<commit_message>
Master system update 2026-05-15 13:18
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1895 +568,1895 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>68.12</v>
+        <v>84.66</v>
       </c>
       <c r="C2" t="n">
-        <v>72.28</v>
+        <v>85.98</v>
       </c>
       <c r="D2" t="n">
-        <v>68.12</v>
+        <v>79.76000000000001</v>
       </c>
       <c r="E2" t="n">
-        <v>71.98</v>
+        <v>85.95999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>48.02</v>
+        <v>53.57</v>
       </c>
       <c r="G2" t="n">
-        <v>49.09</v>
+        <v>55.74</v>
       </c>
       <c r="H2" t="n">
-        <v>47.31</v>
+        <v>53.33</v>
       </c>
       <c r="I2" t="n">
-        <v>48.96</v>
+        <v>55.65</v>
       </c>
       <c r="J2" t="n">
-        <v>26.76</v>
+        <v>21.23</v>
       </c>
       <c r="K2" t="n">
-        <v>26.76</v>
+        <v>22.43</v>
       </c>
       <c r="L2" t="n">
-        <v>25.09</v>
+        <v>20.9</v>
       </c>
       <c r="M2" t="n">
-        <v>25.2</v>
+        <v>20.94</v>
       </c>
       <c r="N2" t="n">
-        <v>69.31999999999999</v>
+        <v>61.88</v>
       </c>
       <c r="O2" t="n">
-        <v>70.3</v>
+        <v>62.15</v>
       </c>
       <c r="P2" t="n">
-        <v>67.72</v>
+        <v>59.35</v>
       </c>
       <c r="Q2" t="n">
-        <v>67.86</v>
+        <v>59.44</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>74.3</v>
+        <v>85.01000000000001</v>
       </c>
       <c r="C3" t="n">
-        <v>78.3</v>
+        <v>89.39</v>
       </c>
       <c r="D3" t="n">
-        <v>74.3</v>
+        <v>83.31</v>
       </c>
       <c r="E3" t="n">
-        <v>76.39</v>
+        <v>88.37</v>
       </c>
       <c r="F3" t="n">
-        <v>49.36</v>
+        <v>56.13</v>
       </c>
       <c r="G3" t="n">
-        <v>49.81</v>
+        <v>56.92</v>
       </c>
       <c r="H3" t="n">
-        <v>48.82</v>
+        <v>55.1</v>
       </c>
       <c r="I3" t="n">
-        <v>49.17</v>
+        <v>56.43</v>
       </c>
       <c r="J3" t="n">
-        <v>24.38</v>
+        <v>21.13</v>
       </c>
       <c r="K3" t="n">
-        <v>24.42</v>
+        <v>21.56</v>
       </c>
       <c r="L3" t="n">
-        <v>23.01</v>
+        <v>20.07</v>
       </c>
       <c r="M3" t="n">
-        <v>23.69</v>
+        <v>20.28</v>
       </c>
       <c r="N3" t="n">
-        <v>67.38</v>
+        <v>58.95</v>
       </c>
       <c r="O3" t="n">
-        <v>68.13</v>
+        <v>60.06</v>
       </c>
       <c r="P3" t="n">
-        <v>66.75</v>
+        <v>58.11</v>
       </c>
       <c r="Q3" t="n">
-        <v>67.62</v>
+        <v>58.61</v>
       </c>
       <c r="R3" t="n">
-        <v>6.1267</v>
+        <v>2.8036</v>
       </c>
       <c r="U3" t="n">
-        <v>0.4289</v>
+        <v>1.4016</v>
       </c>
       <c r="X3" t="n">
-        <v>-5.9921</v>
+        <v>-3.1519</v>
       </c>
       <c r="AA3" t="n">
-        <v>-0.3537</v>
+        <v>-1.3964</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>75.59</v>
+        <v>93.2</v>
       </c>
       <c r="C4" t="n">
-        <v>80.73999999999999</v>
+        <v>94.75</v>
       </c>
       <c r="D4" t="n">
-        <v>75.25</v>
+        <v>90.66</v>
       </c>
       <c r="E4" t="n">
-        <v>80.56</v>
+        <v>94.68000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>48.78</v>
+        <v>57.78</v>
       </c>
       <c r="G4" t="n">
-        <v>50.74</v>
+        <v>58.94</v>
       </c>
       <c r="H4" t="n">
-        <v>48.46</v>
+        <v>57.37</v>
       </c>
       <c r="I4" t="n">
-        <v>50.66</v>
+        <v>58.59</v>
       </c>
       <c r="J4" t="n">
-        <v>23.92</v>
+        <v>19.23</v>
       </c>
       <c r="K4" t="n">
-        <v>24.03</v>
+        <v>19.8</v>
       </c>
       <c r="L4" t="n">
-        <v>22.32</v>
+        <v>18.86</v>
       </c>
       <c r="M4" t="n">
-        <v>22.42</v>
+        <v>18.87</v>
       </c>
       <c r="N4" t="n">
-        <v>68.2</v>
+        <v>57.25</v>
       </c>
       <c r="O4" t="n">
-        <v>68.63</v>
+        <v>57.67</v>
       </c>
       <c r="P4" t="n">
-        <v>65.5</v>
+        <v>56.04</v>
       </c>
       <c r="Q4" t="n">
-        <v>65.56999999999999</v>
+        <v>56.39</v>
       </c>
       <c r="R4" t="n">
-        <v>5.4588</v>
+        <v>7.1404</v>
       </c>
       <c r="U4" t="n">
-        <v>3.0303</v>
+        <v>3.8278</v>
       </c>
       <c r="X4" t="n">
-        <v>-5.3609</v>
+        <v>-6.9527</v>
       </c>
       <c r="AA4" t="n">
-        <v>-3.0316</v>
+        <v>-3.7877</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>83.27</v>
+        <v>95.97</v>
       </c>
       <c r="C5" t="n">
-        <v>85.56999999999999</v>
+        <v>96.93000000000001</v>
       </c>
       <c r="D5" t="n">
-        <v>80.70999999999999</v>
+        <v>92.03</v>
       </c>
       <c r="E5" t="n">
-        <v>85.31</v>
+        <v>95.94</v>
       </c>
       <c r="F5" t="n">
-        <v>51.39</v>
+        <v>58.4</v>
       </c>
       <c r="G5" t="n">
-        <v>53.43</v>
+        <v>58.58</v>
       </c>
       <c r="H5" t="n">
-        <v>51.38</v>
+        <v>56.91</v>
       </c>
       <c r="I5" t="n">
-        <v>53.41</v>
+        <v>58.08</v>
       </c>
       <c r="J5" t="n">
-        <v>21.6</v>
+        <v>18.64</v>
       </c>
       <c r="K5" t="n">
-        <v>22.34</v>
+        <v>19.41</v>
       </c>
       <c r="L5" t="n">
-        <v>21</v>
+        <v>18.44</v>
       </c>
       <c r="M5" t="n">
-        <v>21.05</v>
+        <v>18.63</v>
       </c>
       <c r="N5" t="n">
-        <v>64.67</v>
+        <v>56.59</v>
       </c>
       <c r="O5" t="n">
-        <v>64.68000000000001</v>
+        <v>58.04</v>
       </c>
       <c r="P5" t="n">
-        <v>62.02</v>
+        <v>56.41</v>
       </c>
       <c r="Q5" t="n">
-        <v>62.02</v>
+        <v>56.91</v>
       </c>
       <c r="R5" t="n">
-        <v>5.8962</v>
+        <v>1.3308</v>
       </c>
       <c r="S5" t="n">
-        <v>18.519</v>
+        <v>11.6101</v>
       </c>
       <c r="U5" t="n">
-        <v>5.4283</v>
+        <v>-0.8705000000000001</v>
       </c>
       <c r="V5" t="n">
-        <v>9.0891</v>
+        <v>4.3666</v>
       </c>
       <c r="X5" t="n">
-        <v>-6.1106</v>
+        <v>-1.2719</v>
       </c>
       <c r="Y5" t="n">
-        <v>-16.4683</v>
+        <v>-11.0315</v>
       </c>
       <c r="AA5" t="n">
-        <v>-5.4141</v>
+        <v>0.9221</v>
       </c>
       <c r="AB5" t="n">
-        <v>-8.606</v>
+        <v>-4.2564</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>84.66</v>
+        <v>97.97</v>
       </c>
       <c r="C6" t="n">
-        <v>85.98</v>
+        <v>99.95</v>
       </c>
       <c r="D6" t="n">
-        <v>79.76000000000001</v>
+        <v>95.31999999999999</v>
       </c>
       <c r="E6" t="n">
-        <v>85.95999999999999</v>
+        <v>98.09</v>
       </c>
       <c r="F6" t="n">
-        <v>53.57</v>
+        <v>58.48</v>
       </c>
       <c r="G6" t="n">
-        <v>55.74</v>
+        <v>58.97</v>
       </c>
       <c r="H6" t="n">
-        <v>53.33</v>
+        <v>56.82</v>
       </c>
       <c r="I6" t="n">
-        <v>55.65</v>
+        <v>57.4</v>
       </c>
       <c r="J6" t="n">
-        <v>21.23</v>
+        <v>18.25</v>
       </c>
       <c r="K6" t="n">
-        <v>22.43</v>
+        <v>18.76</v>
       </c>
       <c r="L6" t="n">
-        <v>20.9</v>
+        <v>17.85</v>
       </c>
       <c r="M6" t="n">
-        <v>20.94</v>
+        <v>18.2</v>
       </c>
       <c r="N6" t="n">
-        <v>61.88</v>
+        <v>56.52</v>
       </c>
       <c r="O6" t="n">
-        <v>62.15</v>
+        <v>58.15</v>
       </c>
       <c r="P6" t="n">
-        <v>59.35</v>
+        <v>56.04</v>
       </c>
       <c r="Q6" t="n">
-        <v>59.44</v>
+        <v>57.59</v>
       </c>
       <c r="R6" t="n">
-        <v>0.7619</v>
+        <v>2.241</v>
       </c>
       <c r="S6" t="n">
-        <v>12.5278</v>
+        <v>10.9992</v>
       </c>
       <c r="U6" t="n">
-        <v>4.194</v>
+        <v>-1.1708</v>
       </c>
       <c r="V6" t="n">
-        <v>13.1788</v>
+        <v>1.7189</v>
       </c>
       <c r="X6" t="n">
-        <v>-0.5226</v>
+        <v>-2.3081</v>
       </c>
       <c r="Y6" t="n">
-        <v>-11.6083</v>
+        <v>-10.2564</v>
       </c>
       <c r="AA6" t="n">
-        <v>-4.1599</v>
+        <v>1.1949</v>
       </c>
       <c r="AB6" t="n">
-        <v>-12.097</v>
+        <v>-1.7403</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>85.01000000000001</v>
+        <v>102.94</v>
       </c>
       <c r="C7" t="n">
-        <v>89.39</v>
+        <v>106.09</v>
       </c>
       <c r="D7" t="n">
-        <v>83.31</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="E7" t="n">
-        <v>88.37</v>
+        <v>105.64</v>
       </c>
       <c r="F7" t="n">
-        <v>56.13</v>
+        <v>58.93</v>
       </c>
       <c r="G7" t="n">
-        <v>56.92</v>
+        <v>60.3</v>
       </c>
       <c r="H7" t="n">
-        <v>55.1</v>
+        <v>58.49</v>
       </c>
       <c r="I7" t="n">
-        <v>56.43</v>
+        <v>60.21</v>
       </c>
       <c r="J7" t="n">
-        <v>21.13</v>
+        <v>17.37</v>
       </c>
       <c r="K7" t="n">
-        <v>21.56</v>
+        <v>17.95</v>
       </c>
       <c r="L7" t="n">
-        <v>20.07</v>
+        <v>16.72</v>
       </c>
       <c r="M7" t="n">
-        <v>20.28</v>
+        <v>16.8</v>
       </c>
       <c r="N7" t="n">
-        <v>58.95</v>
+        <v>56.05</v>
       </c>
       <c r="O7" t="n">
-        <v>60.06</v>
+        <v>56.49</v>
       </c>
       <c r="P7" t="n">
-        <v>58.11</v>
+        <v>54.66</v>
       </c>
       <c r="Q7" t="n">
-        <v>58.61</v>
+        <v>54.73</v>
       </c>
       <c r="R7" t="n">
-        <v>2.8036</v>
+        <v>7.697</v>
       </c>
       <c r="S7" t="n">
-        <v>9.694599999999999</v>
+        <v>11.5758</v>
       </c>
       <c r="T7" t="n">
-        <v>22.7702</v>
+        <v>22.8944</v>
       </c>
       <c r="U7" t="n">
-        <v>1.4016</v>
+        <v>4.8955</v>
       </c>
       <c r="V7" t="n">
-        <v>11.3897</v>
+        <v>2.765</v>
       </c>
       <c r="W7" t="n">
-        <v>15.2574</v>
+        <v>8.194100000000001</v>
       </c>
       <c r="X7" t="n">
-        <v>-3.1519</v>
+        <v>-7.6923</v>
       </c>
       <c r="Y7" t="n">
-        <v>-9.545</v>
+        <v>-10.9698</v>
       </c>
       <c r="Z7" t="n">
-        <v>-19.5238</v>
+        <v>-19.7708</v>
       </c>
       <c r="AA7" t="n">
-        <v>-1.3964</v>
+        <v>-4.9661</v>
       </c>
       <c r="AB7" t="n">
-        <v>-10.6146</v>
+        <v>-2.9438</v>
       </c>
       <c r="AC7" t="n">
-        <v>-13.631</v>
+        <v>-7.924</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>93.2</v>
+        <v>108.62</v>
       </c>
       <c r="C8" t="n">
-        <v>94.75</v>
+        <v>116.77</v>
       </c>
       <c r="D8" t="n">
-        <v>90.66</v>
+        <v>107.46</v>
       </c>
       <c r="E8" t="n">
-        <v>94.68000000000001</v>
+        <v>112.77</v>
       </c>
       <c r="F8" t="n">
-        <v>57.78</v>
+        <v>59.8</v>
       </c>
       <c r="G8" t="n">
-        <v>58.94</v>
+        <v>60.73</v>
       </c>
       <c r="H8" t="n">
-        <v>57.37</v>
+        <v>57.59</v>
       </c>
       <c r="I8" t="n">
-        <v>58.59</v>
+        <v>59.22</v>
       </c>
       <c r="J8" t="n">
-        <v>19.23</v>
+        <v>16.35</v>
       </c>
       <c r="K8" t="n">
-        <v>19.8</v>
+        <v>16.52</v>
       </c>
       <c r="L8" t="n">
-        <v>18.86</v>
+        <v>15.06</v>
       </c>
       <c r="M8" t="n">
-        <v>18.87</v>
+        <v>15.7</v>
       </c>
       <c r="N8" t="n">
-        <v>57.25</v>
+        <v>55.13</v>
       </c>
       <c r="O8" t="n">
-        <v>57.67</v>
+        <v>57.14</v>
       </c>
       <c r="P8" t="n">
-        <v>56.04</v>
+        <v>54.28</v>
       </c>
       <c r="Q8" t="n">
-        <v>56.39</v>
+        <v>55.66</v>
       </c>
       <c r="R8" t="n">
-        <v>7.1404</v>
+        <v>6.7493</v>
       </c>
       <c r="S8" t="n">
-        <v>10.9835</v>
+        <v>17.5422</v>
       </c>
       <c r="T8" t="n">
-        <v>23.9429</v>
+        <v>27.6112</v>
       </c>
       <c r="U8" t="n">
-        <v>3.8278</v>
+        <v>-1.6442</v>
       </c>
       <c r="V8" t="n">
-        <v>9.698600000000001</v>
+        <v>1.9628</v>
       </c>
       <c r="W8" t="n">
-        <v>19.158</v>
+        <v>4.9442</v>
       </c>
       <c r="X8" t="n">
-        <v>-6.9527</v>
+        <v>-6.5476</v>
       </c>
       <c r="Y8" t="n">
-        <v>-10.3563</v>
+        <v>-15.7273</v>
       </c>
       <c r="Z8" t="n">
-        <v>-20.3461</v>
+        <v>-22.5838</v>
       </c>
       <c r="AA8" t="n">
-        <v>-3.7877</v>
+        <v>1.6993</v>
       </c>
       <c r="AB8" t="n">
-        <v>-9.0777</v>
+        <v>-2.1965</v>
       </c>
       <c r="AC8" t="n">
-        <v>-16.6075</v>
+        <v>-5.0333</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>95.97</v>
+        <v>125.21</v>
       </c>
       <c r="C9" t="n">
-        <v>96.93000000000001</v>
+        <v>130.12</v>
       </c>
       <c r="D9" t="n">
-        <v>92.03</v>
+        <v>120.24</v>
       </c>
       <c r="E9" t="n">
-        <v>95.94</v>
+        <v>128.32</v>
       </c>
       <c r="F9" t="n">
-        <v>58.4</v>
+        <v>61.08</v>
       </c>
       <c r="G9" t="n">
-        <v>58.58</v>
+        <v>62.74</v>
       </c>
       <c r="H9" t="n">
-        <v>56.91</v>
+        <v>60.56</v>
       </c>
       <c r="I9" t="n">
-        <v>58.08</v>
+        <v>62.56</v>
       </c>
       <c r="J9" t="n">
-        <v>18.64</v>
+        <v>13.99</v>
       </c>
       <c r="K9" t="n">
-        <v>19.41</v>
+        <v>14.66</v>
       </c>
       <c r="L9" t="n">
-        <v>18.44</v>
+        <v>13.3</v>
       </c>
       <c r="M9" t="n">
-        <v>18.63</v>
+        <v>13.52</v>
       </c>
       <c r="N9" t="n">
-        <v>56.59</v>
+        <v>53.93</v>
       </c>
       <c r="O9" t="n">
-        <v>58.04</v>
+        <v>54.43</v>
       </c>
       <c r="P9" t="n">
-        <v>56.41</v>
+        <v>52.37</v>
       </c>
       <c r="Q9" t="n">
-        <v>56.91</v>
+        <v>52.5</v>
       </c>
       <c r="R9" t="n">
-        <v>1.3308</v>
+        <v>13.7891</v>
       </c>
       <c r="S9" t="n">
-        <v>11.6101</v>
+        <v>30.8186</v>
       </c>
       <c r="T9" t="n">
-        <v>19.0914</v>
+        <v>35.5302</v>
       </c>
       <c r="U9" t="n">
-        <v>-0.8705000000000001</v>
+        <v>5.64</v>
       </c>
       <c r="V9" t="n">
-        <v>4.3666</v>
+        <v>8.9895</v>
       </c>
       <c r="W9" t="n">
-        <v>14.6467</v>
+        <v>6.7759</v>
       </c>
       <c r="X9" t="n">
-        <v>-1.2719</v>
+        <v>-13.8854</v>
       </c>
       <c r="Y9" t="n">
-        <v>-11.0315</v>
+        <v>-25.7143</v>
       </c>
       <c r="Z9" t="n">
-        <v>-16.9045</v>
+        <v>-28.3519</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.9221</v>
+        <v>-5.6773</v>
       </c>
       <c r="AB9" t="n">
-        <v>-4.2564</v>
+        <v>-8.8383</v>
       </c>
       <c r="AC9" t="n">
-        <v>-13.2073</v>
+        <v>-6.8984</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>97.97</v>
+        <v>128.33</v>
       </c>
       <c r="C10" t="n">
-        <v>99.95</v>
+        <v>129.59</v>
       </c>
       <c r="D10" t="n">
-        <v>95.31999999999999</v>
+        <v>117.79</v>
       </c>
       <c r="E10" t="n">
-        <v>98.09</v>
+        <v>123.39</v>
       </c>
       <c r="F10" t="n">
-        <v>58.48</v>
+        <v>62.41</v>
       </c>
       <c r="G10" t="n">
-        <v>58.97</v>
+        <v>62.7</v>
       </c>
       <c r="H10" t="n">
-        <v>56.82</v>
+        <v>61.64</v>
       </c>
       <c r="I10" t="n">
-        <v>57.4</v>
+        <v>62.64</v>
       </c>
       <c r="J10" t="n">
-        <v>18.25</v>
+        <v>13.51</v>
       </c>
       <c r="K10" t="n">
-        <v>18.76</v>
+        <v>14.63</v>
       </c>
       <c r="L10" t="n">
-        <v>17.85</v>
+        <v>13.41</v>
       </c>
       <c r="M10" t="n">
-        <v>18.2</v>
+        <v>14.03</v>
       </c>
       <c r="N10" t="n">
-        <v>56.52</v>
+        <v>52.67</v>
       </c>
       <c r="O10" t="n">
-        <v>58.15</v>
+        <v>53.31</v>
       </c>
       <c r="P10" t="n">
-        <v>56.04</v>
+        <v>52.42</v>
       </c>
       <c r="Q10" t="n">
-        <v>57.59</v>
+        <v>52.45</v>
       </c>
       <c r="R10" t="n">
-        <v>2.241</v>
+        <v>-3.842</v>
       </c>
       <c r="S10" t="n">
-        <v>10.9992</v>
+        <v>16.8023</v>
       </c>
       <c r="T10" t="n">
-        <v>14.9807</v>
+        <v>28.6116</v>
       </c>
       <c r="U10" t="n">
-        <v>-1.1708</v>
+        <v>0.1279</v>
       </c>
       <c r="V10" t="n">
-        <v>1.7189</v>
+        <v>4.0359</v>
       </c>
       <c r="W10" t="n">
-        <v>7.4705</v>
+        <v>7.8512</v>
       </c>
       <c r="X10" t="n">
-        <v>-2.3081</v>
+        <v>3.7722</v>
       </c>
       <c r="Y10" t="n">
-        <v>-10.2564</v>
+        <v>-16.4881</v>
       </c>
       <c r="Z10" t="n">
-        <v>-13.5392</v>
+        <v>-24.6914</v>
       </c>
       <c r="AA10" t="n">
-        <v>1.1949</v>
+        <v>-0.09520000000000001</v>
       </c>
       <c r="AB10" t="n">
-        <v>-1.7403</v>
+        <v>-4.1659</v>
       </c>
       <c r="AC10" t="n">
-        <v>-7.1429</v>
+        <v>-7.8369</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>102.94</v>
+        <v>108.75</v>
       </c>
       <c r="C11" t="n">
-        <v>106.09</v>
+        <v>115.62</v>
       </c>
       <c r="D11" t="n">
-        <v>99.59999999999999</v>
+        <v>103.99</v>
       </c>
       <c r="E11" t="n">
-        <v>105.64</v>
+        <v>109.56</v>
       </c>
       <c r="F11" t="n">
-        <v>58.93</v>
+        <v>60.72</v>
       </c>
       <c r="G11" t="n">
-        <v>60.3</v>
+        <v>61.33</v>
       </c>
       <c r="H11" t="n">
-        <v>58.49</v>
+        <v>59.68</v>
       </c>
       <c r="I11" t="n">
-        <v>60.21</v>
+        <v>60.74</v>
       </c>
       <c r="J11" t="n">
-        <v>17.37</v>
+        <v>15.71</v>
       </c>
       <c r="K11" t="n">
-        <v>17.95</v>
+        <v>16.27</v>
       </c>
       <c r="L11" t="n">
-        <v>16.72</v>
+        <v>14.93</v>
       </c>
       <c r="M11" t="n">
-        <v>16.8</v>
+        <v>15.59</v>
       </c>
       <c r="N11" t="n">
-        <v>56.05</v>
+        <v>54.09</v>
       </c>
       <c r="O11" t="n">
-        <v>56.49</v>
+        <v>54.96</v>
       </c>
       <c r="P11" t="n">
-        <v>54.66</v>
+        <v>53.58</v>
       </c>
       <c r="Q11" t="n">
-        <v>54.73</v>
+        <v>54.05</v>
       </c>
       <c r="R11" t="n">
-        <v>7.697</v>
+        <v>-11.2084</v>
       </c>
       <c r="S11" t="n">
-        <v>11.5758</v>
+        <v>-2.8465</v>
       </c>
       <c r="T11" t="n">
-        <v>22.8944</v>
+        <v>11.6933</v>
       </c>
       <c r="U11" t="n">
-        <v>4.8955</v>
+        <v>-3.0332</v>
       </c>
       <c r="V11" t="n">
-        <v>2.765</v>
+        <v>2.5667</v>
       </c>
       <c r="W11" t="n">
-        <v>8.194100000000001</v>
+        <v>5.8188</v>
       </c>
       <c r="X11" t="n">
-        <v>-7.6923</v>
+        <v>11.119</v>
       </c>
       <c r="Y11" t="n">
-        <v>-10.9698</v>
+        <v>-0.7006</v>
       </c>
       <c r="Z11" t="n">
-        <v>-19.7708</v>
+        <v>-14.3407</v>
       </c>
       <c r="AA11" t="n">
-        <v>-4.9661</v>
+        <v>3.0505</v>
       </c>
       <c r="AB11" t="n">
-        <v>-2.9438</v>
+        <v>-2.8926</v>
       </c>
       <c r="AC11" t="n">
-        <v>-7.924</v>
+        <v>-6.1469</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>108.62</v>
+        <v>114.76</v>
       </c>
       <c r="C12" t="n">
-        <v>116.77</v>
+        <v>118.32</v>
       </c>
       <c r="D12" t="n">
-        <v>107.46</v>
+        <v>112.3</v>
       </c>
       <c r="E12" t="n">
-        <v>112.77</v>
+        <v>117.97</v>
       </c>
       <c r="F12" t="n">
-        <v>59.8</v>
+        <v>61</v>
       </c>
       <c r="G12" t="n">
-        <v>60.73</v>
+        <v>61.87</v>
       </c>
       <c r="H12" t="n">
-        <v>57.59</v>
+        <v>60.45</v>
       </c>
       <c r="I12" t="n">
-        <v>59.22</v>
+        <v>61.86</v>
       </c>
       <c r="J12" t="n">
-        <v>16.35</v>
+        <v>14.91</v>
       </c>
       <c r="K12" t="n">
-        <v>16.52</v>
+        <v>15.24</v>
       </c>
       <c r="L12" t="n">
-        <v>15.06</v>
+        <v>14.38</v>
       </c>
       <c r="M12" t="n">
-        <v>15.7</v>
+        <v>14.4</v>
       </c>
       <c r="N12" t="n">
-        <v>55.13</v>
+        <v>53.84</v>
       </c>
       <c r="O12" t="n">
-        <v>57.14</v>
+        <v>54.33</v>
       </c>
       <c r="P12" t="n">
-        <v>54.28</v>
+        <v>53.06</v>
       </c>
       <c r="Q12" t="n">
-        <v>55.66</v>
+        <v>53.08</v>
       </c>
       <c r="R12" t="n">
-        <v>6.7493</v>
+        <v>7.6762</v>
       </c>
       <c r="S12" t="n">
-        <v>17.5422</v>
+        <v>-8.065799999999999</v>
       </c>
       <c r="T12" t="n">
-        <v>27.6112</v>
+        <v>11.6717</v>
       </c>
       <c r="U12" t="n">
-        <v>-1.6442</v>
+        <v>1.8439</v>
       </c>
       <c r="V12" t="n">
-        <v>1.9628</v>
+        <v>-1.1189</v>
       </c>
       <c r="W12" t="n">
-        <v>4.9442</v>
+        <v>2.7404</v>
       </c>
       <c r="X12" t="n">
-        <v>-6.5476</v>
+        <v>-7.6331</v>
       </c>
       <c r="Y12" t="n">
-        <v>-15.7273</v>
+        <v>6.5089</v>
       </c>
       <c r="Z12" t="n">
-        <v>-22.5838</v>
+        <v>-14.2857</v>
       </c>
       <c r="AA12" t="n">
-        <v>1.6993</v>
+        <v>-1.7946</v>
       </c>
       <c r="AB12" t="n">
-        <v>-2.1965</v>
+        <v>1.1048</v>
       </c>
       <c r="AC12" t="n">
-        <v>-5.0333</v>
+        <v>-3.0148</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>125.21</v>
+        <v>122.81</v>
       </c>
       <c r="C13" t="n">
-        <v>130.12</v>
+        <v>127.45</v>
       </c>
       <c r="D13" t="n">
-        <v>120.24</v>
+        <v>117.5</v>
       </c>
       <c r="E13" t="n">
-        <v>128.32</v>
+        <v>126.98</v>
       </c>
       <c r="F13" t="n">
-        <v>61.08</v>
+        <v>62.89</v>
       </c>
       <c r="G13" t="n">
-        <v>62.74</v>
+        <v>63.8</v>
       </c>
       <c r="H13" t="n">
-        <v>60.56</v>
+        <v>60.7</v>
       </c>
       <c r="I13" t="n">
-        <v>62.56</v>
+        <v>63.54</v>
       </c>
       <c r="J13" t="n">
-        <v>13.99</v>
+        <v>13.84</v>
       </c>
       <c r="K13" t="n">
-        <v>14.66</v>
+        <v>14.49</v>
       </c>
       <c r="L13" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="M13" t="n">
         <v>13.3</v>
       </c>
-      <c r="M13" t="n">
-        <v>13.52</v>
-      </c>
       <c r="N13" t="n">
-        <v>53.93</v>
+        <v>52.21</v>
       </c>
       <c r="O13" t="n">
-        <v>54.43</v>
+        <v>54.09</v>
       </c>
       <c r="P13" t="n">
-        <v>52.37</v>
+        <v>51.4</v>
       </c>
       <c r="Q13" t="n">
-        <v>52.5</v>
+        <v>51.65</v>
       </c>
       <c r="R13" t="n">
-        <v>13.7891</v>
+        <v>7.6375</v>
       </c>
       <c r="S13" t="n">
-        <v>30.8186</v>
+        <v>2.9095</v>
       </c>
       <c r="T13" t="n">
-        <v>35.5302</v>
+        <v>12.6009</v>
       </c>
       <c r="U13" t="n">
-        <v>5.64</v>
+        <v>2.7158</v>
       </c>
       <c r="V13" t="n">
-        <v>8.9895</v>
+        <v>1.4368</v>
       </c>
       <c r="W13" t="n">
-        <v>6.7759</v>
+        <v>7.2948</v>
       </c>
       <c r="X13" t="n">
-        <v>-13.8854</v>
+        <v>-7.6389</v>
       </c>
       <c r="Y13" t="n">
-        <v>-25.7143</v>
+        <v>-5.2031</v>
       </c>
       <c r="Z13" t="n">
-        <v>-28.3519</v>
+        <v>-15.2866</v>
       </c>
       <c r="AA13" t="n">
-        <v>-5.6773</v>
+        <v>-2.694</v>
       </c>
       <c r="AB13" t="n">
-        <v>-8.8383</v>
+        <v>-1.5253</v>
       </c>
       <c r="AC13" t="n">
-        <v>-6.8984</v>
+        <v>-7.2045</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>128.33</v>
+        <v>124.39</v>
       </c>
       <c r="C14" t="n">
-        <v>129.59</v>
+        <v>131.38</v>
       </c>
       <c r="D14" t="n">
-        <v>117.79</v>
+        <v>121.66</v>
       </c>
       <c r="E14" t="n">
-        <v>123.39</v>
+        <v>130.4</v>
       </c>
       <c r="F14" t="n">
-        <v>62.41</v>
+        <v>63.89</v>
       </c>
       <c r="G14" t="n">
-        <v>62.7</v>
+        <v>65.84</v>
       </c>
       <c r="H14" t="n">
-        <v>61.64</v>
+        <v>63.81</v>
       </c>
       <c r="I14" t="n">
-        <v>62.64</v>
+        <v>65.3</v>
       </c>
       <c r="J14" t="n">
-        <v>13.51</v>
+        <v>13.61</v>
       </c>
       <c r="K14" t="n">
-        <v>14.63</v>
+        <v>13.89</v>
       </c>
       <c r="L14" t="n">
-        <v>13.41</v>
+        <v>12.87</v>
       </c>
       <c r="M14" t="n">
-        <v>14.03</v>
+        <v>12.98</v>
       </c>
       <c r="N14" t="n">
-        <v>52.67</v>
+        <v>51.36</v>
       </c>
       <c r="O14" t="n">
-        <v>53.31</v>
+        <v>51.45</v>
       </c>
       <c r="P14" t="n">
-        <v>52.42</v>
+        <v>49.79</v>
       </c>
       <c r="Q14" t="n">
-        <v>52.45</v>
+        <v>50.22</v>
       </c>
       <c r="R14" t="n">
-        <v>-3.842</v>
+        <v>2.6933</v>
       </c>
       <c r="S14" t="n">
-        <v>16.8023</v>
+        <v>19.0215</v>
       </c>
       <c r="T14" t="n">
-        <v>28.6116</v>
+        <v>1.6209</v>
       </c>
       <c r="U14" t="n">
-        <v>0.1279</v>
+        <v>2.7699</v>
       </c>
       <c r="V14" t="n">
-        <v>4.0359</v>
+        <v>7.5074</v>
       </c>
       <c r="W14" t="n">
-        <v>7.8512</v>
+        <v>4.3798</v>
       </c>
       <c r="X14" t="n">
-        <v>3.7722</v>
+        <v>-2.406</v>
       </c>
       <c r="Y14" t="n">
-        <v>-16.4881</v>
+        <v>-16.7415</v>
       </c>
       <c r="Z14" t="n">
-        <v>-24.6914</v>
+        <v>-3.9941</v>
       </c>
       <c r="AA14" t="n">
-        <v>-0.09520000000000001</v>
+        <v>-2.7686</v>
       </c>
       <c r="AB14" t="n">
-        <v>-4.1659</v>
+        <v>-7.086</v>
       </c>
       <c r="AC14" t="n">
-        <v>-7.8369</v>
+        <v>-4.3429</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>108.75</v>
+        <v>132.2</v>
       </c>
       <c r="C15" t="n">
-        <v>115.62</v>
+        <v>133.67</v>
       </c>
       <c r="D15" t="n">
-        <v>103.99</v>
+        <v>123.8</v>
       </c>
       <c r="E15" t="n">
-        <v>109.56</v>
+        <v>127.55</v>
       </c>
       <c r="F15" t="n">
-        <v>60.72</v>
+        <v>65.44</v>
       </c>
       <c r="G15" t="n">
-        <v>61.33</v>
+        <v>66.05</v>
       </c>
       <c r="H15" t="n">
-        <v>59.68</v>
+        <v>63.78</v>
       </c>
       <c r="I15" t="n">
-        <v>60.74</v>
+        <v>64.91</v>
       </c>
       <c r="J15" t="n">
-        <v>15.71</v>
+        <v>12.8</v>
       </c>
       <c r="K15" t="n">
-        <v>16.27</v>
+        <v>13.64</v>
       </c>
       <c r="L15" t="n">
-        <v>14.93</v>
+        <v>12.65</v>
       </c>
       <c r="M15" t="n">
-        <v>15.59</v>
+        <v>13.26</v>
       </c>
       <c r="N15" t="n">
-        <v>54.09</v>
+        <v>50.12</v>
       </c>
       <c r="O15" t="n">
-        <v>54.96</v>
+        <v>51.43</v>
       </c>
       <c r="P15" t="n">
-        <v>53.58</v>
+        <v>49.65</v>
       </c>
       <c r="Q15" t="n">
-        <v>54.05</v>
+        <v>50.51</v>
       </c>
       <c r="R15" t="n">
-        <v>-11.2084</v>
+        <v>-2.1856</v>
       </c>
       <c r="S15" t="n">
-        <v>-2.8465</v>
+        <v>8.120699999999999</v>
       </c>
       <c r="T15" t="n">
-        <v>11.6933</v>
+        <v>3.3714</v>
       </c>
       <c r="U15" t="n">
-        <v>-3.0332</v>
+        <v>-0.5972</v>
       </c>
       <c r="V15" t="n">
-        <v>2.5667</v>
+        <v>4.9305</v>
       </c>
       <c r="W15" t="n">
-        <v>5.8188</v>
+        <v>3.6239</v>
       </c>
       <c r="X15" t="n">
-        <v>11.119</v>
+        <v>2.1572</v>
       </c>
       <c r="Y15" t="n">
-        <v>-0.7006</v>
+        <v>-7.9167</v>
       </c>
       <c r="Z15" t="n">
-        <v>-14.3407</v>
+        <v>-5.4882</v>
       </c>
       <c r="AA15" t="n">
-        <v>3.0505</v>
+        <v>0.5775</v>
       </c>
       <c r="AB15" t="n">
-        <v>-2.8926</v>
+        <v>-4.8417</v>
       </c>
       <c r="AC15" t="n">
-        <v>-6.1469</v>
+        <v>-3.6988</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>114.76</v>
+        <v>135</v>
       </c>
       <c r="C16" t="n">
-        <v>118.32</v>
+        <v>147.26</v>
       </c>
       <c r="D16" t="n">
-        <v>112.3</v>
+        <v>134.02</v>
       </c>
       <c r="E16" t="n">
-        <v>117.97</v>
+        <v>144.16</v>
       </c>
       <c r="F16" t="n">
-        <v>61</v>
+        <v>66.37</v>
       </c>
       <c r="G16" t="n">
-        <v>61.87</v>
+        <v>67.77</v>
       </c>
       <c r="H16" t="n">
-        <v>60.45</v>
+        <v>66.25</v>
       </c>
       <c r="I16" t="n">
-        <v>61.86</v>
+        <v>67.39</v>
       </c>
       <c r="J16" t="n">
-        <v>14.91</v>
+        <v>12.5</v>
       </c>
       <c r="K16" t="n">
-        <v>15.24</v>
+        <v>12.59</v>
       </c>
       <c r="L16" t="n">
-        <v>14.38</v>
+        <v>11.21</v>
       </c>
       <c r="M16" t="n">
-        <v>14.4</v>
+        <v>11.51</v>
       </c>
       <c r="N16" t="n">
-        <v>53.84</v>
+        <v>49.4</v>
       </c>
       <c r="O16" t="n">
-        <v>54.33</v>
+        <v>49.49</v>
       </c>
       <c r="P16" t="n">
-        <v>53.06</v>
+        <v>48.3</v>
       </c>
       <c r="Q16" t="n">
-        <v>53.08</v>
+        <v>48.59</v>
       </c>
       <c r="R16" t="n">
-        <v>7.6762</v>
+        <v>13.0223</v>
       </c>
       <c r="S16" t="n">
-        <v>-8.065799999999999</v>
+        <v>13.5297</v>
       </c>
       <c r="T16" t="n">
-        <v>11.6717</v>
+        <v>31.5809</v>
       </c>
       <c r="U16" t="n">
-        <v>1.8439</v>
+        <v>3.8207</v>
       </c>
       <c r="V16" t="n">
-        <v>-1.1189</v>
+        <v>6.0592</v>
       </c>
       <c r="W16" t="n">
-        <v>2.7404</v>
+        <v>10.9483</v>
       </c>
       <c r="X16" t="n">
-        <v>-7.6331</v>
+        <v>-13.1976</v>
       </c>
       <c r="Y16" t="n">
-        <v>6.5089</v>
+        <v>-13.4586</v>
       </c>
       <c r="Z16" t="n">
-        <v>-14.2857</v>
+        <v>-26.1706</v>
       </c>
       <c r="AA16" t="n">
-        <v>-1.7946</v>
+        <v>-3.8012</v>
       </c>
       <c r="AB16" t="n">
-        <v>1.1048</v>
+        <v>-5.9245</v>
       </c>
       <c r="AC16" t="n">
-        <v>-3.0148</v>
+        <v>-10.1018</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>122.81</v>
+        <v>157.84</v>
       </c>
       <c r="C17" t="n">
-        <v>127.45</v>
+        <v>166</v>
       </c>
       <c r="D17" t="n">
-        <v>117.5</v>
+        <v>149.06</v>
       </c>
       <c r="E17" t="n">
-        <v>126.98</v>
+        <v>165.85</v>
       </c>
       <c r="F17" t="n">
-        <v>62.89</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>63.8</v>
+        <v>71.66</v>
       </c>
       <c r="H17" t="n">
-        <v>60.7</v>
+        <v>68.88</v>
       </c>
       <c r="I17" t="n">
-        <v>63.54</v>
+        <v>71.56999999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>13.84</v>
+        <v>10.43</v>
       </c>
       <c r="K17" t="n">
-        <v>14.49</v>
+        <v>11.14</v>
       </c>
       <c r="L17" t="n">
-        <v>13.25</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M17" t="n">
-        <v>13.3</v>
+        <v>9.81</v>
       </c>
       <c r="N17" t="n">
-        <v>52.21</v>
+        <v>47.26</v>
       </c>
       <c r="O17" t="n">
-        <v>54.09</v>
+        <v>47.54</v>
       </c>
       <c r="P17" t="n">
-        <v>51.4</v>
+        <v>45.52</v>
       </c>
       <c r="Q17" t="n">
-        <v>51.65</v>
+        <v>45.59</v>
       </c>
       <c r="R17" t="n">
-        <v>7.6375</v>
+        <v>15.0458</v>
       </c>
       <c r="S17" t="n">
-        <v>2.9095</v>
+        <v>27.1856</v>
       </c>
       <c r="T17" t="n">
-        <v>12.6009</v>
+        <v>40.5866</v>
       </c>
       <c r="U17" t="n">
-        <v>2.7158</v>
+        <v>6.2027</v>
       </c>
       <c r="V17" t="n">
-        <v>1.4368</v>
+        <v>9.601800000000001</v>
       </c>
       <c r="W17" t="n">
-        <v>7.2948</v>
+        <v>15.6967</v>
       </c>
       <c r="X17" t="n">
-        <v>-7.6389</v>
+        <v>-14.7698</v>
       </c>
       <c r="Y17" t="n">
-        <v>-5.2031</v>
+        <v>-24.4222</v>
       </c>
       <c r="Z17" t="n">
-        <v>-15.2866</v>
+        <v>-31.875</v>
       </c>
       <c r="AA17" t="n">
-        <v>-2.694</v>
+        <v>-6.1741</v>
       </c>
       <c r="AB17" t="n">
-        <v>-1.5253</v>
+        <v>-9.2194</v>
       </c>
       <c r="AC17" t="n">
-        <v>-7.2045</v>
+        <v>-14.1108</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>124.39</v>
+        <v>162.12</v>
       </c>
       <c r="C18" t="n">
-        <v>131.38</v>
+        <v>162.9</v>
       </c>
       <c r="D18" t="n">
-        <v>121.66</v>
+        <v>147.61</v>
       </c>
       <c r="E18" t="n">
-        <v>130.4</v>
+        <v>152.1</v>
       </c>
       <c r="F18" t="n">
-        <v>63.89</v>
+        <v>71.87</v>
       </c>
       <c r="G18" t="n">
-        <v>65.84</v>
+        <v>73.3</v>
       </c>
       <c r="H18" t="n">
-        <v>63.81</v>
+        <v>70.38</v>
       </c>
       <c r="I18" t="n">
-        <v>65.3</v>
+        <v>71.34</v>
       </c>
       <c r="J18" t="n">
-        <v>13.61</v>
+        <v>10.02</v>
       </c>
       <c r="K18" t="n">
-        <v>13.89</v>
+        <v>10.88</v>
       </c>
       <c r="L18" t="n">
-        <v>12.87</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="M18" t="n">
-        <v>12.98</v>
+        <v>10.6</v>
       </c>
       <c r="N18" t="n">
-        <v>51.36</v>
+        <v>45.41</v>
       </c>
       <c r="O18" t="n">
-        <v>51.45</v>
+        <v>46.36</v>
       </c>
       <c r="P18" t="n">
-        <v>49.79</v>
+        <v>44.5</v>
       </c>
       <c r="Q18" t="n">
-        <v>50.22</v>
+        <v>45.73</v>
       </c>
       <c r="R18" t="n">
-        <v>2.6933</v>
+        <v>-8.2906</v>
       </c>
       <c r="S18" t="n">
-        <v>19.0215</v>
+        <v>19.2474</v>
       </c>
       <c r="T18" t="n">
-        <v>1.6209</v>
+        <v>19.7826</v>
       </c>
       <c r="U18" t="n">
-        <v>2.7699</v>
+        <v>-0.3214</v>
       </c>
       <c r="V18" t="n">
-        <v>7.5074</v>
+        <v>9.906000000000001</v>
       </c>
       <c r="W18" t="n">
-        <v>4.3798</v>
+        <v>12.2757</v>
       </c>
       <c r="X18" t="n">
-        <v>-2.406</v>
+        <v>8.053000000000001</v>
       </c>
       <c r="Y18" t="n">
-        <v>-16.7415</v>
+        <v>-20.0603</v>
       </c>
       <c r="Z18" t="n">
-        <v>-3.9941</v>
+        <v>-20.3008</v>
       </c>
       <c r="AA18" t="n">
-        <v>-2.7686</v>
+        <v>0.3071</v>
       </c>
       <c r="AB18" t="n">
-        <v>-7.086</v>
+        <v>-9.4635</v>
       </c>
       <c r="AC18" t="n">
-        <v>-4.3429</v>
+        <v>-11.4618</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>132.2</v>
+        <v>163</v>
       </c>
       <c r="C19" t="n">
-        <v>133.67</v>
+        <v>177.5</v>
       </c>
       <c r="D19" t="n">
-        <v>123.8</v>
+        <v>161.51</v>
       </c>
       <c r="E19" t="n">
-        <v>127.55</v>
+        <v>176.94</v>
       </c>
       <c r="F19" t="n">
-        <v>65.44</v>
+        <v>72.81999999999999</v>
       </c>
       <c r="G19" t="n">
-        <v>66.05</v>
+        <v>76.31</v>
       </c>
       <c r="H19" t="n">
-        <v>63.78</v>
+        <v>72.7</v>
       </c>
       <c r="I19" t="n">
-        <v>64.91</v>
+        <v>76.28</v>
       </c>
       <c r="J19" t="n">
-        <v>12.8</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="K19" t="n">
-        <v>13.64</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="L19" t="n">
-        <v>12.65</v>
+        <v>8.84</v>
       </c>
       <c r="M19" t="n">
-        <v>13.26</v>
+        <v>8.85</v>
       </c>
       <c r="N19" t="n">
-        <v>50.12</v>
+        <v>44.82</v>
       </c>
       <c r="O19" t="n">
-        <v>51.43</v>
+        <v>44.89</v>
       </c>
       <c r="P19" t="n">
-        <v>49.65</v>
+        <v>42.57</v>
       </c>
       <c r="Q19" t="n">
-        <v>50.51</v>
+        <v>42.57</v>
       </c>
       <c r="R19" t="n">
-        <v>-2.1856</v>
+        <v>16.3314</v>
       </c>
       <c r="S19" t="n">
-        <v>8.120699999999999</v>
+        <v>22.7386</v>
       </c>
       <c r="T19" t="n">
-        <v>3.3714</v>
+        <v>35.6902</v>
       </c>
       <c r="U19" t="n">
-        <v>-0.5972</v>
+        <v>6.9246</v>
       </c>
       <c r="V19" t="n">
-        <v>4.9305</v>
+        <v>13.1919</v>
       </c>
       <c r="W19" t="n">
-        <v>3.6239</v>
+        <v>16.8147</v>
       </c>
       <c r="X19" t="n">
-        <v>2.1572</v>
+        <v>-16.5094</v>
       </c>
       <c r="Y19" t="n">
-        <v>-7.9167</v>
+        <v>-23.1103</v>
       </c>
       <c r="Z19" t="n">
-        <v>-5.4882</v>
+        <v>-31.8182</v>
       </c>
       <c r="AA19" t="n">
-        <v>0.5775</v>
+        <v>-6.9101</v>
       </c>
       <c r="AB19" t="n">
-        <v>-4.8417</v>
+        <v>-12.3894</v>
       </c>
       <c r="AC19" t="n">
-        <v>-3.6988</v>
+        <v>-15.233</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>135</v>
+        <v>181</v>
       </c>
       <c r="C20" t="n">
-        <v>147.26</v>
+        <v>191.29</v>
       </c>
       <c r="D20" t="n">
-        <v>134.02</v>
+        <v>178.94</v>
       </c>
       <c r="E20" t="n">
-        <v>144.16</v>
+        <v>190.42</v>
       </c>
       <c r="F20" t="n">
-        <v>66.37</v>
+        <v>76</v>
       </c>
       <c r="G20" t="n">
-        <v>67.77</v>
+        <v>77.36</v>
       </c>
       <c r="H20" t="n">
-        <v>66.25</v>
+        <v>75.55</v>
       </c>
       <c r="I20" t="n">
-        <v>67.39</v>
+        <v>76.95999999999999</v>
       </c>
       <c r="J20" t="n">
-        <v>12.5</v>
+        <v>8.65</v>
       </c>
       <c r="K20" t="n">
-        <v>12.59</v>
+        <v>8.77</v>
       </c>
       <c r="L20" t="n">
-        <v>11.21</v>
+        <v>8.15</v>
       </c>
       <c r="M20" t="n">
-        <v>11.51</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="N20" t="n">
-        <v>49.4</v>
+        <v>42.74</v>
       </c>
       <c r="O20" t="n">
-        <v>49.49</v>
+        <v>43</v>
       </c>
       <c r="P20" t="n">
-        <v>48.3</v>
+        <v>41.99</v>
       </c>
       <c r="Q20" t="n">
-        <v>48.59</v>
+        <v>42.22</v>
       </c>
       <c r="R20" t="n">
-        <v>13.0223</v>
+        <v>7.6184</v>
       </c>
       <c r="S20" t="n">
-        <v>13.5297</v>
+        <v>14.8146</v>
       </c>
       <c r="T20" t="n">
-        <v>31.5809</v>
+        <v>49.2905</v>
       </c>
       <c r="U20" t="n">
-        <v>3.8207</v>
+        <v>0.8915</v>
       </c>
       <c r="V20" t="n">
-        <v>6.0592</v>
+        <v>7.5311</v>
       </c>
       <c r="W20" t="n">
-        <v>10.9483</v>
+        <v>18.5642</v>
       </c>
       <c r="X20" t="n">
-        <v>-13.1976</v>
+        <v>-7.3446</v>
       </c>
       <c r="Y20" t="n">
-        <v>-13.4586</v>
+        <v>-16.4118</v>
       </c>
       <c r="Z20" t="n">
-        <v>-26.1706</v>
+        <v>-38.1599</v>
       </c>
       <c r="AA20" t="n">
-        <v>-3.8012</v>
+        <v>-0.8222</v>
       </c>
       <c r="AB20" t="n">
-        <v>-5.9245</v>
+        <v>-7.392</v>
       </c>
       <c r="AC20" t="n">
-        <v>-10.1018</v>
+        <v>-16.4126</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>157.84</v>
+        <v>177.62</v>
       </c>
       <c r="C21" t="n">
-        <v>166</v>
+        <v>182.24</v>
       </c>
       <c r="D21" t="n">
-        <v>149.06</v>
+        <v>150.58</v>
       </c>
       <c r="E21" t="n">
-        <v>165.85</v>
+        <v>172.52</v>
       </c>
       <c r="F21" t="n">
-        <v>69.26000000000001</v>
+        <v>75.3</v>
       </c>
       <c r="G21" t="n">
-        <v>71.66</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="H21" t="n">
-        <v>68.88</v>
+        <v>71.55</v>
       </c>
       <c r="I21" t="n">
-        <v>71.56999999999999</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="J21" t="n">
-        <v>10.43</v>
+        <v>8.75</v>
       </c>
       <c r="K21" t="n">
-        <v>11.14</v>
+        <v>9.91</v>
       </c>
       <c r="L21" t="n">
-        <v>9.800000000000001</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="M21" t="n">
-        <v>9.81</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N21" t="n">
-        <v>47.26</v>
+        <v>43.14</v>
       </c>
       <c r="O21" t="n">
-        <v>47.54</v>
+        <v>45.19</v>
       </c>
       <c r="P21" t="n">
-        <v>45.52</v>
+        <v>42.79</v>
       </c>
       <c r="Q21" t="n">
-        <v>45.59</v>
+        <v>43.31</v>
       </c>
       <c r="R21" t="n">
-        <v>15.0458</v>
+        <v>-9.4003</v>
       </c>
       <c r="S21" t="n">
-        <v>27.1856</v>
+        <v>13.4254</v>
       </c>
       <c r="T21" t="n">
-        <v>40.5866</v>
+        <v>19.6726</v>
       </c>
       <c r="U21" t="n">
-        <v>6.2027</v>
+        <v>-2.5988</v>
       </c>
       <c r="V21" t="n">
-        <v>9.601800000000001</v>
+        <v>5.0743</v>
       </c>
       <c r="W21" t="n">
-        <v>15.6967</v>
+        <v>11.2331</v>
       </c>
       <c r="X21" t="n">
-        <v>-14.7698</v>
+        <v>9.1463</v>
       </c>
       <c r="Y21" t="n">
-        <v>-24.4222</v>
+        <v>-15.566</v>
       </c>
       <c r="Z21" t="n">
-        <v>-31.875</v>
+        <v>-22.2415</v>
       </c>
       <c r="AA21" t="n">
-        <v>-6.1741</v>
+        <v>2.5817</v>
       </c>
       <c r="AB21" t="n">
-        <v>-9.2194</v>
+        <v>-5.2919</v>
       </c>
       <c r="AC21" t="n">
-        <v>-14.1108</v>
+        <v>-10.8664</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>162.12</v>
+        <v>183.84</v>
       </c>
       <c r="C22" t="n">
-        <v>162.9</v>
+        <v>188.49</v>
       </c>
       <c r="D22" t="n">
-        <v>147.61</v>
+        <v>172.26</v>
       </c>
       <c r="E22" t="n">
-        <v>152.1</v>
+        <v>184.24</v>
       </c>
       <c r="F22" t="n">
-        <v>71.87</v>
+        <v>75.81</v>
       </c>
       <c r="G22" t="n">
-        <v>73.3</v>
+        <v>77.94</v>
       </c>
       <c r="H22" t="n">
-        <v>70.38</v>
+        <v>74.19</v>
       </c>
       <c r="I22" t="n">
-        <v>71.34</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="J22" t="n">
-        <v>10.02</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K22" t="n">
-        <v>10.88</v>
+        <v>8.98</v>
       </c>
       <c r="L22" t="n">
-        <v>9.970000000000001</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="M22" t="n">
-        <v>10.6</v>
+        <v>8.35</v>
       </c>
       <c r="N22" t="n">
-        <v>45.41</v>
+        <v>42.83</v>
       </c>
       <c r="O22" t="n">
-        <v>46.36</v>
+        <v>43.77</v>
       </c>
       <c r="P22" t="n">
-        <v>44.5</v>
+        <v>41.6</v>
       </c>
       <c r="Q22" t="n">
-        <v>45.73</v>
+        <v>41.99</v>
       </c>
       <c r="R22" t="n">
-        <v>-8.2906</v>
+        <v>6.7934</v>
       </c>
       <c r="S22" t="n">
-        <v>19.2474</v>
+        <v>4.1257</v>
       </c>
       <c r="T22" t="n">
-        <v>19.7826</v>
+        <v>11.0883</v>
       </c>
       <c r="U22" t="n">
-        <v>-0.3214</v>
+        <v>3.0416</v>
       </c>
       <c r="V22" t="n">
-        <v>9.906000000000001</v>
+        <v>1.2585</v>
       </c>
       <c r="W22" t="n">
-        <v>12.2757</v>
+        <v>7.9223</v>
       </c>
       <c r="X22" t="n">
-        <v>8.053000000000001</v>
+        <v>-6.7039</v>
       </c>
       <c r="Y22" t="n">
-        <v>-20.0603</v>
+        <v>-5.6497</v>
       </c>
       <c r="Z22" t="n">
-        <v>-20.3008</v>
+        <v>-14.8828</v>
       </c>
       <c r="AA22" t="n">
-        <v>0.3071</v>
+        <v>-3.0478</v>
       </c>
       <c r="AB22" t="n">
-        <v>-9.4635</v>
+        <v>-1.3625</v>
       </c>
       <c r="AC22" t="n">
-        <v>-11.4618</v>
+        <v>-7.8965</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>163</v>
+        <v>182.67</v>
       </c>
       <c r="C23" t="n">
-        <v>177.495</v>
+        <v>189.56</v>
       </c>
       <c r="D23" t="n">
-        <v>161.51</v>
+        <v>178.28</v>
       </c>
       <c r="E23" t="n">
-        <v>176.94</v>
+        <v>186.19</v>
       </c>
       <c r="F23" t="n">
-        <v>72.825</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G23" t="n">
-        <v>76.31</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H23" t="n">
-        <v>72.69499999999999</v>
+        <v>77.16</v>
       </c>
       <c r="I23" t="n">
-        <v>76.28</v>
+        <v>78.95</v>
       </c>
       <c r="J23" t="n">
-        <v>9.859999999999999</v>
+        <v>8.43</v>
       </c>
       <c r="K23" t="n">
-        <v>9.970000000000001</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L23" t="n">
-        <v>8.84</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M23" t="n">
-        <v>8.85</v>
+        <v>8.27</v>
       </c>
       <c r="N23" t="n">
-        <v>44.8</v>
+        <v>41.98</v>
       </c>
       <c r="O23" t="n">
-        <v>44.89</v>
+        <v>42.06</v>
       </c>
       <c r="P23" t="n">
-        <v>42.57</v>
+        <v>40.68</v>
       </c>
       <c r="Q23" t="n">
-        <v>42.57</v>
+        <v>41.07</v>
       </c>
       <c r="R23" t="n">
-        <v>16.3314</v>
+        <v>1.0584</v>
       </c>
       <c r="S23" t="n">
-        <v>22.7386</v>
+        <v>-2.2214</v>
       </c>
       <c r="T23" t="n">
-        <v>35.6902</v>
+        <v>22.4129</v>
       </c>
       <c r="U23" t="n">
-        <v>6.9246</v>
+        <v>2.2139</v>
       </c>
       <c r="V23" t="n">
-        <v>13.1919</v>
+        <v>2.5858</v>
       </c>
       <c r="W23" t="n">
-        <v>16.8147</v>
+        <v>10.6672</v>
       </c>
       <c r="X23" t="n">
-        <v>-16.5094</v>
+        <v>-0.9581</v>
       </c>
       <c r="Y23" t="n">
-        <v>-23.1103</v>
+        <v>0.8537</v>
       </c>
       <c r="Z23" t="n">
-        <v>-31.8182</v>
+        <v>-21.9811</v>
       </c>
       <c r="AA23" t="n">
-        <v>-6.9101</v>
+        <v>-2.191</v>
       </c>
       <c r="AB23" t="n">
-        <v>-12.3894</v>
+        <v>-2.7238</v>
       </c>
       <c r="AC23" t="n">
-        <v>-15.233</v>
+        <v>-10.1902</v>
       </c>
     </row>
   </sheetData>
@@ -2503,7 +2503,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-05-15 13:30
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC23"/>
+  <dimension ref="A1:AC24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2457,6 +2457,97 @@
       </c>
       <c r="AC23" t="n">
         <v>-10.1902</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>182.67</v>
+      </c>
+      <c r="C24" t="n">
+        <v>167.2739</v>
+      </c>
+      <c r="D24" t="n">
+        <v>165.3105</v>
+      </c>
+      <c r="E24" t="n">
+        <v>165.695</v>
+      </c>
+      <c r="F24" t="n">
+        <v>75.70999999999999</v>
+      </c>
+      <c r="G24" t="n">
+        <v>75.73999999999999</v>
+      </c>
+      <c r="H24" t="n">
+        <v>75.66</v>
+      </c>
+      <c r="I24" t="n">
+        <v>75.68000000000001</v>
+      </c>
+      <c r="J24" t="n">
+        <v>8.43</v>
+      </c>
+      <c r="K24" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="L24" t="n">
+        <v>9.109999999999999</v>
+      </c>
+      <c r="M24" t="n">
+        <v>9.19</v>
+      </c>
+      <c r="N24" t="n">
+        <v>42.77</v>
+      </c>
+      <c r="O24" t="n">
+        <v>42.81</v>
+      </c>
+      <c r="P24" t="n">
+        <v>42.765</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>42.81</v>
+      </c>
+      <c r="R24" t="n">
+        <v>-11.0076</v>
+      </c>
+      <c r="S24" t="n">
+        <v>-3.9561</v>
+      </c>
+      <c r="T24" t="n">
+        <v>-6.3553</v>
+      </c>
+      <c r="U24" t="n">
+        <v>-4.1419</v>
+      </c>
+      <c r="V24" t="n">
+        <v>0.9605</v>
+      </c>
+      <c r="W24" t="n">
+        <v>-0.7866</v>
+      </c>
+      <c r="X24" t="n">
+        <v>11.1245</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>2.6816</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>3.8418</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>4.2367</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>-1.1545</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>0.5638</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Master system update 2026-05-15 22:54
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC24"/>
+  <dimension ref="A1:AC23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1986 +568,1895 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>84.66</v>
+        <v>85.01000000000001</v>
       </c>
       <c r="C2" t="n">
-        <v>85.98</v>
+        <v>89.39</v>
       </c>
       <c r="D2" t="n">
-        <v>79.76000000000001</v>
+        <v>83.31</v>
       </c>
       <c r="E2" t="n">
-        <v>85.95999999999999</v>
+        <v>88.37</v>
       </c>
       <c r="F2" t="n">
-        <v>53.57</v>
+        <v>56.13</v>
       </c>
       <c r="G2" t="n">
-        <v>55.74</v>
+        <v>56.92</v>
       </c>
       <c r="H2" t="n">
-        <v>53.33</v>
+        <v>55.1</v>
       </c>
       <c r="I2" t="n">
-        <v>55.65</v>
+        <v>56.43</v>
       </c>
       <c r="J2" t="n">
-        <v>21.23</v>
+        <v>21.13</v>
       </c>
       <c r="K2" t="n">
-        <v>22.43</v>
+        <v>21.56</v>
       </c>
       <c r="L2" t="n">
-        <v>20.9</v>
+        <v>20.07</v>
       </c>
       <c r="M2" t="n">
-        <v>20.94</v>
+        <v>20.28</v>
       </c>
       <c r="N2" t="n">
-        <v>61.88</v>
+        <v>58.95</v>
       </c>
       <c r="O2" t="n">
-        <v>62.15</v>
+        <v>60.06</v>
       </c>
       <c r="P2" t="n">
-        <v>59.35</v>
+        <v>58.11</v>
       </c>
       <c r="Q2" t="n">
-        <v>59.44</v>
+        <v>58.61</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>85.01000000000001</v>
+        <v>93.2</v>
       </c>
       <c r="C3" t="n">
-        <v>89.39</v>
+        <v>94.75</v>
       </c>
       <c r="D3" t="n">
-        <v>83.31</v>
+        <v>90.66</v>
       </c>
       <c r="E3" t="n">
-        <v>88.37</v>
+        <v>94.68000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>56.13</v>
+        <v>57.78</v>
       </c>
       <c r="G3" t="n">
-        <v>56.92</v>
+        <v>58.94</v>
       </c>
       <c r="H3" t="n">
-        <v>55.1</v>
+        <v>57.37</v>
       </c>
       <c r="I3" t="n">
-        <v>56.43</v>
+        <v>58.59</v>
       </c>
       <c r="J3" t="n">
-        <v>21.13</v>
+        <v>19.23</v>
       </c>
       <c r="K3" t="n">
-        <v>21.56</v>
+        <v>19.8</v>
       </c>
       <c r="L3" t="n">
-        <v>20.07</v>
+        <v>18.86</v>
       </c>
       <c r="M3" t="n">
-        <v>20.28</v>
+        <v>18.87</v>
       </c>
       <c r="N3" t="n">
-        <v>58.95</v>
+        <v>57.25</v>
       </c>
       <c r="O3" t="n">
-        <v>60.06</v>
+        <v>57.67</v>
       </c>
       <c r="P3" t="n">
-        <v>58.11</v>
+        <v>56.04</v>
       </c>
       <c r="Q3" t="n">
-        <v>58.61</v>
+        <v>56.39</v>
       </c>
       <c r="R3" t="n">
-        <v>2.8036</v>
+        <v>7.1404</v>
       </c>
       <c r="U3" t="n">
-        <v>1.4016</v>
+        <v>3.8278</v>
       </c>
       <c r="X3" t="n">
-        <v>-3.1519</v>
+        <v>-6.9527</v>
       </c>
       <c r="AA3" t="n">
-        <v>-1.3964</v>
+        <v>-3.7877</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>93.2</v>
+        <v>95.97</v>
       </c>
       <c r="C4" t="n">
-        <v>94.75</v>
+        <v>96.93000000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>90.66</v>
+        <v>92.03</v>
       </c>
       <c r="E4" t="n">
-        <v>94.68000000000001</v>
+        <v>95.94</v>
       </c>
       <c r="F4" t="n">
-        <v>57.78</v>
+        <v>58.4</v>
       </c>
       <c r="G4" t="n">
-        <v>58.94</v>
+        <v>58.58</v>
       </c>
       <c r="H4" t="n">
-        <v>57.37</v>
+        <v>56.91</v>
       </c>
       <c r="I4" t="n">
-        <v>58.59</v>
+        <v>58.08</v>
       </c>
       <c r="J4" t="n">
-        <v>19.23</v>
+        <v>18.64</v>
       </c>
       <c r="K4" t="n">
-        <v>19.8</v>
+        <v>19.41</v>
       </c>
       <c r="L4" t="n">
-        <v>18.86</v>
+        <v>18.44</v>
       </c>
       <c r="M4" t="n">
-        <v>18.87</v>
+        <v>18.63</v>
       </c>
       <c r="N4" t="n">
-        <v>57.25</v>
+        <v>56.59</v>
       </c>
       <c r="O4" t="n">
-        <v>57.67</v>
+        <v>58.04</v>
       </c>
       <c r="P4" t="n">
-        <v>56.04</v>
+        <v>56.41</v>
       </c>
       <c r="Q4" t="n">
-        <v>56.39</v>
+        <v>56.91</v>
       </c>
       <c r="R4" t="n">
-        <v>7.1404</v>
+        <v>1.3308</v>
       </c>
       <c r="U4" t="n">
-        <v>3.8278</v>
+        <v>-0.8705000000000001</v>
       </c>
       <c r="X4" t="n">
-        <v>-6.9527</v>
+        <v>-1.2719</v>
       </c>
       <c r="AA4" t="n">
-        <v>-3.7877</v>
+        <v>0.9221</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>95.97</v>
+        <v>97.97</v>
       </c>
       <c r="C5" t="n">
-        <v>96.93000000000001</v>
+        <v>99.95</v>
       </c>
       <c r="D5" t="n">
-        <v>92.03</v>
+        <v>95.31999999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>95.94</v>
+        <v>98.09</v>
       </c>
       <c r="F5" t="n">
-        <v>58.4</v>
+        <v>58.48</v>
       </c>
       <c r="G5" t="n">
-        <v>58.58</v>
+        <v>58.97</v>
       </c>
       <c r="H5" t="n">
-        <v>56.91</v>
+        <v>56.82</v>
       </c>
       <c r="I5" t="n">
-        <v>58.08</v>
+        <v>57.4</v>
       </c>
       <c r="J5" t="n">
-        <v>18.64</v>
+        <v>18.25</v>
       </c>
       <c r="K5" t="n">
-        <v>19.41</v>
+        <v>18.76</v>
       </c>
       <c r="L5" t="n">
-        <v>18.44</v>
+        <v>17.85</v>
       </c>
       <c r="M5" t="n">
-        <v>18.63</v>
+        <v>18.2</v>
       </c>
       <c r="N5" t="n">
-        <v>56.59</v>
+        <v>56.52</v>
       </c>
       <c r="O5" t="n">
-        <v>58.04</v>
+        <v>58.15</v>
       </c>
       <c r="P5" t="n">
-        <v>56.41</v>
+        <v>56.04</v>
       </c>
       <c r="Q5" t="n">
-        <v>56.91</v>
+        <v>57.59</v>
       </c>
       <c r="R5" t="n">
-        <v>1.3308</v>
+        <v>2.241</v>
       </c>
       <c r="S5" t="n">
-        <v>11.6101</v>
+        <v>10.9992</v>
       </c>
       <c r="U5" t="n">
-        <v>-0.8705000000000001</v>
+        <v>-1.1708</v>
       </c>
       <c r="V5" t="n">
-        <v>4.3666</v>
+        <v>1.7189</v>
       </c>
       <c r="X5" t="n">
-        <v>-1.2719</v>
+        <v>-2.3081</v>
       </c>
       <c r="Y5" t="n">
-        <v>-11.0315</v>
+        <v>-10.2564</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.9221</v>
+        <v>1.1949</v>
       </c>
       <c r="AB5" t="n">
-        <v>-4.2564</v>
+        <v>-1.7403</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>97.97</v>
+        <v>102.94</v>
       </c>
       <c r="C6" t="n">
-        <v>99.95</v>
+        <v>106.09</v>
       </c>
       <c r="D6" t="n">
-        <v>95.31999999999999</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="E6" t="n">
-        <v>98.09</v>
+        <v>105.64</v>
       </c>
       <c r="F6" t="n">
-        <v>58.48</v>
+        <v>58.93</v>
       </c>
       <c r="G6" t="n">
-        <v>58.97</v>
+        <v>60.3</v>
       </c>
       <c r="H6" t="n">
-        <v>56.82</v>
+        <v>58.49</v>
       </c>
       <c r="I6" t="n">
-        <v>57.4</v>
+        <v>60.21</v>
       </c>
       <c r="J6" t="n">
-        <v>18.25</v>
+        <v>17.37</v>
       </c>
       <c r="K6" t="n">
-        <v>18.76</v>
+        <v>17.95</v>
       </c>
       <c r="L6" t="n">
-        <v>17.85</v>
+        <v>16.72</v>
       </c>
       <c r="M6" t="n">
-        <v>18.2</v>
+        <v>16.8</v>
       </c>
       <c r="N6" t="n">
-        <v>56.52</v>
+        <v>56.05</v>
       </c>
       <c r="O6" t="n">
-        <v>58.15</v>
+        <v>56.49</v>
       </c>
       <c r="P6" t="n">
-        <v>56.04</v>
+        <v>54.66</v>
       </c>
       <c r="Q6" t="n">
-        <v>57.59</v>
+        <v>54.73</v>
       </c>
       <c r="R6" t="n">
-        <v>2.241</v>
+        <v>7.697</v>
       </c>
       <c r="S6" t="n">
-        <v>10.9992</v>
+        <v>11.5758</v>
       </c>
       <c r="U6" t="n">
-        <v>-1.1708</v>
+        <v>4.8955</v>
       </c>
       <c r="V6" t="n">
-        <v>1.7189</v>
+        <v>2.765</v>
       </c>
       <c r="X6" t="n">
-        <v>-2.3081</v>
+        <v>-7.6923</v>
       </c>
       <c r="Y6" t="n">
-        <v>-10.2564</v>
+        <v>-10.9698</v>
       </c>
       <c r="AA6" t="n">
-        <v>1.1949</v>
+        <v>-4.9661</v>
       </c>
       <c r="AB6" t="n">
-        <v>-1.7403</v>
+        <v>-2.9438</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>102.94</v>
+        <v>108.62</v>
       </c>
       <c r="C7" t="n">
-        <v>106.09</v>
+        <v>116.77</v>
       </c>
       <c r="D7" t="n">
-        <v>99.59999999999999</v>
+        <v>107.46</v>
       </c>
       <c r="E7" t="n">
-        <v>105.64</v>
+        <v>112.77</v>
       </c>
       <c r="F7" t="n">
-        <v>58.93</v>
+        <v>59.8</v>
       </c>
       <c r="G7" t="n">
-        <v>60.3</v>
+        <v>60.73</v>
       </c>
       <c r="H7" t="n">
-        <v>58.49</v>
+        <v>57.59</v>
       </c>
       <c r="I7" t="n">
-        <v>60.21</v>
+        <v>59.22</v>
       </c>
       <c r="J7" t="n">
-        <v>17.37</v>
+        <v>16.35</v>
       </c>
       <c r="K7" t="n">
-        <v>17.95</v>
+        <v>16.52</v>
       </c>
       <c r="L7" t="n">
-        <v>16.72</v>
+        <v>15.06</v>
       </c>
       <c r="M7" t="n">
-        <v>16.8</v>
+        <v>15.7</v>
       </c>
       <c r="N7" t="n">
-        <v>56.05</v>
+        <v>55.13</v>
       </c>
       <c r="O7" t="n">
-        <v>56.49</v>
+        <v>57.14</v>
       </c>
       <c r="P7" t="n">
-        <v>54.66</v>
+        <v>54.28</v>
       </c>
       <c r="Q7" t="n">
-        <v>54.73</v>
+        <v>55.66</v>
       </c>
       <c r="R7" t="n">
-        <v>7.697</v>
+        <v>6.7493</v>
       </c>
       <c r="S7" t="n">
-        <v>11.5758</v>
+        <v>17.5422</v>
       </c>
       <c r="T7" t="n">
-        <v>22.8944</v>
+        <v>27.6112</v>
       </c>
       <c r="U7" t="n">
-        <v>4.8955</v>
+        <v>-1.6442</v>
       </c>
       <c r="V7" t="n">
-        <v>2.765</v>
+        <v>1.9628</v>
       </c>
       <c r="W7" t="n">
-        <v>8.194100000000001</v>
+        <v>4.9442</v>
       </c>
       <c r="X7" t="n">
-        <v>-7.6923</v>
+        <v>-6.5476</v>
       </c>
       <c r="Y7" t="n">
-        <v>-10.9698</v>
+        <v>-15.7273</v>
       </c>
       <c r="Z7" t="n">
-        <v>-19.7708</v>
+        <v>-22.5838</v>
       </c>
       <c r="AA7" t="n">
-        <v>-4.9661</v>
+        <v>1.6993</v>
       </c>
       <c r="AB7" t="n">
-        <v>-2.9438</v>
+        <v>-2.1965</v>
       </c>
       <c r="AC7" t="n">
-        <v>-7.924</v>
+        <v>-5.0333</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>108.62</v>
+        <v>125.21</v>
       </c>
       <c r="C8" t="n">
-        <v>116.77</v>
+        <v>130.12</v>
       </c>
       <c r="D8" t="n">
-        <v>107.46</v>
+        <v>120.24</v>
       </c>
       <c r="E8" t="n">
-        <v>112.77</v>
+        <v>128.32</v>
       </c>
       <c r="F8" t="n">
-        <v>59.8</v>
+        <v>61.08</v>
       </c>
       <c r="G8" t="n">
-        <v>60.73</v>
+        <v>62.74</v>
       </c>
       <c r="H8" t="n">
-        <v>57.59</v>
+        <v>60.56</v>
       </c>
       <c r="I8" t="n">
-        <v>59.22</v>
+        <v>62.56</v>
       </c>
       <c r="J8" t="n">
-        <v>16.35</v>
+        <v>13.99</v>
       </c>
       <c r="K8" t="n">
-        <v>16.52</v>
+        <v>14.66</v>
       </c>
       <c r="L8" t="n">
-        <v>15.06</v>
+        <v>13.3</v>
       </c>
       <c r="M8" t="n">
-        <v>15.7</v>
+        <v>13.52</v>
       </c>
       <c r="N8" t="n">
-        <v>55.13</v>
+        <v>53.93</v>
       </c>
       <c r="O8" t="n">
-        <v>57.14</v>
+        <v>54.43</v>
       </c>
       <c r="P8" t="n">
-        <v>54.28</v>
+        <v>52.37</v>
       </c>
       <c r="Q8" t="n">
-        <v>55.66</v>
+        <v>52.5</v>
       </c>
       <c r="R8" t="n">
-        <v>6.7493</v>
+        <v>13.7891</v>
       </c>
       <c r="S8" t="n">
-        <v>17.5422</v>
+        <v>30.8186</v>
       </c>
       <c r="T8" t="n">
-        <v>27.6112</v>
+        <v>35.5302</v>
       </c>
       <c r="U8" t="n">
-        <v>-1.6442</v>
+        <v>5.64</v>
       </c>
       <c r="V8" t="n">
-        <v>1.9628</v>
+        <v>8.9895</v>
       </c>
       <c r="W8" t="n">
-        <v>4.9442</v>
+        <v>6.7759</v>
       </c>
       <c r="X8" t="n">
-        <v>-6.5476</v>
+        <v>-13.8854</v>
       </c>
       <c r="Y8" t="n">
-        <v>-15.7273</v>
+        <v>-25.7143</v>
       </c>
       <c r="Z8" t="n">
-        <v>-22.5838</v>
+        <v>-28.3519</v>
       </c>
       <c r="AA8" t="n">
-        <v>1.6993</v>
+        <v>-5.6773</v>
       </c>
       <c r="AB8" t="n">
-        <v>-2.1965</v>
+        <v>-8.8383</v>
       </c>
       <c r="AC8" t="n">
-        <v>-5.0333</v>
+        <v>-6.8984</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>125.21</v>
+        <v>128.33</v>
       </c>
       <c r="C9" t="n">
-        <v>130.12</v>
+        <v>129.59</v>
       </c>
       <c r="D9" t="n">
-        <v>120.24</v>
+        <v>117.79</v>
       </c>
       <c r="E9" t="n">
-        <v>128.32</v>
+        <v>123.39</v>
       </c>
       <c r="F9" t="n">
-        <v>61.08</v>
+        <v>62.41</v>
       </c>
       <c r="G9" t="n">
-        <v>62.74</v>
+        <v>62.7</v>
       </c>
       <c r="H9" t="n">
-        <v>60.56</v>
+        <v>61.64</v>
       </c>
       <c r="I9" t="n">
-        <v>62.56</v>
+        <v>62.64</v>
       </c>
       <c r="J9" t="n">
-        <v>13.99</v>
+        <v>13.51</v>
       </c>
       <c r="K9" t="n">
-        <v>14.66</v>
+        <v>14.63</v>
       </c>
       <c r="L9" t="n">
-        <v>13.3</v>
+        <v>13.41</v>
       </c>
       <c r="M9" t="n">
-        <v>13.52</v>
+        <v>14.03</v>
       </c>
       <c r="N9" t="n">
-        <v>53.93</v>
+        <v>52.67</v>
       </c>
       <c r="O9" t="n">
-        <v>54.43</v>
+        <v>53.31</v>
       </c>
       <c r="P9" t="n">
-        <v>52.37</v>
+        <v>52.42</v>
       </c>
       <c r="Q9" t="n">
-        <v>52.5</v>
+        <v>52.45</v>
       </c>
       <c r="R9" t="n">
-        <v>13.7891</v>
+        <v>-3.842</v>
       </c>
       <c r="S9" t="n">
-        <v>30.8186</v>
+        <v>16.8023</v>
       </c>
       <c r="T9" t="n">
-        <v>35.5302</v>
+        <v>28.6116</v>
       </c>
       <c r="U9" t="n">
-        <v>5.64</v>
+        <v>0.1279</v>
       </c>
       <c r="V9" t="n">
-        <v>8.9895</v>
+        <v>4.0359</v>
       </c>
       <c r="W9" t="n">
-        <v>6.7759</v>
+        <v>7.8512</v>
       </c>
       <c r="X9" t="n">
-        <v>-13.8854</v>
+        <v>3.7722</v>
       </c>
       <c r="Y9" t="n">
-        <v>-25.7143</v>
+        <v>-16.4881</v>
       </c>
       <c r="Z9" t="n">
-        <v>-28.3519</v>
+        <v>-24.6914</v>
       </c>
       <c r="AA9" t="n">
-        <v>-5.6773</v>
+        <v>-0.09520000000000001</v>
       </c>
       <c r="AB9" t="n">
-        <v>-8.8383</v>
+        <v>-4.1659</v>
       </c>
       <c r="AC9" t="n">
-        <v>-6.8984</v>
+        <v>-7.8369</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>128.33</v>
+        <v>108.75</v>
       </c>
       <c r="C10" t="n">
-        <v>129.59</v>
+        <v>115.62</v>
       </c>
       <c r="D10" t="n">
-        <v>117.79</v>
+        <v>103.99</v>
       </c>
       <c r="E10" t="n">
-        <v>123.39</v>
+        <v>109.56</v>
       </c>
       <c r="F10" t="n">
-        <v>62.41</v>
+        <v>60.72</v>
       </c>
       <c r="G10" t="n">
-        <v>62.7</v>
+        <v>61.33</v>
       </c>
       <c r="H10" t="n">
-        <v>61.64</v>
+        <v>59.68</v>
       </c>
       <c r="I10" t="n">
-        <v>62.64</v>
+        <v>60.74</v>
       </c>
       <c r="J10" t="n">
-        <v>13.51</v>
+        <v>15.71</v>
       </c>
       <c r="K10" t="n">
-        <v>14.63</v>
+        <v>16.27</v>
       </c>
       <c r="L10" t="n">
-        <v>13.41</v>
+        <v>14.93</v>
       </c>
       <c r="M10" t="n">
-        <v>14.03</v>
+        <v>15.59</v>
       </c>
       <c r="N10" t="n">
-        <v>52.67</v>
+        <v>54.09</v>
       </c>
       <c r="O10" t="n">
-        <v>53.31</v>
+        <v>54.96</v>
       </c>
       <c r="P10" t="n">
-        <v>52.42</v>
+        <v>53.58</v>
       </c>
       <c r="Q10" t="n">
-        <v>52.45</v>
+        <v>54.05</v>
       </c>
       <c r="R10" t="n">
-        <v>-3.842</v>
+        <v>-11.2084</v>
       </c>
       <c r="S10" t="n">
-        <v>16.8023</v>
+        <v>-2.8465</v>
       </c>
       <c r="T10" t="n">
-        <v>28.6116</v>
+        <v>11.6933</v>
       </c>
       <c r="U10" t="n">
-        <v>0.1279</v>
+        <v>-3.0332</v>
       </c>
       <c r="V10" t="n">
-        <v>4.0359</v>
+        <v>2.5667</v>
       </c>
       <c r="W10" t="n">
-        <v>7.8512</v>
+        <v>5.8188</v>
       </c>
       <c r="X10" t="n">
-        <v>3.7722</v>
+        <v>11.119</v>
       </c>
       <c r="Y10" t="n">
-        <v>-16.4881</v>
+        <v>-0.7006</v>
       </c>
       <c r="Z10" t="n">
-        <v>-24.6914</v>
+        <v>-14.3407</v>
       </c>
       <c r="AA10" t="n">
-        <v>-0.09520000000000001</v>
+        <v>3.0505</v>
       </c>
       <c r="AB10" t="n">
-        <v>-4.1659</v>
+        <v>-2.8926</v>
       </c>
       <c r="AC10" t="n">
-        <v>-7.8369</v>
+        <v>-6.1469</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>108.75</v>
+        <v>114.76</v>
       </c>
       <c r="C11" t="n">
-        <v>115.62</v>
+        <v>118.32</v>
       </c>
       <c r="D11" t="n">
-        <v>103.99</v>
+        <v>112.3</v>
       </c>
       <c r="E11" t="n">
-        <v>109.56</v>
+        <v>117.97</v>
       </c>
       <c r="F11" t="n">
-        <v>60.72</v>
+        <v>61</v>
       </c>
       <c r="G11" t="n">
-        <v>61.33</v>
+        <v>61.87</v>
       </c>
       <c r="H11" t="n">
-        <v>59.68</v>
+        <v>60.45</v>
       </c>
       <c r="I11" t="n">
-        <v>60.74</v>
+        <v>61.86</v>
       </c>
       <c r="J11" t="n">
-        <v>15.71</v>
+        <v>14.91</v>
       </c>
       <c r="K11" t="n">
-        <v>16.27</v>
+        <v>15.24</v>
       </c>
       <c r="L11" t="n">
-        <v>14.93</v>
+        <v>14.38</v>
       </c>
       <c r="M11" t="n">
-        <v>15.59</v>
+        <v>14.4</v>
       </c>
       <c r="N11" t="n">
-        <v>54.09</v>
+        <v>53.84</v>
       </c>
       <c r="O11" t="n">
-        <v>54.96</v>
+        <v>54.33</v>
       </c>
       <c r="P11" t="n">
-        <v>53.58</v>
+        <v>53.06</v>
       </c>
       <c r="Q11" t="n">
-        <v>54.05</v>
+        <v>53.08</v>
       </c>
       <c r="R11" t="n">
-        <v>-11.2084</v>
+        <v>7.6762</v>
       </c>
       <c r="S11" t="n">
-        <v>-2.8465</v>
+        <v>-8.065799999999999</v>
       </c>
       <c r="T11" t="n">
-        <v>11.6933</v>
+        <v>11.6717</v>
       </c>
       <c r="U11" t="n">
-        <v>-3.0332</v>
+        <v>1.8439</v>
       </c>
       <c r="V11" t="n">
-        <v>2.5667</v>
+        <v>-1.1189</v>
       </c>
       <c r="W11" t="n">
-        <v>5.8188</v>
+        <v>2.7404</v>
       </c>
       <c r="X11" t="n">
-        <v>11.119</v>
+        <v>-7.6331</v>
       </c>
       <c r="Y11" t="n">
-        <v>-0.7006</v>
+        <v>6.5089</v>
       </c>
       <c r="Z11" t="n">
-        <v>-14.3407</v>
+        <v>-14.2857</v>
       </c>
       <c r="AA11" t="n">
-        <v>3.0505</v>
+        <v>-1.7946</v>
       </c>
       <c r="AB11" t="n">
-        <v>-2.8926</v>
+        <v>1.1048</v>
       </c>
       <c r="AC11" t="n">
-        <v>-6.1469</v>
+        <v>-3.0148</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>114.76</v>
+        <v>122.81</v>
       </c>
       <c r="C12" t="n">
-        <v>118.32</v>
+        <v>127.45</v>
       </c>
       <c r="D12" t="n">
-        <v>112.3</v>
+        <v>117.5</v>
       </c>
       <c r="E12" t="n">
-        <v>117.97</v>
+        <v>126.98</v>
       </c>
       <c r="F12" t="n">
-        <v>61</v>
+        <v>62.89</v>
       </c>
       <c r="G12" t="n">
-        <v>61.87</v>
+        <v>63.8</v>
       </c>
       <c r="H12" t="n">
-        <v>60.45</v>
+        <v>60.7</v>
       </c>
       <c r="I12" t="n">
-        <v>61.86</v>
+        <v>63.54</v>
       </c>
       <c r="J12" t="n">
-        <v>14.91</v>
+        <v>13.84</v>
       </c>
       <c r="K12" t="n">
-        <v>15.24</v>
+        <v>14.49</v>
       </c>
       <c r="L12" t="n">
-        <v>14.38</v>
+        <v>13.25</v>
       </c>
       <c r="M12" t="n">
-        <v>14.4</v>
+        <v>13.3</v>
       </c>
       <c r="N12" t="n">
-        <v>53.84</v>
+        <v>52.21</v>
       </c>
       <c r="O12" t="n">
-        <v>54.33</v>
+        <v>54.09</v>
       </c>
       <c r="P12" t="n">
-        <v>53.06</v>
+        <v>51.4</v>
       </c>
       <c r="Q12" t="n">
-        <v>53.08</v>
+        <v>51.65</v>
       </c>
       <c r="R12" t="n">
-        <v>7.6762</v>
+        <v>7.6375</v>
       </c>
       <c r="S12" t="n">
-        <v>-8.065799999999999</v>
+        <v>2.9095</v>
       </c>
       <c r="T12" t="n">
-        <v>11.6717</v>
+        <v>12.6009</v>
       </c>
       <c r="U12" t="n">
-        <v>1.8439</v>
+        <v>2.7158</v>
       </c>
       <c r="V12" t="n">
-        <v>-1.1189</v>
+        <v>1.4368</v>
       </c>
       <c r="W12" t="n">
-        <v>2.7404</v>
+        <v>7.2948</v>
       </c>
       <c r="X12" t="n">
-        <v>-7.6331</v>
+        <v>-7.6389</v>
       </c>
       <c r="Y12" t="n">
-        <v>6.5089</v>
+        <v>-5.2031</v>
       </c>
       <c r="Z12" t="n">
-        <v>-14.2857</v>
+        <v>-15.2866</v>
       </c>
       <c r="AA12" t="n">
-        <v>-1.7946</v>
+        <v>-2.694</v>
       </c>
       <c r="AB12" t="n">
-        <v>1.1048</v>
+        <v>-1.5253</v>
       </c>
       <c r="AC12" t="n">
-        <v>-3.0148</v>
+        <v>-7.2045</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>122.81</v>
+        <v>124.39</v>
       </c>
       <c r="C13" t="n">
-        <v>127.45</v>
+        <v>131.38</v>
       </c>
       <c r="D13" t="n">
-        <v>117.5</v>
+        <v>121.66</v>
       </c>
       <c r="E13" t="n">
-        <v>126.98</v>
+        <v>130.4</v>
       </c>
       <c r="F13" t="n">
-        <v>62.89</v>
+        <v>63.89</v>
       </c>
       <c r="G13" t="n">
-        <v>63.8</v>
+        <v>65.84</v>
       </c>
       <c r="H13" t="n">
-        <v>60.7</v>
+        <v>63.81</v>
       </c>
       <c r="I13" t="n">
-        <v>63.54</v>
+        <v>65.3</v>
       </c>
       <c r="J13" t="n">
-        <v>13.84</v>
+        <v>13.61</v>
       </c>
       <c r="K13" t="n">
-        <v>14.49</v>
+        <v>13.89</v>
       </c>
       <c r="L13" t="n">
-        <v>13.25</v>
+        <v>12.87</v>
       </c>
       <c r="M13" t="n">
-        <v>13.3</v>
+        <v>12.98</v>
       </c>
       <c r="N13" t="n">
-        <v>52.21</v>
+        <v>51.36</v>
       </c>
       <c r="O13" t="n">
-        <v>54.09</v>
+        <v>51.45</v>
       </c>
       <c r="P13" t="n">
-        <v>51.4</v>
+        <v>49.79</v>
       </c>
       <c r="Q13" t="n">
-        <v>51.65</v>
+        <v>50.22</v>
       </c>
       <c r="R13" t="n">
-        <v>7.6375</v>
+        <v>2.6933</v>
       </c>
       <c r="S13" t="n">
-        <v>2.9095</v>
+        <v>19.0215</v>
       </c>
       <c r="T13" t="n">
-        <v>12.6009</v>
+        <v>1.6209</v>
       </c>
       <c r="U13" t="n">
-        <v>2.7158</v>
+        <v>2.7699</v>
       </c>
       <c r="V13" t="n">
-        <v>1.4368</v>
+        <v>7.5074</v>
       </c>
       <c r="W13" t="n">
-        <v>7.2948</v>
+        <v>4.3798</v>
       </c>
       <c r="X13" t="n">
-        <v>-7.6389</v>
+        <v>-2.406</v>
       </c>
       <c r="Y13" t="n">
-        <v>-5.2031</v>
+        <v>-16.7415</v>
       </c>
       <c r="Z13" t="n">
-        <v>-15.2866</v>
+        <v>-3.9941</v>
       </c>
       <c r="AA13" t="n">
-        <v>-2.694</v>
+        <v>-2.7686</v>
       </c>
       <c r="AB13" t="n">
-        <v>-1.5253</v>
+        <v>-7.086</v>
       </c>
       <c r="AC13" t="n">
-        <v>-7.2045</v>
+        <v>-4.3429</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>124.39</v>
+        <v>132.2</v>
       </c>
       <c r="C14" t="n">
-        <v>131.38</v>
+        <v>133.67</v>
       </c>
       <c r="D14" t="n">
-        <v>121.66</v>
+        <v>123.8</v>
       </c>
       <c r="E14" t="n">
-        <v>130.4</v>
+        <v>127.55</v>
       </c>
       <c r="F14" t="n">
-        <v>63.89</v>
+        <v>65.44</v>
       </c>
       <c r="G14" t="n">
-        <v>65.84</v>
+        <v>66.05</v>
       </c>
       <c r="H14" t="n">
-        <v>63.81</v>
+        <v>63.78</v>
       </c>
       <c r="I14" t="n">
-        <v>65.3</v>
+        <v>64.91</v>
       </c>
       <c r="J14" t="n">
-        <v>13.61</v>
+        <v>12.8</v>
       </c>
       <c r="K14" t="n">
-        <v>13.89</v>
+        <v>13.64</v>
       </c>
       <c r="L14" t="n">
-        <v>12.87</v>
+        <v>12.65</v>
       </c>
       <c r="M14" t="n">
-        <v>12.98</v>
+        <v>13.26</v>
       </c>
       <c r="N14" t="n">
-        <v>51.36</v>
+        <v>50.12</v>
       </c>
       <c r="O14" t="n">
-        <v>51.45</v>
+        <v>51.43</v>
       </c>
       <c r="P14" t="n">
-        <v>49.79</v>
+        <v>49.65</v>
       </c>
       <c r="Q14" t="n">
-        <v>50.22</v>
+        <v>50.51</v>
       </c>
       <c r="R14" t="n">
-        <v>2.6933</v>
+        <v>-2.1856</v>
       </c>
       <c r="S14" t="n">
-        <v>19.0215</v>
+        <v>8.120699999999999</v>
       </c>
       <c r="T14" t="n">
-        <v>1.6209</v>
+        <v>3.3714</v>
       </c>
       <c r="U14" t="n">
-        <v>2.7699</v>
+        <v>-0.5972</v>
       </c>
       <c r="V14" t="n">
-        <v>7.5074</v>
+        <v>4.9305</v>
       </c>
       <c r="W14" t="n">
-        <v>4.3798</v>
+        <v>3.6239</v>
       </c>
       <c r="X14" t="n">
-        <v>-2.406</v>
+        <v>2.1572</v>
       </c>
       <c r="Y14" t="n">
-        <v>-16.7415</v>
+        <v>-7.9167</v>
       </c>
       <c r="Z14" t="n">
-        <v>-3.9941</v>
+        <v>-5.4882</v>
       </c>
       <c r="AA14" t="n">
-        <v>-2.7686</v>
+        <v>0.5775</v>
       </c>
       <c r="AB14" t="n">
-        <v>-7.086</v>
+        <v>-4.8417</v>
       </c>
       <c r="AC14" t="n">
-        <v>-4.3429</v>
+        <v>-3.6988</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>132.2</v>
+        <v>135</v>
       </c>
       <c r="C15" t="n">
-        <v>133.67</v>
+        <v>147.26</v>
       </c>
       <c r="D15" t="n">
-        <v>123.8</v>
+        <v>134.02</v>
       </c>
       <c r="E15" t="n">
-        <v>127.55</v>
+        <v>144.16</v>
       </c>
       <c r="F15" t="n">
-        <v>65.44</v>
+        <v>66.37</v>
       </c>
       <c r="G15" t="n">
-        <v>66.05</v>
+        <v>67.77</v>
       </c>
       <c r="H15" t="n">
-        <v>63.78</v>
+        <v>66.25</v>
       </c>
       <c r="I15" t="n">
-        <v>64.91</v>
+        <v>67.39</v>
       </c>
       <c r="J15" t="n">
-        <v>12.8</v>
+        <v>12.5</v>
       </c>
       <c r="K15" t="n">
-        <v>13.64</v>
+        <v>12.59</v>
       </c>
       <c r="L15" t="n">
-        <v>12.65</v>
+        <v>11.21</v>
       </c>
       <c r="M15" t="n">
-        <v>13.26</v>
+        <v>11.51</v>
       </c>
       <c r="N15" t="n">
-        <v>50.12</v>
+        <v>49.4</v>
       </c>
       <c r="O15" t="n">
-        <v>51.43</v>
+        <v>49.49</v>
       </c>
       <c r="P15" t="n">
-        <v>49.65</v>
+        <v>48.3</v>
       </c>
       <c r="Q15" t="n">
-        <v>50.51</v>
+        <v>48.59</v>
       </c>
       <c r="R15" t="n">
-        <v>-2.1856</v>
+        <v>13.0223</v>
       </c>
       <c r="S15" t="n">
-        <v>8.120699999999999</v>
+        <v>13.5297</v>
       </c>
       <c r="T15" t="n">
-        <v>3.3714</v>
+        <v>31.5809</v>
       </c>
       <c r="U15" t="n">
-        <v>-0.5972</v>
+        <v>3.8207</v>
       </c>
       <c r="V15" t="n">
-        <v>4.9305</v>
+        <v>6.0592</v>
       </c>
       <c r="W15" t="n">
-        <v>3.6239</v>
+        <v>10.9483</v>
       </c>
       <c r="X15" t="n">
-        <v>2.1572</v>
+        <v>-13.1976</v>
       </c>
       <c r="Y15" t="n">
-        <v>-7.9167</v>
+        <v>-13.4586</v>
       </c>
       <c r="Z15" t="n">
-        <v>-5.4882</v>
+        <v>-26.1706</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.5775</v>
+        <v>-3.8012</v>
       </c>
       <c r="AB15" t="n">
-        <v>-4.8417</v>
+        <v>-5.9245</v>
       </c>
       <c r="AC15" t="n">
-        <v>-3.6988</v>
+        <v>-10.1018</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>135</v>
+        <v>157.84</v>
       </c>
       <c r="C16" t="n">
-        <v>147.26</v>
+        <v>166</v>
       </c>
       <c r="D16" t="n">
-        <v>134.02</v>
+        <v>149.06</v>
       </c>
       <c r="E16" t="n">
-        <v>144.16</v>
+        <v>165.85</v>
       </c>
       <c r="F16" t="n">
-        <v>66.37</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>67.77</v>
+        <v>71.66</v>
       </c>
       <c r="H16" t="n">
-        <v>66.25</v>
+        <v>68.88</v>
       </c>
       <c r="I16" t="n">
-        <v>67.39</v>
+        <v>71.56999999999999</v>
       </c>
       <c r="J16" t="n">
-        <v>12.5</v>
+        <v>10.43</v>
       </c>
       <c r="K16" t="n">
-        <v>12.59</v>
+        <v>11.14</v>
       </c>
       <c r="L16" t="n">
-        <v>11.21</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M16" t="n">
-        <v>11.51</v>
+        <v>9.81</v>
       </c>
       <c r="N16" t="n">
-        <v>49.4</v>
+        <v>47.26</v>
       </c>
       <c r="O16" t="n">
-        <v>49.49</v>
+        <v>47.54</v>
       </c>
       <c r="P16" t="n">
-        <v>48.3</v>
+        <v>45.52</v>
       </c>
       <c r="Q16" t="n">
-        <v>48.59</v>
+        <v>45.59</v>
       </c>
       <c r="R16" t="n">
-        <v>13.0223</v>
+        <v>15.0458</v>
       </c>
       <c r="S16" t="n">
-        <v>13.5297</v>
+        <v>27.1856</v>
       </c>
       <c r="T16" t="n">
-        <v>31.5809</v>
+        <v>40.5866</v>
       </c>
       <c r="U16" t="n">
-        <v>3.8207</v>
+        <v>6.2027</v>
       </c>
       <c r="V16" t="n">
-        <v>6.0592</v>
+        <v>9.601800000000001</v>
       </c>
       <c r="W16" t="n">
-        <v>10.9483</v>
+        <v>15.6967</v>
       </c>
       <c r="X16" t="n">
-        <v>-13.1976</v>
+        <v>-14.7698</v>
       </c>
       <c r="Y16" t="n">
-        <v>-13.4586</v>
+        <v>-24.4222</v>
       </c>
       <c r="Z16" t="n">
-        <v>-26.1706</v>
+        <v>-31.875</v>
       </c>
       <c r="AA16" t="n">
-        <v>-3.8012</v>
+        <v>-6.1741</v>
       </c>
       <c r="AB16" t="n">
-        <v>-5.9245</v>
+        <v>-9.2194</v>
       </c>
       <c r="AC16" t="n">
-        <v>-10.1018</v>
+        <v>-14.1108</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>157.84</v>
+        <v>162.12</v>
       </c>
       <c r="C17" t="n">
-        <v>166</v>
+        <v>162.9</v>
       </c>
       <c r="D17" t="n">
-        <v>149.06</v>
+        <v>147.61</v>
       </c>
       <c r="E17" t="n">
-        <v>165.85</v>
+        <v>152.1</v>
       </c>
       <c r="F17" t="n">
-        <v>69.26000000000001</v>
+        <v>71.87</v>
       </c>
       <c r="G17" t="n">
-        <v>71.66</v>
+        <v>73.3</v>
       </c>
       <c r="H17" t="n">
-        <v>68.88</v>
+        <v>70.38</v>
       </c>
       <c r="I17" t="n">
-        <v>71.56999999999999</v>
+        <v>71.34</v>
       </c>
       <c r="J17" t="n">
-        <v>10.43</v>
+        <v>10.02</v>
       </c>
       <c r="K17" t="n">
-        <v>11.14</v>
+        <v>10.88</v>
       </c>
       <c r="L17" t="n">
-        <v>9.800000000000001</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="M17" t="n">
-        <v>9.81</v>
+        <v>10.6</v>
       </c>
       <c r="N17" t="n">
-        <v>47.26</v>
+        <v>45.41</v>
       </c>
       <c r="O17" t="n">
-        <v>47.54</v>
+        <v>46.36</v>
       </c>
       <c r="P17" t="n">
-        <v>45.52</v>
+        <v>44.5</v>
       </c>
       <c r="Q17" t="n">
-        <v>45.59</v>
+        <v>45.73</v>
       </c>
       <c r="R17" t="n">
-        <v>15.0458</v>
+        <v>-8.2906</v>
       </c>
       <c r="S17" t="n">
-        <v>27.1856</v>
+        <v>19.2474</v>
       </c>
       <c r="T17" t="n">
-        <v>40.5866</v>
+        <v>19.7826</v>
       </c>
       <c r="U17" t="n">
-        <v>6.2027</v>
+        <v>-0.3214</v>
       </c>
       <c r="V17" t="n">
-        <v>9.601800000000001</v>
+        <v>9.906000000000001</v>
       </c>
       <c r="W17" t="n">
-        <v>15.6967</v>
+        <v>12.2757</v>
       </c>
       <c r="X17" t="n">
-        <v>-14.7698</v>
+        <v>8.053000000000001</v>
       </c>
       <c r="Y17" t="n">
-        <v>-24.4222</v>
+        <v>-20.0603</v>
       </c>
       <c r="Z17" t="n">
-        <v>-31.875</v>
+        <v>-20.3008</v>
       </c>
       <c r="AA17" t="n">
-        <v>-6.1741</v>
+        <v>0.3071</v>
       </c>
       <c r="AB17" t="n">
-        <v>-9.2194</v>
+        <v>-9.4635</v>
       </c>
       <c r="AC17" t="n">
-        <v>-14.1108</v>
+        <v>-11.4618</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>162.12</v>
+        <v>163</v>
       </c>
       <c r="C18" t="n">
-        <v>162.9</v>
+        <v>177.5</v>
       </c>
       <c r="D18" t="n">
-        <v>147.61</v>
+        <v>161.51</v>
       </c>
       <c r="E18" t="n">
-        <v>152.1</v>
+        <v>176.94</v>
       </c>
       <c r="F18" t="n">
-        <v>71.87</v>
+        <v>72.81999999999999</v>
       </c>
       <c r="G18" t="n">
-        <v>73.3</v>
+        <v>76.31</v>
       </c>
       <c r="H18" t="n">
-        <v>70.38</v>
+        <v>72.7</v>
       </c>
       <c r="I18" t="n">
-        <v>71.34</v>
+        <v>76.28</v>
       </c>
       <c r="J18" t="n">
-        <v>10.02</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="K18" t="n">
-        <v>10.88</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="L18" t="n">
-        <v>9.970000000000001</v>
+        <v>8.84</v>
       </c>
       <c r="M18" t="n">
-        <v>10.6</v>
+        <v>8.85</v>
       </c>
       <c r="N18" t="n">
-        <v>45.41</v>
+        <v>44.82</v>
       </c>
       <c r="O18" t="n">
-        <v>46.36</v>
+        <v>44.89</v>
       </c>
       <c r="P18" t="n">
-        <v>44.5</v>
+        <v>42.57</v>
       </c>
       <c r="Q18" t="n">
-        <v>45.73</v>
+        <v>42.57</v>
       </c>
       <c r="R18" t="n">
-        <v>-8.2906</v>
+        <v>16.3314</v>
       </c>
       <c r="S18" t="n">
-        <v>19.2474</v>
+        <v>22.7386</v>
       </c>
       <c r="T18" t="n">
-        <v>19.7826</v>
+        <v>35.6902</v>
       </c>
       <c r="U18" t="n">
-        <v>-0.3214</v>
+        <v>6.9246</v>
       </c>
       <c r="V18" t="n">
-        <v>9.906000000000001</v>
+        <v>13.1919</v>
       </c>
       <c r="W18" t="n">
-        <v>12.2757</v>
+        <v>16.8147</v>
       </c>
       <c r="X18" t="n">
-        <v>8.053000000000001</v>
+        <v>-16.5094</v>
       </c>
       <c r="Y18" t="n">
-        <v>-20.0603</v>
+        <v>-23.1103</v>
       </c>
       <c r="Z18" t="n">
-        <v>-20.3008</v>
+        <v>-31.8182</v>
       </c>
       <c r="AA18" t="n">
-        <v>0.3071</v>
+        <v>-6.9101</v>
       </c>
       <c r="AB18" t="n">
-        <v>-9.4635</v>
+        <v>-12.3894</v>
       </c>
       <c r="AC18" t="n">
-        <v>-11.4618</v>
+        <v>-15.233</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="C19" t="n">
-        <v>177.5</v>
+        <v>191.29</v>
       </c>
       <c r="D19" t="n">
-        <v>161.51</v>
+        <v>178.94</v>
       </c>
       <c r="E19" t="n">
-        <v>176.94</v>
+        <v>190.42</v>
       </c>
       <c r="F19" t="n">
-        <v>72.81999999999999</v>
+        <v>76</v>
       </c>
       <c r="G19" t="n">
-        <v>76.31</v>
+        <v>77.36</v>
       </c>
       <c r="H19" t="n">
-        <v>72.7</v>
+        <v>75.55</v>
       </c>
       <c r="I19" t="n">
-        <v>76.28</v>
+        <v>76.95999999999999</v>
       </c>
       <c r="J19" t="n">
-        <v>9.859999999999999</v>
+        <v>8.65</v>
       </c>
       <c r="K19" t="n">
-        <v>9.970000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="L19" t="n">
-        <v>8.84</v>
+        <v>8.15</v>
       </c>
       <c r="M19" t="n">
-        <v>8.85</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="N19" t="n">
-        <v>44.82</v>
+        <v>42.74</v>
       </c>
       <c r="O19" t="n">
-        <v>44.89</v>
+        <v>43</v>
       </c>
       <c r="P19" t="n">
-        <v>42.57</v>
+        <v>41.99</v>
       </c>
       <c r="Q19" t="n">
-        <v>42.57</v>
+        <v>42.22</v>
       </c>
       <c r="R19" t="n">
-        <v>16.3314</v>
+        <v>7.6184</v>
       </c>
       <c r="S19" t="n">
-        <v>22.7386</v>
+        <v>14.8146</v>
       </c>
       <c r="T19" t="n">
-        <v>35.6902</v>
+        <v>49.2905</v>
       </c>
       <c r="U19" t="n">
-        <v>6.9246</v>
+        <v>0.8915</v>
       </c>
       <c r="V19" t="n">
-        <v>13.1919</v>
+        <v>7.5311</v>
       </c>
       <c r="W19" t="n">
-        <v>16.8147</v>
+        <v>18.5642</v>
       </c>
       <c r="X19" t="n">
-        <v>-16.5094</v>
+        <v>-7.3446</v>
       </c>
       <c r="Y19" t="n">
-        <v>-23.1103</v>
+        <v>-16.4118</v>
       </c>
       <c r="Z19" t="n">
-        <v>-31.8182</v>
+        <v>-38.1599</v>
       </c>
       <c r="AA19" t="n">
-        <v>-6.9101</v>
+        <v>-0.8222</v>
       </c>
       <c r="AB19" t="n">
-        <v>-12.3894</v>
+        <v>-7.392</v>
       </c>
       <c r="AC19" t="n">
-        <v>-15.233</v>
+        <v>-16.4126</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>181</v>
+        <v>177.62</v>
       </c>
       <c r="C20" t="n">
-        <v>191.29</v>
+        <v>182.24</v>
       </c>
       <c r="D20" t="n">
-        <v>178.94</v>
+        <v>150.58</v>
       </c>
       <c r="E20" t="n">
-        <v>190.42</v>
+        <v>172.52</v>
       </c>
       <c r="F20" t="n">
-        <v>76</v>
+        <v>75.3</v>
       </c>
       <c r="G20" t="n">
-        <v>77.36</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="H20" t="n">
-        <v>75.55</v>
+        <v>71.55</v>
       </c>
       <c r="I20" t="n">
-        <v>76.95999999999999</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="J20" t="n">
-        <v>8.65</v>
+        <v>8.75</v>
       </c>
       <c r="K20" t="n">
-        <v>8.77</v>
+        <v>9.91</v>
       </c>
       <c r="L20" t="n">
-        <v>8.15</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="M20" t="n">
-        <v>8.199999999999999</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N20" t="n">
-        <v>42.74</v>
+        <v>43.14</v>
       </c>
       <c r="O20" t="n">
-        <v>43</v>
+        <v>45.19</v>
       </c>
       <c r="P20" t="n">
-        <v>41.99</v>
+        <v>42.79</v>
       </c>
       <c r="Q20" t="n">
-        <v>42.22</v>
+        <v>43.31</v>
       </c>
       <c r="R20" t="n">
-        <v>7.6184</v>
+        <v>-9.4003</v>
       </c>
       <c r="S20" t="n">
-        <v>14.8146</v>
+        <v>13.4254</v>
       </c>
       <c r="T20" t="n">
-        <v>49.2905</v>
+        <v>19.6726</v>
       </c>
       <c r="U20" t="n">
-        <v>0.8915</v>
+        <v>-2.5988</v>
       </c>
       <c r="V20" t="n">
-        <v>7.5311</v>
+        <v>5.0743</v>
       </c>
       <c r="W20" t="n">
-        <v>18.5642</v>
+        <v>11.2331</v>
       </c>
       <c r="X20" t="n">
-        <v>-7.3446</v>
+        <v>9.1463</v>
       </c>
       <c r="Y20" t="n">
-        <v>-16.4118</v>
+        <v>-15.566</v>
       </c>
       <c r="Z20" t="n">
-        <v>-38.1599</v>
+        <v>-22.2415</v>
       </c>
       <c r="AA20" t="n">
-        <v>-0.8222</v>
+        <v>2.5817</v>
       </c>
       <c r="AB20" t="n">
-        <v>-7.392</v>
+        <v>-5.2919</v>
       </c>
       <c r="AC20" t="n">
-        <v>-16.4126</v>
+        <v>-10.8664</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>177.62</v>
+        <v>183.84</v>
       </c>
       <c r="C21" t="n">
-        <v>182.24</v>
+        <v>188.49</v>
       </c>
       <c r="D21" t="n">
-        <v>150.58</v>
+        <v>172.26</v>
       </c>
       <c r="E21" t="n">
-        <v>172.52</v>
+        <v>184.24</v>
       </c>
       <c r="F21" t="n">
-        <v>75.3</v>
+        <v>75.81</v>
       </c>
       <c r="G21" t="n">
-        <v>75.93000000000001</v>
+        <v>77.94</v>
       </c>
       <c r="H21" t="n">
-        <v>71.55</v>
+        <v>74.19</v>
       </c>
       <c r="I21" t="n">
-        <v>74.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="J21" t="n">
-        <v>8.75</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K21" t="n">
-        <v>9.91</v>
+        <v>8.98</v>
       </c>
       <c r="L21" t="n">
-        <v>8.550000000000001</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="M21" t="n">
-        <v>8.949999999999999</v>
+        <v>8.35</v>
       </c>
       <c r="N21" t="n">
-        <v>43.14</v>
+        <v>42.83</v>
       </c>
       <c r="O21" t="n">
-        <v>45.19</v>
+        <v>43.77</v>
       </c>
       <c r="P21" t="n">
-        <v>42.79</v>
+        <v>41.6</v>
       </c>
       <c r="Q21" t="n">
-        <v>43.31</v>
+        <v>41.99</v>
       </c>
       <c r="R21" t="n">
-        <v>-9.4003</v>
+        <v>6.7934</v>
       </c>
       <c r="S21" t="n">
-        <v>13.4254</v>
+        <v>4.1257</v>
       </c>
       <c r="T21" t="n">
-        <v>19.6726</v>
+        <v>11.0883</v>
       </c>
       <c r="U21" t="n">
-        <v>-2.5988</v>
+        <v>3.0416</v>
       </c>
       <c r="V21" t="n">
-        <v>5.0743</v>
+        <v>1.2585</v>
       </c>
       <c r="W21" t="n">
-        <v>11.2331</v>
+        <v>7.9223</v>
       </c>
       <c r="X21" t="n">
-        <v>9.1463</v>
+        <v>-6.7039</v>
       </c>
       <c r="Y21" t="n">
-        <v>-15.566</v>
+        <v>-5.6497</v>
       </c>
       <c r="Z21" t="n">
-        <v>-22.2415</v>
+        <v>-14.8828</v>
       </c>
       <c r="AA21" t="n">
-        <v>2.5817</v>
+        <v>-3.0478</v>
       </c>
       <c r="AB21" t="n">
-        <v>-5.2919</v>
+        <v>-1.3625</v>
       </c>
       <c r="AC21" t="n">
-        <v>-10.8664</v>
+        <v>-7.8965</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>183.84</v>
+        <v>182.67</v>
       </c>
       <c r="C22" t="n">
-        <v>188.49</v>
+        <v>189.56</v>
       </c>
       <c r="D22" t="n">
-        <v>172.26</v>
+        <v>178.28</v>
       </c>
       <c r="E22" t="n">
-        <v>184.24</v>
+        <v>186.19</v>
       </c>
       <c r="F22" t="n">
-        <v>75.81</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G22" t="n">
-        <v>77.94</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>74.19</v>
+        <v>77.16</v>
       </c>
       <c r="I22" t="n">
-        <v>77.23999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="J22" t="n">
-        <v>8.380000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="K22" t="n">
-        <v>8.98</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L22" t="n">
-        <v>8.140000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M22" t="n">
-        <v>8.35</v>
+        <v>8.27</v>
       </c>
       <c r="N22" t="n">
-        <v>42.83</v>
+        <v>41.98</v>
       </c>
       <c r="O22" t="n">
-        <v>43.77</v>
+        <v>42.06</v>
       </c>
       <c r="P22" t="n">
-        <v>41.6</v>
+        <v>40.68</v>
       </c>
       <c r="Q22" t="n">
-        <v>41.99</v>
+        <v>41.07</v>
       </c>
       <c r="R22" t="n">
-        <v>6.7934</v>
+        <v>1.0584</v>
       </c>
       <c r="S22" t="n">
-        <v>4.1257</v>
+        <v>-2.2214</v>
       </c>
       <c r="T22" t="n">
-        <v>11.0883</v>
+        <v>22.4129</v>
       </c>
       <c r="U22" t="n">
-        <v>3.0416</v>
+        <v>2.2139</v>
       </c>
       <c r="V22" t="n">
-        <v>1.2585</v>
+        <v>2.5858</v>
       </c>
       <c r="W22" t="n">
-        <v>7.9223</v>
+        <v>10.6672</v>
       </c>
       <c r="X22" t="n">
-        <v>-6.7039</v>
+        <v>-0.9581</v>
       </c>
       <c r="Y22" t="n">
-        <v>-5.6497</v>
+        <v>0.8537</v>
       </c>
       <c r="Z22" t="n">
-        <v>-14.8828</v>
+        <v>-21.9811</v>
       </c>
       <c r="AA22" t="n">
-        <v>-3.0478</v>
+        <v>-2.191</v>
       </c>
       <c r="AB22" t="n">
-        <v>-1.3625</v>
+        <v>-2.7238</v>
       </c>
       <c r="AC22" t="n">
-        <v>-7.8965</v>
+        <v>-10.1902</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>182.67</v>
+        <v>167</v>
       </c>
       <c r="C23" t="n">
-        <v>189.56</v>
+        <v>174.4</v>
       </c>
       <c r="D23" t="n">
-        <v>178.28</v>
+        <v>161.1402</v>
       </c>
       <c r="E23" t="n">
-        <v>186.19</v>
+        <v>164.18</v>
       </c>
       <c r="F23" t="n">
-        <v>77.29000000000001</v>
+        <v>75.70999999999999</v>
       </c>
       <c r="G23" t="n">
-        <v>79.68000000000001</v>
+        <v>77.36499999999999</v>
       </c>
       <c r="H23" t="n">
-        <v>77.16</v>
+        <v>74.22799999999999</v>
       </c>
       <c r="I23" t="n">
-        <v>78.95</v>
+        <v>75.34</v>
       </c>
       <c r="J23" t="n">
-        <v>8.43</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="K23" t="n">
-        <v>8.630000000000001</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="L23" t="n">
-        <v>8.119999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M23" t="n">
-        <v>8.27</v>
+        <v>9.23</v>
       </c>
       <c r="N23" t="n">
-        <v>41.98</v>
+        <v>42.77</v>
       </c>
       <c r="O23" t="n">
-        <v>42.06</v>
+        <v>43.565</v>
       </c>
       <c r="P23" t="n">
-        <v>40.68</v>
+        <v>41.93</v>
       </c>
       <c r="Q23" t="n">
-        <v>41.07</v>
+        <v>42.98</v>
       </c>
       <c r="R23" t="n">
-        <v>1.0584</v>
+        <v>-11.8213</v>
       </c>
       <c r="S23" t="n">
-        <v>-2.2214</v>
+        <v>-4.8342</v>
       </c>
       <c r="T23" t="n">
-        <v>22.4129</v>
+        <v>-7.2115</v>
       </c>
       <c r="U23" t="n">
-        <v>2.2139</v>
+        <v>-4.5725</v>
       </c>
       <c r="V23" t="n">
-        <v>2.5858</v>
+        <v>0.5069</v>
       </c>
       <c r="W23" t="n">
-        <v>10.6672</v>
+        <v>-1.2323</v>
       </c>
       <c r="X23" t="n">
-        <v>-0.9581</v>
+        <v>11.6082</v>
       </c>
       <c r="Y23" t="n">
-        <v>0.8537</v>
+        <v>3.1285</v>
       </c>
       <c r="Z23" t="n">
-        <v>-21.9811</v>
+        <v>4.2938</v>
       </c>
       <c r="AA23" t="n">
-        <v>-2.191</v>
+        <v>4.6506</v>
       </c>
       <c r="AB23" t="n">
-        <v>-2.7238</v>
+        <v>-0.7619</v>
       </c>
       <c r="AC23" t="n">
-        <v>-10.1902</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>182.67</v>
-      </c>
-      <c r="C24" t="n">
-        <v>167.2739</v>
-      </c>
-      <c r="D24" t="n">
-        <v>165.3105</v>
-      </c>
-      <c r="E24" t="n">
-        <v>165.695</v>
-      </c>
-      <c r="F24" t="n">
-        <v>75.70999999999999</v>
-      </c>
-      <c r="G24" t="n">
-        <v>75.73999999999999</v>
-      </c>
-      <c r="H24" t="n">
-        <v>75.66</v>
-      </c>
-      <c r="I24" t="n">
-        <v>75.68000000000001</v>
-      </c>
-      <c r="J24" t="n">
-        <v>8.43</v>
-      </c>
-      <c r="K24" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="L24" t="n">
-        <v>9.109999999999999</v>
-      </c>
-      <c r="M24" t="n">
-        <v>9.19</v>
-      </c>
-      <c r="N24" t="n">
-        <v>42.77</v>
-      </c>
-      <c r="O24" t="n">
-        <v>42.81</v>
-      </c>
-      <c r="P24" t="n">
-        <v>42.765</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>42.81</v>
-      </c>
-      <c r="R24" t="n">
-        <v>-11.0076</v>
-      </c>
-      <c r="S24" t="n">
-        <v>-3.9561</v>
-      </c>
-      <c r="T24" t="n">
-        <v>-6.3553</v>
-      </c>
-      <c r="U24" t="n">
-        <v>-4.1419</v>
-      </c>
-      <c r="V24" t="n">
-        <v>0.9605</v>
-      </c>
-      <c r="W24" t="n">
-        <v>-0.7866</v>
-      </c>
-      <c r="X24" t="n">
-        <v>11.1245</v>
-      </c>
-      <c r="Y24" t="n">
-        <v>2.6816</v>
-      </c>
-      <c r="Z24" t="n">
-        <v>3.8418</v>
-      </c>
-      <c r="AA24" t="n">
-        <v>4.2367</v>
-      </c>
-      <c r="AB24" t="n">
-        <v>-1.1545</v>
-      </c>
-      <c r="AC24" t="n">
-        <v>0.5638</v>
+        <v>0.9631</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Master system update 2026-05-18 23:01
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC23"/>
+  <dimension ref="A1:AC22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1895 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>85.01000000000001</v>
+        <v>95.97</v>
       </c>
       <c r="C2" t="n">
-        <v>89.39</v>
+        <v>96.93000000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>83.31</v>
+        <v>92.03</v>
       </c>
       <c r="E2" t="n">
-        <v>88.37</v>
+        <v>95.94</v>
       </c>
       <c r="F2" t="n">
-        <v>56.13</v>
+        <v>58.4</v>
       </c>
       <c r="G2" t="n">
-        <v>56.92</v>
+        <v>58.58</v>
       </c>
       <c r="H2" t="n">
-        <v>55.1</v>
+        <v>56.91</v>
       </c>
       <c r="I2" t="n">
-        <v>56.43</v>
+        <v>58.08</v>
       </c>
       <c r="J2" t="n">
-        <v>21.13</v>
+        <v>18.64</v>
       </c>
       <c r="K2" t="n">
-        <v>21.56</v>
+        <v>19.41</v>
       </c>
       <c r="L2" t="n">
-        <v>20.07</v>
+        <v>18.44</v>
       </c>
       <c r="M2" t="n">
-        <v>20.28</v>
+        <v>18.63</v>
       </c>
       <c r="N2" t="n">
-        <v>58.95</v>
+        <v>56.59</v>
       </c>
       <c r="O2" t="n">
-        <v>60.06</v>
+        <v>58.04</v>
       </c>
       <c r="P2" t="n">
-        <v>58.11</v>
+        <v>56.41</v>
       </c>
       <c r="Q2" t="n">
-        <v>58.61</v>
+        <v>56.91</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>93.2</v>
+        <v>97.97</v>
       </c>
       <c r="C3" t="n">
-        <v>94.75</v>
+        <v>99.95</v>
       </c>
       <c r="D3" t="n">
-        <v>90.66</v>
+        <v>95.31999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>94.68000000000001</v>
+        <v>98.09</v>
       </c>
       <c r="F3" t="n">
-        <v>57.78</v>
+        <v>58.48</v>
       </c>
       <c r="G3" t="n">
-        <v>58.94</v>
+        <v>58.97</v>
       </c>
       <c r="H3" t="n">
-        <v>57.37</v>
+        <v>56.82</v>
       </c>
       <c r="I3" t="n">
-        <v>58.59</v>
+        <v>57.4</v>
       </c>
       <c r="J3" t="n">
-        <v>19.23</v>
+        <v>18.25</v>
       </c>
       <c r="K3" t="n">
-        <v>19.8</v>
+        <v>18.76</v>
       </c>
       <c r="L3" t="n">
-        <v>18.86</v>
+        <v>17.85</v>
       </c>
       <c r="M3" t="n">
-        <v>18.87</v>
+        <v>18.2</v>
       </c>
       <c r="N3" t="n">
-        <v>57.25</v>
+        <v>56.52</v>
       </c>
       <c r="O3" t="n">
-        <v>57.67</v>
+        <v>58.15</v>
       </c>
       <c r="P3" t="n">
         <v>56.04</v>
       </c>
       <c r="Q3" t="n">
-        <v>56.39</v>
+        <v>57.59</v>
       </c>
       <c r="R3" t="n">
-        <v>7.1404</v>
+        <v>2.241</v>
       </c>
       <c r="U3" t="n">
-        <v>3.8278</v>
+        <v>-1.1708</v>
       </c>
       <c r="X3" t="n">
-        <v>-6.9527</v>
+        <v>-2.3081</v>
       </c>
       <c r="AA3" t="n">
-        <v>-3.7877</v>
+        <v>1.1949</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>95.97</v>
+        <v>102.94</v>
       </c>
       <c r="C4" t="n">
-        <v>96.93000000000001</v>
+        <v>106.09</v>
       </c>
       <c r="D4" t="n">
-        <v>92.03</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>95.94</v>
+        <v>105.64</v>
       </c>
       <c r="F4" t="n">
-        <v>58.4</v>
+        <v>58.93</v>
       </c>
       <c r="G4" t="n">
-        <v>58.58</v>
+        <v>60.3</v>
       </c>
       <c r="H4" t="n">
-        <v>56.91</v>
+        <v>58.49</v>
       </c>
       <c r="I4" t="n">
-        <v>58.08</v>
+        <v>60.21</v>
       </c>
       <c r="J4" t="n">
-        <v>18.64</v>
+        <v>17.37</v>
       </c>
       <c r="K4" t="n">
-        <v>19.41</v>
+        <v>17.95</v>
       </c>
       <c r="L4" t="n">
-        <v>18.44</v>
+        <v>16.72</v>
       </c>
       <c r="M4" t="n">
-        <v>18.63</v>
+        <v>16.8</v>
       </c>
       <c r="N4" t="n">
-        <v>56.59</v>
+        <v>56.05</v>
       </c>
       <c r="O4" t="n">
-        <v>58.04</v>
+        <v>56.49</v>
       </c>
       <c r="P4" t="n">
-        <v>56.41</v>
+        <v>54.66</v>
       </c>
       <c r="Q4" t="n">
-        <v>56.91</v>
+        <v>54.73</v>
       </c>
       <c r="R4" t="n">
-        <v>1.3308</v>
+        <v>7.697</v>
       </c>
       <c r="U4" t="n">
-        <v>-0.8705000000000001</v>
+        <v>4.8955</v>
       </c>
       <c r="X4" t="n">
-        <v>-1.2719</v>
+        <v>-7.6923</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.9221</v>
+        <v>-4.9661</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>97.97</v>
+        <v>108.62</v>
       </c>
       <c r="C5" t="n">
-        <v>99.95</v>
+        <v>116.77</v>
       </c>
       <c r="D5" t="n">
-        <v>95.31999999999999</v>
+        <v>107.46</v>
       </c>
       <c r="E5" t="n">
-        <v>98.09</v>
+        <v>112.77</v>
       </c>
       <c r="F5" t="n">
-        <v>58.48</v>
+        <v>59.8</v>
       </c>
       <c r="G5" t="n">
-        <v>58.97</v>
+        <v>60.73</v>
       </c>
       <c r="H5" t="n">
-        <v>56.82</v>
+        <v>57.59</v>
       </c>
       <c r="I5" t="n">
-        <v>57.4</v>
+        <v>59.22</v>
       </c>
       <c r="J5" t="n">
-        <v>18.25</v>
+        <v>16.35</v>
       </c>
       <c r="K5" t="n">
-        <v>18.76</v>
+        <v>16.52</v>
       </c>
       <c r="L5" t="n">
-        <v>17.85</v>
+        <v>15.06</v>
       </c>
       <c r="M5" t="n">
-        <v>18.2</v>
+        <v>15.7</v>
       </c>
       <c r="N5" t="n">
-        <v>56.52</v>
+        <v>55.13</v>
       </c>
       <c r="O5" t="n">
-        <v>58.15</v>
+        <v>57.14</v>
       </c>
       <c r="P5" t="n">
-        <v>56.04</v>
+        <v>54.28</v>
       </c>
       <c r="Q5" t="n">
-        <v>57.59</v>
+        <v>55.66</v>
       </c>
       <c r="R5" t="n">
-        <v>2.241</v>
+        <v>6.7493</v>
       </c>
       <c r="S5" t="n">
-        <v>10.9992</v>
+        <v>17.5422</v>
       </c>
       <c r="U5" t="n">
-        <v>-1.1708</v>
+        <v>-1.6442</v>
       </c>
       <c r="V5" t="n">
-        <v>1.7189</v>
+        <v>1.9628</v>
       </c>
       <c r="X5" t="n">
-        <v>-2.3081</v>
+        <v>-6.5476</v>
       </c>
       <c r="Y5" t="n">
-        <v>-10.2564</v>
+        <v>-15.7273</v>
       </c>
       <c r="AA5" t="n">
-        <v>1.1949</v>
+        <v>1.6993</v>
       </c>
       <c r="AB5" t="n">
-        <v>-1.7403</v>
+        <v>-2.1965</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>102.94</v>
+        <v>125.21</v>
       </c>
       <c r="C6" t="n">
-        <v>106.09</v>
+        <v>130.12</v>
       </c>
       <c r="D6" t="n">
-        <v>99.59999999999999</v>
+        <v>120.24</v>
       </c>
       <c r="E6" t="n">
-        <v>105.64</v>
+        <v>128.32</v>
       </c>
       <c r="F6" t="n">
-        <v>58.93</v>
+        <v>61.08</v>
       </c>
       <c r="G6" t="n">
-        <v>60.3</v>
+        <v>62.74</v>
       </c>
       <c r="H6" t="n">
-        <v>58.49</v>
+        <v>60.56</v>
       </c>
       <c r="I6" t="n">
-        <v>60.21</v>
+        <v>62.56</v>
       </c>
       <c r="J6" t="n">
-        <v>17.37</v>
+        <v>13.99</v>
       </c>
       <c r="K6" t="n">
-        <v>17.95</v>
+        <v>14.66</v>
       </c>
       <c r="L6" t="n">
-        <v>16.72</v>
+        <v>13.3</v>
       </c>
       <c r="M6" t="n">
-        <v>16.8</v>
+        <v>13.52</v>
       </c>
       <c r="N6" t="n">
-        <v>56.05</v>
+        <v>53.93</v>
       </c>
       <c r="O6" t="n">
-        <v>56.49</v>
+        <v>54.43</v>
       </c>
       <c r="P6" t="n">
-        <v>54.66</v>
+        <v>52.37</v>
       </c>
       <c r="Q6" t="n">
-        <v>54.73</v>
+        <v>52.5</v>
       </c>
       <c r="R6" t="n">
-        <v>7.697</v>
+        <v>13.7891</v>
       </c>
       <c r="S6" t="n">
-        <v>11.5758</v>
+        <v>30.8186</v>
       </c>
       <c r="U6" t="n">
-        <v>4.8955</v>
+        <v>5.64</v>
       </c>
       <c r="V6" t="n">
-        <v>2.765</v>
+        <v>8.9895</v>
       </c>
       <c r="X6" t="n">
-        <v>-7.6923</v>
+        <v>-13.8854</v>
       </c>
       <c r="Y6" t="n">
-        <v>-10.9698</v>
+        <v>-25.7143</v>
       </c>
       <c r="AA6" t="n">
-        <v>-4.9661</v>
+        <v>-5.6773</v>
       </c>
       <c r="AB6" t="n">
-        <v>-2.9438</v>
+        <v>-8.8383</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>108.62</v>
+        <v>128.33</v>
       </c>
       <c r="C7" t="n">
-        <v>116.77</v>
+        <v>129.59</v>
       </c>
       <c r="D7" t="n">
-        <v>107.46</v>
+        <v>117.79</v>
       </c>
       <c r="E7" t="n">
-        <v>112.77</v>
+        <v>123.39</v>
       </c>
       <c r="F7" t="n">
-        <v>59.8</v>
+        <v>62.41</v>
       </c>
       <c r="G7" t="n">
-        <v>60.73</v>
+        <v>62.7</v>
       </c>
       <c r="H7" t="n">
-        <v>57.59</v>
+        <v>61.64</v>
       </c>
       <c r="I7" t="n">
-        <v>59.22</v>
+        <v>62.64</v>
       </c>
       <c r="J7" t="n">
-        <v>16.35</v>
+        <v>13.51</v>
       </c>
       <c r="K7" t="n">
-        <v>16.52</v>
+        <v>14.63</v>
       </c>
       <c r="L7" t="n">
-        <v>15.06</v>
+        <v>13.41</v>
       </c>
       <c r="M7" t="n">
-        <v>15.7</v>
+        <v>14.03</v>
       </c>
       <c r="N7" t="n">
-        <v>55.13</v>
+        <v>52.67</v>
       </c>
       <c r="O7" t="n">
-        <v>57.14</v>
+        <v>53.31</v>
       </c>
       <c r="P7" t="n">
-        <v>54.28</v>
+        <v>52.42</v>
       </c>
       <c r="Q7" t="n">
-        <v>55.66</v>
+        <v>52.45</v>
       </c>
       <c r="R7" t="n">
-        <v>6.7493</v>
+        <v>-3.842</v>
       </c>
       <c r="S7" t="n">
-        <v>17.5422</v>
+        <v>16.8023</v>
       </c>
       <c r="T7" t="n">
-        <v>27.6112</v>
+        <v>28.6116</v>
       </c>
       <c r="U7" t="n">
-        <v>-1.6442</v>
+        <v>0.1279</v>
       </c>
       <c r="V7" t="n">
-        <v>1.9628</v>
+        <v>4.0359</v>
       </c>
       <c r="W7" t="n">
-        <v>4.9442</v>
+        <v>7.8512</v>
       </c>
       <c r="X7" t="n">
-        <v>-6.5476</v>
+        <v>3.7722</v>
       </c>
       <c r="Y7" t="n">
-        <v>-15.7273</v>
+        <v>-16.4881</v>
       </c>
       <c r="Z7" t="n">
-        <v>-22.5838</v>
+        <v>-24.6914</v>
       </c>
       <c r="AA7" t="n">
-        <v>1.6993</v>
+        <v>-0.09520000000000001</v>
       </c>
       <c r="AB7" t="n">
-        <v>-2.1965</v>
+        <v>-4.1659</v>
       </c>
       <c r="AC7" t="n">
-        <v>-5.0333</v>
+        <v>-7.8369</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>125.21</v>
+        <v>108.75</v>
       </c>
       <c r="C8" t="n">
-        <v>130.12</v>
+        <v>115.62</v>
       </c>
       <c r="D8" t="n">
-        <v>120.24</v>
+        <v>103.99</v>
       </c>
       <c r="E8" t="n">
-        <v>128.32</v>
+        <v>109.56</v>
       </c>
       <c r="F8" t="n">
-        <v>61.08</v>
+        <v>60.72</v>
       </c>
       <c r="G8" t="n">
-        <v>62.74</v>
+        <v>61.33</v>
       </c>
       <c r="H8" t="n">
-        <v>60.56</v>
+        <v>59.68</v>
       </c>
       <c r="I8" t="n">
-        <v>62.56</v>
+        <v>60.74</v>
       </c>
       <c r="J8" t="n">
-        <v>13.99</v>
+        <v>15.71</v>
       </c>
       <c r="K8" t="n">
-        <v>14.66</v>
+        <v>16.27</v>
       </c>
       <c r="L8" t="n">
-        <v>13.3</v>
+        <v>14.93</v>
       </c>
       <c r="M8" t="n">
-        <v>13.52</v>
+        <v>15.59</v>
       </c>
       <c r="N8" t="n">
-        <v>53.93</v>
+        <v>54.09</v>
       </c>
       <c r="O8" t="n">
-        <v>54.43</v>
+        <v>54.96</v>
       </c>
       <c r="P8" t="n">
-        <v>52.37</v>
+        <v>53.58</v>
       </c>
       <c r="Q8" t="n">
-        <v>52.5</v>
+        <v>54.05</v>
       </c>
       <c r="R8" t="n">
-        <v>13.7891</v>
+        <v>-11.2084</v>
       </c>
       <c r="S8" t="n">
-        <v>30.8186</v>
+        <v>-2.8465</v>
       </c>
       <c r="T8" t="n">
-        <v>35.5302</v>
+        <v>11.6933</v>
       </c>
       <c r="U8" t="n">
-        <v>5.64</v>
+        <v>-3.0332</v>
       </c>
       <c r="V8" t="n">
-        <v>8.9895</v>
+        <v>2.5667</v>
       </c>
       <c r="W8" t="n">
-        <v>6.7759</v>
+        <v>5.8188</v>
       </c>
       <c r="X8" t="n">
-        <v>-13.8854</v>
+        <v>11.119</v>
       </c>
       <c r="Y8" t="n">
-        <v>-25.7143</v>
+        <v>-0.7006</v>
       </c>
       <c r="Z8" t="n">
-        <v>-28.3519</v>
+        <v>-14.3407</v>
       </c>
       <c r="AA8" t="n">
-        <v>-5.6773</v>
+        <v>3.0505</v>
       </c>
       <c r="AB8" t="n">
-        <v>-8.8383</v>
+        <v>-2.8926</v>
       </c>
       <c r="AC8" t="n">
-        <v>-6.8984</v>
+        <v>-6.1469</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>128.33</v>
+        <v>114.76</v>
       </c>
       <c r="C9" t="n">
-        <v>129.59</v>
+        <v>118.32</v>
       </c>
       <c r="D9" t="n">
-        <v>117.79</v>
+        <v>112.3</v>
       </c>
       <c r="E9" t="n">
-        <v>123.39</v>
+        <v>117.97</v>
       </c>
       <c r="F9" t="n">
-        <v>62.41</v>
+        <v>61</v>
       </c>
       <c r="G9" t="n">
-        <v>62.7</v>
+        <v>61.87</v>
       </c>
       <c r="H9" t="n">
-        <v>61.64</v>
+        <v>60.45</v>
       </c>
       <c r="I9" t="n">
-        <v>62.64</v>
+        <v>61.86</v>
       </c>
       <c r="J9" t="n">
-        <v>13.51</v>
+        <v>14.91</v>
       </c>
       <c r="K9" t="n">
-        <v>14.63</v>
+        <v>15.24</v>
       </c>
       <c r="L9" t="n">
-        <v>13.41</v>
+        <v>14.38</v>
       </c>
       <c r="M9" t="n">
-        <v>14.03</v>
+        <v>14.4</v>
       </c>
       <c r="N9" t="n">
-        <v>52.67</v>
+        <v>53.84</v>
       </c>
       <c r="O9" t="n">
-        <v>53.31</v>
+        <v>54.33</v>
       </c>
       <c r="P9" t="n">
-        <v>52.42</v>
+        <v>53.06</v>
       </c>
       <c r="Q9" t="n">
-        <v>52.45</v>
+        <v>53.08</v>
       </c>
       <c r="R9" t="n">
-        <v>-3.842</v>
+        <v>7.6762</v>
       </c>
       <c r="S9" t="n">
-        <v>16.8023</v>
+        <v>-8.065799999999999</v>
       </c>
       <c r="T9" t="n">
-        <v>28.6116</v>
+        <v>11.6717</v>
       </c>
       <c r="U9" t="n">
-        <v>0.1279</v>
+        <v>1.8439</v>
       </c>
       <c r="V9" t="n">
-        <v>4.0359</v>
+        <v>-1.1189</v>
       </c>
       <c r="W9" t="n">
-        <v>7.8512</v>
+        <v>2.7404</v>
       </c>
       <c r="X9" t="n">
-        <v>3.7722</v>
+        <v>-7.6331</v>
       </c>
       <c r="Y9" t="n">
-        <v>-16.4881</v>
+        <v>6.5089</v>
       </c>
       <c r="Z9" t="n">
-        <v>-24.6914</v>
+        <v>-14.2857</v>
       </c>
       <c r="AA9" t="n">
-        <v>-0.09520000000000001</v>
+        <v>-1.7946</v>
       </c>
       <c r="AB9" t="n">
-        <v>-4.1659</v>
+        <v>1.1048</v>
       </c>
       <c r="AC9" t="n">
-        <v>-7.8369</v>
+        <v>-3.0148</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>108.75</v>
+        <v>122.81</v>
       </c>
       <c r="C10" t="n">
-        <v>115.62</v>
+        <v>127.45</v>
       </c>
       <c r="D10" t="n">
-        <v>103.99</v>
+        <v>117.5</v>
       </c>
       <c r="E10" t="n">
-        <v>109.56</v>
+        <v>126.98</v>
       </c>
       <c r="F10" t="n">
-        <v>60.72</v>
+        <v>62.89</v>
       </c>
       <c r="G10" t="n">
-        <v>61.33</v>
+        <v>63.8</v>
       </c>
       <c r="H10" t="n">
-        <v>59.68</v>
+        <v>60.7</v>
       </c>
       <c r="I10" t="n">
-        <v>60.74</v>
+        <v>63.54</v>
       </c>
       <c r="J10" t="n">
-        <v>15.71</v>
+        <v>13.84</v>
       </c>
       <c r="K10" t="n">
-        <v>16.27</v>
+        <v>14.49</v>
       </c>
       <c r="L10" t="n">
-        <v>14.93</v>
+        <v>13.25</v>
       </c>
       <c r="M10" t="n">
-        <v>15.59</v>
+        <v>13.3</v>
       </c>
       <c r="N10" t="n">
+        <v>52.21</v>
+      </c>
+      <c r="O10" t="n">
         <v>54.09</v>
       </c>
-      <c r="O10" t="n">
-        <v>54.96</v>
-      </c>
       <c r="P10" t="n">
-        <v>53.58</v>
+        <v>51.4</v>
       </c>
       <c r="Q10" t="n">
-        <v>54.05</v>
+        <v>51.65</v>
       </c>
       <c r="R10" t="n">
-        <v>-11.2084</v>
+        <v>7.6375</v>
       </c>
       <c r="S10" t="n">
-        <v>-2.8465</v>
+        <v>2.9095</v>
       </c>
       <c r="T10" t="n">
-        <v>11.6933</v>
+        <v>12.6009</v>
       </c>
       <c r="U10" t="n">
-        <v>-3.0332</v>
+        <v>2.7158</v>
       </c>
       <c r="V10" t="n">
-        <v>2.5667</v>
+        <v>1.4368</v>
       </c>
       <c r="W10" t="n">
-        <v>5.8188</v>
+        <v>7.2948</v>
       </c>
       <c r="X10" t="n">
-        <v>11.119</v>
+        <v>-7.6389</v>
       </c>
       <c r="Y10" t="n">
-        <v>-0.7006</v>
+        <v>-5.2031</v>
       </c>
       <c r="Z10" t="n">
-        <v>-14.3407</v>
+        <v>-15.2866</v>
       </c>
       <c r="AA10" t="n">
-        <v>3.0505</v>
+        <v>-2.694</v>
       </c>
       <c r="AB10" t="n">
-        <v>-2.8926</v>
+        <v>-1.5253</v>
       </c>
       <c r="AC10" t="n">
-        <v>-6.1469</v>
+        <v>-7.2045</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>114.76</v>
+        <v>124.39</v>
       </c>
       <c r="C11" t="n">
-        <v>118.32</v>
+        <v>131.38</v>
       </c>
       <c r="D11" t="n">
-        <v>112.3</v>
+        <v>121.66</v>
       </c>
       <c r="E11" t="n">
-        <v>117.97</v>
+        <v>130.4</v>
       </c>
       <c r="F11" t="n">
-        <v>61</v>
+        <v>63.89</v>
       </c>
       <c r="G11" t="n">
-        <v>61.87</v>
+        <v>65.84</v>
       </c>
       <c r="H11" t="n">
-        <v>60.45</v>
+        <v>63.81</v>
       </c>
       <c r="I11" t="n">
-        <v>61.86</v>
+        <v>65.3</v>
       </c>
       <c r="J11" t="n">
-        <v>14.91</v>
+        <v>13.61</v>
       </c>
       <c r="K11" t="n">
-        <v>15.24</v>
+        <v>13.89</v>
       </c>
       <c r="L11" t="n">
-        <v>14.38</v>
+        <v>12.87</v>
       </c>
       <c r="M11" t="n">
-        <v>14.4</v>
+        <v>12.98</v>
       </c>
       <c r="N11" t="n">
-        <v>53.84</v>
+        <v>51.36</v>
       </c>
       <c r="O11" t="n">
-        <v>54.33</v>
+        <v>51.45</v>
       </c>
       <c r="P11" t="n">
-        <v>53.06</v>
+        <v>49.79</v>
       </c>
       <c r="Q11" t="n">
-        <v>53.08</v>
+        <v>50.22</v>
       </c>
       <c r="R11" t="n">
-        <v>7.6762</v>
+        <v>2.6933</v>
       </c>
       <c r="S11" t="n">
-        <v>-8.065799999999999</v>
+        <v>19.0215</v>
       </c>
       <c r="T11" t="n">
-        <v>11.6717</v>
+        <v>1.6209</v>
       </c>
       <c r="U11" t="n">
-        <v>1.8439</v>
+        <v>2.7699</v>
       </c>
       <c r="V11" t="n">
-        <v>-1.1189</v>
+        <v>7.5074</v>
       </c>
       <c r="W11" t="n">
-        <v>2.7404</v>
+        <v>4.3798</v>
       </c>
       <c r="X11" t="n">
-        <v>-7.6331</v>
+        <v>-2.406</v>
       </c>
       <c r="Y11" t="n">
-        <v>6.5089</v>
+        <v>-16.7415</v>
       </c>
       <c r="Z11" t="n">
-        <v>-14.2857</v>
+        <v>-3.9941</v>
       </c>
       <c r="AA11" t="n">
-        <v>-1.7946</v>
+        <v>-2.7686</v>
       </c>
       <c r="AB11" t="n">
-        <v>1.1048</v>
+        <v>-7.086</v>
       </c>
       <c r="AC11" t="n">
-        <v>-3.0148</v>
+        <v>-4.3429</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>122.81</v>
+        <v>132.2</v>
       </c>
       <c r="C12" t="n">
-        <v>127.45</v>
+        <v>133.67</v>
       </c>
       <c r="D12" t="n">
-        <v>117.5</v>
+        <v>123.8</v>
       </c>
       <c r="E12" t="n">
-        <v>126.98</v>
+        <v>127.55</v>
       </c>
       <c r="F12" t="n">
-        <v>62.89</v>
+        <v>65.44</v>
       </c>
       <c r="G12" t="n">
-        <v>63.8</v>
+        <v>66.05</v>
       </c>
       <c r="H12" t="n">
-        <v>60.7</v>
+        <v>63.78</v>
       </c>
       <c r="I12" t="n">
-        <v>63.54</v>
+        <v>64.91</v>
       </c>
       <c r="J12" t="n">
-        <v>13.84</v>
+        <v>12.8</v>
       </c>
       <c r="K12" t="n">
-        <v>14.49</v>
+        <v>13.64</v>
       </c>
       <c r="L12" t="n">
-        <v>13.25</v>
+        <v>12.65</v>
       </c>
       <c r="M12" t="n">
-        <v>13.3</v>
+        <v>13.26</v>
       </c>
       <c r="N12" t="n">
-        <v>52.21</v>
+        <v>50.12</v>
       </c>
       <c r="O12" t="n">
-        <v>54.09</v>
+        <v>51.43</v>
       </c>
       <c r="P12" t="n">
-        <v>51.4</v>
+        <v>49.65</v>
       </c>
       <c r="Q12" t="n">
-        <v>51.65</v>
+        <v>50.51</v>
       </c>
       <c r="R12" t="n">
-        <v>7.6375</v>
+        <v>-2.1856</v>
       </c>
       <c r="S12" t="n">
-        <v>2.9095</v>
+        <v>8.120699999999999</v>
       </c>
       <c r="T12" t="n">
-        <v>12.6009</v>
+        <v>3.3714</v>
       </c>
       <c r="U12" t="n">
-        <v>2.7158</v>
+        <v>-0.5972</v>
       </c>
       <c r="V12" t="n">
-        <v>1.4368</v>
+        <v>4.9305</v>
       </c>
       <c r="W12" t="n">
-        <v>7.2948</v>
+        <v>3.6239</v>
       </c>
       <c r="X12" t="n">
-        <v>-7.6389</v>
+        <v>2.1572</v>
       </c>
       <c r="Y12" t="n">
-        <v>-5.2031</v>
+        <v>-7.9167</v>
       </c>
       <c r="Z12" t="n">
-        <v>-15.2866</v>
+        <v>-5.4882</v>
       </c>
       <c r="AA12" t="n">
-        <v>-2.694</v>
+        <v>0.5775</v>
       </c>
       <c r="AB12" t="n">
-        <v>-1.5253</v>
+        <v>-4.8417</v>
       </c>
       <c r="AC12" t="n">
-        <v>-7.2045</v>
+        <v>-3.6988</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>124.39</v>
+        <v>135</v>
       </c>
       <c r="C13" t="n">
-        <v>131.38</v>
+        <v>147.26</v>
       </c>
       <c r="D13" t="n">
-        <v>121.66</v>
+        <v>134.02</v>
       </c>
       <c r="E13" t="n">
-        <v>130.4</v>
+        <v>144.16</v>
       </c>
       <c r="F13" t="n">
-        <v>63.89</v>
+        <v>66.37</v>
       </c>
       <c r="G13" t="n">
-        <v>65.84</v>
+        <v>67.77</v>
       </c>
       <c r="H13" t="n">
-        <v>63.81</v>
+        <v>66.25</v>
       </c>
       <c r="I13" t="n">
-        <v>65.3</v>
+        <v>67.39</v>
       </c>
       <c r="J13" t="n">
-        <v>13.61</v>
+        <v>12.5</v>
       </c>
       <c r="K13" t="n">
-        <v>13.89</v>
+        <v>12.59</v>
       </c>
       <c r="L13" t="n">
-        <v>12.87</v>
+        <v>11.21</v>
       </c>
       <c r="M13" t="n">
-        <v>12.98</v>
+        <v>11.51</v>
       </c>
       <c r="N13" t="n">
-        <v>51.36</v>
+        <v>49.4</v>
       </c>
       <c r="O13" t="n">
-        <v>51.45</v>
+        <v>49.49</v>
       </c>
       <c r="P13" t="n">
-        <v>49.79</v>
+        <v>48.3</v>
       </c>
       <c r="Q13" t="n">
-        <v>50.22</v>
+        <v>48.59</v>
       </c>
       <c r="R13" t="n">
-        <v>2.6933</v>
+        <v>13.0223</v>
       </c>
       <c r="S13" t="n">
-        <v>19.0215</v>
+        <v>13.5297</v>
       </c>
       <c r="T13" t="n">
-        <v>1.6209</v>
+        <v>31.5809</v>
       </c>
       <c r="U13" t="n">
-        <v>2.7699</v>
+        <v>3.8207</v>
       </c>
       <c r="V13" t="n">
-        <v>7.5074</v>
+        <v>6.0592</v>
       </c>
       <c r="W13" t="n">
-        <v>4.3798</v>
+        <v>10.9483</v>
       </c>
       <c r="X13" t="n">
-        <v>-2.406</v>
+        <v>-13.1976</v>
       </c>
       <c r="Y13" t="n">
-        <v>-16.7415</v>
+        <v>-13.4586</v>
       </c>
       <c r="Z13" t="n">
-        <v>-3.9941</v>
+        <v>-26.1706</v>
       </c>
       <c r="AA13" t="n">
-        <v>-2.7686</v>
+        <v>-3.8012</v>
       </c>
       <c r="AB13" t="n">
-        <v>-7.086</v>
+        <v>-5.9245</v>
       </c>
       <c r="AC13" t="n">
-        <v>-4.3429</v>
+        <v>-10.1018</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>132.2</v>
+        <v>157.84</v>
       </c>
       <c r="C14" t="n">
-        <v>133.67</v>
+        <v>166</v>
       </c>
       <c r="D14" t="n">
-        <v>123.8</v>
+        <v>149.06</v>
       </c>
       <c r="E14" t="n">
-        <v>127.55</v>
+        <v>165.85</v>
       </c>
       <c r="F14" t="n">
-        <v>65.44</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>66.05</v>
+        <v>71.66</v>
       </c>
       <c r="H14" t="n">
-        <v>63.78</v>
+        <v>68.88</v>
       </c>
       <c r="I14" t="n">
-        <v>64.91</v>
+        <v>71.56999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>12.8</v>
+        <v>10.43</v>
       </c>
       <c r="K14" t="n">
-        <v>13.64</v>
+        <v>11.14</v>
       </c>
       <c r="L14" t="n">
-        <v>12.65</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M14" t="n">
-        <v>13.26</v>
+        <v>9.81</v>
       </c>
       <c r="N14" t="n">
-        <v>50.12</v>
+        <v>47.26</v>
       </c>
       <c r="O14" t="n">
-        <v>51.43</v>
+        <v>47.54</v>
       </c>
       <c r="P14" t="n">
-        <v>49.65</v>
+        <v>45.52</v>
       </c>
       <c r="Q14" t="n">
-        <v>50.51</v>
+        <v>45.59</v>
       </c>
       <c r="R14" t="n">
-        <v>-2.1856</v>
+        <v>15.0458</v>
       </c>
       <c r="S14" t="n">
-        <v>8.120699999999999</v>
+        <v>27.1856</v>
       </c>
       <c r="T14" t="n">
-        <v>3.3714</v>
+        <v>40.5866</v>
       </c>
       <c r="U14" t="n">
-        <v>-0.5972</v>
+        <v>6.2027</v>
       </c>
       <c r="V14" t="n">
-        <v>4.9305</v>
+        <v>9.601800000000001</v>
       </c>
       <c r="W14" t="n">
-        <v>3.6239</v>
+        <v>15.6967</v>
       </c>
       <c r="X14" t="n">
-        <v>2.1572</v>
+        <v>-14.7698</v>
       </c>
       <c r="Y14" t="n">
-        <v>-7.9167</v>
+        <v>-24.4222</v>
       </c>
       <c r="Z14" t="n">
-        <v>-5.4882</v>
+        <v>-31.875</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.5775</v>
+        <v>-6.1741</v>
       </c>
       <c r="AB14" t="n">
-        <v>-4.8417</v>
+        <v>-9.2194</v>
       </c>
       <c r="AC14" t="n">
-        <v>-3.6988</v>
+        <v>-14.1108</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>135</v>
+        <v>162.12</v>
       </c>
       <c r="C15" t="n">
-        <v>147.26</v>
+        <v>162.9</v>
       </c>
       <c r="D15" t="n">
-        <v>134.02</v>
+        <v>147.61</v>
       </c>
       <c r="E15" t="n">
-        <v>144.16</v>
+        <v>152.1</v>
       </c>
       <c r="F15" t="n">
-        <v>66.37</v>
+        <v>71.87</v>
       </c>
       <c r="G15" t="n">
-        <v>67.77</v>
+        <v>73.3</v>
       </c>
       <c r="H15" t="n">
-        <v>66.25</v>
+        <v>70.38</v>
       </c>
       <c r="I15" t="n">
-        <v>67.39</v>
+        <v>71.34</v>
       </c>
       <c r="J15" t="n">
-        <v>12.5</v>
+        <v>10.02</v>
       </c>
       <c r="K15" t="n">
-        <v>12.59</v>
+        <v>10.88</v>
       </c>
       <c r="L15" t="n">
-        <v>11.21</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="M15" t="n">
-        <v>11.51</v>
+        <v>10.6</v>
       </c>
       <c r="N15" t="n">
-        <v>49.4</v>
+        <v>45.41</v>
       </c>
       <c r="O15" t="n">
-        <v>49.49</v>
+        <v>46.36</v>
       </c>
       <c r="P15" t="n">
-        <v>48.3</v>
+        <v>44.5</v>
       </c>
       <c r="Q15" t="n">
-        <v>48.59</v>
+        <v>45.73</v>
       </c>
       <c r="R15" t="n">
-        <v>13.0223</v>
+        <v>-8.2906</v>
       </c>
       <c r="S15" t="n">
-        <v>13.5297</v>
+        <v>19.2474</v>
       </c>
       <c r="T15" t="n">
-        <v>31.5809</v>
+        <v>19.7826</v>
       </c>
       <c r="U15" t="n">
-        <v>3.8207</v>
+        <v>-0.3214</v>
       </c>
       <c r="V15" t="n">
-        <v>6.0592</v>
+        <v>9.906000000000001</v>
       </c>
       <c r="W15" t="n">
-        <v>10.9483</v>
+        <v>12.2757</v>
       </c>
       <c r="X15" t="n">
-        <v>-13.1976</v>
+        <v>8.053000000000001</v>
       </c>
       <c r="Y15" t="n">
-        <v>-13.4586</v>
+        <v>-20.0603</v>
       </c>
       <c r="Z15" t="n">
-        <v>-26.1706</v>
+        <v>-20.3008</v>
       </c>
       <c r="AA15" t="n">
-        <v>-3.8012</v>
+        <v>0.3071</v>
       </c>
       <c r="AB15" t="n">
-        <v>-5.9245</v>
+        <v>-9.4635</v>
       </c>
       <c r="AC15" t="n">
-        <v>-10.1018</v>
+        <v>-11.4618</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>157.84</v>
+        <v>163</v>
       </c>
       <c r="C16" t="n">
-        <v>166</v>
+        <v>177.5</v>
       </c>
       <c r="D16" t="n">
-        <v>149.06</v>
+        <v>161.51</v>
       </c>
       <c r="E16" t="n">
-        <v>165.85</v>
+        <v>176.94</v>
       </c>
       <c r="F16" t="n">
-        <v>69.26000000000001</v>
+        <v>72.81999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>71.66</v>
+        <v>76.31</v>
       </c>
       <c r="H16" t="n">
-        <v>68.88</v>
+        <v>72.7</v>
       </c>
       <c r="I16" t="n">
-        <v>71.56999999999999</v>
+        <v>76.28</v>
       </c>
       <c r="J16" t="n">
-        <v>10.43</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="K16" t="n">
-        <v>11.14</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="L16" t="n">
-        <v>9.800000000000001</v>
+        <v>8.84</v>
       </c>
       <c r="M16" t="n">
-        <v>9.81</v>
+        <v>8.85</v>
       </c>
       <c r="N16" t="n">
-        <v>47.26</v>
+        <v>44.82</v>
       </c>
       <c r="O16" t="n">
-        <v>47.54</v>
+        <v>44.89</v>
       </c>
       <c r="P16" t="n">
-        <v>45.52</v>
+        <v>42.57</v>
       </c>
       <c r="Q16" t="n">
-        <v>45.59</v>
+        <v>42.57</v>
       </c>
       <c r="R16" t="n">
-        <v>15.0458</v>
+        <v>16.3314</v>
       </c>
       <c r="S16" t="n">
-        <v>27.1856</v>
+        <v>22.7386</v>
       </c>
       <c r="T16" t="n">
-        <v>40.5866</v>
+        <v>35.6902</v>
       </c>
       <c r="U16" t="n">
-        <v>6.2027</v>
+        <v>6.9246</v>
       </c>
       <c r="V16" t="n">
-        <v>9.601800000000001</v>
+        <v>13.1919</v>
       </c>
       <c r="W16" t="n">
-        <v>15.6967</v>
+        <v>16.8147</v>
       </c>
       <c r="X16" t="n">
-        <v>-14.7698</v>
+        <v>-16.5094</v>
       </c>
       <c r="Y16" t="n">
-        <v>-24.4222</v>
+        <v>-23.1103</v>
       </c>
       <c r="Z16" t="n">
-        <v>-31.875</v>
+        <v>-31.8182</v>
       </c>
       <c r="AA16" t="n">
-        <v>-6.1741</v>
+        <v>-6.9101</v>
       </c>
       <c r="AB16" t="n">
-        <v>-9.2194</v>
+        <v>-12.3894</v>
       </c>
       <c r="AC16" t="n">
-        <v>-14.1108</v>
+        <v>-15.233</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>162.12</v>
+        <v>181</v>
       </c>
       <c r="C17" t="n">
-        <v>162.9</v>
+        <v>191.29</v>
       </c>
       <c r="D17" t="n">
-        <v>147.61</v>
+        <v>178.94</v>
       </c>
       <c r="E17" t="n">
-        <v>152.1</v>
+        <v>190.42</v>
       </c>
       <c r="F17" t="n">
-        <v>71.87</v>
+        <v>76</v>
       </c>
       <c r="G17" t="n">
-        <v>73.3</v>
+        <v>77.36</v>
       </c>
       <c r="H17" t="n">
-        <v>70.38</v>
+        <v>75.55</v>
       </c>
       <c r="I17" t="n">
-        <v>71.34</v>
+        <v>76.95999999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>10.02</v>
+        <v>8.65</v>
       </c>
       <c r="K17" t="n">
-        <v>10.88</v>
+        <v>8.77</v>
       </c>
       <c r="L17" t="n">
-        <v>9.970000000000001</v>
+        <v>8.15</v>
       </c>
       <c r="M17" t="n">
-        <v>10.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="N17" t="n">
-        <v>45.41</v>
+        <v>42.74</v>
       </c>
       <c r="O17" t="n">
-        <v>46.36</v>
+        <v>43</v>
       </c>
       <c r="P17" t="n">
-        <v>44.5</v>
+        <v>41.99</v>
       </c>
       <c r="Q17" t="n">
-        <v>45.73</v>
+        <v>42.22</v>
       </c>
       <c r="R17" t="n">
-        <v>-8.2906</v>
+        <v>7.6184</v>
       </c>
       <c r="S17" t="n">
-        <v>19.2474</v>
+        <v>14.8146</v>
       </c>
       <c r="T17" t="n">
-        <v>19.7826</v>
+        <v>49.2905</v>
       </c>
       <c r="U17" t="n">
-        <v>-0.3214</v>
+        <v>0.8915</v>
       </c>
       <c r="V17" t="n">
-        <v>9.906000000000001</v>
+        <v>7.5311</v>
       </c>
       <c r="W17" t="n">
-        <v>12.2757</v>
+        <v>18.5642</v>
       </c>
       <c r="X17" t="n">
-        <v>8.053000000000001</v>
+        <v>-7.3446</v>
       </c>
       <c r="Y17" t="n">
-        <v>-20.0603</v>
+        <v>-16.4118</v>
       </c>
       <c r="Z17" t="n">
-        <v>-20.3008</v>
+        <v>-38.1599</v>
       </c>
       <c r="AA17" t="n">
-        <v>0.3071</v>
+        <v>-0.8222</v>
       </c>
       <c r="AB17" t="n">
-        <v>-9.4635</v>
+        <v>-7.392</v>
       </c>
       <c r="AC17" t="n">
-        <v>-11.4618</v>
+        <v>-16.4126</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>163</v>
+        <v>177.62</v>
       </c>
       <c r="C18" t="n">
-        <v>177.5</v>
+        <v>182.24</v>
       </c>
       <c r="D18" t="n">
-        <v>161.51</v>
+        <v>150.58</v>
       </c>
       <c r="E18" t="n">
-        <v>176.94</v>
+        <v>172.52</v>
       </c>
       <c r="F18" t="n">
-        <v>72.81999999999999</v>
+        <v>75.3</v>
       </c>
       <c r="G18" t="n">
-        <v>76.31</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="H18" t="n">
-        <v>72.7</v>
+        <v>71.55</v>
       </c>
       <c r="I18" t="n">
-        <v>76.28</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="J18" t="n">
-        <v>9.859999999999999</v>
+        <v>8.75</v>
       </c>
       <c r="K18" t="n">
-        <v>9.970000000000001</v>
+        <v>9.91</v>
       </c>
       <c r="L18" t="n">
-        <v>8.84</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="M18" t="n">
-        <v>8.85</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N18" t="n">
-        <v>44.82</v>
+        <v>43.14</v>
       </c>
       <c r="O18" t="n">
-        <v>44.89</v>
+        <v>45.19</v>
       </c>
       <c r="P18" t="n">
-        <v>42.57</v>
+        <v>42.79</v>
       </c>
       <c r="Q18" t="n">
-        <v>42.57</v>
+        <v>43.31</v>
       </c>
       <c r="R18" t="n">
-        <v>16.3314</v>
+        <v>-9.4003</v>
       </c>
       <c r="S18" t="n">
-        <v>22.7386</v>
+        <v>13.4254</v>
       </c>
       <c r="T18" t="n">
-        <v>35.6902</v>
+        <v>19.6726</v>
       </c>
       <c r="U18" t="n">
-        <v>6.9246</v>
+        <v>-2.5988</v>
       </c>
       <c r="V18" t="n">
-        <v>13.1919</v>
+        <v>5.0743</v>
       </c>
       <c r="W18" t="n">
-        <v>16.8147</v>
+        <v>11.2331</v>
       </c>
       <c r="X18" t="n">
-        <v>-16.5094</v>
+        <v>9.1463</v>
       </c>
       <c r="Y18" t="n">
-        <v>-23.1103</v>
+        <v>-15.566</v>
       </c>
       <c r="Z18" t="n">
-        <v>-31.8182</v>
+        <v>-22.2415</v>
       </c>
       <c r="AA18" t="n">
-        <v>-6.9101</v>
+        <v>2.5817</v>
       </c>
       <c r="AB18" t="n">
-        <v>-12.3894</v>
+        <v>-5.2919</v>
       </c>
       <c r="AC18" t="n">
-        <v>-15.233</v>
+        <v>-10.8664</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>181</v>
+        <v>183.84</v>
       </c>
       <c r="C19" t="n">
-        <v>191.29</v>
+        <v>188.49</v>
       </c>
       <c r="D19" t="n">
-        <v>178.94</v>
+        <v>172.26</v>
       </c>
       <c r="E19" t="n">
-        <v>190.42</v>
+        <v>184.24</v>
       </c>
       <c r="F19" t="n">
-        <v>76</v>
+        <v>75.81</v>
       </c>
       <c r="G19" t="n">
-        <v>77.36</v>
+        <v>77.94</v>
       </c>
       <c r="H19" t="n">
-        <v>75.55</v>
+        <v>74.19</v>
       </c>
       <c r="I19" t="n">
-        <v>76.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="J19" t="n">
-        <v>8.65</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K19" t="n">
-        <v>8.77</v>
+        <v>8.98</v>
       </c>
       <c r="L19" t="n">
-        <v>8.15</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="M19" t="n">
-        <v>8.199999999999999</v>
+        <v>8.35</v>
       </c>
       <c r="N19" t="n">
-        <v>42.74</v>
+        <v>42.83</v>
       </c>
       <c r="O19" t="n">
-        <v>43</v>
+        <v>43.77</v>
       </c>
       <c r="P19" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="Q19" t="n">
         <v>41.99</v>
       </c>
-      <c r="Q19" t="n">
-        <v>42.22</v>
-      </c>
       <c r="R19" t="n">
-        <v>7.6184</v>
+        <v>6.7934</v>
       </c>
       <c r="S19" t="n">
-        <v>14.8146</v>
+        <v>4.1257</v>
       </c>
       <c r="T19" t="n">
-        <v>49.2905</v>
+        <v>11.0883</v>
       </c>
       <c r="U19" t="n">
-        <v>0.8915</v>
+        <v>3.0416</v>
       </c>
       <c r="V19" t="n">
-        <v>7.5311</v>
+        <v>1.2585</v>
       </c>
       <c r="W19" t="n">
-        <v>18.5642</v>
+        <v>7.9223</v>
       </c>
       <c r="X19" t="n">
-        <v>-7.3446</v>
+        <v>-6.7039</v>
       </c>
       <c r="Y19" t="n">
-        <v>-16.4118</v>
+        <v>-5.6497</v>
       </c>
       <c r="Z19" t="n">
-        <v>-38.1599</v>
+        <v>-14.8828</v>
       </c>
       <c r="AA19" t="n">
-        <v>-0.8222</v>
+        <v>-3.0478</v>
       </c>
       <c r="AB19" t="n">
-        <v>-7.392</v>
+        <v>-1.3625</v>
       </c>
       <c r="AC19" t="n">
-        <v>-16.4126</v>
+        <v>-7.8965</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>177.62</v>
+        <v>182.67</v>
       </c>
       <c r="C20" t="n">
-        <v>182.24</v>
+        <v>189.56</v>
       </c>
       <c r="D20" t="n">
-        <v>150.58</v>
+        <v>178.28</v>
       </c>
       <c r="E20" t="n">
-        <v>172.52</v>
+        <v>186.19</v>
       </c>
       <c r="F20" t="n">
-        <v>75.3</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>75.93000000000001</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H20" t="n">
-        <v>71.55</v>
+        <v>77.16</v>
       </c>
       <c r="I20" t="n">
-        <v>74.95999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="J20" t="n">
-        <v>8.75</v>
+        <v>8.43</v>
       </c>
       <c r="K20" t="n">
-        <v>9.91</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L20" t="n">
-        <v>8.550000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M20" t="n">
-        <v>8.949999999999999</v>
+        <v>8.27</v>
       </c>
       <c r="N20" t="n">
-        <v>43.14</v>
+        <v>41.98</v>
       </c>
       <c r="O20" t="n">
-        <v>45.19</v>
+        <v>42.06</v>
       </c>
       <c r="P20" t="n">
-        <v>42.79</v>
+        <v>40.68</v>
       </c>
       <c r="Q20" t="n">
-        <v>43.31</v>
+        <v>41.07</v>
       </c>
       <c r="R20" t="n">
-        <v>-9.4003</v>
+        <v>1.0584</v>
       </c>
       <c r="S20" t="n">
-        <v>13.4254</v>
+        <v>-2.2214</v>
       </c>
       <c r="T20" t="n">
-        <v>19.6726</v>
+        <v>22.4129</v>
       </c>
       <c r="U20" t="n">
-        <v>-2.5988</v>
+        <v>2.2139</v>
       </c>
       <c r="V20" t="n">
-        <v>5.0743</v>
+        <v>2.5858</v>
       </c>
       <c r="W20" t="n">
-        <v>11.2331</v>
+        <v>10.6672</v>
       </c>
       <c r="X20" t="n">
-        <v>9.1463</v>
+        <v>-0.9581</v>
       </c>
       <c r="Y20" t="n">
-        <v>-15.566</v>
+        <v>0.8537</v>
       </c>
       <c r="Z20" t="n">
-        <v>-22.2415</v>
+        <v>-21.9811</v>
       </c>
       <c r="AA20" t="n">
-        <v>2.5817</v>
+        <v>-2.191</v>
       </c>
       <c r="AB20" t="n">
-        <v>-5.2919</v>
+        <v>-2.7238</v>
       </c>
       <c r="AC20" t="n">
-        <v>-10.8664</v>
+        <v>-10.1902</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>183.84</v>
+        <v>167</v>
       </c>
       <c r="C21" t="n">
-        <v>188.49</v>
+        <v>174.4</v>
       </c>
       <c r="D21" t="n">
-        <v>172.26</v>
+        <v>161.14</v>
       </c>
       <c r="E21" t="n">
-        <v>184.24</v>
+        <v>164.18</v>
       </c>
       <c r="F21" t="n">
-        <v>75.81</v>
+        <v>75.73</v>
       </c>
       <c r="G21" t="n">
-        <v>77.94</v>
+        <v>77.37</v>
       </c>
       <c r="H21" t="n">
-        <v>74.19</v>
+        <v>74.23</v>
       </c>
       <c r="I21" t="n">
-        <v>77.23999999999999</v>
+        <v>75.34</v>
       </c>
       <c r="J21" t="n">
-        <v>8.380000000000001</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="K21" t="n">
-        <v>8.98</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="L21" t="n">
-        <v>8.140000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M21" t="n">
-        <v>8.35</v>
+        <v>9.23</v>
       </c>
       <c r="N21" t="n">
-        <v>42.83</v>
+        <v>42.77</v>
       </c>
       <c r="O21" t="n">
-        <v>43.77</v>
+        <v>43.57</v>
       </c>
       <c r="P21" t="n">
-        <v>41.6</v>
+        <v>41.93</v>
       </c>
       <c r="Q21" t="n">
-        <v>41.99</v>
+        <v>42.98</v>
       </c>
       <c r="R21" t="n">
-        <v>6.7934</v>
+        <v>-11.8213</v>
       </c>
       <c r="S21" t="n">
-        <v>4.1257</v>
+        <v>-4.8342</v>
       </c>
       <c r="T21" t="n">
-        <v>11.0883</v>
+        <v>-7.2115</v>
       </c>
       <c r="U21" t="n">
-        <v>3.0416</v>
+        <v>-4.5725</v>
       </c>
       <c r="V21" t="n">
-        <v>1.2585</v>
+        <v>0.5069</v>
       </c>
       <c r="W21" t="n">
-        <v>7.9223</v>
+        <v>-1.2323</v>
       </c>
       <c r="X21" t="n">
-        <v>-6.7039</v>
+        <v>11.6082</v>
       </c>
       <c r="Y21" t="n">
-        <v>-5.6497</v>
+        <v>3.1285</v>
       </c>
       <c r="Z21" t="n">
-        <v>-14.8828</v>
+        <v>4.2938</v>
       </c>
       <c r="AA21" t="n">
-        <v>-3.0478</v>
+        <v>4.6506</v>
       </c>
       <c r="AB21" t="n">
-        <v>-1.3625</v>
+        <v>-0.7619</v>
       </c>
       <c r="AC21" t="n">
-        <v>-7.8965</v>
+        <v>0.9631</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>182.67</v>
+        <v>172.95</v>
       </c>
       <c r="C22" t="n">
-        <v>189.56</v>
+        <v>174.61</v>
       </c>
       <c r="D22" t="n">
-        <v>178.28</v>
+        <v>142.69</v>
       </c>
       <c r="E22" t="n">
-        <v>186.19</v>
+        <v>151.75</v>
       </c>
       <c r="F22" t="n">
-        <v>77.29000000000001</v>
+        <v>76.13500000000001</v>
       </c>
       <c r="G22" t="n">
-        <v>79.68000000000001</v>
+        <v>76.2713</v>
       </c>
       <c r="H22" t="n">
-        <v>77.16</v>
+        <v>72.101</v>
       </c>
       <c r="I22" t="n">
-        <v>78.95</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="J22" t="n">
-        <v>8.43</v>
+        <v>8.77</v>
       </c>
       <c r="K22" t="n">
-        <v>8.630000000000001</v>
+        <v>10.47</v>
       </c>
       <c r="L22" t="n">
-        <v>8.119999999999999</v>
+        <v>8.68</v>
       </c>
       <c r="M22" t="n">
-        <v>8.27</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="N22" t="n">
-        <v>41.98</v>
+        <v>42.515</v>
       </c>
       <c r="O22" t="n">
-        <v>42.06</v>
+        <v>44.8201</v>
       </c>
       <c r="P22" t="n">
-        <v>40.68</v>
+        <v>42.44</v>
       </c>
       <c r="Q22" t="n">
-        <v>41.07</v>
+        <v>43.54</v>
       </c>
       <c r="R22" t="n">
-        <v>1.0584</v>
+        <v>-7.571</v>
       </c>
       <c r="S22" t="n">
-        <v>-2.2214</v>
+        <v>-17.6346</v>
       </c>
       <c r="T22" t="n">
-        <v>22.4129</v>
+        <v>-20.3077</v>
       </c>
       <c r="U22" t="n">
-        <v>2.2139</v>
+        <v>-1.3539</v>
       </c>
       <c r="V22" t="n">
-        <v>2.5858</v>
+        <v>-3.7804</v>
       </c>
       <c r="W22" t="n">
-        <v>10.6672</v>
+        <v>-3.4304</v>
       </c>
       <c r="X22" t="n">
-        <v>-0.9581</v>
+        <v>7.8007</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.8537</v>
+        <v>19.1617</v>
       </c>
       <c r="Z22" t="n">
-        <v>-21.9811</v>
+        <v>21.3415</v>
       </c>
       <c r="AA22" t="n">
-        <v>-2.191</v>
+        <v>1.3029</v>
       </c>
       <c r="AB22" t="n">
-        <v>-2.7238</v>
+        <v>3.6914</v>
       </c>
       <c r="AC22" t="n">
-        <v>-10.1902</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>167</v>
-      </c>
-      <c r="C23" t="n">
-        <v>174.4</v>
-      </c>
-      <c r="D23" t="n">
-        <v>161.1402</v>
-      </c>
-      <c r="E23" t="n">
-        <v>164.18</v>
-      </c>
-      <c r="F23" t="n">
-        <v>75.70999999999999</v>
-      </c>
-      <c r="G23" t="n">
-        <v>77.36499999999999</v>
-      </c>
-      <c r="H23" t="n">
-        <v>74.22799999999999</v>
-      </c>
-      <c r="I23" t="n">
-        <v>75.34</v>
-      </c>
-      <c r="J23" t="n">
-        <v>9.130000000000001</v>
-      </c>
-      <c r="K23" t="n">
-        <v>9.390000000000001</v>
-      </c>
-      <c r="L23" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="M23" t="n">
-        <v>9.23</v>
-      </c>
-      <c r="N23" t="n">
-        <v>42.77</v>
-      </c>
-      <c r="O23" t="n">
-        <v>43.565</v>
-      </c>
-      <c r="P23" t="n">
-        <v>41.93</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>42.98</v>
-      </c>
-      <c r="R23" t="n">
-        <v>-11.8213</v>
-      </c>
-      <c r="S23" t="n">
-        <v>-4.8342</v>
-      </c>
-      <c r="T23" t="n">
-        <v>-7.2115</v>
-      </c>
-      <c r="U23" t="n">
-        <v>-4.5725</v>
-      </c>
-      <c r="V23" t="n">
-        <v>0.5069</v>
-      </c>
-      <c r="W23" t="n">
-        <v>-1.2323</v>
-      </c>
-      <c r="X23" t="n">
-        <v>11.6082</v>
-      </c>
-      <c r="Y23" t="n">
-        <v>3.1285</v>
-      </c>
-      <c r="Z23" t="n">
-        <v>4.2938</v>
-      </c>
-      <c r="AA23" t="n">
-        <v>4.6506</v>
-      </c>
-      <c r="AB23" t="n">
-        <v>-0.7619</v>
-      </c>
-      <c r="AC23" t="n">
-        <v>0.9631</v>
+        <v>3.1265</v>
       </c>
     </row>
   </sheetData>
@@ -2503,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-05-19 19:33
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC22"/>
+  <dimension ref="A1:AC23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2296,13 +2296,13 @@
         <v>151.75</v>
       </c>
       <c r="F22" t="n">
-        <v>76.13500000000001</v>
+        <v>76.13</v>
       </c>
       <c r="G22" t="n">
-        <v>76.2713</v>
+        <v>76.27</v>
       </c>
       <c r="H22" t="n">
-        <v>72.101</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I22" t="n">
         <v>74.31999999999999</v>
@@ -2320,10 +2320,10 @@
         <v>9.949999999999999</v>
       </c>
       <c r="N22" t="n">
-        <v>42.515</v>
+        <v>42.51</v>
       </c>
       <c r="O22" t="n">
-        <v>44.8201</v>
+        <v>44.82</v>
       </c>
       <c r="P22" t="n">
         <v>42.44</v>
@@ -2366,6 +2366,97 @@
       </c>
       <c r="AC22" t="n">
         <v>3.1265</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>141.24</v>
+      </c>
+      <c r="C23" t="n">
+        <v>160.58</v>
+      </c>
+      <c r="D23" t="n">
+        <v>135.02</v>
+      </c>
+      <c r="E23" t="n">
+        <v>154.9699</v>
+      </c>
+      <c r="F23" t="n">
+        <v>72.41</v>
+      </c>
+      <c r="G23" t="n">
+        <v>74.5</v>
+      </c>
+      <c r="H23" t="n">
+        <v>70.9616</v>
+      </c>
+      <c r="I23" t="n">
+        <v>73.41</v>
+      </c>
+      <c r="J23" t="n">
+        <v>10.6403</v>
+      </c>
+      <c r="K23" t="n">
+        <v>11.07</v>
+      </c>
+      <c r="L23" t="n">
+        <v>9.369999999999999</v>
+      </c>
+      <c r="M23" t="n">
+        <v>9.7499</v>
+      </c>
+      <c r="N23" t="n">
+        <v>44.69</v>
+      </c>
+      <c r="O23" t="n">
+        <v>45.53</v>
+      </c>
+      <c r="P23" t="n">
+        <v>43.455</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>44.09</v>
+      </c>
+      <c r="R23" t="n">
+        <v>2.1218</v>
+      </c>
+      <c r="S23" t="n">
+        <v>-16.7679</v>
+      </c>
+      <c r="T23" t="n">
+        <v>-10.1728</v>
+      </c>
+      <c r="U23" t="n">
+        <v>-1.2244</v>
+      </c>
+      <c r="V23" t="n">
+        <v>-7.0171</v>
+      </c>
+      <c r="W23" t="n">
+        <v>-2.0678</v>
+      </c>
+      <c r="X23" t="n">
+        <v>-2.0111</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>17.8948</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>8.9374</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>1.2632</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>7.3533</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>1.801</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2503,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-05-19 23:02
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -2384,7 +2384,7 @@
         <v>135.02</v>
       </c>
       <c r="E23" t="n">
-        <v>154.9699</v>
+        <v>151.89</v>
       </c>
       <c r="F23" t="n">
         <v>72.41</v>
@@ -2396,7 +2396,7 @@
         <v>70.9616</v>
       </c>
       <c r="I23" t="n">
-        <v>73.41</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J23" t="n">
         <v>10.6403</v>
@@ -2408,7 +2408,7 @@
         <v>9.369999999999999</v>
       </c>
       <c r="M23" t="n">
-        <v>9.7499</v>
+        <v>9.93</v>
       </c>
       <c r="N23" t="n">
         <v>44.69</v>
@@ -2420,43 +2420,43 @@
         <v>43.455</v>
       </c>
       <c r="Q23" t="n">
-        <v>44.09</v>
+        <v>44.37</v>
       </c>
       <c r="R23" t="n">
-        <v>2.1218</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="S23" t="n">
-        <v>-16.7679</v>
+        <v>-18.422</v>
       </c>
       <c r="T23" t="n">
-        <v>-10.1728</v>
+        <v>-11.958</v>
       </c>
       <c r="U23" t="n">
-        <v>-1.2244</v>
+        <v>-1.8703</v>
       </c>
       <c r="V23" t="n">
-        <v>-7.0171</v>
+        <v>-7.6251</v>
       </c>
       <c r="W23" t="n">
-        <v>-2.0678</v>
+        <v>-2.7081</v>
       </c>
       <c r="X23" t="n">
-        <v>-2.0111</v>
+        <v>-0.201</v>
       </c>
       <c r="Y23" t="n">
-        <v>17.8948</v>
+        <v>20.0726</v>
       </c>
       <c r="Z23" t="n">
-        <v>8.9374</v>
+        <v>10.9497</v>
       </c>
       <c r="AA23" t="n">
-        <v>1.2632</v>
+        <v>1.9063</v>
       </c>
       <c r="AB23" t="n">
-        <v>7.3533</v>
+        <v>8.0351</v>
       </c>
       <c r="AC23" t="n">
-        <v>1.801</v>
+        <v>2.4475</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Master system update 2026-05-20 23:14
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1895 +568,1895 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>95.97</v>
+        <v>97.97</v>
       </c>
       <c r="C2" t="n">
-        <v>96.93000000000001</v>
+        <v>99.95</v>
       </c>
       <c r="D2" t="n">
-        <v>92.03</v>
+        <v>95.31999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>95.94</v>
+        <v>98.09</v>
       </c>
       <c r="F2" t="n">
-        <v>58.4</v>
+        <v>58.48</v>
       </c>
       <c r="G2" t="n">
-        <v>58.58</v>
+        <v>58.97</v>
       </c>
       <c r="H2" t="n">
-        <v>56.91</v>
+        <v>56.82</v>
       </c>
       <c r="I2" t="n">
-        <v>58.08</v>
+        <v>57.4</v>
       </c>
       <c r="J2" t="n">
-        <v>18.64</v>
+        <v>18.25</v>
       </c>
       <c r="K2" t="n">
-        <v>19.41</v>
+        <v>18.76</v>
       </c>
       <c r="L2" t="n">
-        <v>18.44</v>
+        <v>17.85</v>
       </c>
       <c r="M2" t="n">
-        <v>18.63</v>
+        <v>18.2</v>
       </c>
       <c r="N2" t="n">
-        <v>56.59</v>
+        <v>56.52</v>
       </c>
       <c r="O2" t="n">
-        <v>58.04</v>
+        <v>58.15</v>
       </c>
       <c r="P2" t="n">
-        <v>56.41</v>
+        <v>56.04</v>
       </c>
       <c r="Q2" t="n">
-        <v>56.91</v>
+        <v>57.59</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>97.97</v>
+        <v>102.94</v>
       </c>
       <c r="C3" t="n">
-        <v>99.95</v>
+        <v>106.09</v>
       </c>
       <c r="D3" t="n">
-        <v>95.31999999999999</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>98.09</v>
+        <v>105.64</v>
       </c>
       <c r="F3" t="n">
-        <v>58.48</v>
+        <v>58.93</v>
       </c>
       <c r="G3" t="n">
-        <v>58.97</v>
+        <v>60.3</v>
       </c>
       <c r="H3" t="n">
-        <v>56.82</v>
+        <v>58.49</v>
       </c>
       <c r="I3" t="n">
-        <v>57.4</v>
+        <v>60.21</v>
       </c>
       <c r="J3" t="n">
-        <v>18.25</v>
+        <v>17.37</v>
       </c>
       <c r="K3" t="n">
-        <v>18.76</v>
+        <v>17.95</v>
       </c>
       <c r="L3" t="n">
-        <v>17.85</v>
+        <v>16.72</v>
       </c>
       <c r="M3" t="n">
-        <v>18.2</v>
+        <v>16.8</v>
       </c>
       <c r="N3" t="n">
-        <v>56.52</v>
+        <v>56.05</v>
       </c>
       <c r="O3" t="n">
-        <v>58.15</v>
+        <v>56.49</v>
       </c>
       <c r="P3" t="n">
-        <v>56.04</v>
+        <v>54.66</v>
       </c>
       <c r="Q3" t="n">
-        <v>57.59</v>
+        <v>54.73</v>
       </c>
       <c r="R3" t="n">
-        <v>2.241</v>
+        <v>7.697</v>
       </c>
       <c r="U3" t="n">
-        <v>-1.1708</v>
+        <v>4.8955</v>
       </c>
       <c r="X3" t="n">
-        <v>-2.3081</v>
+        <v>-7.6923</v>
       </c>
       <c r="AA3" t="n">
-        <v>1.1949</v>
+        <v>-4.9661</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>102.94</v>
+        <v>108.62</v>
       </c>
       <c r="C4" t="n">
-        <v>106.09</v>
+        <v>116.77</v>
       </c>
       <c r="D4" t="n">
-        <v>99.59999999999999</v>
+        <v>107.46</v>
       </c>
       <c r="E4" t="n">
-        <v>105.64</v>
+        <v>112.77</v>
       </c>
       <c r="F4" t="n">
-        <v>58.93</v>
+        <v>59.8</v>
       </c>
       <c r="G4" t="n">
-        <v>60.3</v>
+        <v>60.73</v>
       </c>
       <c r="H4" t="n">
-        <v>58.49</v>
+        <v>57.59</v>
       </c>
       <c r="I4" t="n">
-        <v>60.21</v>
+        <v>59.22</v>
       </c>
       <c r="J4" t="n">
-        <v>17.37</v>
+        <v>16.35</v>
       </c>
       <c r="K4" t="n">
-        <v>17.95</v>
+        <v>16.52</v>
       </c>
       <c r="L4" t="n">
-        <v>16.72</v>
+        <v>15.06</v>
       </c>
       <c r="M4" t="n">
-        <v>16.8</v>
+        <v>15.7</v>
       </c>
       <c r="N4" t="n">
-        <v>56.05</v>
+        <v>55.13</v>
       </c>
       <c r="O4" t="n">
-        <v>56.49</v>
+        <v>57.14</v>
       </c>
       <c r="P4" t="n">
-        <v>54.66</v>
+        <v>54.28</v>
       </c>
       <c r="Q4" t="n">
-        <v>54.73</v>
+        <v>55.66</v>
       </c>
       <c r="R4" t="n">
-        <v>7.697</v>
+        <v>6.7493</v>
       </c>
       <c r="U4" t="n">
-        <v>4.8955</v>
+        <v>-1.6442</v>
       </c>
       <c r="X4" t="n">
-        <v>-7.6923</v>
+        <v>-6.5476</v>
       </c>
       <c r="AA4" t="n">
-        <v>-4.9661</v>
+        <v>1.6993</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>108.62</v>
+        <v>125.21</v>
       </c>
       <c r="C5" t="n">
-        <v>116.77</v>
+        <v>130.12</v>
       </c>
       <c r="D5" t="n">
-        <v>107.46</v>
+        <v>120.24</v>
       </c>
       <c r="E5" t="n">
-        <v>112.77</v>
+        <v>128.32</v>
       </c>
       <c r="F5" t="n">
-        <v>59.8</v>
+        <v>61.08</v>
       </c>
       <c r="G5" t="n">
-        <v>60.73</v>
+        <v>62.74</v>
       </c>
       <c r="H5" t="n">
-        <v>57.59</v>
+        <v>60.56</v>
       </c>
       <c r="I5" t="n">
-        <v>59.22</v>
+        <v>62.56</v>
       </c>
       <c r="J5" t="n">
-        <v>16.35</v>
+        <v>13.99</v>
       </c>
       <c r="K5" t="n">
-        <v>16.52</v>
+        <v>14.66</v>
       </c>
       <c r="L5" t="n">
-        <v>15.06</v>
+        <v>13.3</v>
       </c>
       <c r="M5" t="n">
-        <v>15.7</v>
+        <v>13.52</v>
       </c>
       <c r="N5" t="n">
-        <v>55.13</v>
+        <v>53.93</v>
       </c>
       <c r="O5" t="n">
-        <v>57.14</v>
+        <v>54.43</v>
       </c>
       <c r="P5" t="n">
-        <v>54.28</v>
+        <v>52.37</v>
       </c>
       <c r="Q5" t="n">
-        <v>55.66</v>
+        <v>52.5</v>
       </c>
       <c r="R5" t="n">
-        <v>6.7493</v>
+        <v>13.7891</v>
       </c>
       <c r="S5" t="n">
-        <v>17.5422</v>
+        <v>30.8186</v>
       </c>
       <c r="U5" t="n">
-        <v>-1.6442</v>
+        <v>5.64</v>
       </c>
       <c r="V5" t="n">
-        <v>1.9628</v>
+        <v>8.9895</v>
       </c>
       <c r="X5" t="n">
-        <v>-6.5476</v>
+        <v>-13.8854</v>
       </c>
       <c r="Y5" t="n">
-        <v>-15.7273</v>
+        <v>-25.7143</v>
       </c>
       <c r="AA5" t="n">
-        <v>1.6993</v>
+        <v>-5.6773</v>
       </c>
       <c r="AB5" t="n">
-        <v>-2.1965</v>
+        <v>-8.8383</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>125.21</v>
+        <v>128.33</v>
       </c>
       <c r="C6" t="n">
-        <v>130.12</v>
+        <v>129.59</v>
       </c>
       <c r="D6" t="n">
-        <v>120.24</v>
+        <v>117.79</v>
       </c>
       <c r="E6" t="n">
-        <v>128.32</v>
+        <v>123.39</v>
       </c>
       <c r="F6" t="n">
-        <v>61.08</v>
+        <v>62.41</v>
       </c>
       <c r="G6" t="n">
-        <v>62.74</v>
+        <v>62.7</v>
       </c>
       <c r="H6" t="n">
-        <v>60.56</v>
+        <v>61.64</v>
       </c>
       <c r="I6" t="n">
-        <v>62.56</v>
+        <v>62.64</v>
       </c>
       <c r="J6" t="n">
-        <v>13.99</v>
+        <v>13.51</v>
       </c>
       <c r="K6" t="n">
-        <v>14.66</v>
+        <v>14.63</v>
       </c>
       <c r="L6" t="n">
-        <v>13.3</v>
+        <v>13.41</v>
       </c>
       <c r="M6" t="n">
-        <v>13.52</v>
+        <v>14.03</v>
       </c>
       <c r="N6" t="n">
-        <v>53.93</v>
+        <v>52.67</v>
       </c>
       <c r="O6" t="n">
-        <v>54.43</v>
+        <v>53.31</v>
       </c>
       <c r="P6" t="n">
-        <v>52.37</v>
+        <v>52.42</v>
       </c>
       <c r="Q6" t="n">
-        <v>52.5</v>
+        <v>52.45</v>
       </c>
       <c r="R6" t="n">
-        <v>13.7891</v>
+        <v>-3.842</v>
       </c>
       <c r="S6" t="n">
-        <v>30.8186</v>
+        <v>16.8023</v>
       </c>
       <c r="U6" t="n">
-        <v>5.64</v>
+        <v>0.1279</v>
       </c>
       <c r="V6" t="n">
-        <v>8.9895</v>
+        <v>4.0359</v>
       </c>
       <c r="X6" t="n">
-        <v>-13.8854</v>
+        <v>3.7722</v>
       </c>
       <c r="Y6" t="n">
-        <v>-25.7143</v>
+        <v>-16.4881</v>
       </c>
       <c r="AA6" t="n">
-        <v>-5.6773</v>
+        <v>-0.09520000000000001</v>
       </c>
       <c r="AB6" t="n">
-        <v>-8.8383</v>
+        <v>-4.1659</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>128.33</v>
+        <v>108.75</v>
       </c>
       <c r="C7" t="n">
-        <v>129.59</v>
+        <v>115.62</v>
       </c>
       <c r="D7" t="n">
-        <v>117.79</v>
+        <v>103.99</v>
       </c>
       <c r="E7" t="n">
-        <v>123.39</v>
+        <v>109.56</v>
       </c>
       <c r="F7" t="n">
-        <v>62.41</v>
+        <v>60.72</v>
       </c>
       <c r="G7" t="n">
-        <v>62.7</v>
+        <v>61.33</v>
       </c>
       <c r="H7" t="n">
-        <v>61.64</v>
+        <v>59.68</v>
       </c>
       <c r="I7" t="n">
-        <v>62.64</v>
+        <v>60.74</v>
       </c>
       <c r="J7" t="n">
-        <v>13.51</v>
+        <v>15.71</v>
       </c>
       <c r="K7" t="n">
-        <v>14.63</v>
+        <v>16.27</v>
       </c>
       <c r="L7" t="n">
-        <v>13.41</v>
+        <v>14.93</v>
       </c>
       <c r="M7" t="n">
-        <v>14.03</v>
+        <v>15.59</v>
       </c>
       <c r="N7" t="n">
-        <v>52.67</v>
+        <v>54.09</v>
       </c>
       <c r="O7" t="n">
-        <v>53.31</v>
+        <v>54.96</v>
       </c>
       <c r="P7" t="n">
-        <v>52.42</v>
+        <v>53.58</v>
       </c>
       <c r="Q7" t="n">
-        <v>52.45</v>
+        <v>54.05</v>
       </c>
       <c r="R7" t="n">
-        <v>-3.842</v>
+        <v>-11.2084</v>
       </c>
       <c r="S7" t="n">
-        <v>16.8023</v>
+        <v>-2.8465</v>
       </c>
       <c r="T7" t="n">
-        <v>28.6116</v>
+        <v>11.6933</v>
       </c>
       <c r="U7" t="n">
-        <v>0.1279</v>
+        <v>-3.0332</v>
       </c>
       <c r="V7" t="n">
-        <v>4.0359</v>
+        <v>2.5667</v>
       </c>
       <c r="W7" t="n">
-        <v>7.8512</v>
+        <v>5.8188</v>
       </c>
       <c r="X7" t="n">
-        <v>3.7722</v>
+        <v>11.119</v>
       </c>
       <c r="Y7" t="n">
-        <v>-16.4881</v>
+        <v>-0.7006</v>
       </c>
       <c r="Z7" t="n">
-        <v>-24.6914</v>
+        <v>-14.3407</v>
       </c>
       <c r="AA7" t="n">
-        <v>-0.09520000000000001</v>
+        <v>3.0505</v>
       </c>
       <c r="AB7" t="n">
-        <v>-4.1659</v>
+        <v>-2.8926</v>
       </c>
       <c r="AC7" t="n">
-        <v>-7.8369</v>
+        <v>-6.1469</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>108.75</v>
+        <v>114.76</v>
       </c>
       <c r="C8" t="n">
-        <v>115.62</v>
+        <v>118.32</v>
       </c>
       <c r="D8" t="n">
-        <v>103.99</v>
+        <v>112.3</v>
       </c>
       <c r="E8" t="n">
-        <v>109.56</v>
+        <v>117.97</v>
       </c>
       <c r="F8" t="n">
-        <v>60.72</v>
+        <v>61</v>
       </c>
       <c r="G8" t="n">
-        <v>61.33</v>
+        <v>61.87</v>
       </c>
       <c r="H8" t="n">
-        <v>59.68</v>
+        <v>60.45</v>
       </c>
       <c r="I8" t="n">
-        <v>60.74</v>
+        <v>61.86</v>
       </c>
       <c r="J8" t="n">
-        <v>15.71</v>
+        <v>14.91</v>
       </c>
       <c r="K8" t="n">
-        <v>16.27</v>
+        <v>15.24</v>
       </c>
       <c r="L8" t="n">
-        <v>14.93</v>
+        <v>14.38</v>
       </c>
       <c r="M8" t="n">
-        <v>15.59</v>
+        <v>14.4</v>
       </c>
       <c r="N8" t="n">
-        <v>54.09</v>
+        <v>53.84</v>
       </c>
       <c r="O8" t="n">
-        <v>54.96</v>
+        <v>54.33</v>
       </c>
       <c r="P8" t="n">
-        <v>53.58</v>
+        <v>53.06</v>
       </c>
       <c r="Q8" t="n">
-        <v>54.05</v>
+        <v>53.08</v>
       </c>
       <c r="R8" t="n">
-        <v>-11.2084</v>
+        <v>7.6762</v>
       </c>
       <c r="S8" t="n">
-        <v>-2.8465</v>
+        <v>-8.065799999999999</v>
       </c>
       <c r="T8" t="n">
-        <v>11.6933</v>
+        <v>11.6717</v>
       </c>
       <c r="U8" t="n">
-        <v>-3.0332</v>
+        <v>1.8439</v>
       </c>
       <c r="V8" t="n">
-        <v>2.5667</v>
+        <v>-1.1189</v>
       </c>
       <c r="W8" t="n">
-        <v>5.8188</v>
+        <v>2.7404</v>
       </c>
       <c r="X8" t="n">
-        <v>11.119</v>
+        <v>-7.6331</v>
       </c>
       <c r="Y8" t="n">
-        <v>-0.7006</v>
+        <v>6.5089</v>
       </c>
       <c r="Z8" t="n">
-        <v>-14.3407</v>
+        <v>-14.2857</v>
       </c>
       <c r="AA8" t="n">
-        <v>3.0505</v>
+        <v>-1.7946</v>
       </c>
       <c r="AB8" t="n">
-        <v>-2.8926</v>
+        <v>1.1048</v>
       </c>
       <c r="AC8" t="n">
-        <v>-6.1469</v>
+        <v>-3.0148</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>114.76</v>
+        <v>122.81</v>
       </c>
       <c r="C9" t="n">
-        <v>118.32</v>
+        <v>127.45</v>
       </c>
       <c r="D9" t="n">
-        <v>112.3</v>
+        <v>117.5</v>
       </c>
       <c r="E9" t="n">
-        <v>117.97</v>
+        <v>126.98</v>
       </c>
       <c r="F9" t="n">
-        <v>61</v>
+        <v>62.89</v>
       </c>
       <c r="G9" t="n">
-        <v>61.87</v>
+        <v>63.8</v>
       </c>
       <c r="H9" t="n">
-        <v>60.45</v>
+        <v>60.7</v>
       </c>
       <c r="I9" t="n">
-        <v>61.86</v>
+        <v>63.54</v>
       </c>
       <c r="J9" t="n">
-        <v>14.91</v>
+        <v>13.84</v>
       </c>
       <c r="K9" t="n">
-        <v>15.24</v>
+        <v>14.49</v>
       </c>
       <c r="L9" t="n">
-        <v>14.38</v>
+        <v>13.25</v>
       </c>
       <c r="M9" t="n">
-        <v>14.4</v>
+        <v>13.3</v>
       </c>
       <c r="N9" t="n">
-        <v>53.84</v>
+        <v>52.21</v>
       </c>
       <c r="O9" t="n">
-        <v>54.33</v>
+        <v>54.09</v>
       </c>
       <c r="P9" t="n">
-        <v>53.06</v>
+        <v>51.4</v>
       </c>
       <c r="Q9" t="n">
-        <v>53.08</v>
+        <v>51.65</v>
       </c>
       <c r="R9" t="n">
-        <v>7.6762</v>
+        <v>7.6375</v>
       </c>
       <c r="S9" t="n">
-        <v>-8.065799999999999</v>
+        <v>2.9095</v>
       </c>
       <c r="T9" t="n">
-        <v>11.6717</v>
+        <v>12.6009</v>
       </c>
       <c r="U9" t="n">
-        <v>1.8439</v>
+        <v>2.7158</v>
       </c>
       <c r="V9" t="n">
-        <v>-1.1189</v>
+        <v>1.4368</v>
       </c>
       <c r="W9" t="n">
-        <v>2.7404</v>
+        <v>7.2948</v>
       </c>
       <c r="X9" t="n">
-        <v>-7.6331</v>
+        <v>-7.6389</v>
       </c>
       <c r="Y9" t="n">
-        <v>6.5089</v>
+        <v>-5.2031</v>
       </c>
       <c r="Z9" t="n">
-        <v>-14.2857</v>
+        <v>-15.2866</v>
       </c>
       <c r="AA9" t="n">
-        <v>-1.7946</v>
+        <v>-2.694</v>
       </c>
       <c r="AB9" t="n">
-        <v>1.1048</v>
+        <v>-1.5253</v>
       </c>
       <c r="AC9" t="n">
-        <v>-3.0148</v>
+        <v>-7.2045</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>122.81</v>
+        <v>124.39</v>
       </c>
       <c r="C10" t="n">
-        <v>127.45</v>
+        <v>131.38</v>
       </c>
       <c r="D10" t="n">
-        <v>117.5</v>
+        <v>121.66</v>
       </c>
       <c r="E10" t="n">
-        <v>126.98</v>
+        <v>130.4</v>
       </c>
       <c r="F10" t="n">
-        <v>62.89</v>
+        <v>63.89</v>
       </c>
       <c r="G10" t="n">
-        <v>63.8</v>
+        <v>65.84</v>
       </c>
       <c r="H10" t="n">
-        <v>60.7</v>
+        <v>63.81</v>
       </c>
       <c r="I10" t="n">
-        <v>63.54</v>
+        <v>65.3</v>
       </c>
       <c r="J10" t="n">
-        <v>13.84</v>
+        <v>13.61</v>
       </c>
       <c r="K10" t="n">
-        <v>14.49</v>
+        <v>13.89</v>
       </c>
       <c r="L10" t="n">
-        <v>13.25</v>
+        <v>12.87</v>
       </c>
       <c r="M10" t="n">
-        <v>13.3</v>
+        <v>12.98</v>
       </c>
       <c r="N10" t="n">
-        <v>52.21</v>
+        <v>51.36</v>
       </c>
       <c r="O10" t="n">
-        <v>54.09</v>
+        <v>51.45</v>
       </c>
       <c r="P10" t="n">
-        <v>51.4</v>
+        <v>49.79</v>
       </c>
       <c r="Q10" t="n">
-        <v>51.65</v>
+        <v>50.22</v>
       </c>
       <c r="R10" t="n">
-        <v>7.6375</v>
+        <v>2.6933</v>
       </c>
       <c r="S10" t="n">
-        <v>2.9095</v>
+        <v>19.0215</v>
       </c>
       <c r="T10" t="n">
-        <v>12.6009</v>
+        <v>1.6209</v>
       </c>
       <c r="U10" t="n">
-        <v>2.7158</v>
+        <v>2.7699</v>
       </c>
       <c r="V10" t="n">
-        <v>1.4368</v>
+        <v>7.5074</v>
       </c>
       <c r="W10" t="n">
-        <v>7.2948</v>
+        <v>4.3798</v>
       </c>
       <c r="X10" t="n">
-        <v>-7.6389</v>
+        <v>-2.406</v>
       </c>
       <c r="Y10" t="n">
-        <v>-5.2031</v>
+        <v>-16.7415</v>
       </c>
       <c r="Z10" t="n">
-        <v>-15.2866</v>
+        <v>-3.9941</v>
       </c>
       <c r="AA10" t="n">
-        <v>-2.694</v>
+        <v>-2.7686</v>
       </c>
       <c r="AB10" t="n">
-        <v>-1.5253</v>
+        <v>-7.086</v>
       </c>
       <c r="AC10" t="n">
-        <v>-7.2045</v>
+        <v>-4.3429</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>124.39</v>
+        <v>132.2</v>
       </c>
       <c r="C11" t="n">
-        <v>131.38</v>
+        <v>133.67</v>
       </c>
       <c r="D11" t="n">
-        <v>121.66</v>
+        <v>123.8</v>
       </c>
       <c r="E11" t="n">
-        <v>130.4</v>
+        <v>127.55</v>
       </c>
       <c r="F11" t="n">
-        <v>63.89</v>
+        <v>65.44</v>
       </c>
       <c r="G11" t="n">
-        <v>65.84</v>
+        <v>66.05</v>
       </c>
       <c r="H11" t="n">
-        <v>63.81</v>
+        <v>63.78</v>
       </c>
       <c r="I11" t="n">
-        <v>65.3</v>
+        <v>64.91</v>
       </c>
       <c r="J11" t="n">
-        <v>13.61</v>
+        <v>12.8</v>
       </c>
       <c r="K11" t="n">
-        <v>13.89</v>
+        <v>13.64</v>
       </c>
       <c r="L11" t="n">
-        <v>12.87</v>
+        <v>12.65</v>
       </c>
       <c r="M11" t="n">
-        <v>12.98</v>
+        <v>13.26</v>
       </c>
       <c r="N11" t="n">
-        <v>51.36</v>
+        <v>50.12</v>
       </c>
       <c r="O11" t="n">
-        <v>51.45</v>
+        <v>51.43</v>
       </c>
       <c r="P11" t="n">
-        <v>49.79</v>
+        <v>49.65</v>
       </c>
       <c r="Q11" t="n">
-        <v>50.22</v>
+        <v>50.51</v>
       </c>
       <c r="R11" t="n">
-        <v>2.6933</v>
+        <v>-2.1856</v>
       </c>
       <c r="S11" t="n">
-        <v>19.0215</v>
+        <v>8.120699999999999</v>
       </c>
       <c r="T11" t="n">
-        <v>1.6209</v>
+        <v>3.3714</v>
       </c>
       <c r="U11" t="n">
-        <v>2.7699</v>
+        <v>-0.5972</v>
       </c>
       <c r="V11" t="n">
-        <v>7.5074</v>
+        <v>4.9305</v>
       </c>
       <c r="W11" t="n">
-        <v>4.3798</v>
+        <v>3.6239</v>
       </c>
       <c r="X11" t="n">
-        <v>-2.406</v>
+        <v>2.1572</v>
       </c>
       <c r="Y11" t="n">
-        <v>-16.7415</v>
+        <v>-7.9167</v>
       </c>
       <c r="Z11" t="n">
-        <v>-3.9941</v>
+        <v>-5.4882</v>
       </c>
       <c r="AA11" t="n">
-        <v>-2.7686</v>
+        <v>0.5775</v>
       </c>
       <c r="AB11" t="n">
-        <v>-7.086</v>
+        <v>-4.8417</v>
       </c>
       <c r="AC11" t="n">
-        <v>-4.3429</v>
+        <v>-3.6988</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>132.2</v>
+        <v>135</v>
       </c>
       <c r="C12" t="n">
-        <v>133.67</v>
+        <v>147.26</v>
       </c>
       <c r="D12" t="n">
-        <v>123.8</v>
+        <v>134.02</v>
       </c>
       <c r="E12" t="n">
-        <v>127.55</v>
+        <v>144.16</v>
       </c>
       <c r="F12" t="n">
-        <v>65.44</v>
+        <v>66.37</v>
       </c>
       <c r="G12" t="n">
-        <v>66.05</v>
+        <v>67.77</v>
       </c>
       <c r="H12" t="n">
-        <v>63.78</v>
+        <v>66.25</v>
       </c>
       <c r="I12" t="n">
-        <v>64.91</v>
+        <v>67.39</v>
       </c>
       <c r="J12" t="n">
-        <v>12.8</v>
+        <v>12.5</v>
       </c>
       <c r="K12" t="n">
-        <v>13.64</v>
+        <v>12.59</v>
       </c>
       <c r="L12" t="n">
-        <v>12.65</v>
+        <v>11.21</v>
       </c>
       <c r="M12" t="n">
-        <v>13.26</v>
+        <v>11.51</v>
       </c>
       <c r="N12" t="n">
-        <v>50.12</v>
+        <v>49.4</v>
       </c>
       <c r="O12" t="n">
-        <v>51.43</v>
+        <v>49.49</v>
       </c>
       <c r="P12" t="n">
-        <v>49.65</v>
+        <v>48.3</v>
       </c>
       <c r="Q12" t="n">
-        <v>50.51</v>
+        <v>48.59</v>
       </c>
       <c r="R12" t="n">
-        <v>-2.1856</v>
+        <v>13.0223</v>
       </c>
       <c r="S12" t="n">
-        <v>8.120699999999999</v>
+        <v>13.5297</v>
       </c>
       <c r="T12" t="n">
-        <v>3.3714</v>
+        <v>31.5809</v>
       </c>
       <c r="U12" t="n">
-        <v>-0.5972</v>
+        <v>3.8207</v>
       </c>
       <c r="V12" t="n">
-        <v>4.9305</v>
+        <v>6.0592</v>
       </c>
       <c r="W12" t="n">
-        <v>3.6239</v>
+        <v>10.9483</v>
       </c>
       <c r="X12" t="n">
-        <v>2.1572</v>
+        <v>-13.1976</v>
       </c>
       <c r="Y12" t="n">
-        <v>-7.9167</v>
+        <v>-13.4586</v>
       </c>
       <c r="Z12" t="n">
-        <v>-5.4882</v>
+        <v>-26.1706</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.5775</v>
+        <v>-3.8012</v>
       </c>
       <c r="AB12" t="n">
-        <v>-4.8417</v>
+        <v>-5.9245</v>
       </c>
       <c r="AC12" t="n">
-        <v>-3.6988</v>
+        <v>-10.1018</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>135</v>
+        <v>157.84</v>
       </c>
       <c r="C13" t="n">
-        <v>147.26</v>
+        <v>166</v>
       </c>
       <c r="D13" t="n">
-        <v>134.02</v>
+        <v>149.06</v>
       </c>
       <c r="E13" t="n">
-        <v>144.16</v>
+        <v>165.85</v>
       </c>
       <c r="F13" t="n">
-        <v>66.37</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>67.77</v>
+        <v>71.66</v>
       </c>
       <c r="H13" t="n">
-        <v>66.25</v>
+        <v>68.88</v>
       </c>
       <c r="I13" t="n">
-        <v>67.39</v>
+        <v>71.56999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>12.5</v>
+        <v>10.43</v>
       </c>
       <c r="K13" t="n">
-        <v>12.59</v>
+        <v>11.14</v>
       </c>
       <c r="L13" t="n">
-        <v>11.21</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M13" t="n">
-        <v>11.51</v>
+        <v>9.81</v>
       </c>
       <c r="N13" t="n">
-        <v>49.4</v>
+        <v>47.26</v>
       </c>
       <c r="O13" t="n">
-        <v>49.49</v>
+        <v>47.54</v>
       </c>
       <c r="P13" t="n">
-        <v>48.3</v>
+        <v>45.52</v>
       </c>
       <c r="Q13" t="n">
-        <v>48.59</v>
+        <v>45.59</v>
       </c>
       <c r="R13" t="n">
-        <v>13.0223</v>
+        <v>15.0458</v>
       </c>
       <c r="S13" t="n">
-        <v>13.5297</v>
+        <v>27.1856</v>
       </c>
       <c r="T13" t="n">
-        <v>31.5809</v>
+        <v>40.5866</v>
       </c>
       <c r="U13" t="n">
-        <v>3.8207</v>
+        <v>6.2027</v>
       </c>
       <c r="V13" t="n">
-        <v>6.0592</v>
+        <v>9.601800000000001</v>
       </c>
       <c r="W13" t="n">
-        <v>10.9483</v>
+        <v>15.6967</v>
       </c>
       <c r="X13" t="n">
-        <v>-13.1976</v>
+        <v>-14.7698</v>
       </c>
       <c r="Y13" t="n">
-        <v>-13.4586</v>
+        <v>-24.4222</v>
       </c>
       <c r="Z13" t="n">
-        <v>-26.1706</v>
+        <v>-31.875</v>
       </c>
       <c r="AA13" t="n">
-        <v>-3.8012</v>
+        <v>-6.1741</v>
       </c>
       <c r="AB13" t="n">
-        <v>-5.9245</v>
+        <v>-9.2194</v>
       </c>
       <c r="AC13" t="n">
-        <v>-10.1018</v>
+        <v>-14.1108</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>157.84</v>
+        <v>162.12</v>
       </c>
       <c r="C14" t="n">
-        <v>166</v>
+        <v>162.9</v>
       </c>
       <c r="D14" t="n">
-        <v>149.06</v>
+        <v>147.61</v>
       </c>
       <c r="E14" t="n">
-        <v>165.85</v>
+        <v>152.1</v>
       </c>
       <c r="F14" t="n">
-        <v>69.26000000000001</v>
+        <v>71.87</v>
       </c>
       <c r="G14" t="n">
-        <v>71.66</v>
+        <v>73.3</v>
       </c>
       <c r="H14" t="n">
-        <v>68.88</v>
+        <v>70.38</v>
       </c>
       <c r="I14" t="n">
-        <v>71.56999999999999</v>
+        <v>71.34</v>
       </c>
       <c r="J14" t="n">
-        <v>10.43</v>
+        <v>10.02</v>
       </c>
       <c r="K14" t="n">
-        <v>11.14</v>
+        <v>10.88</v>
       </c>
       <c r="L14" t="n">
-        <v>9.800000000000001</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="M14" t="n">
-        <v>9.81</v>
+        <v>10.6</v>
       </c>
       <c r="N14" t="n">
-        <v>47.26</v>
+        <v>45.41</v>
       </c>
       <c r="O14" t="n">
-        <v>47.54</v>
+        <v>46.36</v>
       </c>
       <c r="P14" t="n">
-        <v>45.52</v>
+        <v>44.5</v>
       </c>
       <c r="Q14" t="n">
-        <v>45.59</v>
+        <v>45.73</v>
       </c>
       <c r="R14" t="n">
-        <v>15.0458</v>
+        <v>-8.2906</v>
       </c>
       <c r="S14" t="n">
-        <v>27.1856</v>
+        <v>19.2474</v>
       </c>
       <c r="T14" t="n">
-        <v>40.5866</v>
+        <v>19.7826</v>
       </c>
       <c r="U14" t="n">
-        <v>6.2027</v>
+        <v>-0.3214</v>
       </c>
       <c r="V14" t="n">
-        <v>9.601800000000001</v>
+        <v>9.906000000000001</v>
       </c>
       <c r="W14" t="n">
-        <v>15.6967</v>
+        <v>12.2757</v>
       </c>
       <c r="X14" t="n">
-        <v>-14.7698</v>
+        <v>8.053000000000001</v>
       </c>
       <c r="Y14" t="n">
-        <v>-24.4222</v>
+        <v>-20.0603</v>
       </c>
       <c r="Z14" t="n">
-        <v>-31.875</v>
+        <v>-20.3008</v>
       </c>
       <c r="AA14" t="n">
-        <v>-6.1741</v>
+        <v>0.3071</v>
       </c>
       <c r="AB14" t="n">
-        <v>-9.2194</v>
+        <v>-9.4635</v>
       </c>
       <c r="AC14" t="n">
-        <v>-14.1108</v>
+        <v>-11.4618</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>162.12</v>
+        <v>163</v>
       </c>
       <c r="C15" t="n">
-        <v>162.9</v>
+        <v>177.5</v>
       </c>
       <c r="D15" t="n">
-        <v>147.61</v>
+        <v>161.51</v>
       </c>
       <c r="E15" t="n">
-        <v>152.1</v>
+        <v>176.94</v>
       </c>
       <c r="F15" t="n">
-        <v>71.87</v>
+        <v>72.81999999999999</v>
       </c>
       <c r="G15" t="n">
-        <v>73.3</v>
+        <v>76.31</v>
       </c>
       <c r="H15" t="n">
-        <v>70.38</v>
+        <v>72.7</v>
       </c>
       <c r="I15" t="n">
-        <v>71.34</v>
+        <v>76.28</v>
       </c>
       <c r="J15" t="n">
-        <v>10.02</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="K15" t="n">
-        <v>10.88</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="L15" t="n">
-        <v>9.970000000000001</v>
+        <v>8.84</v>
       </c>
       <c r="M15" t="n">
-        <v>10.6</v>
+        <v>8.85</v>
       </c>
       <c r="N15" t="n">
-        <v>45.41</v>
+        <v>44.82</v>
       </c>
       <c r="O15" t="n">
-        <v>46.36</v>
+        <v>44.89</v>
       </c>
       <c r="P15" t="n">
-        <v>44.5</v>
+        <v>42.57</v>
       </c>
       <c r="Q15" t="n">
-        <v>45.73</v>
+        <v>42.57</v>
       </c>
       <c r="R15" t="n">
-        <v>-8.2906</v>
+        <v>16.3314</v>
       </c>
       <c r="S15" t="n">
-        <v>19.2474</v>
+        <v>22.7386</v>
       </c>
       <c r="T15" t="n">
-        <v>19.7826</v>
+        <v>35.6902</v>
       </c>
       <c r="U15" t="n">
-        <v>-0.3214</v>
+        <v>6.9246</v>
       </c>
       <c r="V15" t="n">
-        <v>9.906000000000001</v>
+        <v>13.1919</v>
       </c>
       <c r="W15" t="n">
-        <v>12.2757</v>
+        <v>16.8147</v>
       </c>
       <c r="X15" t="n">
-        <v>8.053000000000001</v>
+        <v>-16.5094</v>
       </c>
       <c r="Y15" t="n">
-        <v>-20.0603</v>
+        <v>-23.1103</v>
       </c>
       <c r="Z15" t="n">
-        <v>-20.3008</v>
+        <v>-31.8182</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.3071</v>
+        <v>-6.9101</v>
       </c>
       <c r="AB15" t="n">
-        <v>-9.4635</v>
+        <v>-12.3894</v>
       </c>
       <c r="AC15" t="n">
-        <v>-11.4618</v>
+        <v>-15.233</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="C16" t="n">
-        <v>177.5</v>
+        <v>191.29</v>
       </c>
       <c r="D16" t="n">
-        <v>161.51</v>
+        <v>178.94</v>
       </c>
       <c r="E16" t="n">
-        <v>176.94</v>
+        <v>190.42</v>
       </c>
       <c r="F16" t="n">
-        <v>72.81999999999999</v>
+        <v>76</v>
       </c>
       <c r="G16" t="n">
-        <v>76.31</v>
+        <v>77.36</v>
       </c>
       <c r="H16" t="n">
-        <v>72.7</v>
+        <v>75.55</v>
       </c>
       <c r="I16" t="n">
-        <v>76.28</v>
+        <v>76.95999999999999</v>
       </c>
       <c r="J16" t="n">
-        <v>9.859999999999999</v>
+        <v>8.65</v>
       </c>
       <c r="K16" t="n">
-        <v>9.970000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="L16" t="n">
-        <v>8.84</v>
+        <v>8.15</v>
       </c>
       <c r="M16" t="n">
-        <v>8.85</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="N16" t="n">
-        <v>44.82</v>
+        <v>42.74</v>
       </c>
       <c r="O16" t="n">
-        <v>44.89</v>
+        <v>43</v>
       </c>
       <c r="P16" t="n">
-        <v>42.57</v>
+        <v>41.99</v>
       </c>
       <c r="Q16" t="n">
-        <v>42.57</v>
+        <v>42.22</v>
       </c>
       <c r="R16" t="n">
-        <v>16.3314</v>
+        <v>7.6184</v>
       </c>
       <c r="S16" t="n">
-        <v>22.7386</v>
+        <v>14.8146</v>
       </c>
       <c r="T16" t="n">
-        <v>35.6902</v>
+        <v>49.2905</v>
       </c>
       <c r="U16" t="n">
-        <v>6.9246</v>
+        <v>0.8915</v>
       </c>
       <c r="V16" t="n">
-        <v>13.1919</v>
+        <v>7.5311</v>
       </c>
       <c r="W16" t="n">
-        <v>16.8147</v>
+        <v>18.5642</v>
       </c>
       <c r="X16" t="n">
-        <v>-16.5094</v>
+        <v>-7.3446</v>
       </c>
       <c r="Y16" t="n">
-        <v>-23.1103</v>
+        <v>-16.4118</v>
       </c>
       <c r="Z16" t="n">
-        <v>-31.8182</v>
+        <v>-38.1599</v>
       </c>
       <c r="AA16" t="n">
-        <v>-6.9101</v>
+        <v>-0.8222</v>
       </c>
       <c r="AB16" t="n">
-        <v>-12.3894</v>
+        <v>-7.392</v>
       </c>
       <c r="AC16" t="n">
-        <v>-15.233</v>
+        <v>-16.4126</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>181</v>
+        <v>177.62</v>
       </c>
       <c r="C17" t="n">
-        <v>191.29</v>
+        <v>182.24</v>
       </c>
       <c r="D17" t="n">
-        <v>178.94</v>
+        <v>150.58</v>
       </c>
       <c r="E17" t="n">
-        <v>190.42</v>
+        <v>172.52</v>
       </c>
       <c r="F17" t="n">
-        <v>76</v>
+        <v>75.3</v>
       </c>
       <c r="G17" t="n">
-        <v>77.36</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="H17" t="n">
-        <v>75.55</v>
+        <v>71.55</v>
       </c>
       <c r="I17" t="n">
-        <v>76.95999999999999</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>8.65</v>
+        <v>8.75</v>
       </c>
       <c r="K17" t="n">
-        <v>8.77</v>
+        <v>9.91</v>
       </c>
       <c r="L17" t="n">
-        <v>8.15</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="M17" t="n">
-        <v>8.199999999999999</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N17" t="n">
-        <v>42.74</v>
+        <v>43.14</v>
       </c>
       <c r="O17" t="n">
-        <v>43</v>
+        <v>45.19</v>
       </c>
       <c r="P17" t="n">
-        <v>41.99</v>
+        <v>42.79</v>
       </c>
       <c r="Q17" t="n">
-        <v>42.22</v>
+        <v>43.31</v>
       </c>
       <c r="R17" t="n">
-        <v>7.6184</v>
+        <v>-9.4003</v>
       </c>
       <c r="S17" t="n">
-        <v>14.8146</v>
+        <v>13.4254</v>
       </c>
       <c r="T17" t="n">
-        <v>49.2905</v>
+        <v>19.6726</v>
       </c>
       <c r="U17" t="n">
-        <v>0.8915</v>
+        <v>-2.5988</v>
       </c>
       <c r="V17" t="n">
-        <v>7.5311</v>
+        <v>5.0743</v>
       </c>
       <c r="W17" t="n">
-        <v>18.5642</v>
+        <v>11.2331</v>
       </c>
       <c r="X17" t="n">
-        <v>-7.3446</v>
+        <v>9.1463</v>
       </c>
       <c r="Y17" t="n">
-        <v>-16.4118</v>
+        <v>-15.566</v>
       </c>
       <c r="Z17" t="n">
-        <v>-38.1599</v>
+        <v>-22.2415</v>
       </c>
       <c r="AA17" t="n">
-        <v>-0.8222</v>
+        <v>2.5817</v>
       </c>
       <c r="AB17" t="n">
-        <v>-7.392</v>
+        <v>-5.2919</v>
       </c>
       <c r="AC17" t="n">
-        <v>-16.4126</v>
+        <v>-10.8664</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>177.62</v>
+        <v>183.84</v>
       </c>
       <c r="C18" t="n">
-        <v>182.24</v>
+        <v>188.49</v>
       </c>
       <c r="D18" t="n">
-        <v>150.58</v>
+        <v>172.26</v>
       </c>
       <c r="E18" t="n">
-        <v>172.52</v>
+        <v>184.24</v>
       </c>
       <c r="F18" t="n">
-        <v>75.3</v>
+        <v>75.81</v>
       </c>
       <c r="G18" t="n">
-        <v>75.93000000000001</v>
+        <v>77.94</v>
       </c>
       <c r="H18" t="n">
-        <v>71.55</v>
+        <v>74.19</v>
       </c>
       <c r="I18" t="n">
-        <v>74.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="J18" t="n">
-        <v>8.75</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>9.91</v>
+        <v>8.98</v>
       </c>
       <c r="L18" t="n">
-        <v>8.550000000000001</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="M18" t="n">
-        <v>8.949999999999999</v>
+        <v>8.35</v>
       </c>
       <c r="N18" t="n">
-        <v>43.14</v>
+        <v>42.83</v>
       </c>
       <c r="O18" t="n">
-        <v>45.19</v>
+        <v>43.77</v>
       </c>
       <c r="P18" t="n">
-        <v>42.79</v>
+        <v>41.6</v>
       </c>
       <c r="Q18" t="n">
-        <v>43.31</v>
+        <v>41.99</v>
       </c>
       <c r="R18" t="n">
-        <v>-9.4003</v>
+        <v>6.7934</v>
       </c>
       <c r="S18" t="n">
-        <v>13.4254</v>
+        <v>4.1257</v>
       </c>
       <c r="T18" t="n">
-        <v>19.6726</v>
+        <v>11.0883</v>
       </c>
       <c r="U18" t="n">
-        <v>-2.5988</v>
+        <v>3.0416</v>
       </c>
       <c r="V18" t="n">
-        <v>5.0743</v>
+        <v>1.2585</v>
       </c>
       <c r="W18" t="n">
-        <v>11.2331</v>
+        <v>7.9223</v>
       </c>
       <c r="X18" t="n">
-        <v>9.1463</v>
+        <v>-6.7039</v>
       </c>
       <c r="Y18" t="n">
-        <v>-15.566</v>
+        <v>-5.6497</v>
       </c>
       <c r="Z18" t="n">
-        <v>-22.2415</v>
+        <v>-14.8828</v>
       </c>
       <c r="AA18" t="n">
-        <v>2.5817</v>
+        <v>-3.0478</v>
       </c>
       <c r="AB18" t="n">
-        <v>-5.2919</v>
+        <v>-1.3625</v>
       </c>
       <c r="AC18" t="n">
-        <v>-10.8664</v>
+        <v>-7.8965</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>183.84</v>
+        <v>182.67</v>
       </c>
       <c r="C19" t="n">
-        <v>188.49</v>
+        <v>189.56</v>
       </c>
       <c r="D19" t="n">
-        <v>172.26</v>
+        <v>178.28</v>
       </c>
       <c r="E19" t="n">
-        <v>184.24</v>
+        <v>186.19</v>
       </c>
       <c r="F19" t="n">
-        <v>75.81</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>77.94</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>74.19</v>
+        <v>77.16</v>
       </c>
       <c r="I19" t="n">
-        <v>77.23999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="J19" t="n">
-        <v>8.380000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="K19" t="n">
-        <v>8.98</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L19" t="n">
-        <v>8.140000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M19" t="n">
-        <v>8.35</v>
+        <v>8.27</v>
       </c>
       <c r="N19" t="n">
-        <v>42.83</v>
+        <v>41.98</v>
       </c>
       <c r="O19" t="n">
-        <v>43.77</v>
+        <v>42.06</v>
       </c>
       <c r="P19" t="n">
-        <v>41.6</v>
+        <v>40.68</v>
       </c>
       <c r="Q19" t="n">
-        <v>41.99</v>
+        <v>41.07</v>
       </c>
       <c r="R19" t="n">
-        <v>6.7934</v>
+        <v>1.0584</v>
       </c>
       <c r="S19" t="n">
-        <v>4.1257</v>
+        <v>-2.2214</v>
       </c>
       <c r="T19" t="n">
-        <v>11.0883</v>
+        <v>22.4129</v>
       </c>
       <c r="U19" t="n">
-        <v>3.0416</v>
+        <v>2.2139</v>
       </c>
       <c r="V19" t="n">
-        <v>1.2585</v>
+        <v>2.5858</v>
       </c>
       <c r="W19" t="n">
-        <v>7.9223</v>
+        <v>10.6672</v>
       </c>
       <c r="X19" t="n">
-        <v>-6.7039</v>
+        <v>-0.9581</v>
       </c>
       <c r="Y19" t="n">
-        <v>-5.6497</v>
+        <v>0.8537</v>
       </c>
       <c r="Z19" t="n">
-        <v>-14.8828</v>
+        <v>-21.9811</v>
       </c>
       <c r="AA19" t="n">
-        <v>-3.0478</v>
+        <v>-2.191</v>
       </c>
       <c r="AB19" t="n">
-        <v>-1.3625</v>
+        <v>-2.7238</v>
       </c>
       <c r="AC19" t="n">
-        <v>-7.8965</v>
+        <v>-10.1902</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>182.67</v>
+        <v>167</v>
       </c>
       <c r="C20" t="n">
-        <v>189.56</v>
+        <v>174.4</v>
       </c>
       <c r="D20" t="n">
-        <v>178.28</v>
+        <v>161.14</v>
       </c>
       <c r="E20" t="n">
-        <v>186.19</v>
+        <v>164.18</v>
       </c>
       <c r="F20" t="n">
-        <v>77.29000000000001</v>
+        <v>75.73</v>
       </c>
       <c r="G20" t="n">
-        <v>79.68000000000001</v>
+        <v>77.37</v>
       </c>
       <c r="H20" t="n">
-        <v>77.16</v>
+        <v>74.23</v>
       </c>
       <c r="I20" t="n">
-        <v>78.95</v>
+        <v>75.34</v>
       </c>
       <c r="J20" t="n">
-        <v>8.43</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="K20" t="n">
-        <v>8.630000000000001</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="L20" t="n">
-        <v>8.119999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M20" t="n">
-        <v>8.27</v>
+        <v>9.23</v>
       </c>
       <c r="N20" t="n">
-        <v>41.98</v>
+        <v>42.77</v>
       </c>
       <c r="O20" t="n">
-        <v>42.06</v>
+        <v>43.57</v>
       </c>
       <c r="P20" t="n">
-        <v>40.68</v>
+        <v>41.93</v>
       </c>
       <c r="Q20" t="n">
-        <v>41.07</v>
+        <v>42.98</v>
       </c>
       <c r="R20" t="n">
-        <v>1.0584</v>
+        <v>-11.8213</v>
       </c>
       <c r="S20" t="n">
-        <v>-2.2214</v>
+        <v>-4.8342</v>
       </c>
       <c r="T20" t="n">
-        <v>22.4129</v>
+        <v>-7.2115</v>
       </c>
       <c r="U20" t="n">
-        <v>2.2139</v>
+        <v>-4.5725</v>
       </c>
       <c r="V20" t="n">
-        <v>2.5858</v>
+        <v>0.5069</v>
       </c>
       <c r="W20" t="n">
-        <v>10.6672</v>
+        <v>-1.2323</v>
       </c>
       <c r="X20" t="n">
-        <v>-0.9581</v>
+        <v>11.6082</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.8537</v>
+        <v>3.1285</v>
       </c>
       <c r="Z20" t="n">
-        <v>-21.9811</v>
+        <v>4.2938</v>
       </c>
       <c r="AA20" t="n">
-        <v>-2.191</v>
+        <v>4.6506</v>
       </c>
       <c r="AB20" t="n">
-        <v>-2.7238</v>
+        <v>-0.7619</v>
       </c>
       <c r="AC20" t="n">
-        <v>-10.1902</v>
+        <v>0.9631</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>167</v>
+        <v>172.95</v>
       </c>
       <c r="C21" t="n">
-        <v>174.4</v>
+        <v>174.61</v>
       </c>
       <c r="D21" t="n">
-        <v>161.14</v>
+        <v>142.69</v>
       </c>
       <c r="E21" t="n">
-        <v>164.18</v>
+        <v>151.75</v>
       </c>
       <c r="F21" t="n">
-        <v>75.73</v>
+        <v>76.13</v>
       </c>
       <c r="G21" t="n">
-        <v>77.37</v>
+        <v>76.27</v>
       </c>
       <c r="H21" t="n">
-        <v>74.23</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I21" t="n">
-        <v>75.34</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="J21" t="n">
-        <v>9.130000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="K21" t="n">
-        <v>9.390000000000001</v>
+        <v>10.47</v>
       </c>
       <c r="L21" t="n">
-        <v>8.800000000000001</v>
+        <v>8.68</v>
       </c>
       <c r="M21" t="n">
-        <v>9.23</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="N21" t="n">
-        <v>42.77</v>
+        <v>42.51</v>
       </c>
       <c r="O21" t="n">
-        <v>43.57</v>
+        <v>44.82</v>
       </c>
       <c r="P21" t="n">
-        <v>41.93</v>
+        <v>42.44</v>
       </c>
       <c r="Q21" t="n">
-        <v>42.98</v>
+        <v>43.54</v>
       </c>
       <c r="R21" t="n">
-        <v>-11.8213</v>
+        <v>-7.571</v>
       </c>
       <c r="S21" t="n">
-        <v>-4.8342</v>
+        <v>-17.6346</v>
       </c>
       <c r="T21" t="n">
-        <v>-7.2115</v>
+        <v>-20.3077</v>
       </c>
       <c r="U21" t="n">
-        <v>-4.5725</v>
+        <v>-1.3539</v>
       </c>
       <c r="V21" t="n">
-        <v>0.5069</v>
+        <v>-3.7804</v>
       </c>
       <c r="W21" t="n">
-        <v>-1.2323</v>
+        <v>-3.4304</v>
       </c>
       <c r="X21" t="n">
-        <v>11.6082</v>
+        <v>7.8007</v>
       </c>
       <c r="Y21" t="n">
-        <v>3.1285</v>
+        <v>19.1617</v>
       </c>
       <c r="Z21" t="n">
-        <v>4.2938</v>
+        <v>21.3415</v>
       </c>
       <c r="AA21" t="n">
-        <v>4.6506</v>
+        <v>1.3029</v>
       </c>
       <c r="AB21" t="n">
-        <v>-0.7619</v>
+        <v>3.6914</v>
       </c>
       <c r="AC21" t="n">
-        <v>0.9631</v>
+        <v>3.1265</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>172.95</v>
+        <v>141.24</v>
       </c>
       <c r="C22" t="n">
-        <v>174.61</v>
+        <v>160.6</v>
       </c>
       <c r="D22" t="n">
-        <v>142.69</v>
+        <v>135.02</v>
       </c>
       <c r="E22" t="n">
-        <v>151.75</v>
+        <v>151.89</v>
       </c>
       <c r="F22" t="n">
-        <v>76.13</v>
+        <v>72.41</v>
       </c>
       <c r="G22" t="n">
-        <v>76.27</v>
+        <v>74.5</v>
       </c>
       <c r="H22" t="n">
-        <v>72.09999999999999</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="I22" t="n">
-        <v>74.31999999999999</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J22" t="n">
-        <v>8.77</v>
+        <v>10.64</v>
       </c>
       <c r="K22" t="n">
-        <v>10.47</v>
+        <v>11.07</v>
       </c>
       <c r="L22" t="n">
-        <v>8.68</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="M22" t="n">
-        <v>9.949999999999999</v>
+        <v>9.93</v>
       </c>
       <c r="N22" t="n">
-        <v>42.51</v>
+        <v>44.68</v>
       </c>
       <c r="O22" t="n">
-        <v>44.82</v>
+        <v>45.53</v>
       </c>
       <c r="P22" t="n">
-        <v>42.44</v>
+        <v>43.46</v>
       </c>
       <c r="Q22" t="n">
-        <v>43.54</v>
+        <v>44.37</v>
       </c>
       <c r="R22" t="n">
-        <v>-7.571</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="S22" t="n">
-        <v>-17.6346</v>
+        <v>-18.422</v>
       </c>
       <c r="T22" t="n">
-        <v>-20.3077</v>
+        <v>-11.958</v>
       </c>
       <c r="U22" t="n">
-        <v>-1.3539</v>
+        <v>-1.8703</v>
       </c>
       <c r="V22" t="n">
-        <v>-3.7804</v>
+        <v>-7.6251</v>
       </c>
       <c r="W22" t="n">
-        <v>-3.4304</v>
+        <v>-2.7081</v>
       </c>
       <c r="X22" t="n">
-        <v>7.8007</v>
+        <v>-0.201</v>
       </c>
       <c r="Y22" t="n">
-        <v>19.1617</v>
+        <v>20.0726</v>
       </c>
       <c r="Z22" t="n">
-        <v>21.3415</v>
+        <v>10.9497</v>
       </c>
       <c r="AA22" t="n">
-        <v>1.3029</v>
+        <v>1.9063</v>
       </c>
       <c r="AB22" t="n">
-        <v>3.6914</v>
+        <v>8.0351</v>
       </c>
       <c r="AC22" t="n">
-        <v>3.1265</v>
+        <v>2.4475</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>141.24</v>
+        <v>161</v>
       </c>
       <c r="C23" t="n">
-        <v>160.58</v>
+        <v>173.69</v>
       </c>
       <c r="D23" t="n">
-        <v>135.02</v>
+        <v>161.04</v>
       </c>
       <c r="E23" t="n">
-        <v>151.89</v>
+        <v>173.2</v>
       </c>
       <c r="F23" t="n">
-        <v>72.41</v>
+        <v>74.084</v>
       </c>
       <c r="G23" t="n">
-        <v>74.5</v>
+        <v>76.53</v>
       </c>
       <c r="H23" t="n">
-        <v>70.9616</v>
+        <v>73.61499999999999</v>
       </c>
       <c r="I23" t="n">
-        <v>72.93000000000001</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J23" t="n">
-        <v>10.6403</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K23" t="n">
-        <v>11.07</v>
+        <v>9.35</v>
       </c>
       <c r="L23" t="n">
-        <v>9.369999999999999</v>
+        <v>8.51</v>
       </c>
       <c r="M23" t="n">
-        <v>9.93</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N23" t="n">
-        <v>44.69</v>
+        <v>43.675</v>
       </c>
       <c r="O23" t="n">
-        <v>45.53</v>
+        <v>43.965</v>
       </c>
       <c r="P23" t="n">
-        <v>43.455</v>
+        <v>42.19</v>
       </c>
       <c r="Q23" t="n">
-        <v>44.37</v>
+        <v>42.19</v>
       </c>
       <c r="R23" t="n">
-        <v>0.09229999999999999</v>
+        <v>14.0299</v>
       </c>
       <c r="S23" t="n">
-        <v>-18.422</v>
+        <v>5.494</v>
       </c>
       <c r="T23" t="n">
-        <v>-11.958</v>
+        <v>-5.9922</v>
       </c>
       <c r="U23" t="n">
-        <v>-1.8703</v>
+        <v>4.9088</v>
       </c>
       <c r="V23" t="n">
-        <v>-7.6251</v>
+        <v>1.553</v>
       </c>
       <c r="W23" t="n">
-        <v>-2.7081</v>
+        <v>-0.9451000000000001</v>
       </c>
       <c r="X23" t="n">
-        <v>-0.201</v>
+        <v>-13.998</v>
       </c>
       <c r="Y23" t="n">
-        <v>20.0726</v>
+        <v>-7.4756</v>
       </c>
       <c r="Z23" t="n">
-        <v>10.9497</v>
+        <v>2.2754</v>
       </c>
       <c r="AA23" t="n">
-        <v>1.9063</v>
+        <v>-4.9132</v>
       </c>
       <c r="AB23" t="n">
-        <v>8.0351</v>
+        <v>-1.8381</v>
       </c>
       <c r="AC23" t="n">
-        <v>2.4475</v>
+        <v>0.4763</v>
       </c>
     </row>
   </sheetData>
@@ -2503,7 +2503,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-05-21 23:03
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1895 +568,1895 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>97.97</v>
+        <v>102.94</v>
       </c>
       <c r="C2" t="n">
-        <v>99.95</v>
+        <v>106.09</v>
       </c>
       <c r="D2" t="n">
-        <v>95.31999999999999</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>98.09</v>
+        <v>105.64</v>
       </c>
       <c r="F2" t="n">
-        <v>58.48</v>
+        <v>58.93</v>
       </c>
       <c r="G2" t="n">
-        <v>58.97</v>
+        <v>60.3</v>
       </c>
       <c r="H2" t="n">
-        <v>56.82</v>
+        <v>58.49</v>
       </c>
       <c r="I2" t="n">
-        <v>57.4</v>
+        <v>60.21</v>
       </c>
       <c r="J2" t="n">
-        <v>18.25</v>
+        <v>17.37</v>
       </c>
       <c r="K2" t="n">
-        <v>18.76</v>
+        <v>17.95</v>
       </c>
       <c r="L2" t="n">
-        <v>17.85</v>
+        <v>16.72</v>
       </c>
       <c r="M2" t="n">
-        <v>18.2</v>
+        <v>16.8</v>
       </c>
       <c r="N2" t="n">
-        <v>56.52</v>
+        <v>56.05</v>
       </c>
       <c r="O2" t="n">
-        <v>58.15</v>
+        <v>56.49</v>
       </c>
       <c r="P2" t="n">
-        <v>56.04</v>
+        <v>54.66</v>
       </c>
       <c r="Q2" t="n">
-        <v>57.59</v>
+        <v>54.73</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>102.94</v>
+        <v>108.62</v>
       </c>
       <c r="C3" t="n">
-        <v>106.09</v>
+        <v>116.77</v>
       </c>
       <c r="D3" t="n">
-        <v>99.59999999999999</v>
+        <v>107.46</v>
       </c>
       <c r="E3" t="n">
-        <v>105.64</v>
+        <v>112.77</v>
       </c>
       <c r="F3" t="n">
-        <v>58.93</v>
+        <v>59.8</v>
       </c>
       <c r="G3" t="n">
-        <v>60.3</v>
+        <v>60.73</v>
       </c>
       <c r="H3" t="n">
-        <v>58.49</v>
+        <v>57.59</v>
       </c>
       <c r="I3" t="n">
-        <v>60.21</v>
+        <v>59.22</v>
       </c>
       <c r="J3" t="n">
-        <v>17.37</v>
+        <v>16.35</v>
       </c>
       <c r="K3" t="n">
-        <v>17.95</v>
+        <v>16.52</v>
       </c>
       <c r="L3" t="n">
-        <v>16.72</v>
+        <v>15.06</v>
       </c>
       <c r="M3" t="n">
-        <v>16.8</v>
+        <v>15.7</v>
       </c>
       <c r="N3" t="n">
-        <v>56.05</v>
+        <v>55.13</v>
       </c>
       <c r="O3" t="n">
-        <v>56.49</v>
+        <v>57.14</v>
       </c>
       <c r="P3" t="n">
-        <v>54.66</v>
+        <v>54.28</v>
       </c>
       <c r="Q3" t="n">
-        <v>54.73</v>
+        <v>55.66</v>
       </c>
       <c r="R3" t="n">
-        <v>7.697</v>
+        <v>6.7493</v>
       </c>
       <c r="U3" t="n">
-        <v>4.8955</v>
+        <v>-1.6442</v>
       </c>
       <c r="X3" t="n">
-        <v>-7.6923</v>
+        <v>-6.5476</v>
       </c>
       <c r="AA3" t="n">
-        <v>-4.9661</v>
+        <v>1.6993</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>108.62</v>
+        <v>125.21</v>
       </c>
       <c r="C4" t="n">
-        <v>116.77</v>
+        <v>130.12</v>
       </c>
       <c r="D4" t="n">
-        <v>107.46</v>
+        <v>120.24</v>
       </c>
       <c r="E4" t="n">
-        <v>112.77</v>
+        <v>128.32</v>
       </c>
       <c r="F4" t="n">
-        <v>59.8</v>
+        <v>61.08</v>
       </c>
       <c r="G4" t="n">
-        <v>60.73</v>
+        <v>62.74</v>
       </c>
       <c r="H4" t="n">
-        <v>57.59</v>
+        <v>60.56</v>
       </c>
       <c r="I4" t="n">
-        <v>59.22</v>
+        <v>62.56</v>
       </c>
       <c r="J4" t="n">
-        <v>16.35</v>
+        <v>13.99</v>
       </c>
       <c r="K4" t="n">
-        <v>16.52</v>
+        <v>14.66</v>
       </c>
       <c r="L4" t="n">
-        <v>15.06</v>
+        <v>13.3</v>
       </c>
       <c r="M4" t="n">
-        <v>15.7</v>
+        <v>13.52</v>
       </c>
       <c r="N4" t="n">
-        <v>55.13</v>
+        <v>53.93</v>
       </c>
       <c r="O4" t="n">
-        <v>57.14</v>
+        <v>54.43</v>
       </c>
       <c r="P4" t="n">
-        <v>54.28</v>
+        <v>52.37</v>
       </c>
       <c r="Q4" t="n">
-        <v>55.66</v>
+        <v>52.5</v>
       </c>
       <c r="R4" t="n">
-        <v>6.7493</v>
+        <v>13.7891</v>
       </c>
       <c r="U4" t="n">
-        <v>-1.6442</v>
+        <v>5.64</v>
       </c>
       <c r="X4" t="n">
-        <v>-6.5476</v>
+        <v>-13.8854</v>
       </c>
       <c r="AA4" t="n">
-        <v>1.6993</v>
+        <v>-5.6773</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>125.21</v>
+        <v>128.33</v>
       </c>
       <c r="C5" t="n">
-        <v>130.12</v>
+        <v>129.59</v>
       </c>
       <c r="D5" t="n">
-        <v>120.24</v>
+        <v>117.79</v>
       </c>
       <c r="E5" t="n">
-        <v>128.32</v>
+        <v>123.39</v>
       </c>
       <c r="F5" t="n">
-        <v>61.08</v>
+        <v>62.41</v>
       </c>
       <c r="G5" t="n">
-        <v>62.74</v>
+        <v>62.7</v>
       </c>
       <c r="H5" t="n">
-        <v>60.56</v>
+        <v>61.64</v>
       </c>
       <c r="I5" t="n">
-        <v>62.56</v>
+        <v>62.64</v>
       </c>
       <c r="J5" t="n">
-        <v>13.99</v>
+        <v>13.51</v>
       </c>
       <c r="K5" t="n">
-        <v>14.66</v>
+        <v>14.63</v>
       </c>
       <c r="L5" t="n">
-        <v>13.3</v>
+        <v>13.41</v>
       </c>
       <c r="M5" t="n">
-        <v>13.52</v>
+        <v>14.03</v>
       </c>
       <c r="N5" t="n">
-        <v>53.93</v>
+        <v>52.67</v>
       </c>
       <c r="O5" t="n">
-        <v>54.43</v>
+        <v>53.31</v>
       </c>
       <c r="P5" t="n">
-        <v>52.37</v>
+        <v>52.42</v>
       </c>
       <c r="Q5" t="n">
-        <v>52.5</v>
+        <v>52.45</v>
       </c>
       <c r="R5" t="n">
-        <v>13.7891</v>
+        <v>-3.842</v>
       </c>
       <c r="S5" t="n">
-        <v>30.8186</v>
+        <v>16.8023</v>
       </c>
       <c r="U5" t="n">
-        <v>5.64</v>
+        <v>0.1279</v>
       </c>
       <c r="V5" t="n">
-        <v>8.9895</v>
+        <v>4.0359</v>
       </c>
       <c r="X5" t="n">
-        <v>-13.8854</v>
+        <v>3.7722</v>
       </c>
       <c r="Y5" t="n">
-        <v>-25.7143</v>
+        <v>-16.4881</v>
       </c>
       <c r="AA5" t="n">
-        <v>-5.6773</v>
+        <v>-0.09520000000000001</v>
       </c>
       <c r="AB5" t="n">
-        <v>-8.8383</v>
+        <v>-4.1659</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>128.33</v>
+        <v>108.75</v>
       </c>
       <c r="C6" t="n">
-        <v>129.59</v>
+        <v>115.62</v>
       </c>
       <c r="D6" t="n">
-        <v>117.79</v>
+        <v>103.99</v>
       </c>
       <c r="E6" t="n">
-        <v>123.39</v>
+        <v>109.56</v>
       </c>
       <c r="F6" t="n">
-        <v>62.41</v>
+        <v>60.72</v>
       </c>
       <c r="G6" t="n">
-        <v>62.7</v>
+        <v>61.33</v>
       </c>
       <c r="H6" t="n">
-        <v>61.64</v>
+        <v>59.68</v>
       </c>
       <c r="I6" t="n">
-        <v>62.64</v>
+        <v>60.74</v>
       </c>
       <c r="J6" t="n">
-        <v>13.51</v>
+        <v>15.71</v>
       </c>
       <c r="K6" t="n">
-        <v>14.63</v>
+        <v>16.27</v>
       </c>
       <c r="L6" t="n">
-        <v>13.41</v>
+        <v>14.93</v>
       </c>
       <c r="M6" t="n">
-        <v>14.03</v>
+        <v>15.59</v>
       </c>
       <c r="N6" t="n">
-        <v>52.67</v>
+        <v>54.09</v>
       </c>
       <c r="O6" t="n">
-        <v>53.31</v>
+        <v>54.96</v>
       </c>
       <c r="P6" t="n">
-        <v>52.42</v>
+        <v>53.58</v>
       </c>
       <c r="Q6" t="n">
-        <v>52.45</v>
+        <v>54.05</v>
       </c>
       <c r="R6" t="n">
-        <v>-3.842</v>
+        <v>-11.2084</v>
       </c>
       <c r="S6" t="n">
-        <v>16.8023</v>
+        <v>-2.8465</v>
       </c>
       <c r="U6" t="n">
-        <v>0.1279</v>
+        <v>-3.0332</v>
       </c>
       <c r="V6" t="n">
-        <v>4.0359</v>
+        <v>2.5667</v>
       </c>
       <c r="X6" t="n">
-        <v>3.7722</v>
+        <v>11.119</v>
       </c>
       <c r="Y6" t="n">
-        <v>-16.4881</v>
+        <v>-0.7006</v>
       </c>
       <c r="AA6" t="n">
-        <v>-0.09520000000000001</v>
+        <v>3.0505</v>
       </c>
       <c r="AB6" t="n">
-        <v>-4.1659</v>
+        <v>-2.8926</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>108.75</v>
+        <v>114.76</v>
       </c>
       <c r="C7" t="n">
-        <v>115.62</v>
+        <v>118.32</v>
       </c>
       <c r="D7" t="n">
-        <v>103.99</v>
+        <v>112.3</v>
       </c>
       <c r="E7" t="n">
-        <v>109.56</v>
+        <v>117.97</v>
       </c>
       <c r="F7" t="n">
-        <v>60.72</v>
+        <v>61</v>
       </c>
       <c r="G7" t="n">
-        <v>61.33</v>
+        <v>61.87</v>
       </c>
       <c r="H7" t="n">
-        <v>59.68</v>
+        <v>60.45</v>
       </c>
       <c r="I7" t="n">
-        <v>60.74</v>
+        <v>61.86</v>
       </c>
       <c r="J7" t="n">
-        <v>15.71</v>
+        <v>14.91</v>
       </c>
       <c r="K7" t="n">
-        <v>16.27</v>
+        <v>15.24</v>
       </c>
       <c r="L7" t="n">
-        <v>14.93</v>
+        <v>14.38</v>
       </c>
       <c r="M7" t="n">
-        <v>15.59</v>
+        <v>14.4</v>
       </c>
       <c r="N7" t="n">
-        <v>54.09</v>
+        <v>53.84</v>
       </c>
       <c r="O7" t="n">
-        <v>54.96</v>
+        <v>54.33</v>
       </c>
       <c r="P7" t="n">
-        <v>53.58</v>
+        <v>53.06</v>
       </c>
       <c r="Q7" t="n">
-        <v>54.05</v>
+        <v>53.08</v>
       </c>
       <c r="R7" t="n">
-        <v>-11.2084</v>
+        <v>7.6762</v>
       </c>
       <c r="S7" t="n">
-        <v>-2.8465</v>
+        <v>-8.065799999999999</v>
       </c>
       <c r="T7" t="n">
-        <v>11.6933</v>
+        <v>11.6717</v>
       </c>
       <c r="U7" t="n">
-        <v>-3.0332</v>
+        <v>1.8439</v>
       </c>
       <c r="V7" t="n">
-        <v>2.5667</v>
+        <v>-1.1189</v>
       </c>
       <c r="W7" t="n">
-        <v>5.8188</v>
+        <v>2.7404</v>
       </c>
       <c r="X7" t="n">
-        <v>11.119</v>
+        <v>-7.6331</v>
       </c>
       <c r="Y7" t="n">
-        <v>-0.7006</v>
+        <v>6.5089</v>
       </c>
       <c r="Z7" t="n">
-        <v>-14.3407</v>
+        <v>-14.2857</v>
       </c>
       <c r="AA7" t="n">
-        <v>3.0505</v>
+        <v>-1.7946</v>
       </c>
       <c r="AB7" t="n">
-        <v>-2.8926</v>
+        <v>1.1048</v>
       </c>
       <c r="AC7" t="n">
-        <v>-6.1469</v>
+        <v>-3.0148</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>114.76</v>
+        <v>122.81</v>
       </c>
       <c r="C8" t="n">
-        <v>118.32</v>
+        <v>127.45</v>
       </c>
       <c r="D8" t="n">
-        <v>112.3</v>
+        <v>117.5</v>
       </c>
       <c r="E8" t="n">
-        <v>117.97</v>
+        <v>126.98</v>
       </c>
       <c r="F8" t="n">
-        <v>61</v>
+        <v>62.89</v>
       </c>
       <c r="G8" t="n">
-        <v>61.87</v>
+        <v>63.8</v>
       </c>
       <c r="H8" t="n">
-        <v>60.45</v>
+        <v>60.7</v>
       </c>
       <c r="I8" t="n">
-        <v>61.86</v>
+        <v>63.54</v>
       </c>
       <c r="J8" t="n">
-        <v>14.91</v>
+        <v>13.84</v>
       </c>
       <c r="K8" t="n">
-        <v>15.24</v>
+        <v>14.49</v>
       </c>
       <c r="L8" t="n">
-        <v>14.38</v>
+        <v>13.25</v>
       </c>
       <c r="M8" t="n">
-        <v>14.4</v>
+        <v>13.3</v>
       </c>
       <c r="N8" t="n">
-        <v>53.84</v>
+        <v>52.21</v>
       </c>
       <c r="O8" t="n">
-        <v>54.33</v>
+        <v>54.09</v>
       </c>
       <c r="P8" t="n">
-        <v>53.06</v>
+        <v>51.4</v>
       </c>
       <c r="Q8" t="n">
-        <v>53.08</v>
+        <v>51.65</v>
       </c>
       <c r="R8" t="n">
-        <v>7.6762</v>
+        <v>7.6375</v>
       </c>
       <c r="S8" t="n">
-        <v>-8.065799999999999</v>
+        <v>2.9095</v>
       </c>
       <c r="T8" t="n">
-        <v>11.6717</v>
+        <v>12.6009</v>
       </c>
       <c r="U8" t="n">
-        <v>1.8439</v>
+        <v>2.7158</v>
       </c>
       <c r="V8" t="n">
-        <v>-1.1189</v>
+        <v>1.4368</v>
       </c>
       <c r="W8" t="n">
-        <v>2.7404</v>
+        <v>7.2948</v>
       </c>
       <c r="X8" t="n">
-        <v>-7.6331</v>
+        <v>-7.6389</v>
       </c>
       <c r="Y8" t="n">
-        <v>6.5089</v>
+        <v>-5.2031</v>
       </c>
       <c r="Z8" t="n">
-        <v>-14.2857</v>
+        <v>-15.2866</v>
       </c>
       <c r="AA8" t="n">
-        <v>-1.7946</v>
+        <v>-2.694</v>
       </c>
       <c r="AB8" t="n">
-        <v>1.1048</v>
+        <v>-1.5253</v>
       </c>
       <c r="AC8" t="n">
-        <v>-3.0148</v>
+        <v>-7.2045</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>122.81</v>
+        <v>124.39</v>
       </c>
       <c r="C9" t="n">
-        <v>127.45</v>
+        <v>131.38</v>
       </c>
       <c r="D9" t="n">
-        <v>117.5</v>
+        <v>121.66</v>
       </c>
       <c r="E9" t="n">
-        <v>126.98</v>
+        <v>130.4</v>
       </c>
       <c r="F9" t="n">
-        <v>62.89</v>
+        <v>63.89</v>
       </c>
       <c r="G9" t="n">
-        <v>63.8</v>
+        <v>65.84</v>
       </c>
       <c r="H9" t="n">
-        <v>60.7</v>
+        <v>63.81</v>
       </c>
       <c r="I9" t="n">
-        <v>63.54</v>
+        <v>65.3</v>
       </c>
       <c r="J9" t="n">
-        <v>13.84</v>
+        <v>13.61</v>
       </c>
       <c r="K9" t="n">
-        <v>14.49</v>
+        <v>13.89</v>
       </c>
       <c r="L9" t="n">
-        <v>13.25</v>
+        <v>12.87</v>
       </c>
       <c r="M9" t="n">
-        <v>13.3</v>
+        <v>12.98</v>
       </c>
       <c r="N9" t="n">
-        <v>52.21</v>
+        <v>51.36</v>
       </c>
       <c r="O9" t="n">
-        <v>54.09</v>
+        <v>51.45</v>
       </c>
       <c r="P9" t="n">
-        <v>51.4</v>
+        <v>49.79</v>
       </c>
       <c r="Q9" t="n">
-        <v>51.65</v>
+        <v>50.22</v>
       </c>
       <c r="R9" t="n">
-        <v>7.6375</v>
+        <v>2.6933</v>
       </c>
       <c r="S9" t="n">
-        <v>2.9095</v>
+        <v>19.0215</v>
       </c>
       <c r="T9" t="n">
-        <v>12.6009</v>
+        <v>1.6209</v>
       </c>
       <c r="U9" t="n">
-        <v>2.7158</v>
+        <v>2.7699</v>
       </c>
       <c r="V9" t="n">
-        <v>1.4368</v>
+        <v>7.5074</v>
       </c>
       <c r="W9" t="n">
-        <v>7.2948</v>
+        <v>4.3798</v>
       </c>
       <c r="X9" t="n">
-        <v>-7.6389</v>
+        <v>-2.406</v>
       </c>
       <c r="Y9" t="n">
-        <v>-5.2031</v>
+        <v>-16.7415</v>
       </c>
       <c r="Z9" t="n">
-        <v>-15.2866</v>
+        <v>-3.9941</v>
       </c>
       <c r="AA9" t="n">
-        <v>-2.694</v>
+        <v>-2.7686</v>
       </c>
       <c r="AB9" t="n">
-        <v>-1.5253</v>
+        <v>-7.086</v>
       </c>
       <c r="AC9" t="n">
-        <v>-7.2045</v>
+        <v>-4.3429</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>124.39</v>
+        <v>132.2</v>
       </c>
       <c r="C10" t="n">
-        <v>131.38</v>
+        <v>133.67</v>
       </c>
       <c r="D10" t="n">
-        <v>121.66</v>
+        <v>123.8</v>
       </c>
       <c r="E10" t="n">
-        <v>130.4</v>
+        <v>127.55</v>
       </c>
       <c r="F10" t="n">
-        <v>63.89</v>
+        <v>65.44</v>
       </c>
       <c r="G10" t="n">
-        <v>65.84</v>
+        <v>66.05</v>
       </c>
       <c r="H10" t="n">
-        <v>63.81</v>
+        <v>63.78</v>
       </c>
       <c r="I10" t="n">
-        <v>65.3</v>
+        <v>64.91</v>
       </c>
       <c r="J10" t="n">
-        <v>13.61</v>
+        <v>12.8</v>
       </c>
       <c r="K10" t="n">
-        <v>13.89</v>
+        <v>13.64</v>
       </c>
       <c r="L10" t="n">
-        <v>12.87</v>
+        <v>12.65</v>
       </c>
       <c r="M10" t="n">
-        <v>12.98</v>
+        <v>13.26</v>
       </c>
       <c r="N10" t="n">
-        <v>51.36</v>
+        <v>50.12</v>
       </c>
       <c r="O10" t="n">
-        <v>51.45</v>
+        <v>51.43</v>
       </c>
       <c r="P10" t="n">
-        <v>49.79</v>
+        <v>49.65</v>
       </c>
       <c r="Q10" t="n">
-        <v>50.22</v>
+        <v>50.51</v>
       </c>
       <c r="R10" t="n">
-        <v>2.6933</v>
+        <v>-2.1856</v>
       </c>
       <c r="S10" t="n">
-        <v>19.0215</v>
+        <v>8.120699999999999</v>
       </c>
       <c r="T10" t="n">
-        <v>1.6209</v>
+        <v>3.3714</v>
       </c>
       <c r="U10" t="n">
-        <v>2.7699</v>
+        <v>-0.5972</v>
       </c>
       <c r="V10" t="n">
-        <v>7.5074</v>
+        <v>4.9305</v>
       </c>
       <c r="W10" t="n">
-        <v>4.3798</v>
+        <v>3.6239</v>
       </c>
       <c r="X10" t="n">
-        <v>-2.406</v>
+        <v>2.1572</v>
       </c>
       <c r="Y10" t="n">
-        <v>-16.7415</v>
+        <v>-7.9167</v>
       </c>
       <c r="Z10" t="n">
-        <v>-3.9941</v>
+        <v>-5.4882</v>
       </c>
       <c r="AA10" t="n">
-        <v>-2.7686</v>
+        <v>0.5775</v>
       </c>
       <c r="AB10" t="n">
-        <v>-7.086</v>
+        <v>-4.8417</v>
       </c>
       <c r="AC10" t="n">
-        <v>-4.3429</v>
+        <v>-3.6988</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>132.2</v>
+        <v>135</v>
       </c>
       <c r="C11" t="n">
-        <v>133.67</v>
+        <v>147.26</v>
       </c>
       <c r="D11" t="n">
-        <v>123.8</v>
+        <v>134.02</v>
       </c>
       <c r="E11" t="n">
-        <v>127.55</v>
+        <v>144.16</v>
       </c>
       <c r="F11" t="n">
-        <v>65.44</v>
+        <v>66.37</v>
       </c>
       <c r="G11" t="n">
-        <v>66.05</v>
+        <v>67.77</v>
       </c>
       <c r="H11" t="n">
-        <v>63.78</v>
+        <v>66.25</v>
       </c>
       <c r="I11" t="n">
-        <v>64.91</v>
+        <v>67.39</v>
       </c>
       <c r="J11" t="n">
-        <v>12.8</v>
+        <v>12.5</v>
       </c>
       <c r="K11" t="n">
-        <v>13.64</v>
+        <v>12.59</v>
       </c>
       <c r="L11" t="n">
-        <v>12.65</v>
+        <v>11.21</v>
       </c>
       <c r="M11" t="n">
-        <v>13.26</v>
+        <v>11.51</v>
       </c>
       <c r="N11" t="n">
-        <v>50.12</v>
+        <v>49.4</v>
       </c>
       <c r="O11" t="n">
-        <v>51.43</v>
+        <v>49.49</v>
       </c>
       <c r="P11" t="n">
-        <v>49.65</v>
+        <v>48.3</v>
       </c>
       <c r="Q11" t="n">
-        <v>50.51</v>
+        <v>48.59</v>
       </c>
       <c r="R11" t="n">
-        <v>-2.1856</v>
+        <v>13.0223</v>
       </c>
       <c r="S11" t="n">
-        <v>8.120699999999999</v>
+        <v>13.5297</v>
       </c>
       <c r="T11" t="n">
-        <v>3.3714</v>
+        <v>31.5809</v>
       </c>
       <c r="U11" t="n">
-        <v>-0.5972</v>
+        <v>3.8207</v>
       </c>
       <c r="V11" t="n">
-        <v>4.9305</v>
+        <v>6.0592</v>
       </c>
       <c r="W11" t="n">
-        <v>3.6239</v>
+        <v>10.9483</v>
       </c>
       <c r="X11" t="n">
-        <v>2.1572</v>
+        <v>-13.1976</v>
       </c>
       <c r="Y11" t="n">
-        <v>-7.9167</v>
+        <v>-13.4586</v>
       </c>
       <c r="Z11" t="n">
-        <v>-5.4882</v>
+        <v>-26.1706</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.5775</v>
+        <v>-3.8012</v>
       </c>
       <c r="AB11" t="n">
-        <v>-4.8417</v>
+        <v>-5.9245</v>
       </c>
       <c r="AC11" t="n">
-        <v>-3.6988</v>
+        <v>-10.1018</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>135</v>
+        <v>157.84</v>
       </c>
       <c r="C12" t="n">
-        <v>147.26</v>
+        <v>166</v>
       </c>
       <c r="D12" t="n">
-        <v>134.02</v>
+        <v>149.06</v>
       </c>
       <c r="E12" t="n">
-        <v>144.16</v>
+        <v>165.85</v>
       </c>
       <c r="F12" t="n">
-        <v>66.37</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>67.77</v>
+        <v>71.66</v>
       </c>
       <c r="H12" t="n">
-        <v>66.25</v>
+        <v>68.88</v>
       </c>
       <c r="I12" t="n">
-        <v>67.39</v>
+        <v>71.56999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>12.5</v>
+        <v>10.43</v>
       </c>
       <c r="K12" t="n">
-        <v>12.59</v>
+        <v>11.14</v>
       </c>
       <c r="L12" t="n">
-        <v>11.21</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M12" t="n">
-        <v>11.51</v>
+        <v>9.81</v>
       </c>
       <c r="N12" t="n">
-        <v>49.4</v>
+        <v>47.26</v>
       </c>
       <c r="O12" t="n">
-        <v>49.49</v>
+        <v>47.54</v>
       </c>
       <c r="P12" t="n">
-        <v>48.3</v>
+        <v>45.52</v>
       </c>
       <c r="Q12" t="n">
-        <v>48.59</v>
+        <v>45.59</v>
       </c>
       <c r="R12" t="n">
-        <v>13.0223</v>
+        <v>15.0458</v>
       </c>
       <c r="S12" t="n">
-        <v>13.5297</v>
+        <v>27.1856</v>
       </c>
       <c r="T12" t="n">
-        <v>31.5809</v>
+        <v>40.5866</v>
       </c>
       <c r="U12" t="n">
-        <v>3.8207</v>
+        <v>6.2027</v>
       </c>
       <c r="V12" t="n">
-        <v>6.0592</v>
+        <v>9.601800000000001</v>
       </c>
       <c r="W12" t="n">
-        <v>10.9483</v>
+        <v>15.6967</v>
       </c>
       <c r="X12" t="n">
-        <v>-13.1976</v>
+        <v>-14.7698</v>
       </c>
       <c r="Y12" t="n">
-        <v>-13.4586</v>
+        <v>-24.4222</v>
       </c>
       <c r="Z12" t="n">
-        <v>-26.1706</v>
+        <v>-31.875</v>
       </c>
       <c r="AA12" t="n">
-        <v>-3.8012</v>
+        <v>-6.1741</v>
       </c>
       <c r="AB12" t="n">
-        <v>-5.9245</v>
+        <v>-9.2194</v>
       </c>
       <c r="AC12" t="n">
-        <v>-10.1018</v>
+        <v>-14.1108</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>157.84</v>
+        <v>162.12</v>
       </c>
       <c r="C13" t="n">
-        <v>166</v>
+        <v>162.9</v>
       </c>
       <c r="D13" t="n">
-        <v>149.06</v>
+        <v>147.61</v>
       </c>
       <c r="E13" t="n">
-        <v>165.85</v>
+        <v>152.1</v>
       </c>
       <c r="F13" t="n">
-        <v>69.26000000000001</v>
+        <v>71.87</v>
       </c>
       <c r="G13" t="n">
-        <v>71.66</v>
+        <v>73.3</v>
       </c>
       <c r="H13" t="n">
-        <v>68.88</v>
+        <v>70.38</v>
       </c>
       <c r="I13" t="n">
-        <v>71.56999999999999</v>
+        <v>71.34</v>
       </c>
       <c r="J13" t="n">
-        <v>10.43</v>
+        <v>10.02</v>
       </c>
       <c r="K13" t="n">
-        <v>11.14</v>
+        <v>10.88</v>
       </c>
       <c r="L13" t="n">
-        <v>9.800000000000001</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="M13" t="n">
-        <v>9.81</v>
+        <v>10.6</v>
       </c>
       <c r="N13" t="n">
-        <v>47.26</v>
+        <v>45.41</v>
       </c>
       <c r="O13" t="n">
-        <v>47.54</v>
+        <v>46.36</v>
       </c>
       <c r="P13" t="n">
-        <v>45.52</v>
+        <v>44.5</v>
       </c>
       <c r="Q13" t="n">
-        <v>45.59</v>
+        <v>45.73</v>
       </c>
       <c r="R13" t="n">
-        <v>15.0458</v>
+        <v>-8.2906</v>
       </c>
       <c r="S13" t="n">
-        <v>27.1856</v>
+        <v>19.2474</v>
       </c>
       <c r="T13" t="n">
-        <v>40.5866</v>
+        <v>19.7826</v>
       </c>
       <c r="U13" t="n">
-        <v>6.2027</v>
+        <v>-0.3214</v>
       </c>
       <c r="V13" t="n">
-        <v>9.601800000000001</v>
+        <v>9.906000000000001</v>
       </c>
       <c r="W13" t="n">
-        <v>15.6967</v>
+        <v>12.2757</v>
       </c>
       <c r="X13" t="n">
-        <v>-14.7698</v>
+        <v>8.053000000000001</v>
       </c>
       <c r="Y13" t="n">
-        <v>-24.4222</v>
+        <v>-20.0603</v>
       </c>
       <c r="Z13" t="n">
-        <v>-31.875</v>
+        <v>-20.3008</v>
       </c>
       <c r="AA13" t="n">
-        <v>-6.1741</v>
+        <v>0.3071</v>
       </c>
       <c r="AB13" t="n">
-        <v>-9.2194</v>
+        <v>-9.4635</v>
       </c>
       <c r="AC13" t="n">
-        <v>-14.1108</v>
+        <v>-11.4618</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>162.12</v>
+        <v>163</v>
       </c>
       <c r="C14" t="n">
-        <v>162.9</v>
+        <v>177.5</v>
       </c>
       <c r="D14" t="n">
-        <v>147.61</v>
+        <v>161.51</v>
       </c>
       <c r="E14" t="n">
-        <v>152.1</v>
+        <v>176.94</v>
       </c>
       <c r="F14" t="n">
-        <v>71.87</v>
+        <v>72.81999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>73.3</v>
+        <v>76.31</v>
       </c>
       <c r="H14" t="n">
-        <v>70.38</v>
+        <v>72.7</v>
       </c>
       <c r="I14" t="n">
-        <v>71.34</v>
+        <v>76.28</v>
       </c>
       <c r="J14" t="n">
-        <v>10.02</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="K14" t="n">
-        <v>10.88</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="L14" t="n">
-        <v>9.970000000000001</v>
+        <v>8.84</v>
       </c>
       <c r="M14" t="n">
-        <v>10.6</v>
+        <v>8.85</v>
       </c>
       <c r="N14" t="n">
-        <v>45.41</v>
+        <v>44.82</v>
       </c>
       <c r="O14" t="n">
-        <v>46.36</v>
+        <v>44.89</v>
       </c>
       <c r="P14" t="n">
-        <v>44.5</v>
+        <v>42.57</v>
       </c>
       <c r="Q14" t="n">
-        <v>45.73</v>
+        <v>42.57</v>
       </c>
       <c r="R14" t="n">
-        <v>-8.2906</v>
+        <v>16.3314</v>
       </c>
       <c r="S14" t="n">
-        <v>19.2474</v>
+        <v>22.7386</v>
       </c>
       <c r="T14" t="n">
-        <v>19.7826</v>
+        <v>35.6902</v>
       </c>
       <c r="U14" t="n">
-        <v>-0.3214</v>
+        <v>6.9246</v>
       </c>
       <c r="V14" t="n">
-        <v>9.906000000000001</v>
+        <v>13.1919</v>
       </c>
       <c r="W14" t="n">
-        <v>12.2757</v>
+        <v>16.8147</v>
       </c>
       <c r="X14" t="n">
-        <v>8.053000000000001</v>
+        <v>-16.5094</v>
       </c>
       <c r="Y14" t="n">
-        <v>-20.0603</v>
+        <v>-23.1103</v>
       </c>
       <c r="Z14" t="n">
-        <v>-20.3008</v>
+        <v>-31.8182</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.3071</v>
+        <v>-6.9101</v>
       </c>
       <c r="AB14" t="n">
-        <v>-9.4635</v>
+        <v>-12.3894</v>
       </c>
       <c r="AC14" t="n">
-        <v>-11.4618</v>
+        <v>-15.233</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="C15" t="n">
-        <v>177.5</v>
+        <v>191.29</v>
       </c>
       <c r="D15" t="n">
-        <v>161.51</v>
+        <v>178.94</v>
       </c>
       <c r="E15" t="n">
-        <v>176.94</v>
+        <v>190.42</v>
       </c>
       <c r="F15" t="n">
-        <v>72.81999999999999</v>
+        <v>76</v>
       </c>
       <c r="G15" t="n">
-        <v>76.31</v>
+        <v>77.36</v>
       </c>
       <c r="H15" t="n">
-        <v>72.7</v>
+        <v>75.55</v>
       </c>
       <c r="I15" t="n">
-        <v>76.28</v>
+        <v>76.95999999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>9.859999999999999</v>
+        <v>8.65</v>
       </c>
       <c r="K15" t="n">
-        <v>9.970000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="L15" t="n">
-        <v>8.84</v>
+        <v>8.15</v>
       </c>
       <c r="M15" t="n">
-        <v>8.85</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="N15" t="n">
-        <v>44.82</v>
+        <v>42.74</v>
       </c>
       <c r="O15" t="n">
-        <v>44.89</v>
+        <v>43</v>
       </c>
       <c r="P15" t="n">
-        <v>42.57</v>
+        <v>41.99</v>
       </c>
       <c r="Q15" t="n">
-        <v>42.57</v>
+        <v>42.22</v>
       </c>
       <c r="R15" t="n">
-        <v>16.3314</v>
+        <v>7.6184</v>
       </c>
       <c r="S15" t="n">
-        <v>22.7386</v>
+        <v>14.8146</v>
       </c>
       <c r="T15" t="n">
-        <v>35.6902</v>
+        <v>49.2905</v>
       </c>
       <c r="U15" t="n">
-        <v>6.9246</v>
+        <v>0.8915</v>
       </c>
       <c r="V15" t="n">
-        <v>13.1919</v>
+        <v>7.5311</v>
       </c>
       <c r="W15" t="n">
-        <v>16.8147</v>
+        <v>18.5642</v>
       </c>
       <c r="X15" t="n">
-        <v>-16.5094</v>
+        <v>-7.3446</v>
       </c>
       <c r="Y15" t="n">
-        <v>-23.1103</v>
+        <v>-16.4118</v>
       </c>
       <c r="Z15" t="n">
-        <v>-31.8182</v>
+        <v>-38.1599</v>
       </c>
       <c r="AA15" t="n">
-        <v>-6.9101</v>
+        <v>-0.8222</v>
       </c>
       <c r="AB15" t="n">
-        <v>-12.3894</v>
+        <v>-7.392</v>
       </c>
       <c r="AC15" t="n">
-        <v>-15.233</v>
+        <v>-16.4126</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>181</v>
+        <v>177.62</v>
       </c>
       <c r="C16" t="n">
-        <v>191.29</v>
+        <v>182.24</v>
       </c>
       <c r="D16" t="n">
-        <v>178.94</v>
+        <v>150.58</v>
       </c>
       <c r="E16" t="n">
-        <v>190.42</v>
+        <v>172.52</v>
       </c>
       <c r="F16" t="n">
-        <v>76</v>
+        <v>75.3</v>
       </c>
       <c r="G16" t="n">
-        <v>77.36</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="H16" t="n">
-        <v>75.55</v>
+        <v>71.55</v>
       </c>
       <c r="I16" t="n">
-        <v>76.95999999999999</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="J16" t="n">
-        <v>8.65</v>
+        <v>8.75</v>
       </c>
       <c r="K16" t="n">
-        <v>8.77</v>
+        <v>9.91</v>
       </c>
       <c r="L16" t="n">
-        <v>8.15</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="M16" t="n">
-        <v>8.199999999999999</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N16" t="n">
-        <v>42.74</v>
+        <v>43.14</v>
       </c>
       <c r="O16" t="n">
-        <v>43</v>
+        <v>45.19</v>
       </c>
       <c r="P16" t="n">
-        <v>41.99</v>
+        <v>42.79</v>
       </c>
       <c r="Q16" t="n">
-        <v>42.22</v>
+        <v>43.31</v>
       </c>
       <c r="R16" t="n">
-        <v>7.6184</v>
+        <v>-9.4003</v>
       </c>
       <c r="S16" t="n">
-        <v>14.8146</v>
+        <v>13.4254</v>
       </c>
       <c r="T16" t="n">
-        <v>49.2905</v>
+        <v>19.6726</v>
       </c>
       <c r="U16" t="n">
-        <v>0.8915</v>
+        <v>-2.5988</v>
       </c>
       <c r="V16" t="n">
-        <v>7.5311</v>
+        <v>5.0743</v>
       </c>
       <c r="W16" t="n">
-        <v>18.5642</v>
+        <v>11.2331</v>
       </c>
       <c r="X16" t="n">
-        <v>-7.3446</v>
+        <v>9.1463</v>
       </c>
       <c r="Y16" t="n">
-        <v>-16.4118</v>
+        <v>-15.566</v>
       </c>
       <c r="Z16" t="n">
-        <v>-38.1599</v>
+        <v>-22.2415</v>
       </c>
       <c r="AA16" t="n">
-        <v>-0.8222</v>
+        <v>2.5817</v>
       </c>
       <c r="AB16" t="n">
-        <v>-7.392</v>
+        <v>-5.2919</v>
       </c>
       <c r="AC16" t="n">
-        <v>-16.4126</v>
+        <v>-10.8664</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>177.62</v>
+        <v>183.84</v>
       </c>
       <c r="C17" t="n">
-        <v>182.24</v>
+        <v>188.49</v>
       </c>
       <c r="D17" t="n">
-        <v>150.58</v>
+        <v>172.26</v>
       </c>
       <c r="E17" t="n">
-        <v>172.52</v>
+        <v>184.24</v>
       </c>
       <c r="F17" t="n">
-        <v>75.3</v>
+        <v>75.81</v>
       </c>
       <c r="G17" t="n">
-        <v>75.93000000000001</v>
+        <v>77.94</v>
       </c>
       <c r="H17" t="n">
-        <v>71.55</v>
+        <v>74.19</v>
       </c>
       <c r="I17" t="n">
-        <v>74.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>8.75</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K17" t="n">
-        <v>9.91</v>
+        <v>8.98</v>
       </c>
       <c r="L17" t="n">
-        <v>8.550000000000001</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="M17" t="n">
-        <v>8.949999999999999</v>
+        <v>8.35</v>
       </c>
       <c r="N17" t="n">
-        <v>43.14</v>
+        <v>42.83</v>
       </c>
       <c r="O17" t="n">
-        <v>45.19</v>
+        <v>43.77</v>
       </c>
       <c r="P17" t="n">
-        <v>42.79</v>
+        <v>41.6</v>
       </c>
       <c r="Q17" t="n">
-        <v>43.31</v>
+        <v>41.99</v>
       </c>
       <c r="R17" t="n">
-        <v>-9.4003</v>
+        <v>6.7934</v>
       </c>
       <c r="S17" t="n">
-        <v>13.4254</v>
+        <v>4.1257</v>
       </c>
       <c r="T17" t="n">
-        <v>19.6726</v>
+        <v>11.0883</v>
       </c>
       <c r="U17" t="n">
-        <v>-2.5988</v>
+        <v>3.0416</v>
       </c>
       <c r="V17" t="n">
-        <v>5.0743</v>
+        <v>1.2585</v>
       </c>
       <c r="W17" t="n">
-        <v>11.2331</v>
+        <v>7.9223</v>
       </c>
       <c r="X17" t="n">
-        <v>9.1463</v>
+        <v>-6.7039</v>
       </c>
       <c r="Y17" t="n">
-        <v>-15.566</v>
+        <v>-5.6497</v>
       </c>
       <c r="Z17" t="n">
-        <v>-22.2415</v>
+        <v>-14.8828</v>
       </c>
       <c r="AA17" t="n">
-        <v>2.5817</v>
+        <v>-3.0478</v>
       </c>
       <c r="AB17" t="n">
-        <v>-5.2919</v>
+        <v>-1.3625</v>
       </c>
       <c r="AC17" t="n">
-        <v>-10.8664</v>
+        <v>-7.8965</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>183.84</v>
+        <v>182.67</v>
       </c>
       <c r="C18" t="n">
-        <v>188.49</v>
+        <v>189.56</v>
       </c>
       <c r="D18" t="n">
-        <v>172.26</v>
+        <v>178.28</v>
       </c>
       <c r="E18" t="n">
-        <v>184.24</v>
+        <v>186.19</v>
       </c>
       <c r="F18" t="n">
-        <v>75.81</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>77.94</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H18" t="n">
-        <v>74.19</v>
+        <v>77.16</v>
       </c>
       <c r="I18" t="n">
-        <v>77.23999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="J18" t="n">
-        <v>8.380000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="K18" t="n">
-        <v>8.98</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L18" t="n">
-        <v>8.140000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M18" t="n">
-        <v>8.35</v>
+        <v>8.27</v>
       </c>
       <c r="N18" t="n">
-        <v>42.83</v>
+        <v>41.98</v>
       </c>
       <c r="O18" t="n">
-        <v>43.77</v>
+        <v>42.06</v>
       </c>
       <c r="P18" t="n">
-        <v>41.6</v>
+        <v>40.68</v>
       </c>
       <c r="Q18" t="n">
-        <v>41.99</v>
+        <v>41.07</v>
       </c>
       <c r="R18" t="n">
-        <v>6.7934</v>
+        <v>1.0584</v>
       </c>
       <c r="S18" t="n">
-        <v>4.1257</v>
+        <v>-2.2214</v>
       </c>
       <c r="T18" t="n">
-        <v>11.0883</v>
+        <v>22.4129</v>
       </c>
       <c r="U18" t="n">
-        <v>3.0416</v>
+        <v>2.2139</v>
       </c>
       <c r="V18" t="n">
-        <v>1.2585</v>
+        <v>2.5858</v>
       </c>
       <c r="W18" t="n">
-        <v>7.9223</v>
+        <v>10.6672</v>
       </c>
       <c r="X18" t="n">
-        <v>-6.7039</v>
+        <v>-0.9581</v>
       </c>
       <c r="Y18" t="n">
-        <v>-5.6497</v>
+        <v>0.8537</v>
       </c>
       <c r="Z18" t="n">
-        <v>-14.8828</v>
+        <v>-21.9811</v>
       </c>
       <c r="AA18" t="n">
-        <v>-3.0478</v>
+        <v>-2.191</v>
       </c>
       <c r="AB18" t="n">
-        <v>-1.3625</v>
+        <v>-2.7238</v>
       </c>
       <c r="AC18" t="n">
-        <v>-7.8965</v>
+        <v>-10.1902</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>182.67</v>
+        <v>167</v>
       </c>
       <c r="C19" t="n">
-        <v>189.56</v>
+        <v>174.4</v>
       </c>
       <c r="D19" t="n">
-        <v>178.28</v>
+        <v>161.14</v>
       </c>
       <c r="E19" t="n">
-        <v>186.19</v>
+        <v>164.18</v>
       </c>
       <c r="F19" t="n">
-        <v>77.29000000000001</v>
+        <v>75.73</v>
       </c>
       <c r="G19" t="n">
-        <v>79.68000000000001</v>
+        <v>77.37</v>
       </c>
       <c r="H19" t="n">
-        <v>77.16</v>
+        <v>74.23</v>
       </c>
       <c r="I19" t="n">
-        <v>78.95</v>
+        <v>75.34</v>
       </c>
       <c r="J19" t="n">
-        <v>8.43</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="K19" t="n">
-        <v>8.630000000000001</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="L19" t="n">
-        <v>8.119999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M19" t="n">
-        <v>8.27</v>
+        <v>9.23</v>
       </c>
       <c r="N19" t="n">
-        <v>41.98</v>
+        <v>42.77</v>
       </c>
       <c r="O19" t="n">
-        <v>42.06</v>
+        <v>43.57</v>
       </c>
       <c r="P19" t="n">
-        <v>40.68</v>
+        <v>41.93</v>
       </c>
       <c r="Q19" t="n">
-        <v>41.07</v>
+        <v>42.98</v>
       </c>
       <c r="R19" t="n">
-        <v>1.0584</v>
+        <v>-11.8213</v>
       </c>
       <c r="S19" t="n">
-        <v>-2.2214</v>
+        <v>-4.8342</v>
       </c>
       <c r="T19" t="n">
-        <v>22.4129</v>
+        <v>-7.2115</v>
       </c>
       <c r="U19" t="n">
-        <v>2.2139</v>
+        <v>-4.5725</v>
       </c>
       <c r="V19" t="n">
-        <v>2.5858</v>
+        <v>0.5069</v>
       </c>
       <c r="W19" t="n">
-        <v>10.6672</v>
+        <v>-1.2323</v>
       </c>
       <c r="X19" t="n">
-        <v>-0.9581</v>
+        <v>11.6082</v>
       </c>
       <c r="Y19" t="n">
-        <v>0.8537</v>
+        <v>3.1285</v>
       </c>
       <c r="Z19" t="n">
-        <v>-21.9811</v>
+        <v>4.2938</v>
       </c>
       <c r="AA19" t="n">
-        <v>-2.191</v>
+        <v>4.6506</v>
       </c>
       <c r="AB19" t="n">
-        <v>-2.7238</v>
+        <v>-0.7619</v>
       </c>
       <c r="AC19" t="n">
-        <v>-10.1902</v>
+        <v>0.9631</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>167</v>
+        <v>172.95</v>
       </c>
       <c r="C20" t="n">
-        <v>174.4</v>
+        <v>174.61</v>
       </c>
       <c r="D20" t="n">
-        <v>161.14</v>
+        <v>142.69</v>
       </c>
       <c r="E20" t="n">
-        <v>164.18</v>
+        <v>151.75</v>
       </c>
       <c r="F20" t="n">
-        <v>75.73</v>
+        <v>76.13</v>
       </c>
       <c r="G20" t="n">
-        <v>77.37</v>
+        <v>76.27</v>
       </c>
       <c r="H20" t="n">
-        <v>74.23</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>75.34</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="J20" t="n">
-        <v>9.130000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="K20" t="n">
-        <v>9.390000000000001</v>
+        <v>10.47</v>
       </c>
       <c r="L20" t="n">
-        <v>8.800000000000001</v>
+        <v>8.68</v>
       </c>
       <c r="M20" t="n">
-        <v>9.23</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="N20" t="n">
-        <v>42.77</v>
+        <v>42.51</v>
       </c>
       <c r="O20" t="n">
-        <v>43.57</v>
+        <v>44.82</v>
       </c>
       <c r="P20" t="n">
-        <v>41.93</v>
+        <v>42.44</v>
       </c>
       <c r="Q20" t="n">
-        <v>42.98</v>
+        <v>43.54</v>
       </c>
       <c r="R20" t="n">
-        <v>-11.8213</v>
+        <v>-7.571</v>
       </c>
       <c r="S20" t="n">
-        <v>-4.8342</v>
+        <v>-17.6346</v>
       </c>
       <c r="T20" t="n">
-        <v>-7.2115</v>
+        <v>-20.3077</v>
       </c>
       <c r="U20" t="n">
-        <v>-4.5725</v>
+        <v>-1.3539</v>
       </c>
       <c r="V20" t="n">
-        <v>0.5069</v>
+        <v>-3.7804</v>
       </c>
       <c r="W20" t="n">
-        <v>-1.2323</v>
+        <v>-3.4304</v>
       </c>
       <c r="X20" t="n">
-        <v>11.6082</v>
+        <v>7.8007</v>
       </c>
       <c r="Y20" t="n">
-        <v>3.1285</v>
+        <v>19.1617</v>
       </c>
       <c r="Z20" t="n">
-        <v>4.2938</v>
+        <v>21.3415</v>
       </c>
       <c r="AA20" t="n">
-        <v>4.6506</v>
+        <v>1.3029</v>
       </c>
       <c r="AB20" t="n">
-        <v>-0.7619</v>
+        <v>3.6914</v>
       </c>
       <c r="AC20" t="n">
-        <v>0.9631</v>
+        <v>3.1265</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>172.95</v>
+        <v>141.24</v>
       </c>
       <c r="C21" t="n">
-        <v>174.61</v>
+        <v>160.6</v>
       </c>
       <c r="D21" t="n">
-        <v>142.69</v>
+        <v>135.02</v>
       </c>
       <c r="E21" t="n">
-        <v>151.75</v>
+        <v>151.89</v>
       </c>
       <c r="F21" t="n">
-        <v>76.13</v>
+        <v>72.41</v>
       </c>
       <c r="G21" t="n">
-        <v>76.27</v>
+        <v>74.5</v>
       </c>
       <c r="H21" t="n">
-        <v>72.09999999999999</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="I21" t="n">
-        <v>74.31999999999999</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>8.77</v>
+        <v>10.64</v>
       </c>
       <c r="K21" t="n">
-        <v>10.47</v>
+        <v>11.07</v>
       </c>
       <c r="L21" t="n">
-        <v>8.68</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="M21" t="n">
-        <v>9.949999999999999</v>
+        <v>9.93</v>
       </c>
       <c r="N21" t="n">
-        <v>42.51</v>
+        <v>44.68</v>
       </c>
       <c r="O21" t="n">
-        <v>44.82</v>
+        <v>45.53</v>
       </c>
       <c r="P21" t="n">
-        <v>42.44</v>
+        <v>43.46</v>
       </c>
       <c r="Q21" t="n">
-        <v>43.54</v>
+        <v>44.37</v>
       </c>
       <c r="R21" t="n">
-        <v>-7.571</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="S21" t="n">
-        <v>-17.6346</v>
+        <v>-18.422</v>
       </c>
       <c r="T21" t="n">
-        <v>-20.3077</v>
+        <v>-11.958</v>
       </c>
       <c r="U21" t="n">
-        <v>-1.3539</v>
+        <v>-1.8703</v>
       </c>
       <c r="V21" t="n">
-        <v>-3.7804</v>
+        <v>-7.6251</v>
       </c>
       <c r="W21" t="n">
-        <v>-3.4304</v>
+        <v>-2.7081</v>
       </c>
       <c r="X21" t="n">
-        <v>7.8007</v>
+        <v>-0.201</v>
       </c>
       <c r="Y21" t="n">
-        <v>19.1617</v>
+        <v>20.0726</v>
       </c>
       <c r="Z21" t="n">
-        <v>21.3415</v>
+        <v>10.9497</v>
       </c>
       <c r="AA21" t="n">
-        <v>1.3029</v>
+        <v>1.9063</v>
       </c>
       <c r="AB21" t="n">
-        <v>3.6914</v>
+        <v>8.0351</v>
       </c>
       <c r="AC21" t="n">
-        <v>3.1265</v>
+        <v>2.4475</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>141.24</v>
+        <v>161</v>
       </c>
       <c r="C22" t="n">
-        <v>160.6</v>
+        <v>173.7</v>
       </c>
       <c r="D22" t="n">
-        <v>135.02</v>
+        <v>161</v>
       </c>
       <c r="E22" t="n">
-        <v>151.89</v>
+        <v>173.2</v>
       </c>
       <c r="F22" t="n">
-        <v>72.41</v>
+        <v>74.09</v>
       </c>
       <c r="G22" t="n">
-        <v>74.5</v>
+        <v>76.53</v>
       </c>
       <c r="H22" t="n">
-        <v>70.95999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="I22" t="n">
-        <v>72.93000000000001</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J22" t="n">
-        <v>10.64</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K22" t="n">
-        <v>11.07</v>
+        <v>9.35</v>
       </c>
       <c r="L22" t="n">
-        <v>9.369999999999999</v>
+        <v>8.51</v>
       </c>
       <c r="M22" t="n">
-        <v>9.93</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N22" t="n">
-        <v>44.68</v>
+        <v>43.67</v>
       </c>
       <c r="O22" t="n">
-        <v>45.53</v>
+        <v>43.97</v>
       </c>
       <c r="P22" t="n">
-        <v>43.46</v>
+        <v>42.19</v>
       </c>
       <c r="Q22" t="n">
-        <v>44.37</v>
+        <v>42.19</v>
       </c>
       <c r="R22" t="n">
-        <v>0.09229999999999999</v>
+        <v>14.0299</v>
       </c>
       <c r="S22" t="n">
-        <v>-18.422</v>
+        <v>5.494</v>
       </c>
       <c r="T22" t="n">
-        <v>-11.958</v>
+        <v>-5.9922</v>
       </c>
       <c r="U22" t="n">
-        <v>-1.8703</v>
+        <v>4.9088</v>
       </c>
       <c r="V22" t="n">
-        <v>-7.6251</v>
+        <v>1.553</v>
       </c>
       <c r="W22" t="n">
-        <v>-2.7081</v>
+        <v>-0.9451000000000001</v>
       </c>
       <c r="X22" t="n">
-        <v>-0.201</v>
+        <v>-13.998</v>
       </c>
       <c r="Y22" t="n">
-        <v>20.0726</v>
+        <v>-7.4756</v>
       </c>
       <c r="Z22" t="n">
-        <v>10.9497</v>
+        <v>2.2754</v>
       </c>
       <c r="AA22" t="n">
-        <v>1.9063</v>
+        <v>-4.9132</v>
       </c>
       <c r="AB22" t="n">
-        <v>8.0351</v>
+        <v>-1.8381</v>
       </c>
       <c r="AC22" t="n">
-        <v>2.4475</v>
+        <v>0.4763</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>161</v>
+        <v>171.26</v>
       </c>
       <c r="C23" t="n">
-        <v>173.69</v>
+        <v>179.97</v>
       </c>
       <c r="D23" t="n">
-        <v>161.04</v>
+        <v>168.2501</v>
       </c>
       <c r="E23" t="n">
-        <v>173.2</v>
+        <v>178.39</v>
       </c>
       <c r="F23" t="n">
-        <v>74.084</v>
+        <v>75.19</v>
       </c>
       <c r="G23" t="n">
-        <v>76.53</v>
+        <v>77.7895</v>
       </c>
       <c r="H23" t="n">
-        <v>73.61499999999999</v>
+        <v>74.471</v>
       </c>
       <c r="I23" t="n">
-        <v>76.51000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J23" t="n">
-        <v>9.300000000000001</v>
+        <v>8.645</v>
       </c>
       <c r="K23" t="n">
-        <v>9.35</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L23" t="n">
-        <v>8.51</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M23" t="n">
-        <v>8.539999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N23" t="n">
-        <v>43.675</v>
+        <v>42.97</v>
       </c>
       <c r="O23" t="n">
-        <v>43.965</v>
+        <v>43.3305</v>
       </c>
       <c r="P23" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="Q23" t="n">
-        <v>42.19</v>
+        <v>41.96</v>
       </c>
       <c r="R23" t="n">
-        <v>14.0299</v>
+        <v>2.9965</v>
       </c>
       <c r="S23" t="n">
-        <v>5.494</v>
+        <v>17.5552</v>
       </c>
       <c r="T23" t="n">
-        <v>-5.9922</v>
+        <v>-4.1893</v>
       </c>
       <c r="U23" t="n">
-        <v>4.9088</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="V23" t="n">
-        <v>1.553</v>
+        <v>3.5388</v>
       </c>
       <c r="W23" t="n">
-        <v>-0.9451000000000001</v>
+        <v>-2.5332</v>
       </c>
       <c r="X23" t="n">
-        <v>-13.998</v>
+        <v>-2.9274</v>
       </c>
       <c r="Y23" t="n">
-        <v>-7.4756</v>
+        <v>-16.6834</v>
       </c>
       <c r="Z23" t="n">
-        <v>2.2754</v>
+        <v>0.2418</v>
       </c>
       <c r="AA23" t="n">
-        <v>-4.9132</v>
+        <v>-0.5452</v>
       </c>
       <c r="AB23" t="n">
-        <v>-1.8381</v>
+        <v>-3.6288</v>
       </c>
       <c r="AC23" t="n">
-        <v>0.4763</v>
+        <v>2.167</v>
       </c>
     </row>
   </sheetData>
@@ -2503,7 +2503,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-05-22 22:59
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1895 +568,1895 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>102.94</v>
+        <v>108.62</v>
       </c>
       <c r="C2" t="n">
-        <v>106.09</v>
+        <v>116.77</v>
       </c>
       <c r="D2" t="n">
-        <v>99.59999999999999</v>
+        <v>107.46</v>
       </c>
       <c r="E2" t="n">
-        <v>105.64</v>
+        <v>112.77</v>
       </c>
       <c r="F2" t="n">
-        <v>58.93</v>
+        <v>59.8</v>
       </c>
       <c r="G2" t="n">
-        <v>60.3</v>
+        <v>60.73</v>
       </c>
       <c r="H2" t="n">
-        <v>58.49</v>
+        <v>57.59</v>
       </c>
       <c r="I2" t="n">
-        <v>60.21</v>
+        <v>59.22</v>
       </c>
       <c r="J2" t="n">
-        <v>17.37</v>
+        <v>16.35</v>
       </c>
       <c r="K2" t="n">
-        <v>17.95</v>
+        <v>16.52</v>
       </c>
       <c r="L2" t="n">
-        <v>16.72</v>
+        <v>15.06</v>
       </c>
       <c r="M2" t="n">
-        <v>16.8</v>
+        <v>15.7</v>
       </c>
       <c r="N2" t="n">
-        <v>56.05</v>
+        <v>55.13</v>
       </c>
       <c r="O2" t="n">
-        <v>56.49</v>
+        <v>57.14</v>
       </c>
       <c r="P2" t="n">
-        <v>54.66</v>
+        <v>54.28</v>
       </c>
       <c r="Q2" t="n">
-        <v>54.73</v>
+        <v>55.66</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>108.62</v>
+        <v>125.21</v>
       </c>
       <c r="C3" t="n">
-        <v>116.77</v>
+        <v>130.12</v>
       </c>
       <c r="D3" t="n">
-        <v>107.46</v>
+        <v>120.24</v>
       </c>
       <c r="E3" t="n">
-        <v>112.77</v>
+        <v>128.32</v>
       </c>
       <c r="F3" t="n">
-        <v>59.8</v>
+        <v>61.08</v>
       </c>
       <c r="G3" t="n">
-        <v>60.73</v>
+        <v>62.74</v>
       </c>
       <c r="H3" t="n">
-        <v>57.59</v>
+        <v>60.56</v>
       </c>
       <c r="I3" t="n">
-        <v>59.22</v>
+        <v>62.56</v>
       </c>
       <c r="J3" t="n">
-        <v>16.35</v>
+        <v>13.99</v>
       </c>
       <c r="K3" t="n">
-        <v>16.52</v>
+        <v>14.66</v>
       </c>
       <c r="L3" t="n">
-        <v>15.06</v>
+        <v>13.3</v>
       </c>
       <c r="M3" t="n">
-        <v>15.7</v>
+        <v>13.52</v>
       </c>
       <c r="N3" t="n">
-        <v>55.13</v>
+        <v>53.93</v>
       </c>
       <c r="O3" t="n">
-        <v>57.14</v>
+        <v>54.43</v>
       </c>
       <c r="P3" t="n">
-        <v>54.28</v>
+        <v>52.37</v>
       </c>
       <c r="Q3" t="n">
-        <v>55.66</v>
+        <v>52.5</v>
       </c>
       <c r="R3" t="n">
-        <v>6.7493</v>
+        <v>13.7891</v>
       </c>
       <c r="U3" t="n">
-        <v>-1.6442</v>
+        <v>5.64</v>
       </c>
       <c r="X3" t="n">
-        <v>-6.5476</v>
+        <v>-13.8854</v>
       </c>
       <c r="AA3" t="n">
-        <v>1.6993</v>
+        <v>-5.6773</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>125.21</v>
+        <v>128.33</v>
       </c>
       <c r="C4" t="n">
-        <v>130.12</v>
+        <v>129.59</v>
       </c>
       <c r="D4" t="n">
-        <v>120.24</v>
+        <v>117.79</v>
       </c>
       <c r="E4" t="n">
-        <v>128.32</v>
+        <v>123.39</v>
       </c>
       <c r="F4" t="n">
-        <v>61.08</v>
+        <v>62.41</v>
       </c>
       <c r="G4" t="n">
-        <v>62.74</v>
+        <v>62.7</v>
       </c>
       <c r="H4" t="n">
-        <v>60.56</v>
+        <v>61.64</v>
       </c>
       <c r="I4" t="n">
-        <v>62.56</v>
+        <v>62.64</v>
       </c>
       <c r="J4" t="n">
-        <v>13.99</v>
+        <v>13.51</v>
       </c>
       <c r="K4" t="n">
-        <v>14.66</v>
+        <v>14.63</v>
       </c>
       <c r="L4" t="n">
-        <v>13.3</v>
+        <v>13.41</v>
       </c>
       <c r="M4" t="n">
-        <v>13.52</v>
+        <v>14.03</v>
       </c>
       <c r="N4" t="n">
-        <v>53.93</v>
+        <v>52.67</v>
       </c>
       <c r="O4" t="n">
-        <v>54.43</v>
+        <v>53.31</v>
       </c>
       <c r="P4" t="n">
-        <v>52.37</v>
+        <v>52.42</v>
       </c>
       <c r="Q4" t="n">
-        <v>52.5</v>
+        <v>52.45</v>
       </c>
       <c r="R4" t="n">
-        <v>13.7891</v>
+        <v>-3.842</v>
       </c>
       <c r="U4" t="n">
-        <v>5.64</v>
+        <v>0.1279</v>
       </c>
       <c r="X4" t="n">
-        <v>-13.8854</v>
+        <v>3.7722</v>
       </c>
       <c r="AA4" t="n">
-        <v>-5.6773</v>
+        <v>-0.09520000000000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>128.33</v>
+        <v>108.75</v>
       </c>
       <c r="C5" t="n">
-        <v>129.59</v>
+        <v>115.62</v>
       </c>
       <c r="D5" t="n">
-        <v>117.79</v>
+        <v>103.99</v>
       </c>
       <c r="E5" t="n">
-        <v>123.39</v>
+        <v>109.56</v>
       </c>
       <c r="F5" t="n">
-        <v>62.41</v>
+        <v>60.72</v>
       </c>
       <c r="G5" t="n">
-        <v>62.7</v>
+        <v>61.33</v>
       </c>
       <c r="H5" t="n">
-        <v>61.64</v>
+        <v>59.68</v>
       </c>
       <c r="I5" t="n">
-        <v>62.64</v>
+        <v>60.74</v>
       </c>
       <c r="J5" t="n">
-        <v>13.51</v>
+        <v>15.71</v>
       </c>
       <c r="K5" t="n">
-        <v>14.63</v>
+        <v>16.27</v>
       </c>
       <c r="L5" t="n">
-        <v>13.41</v>
+        <v>14.93</v>
       </c>
       <c r="M5" t="n">
-        <v>14.03</v>
+        <v>15.59</v>
       </c>
       <c r="N5" t="n">
-        <v>52.67</v>
+        <v>54.09</v>
       </c>
       <c r="O5" t="n">
-        <v>53.31</v>
+        <v>54.96</v>
       </c>
       <c r="P5" t="n">
-        <v>52.42</v>
+        <v>53.58</v>
       </c>
       <c r="Q5" t="n">
-        <v>52.45</v>
+        <v>54.05</v>
       </c>
       <c r="R5" t="n">
-        <v>-3.842</v>
+        <v>-11.2084</v>
       </c>
       <c r="S5" t="n">
-        <v>16.8023</v>
+        <v>-2.8465</v>
       </c>
       <c r="U5" t="n">
-        <v>0.1279</v>
+        <v>-3.0332</v>
       </c>
       <c r="V5" t="n">
-        <v>4.0359</v>
+        <v>2.5667</v>
       </c>
       <c r="X5" t="n">
-        <v>3.7722</v>
+        <v>11.119</v>
       </c>
       <c r="Y5" t="n">
-        <v>-16.4881</v>
+        <v>-0.7006</v>
       </c>
       <c r="AA5" t="n">
-        <v>-0.09520000000000001</v>
+        <v>3.0505</v>
       </c>
       <c r="AB5" t="n">
-        <v>-4.1659</v>
+        <v>-2.8926</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>108.75</v>
+        <v>114.76</v>
       </c>
       <c r="C6" t="n">
-        <v>115.62</v>
+        <v>118.32</v>
       </c>
       <c r="D6" t="n">
-        <v>103.99</v>
+        <v>112.3</v>
       </c>
       <c r="E6" t="n">
-        <v>109.56</v>
+        <v>117.97</v>
       </c>
       <c r="F6" t="n">
-        <v>60.72</v>
+        <v>61</v>
       </c>
       <c r="G6" t="n">
-        <v>61.33</v>
+        <v>61.87</v>
       </c>
       <c r="H6" t="n">
-        <v>59.68</v>
+        <v>60.45</v>
       </c>
       <c r="I6" t="n">
-        <v>60.74</v>
+        <v>61.86</v>
       </c>
       <c r="J6" t="n">
-        <v>15.71</v>
+        <v>14.91</v>
       </c>
       <c r="K6" t="n">
-        <v>16.27</v>
+        <v>15.24</v>
       </c>
       <c r="L6" t="n">
-        <v>14.93</v>
+        <v>14.38</v>
       </c>
       <c r="M6" t="n">
-        <v>15.59</v>
+        <v>14.4</v>
       </c>
       <c r="N6" t="n">
-        <v>54.09</v>
+        <v>53.84</v>
       </c>
       <c r="O6" t="n">
-        <v>54.96</v>
+        <v>54.33</v>
       </c>
       <c r="P6" t="n">
-        <v>53.58</v>
+        <v>53.06</v>
       </c>
       <c r="Q6" t="n">
-        <v>54.05</v>
+        <v>53.08</v>
       </c>
       <c r="R6" t="n">
-        <v>-11.2084</v>
+        <v>7.6762</v>
       </c>
       <c r="S6" t="n">
-        <v>-2.8465</v>
+        <v>-8.065799999999999</v>
       </c>
       <c r="U6" t="n">
-        <v>-3.0332</v>
+        <v>1.8439</v>
       </c>
       <c r="V6" t="n">
-        <v>2.5667</v>
+        <v>-1.1189</v>
       </c>
       <c r="X6" t="n">
-        <v>11.119</v>
+        <v>-7.6331</v>
       </c>
       <c r="Y6" t="n">
-        <v>-0.7006</v>
+        <v>6.5089</v>
       </c>
       <c r="AA6" t="n">
-        <v>3.0505</v>
+        <v>-1.7946</v>
       </c>
       <c r="AB6" t="n">
-        <v>-2.8926</v>
+        <v>1.1048</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>114.76</v>
+        <v>122.81</v>
       </c>
       <c r="C7" t="n">
-        <v>118.32</v>
+        <v>127.45</v>
       </c>
       <c r="D7" t="n">
-        <v>112.3</v>
+        <v>117.5</v>
       </c>
       <c r="E7" t="n">
-        <v>117.97</v>
+        <v>126.98</v>
       </c>
       <c r="F7" t="n">
-        <v>61</v>
+        <v>62.89</v>
       </c>
       <c r="G7" t="n">
-        <v>61.87</v>
+        <v>63.8</v>
       </c>
       <c r="H7" t="n">
-        <v>60.45</v>
+        <v>60.7</v>
       </c>
       <c r="I7" t="n">
-        <v>61.86</v>
+        <v>63.54</v>
       </c>
       <c r="J7" t="n">
-        <v>14.91</v>
+        <v>13.84</v>
       </c>
       <c r="K7" t="n">
-        <v>15.24</v>
+        <v>14.49</v>
       </c>
       <c r="L7" t="n">
-        <v>14.38</v>
+        <v>13.25</v>
       </c>
       <c r="M7" t="n">
-        <v>14.4</v>
+        <v>13.3</v>
       </c>
       <c r="N7" t="n">
-        <v>53.84</v>
+        <v>52.21</v>
       </c>
       <c r="O7" t="n">
-        <v>54.33</v>
+        <v>54.09</v>
       </c>
       <c r="P7" t="n">
-        <v>53.06</v>
+        <v>51.4</v>
       </c>
       <c r="Q7" t="n">
-        <v>53.08</v>
+        <v>51.65</v>
       </c>
       <c r="R7" t="n">
-        <v>7.6762</v>
+        <v>7.6375</v>
       </c>
       <c r="S7" t="n">
-        <v>-8.065799999999999</v>
+        <v>2.9095</v>
       </c>
       <c r="T7" t="n">
-        <v>11.6717</v>
+        <v>12.6009</v>
       </c>
       <c r="U7" t="n">
-        <v>1.8439</v>
+        <v>2.7158</v>
       </c>
       <c r="V7" t="n">
-        <v>-1.1189</v>
+        <v>1.4368</v>
       </c>
       <c r="W7" t="n">
-        <v>2.7404</v>
+        <v>7.2948</v>
       </c>
       <c r="X7" t="n">
-        <v>-7.6331</v>
+        <v>-7.6389</v>
       </c>
       <c r="Y7" t="n">
-        <v>6.5089</v>
+        <v>-5.2031</v>
       </c>
       <c r="Z7" t="n">
-        <v>-14.2857</v>
+        <v>-15.2866</v>
       </c>
       <c r="AA7" t="n">
-        <v>-1.7946</v>
+        <v>-2.694</v>
       </c>
       <c r="AB7" t="n">
-        <v>1.1048</v>
+        <v>-1.5253</v>
       </c>
       <c r="AC7" t="n">
-        <v>-3.0148</v>
+        <v>-7.2045</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>122.81</v>
+        <v>124.39</v>
       </c>
       <c r="C8" t="n">
-        <v>127.45</v>
+        <v>131.38</v>
       </c>
       <c r="D8" t="n">
-        <v>117.5</v>
+        <v>121.66</v>
       </c>
       <c r="E8" t="n">
-        <v>126.98</v>
+        <v>130.4</v>
       </c>
       <c r="F8" t="n">
-        <v>62.89</v>
+        <v>63.89</v>
       </c>
       <c r="G8" t="n">
-        <v>63.8</v>
+        <v>65.84</v>
       </c>
       <c r="H8" t="n">
-        <v>60.7</v>
+        <v>63.81</v>
       </c>
       <c r="I8" t="n">
-        <v>63.54</v>
+        <v>65.3</v>
       </c>
       <c r="J8" t="n">
-        <v>13.84</v>
+        <v>13.61</v>
       </c>
       <c r="K8" t="n">
-        <v>14.49</v>
+        <v>13.89</v>
       </c>
       <c r="L8" t="n">
-        <v>13.25</v>
+        <v>12.87</v>
       </c>
       <c r="M8" t="n">
-        <v>13.3</v>
+        <v>12.98</v>
       </c>
       <c r="N8" t="n">
-        <v>52.21</v>
+        <v>51.36</v>
       </c>
       <c r="O8" t="n">
-        <v>54.09</v>
+        <v>51.45</v>
       </c>
       <c r="P8" t="n">
-        <v>51.4</v>
+        <v>49.79</v>
       </c>
       <c r="Q8" t="n">
-        <v>51.65</v>
+        <v>50.22</v>
       </c>
       <c r="R8" t="n">
-        <v>7.6375</v>
+        <v>2.6933</v>
       </c>
       <c r="S8" t="n">
-        <v>2.9095</v>
+        <v>19.0215</v>
       </c>
       <c r="T8" t="n">
-        <v>12.6009</v>
+        <v>1.6209</v>
       </c>
       <c r="U8" t="n">
-        <v>2.7158</v>
+        <v>2.7699</v>
       </c>
       <c r="V8" t="n">
-        <v>1.4368</v>
+        <v>7.5074</v>
       </c>
       <c r="W8" t="n">
-        <v>7.2948</v>
+        <v>4.3798</v>
       </c>
       <c r="X8" t="n">
-        <v>-7.6389</v>
+        <v>-2.406</v>
       </c>
       <c r="Y8" t="n">
-        <v>-5.2031</v>
+        <v>-16.7415</v>
       </c>
       <c r="Z8" t="n">
-        <v>-15.2866</v>
+        <v>-3.9941</v>
       </c>
       <c r="AA8" t="n">
-        <v>-2.694</v>
+        <v>-2.7686</v>
       </c>
       <c r="AB8" t="n">
-        <v>-1.5253</v>
+        <v>-7.086</v>
       </c>
       <c r="AC8" t="n">
-        <v>-7.2045</v>
+        <v>-4.3429</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>124.39</v>
+        <v>132.2</v>
       </c>
       <c r="C9" t="n">
-        <v>131.38</v>
+        <v>133.67</v>
       </c>
       <c r="D9" t="n">
-        <v>121.66</v>
+        <v>123.8</v>
       </c>
       <c r="E9" t="n">
-        <v>130.4</v>
+        <v>127.55</v>
       </c>
       <c r="F9" t="n">
-        <v>63.89</v>
+        <v>65.44</v>
       </c>
       <c r="G9" t="n">
-        <v>65.84</v>
+        <v>66.05</v>
       </c>
       <c r="H9" t="n">
-        <v>63.81</v>
+        <v>63.78</v>
       </c>
       <c r="I9" t="n">
-        <v>65.3</v>
+        <v>64.91</v>
       </c>
       <c r="J9" t="n">
-        <v>13.61</v>
+        <v>12.8</v>
       </c>
       <c r="K9" t="n">
-        <v>13.89</v>
+        <v>13.64</v>
       </c>
       <c r="L9" t="n">
-        <v>12.87</v>
+        <v>12.65</v>
       </c>
       <c r="M9" t="n">
-        <v>12.98</v>
+        <v>13.26</v>
       </c>
       <c r="N9" t="n">
-        <v>51.36</v>
+        <v>50.12</v>
       </c>
       <c r="O9" t="n">
-        <v>51.45</v>
+        <v>51.43</v>
       </c>
       <c r="P9" t="n">
-        <v>49.79</v>
+        <v>49.65</v>
       </c>
       <c r="Q9" t="n">
-        <v>50.22</v>
+        <v>50.51</v>
       </c>
       <c r="R9" t="n">
-        <v>2.6933</v>
+        <v>-2.1856</v>
       </c>
       <c r="S9" t="n">
-        <v>19.0215</v>
+        <v>8.120699999999999</v>
       </c>
       <c r="T9" t="n">
-        <v>1.6209</v>
+        <v>3.3714</v>
       </c>
       <c r="U9" t="n">
-        <v>2.7699</v>
+        <v>-0.5972</v>
       </c>
       <c r="V9" t="n">
-        <v>7.5074</v>
+        <v>4.9305</v>
       </c>
       <c r="W9" t="n">
-        <v>4.3798</v>
+        <v>3.6239</v>
       </c>
       <c r="X9" t="n">
-        <v>-2.406</v>
+        <v>2.1572</v>
       </c>
       <c r="Y9" t="n">
-        <v>-16.7415</v>
+        <v>-7.9167</v>
       </c>
       <c r="Z9" t="n">
-        <v>-3.9941</v>
+        <v>-5.4882</v>
       </c>
       <c r="AA9" t="n">
-        <v>-2.7686</v>
+        <v>0.5775</v>
       </c>
       <c r="AB9" t="n">
-        <v>-7.086</v>
+        <v>-4.8417</v>
       </c>
       <c r="AC9" t="n">
-        <v>-4.3429</v>
+        <v>-3.6988</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>132.2</v>
+        <v>135</v>
       </c>
       <c r="C10" t="n">
-        <v>133.67</v>
+        <v>147.26</v>
       </c>
       <c r="D10" t="n">
-        <v>123.8</v>
+        <v>134.02</v>
       </c>
       <c r="E10" t="n">
-        <v>127.55</v>
+        <v>144.16</v>
       </c>
       <c r="F10" t="n">
-        <v>65.44</v>
+        <v>66.37</v>
       </c>
       <c r="G10" t="n">
-        <v>66.05</v>
+        <v>67.77</v>
       </c>
       <c r="H10" t="n">
-        <v>63.78</v>
+        <v>66.25</v>
       </c>
       <c r="I10" t="n">
-        <v>64.91</v>
+        <v>67.39</v>
       </c>
       <c r="J10" t="n">
-        <v>12.8</v>
+        <v>12.5</v>
       </c>
       <c r="K10" t="n">
-        <v>13.64</v>
+        <v>12.59</v>
       </c>
       <c r="L10" t="n">
-        <v>12.65</v>
+        <v>11.21</v>
       </c>
       <c r="M10" t="n">
-        <v>13.26</v>
+        <v>11.51</v>
       </c>
       <c r="N10" t="n">
-        <v>50.12</v>
+        <v>49.4</v>
       </c>
       <c r="O10" t="n">
-        <v>51.43</v>
+        <v>49.49</v>
       </c>
       <c r="P10" t="n">
-        <v>49.65</v>
+        <v>48.3</v>
       </c>
       <c r="Q10" t="n">
-        <v>50.51</v>
+        <v>48.59</v>
       </c>
       <c r="R10" t="n">
-        <v>-2.1856</v>
+        <v>13.0223</v>
       </c>
       <c r="S10" t="n">
-        <v>8.120699999999999</v>
+        <v>13.5297</v>
       </c>
       <c r="T10" t="n">
-        <v>3.3714</v>
+        <v>31.5809</v>
       </c>
       <c r="U10" t="n">
-        <v>-0.5972</v>
+        <v>3.8207</v>
       </c>
       <c r="V10" t="n">
-        <v>4.9305</v>
+        <v>6.0592</v>
       </c>
       <c r="W10" t="n">
-        <v>3.6239</v>
+        <v>10.9483</v>
       </c>
       <c r="X10" t="n">
-        <v>2.1572</v>
+        <v>-13.1976</v>
       </c>
       <c r="Y10" t="n">
-        <v>-7.9167</v>
+        <v>-13.4586</v>
       </c>
       <c r="Z10" t="n">
-        <v>-5.4882</v>
+        <v>-26.1706</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.5775</v>
+        <v>-3.8012</v>
       </c>
       <c r="AB10" t="n">
-        <v>-4.8417</v>
+        <v>-5.9245</v>
       </c>
       <c r="AC10" t="n">
-        <v>-3.6988</v>
+        <v>-10.1018</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>135</v>
+        <v>157.84</v>
       </c>
       <c r="C11" t="n">
-        <v>147.26</v>
+        <v>166</v>
       </c>
       <c r="D11" t="n">
-        <v>134.02</v>
+        <v>149.06</v>
       </c>
       <c r="E11" t="n">
-        <v>144.16</v>
+        <v>165.85</v>
       </c>
       <c r="F11" t="n">
-        <v>66.37</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>67.77</v>
+        <v>71.66</v>
       </c>
       <c r="H11" t="n">
-        <v>66.25</v>
+        <v>68.88</v>
       </c>
       <c r="I11" t="n">
-        <v>67.39</v>
+        <v>71.56999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>12.5</v>
+        <v>10.43</v>
       </c>
       <c r="K11" t="n">
-        <v>12.59</v>
+        <v>11.14</v>
       </c>
       <c r="L11" t="n">
-        <v>11.21</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M11" t="n">
-        <v>11.51</v>
+        <v>9.81</v>
       </c>
       <c r="N11" t="n">
-        <v>49.4</v>
+        <v>47.26</v>
       </c>
       <c r="O11" t="n">
-        <v>49.49</v>
+        <v>47.54</v>
       </c>
       <c r="P11" t="n">
-        <v>48.3</v>
+        <v>45.52</v>
       </c>
       <c r="Q11" t="n">
-        <v>48.59</v>
+        <v>45.59</v>
       </c>
       <c r="R11" t="n">
-        <v>13.0223</v>
+        <v>15.0458</v>
       </c>
       <c r="S11" t="n">
-        <v>13.5297</v>
+        <v>27.1856</v>
       </c>
       <c r="T11" t="n">
-        <v>31.5809</v>
+        <v>40.5866</v>
       </c>
       <c r="U11" t="n">
-        <v>3.8207</v>
+        <v>6.2027</v>
       </c>
       <c r="V11" t="n">
-        <v>6.0592</v>
+        <v>9.601800000000001</v>
       </c>
       <c r="W11" t="n">
-        <v>10.9483</v>
+        <v>15.6967</v>
       </c>
       <c r="X11" t="n">
-        <v>-13.1976</v>
+        <v>-14.7698</v>
       </c>
       <c r="Y11" t="n">
-        <v>-13.4586</v>
+        <v>-24.4222</v>
       </c>
       <c r="Z11" t="n">
-        <v>-26.1706</v>
+        <v>-31.875</v>
       </c>
       <c r="AA11" t="n">
-        <v>-3.8012</v>
+        <v>-6.1741</v>
       </c>
       <c r="AB11" t="n">
-        <v>-5.9245</v>
+        <v>-9.2194</v>
       </c>
       <c r="AC11" t="n">
-        <v>-10.1018</v>
+        <v>-14.1108</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>157.84</v>
+        <v>162.12</v>
       </c>
       <c r="C12" t="n">
-        <v>166</v>
+        <v>162.9</v>
       </c>
       <c r="D12" t="n">
-        <v>149.06</v>
+        <v>147.61</v>
       </c>
       <c r="E12" t="n">
-        <v>165.85</v>
+        <v>152.1</v>
       </c>
       <c r="F12" t="n">
-        <v>69.26000000000001</v>
+        <v>71.87</v>
       </c>
       <c r="G12" t="n">
-        <v>71.66</v>
+        <v>73.3</v>
       </c>
       <c r="H12" t="n">
-        <v>68.88</v>
+        <v>70.38</v>
       </c>
       <c r="I12" t="n">
-        <v>71.56999999999999</v>
+        <v>71.34</v>
       </c>
       <c r="J12" t="n">
-        <v>10.43</v>
+        <v>10.02</v>
       </c>
       <c r="K12" t="n">
-        <v>11.14</v>
+        <v>10.88</v>
       </c>
       <c r="L12" t="n">
-        <v>9.800000000000001</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="M12" t="n">
-        <v>9.81</v>
+        <v>10.6</v>
       </c>
       <c r="N12" t="n">
-        <v>47.26</v>
+        <v>45.41</v>
       </c>
       <c r="O12" t="n">
-        <v>47.54</v>
+        <v>46.36</v>
       </c>
       <c r="P12" t="n">
-        <v>45.52</v>
+        <v>44.5</v>
       </c>
       <c r="Q12" t="n">
-        <v>45.59</v>
+        <v>45.73</v>
       </c>
       <c r="R12" t="n">
-        <v>15.0458</v>
+        <v>-8.2906</v>
       </c>
       <c r="S12" t="n">
-        <v>27.1856</v>
+        <v>19.2474</v>
       </c>
       <c r="T12" t="n">
-        <v>40.5866</v>
+        <v>19.7826</v>
       </c>
       <c r="U12" t="n">
-        <v>6.2027</v>
+        <v>-0.3214</v>
       </c>
       <c r="V12" t="n">
-        <v>9.601800000000001</v>
+        <v>9.906000000000001</v>
       </c>
       <c r="W12" t="n">
-        <v>15.6967</v>
+        <v>12.2757</v>
       </c>
       <c r="X12" t="n">
-        <v>-14.7698</v>
+        <v>8.053000000000001</v>
       </c>
       <c r="Y12" t="n">
-        <v>-24.4222</v>
+        <v>-20.0603</v>
       </c>
       <c r="Z12" t="n">
-        <v>-31.875</v>
+        <v>-20.3008</v>
       </c>
       <c r="AA12" t="n">
-        <v>-6.1741</v>
+        <v>0.3071</v>
       </c>
       <c r="AB12" t="n">
-        <v>-9.2194</v>
+        <v>-9.4635</v>
       </c>
       <c r="AC12" t="n">
-        <v>-14.1108</v>
+        <v>-11.4618</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>162.12</v>
+        <v>163</v>
       </c>
       <c r="C13" t="n">
-        <v>162.9</v>
+        <v>177.5</v>
       </c>
       <c r="D13" t="n">
-        <v>147.61</v>
+        <v>161.51</v>
       </c>
       <c r="E13" t="n">
-        <v>152.1</v>
+        <v>176.94</v>
       </c>
       <c r="F13" t="n">
-        <v>71.87</v>
+        <v>72.81999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>73.3</v>
+        <v>76.31</v>
       </c>
       <c r="H13" t="n">
-        <v>70.38</v>
+        <v>72.7</v>
       </c>
       <c r="I13" t="n">
-        <v>71.34</v>
+        <v>76.28</v>
       </c>
       <c r="J13" t="n">
-        <v>10.02</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="K13" t="n">
-        <v>10.88</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="L13" t="n">
-        <v>9.970000000000001</v>
+        <v>8.84</v>
       </c>
       <c r="M13" t="n">
-        <v>10.6</v>
+        <v>8.85</v>
       </c>
       <c r="N13" t="n">
-        <v>45.41</v>
+        <v>44.82</v>
       </c>
       <c r="O13" t="n">
-        <v>46.36</v>
+        <v>44.89</v>
       </c>
       <c r="P13" t="n">
-        <v>44.5</v>
+        <v>42.57</v>
       </c>
       <c r="Q13" t="n">
-        <v>45.73</v>
+        <v>42.57</v>
       </c>
       <c r="R13" t="n">
-        <v>-8.2906</v>
+        <v>16.3314</v>
       </c>
       <c r="S13" t="n">
-        <v>19.2474</v>
+        <v>22.7386</v>
       </c>
       <c r="T13" t="n">
-        <v>19.7826</v>
+        <v>35.6902</v>
       </c>
       <c r="U13" t="n">
-        <v>-0.3214</v>
+        <v>6.9246</v>
       </c>
       <c r="V13" t="n">
-        <v>9.906000000000001</v>
+        <v>13.1919</v>
       </c>
       <c r="W13" t="n">
-        <v>12.2757</v>
+        <v>16.8147</v>
       </c>
       <c r="X13" t="n">
-        <v>8.053000000000001</v>
+        <v>-16.5094</v>
       </c>
       <c r="Y13" t="n">
-        <v>-20.0603</v>
+        <v>-23.1103</v>
       </c>
       <c r="Z13" t="n">
-        <v>-20.3008</v>
+        <v>-31.8182</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.3071</v>
+        <v>-6.9101</v>
       </c>
       <c r="AB13" t="n">
-        <v>-9.4635</v>
+        <v>-12.3894</v>
       </c>
       <c r="AC13" t="n">
-        <v>-11.4618</v>
+        <v>-15.233</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="C14" t="n">
-        <v>177.5</v>
+        <v>191.29</v>
       </c>
       <c r="D14" t="n">
-        <v>161.51</v>
+        <v>178.94</v>
       </c>
       <c r="E14" t="n">
-        <v>176.94</v>
+        <v>190.42</v>
       </c>
       <c r="F14" t="n">
-        <v>72.81999999999999</v>
+        <v>76</v>
       </c>
       <c r="G14" t="n">
-        <v>76.31</v>
+        <v>77.36</v>
       </c>
       <c r="H14" t="n">
-        <v>72.7</v>
+        <v>75.55</v>
       </c>
       <c r="I14" t="n">
-        <v>76.28</v>
+        <v>76.95999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>9.859999999999999</v>
+        <v>8.65</v>
       </c>
       <c r="K14" t="n">
-        <v>9.970000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="L14" t="n">
-        <v>8.84</v>
+        <v>8.15</v>
       </c>
       <c r="M14" t="n">
-        <v>8.85</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="N14" t="n">
-        <v>44.82</v>
+        <v>42.74</v>
       </c>
       <c r="O14" t="n">
-        <v>44.89</v>
+        <v>43</v>
       </c>
       <c r="P14" t="n">
-        <v>42.57</v>
+        <v>41.99</v>
       </c>
       <c r="Q14" t="n">
-        <v>42.57</v>
+        <v>42.22</v>
       </c>
       <c r="R14" t="n">
-        <v>16.3314</v>
+        <v>7.6184</v>
       </c>
       <c r="S14" t="n">
-        <v>22.7386</v>
+        <v>14.8146</v>
       </c>
       <c r="T14" t="n">
-        <v>35.6902</v>
+        <v>49.2905</v>
       </c>
       <c r="U14" t="n">
-        <v>6.9246</v>
+        <v>0.8915</v>
       </c>
       <c r="V14" t="n">
-        <v>13.1919</v>
+        <v>7.5311</v>
       </c>
       <c r="W14" t="n">
-        <v>16.8147</v>
+        <v>18.5642</v>
       </c>
       <c r="X14" t="n">
-        <v>-16.5094</v>
+        <v>-7.3446</v>
       </c>
       <c r="Y14" t="n">
-        <v>-23.1103</v>
+        <v>-16.4118</v>
       </c>
       <c r="Z14" t="n">
-        <v>-31.8182</v>
+        <v>-38.1599</v>
       </c>
       <c r="AA14" t="n">
-        <v>-6.9101</v>
+        <v>-0.8222</v>
       </c>
       <c r="AB14" t="n">
-        <v>-12.3894</v>
+        <v>-7.392</v>
       </c>
       <c r="AC14" t="n">
-        <v>-15.233</v>
+        <v>-16.4126</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>181</v>
+        <v>177.62</v>
       </c>
       <c r="C15" t="n">
-        <v>191.29</v>
+        <v>182.24</v>
       </c>
       <c r="D15" t="n">
-        <v>178.94</v>
+        <v>150.58</v>
       </c>
       <c r="E15" t="n">
-        <v>190.42</v>
+        <v>172.52</v>
       </c>
       <c r="F15" t="n">
-        <v>76</v>
+        <v>75.3</v>
       </c>
       <c r="G15" t="n">
-        <v>77.36</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="H15" t="n">
-        <v>75.55</v>
+        <v>71.55</v>
       </c>
       <c r="I15" t="n">
-        <v>76.95999999999999</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>8.65</v>
+        <v>8.75</v>
       </c>
       <c r="K15" t="n">
-        <v>8.77</v>
+        <v>9.91</v>
       </c>
       <c r="L15" t="n">
-        <v>8.15</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="M15" t="n">
-        <v>8.199999999999999</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N15" t="n">
-        <v>42.74</v>
+        <v>43.14</v>
       </c>
       <c r="O15" t="n">
-        <v>43</v>
+        <v>45.19</v>
       </c>
       <c r="P15" t="n">
-        <v>41.99</v>
+        <v>42.79</v>
       </c>
       <c r="Q15" t="n">
-        <v>42.22</v>
+        <v>43.31</v>
       </c>
       <c r="R15" t="n">
-        <v>7.6184</v>
+        <v>-9.4003</v>
       </c>
       <c r="S15" t="n">
-        <v>14.8146</v>
+        <v>13.4254</v>
       </c>
       <c r="T15" t="n">
-        <v>49.2905</v>
+        <v>19.6726</v>
       </c>
       <c r="U15" t="n">
-        <v>0.8915</v>
+        <v>-2.5988</v>
       </c>
       <c r="V15" t="n">
-        <v>7.5311</v>
+        <v>5.0743</v>
       </c>
       <c r="W15" t="n">
-        <v>18.5642</v>
+        <v>11.2331</v>
       </c>
       <c r="X15" t="n">
-        <v>-7.3446</v>
+        <v>9.1463</v>
       </c>
       <c r="Y15" t="n">
-        <v>-16.4118</v>
+        <v>-15.566</v>
       </c>
       <c r="Z15" t="n">
-        <v>-38.1599</v>
+        <v>-22.2415</v>
       </c>
       <c r="AA15" t="n">
-        <v>-0.8222</v>
+        <v>2.5817</v>
       </c>
       <c r="AB15" t="n">
-        <v>-7.392</v>
+        <v>-5.2919</v>
       </c>
       <c r="AC15" t="n">
-        <v>-16.4126</v>
+        <v>-10.8664</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>177.62</v>
+        <v>183.84</v>
       </c>
       <c r="C16" t="n">
-        <v>182.24</v>
+        <v>188.49</v>
       </c>
       <c r="D16" t="n">
-        <v>150.58</v>
+        <v>172.26</v>
       </c>
       <c r="E16" t="n">
-        <v>172.52</v>
+        <v>184.24</v>
       </c>
       <c r="F16" t="n">
-        <v>75.3</v>
+        <v>75.81</v>
       </c>
       <c r="G16" t="n">
-        <v>75.93000000000001</v>
+        <v>77.94</v>
       </c>
       <c r="H16" t="n">
-        <v>71.55</v>
+        <v>74.19</v>
       </c>
       <c r="I16" t="n">
-        <v>74.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="J16" t="n">
-        <v>8.75</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>9.91</v>
+        <v>8.98</v>
       </c>
       <c r="L16" t="n">
-        <v>8.550000000000001</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="M16" t="n">
-        <v>8.949999999999999</v>
+        <v>8.35</v>
       </c>
       <c r="N16" t="n">
-        <v>43.14</v>
+        <v>42.83</v>
       </c>
       <c r="O16" t="n">
-        <v>45.19</v>
+        <v>43.77</v>
       </c>
       <c r="P16" t="n">
-        <v>42.79</v>
+        <v>41.6</v>
       </c>
       <c r="Q16" t="n">
-        <v>43.31</v>
+        <v>41.99</v>
       </c>
       <c r="R16" t="n">
-        <v>-9.4003</v>
+        <v>6.7934</v>
       </c>
       <c r="S16" t="n">
-        <v>13.4254</v>
+        <v>4.1257</v>
       </c>
       <c r="T16" t="n">
-        <v>19.6726</v>
+        <v>11.0883</v>
       </c>
       <c r="U16" t="n">
-        <v>-2.5988</v>
+        <v>3.0416</v>
       </c>
       <c r="V16" t="n">
-        <v>5.0743</v>
+        <v>1.2585</v>
       </c>
       <c r="W16" t="n">
-        <v>11.2331</v>
+        <v>7.9223</v>
       </c>
       <c r="X16" t="n">
-        <v>9.1463</v>
+        <v>-6.7039</v>
       </c>
       <c r="Y16" t="n">
-        <v>-15.566</v>
+        <v>-5.6497</v>
       </c>
       <c r="Z16" t="n">
-        <v>-22.2415</v>
+        <v>-14.8828</v>
       </c>
       <c r="AA16" t="n">
-        <v>2.5817</v>
+        <v>-3.0478</v>
       </c>
       <c r="AB16" t="n">
-        <v>-5.2919</v>
+        <v>-1.3625</v>
       </c>
       <c r="AC16" t="n">
-        <v>-10.8664</v>
+        <v>-7.8965</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>183.84</v>
+        <v>182.67</v>
       </c>
       <c r="C17" t="n">
-        <v>188.49</v>
+        <v>189.56</v>
       </c>
       <c r="D17" t="n">
-        <v>172.26</v>
+        <v>178.28</v>
       </c>
       <c r="E17" t="n">
-        <v>184.24</v>
+        <v>186.19</v>
       </c>
       <c r="F17" t="n">
-        <v>75.81</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>77.94</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H17" t="n">
-        <v>74.19</v>
+        <v>77.16</v>
       </c>
       <c r="I17" t="n">
-        <v>77.23999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="J17" t="n">
-        <v>8.380000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="K17" t="n">
-        <v>8.98</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L17" t="n">
-        <v>8.140000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M17" t="n">
-        <v>8.35</v>
+        <v>8.27</v>
       </c>
       <c r="N17" t="n">
-        <v>42.83</v>
+        <v>41.98</v>
       </c>
       <c r="O17" t="n">
-        <v>43.77</v>
+        <v>42.06</v>
       </c>
       <c r="P17" t="n">
-        <v>41.6</v>
+        <v>40.68</v>
       </c>
       <c r="Q17" t="n">
-        <v>41.99</v>
+        <v>41.07</v>
       </c>
       <c r="R17" t="n">
-        <v>6.7934</v>
+        <v>1.0584</v>
       </c>
       <c r="S17" t="n">
-        <v>4.1257</v>
+        <v>-2.2214</v>
       </c>
       <c r="T17" t="n">
-        <v>11.0883</v>
+        <v>22.4129</v>
       </c>
       <c r="U17" t="n">
-        <v>3.0416</v>
+        <v>2.2139</v>
       </c>
       <c r="V17" t="n">
-        <v>1.2585</v>
+        <v>2.5858</v>
       </c>
       <c r="W17" t="n">
-        <v>7.9223</v>
+        <v>10.6672</v>
       </c>
       <c r="X17" t="n">
-        <v>-6.7039</v>
+        <v>-0.9581</v>
       </c>
       <c r="Y17" t="n">
-        <v>-5.6497</v>
+        <v>0.8537</v>
       </c>
       <c r="Z17" t="n">
-        <v>-14.8828</v>
+        <v>-21.9811</v>
       </c>
       <c r="AA17" t="n">
-        <v>-3.0478</v>
+        <v>-2.191</v>
       </c>
       <c r="AB17" t="n">
-        <v>-1.3625</v>
+        <v>-2.7238</v>
       </c>
       <c r="AC17" t="n">
-        <v>-7.8965</v>
+        <v>-10.1902</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>182.67</v>
+        <v>167</v>
       </c>
       <c r="C18" t="n">
-        <v>189.56</v>
+        <v>174.4</v>
       </c>
       <c r="D18" t="n">
-        <v>178.28</v>
+        <v>161.14</v>
       </c>
       <c r="E18" t="n">
-        <v>186.19</v>
+        <v>164.18</v>
       </c>
       <c r="F18" t="n">
-        <v>77.29000000000001</v>
+        <v>75.73</v>
       </c>
       <c r="G18" t="n">
-        <v>79.68000000000001</v>
+        <v>77.37</v>
       </c>
       <c r="H18" t="n">
-        <v>77.16</v>
+        <v>74.23</v>
       </c>
       <c r="I18" t="n">
-        <v>78.95</v>
+        <v>75.34</v>
       </c>
       <c r="J18" t="n">
-        <v>8.43</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>8.630000000000001</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="L18" t="n">
-        <v>8.119999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M18" t="n">
-        <v>8.27</v>
+        <v>9.23</v>
       </c>
       <c r="N18" t="n">
-        <v>41.98</v>
+        <v>42.77</v>
       </c>
       <c r="O18" t="n">
-        <v>42.06</v>
+        <v>43.57</v>
       </c>
       <c r="P18" t="n">
-        <v>40.68</v>
+        <v>41.93</v>
       </c>
       <c r="Q18" t="n">
-        <v>41.07</v>
+        <v>42.98</v>
       </c>
       <c r="R18" t="n">
-        <v>1.0584</v>
+        <v>-11.8213</v>
       </c>
       <c r="S18" t="n">
-        <v>-2.2214</v>
+        <v>-4.8342</v>
       </c>
       <c r="T18" t="n">
-        <v>22.4129</v>
+        <v>-7.2115</v>
       </c>
       <c r="U18" t="n">
-        <v>2.2139</v>
+        <v>-4.5725</v>
       </c>
       <c r="V18" t="n">
-        <v>2.5858</v>
+        <v>0.5069</v>
       </c>
       <c r="W18" t="n">
-        <v>10.6672</v>
+        <v>-1.2323</v>
       </c>
       <c r="X18" t="n">
-        <v>-0.9581</v>
+        <v>11.6082</v>
       </c>
       <c r="Y18" t="n">
-        <v>0.8537</v>
+        <v>3.1285</v>
       </c>
       <c r="Z18" t="n">
-        <v>-21.9811</v>
+        <v>4.2938</v>
       </c>
       <c r="AA18" t="n">
-        <v>-2.191</v>
+        <v>4.6506</v>
       </c>
       <c r="AB18" t="n">
-        <v>-2.7238</v>
+        <v>-0.7619</v>
       </c>
       <c r="AC18" t="n">
-        <v>-10.1902</v>
+        <v>0.9631</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>167</v>
+        <v>172.95</v>
       </c>
       <c r="C19" t="n">
-        <v>174.4</v>
+        <v>174.61</v>
       </c>
       <c r="D19" t="n">
-        <v>161.14</v>
+        <v>142.69</v>
       </c>
       <c r="E19" t="n">
-        <v>164.18</v>
+        <v>151.75</v>
       </c>
       <c r="F19" t="n">
-        <v>75.73</v>
+        <v>76.13</v>
       </c>
       <c r="G19" t="n">
-        <v>77.37</v>
+        <v>76.27</v>
       </c>
       <c r="H19" t="n">
-        <v>74.23</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>75.34</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="J19" t="n">
-        <v>9.130000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="K19" t="n">
-        <v>9.390000000000001</v>
+        <v>10.47</v>
       </c>
       <c r="L19" t="n">
-        <v>8.800000000000001</v>
+        <v>8.68</v>
       </c>
       <c r="M19" t="n">
-        <v>9.23</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="N19" t="n">
-        <v>42.77</v>
+        <v>42.51</v>
       </c>
       <c r="O19" t="n">
-        <v>43.57</v>
+        <v>44.82</v>
       </c>
       <c r="P19" t="n">
-        <v>41.93</v>
+        <v>42.44</v>
       </c>
       <c r="Q19" t="n">
-        <v>42.98</v>
+        <v>43.54</v>
       </c>
       <c r="R19" t="n">
-        <v>-11.8213</v>
+        <v>-7.571</v>
       </c>
       <c r="S19" t="n">
-        <v>-4.8342</v>
+        <v>-17.6346</v>
       </c>
       <c r="T19" t="n">
-        <v>-7.2115</v>
+        <v>-20.3077</v>
       </c>
       <c r="U19" t="n">
-        <v>-4.5725</v>
+        <v>-1.3539</v>
       </c>
       <c r="V19" t="n">
-        <v>0.5069</v>
+        <v>-3.7804</v>
       </c>
       <c r="W19" t="n">
-        <v>-1.2323</v>
+        <v>-3.4304</v>
       </c>
       <c r="X19" t="n">
-        <v>11.6082</v>
+        <v>7.8007</v>
       </c>
       <c r="Y19" t="n">
-        <v>3.1285</v>
+        <v>19.1617</v>
       </c>
       <c r="Z19" t="n">
-        <v>4.2938</v>
+        <v>21.3415</v>
       </c>
       <c r="AA19" t="n">
-        <v>4.6506</v>
+        <v>1.3029</v>
       </c>
       <c r="AB19" t="n">
-        <v>-0.7619</v>
+        <v>3.6914</v>
       </c>
       <c r="AC19" t="n">
-        <v>0.9631</v>
+        <v>3.1265</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>172.95</v>
+        <v>141.24</v>
       </c>
       <c r="C20" t="n">
-        <v>174.61</v>
+        <v>160.6</v>
       </c>
       <c r="D20" t="n">
-        <v>142.69</v>
+        <v>135.02</v>
       </c>
       <c r="E20" t="n">
-        <v>151.75</v>
+        <v>151.89</v>
       </c>
       <c r="F20" t="n">
-        <v>76.13</v>
+        <v>72.41</v>
       </c>
       <c r="G20" t="n">
-        <v>76.27</v>
+        <v>74.5</v>
       </c>
       <c r="H20" t="n">
-        <v>72.09999999999999</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>74.31999999999999</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J20" t="n">
-        <v>8.77</v>
+        <v>10.64</v>
       </c>
       <c r="K20" t="n">
-        <v>10.47</v>
+        <v>11.07</v>
       </c>
       <c r="L20" t="n">
-        <v>8.68</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="M20" t="n">
-        <v>9.949999999999999</v>
+        <v>9.93</v>
       </c>
       <c r="N20" t="n">
-        <v>42.51</v>
+        <v>44.68</v>
       </c>
       <c r="O20" t="n">
-        <v>44.82</v>
+        <v>45.53</v>
       </c>
       <c r="P20" t="n">
-        <v>42.44</v>
+        <v>43.46</v>
       </c>
       <c r="Q20" t="n">
-        <v>43.54</v>
+        <v>44.37</v>
       </c>
       <c r="R20" t="n">
-        <v>-7.571</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="S20" t="n">
-        <v>-17.6346</v>
+        <v>-18.422</v>
       </c>
       <c r="T20" t="n">
-        <v>-20.3077</v>
+        <v>-11.958</v>
       </c>
       <c r="U20" t="n">
-        <v>-1.3539</v>
+        <v>-1.8703</v>
       </c>
       <c r="V20" t="n">
-        <v>-3.7804</v>
+        <v>-7.6251</v>
       </c>
       <c r="W20" t="n">
-        <v>-3.4304</v>
+        <v>-2.7081</v>
       </c>
       <c r="X20" t="n">
-        <v>7.8007</v>
+        <v>-0.201</v>
       </c>
       <c r="Y20" t="n">
-        <v>19.1617</v>
+        <v>20.0726</v>
       </c>
       <c r="Z20" t="n">
-        <v>21.3415</v>
+        <v>10.9497</v>
       </c>
       <c r="AA20" t="n">
-        <v>1.3029</v>
+        <v>1.9063</v>
       </c>
       <c r="AB20" t="n">
-        <v>3.6914</v>
+        <v>8.0351</v>
       </c>
       <c r="AC20" t="n">
-        <v>3.1265</v>
+        <v>2.4475</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>141.24</v>
+        <v>161</v>
       </c>
       <c r="C21" t="n">
-        <v>160.6</v>
+        <v>173.7</v>
       </c>
       <c r="D21" t="n">
-        <v>135.02</v>
+        <v>161</v>
       </c>
       <c r="E21" t="n">
-        <v>151.89</v>
+        <v>173.2</v>
       </c>
       <c r="F21" t="n">
-        <v>72.41</v>
+        <v>74.09</v>
       </c>
       <c r="G21" t="n">
-        <v>74.5</v>
+        <v>76.53</v>
       </c>
       <c r="H21" t="n">
-        <v>70.95999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="I21" t="n">
-        <v>72.93000000000001</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>10.64</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K21" t="n">
-        <v>11.07</v>
+        <v>9.35</v>
       </c>
       <c r="L21" t="n">
-        <v>9.369999999999999</v>
+        <v>8.51</v>
       </c>
       <c r="M21" t="n">
-        <v>9.93</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N21" t="n">
-        <v>44.68</v>
+        <v>43.67</v>
       </c>
       <c r="O21" t="n">
-        <v>45.53</v>
+        <v>43.97</v>
       </c>
       <c r="P21" t="n">
-        <v>43.46</v>
+        <v>42.19</v>
       </c>
       <c r="Q21" t="n">
-        <v>44.37</v>
+        <v>42.19</v>
       </c>
       <c r="R21" t="n">
-        <v>0.09229999999999999</v>
+        <v>14.0299</v>
       </c>
       <c r="S21" t="n">
-        <v>-18.422</v>
+        <v>5.494</v>
       </c>
       <c r="T21" t="n">
-        <v>-11.958</v>
+        <v>-5.9922</v>
       </c>
       <c r="U21" t="n">
-        <v>-1.8703</v>
+        <v>4.9088</v>
       </c>
       <c r="V21" t="n">
-        <v>-7.6251</v>
+        <v>1.553</v>
       </c>
       <c r="W21" t="n">
-        <v>-2.7081</v>
+        <v>-0.9451000000000001</v>
       </c>
       <c r="X21" t="n">
-        <v>-0.201</v>
+        <v>-13.998</v>
       </c>
       <c r="Y21" t="n">
-        <v>20.0726</v>
+        <v>-7.4756</v>
       </c>
       <c r="Z21" t="n">
-        <v>10.9497</v>
+        <v>2.2754</v>
       </c>
       <c r="AA21" t="n">
-        <v>1.9063</v>
+        <v>-4.9132</v>
       </c>
       <c r="AB21" t="n">
-        <v>8.0351</v>
+        <v>-1.8381</v>
       </c>
       <c r="AC21" t="n">
-        <v>2.4475</v>
+        <v>0.4763</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>161</v>
+        <v>171.26</v>
       </c>
       <c r="C22" t="n">
-        <v>173.7</v>
+        <v>179.97</v>
       </c>
       <c r="D22" t="n">
-        <v>161</v>
+        <v>168.23</v>
       </c>
       <c r="E22" t="n">
-        <v>173.2</v>
+        <v>178.39</v>
       </c>
       <c r="F22" t="n">
-        <v>74.09</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G22" t="n">
-        <v>76.53</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>73.62</v>
+        <v>74.47</v>
       </c>
       <c r="I22" t="n">
-        <v>76.51000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J22" t="n">
-        <v>9.300000000000001</v>
+        <v>8.65</v>
       </c>
       <c r="K22" t="n">
-        <v>9.35</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L22" t="n">
-        <v>8.51</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M22" t="n">
-        <v>8.539999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N22" t="n">
-        <v>43.67</v>
+        <v>42.94</v>
       </c>
       <c r="O22" t="n">
-        <v>43.97</v>
+        <v>43.33</v>
       </c>
       <c r="P22" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="Q22" t="n">
-        <v>42.19</v>
+        <v>41.96</v>
       </c>
       <c r="R22" t="n">
-        <v>14.0299</v>
+        <v>2.9965</v>
       </c>
       <c r="S22" t="n">
-        <v>5.494</v>
+        <v>17.5552</v>
       </c>
       <c r="T22" t="n">
-        <v>-5.9922</v>
+        <v>-4.1893</v>
       </c>
       <c r="U22" t="n">
-        <v>4.9088</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="V22" t="n">
-        <v>1.553</v>
+        <v>3.5388</v>
       </c>
       <c r="W22" t="n">
-        <v>-0.9451000000000001</v>
+        <v>-2.5332</v>
       </c>
       <c r="X22" t="n">
-        <v>-13.998</v>
+        <v>-2.9274</v>
       </c>
       <c r="Y22" t="n">
-        <v>-7.4756</v>
+        <v>-16.6834</v>
       </c>
       <c r="Z22" t="n">
-        <v>2.2754</v>
+        <v>0.2418</v>
       </c>
       <c r="AA22" t="n">
-        <v>-4.9132</v>
+        <v>-0.5452</v>
       </c>
       <c r="AB22" t="n">
-        <v>-1.8381</v>
+        <v>-3.6288</v>
       </c>
       <c r="AC22" t="n">
-        <v>0.4763</v>
+        <v>2.167</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>171.26</v>
+        <v>184.8</v>
       </c>
       <c r="C23" t="n">
-        <v>179.97</v>
+        <v>195.255</v>
       </c>
       <c r="D23" t="n">
-        <v>168.2501</v>
+        <v>183.34</v>
       </c>
       <c r="E23" t="n">
-        <v>178.39</v>
+        <v>190.56</v>
       </c>
       <c r="F23" t="n">
-        <v>75.19</v>
+        <v>78.01000000000001</v>
       </c>
       <c r="G23" t="n">
-        <v>77.7895</v>
+        <v>79.33</v>
       </c>
       <c r="H23" t="n">
-        <v>74.471</v>
+        <v>77.33199999999999</v>
       </c>
       <c r="I23" t="n">
-        <v>76.95</v>
+        <v>77.84</v>
       </c>
       <c r="J23" t="n">
-        <v>8.645</v>
+        <v>8</v>
       </c>
       <c r="K23" t="n">
-        <v>8.779999999999999</v>
+        <v>8.06</v>
       </c>
       <c r="L23" t="n">
-        <v>8.210000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="M23" t="n">
-        <v>8.289999999999999</v>
+        <v>7.73</v>
       </c>
       <c r="N23" t="n">
-        <v>42.97</v>
+        <v>41.39</v>
       </c>
       <c r="O23" t="n">
-        <v>43.3305</v>
+        <v>41.78</v>
       </c>
       <c r="P23" t="n">
+        <v>40.68</v>
+      </c>
+      <c r="Q23" t="n">
         <v>41.5</v>
       </c>
-      <c r="Q23" t="n">
-        <v>41.96</v>
-      </c>
       <c r="R23" t="n">
-        <v>2.9965</v>
+        <v>6.8221</v>
       </c>
       <c r="S23" t="n">
-        <v>17.5552</v>
+        <v>25.4592</v>
       </c>
       <c r="T23" t="n">
-        <v>-4.1893</v>
+        <v>16.0677</v>
       </c>
       <c r="U23" t="n">
-        <v>0.5750999999999999</v>
+        <v>1.1566</v>
       </c>
       <c r="V23" t="n">
-        <v>3.5388</v>
+        <v>6.7325</v>
       </c>
       <c r="W23" t="n">
-        <v>-2.5332</v>
+        <v>3.3183</v>
       </c>
       <c r="X23" t="n">
-        <v>-2.9274</v>
+        <v>-6.7551</v>
       </c>
       <c r="Y23" t="n">
-        <v>-16.6834</v>
+        <v>-22.1551</v>
       </c>
       <c r="Z23" t="n">
-        <v>0.2418</v>
+        <v>-16.2514</v>
       </c>
       <c r="AA23" t="n">
-        <v>-0.5452</v>
+        <v>-1.0963</v>
       </c>
       <c r="AB23" t="n">
-        <v>-3.6288</v>
+        <v>-6.4683</v>
       </c>
       <c r="AC23" t="n">
-        <v>2.167</v>
+        <v>-3.4435</v>
       </c>
     </row>
   </sheetData>
@@ -2503,7 +2503,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-05-23 16:26
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -2378,7 +2378,7 @@
         <v>184.8</v>
       </c>
       <c r="C23" t="n">
-        <v>195.255</v>
+        <v>195.27</v>
       </c>
       <c r="D23" t="n">
         <v>183.34</v>
@@ -2387,13 +2387,13 @@
         <v>190.56</v>
       </c>
       <c r="F23" t="n">
-        <v>78.01000000000001</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G23" t="n">
         <v>79.33</v>
       </c>
       <c r="H23" t="n">
-        <v>77.33199999999999</v>
+        <v>77.33</v>
       </c>
       <c r="I23" t="n">
         <v>77.84</v>
@@ -2411,7 +2411,7 @@
         <v>7.73</v>
       </c>
       <c r="N23" t="n">
-        <v>41.39</v>
+        <v>41.4</v>
       </c>
       <c r="O23" t="n">
         <v>41.78</v>
@@ -2503,7 +2503,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-05-25 23:02
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC23"/>
+  <dimension ref="A1:AC21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1894 +568,1712 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>108.62</v>
+        <v>128.33</v>
       </c>
       <c r="C2" t="n">
-        <v>116.77</v>
+        <v>129.59</v>
       </c>
       <c r="D2" t="n">
-        <v>107.46</v>
+        <v>117.79</v>
       </c>
       <c r="E2" t="n">
-        <v>112.77</v>
+        <v>123.39</v>
       </c>
       <c r="F2" t="n">
-        <v>59.8</v>
+        <v>62.41</v>
       </c>
       <c r="G2" t="n">
-        <v>60.73</v>
+        <v>62.7</v>
       </c>
       <c r="H2" t="n">
-        <v>57.59</v>
+        <v>61.64</v>
       </c>
       <c r="I2" t="n">
-        <v>59.22</v>
+        <v>62.64</v>
       </c>
       <c r="J2" t="n">
-        <v>16.35</v>
+        <v>13.51</v>
       </c>
       <c r="K2" t="n">
-        <v>16.52</v>
+        <v>14.63</v>
       </c>
       <c r="L2" t="n">
-        <v>15.06</v>
+        <v>13.41</v>
       </c>
       <c r="M2" t="n">
-        <v>15.7</v>
+        <v>14.03</v>
       </c>
       <c r="N2" t="n">
-        <v>55.13</v>
+        <v>52.67</v>
       </c>
       <c r="O2" t="n">
-        <v>57.14</v>
+        <v>53.31</v>
       </c>
       <c r="P2" t="n">
-        <v>54.28</v>
+        <v>52.42</v>
       </c>
       <c r="Q2" t="n">
-        <v>55.66</v>
+        <v>52.45</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>125.21</v>
+        <v>108.75</v>
       </c>
       <c r="C3" t="n">
-        <v>130.12</v>
+        <v>115.62</v>
       </c>
       <c r="D3" t="n">
-        <v>120.24</v>
+        <v>103.99</v>
       </c>
       <c r="E3" t="n">
-        <v>128.32</v>
+        <v>109.56</v>
       </c>
       <c r="F3" t="n">
-        <v>61.08</v>
+        <v>60.72</v>
       </c>
       <c r="G3" t="n">
-        <v>62.74</v>
+        <v>61.33</v>
       </c>
       <c r="H3" t="n">
-        <v>60.56</v>
+        <v>59.68</v>
       </c>
       <c r="I3" t="n">
-        <v>62.56</v>
+        <v>60.74</v>
       </c>
       <c r="J3" t="n">
-        <v>13.99</v>
+        <v>15.71</v>
       </c>
       <c r="K3" t="n">
-        <v>14.66</v>
+        <v>16.27</v>
       </c>
       <c r="L3" t="n">
-        <v>13.3</v>
+        <v>14.93</v>
       </c>
       <c r="M3" t="n">
-        <v>13.52</v>
+        <v>15.59</v>
       </c>
       <c r="N3" t="n">
-        <v>53.93</v>
+        <v>54.09</v>
       </c>
       <c r="O3" t="n">
-        <v>54.43</v>
+        <v>54.96</v>
       </c>
       <c r="P3" t="n">
-        <v>52.37</v>
+        <v>53.58</v>
       </c>
       <c r="Q3" t="n">
-        <v>52.5</v>
+        <v>54.05</v>
       </c>
       <c r="R3" t="n">
-        <v>13.7891</v>
+        <v>-11.2084</v>
       </c>
       <c r="U3" t="n">
-        <v>5.64</v>
+        <v>-3.0332</v>
       </c>
       <c r="X3" t="n">
-        <v>-13.8854</v>
+        <v>11.119</v>
       </c>
       <c r="AA3" t="n">
-        <v>-5.6773</v>
+        <v>3.0505</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>128.33</v>
+        <v>114.76</v>
       </c>
       <c r="C4" t="n">
-        <v>129.59</v>
+        <v>118.32</v>
       </c>
       <c r="D4" t="n">
-        <v>117.79</v>
+        <v>112.3</v>
       </c>
       <c r="E4" t="n">
-        <v>123.39</v>
+        <v>117.97</v>
       </c>
       <c r="F4" t="n">
-        <v>62.41</v>
+        <v>61</v>
       </c>
       <c r="G4" t="n">
-        <v>62.7</v>
+        <v>61.87</v>
       </c>
       <c r="H4" t="n">
-        <v>61.64</v>
+        <v>60.45</v>
       </c>
       <c r="I4" t="n">
-        <v>62.64</v>
+        <v>61.86</v>
       </c>
       <c r="J4" t="n">
-        <v>13.51</v>
+        <v>14.91</v>
       </c>
       <c r="K4" t="n">
-        <v>14.63</v>
+        <v>15.24</v>
       </c>
       <c r="L4" t="n">
-        <v>13.41</v>
+        <v>14.38</v>
       </c>
       <c r="M4" t="n">
-        <v>14.03</v>
+        <v>14.4</v>
       </c>
       <c r="N4" t="n">
-        <v>52.67</v>
+        <v>53.84</v>
       </c>
       <c r="O4" t="n">
-        <v>53.31</v>
+        <v>54.33</v>
       </c>
       <c r="P4" t="n">
-        <v>52.42</v>
+        <v>53.06</v>
       </c>
       <c r="Q4" t="n">
-        <v>52.45</v>
+        <v>53.08</v>
       </c>
       <c r="R4" t="n">
-        <v>-3.842</v>
+        <v>7.6762</v>
       </c>
       <c r="U4" t="n">
-        <v>0.1279</v>
+        <v>1.8439</v>
       </c>
       <c r="X4" t="n">
-        <v>3.7722</v>
+        <v>-7.6331</v>
       </c>
       <c r="AA4" t="n">
-        <v>-0.09520000000000001</v>
+        <v>-1.7946</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>108.75</v>
+        <v>122.81</v>
       </c>
       <c r="C5" t="n">
-        <v>115.62</v>
+        <v>127.45</v>
       </c>
       <c r="D5" t="n">
-        <v>103.99</v>
+        <v>117.5</v>
       </c>
       <c r="E5" t="n">
-        <v>109.56</v>
+        <v>126.98</v>
       </c>
       <c r="F5" t="n">
-        <v>60.72</v>
+        <v>62.89</v>
       </c>
       <c r="G5" t="n">
-        <v>61.33</v>
+        <v>63.8</v>
       </c>
       <c r="H5" t="n">
-        <v>59.68</v>
+        <v>60.7</v>
       </c>
       <c r="I5" t="n">
-        <v>60.74</v>
+        <v>63.54</v>
       </c>
       <c r="J5" t="n">
-        <v>15.71</v>
+        <v>13.84</v>
       </c>
       <c r="K5" t="n">
-        <v>16.27</v>
+        <v>14.49</v>
       </c>
       <c r="L5" t="n">
-        <v>14.93</v>
+        <v>13.25</v>
       </c>
       <c r="M5" t="n">
-        <v>15.59</v>
+        <v>13.3</v>
       </c>
       <c r="N5" t="n">
+        <v>52.21</v>
+      </c>
+      <c r="O5" t="n">
         <v>54.09</v>
       </c>
-      <c r="O5" t="n">
-        <v>54.96</v>
-      </c>
       <c r="P5" t="n">
-        <v>53.58</v>
+        <v>51.4</v>
       </c>
       <c r="Q5" t="n">
-        <v>54.05</v>
+        <v>51.65</v>
       </c>
       <c r="R5" t="n">
-        <v>-11.2084</v>
+        <v>7.6375</v>
       </c>
       <c r="S5" t="n">
-        <v>-2.8465</v>
+        <v>2.9095</v>
       </c>
       <c r="U5" t="n">
-        <v>-3.0332</v>
+        <v>2.7158</v>
       </c>
       <c r="V5" t="n">
-        <v>2.5667</v>
+        <v>1.4368</v>
       </c>
       <c r="X5" t="n">
-        <v>11.119</v>
+        <v>-7.6389</v>
       </c>
       <c r="Y5" t="n">
-        <v>-0.7006</v>
+        <v>-5.2031</v>
       </c>
       <c r="AA5" t="n">
-        <v>3.0505</v>
+        <v>-2.694</v>
       </c>
       <c r="AB5" t="n">
-        <v>-2.8926</v>
+        <v>-1.5253</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>114.76</v>
+        <v>124.39</v>
       </c>
       <c r="C6" t="n">
-        <v>118.32</v>
+        <v>131.38</v>
       </c>
       <c r="D6" t="n">
-        <v>112.3</v>
+        <v>121.66</v>
       </c>
       <c r="E6" t="n">
-        <v>117.97</v>
+        <v>130.4</v>
       </c>
       <c r="F6" t="n">
-        <v>61</v>
+        <v>63.89</v>
       </c>
       <c r="G6" t="n">
-        <v>61.87</v>
+        <v>65.84</v>
       </c>
       <c r="H6" t="n">
-        <v>60.45</v>
+        <v>63.81</v>
       </c>
       <c r="I6" t="n">
-        <v>61.86</v>
+        <v>65.3</v>
       </c>
       <c r="J6" t="n">
-        <v>14.91</v>
+        <v>13.61</v>
       </c>
       <c r="K6" t="n">
-        <v>15.24</v>
+        <v>13.89</v>
       </c>
       <c r="L6" t="n">
-        <v>14.38</v>
+        <v>12.87</v>
       </c>
       <c r="M6" t="n">
-        <v>14.4</v>
+        <v>12.98</v>
       </c>
       <c r="N6" t="n">
-        <v>53.84</v>
+        <v>51.36</v>
       </c>
       <c r="O6" t="n">
-        <v>54.33</v>
+        <v>51.45</v>
       </c>
       <c r="P6" t="n">
-        <v>53.06</v>
+        <v>49.79</v>
       </c>
       <c r="Q6" t="n">
-        <v>53.08</v>
+        <v>50.22</v>
       </c>
       <c r="R6" t="n">
-        <v>7.6762</v>
+        <v>2.6933</v>
       </c>
       <c r="S6" t="n">
-        <v>-8.065799999999999</v>
+        <v>19.0215</v>
       </c>
       <c r="U6" t="n">
-        <v>1.8439</v>
+        <v>2.7699</v>
       </c>
       <c r="V6" t="n">
-        <v>-1.1189</v>
+        <v>7.5074</v>
       </c>
       <c r="X6" t="n">
-        <v>-7.6331</v>
+        <v>-2.406</v>
       </c>
       <c r="Y6" t="n">
-        <v>6.5089</v>
+        <v>-16.7415</v>
       </c>
       <c r="AA6" t="n">
-        <v>-1.7946</v>
+        <v>-2.7686</v>
       </c>
       <c r="AB6" t="n">
-        <v>1.1048</v>
+        <v>-7.086</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>122.81</v>
+        <v>132.2</v>
       </c>
       <c r="C7" t="n">
-        <v>127.45</v>
+        <v>133.67</v>
       </c>
       <c r="D7" t="n">
-        <v>117.5</v>
+        <v>123.8</v>
       </c>
       <c r="E7" t="n">
-        <v>126.98</v>
+        <v>127.55</v>
       </c>
       <c r="F7" t="n">
-        <v>62.89</v>
+        <v>65.44</v>
       </c>
       <c r="G7" t="n">
-        <v>63.8</v>
+        <v>66.05</v>
       </c>
       <c r="H7" t="n">
-        <v>60.7</v>
+        <v>63.78</v>
       </c>
       <c r="I7" t="n">
-        <v>63.54</v>
+        <v>64.91</v>
       </c>
       <c r="J7" t="n">
-        <v>13.84</v>
+        <v>12.8</v>
       </c>
       <c r="K7" t="n">
-        <v>14.49</v>
+        <v>13.64</v>
       </c>
       <c r="L7" t="n">
-        <v>13.25</v>
+        <v>12.65</v>
       </c>
       <c r="M7" t="n">
-        <v>13.3</v>
+        <v>13.26</v>
       </c>
       <c r="N7" t="n">
-        <v>52.21</v>
+        <v>50.12</v>
       </c>
       <c r="O7" t="n">
-        <v>54.09</v>
+        <v>51.43</v>
       </c>
       <c r="P7" t="n">
-        <v>51.4</v>
+        <v>49.65</v>
       </c>
       <c r="Q7" t="n">
-        <v>51.65</v>
+        <v>50.51</v>
       </c>
       <c r="R7" t="n">
-        <v>7.6375</v>
+        <v>-2.1856</v>
       </c>
       <c r="S7" t="n">
-        <v>2.9095</v>
+        <v>8.120699999999999</v>
       </c>
       <c r="T7" t="n">
-        <v>12.6009</v>
+        <v>3.3714</v>
       </c>
       <c r="U7" t="n">
-        <v>2.7158</v>
+        <v>-0.5972</v>
       </c>
       <c r="V7" t="n">
-        <v>1.4368</v>
+        <v>4.9305</v>
       </c>
       <c r="W7" t="n">
-        <v>7.2948</v>
+        <v>3.6239</v>
       </c>
       <c r="X7" t="n">
-        <v>-7.6389</v>
+        <v>2.1572</v>
       </c>
       <c r="Y7" t="n">
-        <v>-5.2031</v>
+        <v>-7.9167</v>
       </c>
       <c r="Z7" t="n">
-        <v>-15.2866</v>
+        <v>-5.4882</v>
       </c>
       <c r="AA7" t="n">
-        <v>-2.694</v>
+        <v>0.5775</v>
       </c>
       <c r="AB7" t="n">
-        <v>-1.5253</v>
+        <v>-4.8417</v>
       </c>
       <c r="AC7" t="n">
-        <v>-7.2045</v>
+        <v>-3.6988</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>124.39</v>
+        <v>135</v>
       </c>
       <c r="C8" t="n">
-        <v>131.38</v>
+        <v>147.26</v>
       </c>
       <c r="D8" t="n">
-        <v>121.66</v>
+        <v>134.02</v>
       </c>
       <c r="E8" t="n">
-        <v>130.4</v>
+        <v>144.16</v>
       </c>
       <c r="F8" t="n">
-        <v>63.89</v>
+        <v>66.37</v>
       </c>
       <c r="G8" t="n">
-        <v>65.84</v>
+        <v>67.77</v>
       </c>
       <c r="H8" t="n">
-        <v>63.81</v>
+        <v>66.25</v>
       </c>
       <c r="I8" t="n">
-        <v>65.3</v>
+        <v>67.39</v>
       </c>
       <c r="J8" t="n">
-        <v>13.61</v>
+        <v>12.5</v>
       </c>
       <c r="K8" t="n">
-        <v>13.89</v>
+        <v>12.59</v>
       </c>
       <c r="L8" t="n">
-        <v>12.87</v>
+        <v>11.21</v>
       </c>
       <c r="M8" t="n">
-        <v>12.98</v>
+        <v>11.51</v>
       </c>
       <c r="N8" t="n">
-        <v>51.36</v>
+        <v>49.4</v>
       </c>
       <c r="O8" t="n">
-        <v>51.45</v>
+        <v>49.49</v>
       </c>
       <c r="P8" t="n">
-        <v>49.79</v>
+        <v>48.3</v>
       </c>
       <c r="Q8" t="n">
-        <v>50.22</v>
+        <v>48.59</v>
       </c>
       <c r="R8" t="n">
-        <v>2.6933</v>
+        <v>13.0223</v>
       </c>
       <c r="S8" t="n">
-        <v>19.0215</v>
+        <v>13.5297</v>
       </c>
       <c r="T8" t="n">
-        <v>1.6209</v>
+        <v>31.5809</v>
       </c>
       <c r="U8" t="n">
-        <v>2.7699</v>
+        <v>3.8207</v>
       </c>
       <c r="V8" t="n">
-        <v>7.5074</v>
+        <v>6.0592</v>
       </c>
       <c r="W8" t="n">
-        <v>4.3798</v>
+        <v>10.9483</v>
       </c>
       <c r="X8" t="n">
-        <v>-2.406</v>
+        <v>-13.1976</v>
       </c>
       <c r="Y8" t="n">
-        <v>-16.7415</v>
+        <v>-13.4586</v>
       </c>
       <c r="Z8" t="n">
-        <v>-3.9941</v>
+        <v>-26.1706</v>
       </c>
       <c r="AA8" t="n">
-        <v>-2.7686</v>
+        <v>-3.8012</v>
       </c>
       <c r="AB8" t="n">
-        <v>-7.086</v>
+        <v>-5.9245</v>
       </c>
       <c r="AC8" t="n">
-        <v>-4.3429</v>
+        <v>-10.1018</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>132.2</v>
+        <v>157.84</v>
       </c>
       <c r="C9" t="n">
-        <v>133.67</v>
+        <v>166</v>
       </c>
       <c r="D9" t="n">
-        <v>123.8</v>
+        <v>149.06</v>
       </c>
       <c r="E9" t="n">
-        <v>127.55</v>
+        <v>165.85</v>
       </c>
       <c r="F9" t="n">
-        <v>65.44</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>66.05</v>
+        <v>71.66</v>
       </c>
       <c r="H9" t="n">
-        <v>63.78</v>
+        <v>68.88</v>
       </c>
       <c r="I9" t="n">
-        <v>64.91</v>
+        <v>71.56999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>12.8</v>
+        <v>10.43</v>
       </c>
       <c r="K9" t="n">
-        <v>13.64</v>
+        <v>11.14</v>
       </c>
       <c r="L9" t="n">
-        <v>12.65</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M9" t="n">
-        <v>13.26</v>
+        <v>9.81</v>
       </c>
       <c r="N9" t="n">
-        <v>50.12</v>
+        <v>47.26</v>
       </c>
       <c r="O9" t="n">
-        <v>51.43</v>
+        <v>47.54</v>
       </c>
       <c r="P9" t="n">
-        <v>49.65</v>
+        <v>45.52</v>
       </c>
       <c r="Q9" t="n">
-        <v>50.51</v>
+        <v>45.59</v>
       </c>
       <c r="R9" t="n">
-        <v>-2.1856</v>
+        <v>15.0458</v>
       </c>
       <c r="S9" t="n">
-        <v>8.120699999999999</v>
+        <v>27.1856</v>
       </c>
       <c r="T9" t="n">
-        <v>3.3714</v>
+        <v>40.5866</v>
       </c>
       <c r="U9" t="n">
-        <v>-0.5972</v>
+        <v>6.2027</v>
       </c>
       <c r="V9" t="n">
-        <v>4.9305</v>
+        <v>9.601800000000001</v>
       </c>
       <c r="W9" t="n">
-        <v>3.6239</v>
+        <v>15.6967</v>
       </c>
       <c r="X9" t="n">
-        <v>2.1572</v>
+        <v>-14.7698</v>
       </c>
       <c r="Y9" t="n">
-        <v>-7.9167</v>
+        <v>-24.4222</v>
       </c>
       <c r="Z9" t="n">
-        <v>-5.4882</v>
+        <v>-31.875</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.5775</v>
+        <v>-6.1741</v>
       </c>
       <c r="AB9" t="n">
-        <v>-4.8417</v>
+        <v>-9.2194</v>
       </c>
       <c r="AC9" t="n">
-        <v>-3.6988</v>
+        <v>-14.1108</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>135</v>
+        <v>162.12</v>
       </c>
       <c r="C10" t="n">
-        <v>147.26</v>
+        <v>162.9</v>
       </c>
       <c r="D10" t="n">
-        <v>134.02</v>
+        <v>147.61</v>
       </c>
       <c r="E10" t="n">
-        <v>144.16</v>
+        <v>152.1</v>
       </c>
       <c r="F10" t="n">
-        <v>66.37</v>
+        <v>71.87</v>
       </c>
       <c r="G10" t="n">
-        <v>67.77</v>
+        <v>73.3</v>
       </c>
       <c r="H10" t="n">
-        <v>66.25</v>
+        <v>70.38</v>
       </c>
       <c r="I10" t="n">
-        <v>67.39</v>
+        <v>71.34</v>
       </c>
       <c r="J10" t="n">
-        <v>12.5</v>
+        <v>10.02</v>
       </c>
       <c r="K10" t="n">
-        <v>12.59</v>
+        <v>10.88</v>
       </c>
       <c r="L10" t="n">
-        <v>11.21</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="M10" t="n">
-        <v>11.51</v>
+        <v>10.6</v>
       </c>
       <c r="N10" t="n">
-        <v>49.4</v>
+        <v>45.41</v>
       </c>
       <c r="O10" t="n">
-        <v>49.49</v>
+        <v>46.36</v>
       </c>
       <c r="P10" t="n">
-        <v>48.3</v>
+        <v>44.5</v>
       </c>
       <c r="Q10" t="n">
-        <v>48.59</v>
+        <v>45.73</v>
       </c>
       <c r="R10" t="n">
-        <v>13.0223</v>
+        <v>-8.2906</v>
       </c>
       <c r="S10" t="n">
-        <v>13.5297</v>
+        <v>19.2474</v>
       </c>
       <c r="T10" t="n">
-        <v>31.5809</v>
+        <v>19.7826</v>
       </c>
       <c r="U10" t="n">
-        <v>3.8207</v>
+        <v>-0.3214</v>
       </c>
       <c r="V10" t="n">
-        <v>6.0592</v>
+        <v>9.906000000000001</v>
       </c>
       <c r="W10" t="n">
-        <v>10.9483</v>
+        <v>12.2757</v>
       </c>
       <c r="X10" t="n">
-        <v>-13.1976</v>
+        <v>8.053000000000001</v>
       </c>
       <c r="Y10" t="n">
-        <v>-13.4586</v>
+        <v>-20.0603</v>
       </c>
       <c r="Z10" t="n">
-        <v>-26.1706</v>
+        <v>-20.3008</v>
       </c>
       <c r="AA10" t="n">
-        <v>-3.8012</v>
+        <v>0.3071</v>
       </c>
       <c r="AB10" t="n">
-        <v>-5.9245</v>
+        <v>-9.4635</v>
       </c>
       <c r="AC10" t="n">
-        <v>-10.1018</v>
+        <v>-11.4618</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>157.84</v>
+        <v>163</v>
       </c>
       <c r="C11" t="n">
-        <v>166</v>
+        <v>177.5</v>
       </c>
       <c r="D11" t="n">
-        <v>149.06</v>
+        <v>161.51</v>
       </c>
       <c r="E11" t="n">
-        <v>165.85</v>
+        <v>176.94</v>
       </c>
       <c r="F11" t="n">
-        <v>69.26000000000001</v>
+        <v>72.81999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>71.66</v>
+        <v>76.31</v>
       </c>
       <c r="H11" t="n">
-        <v>68.88</v>
+        <v>72.7</v>
       </c>
       <c r="I11" t="n">
-        <v>71.56999999999999</v>
+        <v>76.28</v>
       </c>
       <c r="J11" t="n">
-        <v>10.43</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="K11" t="n">
-        <v>11.14</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="L11" t="n">
-        <v>9.800000000000001</v>
+        <v>8.84</v>
       </c>
       <c r="M11" t="n">
-        <v>9.81</v>
+        <v>8.85</v>
       </c>
       <c r="N11" t="n">
-        <v>47.26</v>
+        <v>44.82</v>
       </c>
       <c r="O11" t="n">
-        <v>47.54</v>
+        <v>44.89</v>
       </c>
       <c r="P11" t="n">
-        <v>45.52</v>
+        <v>42.57</v>
       </c>
       <c r="Q11" t="n">
-        <v>45.59</v>
+        <v>42.57</v>
       </c>
       <c r="R11" t="n">
-        <v>15.0458</v>
+        <v>16.3314</v>
       </c>
       <c r="S11" t="n">
-        <v>27.1856</v>
+        <v>22.7386</v>
       </c>
       <c r="T11" t="n">
-        <v>40.5866</v>
+        <v>35.6902</v>
       </c>
       <c r="U11" t="n">
-        <v>6.2027</v>
+        <v>6.9246</v>
       </c>
       <c r="V11" t="n">
-        <v>9.601800000000001</v>
+        <v>13.1919</v>
       </c>
       <c r="W11" t="n">
-        <v>15.6967</v>
+        <v>16.8147</v>
       </c>
       <c r="X11" t="n">
-        <v>-14.7698</v>
+        <v>-16.5094</v>
       </c>
       <c r="Y11" t="n">
-        <v>-24.4222</v>
+        <v>-23.1103</v>
       </c>
       <c r="Z11" t="n">
-        <v>-31.875</v>
+        <v>-31.8182</v>
       </c>
       <c r="AA11" t="n">
-        <v>-6.1741</v>
+        <v>-6.9101</v>
       </c>
       <c r="AB11" t="n">
-        <v>-9.2194</v>
+        <v>-12.3894</v>
       </c>
       <c r="AC11" t="n">
-        <v>-14.1108</v>
+        <v>-15.233</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>162.12</v>
+        <v>181</v>
       </c>
       <c r="C12" t="n">
-        <v>162.9</v>
+        <v>191.29</v>
       </c>
       <c r="D12" t="n">
-        <v>147.61</v>
+        <v>178.94</v>
       </c>
       <c r="E12" t="n">
-        <v>152.1</v>
+        <v>190.42</v>
       </c>
       <c r="F12" t="n">
-        <v>71.87</v>
+        <v>76</v>
       </c>
       <c r="G12" t="n">
-        <v>73.3</v>
+        <v>77.36</v>
       </c>
       <c r="H12" t="n">
-        <v>70.38</v>
+        <v>75.55</v>
       </c>
       <c r="I12" t="n">
-        <v>71.34</v>
+        <v>76.95999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>10.02</v>
+        <v>8.65</v>
       </c>
       <c r="K12" t="n">
-        <v>10.88</v>
+        <v>8.77</v>
       </c>
       <c r="L12" t="n">
-        <v>9.970000000000001</v>
+        <v>8.15</v>
       </c>
       <c r="M12" t="n">
-        <v>10.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="N12" t="n">
-        <v>45.41</v>
+        <v>42.74</v>
       </c>
       <c r="O12" t="n">
-        <v>46.36</v>
+        <v>43</v>
       </c>
       <c r="P12" t="n">
-        <v>44.5</v>
+        <v>41.99</v>
       </c>
       <c r="Q12" t="n">
-        <v>45.73</v>
+        <v>42.22</v>
       </c>
       <c r="R12" t="n">
-        <v>-8.2906</v>
+        <v>7.6184</v>
       </c>
       <c r="S12" t="n">
-        <v>19.2474</v>
+        <v>14.8146</v>
       </c>
       <c r="T12" t="n">
-        <v>19.7826</v>
+        <v>49.2905</v>
       </c>
       <c r="U12" t="n">
-        <v>-0.3214</v>
+        <v>0.8915</v>
       </c>
       <c r="V12" t="n">
-        <v>9.906000000000001</v>
+        <v>7.5311</v>
       </c>
       <c r="W12" t="n">
-        <v>12.2757</v>
+        <v>18.5642</v>
       </c>
       <c r="X12" t="n">
-        <v>8.053000000000001</v>
+        <v>-7.3446</v>
       </c>
       <c r="Y12" t="n">
-        <v>-20.0603</v>
+        <v>-16.4118</v>
       </c>
       <c r="Z12" t="n">
-        <v>-20.3008</v>
+        <v>-38.1599</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.3071</v>
+        <v>-0.8222</v>
       </c>
       <c r="AB12" t="n">
-        <v>-9.4635</v>
+        <v>-7.392</v>
       </c>
       <c r="AC12" t="n">
-        <v>-11.4618</v>
+        <v>-16.4126</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>163</v>
+        <v>177.62</v>
       </c>
       <c r="C13" t="n">
-        <v>177.5</v>
+        <v>182.24</v>
       </c>
       <c r="D13" t="n">
-        <v>161.51</v>
+        <v>150.58</v>
       </c>
       <c r="E13" t="n">
-        <v>176.94</v>
+        <v>172.52</v>
       </c>
       <c r="F13" t="n">
-        <v>72.81999999999999</v>
+        <v>75.3</v>
       </c>
       <c r="G13" t="n">
-        <v>76.31</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="H13" t="n">
-        <v>72.7</v>
+        <v>71.55</v>
       </c>
       <c r="I13" t="n">
-        <v>76.28</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>9.859999999999999</v>
+        <v>8.75</v>
       </c>
       <c r="K13" t="n">
-        <v>9.970000000000001</v>
+        <v>9.91</v>
       </c>
       <c r="L13" t="n">
-        <v>8.84</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="M13" t="n">
-        <v>8.85</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N13" t="n">
-        <v>44.82</v>
+        <v>43.14</v>
       </c>
       <c r="O13" t="n">
-        <v>44.89</v>
+        <v>45.19</v>
       </c>
       <c r="P13" t="n">
-        <v>42.57</v>
+        <v>42.79</v>
       </c>
       <c r="Q13" t="n">
-        <v>42.57</v>
+        <v>43.31</v>
       </c>
       <c r="R13" t="n">
-        <v>16.3314</v>
+        <v>-9.4003</v>
       </c>
       <c r="S13" t="n">
-        <v>22.7386</v>
+        <v>13.4254</v>
       </c>
       <c r="T13" t="n">
-        <v>35.6902</v>
+        <v>19.6726</v>
       </c>
       <c r="U13" t="n">
-        <v>6.9246</v>
+        <v>-2.5988</v>
       </c>
       <c r="V13" t="n">
-        <v>13.1919</v>
+        <v>5.0743</v>
       </c>
       <c r="W13" t="n">
-        <v>16.8147</v>
+        <v>11.2331</v>
       </c>
       <c r="X13" t="n">
-        <v>-16.5094</v>
+        <v>9.1463</v>
       </c>
       <c r="Y13" t="n">
-        <v>-23.1103</v>
+        <v>-15.566</v>
       </c>
       <c r="Z13" t="n">
-        <v>-31.8182</v>
+        <v>-22.2415</v>
       </c>
       <c r="AA13" t="n">
-        <v>-6.9101</v>
+        <v>2.5817</v>
       </c>
       <c r="AB13" t="n">
-        <v>-12.3894</v>
+        <v>-5.2919</v>
       </c>
       <c r="AC13" t="n">
-        <v>-15.233</v>
+        <v>-10.8664</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>181</v>
+        <v>183.84</v>
       </c>
       <c r="C14" t="n">
-        <v>191.29</v>
+        <v>188.49</v>
       </c>
       <c r="D14" t="n">
-        <v>178.94</v>
+        <v>172.26</v>
       </c>
       <c r="E14" t="n">
-        <v>190.42</v>
+        <v>184.24</v>
       </c>
       <c r="F14" t="n">
-        <v>76</v>
+        <v>75.81</v>
       </c>
       <c r="G14" t="n">
-        <v>77.36</v>
+        <v>77.94</v>
       </c>
       <c r="H14" t="n">
-        <v>75.55</v>
+        <v>74.19</v>
       </c>
       <c r="I14" t="n">
-        <v>76.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>8.65</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>8.77</v>
+        <v>8.98</v>
       </c>
       <c r="L14" t="n">
-        <v>8.15</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="M14" t="n">
-        <v>8.199999999999999</v>
+        <v>8.35</v>
       </c>
       <c r="N14" t="n">
-        <v>42.74</v>
+        <v>42.83</v>
       </c>
       <c r="O14" t="n">
-        <v>43</v>
+        <v>43.77</v>
       </c>
       <c r="P14" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="Q14" t="n">
         <v>41.99</v>
       </c>
-      <c r="Q14" t="n">
-        <v>42.22</v>
-      </c>
       <c r="R14" t="n">
-        <v>7.6184</v>
+        <v>6.7934</v>
       </c>
       <c r="S14" t="n">
-        <v>14.8146</v>
+        <v>4.1257</v>
       </c>
       <c r="T14" t="n">
-        <v>49.2905</v>
+        <v>11.0883</v>
       </c>
       <c r="U14" t="n">
-        <v>0.8915</v>
+        <v>3.0416</v>
       </c>
       <c r="V14" t="n">
-        <v>7.5311</v>
+        <v>1.2585</v>
       </c>
       <c r="W14" t="n">
-        <v>18.5642</v>
+        <v>7.9223</v>
       </c>
       <c r="X14" t="n">
-        <v>-7.3446</v>
+        <v>-6.7039</v>
       </c>
       <c r="Y14" t="n">
-        <v>-16.4118</v>
+        <v>-5.6497</v>
       </c>
       <c r="Z14" t="n">
-        <v>-38.1599</v>
+        <v>-14.8828</v>
       </c>
       <c r="AA14" t="n">
-        <v>-0.8222</v>
+        <v>-3.0478</v>
       </c>
       <c r="AB14" t="n">
-        <v>-7.392</v>
+        <v>-1.3625</v>
       </c>
       <c r="AC14" t="n">
-        <v>-16.4126</v>
+        <v>-7.8965</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>177.62</v>
+        <v>182.67</v>
       </c>
       <c r="C15" t="n">
-        <v>182.24</v>
+        <v>189.56</v>
       </c>
       <c r="D15" t="n">
-        <v>150.58</v>
+        <v>178.28</v>
       </c>
       <c r="E15" t="n">
-        <v>172.52</v>
+        <v>186.19</v>
       </c>
       <c r="F15" t="n">
-        <v>75.3</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>75.93000000000001</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H15" t="n">
-        <v>71.55</v>
+        <v>77.16</v>
       </c>
       <c r="I15" t="n">
-        <v>74.95999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="J15" t="n">
-        <v>8.75</v>
+        <v>8.43</v>
       </c>
       <c r="K15" t="n">
-        <v>9.91</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L15" t="n">
-        <v>8.550000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M15" t="n">
-        <v>8.949999999999999</v>
+        <v>8.27</v>
       </c>
       <c r="N15" t="n">
-        <v>43.14</v>
+        <v>41.98</v>
       </c>
       <c r="O15" t="n">
-        <v>45.19</v>
+        <v>42.06</v>
       </c>
       <c r="P15" t="n">
-        <v>42.79</v>
+        <v>40.68</v>
       </c>
       <c r="Q15" t="n">
-        <v>43.31</v>
+        <v>41.07</v>
       </c>
       <c r="R15" t="n">
-        <v>-9.4003</v>
+        <v>1.0584</v>
       </c>
       <c r="S15" t="n">
-        <v>13.4254</v>
+        <v>-2.2214</v>
       </c>
       <c r="T15" t="n">
-        <v>19.6726</v>
+        <v>22.4129</v>
       </c>
       <c r="U15" t="n">
-        <v>-2.5988</v>
+        <v>2.2139</v>
       </c>
       <c r="V15" t="n">
-        <v>5.0743</v>
+        <v>2.5858</v>
       </c>
       <c r="W15" t="n">
-        <v>11.2331</v>
+        <v>10.6672</v>
       </c>
       <c r="X15" t="n">
-        <v>9.1463</v>
+        <v>-0.9581</v>
       </c>
       <c r="Y15" t="n">
-        <v>-15.566</v>
+        <v>0.8537</v>
       </c>
       <c r="Z15" t="n">
-        <v>-22.2415</v>
+        <v>-21.9811</v>
       </c>
       <c r="AA15" t="n">
-        <v>2.5817</v>
+        <v>-2.191</v>
       </c>
       <c r="AB15" t="n">
-        <v>-5.2919</v>
+        <v>-2.7238</v>
       </c>
       <c r="AC15" t="n">
-        <v>-10.8664</v>
+        <v>-10.1902</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>183.84</v>
+        <v>167</v>
       </c>
       <c r="C16" t="n">
-        <v>188.49</v>
+        <v>174.4</v>
       </c>
       <c r="D16" t="n">
-        <v>172.26</v>
+        <v>161.14</v>
       </c>
       <c r="E16" t="n">
-        <v>184.24</v>
+        <v>164.18</v>
       </c>
       <c r="F16" t="n">
-        <v>75.81</v>
+        <v>75.73</v>
       </c>
       <c r="G16" t="n">
-        <v>77.94</v>
+        <v>77.37</v>
       </c>
       <c r="H16" t="n">
-        <v>74.19</v>
+        <v>74.23</v>
       </c>
       <c r="I16" t="n">
-        <v>77.23999999999999</v>
+        <v>75.34</v>
       </c>
       <c r="J16" t="n">
-        <v>8.380000000000001</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>8.98</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="L16" t="n">
-        <v>8.140000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M16" t="n">
-        <v>8.35</v>
+        <v>9.23</v>
       </c>
       <c r="N16" t="n">
-        <v>42.83</v>
+        <v>42.77</v>
       </c>
       <c r="O16" t="n">
-        <v>43.77</v>
+        <v>43.57</v>
       </c>
       <c r="P16" t="n">
-        <v>41.6</v>
+        <v>41.93</v>
       </c>
       <c r="Q16" t="n">
-        <v>41.99</v>
+        <v>42.98</v>
       </c>
       <c r="R16" t="n">
-        <v>6.7934</v>
+        <v>-11.8213</v>
       </c>
       <c r="S16" t="n">
-        <v>4.1257</v>
+        <v>-4.8342</v>
       </c>
       <c r="T16" t="n">
-        <v>11.0883</v>
+        <v>-7.2115</v>
       </c>
       <c r="U16" t="n">
-        <v>3.0416</v>
+        <v>-4.5725</v>
       </c>
       <c r="V16" t="n">
-        <v>1.2585</v>
+        <v>0.5069</v>
       </c>
       <c r="W16" t="n">
-        <v>7.9223</v>
+        <v>-1.2323</v>
       </c>
       <c r="X16" t="n">
-        <v>-6.7039</v>
+        <v>11.6082</v>
       </c>
       <c r="Y16" t="n">
-        <v>-5.6497</v>
+        <v>3.1285</v>
       </c>
       <c r="Z16" t="n">
-        <v>-14.8828</v>
+        <v>4.2938</v>
       </c>
       <c r="AA16" t="n">
-        <v>-3.0478</v>
+        <v>4.6506</v>
       </c>
       <c r="AB16" t="n">
-        <v>-1.3625</v>
+        <v>-0.7619</v>
       </c>
       <c r="AC16" t="n">
-        <v>-7.8965</v>
+        <v>0.9631</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>182.67</v>
+        <v>172.95</v>
       </c>
       <c r="C17" t="n">
-        <v>189.56</v>
+        <v>174.61</v>
       </c>
       <c r="D17" t="n">
-        <v>178.28</v>
+        <v>142.69</v>
       </c>
       <c r="E17" t="n">
-        <v>186.19</v>
+        <v>151.75</v>
       </c>
       <c r="F17" t="n">
-        <v>77.29000000000001</v>
+        <v>76.13</v>
       </c>
       <c r="G17" t="n">
-        <v>79.68000000000001</v>
+        <v>76.27</v>
       </c>
       <c r="H17" t="n">
-        <v>77.16</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I17" t="n">
-        <v>78.95</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>8.43</v>
+        <v>8.77</v>
       </c>
       <c r="K17" t="n">
-        <v>8.630000000000001</v>
+        <v>10.47</v>
       </c>
       <c r="L17" t="n">
-        <v>8.119999999999999</v>
+        <v>8.68</v>
       </c>
       <c r="M17" t="n">
-        <v>8.27</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="N17" t="n">
-        <v>41.98</v>
+        <v>42.51</v>
       </c>
       <c r="O17" t="n">
-        <v>42.06</v>
+        <v>44.82</v>
       </c>
       <c r="P17" t="n">
-        <v>40.68</v>
+        <v>42.44</v>
       </c>
       <c r="Q17" t="n">
-        <v>41.07</v>
+        <v>43.54</v>
       </c>
       <c r="R17" t="n">
-        <v>1.0584</v>
+        <v>-7.571</v>
       </c>
       <c r="S17" t="n">
-        <v>-2.2214</v>
+        <v>-17.6346</v>
       </c>
       <c r="T17" t="n">
-        <v>22.4129</v>
+        <v>-20.3077</v>
       </c>
       <c r="U17" t="n">
-        <v>2.2139</v>
+        <v>-1.3539</v>
       </c>
       <c r="V17" t="n">
-        <v>2.5858</v>
+        <v>-3.7804</v>
       </c>
       <c r="W17" t="n">
-        <v>10.6672</v>
+        <v>-3.4304</v>
       </c>
       <c r="X17" t="n">
-        <v>-0.9581</v>
+        <v>7.8007</v>
       </c>
       <c r="Y17" t="n">
-        <v>0.8537</v>
+        <v>19.1617</v>
       </c>
       <c r="Z17" t="n">
-        <v>-21.9811</v>
+        <v>21.3415</v>
       </c>
       <c r="AA17" t="n">
-        <v>-2.191</v>
+        <v>1.3029</v>
       </c>
       <c r="AB17" t="n">
-        <v>-2.7238</v>
+        <v>3.6914</v>
       </c>
       <c r="AC17" t="n">
-        <v>-10.1902</v>
+        <v>3.1265</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>167</v>
+        <v>141.24</v>
       </c>
       <c r="C18" t="n">
-        <v>174.4</v>
+        <v>160.6</v>
       </c>
       <c r="D18" t="n">
-        <v>161.14</v>
+        <v>135.02</v>
       </c>
       <c r="E18" t="n">
-        <v>164.18</v>
+        <v>151.89</v>
       </c>
       <c r="F18" t="n">
-        <v>75.73</v>
+        <v>72.41</v>
       </c>
       <c r="G18" t="n">
-        <v>77.37</v>
+        <v>74.5</v>
       </c>
       <c r="H18" t="n">
-        <v>74.23</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="I18" t="n">
-        <v>75.34</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>9.130000000000001</v>
+        <v>10.64</v>
       </c>
       <c r="K18" t="n">
-        <v>9.390000000000001</v>
+        <v>11.07</v>
       </c>
       <c r="L18" t="n">
-        <v>8.800000000000001</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="M18" t="n">
-        <v>9.23</v>
+        <v>9.93</v>
       </c>
       <c r="N18" t="n">
-        <v>42.77</v>
+        <v>44.68</v>
       </c>
       <c r="O18" t="n">
-        <v>43.57</v>
+        <v>45.53</v>
       </c>
       <c r="P18" t="n">
-        <v>41.93</v>
+        <v>43.46</v>
       </c>
       <c r="Q18" t="n">
-        <v>42.98</v>
+        <v>44.37</v>
       </c>
       <c r="R18" t="n">
-        <v>-11.8213</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="S18" t="n">
-        <v>-4.8342</v>
+        <v>-18.422</v>
       </c>
       <c r="T18" t="n">
-        <v>-7.2115</v>
+        <v>-11.958</v>
       </c>
       <c r="U18" t="n">
-        <v>-4.5725</v>
+        <v>-1.8703</v>
       </c>
       <c r="V18" t="n">
-        <v>0.5069</v>
+        <v>-7.6251</v>
       </c>
       <c r="W18" t="n">
-        <v>-1.2323</v>
+        <v>-2.7081</v>
       </c>
       <c r="X18" t="n">
-        <v>11.6082</v>
+        <v>-0.201</v>
       </c>
       <c r="Y18" t="n">
-        <v>3.1285</v>
+        <v>20.0726</v>
       </c>
       <c r="Z18" t="n">
-        <v>4.2938</v>
+        <v>10.9497</v>
       </c>
       <c r="AA18" t="n">
-        <v>4.6506</v>
+        <v>1.9063</v>
       </c>
       <c r="AB18" t="n">
-        <v>-0.7619</v>
+        <v>8.0351</v>
       </c>
       <c r="AC18" t="n">
-        <v>0.9631</v>
+        <v>2.4475</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>172.95</v>
+        <v>161</v>
       </c>
       <c r="C19" t="n">
-        <v>174.61</v>
+        <v>173.7</v>
       </c>
       <c r="D19" t="n">
-        <v>142.69</v>
+        <v>161</v>
       </c>
       <c r="E19" t="n">
-        <v>151.75</v>
+        <v>173.2</v>
       </c>
       <c r="F19" t="n">
-        <v>76.13</v>
+        <v>74.09</v>
       </c>
       <c r="G19" t="n">
-        <v>76.27</v>
+        <v>76.53</v>
       </c>
       <c r="H19" t="n">
-        <v>72.09999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="I19" t="n">
-        <v>74.31999999999999</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J19" t="n">
-        <v>8.77</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K19" t="n">
-        <v>10.47</v>
+        <v>9.35</v>
       </c>
       <c r="L19" t="n">
-        <v>8.68</v>
+        <v>8.51</v>
       </c>
       <c r="M19" t="n">
-        <v>9.949999999999999</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N19" t="n">
-        <v>42.51</v>
+        <v>43.67</v>
       </c>
       <c r="O19" t="n">
-        <v>44.82</v>
+        <v>43.97</v>
       </c>
       <c r="P19" t="n">
-        <v>42.44</v>
+        <v>42.19</v>
       </c>
       <c r="Q19" t="n">
-        <v>43.54</v>
+        <v>42.19</v>
       </c>
       <c r="R19" t="n">
-        <v>-7.571</v>
+        <v>14.0299</v>
       </c>
       <c r="S19" t="n">
-        <v>-17.6346</v>
+        <v>5.494</v>
       </c>
       <c r="T19" t="n">
-        <v>-20.3077</v>
+        <v>-5.9922</v>
       </c>
       <c r="U19" t="n">
-        <v>-1.3539</v>
+        <v>4.9088</v>
       </c>
       <c r="V19" t="n">
-        <v>-3.7804</v>
+        <v>1.553</v>
       </c>
       <c r="W19" t="n">
-        <v>-3.4304</v>
+        <v>-0.9451000000000001</v>
       </c>
       <c r="X19" t="n">
-        <v>7.8007</v>
+        <v>-13.998</v>
       </c>
       <c r="Y19" t="n">
-        <v>19.1617</v>
+        <v>-7.4756</v>
       </c>
       <c r="Z19" t="n">
-        <v>21.3415</v>
+        <v>2.2754</v>
       </c>
       <c r="AA19" t="n">
-        <v>1.3029</v>
+        <v>-4.9132</v>
       </c>
       <c r="AB19" t="n">
-        <v>3.6914</v>
+        <v>-1.8381</v>
       </c>
       <c r="AC19" t="n">
-        <v>3.1265</v>
+        <v>0.4763</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>141.24</v>
+        <v>171.26</v>
       </c>
       <c r="C20" t="n">
-        <v>160.6</v>
+        <v>179.97</v>
       </c>
       <c r="D20" t="n">
-        <v>135.02</v>
+        <v>168.23</v>
       </c>
       <c r="E20" t="n">
-        <v>151.89</v>
+        <v>178.39</v>
       </c>
       <c r="F20" t="n">
-        <v>72.41</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>74.5</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H20" t="n">
-        <v>70.95999999999999</v>
+        <v>74.47</v>
       </c>
       <c r="I20" t="n">
-        <v>72.93000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J20" t="n">
-        <v>10.64</v>
+        <v>8.65</v>
       </c>
       <c r="K20" t="n">
-        <v>11.07</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L20" t="n">
-        <v>9.369999999999999</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M20" t="n">
-        <v>9.93</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N20" t="n">
-        <v>44.68</v>
+        <v>42.94</v>
       </c>
       <c r="O20" t="n">
-        <v>45.53</v>
+        <v>43.33</v>
       </c>
       <c r="P20" t="n">
-        <v>43.46</v>
+        <v>41.5</v>
       </c>
       <c r="Q20" t="n">
-        <v>44.37</v>
+        <v>41.96</v>
       </c>
       <c r="R20" t="n">
-        <v>0.09229999999999999</v>
+        <v>2.9965</v>
       </c>
       <c r="S20" t="n">
-        <v>-18.422</v>
+        <v>17.5552</v>
       </c>
       <c r="T20" t="n">
-        <v>-11.958</v>
+        <v>-4.1893</v>
       </c>
       <c r="U20" t="n">
-        <v>-1.8703</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="V20" t="n">
-        <v>-7.6251</v>
+        <v>3.5388</v>
       </c>
       <c r="W20" t="n">
-        <v>-2.7081</v>
+        <v>-2.5332</v>
       </c>
       <c r="X20" t="n">
-        <v>-0.201</v>
+        <v>-2.9274</v>
       </c>
       <c r="Y20" t="n">
-        <v>20.0726</v>
+        <v>-16.6834</v>
       </c>
       <c r="Z20" t="n">
-        <v>10.9497</v>
+        <v>0.2418</v>
       </c>
       <c r="AA20" t="n">
-        <v>1.9063</v>
+        <v>-0.5452</v>
       </c>
       <c r="AB20" t="n">
-        <v>8.0351</v>
+        <v>-3.6288</v>
       </c>
       <c r="AC20" t="n">
-        <v>2.4475</v>
+        <v>2.167</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>161</v>
+        <v>184.8</v>
       </c>
       <c r="C21" t="n">
-        <v>173.7</v>
+        <v>195.27</v>
       </c>
       <c r="D21" t="n">
-        <v>161</v>
+        <v>183.34</v>
       </c>
       <c r="E21" t="n">
-        <v>173.2</v>
+        <v>190.56</v>
       </c>
       <c r="F21" t="n">
-        <v>74.09</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>76.53</v>
+        <v>79.33</v>
       </c>
       <c r="H21" t="n">
-        <v>73.62</v>
+        <v>77.33</v>
       </c>
       <c r="I21" t="n">
-        <v>76.51000000000001</v>
+        <v>77.84</v>
       </c>
       <c r="J21" t="n">
-        <v>9.300000000000001</v>
+        <v>8</v>
       </c>
       <c r="K21" t="n">
-        <v>9.35</v>
+        <v>8.06</v>
       </c>
       <c r="L21" t="n">
-        <v>8.51</v>
+        <v>7.5</v>
       </c>
       <c r="M21" t="n">
-        <v>8.539999999999999</v>
+        <v>7.73</v>
       </c>
       <c r="N21" t="n">
-        <v>43.67</v>
+        <v>41.4</v>
       </c>
       <c r="O21" t="n">
-        <v>43.97</v>
+        <v>41.78</v>
       </c>
       <c r="P21" t="n">
-        <v>42.19</v>
+        <v>40.68</v>
       </c>
       <c r="Q21" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="R21" t="n">
-        <v>14.0299</v>
+        <v>6.8221</v>
       </c>
       <c r="S21" t="n">
-        <v>5.494</v>
+        <v>25.4592</v>
       </c>
       <c r="T21" t="n">
-        <v>-5.9922</v>
+        <v>16.0677</v>
       </c>
       <c r="U21" t="n">
-        <v>4.9088</v>
+        <v>1.1566</v>
       </c>
       <c r="V21" t="n">
-        <v>1.553</v>
+        <v>6.7325</v>
       </c>
       <c r="W21" t="n">
-        <v>-0.9451000000000001</v>
+        <v>3.3183</v>
       </c>
       <c r="X21" t="n">
-        <v>-13.998</v>
+        <v>-6.7551</v>
       </c>
       <c r="Y21" t="n">
-        <v>-7.4756</v>
+        <v>-22.1551</v>
       </c>
       <c r="Z21" t="n">
-        <v>2.2754</v>
+        <v>-16.2514</v>
       </c>
       <c r="AA21" t="n">
-        <v>-4.9132</v>
+        <v>-1.0963</v>
       </c>
       <c r="AB21" t="n">
-        <v>-1.8381</v>
+        <v>-6.4683</v>
       </c>
       <c r="AC21" t="n">
-        <v>0.4763</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>171.26</v>
-      </c>
-      <c r="C22" t="n">
-        <v>179.97</v>
-      </c>
-      <c r="D22" t="n">
-        <v>168.23</v>
-      </c>
-      <c r="E22" t="n">
-        <v>178.39</v>
-      </c>
-      <c r="F22" t="n">
-        <v>75.18000000000001</v>
-      </c>
-      <c r="G22" t="n">
-        <v>77.79000000000001</v>
-      </c>
-      <c r="H22" t="n">
-        <v>74.47</v>
-      </c>
-      <c r="I22" t="n">
-        <v>76.95</v>
-      </c>
-      <c r="J22" t="n">
-        <v>8.65</v>
-      </c>
-      <c r="K22" t="n">
-        <v>8.779999999999999</v>
-      </c>
-      <c r="L22" t="n">
-        <v>8.210000000000001</v>
-      </c>
-      <c r="M22" t="n">
-        <v>8.289999999999999</v>
-      </c>
-      <c r="N22" t="n">
-        <v>42.94</v>
-      </c>
-      <c r="O22" t="n">
-        <v>43.33</v>
-      </c>
-      <c r="P22" t="n">
-        <v>41.5</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>41.96</v>
-      </c>
-      <c r="R22" t="n">
-        <v>2.9965</v>
-      </c>
-      <c r="S22" t="n">
-        <v>17.5552</v>
-      </c>
-      <c r="T22" t="n">
-        <v>-4.1893</v>
-      </c>
-      <c r="U22" t="n">
-        <v>0.5750999999999999</v>
-      </c>
-      <c r="V22" t="n">
-        <v>3.5388</v>
-      </c>
-      <c r="W22" t="n">
-        <v>-2.5332</v>
-      </c>
-      <c r="X22" t="n">
-        <v>-2.9274</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>-16.6834</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>0.2418</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>-0.5452</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>-3.6288</v>
-      </c>
-      <c r="AC22" t="n">
-        <v>2.167</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>184.8</v>
-      </c>
-      <c r="C23" t="n">
-        <v>195.27</v>
-      </c>
-      <c r="D23" t="n">
-        <v>183.34</v>
-      </c>
-      <c r="E23" t="n">
-        <v>190.56</v>
-      </c>
-      <c r="F23" t="n">
-        <v>78.04000000000001</v>
-      </c>
-      <c r="G23" t="n">
-        <v>79.33</v>
-      </c>
-      <c r="H23" t="n">
-        <v>77.33</v>
-      </c>
-      <c r="I23" t="n">
-        <v>77.84</v>
-      </c>
-      <c r="J23" t="n">
-        <v>8</v>
-      </c>
-      <c r="K23" t="n">
-        <v>8.06</v>
-      </c>
-      <c r="L23" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="M23" t="n">
-        <v>7.73</v>
-      </c>
-      <c r="N23" t="n">
-        <v>41.4</v>
-      </c>
-      <c r="O23" t="n">
-        <v>41.78</v>
-      </c>
-      <c r="P23" t="n">
-        <v>40.68</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>41.5</v>
-      </c>
-      <c r="R23" t="n">
-        <v>6.8221</v>
-      </c>
-      <c r="S23" t="n">
-        <v>25.4592</v>
-      </c>
-      <c r="T23" t="n">
-        <v>16.0677</v>
-      </c>
-      <c r="U23" t="n">
-        <v>1.1566</v>
-      </c>
-      <c r="V23" t="n">
-        <v>6.7325</v>
-      </c>
-      <c r="W23" t="n">
-        <v>3.3183</v>
-      </c>
-      <c r="X23" t="n">
-        <v>-6.7551</v>
-      </c>
-      <c r="Y23" t="n">
-        <v>-22.1551</v>
-      </c>
-      <c r="Z23" t="n">
-        <v>-16.2514</v>
-      </c>
-      <c r="AA23" t="n">
-        <v>-1.0963</v>
-      </c>
-      <c r="AB23" t="n">
-        <v>-6.4683</v>
-      </c>
-      <c r="AC23" t="n">
         <v>-3.4435</v>
       </c>
     </row>
@@ -2503,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-05-26 23:10
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC21"/>
+  <dimension ref="A1:AC22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2275,6 +2275,97 @@
       </c>
       <c r="AC21" t="n">
         <v>-3.4435</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>211.38</v>
+      </c>
+      <c r="C22" t="n">
+        <v>228.5</v>
+      </c>
+      <c r="D22" t="n">
+        <v>209.89</v>
+      </c>
+      <c r="E22" t="n">
+        <v>225.79</v>
+      </c>
+      <c r="F22" t="n">
+        <v>80.56999999999999</v>
+      </c>
+      <c r="G22" t="n">
+        <v>82.27</v>
+      </c>
+      <c r="H22" t="n">
+        <v>79.98</v>
+      </c>
+      <c r="I22" t="n">
+        <v>81.95</v>
+      </c>
+      <c r="J22" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="K22" t="n">
+        <v>6.95</v>
+      </c>
+      <c r="L22" t="n">
+        <v>6.19</v>
+      </c>
+      <c r="M22" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="N22" t="n">
+        <v>40.045</v>
+      </c>
+      <c r="O22" t="n">
+        <v>40.3519</v>
+      </c>
+      <c r="P22" t="n">
+        <v>39.1399</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>39.28</v>
+      </c>
+      <c r="R22" t="n">
+        <v>18.4876</v>
+      </c>
+      <c r="S22" t="n">
+        <v>30.3637</v>
+      </c>
+      <c r="T22" t="n">
+        <v>48.7908</v>
+      </c>
+      <c r="U22" t="n">
+        <v>5.2801</v>
+      </c>
+      <c r="V22" t="n">
+        <v>7.1102</v>
+      </c>
+      <c r="W22" t="n">
+        <v>10.2664</v>
+      </c>
+      <c r="X22" t="n">
+        <v>-18.6287</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>-26.3466</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>-36.7839</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>-5.3494</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>-6.8974</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>-9.7841</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-05-27 23:18
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>128.33</v>
+        <v>108.75</v>
       </c>
       <c r="C2" t="n">
-        <v>129.59</v>
+        <v>115.62</v>
       </c>
       <c r="D2" t="n">
-        <v>117.79</v>
+        <v>103.99</v>
       </c>
       <c r="E2" t="n">
-        <v>123.39</v>
+        <v>109.56</v>
       </c>
       <c r="F2" t="n">
-        <v>62.41</v>
+        <v>60.72</v>
       </c>
       <c r="G2" t="n">
-        <v>62.7</v>
+        <v>61.33</v>
       </c>
       <c r="H2" t="n">
-        <v>61.64</v>
+        <v>59.68</v>
       </c>
       <c r="I2" t="n">
-        <v>62.64</v>
+        <v>60.74</v>
       </c>
       <c r="J2" t="n">
-        <v>13.51</v>
+        <v>15.71</v>
       </c>
       <c r="K2" t="n">
-        <v>14.63</v>
+        <v>16.27</v>
       </c>
       <c r="L2" t="n">
-        <v>13.41</v>
+        <v>14.93</v>
       </c>
       <c r="M2" t="n">
-        <v>14.03</v>
+        <v>15.59</v>
       </c>
       <c r="N2" t="n">
-        <v>52.67</v>
+        <v>54.09</v>
       </c>
       <c r="O2" t="n">
-        <v>53.31</v>
+        <v>54.96</v>
       </c>
       <c r="P2" t="n">
-        <v>52.42</v>
+        <v>53.58</v>
       </c>
       <c r="Q2" t="n">
-        <v>52.45</v>
+        <v>54.05</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>108.75</v>
+        <v>114.76</v>
       </c>
       <c r="C3" t="n">
-        <v>115.62</v>
+        <v>118.32</v>
       </c>
       <c r="D3" t="n">
-        <v>103.99</v>
+        <v>112.3</v>
       </c>
       <c r="E3" t="n">
-        <v>109.56</v>
+        <v>117.97</v>
       </c>
       <c r="F3" t="n">
-        <v>60.72</v>
+        <v>61</v>
       </c>
       <c r="G3" t="n">
-        <v>61.33</v>
+        <v>61.87</v>
       </c>
       <c r="H3" t="n">
-        <v>59.68</v>
+        <v>60.45</v>
       </c>
       <c r="I3" t="n">
-        <v>60.74</v>
+        <v>61.86</v>
       </c>
       <c r="J3" t="n">
-        <v>15.71</v>
+        <v>14.91</v>
       </c>
       <c r="K3" t="n">
-        <v>16.27</v>
+        <v>15.24</v>
       </c>
       <c r="L3" t="n">
-        <v>14.93</v>
+        <v>14.38</v>
       </c>
       <c r="M3" t="n">
-        <v>15.59</v>
+        <v>14.4</v>
       </c>
       <c r="N3" t="n">
-        <v>54.09</v>
+        <v>53.84</v>
       </c>
       <c r="O3" t="n">
-        <v>54.96</v>
+        <v>54.33</v>
       </c>
       <c r="P3" t="n">
-        <v>53.58</v>
+        <v>53.06</v>
       </c>
       <c r="Q3" t="n">
-        <v>54.05</v>
+        <v>53.08</v>
       </c>
       <c r="R3" t="n">
-        <v>-11.2084</v>
+        <v>7.6762</v>
       </c>
       <c r="U3" t="n">
-        <v>-3.0332</v>
+        <v>1.8439</v>
       </c>
       <c r="X3" t="n">
-        <v>11.119</v>
+        <v>-7.6331</v>
       </c>
       <c r="AA3" t="n">
-        <v>3.0505</v>
+        <v>-1.7946</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>114.76</v>
+        <v>122.81</v>
       </c>
       <c r="C4" t="n">
-        <v>118.32</v>
+        <v>127.45</v>
       </c>
       <c r="D4" t="n">
-        <v>112.3</v>
+        <v>117.5</v>
       </c>
       <c r="E4" t="n">
-        <v>117.97</v>
+        <v>126.98</v>
       </c>
       <c r="F4" t="n">
-        <v>61</v>
+        <v>62.89</v>
       </c>
       <c r="G4" t="n">
-        <v>61.87</v>
+        <v>63.8</v>
       </c>
       <c r="H4" t="n">
-        <v>60.45</v>
+        <v>60.7</v>
       </c>
       <c r="I4" t="n">
-        <v>61.86</v>
+        <v>63.54</v>
       </c>
       <c r="J4" t="n">
-        <v>14.91</v>
+        <v>13.84</v>
       </c>
       <c r="K4" t="n">
-        <v>15.24</v>
+        <v>14.49</v>
       </c>
       <c r="L4" t="n">
-        <v>14.38</v>
+        <v>13.25</v>
       </c>
       <c r="M4" t="n">
-        <v>14.4</v>
+        <v>13.3</v>
       </c>
       <c r="N4" t="n">
-        <v>53.84</v>
+        <v>52.21</v>
       </c>
       <c r="O4" t="n">
-        <v>54.33</v>
+        <v>54.09</v>
       </c>
       <c r="P4" t="n">
-        <v>53.06</v>
+        <v>51.4</v>
       </c>
       <c r="Q4" t="n">
-        <v>53.08</v>
+        <v>51.65</v>
       </c>
       <c r="R4" t="n">
-        <v>7.6762</v>
+        <v>7.6375</v>
       </c>
       <c r="U4" t="n">
-        <v>1.8439</v>
+        <v>2.7158</v>
       </c>
       <c r="X4" t="n">
-        <v>-7.6331</v>
+        <v>-7.6389</v>
       </c>
       <c r="AA4" t="n">
-        <v>-1.7946</v>
+        <v>-2.694</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>122.81</v>
+        <v>124.39</v>
       </c>
       <c r="C5" t="n">
-        <v>127.45</v>
+        <v>131.38</v>
       </c>
       <c r="D5" t="n">
-        <v>117.5</v>
+        <v>121.66</v>
       </c>
       <c r="E5" t="n">
-        <v>126.98</v>
+        <v>130.4</v>
       </c>
       <c r="F5" t="n">
-        <v>62.89</v>
+        <v>63.89</v>
       </c>
       <c r="G5" t="n">
-        <v>63.8</v>
+        <v>65.84</v>
       </c>
       <c r="H5" t="n">
-        <v>60.7</v>
+        <v>63.81</v>
       </c>
       <c r="I5" t="n">
-        <v>63.54</v>
+        <v>65.3</v>
       </c>
       <c r="J5" t="n">
-        <v>13.84</v>
+        <v>13.61</v>
       </c>
       <c r="K5" t="n">
-        <v>14.49</v>
+        <v>13.89</v>
       </c>
       <c r="L5" t="n">
-        <v>13.25</v>
+        <v>12.87</v>
       </c>
       <c r="M5" t="n">
-        <v>13.3</v>
+        <v>12.98</v>
       </c>
       <c r="N5" t="n">
-        <v>52.21</v>
+        <v>51.36</v>
       </c>
       <c r="O5" t="n">
-        <v>54.09</v>
+        <v>51.45</v>
       </c>
       <c r="P5" t="n">
-        <v>51.4</v>
+        <v>49.79</v>
       </c>
       <c r="Q5" t="n">
-        <v>51.65</v>
+        <v>50.22</v>
       </c>
       <c r="R5" t="n">
-        <v>7.6375</v>
+        <v>2.6933</v>
       </c>
       <c r="S5" t="n">
-        <v>2.9095</v>
+        <v>19.0215</v>
       </c>
       <c r="U5" t="n">
-        <v>2.7158</v>
+        <v>2.7699</v>
       </c>
       <c r="V5" t="n">
-        <v>1.4368</v>
+        <v>7.5074</v>
       </c>
       <c r="X5" t="n">
-        <v>-7.6389</v>
+        <v>-2.406</v>
       </c>
       <c r="Y5" t="n">
-        <v>-5.2031</v>
+        <v>-16.7415</v>
       </c>
       <c r="AA5" t="n">
-        <v>-2.694</v>
+        <v>-2.7686</v>
       </c>
       <c r="AB5" t="n">
-        <v>-1.5253</v>
+        <v>-7.086</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>124.39</v>
+        <v>132.2</v>
       </c>
       <c r="C6" t="n">
-        <v>131.38</v>
+        <v>133.67</v>
       </c>
       <c r="D6" t="n">
-        <v>121.66</v>
+        <v>123.8</v>
       </c>
       <c r="E6" t="n">
-        <v>130.4</v>
+        <v>127.55</v>
       </c>
       <c r="F6" t="n">
-        <v>63.89</v>
+        <v>65.44</v>
       </c>
       <c r="G6" t="n">
-        <v>65.84</v>
+        <v>66.05</v>
       </c>
       <c r="H6" t="n">
-        <v>63.81</v>
+        <v>63.78</v>
       </c>
       <c r="I6" t="n">
-        <v>65.3</v>
+        <v>64.91</v>
       </c>
       <c r="J6" t="n">
-        <v>13.61</v>
+        <v>12.8</v>
       </c>
       <c r="K6" t="n">
-        <v>13.89</v>
+        <v>13.64</v>
       </c>
       <c r="L6" t="n">
-        <v>12.87</v>
+        <v>12.65</v>
       </c>
       <c r="M6" t="n">
-        <v>12.98</v>
+        <v>13.26</v>
       </c>
       <c r="N6" t="n">
-        <v>51.36</v>
+        <v>50.12</v>
       </c>
       <c r="O6" t="n">
-        <v>51.45</v>
+        <v>51.43</v>
       </c>
       <c r="P6" t="n">
-        <v>49.79</v>
+        <v>49.65</v>
       </c>
       <c r="Q6" t="n">
-        <v>50.22</v>
+        <v>50.51</v>
       </c>
       <c r="R6" t="n">
-        <v>2.6933</v>
+        <v>-2.1856</v>
       </c>
       <c r="S6" t="n">
-        <v>19.0215</v>
+        <v>8.120699999999999</v>
       </c>
       <c r="U6" t="n">
-        <v>2.7699</v>
+        <v>-0.5972</v>
       </c>
       <c r="V6" t="n">
-        <v>7.5074</v>
+        <v>4.9305</v>
       </c>
       <c r="X6" t="n">
-        <v>-2.406</v>
+        <v>2.1572</v>
       </c>
       <c r="Y6" t="n">
-        <v>-16.7415</v>
+        <v>-7.9167</v>
       </c>
       <c r="AA6" t="n">
-        <v>-2.7686</v>
+        <v>0.5775</v>
       </c>
       <c r="AB6" t="n">
-        <v>-7.086</v>
+        <v>-4.8417</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>132.2</v>
+        <v>135</v>
       </c>
       <c r="C7" t="n">
-        <v>133.67</v>
+        <v>147.26</v>
       </c>
       <c r="D7" t="n">
-        <v>123.8</v>
+        <v>134.02</v>
       </c>
       <c r="E7" t="n">
-        <v>127.55</v>
+        <v>144.16</v>
       </c>
       <c r="F7" t="n">
-        <v>65.44</v>
+        <v>66.37</v>
       </c>
       <c r="G7" t="n">
-        <v>66.05</v>
+        <v>67.77</v>
       </c>
       <c r="H7" t="n">
-        <v>63.78</v>
+        <v>66.25</v>
       </c>
       <c r="I7" t="n">
-        <v>64.91</v>
+        <v>67.39</v>
       </c>
       <c r="J7" t="n">
-        <v>12.8</v>
+        <v>12.5</v>
       </c>
       <c r="K7" t="n">
-        <v>13.64</v>
+        <v>12.59</v>
       </c>
       <c r="L7" t="n">
-        <v>12.65</v>
+        <v>11.21</v>
       </c>
       <c r="M7" t="n">
-        <v>13.26</v>
+        <v>11.51</v>
       </c>
       <c r="N7" t="n">
-        <v>50.12</v>
+        <v>49.4</v>
       </c>
       <c r="O7" t="n">
-        <v>51.43</v>
+        <v>49.49</v>
       </c>
       <c r="P7" t="n">
-        <v>49.65</v>
+        <v>48.3</v>
       </c>
       <c r="Q7" t="n">
-        <v>50.51</v>
+        <v>48.59</v>
       </c>
       <c r="R7" t="n">
-        <v>-2.1856</v>
+        <v>13.0223</v>
       </c>
       <c r="S7" t="n">
-        <v>8.120699999999999</v>
+        <v>13.5297</v>
       </c>
       <c r="T7" t="n">
-        <v>3.3714</v>
+        <v>31.5809</v>
       </c>
       <c r="U7" t="n">
-        <v>-0.5972</v>
+        <v>3.8207</v>
       </c>
       <c r="V7" t="n">
-        <v>4.9305</v>
+        <v>6.0592</v>
       </c>
       <c r="W7" t="n">
-        <v>3.6239</v>
+        <v>10.9483</v>
       </c>
       <c r="X7" t="n">
-        <v>2.1572</v>
+        <v>-13.1976</v>
       </c>
       <c r="Y7" t="n">
-        <v>-7.9167</v>
+        <v>-13.4586</v>
       </c>
       <c r="Z7" t="n">
-        <v>-5.4882</v>
+        <v>-26.1706</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.5775</v>
+        <v>-3.8012</v>
       </c>
       <c r="AB7" t="n">
-        <v>-4.8417</v>
+        <v>-5.9245</v>
       </c>
       <c r="AC7" t="n">
-        <v>-3.6988</v>
+        <v>-10.1018</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>135</v>
+        <v>157.84</v>
       </c>
       <c r="C8" t="n">
-        <v>147.26</v>
+        <v>166</v>
       </c>
       <c r="D8" t="n">
-        <v>134.02</v>
+        <v>149.06</v>
       </c>
       <c r="E8" t="n">
-        <v>144.16</v>
+        <v>165.85</v>
       </c>
       <c r="F8" t="n">
-        <v>66.37</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>67.77</v>
+        <v>71.66</v>
       </c>
       <c r="H8" t="n">
-        <v>66.25</v>
+        <v>68.88</v>
       </c>
       <c r="I8" t="n">
-        <v>67.39</v>
+        <v>71.56999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>12.5</v>
+        <v>10.43</v>
       </c>
       <c r="K8" t="n">
-        <v>12.59</v>
+        <v>11.14</v>
       </c>
       <c r="L8" t="n">
-        <v>11.21</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>11.51</v>
+        <v>9.81</v>
       </c>
       <c r="N8" t="n">
-        <v>49.4</v>
+        <v>47.26</v>
       </c>
       <c r="O8" t="n">
-        <v>49.49</v>
+        <v>47.54</v>
       </c>
       <c r="P8" t="n">
-        <v>48.3</v>
+        <v>45.52</v>
       </c>
       <c r="Q8" t="n">
-        <v>48.59</v>
+        <v>45.59</v>
       </c>
       <c r="R8" t="n">
-        <v>13.0223</v>
+        <v>15.0458</v>
       </c>
       <c r="S8" t="n">
-        <v>13.5297</v>
+        <v>27.1856</v>
       </c>
       <c r="T8" t="n">
-        <v>31.5809</v>
+        <v>40.5866</v>
       </c>
       <c r="U8" t="n">
-        <v>3.8207</v>
+        <v>6.2027</v>
       </c>
       <c r="V8" t="n">
-        <v>6.0592</v>
+        <v>9.601800000000001</v>
       </c>
       <c r="W8" t="n">
-        <v>10.9483</v>
+        <v>15.6967</v>
       </c>
       <c r="X8" t="n">
-        <v>-13.1976</v>
+        <v>-14.7698</v>
       </c>
       <c r="Y8" t="n">
-        <v>-13.4586</v>
+        <v>-24.4222</v>
       </c>
       <c r="Z8" t="n">
-        <v>-26.1706</v>
+        <v>-31.875</v>
       </c>
       <c r="AA8" t="n">
-        <v>-3.8012</v>
+        <v>-6.1741</v>
       </c>
       <c r="AB8" t="n">
-        <v>-5.9245</v>
+        <v>-9.2194</v>
       </c>
       <c r="AC8" t="n">
-        <v>-10.1018</v>
+        <v>-14.1108</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>157.84</v>
+        <v>162.12</v>
       </c>
       <c r="C9" t="n">
-        <v>166</v>
+        <v>162.9</v>
       </c>
       <c r="D9" t="n">
-        <v>149.06</v>
+        <v>147.61</v>
       </c>
       <c r="E9" t="n">
-        <v>165.85</v>
+        <v>152.1</v>
       </c>
       <c r="F9" t="n">
-        <v>69.26000000000001</v>
+        <v>71.87</v>
       </c>
       <c r="G9" t="n">
-        <v>71.66</v>
+        <v>73.3</v>
       </c>
       <c r="H9" t="n">
-        <v>68.88</v>
+        <v>70.38</v>
       </c>
       <c r="I9" t="n">
-        <v>71.56999999999999</v>
+        <v>71.34</v>
       </c>
       <c r="J9" t="n">
-        <v>10.43</v>
+        <v>10.02</v>
       </c>
       <c r="K9" t="n">
-        <v>11.14</v>
+        <v>10.88</v>
       </c>
       <c r="L9" t="n">
-        <v>9.800000000000001</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="M9" t="n">
-        <v>9.81</v>
+        <v>10.6</v>
       </c>
       <c r="N9" t="n">
-        <v>47.26</v>
+        <v>45.41</v>
       </c>
       <c r="O9" t="n">
-        <v>47.54</v>
+        <v>46.36</v>
       </c>
       <c r="P9" t="n">
-        <v>45.52</v>
+        <v>44.5</v>
       </c>
       <c r="Q9" t="n">
-        <v>45.59</v>
+        <v>45.73</v>
       </c>
       <c r="R9" t="n">
-        <v>15.0458</v>
+        <v>-8.2906</v>
       </c>
       <c r="S9" t="n">
-        <v>27.1856</v>
+        <v>19.2474</v>
       </c>
       <c r="T9" t="n">
-        <v>40.5866</v>
+        <v>19.7826</v>
       </c>
       <c r="U9" t="n">
-        <v>6.2027</v>
+        <v>-0.3214</v>
       </c>
       <c r="V9" t="n">
-        <v>9.601800000000001</v>
+        <v>9.906000000000001</v>
       </c>
       <c r="W9" t="n">
-        <v>15.6967</v>
+        <v>12.2757</v>
       </c>
       <c r="X9" t="n">
-        <v>-14.7698</v>
+        <v>8.053000000000001</v>
       </c>
       <c r="Y9" t="n">
-        <v>-24.4222</v>
+        <v>-20.0603</v>
       </c>
       <c r="Z9" t="n">
-        <v>-31.875</v>
+        <v>-20.3008</v>
       </c>
       <c r="AA9" t="n">
-        <v>-6.1741</v>
+        <v>0.3071</v>
       </c>
       <c r="AB9" t="n">
-        <v>-9.2194</v>
+        <v>-9.4635</v>
       </c>
       <c r="AC9" t="n">
-        <v>-14.1108</v>
+        <v>-11.4618</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>162.12</v>
+        <v>163</v>
       </c>
       <c r="C10" t="n">
-        <v>162.9</v>
+        <v>177.5</v>
       </c>
       <c r="D10" t="n">
-        <v>147.61</v>
+        <v>161.51</v>
       </c>
       <c r="E10" t="n">
-        <v>152.1</v>
+        <v>176.94</v>
       </c>
       <c r="F10" t="n">
-        <v>71.87</v>
+        <v>72.81999999999999</v>
       </c>
       <c r="G10" t="n">
-        <v>73.3</v>
+        <v>76.31</v>
       </c>
       <c r="H10" t="n">
-        <v>70.38</v>
+        <v>72.7</v>
       </c>
       <c r="I10" t="n">
-        <v>71.34</v>
+        <v>76.28</v>
       </c>
       <c r="J10" t="n">
-        <v>10.02</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="K10" t="n">
-        <v>10.88</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="L10" t="n">
-        <v>9.970000000000001</v>
+        <v>8.84</v>
       </c>
       <c r="M10" t="n">
-        <v>10.6</v>
+        <v>8.85</v>
       </c>
       <c r="N10" t="n">
-        <v>45.41</v>
+        <v>44.82</v>
       </c>
       <c r="O10" t="n">
-        <v>46.36</v>
+        <v>44.89</v>
       </c>
       <c r="P10" t="n">
-        <v>44.5</v>
+        <v>42.57</v>
       </c>
       <c r="Q10" t="n">
-        <v>45.73</v>
+        <v>42.57</v>
       </c>
       <c r="R10" t="n">
-        <v>-8.2906</v>
+        <v>16.3314</v>
       </c>
       <c r="S10" t="n">
-        <v>19.2474</v>
+        <v>22.7386</v>
       </c>
       <c r="T10" t="n">
-        <v>19.7826</v>
+        <v>35.6902</v>
       </c>
       <c r="U10" t="n">
-        <v>-0.3214</v>
+        <v>6.9246</v>
       </c>
       <c r="V10" t="n">
-        <v>9.906000000000001</v>
+        <v>13.1919</v>
       </c>
       <c r="W10" t="n">
-        <v>12.2757</v>
+        <v>16.8147</v>
       </c>
       <c r="X10" t="n">
-        <v>8.053000000000001</v>
+        <v>-16.5094</v>
       </c>
       <c r="Y10" t="n">
-        <v>-20.0603</v>
+        <v>-23.1103</v>
       </c>
       <c r="Z10" t="n">
-        <v>-20.3008</v>
+        <v>-31.8182</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.3071</v>
+        <v>-6.9101</v>
       </c>
       <c r="AB10" t="n">
-        <v>-9.4635</v>
+        <v>-12.3894</v>
       </c>
       <c r="AC10" t="n">
-        <v>-11.4618</v>
+        <v>-15.233</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="C11" t="n">
-        <v>177.5</v>
+        <v>191.29</v>
       </c>
       <c r="D11" t="n">
-        <v>161.51</v>
+        <v>178.94</v>
       </c>
       <c r="E11" t="n">
-        <v>176.94</v>
+        <v>190.42</v>
       </c>
       <c r="F11" t="n">
-        <v>72.81999999999999</v>
+        <v>76</v>
       </c>
       <c r="G11" t="n">
-        <v>76.31</v>
+        <v>77.36</v>
       </c>
       <c r="H11" t="n">
-        <v>72.7</v>
+        <v>75.55</v>
       </c>
       <c r="I11" t="n">
-        <v>76.28</v>
+        <v>76.95999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>9.859999999999999</v>
+        <v>8.65</v>
       </c>
       <c r="K11" t="n">
-        <v>9.970000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="L11" t="n">
-        <v>8.84</v>
+        <v>8.15</v>
       </c>
       <c r="M11" t="n">
-        <v>8.85</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>44.82</v>
+        <v>42.74</v>
       </c>
       <c r="O11" t="n">
-        <v>44.89</v>
+        <v>43</v>
       </c>
       <c r="P11" t="n">
-        <v>42.57</v>
+        <v>41.99</v>
       </c>
       <c r="Q11" t="n">
-        <v>42.57</v>
+        <v>42.22</v>
       </c>
       <c r="R11" t="n">
-        <v>16.3314</v>
+        <v>7.6184</v>
       </c>
       <c r="S11" t="n">
-        <v>22.7386</v>
+        <v>14.8146</v>
       </c>
       <c r="T11" t="n">
-        <v>35.6902</v>
+        <v>49.2905</v>
       </c>
       <c r="U11" t="n">
-        <v>6.9246</v>
+        <v>0.8915</v>
       </c>
       <c r="V11" t="n">
-        <v>13.1919</v>
+        <v>7.5311</v>
       </c>
       <c r="W11" t="n">
-        <v>16.8147</v>
+        <v>18.5642</v>
       </c>
       <c r="X11" t="n">
-        <v>-16.5094</v>
+        <v>-7.3446</v>
       </c>
       <c r="Y11" t="n">
-        <v>-23.1103</v>
+        <v>-16.4118</v>
       </c>
       <c r="Z11" t="n">
-        <v>-31.8182</v>
+        <v>-38.1599</v>
       </c>
       <c r="AA11" t="n">
-        <v>-6.9101</v>
+        <v>-0.8222</v>
       </c>
       <c r="AB11" t="n">
-        <v>-12.3894</v>
+        <v>-7.392</v>
       </c>
       <c r="AC11" t="n">
-        <v>-15.233</v>
+        <v>-16.4126</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>181</v>
+        <v>177.62</v>
       </c>
       <c r="C12" t="n">
-        <v>191.29</v>
+        <v>182.24</v>
       </c>
       <c r="D12" t="n">
-        <v>178.94</v>
+        <v>150.58</v>
       </c>
       <c r="E12" t="n">
-        <v>190.42</v>
+        <v>172.52</v>
       </c>
       <c r="F12" t="n">
-        <v>76</v>
+        <v>75.3</v>
       </c>
       <c r="G12" t="n">
-        <v>77.36</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>75.55</v>
+        <v>71.55</v>
       </c>
       <c r="I12" t="n">
-        <v>76.95999999999999</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>8.65</v>
+        <v>8.75</v>
       </c>
       <c r="K12" t="n">
-        <v>8.77</v>
+        <v>9.91</v>
       </c>
       <c r="L12" t="n">
-        <v>8.15</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="M12" t="n">
-        <v>8.199999999999999</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N12" t="n">
-        <v>42.74</v>
+        <v>43.14</v>
       </c>
       <c r="O12" t="n">
-        <v>43</v>
+        <v>45.19</v>
       </c>
       <c r="P12" t="n">
-        <v>41.99</v>
+        <v>42.79</v>
       </c>
       <c r="Q12" t="n">
-        <v>42.22</v>
+        <v>43.31</v>
       </c>
       <c r="R12" t="n">
-        <v>7.6184</v>
+        <v>-9.4003</v>
       </c>
       <c r="S12" t="n">
-        <v>14.8146</v>
+        <v>13.4254</v>
       </c>
       <c r="T12" t="n">
-        <v>49.2905</v>
+        <v>19.6726</v>
       </c>
       <c r="U12" t="n">
-        <v>0.8915</v>
+        <v>-2.5988</v>
       </c>
       <c r="V12" t="n">
-        <v>7.5311</v>
+        <v>5.0743</v>
       </c>
       <c r="W12" t="n">
-        <v>18.5642</v>
+        <v>11.2331</v>
       </c>
       <c r="X12" t="n">
-        <v>-7.3446</v>
+        <v>9.1463</v>
       </c>
       <c r="Y12" t="n">
-        <v>-16.4118</v>
+        <v>-15.566</v>
       </c>
       <c r="Z12" t="n">
-        <v>-38.1599</v>
+        <v>-22.2415</v>
       </c>
       <c r="AA12" t="n">
-        <v>-0.8222</v>
+        <v>2.5817</v>
       </c>
       <c r="AB12" t="n">
-        <v>-7.392</v>
+        <v>-5.2919</v>
       </c>
       <c r="AC12" t="n">
-        <v>-16.4126</v>
+        <v>-10.8664</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>177.62</v>
+        <v>183.84</v>
       </c>
       <c r="C13" t="n">
-        <v>182.24</v>
+        <v>188.49</v>
       </c>
       <c r="D13" t="n">
-        <v>150.58</v>
+        <v>172.26</v>
       </c>
       <c r="E13" t="n">
-        <v>172.52</v>
+        <v>184.24</v>
       </c>
       <c r="F13" t="n">
-        <v>75.3</v>
+        <v>75.81</v>
       </c>
       <c r="G13" t="n">
-        <v>75.93000000000001</v>
+        <v>77.94</v>
       </c>
       <c r="H13" t="n">
-        <v>71.55</v>
+        <v>74.19</v>
       </c>
       <c r="I13" t="n">
-        <v>74.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>8.75</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>9.91</v>
+        <v>8.98</v>
       </c>
       <c r="L13" t="n">
-        <v>8.550000000000001</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="M13" t="n">
-        <v>8.949999999999999</v>
+        <v>8.35</v>
       </c>
       <c r="N13" t="n">
-        <v>43.14</v>
+        <v>42.83</v>
       </c>
       <c r="O13" t="n">
-        <v>45.19</v>
+        <v>43.77</v>
       </c>
       <c r="P13" t="n">
-        <v>42.79</v>
+        <v>41.6</v>
       </c>
       <c r="Q13" t="n">
-        <v>43.31</v>
+        <v>41.99</v>
       </c>
       <c r="R13" t="n">
-        <v>-9.4003</v>
+        <v>6.7934</v>
       </c>
       <c r="S13" t="n">
-        <v>13.4254</v>
+        <v>4.1257</v>
       </c>
       <c r="T13" t="n">
-        <v>19.6726</v>
+        <v>11.0883</v>
       </c>
       <c r="U13" t="n">
-        <v>-2.5988</v>
+        <v>3.0416</v>
       </c>
       <c r="V13" t="n">
-        <v>5.0743</v>
+        <v>1.2585</v>
       </c>
       <c r="W13" t="n">
-        <v>11.2331</v>
+        <v>7.9223</v>
       </c>
       <c r="X13" t="n">
-        <v>9.1463</v>
+        <v>-6.7039</v>
       </c>
       <c r="Y13" t="n">
-        <v>-15.566</v>
+        <v>-5.6497</v>
       </c>
       <c r="Z13" t="n">
-        <v>-22.2415</v>
+        <v>-14.8828</v>
       </c>
       <c r="AA13" t="n">
-        <v>2.5817</v>
+        <v>-3.0478</v>
       </c>
       <c r="AB13" t="n">
-        <v>-5.2919</v>
+        <v>-1.3625</v>
       </c>
       <c r="AC13" t="n">
-        <v>-10.8664</v>
+        <v>-7.8965</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>183.84</v>
+        <v>182.67</v>
       </c>
       <c r="C14" t="n">
-        <v>188.49</v>
+        <v>189.56</v>
       </c>
       <c r="D14" t="n">
-        <v>172.26</v>
+        <v>178.28</v>
       </c>
       <c r="E14" t="n">
-        <v>184.24</v>
+        <v>186.19</v>
       </c>
       <c r="F14" t="n">
-        <v>75.81</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>77.94</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H14" t="n">
-        <v>74.19</v>
+        <v>77.16</v>
       </c>
       <c r="I14" t="n">
-        <v>77.23999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="J14" t="n">
-        <v>8.380000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="K14" t="n">
-        <v>8.98</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L14" t="n">
-        <v>8.140000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M14" t="n">
-        <v>8.35</v>
+        <v>8.27</v>
       </c>
       <c r="N14" t="n">
-        <v>42.83</v>
+        <v>41.98</v>
       </c>
       <c r="O14" t="n">
-        <v>43.77</v>
+        <v>42.06</v>
       </c>
       <c r="P14" t="n">
-        <v>41.6</v>
+        <v>40.68</v>
       </c>
       <c r="Q14" t="n">
-        <v>41.99</v>
+        <v>41.07</v>
       </c>
       <c r="R14" t="n">
-        <v>6.7934</v>
+        <v>1.0584</v>
       </c>
       <c r="S14" t="n">
-        <v>4.1257</v>
+        <v>-2.2214</v>
       </c>
       <c r="T14" t="n">
-        <v>11.0883</v>
+        <v>22.4129</v>
       </c>
       <c r="U14" t="n">
-        <v>3.0416</v>
+        <v>2.2139</v>
       </c>
       <c r="V14" t="n">
-        <v>1.2585</v>
+        <v>2.5858</v>
       </c>
       <c r="W14" t="n">
-        <v>7.9223</v>
+        <v>10.6672</v>
       </c>
       <c r="X14" t="n">
-        <v>-6.7039</v>
+        <v>-0.9581</v>
       </c>
       <c r="Y14" t="n">
-        <v>-5.6497</v>
+        <v>0.8537</v>
       </c>
       <c r="Z14" t="n">
-        <v>-14.8828</v>
+        <v>-21.9811</v>
       </c>
       <c r="AA14" t="n">
-        <v>-3.0478</v>
+        <v>-2.191</v>
       </c>
       <c r="AB14" t="n">
-        <v>-1.3625</v>
+        <v>-2.7238</v>
       </c>
       <c r="AC14" t="n">
-        <v>-7.8965</v>
+        <v>-10.1902</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>182.67</v>
+        <v>167</v>
       </c>
       <c r="C15" t="n">
-        <v>189.56</v>
+        <v>174.4</v>
       </c>
       <c r="D15" t="n">
-        <v>178.28</v>
+        <v>161.14</v>
       </c>
       <c r="E15" t="n">
-        <v>186.19</v>
+        <v>164.18</v>
       </c>
       <c r="F15" t="n">
-        <v>77.29000000000001</v>
+        <v>75.73</v>
       </c>
       <c r="G15" t="n">
-        <v>79.68000000000001</v>
+        <v>77.37</v>
       </c>
       <c r="H15" t="n">
-        <v>77.16</v>
+        <v>74.23</v>
       </c>
       <c r="I15" t="n">
-        <v>78.95</v>
+        <v>75.34</v>
       </c>
       <c r="J15" t="n">
-        <v>8.43</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>8.630000000000001</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="L15" t="n">
-        <v>8.119999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M15" t="n">
-        <v>8.27</v>
+        <v>9.23</v>
       </c>
       <c r="N15" t="n">
-        <v>41.98</v>
+        <v>42.77</v>
       </c>
       <c r="O15" t="n">
-        <v>42.06</v>
+        <v>43.57</v>
       </c>
       <c r="P15" t="n">
-        <v>40.68</v>
+        <v>41.93</v>
       </c>
       <c r="Q15" t="n">
-        <v>41.07</v>
+        <v>42.98</v>
       </c>
       <c r="R15" t="n">
-        <v>1.0584</v>
+        <v>-11.8213</v>
       </c>
       <c r="S15" t="n">
-        <v>-2.2214</v>
+        <v>-4.8342</v>
       </c>
       <c r="T15" t="n">
-        <v>22.4129</v>
+        <v>-7.2115</v>
       </c>
       <c r="U15" t="n">
-        <v>2.2139</v>
+        <v>-4.5725</v>
       </c>
       <c r="V15" t="n">
-        <v>2.5858</v>
+        <v>0.5069</v>
       </c>
       <c r="W15" t="n">
-        <v>10.6672</v>
+        <v>-1.2323</v>
       </c>
       <c r="X15" t="n">
-        <v>-0.9581</v>
+        <v>11.6082</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.8537</v>
+        <v>3.1285</v>
       </c>
       <c r="Z15" t="n">
-        <v>-21.9811</v>
+        <v>4.2938</v>
       </c>
       <c r="AA15" t="n">
-        <v>-2.191</v>
+        <v>4.6506</v>
       </c>
       <c r="AB15" t="n">
-        <v>-2.7238</v>
+        <v>-0.7619</v>
       </c>
       <c r="AC15" t="n">
-        <v>-10.1902</v>
+        <v>0.9631</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>167</v>
+        <v>172.95</v>
       </c>
       <c r="C16" t="n">
-        <v>174.4</v>
+        <v>174.61</v>
       </c>
       <c r="D16" t="n">
-        <v>161.14</v>
+        <v>142.69</v>
       </c>
       <c r="E16" t="n">
-        <v>164.18</v>
+        <v>151.75</v>
       </c>
       <c r="F16" t="n">
-        <v>75.73</v>
+        <v>76.13</v>
       </c>
       <c r="G16" t="n">
-        <v>77.37</v>
+        <v>76.27</v>
       </c>
       <c r="H16" t="n">
-        <v>74.23</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I16" t="n">
-        <v>75.34</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="J16" t="n">
-        <v>9.130000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="K16" t="n">
-        <v>9.390000000000001</v>
+        <v>10.47</v>
       </c>
       <c r="L16" t="n">
-        <v>8.800000000000001</v>
+        <v>8.68</v>
       </c>
       <c r="M16" t="n">
-        <v>9.23</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="N16" t="n">
-        <v>42.77</v>
+        <v>42.51</v>
       </c>
       <c r="O16" t="n">
-        <v>43.57</v>
+        <v>44.82</v>
       </c>
       <c r="P16" t="n">
-        <v>41.93</v>
+        <v>42.44</v>
       </c>
       <c r="Q16" t="n">
-        <v>42.98</v>
+        <v>43.54</v>
       </c>
       <c r="R16" t="n">
-        <v>-11.8213</v>
+        <v>-7.571</v>
       </c>
       <c r="S16" t="n">
-        <v>-4.8342</v>
+        <v>-17.6346</v>
       </c>
       <c r="T16" t="n">
-        <v>-7.2115</v>
+        <v>-20.3077</v>
       </c>
       <c r="U16" t="n">
-        <v>-4.5725</v>
+        <v>-1.3539</v>
       </c>
       <c r="V16" t="n">
-        <v>0.5069</v>
+        <v>-3.7804</v>
       </c>
       <c r="W16" t="n">
-        <v>-1.2323</v>
+        <v>-3.4304</v>
       </c>
       <c r="X16" t="n">
-        <v>11.6082</v>
+        <v>7.8007</v>
       </c>
       <c r="Y16" t="n">
-        <v>3.1285</v>
+        <v>19.1617</v>
       </c>
       <c r="Z16" t="n">
-        <v>4.2938</v>
+        <v>21.3415</v>
       </c>
       <c r="AA16" t="n">
-        <v>4.6506</v>
+        <v>1.3029</v>
       </c>
       <c r="AB16" t="n">
-        <v>-0.7619</v>
+        <v>3.6914</v>
       </c>
       <c r="AC16" t="n">
-        <v>0.9631</v>
+        <v>3.1265</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>172.95</v>
+        <v>141.24</v>
       </c>
       <c r="C17" t="n">
-        <v>174.61</v>
+        <v>160.6</v>
       </c>
       <c r="D17" t="n">
-        <v>142.69</v>
+        <v>135.02</v>
       </c>
       <c r="E17" t="n">
-        <v>151.75</v>
+        <v>151.89</v>
       </c>
       <c r="F17" t="n">
-        <v>76.13</v>
+        <v>72.41</v>
       </c>
       <c r="G17" t="n">
-        <v>76.27</v>
+        <v>74.5</v>
       </c>
       <c r="H17" t="n">
-        <v>72.09999999999999</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="I17" t="n">
-        <v>74.31999999999999</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J17" t="n">
-        <v>8.77</v>
+        <v>10.64</v>
       </c>
       <c r="K17" t="n">
-        <v>10.47</v>
+        <v>11.07</v>
       </c>
       <c r="L17" t="n">
-        <v>8.68</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="M17" t="n">
-        <v>9.949999999999999</v>
+        <v>9.93</v>
       </c>
       <c r="N17" t="n">
-        <v>42.51</v>
+        <v>44.68</v>
       </c>
       <c r="O17" t="n">
-        <v>44.82</v>
+        <v>45.53</v>
       </c>
       <c r="P17" t="n">
-        <v>42.44</v>
+        <v>43.46</v>
       </c>
       <c r="Q17" t="n">
-        <v>43.54</v>
+        <v>44.37</v>
       </c>
       <c r="R17" t="n">
-        <v>-7.571</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="S17" t="n">
-        <v>-17.6346</v>
+        <v>-18.422</v>
       </c>
       <c r="T17" t="n">
-        <v>-20.3077</v>
+        <v>-11.958</v>
       </c>
       <c r="U17" t="n">
-        <v>-1.3539</v>
+        <v>-1.8703</v>
       </c>
       <c r="V17" t="n">
-        <v>-3.7804</v>
+        <v>-7.6251</v>
       </c>
       <c r="W17" t="n">
-        <v>-3.4304</v>
+        <v>-2.7081</v>
       </c>
       <c r="X17" t="n">
-        <v>7.8007</v>
+        <v>-0.201</v>
       </c>
       <c r="Y17" t="n">
-        <v>19.1617</v>
+        <v>20.0726</v>
       </c>
       <c r="Z17" t="n">
-        <v>21.3415</v>
+        <v>10.9497</v>
       </c>
       <c r="AA17" t="n">
-        <v>1.3029</v>
+        <v>1.9063</v>
       </c>
       <c r="AB17" t="n">
-        <v>3.6914</v>
+        <v>8.0351</v>
       </c>
       <c r="AC17" t="n">
-        <v>3.1265</v>
+        <v>2.4475</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>141.24</v>
+        <v>161</v>
       </c>
       <c r="C18" t="n">
-        <v>160.6</v>
+        <v>173.7</v>
       </c>
       <c r="D18" t="n">
-        <v>135.02</v>
+        <v>161</v>
       </c>
       <c r="E18" t="n">
-        <v>151.89</v>
+        <v>173.2</v>
       </c>
       <c r="F18" t="n">
-        <v>72.41</v>
+        <v>74.09</v>
       </c>
       <c r="G18" t="n">
-        <v>74.5</v>
+        <v>76.53</v>
       </c>
       <c r="H18" t="n">
-        <v>70.95999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="I18" t="n">
-        <v>72.93000000000001</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>10.64</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>11.07</v>
+        <v>9.35</v>
       </c>
       <c r="L18" t="n">
-        <v>9.369999999999999</v>
+        <v>8.51</v>
       </c>
       <c r="M18" t="n">
-        <v>9.93</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N18" t="n">
-        <v>44.68</v>
+        <v>43.67</v>
       </c>
       <c r="O18" t="n">
-        <v>45.53</v>
+        <v>43.97</v>
       </c>
       <c r="P18" t="n">
-        <v>43.46</v>
+        <v>42.19</v>
       </c>
       <c r="Q18" t="n">
-        <v>44.37</v>
+        <v>42.19</v>
       </c>
       <c r="R18" t="n">
-        <v>0.09229999999999999</v>
+        <v>14.0299</v>
       </c>
       <c r="S18" t="n">
-        <v>-18.422</v>
+        <v>5.494</v>
       </c>
       <c r="T18" t="n">
-        <v>-11.958</v>
+        <v>-5.9922</v>
       </c>
       <c r="U18" t="n">
-        <v>-1.8703</v>
+        <v>4.9088</v>
       </c>
       <c r="V18" t="n">
-        <v>-7.6251</v>
+        <v>1.553</v>
       </c>
       <c r="W18" t="n">
-        <v>-2.7081</v>
+        <v>-0.9451000000000001</v>
       </c>
       <c r="X18" t="n">
-        <v>-0.201</v>
+        <v>-13.998</v>
       </c>
       <c r="Y18" t="n">
-        <v>20.0726</v>
+        <v>-7.4756</v>
       </c>
       <c r="Z18" t="n">
-        <v>10.9497</v>
+        <v>2.2754</v>
       </c>
       <c r="AA18" t="n">
-        <v>1.9063</v>
+        <v>-4.9132</v>
       </c>
       <c r="AB18" t="n">
-        <v>8.0351</v>
+        <v>-1.8381</v>
       </c>
       <c r="AC18" t="n">
-        <v>2.4475</v>
+        <v>0.4763</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>161</v>
+        <v>171.26</v>
       </c>
       <c r="C19" t="n">
-        <v>173.7</v>
+        <v>179.97</v>
       </c>
       <c r="D19" t="n">
-        <v>161</v>
+        <v>168.23</v>
       </c>
       <c r="E19" t="n">
-        <v>173.2</v>
+        <v>178.39</v>
       </c>
       <c r="F19" t="n">
-        <v>74.09</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>76.53</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>73.62</v>
+        <v>74.47</v>
       </c>
       <c r="I19" t="n">
-        <v>76.51000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J19" t="n">
-        <v>9.300000000000001</v>
+        <v>8.65</v>
       </c>
       <c r="K19" t="n">
-        <v>9.35</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L19" t="n">
-        <v>8.51</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M19" t="n">
-        <v>8.539999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N19" t="n">
-        <v>43.67</v>
+        <v>42.94</v>
       </c>
       <c r="O19" t="n">
-        <v>43.97</v>
+        <v>43.33</v>
       </c>
       <c r="P19" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="Q19" t="n">
-        <v>42.19</v>
+        <v>41.96</v>
       </c>
       <c r="R19" t="n">
-        <v>14.0299</v>
+        <v>2.9965</v>
       </c>
       <c r="S19" t="n">
-        <v>5.494</v>
+        <v>17.5552</v>
       </c>
       <c r="T19" t="n">
-        <v>-5.9922</v>
+        <v>-4.1893</v>
       </c>
       <c r="U19" t="n">
-        <v>4.9088</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="V19" t="n">
-        <v>1.553</v>
+        <v>3.5388</v>
       </c>
       <c r="W19" t="n">
-        <v>-0.9451000000000001</v>
+        <v>-2.5332</v>
       </c>
       <c r="X19" t="n">
-        <v>-13.998</v>
+        <v>-2.9274</v>
       </c>
       <c r="Y19" t="n">
-        <v>-7.4756</v>
+        <v>-16.6834</v>
       </c>
       <c r="Z19" t="n">
-        <v>2.2754</v>
+        <v>0.2418</v>
       </c>
       <c r="AA19" t="n">
-        <v>-4.9132</v>
+        <v>-0.5452</v>
       </c>
       <c r="AB19" t="n">
-        <v>-1.8381</v>
+        <v>-3.6288</v>
       </c>
       <c r="AC19" t="n">
-        <v>0.4763</v>
+        <v>2.167</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>171.26</v>
+        <v>184.8</v>
       </c>
       <c r="C20" t="n">
-        <v>179.97</v>
+        <v>195.27</v>
       </c>
       <c r="D20" t="n">
-        <v>168.23</v>
+        <v>183.34</v>
       </c>
       <c r="E20" t="n">
-        <v>178.39</v>
+        <v>190.56</v>
       </c>
       <c r="F20" t="n">
-        <v>75.18000000000001</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>77.79000000000001</v>
+        <v>79.33</v>
       </c>
       <c r="H20" t="n">
-        <v>74.47</v>
+        <v>77.33</v>
       </c>
       <c r="I20" t="n">
-        <v>76.95</v>
+        <v>77.84</v>
       </c>
       <c r="J20" t="n">
-        <v>8.65</v>
+        <v>8</v>
       </c>
       <c r="K20" t="n">
-        <v>8.779999999999999</v>
+        <v>8.06</v>
       </c>
       <c r="L20" t="n">
-        <v>8.210000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="M20" t="n">
-        <v>8.289999999999999</v>
+        <v>7.73</v>
       </c>
       <c r="N20" t="n">
-        <v>42.94</v>
+        <v>41.4</v>
       </c>
       <c r="O20" t="n">
-        <v>43.33</v>
+        <v>41.78</v>
       </c>
       <c r="P20" t="n">
+        <v>40.68</v>
+      </c>
+      <c r="Q20" t="n">
         <v>41.5</v>
       </c>
-      <c r="Q20" t="n">
-        <v>41.96</v>
-      </c>
       <c r="R20" t="n">
-        <v>2.9965</v>
+        <v>6.8221</v>
       </c>
       <c r="S20" t="n">
-        <v>17.5552</v>
+        <v>25.4592</v>
       </c>
       <c r="T20" t="n">
-        <v>-4.1893</v>
+        <v>16.0677</v>
       </c>
       <c r="U20" t="n">
-        <v>0.5750999999999999</v>
+        <v>1.1566</v>
       </c>
       <c r="V20" t="n">
-        <v>3.5388</v>
+        <v>6.7325</v>
       </c>
       <c r="W20" t="n">
-        <v>-2.5332</v>
+        <v>3.3183</v>
       </c>
       <c r="X20" t="n">
-        <v>-2.9274</v>
+        <v>-6.7551</v>
       </c>
       <c r="Y20" t="n">
-        <v>-16.6834</v>
+        <v>-22.1551</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.2418</v>
+        <v>-16.2514</v>
       </c>
       <c r="AA20" t="n">
-        <v>-0.5452</v>
+        <v>-1.0963</v>
       </c>
       <c r="AB20" t="n">
-        <v>-3.6288</v>
+        <v>-6.4683</v>
       </c>
       <c r="AC20" t="n">
-        <v>2.167</v>
+        <v>-3.4435</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>184.8</v>
+        <v>211.38</v>
       </c>
       <c r="C21" t="n">
-        <v>195.27</v>
+        <v>228.5</v>
       </c>
       <c r="D21" t="n">
-        <v>183.34</v>
+        <v>209.89</v>
       </c>
       <c r="E21" t="n">
-        <v>190.56</v>
+        <v>225.79</v>
       </c>
       <c r="F21" t="n">
-        <v>78.04000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="G21" t="n">
-        <v>79.33</v>
+        <v>82.27</v>
       </c>
       <c r="H21" t="n">
-        <v>77.33</v>
+        <v>79.98</v>
       </c>
       <c r="I21" t="n">
-        <v>77.84</v>
+        <v>81.95</v>
       </c>
       <c r="J21" t="n">
-        <v>8</v>
+        <v>6.9</v>
       </c>
       <c r="K21" t="n">
-        <v>8.06</v>
+        <v>6.95</v>
       </c>
       <c r="L21" t="n">
-        <v>7.5</v>
+        <v>6.19</v>
       </c>
       <c r="M21" t="n">
-        <v>7.73</v>
+        <v>6.29</v>
       </c>
       <c r="N21" t="n">
-        <v>41.4</v>
+        <v>40.05</v>
       </c>
       <c r="O21" t="n">
-        <v>41.78</v>
+        <v>40.35</v>
       </c>
       <c r="P21" t="n">
-        <v>40.68</v>
+        <v>39.14</v>
       </c>
       <c r="Q21" t="n">
-        <v>41.5</v>
+        <v>39.28</v>
       </c>
       <c r="R21" t="n">
-        <v>6.8221</v>
+        <v>18.4876</v>
       </c>
       <c r="S21" t="n">
-        <v>25.4592</v>
+        <v>30.3637</v>
       </c>
       <c r="T21" t="n">
-        <v>16.0677</v>
+        <v>48.7908</v>
       </c>
       <c r="U21" t="n">
-        <v>1.1566</v>
+        <v>5.2801</v>
       </c>
       <c r="V21" t="n">
-        <v>6.7325</v>
+        <v>7.1102</v>
       </c>
       <c r="W21" t="n">
-        <v>3.3183</v>
+        <v>10.2664</v>
       </c>
       <c r="X21" t="n">
-        <v>-6.7551</v>
+        <v>-18.6287</v>
       </c>
       <c r="Y21" t="n">
-        <v>-22.1551</v>
+        <v>-26.3466</v>
       </c>
       <c r="Z21" t="n">
-        <v>-16.2514</v>
+        <v>-36.7839</v>
       </c>
       <c r="AA21" t="n">
-        <v>-1.0963</v>
+        <v>-5.3494</v>
       </c>
       <c r="AB21" t="n">
-        <v>-6.4683</v>
+        <v>-6.8974</v>
       </c>
       <c r="AC21" t="n">
-        <v>-3.4435</v>
+        <v>-9.7841</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>211.38</v>
+        <v>242.66</v>
       </c>
       <c r="C22" t="n">
-        <v>228.5</v>
+        <v>242.66</v>
       </c>
       <c r="D22" t="n">
-        <v>209.89</v>
+        <v>204</v>
       </c>
       <c r="E22" t="n">
-        <v>225.79</v>
+        <v>217.98</v>
       </c>
       <c r="F22" t="n">
-        <v>80.56999999999999</v>
+        <v>82.87</v>
       </c>
       <c r="G22" t="n">
-        <v>82.27</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>79.98</v>
+        <v>80.33</v>
       </c>
       <c r="I22" t="n">
-        <v>81.95</v>
+        <v>81.67</v>
       </c>
       <c r="J22" t="n">
-        <v>6.9</v>
+        <v>5.83</v>
       </c>
       <c r="K22" t="n">
-        <v>6.95</v>
+        <v>6.91</v>
       </c>
       <c r="L22" t="n">
-        <v>6.19</v>
+        <v>5.84</v>
       </c>
       <c r="M22" t="n">
-        <v>6.29</v>
+        <v>6.53</v>
       </c>
       <c r="N22" t="n">
-        <v>40.045</v>
+        <v>38.87</v>
       </c>
       <c r="O22" t="n">
-        <v>40.3519</v>
+        <v>40.09</v>
       </c>
       <c r="P22" t="n">
-        <v>39.1399</v>
+        <v>38.86</v>
       </c>
       <c r="Q22" t="n">
-        <v>39.28</v>
+        <v>39.44</v>
       </c>
       <c r="R22" t="n">
-        <v>18.4876</v>
+        <v>-3.459</v>
       </c>
       <c r="S22" t="n">
-        <v>30.3637</v>
+        <v>22.1929</v>
       </c>
       <c r="T22" t="n">
-        <v>48.7908</v>
+        <v>43.5118</v>
       </c>
       <c r="U22" t="n">
-        <v>5.2801</v>
+        <v>-0.3417</v>
       </c>
       <c r="V22" t="n">
-        <v>7.1102</v>
+        <v>6.1339</v>
       </c>
       <c r="W22" t="n">
-        <v>10.2664</v>
+        <v>11.9841</v>
       </c>
       <c r="X22" t="n">
-        <v>-18.6287</v>
+        <v>3.8156</v>
       </c>
       <c r="Y22" t="n">
-        <v>-26.3466</v>
+        <v>-21.2304</v>
       </c>
       <c r="Z22" t="n">
-        <v>-36.7839</v>
+        <v>-34.2397</v>
       </c>
       <c r="AA22" t="n">
-        <v>-5.3494</v>
+        <v>0.4073</v>
       </c>
       <c r="AB22" t="n">
-        <v>-6.8974</v>
+        <v>-6.0057</v>
       </c>
       <c r="AC22" t="n">
-        <v>-9.7841</v>
+        <v>-11.1111</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-05-28 23:17
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>108.75</v>
+        <v>114.76</v>
       </c>
       <c r="C2" t="n">
-        <v>115.62</v>
+        <v>118.32</v>
       </c>
       <c r="D2" t="n">
-        <v>103.99</v>
+        <v>112.3</v>
       </c>
       <c r="E2" t="n">
-        <v>109.56</v>
+        <v>117.97</v>
       </c>
       <c r="F2" t="n">
-        <v>60.72</v>
+        <v>61</v>
       </c>
       <c r="G2" t="n">
-        <v>61.33</v>
+        <v>61.87</v>
       </c>
       <c r="H2" t="n">
-        <v>59.68</v>
+        <v>60.45</v>
       </c>
       <c r="I2" t="n">
-        <v>60.74</v>
+        <v>61.86</v>
       </c>
       <c r="J2" t="n">
-        <v>15.71</v>
+        <v>14.91</v>
       </c>
       <c r="K2" t="n">
-        <v>16.27</v>
+        <v>15.24</v>
       </c>
       <c r="L2" t="n">
-        <v>14.93</v>
+        <v>14.38</v>
       </c>
       <c r="M2" t="n">
-        <v>15.59</v>
+        <v>14.4</v>
       </c>
       <c r="N2" t="n">
-        <v>54.09</v>
+        <v>53.84</v>
       </c>
       <c r="O2" t="n">
-        <v>54.96</v>
+        <v>54.33</v>
       </c>
       <c r="P2" t="n">
-        <v>53.58</v>
+        <v>53.06</v>
       </c>
       <c r="Q2" t="n">
-        <v>54.05</v>
+        <v>53.08</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>114.76</v>
+        <v>122.81</v>
       </c>
       <c r="C3" t="n">
-        <v>118.32</v>
+        <v>127.45</v>
       </c>
       <c r="D3" t="n">
-        <v>112.3</v>
+        <v>117.5</v>
       </c>
       <c r="E3" t="n">
-        <v>117.97</v>
+        <v>126.98</v>
       </c>
       <c r="F3" t="n">
-        <v>61</v>
+        <v>62.89</v>
       </c>
       <c r="G3" t="n">
-        <v>61.87</v>
+        <v>63.8</v>
       </c>
       <c r="H3" t="n">
-        <v>60.45</v>
+        <v>60.7</v>
       </c>
       <c r="I3" t="n">
-        <v>61.86</v>
+        <v>63.54</v>
       </c>
       <c r="J3" t="n">
-        <v>14.91</v>
+        <v>13.84</v>
       </c>
       <c r="K3" t="n">
-        <v>15.24</v>
+        <v>14.49</v>
       </c>
       <c r="L3" t="n">
-        <v>14.38</v>
+        <v>13.25</v>
       </c>
       <c r="M3" t="n">
-        <v>14.4</v>
+        <v>13.3</v>
       </c>
       <c r="N3" t="n">
-        <v>53.84</v>
+        <v>52.21</v>
       </c>
       <c r="O3" t="n">
-        <v>54.33</v>
+        <v>54.09</v>
       </c>
       <c r="P3" t="n">
-        <v>53.06</v>
+        <v>51.4</v>
       </c>
       <c r="Q3" t="n">
-        <v>53.08</v>
+        <v>51.65</v>
       </c>
       <c r="R3" t="n">
-        <v>7.6762</v>
+        <v>7.6375</v>
       </c>
       <c r="U3" t="n">
-        <v>1.8439</v>
+        <v>2.7158</v>
       </c>
       <c r="X3" t="n">
-        <v>-7.6331</v>
+        <v>-7.6389</v>
       </c>
       <c r="AA3" t="n">
-        <v>-1.7946</v>
+        <v>-2.694</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>122.81</v>
+        <v>124.39</v>
       </c>
       <c r="C4" t="n">
-        <v>127.45</v>
+        <v>131.38</v>
       </c>
       <c r="D4" t="n">
-        <v>117.5</v>
+        <v>121.66</v>
       </c>
       <c r="E4" t="n">
-        <v>126.98</v>
+        <v>130.4</v>
       </c>
       <c r="F4" t="n">
-        <v>62.89</v>
+        <v>63.89</v>
       </c>
       <c r="G4" t="n">
-        <v>63.8</v>
+        <v>65.84</v>
       </c>
       <c r="H4" t="n">
-        <v>60.7</v>
+        <v>63.81</v>
       </c>
       <c r="I4" t="n">
-        <v>63.54</v>
+        <v>65.3</v>
       </c>
       <c r="J4" t="n">
-        <v>13.84</v>
+        <v>13.61</v>
       </c>
       <c r="K4" t="n">
-        <v>14.49</v>
+        <v>13.89</v>
       </c>
       <c r="L4" t="n">
-        <v>13.25</v>
+        <v>12.87</v>
       </c>
       <c r="M4" t="n">
-        <v>13.3</v>
+        <v>12.98</v>
       </c>
       <c r="N4" t="n">
-        <v>52.21</v>
+        <v>51.36</v>
       </c>
       <c r="O4" t="n">
-        <v>54.09</v>
+        <v>51.45</v>
       </c>
       <c r="P4" t="n">
-        <v>51.4</v>
+        <v>49.79</v>
       </c>
       <c r="Q4" t="n">
-        <v>51.65</v>
+        <v>50.22</v>
       </c>
       <c r="R4" t="n">
-        <v>7.6375</v>
+        <v>2.6933</v>
       </c>
       <c r="U4" t="n">
-        <v>2.7158</v>
+        <v>2.7699</v>
       </c>
       <c r="X4" t="n">
-        <v>-7.6389</v>
+        <v>-2.406</v>
       </c>
       <c r="AA4" t="n">
-        <v>-2.694</v>
+        <v>-2.7686</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>124.39</v>
+        <v>132.2</v>
       </c>
       <c r="C5" t="n">
-        <v>131.38</v>
+        <v>133.67</v>
       </c>
       <c r="D5" t="n">
-        <v>121.66</v>
+        <v>123.8</v>
       </c>
       <c r="E5" t="n">
-        <v>130.4</v>
+        <v>127.55</v>
       </c>
       <c r="F5" t="n">
-        <v>63.89</v>
+        <v>65.44</v>
       </c>
       <c r="G5" t="n">
-        <v>65.84</v>
+        <v>66.05</v>
       </c>
       <c r="H5" t="n">
-        <v>63.81</v>
+        <v>63.78</v>
       </c>
       <c r="I5" t="n">
-        <v>65.3</v>
+        <v>64.91</v>
       </c>
       <c r="J5" t="n">
-        <v>13.61</v>
+        <v>12.8</v>
       </c>
       <c r="K5" t="n">
-        <v>13.89</v>
+        <v>13.64</v>
       </c>
       <c r="L5" t="n">
-        <v>12.87</v>
+        <v>12.65</v>
       </c>
       <c r="M5" t="n">
-        <v>12.98</v>
+        <v>13.26</v>
       </c>
       <c r="N5" t="n">
-        <v>51.36</v>
+        <v>50.12</v>
       </c>
       <c r="O5" t="n">
-        <v>51.45</v>
+        <v>51.43</v>
       </c>
       <c r="P5" t="n">
-        <v>49.79</v>
+        <v>49.65</v>
       </c>
       <c r="Q5" t="n">
-        <v>50.22</v>
+        <v>50.51</v>
       </c>
       <c r="R5" t="n">
-        <v>2.6933</v>
+        <v>-2.1856</v>
       </c>
       <c r="S5" t="n">
-        <v>19.0215</v>
+        <v>8.120699999999999</v>
       </c>
       <c r="U5" t="n">
-        <v>2.7699</v>
+        <v>-0.5972</v>
       </c>
       <c r="V5" t="n">
-        <v>7.5074</v>
+        <v>4.9305</v>
       </c>
       <c r="X5" t="n">
-        <v>-2.406</v>
+        <v>2.1572</v>
       </c>
       <c r="Y5" t="n">
-        <v>-16.7415</v>
+        <v>-7.9167</v>
       </c>
       <c r="AA5" t="n">
-        <v>-2.7686</v>
+        <v>0.5775</v>
       </c>
       <c r="AB5" t="n">
-        <v>-7.086</v>
+        <v>-4.8417</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>132.2</v>
+        <v>135</v>
       </c>
       <c r="C6" t="n">
-        <v>133.67</v>
+        <v>147.26</v>
       </c>
       <c r="D6" t="n">
-        <v>123.8</v>
+        <v>134.02</v>
       </c>
       <c r="E6" t="n">
-        <v>127.55</v>
+        <v>144.16</v>
       </c>
       <c r="F6" t="n">
-        <v>65.44</v>
+        <v>66.37</v>
       </c>
       <c r="G6" t="n">
-        <v>66.05</v>
+        <v>67.77</v>
       </c>
       <c r="H6" t="n">
-        <v>63.78</v>
+        <v>66.25</v>
       </c>
       <c r="I6" t="n">
-        <v>64.91</v>
+        <v>67.39</v>
       </c>
       <c r="J6" t="n">
-        <v>12.8</v>
+        <v>12.5</v>
       </c>
       <c r="K6" t="n">
-        <v>13.64</v>
+        <v>12.59</v>
       </c>
       <c r="L6" t="n">
-        <v>12.65</v>
+        <v>11.21</v>
       </c>
       <c r="M6" t="n">
-        <v>13.26</v>
+        <v>11.51</v>
       </c>
       <c r="N6" t="n">
-        <v>50.12</v>
+        <v>49.4</v>
       </c>
       <c r="O6" t="n">
-        <v>51.43</v>
+        <v>49.49</v>
       </c>
       <c r="P6" t="n">
-        <v>49.65</v>
+        <v>48.3</v>
       </c>
       <c r="Q6" t="n">
-        <v>50.51</v>
+        <v>48.59</v>
       </c>
       <c r="R6" t="n">
-        <v>-2.1856</v>
+        <v>13.0223</v>
       </c>
       <c r="S6" t="n">
-        <v>8.120699999999999</v>
+        <v>13.5297</v>
       </c>
       <c r="U6" t="n">
-        <v>-0.5972</v>
+        <v>3.8207</v>
       </c>
       <c r="V6" t="n">
-        <v>4.9305</v>
+        <v>6.0592</v>
       </c>
       <c r="X6" t="n">
-        <v>2.1572</v>
+        <v>-13.1976</v>
       </c>
       <c r="Y6" t="n">
-        <v>-7.9167</v>
+        <v>-13.4586</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.5775</v>
+        <v>-3.8012</v>
       </c>
       <c r="AB6" t="n">
-        <v>-4.8417</v>
+        <v>-5.9245</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>135</v>
+        <v>157.84</v>
       </c>
       <c r="C7" t="n">
-        <v>147.26</v>
+        <v>166</v>
       </c>
       <c r="D7" t="n">
-        <v>134.02</v>
+        <v>149.06</v>
       </c>
       <c r="E7" t="n">
-        <v>144.16</v>
+        <v>165.85</v>
       </c>
       <c r="F7" t="n">
-        <v>66.37</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>67.77</v>
+        <v>71.66</v>
       </c>
       <c r="H7" t="n">
-        <v>66.25</v>
+        <v>68.88</v>
       </c>
       <c r="I7" t="n">
-        <v>67.39</v>
+        <v>71.56999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>12.5</v>
+        <v>10.43</v>
       </c>
       <c r="K7" t="n">
-        <v>12.59</v>
+        <v>11.14</v>
       </c>
       <c r="L7" t="n">
-        <v>11.21</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M7" t="n">
-        <v>11.51</v>
+        <v>9.81</v>
       </c>
       <c r="N7" t="n">
-        <v>49.4</v>
+        <v>47.26</v>
       </c>
       <c r="O7" t="n">
-        <v>49.49</v>
+        <v>47.54</v>
       </c>
       <c r="P7" t="n">
-        <v>48.3</v>
+        <v>45.52</v>
       </c>
       <c r="Q7" t="n">
-        <v>48.59</v>
+        <v>45.59</v>
       </c>
       <c r="R7" t="n">
-        <v>13.0223</v>
+        <v>15.0458</v>
       </c>
       <c r="S7" t="n">
-        <v>13.5297</v>
+        <v>27.1856</v>
       </c>
       <c r="T7" t="n">
-        <v>31.5809</v>
+        <v>40.5866</v>
       </c>
       <c r="U7" t="n">
-        <v>3.8207</v>
+        <v>6.2027</v>
       </c>
       <c r="V7" t="n">
-        <v>6.0592</v>
+        <v>9.601800000000001</v>
       </c>
       <c r="W7" t="n">
-        <v>10.9483</v>
+        <v>15.6967</v>
       </c>
       <c r="X7" t="n">
-        <v>-13.1976</v>
+        <v>-14.7698</v>
       </c>
       <c r="Y7" t="n">
-        <v>-13.4586</v>
+        <v>-24.4222</v>
       </c>
       <c r="Z7" t="n">
-        <v>-26.1706</v>
+        <v>-31.875</v>
       </c>
       <c r="AA7" t="n">
-        <v>-3.8012</v>
+        <v>-6.1741</v>
       </c>
       <c r="AB7" t="n">
-        <v>-5.9245</v>
+        <v>-9.2194</v>
       </c>
       <c r="AC7" t="n">
-        <v>-10.1018</v>
+        <v>-14.1108</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>157.84</v>
+        <v>162.12</v>
       </c>
       <c r="C8" t="n">
-        <v>166</v>
+        <v>162.9</v>
       </c>
       <c r="D8" t="n">
-        <v>149.06</v>
+        <v>147.61</v>
       </c>
       <c r="E8" t="n">
-        <v>165.85</v>
+        <v>152.1</v>
       </c>
       <c r="F8" t="n">
-        <v>69.26000000000001</v>
+        <v>71.87</v>
       </c>
       <c r="G8" t="n">
-        <v>71.66</v>
+        <v>73.3</v>
       </c>
       <c r="H8" t="n">
-        <v>68.88</v>
+        <v>70.38</v>
       </c>
       <c r="I8" t="n">
-        <v>71.56999999999999</v>
+        <v>71.34</v>
       </c>
       <c r="J8" t="n">
-        <v>10.43</v>
+        <v>10.02</v>
       </c>
       <c r="K8" t="n">
-        <v>11.14</v>
+        <v>10.88</v>
       </c>
       <c r="L8" t="n">
-        <v>9.800000000000001</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>9.81</v>
+        <v>10.6</v>
       </c>
       <c r="N8" t="n">
-        <v>47.26</v>
+        <v>45.41</v>
       </c>
       <c r="O8" t="n">
-        <v>47.54</v>
+        <v>46.36</v>
       </c>
       <c r="P8" t="n">
-        <v>45.52</v>
+        <v>44.5</v>
       </c>
       <c r="Q8" t="n">
-        <v>45.59</v>
+        <v>45.73</v>
       </c>
       <c r="R8" t="n">
-        <v>15.0458</v>
+        <v>-8.2906</v>
       </c>
       <c r="S8" t="n">
-        <v>27.1856</v>
+        <v>19.2474</v>
       </c>
       <c r="T8" t="n">
-        <v>40.5866</v>
+        <v>19.7826</v>
       </c>
       <c r="U8" t="n">
-        <v>6.2027</v>
+        <v>-0.3214</v>
       </c>
       <c r="V8" t="n">
-        <v>9.601800000000001</v>
+        <v>9.906000000000001</v>
       </c>
       <c r="W8" t="n">
-        <v>15.6967</v>
+        <v>12.2757</v>
       </c>
       <c r="X8" t="n">
-        <v>-14.7698</v>
+        <v>8.053000000000001</v>
       </c>
       <c r="Y8" t="n">
-        <v>-24.4222</v>
+        <v>-20.0603</v>
       </c>
       <c r="Z8" t="n">
-        <v>-31.875</v>
+        <v>-20.3008</v>
       </c>
       <c r="AA8" t="n">
-        <v>-6.1741</v>
+        <v>0.3071</v>
       </c>
       <c r="AB8" t="n">
-        <v>-9.2194</v>
+        <v>-9.4635</v>
       </c>
       <c r="AC8" t="n">
-        <v>-14.1108</v>
+        <v>-11.4618</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>162.12</v>
+        <v>163</v>
       </c>
       <c r="C9" t="n">
-        <v>162.9</v>
+        <v>177.5</v>
       </c>
       <c r="D9" t="n">
-        <v>147.61</v>
+        <v>161.51</v>
       </c>
       <c r="E9" t="n">
-        <v>152.1</v>
+        <v>176.94</v>
       </c>
       <c r="F9" t="n">
-        <v>71.87</v>
+        <v>72.81999999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>73.3</v>
+        <v>76.31</v>
       </c>
       <c r="H9" t="n">
-        <v>70.38</v>
+        <v>72.7</v>
       </c>
       <c r="I9" t="n">
-        <v>71.34</v>
+        <v>76.28</v>
       </c>
       <c r="J9" t="n">
-        <v>10.02</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="K9" t="n">
-        <v>10.88</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="L9" t="n">
-        <v>9.970000000000001</v>
+        <v>8.84</v>
       </c>
       <c r="M9" t="n">
-        <v>10.6</v>
+        <v>8.85</v>
       </c>
       <c r="N9" t="n">
-        <v>45.41</v>
+        <v>44.82</v>
       </c>
       <c r="O9" t="n">
-        <v>46.36</v>
+        <v>44.89</v>
       </c>
       <c r="P9" t="n">
-        <v>44.5</v>
+        <v>42.57</v>
       </c>
       <c r="Q9" t="n">
-        <v>45.73</v>
+        <v>42.57</v>
       </c>
       <c r="R9" t="n">
-        <v>-8.2906</v>
+        <v>16.3314</v>
       </c>
       <c r="S9" t="n">
-        <v>19.2474</v>
+        <v>22.7386</v>
       </c>
       <c r="T9" t="n">
-        <v>19.7826</v>
+        <v>35.6902</v>
       </c>
       <c r="U9" t="n">
-        <v>-0.3214</v>
+        <v>6.9246</v>
       </c>
       <c r="V9" t="n">
-        <v>9.906000000000001</v>
+        <v>13.1919</v>
       </c>
       <c r="W9" t="n">
-        <v>12.2757</v>
+        <v>16.8147</v>
       </c>
       <c r="X9" t="n">
-        <v>8.053000000000001</v>
+        <v>-16.5094</v>
       </c>
       <c r="Y9" t="n">
-        <v>-20.0603</v>
+        <v>-23.1103</v>
       </c>
       <c r="Z9" t="n">
-        <v>-20.3008</v>
+        <v>-31.8182</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.3071</v>
+        <v>-6.9101</v>
       </c>
       <c r="AB9" t="n">
-        <v>-9.4635</v>
+        <v>-12.3894</v>
       </c>
       <c r="AC9" t="n">
-        <v>-11.4618</v>
+        <v>-15.233</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="C10" t="n">
-        <v>177.5</v>
+        <v>191.29</v>
       </c>
       <c r="D10" t="n">
-        <v>161.51</v>
+        <v>178.94</v>
       </c>
       <c r="E10" t="n">
-        <v>176.94</v>
+        <v>190.42</v>
       </c>
       <c r="F10" t="n">
-        <v>72.81999999999999</v>
+        <v>76</v>
       </c>
       <c r="G10" t="n">
-        <v>76.31</v>
+        <v>77.36</v>
       </c>
       <c r="H10" t="n">
-        <v>72.7</v>
+        <v>75.55</v>
       </c>
       <c r="I10" t="n">
-        <v>76.28</v>
+        <v>76.95999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>9.859999999999999</v>
+        <v>8.65</v>
       </c>
       <c r="K10" t="n">
-        <v>9.970000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="L10" t="n">
-        <v>8.84</v>
+        <v>8.15</v>
       </c>
       <c r="M10" t="n">
-        <v>8.85</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="N10" t="n">
-        <v>44.82</v>
+        <v>42.74</v>
       </c>
       <c r="O10" t="n">
-        <v>44.89</v>
+        <v>43</v>
       </c>
       <c r="P10" t="n">
-        <v>42.57</v>
+        <v>41.99</v>
       </c>
       <c r="Q10" t="n">
-        <v>42.57</v>
+        <v>42.22</v>
       </c>
       <c r="R10" t="n">
-        <v>16.3314</v>
+        <v>7.6184</v>
       </c>
       <c r="S10" t="n">
-        <v>22.7386</v>
+        <v>14.8146</v>
       </c>
       <c r="T10" t="n">
-        <v>35.6902</v>
+        <v>49.2905</v>
       </c>
       <c r="U10" t="n">
-        <v>6.9246</v>
+        <v>0.8915</v>
       </c>
       <c r="V10" t="n">
-        <v>13.1919</v>
+        <v>7.5311</v>
       </c>
       <c r="W10" t="n">
-        <v>16.8147</v>
+        <v>18.5642</v>
       </c>
       <c r="X10" t="n">
-        <v>-16.5094</v>
+        <v>-7.3446</v>
       </c>
       <c r="Y10" t="n">
-        <v>-23.1103</v>
+        <v>-16.4118</v>
       </c>
       <c r="Z10" t="n">
-        <v>-31.8182</v>
+        <v>-38.1599</v>
       </c>
       <c r="AA10" t="n">
-        <v>-6.9101</v>
+        <v>-0.8222</v>
       </c>
       <c r="AB10" t="n">
-        <v>-12.3894</v>
+        <v>-7.392</v>
       </c>
       <c r="AC10" t="n">
-        <v>-15.233</v>
+        <v>-16.4126</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>181</v>
+        <v>177.62</v>
       </c>
       <c r="C11" t="n">
-        <v>191.29</v>
+        <v>182.24</v>
       </c>
       <c r="D11" t="n">
-        <v>178.94</v>
+        <v>150.58</v>
       </c>
       <c r="E11" t="n">
-        <v>190.42</v>
+        <v>172.52</v>
       </c>
       <c r="F11" t="n">
-        <v>76</v>
+        <v>75.3</v>
       </c>
       <c r="G11" t="n">
-        <v>77.36</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>75.55</v>
+        <v>71.55</v>
       </c>
       <c r="I11" t="n">
-        <v>76.95999999999999</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>8.65</v>
+        <v>8.75</v>
       </c>
       <c r="K11" t="n">
-        <v>8.77</v>
+        <v>9.91</v>
       </c>
       <c r="L11" t="n">
-        <v>8.15</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="M11" t="n">
-        <v>8.199999999999999</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>42.74</v>
+        <v>43.14</v>
       </c>
       <c r="O11" t="n">
-        <v>43</v>
+        <v>45.19</v>
       </c>
       <c r="P11" t="n">
-        <v>41.99</v>
+        <v>42.79</v>
       </c>
       <c r="Q11" t="n">
-        <v>42.22</v>
+        <v>43.31</v>
       </c>
       <c r="R11" t="n">
-        <v>7.6184</v>
+        <v>-9.4003</v>
       </c>
       <c r="S11" t="n">
-        <v>14.8146</v>
+        <v>13.4254</v>
       </c>
       <c r="T11" t="n">
-        <v>49.2905</v>
+        <v>19.6726</v>
       </c>
       <c r="U11" t="n">
-        <v>0.8915</v>
+        <v>-2.5988</v>
       </c>
       <c r="V11" t="n">
-        <v>7.5311</v>
+        <v>5.0743</v>
       </c>
       <c r="W11" t="n">
-        <v>18.5642</v>
+        <v>11.2331</v>
       </c>
       <c r="X11" t="n">
-        <v>-7.3446</v>
+        <v>9.1463</v>
       </c>
       <c r="Y11" t="n">
-        <v>-16.4118</v>
+        <v>-15.566</v>
       </c>
       <c r="Z11" t="n">
-        <v>-38.1599</v>
+        <v>-22.2415</v>
       </c>
       <c r="AA11" t="n">
-        <v>-0.8222</v>
+        <v>2.5817</v>
       </c>
       <c r="AB11" t="n">
-        <v>-7.392</v>
+        <v>-5.2919</v>
       </c>
       <c r="AC11" t="n">
-        <v>-16.4126</v>
+        <v>-10.8664</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>177.62</v>
+        <v>183.84</v>
       </c>
       <c r="C12" t="n">
-        <v>182.24</v>
+        <v>188.49</v>
       </c>
       <c r="D12" t="n">
-        <v>150.58</v>
+        <v>172.26</v>
       </c>
       <c r="E12" t="n">
-        <v>172.52</v>
+        <v>184.24</v>
       </c>
       <c r="F12" t="n">
-        <v>75.3</v>
+        <v>75.81</v>
       </c>
       <c r="G12" t="n">
-        <v>75.93000000000001</v>
+        <v>77.94</v>
       </c>
       <c r="H12" t="n">
-        <v>71.55</v>
+        <v>74.19</v>
       </c>
       <c r="I12" t="n">
-        <v>74.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>8.75</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>9.91</v>
+        <v>8.98</v>
       </c>
       <c r="L12" t="n">
-        <v>8.550000000000001</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="M12" t="n">
-        <v>8.949999999999999</v>
+        <v>8.35</v>
       </c>
       <c r="N12" t="n">
-        <v>43.14</v>
+        <v>42.83</v>
       </c>
       <c r="O12" t="n">
-        <v>45.19</v>
+        <v>43.77</v>
       </c>
       <c r="P12" t="n">
-        <v>42.79</v>
+        <v>41.6</v>
       </c>
       <c r="Q12" t="n">
-        <v>43.31</v>
+        <v>41.99</v>
       </c>
       <c r="R12" t="n">
-        <v>-9.4003</v>
+        <v>6.7934</v>
       </c>
       <c r="S12" t="n">
-        <v>13.4254</v>
+        <v>4.1257</v>
       </c>
       <c r="T12" t="n">
-        <v>19.6726</v>
+        <v>11.0883</v>
       </c>
       <c r="U12" t="n">
-        <v>-2.5988</v>
+        <v>3.0416</v>
       </c>
       <c r="V12" t="n">
-        <v>5.0743</v>
+        <v>1.2585</v>
       </c>
       <c r="W12" t="n">
-        <v>11.2331</v>
+        <v>7.9223</v>
       </c>
       <c r="X12" t="n">
-        <v>9.1463</v>
+        <v>-6.7039</v>
       </c>
       <c r="Y12" t="n">
-        <v>-15.566</v>
+        <v>-5.6497</v>
       </c>
       <c r="Z12" t="n">
-        <v>-22.2415</v>
+        <v>-14.8828</v>
       </c>
       <c r="AA12" t="n">
-        <v>2.5817</v>
+        <v>-3.0478</v>
       </c>
       <c r="AB12" t="n">
-        <v>-5.2919</v>
+        <v>-1.3625</v>
       </c>
       <c r="AC12" t="n">
-        <v>-10.8664</v>
+        <v>-7.8965</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>183.84</v>
+        <v>182.67</v>
       </c>
       <c r="C13" t="n">
-        <v>188.49</v>
+        <v>189.56</v>
       </c>
       <c r="D13" t="n">
-        <v>172.26</v>
+        <v>178.28</v>
       </c>
       <c r="E13" t="n">
-        <v>184.24</v>
+        <v>186.19</v>
       </c>
       <c r="F13" t="n">
-        <v>75.81</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>77.94</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H13" t="n">
-        <v>74.19</v>
+        <v>77.16</v>
       </c>
       <c r="I13" t="n">
-        <v>77.23999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="J13" t="n">
-        <v>8.380000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="K13" t="n">
-        <v>8.98</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L13" t="n">
-        <v>8.140000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M13" t="n">
-        <v>8.35</v>
+        <v>8.27</v>
       </c>
       <c r="N13" t="n">
-        <v>42.83</v>
+        <v>41.98</v>
       </c>
       <c r="O13" t="n">
-        <v>43.77</v>
+        <v>42.06</v>
       </c>
       <c r="P13" t="n">
-        <v>41.6</v>
+        <v>40.68</v>
       </c>
       <c r="Q13" t="n">
-        <v>41.99</v>
+        <v>41.07</v>
       </c>
       <c r="R13" t="n">
-        <v>6.7934</v>
+        <v>1.0584</v>
       </c>
       <c r="S13" t="n">
-        <v>4.1257</v>
+        <v>-2.2214</v>
       </c>
       <c r="T13" t="n">
-        <v>11.0883</v>
+        <v>22.4129</v>
       </c>
       <c r="U13" t="n">
-        <v>3.0416</v>
+        <v>2.2139</v>
       </c>
       <c r="V13" t="n">
-        <v>1.2585</v>
+        <v>2.5858</v>
       </c>
       <c r="W13" t="n">
-        <v>7.9223</v>
+        <v>10.6672</v>
       </c>
       <c r="X13" t="n">
-        <v>-6.7039</v>
+        <v>-0.9581</v>
       </c>
       <c r="Y13" t="n">
-        <v>-5.6497</v>
+        <v>0.8537</v>
       </c>
       <c r="Z13" t="n">
-        <v>-14.8828</v>
+        <v>-21.9811</v>
       </c>
       <c r="AA13" t="n">
-        <v>-3.0478</v>
+        <v>-2.191</v>
       </c>
       <c r="AB13" t="n">
-        <v>-1.3625</v>
+        <v>-2.7238</v>
       </c>
       <c r="AC13" t="n">
-        <v>-7.8965</v>
+        <v>-10.1902</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>182.67</v>
+        <v>167</v>
       </c>
       <c r="C14" t="n">
-        <v>189.56</v>
+        <v>174.4</v>
       </c>
       <c r="D14" t="n">
-        <v>178.28</v>
+        <v>161.14</v>
       </c>
       <c r="E14" t="n">
-        <v>186.19</v>
+        <v>164.18</v>
       </c>
       <c r="F14" t="n">
-        <v>77.29000000000001</v>
+        <v>75.73</v>
       </c>
       <c r="G14" t="n">
-        <v>79.68000000000001</v>
+        <v>77.37</v>
       </c>
       <c r="H14" t="n">
-        <v>77.16</v>
+        <v>74.23</v>
       </c>
       <c r="I14" t="n">
-        <v>78.95</v>
+        <v>75.34</v>
       </c>
       <c r="J14" t="n">
-        <v>8.43</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>8.630000000000001</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="L14" t="n">
-        <v>8.119999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M14" t="n">
-        <v>8.27</v>
+        <v>9.23</v>
       </c>
       <c r="N14" t="n">
-        <v>41.98</v>
+        <v>42.77</v>
       </c>
       <c r="O14" t="n">
-        <v>42.06</v>
+        <v>43.57</v>
       </c>
       <c r="P14" t="n">
-        <v>40.68</v>
+        <v>41.93</v>
       </c>
       <c r="Q14" t="n">
-        <v>41.07</v>
+        <v>42.98</v>
       </c>
       <c r="R14" t="n">
-        <v>1.0584</v>
+        <v>-11.8213</v>
       </c>
       <c r="S14" t="n">
-        <v>-2.2214</v>
+        <v>-4.8342</v>
       </c>
       <c r="T14" t="n">
-        <v>22.4129</v>
+        <v>-7.2115</v>
       </c>
       <c r="U14" t="n">
-        <v>2.2139</v>
+        <v>-4.5725</v>
       </c>
       <c r="V14" t="n">
-        <v>2.5858</v>
+        <v>0.5069</v>
       </c>
       <c r="W14" t="n">
-        <v>10.6672</v>
+        <v>-1.2323</v>
       </c>
       <c r="X14" t="n">
-        <v>-0.9581</v>
+        <v>11.6082</v>
       </c>
       <c r="Y14" t="n">
-        <v>0.8537</v>
+        <v>3.1285</v>
       </c>
       <c r="Z14" t="n">
-        <v>-21.9811</v>
+        <v>4.2938</v>
       </c>
       <c r="AA14" t="n">
-        <v>-2.191</v>
+        <v>4.6506</v>
       </c>
       <c r="AB14" t="n">
-        <v>-2.7238</v>
+        <v>-0.7619</v>
       </c>
       <c r="AC14" t="n">
-        <v>-10.1902</v>
+        <v>0.9631</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>167</v>
+        <v>172.95</v>
       </c>
       <c r="C15" t="n">
-        <v>174.4</v>
+        <v>174.61</v>
       </c>
       <c r="D15" t="n">
-        <v>161.14</v>
+        <v>142.69</v>
       </c>
       <c r="E15" t="n">
-        <v>164.18</v>
+        <v>151.75</v>
       </c>
       <c r="F15" t="n">
-        <v>75.73</v>
+        <v>76.13</v>
       </c>
       <c r="G15" t="n">
-        <v>77.37</v>
+        <v>76.27</v>
       </c>
       <c r="H15" t="n">
-        <v>74.23</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I15" t="n">
-        <v>75.34</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>9.130000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="K15" t="n">
-        <v>9.390000000000001</v>
+        <v>10.47</v>
       </c>
       <c r="L15" t="n">
-        <v>8.800000000000001</v>
+        <v>8.68</v>
       </c>
       <c r="M15" t="n">
-        <v>9.23</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="N15" t="n">
-        <v>42.77</v>
+        <v>42.51</v>
       </c>
       <c r="O15" t="n">
-        <v>43.57</v>
+        <v>44.82</v>
       </c>
       <c r="P15" t="n">
-        <v>41.93</v>
+        <v>42.44</v>
       </c>
       <c r="Q15" t="n">
-        <v>42.98</v>
+        <v>43.54</v>
       </c>
       <c r="R15" t="n">
-        <v>-11.8213</v>
+        <v>-7.571</v>
       </c>
       <c r="S15" t="n">
-        <v>-4.8342</v>
+        <v>-17.6346</v>
       </c>
       <c r="T15" t="n">
-        <v>-7.2115</v>
+        <v>-20.3077</v>
       </c>
       <c r="U15" t="n">
-        <v>-4.5725</v>
+        <v>-1.3539</v>
       </c>
       <c r="V15" t="n">
-        <v>0.5069</v>
+        <v>-3.7804</v>
       </c>
       <c r="W15" t="n">
-        <v>-1.2323</v>
+        <v>-3.4304</v>
       </c>
       <c r="X15" t="n">
-        <v>11.6082</v>
+        <v>7.8007</v>
       </c>
       <c r="Y15" t="n">
-        <v>3.1285</v>
+        <v>19.1617</v>
       </c>
       <c r="Z15" t="n">
-        <v>4.2938</v>
+        <v>21.3415</v>
       </c>
       <c r="AA15" t="n">
-        <v>4.6506</v>
+        <v>1.3029</v>
       </c>
       <c r="AB15" t="n">
-        <v>-0.7619</v>
+        <v>3.6914</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.9631</v>
+        <v>3.1265</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>172.95</v>
+        <v>141.24</v>
       </c>
       <c r="C16" t="n">
-        <v>174.61</v>
+        <v>160.6</v>
       </c>
       <c r="D16" t="n">
-        <v>142.69</v>
+        <v>135.02</v>
       </c>
       <c r="E16" t="n">
-        <v>151.75</v>
+        <v>151.89</v>
       </c>
       <c r="F16" t="n">
-        <v>76.13</v>
+        <v>72.41</v>
       </c>
       <c r="G16" t="n">
-        <v>76.27</v>
+        <v>74.5</v>
       </c>
       <c r="H16" t="n">
-        <v>72.09999999999999</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="I16" t="n">
-        <v>74.31999999999999</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J16" t="n">
-        <v>8.77</v>
+        <v>10.64</v>
       </c>
       <c r="K16" t="n">
-        <v>10.47</v>
+        <v>11.07</v>
       </c>
       <c r="L16" t="n">
-        <v>8.68</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="M16" t="n">
-        <v>9.949999999999999</v>
+        <v>9.93</v>
       </c>
       <c r="N16" t="n">
-        <v>42.51</v>
+        <v>44.68</v>
       </c>
       <c r="O16" t="n">
-        <v>44.82</v>
+        <v>45.53</v>
       </c>
       <c r="P16" t="n">
-        <v>42.44</v>
+        <v>43.46</v>
       </c>
       <c r="Q16" t="n">
-        <v>43.54</v>
+        <v>44.37</v>
       </c>
       <c r="R16" t="n">
-        <v>-7.571</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="S16" t="n">
-        <v>-17.6346</v>
+        <v>-18.422</v>
       </c>
       <c r="T16" t="n">
-        <v>-20.3077</v>
+        <v>-11.958</v>
       </c>
       <c r="U16" t="n">
-        <v>-1.3539</v>
+        <v>-1.8703</v>
       </c>
       <c r="V16" t="n">
-        <v>-3.7804</v>
+        <v>-7.6251</v>
       </c>
       <c r="W16" t="n">
-        <v>-3.4304</v>
+        <v>-2.7081</v>
       </c>
       <c r="X16" t="n">
-        <v>7.8007</v>
+        <v>-0.201</v>
       </c>
       <c r="Y16" t="n">
-        <v>19.1617</v>
+        <v>20.0726</v>
       </c>
       <c r="Z16" t="n">
-        <v>21.3415</v>
+        <v>10.9497</v>
       </c>
       <c r="AA16" t="n">
-        <v>1.3029</v>
+        <v>1.9063</v>
       </c>
       <c r="AB16" t="n">
-        <v>3.6914</v>
+        <v>8.0351</v>
       </c>
       <c r="AC16" t="n">
-        <v>3.1265</v>
+        <v>2.4475</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>141.24</v>
+        <v>161</v>
       </c>
       <c r="C17" t="n">
-        <v>160.6</v>
+        <v>173.7</v>
       </c>
       <c r="D17" t="n">
-        <v>135.02</v>
+        <v>161</v>
       </c>
       <c r="E17" t="n">
-        <v>151.89</v>
+        <v>173.2</v>
       </c>
       <c r="F17" t="n">
-        <v>72.41</v>
+        <v>74.09</v>
       </c>
       <c r="G17" t="n">
-        <v>74.5</v>
+        <v>76.53</v>
       </c>
       <c r="H17" t="n">
-        <v>70.95999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="I17" t="n">
-        <v>72.93000000000001</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J17" t="n">
-        <v>10.64</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K17" t="n">
-        <v>11.07</v>
+        <v>9.35</v>
       </c>
       <c r="L17" t="n">
-        <v>9.369999999999999</v>
+        <v>8.51</v>
       </c>
       <c r="M17" t="n">
-        <v>9.93</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N17" t="n">
-        <v>44.68</v>
+        <v>43.67</v>
       </c>
       <c r="O17" t="n">
-        <v>45.53</v>
+        <v>43.97</v>
       </c>
       <c r="P17" t="n">
-        <v>43.46</v>
+        <v>42.19</v>
       </c>
       <c r="Q17" t="n">
-        <v>44.37</v>
+        <v>42.19</v>
       </c>
       <c r="R17" t="n">
-        <v>0.09229999999999999</v>
+        <v>14.0299</v>
       </c>
       <c r="S17" t="n">
-        <v>-18.422</v>
+        <v>5.494</v>
       </c>
       <c r="T17" t="n">
-        <v>-11.958</v>
+        <v>-5.9922</v>
       </c>
       <c r="U17" t="n">
-        <v>-1.8703</v>
+        <v>4.9088</v>
       </c>
       <c r="V17" t="n">
-        <v>-7.6251</v>
+        <v>1.553</v>
       </c>
       <c r="W17" t="n">
-        <v>-2.7081</v>
+        <v>-0.9451000000000001</v>
       </c>
       <c r="X17" t="n">
-        <v>-0.201</v>
+        <v>-13.998</v>
       </c>
       <c r="Y17" t="n">
-        <v>20.0726</v>
+        <v>-7.4756</v>
       </c>
       <c r="Z17" t="n">
-        <v>10.9497</v>
+        <v>2.2754</v>
       </c>
       <c r="AA17" t="n">
-        <v>1.9063</v>
+        <v>-4.9132</v>
       </c>
       <c r="AB17" t="n">
-        <v>8.0351</v>
+        <v>-1.8381</v>
       </c>
       <c r="AC17" t="n">
-        <v>2.4475</v>
+        <v>0.4763</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>161</v>
+        <v>171.26</v>
       </c>
       <c r="C18" t="n">
-        <v>173.7</v>
+        <v>179.97</v>
       </c>
       <c r="D18" t="n">
-        <v>161</v>
+        <v>168.23</v>
       </c>
       <c r="E18" t="n">
-        <v>173.2</v>
+        <v>178.39</v>
       </c>
       <c r="F18" t="n">
-        <v>74.09</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>76.53</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H18" t="n">
-        <v>73.62</v>
+        <v>74.47</v>
       </c>
       <c r="I18" t="n">
-        <v>76.51000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J18" t="n">
-        <v>9.300000000000001</v>
+        <v>8.65</v>
       </c>
       <c r="K18" t="n">
-        <v>9.35</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L18" t="n">
-        <v>8.51</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M18" t="n">
-        <v>8.539999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N18" t="n">
-        <v>43.67</v>
+        <v>42.94</v>
       </c>
       <c r="O18" t="n">
-        <v>43.97</v>
+        <v>43.33</v>
       </c>
       <c r="P18" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="Q18" t="n">
-        <v>42.19</v>
+        <v>41.96</v>
       </c>
       <c r="R18" t="n">
-        <v>14.0299</v>
+        <v>2.9965</v>
       </c>
       <c r="S18" t="n">
-        <v>5.494</v>
+        <v>17.5552</v>
       </c>
       <c r="T18" t="n">
-        <v>-5.9922</v>
+        <v>-4.1893</v>
       </c>
       <c r="U18" t="n">
-        <v>4.9088</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="V18" t="n">
-        <v>1.553</v>
+        <v>3.5388</v>
       </c>
       <c r="W18" t="n">
-        <v>-0.9451000000000001</v>
+        <v>-2.5332</v>
       </c>
       <c r="X18" t="n">
-        <v>-13.998</v>
+        <v>-2.9274</v>
       </c>
       <c r="Y18" t="n">
-        <v>-7.4756</v>
+        <v>-16.6834</v>
       </c>
       <c r="Z18" t="n">
-        <v>2.2754</v>
+        <v>0.2418</v>
       </c>
       <c r="AA18" t="n">
-        <v>-4.9132</v>
+        <v>-0.5452</v>
       </c>
       <c r="AB18" t="n">
-        <v>-1.8381</v>
+        <v>-3.6288</v>
       </c>
       <c r="AC18" t="n">
-        <v>0.4763</v>
+        <v>2.167</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>171.26</v>
+        <v>184.8</v>
       </c>
       <c r="C19" t="n">
-        <v>179.97</v>
+        <v>195.27</v>
       </c>
       <c r="D19" t="n">
-        <v>168.23</v>
+        <v>183.34</v>
       </c>
       <c r="E19" t="n">
-        <v>178.39</v>
+        <v>190.56</v>
       </c>
       <c r="F19" t="n">
-        <v>75.18000000000001</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>77.79000000000001</v>
+        <v>79.33</v>
       </c>
       <c r="H19" t="n">
-        <v>74.47</v>
+        <v>77.33</v>
       </c>
       <c r="I19" t="n">
-        <v>76.95</v>
+        <v>77.84</v>
       </c>
       <c r="J19" t="n">
-        <v>8.65</v>
+        <v>8</v>
       </c>
       <c r="K19" t="n">
-        <v>8.779999999999999</v>
+        <v>8.06</v>
       </c>
       <c r="L19" t="n">
-        <v>8.210000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="M19" t="n">
-        <v>8.289999999999999</v>
+        <v>7.73</v>
       </c>
       <c r="N19" t="n">
-        <v>42.94</v>
+        <v>41.4</v>
       </c>
       <c r="O19" t="n">
-        <v>43.33</v>
+        <v>41.78</v>
       </c>
       <c r="P19" t="n">
+        <v>40.68</v>
+      </c>
+      <c r="Q19" t="n">
         <v>41.5</v>
       </c>
-      <c r="Q19" t="n">
-        <v>41.96</v>
-      </c>
       <c r="R19" t="n">
-        <v>2.9965</v>
+        <v>6.8221</v>
       </c>
       <c r="S19" t="n">
-        <v>17.5552</v>
+        <v>25.4592</v>
       </c>
       <c r="T19" t="n">
-        <v>-4.1893</v>
+        <v>16.0677</v>
       </c>
       <c r="U19" t="n">
-        <v>0.5750999999999999</v>
+        <v>1.1566</v>
       </c>
       <c r="V19" t="n">
-        <v>3.5388</v>
+        <v>6.7325</v>
       </c>
       <c r="W19" t="n">
-        <v>-2.5332</v>
+        <v>3.3183</v>
       </c>
       <c r="X19" t="n">
-        <v>-2.9274</v>
+        <v>-6.7551</v>
       </c>
       <c r="Y19" t="n">
-        <v>-16.6834</v>
+        <v>-22.1551</v>
       </c>
       <c r="Z19" t="n">
-        <v>0.2418</v>
+        <v>-16.2514</v>
       </c>
       <c r="AA19" t="n">
-        <v>-0.5452</v>
+        <v>-1.0963</v>
       </c>
       <c r="AB19" t="n">
-        <v>-3.6288</v>
+        <v>-6.4683</v>
       </c>
       <c r="AC19" t="n">
-        <v>2.167</v>
+        <v>-3.4435</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>184.8</v>
+        <v>211.38</v>
       </c>
       <c r="C20" t="n">
-        <v>195.27</v>
+        <v>228.5</v>
       </c>
       <c r="D20" t="n">
-        <v>183.34</v>
+        <v>209.89</v>
       </c>
       <c r="E20" t="n">
-        <v>190.56</v>
+        <v>225.79</v>
       </c>
       <c r="F20" t="n">
-        <v>78.04000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="G20" t="n">
-        <v>79.33</v>
+        <v>82.27</v>
       </c>
       <c r="H20" t="n">
-        <v>77.33</v>
+        <v>79.98</v>
       </c>
       <c r="I20" t="n">
-        <v>77.84</v>
+        <v>81.95</v>
       </c>
       <c r="J20" t="n">
-        <v>8</v>
+        <v>6.9</v>
       </c>
       <c r="K20" t="n">
-        <v>8.06</v>
+        <v>6.95</v>
       </c>
       <c r="L20" t="n">
-        <v>7.5</v>
+        <v>6.19</v>
       </c>
       <c r="M20" t="n">
-        <v>7.73</v>
+        <v>6.29</v>
       </c>
       <c r="N20" t="n">
-        <v>41.4</v>
+        <v>40.05</v>
       </c>
       <c r="O20" t="n">
-        <v>41.78</v>
+        <v>40.35</v>
       </c>
       <c r="P20" t="n">
-        <v>40.68</v>
+        <v>39.14</v>
       </c>
       <c r="Q20" t="n">
-        <v>41.5</v>
+        <v>39.28</v>
       </c>
       <c r="R20" t="n">
-        <v>6.8221</v>
+        <v>18.4876</v>
       </c>
       <c r="S20" t="n">
-        <v>25.4592</v>
+        <v>30.3637</v>
       </c>
       <c r="T20" t="n">
-        <v>16.0677</v>
+        <v>48.7908</v>
       </c>
       <c r="U20" t="n">
-        <v>1.1566</v>
+        <v>5.2801</v>
       </c>
       <c r="V20" t="n">
-        <v>6.7325</v>
+        <v>7.1102</v>
       </c>
       <c r="W20" t="n">
-        <v>3.3183</v>
+        <v>10.2664</v>
       </c>
       <c r="X20" t="n">
-        <v>-6.7551</v>
+        <v>-18.6287</v>
       </c>
       <c r="Y20" t="n">
-        <v>-22.1551</v>
+        <v>-26.3466</v>
       </c>
       <c r="Z20" t="n">
-        <v>-16.2514</v>
+        <v>-36.7839</v>
       </c>
       <c r="AA20" t="n">
-        <v>-1.0963</v>
+        <v>-5.3494</v>
       </c>
       <c r="AB20" t="n">
-        <v>-6.4683</v>
+        <v>-6.8974</v>
       </c>
       <c r="AC20" t="n">
-        <v>-3.4435</v>
+        <v>-9.7841</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>211.38</v>
+        <v>242.66</v>
       </c>
       <c r="C21" t="n">
-        <v>228.5</v>
+        <v>242.66</v>
       </c>
       <c r="D21" t="n">
-        <v>209.89</v>
+        <v>204</v>
       </c>
       <c r="E21" t="n">
-        <v>225.79</v>
+        <v>217.98</v>
       </c>
       <c r="F21" t="n">
-        <v>80.59</v>
+        <v>82.87</v>
       </c>
       <c r="G21" t="n">
-        <v>82.27</v>
+        <v>82.91</v>
       </c>
       <c r="H21" t="n">
-        <v>79.98</v>
+        <v>80.33</v>
       </c>
       <c r="I21" t="n">
-        <v>81.95</v>
+        <v>81.67</v>
       </c>
       <c r="J21" t="n">
-        <v>6.9</v>
+        <v>5.83</v>
       </c>
       <c r="K21" t="n">
-        <v>6.95</v>
+        <v>6.91</v>
       </c>
       <c r="L21" t="n">
-        <v>6.19</v>
+        <v>5.83</v>
       </c>
       <c r="M21" t="n">
-        <v>6.29</v>
+        <v>6.53</v>
       </c>
       <c r="N21" t="n">
-        <v>40.05</v>
+        <v>38.87</v>
       </c>
       <c r="O21" t="n">
-        <v>40.35</v>
+        <v>40.09</v>
       </c>
       <c r="P21" t="n">
-        <v>39.14</v>
+        <v>38.86</v>
       </c>
       <c r="Q21" t="n">
-        <v>39.28</v>
+        <v>39.44</v>
       </c>
       <c r="R21" t="n">
-        <v>18.4876</v>
+        <v>-3.459</v>
       </c>
       <c r="S21" t="n">
-        <v>30.3637</v>
+        <v>22.1929</v>
       </c>
       <c r="T21" t="n">
-        <v>48.7908</v>
+        <v>43.5118</v>
       </c>
       <c r="U21" t="n">
-        <v>5.2801</v>
+        <v>-0.3417</v>
       </c>
       <c r="V21" t="n">
-        <v>7.1102</v>
+        <v>6.1339</v>
       </c>
       <c r="W21" t="n">
-        <v>10.2664</v>
+        <v>11.9841</v>
       </c>
       <c r="X21" t="n">
-        <v>-18.6287</v>
+        <v>3.8156</v>
       </c>
       <c r="Y21" t="n">
-        <v>-26.3466</v>
+        <v>-21.2304</v>
       </c>
       <c r="Z21" t="n">
-        <v>-36.7839</v>
+        <v>-34.2397</v>
       </c>
       <c r="AA21" t="n">
-        <v>-5.3494</v>
+        <v>0.4073</v>
       </c>
       <c r="AB21" t="n">
-        <v>-6.8974</v>
+        <v>-6.0057</v>
       </c>
       <c r="AC21" t="n">
-        <v>-9.7841</v>
+        <v>-11.1111</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>242.66</v>
+        <v>219</v>
       </c>
       <c r="C22" t="n">
-        <v>242.66</v>
+        <v>231.89</v>
       </c>
       <c r="D22" t="n">
-        <v>204</v>
+        <v>207.61</v>
       </c>
       <c r="E22" t="n">
-        <v>217.98</v>
+        <v>224.63</v>
       </c>
       <c r="F22" t="n">
-        <v>82.87</v>
+        <v>81.73</v>
       </c>
       <c r="G22" t="n">
-        <v>82.90000000000001</v>
+        <v>84.05</v>
       </c>
       <c r="H22" t="n">
-        <v>80.33</v>
+        <v>80.66</v>
       </c>
       <c r="I22" t="n">
-        <v>81.67</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="J22" t="n">
-        <v>5.83</v>
+        <v>6.49</v>
       </c>
       <c r="K22" t="n">
-        <v>6.91</v>
+        <v>6.83</v>
       </c>
       <c r="L22" t="n">
-        <v>5.84</v>
+        <v>6.1</v>
       </c>
       <c r="M22" t="n">
-        <v>6.53</v>
+        <v>6.31</v>
       </c>
       <c r="N22" t="n">
-        <v>38.87</v>
+        <v>39.41</v>
       </c>
       <c r="O22" t="n">
-        <v>40.09</v>
+        <v>39.94</v>
       </c>
       <c r="P22" t="n">
-        <v>38.86</v>
+        <v>38.3</v>
       </c>
       <c r="Q22" t="n">
-        <v>39.44</v>
+        <v>38.47</v>
       </c>
       <c r="R22" t="n">
-        <v>-3.459</v>
+        <v>3.0507</v>
       </c>
       <c r="S22" t="n">
-        <v>22.1929</v>
+        <v>17.8789</v>
       </c>
       <c r="T22" t="n">
-        <v>43.5118</v>
+        <v>29.694</v>
       </c>
       <c r="U22" t="n">
-        <v>-0.3417</v>
+        <v>2.4611</v>
       </c>
       <c r="V22" t="n">
-        <v>6.1339</v>
+        <v>7.5026</v>
       </c>
       <c r="W22" t="n">
-        <v>11.9841</v>
+        <v>9.3713</v>
       </c>
       <c r="X22" t="n">
-        <v>3.8156</v>
+        <v>-3.3691</v>
       </c>
       <c r="Y22" t="n">
-        <v>-21.2304</v>
+        <v>-18.37</v>
       </c>
       <c r="Z22" t="n">
-        <v>-34.2397</v>
+        <v>-26.1124</v>
       </c>
       <c r="AA22" t="n">
-        <v>0.4073</v>
+        <v>-2.4594</v>
       </c>
       <c r="AB22" t="n">
-        <v>-6.0057</v>
+        <v>-7.3012</v>
       </c>
       <c r="AC22" t="n">
-        <v>-11.1111</v>
+        <v>-8.817299999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-05-29 23:13
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>114.76</v>
+        <v>122.81</v>
       </c>
       <c r="C2" t="n">
-        <v>118.32</v>
+        <v>127.45</v>
       </c>
       <c r="D2" t="n">
-        <v>112.3</v>
+        <v>117.5</v>
       </c>
       <c r="E2" t="n">
-        <v>117.97</v>
+        <v>126.98</v>
       </c>
       <c r="F2" t="n">
-        <v>61</v>
+        <v>62.89</v>
       </c>
       <c r="G2" t="n">
-        <v>61.87</v>
+        <v>63.8</v>
       </c>
       <c r="H2" t="n">
-        <v>60.45</v>
+        <v>60.7</v>
       </c>
       <c r="I2" t="n">
-        <v>61.86</v>
+        <v>63.54</v>
       </c>
       <c r="J2" t="n">
-        <v>14.91</v>
+        <v>13.84</v>
       </c>
       <c r="K2" t="n">
-        <v>15.24</v>
+        <v>14.49</v>
       </c>
       <c r="L2" t="n">
-        <v>14.38</v>
+        <v>13.25</v>
       </c>
       <c r="M2" t="n">
-        <v>14.4</v>
+        <v>13.3</v>
       </c>
       <c r="N2" t="n">
-        <v>53.84</v>
+        <v>52.21</v>
       </c>
       <c r="O2" t="n">
-        <v>54.33</v>
+        <v>54.09</v>
       </c>
       <c r="P2" t="n">
-        <v>53.06</v>
+        <v>51.4</v>
       </c>
       <c r="Q2" t="n">
-        <v>53.08</v>
+        <v>51.65</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>122.81</v>
+        <v>124.39</v>
       </c>
       <c r="C3" t="n">
-        <v>127.45</v>
+        <v>131.38</v>
       </c>
       <c r="D3" t="n">
-        <v>117.5</v>
+        <v>121.66</v>
       </c>
       <c r="E3" t="n">
-        <v>126.98</v>
+        <v>130.4</v>
       </c>
       <c r="F3" t="n">
-        <v>62.89</v>
+        <v>63.89</v>
       </c>
       <c r="G3" t="n">
-        <v>63.8</v>
+        <v>65.84</v>
       </c>
       <c r="H3" t="n">
-        <v>60.7</v>
+        <v>63.81</v>
       </c>
       <c r="I3" t="n">
-        <v>63.54</v>
+        <v>65.3</v>
       </c>
       <c r="J3" t="n">
-        <v>13.84</v>
+        <v>13.61</v>
       </c>
       <c r="K3" t="n">
-        <v>14.49</v>
+        <v>13.89</v>
       </c>
       <c r="L3" t="n">
-        <v>13.25</v>
+        <v>12.87</v>
       </c>
       <c r="M3" t="n">
-        <v>13.3</v>
+        <v>12.98</v>
       </c>
       <c r="N3" t="n">
-        <v>52.21</v>
+        <v>51.36</v>
       </c>
       <c r="O3" t="n">
-        <v>54.09</v>
+        <v>51.45</v>
       </c>
       <c r="P3" t="n">
-        <v>51.4</v>
+        <v>49.79</v>
       </c>
       <c r="Q3" t="n">
-        <v>51.65</v>
+        <v>50.22</v>
       </c>
       <c r="R3" t="n">
-        <v>7.6375</v>
+        <v>2.6933</v>
       </c>
       <c r="U3" t="n">
-        <v>2.7158</v>
+        <v>2.7699</v>
       </c>
       <c r="X3" t="n">
-        <v>-7.6389</v>
+        <v>-2.406</v>
       </c>
       <c r="AA3" t="n">
-        <v>-2.694</v>
+        <v>-2.7686</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>124.39</v>
+        <v>132.2</v>
       </c>
       <c r="C4" t="n">
-        <v>131.38</v>
+        <v>133.67</v>
       </c>
       <c r="D4" t="n">
-        <v>121.66</v>
+        <v>123.8</v>
       </c>
       <c r="E4" t="n">
-        <v>130.4</v>
+        <v>127.55</v>
       </c>
       <c r="F4" t="n">
-        <v>63.89</v>
+        <v>65.44</v>
       </c>
       <c r="G4" t="n">
-        <v>65.84</v>
+        <v>66.05</v>
       </c>
       <c r="H4" t="n">
-        <v>63.81</v>
+        <v>63.78</v>
       </c>
       <c r="I4" t="n">
-        <v>65.3</v>
+        <v>64.91</v>
       </c>
       <c r="J4" t="n">
-        <v>13.61</v>
+        <v>12.8</v>
       </c>
       <c r="K4" t="n">
-        <v>13.89</v>
+        <v>13.64</v>
       </c>
       <c r="L4" t="n">
-        <v>12.87</v>
+        <v>12.65</v>
       </c>
       <c r="M4" t="n">
-        <v>12.98</v>
+        <v>13.26</v>
       </c>
       <c r="N4" t="n">
-        <v>51.36</v>
+        <v>50.12</v>
       </c>
       <c r="O4" t="n">
-        <v>51.45</v>
+        <v>51.43</v>
       </c>
       <c r="P4" t="n">
-        <v>49.79</v>
+        <v>49.65</v>
       </c>
       <c r="Q4" t="n">
-        <v>50.22</v>
+        <v>50.51</v>
       </c>
       <c r="R4" t="n">
-        <v>2.6933</v>
+        <v>-2.1856</v>
       </c>
       <c r="U4" t="n">
-        <v>2.7699</v>
+        <v>-0.5972</v>
       </c>
       <c r="X4" t="n">
-        <v>-2.406</v>
+        <v>2.1572</v>
       </c>
       <c r="AA4" t="n">
-        <v>-2.7686</v>
+        <v>0.5775</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>132.2</v>
+        <v>135</v>
       </c>
       <c r="C5" t="n">
-        <v>133.67</v>
+        <v>147.26</v>
       </c>
       <c r="D5" t="n">
-        <v>123.8</v>
+        <v>134.02</v>
       </c>
       <c r="E5" t="n">
-        <v>127.55</v>
+        <v>144.16</v>
       </c>
       <c r="F5" t="n">
-        <v>65.44</v>
+        <v>66.37</v>
       </c>
       <c r="G5" t="n">
-        <v>66.05</v>
+        <v>67.77</v>
       </c>
       <c r="H5" t="n">
-        <v>63.78</v>
+        <v>66.25</v>
       </c>
       <c r="I5" t="n">
-        <v>64.91</v>
+        <v>67.39</v>
       </c>
       <c r="J5" t="n">
-        <v>12.8</v>
+        <v>12.5</v>
       </c>
       <c r="K5" t="n">
-        <v>13.64</v>
+        <v>12.59</v>
       </c>
       <c r="L5" t="n">
-        <v>12.65</v>
+        <v>11.21</v>
       </c>
       <c r="M5" t="n">
-        <v>13.26</v>
+        <v>11.51</v>
       </c>
       <c r="N5" t="n">
-        <v>50.12</v>
+        <v>49.4</v>
       </c>
       <c r="O5" t="n">
-        <v>51.43</v>
+        <v>49.49</v>
       </c>
       <c r="P5" t="n">
-        <v>49.65</v>
+        <v>48.3</v>
       </c>
       <c r="Q5" t="n">
-        <v>50.51</v>
+        <v>48.59</v>
       </c>
       <c r="R5" t="n">
-        <v>-2.1856</v>
+        <v>13.0223</v>
       </c>
       <c r="S5" t="n">
-        <v>8.120699999999999</v>
+        <v>13.5297</v>
       </c>
       <c r="U5" t="n">
-        <v>-0.5972</v>
+        <v>3.8207</v>
       </c>
       <c r="V5" t="n">
-        <v>4.9305</v>
+        <v>6.0592</v>
       </c>
       <c r="X5" t="n">
-        <v>2.1572</v>
+        <v>-13.1976</v>
       </c>
       <c r="Y5" t="n">
-        <v>-7.9167</v>
+        <v>-13.4586</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.5775</v>
+        <v>-3.8012</v>
       </c>
       <c r="AB5" t="n">
-        <v>-4.8417</v>
+        <v>-5.9245</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>135</v>
+        <v>157.84</v>
       </c>
       <c r="C6" t="n">
-        <v>147.26</v>
+        <v>166</v>
       </c>
       <c r="D6" t="n">
-        <v>134.02</v>
+        <v>149.06</v>
       </c>
       <c r="E6" t="n">
-        <v>144.16</v>
+        <v>165.85</v>
       </c>
       <c r="F6" t="n">
-        <v>66.37</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>67.77</v>
+        <v>71.66</v>
       </c>
       <c r="H6" t="n">
-        <v>66.25</v>
+        <v>68.88</v>
       </c>
       <c r="I6" t="n">
-        <v>67.39</v>
+        <v>71.56999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>12.5</v>
+        <v>10.43</v>
       </c>
       <c r="K6" t="n">
-        <v>12.59</v>
+        <v>11.14</v>
       </c>
       <c r="L6" t="n">
-        <v>11.21</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M6" t="n">
-        <v>11.51</v>
+        <v>9.81</v>
       </c>
       <c r="N6" t="n">
-        <v>49.4</v>
+        <v>47.26</v>
       </c>
       <c r="O6" t="n">
-        <v>49.49</v>
+        <v>47.54</v>
       </c>
       <c r="P6" t="n">
-        <v>48.3</v>
+        <v>45.52</v>
       </c>
       <c r="Q6" t="n">
-        <v>48.59</v>
+        <v>45.59</v>
       </c>
       <c r="R6" t="n">
-        <v>13.0223</v>
+        <v>15.0458</v>
       </c>
       <c r="S6" t="n">
-        <v>13.5297</v>
+        <v>27.1856</v>
       </c>
       <c r="U6" t="n">
-        <v>3.8207</v>
+        <v>6.2027</v>
       </c>
       <c r="V6" t="n">
-        <v>6.0592</v>
+        <v>9.601800000000001</v>
       </c>
       <c r="X6" t="n">
-        <v>-13.1976</v>
+        <v>-14.7698</v>
       </c>
       <c r="Y6" t="n">
-        <v>-13.4586</v>
+        <v>-24.4222</v>
       </c>
       <c r="AA6" t="n">
-        <v>-3.8012</v>
+        <v>-6.1741</v>
       </c>
       <c r="AB6" t="n">
-        <v>-5.9245</v>
+        <v>-9.2194</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>157.84</v>
+        <v>162.12</v>
       </c>
       <c r="C7" t="n">
-        <v>166</v>
+        <v>162.9</v>
       </c>
       <c r="D7" t="n">
-        <v>149.06</v>
+        <v>147.61</v>
       </c>
       <c r="E7" t="n">
-        <v>165.85</v>
+        <v>152.1</v>
       </c>
       <c r="F7" t="n">
-        <v>69.26000000000001</v>
+        <v>71.87</v>
       </c>
       <c r="G7" t="n">
-        <v>71.66</v>
+        <v>73.3</v>
       </c>
       <c r="H7" t="n">
-        <v>68.88</v>
+        <v>70.38</v>
       </c>
       <c r="I7" t="n">
-        <v>71.56999999999999</v>
+        <v>71.34</v>
       </c>
       <c r="J7" t="n">
-        <v>10.43</v>
+        <v>10.02</v>
       </c>
       <c r="K7" t="n">
-        <v>11.14</v>
+        <v>10.88</v>
       </c>
       <c r="L7" t="n">
-        <v>9.800000000000001</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="M7" t="n">
-        <v>9.81</v>
+        <v>10.6</v>
       </c>
       <c r="N7" t="n">
-        <v>47.26</v>
+        <v>45.41</v>
       </c>
       <c r="O7" t="n">
-        <v>47.54</v>
+        <v>46.36</v>
       </c>
       <c r="P7" t="n">
-        <v>45.52</v>
+        <v>44.5</v>
       </c>
       <c r="Q7" t="n">
-        <v>45.59</v>
+        <v>45.73</v>
       </c>
       <c r="R7" t="n">
-        <v>15.0458</v>
+        <v>-8.2906</v>
       </c>
       <c r="S7" t="n">
-        <v>27.1856</v>
+        <v>19.2474</v>
       </c>
       <c r="T7" t="n">
-        <v>40.5866</v>
+        <v>19.7826</v>
       </c>
       <c r="U7" t="n">
-        <v>6.2027</v>
+        <v>-0.3214</v>
       </c>
       <c r="V7" t="n">
-        <v>9.601800000000001</v>
+        <v>9.906000000000001</v>
       </c>
       <c r="W7" t="n">
-        <v>15.6967</v>
+        <v>12.2757</v>
       </c>
       <c r="X7" t="n">
-        <v>-14.7698</v>
+        <v>8.053000000000001</v>
       </c>
       <c r="Y7" t="n">
-        <v>-24.4222</v>
+        <v>-20.0603</v>
       </c>
       <c r="Z7" t="n">
-        <v>-31.875</v>
+        <v>-20.3008</v>
       </c>
       <c r="AA7" t="n">
-        <v>-6.1741</v>
+        <v>0.3071</v>
       </c>
       <c r="AB7" t="n">
-        <v>-9.2194</v>
+        <v>-9.4635</v>
       </c>
       <c r="AC7" t="n">
-        <v>-14.1108</v>
+        <v>-11.4618</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>162.12</v>
+        <v>163</v>
       </c>
       <c r="C8" t="n">
-        <v>162.9</v>
+        <v>177.5</v>
       </c>
       <c r="D8" t="n">
-        <v>147.61</v>
+        <v>161.51</v>
       </c>
       <c r="E8" t="n">
-        <v>152.1</v>
+        <v>176.94</v>
       </c>
       <c r="F8" t="n">
-        <v>71.87</v>
+        <v>72.81999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>73.3</v>
+        <v>76.31</v>
       </c>
       <c r="H8" t="n">
-        <v>70.38</v>
+        <v>72.7</v>
       </c>
       <c r="I8" t="n">
-        <v>71.34</v>
+        <v>76.28</v>
       </c>
       <c r="J8" t="n">
-        <v>10.02</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="K8" t="n">
-        <v>10.88</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="L8" t="n">
-        <v>9.970000000000001</v>
+        <v>8.84</v>
       </c>
       <c r="M8" t="n">
-        <v>10.6</v>
+        <v>8.85</v>
       </c>
       <c r="N8" t="n">
-        <v>45.41</v>
+        <v>44.82</v>
       </c>
       <c r="O8" t="n">
-        <v>46.36</v>
+        <v>44.89</v>
       </c>
       <c r="P8" t="n">
-        <v>44.5</v>
+        <v>42.57</v>
       </c>
       <c r="Q8" t="n">
-        <v>45.73</v>
+        <v>42.57</v>
       </c>
       <c r="R8" t="n">
-        <v>-8.2906</v>
+        <v>16.3314</v>
       </c>
       <c r="S8" t="n">
-        <v>19.2474</v>
+        <v>22.7386</v>
       </c>
       <c r="T8" t="n">
-        <v>19.7826</v>
+        <v>35.6902</v>
       </c>
       <c r="U8" t="n">
-        <v>-0.3214</v>
+        <v>6.9246</v>
       </c>
       <c r="V8" t="n">
-        <v>9.906000000000001</v>
+        <v>13.1919</v>
       </c>
       <c r="W8" t="n">
-        <v>12.2757</v>
+        <v>16.8147</v>
       </c>
       <c r="X8" t="n">
-        <v>8.053000000000001</v>
+        <v>-16.5094</v>
       </c>
       <c r="Y8" t="n">
-        <v>-20.0603</v>
+        <v>-23.1103</v>
       </c>
       <c r="Z8" t="n">
-        <v>-20.3008</v>
+        <v>-31.8182</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.3071</v>
+        <v>-6.9101</v>
       </c>
       <c r="AB8" t="n">
-        <v>-9.4635</v>
+        <v>-12.3894</v>
       </c>
       <c r="AC8" t="n">
-        <v>-11.4618</v>
+        <v>-15.233</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="C9" t="n">
-        <v>177.5</v>
+        <v>191.29</v>
       </c>
       <c r="D9" t="n">
-        <v>161.51</v>
+        <v>178.94</v>
       </c>
       <c r="E9" t="n">
-        <v>176.94</v>
+        <v>190.42</v>
       </c>
       <c r="F9" t="n">
-        <v>72.81999999999999</v>
+        <v>76</v>
       </c>
       <c r="G9" t="n">
-        <v>76.31</v>
+        <v>77.36</v>
       </c>
       <c r="H9" t="n">
-        <v>72.7</v>
+        <v>75.55</v>
       </c>
       <c r="I9" t="n">
-        <v>76.28</v>
+        <v>76.95999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>9.859999999999999</v>
+        <v>8.65</v>
       </c>
       <c r="K9" t="n">
-        <v>9.970000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="L9" t="n">
-        <v>8.84</v>
+        <v>8.15</v>
       </c>
       <c r="M9" t="n">
-        <v>8.85</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="N9" t="n">
-        <v>44.82</v>
+        <v>42.74</v>
       </c>
       <c r="O9" t="n">
-        <v>44.89</v>
+        <v>43</v>
       </c>
       <c r="P9" t="n">
-        <v>42.57</v>
+        <v>41.99</v>
       </c>
       <c r="Q9" t="n">
-        <v>42.57</v>
+        <v>42.22</v>
       </c>
       <c r="R9" t="n">
-        <v>16.3314</v>
+        <v>7.6184</v>
       </c>
       <c r="S9" t="n">
-        <v>22.7386</v>
+        <v>14.8146</v>
       </c>
       <c r="T9" t="n">
-        <v>35.6902</v>
+        <v>49.2905</v>
       </c>
       <c r="U9" t="n">
-        <v>6.9246</v>
+        <v>0.8915</v>
       </c>
       <c r="V9" t="n">
-        <v>13.1919</v>
+        <v>7.5311</v>
       </c>
       <c r="W9" t="n">
-        <v>16.8147</v>
+        <v>18.5642</v>
       </c>
       <c r="X9" t="n">
-        <v>-16.5094</v>
+        <v>-7.3446</v>
       </c>
       <c r="Y9" t="n">
-        <v>-23.1103</v>
+        <v>-16.4118</v>
       </c>
       <c r="Z9" t="n">
-        <v>-31.8182</v>
+        <v>-38.1599</v>
       </c>
       <c r="AA9" t="n">
-        <v>-6.9101</v>
+        <v>-0.8222</v>
       </c>
       <c r="AB9" t="n">
-        <v>-12.3894</v>
+        <v>-7.392</v>
       </c>
       <c r="AC9" t="n">
-        <v>-15.233</v>
+        <v>-16.4126</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>181</v>
+        <v>177.62</v>
       </c>
       <c r="C10" t="n">
-        <v>191.29</v>
+        <v>182.24</v>
       </c>
       <c r="D10" t="n">
-        <v>178.94</v>
+        <v>150.58</v>
       </c>
       <c r="E10" t="n">
-        <v>190.42</v>
+        <v>172.52</v>
       </c>
       <c r="F10" t="n">
-        <v>76</v>
+        <v>75.3</v>
       </c>
       <c r="G10" t="n">
-        <v>77.36</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>75.55</v>
+        <v>71.55</v>
       </c>
       <c r="I10" t="n">
-        <v>76.95999999999999</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>8.65</v>
+        <v>8.75</v>
       </c>
       <c r="K10" t="n">
-        <v>8.77</v>
+        <v>9.91</v>
       </c>
       <c r="L10" t="n">
-        <v>8.15</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="M10" t="n">
-        <v>8.199999999999999</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N10" t="n">
-        <v>42.74</v>
+        <v>43.14</v>
       </c>
       <c r="O10" t="n">
-        <v>43</v>
+        <v>45.19</v>
       </c>
       <c r="P10" t="n">
-        <v>41.99</v>
+        <v>42.79</v>
       </c>
       <c r="Q10" t="n">
-        <v>42.22</v>
+        <v>43.31</v>
       </c>
       <c r="R10" t="n">
-        <v>7.6184</v>
+        <v>-9.4003</v>
       </c>
       <c r="S10" t="n">
-        <v>14.8146</v>
+        <v>13.4254</v>
       </c>
       <c r="T10" t="n">
-        <v>49.2905</v>
+        <v>19.6726</v>
       </c>
       <c r="U10" t="n">
-        <v>0.8915</v>
+        <v>-2.5988</v>
       </c>
       <c r="V10" t="n">
-        <v>7.5311</v>
+        <v>5.0743</v>
       </c>
       <c r="W10" t="n">
-        <v>18.5642</v>
+        <v>11.2331</v>
       </c>
       <c r="X10" t="n">
-        <v>-7.3446</v>
+        <v>9.1463</v>
       </c>
       <c r="Y10" t="n">
-        <v>-16.4118</v>
+        <v>-15.566</v>
       </c>
       <c r="Z10" t="n">
-        <v>-38.1599</v>
+        <v>-22.2415</v>
       </c>
       <c r="AA10" t="n">
-        <v>-0.8222</v>
+        <v>2.5817</v>
       </c>
       <c r="AB10" t="n">
-        <v>-7.392</v>
+        <v>-5.2919</v>
       </c>
       <c r="AC10" t="n">
-        <v>-16.4126</v>
+        <v>-10.8664</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>177.62</v>
+        <v>183.84</v>
       </c>
       <c r="C11" t="n">
-        <v>182.24</v>
+        <v>188.49</v>
       </c>
       <c r="D11" t="n">
-        <v>150.58</v>
+        <v>172.26</v>
       </c>
       <c r="E11" t="n">
-        <v>172.52</v>
+        <v>184.24</v>
       </c>
       <c r="F11" t="n">
-        <v>75.3</v>
+        <v>75.81</v>
       </c>
       <c r="G11" t="n">
-        <v>75.93000000000001</v>
+        <v>77.94</v>
       </c>
       <c r="H11" t="n">
-        <v>71.55</v>
+        <v>74.19</v>
       </c>
       <c r="I11" t="n">
-        <v>74.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>8.75</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>9.91</v>
+        <v>8.98</v>
       </c>
       <c r="L11" t="n">
-        <v>8.550000000000001</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="M11" t="n">
-        <v>8.949999999999999</v>
+        <v>8.35</v>
       </c>
       <c r="N11" t="n">
-        <v>43.14</v>
+        <v>42.83</v>
       </c>
       <c r="O11" t="n">
-        <v>45.19</v>
+        <v>43.77</v>
       </c>
       <c r="P11" t="n">
-        <v>42.79</v>
+        <v>41.6</v>
       </c>
       <c r="Q11" t="n">
-        <v>43.31</v>
+        <v>41.99</v>
       </c>
       <c r="R11" t="n">
-        <v>-9.4003</v>
+        <v>6.7934</v>
       </c>
       <c r="S11" t="n">
-        <v>13.4254</v>
+        <v>4.1257</v>
       </c>
       <c r="T11" t="n">
-        <v>19.6726</v>
+        <v>11.0883</v>
       </c>
       <c r="U11" t="n">
-        <v>-2.5988</v>
+        <v>3.0416</v>
       </c>
       <c r="V11" t="n">
-        <v>5.0743</v>
+        <v>1.2585</v>
       </c>
       <c r="W11" t="n">
-        <v>11.2331</v>
+        <v>7.9223</v>
       </c>
       <c r="X11" t="n">
-        <v>9.1463</v>
+        <v>-6.7039</v>
       </c>
       <c r="Y11" t="n">
-        <v>-15.566</v>
+        <v>-5.6497</v>
       </c>
       <c r="Z11" t="n">
-        <v>-22.2415</v>
+        <v>-14.8828</v>
       </c>
       <c r="AA11" t="n">
-        <v>2.5817</v>
+        <v>-3.0478</v>
       </c>
       <c r="AB11" t="n">
-        <v>-5.2919</v>
+        <v>-1.3625</v>
       </c>
       <c r="AC11" t="n">
-        <v>-10.8664</v>
+        <v>-7.8965</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>183.84</v>
+        <v>182.67</v>
       </c>
       <c r="C12" t="n">
-        <v>188.49</v>
+        <v>189.56</v>
       </c>
       <c r="D12" t="n">
-        <v>172.26</v>
+        <v>178.28</v>
       </c>
       <c r="E12" t="n">
-        <v>184.24</v>
+        <v>186.19</v>
       </c>
       <c r="F12" t="n">
-        <v>75.81</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>77.94</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>74.19</v>
+        <v>77.16</v>
       </c>
       <c r="I12" t="n">
-        <v>77.23999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="J12" t="n">
-        <v>8.380000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="K12" t="n">
-        <v>8.98</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L12" t="n">
-        <v>8.140000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M12" t="n">
-        <v>8.35</v>
+        <v>8.27</v>
       </c>
       <c r="N12" t="n">
-        <v>42.83</v>
+        <v>41.98</v>
       </c>
       <c r="O12" t="n">
-        <v>43.77</v>
+        <v>42.06</v>
       </c>
       <c r="P12" t="n">
-        <v>41.6</v>
+        <v>40.68</v>
       </c>
       <c r="Q12" t="n">
-        <v>41.99</v>
+        <v>41.07</v>
       </c>
       <c r="R12" t="n">
-        <v>6.7934</v>
+        <v>1.0584</v>
       </c>
       <c r="S12" t="n">
-        <v>4.1257</v>
+        <v>-2.2214</v>
       </c>
       <c r="T12" t="n">
-        <v>11.0883</v>
+        <v>22.4129</v>
       </c>
       <c r="U12" t="n">
-        <v>3.0416</v>
+        <v>2.2139</v>
       </c>
       <c r="V12" t="n">
-        <v>1.2585</v>
+        <v>2.5858</v>
       </c>
       <c r="W12" t="n">
-        <v>7.9223</v>
+        <v>10.6672</v>
       </c>
       <c r="X12" t="n">
-        <v>-6.7039</v>
+        <v>-0.9581</v>
       </c>
       <c r="Y12" t="n">
-        <v>-5.6497</v>
+        <v>0.8537</v>
       </c>
       <c r="Z12" t="n">
-        <v>-14.8828</v>
+        <v>-21.9811</v>
       </c>
       <c r="AA12" t="n">
-        <v>-3.0478</v>
+        <v>-2.191</v>
       </c>
       <c r="AB12" t="n">
-        <v>-1.3625</v>
+        <v>-2.7238</v>
       </c>
       <c r="AC12" t="n">
-        <v>-7.8965</v>
+        <v>-10.1902</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>182.67</v>
+        <v>167</v>
       </c>
       <c r="C13" t="n">
-        <v>189.56</v>
+        <v>174.4</v>
       </c>
       <c r="D13" t="n">
-        <v>178.28</v>
+        <v>161.14</v>
       </c>
       <c r="E13" t="n">
-        <v>186.19</v>
+        <v>164.18</v>
       </c>
       <c r="F13" t="n">
-        <v>77.29000000000001</v>
+        <v>75.73</v>
       </c>
       <c r="G13" t="n">
-        <v>79.68000000000001</v>
+        <v>77.37</v>
       </c>
       <c r="H13" t="n">
-        <v>77.16</v>
+        <v>74.23</v>
       </c>
       <c r="I13" t="n">
-        <v>78.95</v>
+        <v>75.34</v>
       </c>
       <c r="J13" t="n">
-        <v>8.43</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>8.630000000000001</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="L13" t="n">
-        <v>8.119999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M13" t="n">
-        <v>8.27</v>
+        <v>9.23</v>
       </c>
       <c r="N13" t="n">
-        <v>41.98</v>
+        <v>42.77</v>
       </c>
       <c r="O13" t="n">
-        <v>42.06</v>
+        <v>43.57</v>
       </c>
       <c r="P13" t="n">
-        <v>40.68</v>
+        <v>41.93</v>
       </c>
       <c r="Q13" t="n">
-        <v>41.07</v>
+        <v>42.98</v>
       </c>
       <c r="R13" t="n">
-        <v>1.0584</v>
+        <v>-11.8213</v>
       </c>
       <c r="S13" t="n">
-        <v>-2.2214</v>
+        <v>-4.8342</v>
       </c>
       <c r="T13" t="n">
-        <v>22.4129</v>
+        <v>-7.2115</v>
       </c>
       <c r="U13" t="n">
-        <v>2.2139</v>
+        <v>-4.5725</v>
       </c>
       <c r="V13" t="n">
-        <v>2.5858</v>
+        <v>0.5069</v>
       </c>
       <c r="W13" t="n">
-        <v>10.6672</v>
+        <v>-1.2323</v>
       </c>
       <c r="X13" t="n">
-        <v>-0.9581</v>
+        <v>11.6082</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.8537</v>
+        <v>3.1285</v>
       </c>
       <c r="Z13" t="n">
-        <v>-21.9811</v>
+        <v>4.2938</v>
       </c>
       <c r="AA13" t="n">
-        <v>-2.191</v>
+        <v>4.6506</v>
       </c>
       <c r="AB13" t="n">
-        <v>-2.7238</v>
+        <v>-0.7619</v>
       </c>
       <c r="AC13" t="n">
-        <v>-10.1902</v>
+        <v>0.9631</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>167</v>
+        <v>172.95</v>
       </c>
       <c r="C14" t="n">
-        <v>174.4</v>
+        <v>174.61</v>
       </c>
       <c r="D14" t="n">
-        <v>161.14</v>
+        <v>142.69</v>
       </c>
       <c r="E14" t="n">
-        <v>164.18</v>
+        <v>151.75</v>
       </c>
       <c r="F14" t="n">
-        <v>75.73</v>
+        <v>76.13</v>
       </c>
       <c r="G14" t="n">
-        <v>77.37</v>
+        <v>76.27</v>
       </c>
       <c r="H14" t="n">
-        <v>74.23</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I14" t="n">
-        <v>75.34</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>9.130000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="K14" t="n">
-        <v>9.390000000000001</v>
+        <v>10.47</v>
       </c>
       <c r="L14" t="n">
-        <v>8.800000000000001</v>
+        <v>8.68</v>
       </c>
       <c r="M14" t="n">
-        <v>9.23</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="N14" t="n">
-        <v>42.77</v>
+        <v>42.51</v>
       </c>
       <c r="O14" t="n">
-        <v>43.57</v>
+        <v>44.82</v>
       </c>
       <c r="P14" t="n">
-        <v>41.93</v>
+        <v>42.44</v>
       </c>
       <c r="Q14" t="n">
-        <v>42.98</v>
+        <v>43.54</v>
       </c>
       <c r="R14" t="n">
-        <v>-11.8213</v>
+        <v>-7.571</v>
       </c>
       <c r="S14" t="n">
-        <v>-4.8342</v>
+        <v>-17.6346</v>
       </c>
       <c r="T14" t="n">
-        <v>-7.2115</v>
+        <v>-20.3077</v>
       </c>
       <c r="U14" t="n">
-        <v>-4.5725</v>
+        <v>-1.3539</v>
       </c>
       <c r="V14" t="n">
-        <v>0.5069</v>
+        <v>-3.7804</v>
       </c>
       <c r="W14" t="n">
-        <v>-1.2323</v>
+        <v>-3.4304</v>
       </c>
       <c r="X14" t="n">
-        <v>11.6082</v>
+        <v>7.8007</v>
       </c>
       <c r="Y14" t="n">
-        <v>3.1285</v>
+        <v>19.1617</v>
       </c>
       <c r="Z14" t="n">
-        <v>4.2938</v>
+        <v>21.3415</v>
       </c>
       <c r="AA14" t="n">
-        <v>4.6506</v>
+        <v>1.3029</v>
       </c>
       <c r="AB14" t="n">
-        <v>-0.7619</v>
+        <v>3.6914</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.9631</v>
+        <v>3.1265</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>172.95</v>
+        <v>141.24</v>
       </c>
       <c r="C15" t="n">
-        <v>174.61</v>
+        <v>160.6</v>
       </c>
       <c r="D15" t="n">
-        <v>142.69</v>
+        <v>135.02</v>
       </c>
       <c r="E15" t="n">
-        <v>151.75</v>
+        <v>151.89</v>
       </c>
       <c r="F15" t="n">
-        <v>76.13</v>
+        <v>72.41</v>
       </c>
       <c r="G15" t="n">
-        <v>76.27</v>
+        <v>74.5</v>
       </c>
       <c r="H15" t="n">
-        <v>72.09999999999999</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="I15" t="n">
-        <v>74.31999999999999</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J15" t="n">
-        <v>8.77</v>
+        <v>10.64</v>
       </c>
       <c r="K15" t="n">
-        <v>10.47</v>
+        <v>11.07</v>
       </c>
       <c r="L15" t="n">
-        <v>8.68</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="M15" t="n">
-        <v>9.949999999999999</v>
+        <v>9.93</v>
       </c>
       <c r="N15" t="n">
-        <v>42.51</v>
+        <v>44.68</v>
       </c>
       <c r="O15" t="n">
-        <v>44.82</v>
+        <v>45.53</v>
       </c>
       <c r="P15" t="n">
-        <v>42.44</v>
+        <v>43.46</v>
       </c>
       <c r="Q15" t="n">
-        <v>43.54</v>
+        <v>44.37</v>
       </c>
       <c r="R15" t="n">
-        <v>-7.571</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="S15" t="n">
-        <v>-17.6346</v>
+        <v>-18.422</v>
       </c>
       <c r="T15" t="n">
-        <v>-20.3077</v>
+        <v>-11.958</v>
       </c>
       <c r="U15" t="n">
-        <v>-1.3539</v>
+        <v>-1.8703</v>
       </c>
       <c r="V15" t="n">
-        <v>-3.7804</v>
+        <v>-7.6251</v>
       </c>
       <c r="W15" t="n">
-        <v>-3.4304</v>
+        <v>-2.7081</v>
       </c>
       <c r="X15" t="n">
-        <v>7.8007</v>
+        <v>-0.201</v>
       </c>
       <c r="Y15" t="n">
-        <v>19.1617</v>
+        <v>20.0726</v>
       </c>
       <c r="Z15" t="n">
-        <v>21.3415</v>
+        <v>10.9497</v>
       </c>
       <c r="AA15" t="n">
-        <v>1.3029</v>
+        <v>1.9063</v>
       </c>
       <c r="AB15" t="n">
-        <v>3.6914</v>
+        <v>8.0351</v>
       </c>
       <c r="AC15" t="n">
-        <v>3.1265</v>
+        <v>2.4475</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>141.24</v>
+        <v>161</v>
       </c>
       <c r="C16" t="n">
-        <v>160.6</v>
+        <v>173.7</v>
       </c>
       <c r="D16" t="n">
-        <v>135.02</v>
+        <v>161</v>
       </c>
       <c r="E16" t="n">
-        <v>151.89</v>
+        <v>173.2</v>
       </c>
       <c r="F16" t="n">
-        <v>72.41</v>
+        <v>74.09</v>
       </c>
       <c r="G16" t="n">
-        <v>74.5</v>
+        <v>76.53</v>
       </c>
       <c r="H16" t="n">
-        <v>70.95999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="I16" t="n">
-        <v>72.93000000000001</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J16" t="n">
-        <v>10.64</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>11.07</v>
+        <v>9.35</v>
       </c>
       <c r="L16" t="n">
-        <v>9.369999999999999</v>
+        <v>8.51</v>
       </c>
       <c r="M16" t="n">
-        <v>9.93</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N16" t="n">
-        <v>44.68</v>
+        <v>43.67</v>
       </c>
       <c r="O16" t="n">
-        <v>45.53</v>
+        <v>43.97</v>
       </c>
       <c r="P16" t="n">
-        <v>43.46</v>
+        <v>42.19</v>
       </c>
       <c r="Q16" t="n">
-        <v>44.37</v>
+        <v>42.19</v>
       </c>
       <c r="R16" t="n">
-        <v>0.09229999999999999</v>
+        <v>14.0299</v>
       </c>
       <c r="S16" t="n">
-        <v>-18.422</v>
+        <v>5.494</v>
       </c>
       <c r="T16" t="n">
-        <v>-11.958</v>
+        <v>-5.9922</v>
       </c>
       <c r="U16" t="n">
-        <v>-1.8703</v>
+        <v>4.9088</v>
       </c>
       <c r="V16" t="n">
-        <v>-7.6251</v>
+        <v>1.553</v>
       </c>
       <c r="W16" t="n">
-        <v>-2.7081</v>
+        <v>-0.9451000000000001</v>
       </c>
       <c r="X16" t="n">
-        <v>-0.201</v>
+        <v>-13.998</v>
       </c>
       <c r="Y16" t="n">
-        <v>20.0726</v>
+        <v>-7.4756</v>
       </c>
       <c r="Z16" t="n">
-        <v>10.9497</v>
+        <v>2.2754</v>
       </c>
       <c r="AA16" t="n">
-        <v>1.9063</v>
+        <v>-4.9132</v>
       </c>
       <c r="AB16" t="n">
-        <v>8.0351</v>
+        <v>-1.8381</v>
       </c>
       <c r="AC16" t="n">
-        <v>2.4475</v>
+        <v>0.4763</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>161</v>
+        <v>171.26</v>
       </c>
       <c r="C17" t="n">
-        <v>173.7</v>
+        <v>179.97</v>
       </c>
       <c r="D17" t="n">
-        <v>161</v>
+        <v>168.23</v>
       </c>
       <c r="E17" t="n">
-        <v>173.2</v>
+        <v>178.39</v>
       </c>
       <c r="F17" t="n">
-        <v>74.09</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>76.53</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H17" t="n">
-        <v>73.62</v>
+        <v>74.47</v>
       </c>
       <c r="I17" t="n">
-        <v>76.51000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J17" t="n">
-        <v>9.300000000000001</v>
+        <v>8.65</v>
       </c>
       <c r="K17" t="n">
-        <v>9.35</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L17" t="n">
-        <v>8.51</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M17" t="n">
-        <v>8.539999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N17" t="n">
-        <v>43.67</v>
+        <v>42.94</v>
       </c>
       <c r="O17" t="n">
-        <v>43.97</v>
+        <v>43.33</v>
       </c>
       <c r="P17" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="Q17" t="n">
-        <v>42.19</v>
+        <v>41.96</v>
       </c>
       <c r="R17" t="n">
-        <v>14.0299</v>
+        <v>2.9965</v>
       </c>
       <c r="S17" t="n">
-        <v>5.494</v>
+        <v>17.5552</v>
       </c>
       <c r="T17" t="n">
-        <v>-5.9922</v>
+        <v>-4.1893</v>
       </c>
       <c r="U17" t="n">
-        <v>4.9088</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="V17" t="n">
-        <v>1.553</v>
+        <v>3.5388</v>
       </c>
       <c r="W17" t="n">
-        <v>-0.9451000000000001</v>
+        <v>-2.5332</v>
       </c>
       <c r="X17" t="n">
-        <v>-13.998</v>
+        <v>-2.9274</v>
       </c>
       <c r="Y17" t="n">
-        <v>-7.4756</v>
+        <v>-16.6834</v>
       </c>
       <c r="Z17" t="n">
-        <v>2.2754</v>
+        <v>0.2418</v>
       </c>
       <c r="AA17" t="n">
-        <v>-4.9132</v>
+        <v>-0.5452</v>
       </c>
       <c r="AB17" t="n">
-        <v>-1.8381</v>
+        <v>-3.6288</v>
       </c>
       <c r="AC17" t="n">
-        <v>0.4763</v>
+        <v>2.167</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>171.26</v>
+        <v>184.8</v>
       </c>
       <c r="C18" t="n">
-        <v>179.97</v>
+        <v>195.27</v>
       </c>
       <c r="D18" t="n">
-        <v>168.23</v>
+        <v>183.34</v>
       </c>
       <c r="E18" t="n">
-        <v>178.39</v>
+        <v>190.56</v>
       </c>
       <c r="F18" t="n">
-        <v>75.18000000000001</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>77.79000000000001</v>
+        <v>79.33</v>
       </c>
       <c r="H18" t="n">
-        <v>74.47</v>
+        <v>77.33</v>
       </c>
       <c r="I18" t="n">
-        <v>76.95</v>
+        <v>77.84</v>
       </c>
       <c r="J18" t="n">
-        <v>8.65</v>
+        <v>8</v>
       </c>
       <c r="K18" t="n">
-        <v>8.779999999999999</v>
+        <v>8.06</v>
       </c>
       <c r="L18" t="n">
-        <v>8.210000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="M18" t="n">
-        <v>8.289999999999999</v>
+        <v>7.73</v>
       </c>
       <c r="N18" t="n">
-        <v>42.94</v>
+        <v>41.4</v>
       </c>
       <c r="O18" t="n">
-        <v>43.33</v>
+        <v>41.78</v>
       </c>
       <c r="P18" t="n">
+        <v>40.68</v>
+      </c>
+      <c r="Q18" t="n">
         <v>41.5</v>
       </c>
-      <c r="Q18" t="n">
-        <v>41.96</v>
-      </c>
       <c r="R18" t="n">
-        <v>2.9965</v>
+        <v>6.8221</v>
       </c>
       <c r="S18" t="n">
-        <v>17.5552</v>
+        <v>25.4592</v>
       </c>
       <c r="T18" t="n">
-        <v>-4.1893</v>
+        <v>16.0677</v>
       </c>
       <c r="U18" t="n">
-        <v>0.5750999999999999</v>
+        <v>1.1566</v>
       </c>
       <c r="V18" t="n">
-        <v>3.5388</v>
+        <v>6.7325</v>
       </c>
       <c r="W18" t="n">
-        <v>-2.5332</v>
+        <v>3.3183</v>
       </c>
       <c r="X18" t="n">
-        <v>-2.9274</v>
+        <v>-6.7551</v>
       </c>
       <c r="Y18" t="n">
-        <v>-16.6834</v>
+        <v>-22.1551</v>
       </c>
       <c r="Z18" t="n">
-        <v>0.2418</v>
+        <v>-16.2514</v>
       </c>
       <c r="AA18" t="n">
-        <v>-0.5452</v>
+        <v>-1.0963</v>
       </c>
       <c r="AB18" t="n">
-        <v>-3.6288</v>
+        <v>-6.4683</v>
       </c>
       <c r="AC18" t="n">
-        <v>2.167</v>
+        <v>-3.4435</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>184.8</v>
+        <v>211.38</v>
       </c>
       <c r="C19" t="n">
-        <v>195.27</v>
+        <v>228.5</v>
       </c>
       <c r="D19" t="n">
-        <v>183.34</v>
+        <v>209.89</v>
       </c>
       <c r="E19" t="n">
-        <v>190.56</v>
+        <v>225.79</v>
       </c>
       <c r="F19" t="n">
-        <v>78.04000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="G19" t="n">
-        <v>79.33</v>
+        <v>82.27</v>
       </c>
       <c r="H19" t="n">
-        <v>77.33</v>
+        <v>79.98</v>
       </c>
       <c r="I19" t="n">
-        <v>77.84</v>
+        <v>81.95</v>
       </c>
       <c r="J19" t="n">
-        <v>8</v>
+        <v>6.9</v>
       </c>
       <c r="K19" t="n">
-        <v>8.06</v>
+        <v>6.95</v>
       </c>
       <c r="L19" t="n">
-        <v>7.5</v>
+        <v>6.19</v>
       </c>
       <c r="M19" t="n">
-        <v>7.73</v>
+        <v>6.29</v>
       </c>
       <c r="N19" t="n">
-        <v>41.4</v>
+        <v>40.05</v>
       </c>
       <c r="O19" t="n">
-        <v>41.78</v>
+        <v>40.35</v>
       </c>
       <c r="P19" t="n">
-        <v>40.68</v>
+        <v>39.14</v>
       </c>
       <c r="Q19" t="n">
-        <v>41.5</v>
+        <v>39.28</v>
       </c>
       <c r="R19" t="n">
-        <v>6.8221</v>
+        <v>18.4876</v>
       </c>
       <c r="S19" t="n">
-        <v>25.4592</v>
+        <v>30.3637</v>
       </c>
       <c r="T19" t="n">
-        <v>16.0677</v>
+        <v>48.7908</v>
       </c>
       <c r="U19" t="n">
-        <v>1.1566</v>
+        <v>5.2801</v>
       </c>
       <c r="V19" t="n">
-        <v>6.7325</v>
+        <v>7.1102</v>
       </c>
       <c r="W19" t="n">
-        <v>3.3183</v>
+        <v>10.2664</v>
       </c>
       <c r="X19" t="n">
-        <v>-6.7551</v>
+        <v>-18.6287</v>
       </c>
       <c r="Y19" t="n">
-        <v>-22.1551</v>
+        <v>-26.3466</v>
       </c>
       <c r="Z19" t="n">
-        <v>-16.2514</v>
+        <v>-36.7839</v>
       </c>
       <c r="AA19" t="n">
-        <v>-1.0963</v>
+        <v>-5.3494</v>
       </c>
       <c r="AB19" t="n">
-        <v>-6.4683</v>
+        <v>-6.8974</v>
       </c>
       <c r="AC19" t="n">
-        <v>-3.4435</v>
+        <v>-9.7841</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>211.38</v>
+        <v>242.66</v>
       </c>
       <c r="C20" t="n">
-        <v>228.5</v>
+        <v>242.66</v>
       </c>
       <c r="D20" t="n">
-        <v>209.89</v>
+        <v>204</v>
       </c>
       <c r="E20" t="n">
-        <v>225.79</v>
+        <v>217.98</v>
       </c>
       <c r="F20" t="n">
-        <v>80.59</v>
+        <v>82.87</v>
       </c>
       <c r="G20" t="n">
-        <v>82.27</v>
+        <v>82.91</v>
       </c>
       <c r="H20" t="n">
-        <v>79.98</v>
+        <v>80.33</v>
       </c>
       <c r="I20" t="n">
-        <v>81.95</v>
+        <v>81.67</v>
       </c>
       <c r="J20" t="n">
-        <v>6.9</v>
+        <v>5.83</v>
       </c>
       <c r="K20" t="n">
-        <v>6.95</v>
+        <v>6.91</v>
       </c>
       <c r="L20" t="n">
-        <v>6.19</v>
+        <v>5.83</v>
       </c>
       <c r="M20" t="n">
-        <v>6.29</v>
+        <v>6.53</v>
       </c>
       <c r="N20" t="n">
-        <v>40.05</v>
+        <v>38.87</v>
       </c>
       <c r="O20" t="n">
-        <v>40.35</v>
+        <v>40.09</v>
       </c>
       <c r="P20" t="n">
-        <v>39.14</v>
+        <v>38.86</v>
       </c>
       <c r="Q20" t="n">
-        <v>39.28</v>
+        <v>39.44</v>
       </c>
       <c r="R20" t="n">
-        <v>18.4876</v>
+        <v>-3.459</v>
       </c>
       <c r="S20" t="n">
-        <v>30.3637</v>
+        <v>22.1929</v>
       </c>
       <c r="T20" t="n">
-        <v>48.7908</v>
+        <v>43.5118</v>
       </c>
       <c r="U20" t="n">
-        <v>5.2801</v>
+        <v>-0.3417</v>
       </c>
       <c r="V20" t="n">
-        <v>7.1102</v>
+        <v>6.1339</v>
       </c>
       <c r="W20" t="n">
-        <v>10.2664</v>
+        <v>11.9841</v>
       </c>
       <c r="X20" t="n">
-        <v>-18.6287</v>
+        <v>3.8156</v>
       </c>
       <c r="Y20" t="n">
-        <v>-26.3466</v>
+        <v>-21.2304</v>
       </c>
       <c r="Z20" t="n">
-        <v>-36.7839</v>
+        <v>-34.2397</v>
       </c>
       <c r="AA20" t="n">
-        <v>-5.3494</v>
+        <v>0.4073</v>
       </c>
       <c r="AB20" t="n">
-        <v>-6.8974</v>
+        <v>-6.0057</v>
       </c>
       <c r="AC20" t="n">
-        <v>-9.7841</v>
+        <v>-11.1111</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>242.66</v>
+        <v>219</v>
       </c>
       <c r="C21" t="n">
-        <v>242.66</v>
+        <v>231.89</v>
       </c>
       <c r="D21" t="n">
-        <v>204</v>
+        <v>207.56</v>
       </c>
       <c r="E21" t="n">
-        <v>217.98</v>
+        <v>224.63</v>
       </c>
       <c r="F21" t="n">
-        <v>82.87</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="G21" t="n">
-        <v>82.91</v>
+        <v>84.05</v>
       </c>
       <c r="H21" t="n">
-        <v>80.33</v>
+        <v>80.66</v>
       </c>
       <c r="I21" t="n">
-        <v>81.67</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>5.83</v>
+        <v>6.49</v>
       </c>
       <c r="K21" t="n">
-        <v>6.91</v>
+        <v>6.83</v>
       </c>
       <c r="L21" t="n">
-        <v>5.83</v>
+        <v>6.1</v>
       </c>
       <c r="M21" t="n">
-        <v>6.53</v>
+        <v>6.31</v>
       </c>
       <c r="N21" t="n">
-        <v>38.87</v>
+        <v>39.41</v>
       </c>
       <c r="O21" t="n">
-        <v>40.09</v>
+        <v>39.94</v>
       </c>
       <c r="P21" t="n">
-        <v>38.86</v>
+        <v>38.3</v>
       </c>
       <c r="Q21" t="n">
-        <v>39.44</v>
+        <v>38.47</v>
       </c>
       <c r="R21" t="n">
-        <v>-3.459</v>
+        <v>3.0507</v>
       </c>
       <c r="S21" t="n">
-        <v>22.1929</v>
+        <v>17.8789</v>
       </c>
       <c r="T21" t="n">
-        <v>43.5118</v>
+        <v>29.694</v>
       </c>
       <c r="U21" t="n">
-        <v>-0.3417</v>
+        <v>2.4611</v>
       </c>
       <c r="V21" t="n">
-        <v>6.1339</v>
+        <v>7.5026</v>
       </c>
       <c r="W21" t="n">
-        <v>11.9841</v>
+        <v>9.3713</v>
       </c>
       <c r="X21" t="n">
-        <v>3.8156</v>
+        <v>-3.3691</v>
       </c>
       <c r="Y21" t="n">
-        <v>-21.2304</v>
+        <v>-18.37</v>
       </c>
       <c r="Z21" t="n">
-        <v>-34.2397</v>
+        <v>-26.1124</v>
       </c>
       <c r="AA21" t="n">
-        <v>0.4073</v>
+        <v>-2.4594</v>
       </c>
       <c r="AB21" t="n">
-        <v>-6.0057</v>
+        <v>-7.3012</v>
       </c>
       <c r="AC21" t="n">
-        <v>-11.1111</v>
+        <v>-8.817299999999999</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>219</v>
+        <v>231.82</v>
       </c>
       <c r="C22" t="n">
-        <v>231.89</v>
+        <v>239.05</v>
       </c>
       <c r="D22" t="n">
-        <v>207.61</v>
+        <v>218.56</v>
       </c>
       <c r="E22" t="n">
-        <v>224.63</v>
+        <v>224.34</v>
       </c>
       <c r="F22" t="n">
-        <v>81.73</v>
+        <v>84.42</v>
       </c>
       <c r="G22" t="n">
-        <v>84.05</v>
+        <v>85.7</v>
       </c>
       <c r="H22" t="n">
-        <v>80.66</v>
+        <v>83.53</v>
       </c>
       <c r="I22" t="n">
-        <v>83.68000000000001</v>
+        <v>84.56</v>
       </c>
       <c r="J22" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="K22" t="n">
         <v>6.49</v>
       </c>
-      <c r="K22" t="n">
-        <v>6.83</v>
-      </c>
       <c r="L22" t="n">
-        <v>6.1</v>
+        <v>5.9107</v>
       </c>
       <c r="M22" t="n">
-        <v>6.31</v>
+        <v>6.33</v>
       </c>
       <c r="N22" t="n">
-        <v>39.41</v>
+        <v>38.16</v>
       </c>
       <c r="O22" t="n">
-        <v>39.94</v>
+        <v>38.5599</v>
       </c>
       <c r="P22" t="n">
-        <v>38.3</v>
+        <v>37.57</v>
       </c>
       <c r="Q22" t="n">
-        <v>38.47</v>
+        <v>38.08</v>
       </c>
       <c r="R22" t="n">
-        <v>3.0507</v>
+        <v>-0.1291</v>
       </c>
       <c r="S22" t="n">
-        <v>17.8789</v>
+        <v>-0.6422</v>
       </c>
       <c r="T22" t="n">
-        <v>29.694</v>
+        <v>25.7582</v>
       </c>
       <c r="U22" t="n">
-        <v>2.4611</v>
+        <v>1.0516</v>
       </c>
       <c r="V22" t="n">
-        <v>7.5026</v>
+        <v>3.1849</v>
       </c>
       <c r="W22" t="n">
-        <v>9.3713</v>
+        <v>9.8895</v>
       </c>
       <c r="X22" t="n">
-        <v>-3.3691</v>
+        <v>0.317</v>
       </c>
       <c r="Y22" t="n">
-        <v>-18.37</v>
+        <v>0.6359</v>
       </c>
       <c r="Z22" t="n">
-        <v>-26.1124</v>
+        <v>-23.6429</v>
       </c>
       <c r="AA22" t="n">
-        <v>-2.4594</v>
+        <v>-1.0138</v>
       </c>
       <c r="AB22" t="n">
-        <v>-7.3012</v>
+        <v>-3.055</v>
       </c>
       <c r="AC22" t="n">
-        <v>-8.817299999999999</v>
+        <v>-9.2469</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-01 23:27
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC22"/>
+  <dimension ref="A1:AC21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1804 +568,1713 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>122.81</v>
+        <v>132.2</v>
       </c>
       <c r="C2" t="n">
-        <v>127.45</v>
+        <v>133.67</v>
       </c>
       <c r="D2" t="n">
-        <v>117.5</v>
+        <v>123.8</v>
       </c>
       <c r="E2" t="n">
-        <v>126.98</v>
+        <v>127.55</v>
       </c>
       <c r="F2" t="n">
-        <v>62.89</v>
+        <v>65.44</v>
       </c>
       <c r="G2" t="n">
-        <v>63.8</v>
+        <v>66.05</v>
       </c>
       <c r="H2" t="n">
-        <v>60.7</v>
+        <v>63.78</v>
       </c>
       <c r="I2" t="n">
-        <v>63.54</v>
+        <v>64.91</v>
       </c>
       <c r="J2" t="n">
-        <v>13.84</v>
+        <v>12.8</v>
       </c>
       <c r="K2" t="n">
-        <v>14.49</v>
+        <v>13.64</v>
       </c>
       <c r="L2" t="n">
-        <v>13.25</v>
+        <v>12.65</v>
       </c>
       <c r="M2" t="n">
-        <v>13.3</v>
+        <v>13.26</v>
       </c>
       <c r="N2" t="n">
-        <v>52.21</v>
+        <v>50.12</v>
       </c>
       <c r="O2" t="n">
-        <v>54.09</v>
+        <v>51.43</v>
       </c>
       <c r="P2" t="n">
-        <v>51.4</v>
+        <v>49.65</v>
       </c>
       <c r="Q2" t="n">
-        <v>51.65</v>
+        <v>50.51</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>124.39</v>
+        <v>135</v>
       </c>
       <c r="C3" t="n">
-        <v>131.38</v>
+        <v>147.26</v>
       </c>
       <c r="D3" t="n">
-        <v>121.66</v>
+        <v>134.02</v>
       </c>
       <c r="E3" t="n">
-        <v>130.4</v>
+        <v>144.16</v>
       </c>
       <c r="F3" t="n">
-        <v>63.89</v>
+        <v>66.37</v>
       </c>
       <c r="G3" t="n">
-        <v>65.84</v>
+        <v>67.77</v>
       </c>
       <c r="H3" t="n">
-        <v>63.81</v>
+        <v>66.25</v>
       </c>
       <c r="I3" t="n">
-        <v>65.3</v>
+        <v>67.39</v>
       </c>
       <c r="J3" t="n">
-        <v>13.61</v>
+        <v>12.5</v>
       </c>
       <c r="K3" t="n">
-        <v>13.89</v>
+        <v>12.59</v>
       </c>
       <c r="L3" t="n">
-        <v>12.87</v>
+        <v>11.21</v>
       </c>
       <c r="M3" t="n">
-        <v>12.98</v>
+        <v>11.51</v>
       </c>
       <c r="N3" t="n">
-        <v>51.36</v>
+        <v>49.4</v>
       </c>
       <c r="O3" t="n">
-        <v>51.45</v>
+        <v>49.49</v>
       </c>
       <c r="P3" t="n">
-        <v>49.79</v>
+        <v>48.3</v>
       </c>
       <c r="Q3" t="n">
-        <v>50.22</v>
+        <v>48.59</v>
       </c>
       <c r="R3" t="n">
-        <v>2.6933</v>
+        <v>13.0223</v>
       </c>
       <c r="U3" t="n">
-        <v>2.7699</v>
+        <v>3.8207</v>
       </c>
       <c r="X3" t="n">
-        <v>-2.406</v>
+        <v>-13.1976</v>
       </c>
       <c r="AA3" t="n">
-        <v>-2.7686</v>
+        <v>-3.8012</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>132.2</v>
+        <v>157.84</v>
       </c>
       <c r="C4" t="n">
-        <v>133.67</v>
+        <v>166</v>
       </c>
       <c r="D4" t="n">
-        <v>123.8</v>
+        <v>149.06</v>
       </c>
       <c r="E4" t="n">
-        <v>127.55</v>
+        <v>165.85</v>
       </c>
       <c r="F4" t="n">
-        <v>65.44</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>66.05</v>
+        <v>71.66</v>
       </c>
       <c r="H4" t="n">
-        <v>63.78</v>
+        <v>68.88</v>
       </c>
       <c r="I4" t="n">
-        <v>64.91</v>
+        <v>71.56999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>12.8</v>
+        <v>10.43</v>
       </c>
       <c r="K4" t="n">
-        <v>13.64</v>
+        <v>11.14</v>
       </c>
       <c r="L4" t="n">
-        <v>12.65</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>13.26</v>
+        <v>9.81</v>
       </c>
       <c r="N4" t="n">
-        <v>50.12</v>
+        <v>47.26</v>
       </c>
       <c r="O4" t="n">
-        <v>51.43</v>
+        <v>47.54</v>
       </c>
       <c r="P4" t="n">
-        <v>49.65</v>
+        <v>45.52</v>
       </c>
       <c r="Q4" t="n">
-        <v>50.51</v>
+        <v>45.59</v>
       </c>
       <c r="R4" t="n">
-        <v>-2.1856</v>
+        <v>15.0458</v>
       </c>
       <c r="U4" t="n">
-        <v>-0.5972</v>
+        <v>6.2027</v>
       </c>
       <c r="X4" t="n">
-        <v>2.1572</v>
+        <v>-14.7698</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.5775</v>
+        <v>-6.1741</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>135</v>
+        <v>162.12</v>
       </c>
       <c r="C5" t="n">
-        <v>147.26</v>
+        <v>162.9</v>
       </c>
       <c r="D5" t="n">
-        <v>134.02</v>
+        <v>147.61</v>
       </c>
       <c r="E5" t="n">
-        <v>144.16</v>
+        <v>152.1</v>
       </c>
       <c r="F5" t="n">
-        <v>66.37</v>
+        <v>71.87</v>
       </c>
       <c r="G5" t="n">
-        <v>67.77</v>
+        <v>73.3</v>
       </c>
       <c r="H5" t="n">
-        <v>66.25</v>
+        <v>70.38</v>
       </c>
       <c r="I5" t="n">
-        <v>67.39</v>
+        <v>71.34</v>
       </c>
       <c r="J5" t="n">
-        <v>12.5</v>
+        <v>10.02</v>
       </c>
       <c r="K5" t="n">
-        <v>12.59</v>
+        <v>10.88</v>
       </c>
       <c r="L5" t="n">
-        <v>11.21</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>11.51</v>
+        <v>10.6</v>
       </c>
       <c r="N5" t="n">
-        <v>49.4</v>
+        <v>45.41</v>
       </c>
       <c r="O5" t="n">
-        <v>49.49</v>
+        <v>46.36</v>
       </c>
       <c r="P5" t="n">
-        <v>48.3</v>
+        <v>44.5</v>
       </c>
       <c r="Q5" t="n">
-        <v>48.59</v>
+        <v>45.73</v>
       </c>
       <c r="R5" t="n">
-        <v>13.0223</v>
+        <v>-8.2906</v>
       </c>
       <c r="S5" t="n">
-        <v>13.5297</v>
+        <v>19.2474</v>
       </c>
       <c r="U5" t="n">
-        <v>3.8207</v>
+        <v>-0.3214</v>
       </c>
       <c r="V5" t="n">
-        <v>6.0592</v>
+        <v>9.906000000000001</v>
       </c>
       <c r="X5" t="n">
-        <v>-13.1976</v>
+        <v>8.053000000000001</v>
       </c>
       <c r="Y5" t="n">
-        <v>-13.4586</v>
+        <v>-20.0603</v>
       </c>
       <c r="AA5" t="n">
-        <v>-3.8012</v>
+        <v>0.3071</v>
       </c>
       <c r="AB5" t="n">
-        <v>-5.9245</v>
+        <v>-9.4635</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>157.84</v>
+        <v>163</v>
       </c>
       <c r="C6" t="n">
-        <v>166</v>
+        <v>177.5</v>
       </c>
       <c r="D6" t="n">
-        <v>149.06</v>
+        <v>161.51</v>
       </c>
       <c r="E6" t="n">
-        <v>165.85</v>
+        <v>176.94</v>
       </c>
       <c r="F6" t="n">
-        <v>69.26000000000001</v>
+        <v>72.81999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>71.66</v>
+        <v>76.31</v>
       </c>
       <c r="H6" t="n">
-        <v>68.88</v>
+        <v>72.7</v>
       </c>
       <c r="I6" t="n">
-        <v>71.56999999999999</v>
+        <v>76.28</v>
       </c>
       <c r="J6" t="n">
-        <v>10.43</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="K6" t="n">
-        <v>11.14</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="L6" t="n">
-        <v>9.800000000000001</v>
+        <v>8.84</v>
       </c>
       <c r="M6" t="n">
-        <v>9.81</v>
+        <v>8.85</v>
       </c>
       <c r="N6" t="n">
-        <v>47.26</v>
+        <v>44.82</v>
       </c>
       <c r="O6" t="n">
-        <v>47.54</v>
+        <v>44.89</v>
       </c>
       <c r="P6" t="n">
-        <v>45.52</v>
+        <v>42.57</v>
       </c>
       <c r="Q6" t="n">
-        <v>45.59</v>
+        <v>42.57</v>
       </c>
       <c r="R6" t="n">
-        <v>15.0458</v>
+        <v>16.3314</v>
       </c>
       <c r="S6" t="n">
-        <v>27.1856</v>
+        <v>22.7386</v>
       </c>
       <c r="U6" t="n">
-        <v>6.2027</v>
+        <v>6.9246</v>
       </c>
       <c r="V6" t="n">
-        <v>9.601800000000001</v>
+        <v>13.1919</v>
       </c>
       <c r="X6" t="n">
-        <v>-14.7698</v>
+        <v>-16.5094</v>
       </c>
       <c r="Y6" t="n">
-        <v>-24.4222</v>
+        <v>-23.1103</v>
       </c>
       <c r="AA6" t="n">
-        <v>-6.1741</v>
+        <v>-6.9101</v>
       </c>
       <c r="AB6" t="n">
-        <v>-9.2194</v>
+        <v>-12.3894</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>162.12</v>
+        <v>181</v>
       </c>
       <c r="C7" t="n">
-        <v>162.9</v>
+        <v>191.29</v>
       </c>
       <c r="D7" t="n">
-        <v>147.61</v>
+        <v>178.94</v>
       </c>
       <c r="E7" t="n">
-        <v>152.1</v>
+        <v>190.42</v>
       </c>
       <c r="F7" t="n">
-        <v>71.87</v>
+        <v>76</v>
       </c>
       <c r="G7" t="n">
-        <v>73.3</v>
+        <v>77.36</v>
       </c>
       <c r="H7" t="n">
-        <v>70.38</v>
+        <v>75.55</v>
       </c>
       <c r="I7" t="n">
-        <v>71.34</v>
+        <v>76.95999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>10.02</v>
+        <v>8.65</v>
       </c>
       <c r="K7" t="n">
-        <v>10.88</v>
+        <v>8.77</v>
       </c>
       <c r="L7" t="n">
-        <v>9.970000000000001</v>
+        <v>8.15</v>
       </c>
       <c r="M7" t="n">
-        <v>10.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="N7" t="n">
-        <v>45.41</v>
+        <v>42.74</v>
       </c>
       <c r="O7" t="n">
-        <v>46.36</v>
+        <v>43</v>
       </c>
       <c r="P7" t="n">
-        <v>44.5</v>
+        <v>41.99</v>
       </c>
       <c r="Q7" t="n">
-        <v>45.73</v>
+        <v>42.22</v>
       </c>
       <c r="R7" t="n">
-        <v>-8.2906</v>
+        <v>7.6184</v>
       </c>
       <c r="S7" t="n">
-        <v>19.2474</v>
+        <v>14.8146</v>
       </c>
       <c r="T7" t="n">
-        <v>19.7826</v>
+        <v>49.2905</v>
       </c>
       <c r="U7" t="n">
-        <v>-0.3214</v>
+        <v>0.8915</v>
       </c>
       <c r="V7" t="n">
-        <v>9.906000000000001</v>
+        <v>7.5311</v>
       </c>
       <c r="W7" t="n">
-        <v>12.2757</v>
+        <v>18.5642</v>
       </c>
       <c r="X7" t="n">
-        <v>8.053000000000001</v>
+        <v>-7.3446</v>
       </c>
       <c r="Y7" t="n">
-        <v>-20.0603</v>
+        <v>-16.4118</v>
       </c>
       <c r="Z7" t="n">
-        <v>-20.3008</v>
+        <v>-38.1599</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.3071</v>
+        <v>-0.8222</v>
       </c>
       <c r="AB7" t="n">
-        <v>-9.4635</v>
+        <v>-7.392</v>
       </c>
       <c r="AC7" t="n">
-        <v>-11.4618</v>
+        <v>-16.4126</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>163</v>
+        <v>177.62</v>
       </c>
       <c r="C8" t="n">
-        <v>177.5</v>
+        <v>182.24</v>
       </c>
       <c r="D8" t="n">
-        <v>161.51</v>
+        <v>150.58</v>
       </c>
       <c r="E8" t="n">
-        <v>176.94</v>
+        <v>172.52</v>
       </c>
       <c r="F8" t="n">
-        <v>72.81999999999999</v>
+        <v>75.3</v>
       </c>
       <c r="G8" t="n">
-        <v>76.31</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="H8" t="n">
-        <v>72.7</v>
+        <v>71.55</v>
       </c>
       <c r="I8" t="n">
-        <v>76.28</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>9.859999999999999</v>
+        <v>8.75</v>
       </c>
       <c r="K8" t="n">
-        <v>9.970000000000001</v>
+        <v>9.91</v>
       </c>
       <c r="L8" t="n">
-        <v>8.84</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>8.85</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>44.82</v>
+        <v>43.14</v>
       </c>
       <c r="O8" t="n">
-        <v>44.89</v>
+        <v>45.19</v>
       </c>
       <c r="P8" t="n">
-        <v>42.57</v>
+        <v>42.79</v>
       </c>
       <c r="Q8" t="n">
-        <v>42.57</v>
+        <v>43.31</v>
       </c>
       <c r="R8" t="n">
-        <v>16.3314</v>
+        <v>-9.4003</v>
       </c>
       <c r="S8" t="n">
-        <v>22.7386</v>
+        <v>13.4254</v>
       </c>
       <c r="T8" t="n">
-        <v>35.6902</v>
+        <v>19.6726</v>
       </c>
       <c r="U8" t="n">
-        <v>6.9246</v>
+        <v>-2.5988</v>
       </c>
       <c r="V8" t="n">
-        <v>13.1919</v>
+        <v>5.0743</v>
       </c>
       <c r="W8" t="n">
-        <v>16.8147</v>
+        <v>11.2331</v>
       </c>
       <c r="X8" t="n">
-        <v>-16.5094</v>
+        <v>9.1463</v>
       </c>
       <c r="Y8" t="n">
-        <v>-23.1103</v>
+        <v>-15.566</v>
       </c>
       <c r="Z8" t="n">
-        <v>-31.8182</v>
+        <v>-22.2415</v>
       </c>
       <c r="AA8" t="n">
-        <v>-6.9101</v>
+        <v>2.5817</v>
       </c>
       <c r="AB8" t="n">
-        <v>-12.3894</v>
+        <v>-5.2919</v>
       </c>
       <c r="AC8" t="n">
-        <v>-15.233</v>
+        <v>-10.8664</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>181</v>
+        <v>183.84</v>
       </c>
       <c r="C9" t="n">
-        <v>191.29</v>
+        <v>188.49</v>
       </c>
       <c r="D9" t="n">
-        <v>178.94</v>
+        <v>172.26</v>
       </c>
       <c r="E9" t="n">
-        <v>190.42</v>
+        <v>184.24</v>
       </c>
       <c r="F9" t="n">
-        <v>76</v>
+        <v>75.81</v>
       </c>
       <c r="G9" t="n">
-        <v>77.36</v>
+        <v>77.94</v>
       </c>
       <c r="H9" t="n">
-        <v>75.55</v>
+        <v>74.19</v>
       </c>
       <c r="I9" t="n">
-        <v>76.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>8.65</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>8.77</v>
+        <v>8.98</v>
       </c>
       <c r="L9" t="n">
-        <v>8.15</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="M9" t="n">
-        <v>8.199999999999999</v>
+        <v>8.35</v>
       </c>
       <c r="N9" t="n">
-        <v>42.74</v>
+        <v>42.83</v>
       </c>
       <c r="O9" t="n">
-        <v>43</v>
+        <v>43.77</v>
       </c>
       <c r="P9" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="Q9" t="n">
         <v>41.99</v>
       </c>
-      <c r="Q9" t="n">
-        <v>42.22</v>
-      </c>
       <c r="R9" t="n">
-        <v>7.6184</v>
+        <v>6.7934</v>
       </c>
       <c r="S9" t="n">
-        <v>14.8146</v>
+        <v>4.1257</v>
       </c>
       <c r="T9" t="n">
-        <v>49.2905</v>
+        <v>11.0883</v>
       </c>
       <c r="U9" t="n">
-        <v>0.8915</v>
+        <v>3.0416</v>
       </c>
       <c r="V9" t="n">
-        <v>7.5311</v>
+        <v>1.2585</v>
       </c>
       <c r="W9" t="n">
-        <v>18.5642</v>
+        <v>7.9223</v>
       </c>
       <c r="X9" t="n">
-        <v>-7.3446</v>
+        <v>-6.7039</v>
       </c>
       <c r="Y9" t="n">
-        <v>-16.4118</v>
+        <v>-5.6497</v>
       </c>
       <c r="Z9" t="n">
-        <v>-38.1599</v>
+        <v>-14.8828</v>
       </c>
       <c r="AA9" t="n">
-        <v>-0.8222</v>
+        <v>-3.0478</v>
       </c>
       <c r="AB9" t="n">
-        <v>-7.392</v>
+        <v>-1.3625</v>
       </c>
       <c r="AC9" t="n">
-        <v>-16.4126</v>
+        <v>-7.8965</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>177.62</v>
+        <v>182.67</v>
       </c>
       <c r="C10" t="n">
-        <v>182.24</v>
+        <v>189.56</v>
       </c>
       <c r="D10" t="n">
-        <v>150.58</v>
+        <v>178.28</v>
       </c>
       <c r="E10" t="n">
-        <v>172.52</v>
+        <v>186.19</v>
       </c>
       <c r="F10" t="n">
-        <v>75.3</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>75.93000000000001</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>71.55</v>
+        <v>77.16</v>
       </c>
       <c r="I10" t="n">
-        <v>74.95999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="J10" t="n">
-        <v>8.75</v>
+        <v>8.43</v>
       </c>
       <c r="K10" t="n">
-        <v>9.91</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L10" t="n">
-        <v>8.550000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M10" t="n">
-        <v>8.949999999999999</v>
+        <v>8.27</v>
       </c>
       <c r="N10" t="n">
-        <v>43.14</v>
+        <v>41.98</v>
       </c>
       <c r="O10" t="n">
-        <v>45.19</v>
+        <v>42.06</v>
       </c>
       <c r="P10" t="n">
-        <v>42.79</v>
+        <v>40.68</v>
       </c>
       <c r="Q10" t="n">
-        <v>43.31</v>
+        <v>41.07</v>
       </c>
       <c r="R10" t="n">
-        <v>-9.4003</v>
+        <v>1.0584</v>
       </c>
       <c r="S10" t="n">
-        <v>13.4254</v>
+        <v>-2.2214</v>
       </c>
       <c r="T10" t="n">
-        <v>19.6726</v>
+        <v>22.4129</v>
       </c>
       <c r="U10" t="n">
-        <v>-2.5988</v>
+        <v>2.2139</v>
       </c>
       <c r="V10" t="n">
-        <v>5.0743</v>
+        <v>2.5858</v>
       </c>
       <c r="W10" t="n">
-        <v>11.2331</v>
+        <v>10.6672</v>
       </c>
       <c r="X10" t="n">
-        <v>9.1463</v>
+        <v>-0.9581</v>
       </c>
       <c r="Y10" t="n">
-        <v>-15.566</v>
+        <v>0.8537</v>
       </c>
       <c r="Z10" t="n">
-        <v>-22.2415</v>
+        <v>-21.9811</v>
       </c>
       <c r="AA10" t="n">
-        <v>2.5817</v>
+        <v>-2.191</v>
       </c>
       <c r="AB10" t="n">
-        <v>-5.2919</v>
+        <v>-2.7238</v>
       </c>
       <c r="AC10" t="n">
-        <v>-10.8664</v>
+        <v>-10.1902</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>183.84</v>
+        <v>167</v>
       </c>
       <c r="C11" t="n">
-        <v>188.49</v>
+        <v>174.4</v>
       </c>
       <c r="D11" t="n">
-        <v>172.26</v>
+        <v>161.14</v>
       </c>
       <c r="E11" t="n">
-        <v>184.24</v>
+        <v>164.18</v>
       </c>
       <c r="F11" t="n">
-        <v>75.81</v>
+        <v>75.73</v>
       </c>
       <c r="G11" t="n">
-        <v>77.94</v>
+        <v>77.37</v>
       </c>
       <c r="H11" t="n">
-        <v>74.19</v>
+        <v>74.23</v>
       </c>
       <c r="I11" t="n">
-        <v>77.23999999999999</v>
+        <v>75.34</v>
       </c>
       <c r="J11" t="n">
-        <v>8.380000000000001</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>8.98</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="L11" t="n">
-        <v>8.140000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M11" t="n">
-        <v>8.35</v>
+        <v>9.23</v>
       </c>
       <c r="N11" t="n">
-        <v>42.83</v>
+        <v>42.77</v>
       </c>
       <c r="O11" t="n">
-        <v>43.77</v>
+        <v>43.57</v>
       </c>
       <c r="P11" t="n">
-        <v>41.6</v>
+        <v>41.93</v>
       </c>
       <c r="Q11" t="n">
-        <v>41.99</v>
+        <v>42.98</v>
       </c>
       <c r="R11" t="n">
-        <v>6.7934</v>
+        <v>-11.8213</v>
       </c>
       <c r="S11" t="n">
-        <v>4.1257</v>
+        <v>-4.8342</v>
       </c>
       <c r="T11" t="n">
-        <v>11.0883</v>
+        <v>-7.2115</v>
       </c>
       <c r="U11" t="n">
-        <v>3.0416</v>
+        <v>-4.5725</v>
       </c>
       <c r="V11" t="n">
-        <v>1.2585</v>
+        <v>0.5069</v>
       </c>
       <c r="W11" t="n">
-        <v>7.9223</v>
+        <v>-1.2323</v>
       </c>
       <c r="X11" t="n">
-        <v>-6.7039</v>
+        <v>11.6082</v>
       </c>
       <c r="Y11" t="n">
-        <v>-5.6497</v>
+        <v>3.1285</v>
       </c>
       <c r="Z11" t="n">
-        <v>-14.8828</v>
+        <v>4.2938</v>
       </c>
       <c r="AA11" t="n">
-        <v>-3.0478</v>
+        <v>4.6506</v>
       </c>
       <c r="AB11" t="n">
-        <v>-1.3625</v>
+        <v>-0.7619</v>
       </c>
       <c r="AC11" t="n">
-        <v>-7.8965</v>
+        <v>0.9631</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>182.67</v>
+        <v>172.95</v>
       </c>
       <c r="C12" t="n">
-        <v>189.56</v>
+        <v>174.61</v>
       </c>
       <c r="D12" t="n">
-        <v>178.28</v>
+        <v>142.69</v>
       </c>
       <c r="E12" t="n">
-        <v>186.19</v>
+        <v>151.75</v>
       </c>
       <c r="F12" t="n">
-        <v>77.29000000000001</v>
+        <v>76.13</v>
       </c>
       <c r="G12" t="n">
-        <v>79.68000000000001</v>
+        <v>76.27</v>
       </c>
       <c r="H12" t="n">
-        <v>77.16</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>78.95</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>8.43</v>
+        <v>8.77</v>
       </c>
       <c r="K12" t="n">
-        <v>8.630000000000001</v>
+        <v>10.47</v>
       </c>
       <c r="L12" t="n">
-        <v>8.119999999999999</v>
+        <v>8.68</v>
       </c>
       <c r="M12" t="n">
-        <v>8.27</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="N12" t="n">
-        <v>41.98</v>
+        <v>42.51</v>
       </c>
       <c r="O12" t="n">
-        <v>42.06</v>
+        <v>44.82</v>
       </c>
       <c r="P12" t="n">
-        <v>40.68</v>
+        <v>42.44</v>
       </c>
       <c r="Q12" t="n">
-        <v>41.07</v>
+        <v>43.54</v>
       </c>
       <c r="R12" t="n">
-        <v>1.0584</v>
+        <v>-7.571</v>
       </c>
       <c r="S12" t="n">
-        <v>-2.2214</v>
+        <v>-17.6346</v>
       </c>
       <c r="T12" t="n">
-        <v>22.4129</v>
+        <v>-20.3077</v>
       </c>
       <c r="U12" t="n">
-        <v>2.2139</v>
+        <v>-1.3539</v>
       </c>
       <c r="V12" t="n">
-        <v>2.5858</v>
+        <v>-3.7804</v>
       </c>
       <c r="W12" t="n">
-        <v>10.6672</v>
+        <v>-3.4304</v>
       </c>
       <c r="X12" t="n">
-        <v>-0.9581</v>
+        <v>7.8007</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.8537</v>
+        <v>19.1617</v>
       </c>
       <c r="Z12" t="n">
-        <v>-21.9811</v>
+        <v>21.3415</v>
       </c>
       <c r="AA12" t="n">
-        <v>-2.191</v>
+        <v>1.3029</v>
       </c>
       <c r="AB12" t="n">
-        <v>-2.7238</v>
+        <v>3.6914</v>
       </c>
       <c r="AC12" t="n">
-        <v>-10.1902</v>
+        <v>3.1265</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>167</v>
+        <v>141.24</v>
       </c>
       <c r="C13" t="n">
-        <v>174.4</v>
+        <v>160.6</v>
       </c>
       <c r="D13" t="n">
-        <v>161.14</v>
+        <v>135.02</v>
       </c>
       <c r="E13" t="n">
-        <v>164.18</v>
+        <v>151.89</v>
       </c>
       <c r="F13" t="n">
-        <v>75.73</v>
+        <v>72.41</v>
       </c>
       <c r="G13" t="n">
-        <v>77.37</v>
+        <v>74.5</v>
       </c>
       <c r="H13" t="n">
-        <v>74.23</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>75.34</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>9.130000000000001</v>
+        <v>10.64</v>
       </c>
       <c r="K13" t="n">
-        <v>9.390000000000001</v>
+        <v>11.07</v>
       </c>
       <c r="L13" t="n">
-        <v>8.800000000000001</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="M13" t="n">
-        <v>9.23</v>
+        <v>9.93</v>
       </c>
       <c r="N13" t="n">
-        <v>42.77</v>
+        <v>44.68</v>
       </c>
       <c r="O13" t="n">
-        <v>43.57</v>
+        <v>45.53</v>
       </c>
       <c r="P13" t="n">
-        <v>41.93</v>
+        <v>43.46</v>
       </c>
       <c r="Q13" t="n">
-        <v>42.98</v>
+        <v>44.37</v>
       </c>
       <c r="R13" t="n">
-        <v>-11.8213</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="S13" t="n">
-        <v>-4.8342</v>
+        <v>-18.422</v>
       </c>
       <c r="T13" t="n">
-        <v>-7.2115</v>
+        <v>-11.958</v>
       </c>
       <c r="U13" t="n">
-        <v>-4.5725</v>
+        <v>-1.8703</v>
       </c>
       <c r="V13" t="n">
-        <v>0.5069</v>
+        <v>-7.6251</v>
       </c>
       <c r="W13" t="n">
-        <v>-1.2323</v>
+        <v>-2.7081</v>
       </c>
       <c r="X13" t="n">
-        <v>11.6082</v>
+        <v>-0.201</v>
       </c>
       <c r="Y13" t="n">
-        <v>3.1285</v>
+        <v>20.0726</v>
       </c>
       <c r="Z13" t="n">
-        <v>4.2938</v>
+        <v>10.9497</v>
       </c>
       <c r="AA13" t="n">
-        <v>4.6506</v>
+        <v>1.9063</v>
       </c>
       <c r="AB13" t="n">
-        <v>-0.7619</v>
+        <v>8.0351</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.9631</v>
+        <v>2.4475</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>172.95</v>
+        <v>161</v>
       </c>
       <c r="C14" t="n">
-        <v>174.61</v>
+        <v>173.7</v>
       </c>
       <c r="D14" t="n">
-        <v>142.69</v>
+        <v>161</v>
       </c>
       <c r="E14" t="n">
-        <v>151.75</v>
+        <v>173.2</v>
       </c>
       <c r="F14" t="n">
-        <v>76.13</v>
+        <v>74.09</v>
       </c>
       <c r="G14" t="n">
-        <v>76.27</v>
+        <v>76.53</v>
       </c>
       <c r="H14" t="n">
-        <v>72.09999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="I14" t="n">
-        <v>74.31999999999999</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J14" t="n">
-        <v>8.77</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>10.47</v>
+        <v>9.35</v>
       </c>
       <c r="L14" t="n">
-        <v>8.68</v>
+        <v>8.51</v>
       </c>
       <c r="M14" t="n">
-        <v>9.949999999999999</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N14" t="n">
-        <v>42.51</v>
+        <v>43.67</v>
       </c>
       <c r="O14" t="n">
-        <v>44.82</v>
+        <v>43.97</v>
       </c>
       <c r="P14" t="n">
-        <v>42.44</v>
+        <v>42.19</v>
       </c>
       <c r="Q14" t="n">
-        <v>43.54</v>
+        <v>42.19</v>
       </c>
       <c r="R14" t="n">
-        <v>-7.571</v>
+        <v>14.0299</v>
       </c>
       <c r="S14" t="n">
-        <v>-17.6346</v>
+        <v>5.494</v>
       </c>
       <c r="T14" t="n">
-        <v>-20.3077</v>
+        <v>-5.9922</v>
       </c>
       <c r="U14" t="n">
-        <v>-1.3539</v>
+        <v>4.9088</v>
       </c>
       <c r="V14" t="n">
-        <v>-3.7804</v>
+        <v>1.553</v>
       </c>
       <c r="W14" t="n">
-        <v>-3.4304</v>
+        <v>-0.9451000000000001</v>
       </c>
       <c r="X14" t="n">
-        <v>7.8007</v>
+        <v>-13.998</v>
       </c>
       <c r="Y14" t="n">
-        <v>19.1617</v>
+        <v>-7.4756</v>
       </c>
       <c r="Z14" t="n">
-        <v>21.3415</v>
+        <v>2.2754</v>
       </c>
       <c r="AA14" t="n">
-        <v>1.3029</v>
+        <v>-4.9132</v>
       </c>
       <c r="AB14" t="n">
-        <v>3.6914</v>
+        <v>-1.8381</v>
       </c>
       <c r="AC14" t="n">
-        <v>3.1265</v>
+        <v>0.4763</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>141.24</v>
+        <v>171.26</v>
       </c>
       <c r="C15" t="n">
-        <v>160.6</v>
+        <v>179.97</v>
       </c>
       <c r="D15" t="n">
-        <v>135.02</v>
+        <v>168.23</v>
       </c>
       <c r="E15" t="n">
-        <v>151.89</v>
+        <v>178.39</v>
       </c>
       <c r="F15" t="n">
-        <v>72.41</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>74.5</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H15" t="n">
-        <v>70.95999999999999</v>
+        <v>74.47</v>
       </c>
       <c r="I15" t="n">
-        <v>72.93000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J15" t="n">
-        <v>10.64</v>
+        <v>8.65</v>
       </c>
       <c r="K15" t="n">
-        <v>11.07</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L15" t="n">
-        <v>9.369999999999999</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M15" t="n">
-        <v>9.93</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N15" t="n">
-        <v>44.68</v>
+        <v>42.94</v>
       </c>
       <c r="O15" t="n">
-        <v>45.53</v>
+        <v>43.33</v>
       </c>
       <c r="P15" t="n">
-        <v>43.46</v>
+        <v>41.5</v>
       </c>
       <c r="Q15" t="n">
-        <v>44.37</v>
+        <v>41.96</v>
       </c>
       <c r="R15" t="n">
-        <v>0.09229999999999999</v>
+        <v>2.9965</v>
       </c>
       <c r="S15" t="n">
-        <v>-18.422</v>
+        <v>17.5552</v>
       </c>
       <c r="T15" t="n">
-        <v>-11.958</v>
+        <v>-4.1893</v>
       </c>
       <c r="U15" t="n">
-        <v>-1.8703</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="V15" t="n">
-        <v>-7.6251</v>
+        <v>3.5388</v>
       </c>
       <c r="W15" t="n">
-        <v>-2.7081</v>
+        <v>-2.5332</v>
       </c>
       <c r="X15" t="n">
-        <v>-0.201</v>
+        <v>-2.9274</v>
       </c>
       <c r="Y15" t="n">
-        <v>20.0726</v>
+        <v>-16.6834</v>
       </c>
       <c r="Z15" t="n">
-        <v>10.9497</v>
+        <v>0.2418</v>
       </c>
       <c r="AA15" t="n">
-        <v>1.9063</v>
+        <v>-0.5452</v>
       </c>
       <c r="AB15" t="n">
-        <v>8.0351</v>
+        <v>-3.6288</v>
       </c>
       <c r="AC15" t="n">
-        <v>2.4475</v>
+        <v>2.167</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>161</v>
+        <v>184.8</v>
       </c>
       <c r="C16" t="n">
-        <v>173.7</v>
+        <v>195.27</v>
       </c>
       <c r="D16" t="n">
-        <v>161</v>
+        <v>183.34</v>
       </c>
       <c r="E16" t="n">
-        <v>173.2</v>
+        <v>190.56</v>
       </c>
       <c r="F16" t="n">
-        <v>74.09</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>76.53</v>
+        <v>79.33</v>
       </c>
       <c r="H16" t="n">
-        <v>73.62</v>
+        <v>77.33</v>
       </c>
       <c r="I16" t="n">
-        <v>76.51000000000001</v>
+        <v>77.84</v>
       </c>
       <c r="J16" t="n">
-        <v>9.300000000000001</v>
+        <v>8</v>
       </c>
       <c r="K16" t="n">
-        <v>9.35</v>
+        <v>8.06</v>
       </c>
       <c r="L16" t="n">
-        <v>8.51</v>
+        <v>7.5</v>
       </c>
       <c r="M16" t="n">
-        <v>8.539999999999999</v>
+        <v>7.73</v>
       </c>
       <c r="N16" t="n">
-        <v>43.67</v>
+        <v>41.4</v>
       </c>
       <c r="O16" t="n">
-        <v>43.97</v>
+        <v>41.78</v>
       </c>
       <c r="P16" t="n">
-        <v>42.19</v>
+        <v>40.68</v>
       </c>
       <c r="Q16" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="R16" t="n">
-        <v>14.0299</v>
+        <v>6.8221</v>
       </c>
       <c r="S16" t="n">
-        <v>5.494</v>
+        <v>25.4592</v>
       </c>
       <c r="T16" t="n">
-        <v>-5.9922</v>
+        <v>16.0677</v>
       </c>
       <c r="U16" t="n">
-        <v>4.9088</v>
+        <v>1.1566</v>
       </c>
       <c r="V16" t="n">
-        <v>1.553</v>
+        <v>6.7325</v>
       </c>
       <c r="W16" t="n">
-        <v>-0.9451000000000001</v>
+        <v>3.3183</v>
       </c>
       <c r="X16" t="n">
-        <v>-13.998</v>
+        <v>-6.7551</v>
       </c>
       <c r="Y16" t="n">
-        <v>-7.4756</v>
+        <v>-22.1551</v>
       </c>
       <c r="Z16" t="n">
-        <v>2.2754</v>
+        <v>-16.2514</v>
       </c>
       <c r="AA16" t="n">
-        <v>-4.9132</v>
+        <v>-1.0963</v>
       </c>
       <c r="AB16" t="n">
-        <v>-1.8381</v>
+        <v>-6.4683</v>
       </c>
       <c r="AC16" t="n">
-        <v>0.4763</v>
+        <v>-3.4435</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>171.26</v>
+        <v>211.38</v>
       </c>
       <c r="C17" t="n">
-        <v>179.97</v>
+        <v>228.5</v>
       </c>
       <c r="D17" t="n">
-        <v>168.23</v>
+        <v>209.89</v>
       </c>
       <c r="E17" t="n">
-        <v>178.39</v>
+        <v>225.79</v>
       </c>
       <c r="F17" t="n">
-        <v>75.18000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="G17" t="n">
-        <v>77.79000000000001</v>
+        <v>82.27</v>
       </c>
       <c r="H17" t="n">
-        <v>74.47</v>
+        <v>79.98</v>
       </c>
       <c r="I17" t="n">
-        <v>76.95</v>
+        <v>81.95</v>
       </c>
       <c r="J17" t="n">
-        <v>8.65</v>
+        <v>6.9</v>
       </c>
       <c r="K17" t="n">
-        <v>8.779999999999999</v>
+        <v>6.95</v>
       </c>
       <c r="L17" t="n">
-        <v>8.210000000000001</v>
+        <v>6.19</v>
       </c>
       <c r="M17" t="n">
-        <v>8.289999999999999</v>
+        <v>6.29</v>
       </c>
       <c r="N17" t="n">
-        <v>42.94</v>
+        <v>40.05</v>
       </c>
       <c r="O17" t="n">
-        <v>43.33</v>
+        <v>40.35</v>
       </c>
       <c r="P17" t="n">
-        <v>41.5</v>
+        <v>39.14</v>
       </c>
       <c r="Q17" t="n">
-        <v>41.96</v>
+        <v>39.28</v>
       </c>
       <c r="R17" t="n">
-        <v>2.9965</v>
+        <v>18.4876</v>
       </c>
       <c r="S17" t="n">
-        <v>17.5552</v>
+        <v>30.3637</v>
       </c>
       <c r="T17" t="n">
-        <v>-4.1893</v>
+        <v>48.7908</v>
       </c>
       <c r="U17" t="n">
-        <v>0.5750999999999999</v>
+        <v>5.2801</v>
       </c>
       <c r="V17" t="n">
-        <v>3.5388</v>
+        <v>7.1102</v>
       </c>
       <c r="W17" t="n">
-        <v>-2.5332</v>
+        <v>10.2664</v>
       </c>
       <c r="X17" t="n">
-        <v>-2.9274</v>
+        <v>-18.6287</v>
       </c>
       <c r="Y17" t="n">
-        <v>-16.6834</v>
+        <v>-26.3466</v>
       </c>
       <c r="Z17" t="n">
-        <v>0.2418</v>
+        <v>-36.7839</v>
       </c>
       <c r="AA17" t="n">
-        <v>-0.5452</v>
+        <v>-5.3494</v>
       </c>
       <c r="AB17" t="n">
-        <v>-3.6288</v>
+        <v>-6.8974</v>
       </c>
       <c r="AC17" t="n">
-        <v>2.167</v>
+        <v>-9.7841</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>184.8</v>
+        <v>242.66</v>
       </c>
       <c r="C18" t="n">
-        <v>195.27</v>
+        <v>242.66</v>
       </c>
       <c r="D18" t="n">
-        <v>183.34</v>
+        <v>204</v>
       </c>
       <c r="E18" t="n">
-        <v>190.56</v>
+        <v>217.98</v>
       </c>
       <c r="F18" t="n">
-        <v>78.04000000000001</v>
+        <v>82.87</v>
       </c>
       <c r="G18" t="n">
-        <v>79.33</v>
+        <v>82.91</v>
       </c>
       <c r="H18" t="n">
-        <v>77.33</v>
+        <v>80.33</v>
       </c>
       <c r="I18" t="n">
-        <v>77.84</v>
+        <v>81.67</v>
       </c>
       <c r="J18" t="n">
-        <v>8</v>
+        <v>5.83</v>
       </c>
       <c r="K18" t="n">
-        <v>8.06</v>
+        <v>6.91</v>
       </c>
       <c r="L18" t="n">
-        <v>7.5</v>
+        <v>5.83</v>
       </c>
       <c r="M18" t="n">
-        <v>7.73</v>
+        <v>6.53</v>
       </c>
       <c r="N18" t="n">
-        <v>41.4</v>
+        <v>38.87</v>
       </c>
       <c r="O18" t="n">
-        <v>41.78</v>
+        <v>40.09</v>
       </c>
       <c r="P18" t="n">
-        <v>40.68</v>
+        <v>38.86</v>
       </c>
       <c r="Q18" t="n">
-        <v>41.5</v>
+        <v>39.44</v>
       </c>
       <c r="R18" t="n">
-        <v>6.8221</v>
+        <v>-3.459</v>
       </c>
       <c r="S18" t="n">
-        <v>25.4592</v>
+        <v>22.1929</v>
       </c>
       <c r="T18" t="n">
-        <v>16.0677</v>
+        <v>43.5118</v>
       </c>
       <c r="U18" t="n">
-        <v>1.1566</v>
+        <v>-0.3417</v>
       </c>
       <c r="V18" t="n">
-        <v>6.7325</v>
+        <v>6.1339</v>
       </c>
       <c r="W18" t="n">
-        <v>3.3183</v>
+        <v>11.9841</v>
       </c>
       <c r="X18" t="n">
-        <v>-6.7551</v>
+        <v>3.8156</v>
       </c>
       <c r="Y18" t="n">
-        <v>-22.1551</v>
+        <v>-21.2304</v>
       </c>
       <c r="Z18" t="n">
-        <v>-16.2514</v>
+        <v>-34.2397</v>
       </c>
       <c r="AA18" t="n">
-        <v>-1.0963</v>
+        <v>0.4073</v>
       </c>
       <c r="AB18" t="n">
-        <v>-6.4683</v>
+        <v>-6.0057</v>
       </c>
       <c r="AC18" t="n">
-        <v>-3.4435</v>
+        <v>-11.1111</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>211.38</v>
+        <v>219</v>
       </c>
       <c r="C19" t="n">
-        <v>228.5</v>
+        <v>231.89</v>
       </c>
       <c r="D19" t="n">
-        <v>209.89</v>
+        <v>207.56</v>
       </c>
       <c r="E19" t="n">
-        <v>225.79</v>
+        <v>224.63</v>
       </c>
       <c r="F19" t="n">
-        <v>80.59</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="G19" t="n">
-        <v>82.27</v>
+        <v>84.05</v>
       </c>
       <c r="H19" t="n">
-        <v>79.98</v>
+        <v>80.66</v>
       </c>
       <c r="I19" t="n">
-        <v>81.95</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="J19" t="n">
-        <v>6.9</v>
+        <v>6.49</v>
       </c>
       <c r="K19" t="n">
-        <v>6.95</v>
+        <v>6.83</v>
       </c>
       <c r="L19" t="n">
-        <v>6.19</v>
+        <v>6.1</v>
       </c>
       <c r="M19" t="n">
-        <v>6.29</v>
+        <v>6.31</v>
       </c>
       <c r="N19" t="n">
-        <v>40.05</v>
+        <v>39.41</v>
       </c>
       <c r="O19" t="n">
-        <v>40.35</v>
+        <v>39.94</v>
       </c>
       <c r="P19" t="n">
-        <v>39.14</v>
+        <v>38.3</v>
       </c>
       <c r="Q19" t="n">
-        <v>39.28</v>
+        <v>38.47</v>
       </c>
       <c r="R19" t="n">
-        <v>18.4876</v>
+        <v>3.0507</v>
       </c>
       <c r="S19" t="n">
-        <v>30.3637</v>
+        <v>17.8789</v>
       </c>
       <c r="T19" t="n">
-        <v>48.7908</v>
+        <v>29.694</v>
       </c>
       <c r="U19" t="n">
-        <v>5.2801</v>
+        <v>2.4611</v>
       </c>
       <c r="V19" t="n">
-        <v>7.1102</v>
+        <v>7.5026</v>
       </c>
       <c r="W19" t="n">
-        <v>10.2664</v>
+        <v>9.3713</v>
       </c>
       <c r="X19" t="n">
-        <v>-18.6287</v>
+        <v>-3.3691</v>
       </c>
       <c r="Y19" t="n">
-        <v>-26.3466</v>
+        <v>-18.37</v>
       </c>
       <c r="Z19" t="n">
-        <v>-36.7839</v>
+        <v>-26.1124</v>
       </c>
       <c r="AA19" t="n">
-        <v>-5.3494</v>
+        <v>-2.4594</v>
       </c>
       <c r="AB19" t="n">
-        <v>-6.8974</v>
+        <v>-7.3012</v>
       </c>
       <c r="AC19" t="n">
-        <v>-9.7841</v>
+        <v>-8.817299999999999</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>242.66</v>
+        <v>231.82</v>
       </c>
       <c r="C20" t="n">
-        <v>242.66</v>
+        <v>239.07</v>
       </c>
       <c r="D20" t="n">
-        <v>204</v>
+        <v>218.56</v>
       </c>
       <c r="E20" t="n">
-        <v>217.98</v>
+        <v>224.34</v>
       </c>
       <c r="F20" t="n">
-        <v>82.87</v>
+        <v>84.41</v>
       </c>
       <c r="G20" t="n">
-        <v>82.91</v>
+        <v>85.7</v>
       </c>
       <c r="H20" t="n">
-        <v>80.33</v>
+        <v>83.53</v>
       </c>
       <c r="I20" t="n">
-        <v>81.67</v>
+        <v>84.56</v>
       </c>
       <c r="J20" t="n">
-        <v>5.83</v>
+        <v>6.11</v>
       </c>
       <c r="K20" t="n">
-        <v>6.91</v>
+        <v>6.49</v>
       </c>
       <c r="L20" t="n">
-        <v>5.83</v>
+        <v>5.91</v>
       </c>
       <c r="M20" t="n">
-        <v>6.53</v>
+        <v>6.33</v>
       </c>
       <c r="N20" t="n">
-        <v>38.87</v>
+        <v>38.15</v>
       </c>
       <c r="O20" t="n">
-        <v>40.09</v>
+        <v>38.56</v>
       </c>
       <c r="P20" t="n">
-        <v>38.86</v>
+        <v>37.56</v>
       </c>
       <c r="Q20" t="n">
-        <v>39.44</v>
+        <v>38.08</v>
       </c>
       <c r="R20" t="n">
-        <v>-3.459</v>
+        <v>-0.1291</v>
       </c>
       <c r="S20" t="n">
-        <v>22.1929</v>
+        <v>-0.6422</v>
       </c>
       <c r="T20" t="n">
-        <v>43.5118</v>
+        <v>25.7582</v>
       </c>
       <c r="U20" t="n">
-        <v>-0.3417</v>
+        <v>1.0516</v>
       </c>
       <c r="V20" t="n">
-        <v>6.1339</v>
+        <v>3.1849</v>
       </c>
       <c r="W20" t="n">
-        <v>11.9841</v>
+        <v>9.8895</v>
       </c>
       <c r="X20" t="n">
-        <v>3.8156</v>
+        <v>0.317</v>
       </c>
       <c r="Y20" t="n">
-        <v>-21.2304</v>
+        <v>0.6359</v>
       </c>
       <c r="Z20" t="n">
-        <v>-34.2397</v>
+        <v>-23.6429</v>
       </c>
       <c r="AA20" t="n">
-        <v>0.4073</v>
+        <v>-1.0138</v>
       </c>
       <c r="AB20" t="n">
-        <v>-6.0057</v>
+        <v>-3.055</v>
       </c>
       <c r="AC20" t="n">
-        <v>-11.1111</v>
+        <v>-9.2469</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>219</v>
+        <v>217.265</v>
       </c>
       <c r="C21" t="n">
-        <v>231.89</v>
+        <v>234.06</v>
       </c>
       <c r="D21" t="n">
-        <v>207.56</v>
+        <v>210.14</v>
       </c>
       <c r="E21" t="n">
-        <v>224.63</v>
+        <v>227.03</v>
       </c>
       <c r="F21" t="n">
-        <v>81.73999999999999</v>
+        <v>84.14749999999999</v>
       </c>
       <c r="G21" t="n">
-        <v>84.05</v>
+        <v>87.06</v>
       </c>
       <c r="H21" t="n">
-        <v>80.66</v>
+        <v>83.75</v>
       </c>
       <c r="I21" t="n">
-        <v>83.68000000000001</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>6.49</v>
+        <v>6.55</v>
       </c>
       <c r="K21" t="n">
-        <v>6.83</v>
+        <v>6.74</v>
       </c>
       <c r="L21" t="n">
-        <v>6.1</v>
+        <v>6.05</v>
       </c>
       <c r="M21" t="n">
-        <v>6.31</v>
+        <v>6.26</v>
       </c>
       <c r="N21" t="n">
-        <v>39.41</v>
+        <v>38.27</v>
       </c>
       <c r="O21" t="n">
-        <v>39.94</v>
+        <v>38.4599</v>
       </c>
       <c r="P21" t="n">
-        <v>38.3</v>
+        <v>36.96</v>
       </c>
       <c r="Q21" t="n">
-        <v>38.47</v>
+        <v>37.42</v>
       </c>
       <c r="R21" t="n">
-        <v>3.0507</v>
+        <v>1.1991</v>
       </c>
       <c r="S21" t="n">
-        <v>17.8789</v>
+        <v>4.1518</v>
       </c>
       <c r="T21" t="n">
-        <v>29.694</v>
+        <v>19.1383</v>
       </c>
       <c r="U21" t="n">
-        <v>2.4611</v>
+        <v>1.7502</v>
       </c>
       <c r="V21" t="n">
-        <v>7.5026</v>
+        <v>5.3508</v>
       </c>
       <c r="W21" t="n">
-        <v>9.3713</v>
+        <v>10.5344</v>
       </c>
       <c r="X21" t="n">
-        <v>-3.3691</v>
+        <v>-1.1058</v>
       </c>
       <c r="Y21" t="n">
-        <v>-18.37</v>
+        <v>-4.1348</v>
       </c>
       <c r="Z21" t="n">
-        <v>-26.1124</v>
+        <v>-19.0168</v>
       </c>
       <c r="AA21" t="n">
-        <v>-2.4594</v>
+        <v>-1.7332</v>
       </c>
       <c r="AB21" t="n">
-        <v>-7.3012</v>
+        <v>-5.1217</v>
       </c>
       <c r="AC21" t="n">
-        <v>-8.817299999999999</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>231.82</v>
-      </c>
-      <c r="C22" t="n">
-        <v>239.05</v>
-      </c>
-      <c r="D22" t="n">
-        <v>218.56</v>
-      </c>
-      <c r="E22" t="n">
-        <v>224.34</v>
-      </c>
-      <c r="F22" t="n">
-        <v>84.42</v>
-      </c>
-      <c r="G22" t="n">
-        <v>85.7</v>
-      </c>
-      <c r="H22" t="n">
-        <v>83.53</v>
-      </c>
-      <c r="I22" t="n">
-        <v>84.56</v>
-      </c>
-      <c r="J22" t="n">
-        <v>6.11</v>
-      </c>
-      <c r="K22" t="n">
-        <v>6.49</v>
-      </c>
-      <c r="L22" t="n">
-        <v>5.9107</v>
-      </c>
-      <c r="M22" t="n">
-        <v>6.33</v>
-      </c>
-      <c r="N22" t="n">
-        <v>38.16</v>
-      </c>
-      <c r="O22" t="n">
-        <v>38.5599</v>
-      </c>
-      <c r="P22" t="n">
-        <v>37.57</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>38.08</v>
-      </c>
-      <c r="R22" t="n">
-        <v>-0.1291</v>
-      </c>
-      <c r="S22" t="n">
-        <v>-0.6422</v>
-      </c>
-      <c r="T22" t="n">
-        <v>25.7582</v>
-      </c>
-      <c r="U22" t="n">
-        <v>1.0516</v>
-      </c>
-      <c r="V22" t="n">
-        <v>3.1849</v>
-      </c>
-      <c r="W22" t="n">
-        <v>9.8895</v>
-      </c>
-      <c r="X22" t="n">
-        <v>0.317</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>0.6359</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>-23.6429</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>-1.0138</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>-3.055</v>
-      </c>
-      <c r="AC22" t="n">
-        <v>-9.2469</v>
+        <v>-9.831300000000001</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-02 23:45
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC21"/>
+  <dimension ref="A1:AC22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2193,7 +2193,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>217.265</v>
+        <v>217.27</v>
       </c>
       <c r="C21" t="n">
         <v>234.06</v>
@@ -2205,7 +2205,7 @@
         <v>227.03</v>
       </c>
       <c r="F21" t="n">
-        <v>84.14749999999999</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="G21" t="n">
         <v>87.06</v>
@@ -2232,7 +2232,7 @@
         <v>38.27</v>
       </c>
       <c r="O21" t="n">
-        <v>38.4599</v>
+        <v>38.46</v>
       </c>
       <c r="P21" t="n">
         <v>36.96</v>
@@ -2275,6 +2275,97 @@
       </c>
       <c r="AC21" t="n">
         <v>-9.831300000000001</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>243.18</v>
+      </c>
+      <c r="C22" t="n">
+        <v>267.08</v>
+      </c>
+      <c r="D22" t="n">
+        <v>238.8233</v>
+      </c>
+      <c r="E22" t="n">
+        <v>266.32</v>
+      </c>
+      <c r="F22" t="n">
+        <v>85.95</v>
+      </c>
+      <c r="G22" t="n">
+        <v>87.31999999999999</v>
+      </c>
+      <c r="H22" t="n">
+        <v>84.8313</v>
+      </c>
+      <c r="I22" t="n">
+        <v>87.22</v>
+      </c>
+      <c r="J22" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="K22" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="L22" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="M22" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="N22" t="n">
+        <v>37.46</v>
+      </c>
+      <c r="O22" t="n">
+        <v>37.95</v>
+      </c>
+      <c r="P22" t="n">
+        <v>36.86</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>36.91</v>
+      </c>
+      <c r="R22" t="n">
+        <v>17.3061</v>
+      </c>
+      <c r="S22" t="n">
+        <v>18.5594</v>
+      </c>
+      <c r="T22" t="n">
+        <v>17.9503</v>
+      </c>
+      <c r="U22" t="n">
+        <v>1.3715</v>
+      </c>
+      <c r="V22" t="n">
+        <v>4.2304</v>
+      </c>
+      <c r="W22" t="n">
+        <v>6.4308</v>
+      </c>
+      <c r="X22" t="n">
+        <v>-17.4121</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>-18.0666</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>-17.806</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>-1.3629</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>-4.0551</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>-6.0336</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-03 23:44
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>132.2</v>
+        <v>135</v>
       </c>
       <c r="C2" t="n">
-        <v>133.67</v>
+        <v>147.26</v>
       </c>
       <c r="D2" t="n">
-        <v>123.8</v>
+        <v>134.02</v>
       </c>
       <c r="E2" t="n">
-        <v>127.55</v>
+        <v>144.16</v>
       </c>
       <c r="F2" t="n">
-        <v>65.44</v>
+        <v>66.37</v>
       </c>
       <c r="G2" t="n">
-        <v>66.05</v>
+        <v>67.77</v>
       </c>
       <c r="H2" t="n">
-        <v>63.78</v>
+        <v>66.25</v>
       </c>
       <c r="I2" t="n">
-        <v>64.91</v>
+        <v>67.39</v>
       </c>
       <c r="J2" t="n">
-        <v>12.8</v>
+        <v>12.5</v>
       </c>
       <c r="K2" t="n">
-        <v>13.64</v>
+        <v>12.59</v>
       </c>
       <c r="L2" t="n">
-        <v>12.65</v>
+        <v>11.21</v>
       </c>
       <c r="M2" t="n">
-        <v>13.26</v>
+        <v>11.51</v>
       </c>
       <c r="N2" t="n">
-        <v>50.12</v>
+        <v>49.4</v>
       </c>
       <c r="O2" t="n">
-        <v>51.43</v>
+        <v>49.49</v>
       </c>
       <c r="P2" t="n">
-        <v>49.65</v>
+        <v>48.3</v>
       </c>
       <c r="Q2" t="n">
-        <v>50.51</v>
+        <v>48.59</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>135</v>
+        <v>157.84</v>
       </c>
       <c r="C3" t="n">
-        <v>147.26</v>
+        <v>166</v>
       </c>
       <c r="D3" t="n">
-        <v>134.02</v>
+        <v>149.06</v>
       </c>
       <c r="E3" t="n">
-        <v>144.16</v>
+        <v>165.85</v>
       </c>
       <c r="F3" t="n">
-        <v>66.37</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>67.77</v>
+        <v>71.66</v>
       </c>
       <c r="H3" t="n">
-        <v>66.25</v>
+        <v>68.88</v>
       </c>
       <c r="I3" t="n">
-        <v>67.39</v>
+        <v>71.56999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>12.5</v>
+        <v>10.43</v>
       </c>
       <c r="K3" t="n">
-        <v>12.59</v>
+        <v>11.14</v>
       </c>
       <c r="L3" t="n">
-        <v>11.21</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M3" t="n">
-        <v>11.51</v>
+        <v>9.81</v>
       </c>
       <c r="N3" t="n">
-        <v>49.4</v>
+        <v>47.26</v>
       </c>
       <c r="O3" t="n">
-        <v>49.49</v>
+        <v>47.54</v>
       </c>
       <c r="P3" t="n">
-        <v>48.3</v>
+        <v>45.52</v>
       </c>
       <c r="Q3" t="n">
-        <v>48.59</v>
+        <v>45.59</v>
       </c>
       <c r="R3" t="n">
-        <v>13.0223</v>
+        <v>15.0458</v>
       </c>
       <c r="U3" t="n">
-        <v>3.8207</v>
+        <v>6.2027</v>
       </c>
       <c r="X3" t="n">
-        <v>-13.1976</v>
+        <v>-14.7698</v>
       </c>
       <c r="AA3" t="n">
-        <v>-3.8012</v>
+        <v>-6.1741</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>157.84</v>
+        <v>162.12</v>
       </c>
       <c r="C4" t="n">
-        <v>166</v>
+        <v>162.9</v>
       </c>
       <c r="D4" t="n">
-        <v>149.06</v>
+        <v>147.61</v>
       </c>
       <c r="E4" t="n">
-        <v>165.85</v>
+        <v>152.1</v>
       </c>
       <c r="F4" t="n">
-        <v>69.26000000000001</v>
+        <v>71.87</v>
       </c>
       <c r="G4" t="n">
-        <v>71.66</v>
+        <v>73.3</v>
       </c>
       <c r="H4" t="n">
-        <v>68.88</v>
+        <v>70.38</v>
       </c>
       <c r="I4" t="n">
-        <v>71.56999999999999</v>
+        <v>71.34</v>
       </c>
       <c r="J4" t="n">
-        <v>10.43</v>
+        <v>10.02</v>
       </c>
       <c r="K4" t="n">
-        <v>11.14</v>
+        <v>10.88</v>
       </c>
       <c r="L4" t="n">
-        <v>9.800000000000001</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>9.81</v>
+        <v>10.6</v>
       </c>
       <c r="N4" t="n">
-        <v>47.26</v>
+        <v>45.41</v>
       </c>
       <c r="O4" t="n">
-        <v>47.54</v>
+        <v>46.36</v>
       </c>
       <c r="P4" t="n">
-        <v>45.52</v>
+        <v>44.5</v>
       </c>
       <c r="Q4" t="n">
-        <v>45.59</v>
+        <v>45.73</v>
       </c>
       <c r="R4" t="n">
-        <v>15.0458</v>
+        <v>-8.2906</v>
       </c>
       <c r="U4" t="n">
-        <v>6.2027</v>
+        <v>-0.3214</v>
       </c>
       <c r="X4" t="n">
-        <v>-14.7698</v>
+        <v>8.053000000000001</v>
       </c>
       <c r="AA4" t="n">
-        <v>-6.1741</v>
+        <v>0.3071</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>162.12</v>
+        <v>163</v>
       </c>
       <c r="C5" t="n">
-        <v>162.9</v>
+        <v>177.5</v>
       </c>
       <c r="D5" t="n">
-        <v>147.61</v>
+        <v>161.51</v>
       </c>
       <c r="E5" t="n">
-        <v>152.1</v>
+        <v>176.94</v>
       </c>
       <c r="F5" t="n">
-        <v>71.87</v>
+        <v>72.81999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>73.3</v>
+        <v>76.31</v>
       </c>
       <c r="H5" t="n">
-        <v>70.38</v>
+        <v>72.7</v>
       </c>
       <c r="I5" t="n">
-        <v>71.34</v>
+        <v>76.28</v>
       </c>
       <c r="J5" t="n">
-        <v>10.02</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="K5" t="n">
-        <v>10.88</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="L5" t="n">
-        <v>9.970000000000001</v>
+        <v>8.84</v>
       </c>
       <c r="M5" t="n">
-        <v>10.6</v>
+        <v>8.85</v>
       </c>
       <c r="N5" t="n">
-        <v>45.41</v>
+        <v>44.82</v>
       </c>
       <c r="O5" t="n">
-        <v>46.36</v>
+        <v>44.89</v>
       </c>
       <c r="P5" t="n">
-        <v>44.5</v>
+        <v>42.57</v>
       </c>
       <c r="Q5" t="n">
-        <v>45.73</v>
+        <v>42.57</v>
       </c>
       <c r="R5" t="n">
-        <v>-8.2906</v>
+        <v>16.3314</v>
       </c>
       <c r="S5" t="n">
-        <v>19.2474</v>
+        <v>22.7386</v>
       </c>
       <c r="U5" t="n">
-        <v>-0.3214</v>
+        <v>6.9246</v>
       </c>
       <c r="V5" t="n">
-        <v>9.906000000000001</v>
+        <v>13.1919</v>
       </c>
       <c r="X5" t="n">
-        <v>8.053000000000001</v>
+        <v>-16.5094</v>
       </c>
       <c r="Y5" t="n">
-        <v>-20.0603</v>
+        <v>-23.1103</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.3071</v>
+        <v>-6.9101</v>
       </c>
       <c r="AB5" t="n">
-        <v>-9.4635</v>
+        <v>-12.3894</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="C6" t="n">
-        <v>177.5</v>
+        <v>191.29</v>
       </c>
       <c r="D6" t="n">
-        <v>161.51</v>
+        <v>178.94</v>
       </c>
       <c r="E6" t="n">
-        <v>176.94</v>
+        <v>190.42</v>
       </c>
       <c r="F6" t="n">
-        <v>72.81999999999999</v>
+        <v>76</v>
       </c>
       <c r="G6" t="n">
-        <v>76.31</v>
+        <v>77.36</v>
       </c>
       <c r="H6" t="n">
-        <v>72.7</v>
+        <v>75.55</v>
       </c>
       <c r="I6" t="n">
-        <v>76.28</v>
+        <v>76.95999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>9.859999999999999</v>
+        <v>8.65</v>
       </c>
       <c r="K6" t="n">
-        <v>9.970000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="L6" t="n">
-        <v>8.84</v>
+        <v>8.15</v>
       </c>
       <c r="M6" t="n">
-        <v>8.85</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="N6" t="n">
-        <v>44.82</v>
+        <v>42.74</v>
       </c>
       <c r="O6" t="n">
-        <v>44.89</v>
+        <v>43</v>
       </c>
       <c r="P6" t="n">
-        <v>42.57</v>
+        <v>41.99</v>
       </c>
       <c r="Q6" t="n">
-        <v>42.57</v>
+        <v>42.22</v>
       </c>
       <c r="R6" t="n">
-        <v>16.3314</v>
+        <v>7.6184</v>
       </c>
       <c r="S6" t="n">
-        <v>22.7386</v>
+        <v>14.8146</v>
       </c>
       <c r="U6" t="n">
-        <v>6.9246</v>
+        <v>0.8915</v>
       </c>
       <c r="V6" t="n">
-        <v>13.1919</v>
+        <v>7.5311</v>
       </c>
       <c r="X6" t="n">
-        <v>-16.5094</v>
+        <v>-7.3446</v>
       </c>
       <c r="Y6" t="n">
-        <v>-23.1103</v>
+        <v>-16.4118</v>
       </c>
       <c r="AA6" t="n">
-        <v>-6.9101</v>
+        <v>-0.8222</v>
       </c>
       <c r="AB6" t="n">
-        <v>-12.3894</v>
+        <v>-7.392</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>181</v>
+        <v>177.62</v>
       </c>
       <c r="C7" t="n">
-        <v>191.29</v>
+        <v>182.24</v>
       </c>
       <c r="D7" t="n">
-        <v>178.94</v>
+        <v>150.58</v>
       </c>
       <c r="E7" t="n">
-        <v>190.42</v>
+        <v>172.52</v>
       </c>
       <c r="F7" t="n">
-        <v>76</v>
+        <v>75.3</v>
       </c>
       <c r="G7" t="n">
-        <v>77.36</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>75.55</v>
+        <v>71.55</v>
       </c>
       <c r="I7" t="n">
-        <v>76.95999999999999</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>8.65</v>
+        <v>8.75</v>
       </c>
       <c r="K7" t="n">
-        <v>8.77</v>
+        <v>9.91</v>
       </c>
       <c r="L7" t="n">
-        <v>8.15</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="M7" t="n">
-        <v>8.199999999999999</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N7" t="n">
-        <v>42.74</v>
+        <v>43.14</v>
       </c>
       <c r="O7" t="n">
-        <v>43</v>
+        <v>45.19</v>
       </c>
       <c r="P7" t="n">
-        <v>41.99</v>
+        <v>42.79</v>
       </c>
       <c r="Q7" t="n">
-        <v>42.22</v>
+        <v>43.31</v>
       </c>
       <c r="R7" t="n">
-        <v>7.6184</v>
+        <v>-9.4003</v>
       </c>
       <c r="S7" t="n">
-        <v>14.8146</v>
+        <v>13.4254</v>
       </c>
       <c r="T7" t="n">
-        <v>49.2905</v>
+        <v>19.6726</v>
       </c>
       <c r="U7" t="n">
-        <v>0.8915</v>
+        <v>-2.5988</v>
       </c>
       <c r="V7" t="n">
-        <v>7.5311</v>
+        <v>5.0743</v>
       </c>
       <c r="W7" t="n">
-        <v>18.5642</v>
+        <v>11.2331</v>
       </c>
       <c r="X7" t="n">
-        <v>-7.3446</v>
+        <v>9.1463</v>
       </c>
       <c r="Y7" t="n">
-        <v>-16.4118</v>
+        <v>-15.566</v>
       </c>
       <c r="Z7" t="n">
-        <v>-38.1599</v>
+        <v>-22.2415</v>
       </c>
       <c r="AA7" t="n">
-        <v>-0.8222</v>
+        <v>2.5817</v>
       </c>
       <c r="AB7" t="n">
-        <v>-7.392</v>
+        <v>-5.2919</v>
       </c>
       <c r="AC7" t="n">
-        <v>-16.4126</v>
+        <v>-10.8664</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>177.62</v>
+        <v>183.84</v>
       </c>
       <c r="C8" t="n">
-        <v>182.24</v>
+        <v>188.49</v>
       </c>
       <c r="D8" t="n">
-        <v>150.58</v>
+        <v>172.26</v>
       </c>
       <c r="E8" t="n">
-        <v>172.52</v>
+        <v>184.24</v>
       </c>
       <c r="F8" t="n">
-        <v>75.3</v>
+        <v>75.81</v>
       </c>
       <c r="G8" t="n">
-        <v>75.93000000000001</v>
+        <v>77.94</v>
       </c>
       <c r="H8" t="n">
-        <v>71.55</v>
+        <v>74.19</v>
       </c>
       <c r="I8" t="n">
-        <v>74.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>8.75</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>9.91</v>
+        <v>8.98</v>
       </c>
       <c r="L8" t="n">
-        <v>8.550000000000001</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>8.949999999999999</v>
+        <v>8.35</v>
       </c>
       <c r="N8" t="n">
-        <v>43.14</v>
+        <v>42.83</v>
       </c>
       <c r="O8" t="n">
-        <v>45.19</v>
+        <v>43.77</v>
       </c>
       <c r="P8" t="n">
-        <v>42.79</v>
+        <v>41.6</v>
       </c>
       <c r="Q8" t="n">
-        <v>43.31</v>
+        <v>41.99</v>
       </c>
       <c r="R8" t="n">
-        <v>-9.4003</v>
+        <v>6.7934</v>
       </c>
       <c r="S8" t="n">
-        <v>13.4254</v>
+        <v>4.1257</v>
       </c>
       <c r="T8" t="n">
-        <v>19.6726</v>
+        <v>11.0883</v>
       </c>
       <c r="U8" t="n">
-        <v>-2.5988</v>
+        <v>3.0416</v>
       </c>
       <c r="V8" t="n">
-        <v>5.0743</v>
+        <v>1.2585</v>
       </c>
       <c r="W8" t="n">
-        <v>11.2331</v>
+        <v>7.9223</v>
       </c>
       <c r="X8" t="n">
-        <v>9.1463</v>
+        <v>-6.7039</v>
       </c>
       <c r="Y8" t="n">
-        <v>-15.566</v>
+        <v>-5.6497</v>
       </c>
       <c r="Z8" t="n">
-        <v>-22.2415</v>
+        <v>-14.8828</v>
       </c>
       <c r="AA8" t="n">
-        <v>2.5817</v>
+        <v>-3.0478</v>
       </c>
       <c r="AB8" t="n">
-        <v>-5.2919</v>
+        <v>-1.3625</v>
       </c>
       <c r="AC8" t="n">
-        <v>-10.8664</v>
+        <v>-7.8965</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>183.84</v>
+        <v>182.67</v>
       </c>
       <c r="C9" t="n">
-        <v>188.49</v>
+        <v>189.56</v>
       </c>
       <c r="D9" t="n">
-        <v>172.26</v>
+        <v>178.28</v>
       </c>
       <c r="E9" t="n">
-        <v>184.24</v>
+        <v>186.19</v>
       </c>
       <c r="F9" t="n">
-        <v>75.81</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>77.94</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>74.19</v>
+        <v>77.16</v>
       </c>
       <c r="I9" t="n">
-        <v>77.23999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="J9" t="n">
-        <v>8.380000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="K9" t="n">
-        <v>8.98</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L9" t="n">
-        <v>8.140000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M9" t="n">
-        <v>8.35</v>
+        <v>8.27</v>
       </c>
       <c r="N9" t="n">
-        <v>42.83</v>
+        <v>41.98</v>
       </c>
       <c r="O9" t="n">
-        <v>43.77</v>
+        <v>42.06</v>
       </c>
       <c r="P9" t="n">
-        <v>41.6</v>
+        <v>40.68</v>
       </c>
       <c r="Q9" t="n">
-        <v>41.99</v>
+        <v>41.07</v>
       </c>
       <c r="R9" t="n">
-        <v>6.7934</v>
+        <v>1.0584</v>
       </c>
       <c r="S9" t="n">
-        <v>4.1257</v>
+        <v>-2.2214</v>
       </c>
       <c r="T9" t="n">
-        <v>11.0883</v>
+        <v>22.4129</v>
       </c>
       <c r="U9" t="n">
-        <v>3.0416</v>
+        <v>2.2139</v>
       </c>
       <c r="V9" t="n">
-        <v>1.2585</v>
+        <v>2.5858</v>
       </c>
       <c r="W9" t="n">
-        <v>7.9223</v>
+        <v>10.6672</v>
       </c>
       <c r="X9" t="n">
-        <v>-6.7039</v>
+        <v>-0.9581</v>
       </c>
       <c r="Y9" t="n">
-        <v>-5.6497</v>
+        <v>0.8537</v>
       </c>
       <c r="Z9" t="n">
-        <v>-14.8828</v>
+        <v>-21.9811</v>
       </c>
       <c r="AA9" t="n">
-        <v>-3.0478</v>
+        <v>-2.191</v>
       </c>
       <c r="AB9" t="n">
-        <v>-1.3625</v>
+        <v>-2.7238</v>
       </c>
       <c r="AC9" t="n">
-        <v>-7.8965</v>
+        <v>-10.1902</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>182.67</v>
+        <v>167</v>
       </c>
       <c r="C10" t="n">
-        <v>189.56</v>
+        <v>174.4</v>
       </c>
       <c r="D10" t="n">
-        <v>178.28</v>
+        <v>161.14</v>
       </c>
       <c r="E10" t="n">
-        <v>186.19</v>
+        <v>164.18</v>
       </c>
       <c r="F10" t="n">
-        <v>77.29000000000001</v>
+        <v>75.73</v>
       </c>
       <c r="G10" t="n">
-        <v>79.68000000000001</v>
+        <v>77.37</v>
       </c>
       <c r="H10" t="n">
-        <v>77.16</v>
+        <v>74.23</v>
       </c>
       <c r="I10" t="n">
-        <v>78.95</v>
+        <v>75.34</v>
       </c>
       <c r="J10" t="n">
-        <v>8.43</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>8.630000000000001</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="L10" t="n">
-        <v>8.119999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M10" t="n">
-        <v>8.27</v>
+        <v>9.23</v>
       </c>
       <c r="N10" t="n">
-        <v>41.98</v>
+        <v>42.77</v>
       </c>
       <c r="O10" t="n">
-        <v>42.06</v>
+        <v>43.57</v>
       </c>
       <c r="P10" t="n">
-        <v>40.68</v>
+        <v>41.93</v>
       </c>
       <c r="Q10" t="n">
-        <v>41.07</v>
+        <v>42.98</v>
       </c>
       <c r="R10" t="n">
-        <v>1.0584</v>
+        <v>-11.8213</v>
       </c>
       <c r="S10" t="n">
-        <v>-2.2214</v>
+        <v>-4.8342</v>
       </c>
       <c r="T10" t="n">
-        <v>22.4129</v>
+        <v>-7.2115</v>
       </c>
       <c r="U10" t="n">
-        <v>2.2139</v>
+        <v>-4.5725</v>
       </c>
       <c r="V10" t="n">
-        <v>2.5858</v>
+        <v>0.5069</v>
       </c>
       <c r="W10" t="n">
-        <v>10.6672</v>
+        <v>-1.2323</v>
       </c>
       <c r="X10" t="n">
-        <v>-0.9581</v>
+        <v>11.6082</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.8537</v>
+        <v>3.1285</v>
       </c>
       <c r="Z10" t="n">
-        <v>-21.9811</v>
+        <v>4.2938</v>
       </c>
       <c r="AA10" t="n">
-        <v>-2.191</v>
+        <v>4.6506</v>
       </c>
       <c r="AB10" t="n">
-        <v>-2.7238</v>
+        <v>-0.7619</v>
       </c>
       <c r="AC10" t="n">
-        <v>-10.1902</v>
+        <v>0.9631</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>167</v>
+        <v>172.95</v>
       </c>
       <c r="C11" t="n">
-        <v>174.4</v>
+        <v>174.61</v>
       </c>
       <c r="D11" t="n">
-        <v>161.14</v>
+        <v>142.69</v>
       </c>
       <c r="E11" t="n">
-        <v>164.18</v>
+        <v>151.75</v>
       </c>
       <c r="F11" t="n">
-        <v>75.73</v>
+        <v>76.13</v>
       </c>
       <c r="G11" t="n">
-        <v>77.37</v>
+        <v>76.27</v>
       </c>
       <c r="H11" t="n">
-        <v>74.23</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>75.34</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>9.130000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="K11" t="n">
-        <v>9.390000000000001</v>
+        <v>10.47</v>
       </c>
       <c r="L11" t="n">
-        <v>8.800000000000001</v>
+        <v>8.68</v>
       </c>
       <c r="M11" t="n">
-        <v>9.23</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>42.77</v>
+        <v>42.51</v>
       </c>
       <c r="O11" t="n">
-        <v>43.57</v>
+        <v>44.82</v>
       </c>
       <c r="P11" t="n">
-        <v>41.93</v>
+        <v>42.44</v>
       </c>
       <c r="Q11" t="n">
-        <v>42.98</v>
+        <v>43.54</v>
       </c>
       <c r="R11" t="n">
-        <v>-11.8213</v>
+        <v>-7.571</v>
       </c>
       <c r="S11" t="n">
-        <v>-4.8342</v>
+        <v>-17.6346</v>
       </c>
       <c r="T11" t="n">
-        <v>-7.2115</v>
+        <v>-20.3077</v>
       </c>
       <c r="U11" t="n">
-        <v>-4.5725</v>
+        <v>-1.3539</v>
       </c>
       <c r="V11" t="n">
-        <v>0.5069</v>
+        <v>-3.7804</v>
       </c>
       <c r="W11" t="n">
-        <v>-1.2323</v>
+        <v>-3.4304</v>
       </c>
       <c r="X11" t="n">
-        <v>11.6082</v>
+        <v>7.8007</v>
       </c>
       <c r="Y11" t="n">
-        <v>3.1285</v>
+        <v>19.1617</v>
       </c>
       <c r="Z11" t="n">
-        <v>4.2938</v>
+        <v>21.3415</v>
       </c>
       <c r="AA11" t="n">
-        <v>4.6506</v>
+        <v>1.3029</v>
       </c>
       <c r="AB11" t="n">
-        <v>-0.7619</v>
+        <v>3.6914</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.9631</v>
+        <v>3.1265</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>172.95</v>
+        <v>141.24</v>
       </c>
       <c r="C12" t="n">
-        <v>174.61</v>
+        <v>160.6</v>
       </c>
       <c r="D12" t="n">
-        <v>142.69</v>
+        <v>135.02</v>
       </c>
       <c r="E12" t="n">
-        <v>151.75</v>
+        <v>151.89</v>
       </c>
       <c r="F12" t="n">
-        <v>76.13</v>
+        <v>72.41</v>
       </c>
       <c r="G12" t="n">
-        <v>76.27</v>
+        <v>74.5</v>
       </c>
       <c r="H12" t="n">
-        <v>72.09999999999999</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>74.31999999999999</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>8.77</v>
+        <v>10.64</v>
       </c>
       <c r="K12" t="n">
-        <v>10.47</v>
+        <v>11.07</v>
       </c>
       <c r="L12" t="n">
-        <v>8.68</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="M12" t="n">
-        <v>9.949999999999999</v>
+        <v>9.93</v>
       </c>
       <c r="N12" t="n">
-        <v>42.51</v>
+        <v>44.68</v>
       </c>
       <c r="O12" t="n">
-        <v>44.82</v>
+        <v>45.53</v>
       </c>
       <c r="P12" t="n">
-        <v>42.44</v>
+        <v>43.46</v>
       </c>
       <c r="Q12" t="n">
-        <v>43.54</v>
+        <v>44.37</v>
       </c>
       <c r="R12" t="n">
-        <v>-7.571</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="S12" t="n">
-        <v>-17.6346</v>
+        <v>-18.422</v>
       </c>
       <c r="T12" t="n">
-        <v>-20.3077</v>
+        <v>-11.958</v>
       </c>
       <c r="U12" t="n">
-        <v>-1.3539</v>
+        <v>-1.8703</v>
       </c>
       <c r="V12" t="n">
-        <v>-3.7804</v>
+        <v>-7.6251</v>
       </c>
       <c r="W12" t="n">
-        <v>-3.4304</v>
+        <v>-2.7081</v>
       </c>
       <c r="X12" t="n">
-        <v>7.8007</v>
+        <v>-0.201</v>
       </c>
       <c r="Y12" t="n">
-        <v>19.1617</v>
+        <v>20.0726</v>
       </c>
       <c r="Z12" t="n">
-        <v>21.3415</v>
+        <v>10.9497</v>
       </c>
       <c r="AA12" t="n">
-        <v>1.3029</v>
+        <v>1.9063</v>
       </c>
       <c r="AB12" t="n">
-        <v>3.6914</v>
+        <v>8.0351</v>
       </c>
       <c r="AC12" t="n">
-        <v>3.1265</v>
+        <v>2.4475</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>141.24</v>
+        <v>161</v>
       </c>
       <c r="C13" t="n">
-        <v>160.6</v>
+        <v>173.7</v>
       </c>
       <c r="D13" t="n">
-        <v>135.02</v>
+        <v>161</v>
       </c>
       <c r="E13" t="n">
-        <v>151.89</v>
+        <v>173.2</v>
       </c>
       <c r="F13" t="n">
-        <v>72.41</v>
+        <v>74.09</v>
       </c>
       <c r="G13" t="n">
-        <v>74.5</v>
+        <v>76.53</v>
       </c>
       <c r="H13" t="n">
-        <v>70.95999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="I13" t="n">
-        <v>72.93000000000001</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>10.64</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>11.07</v>
+        <v>9.35</v>
       </c>
       <c r="L13" t="n">
-        <v>9.369999999999999</v>
+        <v>8.51</v>
       </c>
       <c r="M13" t="n">
-        <v>9.93</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N13" t="n">
-        <v>44.68</v>
+        <v>43.67</v>
       </c>
       <c r="O13" t="n">
-        <v>45.53</v>
+        <v>43.97</v>
       </c>
       <c r="P13" t="n">
-        <v>43.46</v>
+        <v>42.19</v>
       </c>
       <c r="Q13" t="n">
-        <v>44.37</v>
+        <v>42.19</v>
       </c>
       <c r="R13" t="n">
-        <v>0.09229999999999999</v>
+        <v>14.0299</v>
       </c>
       <c r="S13" t="n">
-        <v>-18.422</v>
+        <v>5.494</v>
       </c>
       <c r="T13" t="n">
-        <v>-11.958</v>
+        <v>-5.9922</v>
       </c>
       <c r="U13" t="n">
-        <v>-1.8703</v>
+        <v>4.9088</v>
       </c>
       <c r="V13" t="n">
-        <v>-7.6251</v>
+        <v>1.553</v>
       </c>
       <c r="W13" t="n">
-        <v>-2.7081</v>
+        <v>-0.9451000000000001</v>
       </c>
       <c r="X13" t="n">
-        <v>-0.201</v>
+        <v>-13.998</v>
       </c>
       <c r="Y13" t="n">
-        <v>20.0726</v>
+        <v>-7.4756</v>
       </c>
       <c r="Z13" t="n">
-        <v>10.9497</v>
+        <v>2.2754</v>
       </c>
       <c r="AA13" t="n">
-        <v>1.9063</v>
+        <v>-4.9132</v>
       </c>
       <c r="AB13" t="n">
-        <v>8.0351</v>
+        <v>-1.8381</v>
       </c>
       <c r="AC13" t="n">
-        <v>2.4475</v>
+        <v>0.4763</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>161</v>
+        <v>171.26</v>
       </c>
       <c r="C14" t="n">
-        <v>173.7</v>
+        <v>179.97</v>
       </c>
       <c r="D14" t="n">
-        <v>161</v>
+        <v>168.23</v>
       </c>
       <c r="E14" t="n">
-        <v>173.2</v>
+        <v>178.39</v>
       </c>
       <c r="F14" t="n">
-        <v>74.09</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>76.53</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H14" t="n">
-        <v>73.62</v>
+        <v>74.47</v>
       </c>
       <c r="I14" t="n">
-        <v>76.51000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J14" t="n">
-        <v>9.300000000000001</v>
+        <v>8.65</v>
       </c>
       <c r="K14" t="n">
-        <v>9.35</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L14" t="n">
-        <v>8.51</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M14" t="n">
-        <v>8.539999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N14" t="n">
-        <v>43.67</v>
+        <v>42.94</v>
       </c>
       <c r="O14" t="n">
-        <v>43.97</v>
+        <v>43.33</v>
       </c>
       <c r="P14" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="Q14" t="n">
-        <v>42.19</v>
+        <v>41.96</v>
       </c>
       <c r="R14" t="n">
-        <v>14.0299</v>
+        <v>2.9965</v>
       </c>
       <c r="S14" t="n">
-        <v>5.494</v>
+        <v>17.5552</v>
       </c>
       <c r="T14" t="n">
-        <v>-5.9922</v>
+        <v>-4.1893</v>
       </c>
       <c r="U14" t="n">
-        <v>4.9088</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="V14" t="n">
-        <v>1.553</v>
+        <v>3.5388</v>
       </c>
       <c r="W14" t="n">
-        <v>-0.9451000000000001</v>
+        <v>-2.5332</v>
       </c>
       <c r="X14" t="n">
-        <v>-13.998</v>
+        <v>-2.9274</v>
       </c>
       <c r="Y14" t="n">
-        <v>-7.4756</v>
+        <v>-16.6834</v>
       </c>
       <c r="Z14" t="n">
-        <v>2.2754</v>
+        <v>0.2418</v>
       </c>
       <c r="AA14" t="n">
-        <v>-4.9132</v>
+        <v>-0.5452</v>
       </c>
       <c r="AB14" t="n">
-        <v>-1.8381</v>
+        <v>-3.6288</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.4763</v>
+        <v>2.167</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>171.26</v>
+        <v>184.8</v>
       </c>
       <c r="C15" t="n">
-        <v>179.97</v>
+        <v>195.27</v>
       </c>
       <c r="D15" t="n">
-        <v>168.23</v>
+        <v>183.34</v>
       </c>
       <c r="E15" t="n">
-        <v>178.39</v>
+        <v>190.56</v>
       </c>
       <c r="F15" t="n">
-        <v>75.18000000000001</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>77.79000000000001</v>
+        <v>79.33</v>
       </c>
       <c r="H15" t="n">
-        <v>74.47</v>
+        <v>77.33</v>
       </c>
       <c r="I15" t="n">
-        <v>76.95</v>
+        <v>77.84</v>
       </c>
       <c r="J15" t="n">
-        <v>8.65</v>
+        <v>8</v>
       </c>
       <c r="K15" t="n">
-        <v>8.779999999999999</v>
+        <v>8.06</v>
       </c>
       <c r="L15" t="n">
-        <v>8.210000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="M15" t="n">
-        <v>8.289999999999999</v>
+        <v>7.73</v>
       </c>
       <c r="N15" t="n">
-        <v>42.94</v>
+        <v>41.4</v>
       </c>
       <c r="O15" t="n">
-        <v>43.33</v>
+        <v>41.78</v>
       </c>
       <c r="P15" t="n">
+        <v>40.68</v>
+      </c>
+      <c r="Q15" t="n">
         <v>41.5</v>
       </c>
-      <c r="Q15" t="n">
-        <v>41.96</v>
-      </c>
       <c r="R15" t="n">
-        <v>2.9965</v>
+        <v>6.8221</v>
       </c>
       <c r="S15" t="n">
-        <v>17.5552</v>
+        <v>25.4592</v>
       </c>
       <c r="T15" t="n">
-        <v>-4.1893</v>
+        <v>16.0677</v>
       </c>
       <c r="U15" t="n">
-        <v>0.5750999999999999</v>
+        <v>1.1566</v>
       </c>
       <c r="V15" t="n">
-        <v>3.5388</v>
+        <v>6.7325</v>
       </c>
       <c r="W15" t="n">
-        <v>-2.5332</v>
+        <v>3.3183</v>
       </c>
       <c r="X15" t="n">
-        <v>-2.9274</v>
+        <v>-6.7551</v>
       </c>
       <c r="Y15" t="n">
-        <v>-16.6834</v>
+        <v>-22.1551</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.2418</v>
+        <v>-16.2514</v>
       </c>
       <c r="AA15" t="n">
-        <v>-0.5452</v>
+        <v>-1.0963</v>
       </c>
       <c r="AB15" t="n">
-        <v>-3.6288</v>
+        <v>-6.4683</v>
       </c>
       <c r="AC15" t="n">
-        <v>2.167</v>
+        <v>-3.4435</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>184.8</v>
+        <v>211.38</v>
       </c>
       <c r="C16" t="n">
-        <v>195.27</v>
+        <v>228.5</v>
       </c>
       <c r="D16" t="n">
-        <v>183.34</v>
+        <v>209.89</v>
       </c>
       <c r="E16" t="n">
-        <v>190.56</v>
+        <v>225.79</v>
       </c>
       <c r="F16" t="n">
-        <v>78.04000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="G16" t="n">
-        <v>79.33</v>
+        <v>82.27</v>
       </c>
       <c r="H16" t="n">
-        <v>77.33</v>
+        <v>79.98</v>
       </c>
       <c r="I16" t="n">
-        <v>77.84</v>
+        <v>81.95</v>
       </c>
       <c r="J16" t="n">
-        <v>8</v>
+        <v>6.9</v>
       </c>
       <c r="K16" t="n">
-        <v>8.06</v>
+        <v>6.95</v>
       </c>
       <c r="L16" t="n">
-        <v>7.5</v>
+        <v>6.19</v>
       </c>
       <c r="M16" t="n">
-        <v>7.73</v>
+        <v>6.29</v>
       </c>
       <c r="N16" t="n">
-        <v>41.4</v>
+        <v>40.05</v>
       </c>
       <c r="O16" t="n">
-        <v>41.78</v>
+        <v>40.35</v>
       </c>
       <c r="P16" t="n">
-        <v>40.68</v>
+        <v>39.14</v>
       </c>
       <c r="Q16" t="n">
-        <v>41.5</v>
+        <v>39.28</v>
       </c>
       <c r="R16" t="n">
-        <v>6.8221</v>
+        <v>18.4876</v>
       </c>
       <c r="S16" t="n">
-        <v>25.4592</v>
+        <v>30.3637</v>
       </c>
       <c r="T16" t="n">
-        <v>16.0677</v>
+        <v>48.7908</v>
       </c>
       <c r="U16" t="n">
-        <v>1.1566</v>
+        <v>5.2801</v>
       </c>
       <c r="V16" t="n">
-        <v>6.7325</v>
+        <v>7.1102</v>
       </c>
       <c r="W16" t="n">
-        <v>3.3183</v>
+        <v>10.2664</v>
       </c>
       <c r="X16" t="n">
-        <v>-6.7551</v>
+        <v>-18.6287</v>
       </c>
       <c r="Y16" t="n">
-        <v>-22.1551</v>
+        <v>-26.3466</v>
       </c>
       <c r="Z16" t="n">
-        <v>-16.2514</v>
+        <v>-36.7839</v>
       </c>
       <c r="AA16" t="n">
-        <v>-1.0963</v>
+        <v>-5.3494</v>
       </c>
       <c r="AB16" t="n">
-        <v>-6.4683</v>
+        <v>-6.8974</v>
       </c>
       <c r="AC16" t="n">
-        <v>-3.4435</v>
+        <v>-9.7841</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>211.38</v>
+        <v>242.66</v>
       </c>
       <c r="C17" t="n">
-        <v>228.5</v>
+        <v>242.66</v>
       </c>
       <c r="D17" t="n">
-        <v>209.89</v>
+        <v>204</v>
       </c>
       <c r="E17" t="n">
-        <v>225.79</v>
+        <v>217.98</v>
       </c>
       <c r="F17" t="n">
-        <v>80.59</v>
+        <v>82.87</v>
       </c>
       <c r="G17" t="n">
-        <v>82.27</v>
+        <v>82.91</v>
       </c>
       <c r="H17" t="n">
-        <v>79.98</v>
+        <v>80.33</v>
       </c>
       <c r="I17" t="n">
-        <v>81.95</v>
+        <v>81.67</v>
       </c>
       <c r="J17" t="n">
-        <v>6.9</v>
+        <v>5.83</v>
       </c>
       <c r="K17" t="n">
-        <v>6.95</v>
+        <v>6.91</v>
       </c>
       <c r="L17" t="n">
-        <v>6.19</v>
+        <v>5.83</v>
       </c>
       <c r="M17" t="n">
-        <v>6.29</v>
+        <v>6.53</v>
       </c>
       <c r="N17" t="n">
-        <v>40.05</v>
+        <v>38.87</v>
       </c>
       <c r="O17" t="n">
-        <v>40.35</v>
+        <v>40.09</v>
       </c>
       <c r="P17" t="n">
-        <v>39.14</v>
+        <v>38.86</v>
       </c>
       <c r="Q17" t="n">
-        <v>39.28</v>
+        <v>39.44</v>
       </c>
       <c r="R17" t="n">
-        <v>18.4876</v>
+        <v>-3.459</v>
       </c>
       <c r="S17" t="n">
-        <v>30.3637</v>
+        <v>22.1929</v>
       </c>
       <c r="T17" t="n">
-        <v>48.7908</v>
+        <v>43.5118</v>
       </c>
       <c r="U17" t="n">
-        <v>5.2801</v>
+        <v>-0.3417</v>
       </c>
       <c r="V17" t="n">
-        <v>7.1102</v>
+        <v>6.1339</v>
       </c>
       <c r="W17" t="n">
-        <v>10.2664</v>
+        <v>11.9841</v>
       </c>
       <c r="X17" t="n">
-        <v>-18.6287</v>
+        <v>3.8156</v>
       </c>
       <c r="Y17" t="n">
-        <v>-26.3466</v>
+        <v>-21.2304</v>
       </c>
       <c r="Z17" t="n">
-        <v>-36.7839</v>
+        <v>-34.2397</v>
       </c>
       <c r="AA17" t="n">
-        <v>-5.3494</v>
+        <v>0.4073</v>
       </c>
       <c r="AB17" t="n">
-        <v>-6.8974</v>
+        <v>-6.0057</v>
       </c>
       <c r="AC17" t="n">
-        <v>-9.7841</v>
+        <v>-11.1111</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>242.66</v>
+        <v>219</v>
       </c>
       <c r="C18" t="n">
-        <v>242.66</v>
+        <v>231.89</v>
       </c>
       <c r="D18" t="n">
-        <v>204</v>
+        <v>207.56</v>
       </c>
       <c r="E18" t="n">
-        <v>217.98</v>
+        <v>224.63</v>
       </c>
       <c r="F18" t="n">
-        <v>82.87</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="G18" t="n">
-        <v>82.91</v>
+        <v>84.05</v>
       </c>
       <c r="H18" t="n">
-        <v>80.33</v>
+        <v>80.66</v>
       </c>
       <c r="I18" t="n">
-        <v>81.67</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>5.83</v>
+        <v>6.49</v>
       </c>
       <c r="K18" t="n">
-        <v>6.91</v>
+        <v>6.83</v>
       </c>
       <c r="L18" t="n">
-        <v>5.83</v>
+        <v>6.1</v>
       </c>
       <c r="M18" t="n">
-        <v>6.53</v>
+        <v>6.31</v>
       </c>
       <c r="N18" t="n">
-        <v>38.87</v>
+        <v>39.41</v>
       </c>
       <c r="O18" t="n">
-        <v>40.09</v>
+        <v>39.94</v>
       </c>
       <c r="P18" t="n">
-        <v>38.86</v>
+        <v>38.3</v>
       </c>
       <c r="Q18" t="n">
-        <v>39.44</v>
+        <v>38.47</v>
       </c>
       <c r="R18" t="n">
-        <v>-3.459</v>
+        <v>3.0507</v>
       </c>
       <c r="S18" t="n">
-        <v>22.1929</v>
+        <v>17.8789</v>
       </c>
       <c r="T18" t="n">
-        <v>43.5118</v>
+        <v>29.694</v>
       </c>
       <c r="U18" t="n">
-        <v>-0.3417</v>
+        <v>2.4611</v>
       </c>
       <c r="V18" t="n">
-        <v>6.1339</v>
+        <v>7.5026</v>
       </c>
       <c r="W18" t="n">
-        <v>11.9841</v>
+        <v>9.3713</v>
       </c>
       <c r="X18" t="n">
-        <v>3.8156</v>
+        <v>-3.3691</v>
       </c>
       <c r="Y18" t="n">
-        <v>-21.2304</v>
+        <v>-18.37</v>
       </c>
       <c r="Z18" t="n">
-        <v>-34.2397</v>
+        <v>-26.1124</v>
       </c>
       <c r="AA18" t="n">
-        <v>0.4073</v>
+        <v>-2.4594</v>
       </c>
       <c r="AB18" t="n">
-        <v>-6.0057</v>
+        <v>-7.3012</v>
       </c>
       <c r="AC18" t="n">
-        <v>-11.1111</v>
+        <v>-8.817299999999999</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>219</v>
+        <v>231.82</v>
       </c>
       <c r="C19" t="n">
-        <v>231.89</v>
+        <v>239.07</v>
       </c>
       <c r="D19" t="n">
-        <v>207.56</v>
+        <v>218.56</v>
       </c>
       <c r="E19" t="n">
-        <v>224.63</v>
+        <v>224.34</v>
       </c>
       <c r="F19" t="n">
-        <v>81.73999999999999</v>
+        <v>84.41</v>
       </c>
       <c r="G19" t="n">
-        <v>84.05</v>
+        <v>85.7</v>
       </c>
       <c r="H19" t="n">
-        <v>80.66</v>
+        <v>83.53</v>
       </c>
       <c r="I19" t="n">
-        <v>83.68000000000001</v>
+        <v>84.56</v>
       </c>
       <c r="J19" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="K19" t="n">
         <v>6.49</v>
       </c>
-      <c r="K19" t="n">
-        <v>6.83</v>
-      </c>
       <c r="L19" t="n">
-        <v>6.1</v>
+        <v>5.91</v>
       </c>
       <c r="M19" t="n">
-        <v>6.31</v>
+        <v>6.33</v>
       </c>
       <c r="N19" t="n">
-        <v>39.41</v>
+        <v>38.15</v>
       </c>
       <c r="O19" t="n">
-        <v>39.94</v>
+        <v>38.56</v>
       </c>
       <c r="P19" t="n">
-        <v>38.3</v>
+        <v>37.56</v>
       </c>
       <c r="Q19" t="n">
-        <v>38.47</v>
+        <v>38.08</v>
       </c>
       <c r="R19" t="n">
-        <v>3.0507</v>
+        <v>-0.1291</v>
       </c>
       <c r="S19" t="n">
-        <v>17.8789</v>
+        <v>-0.6422</v>
       </c>
       <c r="T19" t="n">
-        <v>29.694</v>
+        <v>25.7582</v>
       </c>
       <c r="U19" t="n">
-        <v>2.4611</v>
+        <v>1.0516</v>
       </c>
       <c r="V19" t="n">
-        <v>7.5026</v>
+        <v>3.1849</v>
       </c>
       <c r="W19" t="n">
-        <v>9.3713</v>
+        <v>9.8895</v>
       </c>
       <c r="X19" t="n">
-        <v>-3.3691</v>
+        <v>0.317</v>
       </c>
       <c r="Y19" t="n">
-        <v>-18.37</v>
+        <v>0.6359</v>
       </c>
       <c r="Z19" t="n">
-        <v>-26.1124</v>
+        <v>-23.6429</v>
       </c>
       <c r="AA19" t="n">
-        <v>-2.4594</v>
+        <v>-1.0138</v>
       </c>
       <c r="AB19" t="n">
-        <v>-7.3012</v>
+        <v>-3.055</v>
       </c>
       <c r="AC19" t="n">
-        <v>-8.817299999999999</v>
+        <v>-9.2469</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>231.82</v>
+        <v>217.27</v>
       </c>
       <c r="C20" t="n">
-        <v>239.07</v>
+        <v>234.06</v>
       </c>
       <c r="D20" t="n">
-        <v>218.56</v>
+        <v>210.14</v>
       </c>
       <c r="E20" t="n">
-        <v>224.34</v>
+        <v>227.03</v>
       </c>
       <c r="F20" t="n">
-        <v>84.41</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>85.7</v>
+        <v>87.06</v>
       </c>
       <c r="H20" t="n">
-        <v>83.53</v>
+        <v>83.75</v>
       </c>
       <c r="I20" t="n">
-        <v>84.56</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="J20" t="n">
-        <v>6.11</v>
+        <v>6.55</v>
       </c>
       <c r="K20" t="n">
-        <v>6.49</v>
+        <v>6.74</v>
       </c>
       <c r="L20" t="n">
-        <v>5.91</v>
+        <v>6.05</v>
       </c>
       <c r="M20" t="n">
-        <v>6.33</v>
+        <v>6.26</v>
       </c>
       <c r="N20" t="n">
-        <v>38.15</v>
+        <v>38.27</v>
       </c>
       <c r="O20" t="n">
-        <v>38.56</v>
+        <v>38.46</v>
       </c>
       <c r="P20" t="n">
-        <v>37.56</v>
+        <v>36.96</v>
       </c>
       <c r="Q20" t="n">
-        <v>38.08</v>
+        <v>37.42</v>
       </c>
       <c r="R20" t="n">
-        <v>-0.1291</v>
+        <v>1.1991</v>
       </c>
       <c r="S20" t="n">
-        <v>-0.6422</v>
+        <v>4.1518</v>
       </c>
       <c r="T20" t="n">
-        <v>25.7582</v>
+        <v>19.1383</v>
       </c>
       <c r="U20" t="n">
-        <v>1.0516</v>
+        <v>1.7502</v>
       </c>
       <c r="V20" t="n">
-        <v>3.1849</v>
+        <v>5.3508</v>
       </c>
       <c r="W20" t="n">
-        <v>9.8895</v>
+        <v>10.5344</v>
       </c>
       <c r="X20" t="n">
-        <v>0.317</v>
+        <v>-1.1058</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.6359</v>
+        <v>-4.1348</v>
       </c>
       <c r="Z20" t="n">
-        <v>-23.6429</v>
+        <v>-19.0168</v>
       </c>
       <c r="AA20" t="n">
-        <v>-1.0138</v>
+        <v>-1.7332</v>
       </c>
       <c r="AB20" t="n">
-        <v>-3.055</v>
+        <v>-5.1217</v>
       </c>
       <c r="AC20" t="n">
-        <v>-9.2469</v>
+        <v>-9.831300000000001</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>217.27</v>
+        <v>243.18</v>
       </c>
       <c r="C21" t="n">
-        <v>234.06</v>
+        <v>267.08</v>
       </c>
       <c r="D21" t="n">
-        <v>210.14</v>
+        <v>238.82</v>
       </c>
       <c r="E21" t="n">
-        <v>227.03</v>
+        <v>266.32</v>
       </c>
       <c r="F21" t="n">
-        <v>84.15000000000001</v>
+        <v>85.94</v>
       </c>
       <c r="G21" t="n">
-        <v>87.06</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>83.75</v>
+        <v>84.83</v>
       </c>
       <c r="I21" t="n">
-        <v>86.04000000000001</v>
+        <v>87.22</v>
       </c>
       <c r="J21" t="n">
-        <v>6.55</v>
+        <v>5.8</v>
       </c>
       <c r="K21" t="n">
-        <v>6.74</v>
+        <v>5.93</v>
       </c>
       <c r="L21" t="n">
-        <v>6.05</v>
+        <v>5.15</v>
       </c>
       <c r="M21" t="n">
-        <v>6.26</v>
+        <v>5.17</v>
       </c>
       <c r="N21" t="n">
-        <v>38.27</v>
+        <v>37.47</v>
       </c>
       <c r="O21" t="n">
-        <v>38.46</v>
+        <v>37.95</v>
       </c>
       <c r="P21" t="n">
-        <v>36.96</v>
+        <v>36.86</v>
       </c>
       <c r="Q21" t="n">
-        <v>37.42</v>
+        <v>36.91</v>
       </c>
       <c r="R21" t="n">
-        <v>1.1991</v>
+        <v>17.3061</v>
       </c>
       <c r="S21" t="n">
-        <v>4.1518</v>
+        <v>18.5594</v>
       </c>
       <c r="T21" t="n">
-        <v>19.1383</v>
+        <v>17.9503</v>
       </c>
       <c r="U21" t="n">
-        <v>1.7502</v>
+        <v>1.3715</v>
       </c>
       <c r="V21" t="n">
-        <v>5.3508</v>
+        <v>4.2304</v>
       </c>
       <c r="W21" t="n">
-        <v>10.5344</v>
+        <v>6.4308</v>
       </c>
       <c r="X21" t="n">
-        <v>-1.1058</v>
+        <v>-17.4121</v>
       </c>
       <c r="Y21" t="n">
-        <v>-4.1348</v>
+        <v>-18.0666</v>
       </c>
       <c r="Z21" t="n">
-        <v>-19.0168</v>
+        <v>-17.806</v>
       </c>
       <c r="AA21" t="n">
-        <v>-1.7332</v>
+        <v>-1.3629</v>
       </c>
       <c r="AB21" t="n">
-        <v>-5.1217</v>
+        <v>-4.0551</v>
       </c>
       <c r="AC21" t="n">
-        <v>-9.831300000000001</v>
+        <v>-6.0336</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>243.18</v>
+        <v>281.47</v>
       </c>
       <c r="C22" t="n">
-        <v>267.08</v>
+        <v>284.58</v>
       </c>
       <c r="D22" t="n">
-        <v>238.8233</v>
+        <v>257.2601</v>
       </c>
       <c r="E22" t="n">
-        <v>266.32</v>
+        <v>280.54</v>
       </c>
       <c r="F22" t="n">
-        <v>85.95</v>
+        <v>87.675</v>
       </c>
       <c r="G22" t="n">
-        <v>87.31999999999999</v>
+        <v>88.09</v>
       </c>
       <c r="H22" t="n">
-        <v>84.8313</v>
+        <v>85.41</v>
       </c>
       <c r="I22" t="n">
-        <v>87.22</v>
+        <v>86.56</v>
       </c>
       <c r="J22" t="n">
-        <v>5.8</v>
+        <v>4.88</v>
       </c>
       <c r="K22" t="n">
-        <v>5.93</v>
+        <v>5.35</v>
       </c>
       <c r="L22" t="n">
-        <v>5.15</v>
+        <v>4.82</v>
       </c>
       <c r="M22" t="n">
-        <v>5.17</v>
+        <v>4.91</v>
       </c>
       <c r="N22" t="n">
-        <v>37.46</v>
+        <v>36.73</v>
       </c>
       <c r="O22" t="n">
-        <v>37.95</v>
+        <v>37.6869</v>
       </c>
       <c r="P22" t="n">
-        <v>36.86</v>
+        <v>36.55</v>
       </c>
       <c r="Q22" t="n">
-        <v>36.91</v>
+        <v>37.19</v>
       </c>
       <c r="R22" t="n">
-        <v>17.3061</v>
+        <v>5.3394</v>
       </c>
       <c r="S22" t="n">
-        <v>18.5594</v>
+        <v>25.0513</v>
       </c>
       <c r="T22" t="n">
-        <v>17.9503</v>
+        <v>28.6999</v>
       </c>
       <c r="U22" t="n">
-        <v>1.3715</v>
+        <v>-0.7567</v>
       </c>
       <c r="V22" t="n">
-        <v>4.2304</v>
+        <v>2.3652</v>
       </c>
       <c r="W22" t="n">
-        <v>6.4308</v>
+        <v>5.9875</v>
       </c>
       <c r="X22" t="n">
-        <v>-17.4121</v>
+        <v>-5.029</v>
       </c>
       <c r="Y22" t="n">
-        <v>-18.0666</v>
+        <v>-22.4329</v>
       </c>
       <c r="Z22" t="n">
-        <v>-17.806</v>
+        <v>-24.8086</v>
       </c>
       <c r="AA22" t="n">
-        <v>-1.3629</v>
+        <v>0.7586000000000001</v>
       </c>
       <c r="AB22" t="n">
-        <v>-4.0551</v>
+        <v>-2.3372</v>
       </c>
       <c r="AC22" t="n">
-        <v>-6.0336</v>
+        <v>-5.7049</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Master system update 2026-06-04 23:09
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>135</v>
+        <v>157.84</v>
       </c>
       <c r="C2" t="n">
-        <v>147.26</v>
+        <v>166</v>
       </c>
       <c r="D2" t="n">
-        <v>134.02</v>
+        <v>149.06</v>
       </c>
       <c r="E2" t="n">
-        <v>144.16</v>
+        <v>165.85</v>
       </c>
       <c r="F2" t="n">
-        <v>66.37</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>67.77</v>
+        <v>71.66</v>
       </c>
       <c r="H2" t="n">
-        <v>66.25</v>
+        <v>68.88</v>
       </c>
       <c r="I2" t="n">
-        <v>67.39</v>
+        <v>71.56999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>12.5</v>
+        <v>10.43</v>
       </c>
       <c r="K2" t="n">
-        <v>12.59</v>
+        <v>11.14</v>
       </c>
       <c r="L2" t="n">
-        <v>11.21</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M2" t="n">
-        <v>11.51</v>
+        <v>9.81</v>
       </c>
       <c r="N2" t="n">
-        <v>49.4</v>
+        <v>47.26</v>
       </c>
       <c r="O2" t="n">
-        <v>49.49</v>
+        <v>47.54</v>
       </c>
       <c r="P2" t="n">
-        <v>48.3</v>
+        <v>45.52</v>
       </c>
       <c r="Q2" t="n">
-        <v>48.59</v>
+        <v>45.59</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>157.84</v>
+        <v>162.12</v>
       </c>
       <c r="C3" t="n">
-        <v>166</v>
+        <v>162.9</v>
       </c>
       <c r="D3" t="n">
-        <v>149.06</v>
+        <v>147.61</v>
       </c>
       <c r="E3" t="n">
-        <v>165.85</v>
+        <v>152.1</v>
       </c>
       <c r="F3" t="n">
-        <v>69.26000000000001</v>
+        <v>71.87</v>
       </c>
       <c r="G3" t="n">
-        <v>71.66</v>
+        <v>73.3</v>
       </c>
       <c r="H3" t="n">
-        <v>68.88</v>
+        <v>70.38</v>
       </c>
       <c r="I3" t="n">
-        <v>71.56999999999999</v>
+        <v>71.34</v>
       </c>
       <c r="J3" t="n">
-        <v>10.43</v>
+        <v>10.02</v>
       </c>
       <c r="K3" t="n">
-        <v>11.14</v>
+        <v>10.88</v>
       </c>
       <c r="L3" t="n">
-        <v>9.800000000000001</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="M3" t="n">
-        <v>9.81</v>
+        <v>10.6</v>
       </c>
       <c r="N3" t="n">
-        <v>47.26</v>
+        <v>45.41</v>
       </c>
       <c r="O3" t="n">
-        <v>47.54</v>
+        <v>46.36</v>
       </c>
       <c r="P3" t="n">
-        <v>45.52</v>
+        <v>44.5</v>
       </c>
       <c r="Q3" t="n">
-        <v>45.59</v>
+        <v>45.73</v>
       </c>
       <c r="R3" t="n">
-        <v>15.0458</v>
+        <v>-8.2906</v>
       </c>
       <c r="U3" t="n">
-        <v>6.2027</v>
+        <v>-0.3214</v>
       </c>
       <c r="X3" t="n">
-        <v>-14.7698</v>
+        <v>8.053000000000001</v>
       </c>
       <c r="AA3" t="n">
-        <v>-6.1741</v>
+        <v>0.3071</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>162.12</v>
+        <v>163</v>
       </c>
       <c r="C4" t="n">
-        <v>162.9</v>
+        <v>177.5</v>
       </c>
       <c r="D4" t="n">
-        <v>147.61</v>
+        <v>161.51</v>
       </c>
       <c r="E4" t="n">
-        <v>152.1</v>
+        <v>176.94</v>
       </c>
       <c r="F4" t="n">
-        <v>71.87</v>
+        <v>72.81999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>73.3</v>
+        <v>76.31</v>
       </c>
       <c r="H4" t="n">
-        <v>70.38</v>
+        <v>72.7</v>
       </c>
       <c r="I4" t="n">
-        <v>71.34</v>
+        <v>76.28</v>
       </c>
       <c r="J4" t="n">
-        <v>10.02</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="K4" t="n">
-        <v>10.88</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="L4" t="n">
-        <v>9.970000000000001</v>
+        <v>8.84</v>
       </c>
       <c r="M4" t="n">
-        <v>10.6</v>
+        <v>8.85</v>
       </c>
       <c r="N4" t="n">
-        <v>45.41</v>
+        <v>44.82</v>
       </c>
       <c r="O4" t="n">
-        <v>46.36</v>
+        <v>44.89</v>
       </c>
       <c r="P4" t="n">
-        <v>44.5</v>
+        <v>42.57</v>
       </c>
       <c r="Q4" t="n">
-        <v>45.73</v>
+        <v>42.57</v>
       </c>
       <c r="R4" t="n">
-        <v>-8.2906</v>
+        <v>16.3314</v>
       </c>
       <c r="U4" t="n">
-        <v>-0.3214</v>
+        <v>6.9246</v>
       </c>
       <c r="X4" t="n">
-        <v>8.053000000000001</v>
+        <v>-16.5094</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.3071</v>
+        <v>-6.9101</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="C5" t="n">
-        <v>177.5</v>
+        <v>191.29</v>
       </c>
       <c r="D5" t="n">
-        <v>161.51</v>
+        <v>178.94</v>
       </c>
       <c r="E5" t="n">
-        <v>176.94</v>
+        <v>190.42</v>
       </c>
       <c r="F5" t="n">
-        <v>72.81999999999999</v>
+        <v>76</v>
       </c>
       <c r="G5" t="n">
-        <v>76.31</v>
+        <v>77.36</v>
       </c>
       <c r="H5" t="n">
-        <v>72.7</v>
+        <v>75.55</v>
       </c>
       <c r="I5" t="n">
-        <v>76.28</v>
+        <v>76.95999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>9.859999999999999</v>
+        <v>8.65</v>
       </c>
       <c r="K5" t="n">
-        <v>9.970000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="L5" t="n">
-        <v>8.84</v>
+        <v>8.15</v>
       </c>
       <c r="M5" t="n">
-        <v>8.85</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="N5" t="n">
-        <v>44.82</v>
+        <v>42.74</v>
       </c>
       <c r="O5" t="n">
-        <v>44.89</v>
+        <v>43</v>
       </c>
       <c r="P5" t="n">
-        <v>42.57</v>
+        <v>41.99</v>
       </c>
       <c r="Q5" t="n">
-        <v>42.57</v>
+        <v>42.22</v>
       </c>
       <c r="R5" t="n">
-        <v>16.3314</v>
+        <v>7.6184</v>
       </c>
       <c r="S5" t="n">
-        <v>22.7386</v>
+        <v>14.8146</v>
       </c>
       <c r="U5" t="n">
-        <v>6.9246</v>
+        <v>0.8915</v>
       </c>
       <c r="V5" t="n">
-        <v>13.1919</v>
+        <v>7.5311</v>
       </c>
       <c r="X5" t="n">
-        <v>-16.5094</v>
+        <v>-7.3446</v>
       </c>
       <c r="Y5" t="n">
-        <v>-23.1103</v>
+        <v>-16.4118</v>
       </c>
       <c r="AA5" t="n">
-        <v>-6.9101</v>
+        <v>-0.8222</v>
       </c>
       <c r="AB5" t="n">
-        <v>-12.3894</v>
+        <v>-7.392</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>181</v>
+        <v>177.62</v>
       </c>
       <c r="C6" t="n">
-        <v>191.29</v>
+        <v>182.24</v>
       </c>
       <c r="D6" t="n">
-        <v>178.94</v>
+        <v>150.58</v>
       </c>
       <c r="E6" t="n">
-        <v>190.42</v>
+        <v>172.52</v>
       </c>
       <c r="F6" t="n">
-        <v>76</v>
+        <v>75.3</v>
       </c>
       <c r="G6" t="n">
-        <v>77.36</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>75.55</v>
+        <v>71.55</v>
       </c>
       <c r="I6" t="n">
-        <v>76.95999999999999</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>8.65</v>
+        <v>8.75</v>
       </c>
       <c r="K6" t="n">
-        <v>8.77</v>
+        <v>9.91</v>
       </c>
       <c r="L6" t="n">
-        <v>8.15</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="M6" t="n">
-        <v>8.199999999999999</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N6" t="n">
-        <v>42.74</v>
+        <v>43.14</v>
       </c>
       <c r="O6" t="n">
-        <v>43</v>
+        <v>45.19</v>
       </c>
       <c r="P6" t="n">
-        <v>41.99</v>
+        <v>42.79</v>
       </c>
       <c r="Q6" t="n">
-        <v>42.22</v>
+        <v>43.31</v>
       </c>
       <c r="R6" t="n">
-        <v>7.6184</v>
+        <v>-9.4003</v>
       </c>
       <c r="S6" t="n">
-        <v>14.8146</v>
+        <v>13.4254</v>
       </c>
       <c r="U6" t="n">
-        <v>0.8915</v>
+        <v>-2.5988</v>
       </c>
       <c r="V6" t="n">
-        <v>7.5311</v>
+        <v>5.0743</v>
       </c>
       <c r="X6" t="n">
-        <v>-7.3446</v>
+        <v>9.1463</v>
       </c>
       <c r="Y6" t="n">
-        <v>-16.4118</v>
+        <v>-15.566</v>
       </c>
       <c r="AA6" t="n">
-        <v>-0.8222</v>
+        <v>2.5817</v>
       </c>
       <c r="AB6" t="n">
-        <v>-7.392</v>
+        <v>-5.2919</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>177.62</v>
+        <v>183.84</v>
       </c>
       <c r="C7" t="n">
-        <v>182.24</v>
+        <v>188.49</v>
       </c>
       <c r="D7" t="n">
-        <v>150.58</v>
+        <v>172.26</v>
       </c>
       <c r="E7" t="n">
-        <v>172.52</v>
+        <v>184.24</v>
       </c>
       <c r="F7" t="n">
-        <v>75.3</v>
+        <v>75.81</v>
       </c>
       <c r="G7" t="n">
-        <v>75.93000000000001</v>
+        <v>77.94</v>
       </c>
       <c r="H7" t="n">
-        <v>71.55</v>
+        <v>74.19</v>
       </c>
       <c r="I7" t="n">
-        <v>74.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>8.75</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>9.91</v>
+        <v>8.98</v>
       </c>
       <c r="L7" t="n">
-        <v>8.550000000000001</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="M7" t="n">
-        <v>8.949999999999999</v>
+        <v>8.35</v>
       </c>
       <c r="N7" t="n">
-        <v>43.14</v>
+        <v>42.83</v>
       </c>
       <c r="O7" t="n">
-        <v>45.19</v>
+        <v>43.77</v>
       </c>
       <c r="P7" t="n">
-        <v>42.79</v>
+        <v>41.6</v>
       </c>
       <c r="Q7" t="n">
-        <v>43.31</v>
+        <v>41.99</v>
       </c>
       <c r="R7" t="n">
-        <v>-9.4003</v>
+        <v>6.7934</v>
       </c>
       <c r="S7" t="n">
-        <v>13.4254</v>
+        <v>4.1257</v>
       </c>
       <c r="T7" t="n">
-        <v>19.6726</v>
+        <v>11.0883</v>
       </c>
       <c r="U7" t="n">
-        <v>-2.5988</v>
+        <v>3.0416</v>
       </c>
       <c r="V7" t="n">
-        <v>5.0743</v>
+        <v>1.2585</v>
       </c>
       <c r="W7" t="n">
-        <v>11.2331</v>
+        <v>7.9223</v>
       </c>
       <c r="X7" t="n">
-        <v>9.1463</v>
+        <v>-6.7039</v>
       </c>
       <c r="Y7" t="n">
-        <v>-15.566</v>
+        <v>-5.6497</v>
       </c>
       <c r="Z7" t="n">
-        <v>-22.2415</v>
+        <v>-14.8828</v>
       </c>
       <c r="AA7" t="n">
-        <v>2.5817</v>
+        <v>-3.0478</v>
       </c>
       <c r="AB7" t="n">
-        <v>-5.2919</v>
+        <v>-1.3625</v>
       </c>
       <c r="AC7" t="n">
-        <v>-10.8664</v>
+        <v>-7.8965</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>183.84</v>
+        <v>182.67</v>
       </c>
       <c r="C8" t="n">
-        <v>188.49</v>
+        <v>189.56</v>
       </c>
       <c r="D8" t="n">
-        <v>172.26</v>
+        <v>178.28</v>
       </c>
       <c r="E8" t="n">
-        <v>184.24</v>
+        <v>186.19</v>
       </c>
       <c r="F8" t="n">
-        <v>75.81</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>77.94</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H8" t="n">
-        <v>74.19</v>
+        <v>77.16</v>
       </c>
       <c r="I8" t="n">
-        <v>77.23999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="J8" t="n">
-        <v>8.380000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="K8" t="n">
-        <v>8.98</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L8" t="n">
-        <v>8.140000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>8.35</v>
+        <v>8.27</v>
       </c>
       <c r="N8" t="n">
-        <v>42.83</v>
+        <v>41.98</v>
       </c>
       <c r="O8" t="n">
-        <v>43.77</v>
+        <v>42.06</v>
       </c>
       <c r="P8" t="n">
-        <v>41.6</v>
+        <v>40.68</v>
       </c>
       <c r="Q8" t="n">
-        <v>41.99</v>
+        <v>41.07</v>
       </c>
       <c r="R8" t="n">
-        <v>6.7934</v>
+        <v>1.0584</v>
       </c>
       <c r="S8" t="n">
-        <v>4.1257</v>
+        <v>-2.2214</v>
       </c>
       <c r="T8" t="n">
-        <v>11.0883</v>
+        <v>22.4129</v>
       </c>
       <c r="U8" t="n">
-        <v>3.0416</v>
+        <v>2.2139</v>
       </c>
       <c r="V8" t="n">
-        <v>1.2585</v>
+        <v>2.5858</v>
       </c>
       <c r="W8" t="n">
-        <v>7.9223</v>
+        <v>10.6672</v>
       </c>
       <c r="X8" t="n">
-        <v>-6.7039</v>
+        <v>-0.9581</v>
       </c>
       <c r="Y8" t="n">
-        <v>-5.6497</v>
+        <v>0.8537</v>
       </c>
       <c r="Z8" t="n">
-        <v>-14.8828</v>
+        <v>-21.9811</v>
       </c>
       <c r="AA8" t="n">
-        <v>-3.0478</v>
+        <v>-2.191</v>
       </c>
       <c r="AB8" t="n">
-        <v>-1.3625</v>
+        <v>-2.7238</v>
       </c>
       <c r="AC8" t="n">
-        <v>-7.8965</v>
+        <v>-10.1902</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>182.67</v>
+        <v>167</v>
       </c>
       <c r="C9" t="n">
-        <v>189.56</v>
+        <v>174.4</v>
       </c>
       <c r="D9" t="n">
-        <v>178.28</v>
+        <v>161.14</v>
       </c>
       <c r="E9" t="n">
-        <v>186.19</v>
+        <v>164.18</v>
       </c>
       <c r="F9" t="n">
-        <v>77.29000000000001</v>
+        <v>75.73</v>
       </c>
       <c r="G9" t="n">
-        <v>79.68000000000001</v>
+        <v>77.37</v>
       </c>
       <c r="H9" t="n">
-        <v>77.16</v>
+        <v>74.23</v>
       </c>
       <c r="I9" t="n">
-        <v>78.95</v>
+        <v>75.34</v>
       </c>
       <c r="J9" t="n">
-        <v>8.43</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>8.630000000000001</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="L9" t="n">
-        <v>8.119999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M9" t="n">
-        <v>8.27</v>
+        <v>9.23</v>
       </c>
       <c r="N9" t="n">
-        <v>41.98</v>
+        <v>42.77</v>
       </c>
       <c r="O9" t="n">
-        <v>42.06</v>
+        <v>43.57</v>
       </c>
       <c r="P9" t="n">
-        <v>40.68</v>
+        <v>41.93</v>
       </c>
       <c r="Q9" t="n">
-        <v>41.07</v>
+        <v>42.98</v>
       </c>
       <c r="R9" t="n">
-        <v>1.0584</v>
+        <v>-11.8213</v>
       </c>
       <c r="S9" t="n">
-        <v>-2.2214</v>
+        <v>-4.8342</v>
       </c>
       <c r="T9" t="n">
-        <v>22.4129</v>
+        <v>-7.2115</v>
       </c>
       <c r="U9" t="n">
-        <v>2.2139</v>
+        <v>-4.5725</v>
       </c>
       <c r="V9" t="n">
-        <v>2.5858</v>
+        <v>0.5069</v>
       </c>
       <c r="W9" t="n">
-        <v>10.6672</v>
+        <v>-1.2323</v>
       </c>
       <c r="X9" t="n">
-        <v>-0.9581</v>
+        <v>11.6082</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.8537</v>
+        <v>3.1285</v>
       </c>
       <c r="Z9" t="n">
-        <v>-21.9811</v>
+        <v>4.2938</v>
       </c>
       <c r="AA9" t="n">
-        <v>-2.191</v>
+        <v>4.6506</v>
       </c>
       <c r="AB9" t="n">
-        <v>-2.7238</v>
+        <v>-0.7619</v>
       </c>
       <c r="AC9" t="n">
-        <v>-10.1902</v>
+        <v>0.9631</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>167</v>
+        <v>172.95</v>
       </c>
       <c r="C10" t="n">
-        <v>174.4</v>
+        <v>174.61</v>
       </c>
       <c r="D10" t="n">
-        <v>161.14</v>
+        <v>142.69</v>
       </c>
       <c r="E10" t="n">
-        <v>164.18</v>
+        <v>151.75</v>
       </c>
       <c r="F10" t="n">
-        <v>75.73</v>
+        <v>76.13</v>
       </c>
       <c r="G10" t="n">
-        <v>77.37</v>
+        <v>76.27</v>
       </c>
       <c r="H10" t="n">
-        <v>74.23</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>75.34</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>9.130000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="K10" t="n">
-        <v>9.390000000000001</v>
+        <v>10.47</v>
       </c>
       <c r="L10" t="n">
-        <v>8.800000000000001</v>
+        <v>8.68</v>
       </c>
       <c r="M10" t="n">
-        <v>9.23</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="N10" t="n">
-        <v>42.77</v>
+        <v>42.51</v>
       </c>
       <c r="O10" t="n">
-        <v>43.57</v>
+        <v>44.82</v>
       </c>
       <c r="P10" t="n">
-        <v>41.93</v>
+        <v>42.44</v>
       </c>
       <c r="Q10" t="n">
-        <v>42.98</v>
+        <v>43.54</v>
       </c>
       <c r="R10" t="n">
-        <v>-11.8213</v>
+        <v>-7.571</v>
       </c>
       <c r="S10" t="n">
-        <v>-4.8342</v>
+        <v>-17.6346</v>
       </c>
       <c r="T10" t="n">
-        <v>-7.2115</v>
+        <v>-20.3077</v>
       </c>
       <c r="U10" t="n">
-        <v>-4.5725</v>
+        <v>-1.3539</v>
       </c>
       <c r="V10" t="n">
-        <v>0.5069</v>
+        <v>-3.7804</v>
       </c>
       <c r="W10" t="n">
-        <v>-1.2323</v>
+        <v>-3.4304</v>
       </c>
       <c r="X10" t="n">
-        <v>11.6082</v>
+        <v>7.8007</v>
       </c>
       <c r="Y10" t="n">
-        <v>3.1285</v>
+        <v>19.1617</v>
       </c>
       <c r="Z10" t="n">
-        <v>4.2938</v>
+        <v>21.3415</v>
       </c>
       <c r="AA10" t="n">
-        <v>4.6506</v>
+        <v>1.3029</v>
       </c>
       <c r="AB10" t="n">
-        <v>-0.7619</v>
+        <v>3.6914</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.9631</v>
+        <v>3.1265</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>172.95</v>
+        <v>141.24</v>
       </c>
       <c r="C11" t="n">
-        <v>174.61</v>
+        <v>160.6</v>
       </c>
       <c r="D11" t="n">
-        <v>142.69</v>
+        <v>135.02</v>
       </c>
       <c r="E11" t="n">
-        <v>151.75</v>
+        <v>151.89</v>
       </c>
       <c r="F11" t="n">
-        <v>76.13</v>
+        <v>72.41</v>
       </c>
       <c r="G11" t="n">
-        <v>76.27</v>
+        <v>74.5</v>
       </c>
       <c r="H11" t="n">
-        <v>72.09999999999999</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>74.31999999999999</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>8.77</v>
+        <v>10.64</v>
       </c>
       <c r="K11" t="n">
-        <v>10.47</v>
+        <v>11.07</v>
       </c>
       <c r="L11" t="n">
-        <v>8.68</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="M11" t="n">
-        <v>9.949999999999999</v>
+        <v>9.93</v>
       </c>
       <c r="N11" t="n">
-        <v>42.51</v>
+        <v>44.68</v>
       </c>
       <c r="O11" t="n">
-        <v>44.82</v>
+        <v>45.53</v>
       </c>
       <c r="P11" t="n">
-        <v>42.44</v>
+        <v>43.46</v>
       </c>
       <c r="Q11" t="n">
-        <v>43.54</v>
+        <v>44.37</v>
       </c>
       <c r="R11" t="n">
-        <v>-7.571</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="S11" t="n">
-        <v>-17.6346</v>
+        <v>-18.422</v>
       </c>
       <c r="T11" t="n">
-        <v>-20.3077</v>
+        <v>-11.958</v>
       </c>
       <c r="U11" t="n">
-        <v>-1.3539</v>
+        <v>-1.8703</v>
       </c>
       <c r="V11" t="n">
-        <v>-3.7804</v>
+        <v>-7.6251</v>
       </c>
       <c r="W11" t="n">
-        <v>-3.4304</v>
+        <v>-2.7081</v>
       </c>
       <c r="X11" t="n">
-        <v>7.8007</v>
+        <v>-0.201</v>
       </c>
       <c r="Y11" t="n">
-        <v>19.1617</v>
+        <v>20.0726</v>
       </c>
       <c r="Z11" t="n">
-        <v>21.3415</v>
+        <v>10.9497</v>
       </c>
       <c r="AA11" t="n">
-        <v>1.3029</v>
+        <v>1.9063</v>
       </c>
       <c r="AB11" t="n">
-        <v>3.6914</v>
+        <v>8.0351</v>
       </c>
       <c r="AC11" t="n">
-        <v>3.1265</v>
+        <v>2.4475</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>141.24</v>
+        <v>161</v>
       </c>
       <c r="C12" t="n">
-        <v>160.6</v>
+        <v>173.7</v>
       </c>
       <c r="D12" t="n">
-        <v>135.02</v>
+        <v>161</v>
       </c>
       <c r="E12" t="n">
-        <v>151.89</v>
+        <v>173.2</v>
       </c>
       <c r="F12" t="n">
-        <v>72.41</v>
+        <v>74.09</v>
       </c>
       <c r="G12" t="n">
-        <v>74.5</v>
+        <v>76.53</v>
       </c>
       <c r="H12" t="n">
-        <v>70.95999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="I12" t="n">
-        <v>72.93000000000001</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>10.64</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>11.07</v>
+        <v>9.35</v>
       </c>
       <c r="L12" t="n">
-        <v>9.369999999999999</v>
+        <v>8.51</v>
       </c>
       <c r="M12" t="n">
-        <v>9.93</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N12" t="n">
-        <v>44.68</v>
+        <v>43.67</v>
       </c>
       <c r="O12" t="n">
-        <v>45.53</v>
+        <v>43.97</v>
       </c>
       <c r="P12" t="n">
-        <v>43.46</v>
+        <v>42.19</v>
       </c>
       <c r="Q12" t="n">
-        <v>44.37</v>
+        <v>42.19</v>
       </c>
       <c r="R12" t="n">
-        <v>0.09229999999999999</v>
+        <v>14.0299</v>
       </c>
       <c r="S12" t="n">
-        <v>-18.422</v>
+        <v>5.494</v>
       </c>
       <c r="T12" t="n">
-        <v>-11.958</v>
+        <v>-5.9922</v>
       </c>
       <c r="U12" t="n">
-        <v>-1.8703</v>
+        <v>4.9088</v>
       </c>
       <c r="V12" t="n">
-        <v>-7.6251</v>
+        <v>1.553</v>
       </c>
       <c r="W12" t="n">
-        <v>-2.7081</v>
+        <v>-0.9451000000000001</v>
       </c>
       <c r="X12" t="n">
-        <v>-0.201</v>
+        <v>-13.998</v>
       </c>
       <c r="Y12" t="n">
-        <v>20.0726</v>
+        <v>-7.4756</v>
       </c>
       <c r="Z12" t="n">
-        <v>10.9497</v>
+        <v>2.2754</v>
       </c>
       <c r="AA12" t="n">
-        <v>1.9063</v>
+        <v>-4.9132</v>
       </c>
       <c r="AB12" t="n">
-        <v>8.0351</v>
+        <v>-1.8381</v>
       </c>
       <c r="AC12" t="n">
-        <v>2.4475</v>
+        <v>0.4763</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>161</v>
+        <v>171.26</v>
       </c>
       <c r="C13" t="n">
-        <v>173.7</v>
+        <v>179.97</v>
       </c>
       <c r="D13" t="n">
-        <v>161</v>
+        <v>168.23</v>
       </c>
       <c r="E13" t="n">
-        <v>173.2</v>
+        <v>178.39</v>
       </c>
       <c r="F13" t="n">
-        <v>74.09</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>76.53</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H13" t="n">
-        <v>73.62</v>
+        <v>74.47</v>
       </c>
       <c r="I13" t="n">
-        <v>76.51000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J13" t="n">
-        <v>9.300000000000001</v>
+        <v>8.65</v>
       </c>
       <c r="K13" t="n">
-        <v>9.35</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L13" t="n">
-        <v>8.51</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M13" t="n">
-        <v>8.539999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N13" t="n">
-        <v>43.67</v>
+        <v>42.94</v>
       </c>
       <c r="O13" t="n">
-        <v>43.97</v>
+        <v>43.33</v>
       </c>
       <c r="P13" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="Q13" t="n">
-        <v>42.19</v>
+        <v>41.96</v>
       </c>
       <c r="R13" t="n">
-        <v>14.0299</v>
+        <v>2.9965</v>
       </c>
       <c r="S13" t="n">
-        <v>5.494</v>
+        <v>17.5552</v>
       </c>
       <c r="T13" t="n">
-        <v>-5.9922</v>
+        <v>-4.1893</v>
       </c>
       <c r="U13" t="n">
-        <v>4.9088</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="V13" t="n">
-        <v>1.553</v>
+        <v>3.5388</v>
       </c>
       <c r="W13" t="n">
-        <v>-0.9451000000000001</v>
+        <v>-2.5332</v>
       </c>
       <c r="X13" t="n">
-        <v>-13.998</v>
+        <v>-2.9274</v>
       </c>
       <c r="Y13" t="n">
-        <v>-7.4756</v>
+        <v>-16.6834</v>
       </c>
       <c r="Z13" t="n">
-        <v>2.2754</v>
+        <v>0.2418</v>
       </c>
       <c r="AA13" t="n">
-        <v>-4.9132</v>
+        <v>-0.5452</v>
       </c>
       <c r="AB13" t="n">
-        <v>-1.8381</v>
+        <v>-3.6288</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.4763</v>
+        <v>2.167</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>171.26</v>
+        <v>184.8</v>
       </c>
       <c r="C14" t="n">
-        <v>179.97</v>
+        <v>195.27</v>
       </c>
       <c r="D14" t="n">
-        <v>168.23</v>
+        <v>183.34</v>
       </c>
       <c r="E14" t="n">
-        <v>178.39</v>
+        <v>190.56</v>
       </c>
       <c r="F14" t="n">
-        <v>75.18000000000001</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>77.79000000000001</v>
+        <v>79.33</v>
       </c>
       <c r="H14" t="n">
-        <v>74.47</v>
+        <v>77.33</v>
       </c>
       <c r="I14" t="n">
-        <v>76.95</v>
+        <v>77.84</v>
       </c>
       <c r="J14" t="n">
-        <v>8.65</v>
+        <v>8</v>
       </c>
       <c r="K14" t="n">
-        <v>8.779999999999999</v>
+        <v>8.06</v>
       </c>
       <c r="L14" t="n">
-        <v>8.210000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="M14" t="n">
-        <v>8.289999999999999</v>
+        <v>7.73</v>
       </c>
       <c r="N14" t="n">
-        <v>42.94</v>
+        <v>41.4</v>
       </c>
       <c r="O14" t="n">
-        <v>43.33</v>
+        <v>41.78</v>
       </c>
       <c r="P14" t="n">
+        <v>40.68</v>
+      </c>
+      <c r="Q14" t="n">
         <v>41.5</v>
       </c>
-      <c r="Q14" t="n">
-        <v>41.96</v>
-      </c>
       <c r="R14" t="n">
-        <v>2.9965</v>
+        <v>6.8221</v>
       </c>
       <c r="S14" t="n">
-        <v>17.5552</v>
+        <v>25.4592</v>
       </c>
       <c r="T14" t="n">
-        <v>-4.1893</v>
+        <v>16.0677</v>
       </c>
       <c r="U14" t="n">
-        <v>0.5750999999999999</v>
+        <v>1.1566</v>
       </c>
       <c r="V14" t="n">
-        <v>3.5388</v>
+        <v>6.7325</v>
       </c>
       <c r="W14" t="n">
-        <v>-2.5332</v>
+        <v>3.3183</v>
       </c>
       <c r="X14" t="n">
-        <v>-2.9274</v>
+        <v>-6.7551</v>
       </c>
       <c r="Y14" t="n">
-        <v>-16.6834</v>
+        <v>-22.1551</v>
       </c>
       <c r="Z14" t="n">
-        <v>0.2418</v>
+        <v>-16.2514</v>
       </c>
       <c r="AA14" t="n">
-        <v>-0.5452</v>
+        <v>-1.0963</v>
       </c>
       <c r="AB14" t="n">
-        <v>-3.6288</v>
+        <v>-6.4683</v>
       </c>
       <c r="AC14" t="n">
-        <v>2.167</v>
+        <v>-3.4435</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>184.8</v>
+        <v>211.38</v>
       </c>
       <c r="C15" t="n">
-        <v>195.27</v>
+        <v>228.5</v>
       </c>
       <c r="D15" t="n">
-        <v>183.34</v>
+        <v>209.89</v>
       </c>
       <c r="E15" t="n">
-        <v>190.56</v>
+        <v>225.79</v>
       </c>
       <c r="F15" t="n">
-        <v>78.04000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="G15" t="n">
-        <v>79.33</v>
+        <v>82.27</v>
       </c>
       <c r="H15" t="n">
-        <v>77.33</v>
+        <v>79.98</v>
       </c>
       <c r="I15" t="n">
-        <v>77.84</v>
+        <v>81.95</v>
       </c>
       <c r="J15" t="n">
-        <v>8</v>
+        <v>6.9</v>
       </c>
       <c r="K15" t="n">
-        <v>8.06</v>
+        <v>6.95</v>
       </c>
       <c r="L15" t="n">
-        <v>7.5</v>
+        <v>6.19</v>
       </c>
       <c r="M15" t="n">
-        <v>7.73</v>
+        <v>6.29</v>
       </c>
       <c r="N15" t="n">
-        <v>41.4</v>
+        <v>40.05</v>
       </c>
       <c r="O15" t="n">
-        <v>41.78</v>
+        <v>40.35</v>
       </c>
       <c r="P15" t="n">
-        <v>40.68</v>
+        <v>39.14</v>
       </c>
       <c r="Q15" t="n">
-        <v>41.5</v>
+        <v>39.28</v>
       </c>
       <c r="R15" t="n">
-        <v>6.8221</v>
+        <v>18.4876</v>
       </c>
       <c r="S15" t="n">
-        <v>25.4592</v>
+        <v>30.3637</v>
       </c>
       <c r="T15" t="n">
-        <v>16.0677</v>
+        <v>48.7908</v>
       </c>
       <c r="U15" t="n">
-        <v>1.1566</v>
+        <v>5.2801</v>
       </c>
       <c r="V15" t="n">
-        <v>6.7325</v>
+        <v>7.1102</v>
       </c>
       <c r="W15" t="n">
-        <v>3.3183</v>
+        <v>10.2664</v>
       </c>
       <c r="X15" t="n">
-        <v>-6.7551</v>
+        <v>-18.6287</v>
       </c>
       <c r="Y15" t="n">
-        <v>-22.1551</v>
+        <v>-26.3466</v>
       </c>
       <c r="Z15" t="n">
-        <v>-16.2514</v>
+        <v>-36.7839</v>
       </c>
       <c r="AA15" t="n">
-        <v>-1.0963</v>
+        <v>-5.3494</v>
       </c>
       <c r="AB15" t="n">
-        <v>-6.4683</v>
+        <v>-6.8974</v>
       </c>
       <c r="AC15" t="n">
-        <v>-3.4435</v>
+        <v>-9.7841</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>211.38</v>
+        <v>242.66</v>
       </c>
       <c r="C16" t="n">
-        <v>228.5</v>
+        <v>242.66</v>
       </c>
       <c r="D16" t="n">
-        <v>209.89</v>
+        <v>204</v>
       </c>
       <c r="E16" t="n">
-        <v>225.79</v>
+        <v>217.98</v>
       </c>
       <c r="F16" t="n">
-        <v>80.59</v>
+        <v>82.87</v>
       </c>
       <c r="G16" t="n">
-        <v>82.27</v>
+        <v>82.91</v>
       </c>
       <c r="H16" t="n">
-        <v>79.98</v>
+        <v>80.33</v>
       </c>
       <c r="I16" t="n">
-        <v>81.95</v>
+        <v>81.67</v>
       </c>
       <c r="J16" t="n">
-        <v>6.9</v>
+        <v>5.83</v>
       </c>
       <c r="K16" t="n">
-        <v>6.95</v>
+        <v>6.91</v>
       </c>
       <c r="L16" t="n">
-        <v>6.19</v>
+        <v>5.83</v>
       </c>
       <c r="M16" t="n">
-        <v>6.29</v>
+        <v>6.53</v>
       </c>
       <c r="N16" t="n">
-        <v>40.05</v>
+        <v>38.87</v>
       </c>
       <c r="O16" t="n">
-        <v>40.35</v>
+        <v>40.09</v>
       </c>
       <c r="P16" t="n">
-        <v>39.14</v>
+        <v>38.86</v>
       </c>
       <c r="Q16" t="n">
-        <v>39.28</v>
+        <v>39.44</v>
       </c>
       <c r="R16" t="n">
-        <v>18.4876</v>
+        <v>-3.459</v>
       </c>
       <c r="S16" t="n">
-        <v>30.3637</v>
+        <v>22.1929</v>
       </c>
       <c r="T16" t="n">
-        <v>48.7908</v>
+        <v>43.5118</v>
       </c>
       <c r="U16" t="n">
-        <v>5.2801</v>
+        <v>-0.3417</v>
       </c>
       <c r="V16" t="n">
-        <v>7.1102</v>
+        <v>6.1339</v>
       </c>
       <c r="W16" t="n">
-        <v>10.2664</v>
+        <v>11.9841</v>
       </c>
       <c r="X16" t="n">
-        <v>-18.6287</v>
+        <v>3.8156</v>
       </c>
       <c r="Y16" t="n">
-        <v>-26.3466</v>
+        <v>-21.2304</v>
       </c>
       <c r="Z16" t="n">
-        <v>-36.7839</v>
+        <v>-34.2397</v>
       </c>
       <c r="AA16" t="n">
-        <v>-5.3494</v>
+        <v>0.4073</v>
       </c>
       <c r="AB16" t="n">
-        <v>-6.8974</v>
+        <v>-6.0057</v>
       </c>
       <c r="AC16" t="n">
-        <v>-9.7841</v>
+        <v>-11.1111</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>242.66</v>
+        <v>219</v>
       </c>
       <c r="C17" t="n">
-        <v>242.66</v>
+        <v>231.89</v>
       </c>
       <c r="D17" t="n">
-        <v>204</v>
+        <v>207.56</v>
       </c>
       <c r="E17" t="n">
-        <v>217.98</v>
+        <v>224.63</v>
       </c>
       <c r="F17" t="n">
-        <v>82.87</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="G17" t="n">
-        <v>82.91</v>
+        <v>84.05</v>
       </c>
       <c r="H17" t="n">
-        <v>80.33</v>
+        <v>80.66</v>
       </c>
       <c r="I17" t="n">
-        <v>81.67</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="J17" t="n">
-        <v>5.83</v>
+        <v>6.49</v>
       </c>
       <c r="K17" t="n">
-        <v>6.91</v>
+        <v>6.83</v>
       </c>
       <c r="L17" t="n">
-        <v>5.83</v>
+        <v>6.1</v>
       </c>
       <c r="M17" t="n">
-        <v>6.53</v>
+        <v>6.31</v>
       </c>
       <c r="N17" t="n">
-        <v>38.87</v>
+        <v>39.41</v>
       </c>
       <c r="O17" t="n">
-        <v>40.09</v>
+        <v>39.94</v>
       </c>
       <c r="P17" t="n">
-        <v>38.86</v>
+        <v>38.3</v>
       </c>
       <c r="Q17" t="n">
-        <v>39.44</v>
+        <v>38.47</v>
       </c>
       <c r="R17" t="n">
-        <v>-3.459</v>
+        <v>3.0507</v>
       </c>
       <c r="S17" t="n">
-        <v>22.1929</v>
+        <v>17.8789</v>
       </c>
       <c r="T17" t="n">
-        <v>43.5118</v>
+        <v>29.694</v>
       </c>
       <c r="U17" t="n">
-        <v>-0.3417</v>
+        <v>2.4611</v>
       </c>
       <c r="V17" t="n">
-        <v>6.1339</v>
+        <v>7.5026</v>
       </c>
       <c r="W17" t="n">
-        <v>11.9841</v>
+        <v>9.3713</v>
       </c>
       <c r="X17" t="n">
-        <v>3.8156</v>
+        <v>-3.3691</v>
       </c>
       <c r="Y17" t="n">
-        <v>-21.2304</v>
+        <v>-18.37</v>
       </c>
       <c r="Z17" t="n">
-        <v>-34.2397</v>
+        <v>-26.1124</v>
       </c>
       <c r="AA17" t="n">
-        <v>0.4073</v>
+        <v>-2.4594</v>
       </c>
       <c r="AB17" t="n">
-        <v>-6.0057</v>
+        <v>-7.3012</v>
       </c>
       <c r="AC17" t="n">
-        <v>-11.1111</v>
+        <v>-8.817299999999999</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>219</v>
+        <v>231.82</v>
       </c>
       <c r="C18" t="n">
-        <v>231.89</v>
+        <v>239.07</v>
       </c>
       <c r="D18" t="n">
-        <v>207.56</v>
+        <v>218.56</v>
       </c>
       <c r="E18" t="n">
-        <v>224.63</v>
+        <v>224.34</v>
       </c>
       <c r="F18" t="n">
-        <v>81.73999999999999</v>
+        <v>84.41</v>
       </c>
       <c r="G18" t="n">
-        <v>84.05</v>
+        <v>85.7</v>
       </c>
       <c r="H18" t="n">
-        <v>80.66</v>
+        <v>83.53</v>
       </c>
       <c r="I18" t="n">
-        <v>83.68000000000001</v>
+        <v>84.56</v>
       </c>
       <c r="J18" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="K18" t="n">
         <v>6.49</v>
       </c>
-      <c r="K18" t="n">
-        <v>6.83</v>
-      </c>
       <c r="L18" t="n">
-        <v>6.1</v>
+        <v>5.91</v>
       </c>
       <c r="M18" t="n">
-        <v>6.31</v>
+        <v>6.33</v>
       </c>
       <c r="N18" t="n">
-        <v>39.41</v>
+        <v>38.15</v>
       </c>
       <c r="O18" t="n">
-        <v>39.94</v>
+        <v>38.56</v>
       </c>
       <c r="P18" t="n">
-        <v>38.3</v>
+        <v>37.56</v>
       </c>
       <c r="Q18" t="n">
-        <v>38.47</v>
+        <v>38.08</v>
       </c>
       <c r="R18" t="n">
-        <v>3.0507</v>
+        <v>-0.1291</v>
       </c>
       <c r="S18" t="n">
-        <v>17.8789</v>
+        <v>-0.6422</v>
       </c>
       <c r="T18" t="n">
-        <v>29.694</v>
+        <v>25.7582</v>
       </c>
       <c r="U18" t="n">
-        <v>2.4611</v>
+        <v>1.0516</v>
       </c>
       <c r="V18" t="n">
-        <v>7.5026</v>
+        <v>3.1849</v>
       </c>
       <c r="W18" t="n">
-        <v>9.3713</v>
+        <v>9.8895</v>
       </c>
       <c r="X18" t="n">
-        <v>-3.3691</v>
+        <v>0.317</v>
       </c>
       <c r="Y18" t="n">
-        <v>-18.37</v>
+        <v>0.6359</v>
       </c>
       <c r="Z18" t="n">
-        <v>-26.1124</v>
+        <v>-23.6429</v>
       </c>
       <c r="AA18" t="n">
-        <v>-2.4594</v>
+        <v>-1.0138</v>
       </c>
       <c r="AB18" t="n">
-        <v>-7.3012</v>
+        <v>-3.055</v>
       </c>
       <c r="AC18" t="n">
-        <v>-8.817299999999999</v>
+        <v>-9.2469</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>231.82</v>
+        <v>217.27</v>
       </c>
       <c r="C19" t="n">
-        <v>239.07</v>
+        <v>234.06</v>
       </c>
       <c r="D19" t="n">
-        <v>218.56</v>
+        <v>210.14</v>
       </c>
       <c r="E19" t="n">
-        <v>224.34</v>
+        <v>227.03</v>
       </c>
       <c r="F19" t="n">
-        <v>84.41</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>85.7</v>
+        <v>87.06</v>
       </c>
       <c r="H19" t="n">
-        <v>83.53</v>
+        <v>83.75</v>
       </c>
       <c r="I19" t="n">
-        <v>84.56</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="J19" t="n">
-        <v>6.11</v>
+        <v>6.55</v>
       </c>
       <c r="K19" t="n">
-        <v>6.49</v>
+        <v>6.74</v>
       </c>
       <c r="L19" t="n">
-        <v>5.91</v>
+        <v>6.05</v>
       </c>
       <c r="M19" t="n">
-        <v>6.33</v>
+        <v>6.26</v>
       </c>
       <c r="N19" t="n">
-        <v>38.15</v>
+        <v>38.27</v>
       </c>
       <c r="O19" t="n">
-        <v>38.56</v>
+        <v>38.46</v>
       </c>
       <c r="P19" t="n">
-        <v>37.56</v>
+        <v>36.96</v>
       </c>
       <c r="Q19" t="n">
-        <v>38.08</v>
+        <v>37.42</v>
       </c>
       <c r="R19" t="n">
-        <v>-0.1291</v>
+        <v>1.1991</v>
       </c>
       <c r="S19" t="n">
-        <v>-0.6422</v>
+        <v>4.1518</v>
       </c>
       <c r="T19" t="n">
-        <v>25.7582</v>
+        <v>19.1383</v>
       </c>
       <c r="U19" t="n">
-        <v>1.0516</v>
+        <v>1.7502</v>
       </c>
       <c r="V19" t="n">
-        <v>3.1849</v>
+        <v>5.3508</v>
       </c>
       <c r="W19" t="n">
-        <v>9.8895</v>
+        <v>10.5344</v>
       </c>
       <c r="X19" t="n">
-        <v>0.317</v>
+        <v>-1.1058</v>
       </c>
       <c r="Y19" t="n">
-        <v>0.6359</v>
+        <v>-4.1348</v>
       </c>
       <c r="Z19" t="n">
-        <v>-23.6429</v>
+        <v>-19.0168</v>
       </c>
       <c r="AA19" t="n">
-        <v>-1.0138</v>
+        <v>-1.7332</v>
       </c>
       <c r="AB19" t="n">
-        <v>-3.055</v>
+        <v>-5.1217</v>
       </c>
       <c r="AC19" t="n">
-        <v>-9.2469</v>
+        <v>-9.831300000000001</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>217.27</v>
+        <v>243.18</v>
       </c>
       <c r="C20" t="n">
-        <v>234.06</v>
+        <v>267.08</v>
       </c>
       <c r="D20" t="n">
-        <v>210.14</v>
+        <v>238.82</v>
       </c>
       <c r="E20" t="n">
-        <v>227.03</v>
+        <v>266.32</v>
       </c>
       <c r="F20" t="n">
-        <v>84.15000000000001</v>
+        <v>85.94</v>
       </c>
       <c r="G20" t="n">
-        <v>87.06</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="H20" t="n">
-        <v>83.75</v>
+        <v>84.83</v>
       </c>
       <c r="I20" t="n">
-        <v>86.04000000000001</v>
+        <v>87.22</v>
       </c>
       <c r="J20" t="n">
-        <v>6.55</v>
+        <v>5.8</v>
       </c>
       <c r="K20" t="n">
-        <v>6.74</v>
+        <v>5.93</v>
       </c>
       <c r="L20" t="n">
-        <v>6.05</v>
+        <v>5.15</v>
       </c>
       <c r="M20" t="n">
-        <v>6.26</v>
+        <v>5.17</v>
       </c>
       <c r="N20" t="n">
-        <v>38.27</v>
+        <v>37.47</v>
       </c>
       <c r="O20" t="n">
-        <v>38.46</v>
+        <v>37.95</v>
       </c>
       <c r="P20" t="n">
-        <v>36.96</v>
+        <v>36.86</v>
       </c>
       <c r="Q20" t="n">
-        <v>37.42</v>
+        <v>36.91</v>
       </c>
       <c r="R20" t="n">
-        <v>1.1991</v>
+        <v>17.3061</v>
       </c>
       <c r="S20" t="n">
-        <v>4.1518</v>
+        <v>18.5594</v>
       </c>
       <c r="T20" t="n">
-        <v>19.1383</v>
+        <v>17.9503</v>
       </c>
       <c r="U20" t="n">
-        <v>1.7502</v>
+        <v>1.3715</v>
       </c>
       <c r="V20" t="n">
-        <v>5.3508</v>
+        <v>4.2304</v>
       </c>
       <c r="W20" t="n">
-        <v>10.5344</v>
+        <v>6.4308</v>
       </c>
       <c r="X20" t="n">
-        <v>-1.1058</v>
+        <v>-17.4121</v>
       </c>
       <c r="Y20" t="n">
-        <v>-4.1348</v>
+        <v>-18.0666</v>
       </c>
       <c r="Z20" t="n">
-        <v>-19.0168</v>
+        <v>-17.806</v>
       </c>
       <c r="AA20" t="n">
-        <v>-1.7332</v>
+        <v>-1.3629</v>
       </c>
       <c r="AB20" t="n">
-        <v>-5.1217</v>
+        <v>-4.0551</v>
       </c>
       <c r="AC20" t="n">
-        <v>-9.831300000000001</v>
+        <v>-6.0336</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>243.18</v>
+        <v>281.47</v>
       </c>
       <c r="C21" t="n">
-        <v>267.08</v>
+        <v>284.58</v>
       </c>
       <c r="D21" t="n">
-        <v>238.82</v>
+        <v>257.26</v>
       </c>
       <c r="E21" t="n">
-        <v>266.32</v>
+        <v>280.54</v>
       </c>
       <c r="F21" t="n">
-        <v>85.94</v>
+        <v>87.68000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>87.31999999999999</v>
+        <v>88.09</v>
       </c>
       <c r="H21" t="n">
-        <v>84.83</v>
+        <v>85.41</v>
       </c>
       <c r="I21" t="n">
-        <v>87.22</v>
+        <v>86.56</v>
       </c>
       <c r="J21" t="n">
-        <v>5.8</v>
+        <v>4.88</v>
       </c>
       <c r="K21" t="n">
-        <v>5.93</v>
+        <v>5.35</v>
       </c>
       <c r="L21" t="n">
-        <v>5.15</v>
+        <v>4.82</v>
       </c>
       <c r="M21" t="n">
-        <v>5.17</v>
+        <v>4.91</v>
       </c>
       <c r="N21" t="n">
-        <v>37.47</v>
+        <v>36.73</v>
       </c>
       <c r="O21" t="n">
-        <v>37.95</v>
+        <v>37.69</v>
       </c>
       <c r="P21" t="n">
-        <v>36.86</v>
+        <v>36.55</v>
       </c>
       <c r="Q21" t="n">
-        <v>36.91</v>
+        <v>37.19</v>
       </c>
       <c r="R21" t="n">
-        <v>17.3061</v>
+        <v>5.3394</v>
       </c>
       <c r="S21" t="n">
-        <v>18.5594</v>
+        <v>25.0513</v>
       </c>
       <c r="T21" t="n">
-        <v>17.9503</v>
+        <v>28.6999</v>
       </c>
       <c r="U21" t="n">
-        <v>1.3715</v>
+        <v>-0.7567</v>
       </c>
       <c r="V21" t="n">
-        <v>4.2304</v>
+        <v>2.3652</v>
       </c>
       <c r="W21" t="n">
-        <v>6.4308</v>
+        <v>5.9875</v>
       </c>
       <c r="X21" t="n">
-        <v>-17.4121</v>
+        <v>-5.029</v>
       </c>
       <c r="Y21" t="n">
-        <v>-18.0666</v>
+        <v>-22.4329</v>
       </c>
       <c r="Z21" t="n">
-        <v>-17.806</v>
+        <v>-24.8086</v>
       </c>
       <c r="AA21" t="n">
-        <v>-1.3629</v>
+        <v>0.7586000000000001</v>
       </c>
       <c r="AB21" t="n">
-        <v>-4.0551</v>
+        <v>-2.3372</v>
       </c>
       <c r="AC21" t="n">
-        <v>-6.0336</v>
+        <v>-5.7049</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>281.47</v>
+        <v>242.04</v>
       </c>
       <c r="C22" t="n">
-        <v>284.58</v>
+        <v>274.5</v>
       </c>
       <c r="D22" t="n">
-        <v>257.2601</v>
+        <v>228.55</v>
       </c>
       <c r="E22" t="n">
-        <v>280.54</v>
+        <v>262.7</v>
       </c>
       <c r="F22" t="n">
-        <v>87.675</v>
+        <v>83.47</v>
       </c>
       <c r="G22" t="n">
-        <v>88.09</v>
+        <v>86.245</v>
       </c>
       <c r="H22" t="n">
-        <v>85.41</v>
+        <v>82.47499999999999</v>
       </c>
       <c r="I22" t="n">
-        <v>86.56</v>
+        <v>85.22</v>
       </c>
       <c r="J22" t="n">
-        <v>4.88</v>
+        <v>5.57</v>
       </c>
       <c r="K22" t="n">
-        <v>5.35</v>
+        <v>5.81</v>
       </c>
       <c r="L22" t="n">
-        <v>4.82</v>
+        <v>5</v>
       </c>
       <c r="M22" t="n">
-        <v>4.91</v>
+        <v>5.2</v>
       </c>
       <c r="N22" t="n">
-        <v>36.73</v>
+        <v>38.53</v>
       </c>
       <c r="O22" t="n">
-        <v>37.6869</v>
+        <v>38.96</v>
       </c>
       <c r="P22" t="n">
-        <v>36.55</v>
+        <v>37.33</v>
       </c>
       <c r="Q22" t="n">
-        <v>37.19</v>
+        <v>37.76</v>
       </c>
       <c r="R22" t="n">
-        <v>5.3394</v>
+        <v>-6.3592</v>
       </c>
       <c r="S22" t="n">
-        <v>25.0513</v>
+        <v>15.7116</v>
       </c>
       <c r="T22" t="n">
-        <v>28.6999</v>
+        <v>16.9479</v>
       </c>
       <c r="U22" t="n">
-        <v>-0.7567</v>
+        <v>-1.5481</v>
       </c>
       <c r="V22" t="n">
-        <v>2.3652</v>
+        <v>-0.953</v>
       </c>
       <c r="W22" t="n">
-        <v>5.9875</v>
+        <v>1.8403</v>
       </c>
       <c r="X22" t="n">
-        <v>-5.029</v>
+        <v>5.9063</v>
       </c>
       <c r="Y22" t="n">
-        <v>-22.4329</v>
+        <v>-16.9329</v>
       </c>
       <c r="Z22" t="n">
-        <v>-24.8086</v>
+        <v>-17.5911</v>
       </c>
       <c r="AA22" t="n">
-        <v>0.7586000000000001</v>
+        <v>1.5327</v>
       </c>
       <c r="AB22" t="n">
-        <v>-2.3372</v>
+        <v>0.9086</v>
       </c>
       <c r="AC22" t="n">
-        <v>-5.7049</v>
+        <v>-1.8456</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-05 23:09
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>157.84</v>
+        <v>162.12</v>
       </c>
       <c r="C2" t="n">
-        <v>166</v>
+        <v>162.9</v>
       </c>
       <c r="D2" t="n">
-        <v>149.06</v>
+        <v>147.61</v>
       </c>
       <c r="E2" t="n">
-        <v>165.85</v>
+        <v>152.1</v>
       </c>
       <c r="F2" t="n">
-        <v>69.26000000000001</v>
+        <v>71.87</v>
       </c>
       <c r="G2" t="n">
-        <v>71.66</v>
+        <v>73.3</v>
       </c>
       <c r="H2" t="n">
-        <v>68.88</v>
+        <v>70.38</v>
       </c>
       <c r="I2" t="n">
-        <v>71.56999999999999</v>
+        <v>71.34</v>
       </c>
       <c r="J2" t="n">
-        <v>10.43</v>
+        <v>10.02</v>
       </c>
       <c r="K2" t="n">
-        <v>11.14</v>
+        <v>10.88</v>
       </c>
       <c r="L2" t="n">
-        <v>9.800000000000001</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="M2" t="n">
-        <v>9.81</v>
+        <v>10.6</v>
       </c>
       <c r="N2" t="n">
-        <v>47.26</v>
+        <v>45.41</v>
       </c>
       <c r="O2" t="n">
-        <v>47.54</v>
+        <v>46.36</v>
       </c>
       <c r="P2" t="n">
-        <v>45.52</v>
+        <v>44.5</v>
       </c>
       <c r="Q2" t="n">
-        <v>45.59</v>
+        <v>45.73</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>162.12</v>
+        <v>163</v>
       </c>
       <c r="C3" t="n">
-        <v>162.9</v>
+        <v>177.5</v>
       </c>
       <c r="D3" t="n">
-        <v>147.61</v>
+        <v>161.51</v>
       </c>
       <c r="E3" t="n">
-        <v>152.1</v>
+        <v>176.94</v>
       </c>
       <c r="F3" t="n">
-        <v>71.87</v>
+        <v>72.81999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>73.3</v>
+        <v>76.31</v>
       </c>
       <c r="H3" t="n">
-        <v>70.38</v>
+        <v>72.7</v>
       </c>
       <c r="I3" t="n">
-        <v>71.34</v>
+        <v>76.28</v>
       </c>
       <c r="J3" t="n">
-        <v>10.02</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="K3" t="n">
-        <v>10.88</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="L3" t="n">
-        <v>9.970000000000001</v>
+        <v>8.84</v>
       </c>
       <c r="M3" t="n">
-        <v>10.6</v>
+        <v>8.85</v>
       </c>
       <c r="N3" t="n">
-        <v>45.41</v>
+        <v>44.82</v>
       </c>
       <c r="O3" t="n">
-        <v>46.36</v>
+        <v>44.89</v>
       </c>
       <c r="P3" t="n">
-        <v>44.5</v>
+        <v>42.57</v>
       </c>
       <c r="Q3" t="n">
-        <v>45.73</v>
+        <v>42.57</v>
       </c>
       <c r="R3" t="n">
-        <v>-8.2906</v>
+        <v>16.3314</v>
       </c>
       <c r="U3" t="n">
-        <v>-0.3214</v>
+        <v>6.9246</v>
       </c>
       <c r="X3" t="n">
-        <v>8.053000000000001</v>
+        <v>-16.5094</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.3071</v>
+        <v>-6.9101</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="C4" t="n">
-        <v>177.5</v>
+        <v>191.29</v>
       </c>
       <c r="D4" t="n">
-        <v>161.51</v>
+        <v>178.94</v>
       </c>
       <c r="E4" t="n">
-        <v>176.94</v>
+        <v>190.42</v>
       </c>
       <c r="F4" t="n">
-        <v>72.81999999999999</v>
+        <v>76</v>
       </c>
       <c r="G4" t="n">
-        <v>76.31</v>
+        <v>77.36</v>
       </c>
       <c r="H4" t="n">
-        <v>72.7</v>
+        <v>75.55</v>
       </c>
       <c r="I4" t="n">
-        <v>76.28</v>
+        <v>76.95999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>9.859999999999999</v>
+        <v>8.65</v>
       </c>
       <c r="K4" t="n">
-        <v>9.970000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="L4" t="n">
-        <v>8.84</v>
+        <v>8.15</v>
       </c>
       <c r="M4" t="n">
-        <v>8.85</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="N4" t="n">
-        <v>44.82</v>
+        <v>42.74</v>
       </c>
       <c r="O4" t="n">
-        <v>44.89</v>
+        <v>43</v>
       </c>
       <c r="P4" t="n">
-        <v>42.57</v>
+        <v>41.99</v>
       </c>
       <c r="Q4" t="n">
-        <v>42.57</v>
+        <v>42.22</v>
       </c>
       <c r="R4" t="n">
-        <v>16.3314</v>
+        <v>7.6184</v>
       </c>
       <c r="U4" t="n">
-        <v>6.9246</v>
+        <v>0.8915</v>
       </c>
       <c r="X4" t="n">
-        <v>-16.5094</v>
+        <v>-7.3446</v>
       </c>
       <c r="AA4" t="n">
-        <v>-6.9101</v>
+        <v>-0.8222</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>181</v>
+        <v>177.62</v>
       </c>
       <c r="C5" t="n">
-        <v>191.29</v>
+        <v>182.24</v>
       </c>
       <c r="D5" t="n">
-        <v>178.94</v>
+        <v>150.58</v>
       </c>
       <c r="E5" t="n">
-        <v>190.42</v>
+        <v>172.52</v>
       </c>
       <c r="F5" t="n">
-        <v>76</v>
+        <v>75.3</v>
       </c>
       <c r="G5" t="n">
-        <v>77.36</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>75.55</v>
+        <v>71.55</v>
       </c>
       <c r="I5" t="n">
-        <v>76.95999999999999</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>8.65</v>
+        <v>8.75</v>
       </c>
       <c r="K5" t="n">
-        <v>8.77</v>
+        <v>9.91</v>
       </c>
       <c r="L5" t="n">
-        <v>8.15</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>8.199999999999999</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N5" t="n">
-        <v>42.74</v>
+        <v>43.14</v>
       </c>
       <c r="O5" t="n">
-        <v>43</v>
+        <v>45.19</v>
       </c>
       <c r="P5" t="n">
-        <v>41.99</v>
+        <v>42.79</v>
       </c>
       <c r="Q5" t="n">
-        <v>42.22</v>
+        <v>43.31</v>
       </c>
       <c r="R5" t="n">
-        <v>7.6184</v>
+        <v>-9.4003</v>
       </c>
       <c r="S5" t="n">
-        <v>14.8146</v>
+        <v>13.4254</v>
       </c>
       <c r="U5" t="n">
-        <v>0.8915</v>
+        <v>-2.5988</v>
       </c>
       <c r="V5" t="n">
-        <v>7.5311</v>
+        <v>5.0743</v>
       </c>
       <c r="X5" t="n">
-        <v>-7.3446</v>
+        <v>9.1463</v>
       </c>
       <c r="Y5" t="n">
-        <v>-16.4118</v>
+        <v>-15.566</v>
       </c>
       <c r="AA5" t="n">
-        <v>-0.8222</v>
+        <v>2.5817</v>
       </c>
       <c r="AB5" t="n">
-        <v>-7.392</v>
+        <v>-5.2919</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>177.62</v>
+        <v>183.84</v>
       </c>
       <c r="C6" t="n">
-        <v>182.24</v>
+        <v>188.49</v>
       </c>
       <c r="D6" t="n">
-        <v>150.58</v>
+        <v>172.26</v>
       </c>
       <c r="E6" t="n">
-        <v>172.52</v>
+        <v>184.24</v>
       </c>
       <c r="F6" t="n">
-        <v>75.3</v>
+        <v>75.81</v>
       </c>
       <c r="G6" t="n">
-        <v>75.93000000000001</v>
+        <v>77.94</v>
       </c>
       <c r="H6" t="n">
-        <v>71.55</v>
+        <v>74.19</v>
       </c>
       <c r="I6" t="n">
-        <v>74.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>8.75</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>9.91</v>
+        <v>8.98</v>
       </c>
       <c r="L6" t="n">
-        <v>8.550000000000001</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="M6" t="n">
-        <v>8.949999999999999</v>
+        <v>8.35</v>
       </c>
       <c r="N6" t="n">
-        <v>43.14</v>
+        <v>42.83</v>
       </c>
       <c r="O6" t="n">
-        <v>45.19</v>
+        <v>43.77</v>
       </c>
       <c r="P6" t="n">
-        <v>42.79</v>
+        <v>41.6</v>
       </c>
       <c r="Q6" t="n">
-        <v>43.31</v>
+        <v>41.99</v>
       </c>
       <c r="R6" t="n">
-        <v>-9.4003</v>
+        <v>6.7934</v>
       </c>
       <c r="S6" t="n">
-        <v>13.4254</v>
+        <v>4.1257</v>
       </c>
       <c r="U6" t="n">
-        <v>-2.5988</v>
+        <v>3.0416</v>
       </c>
       <c r="V6" t="n">
-        <v>5.0743</v>
+        <v>1.2585</v>
       </c>
       <c r="X6" t="n">
-        <v>9.1463</v>
+        <v>-6.7039</v>
       </c>
       <c r="Y6" t="n">
-        <v>-15.566</v>
+        <v>-5.6497</v>
       </c>
       <c r="AA6" t="n">
-        <v>2.5817</v>
+        <v>-3.0478</v>
       </c>
       <c r="AB6" t="n">
-        <v>-5.2919</v>
+        <v>-1.3625</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>183.84</v>
+        <v>182.67</v>
       </c>
       <c r="C7" t="n">
-        <v>188.49</v>
+        <v>189.56</v>
       </c>
       <c r="D7" t="n">
-        <v>172.26</v>
+        <v>178.28</v>
       </c>
       <c r="E7" t="n">
-        <v>184.24</v>
+        <v>186.19</v>
       </c>
       <c r="F7" t="n">
-        <v>75.81</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>77.94</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>74.19</v>
+        <v>77.16</v>
       </c>
       <c r="I7" t="n">
-        <v>77.23999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="J7" t="n">
-        <v>8.380000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="K7" t="n">
-        <v>8.98</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L7" t="n">
-        <v>8.140000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M7" t="n">
-        <v>8.35</v>
+        <v>8.27</v>
       </c>
       <c r="N7" t="n">
-        <v>42.83</v>
+        <v>41.98</v>
       </c>
       <c r="O7" t="n">
-        <v>43.77</v>
+        <v>42.06</v>
       </c>
       <c r="P7" t="n">
-        <v>41.6</v>
+        <v>40.68</v>
       </c>
       <c r="Q7" t="n">
-        <v>41.99</v>
+        <v>41.07</v>
       </c>
       <c r="R7" t="n">
-        <v>6.7934</v>
+        <v>1.0584</v>
       </c>
       <c r="S7" t="n">
-        <v>4.1257</v>
+        <v>-2.2214</v>
       </c>
       <c r="T7" t="n">
-        <v>11.0883</v>
+        <v>22.4129</v>
       </c>
       <c r="U7" t="n">
-        <v>3.0416</v>
+        <v>2.2139</v>
       </c>
       <c r="V7" t="n">
-        <v>1.2585</v>
+        <v>2.5858</v>
       </c>
       <c r="W7" t="n">
-        <v>7.9223</v>
+        <v>10.6672</v>
       </c>
       <c r="X7" t="n">
-        <v>-6.7039</v>
+        <v>-0.9581</v>
       </c>
       <c r="Y7" t="n">
-        <v>-5.6497</v>
+        <v>0.8537</v>
       </c>
       <c r="Z7" t="n">
-        <v>-14.8828</v>
+        <v>-21.9811</v>
       </c>
       <c r="AA7" t="n">
-        <v>-3.0478</v>
+        <v>-2.191</v>
       </c>
       <c r="AB7" t="n">
-        <v>-1.3625</v>
+        <v>-2.7238</v>
       </c>
       <c r="AC7" t="n">
-        <v>-7.8965</v>
+        <v>-10.1902</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>182.67</v>
+        <v>167</v>
       </c>
       <c r="C8" t="n">
-        <v>189.56</v>
+        <v>174.4</v>
       </c>
       <c r="D8" t="n">
-        <v>178.28</v>
+        <v>161.14</v>
       </c>
       <c r="E8" t="n">
-        <v>186.19</v>
+        <v>164.18</v>
       </c>
       <c r="F8" t="n">
-        <v>77.29000000000001</v>
+        <v>75.73</v>
       </c>
       <c r="G8" t="n">
-        <v>79.68000000000001</v>
+        <v>77.37</v>
       </c>
       <c r="H8" t="n">
-        <v>77.16</v>
+        <v>74.23</v>
       </c>
       <c r="I8" t="n">
-        <v>78.95</v>
+        <v>75.34</v>
       </c>
       <c r="J8" t="n">
-        <v>8.43</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>8.630000000000001</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="L8" t="n">
-        <v>8.119999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>8.27</v>
+        <v>9.23</v>
       </c>
       <c r="N8" t="n">
-        <v>41.98</v>
+        <v>42.77</v>
       </c>
       <c r="O8" t="n">
-        <v>42.06</v>
+        <v>43.57</v>
       </c>
       <c r="P8" t="n">
-        <v>40.68</v>
+        <v>41.93</v>
       </c>
       <c r="Q8" t="n">
-        <v>41.07</v>
+        <v>42.98</v>
       </c>
       <c r="R8" t="n">
-        <v>1.0584</v>
+        <v>-11.8213</v>
       </c>
       <c r="S8" t="n">
-        <v>-2.2214</v>
+        <v>-4.8342</v>
       </c>
       <c r="T8" t="n">
-        <v>22.4129</v>
+        <v>-7.2115</v>
       </c>
       <c r="U8" t="n">
-        <v>2.2139</v>
+        <v>-4.5725</v>
       </c>
       <c r="V8" t="n">
-        <v>2.5858</v>
+        <v>0.5069</v>
       </c>
       <c r="W8" t="n">
-        <v>10.6672</v>
+        <v>-1.2323</v>
       </c>
       <c r="X8" t="n">
-        <v>-0.9581</v>
+        <v>11.6082</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.8537</v>
+        <v>3.1285</v>
       </c>
       <c r="Z8" t="n">
-        <v>-21.9811</v>
+        <v>4.2938</v>
       </c>
       <c r="AA8" t="n">
-        <v>-2.191</v>
+        <v>4.6506</v>
       </c>
       <c r="AB8" t="n">
-        <v>-2.7238</v>
+        <v>-0.7619</v>
       </c>
       <c r="AC8" t="n">
-        <v>-10.1902</v>
+        <v>0.9631</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>167</v>
+        <v>172.95</v>
       </c>
       <c r="C9" t="n">
-        <v>174.4</v>
+        <v>174.61</v>
       </c>
       <c r="D9" t="n">
-        <v>161.14</v>
+        <v>142.69</v>
       </c>
       <c r="E9" t="n">
-        <v>164.18</v>
+        <v>151.75</v>
       </c>
       <c r="F9" t="n">
-        <v>75.73</v>
+        <v>76.13</v>
       </c>
       <c r="G9" t="n">
-        <v>77.37</v>
+        <v>76.27</v>
       </c>
       <c r="H9" t="n">
-        <v>74.23</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I9" t="n">
-        <v>75.34</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>9.130000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="K9" t="n">
-        <v>9.390000000000001</v>
+        <v>10.47</v>
       </c>
       <c r="L9" t="n">
-        <v>8.800000000000001</v>
+        <v>8.68</v>
       </c>
       <c r="M9" t="n">
-        <v>9.23</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="N9" t="n">
-        <v>42.77</v>
+        <v>42.51</v>
       </c>
       <c r="O9" t="n">
-        <v>43.57</v>
+        <v>44.82</v>
       </c>
       <c r="P9" t="n">
-        <v>41.93</v>
+        <v>42.44</v>
       </c>
       <c r="Q9" t="n">
-        <v>42.98</v>
+        <v>43.54</v>
       </c>
       <c r="R9" t="n">
-        <v>-11.8213</v>
+        <v>-7.571</v>
       </c>
       <c r="S9" t="n">
-        <v>-4.8342</v>
+        <v>-17.6346</v>
       </c>
       <c r="T9" t="n">
-        <v>-7.2115</v>
+        <v>-20.3077</v>
       </c>
       <c r="U9" t="n">
-        <v>-4.5725</v>
+        <v>-1.3539</v>
       </c>
       <c r="V9" t="n">
-        <v>0.5069</v>
+        <v>-3.7804</v>
       </c>
       <c r="W9" t="n">
-        <v>-1.2323</v>
+        <v>-3.4304</v>
       </c>
       <c r="X9" t="n">
-        <v>11.6082</v>
+        <v>7.8007</v>
       </c>
       <c r="Y9" t="n">
-        <v>3.1285</v>
+        <v>19.1617</v>
       </c>
       <c r="Z9" t="n">
-        <v>4.2938</v>
+        <v>21.3415</v>
       </c>
       <c r="AA9" t="n">
-        <v>4.6506</v>
+        <v>1.3029</v>
       </c>
       <c r="AB9" t="n">
-        <v>-0.7619</v>
+        <v>3.6914</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.9631</v>
+        <v>3.1265</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>172.95</v>
+        <v>141.24</v>
       </c>
       <c r="C10" t="n">
-        <v>174.61</v>
+        <v>160.6</v>
       </c>
       <c r="D10" t="n">
-        <v>142.69</v>
+        <v>135.02</v>
       </c>
       <c r="E10" t="n">
-        <v>151.75</v>
+        <v>151.89</v>
       </c>
       <c r="F10" t="n">
-        <v>76.13</v>
+        <v>72.41</v>
       </c>
       <c r="G10" t="n">
-        <v>76.27</v>
+        <v>74.5</v>
       </c>
       <c r="H10" t="n">
-        <v>72.09999999999999</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>74.31999999999999</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>8.77</v>
+        <v>10.64</v>
       </c>
       <c r="K10" t="n">
-        <v>10.47</v>
+        <v>11.07</v>
       </c>
       <c r="L10" t="n">
-        <v>8.68</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="M10" t="n">
-        <v>9.949999999999999</v>
+        <v>9.93</v>
       </c>
       <c r="N10" t="n">
-        <v>42.51</v>
+        <v>44.68</v>
       </c>
       <c r="O10" t="n">
-        <v>44.82</v>
+        <v>45.53</v>
       </c>
       <c r="P10" t="n">
-        <v>42.44</v>
+        <v>43.46</v>
       </c>
       <c r="Q10" t="n">
-        <v>43.54</v>
+        <v>44.37</v>
       </c>
       <c r="R10" t="n">
-        <v>-7.571</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="S10" t="n">
-        <v>-17.6346</v>
+        <v>-18.422</v>
       </c>
       <c r="T10" t="n">
-        <v>-20.3077</v>
+        <v>-11.958</v>
       </c>
       <c r="U10" t="n">
-        <v>-1.3539</v>
+        <v>-1.8703</v>
       </c>
       <c r="V10" t="n">
-        <v>-3.7804</v>
+        <v>-7.6251</v>
       </c>
       <c r="W10" t="n">
-        <v>-3.4304</v>
+        <v>-2.7081</v>
       </c>
       <c r="X10" t="n">
-        <v>7.8007</v>
+        <v>-0.201</v>
       </c>
       <c r="Y10" t="n">
-        <v>19.1617</v>
+        <v>20.0726</v>
       </c>
       <c r="Z10" t="n">
-        <v>21.3415</v>
+        <v>10.9497</v>
       </c>
       <c r="AA10" t="n">
-        <v>1.3029</v>
+        <v>1.9063</v>
       </c>
       <c r="AB10" t="n">
-        <v>3.6914</v>
+        <v>8.0351</v>
       </c>
       <c r="AC10" t="n">
-        <v>3.1265</v>
+        <v>2.4475</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>141.24</v>
+        <v>161</v>
       </c>
       <c r="C11" t="n">
-        <v>160.6</v>
+        <v>173.7</v>
       </c>
       <c r="D11" t="n">
-        <v>135.02</v>
+        <v>161</v>
       </c>
       <c r="E11" t="n">
-        <v>151.89</v>
+        <v>173.2</v>
       </c>
       <c r="F11" t="n">
-        <v>72.41</v>
+        <v>74.09</v>
       </c>
       <c r="G11" t="n">
-        <v>74.5</v>
+        <v>76.53</v>
       </c>
       <c r="H11" t="n">
-        <v>70.95999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="I11" t="n">
-        <v>72.93000000000001</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>10.64</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K11" t="n">
-        <v>11.07</v>
+        <v>9.35</v>
       </c>
       <c r="L11" t="n">
-        <v>9.369999999999999</v>
+        <v>8.51</v>
       </c>
       <c r="M11" t="n">
-        <v>9.93</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>44.68</v>
+        <v>43.67</v>
       </c>
       <c r="O11" t="n">
-        <v>45.53</v>
+        <v>43.97</v>
       </c>
       <c r="P11" t="n">
-        <v>43.46</v>
+        <v>42.19</v>
       </c>
       <c r="Q11" t="n">
-        <v>44.37</v>
+        <v>42.19</v>
       </c>
       <c r="R11" t="n">
-        <v>0.09229999999999999</v>
+        <v>14.0299</v>
       </c>
       <c r="S11" t="n">
-        <v>-18.422</v>
+        <v>5.494</v>
       </c>
       <c r="T11" t="n">
-        <v>-11.958</v>
+        <v>-5.9922</v>
       </c>
       <c r="U11" t="n">
-        <v>-1.8703</v>
+        <v>4.9088</v>
       </c>
       <c r="V11" t="n">
-        <v>-7.6251</v>
+        <v>1.553</v>
       </c>
       <c r="W11" t="n">
-        <v>-2.7081</v>
+        <v>-0.9451000000000001</v>
       </c>
       <c r="X11" t="n">
-        <v>-0.201</v>
+        <v>-13.998</v>
       </c>
       <c r="Y11" t="n">
-        <v>20.0726</v>
+        <v>-7.4756</v>
       </c>
       <c r="Z11" t="n">
-        <v>10.9497</v>
+        <v>2.2754</v>
       </c>
       <c r="AA11" t="n">
-        <v>1.9063</v>
+        <v>-4.9132</v>
       </c>
       <c r="AB11" t="n">
-        <v>8.0351</v>
+        <v>-1.8381</v>
       </c>
       <c r="AC11" t="n">
-        <v>2.4475</v>
+        <v>0.4763</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>161</v>
+        <v>171.26</v>
       </c>
       <c r="C12" t="n">
-        <v>173.7</v>
+        <v>179.97</v>
       </c>
       <c r="D12" t="n">
-        <v>161</v>
+        <v>168.23</v>
       </c>
       <c r="E12" t="n">
-        <v>173.2</v>
+        <v>178.39</v>
       </c>
       <c r="F12" t="n">
-        <v>74.09</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>76.53</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>73.62</v>
+        <v>74.47</v>
       </c>
       <c r="I12" t="n">
-        <v>76.51000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J12" t="n">
-        <v>9.300000000000001</v>
+        <v>8.65</v>
       </c>
       <c r="K12" t="n">
-        <v>9.35</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L12" t="n">
-        <v>8.51</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M12" t="n">
-        <v>8.539999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N12" t="n">
-        <v>43.67</v>
+        <v>42.94</v>
       </c>
       <c r="O12" t="n">
-        <v>43.97</v>
+        <v>43.33</v>
       </c>
       <c r="P12" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="Q12" t="n">
-        <v>42.19</v>
+        <v>41.96</v>
       </c>
       <c r="R12" t="n">
-        <v>14.0299</v>
+        <v>2.9965</v>
       </c>
       <c r="S12" t="n">
-        <v>5.494</v>
+        <v>17.5552</v>
       </c>
       <c r="T12" t="n">
-        <v>-5.9922</v>
+        <v>-4.1893</v>
       </c>
       <c r="U12" t="n">
-        <v>4.9088</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="V12" t="n">
-        <v>1.553</v>
+        <v>3.5388</v>
       </c>
       <c r="W12" t="n">
-        <v>-0.9451000000000001</v>
+        <v>-2.5332</v>
       </c>
       <c r="X12" t="n">
-        <v>-13.998</v>
+        <v>-2.9274</v>
       </c>
       <c r="Y12" t="n">
-        <v>-7.4756</v>
+        <v>-16.6834</v>
       </c>
       <c r="Z12" t="n">
-        <v>2.2754</v>
+        <v>0.2418</v>
       </c>
       <c r="AA12" t="n">
-        <v>-4.9132</v>
+        <v>-0.5452</v>
       </c>
       <c r="AB12" t="n">
-        <v>-1.8381</v>
+        <v>-3.6288</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.4763</v>
+        <v>2.167</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>171.26</v>
+        <v>184.8</v>
       </c>
       <c r="C13" t="n">
-        <v>179.97</v>
+        <v>195.27</v>
       </c>
       <c r="D13" t="n">
-        <v>168.23</v>
+        <v>183.34</v>
       </c>
       <c r="E13" t="n">
-        <v>178.39</v>
+        <v>190.56</v>
       </c>
       <c r="F13" t="n">
-        <v>75.18000000000001</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>77.79000000000001</v>
+        <v>79.33</v>
       </c>
       <c r="H13" t="n">
-        <v>74.47</v>
+        <v>77.33</v>
       </c>
       <c r="I13" t="n">
-        <v>76.95</v>
+        <v>77.84</v>
       </c>
       <c r="J13" t="n">
-        <v>8.65</v>
+        <v>8</v>
       </c>
       <c r="K13" t="n">
-        <v>8.779999999999999</v>
+        <v>8.06</v>
       </c>
       <c r="L13" t="n">
-        <v>8.210000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="M13" t="n">
-        <v>8.289999999999999</v>
+        <v>7.73</v>
       </c>
       <c r="N13" t="n">
-        <v>42.94</v>
+        <v>41.4</v>
       </c>
       <c r="O13" t="n">
-        <v>43.33</v>
+        <v>41.78</v>
       </c>
       <c r="P13" t="n">
+        <v>40.68</v>
+      </c>
+      <c r="Q13" t="n">
         <v>41.5</v>
       </c>
-      <c r="Q13" t="n">
-        <v>41.96</v>
-      </c>
       <c r="R13" t="n">
-        <v>2.9965</v>
+        <v>6.8221</v>
       </c>
       <c r="S13" t="n">
-        <v>17.5552</v>
+        <v>25.4592</v>
       </c>
       <c r="T13" t="n">
-        <v>-4.1893</v>
+        <v>16.0677</v>
       </c>
       <c r="U13" t="n">
-        <v>0.5750999999999999</v>
+        <v>1.1566</v>
       </c>
       <c r="V13" t="n">
-        <v>3.5388</v>
+        <v>6.7325</v>
       </c>
       <c r="W13" t="n">
-        <v>-2.5332</v>
+        <v>3.3183</v>
       </c>
       <c r="X13" t="n">
-        <v>-2.9274</v>
+        <v>-6.7551</v>
       </c>
       <c r="Y13" t="n">
-        <v>-16.6834</v>
+        <v>-22.1551</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.2418</v>
+        <v>-16.2514</v>
       </c>
       <c r="AA13" t="n">
-        <v>-0.5452</v>
+        <v>-1.0963</v>
       </c>
       <c r="AB13" t="n">
-        <v>-3.6288</v>
+        <v>-6.4683</v>
       </c>
       <c r="AC13" t="n">
-        <v>2.167</v>
+        <v>-3.4435</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>184.8</v>
+        <v>211.38</v>
       </c>
       <c r="C14" t="n">
-        <v>195.27</v>
+        <v>228.5</v>
       </c>
       <c r="D14" t="n">
-        <v>183.34</v>
+        <v>209.89</v>
       </c>
       <c r="E14" t="n">
-        <v>190.56</v>
+        <v>225.79</v>
       </c>
       <c r="F14" t="n">
-        <v>78.04000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="G14" t="n">
-        <v>79.33</v>
+        <v>82.27</v>
       </c>
       <c r="H14" t="n">
-        <v>77.33</v>
+        <v>79.98</v>
       </c>
       <c r="I14" t="n">
-        <v>77.84</v>
+        <v>81.95</v>
       </c>
       <c r="J14" t="n">
-        <v>8</v>
+        <v>6.9</v>
       </c>
       <c r="K14" t="n">
-        <v>8.06</v>
+        <v>6.95</v>
       </c>
       <c r="L14" t="n">
-        <v>7.5</v>
+        <v>6.19</v>
       </c>
       <c r="M14" t="n">
-        <v>7.73</v>
+        <v>6.29</v>
       </c>
       <c r="N14" t="n">
-        <v>41.4</v>
+        <v>40.05</v>
       </c>
       <c r="O14" t="n">
-        <v>41.78</v>
+        <v>40.35</v>
       </c>
       <c r="P14" t="n">
-        <v>40.68</v>
+        <v>39.14</v>
       </c>
       <c r="Q14" t="n">
-        <v>41.5</v>
+        <v>39.28</v>
       </c>
       <c r="R14" t="n">
-        <v>6.8221</v>
+        <v>18.4876</v>
       </c>
       <c r="S14" t="n">
-        <v>25.4592</v>
+        <v>30.3637</v>
       </c>
       <c r="T14" t="n">
-        <v>16.0677</v>
+        <v>48.7908</v>
       </c>
       <c r="U14" t="n">
-        <v>1.1566</v>
+        <v>5.2801</v>
       </c>
       <c r="V14" t="n">
-        <v>6.7325</v>
+        <v>7.1102</v>
       </c>
       <c r="W14" t="n">
-        <v>3.3183</v>
+        <v>10.2664</v>
       </c>
       <c r="X14" t="n">
-        <v>-6.7551</v>
+        <v>-18.6287</v>
       </c>
       <c r="Y14" t="n">
-        <v>-22.1551</v>
+        <v>-26.3466</v>
       </c>
       <c r="Z14" t="n">
-        <v>-16.2514</v>
+        <v>-36.7839</v>
       </c>
       <c r="AA14" t="n">
-        <v>-1.0963</v>
+        <v>-5.3494</v>
       </c>
       <c r="AB14" t="n">
-        <v>-6.4683</v>
+        <v>-6.8974</v>
       </c>
       <c r="AC14" t="n">
-        <v>-3.4435</v>
+        <v>-9.7841</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>211.38</v>
+        <v>242.66</v>
       </c>
       <c r="C15" t="n">
-        <v>228.5</v>
+        <v>242.66</v>
       </c>
       <c r="D15" t="n">
-        <v>209.89</v>
+        <v>204</v>
       </c>
       <c r="E15" t="n">
-        <v>225.79</v>
+        <v>217.98</v>
       </c>
       <c r="F15" t="n">
-        <v>80.59</v>
+        <v>82.87</v>
       </c>
       <c r="G15" t="n">
-        <v>82.27</v>
+        <v>82.91</v>
       </c>
       <c r="H15" t="n">
-        <v>79.98</v>
+        <v>80.33</v>
       </c>
       <c r="I15" t="n">
-        <v>81.95</v>
+        <v>81.67</v>
       </c>
       <c r="J15" t="n">
-        <v>6.9</v>
+        <v>5.83</v>
       </c>
       <c r="K15" t="n">
-        <v>6.95</v>
+        <v>6.91</v>
       </c>
       <c r="L15" t="n">
-        <v>6.19</v>
+        <v>5.83</v>
       </c>
       <c r="M15" t="n">
-        <v>6.29</v>
+        <v>6.53</v>
       </c>
       <c r="N15" t="n">
-        <v>40.05</v>
+        <v>38.87</v>
       </c>
       <c r="O15" t="n">
-        <v>40.35</v>
+        <v>40.09</v>
       </c>
       <c r="P15" t="n">
-        <v>39.14</v>
+        <v>38.86</v>
       </c>
       <c r="Q15" t="n">
-        <v>39.28</v>
+        <v>39.44</v>
       </c>
       <c r="R15" t="n">
-        <v>18.4876</v>
+        <v>-3.459</v>
       </c>
       <c r="S15" t="n">
-        <v>30.3637</v>
+        <v>22.1929</v>
       </c>
       <c r="T15" t="n">
-        <v>48.7908</v>
+        <v>43.5118</v>
       </c>
       <c r="U15" t="n">
-        <v>5.2801</v>
+        <v>-0.3417</v>
       </c>
       <c r="V15" t="n">
-        <v>7.1102</v>
+        <v>6.1339</v>
       </c>
       <c r="W15" t="n">
-        <v>10.2664</v>
+        <v>11.9841</v>
       </c>
       <c r="X15" t="n">
-        <v>-18.6287</v>
+        <v>3.8156</v>
       </c>
       <c r="Y15" t="n">
-        <v>-26.3466</v>
+        <v>-21.2304</v>
       </c>
       <c r="Z15" t="n">
-        <v>-36.7839</v>
+        <v>-34.2397</v>
       </c>
       <c r="AA15" t="n">
-        <v>-5.3494</v>
+        <v>0.4073</v>
       </c>
       <c r="AB15" t="n">
-        <v>-6.8974</v>
+        <v>-6.0057</v>
       </c>
       <c r="AC15" t="n">
-        <v>-9.7841</v>
+        <v>-11.1111</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>242.66</v>
+        <v>219</v>
       </c>
       <c r="C16" t="n">
-        <v>242.66</v>
+        <v>231.89</v>
       </c>
       <c r="D16" t="n">
-        <v>204</v>
+        <v>207.56</v>
       </c>
       <c r="E16" t="n">
-        <v>217.98</v>
+        <v>224.63</v>
       </c>
       <c r="F16" t="n">
-        <v>82.87</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>82.91</v>
+        <v>84.05</v>
       </c>
       <c r="H16" t="n">
-        <v>80.33</v>
+        <v>80.66</v>
       </c>
       <c r="I16" t="n">
-        <v>81.67</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="J16" t="n">
-        <v>5.83</v>
+        <v>6.49</v>
       </c>
       <c r="K16" t="n">
-        <v>6.91</v>
+        <v>6.83</v>
       </c>
       <c r="L16" t="n">
-        <v>5.83</v>
+        <v>6.1</v>
       </c>
       <c r="M16" t="n">
-        <v>6.53</v>
+        <v>6.31</v>
       </c>
       <c r="N16" t="n">
-        <v>38.87</v>
+        <v>39.41</v>
       </c>
       <c r="O16" t="n">
-        <v>40.09</v>
+        <v>39.94</v>
       </c>
       <c r="P16" t="n">
-        <v>38.86</v>
+        <v>38.3</v>
       </c>
       <c r="Q16" t="n">
-        <v>39.44</v>
+        <v>38.47</v>
       </c>
       <c r="R16" t="n">
-        <v>-3.459</v>
+        <v>3.0507</v>
       </c>
       <c r="S16" t="n">
-        <v>22.1929</v>
+        <v>17.8789</v>
       </c>
       <c r="T16" t="n">
-        <v>43.5118</v>
+        <v>29.694</v>
       </c>
       <c r="U16" t="n">
-        <v>-0.3417</v>
+        <v>2.4611</v>
       </c>
       <c r="V16" t="n">
-        <v>6.1339</v>
+        <v>7.5026</v>
       </c>
       <c r="W16" t="n">
-        <v>11.9841</v>
+        <v>9.3713</v>
       </c>
       <c r="X16" t="n">
-        <v>3.8156</v>
+        <v>-3.3691</v>
       </c>
       <c r="Y16" t="n">
-        <v>-21.2304</v>
+        <v>-18.37</v>
       </c>
       <c r="Z16" t="n">
-        <v>-34.2397</v>
+        <v>-26.1124</v>
       </c>
       <c r="AA16" t="n">
-        <v>0.4073</v>
+        <v>-2.4594</v>
       </c>
       <c r="AB16" t="n">
-        <v>-6.0057</v>
+        <v>-7.3012</v>
       </c>
       <c r="AC16" t="n">
-        <v>-11.1111</v>
+        <v>-8.817299999999999</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>219</v>
+        <v>231.82</v>
       </c>
       <c r="C17" t="n">
-        <v>231.89</v>
+        <v>239.07</v>
       </c>
       <c r="D17" t="n">
-        <v>207.56</v>
+        <v>218.56</v>
       </c>
       <c r="E17" t="n">
-        <v>224.63</v>
+        <v>224.34</v>
       </c>
       <c r="F17" t="n">
-        <v>81.73999999999999</v>
+        <v>84.41</v>
       </c>
       <c r="G17" t="n">
-        <v>84.05</v>
+        <v>85.7</v>
       </c>
       <c r="H17" t="n">
-        <v>80.66</v>
+        <v>83.53</v>
       </c>
       <c r="I17" t="n">
-        <v>83.68000000000001</v>
+        <v>84.56</v>
       </c>
       <c r="J17" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="K17" t="n">
         <v>6.49</v>
       </c>
-      <c r="K17" t="n">
-        <v>6.83</v>
-      </c>
       <c r="L17" t="n">
-        <v>6.1</v>
+        <v>5.91</v>
       </c>
       <c r="M17" t="n">
-        <v>6.31</v>
+        <v>6.33</v>
       </c>
       <c r="N17" t="n">
-        <v>39.41</v>
+        <v>38.15</v>
       </c>
       <c r="O17" t="n">
-        <v>39.94</v>
+        <v>38.56</v>
       </c>
       <c r="P17" t="n">
-        <v>38.3</v>
+        <v>37.56</v>
       </c>
       <c r="Q17" t="n">
-        <v>38.47</v>
+        <v>38.08</v>
       </c>
       <c r="R17" t="n">
-        <v>3.0507</v>
+        <v>-0.1291</v>
       </c>
       <c r="S17" t="n">
-        <v>17.8789</v>
+        <v>-0.6422</v>
       </c>
       <c r="T17" t="n">
-        <v>29.694</v>
+        <v>25.7582</v>
       </c>
       <c r="U17" t="n">
-        <v>2.4611</v>
+        <v>1.0516</v>
       </c>
       <c r="V17" t="n">
-        <v>7.5026</v>
+        <v>3.1849</v>
       </c>
       <c r="W17" t="n">
-        <v>9.3713</v>
+        <v>9.8895</v>
       </c>
       <c r="X17" t="n">
-        <v>-3.3691</v>
+        <v>0.317</v>
       </c>
       <c r="Y17" t="n">
-        <v>-18.37</v>
+        <v>0.6359</v>
       </c>
       <c r="Z17" t="n">
-        <v>-26.1124</v>
+        <v>-23.6429</v>
       </c>
       <c r="AA17" t="n">
-        <v>-2.4594</v>
+        <v>-1.0138</v>
       </c>
       <c r="AB17" t="n">
-        <v>-7.3012</v>
+        <v>-3.055</v>
       </c>
       <c r="AC17" t="n">
-        <v>-8.817299999999999</v>
+        <v>-9.2469</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>231.82</v>
+        <v>217.27</v>
       </c>
       <c r="C18" t="n">
-        <v>239.07</v>
+        <v>234.06</v>
       </c>
       <c r="D18" t="n">
-        <v>218.56</v>
+        <v>210.14</v>
       </c>
       <c r="E18" t="n">
-        <v>224.34</v>
+        <v>227.03</v>
       </c>
       <c r="F18" t="n">
-        <v>84.41</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>85.7</v>
+        <v>87.06</v>
       </c>
       <c r="H18" t="n">
-        <v>83.53</v>
+        <v>83.75</v>
       </c>
       <c r="I18" t="n">
-        <v>84.56</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>6.11</v>
+        <v>6.55</v>
       </c>
       <c r="K18" t="n">
-        <v>6.49</v>
+        <v>6.74</v>
       </c>
       <c r="L18" t="n">
-        <v>5.91</v>
+        <v>6.05</v>
       </c>
       <c r="M18" t="n">
-        <v>6.33</v>
+        <v>6.26</v>
       </c>
       <c r="N18" t="n">
-        <v>38.15</v>
+        <v>38.27</v>
       </c>
       <c r="O18" t="n">
-        <v>38.56</v>
+        <v>38.46</v>
       </c>
       <c r="P18" t="n">
-        <v>37.56</v>
+        <v>36.96</v>
       </c>
       <c r="Q18" t="n">
-        <v>38.08</v>
+        <v>37.42</v>
       </c>
       <c r="R18" t="n">
-        <v>-0.1291</v>
+        <v>1.1991</v>
       </c>
       <c r="S18" t="n">
-        <v>-0.6422</v>
+        <v>4.1518</v>
       </c>
       <c r="T18" t="n">
-        <v>25.7582</v>
+        <v>19.1383</v>
       </c>
       <c r="U18" t="n">
-        <v>1.0516</v>
+        <v>1.7502</v>
       </c>
       <c r="V18" t="n">
-        <v>3.1849</v>
+        <v>5.3508</v>
       </c>
       <c r="W18" t="n">
-        <v>9.8895</v>
+        <v>10.5344</v>
       </c>
       <c r="X18" t="n">
-        <v>0.317</v>
+        <v>-1.1058</v>
       </c>
       <c r="Y18" t="n">
-        <v>0.6359</v>
+        <v>-4.1348</v>
       </c>
       <c r="Z18" t="n">
-        <v>-23.6429</v>
+        <v>-19.0168</v>
       </c>
       <c r="AA18" t="n">
-        <v>-1.0138</v>
+        <v>-1.7332</v>
       </c>
       <c r="AB18" t="n">
-        <v>-3.055</v>
+        <v>-5.1217</v>
       </c>
       <c r="AC18" t="n">
-        <v>-9.2469</v>
+        <v>-9.831300000000001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>217.27</v>
+        <v>243.18</v>
       </c>
       <c r="C19" t="n">
-        <v>234.06</v>
+        <v>267.08</v>
       </c>
       <c r="D19" t="n">
-        <v>210.14</v>
+        <v>238.82</v>
       </c>
       <c r="E19" t="n">
-        <v>227.03</v>
+        <v>266.32</v>
       </c>
       <c r="F19" t="n">
-        <v>84.15000000000001</v>
+        <v>85.94</v>
       </c>
       <c r="G19" t="n">
-        <v>87.06</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>83.75</v>
+        <v>84.83</v>
       </c>
       <c r="I19" t="n">
-        <v>86.04000000000001</v>
+        <v>87.22</v>
       </c>
       <c r="J19" t="n">
-        <v>6.55</v>
+        <v>5.8</v>
       </c>
       <c r="K19" t="n">
-        <v>6.74</v>
+        <v>5.93</v>
       </c>
       <c r="L19" t="n">
-        <v>6.05</v>
+        <v>5.15</v>
       </c>
       <c r="M19" t="n">
-        <v>6.26</v>
+        <v>5.17</v>
       </c>
       <c r="N19" t="n">
-        <v>38.27</v>
+        <v>37.47</v>
       </c>
       <c r="O19" t="n">
-        <v>38.46</v>
+        <v>37.95</v>
       </c>
       <c r="P19" t="n">
-        <v>36.96</v>
+        <v>36.86</v>
       </c>
       <c r="Q19" t="n">
-        <v>37.42</v>
+        <v>36.91</v>
       </c>
       <c r="R19" t="n">
-        <v>1.1991</v>
+        <v>17.3061</v>
       </c>
       <c r="S19" t="n">
-        <v>4.1518</v>
+        <v>18.5594</v>
       </c>
       <c r="T19" t="n">
-        <v>19.1383</v>
+        <v>17.9503</v>
       </c>
       <c r="U19" t="n">
-        <v>1.7502</v>
+        <v>1.3715</v>
       </c>
       <c r="V19" t="n">
-        <v>5.3508</v>
+        <v>4.2304</v>
       </c>
       <c r="W19" t="n">
-        <v>10.5344</v>
+        <v>6.4308</v>
       </c>
       <c r="X19" t="n">
-        <v>-1.1058</v>
+        <v>-17.4121</v>
       </c>
       <c r="Y19" t="n">
-        <v>-4.1348</v>
+        <v>-18.0666</v>
       </c>
       <c r="Z19" t="n">
-        <v>-19.0168</v>
+        <v>-17.806</v>
       </c>
       <c r="AA19" t="n">
-        <v>-1.7332</v>
+        <v>-1.3629</v>
       </c>
       <c r="AB19" t="n">
-        <v>-5.1217</v>
+        <v>-4.0551</v>
       </c>
       <c r="AC19" t="n">
-        <v>-9.831300000000001</v>
+        <v>-6.0336</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>243.18</v>
+        <v>281.47</v>
       </c>
       <c r="C20" t="n">
-        <v>267.08</v>
+        <v>284.58</v>
       </c>
       <c r="D20" t="n">
-        <v>238.82</v>
+        <v>257.26</v>
       </c>
       <c r="E20" t="n">
-        <v>266.32</v>
+        <v>280.54</v>
       </c>
       <c r="F20" t="n">
-        <v>85.94</v>
+        <v>87.68000000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>87.31999999999999</v>
+        <v>88.09</v>
       </c>
       <c r="H20" t="n">
-        <v>84.83</v>
+        <v>85.41</v>
       </c>
       <c r="I20" t="n">
-        <v>87.22</v>
+        <v>86.56</v>
       </c>
       <c r="J20" t="n">
-        <v>5.8</v>
+        <v>4.88</v>
       </c>
       <c r="K20" t="n">
-        <v>5.93</v>
+        <v>5.35</v>
       </c>
       <c r="L20" t="n">
-        <v>5.15</v>
+        <v>4.82</v>
       </c>
       <c r="M20" t="n">
-        <v>5.17</v>
+        <v>4.91</v>
       </c>
       <c r="N20" t="n">
-        <v>37.47</v>
+        <v>36.73</v>
       </c>
       <c r="O20" t="n">
-        <v>37.95</v>
+        <v>37.69</v>
       </c>
       <c r="P20" t="n">
-        <v>36.86</v>
+        <v>36.55</v>
       </c>
       <c r="Q20" t="n">
-        <v>36.91</v>
+        <v>37.19</v>
       </c>
       <c r="R20" t="n">
-        <v>17.3061</v>
+        <v>5.3394</v>
       </c>
       <c r="S20" t="n">
-        <v>18.5594</v>
+        <v>25.0513</v>
       </c>
       <c r="T20" t="n">
-        <v>17.9503</v>
+        <v>28.6999</v>
       </c>
       <c r="U20" t="n">
-        <v>1.3715</v>
+        <v>-0.7567</v>
       </c>
       <c r="V20" t="n">
-        <v>4.2304</v>
+        <v>2.3652</v>
       </c>
       <c r="W20" t="n">
-        <v>6.4308</v>
+        <v>5.9875</v>
       </c>
       <c r="X20" t="n">
-        <v>-17.4121</v>
+        <v>-5.029</v>
       </c>
       <c r="Y20" t="n">
-        <v>-18.0666</v>
+        <v>-22.4329</v>
       </c>
       <c r="Z20" t="n">
-        <v>-17.806</v>
+        <v>-24.8086</v>
       </c>
       <c r="AA20" t="n">
-        <v>-1.3629</v>
+        <v>0.7586000000000001</v>
       </c>
       <c r="AB20" t="n">
-        <v>-4.0551</v>
+        <v>-2.3372</v>
       </c>
       <c r="AC20" t="n">
-        <v>-6.0336</v>
+        <v>-5.7049</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>281.47</v>
+        <v>242.04</v>
       </c>
       <c r="C21" t="n">
-        <v>284.58</v>
+        <v>274.5</v>
       </c>
       <c r="D21" t="n">
-        <v>257.26</v>
+        <v>228.55</v>
       </c>
       <c r="E21" t="n">
-        <v>280.54</v>
+        <v>262.7</v>
       </c>
       <c r="F21" t="n">
-        <v>87.68000000000001</v>
+        <v>83.47</v>
       </c>
       <c r="G21" t="n">
-        <v>88.09</v>
+        <v>86.25</v>
       </c>
       <c r="H21" t="n">
-        <v>85.41</v>
+        <v>82.48</v>
       </c>
       <c r="I21" t="n">
-        <v>86.56</v>
+        <v>85.22</v>
       </c>
       <c r="J21" t="n">
-        <v>4.88</v>
+        <v>5.57</v>
       </c>
       <c r="K21" t="n">
-        <v>5.35</v>
+        <v>5.81</v>
       </c>
       <c r="L21" t="n">
-        <v>4.82</v>
+        <v>5</v>
       </c>
       <c r="M21" t="n">
-        <v>4.91</v>
+        <v>5.2</v>
       </c>
       <c r="N21" t="n">
-        <v>36.73</v>
+        <v>38.53</v>
       </c>
       <c r="O21" t="n">
-        <v>37.69</v>
+        <v>38.96</v>
       </c>
       <c r="P21" t="n">
-        <v>36.55</v>
+        <v>37.33</v>
       </c>
       <c r="Q21" t="n">
-        <v>37.19</v>
+        <v>37.76</v>
       </c>
       <c r="R21" t="n">
-        <v>5.3394</v>
+        <v>-6.3592</v>
       </c>
       <c r="S21" t="n">
-        <v>25.0513</v>
+        <v>15.7116</v>
       </c>
       <c r="T21" t="n">
-        <v>28.6999</v>
+        <v>16.9479</v>
       </c>
       <c r="U21" t="n">
-        <v>-0.7567</v>
+        <v>-1.5481</v>
       </c>
       <c r="V21" t="n">
-        <v>2.3652</v>
+        <v>-0.953</v>
       </c>
       <c r="W21" t="n">
-        <v>5.9875</v>
+        <v>1.8403</v>
       </c>
       <c r="X21" t="n">
-        <v>-5.029</v>
+        <v>5.9063</v>
       </c>
       <c r="Y21" t="n">
-        <v>-22.4329</v>
+        <v>-16.9329</v>
       </c>
       <c r="Z21" t="n">
-        <v>-24.8086</v>
+        <v>-17.5911</v>
       </c>
       <c r="AA21" t="n">
-        <v>0.7586000000000001</v>
+        <v>1.5327</v>
       </c>
       <c r="AB21" t="n">
-        <v>-2.3372</v>
+        <v>0.9086</v>
       </c>
       <c r="AC21" t="n">
-        <v>-5.7049</v>
+        <v>-1.8456</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>242.04</v>
+        <v>230.8482</v>
       </c>
       <c r="C22" t="n">
-        <v>274.5</v>
+        <v>233.69</v>
       </c>
       <c r="D22" t="n">
-        <v>228.55</v>
+        <v>182.0033</v>
       </c>
       <c r="E22" t="n">
-        <v>262.7</v>
+        <v>182.54</v>
       </c>
       <c r="F22" t="n">
-        <v>83.47</v>
+        <v>81.55</v>
       </c>
       <c r="G22" t="n">
-        <v>86.245</v>
+        <v>82.08</v>
       </c>
       <c r="H22" t="n">
-        <v>82.47499999999999</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="I22" t="n">
-        <v>85.22</v>
+        <v>73.05</v>
       </c>
       <c r="J22" t="n">
-        <v>5.57</v>
+        <v>5.855</v>
       </c>
       <c r="K22" t="n">
-        <v>5.81</v>
+        <v>6.85</v>
       </c>
       <c r="L22" t="n">
-        <v>5</v>
+        <v>5.79</v>
       </c>
       <c r="M22" t="n">
-        <v>5.2</v>
+        <v>6.84</v>
       </c>
       <c r="N22" t="n">
-        <v>38.53</v>
+        <v>39.45</v>
       </c>
       <c r="O22" t="n">
-        <v>38.96</v>
+        <v>43.35</v>
       </c>
       <c r="P22" t="n">
-        <v>37.33</v>
+        <v>39.185</v>
       </c>
       <c r="Q22" t="n">
-        <v>37.76</v>
+        <v>43.19</v>
       </c>
       <c r="R22" t="n">
-        <v>-6.3592</v>
+        <v>-30.5139</v>
       </c>
       <c r="S22" t="n">
-        <v>15.7116</v>
+        <v>-31.4584</v>
       </c>
       <c r="T22" t="n">
-        <v>16.9479</v>
+        <v>-18.6324</v>
       </c>
       <c r="U22" t="n">
-        <v>-1.5481</v>
+        <v>-14.2807</v>
       </c>
       <c r="V22" t="n">
-        <v>-0.953</v>
+        <v>-16.2463</v>
       </c>
       <c r="W22" t="n">
-        <v>1.8403</v>
+        <v>-13.6116</v>
       </c>
       <c r="X22" t="n">
-        <v>5.9063</v>
+        <v>31.5385</v>
       </c>
       <c r="Y22" t="n">
-        <v>-16.9329</v>
+        <v>32.3017</v>
       </c>
       <c r="Z22" t="n">
-        <v>-17.5911</v>
+        <v>8.056900000000001</v>
       </c>
       <c r="AA22" t="n">
-        <v>1.5327</v>
+        <v>14.3803</v>
       </c>
       <c r="AB22" t="n">
-        <v>0.9086</v>
+        <v>17.0144</v>
       </c>
       <c r="AC22" t="n">
-        <v>-1.8456</v>
+        <v>13.4191</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-08 23:12
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC22"/>
+  <dimension ref="A1:AC21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1804 +568,1713 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>162.12</v>
+        <v>181</v>
       </c>
       <c r="C2" t="n">
-        <v>162.9</v>
+        <v>191.29</v>
       </c>
       <c r="D2" t="n">
-        <v>147.61</v>
+        <v>178.94</v>
       </c>
       <c r="E2" t="n">
-        <v>152.1</v>
+        <v>190.42</v>
       </c>
       <c r="F2" t="n">
-        <v>71.87</v>
+        <v>76</v>
       </c>
       <c r="G2" t="n">
-        <v>73.3</v>
+        <v>77.36</v>
       </c>
       <c r="H2" t="n">
-        <v>70.38</v>
+        <v>75.55</v>
       </c>
       <c r="I2" t="n">
-        <v>71.34</v>
+        <v>76.95999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>10.02</v>
+        <v>8.65</v>
       </c>
       <c r="K2" t="n">
-        <v>10.88</v>
+        <v>8.77</v>
       </c>
       <c r="L2" t="n">
-        <v>9.970000000000001</v>
+        <v>8.15</v>
       </c>
       <c r="M2" t="n">
-        <v>10.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="N2" t="n">
-        <v>45.41</v>
+        <v>42.74</v>
       </c>
       <c r="O2" t="n">
-        <v>46.36</v>
+        <v>43</v>
       </c>
       <c r="P2" t="n">
-        <v>44.5</v>
+        <v>41.99</v>
       </c>
       <c r="Q2" t="n">
-        <v>45.73</v>
+        <v>42.22</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>163</v>
+        <v>177.62</v>
       </c>
       <c r="C3" t="n">
-        <v>177.5</v>
+        <v>182.24</v>
       </c>
       <c r="D3" t="n">
-        <v>161.51</v>
+        <v>150.58</v>
       </c>
       <c r="E3" t="n">
-        <v>176.94</v>
+        <v>172.52</v>
       </c>
       <c r="F3" t="n">
-        <v>72.81999999999999</v>
+        <v>75.3</v>
       </c>
       <c r="G3" t="n">
-        <v>76.31</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>72.7</v>
+        <v>71.55</v>
       </c>
       <c r="I3" t="n">
-        <v>76.28</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>9.859999999999999</v>
+        <v>8.75</v>
       </c>
       <c r="K3" t="n">
-        <v>9.970000000000001</v>
+        <v>9.91</v>
       </c>
       <c r="L3" t="n">
-        <v>8.84</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="M3" t="n">
-        <v>8.85</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N3" t="n">
-        <v>44.82</v>
+        <v>43.14</v>
       </c>
       <c r="O3" t="n">
-        <v>44.89</v>
+        <v>45.19</v>
       </c>
       <c r="P3" t="n">
-        <v>42.57</v>
+        <v>42.79</v>
       </c>
       <c r="Q3" t="n">
-        <v>42.57</v>
+        <v>43.31</v>
       </c>
       <c r="R3" t="n">
-        <v>16.3314</v>
+        <v>-9.4003</v>
       </c>
       <c r="U3" t="n">
-        <v>6.9246</v>
+        <v>-2.5988</v>
       </c>
       <c r="X3" t="n">
-        <v>-16.5094</v>
+        <v>9.1463</v>
       </c>
       <c r="AA3" t="n">
-        <v>-6.9101</v>
+        <v>2.5817</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>181</v>
+        <v>183.84</v>
       </c>
       <c r="C4" t="n">
-        <v>191.29</v>
+        <v>188.49</v>
       </c>
       <c r="D4" t="n">
-        <v>178.94</v>
+        <v>172.26</v>
       </c>
       <c r="E4" t="n">
-        <v>190.42</v>
+        <v>184.24</v>
       </c>
       <c r="F4" t="n">
-        <v>76</v>
+        <v>75.81</v>
       </c>
       <c r="G4" t="n">
-        <v>77.36</v>
+        <v>77.94</v>
       </c>
       <c r="H4" t="n">
-        <v>75.55</v>
+        <v>74.19</v>
       </c>
       <c r="I4" t="n">
-        <v>76.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>8.65</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>8.77</v>
+        <v>8.98</v>
       </c>
       <c r="L4" t="n">
-        <v>8.15</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>8.199999999999999</v>
+        <v>8.35</v>
       </c>
       <c r="N4" t="n">
-        <v>42.74</v>
+        <v>42.83</v>
       </c>
       <c r="O4" t="n">
-        <v>43</v>
+        <v>43.77</v>
       </c>
       <c r="P4" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="Q4" t="n">
         <v>41.99</v>
       </c>
-      <c r="Q4" t="n">
-        <v>42.22</v>
-      </c>
       <c r="R4" t="n">
-        <v>7.6184</v>
+        <v>6.7934</v>
       </c>
       <c r="U4" t="n">
-        <v>0.8915</v>
+        <v>3.0416</v>
       </c>
       <c r="X4" t="n">
-        <v>-7.3446</v>
+        <v>-6.7039</v>
       </c>
       <c r="AA4" t="n">
-        <v>-0.8222</v>
+        <v>-3.0478</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>177.62</v>
+        <v>182.67</v>
       </c>
       <c r="C5" t="n">
-        <v>182.24</v>
+        <v>189.56</v>
       </c>
       <c r="D5" t="n">
-        <v>150.58</v>
+        <v>178.28</v>
       </c>
       <c r="E5" t="n">
-        <v>172.52</v>
+        <v>186.19</v>
       </c>
       <c r="F5" t="n">
-        <v>75.3</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>75.93000000000001</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>71.55</v>
+        <v>77.16</v>
       </c>
       <c r="I5" t="n">
-        <v>74.95999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="J5" t="n">
-        <v>8.75</v>
+        <v>8.43</v>
       </c>
       <c r="K5" t="n">
-        <v>9.91</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L5" t="n">
-        <v>8.550000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M5" t="n">
-        <v>8.949999999999999</v>
+        <v>8.27</v>
       </c>
       <c r="N5" t="n">
-        <v>43.14</v>
+        <v>41.98</v>
       </c>
       <c r="O5" t="n">
-        <v>45.19</v>
+        <v>42.06</v>
       </c>
       <c r="P5" t="n">
-        <v>42.79</v>
+        <v>40.68</v>
       </c>
       <c r="Q5" t="n">
-        <v>43.31</v>
+        <v>41.07</v>
       </c>
       <c r="R5" t="n">
-        <v>-9.4003</v>
+        <v>1.0584</v>
       </c>
       <c r="S5" t="n">
-        <v>13.4254</v>
+        <v>-2.2214</v>
       </c>
       <c r="U5" t="n">
-        <v>-2.5988</v>
+        <v>2.2139</v>
       </c>
       <c r="V5" t="n">
-        <v>5.0743</v>
+        <v>2.5858</v>
       </c>
       <c r="X5" t="n">
-        <v>9.1463</v>
+        <v>-0.9581</v>
       </c>
       <c r="Y5" t="n">
-        <v>-15.566</v>
+        <v>0.8537</v>
       </c>
       <c r="AA5" t="n">
-        <v>2.5817</v>
+        <v>-2.191</v>
       </c>
       <c r="AB5" t="n">
-        <v>-5.2919</v>
+        <v>-2.7238</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>183.84</v>
+        <v>167</v>
       </c>
       <c r="C6" t="n">
-        <v>188.49</v>
+        <v>174.4</v>
       </c>
       <c r="D6" t="n">
-        <v>172.26</v>
+        <v>161.14</v>
       </c>
       <c r="E6" t="n">
-        <v>184.24</v>
+        <v>164.18</v>
       </c>
       <c r="F6" t="n">
-        <v>75.81</v>
+        <v>75.73</v>
       </c>
       <c r="G6" t="n">
-        <v>77.94</v>
+        <v>77.37</v>
       </c>
       <c r="H6" t="n">
-        <v>74.19</v>
+        <v>74.23</v>
       </c>
       <c r="I6" t="n">
-        <v>77.23999999999999</v>
+        <v>75.34</v>
       </c>
       <c r="J6" t="n">
-        <v>8.380000000000001</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>8.98</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="L6" t="n">
-        <v>8.140000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M6" t="n">
-        <v>8.35</v>
+        <v>9.23</v>
       </c>
       <c r="N6" t="n">
-        <v>42.83</v>
+        <v>42.77</v>
       </c>
       <c r="O6" t="n">
-        <v>43.77</v>
+        <v>43.57</v>
       </c>
       <c r="P6" t="n">
-        <v>41.6</v>
+        <v>41.93</v>
       </c>
       <c r="Q6" t="n">
-        <v>41.99</v>
+        <v>42.98</v>
       </c>
       <c r="R6" t="n">
-        <v>6.7934</v>
+        <v>-11.8213</v>
       </c>
       <c r="S6" t="n">
-        <v>4.1257</v>
+        <v>-4.8342</v>
       </c>
       <c r="U6" t="n">
-        <v>3.0416</v>
+        <v>-4.5725</v>
       </c>
       <c r="V6" t="n">
-        <v>1.2585</v>
+        <v>0.5069</v>
       </c>
       <c r="X6" t="n">
-        <v>-6.7039</v>
+        <v>11.6082</v>
       </c>
       <c r="Y6" t="n">
-        <v>-5.6497</v>
+        <v>3.1285</v>
       </c>
       <c r="AA6" t="n">
-        <v>-3.0478</v>
+        <v>4.6506</v>
       </c>
       <c r="AB6" t="n">
-        <v>-1.3625</v>
+        <v>-0.7619</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>182.67</v>
+        <v>172.95</v>
       </c>
       <c r="C7" t="n">
-        <v>189.56</v>
+        <v>174.61</v>
       </c>
       <c r="D7" t="n">
-        <v>178.28</v>
+        <v>142.69</v>
       </c>
       <c r="E7" t="n">
-        <v>186.19</v>
+        <v>151.75</v>
       </c>
       <c r="F7" t="n">
-        <v>77.29000000000001</v>
+        <v>76.13</v>
       </c>
       <c r="G7" t="n">
-        <v>79.68000000000001</v>
+        <v>76.27</v>
       </c>
       <c r="H7" t="n">
-        <v>77.16</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>78.95</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>8.43</v>
+        <v>8.77</v>
       </c>
       <c r="K7" t="n">
-        <v>8.630000000000001</v>
+        <v>10.47</v>
       </c>
       <c r="L7" t="n">
-        <v>8.119999999999999</v>
+        <v>8.68</v>
       </c>
       <c r="M7" t="n">
-        <v>8.27</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="N7" t="n">
-        <v>41.98</v>
+        <v>42.51</v>
       </c>
       <c r="O7" t="n">
-        <v>42.06</v>
+        <v>44.82</v>
       </c>
       <c r="P7" t="n">
-        <v>40.68</v>
+        <v>42.44</v>
       </c>
       <c r="Q7" t="n">
-        <v>41.07</v>
+        <v>43.54</v>
       </c>
       <c r="R7" t="n">
-        <v>1.0584</v>
+        <v>-7.571</v>
       </c>
       <c r="S7" t="n">
-        <v>-2.2214</v>
+        <v>-17.6346</v>
       </c>
       <c r="T7" t="n">
-        <v>22.4129</v>
+        <v>-20.3077</v>
       </c>
       <c r="U7" t="n">
-        <v>2.2139</v>
+        <v>-1.3539</v>
       </c>
       <c r="V7" t="n">
-        <v>2.5858</v>
+        <v>-3.7804</v>
       </c>
       <c r="W7" t="n">
-        <v>10.6672</v>
+        <v>-3.4304</v>
       </c>
       <c r="X7" t="n">
-        <v>-0.9581</v>
+        <v>7.8007</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.8537</v>
+        <v>19.1617</v>
       </c>
       <c r="Z7" t="n">
-        <v>-21.9811</v>
+        <v>21.3415</v>
       </c>
       <c r="AA7" t="n">
-        <v>-2.191</v>
+        <v>1.3029</v>
       </c>
       <c r="AB7" t="n">
-        <v>-2.7238</v>
+        <v>3.6914</v>
       </c>
       <c r="AC7" t="n">
-        <v>-10.1902</v>
+        <v>3.1265</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>167</v>
+        <v>141.24</v>
       </c>
       <c r="C8" t="n">
-        <v>174.4</v>
+        <v>160.6</v>
       </c>
       <c r="D8" t="n">
-        <v>161.14</v>
+        <v>135.02</v>
       </c>
       <c r="E8" t="n">
-        <v>164.18</v>
+        <v>151.89</v>
       </c>
       <c r="F8" t="n">
-        <v>75.73</v>
+        <v>72.41</v>
       </c>
       <c r="G8" t="n">
-        <v>77.37</v>
+        <v>74.5</v>
       </c>
       <c r="H8" t="n">
-        <v>74.23</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="I8" t="n">
-        <v>75.34</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>9.130000000000001</v>
+        <v>10.64</v>
       </c>
       <c r="K8" t="n">
-        <v>9.390000000000001</v>
+        <v>11.07</v>
       </c>
       <c r="L8" t="n">
-        <v>8.800000000000001</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>9.23</v>
+        <v>9.93</v>
       </c>
       <c r="N8" t="n">
-        <v>42.77</v>
+        <v>44.68</v>
       </c>
       <c r="O8" t="n">
-        <v>43.57</v>
+        <v>45.53</v>
       </c>
       <c r="P8" t="n">
-        <v>41.93</v>
+        <v>43.46</v>
       </c>
       <c r="Q8" t="n">
-        <v>42.98</v>
+        <v>44.37</v>
       </c>
       <c r="R8" t="n">
-        <v>-11.8213</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="S8" t="n">
-        <v>-4.8342</v>
+        <v>-18.422</v>
       </c>
       <c r="T8" t="n">
-        <v>-7.2115</v>
+        <v>-11.958</v>
       </c>
       <c r="U8" t="n">
-        <v>-4.5725</v>
+        <v>-1.8703</v>
       </c>
       <c r="V8" t="n">
-        <v>0.5069</v>
+        <v>-7.6251</v>
       </c>
       <c r="W8" t="n">
-        <v>-1.2323</v>
+        <v>-2.7081</v>
       </c>
       <c r="X8" t="n">
-        <v>11.6082</v>
+        <v>-0.201</v>
       </c>
       <c r="Y8" t="n">
-        <v>3.1285</v>
+        <v>20.0726</v>
       </c>
       <c r="Z8" t="n">
-        <v>4.2938</v>
+        <v>10.9497</v>
       </c>
       <c r="AA8" t="n">
-        <v>4.6506</v>
+        <v>1.9063</v>
       </c>
       <c r="AB8" t="n">
-        <v>-0.7619</v>
+        <v>8.0351</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.9631</v>
+        <v>2.4475</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>172.95</v>
+        <v>161</v>
       </c>
       <c r="C9" t="n">
-        <v>174.61</v>
+        <v>173.7</v>
       </c>
       <c r="D9" t="n">
-        <v>142.69</v>
+        <v>161</v>
       </c>
       <c r="E9" t="n">
-        <v>151.75</v>
+        <v>173.2</v>
       </c>
       <c r="F9" t="n">
-        <v>76.13</v>
+        <v>74.09</v>
       </c>
       <c r="G9" t="n">
-        <v>76.27</v>
+        <v>76.53</v>
       </c>
       <c r="H9" t="n">
-        <v>72.09999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="I9" t="n">
-        <v>74.31999999999999</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>8.77</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>10.47</v>
+        <v>9.35</v>
       </c>
       <c r="L9" t="n">
-        <v>8.68</v>
+        <v>8.51</v>
       </c>
       <c r="M9" t="n">
-        <v>9.949999999999999</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N9" t="n">
-        <v>42.51</v>
+        <v>43.67</v>
       </c>
       <c r="O9" t="n">
-        <v>44.82</v>
+        <v>43.97</v>
       </c>
       <c r="P9" t="n">
-        <v>42.44</v>
+        <v>42.19</v>
       </c>
       <c r="Q9" t="n">
-        <v>43.54</v>
+        <v>42.19</v>
       </c>
       <c r="R9" t="n">
-        <v>-7.571</v>
+        <v>14.0299</v>
       </c>
       <c r="S9" t="n">
-        <v>-17.6346</v>
+        <v>5.494</v>
       </c>
       <c r="T9" t="n">
-        <v>-20.3077</v>
+        <v>-5.9922</v>
       </c>
       <c r="U9" t="n">
-        <v>-1.3539</v>
+        <v>4.9088</v>
       </c>
       <c r="V9" t="n">
-        <v>-3.7804</v>
+        <v>1.553</v>
       </c>
       <c r="W9" t="n">
-        <v>-3.4304</v>
+        <v>-0.9451000000000001</v>
       </c>
       <c r="X9" t="n">
-        <v>7.8007</v>
+        <v>-13.998</v>
       </c>
       <c r="Y9" t="n">
-        <v>19.1617</v>
+        <v>-7.4756</v>
       </c>
       <c r="Z9" t="n">
-        <v>21.3415</v>
+        <v>2.2754</v>
       </c>
       <c r="AA9" t="n">
-        <v>1.3029</v>
+        <v>-4.9132</v>
       </c>
       <c r="AB9" t="n">
-        <v>3.6914</v>
+        <v>-1.8381</v>
       </c>
       <c r="AC9" t="n">
-        <v>3.1265</v>
+        <v>0.4763</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>141.24</v>
+        <v>171.26</v>
       </c>
       <c r="C10" t="n">
-        <v>160.6</v>
+        <v>179.97</v>
       </c>
       <c r="D10" t="n">
-        <v>135.02</v>
+        <v>168.23</v>
       </c>
       <c r="E10" t="n">
-        <v>151.89</v>
+        <v>178.39</v>
       </c>
       <c r="F10" t="n">
-        <v>72.41</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>74.5</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>70.95999999999999</v>
+        <v>74.47</v>
       </c>
       <c r="I10" t="n">
-        <v>72.93000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J10" t="n">
-        <v>10.64</v>
+        <v>8.65</v>
       </c>
       <c r="K10" t="n">
-        <v>11.07</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L10" t="n">
-        <v>9.369999999999999</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M10" t="n">
-        <v>9.93</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N10" t="n">
-        <v>44.68</v>
+        <v>42.94</v>
       </c>
       <c r="O10" t="n">
-        <v>45.53</v>
+        <v>43.33</v>
       </c>
       <c r="P10" t="n">
-        <v>43.46</v>
+        <v>41.5</v>
       </c>
       <c r="Q10" t="n">
-        <v>44.37</v>
+        <v>41.96</v>
       </c>
       <c r="R10" t="n">
-        <v>0.09229999999999999</v>
+        <v>2.9965</v>
       </c>
       <c r="S10" t="n">
-        <v>-18.422</v>
+        <v>17.5552</v>
       </c>
       <c r="T10" t="n">
-        <v>-11.958</v>
+        <v>-4.1893</v>
       </c>
       <c r="U10" t="n">
-        <v>-1.8703</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="V10" t="n">
-        <v>-7.6251</v>
+        <v>3.5388</v>
       </c>
       <c r="W10" t="n">
-        <v>-2.7081</v>
+        <v>-2.5332</v>
       </c>
       <c r="X10" t="n">
-        <v>-0.201</v>
+        <v>-2.9274</v>
       </c>
       <c r="Y10" t="n">
-        <v>20.0726</v>
+        <v>-16.6834</v>
       </c>
       <c r="Z10" t="n">
-        <v>10.9497</v>
+        <v>0.2418</v>
       </c>
       <c r="AA10" t="n">
-        <v>1.9063</v>
+        <v>-0.5452</v>
       </c>
       <c r="AB10" t="n">
-        <v>8.0351</v>
+        <v>-3.6288</v>
       </c>
       <c r="AC10" t="n">
-        <v>2.4475</v>
+        <v>2.167</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>161</v>
+        <v>184.8</v>
       </c>
       <c r="C11" t="n">
-        <v>173.7</v>
+        <v>195.27</v>
       </c>
       <c r="D11" t="n">
-        <v>161</v>
+        <v>183.34</v>
       </c>
       <c r="E11" t="n">
-        <v>173.2</v>
+        <v>190.56</v>
       </c>
       <c r="F11" t="n">
-        <v>74.09</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>76.53</v>
+        <v>79.33</v>
       </c>
       <c r="H11" t="n">
-        <v>73.62</v>
+        <v>77.33</v>
       </c>
       <c r="I11" t="n">
-        <v>76.51000000000001</v>
+        <v>77.84</v>
       </c>
       <c r="J11" t="n">
-        <v>9.300000000000001</v>
+        <v>8</v>
       </c>
       <c r="K11" t="n">
-        <v>9.35</v>
+        <v>8.06</v>
       </c>
       <c r="L11" t="n">
-        <v>8.51</v>
+        <v>7.5</v>
       </c>
       <c r="M11" t="n">
-        <v>8.539999999999999</v>
+        <v>7.73</v>
       </c>
       <c r="N11" t="n">
-        <v>43.67</v>
+        <v>41.4</v>
       </c>
       <c r="O11" t="n">
-        <v>43.97</v>
+        <v>41.78</v>
       </c>
       <c r="P11" t="n">
-        <v>42.19</v>
+        <v>40.68</v>
       </c>
       <c r="Q11" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="R11" t="n">
-        <v>14.0299</v>
+        <v>6.8221</v>
       </c>
       <c r="S11" t="n">
-        <v>5.494</v>
+        <v>25.4592</v>
       </c>
       <c r="T11" t="n">
-        <v>-5.9922</v>
+        <v>16.0677</v>
       </c>
       <c r="U11" t="n">
-        <v>4.9088</v>
+        <v>1.1566</v>
       </c>
       <c r="V11" t="n">
-        <v>1.553</v>
+        <v>6.7325</v>
       </c>
       <c r="W11" t="n">
-        <v>-0.9451000000000001</v>
+        <v>3.3183</v>
       </c>
       <c r="X11" t="n">
-        <v>-13.998</v>
+        <v>-6.7551</v>
       </c>
       <c r="Y11" t="n">
-        <v>-7.4756</v>
+        <v>-22.1551</v>
       </c>
       <c r="Z11" t="n">
-        <v>2.2754</v>
+        <v>-16.2514</v>
       </c>
       <c r="AA11" t="n">
-        <v>-4.9132</v>
+        <v>-1.0963</v>
       </c>
       <c r="AB11" t="n">
-        <v>-1.8381</v>
+        <v>-6.4683</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.4763</v>
+        <v>-3.4435</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>171.26</v>
+        <v>211.38</v>
       </c>
       <c r="C12" t="n">
-        <v>179.97</v>
+        <v>228.5</v>
       </c>
       <c r="D12" t="n">
-        <v>168.23</v>
+        <v>209.89</v>
       </c>
       <c r="E12" t="n">
-        <v>178.39</v>
+        <v>225.79</v>
       </c>
       <c r="F12" t="n">
-        <v>75.18000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="G12" t="n">
-        <v>77.79000000000001</v>
+        <v>82.27</v>
       </c>
       <c r="H12" t="n">
-        <v>74.47</v>
+        <v>79.98</v>
       </c>
       <c r="I12" t="n">
-        <v>76.95</v>
+        <v>81.95</v>
       </c>
       <c r="J12" t="n">
-        <v>8.65</v>
+        <v>6.9</v>
       </c>
       <c r="K12" t="n">
-        <v>8.779999999999999</v>
+        <v>6.95</v>
       </c>
       <c r="L12" t="n">
-        <v>8.210000000000001</v>
+        <v>6.19</v>
       </c>
       <c r="M12" t="n">
-        <v>8.289999999999999</v>
+        <v>6.29</v>
       </c>
       <c r="N12" t="n">
-        <v>42.94</v>
+        <v>40.05</v>
       </c>
       <c r="O12" t="n">
-        <v>43.33</v>
+        <v>40.35</v>
       </c>
       <c r="P12" t="n">
-        <v>41.5</v>
+        <v>39.14</v>
       </c>
       <c r="Q12" t="n">
-        <v>41.96</v>
+        <v>39.28</v>
       </c>
       <c r="R12" t="n">
-        <v>2.9965</v>
+        <v>18.4876</v>
       </c>
       <c r="S12" t="n">
-        <v>17.5552</v>
+        <v>30.3637</v>
       </c>
       <c r="T12" t="n">
-        <v>-4.1893</v>
+        <v>48.7908</v>
       </c>
       <c r="U12" t="n">
-        <v>0.5750999999999999</v>
+        <v>5.2801</v>
       </c>
       <c r="V12" t="n">
-        <v>3.5388</v>
+        <v>7.1102</v>
       </c>
       <c r="W12" t="n">
-        <v>-2.5332</v>
+        <v>10.2664</v>
       </c>
       <c r="X12" t="n">
-        <v>-2.9274</v>
+        <v>-18.6287</v>
       </c>
       <c r="Y12" t="n">
-        <v>-16.6834</v>
+        <v>-26.3466</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.2418</v>
+        <v>-36.7839</v>
       </c>
       <c r="AA12" t="n">
-        <v>-0.5452</v>
+        <v>-5.3494</v>
       </c>
       <c r="AB12" t="n">
-        <v>-3.6288</v>
+        <v>-6.8974</v>
       </c>
       <c r="AC12" t="n">
-        <v>2.167</v>
+        <v>-9.7841</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>184.8</v>
+        <v>242.66</v>
       </c>
       <c r="C13" t="n">
-        <v>195.27</v>
+        <v>242.66</v>
       </c>
       <c r="D13" t="n">
-        <v>183.34</v>
+        <v>204</v>
       </c>
       <c r="E13" t="n">
-        <v>190.56</v>
+        <v>217.98</v>
       </c>
       <c r="F13" t="n">
-        <v>78.04000000000001</v>
+        <v>82.87</v>
       </c>
       <c r="G13" t="n">
-        <v>79.33</v>
+        <v>82.91</v>
       </c>
       <c r="H13" t="n">
-        <v>77.33</v>
+        <v>80.33</v>
       </c>
       <c r="I13" t="n">
-        <v>77.84</v>
+        <v>81.67</v>
       </c>
       <c r="J13" t="n">
-        <v>8</v>
+        <v>5.83</v>
       </c>
       <c r="K13" t="n">
-        <v>8.06</v>
+        <v>6.91</v>
       </c>
       <c r="L13" t="n">
-        <v>7.5</v>
+        <v>5.83</v>
       </c>
       <c r="M13" t="n">
-        <v>7.73</v>
+        <v>6.53</v>
       </c>
       <c r="N13" t="n">
-        <v>41.4</v>
+        <v>38.87</v>
       </c>
       <c r="O13" t="n">
-        <v>41.78</v>
+        <v>40.09</v>
       </c>
       <c r="P13" t="n">
-        <v>40.68</v>
+        <v>38.86</v>
       </c>
       <c r="Q13" t="n">
-        <v>41.5</v>
+        <v>39.44</v>
       </c>
       <c r="R13" t="n">
-        <v>6.8221</v>
+        <v>-3.459</v>
       </c>
       <c r="S13" t="n">
-        <v>25.4592</v>
+        <v>22.1929</v>
       </c>
       <c r="T13" t="n">
-        <v>16.0677</v>
+        <v>43.5118</v>
       </c>
       <c r="U13" t="n">
-        <v>1.1566</v>
+        <v>-0.3417</v>
       </c>
       <c r="V13" t="n">
-        <v>6.7325</v>
+        <v>6.1339</v>
       </c>
       <c r="W13" t="n">
-        <v>3.3183</v>
+        <v>11.9841</v>
       </c>
       <c r="X13" t="n">
-        <v>-6.7551</v>
+        <v>3.8156</v>
       </c>
       <c r="Y13" t="n">
-        <v>-22.1551</v>
+        <v>-21.2304</v>
       </c>
       <c r="Z13" t="n">
-        <v>-16.2514</v>
+        <v>-34.2397</v>
       </c>
       <c r="AA13" t="n">
-        <v>-1.0963</v>
+        <v>0.4073</v>
       </c>
       <c r="AB13" t="n">
-        <v>-6.4683</v>
+        <v>-6.0057</v>
       </c>
       <c r="AC13" t="n">
-        <v>-3.4435</v>
+        <v>-11.1111</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>211.38</v>
+        <v>219</v>
       </c>
       <c r="C14" t="n">
-        <v>228.5</v>
+        <v>231.89</v>
       </c>
       <c r="D14" t="n">
-        <v>209.89</v>
+        <v>207.56</v>
       </c>
       <c r="E14" t="n">
-        <v>225.79</v>
+        <v>224.63</v>
       </c>
       <c r="F14" t="n">
-        <v>80.59</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>82.27</v>
+        <v>84.05</v>
       </c>
       <c r="H14" t="n">
-        <v>79.98</v>
+        <v>80.66</v>
       </c>
       <c r="I14" t="n">
-        <v>81.95</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="J14" t="n">
-        <v>6.9</v>
+        <v>6.49</v>
       </c>
       <c r="K14" t="n">
-        <v>6.95</v>
+        <v>6.83</v>
       </c>
       <c r="L14" t="n">
-        <v>6.19</v>
+        <v>6.1</v>
       </c>
       <c r="M14" t="n">
-        <v>6.29</v>
+        <v>6.31</v>
       </c>
       <c r="N14" t="n">
-        <v>40.05</v>
+        <v>39.41</v>
       </c>
       <c r="O14" t="n">
-        <v>40.35</v>
+        <v>39.94</v>
       </c>
       <c r="P14" t="n">
-        <v>39.14</v>
+        <v>38.3</v>
       </c>
       <c r="Q14" t="n">
-        <v>39.28</v>
+        <v>38.47</v>
       </c>
       <c r="R14" t="n">
-        <v>18.4876</v>
+        <v>3.0507</v>
       </c>
       <c r="S14" t="n">
-        <v>30.3637</v>
+        <v>17.8789</v>
       </c>
       <c r="T14" t="n">
-        <v>48.7908</v>
+        <v>29.694</v>
       </c>
       <c r="U14" t="n">
-        <v>5.2801</v>
+        <v>2.4611</v>
       </c>
       <c r="V14" t="n">
-        <v>7.1102</v>
+        <v>7.5026</v>
       </c>
       <c r="W14" t="n">
-        <v>10.2664</v>
+        <v>9.3713</v>
       </c>
       <c r="X14" t="n">
-        <v>-18.6287</v>
+        <v>-3.3691</v>
       </c>
       <c r="Y14" t="n">
-        <v>-26.3466</v>
+        <v>-18.37</v>
       </c>
       <c r="Z14" t="n">
-        <v>-36.7839</v>
+        <v>-26.1124</v>
       </c>
       <c r="AA14" t="n">
-        <v>-5.3494</v>
+        <v>-2.4594</v>
       </c>
       <c r="AB14" t="n">
-        <v>-6.8974</v>
+        <v>-7.3012</v>
       </c>
       <c r="AC14" t="n">
-        <v>-9.7841</v>
+        <v>-8.817299999999999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>242.66</v>
+        <v>231.82</v>
       </c>
       <c r="C15" t="n">
-        <v>242.66</v>
+        <v>239.07</v>
       </c>
       <c r="D15" t="n">
-        <v>204</v>
+        <v>218.56</v>
       </c>
       <c r="E15" t="n">
-        <v>217.98</v>
+        <v>224.34</v>
       </c>
       <c r="F15" t="n">
-        <v>82.87</v>
+        <v>84.41</v>
       </c>
       <c r="G15" t="n">
-        <v>82.91</v>
+        <v>85.7</v>
       </c>
       <c r="H15" t="n">
-        <v>80.33</v>
+        <v>83.53</v>
       </c>
       <c r="I15" t="n">
-        <v>81.67</v>
+        <v>84.56</v>
       </c>
       <c r="J15" t="n">
-        <v>5.83</v>
+        <v>6.11</v>
       </c>
       <c r="K15" t="n">
-        <v>6.91</v>
+        <v>6.49</v>
       </c>
       <c r="L15" t="n">
-        <v>5.83</v>
+        <v>5.91</v>
       </c>
       <c r="M15" t="n">
-        <v>6.53</v>
+        <v>6.33</v>
       </c>
       <c r="N15" t="n">
-        <v>38.87</v>
+        <v>38.15</v>
       </c>
       <c r="O15" t="n">
-        <v>40.09</v>
+        <v>38.56</v>
       </c>
       <c r="P15" t="n">
-        <v>38.86</v>
+        <v>37.56</v>
       </c>
       <c r="Q15" t="n">
-        <v>39.44</v>
+        <v>38.08</v>
       </c>
       <c r="R15" t="n">
-        <v>-3.459</v>
+        <v>-0.1291</v>
       </c>
       <c r="S15" t="n">
-        <v>22.1929</v>
+        <v>-0.6422</v>
       </c>
       <c r="T15" t="n">
-        <v>43.5118</v>
+        <v>25.7582</v>
       </c>
       <c r="U15" t="n">
-        <v>-0.3417</v>
+        <v>1.0516</v>
       </c>
       <c r="V15" t="n">
-        <v>6.1339</v>
+        <v>3.1849</v>
       </c>
       <c r="W15" t="n">
-        <v>11.9841</v>
+        <v>9.8895</v>
       </c>
       <c r="X15" t="n">
-        <v>3.8156</v>
+        <v>0.317</v>
       </c>
       <c r="Y15" t="n">
-        <v>-21.2304</v>
+        <v>0.6359</v>
       </c>
       <c r="Z15" t="n">
-        <v>-34.2397</v>
+        <v>-23.6429</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.4073</v>
+        <v>-1.0138</v>
       </c>
       <c r="AB15" t="n">
-        <v>-6.0057</v>
+        <v>-3.055</v>
       </c>
       <c r="AC15" t="n">
-        <v>-11.1111</v>
+        <v>-9.2469</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>219</v>
+        <v>217.27</v>
       </c>
       <c r="C16" t="n">
-        <v>231.89</v>
+        <v>234.06</v>
       </c>
       <c r="D16" t="n">
-        <v>207.56</v>
+        <v>210.14</v>
       </c>
       <c r="E16" t="n">
-        <v>224.63</v>
+        <v>227.03</v>
       </c>
       <c r="F16" t="n">
-        <v>81.73999999999999</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>84.05</v>
+        <v>87.06</v>
       </c>
       <c r="H16" t="n">
-        <v>80.66</v>
+        <v>83.75</v>
       </c>
       <c r="I16" t="n">
-        <v>83.68000000000001</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="J16" t="n">
-        <v>6.49</v>
+        <v>6.55</v>
       </c>
       <c r="K16" t="n">
-        <v>6.83</v>
+        <v>6.74</v>
       </c>
       <c r="L16" t="n">
-        <v>6.1</v>
+        <v>6.05</v>
       </c>
       <c r="M16" t="n">
-        <v>6.31</v>
+        <v>6.26</v>
       </c>
       <c r="N16" t="n">
-        <v>39.41</v>
+        <v>38.27</v>
       </c>
       <c r="O16" t="n">
-        <v>39.94</v>
+        <v>38.46</v>
       </c>
       <c r="P16" t="n">
-        <v>38.3</v>
+        <v>36.96</v>
       </c>
       <c r="Q16" t="n">
-        <v>38.47</v>
+        <v>37.42</v>
       </c>
       <c r="R16" t="n">
-        <v>3.0507</v>
+        <v>1.1991</v>
       </c>
       <c r="S16" t="n">
-        <v>17.8789</v>
+        <v>4.1518</v>
       </c>
       <c r="T16" t="n">
-        <v>29.694</v>
+        <v>19.1383</v>
       </c>
       <c r="U16" t="n">
-        <v>2.4611</v>
+        <v>1.7502</v>
       </c>
       <c r="V16" t="n">
-        <v>7.5026</v>
+        <v>5.3508</v>
       </c>
       <c r="W16" t="n">
-        <v>9.3713</v>
+        <v>10.5344</v>
       </c>
       <c r="X16" t="n">
-        <v>-3.3691</v>
+        <v>-1.1058</v>
       </c>
       <c r="Y16" t="n">
-        <v>-18.37</v>
+        <v>-4.1348</v>
       </c>
       <c r="Z16" t="n">
-        <v>-26.1124</v>
+        <v>-19.0168</v>
       </c>
       <c r="AA16" t="n">
-        <v>-2.4594</v>
+        <v>-1.7332</v>
       </c>
       <c r="AB16" t="n">
-        <v>-7.3012</v>
+        <v>-5.1217</v>
       </c>
       <c r="AC16" t="n">
-        <v>-8.817299999999999</v>
+        <v>-9.831300000000001</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>231.82</v>
+        <v>243.18</v>
       </c>
       <c r="C17" t="n">
-        <v>239.07</v>
+        <v>267.08</v>
       </c>
       <c r="D17" t="n">
-        <v>218.56</v>
+        <v>238.82</v>
       </c>
       <c r="E17" t="n">
-        <v>224.34</v>
+        <v>266.32</v>
       </c>
       <c r="F17" t="n">
-        <v>84.41</v>
+        <v>85.94</v>
       </c>
       <c r="G17" t="n">
-        <v>85.7</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="H17" t="n">
-        <v>83.53</v>
+        <v>84.83</v>
       </c>
       <c r="I17" t="n">
-        <v>84.56</v>
+        <v>87.22</v>
       </c>
       <c r="J17" t="n">
-        <v>6.11</v>
+        <v>5.8</v>
       </c>
       <c r="K17" t="n">
-        <v>6.49</v>
+        <v>5.93</v>
       </c>
       <c r="L17" t="n">
-        <v>5.91</v>
+        <v>5.15</v>
       </c>
       <c r="M17" t="n">
-        <v>6.33</v>
+        <v>5.17</v>
       </c>
       <c r="N17" t="n">
-        <v>38.15</v>
+        <v>37.47</v>
       </c>
       <c r="O17" t="n">
-        <v>38.56</v>
+        <v>37.95</v>
       </c>
       <c r="P17" t="n">
-        <v>37.56</v>
+        <v>36.86</v>
       </c>
       <c r="Q17" t="n">
-        <v>38.08</v>
+        <v>36.91</v>
       </c>
       <c r="R17" t="n">
-        <v>-0.1291</v>
+        <v>17.3061</v>
       </c>
       <c r="S17" t="n">
-        <v>-0.6422</v>
+        <v>18.5594</v>
       </c>
       <c r="T17" t="n">
-        <v>25.7582</v>
+        <v>17.9503</v>
       </c>
       <c r="U17" t="n">
-        <v>1.0516</v>
+        <v>1.3715</v>
       </c>
       <c r="V17" t="n">
-        <v>3.1849</v>
+        <v>4.2304</v>
       </c>
       <c r="W17" t="n">
-        <v>9.8895</v>
+        <v>6.4308</v>
       </c>
       <c r="X17" t="n">
-        <v>0.317</v>
+        <v>-17.4121</v>
       </c>
       <c r="Y17" t="n">
-        <v>0.6359</v>
+        <v>-18.0666</v>
       </c>
       <c r="Z17" t="n">
-        <v>-23.6429</v>
+        <v>-17.806</v>
       </c>
       <c r="AA17" t="n">
-        <v>-1.0138</v>
+        <v>-1.3629</v>
       </c>
       <c r="AB17" t="n">
-        <v>-3.055</v>
+        <v>-4.0551</v>
       </c>
       <c r="AC17" t="n">
-        <v>-9.2469</v>
+        <v>-6.0336</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>217.27</v>
+        <v>281.47</v>
       </c>
       <c r="C18" t="n">
-        <v>234.06</v>
+        <v>284.58</v>
       </c>
       <c r="D18" t="n">
-        <v>210.14</v>
+        <v>257.26</v>
       </c>
       <c r="E18" t="n">
-        <v>227.03</v>
+        <v>280.54</v>
       </c>
       <c r="F18" t="n">
-        <v>84.15000000000001</v>
+        <v>87.68000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>87.06</v>
+        <v>88.09</v>
       </c>
       <c r="H18" t="n">
-        <v>83.75</v>
+        <v>85.41</v>
       </c>
       <c r="I18" t="n">
-        <v>86.04000000000001</v>
+        <v>86.56</v>
       </c>
       <c r="J18" t="n">
-        <v>6.55</v>
+        <v>4.88</v>
       </c>
       <c r="K18" t="n">
-        <v>6.74</v>
+        <v>5.35</v>
       </c>
       <c r="L18" t="n">
-        <v>6.05</v>
+        <v>4.82</v>
       </c>
       <c r="M18" t="n">
-        <v>6.26</v>
+        <v>4.91</v>
       </c>
       <c r="N18" t="n">
-        <v>38.27</v>
+        <v>36.73</v>
       </c>
       <c r="O18" t="n">
-        <v>38.46</v>
+        <v>37.69</v>
       </c>
       <c r="P18" t="n">
-        <v>36.96</v>
+        <v>36.55</v>
       </c>
       <c r="Q18" t="n">
-        <v>37.42</v>
+        <v>37.19</v>
       </c>
       <c r="R18" t="n">
-        <v>1.1991</v>
+        <v>5.3394</v>
       </c>
       <c r="S18" t="n">
-        <v>4.1518</v>
+        <v>25.0513</v>
       </c>
       <c r="T18" t="n">
-        <v>19.1383</v>
+        <v>28.6999</v>
       </c>
       <c r="U18" t="n">
-        <v>1.7502</v>
+        <v>-0.7567</v>
       </c>
       <c r="V18" t="n">
-        <v>5.3508</v>
+        <v>2.3652</v>
       </c>
       <c r="W18" t="n">
-        <v>10.5344</v>
+        <v>5.9875</v>
       </c>
       <c r="X18" t="n">
-        <v>-1.1058</v>
+        <v>-5.029</v>
       </c>
       <c r="Y18" t="n">
-        <v>-4.1348</v>
+        <v>-22.4329</v>
       </c>
       <c r="Z18" t="n">
-        <v>-19.0168</v>
+        <v>-24.8086</v>
       </c>
       <c r="AA18" t="n">
-        <v>-1.7332</v>
+        <v>0.7586000000000001</v>
       </c>
       <c r="AB18" t="n">
-        <v>-5.1217</v>
+        <v>-2.3372</v>
       </c>
       <c r="AC18" t="n">
-        <v>-9.831300000000001</v>
+        <v>-5.7049</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>243.18</v>
+        <v>242.04</v>
       </c>
       <c r="C19" t="n">
-        <v>267.08</v>
+        <v>274.5</v>
       </c>
       <c r="D19" t="n">
-        <v>238.82</v>
+        <v>228.55</v>
       </c>
       <c r="E19" t="n">
-        <v>266.32</v>
+        <v>262.7</v>
       </c>
       <c r="F19" t="n">
-        <v>85.94</v>
+        <v>83.47</v>
       </c>
       <c r="G19" t="n">
-        <v>87.31999999999999</v>
+        <v>86.25</v>
       </c>
       <c r="H19" t="n">
-        <v>84.83</v>
+        <v>82.48</v>
       </c>
       <c r="I19" t="n">
-        <v>87.22</v>
+        <v>85.22</v>
       </c>
       <c r="J19" t="n">
-        <v>5.8</v>
+        <v>5.57</v>
       </c>
       <c r="K19" t="n">
-        <v>5.93</v>
+        <v>5.81</v>
       </c>
       <c r="L19" t="n">
-        <v>5.15</v>
+        <v>5</v>
       </c>
       <c r="M19" t="n">
-        <v>5.17</v>
+        <v>5.2</v>
       </c>
       <c r="N19" t="n">
-        <v>37.47</v>
+        <v>38.53</v>
       </c>
       <c r="O19" t="n">
-        <v>37.95</v>
+        <v>38.96</v>
       </c>
       <c r="P19" t="n">
-        <v>36.86</v>
+        <v>37.33</v>
       </c>
       <c r="Q19" t="n">
-        <v>36.91</v>
+        <v>37.76</v>
       </c>
       <c r="R19" t="n">
-        <v>17.3061</v>
+        <v>-6.3592</v>
       </c>
       <c r="S19" t="n">
-        <v>18.5594</v>
+        <v>15.7116</v>
       </c>
       <c r="T19" t="n">
-        <v>17.9503</v>
+        <v>16.9479</v>
       </c>
       <c r="U19" t="n">
-        <v>1.3715</v>
+        <v>-1.5481</v>
       </c>
       <c r="V19" t="n">
-        <v>4.2304</v>
+        <v>-0.953</v>
       </c>
       <c r="W19" t="n">
-        <v>6.4308</v>
+        <v>1.8403</v>
       </c>
       <c r="X19" t="n">
-        <v>-17.4121</v>
+        <v>5.9063</v>
       </c>
       <c r="Y19" t="n">
-        <v>-18.0666</v>
+        <v>-16.9329</v>
       </c>
       <c r="Z19" t="n">
-        <v>-17.806</v>
+        <v>-17.5911</v>
       </c>
       <c r="AA19" t="n">
-        <v>-1.3629</v>
+        <v>1.5327</v>
       </c>
       <c r="AB19" t="n">
-        <v>-4.0551</v>
+        <v>0.9086</v>
       </c>
       <c r="AC19" t="n">
-        <v>-6.0336</v>
+        <v>-1.8456</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>281.47</v>
+        <v>230.85</v>
       </c>
       <c r="C20" t="n">
-        <v>284.58</v>
+        <v>233.69</v>
       </c>
       <c r="D20" t="n">
-        <v>257.26</v>
+        <v>181.81</v>
       </c>
       <c r="E20" t="n">
-        <v>280.54</v>
+        <v>182.54</v>
       </c>
       <c r="F20" t="n">
-        <v>87.68000000000001</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="G20" t="n">
-        <v>88.09</v>
+        <v>82.08</v>
       </c>
       <c r="H20" t="n">
-        <v>85.41</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>86.56</v>
+        <v>73.05</v>
       </c>
       <c r="J20" t="n">
-        <v>4.88</v>
+        <v>5.86</v>
       </c>
       <c r="K20" t="n">
-        <v>5.35</v>
+        <v>6.85</v>
       </c>
       <c r="L20" t="n">
-        <v>4.82</v>
+        <v>5.79</v>
       </c>
       <c r="M20" t="n">
-        <v>4.91</v>
+        <v>6.84</v>
       </c>
       <c r="N20" t="n">
-        <v>36.73</v>
+        <v>39.42</v>
       </c>
       <c r="O20" t="n">
-        <v>37.69</v>
+        <v>43.35</v>
       </c>
       <c r="P20" t="n">
-        <v>36.55</v>
+        <v>39.18</v>
       </c>
       <c r="Q20" t="n">
-        <v>37.19</v>
+        <v>43.19</v>
       </c>
       <c r="R20" t="n">
-        <v>5.3394</v>
+        <v>-30.5139</v>
       </c>
       <c r="S20" t="n">
-        <v>25.0513</v>
+        <v>-31.4584</v>
       </c>
       <c r="T20" t="n">
-        <v>28.6999</v>
+        <v>-18.6324</v>
       </c>
       <c r="U20" t="n">
-        <v>-0.7567</v>
+        <v>-14.2807</v>
       </c>
       <c r="V20" t="n">
-        <v>2.3652</v>
+        <v>-16.2463</v>
       </c>
       <c r="W20" t="n">
-        <v>5.9875</v>
+        <v>-13.6116</v>
       </c>
       <c r="X20" t="n">
-        <v>-5.029</v>
+        <v>31.5385</v>
       </c>
       <c r="Y20" t="n">
-        <v>-22.4329</v>
+        <v>32.3017</v>
       </c>
       <c r="Z20" t="n">
-        <v>-24.8086</v>
+        <v>8.056900000000001</v>
       </c>
       <c r="AA20" t="n">
-        <v>0.7586000000000001</v>
+        <v>14.3803</v>
       </c>
       <c r="AB20" t="n">
-        <v>-2.3372</v>
+        <v>17.0144</v>
       </c>
       <c r="AC20" t="n">
-        <v>-5.7049</v>
+        <v>13.4191</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>242.04</v>
+        <v>210.62</v>
       </c>
       <c r="C21" t="n">
-        <v>274.5</v>
+        <v>222.19</v>
       </c>
       <c r="D21" t="n">
-        <v>228.55</v>
+        <v>201.69</v>
       </c>
       <c r="E21" t="n">
-        <v>262.7</v>
+        <v>211.44</v>
       </c>
       <c r="F21" t="n">
-        <v>83.47</v>
+        <v>76.86</v>
       </c>
       <c r="G21" t="n">
-        <v>86.25</v>
+        <v>78.47</v>
       </c>
       <c r="H21" t="n">
-        <v>82.48</v>
+        <v>75.38</v>
       </c>
       <c r="I21" t="n">
-        <v>85.22</v>
+        <v>76.27</v>
       </c>
       <c r="J21" t="n">
-        <v>5.57</v>
+        <v>5.71</v>
       </c>
       <c r="K21" t="n">
-        <v>5.81</v>
+        <v>6.05</v>
       </c>
       <c r="L21" t="n">
-        <v>5</v>
+        <v>5.27</v>
       </c>
       <c r="M21" t="n">
-        <v>5.2</v>
+        <v>5.69</v>
       </c>
       <c r="N21" t="n">
-        <v>38.53</v>
+        <v>40.925</v>
       </c>
       <c r="O21" t="n">
-        <v>38.96</v>
+        <v>41.78</v>
       </c>
       <c r="P21" t="n">
-        <v>37.33</v>
+        <v>39.96</v>
       </c>
       <c r="Q21" t="n">
-        <v>37.76</v>
+        <v>41.26</v>
       </c>
       <c r="R21" t="n">
-        <v>-6.3592</v>
+        <v>15.8321</v>
       </c>
       <c r="S21" t="n">
-        <v>15.7116</v>
+        <v>-24.6311</v>
       </c>
       <c r="T21" t="n">
-        <v>16.9479</v>
+        <v>-6.8669</v>
       </c>
       <c r="U21" t="n">
-        <v>-1.5481</v>
+        <v>4.4079</v>
       </c>
       <c r="V21" t="n">
-        <v>-0.953</v>
+        <v>-11.8877</v>
       </c>
       <c r="W21" t="n">
-        <v>1.8403</v>
+        <v>-11.3552</v>
       </c>
       <c r="X21" t="n">
-        <v>5.9063</v>
+        <v>-16.8129</v>
       </c>
       <c r="Y21" t="n">
-        <v>-16.9329</v>
+        <v>15.8859</v>
       </c>
       <c r="Z21" t="n">
-        <v>-17.5911</v>
+        <v>-9.105399999999999</v>
       </c>
       <c r="AA21" t="n">
-        <v>1.5327</v>
+        <v>-4.4686</v>
       </c>
       <c r="AB21" t="n">
-        <v>0.9086</v>
+        <v>10.9438</v>
       </c>
       <c r="AC21" t="n">
-        <v>-1.8456</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-06-05</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>230.8482</v>
-      </c>
-      <c r="C22" t="n">
-        <v>233.69</v>
-      </c>
-      <c r="D22" t="n">
-        <v>182.0033</v>
-      </c>
-      <c r="E22" t="n">
-        <v>182.54</v>
-      </c>
-      <c r="F22" t="n">
-        <v>81.55</v>
-      </c>
-      <c r="G22" t="n">
-        <v>82.08</v>
-      </c>
-      <c r="H22" t="n">
-        <v>72.68000000000001</v>
-      </c>
-      <c r="I22" t="n">
-        <v>73.05</v>
-      </c>
-      <c r="J22" t="n">
-        <v>5.855</v>
-      </c>
-      <c r="K22" t="n">
-        <v>6.85</v>
-      </c>
-      <c r="L22" t="n">
-        <v>5.79</v>
-      </c>
-      <c r="M22" t="n">
-        <v>6.84</v>
-      </c>
-      <c r="N22" t="n">
-        <v>39.45</v>
-      </c>
-      <c r="O22" t="n">
-        <v>43.35</v>
-      </c>
-      <c r="P22" t="n">
-        <v>39.185</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>43.19</v>
-      </c>
-      <c r="R22" t="n">
-        <v>-30.5139</v>
-      </c>
-      <c r="S22" t="n">
-        <v>-31.4584</v>
-      </c>
-      <c r="T22" t="n">
-        <v>-18.6324</v>
-      </c>
-      <c r="U22" t="n">
-        <v>-14.2807</v>
-      </c>
-      <c r="V22" t="n">
-        <v>-16.2463</v>
-      </c>
-      <c r="W22" t="n">
-        <v>-13.6116</v>
-      </c>
-      <c r="X22" t="n">
-        <v>31.5385</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>32.3017</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>8.056900000000001</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>14.3803</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>17.0144</v>
-      </c>
-      <c r="AC22" t="n">
-        <v>13.4191</v>
+        <v>10.2619</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-09 23:17
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC21"/>
+  <dimension ref="A1:AC22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2229,7 +2229,7 @@
         <v>5.69</v>
       </c>
       <c r="N21" t="n">
-        <v>40.925</v>
+        <v>40.92</v>
       </c>
       <c r="O21" t="n">
         <v>41.78</v>
@@ -2275,6 +2275,97 @@
       </c>
       <c r="AC21" t="n">
         <v>10.2619</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>227.055</v>
+      </c>
+      <c r="C22" t="n">
+        <v>231.01</v>
+      </c>
+      <c r="D22" t="n">
+        <v>157.561</v>
+      </c>
+      <c r="E22" t="n">
+        <v>201.68</v>
+      </c>
+      <c r="F22" t="n">
+        <v>78.48</v>
+      </c>
+      <c r="G22" t="n">
+        <v>79.3407</v>
+      </c>
+      <c r="H22" t="n">
+        <v>66.79000000000001</v>
+      </c>
+      <c r="I22" t="n">
+        <v>73.72</v>
+      </c>
+      <c r="J22" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="K22" t="n">
+        <v>7.11</v>
+      </c>
+      <c r="L22" t="n">
+        <v>5.14</v>
+      </c>
+      <c r="M22" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="N22" t="n">
+        <v>40.07</v>
+      </c>
+      <c r="O22" t="n">
+        <v>46.38</v>
+      </c>
+      <c r="P22" t="n">
+        <v>39.5936</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>42.67</v>
+      </c>
+      <c r="R22" t="n">
+        <v>-4.616</v>
+      </c>
+      <c r="S22" t="n">
+        <v>-23.228</v>
+      </c>
+      <c r="T22" t="n">
+        <v>-24.2716</v>
+      </c>
+      <c r="U22" t="n">
+        <v>-3.3434</v>
+      </c>
+      <c r="V22" t="n">
+        <v>-13.4945</v>
+      </c>
+      <c r="W22" t="n">
+        <v>-15.4781</v>
+      </c>
+      <c r="X22" t="n">
+        <v>4.2179</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>14.0385</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>14.7002</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>3.4174</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>13.0032</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>15.6055</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-10 23:25
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>181</v>
+        <v>177.62</v>
       </c>
       <c r="C2" t="n">
-        <v>191.29</v>
+        <v>182.24</v>
       </c>
       <c r="D2" t="n">
-        <v>178.94</v>
+        <v>150.58</v>
       </c>
       <c r="E2" t="n">
-        <v>190.42</v>
+        <v>172.52</v>
       </c>
       <c r="F2" t="n">
-        <v>76</v>
+        <v>75.3</v>
       </c>
       <c r="G2" t="n">
-        <v>77.36</v>
+        <v>75.93000000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>75.55</v>
+        <v>71.55</v>
       </c>
       <c r="I2" t="n">
-        <v>76.95999999999999</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>8.65</v>
+        <v>8.75</v>
       </c>
       <c r="K2" t="n">
-        <v>8.77</v>
+        <v>9.91</v>
       </c>
       <c r="L2" t="n">
-        <v>8.15</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="M2" t="n">
-        <v>8.199999999999999</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N2" t="n">
-        <v>42.74</v>
+        <v>43.14</v>
       </c>
       <c r="O2" t="n">
-        <v>43</v>
+        <v>45.19</v>
       </c>
       <c r="P2" t="n">
-        <v>41.99</v>
+        <v>42.79</v>
       </c>
       <c r="Q2" t="n">
-        <v>42.22</v>
+        <v>43.31</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>177.62</v>
+        <v>183.84</v>
       </c>
       <c r="C3" t="n">
-        <v>182.24</v>
+        <v>188.49</v>
       </c>
       <c r="D3" t="n">
-        <v>150.58</v>
+        <v>172.26</v>
       </c>
       <c r="E3" t="n">
-        <v>172.52</v>
+        <v>184.24</v>
       </c>
       <c r="F3" t="n">
-        <v>75.3</v>
+        <v>75.81</v>
       </c>
       <c r="G3" t="n">
-        <v>75.93000000000001</v>
+        <v>77.94</v>
       </c>
       <c r="H3" t="n">
-        <v>71.55</v>
+        <v>74.19</v>
       </c>
       <c r="I3" t="n">
-        <v>74.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>8.75</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>9.91</v>
+        <v>8.98</v>
       </c>
       <c r="L3" t="n">
-        <v>8.550000000000001</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="M3" t="n">
-        <v>8.949999999999999</v>
+        <v>8.35</v>
       </c>
       <c r="N3" t="n">
-        <v>43.14</v>
+        <v>42.83</v>
       </c>
       <c r="O3" t="n">
-        <v>45.19</v>
+        <v>43.77</v>
       </c>
       <c r="P3" t="n">
-        <v>42.79</v>
+        <v>41.6</v>
       </c>
       <c r="Q3" t="n">
-        <v>43.31</v>
+        <v>41.99</v>
       </c>
       <c r="R3" t="n">
-        <v>-9.4003</v>
+        <v>6.7934</v>
       </c>
       <c r="U3" t="n">
-        <v>-2.5988</v>
+        <v>3.0416</v>
       </c>
       <c r="X3" t="n">
-        <v>9.1463</v>
+        <v>-6.7039</v>
       </c>
       <c r="AA3" t="n">
-        <v>2.5817</v>
+        <v>-3.0478</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>183.84</v>
+        <v>182.67</v>
       </c>
       <c r="C4" t="n">
-        <v>188.49</v>
+        <v>189.56</v>
       </c>
       <c r="D4" t="n">
-        <v>172.26</v>
+        <v>178.28</v>
       </c>
       <c r="E4" t="n">
-        <v>184.24</v>
+        <v>186.19</v>
       </c>
       <c r="F4" t="n">
-        <v>75.81</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>77.94</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>74.19</v>
+        <v>77.16</v>
       </c>
       <c r="I4" t="n">
-        <v>77.23999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="J4" t="n">
-        <v>8.380000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="K4" t="n">
-        <v>8.98</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L4" t="n">
-        <v>8.140000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M4" t="n">
-        <v>8.35</v>
+        <v>8.27</v>
       </c>
       <c r="N4" t="n">
-        <v>42.83</v>
+        <v>41.98</v>
       </c>
       <c r="O4" t="n">
-        <v>43.77</v>
+        <v>42.06</v>
       </c>
       <c r="P4" t="n">
-        <v>41.6</v>
+        <v>40.68</v>
       </c>
       <c r="Q4" t="n">
-        <v>41.99</v>
+        <v>41.07</v>
       </c>
       <c r="R4" t="n">
-        <v>6.7934</v>
+        <v>1.0584</v>
       </c>
       <c r="U4" t="n">
-        <v>3.0416</v>
+        <v>2.2139</v>
       </c>
       <c r="X4" t="n">
-        <v>-6.7039</v>
+        <v>-0.9581</v>
       </c>
       <c r="AA4" t="n">
-        <v>-3.0478</v>
+        <v>-2.191</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>182.67</v>
+        <v>167</v>
       </c>
       <c r="C5" t="n">
-        <v>189.56</v>
+        <v>174.4</v>
       </c>
       <c r="D5" t="n">
-        <v>178.28</v>
+        <v>161.14</v>
       </c>
       <c r="E5" t="n">
-        <v>186.19</v>
+        <v>164.18</v>
       </c>
       <c r="F5" t="n">
-        <v>77.29000000000001</v>
+        <v>75.73</v>
       </c>
       <c r="G5" t="n">
-        <v>79.68000000000001</v>
+        <v>77.37</v>
       </c>
       <c r="H5" t="n">
-        <v>77.16</v>
+        <v>74.23</v>
       </c>
       <c r="I5" t="n">
-        <v>78.95</v>
+        <v>75.34</v>
       </c>
       <c r="J5" t="n">
-        <v>8.43</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>8.630000000000001</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="L5" t="n">
-        <v>8.119999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>8.27</v>
+        <v>9.23</v>
       </c>
       <c r="N5" t="n">
-        <v>41.98</v>
+        <v>42.77</v>
       </c>
       <c r="O5" t="n">
-        <v>42.06</v>
+        <v>43.57</v>
       </c>
       <c r="P5" t="n">
-        <v>40.68</v>
+        <v>41.93</v>
       </c>
       <c r="Q5" t="n">
-        <v>41.07</v>
+        <v>42.98</v>
       </c>
       <c r="R5" t="n">
-        <v>1.0584</v>
+        <v>-11.8213</v>
       </c>
       <c r="S5" t="n">
-        <v>-2.2214</v>
+        <v>-4.8342</v>
       </c>
       <c r="U5" t="n">
-        <v>2.2139</v>
+        <v>-4.5725</v>
       </c>
       <c r="V5" t="n">
-        <v>2.5858</v>
+        <v>0.5069</v>
       </c>
       <c r="X5" t="n">
-        <v>-0.9581</v>
+        <v>11.6082</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.8537</v>
+        <v>3.1285</v>
       </c>
       <c r="AA5" t="n">
-        <v>-2.191</v>
+        <v>4.6506</v>
       </c>
       <c r="AB5" t="n">
-        <v>-2.7238</v>
+        <v>-0.7619</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>167</v>
+        <v>172.95</v>
       </c>
       <c r="C6" t="n">
-        <v>174.4</v>
+        <v>174.61</v>
       </c>
       <c r="D6" t="n">
-        <v>161.14</v>
+        <v>142.69</v>
       </c>
       <c r="E6" t="n">
-        <v>164.18</v>
+        <v>151.75</v>
       </c>
       <c r="F6" t="n">
-        <v>75.73</v>
+        <v>76.13</v>
       </c>
       <c r="G6" t="n">
-        <v>77.37</v>
+        <v>76.27</v>
       </c>
       <c r="H6" t="n">
-        <v>74.23</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>75.34</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>9.130000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="K6" t="n">
-        <v>9.390000000000001</v>
+        <v>10.47</v>
       </c>
       <c r="L6" t="n">
-        <v>8.800000000000001</v>
+        <v>8.68</v>
       </c>
       <c r="M6" t="n">
-        <v>9.23</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="N6" t="n">
-        <v>42.77</v>
+        <v>42.51</v>
       </c>
       <c r="O6" t="n">
-        <v>43.57</v>
+        <v>44.82</v>
       </c>
       <c r="P6" t="n">
-        <v>41.93</v>
+        <v>42.44</v>
       </c>
       <c r="Q6" t="n">
-        <v>42.98</v>
+        <v>43.54</v>
       </c>
       <c r="R6" t="n">
-        <v>-11.8213</v>
+        <v>-7.571</v>
       </c>
       <c r="S6" t="n">
-        <v>-4.8342</v>
+        <v>-17.6346</v>
       </c>
       <c r="U6" t="n">
-        <v>-4.5725</v>
+        <v>-1.3539</v>
       </c>
       <c r="V6" t="n">
-        <v>0.5069</v>
+        <v>-3.7804</v>
       </c>
       <c r="X6" t="n">
-        <v>11.6082</v>
+        <v>7.8007</v>
       </c>
       <c r="Y6" t="n">
-        <v>3.1285</v>
+        <v>19.1617</v>
       </c>
       <c r="AA6" t="n">
-        <v>4.6506</v>
+        <v>1.3029</v>
       </c>
       <c r="AB6" t="n">
-        <v>-0.7619</v>
+        <v>3.6914</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>172.95</v>
+        <v>141.24</v>
       </c>
       <c r="C7" t="n">
-        <v>174.61</v>
+        <v>160.6</v>
       </c>
       <c r="D7" t="n">
-        <v>142.69</v>
+        <v>135.02</v>
       </c>
       <c r="E7" t="n">
-        <v>151.75</v>
+        <v>151.89</v>
       </c>
       <c r="F7" t="n">
-        <v>76.13</v>
+        <v>72.41</v>
       </c>
       <c r="G7" t="n">
-        <v>76.27</v>
+        <v>74.5</v>
       </c>
       <c r="H7" t="n">
-        <v>72.09999999999999</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>74.31999999999999</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>8.77</v>
+        <v>10.64</v>
       </c>
       <c r="K7" t="n">
-        <v>10.47</v>
+        <v>11.07</v>
       </c>
       <c r="L7" t="n">
-        <v>8.68</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="M7" t="n">
-        <v>9.949999999999999</v>
+        <v>9.93</v>
       </c>
       <c r="N7" t="n">
-        <v>42.51</v>
+        <v>44.68</v>
       </c>
       <c r="O7" t="n">
-        <v>44.82</v>
+        <v>45.53</v>
       </c>
       <c r="P7" t="n">
-        <v>42.44</v>
+        <v>43.46</v>
       </c>
       <c r="Q7" t="n">
-        <v>43.54</v>
+        <v>44.37</v>
       </c>
       <c r="R7" t="n">
-        <v>-7.571</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="S7" t="n">
-        <v>-17.6346</v>
+        <v>-18.422</v>
       </c>
       <c r="T7" t="n">
-        <v>-20.3077</v>
+        <v>-11.958</v>
       </c>
       <c r="U7" t="n">
-        <v>-1.3539</v>
+        <v>-1.8703</v>
       </c>
       <c r="V7" t="n">
-        <v>-3.7804</v>
+        <v>-7.6251</v>
       </c>
       <c r="W7" t="n">
-        <v>-3.4304</v>
+        <v>-2.7081</v>
       </c>
       <c r="X7" t="n">
-        <v>7.8007</v>
+        <v>-0.201</v>
       </c>
       <c r="Y7" t="n">
-        <v>19.1617</v>
+        <v>20.0726</v>
       </c>
       <c r="Z7" t="n">
-        <v>21.3415</v>
+        <v>10.9497</v>
       </c>
       <c r="AA7" t="n">
-        <v>1.3029</v>
+        <v>1.9063</v>
       </c>
       <c r="AB7" t="n">
-        <v>3.6914</v>
+        <v>8.0351</v>
       </c>
       <c r="AC7" t="n">
-        <v>3.1265</v>
+        <v>2.4475</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>141.24</v>
+        <v>161</v>
       </c>
       <c r="C8" t="n">
-        <v>160.6</v>
+        <v>173.7</v>
       </c>
       <c r="D8" t="n">
-        <v>135.02</v>
+        <v>161</v>
       </c>
       <c r="E8" t="n">
-        <v>151.89</v>
+        <v>173.2</v>
       </c>
       <c r="F8" t="n">
-        <v>72.41</v>
+        <v>74.09</v>
       </c>
       <c r="G8" t="n">
-        <v>74.5</v>
+        <v>76.53</v>
       </c>
       <c r="H8" t="n">
-        <v>70.95999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="I8" t="n">
-        <v>72.93000000000001</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>10.64</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>11.07</v>
+        <v>9.35</v>
       </c>
       <c r="L8" t="n">
-        <v>9.369999999999999</v>
+        <v>8.51</v>
       </c>
       <c r="M8" t="n">
-        <v>9.93</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>44.68</v>
+        <v>43.67</v>
       </c>
       <c r="O8" t="n">
-        <v>45.53</v>
+        <v>43.97</v>
       </c>
       <c r="P8" t="n">
-        <v>43.46</v>
+        <v>42.19</v>
       </c>
       <c r="Q8" t="n">
-        <v>44.37</v>
+        <v>42.19</v>
       </c>
       <c r="R8" t="n">
-        <v>0.09229999999999999</v>
+        <v>14.0299</v>
       </c>
       <c r="S8" t="n">
-        <v>-18.422</v>
+        <v>5.494</v>
       </c>
       <c r="T8" t="n">
-        <v>-11.958</v>
+        <v>-5.9922</v>
       </c>
       <c r="U8" t="n">
-        <v>-1.8703</v>
+        <v>4.9088</v>
       </c>
       <c r="V8" t="n">
-        <v>-7.6251</v>
+        <v>1.553</v>
       </c>
       <c r="W8" t="n">
-        <v>-2.7081</v>
+        <v>-0.9451000000000001</v>
       </c>
       <c r="X8" t="n">
-        <v>-0.201</v>
+        <v>-13.998</v>
       </c>
       <c r="Y8" t="n">
-        <v>20.0726</v>
+        <v>-7.4756</v>
       </c>
       <c r="Z8" t="n">
-        <v>10.9497</v>
+        <v>2.2754</v>
       </c>
       <c r="AA8" t="n">
-        <v>1.9063</v>
+        <v>-4.9132</v>
       </c>
       <c r="AB8" t="n">
-        <v>8.0351</v>
+        <v>-1.8381</v>
       </c>
       <c r="AC8" t="n">
-        <v>2.4475</v>
+        <v>0.4763</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>161</v>
+        <v>171.26</v>
       </c>
       <c r="C9" t="n">
-        <v>173.7</v>
+        <v>179.97</v>
       </c>
       <c r="D9" t="n">
-        <v>161</v>
+        <v>168.23</v>
       </c>
       <c r="E9" t="n">
-        <v>173.2</v>
+        <v>178.39</v>
       </c>
       <c r="F9" t="n">
-        <v>74.09</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>76.53</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>73.62</v>
+        <v>74.47</v>
       </c>
       <c r="I9" t="n">
-        <v>76.51000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J9" t="n">
-        <v>9.300000000000001</v>
+        <v>8.65</v>
       </c>
       <c r="K9" t="n">
-        <v>9.35</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L9" t="n">
-        <v>8.51</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M9" t="n">
-        <v>8.539999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N9" t="n">
-        <v>43.67</v>
+        <v>42.94</v>
       </c>
       <c r="O9" t="n">
-        <v>43.97</v>
+        <v>43.33</v>
       </c>
       <c r="P9" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="Q9" t="n">
-        <v>42.19</v>
+        <v>41.96</v>
       </c>
       <c r="R9" t="n">
-        <v>14.0299</v>
+        <v>2.9965</v>
       </c>
       <c r="S9" t="n">
-        <v>5.494</v>
+        <v>17.5552</v>
       </c>
       <c r="T9" t="n">
-        <v>-5.9922</v>
+        <v>-4.1893</v>
       </c>
       <c r="U9" t="n">
-        <v>4.9088</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="V9" t="n">
-        <v>1.553</v>
+        <v>3.5388</v>
       </c>
       <c r="W9" t="n">
-        <v>-0.9451000000000001</v>
+        <v>-2.5332</v>
       </c>
       <c r="X9" t="n">
-        <v>-13.998</v>
+        <v>-2.9274</v>
       </c>
       <c r="Y9" t="n">
-        <v>-7.4756</v>
+        <v>-16.6834</v>
       </c>
       <c r="Z9" t="n">
-        <v>2.2754</v>
+        <v>0.2418</v>
       </c>
       <c r="AA9" t="n">
-        <v>-4.9132</v>
+        <v>-0.5452</v>
       </c>
       <c r="AB9" t="n">
-        <v>-1.8381</v>
+        <v>-3.6288</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.4763</v>
+        <v>2.167</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>171.26</v>
+        <v>184.8</v>
       </c>
       <c r="C10" t="n">
-        <v>179.97</v>
+        <v>195.27</v>
       </c>
       <c r="D10" t="n">
-        <v>168.23</v>
+        <v>183.34</v>
       </c>
       <c r="E10" t="n">
-        <v>178.39</v>
+        <v>190.56</v>
       </c>
       <c r="F10" t="n">
-        <v>75.18000000000001</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>77.79000000000001</v>
+        <v>79.33</v>
       </c>
       <c r="H10" t="n">
-        <v>74.47</v>
+        <v>77.33</v>
       </c>
       <c r="I10" t="n">
-        <v>76.95</v>
+        <v>77.84</v>
       </c>
       <c r="J10" t="n">
-        <v>8.65</v>
+        <v>8</v>
       </c>
       <c r="K10" t="n">
-        <v>8.779999999999999</v>
+        <v>8.06</v>
       </c>
       <c r="L10" t="n">
-        <v>8.210000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="M10" t="n">
-        <v>8.289999999999999</v>
+        <v>7.73</v>
       </c>
       <c r="N10" t="n">
-        <v>42.94</v>
+        <v>41.4</v>
       </c>
       <c r="O10" t="n">
-        <v>43.33</v>
+        <v>41.78</v>
       </c>
       <c r="P10" t="n">
+        <v>40.68</v>
+      </c>
+      <c r="Q10" t="n">
         <v>41.5</v>
       </c>
-      <c r="Q10" t="n">
-        <v>41.96</v>
-      </c>
       <c r="R10" t="n">
-        <v>2.9965</v>
+        <v>6.8221</v>
       </c>
       <c r="S10" t="n">
-        <v>17.5552</v>
+        <v>25.4592</v>
       </c>
       <c r="T10" t="n">
-        <v>-4.1893</v>
+        <v>16.0677</v>
       </c>
       <c r="U10" t="n">
-        <v>0.5750999999999999</v>
+        <v>1.1566</v>
       </c>
       <c r="V10" t="n">
-        <v>3.5388</v>
+        <v>6.7325</v>
       </c>
       <c r="W10" t="n">
-        <v>-2.5332</v>
+        <v>3.3183</v>
       </c>
       <c r="X10" t="n">
-        <v>-2.9274</v>
+        <v>-6.7551</v>
       </c>
       <c r="Y10" t="n">
-        <v>-16.6834</v>
+        <v>-22.1551</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.2418</v>
+        <v>-16.2514</v>
       </c>
       <c r="AA10" t="n">
-        <v>-0.5452</v>
+        <v>-1.0963</v>
       </c>
       <c r="AB10" t="n">
-        <v>-3.6288</v>
+        <v>-6.4683</v>
       </c>
       <c r="AC10" t="n">
-        <v>2.167</v>
+        <v>-3.4435</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>184.8</v>
+        <v>211.38</v>
       </c>
       <c r="C11" t="n">
-        <v>195.27</v>
+        <v>228.5</v>
       </c>
       <c r="D11" t="n">
-        <v>183.34</v>
+        <v>209.89</v>
       </c>
       <c r="E11" t="n">
-        <v>190.56</v>
+        <v>225.79</v>
       </c>
       <c r="F11" t="n">
-        <v>78.04000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="G11" t="n">
-        <v>79.33</v>
+        <v>82.27</v>
       </c>
       <c r="H11" t="n">
-        <v>77.33</v>
+        <v>79.98</v>
       </c>
       <c r="I11" t="n">
-        <v>77.84</v>
+        <v>81.95</v>
       </c>
       <c r="J11" t="n">
-        <v>8</v>
+        <v>6.9</v>
       </c>
       <c r="K11" t="n">
-        <v>8.06</v>
+        <v>6.95</v>
       </c>
       <c r="L11" t="n">
-        <v>7.5</v>
+        <v>6.19</v>
       </c>
       <c r="M11" t="n">
-        <v>7.73</v>
+        <v>6.29</v>
       </c>
       <c r="N11" t="n">
-        <v>41.4</v>
+        <v>40.05</v>
       </c>
       <c r="O11" t="n">
-        <v>41.78</v>
+        <v>40.35</v>
       </c>
       <c r="P11" t="n">
-        <v>40.68</v>
+        <v>39.14</v>
       </c>
       <c r="Q11" t="n">
-        <v>41.5</v>
+        <v>39.28</v>
       </c>
       <c r="R11" t="n">
-        <v>6.8221</v>
+        <v>18.4876</v>
       </c>
       <c r="S11" t="n">
-        <v>25.4592</v>
+        <v>30.3637</v>
       </c>
       <c r="T11" t="n">
-        <v>16.0677</v>
+        <v>48.7908</v>
       </c>
       <c r="U11" t="n">
-        <v>1.1566</v>
+        <v>5.2801</v>
       </c>
       <c r="V11" t="n">
-        <v>6.7325</v>
+        <v>7.1102</v>
       </c>
       <c r="W11" t="n">
-        <v>3.3183</v>
+        <v>10.2664</v>
       </c>
       <c r="X11" t="n">
-        <v>-6.7551</v>
+        <v>-18.6287</v>
       </c>
       <c r="Y11" t="n">
-        <v>-22.1551</v>
+        <v>-26.3466</v>
       </c>
       <c r="Z11" t="n">
-        <v>-16.2514</v>
+        <v>-36.7839</v>
       </c>
       <c r="AA11" t="n">
-        <v>-1.0963</v>
+        <v>-5.3494</v>
       </c>
       <c r="AB11" t="n">
-        <v>-6.4683</v>
+        <v>-6.8974</v>
       </c>
       <c r="AC11" t="n">
-        <v>-3.4435</v>
+        <v>-9.7841</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>211.38</v>
+        <v>242.66</v>
       </c>
       <c r="C12" t="n">
-        <v>228.5</v>
+        <v>242.66</v>
       </c>
       <c r="D12" t="n">
-        <v>209.89</v>
+        <v>204</v>
       </c>
       <c r="E12" t="n">
-        <v>225.79</v>
+        <v>217.98</v>
       </c>
       <c r="F12" t="n">
-        <v>80.59</v>
+        <v>82.87</v>
       </c>
       <c r="G12" t="n">
-        <v>82.27</v>
+        <v>82.91</v>
       </c>
       <c r="H12" t="n">
-        <v>79.98</v>
+        <v>80.33</v>
       </c>
       <c r="I12" t="n">
-        <v>81.95</v>
+        <v>81.67</v>
       </c>
       <c r="J12" t="n">
-        <v>6.9</v>
+        <v>5.83</v>
       </c>
       <c r="K12" t="n">
-        <v>6.95</v>
+        <v>6.91</v>
       </c>
       <c r="L12" t="n">
-        <v>6.19</v>
+        <v>5.83</v>
       </c>
       <c r="M12" t="n">
-        <v>6.29</v>
+        <v>6.53</v>
       </c>
       <c r="N12" t="n">
-        <v>40.05</v>
+        <v>38.87</v>
       </c>
       <c r="O12" t="n">
-        <v>40.35</v>
+        <v>40.09</v>
       </c>
       <c r="P12" t="n">
-        <v>39.14</v>
+        <v>38.86</v>
       </c>
       <c r="Q12" t="n">
-        <v>39.28</v>
+        <v>39.44</v>
       </c>
       <c r="R12" t="n">
-        <v>18.4876</v>
+        <v>-3.459</v>
       </c>
       <c r="S12" t="n">
-        <v>30.3637</v>
+        <v>22.1929</v>
       </c>
       <c r="T12" t="n">
-        <v>48.7908</v>
+        <v>43.5118</v>
       </c>
       <c r="U12" t="n">
-        <v>5.2801</v>
+        <v>-0.3417</v>
       </c>
       <c r="V12" t="n">
-        <v>7.1102</v>
+        <v>6.1339</v>
       </c>
       <c r="W12" t="n">
-        <v>10.2664</v>
+        <v>11.9841</v>
       </c>
       <c r="X12" t="n">
-        <v>-18.6287</v>
+        <v>3.8156</v>
       </c>
       <c r="Y12" t="n">
-        <v>-26.3466</v>
+        <v>-21.2304</v>
       </c>
       <c r="Z12" t="n">
-        <v>-36.7839</v>
+        <v>-34.2397</v>
       </c>
       <c r="AA12" t="n">
-        <v>-5.3494</v>
+        <v>0.4073</v>
       </c>
       <c r="AB12" t="n">
-        <v>-6.8974</v>
+        <v>-6.0057</v>
       </c>
       <c r="AC12" t="n">
-        <v>-9.7841</v>
+        <v>-11.1111</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>242.66</v>
+        <v>219</v>
       </c>
       <c r="C13" t="n">
-        <v>242.66</v>
+        <v>231.89</v>
       </c>
       <c r="D13" t="n">
-        <v>204</v>
+        <v>207.56</v>
       </c>
       <c r="E13" t="n">
-        <v>217.98</v>
+        <v>224.63</v>
       </c>
       <c r="F13" t="n">
-        <v>82.87</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>82.91</v>
+        <v>84.05</v>
       </c>
       <c r="H13" t="n">
-        <v>80.33</v>
+        <v>80.66</v>
       </c>
       <c r="I13" t="n">
-        <v>81.67</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>5.83</v>
+        <v>6.49</v>
       </c>
       <c r="K13" t="n">
-        <v>6.91</v>
+        <v>6.83</v>
       </c>
       <c r="L13" t="n">
-        <v>5.83</v>
+        <v>6.1</v>
       </c>
       <c r="M13" t="n">
-        <v>6.53</v>
+        <v>6.31</v>
       </c>
       <c r="N13" t="n">
-        <v>38.87</v>
+        <v>39.41</v>
       </c>
       <c r="O13" t="n">
-        <v>40.09</v>
+        <v>39.94</v>
       </c>
       <c r="P13" t="n">
-        <v>38.86</v>
+        <v>38.3</v>
       </c>
       <c r="Q13" t="n">
-        <v>39.44</v>
+        <v>38.47</v>
       </c>
       <c r="R13" t="n">
-        <v>-3.459</v>
+        <v>3.0507</v>
       </c>
       <c r="S13" t="n">
-        <v>22.1929</v>
+        <v>17.8789</v>
       </c>
       <c r="T13" t="n">
-        <v>43.5118</v>
+        <v>29.694</v>
       </c>
       <c r="U13" t="n">
-        <v>-0.3417</v>
+        <v>2.4611</v>
       </c>
       <c r="V13" t="n">
-        <v>6.1339</v>
+        <v>7.5026</v>
       </c>
       <c r="W13" t="n">
-        <v>11.9841</v>
+        <v>9.3713</v>
       </c>
       <c r="X13" t="n">
-        <v>3.8156</v>
+        <v>-3.3691</v>
       </c>
       <c r="Y13" t="n">
-        <v>-21.2304</v>
+        <v>-18.37</v>
       </c>
       <c r="Z13" t="n">
-        <v>-34.2397</v>
+        <v>-26.1124</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.4073</v>
+        <v>-2.4594</v>
       </c>
       <c r="AB13" t="n">
-        <v>-6.0057</v>
+        <v>-7.3012</v>
       </c>
       <c r="AC13" t="n">
-        <v>-11.1111</v>
+        <v>-8.817299999999999</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>219</v>
+        <v>231.82</v>
       </c>
       <c r="C14" t="n">
-        <v>231.89</v>
+        <v>239.07</v>
       </c>
       <c r="D14" t="n">
-        <v>207.56</v>
+        <v>218.56</v>
       </c>
       <c r="E14" t="n">
-        <v>224.63</v>
+        <v>224.34</v>
       </c>
       <c r="F14" t="n">
-        <v>81.73999999999999</v>
+        <v>84.41</v>
       </c>
       <c r="G14" t="n">
-        <v>84.05</v>
+        <v>85.7</v>
       </c>
       <c r="H14" t="n">
-        <v>80.66</v>
+        <v>83.53</v>
       </c>
       <c r="I14" t="n">
-        <v>83.68000000000001</v>
+        <v>84.56</v>
       </c>
       <c r="J14" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="K14" t="n">
         <v>6.49</v>
       </c>
-      <c r="K14" t="n">
-        <v>6.83</v>
-      </c>
       <c r="L14" t="n">
-        <v>6.1</v>
+        <v>5.91</v>
       </c>
       <c r="M14" t="n">
-        <v>6.31</v>
+        <v>6.33</v>
       </c>
       <c r="N14" t="n">
-        <v>39.41</v>
+        <v>38.15</v>
       </c>
       <c r="O14" t="n">
-        <v>39.94</v>
+        <v>38.56</v>
       </c>
       <c r="P14" t="n">
-        <v>38.3</v>
+        <v>37.56</v>
       </c>
       <c r="Q14" t="n">
-        <v>38.47</v>
+        <v>38.08</v>
       </c>
       <c r="R14" t="n">
-        <v>3.0507</v>
+        <v>-0.1291</v>
       </c>
       <c r="S14" t="n">
-        <v>17.8789</v>
+        <v>-0.6422</v>
       </c>
       <c r="T14" t="n">
-        <v>29.694</v>
+        <v>25.7582</v>
       </c>
       <c r="U14" t="n">
-        <v>2.4611</v>
+        <v>1.0516</v>
       </c>
       <c r="V14" t="n">
-        <v>7.5026</v>
+        <v>3.1849</v>
       </c>
       <c r="W14" t="n">
-        <v>9.3713</v>
+        <v>9.8895</v>
       </c>
       <c r="X14" t="n">
-        <v>-3.3691</v>
+        <v>0.317</v>
       </c>
       <c r="Y14" t="n">
-        <v>-18.37</v>
+        <v>0.6359</v>
       </c>
       <c r="Z14" t="n">
-        <v>-26.1124</v>
+        <v>-23.6429</v>
       </c>
       <c r="AA14" t="n">
-        <v>-2.4594</v>
+        <v>-1.0138</v>
       </c>
       <c r="AB14" t="n">
-        <v>-7.3012</v>
+        <v>-3.055</v>
       </c>
       <c r="AC14" t="n">
-        <v>-8.817299999999999</v>
+        <v>-9.2469</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>231.82</v>
+        <v>217.27</v>
       </c>
       <c r="C15" t="n">
-        <v>239.07</v>
+        <v>234.06</v>
       </c>
       <c r="D15" t="n">
-        <v>218.56</v>
+        <v>210.14</v>
       </c>
       <c r="E15" t="n">
-        <v>224.34</v>
+        <v>227.03</v>
       </c>
       <c r="F15" t="n">
-        <v>84.41</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>85.7</v>
+        <v>87.06</v>
       </c>
       <c r="H15" t="n">
-        <v>83.53</v>
+        <v>83.75</v>
       </c>
       <c r="I15" t="n">
-        <v>84.56</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="J15" t="n">
-        <v>6.11</v>
+        <v>6.55</v>
       </c>
       <c r="K15" t="n">
-        <v>6.49</v>
+        <v>6.74</v>
       </c>
       <c r="L15" t="n">
-        <v>5.91</v>
+        <v>6.05</v>
       </c>
       <c r="M15" t="n">
-        <v>6.33</v>
+        <v>6.26</v>
       </c>
       <c r="N15" t="n">
-        <v>38.15</v>
+        <v>38.27</v>
       </c>
       <c r="O15" t="n">
-        <v>38.56</v>
+        <v>38.46</v>
       </c>
       <c r="P15" t="n">
-        <v>37.56</v>
+        <v>36.96</v>
       </c>
       <c r="Q15" t="n">
-        <v>38.08</v>
+        <v>37.42</v>
       </c>
       <c r="R15" t="n">
-        <v>-0.1291</v>
+        <v>1.1991</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.6422</v>
+        <v>4.1518</v>
       </c>
       <c r="T15" t="n">
-        <v>25.7582</v>
+        <v>19.1383</v>
       </c>
       <c r="U15" t="n">
-        <v>1.0516</v>
+        <v>1.7502</v>
       </c>
       <c r="V15" t="n">
-        <v>3.1849</v>
+        <v>5.3508</v>
       </c>
       <c r="W15" t="n">
-        <v>9.8895</v>
+        <v>10.5344</v>
       </c>
       <c r="X15" t="n">
-        <v>0.317</v>
+        <v>-1.1058</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.6359</v>
+        <v>-4.1348</v>
       </c>
       <c r="Z15" t="n">
-        <v>-23.6429</v>
+        <v>-19.0168</v>
       </c>
       <c r="AA15" t="n">
-        <v>-1.0138</v>
+        <v>-1.7332</v>
       </c>
       <c r="AB15" t="n">
-        <v>-3.055</v>
+        <v>-5.1217</v>
       </c>
       <c r="AC15" t="n">
-        <v>-9.2469</v>
+        <v>-9.831300000000001</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>217.27</v>
+        <v>243.18</v>
       </c>
       <c r="C16" t="n">
-        <v>234.06</v>
+        <v>267.08</v>
       </c>
       <c r="D16" t="n">
-        <v>210.14</v>
+        <v>238.82</v>
       </c>
       <c r="E16" t="n">
-        <v>227.03</v>
+        <v>266.32</v>
       </c>
       <c r="F16" t="n">
-        <v>84.15000000000001</v>
+        <v>85.94</v>
       </c>
       <c r="G16" t="n">
-        <v>87.06</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>83.75</v>
+        <v>84.83</v>
       </c>
       <c r="I16" t="n">
-        <v>86.04000000000001</v>
+        <v>87.22</v>
       </c>
       <c r="J16" t="n">
-        <v>6.55</v>
+        <v>5.8</v>
       </c>
       <c r="K16" t="n">
-        <v>6.74</v>
+        <v>5.93</v>
       </c>
       <c r="L16" t="n">
-        <v>6.05</v>
+        <v>5.15</v>
       </c>
       <c r="M16" t="n">
-        <v>6.26</v>
+        <v>5.17</v>
       </c>
       <c r="N16" t="n">
-        <v>38.27</v>
+        <v>37.47</v>
       </c>
       <c r="O16" t="n">
-        <v>38.46</v>
+        <v>37.95</v>
       </c>
       <c r="P16" t="n">
-        <v>36.96</v>
+        <v>36.86</v>
       </c>
       <c r="Q16" t="n">
-        <v>37.42</v>
+        <v>36.91</v>
       </c>
       <c r="R16" t="n">
-        <v>1.1991</v>
+        <v>17.3061</v>
       </c>
       <c r="S16" t="n">
-        <v>4.1518</v>
+        <v>18.5594</v>
       </c>
       <c r="T16" t="n">
-        <v>19.1383</v>
+        <v>17.9503</v>
       </c>
       <c r="U16" t="n">
-        <v>1.7502</v>
+        <v>1.3715</v>
       </c>
       <c r="V16" t="n">
-        <v>5.3508</v>
+        <v>4.2304</v>
       </c>
       <c r="W16" t="n">
-        <v>10.5344</v>
+        <v>6.4308</v>
       </c>
       <c r="X16" t="n">
-        <v>-1.1058</v>
+        <v>-17.4121</v>
       </c>
       <c r="Y16" t="n">
-        <v>-4.1348</v>
+        <v>-18.0666</v>
       </c>
       <c r="Z16" t="n">
-        <v>-19.0168</v>
+        <v>-17.806</v>
       </c>
       <c r="AA16" t="n">
-        <v>-1.7332</v>
+        <v>-1.3629</v>
       </c>
       <c r="AB16" t="n">
-        <v>-5.1217</v>
+        <v>-4.0551</v>
       </c>
       <c r="AC16" t="n">
-        <v>-9.831300000000001</v>
+        <v>-6.0336</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>243.18</v>
+        <v>281.47</v>
       </c>
       <c r="C17" t="n">
-        <v>267.08</v>
+        <v>284.58</v>
       </c>
       <c r="D17" t="n">
-        <v>238.82</v>
+        <v>257.26</v>
       </c>
       <c r="E17" t="n">
-        <v>266.32</v>
+        <v>280.54</v>
       </c>
       <c r="F17" t="n">
-        <v>85.94</v>
+        <v>87.68000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>87.31999999999999</v>
+        <v>88.09</v>
       </c>
       <c r="H17" t="n">
-        <v>84.83</v>
+        <v>85.41</v>
       </c>
       <c r="I17" t="n">
-        <v>87.22</v>
+        <v>86.56</v>
       </c>
       <c r="J17" t="n">
-        <v>5.8</v>
+        <v>4.88</v>
       </c>
       <c r="K17" t="n">
-        <v>5.93</v>
+        <v>5.35</v>
       </c>
       <c r="L17" t="n">
-        <v>5.15</v>
+        <v>4.82</v>
       </c>
       <c r="M17" t="n">
-        <v>5.17</v>
+        <v>4.91</v>
       </c>
       <c r="N17" t="n">
-        <v>37.47</v>
+        <v>36.73</v>
       </c>
       <c r="O17" t="n">
-        <v>37.95</v>
+        <v>37.69</v>
       </c>
       <c r="P17" t="n">
-        <v>36.86</v>
+        <v>36.55</v>
       </c>
       <c r="Q17" t="n">
-        <v>36.91</v>
+        <v>37.19</v>
       </c>
       <c r="R17" t="n">
-        <v>17.3061</v>
+        <v>5.3394</v>
       </c>
       <c r="S17" t="n">
-        <v>18.5594</v>
+        <v>25.0513</v>
       </c>
       <c r="T17" t="n">
-        <v>17.9503</v>
+        <v>28.6999</v>
       </c>
       <c r="U17" t="n">
-        <v>1.3715</v>
+        <v>-0.7567</v>
       </c>
       <c r="V17" t="n">
-        <v>4.2304</v>
+        <v>2.3652</v>
       </c>
       <c r="W17" t="n">
-        <v>6.4308</v>
+        <v>5.9875</v>
       </c>
       <c r="X17" t="n">
-        <v>-17.4121</v>
+        <v>-5.029</v>
       </c>
       <c r="Y17" t="n">
-        <v>-18.0666</v>
+        <v>-22.4329</v>
       </c>
       <c r="Z17" t="n">
-        <v>-17.806</v>
+        <v>-24.8086</v>
       </c>
       <c r="AA17" t="n">
-        <v>-1.3629</v>
+        <v>0.7586000000000001</v>
       </c>
       <c r="AB17" t="n">
-        <v>-4.0551</v>
+        <v>-2.3372</v>
       </c>
       <c r="AC17" t="n">
-        <v>-6.0336</v>
+        <v>-5.7049</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>281.47</v>
+        <v>242.04</v>
       </c>
       <c r="C18" t="n">
-        <v>284.58</v>
+        <v>274.5</v>
       </c>
       <c r="D18" t="n">
-        <v>257.26</v>
+        <v>228.55</v>
       </c>
       <c r="E18" t="n">
-        <v>280.54</v>
+        <v>262.7</v>
       </c>
       <c r="F18" t="n">
-        <v>87.68000000000001</v>
+        <v>83.47</v>
       </c>
       <c r="G18" t="n">
-        <v>88.09</v>
+        <v>86.25</v>
       </c>
       <c r="H18" t="n">
-        <v>85.41</v>
+        <v>82.48</v>
       </c>
       <c r="I18" t="n">
-        <v>86.56</v>
+        <v>85.22</v>
       </c>
       <c r="J18" t="n">
-        <v>4.88</v>
+        <v>5.57</v>
       </c>
       <c r="K18" t="n">
-        <v>5.35</v>
+        <v>5.81</v>
       </c>
       <c r="L18" t="n">
-        <v>4.82</v>
+        <v>5</v>
       </c>
       <c r="M18" t="n">
-        <v>4.91</v>
+        <v>5.2</v>
       </c>
       <c r="N18" t="n">
-        <v>36.73</v>
+        <v>38.53</v>
       </c>
       <c r="O18" t="n">
-        <v>37.69</v>
+        <v>38.96</v>
       </c>
       <c r="P18" t="n">
-        <v>36.55</v>
+        <v>37.33</v>
       </c>
       <c r="Q18" t="n">
-        <v>37.19</v>
+        <v>37.76</v>
       </c>
       <c r="R18" t="n">
-        <v>5.3394</v>
+        <v>-6.3592</v>
       </c>
       <c r="S18" t="n">
-        <v>25.0513</v>
+        <v>15.7116</v>
       </c>
       <c r="T18" t="n">
-        <v>28.6999</v>
+        <v>16.9479</v>
       </c>
       <c r="U18" t="n">
-        <v>-0.7567</v>
+        <v>-1.5481</v>
       </c>
       <c r="V18" t="n">
-        <v>2.3652</v>
+        <v>-0.953</v>
       </c>
       <c r="W18" t="n">
-        <v>5.9875</v>
+        <v>1.8403</v>
       </c>
       <c r="X18" t="n">
-        <v>-5.029</v>
+        <v>5.9063</v>
       </c>
       <c r="Y18" t="n">
-        <v>-22.4329</v>
+        <v>-16.9329</v>
       </c>
       <c r="Z18" t="n">
-        <v>-24.8086</v>
+        <v>-17.5911</v>
       </c>
       <c r="AA18" t="n">
-        <v>0.7586000000000001</v>
+        <v>1.5327</v>
       </c>
       <c r="AB18" t="n">
-        <v>-2.3372</v>
+        <v>0.9086</v>
       </c>
       <c r="AC18" t="n">
-        <v>-5.7049</v>
+        <v>-1.8456</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>242.04</v>
+        <v>230.85</v>
       </c>
       <c r="C19" t="n">
-        <v>274.5</v>
+        <v>233.69</v>
       </c>
       <c r="D19" t="n">
-        <v>228.55</v>
+        <v>181.81</v>
       </c>
       <c r="E19" t="n">
-        <v>262.7</v>
+        <v>182.54</v>
       </c>
       <c r="F19" t="n">
-        <v>83.47</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="G19" t="n">
-        <v>86.25</v>
+        <v>82.08</v>
       </c>
       <c r="H19" t="n">
-        <v>82.48</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="I19" t="n">
-        <v>85.22</v>
+        <v>73.05</v>
       </c>
       <c r="J19" t="n">
-        <v>5.57</v>
+        <v>5.86</v>
       </c>
       <c r="K19" t="n">
-        <v>5.81</v>
+        <v>6.85</v>
       </c>
       <c r="L19" t="n">
-        <v>5</v>
+        <v>5.79</v>
       </c>
       <c r="M19" t="n">
-        <v>5.2</v>
+        <v>6.84</v>
       </c>
       <c r="N19" t="n">
-        <v>38.53</v>
+        <v>39.42</v>
       </c>
       <c r="O19" t="n">
-        <v>38.96</v>
+        <v>43.35</v>
       </c>
       <c r="P19" t="n">
-        <v>37.33</v>
+        <v>39.18</v>
       </c>
       <c r="Q19" t="n">
-        <v>37.76</v>
+        <v>43.19</v>
       </c>
       <c r="R19" t="n">
-        <v>-6.3592</v>
+        <v>-30.5139</v>
       </c>
       <c r="S19" t="n">
-        <v>15.7116</v>
+        <v>-31.4584</v>
       </c>
       <c r="T19" t="n">
-        <v>16.9479</v>
+        <v>-18.6324</v>
       </c>
       <c r="U19" t="n">
-        <v>-1.5481</v>
+        <v>-14.2807</v>
       </c>
       <c r="V19" t="n">
-        <v>-0.953</v>
+        <v>-16.2463</v>
       </c>
       <c r="W19" t="n">
-        <v>1.8403</v>
+        <v>-13.6116</v>
       </c>
       <c r="X19" t="n">
-        <v>5.9063</v>
+        <v>31.5385</v>
       </c>
       <c r="Y19" t="n">
-        <v>-16.9329</v>
+        <v>32.3017</v>
       </c>
       <c r="Z19" t="n">
-        <v>-17.5911</v>
+        <v>8.056900000000001</v>
       </c>
       <c r="AA19" t="n">
-        <v>1.5327</v>
+        <v>14.3803</v>
       </c>
       <c r="AB19" t="n">
-        <v>0.9086</v>
+        <v>17.0144</v>
       </c>
       <c r="AC19" t="n">
-        <v>-1.8456</v>
+        <v>13.4191</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>230.85</v>
+        <v>210.62</v>
       </c>
       <c r="C20" t="n">
-        <v>233.69</v>
+        <v>222.19</v>
       </c>
       <c r="D20" t="n">
-        <v>181.81</v>
+        <v>201.69</v>
       </c>
       <c r="E20" t="n">
-        <v>182.54</v>
+        <v>211.44</v>
       </c>
       <c r="F20" t="n">
-        <v>81.56999999999999</v>
+        <v>76.86</v>
       </c>
       <c r="G20" t="n">
-        <v>82.08</v>
+        <v>78.47</v>
       </c>
       <c r="H20" t="n">
-        <v>72.68000000000001</v>
+        <v>75.38</v>
       </c>
       <c r="I20" t="n">
-        <v>73.05</v>
+        <v>76.27</v>
       </c>
       <c r="J20" t="n">
-        <v>5.86</v>
+        <v>5.71</v>
       </c>
       <c r="K20" t="n">
-        <v>6.85</v>
+        <v>6.05</v>
       </c>
       <c r="L20" t="n">
-        <v>5.79</v>
+        <v>5.27</v>
       </c>
       <c r="M20" t="n">
-        <v>6.84</v>
+        <v>5.69</v>
       </c>
       <c r="N20" t="n">
-        <v>39.42</v>
+        <v>40.92</v>
       </c>
       <c r="O20" t="n">
-        <v>43.35</v>
+        <v>41.78</v>
       </c>
       <c r="P20" t="n">
-        <v>39.18</v>
+        <v>39.96</v>
       </c>
       <c r="Q20" t="n">
-        <v>43.19</v>
+        <v>41.26</v>
       </c>
       <c r="R20" t="n">
-        <v>-30.5139</v>
+        <v>15.8321</v>
       </c>
       <c r="S20" t="n">
-        <v>-31.4584</v>
+        <v>-24.6311</v>
       </c>
       <c r="T20" t="n">
-        <v>-18.6324</v>
+        <v>-6.8669</v>
       </c>
       <c r="U20" t="n">
-        <v>-14.2807</v>
+        <v>4.4079</v>
       </c>
       <c r="V20" t="n">
-        <v>-16.2463</v>
+        <v>-11.8877</v>
       </c>
       <c r="W20" t="n">
-        <v>-13.6116</v>
+        <v>-11.3552</v>
       </c>
       <c r="X20" t="n">
-        <v>31.5385</v>
+        <v>-16.8129</v>
       </c>
       <c r="Y20" t="n">
-        <v>32.3017</v>
+        <v>15.8859</v>
       </c>
       <c r="Z20" t="n">
-        <v>8.056900000000001</v>
+        <v>-9.105399999999999</v>
       </c>
       <c r="AA20" t="n">
-        <v>14.3803</v>
+        <v>-4.4686</v>
       </c>
       <c r="AB20" t="n">
-        <v>17.0144</v>
+        <v>10.9438</v>
       </c>
       <c r="AC20" t="n">
-        <v>13.4191</v>
+        <v>10.2619</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>210.62</v>
+        <v>227.06</v>
       </c>
       <c r="C21" t="n">
-        <v>222.19</v>
+        <v>231.02</v>
       </c>
       <c r="D21" t="n">
-        <v>201.69</v>
+        <v>157.56</v>
       </c>
       <c r="E21" t="n">
-        <v>211.44</v>
+        <v>201.68</v>
       </c>
       <c r="F21" t="n">
-        <v>76.86</v>
+        <v>78.48</v>
       </c>
       <c r="G21" t="n">
-        <v>78.47</v>
+        <v>79.34</v>
       </c>
       <c r="H21" t="n">
-        <v>75.38</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="I21" t="n">
-        <v>76.27</v>
+        <v>73.72</v>
       </c>
       <c r="J21" t="n">
-        <v>5.71</v>
+        <v>5.25</v>
       </c>
       <c r="K21" t="n">
-        <v>6.05</v>
+        <v>7.11</v>
       </c>
       <c r="L21" t="n">
-        <v>5.27</v>
+        <v>5.14</v>
       </c>
       <c r="M21" t="n">
-        <v>5.69</v>
+        <v>5.93</v>
       </c>
       <c r="N21" t="n">
-        <v>40.92</v>
+        <v>40.06</v>
       </c>
       <c r="O21" t="n">
-        <v>41.78</v>
+        <v>46.38</v>
       </c>
       <c r="P21" t="n">
-        <v>39.96</v>
+        <v>39.59</v>
       </c>
       <c r="Q21" t="n">
-        <v>41.26</v>
+        <v>42.67</v>
       </c>
       <c r="R21" t="n">
-        <v>15.8321</v>
+        <v>-4.616</v>
       </c>
       <c r="S21" t="n">
-        <v>-24.6311</v>
+        <v>-23.228</v>
       </c>
       <c r="T21" t="n">
-        <v>-6.8669</v>
+        <v>-24.2716</v>
       </c>
       <c r="U21" t="n">
-        <v>4.4079</v>
+        <v>-3.3434</v>
       </c>
       <c r="V21" t="n">
-        <v>-11.8877</v>
+        <v>-13.4945</v>
       </c>
       <c r="W21" t="n">
-        <v>-11.3552</v>
+        <v>-15.4781</v>
       </c>
       <c r="X21" t="n">
-        <v>-16.8129</v>
+        <v>4.2179</v>
       </c>
       <c r="Y21" t="n">
-        <v>15.8859</v>
+        <v>14.0385</v>
       </c>
       <c r="Z21" t="n">
-        <v>-9.105399999999999</v>
+        <v>14.7002</v>
       </c>
       <c r="AA21" t="n">
-        <v>-4.4686</v>
+        <v>3.4174</v>
       </c>
       <c r="AB21" t="n">
-        <v>10.9438</v>
+        <v>13.0032</v>
       </c>
       <c r="AC21" t="n">
-        <v>10.2619</v>
+        <v>15.6055</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>227.055</v>
+        <v>191.54</v>
       </c>
       <c r="C22" t="n">
-        <v>231.01</v>
+        <v>212.99</v>
       </c>
       <c r="D22" t="n">
-        <v>157.561</v>
+        <v>177.3001</v>
       </c>
       <c r="E22" t="n">
-        <v>201.68</v>
+        <v>180.65</v>
       </c>
       <c r="F22" t="n">
-        <v>78.48</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="G22" t="n">
-        <v>79.3407</v>
+        <v>74.7</v>
       </c>
       <c r="H22" t="n">
-        <v>66.79000000000001</v>
+        <v>69</v>
       </c>
       <c r="I22" t="n">
-        <v>73.72</v>
+        <v>69.27</v>
       </c>
       <c r="J22" t="n">
-        <v>5.25</v>
+        <v>6.24</v>
       </c>
       <c r="K22" t="n">
-        <v>7.11</v>
+        <v>6.65</v>
       </c>
       <c r="L22" t="n">
-        <v>5.14</v>
+        <v>5.6</v>
       </c>
       <c r="M22" t="n">
-        <v>5.93</v>
+        <v>6.57</v>
       </c>
       <c r="N22" t="n">
-        <v>40.07</v>
+        <v>43.81</v>
       </c>
       <c r="O22" t="n">
-        <v>46.38</v>
+        <v>45.3899</v>
       </c>
       <c r="P22" t="n">
-        <v>39.5936</v>
+        <v>42.07</v>
       </c>
       <c r="Q22" t="n">
-        <v>42.67</v>
+        <v>45.25</v>
       </c>
       <c r="R22" t="n">
-        <v>-4.616</v>
+        <v>-10.4274</v>
       </c>
       <c r="S22" t="n">
-        <v>-23.228</v>
+        <v>-1.0354</v>
       </c>
       <c r="T22" t="n">
-        <v>-24.2716</v>
+        <v>-35.6063</v>
       </c>
       <c r="U22" t="n">
-        <v>-3.3434</v>
+        <v>-6.0364</v>
       </c>
       <c r="V22" t="n">
-        <v>-13.4945</v>
+        <v>-5.1745</v>
       </c>
       <c r="W22" t="n">
-        <v>-15.4781</v>
+        <v>-19.9746</v>
       </c>
       <c r="X22" t="n">
-        <v>4.2179</v>
+        <v>10.7926</v>
       </c>
       <c r="Y22" t="n">
-        <v>14.0385</v>
+        <v>-3.9474</v>
       </c>
       <c r="Z22" t="n">
-        <v>14.7002</v>
+        <v>33.8086</v>
       </c>
       <c r="AA22" t="n">
-        <v>3.4174</v>
+        <v>6.0464</v>
       </c>
       <c r="AB22" t="n">
-        <v>13.0032</v>
+        <v>4.7696</v>
       </c>
       <c r="AC22" t="n">
-        <v>15.6055</v>
+        <v>21.6725</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-11 23:22
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>177.62</v>
+        <v>183.84</v>
       </c>
       <c r="C2" t="n">
-        <v>182.24</v>
+        <v>188.49</v>
       </c>
       <c r="D2" t="n">
-        <v>150.58</v>
+        <v>172.26</v>
       </c>
       <c r="E2" t="n">
-        <v>172.52</v>
+        <v>184.24</v>
       </c>
       <c r="F2" t="n">
-        <v>75.3</v>
+        <v>75.81</v>
       </c>
       <c r="G2" t="n">
-        <v>75.93000000000001</v>
+        <v>77.94</v>
       </c>
       <c r="H2" t="n">
-        <v>71.55</v>
+        <v>74.19</v>
       </c>
       <c r="I2" t="n">
-        <v>74.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>8.75</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>9.91</v>
+        <v>8.98</v>
       </c>
       <c r="L2" t="n">
-        <v>8.550000000000001</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="M2" t="n">
-        <v>8.949999999999999</v>
+        <v>8.35</v>
       </c>
       <c r="N2" t="n">
-        <v>43.14</v>
+        <v>42.83</v>
       </c>
       <c r="O2" t="n">
-        <v>45.19</v>
+        <v>43.77</v>
       </c>
       <c r="P2" t="n">
-        <v>42.79</v>
+        <v>41.6</v>
       </c>
       <c r="Q2" t="n">
-        <v>43.31</v>
+        <v>41.99</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>183.84</v>
+        <v>182.67</v>
       </c>
       <c r="C3" t="n">
-        <v>188.49</v>
+        <v>189.56</v>
       </c>
       <c r="D3" t="n">
-        <v>172.26</v>
+        <v>178.28</v>
       </c>
       <c r="E3" t="n">
-        <v>184.24</v>
+        <v>186.19</v>
       </c>
       <c r="F3" t="n">
-        <v>75.81</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>77.94</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>74.19</v>
+        <v>77.16</v>
       </c>
       <c r="I3" t="n">
-        <v>77.23999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="J3" t="n">
-        <v>8.380000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="K3" t="n">
-        <v>8.98</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L3" t="n">
-        <v>8.140000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M3" t="n">
-        <v>8.35</v>
+        <v>8.27</v>
       </c>
       <c r="N3" t="n">
-        <v>42.83</v>
+        <v>41.98</v>
       </c>
       <c r="O3" t="n">
-        <v>43.77</v>
+        <v>42.06</v>
       </c>
       <c r="P3" t="n">
-        <v>41.6</v>
+        <v>40.68</v>
       </c>
       <c r="Q3" t="n">
-        <v>41.99</v>
+        <v>41.07</v>
       </c>
       <c r="R3" t="n">
-        <v>6.7934</v>
+        <v>1.0584</v>
       </c>
       <c r="U3" t="n">
-        <v>3.0416</v>
+        <v>2.2139</v>
       </c>
       <c r="X3" t="n">
-        <v>-6.7039</v>
+        <v>-0.9581</v>
       </c>
       <c r="AA3" t="n">
-        <v>-3.0478</v>
+        <v>-2.191</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>182.67</v>
+        <v>167</v>
       </c>
       <c r="C4" t="n">
-        <v>189.56</v>
+        <v>174.4</v>
       </c>
       <c r="D4" t="n">
-        <v>178.28</v>
+        <v>161.14</v>
       </c>
       <c r="E4" t="n">
-        <v>186.19</v>
+        <v>164.18</v>
       </c>
       <c r="F4" t="n">
-        <v>77.29000000000001</v>
+        <v>75.73</v>
       </c>
       <c r="G4" t="n">
-        <v>79.68000000000001</v>
+        <v>77.37</v>
       </c>
       <c r="H4" t="n">
-        <v>77.16</v>
+        <v>74.23</v>
       </c>
       <c r="I4" t="n">
-        <v>78.95</v>
+        <v>75.34</v>
       </c>
       <c r="J4" t="n">
-        <v>8.43</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>8.630000000000001</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="L4" t="n">
-        <v>8.119999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>8.27</v>
+        <v>9.23</v>
       </c>
       <c r="N4" t="n">
-        <v>41.98</v>
+        <v>42.77</v>
       </c>
       <c r="O4" t="n">
-        <v>42.06</v>
+        <v>43.57</v>
       </c>
       <c r="P4" t="n">
-        <v>40.68</v>
+        <v>41.93</v>
       </c>
       <c r="Q4" t="n">
-        <v>41.07</v>
+        <v>42.98</v>
       </c>
       <c r="R4" t="n">
-        <v>1.0584</v>
+        <v>-11.8213</v>
       </c>
       <c r="U4" t="n">
-        <v>2.2139</v>
+        <v>-4.5725</v>
       </c>
       <c r="X4" t="n">
-        <v>-0.9581</v>
+        <v>11.6082</v>
       </c>
       <c r="AA4" t="n">
-        <v>-2.191</v>
+        <v>4.6506</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>167</v>
+        <v>172.95</v>
       </c>
       <c r="C5" t="n">
-        <v>174.4</v>
+        <v>174.61</v>
       </c>
       <c r="D5" t="n">
-        <v>161.14</v>
+        <v>142.69</v>
       </c>
       <c r="E5" t="n">
-        <v>164.18</v>
+        <v>151.75</v>
       </c>
       <c r="F5" t="n">
-        <v>75.73</v>
+        <v>76.13</v>
       </c>
       <c r="G5" t="n">
-        <v>77.37</v>
+        <v>76.27</v>
       </c>
       <c r="H5" t="n">
-        <v>74.23</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I5" t="n">
-        <v>75.34</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>9.130000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="K5" t="n">
-        <v>9.390000000000001</v>
+        <v>10.47</v>
       </c>
       <c r="L5" t="n">
-        <v>8.800000000000001</v>
+        <v>8.68</v>
       </c>
       <c r="M5" t="n">
-        <v>9.23</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="N5" t="n">
-        <v>42.77</v>
+        <v>42.51</v>
       </c>
       <c r="O5" t="n">
-        <v>43.57</v>
+        <v>44.82</v>
       </c>
       <c r="P5" t="n">
-        <v>41.93</v>
+        <v>42.44</v>
       </c>
       <c r="Q5" t="n">
-        <v>42.98</v>
+        <v>43.54</v>
       </c>
       <c r="R5" t="n">
-        <v>-11.8213</v>
+        <v>-7.571</v>
       </c>
       <c r="S5" t="n">
-        <v>-4.8342</v>
+        <v>-17.6346</v>
       </c>
       <c r="U5" t="n">
-        <v>-4.5725</v>
+        <v>-1.3539</v>
       </c>
       <c r="V5" t="n">
-        <v>0.5069</v>
+        <v>-3.7804</v>
       </c>
       <c r="X5" t="n">
-        <v>11.6082</v>
+        <v>7.8007</v>
       </c>
       <c r="Y5" t="n">
-        <v>3.1285</v>
+        <v>19.1617</v>
       </c>
       <c r="AA5" t="n">
-        <v>4.6506</v>
+        <v>1.3029</v>
       </c>
       <c r="AB5" t="n">
-        <v>-0.7619</v>
+        <v>3.6914</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>172.95</v>
+        <v>141.24</v>
       </c>
       <c r="C6" t="n">
-        <v>174.61</v>
+        <v>160.6</v>
       </c>
       <c r="D6" t="n">
-        <v>142.69</v>
+        <v>135.02</v>
       </c>
       <c r="E6" t="n">
-        <v>151.75</v>
+        <v>151.89</v>
       </c>
       <c r="F6" t="n">
-        <v>76.13</v>
+        <v>72.41</v>
       </c>
       <c r="G6" t="n">
-        <v>76.27</v>
+        <v>74.5</v>
       </c>
       <c r="H6" t="n">
-        <v>72.09999999999999</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>74.31999999999999</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>8.77</v>
+        <v>10.64</v>
       </c>
       <c r="K6" t="n">
-        <v>10.47</v>
+        <v>11.07</v>
       </c>
       <c r="L6" t="n">
-        <v>8.68</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="M6" t="n">
-        <v>9.949999999999999</v>
+        <v>9.93</v>
       </c>
       <c r="N6" t="n">
-        <v>42.51</v>
+        <v>44.68</v>
       </c>
       <c r="O6" t="n">
-        <v>44.82</v>
+        <v>45.53</v>
       </c>
       <c r="P6" t="n">
-        <v>42.44</v>
+        <v>43.46</v>
       </c>
       <c r="Q6" t="n">
-        <v>43.54</v>
+        <v>44.37</v>
       </c>
       <c r="R6" t="n">
-        <v>-7.571</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="S6" t="n">
-        <v>-17.6346</v>
+        <v>-18.422</v>
       </c>
       <c r="U6" t="n">
-        <v>-1.3539</v>
+        <v>-1.8703</v>
       </c>
       <c r="V6" t="n">
-        <v>-3.7804</v>
+        <v>-7.6251</v>
       </c>
       <c r="X6" t="n">
-        <v>7.8007</v>
+        <v>-0.201</v>
       </c>
       <c r="Y6" t="n">
-        <v>19.1617</v>
+        <v>20.0726</v>
       </c>
       <c r="AA6" t="n">
-        <v>1.3029</v>
+        <v>1.9063</v>
       </c>
       <c r="AB6" t="n">
-        <v>3.6914</v>
+        <v>8.0351</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>141.24</v>
+        <v>161</v>
       </c>
       <c r="C7" t="n">
-        <v>160.6</v>
+        <v>173.7</v>
       </c>
       <c r="D7" t="n">
-        <v>135.02</v>
+        <v>161</v>
       </c>
       <c r="E7" t="n">
-        <v>151.89</v>
+        <v>173.2</v>
       </c>
       <c r="F7" t="n">
-        <v>72.41</v>
+        <v>74.09</v>
       </c>
       <c r="G7" t="n">
-        <v>74.5</v>
+        <v>76.53</v>
       </c>
       <c r="H7" t="n">
-        <v>70.95999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="I7" t="n">
-        <v>72.93000000000001</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>10.64</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K7" t="n">
-        <v>11.07</v>
+        <v>9.35</v>
       </c>
       <c r="L7" t="n">
-        <v>9.369999999999999</v>
+        <v>8.51</v>
       </c>
       <c r="M7" t="n">
-        <v>9.93</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N7" t="n">
-        <v>44.68</v>
+        <v>43.67</v>
       </c>
       <c r="O7" t="n">
-        <v>45.53</v>
+        <v>43.97</v>
       </c>
       <c r="P7" t="n">
-        <v>43.46</v>
+        <v>42.19</v>
       </c>
       <c r="Q7" t="n">
-        <v>44.37</v>
+        <v>42.19</v>
       </c>
       <c r="R7" t="n">
-        <v>0.09229999999999999</v>
+        <v>14.0299</v>
       </c>
       <c r="S7" t="n">
-        <v>-18.422</v>
+        <v>5.494</v>
       </c>
       <c r="T7" t="n">
-        <v>-11.958</v>
+        <v>-5.9922</v>
       </c>
       <c r="U7" t="n">
-        <v>-1.8703</v>
+        <v>4.9088</v>
       </c>
       <c r="V7" t="n">
-        <v>-7.6251</v>
+        <v>1.553</v>
       </c>
       <c r="W7" t="n">
-        <v>-2.7081</v>
+        <v>-0.9451000000000001</v>
       </c>
       <c r="X7" t="n">
-        <v>-0.201</v>
+        <v>-13.998</v>
       </c>
       <c r="Y7" t="n">
-        <v>20.0726</v>
+        <v>-7.4756</v>
       </c>
       <c r="Z7" t="n">
-        <v>10.9497</v>
+        <v>2.2754</v>
       </c>
       <c r="AA7" t="n">
-        <v>1.9063</v>
+        <v>-4.9132</v>
       </c>
       <c r="AB7" t="n">
-        <v>8.0351</v>
+        <v>-1.8381</v>
       </c>
       <c r="AC7" t="n">
-        <v>2.4475</v>
+        <v>0.4763</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>161</v>
+        <v>171.26</v>
       </c>
       <c r="C8" t="n">
-        <v>173.7</v>
+        <v>179.97</v>
       </c>
       <c r="D8" t="n">
-        <v>161</v>
+        <v>168.23</v>
       </c>
       <c r="E8" t="n">
-        <v>173.2</v>
+        <v>178.39</v>
       </c>
       <c r="F8" t="n">
-        <v>74.09</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>76.53</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H8" t="n">
-        <v>73.62</v>
+        <v>74.47</v>
       </c>
       <c r="I8" t="n">
-        <v>76.51000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J8" t="n">
-        <v>9.300000000000001</v>
+        <v>8.65</v>
       </c>
       <c r="K8" t="n">
-        <v>9.35</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L8" t="n">
-        <v>8.51</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>8.539999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>43.67</v>
+        <v>42.94</v>
       </c>
       <c r="O8" t="n">
-        <v>43.97</v>
+        <v>43.33</v>
       </c>
       <c r="P8" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="Q8" t="n">
-        <v>42.19</v>
+        <v>41.96</v>
       </c>
       <c r="R8" t="n">
-        <v>14.0299</v>
+        <v>2.9965</v>
       </c>
       <c r="S8" t="n">
-        <v>5.494</v>
+        <v>17.5552</v>
       </c>
       <c r="T8" t="n">
-        <v>-5.9922</v>
+        <v>-4.1893</v>
       </c>
       <c r="U8" t="n">
-        <v>4.9088</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="V8" t="n">
-        <v>1.553</v>
+        <v>3.5388</v>
       </c>
       <c r="W8" t="n">
-        <v>-0.9451000000000001</v>
+        <v>-2.5332</v>
       </c>
       <c r="X8" t="n">
-        <v>-13.998</v>
+        <v>-2.9274</v>
       </c>
       <c r="Y8" t="n">
-        <v>-7.4756</v>
+        <v>-16.6834</v>
       </c>
       <c r="Z8" t="n">
-        <v>2.2754</v>
+        <v>0.2418</v>
       </c>
       <c r="AA8" t="n">
-        <v>-4.9132</v>
+        <v>-0.5452</v>
       </c>
       <c r="AB8" t="n">
-        <v>-1.8381</v>
+        <v>-3.6288</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.4763</v>
+        <v>2.167</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>171.26</v>
+        <v>184.8</v>
       </c>
       <c r="C9" t="n">
-        <v>179.97</v>
+        <v>195.27</v>
       </c>
       <c r="D9" t="n">
-        <v>168.23</v>
+        <v>183.34</v>
       </c>
       <c r="E9" t="n">
-        <v>178.39</v>
+        <v>190.56</v>
       </c>
       <c r="F9" t="n">
-        <v>75.18000000000001</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>77.79000000000001</v>
+        <v>79.33</v>
       </c>
       <c r="H9" t="n">
-        <v>74.47</v>
+        <v>77.33</v>
       </c>
       <c r="I9" t="n">
-        <v>76.95</v>
+        <v>77.84</v>
       </c>
       <c r="J9" t="n">
-        <v>8.65</v>
+        <v>8</v>
       </c>
       <c r="K9" t="n">
-        <v>8.779999999999999</v>
+        <v>8.06</v>
       </c>
       <c r="L9" t="n">
-        <v>8.210000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="M9" t="n">
-        <v>8.289999999999999</v>
+        <v>7.73</v>
       </c>
       <c r="N9" t="n">
-        <v>42.94</v>
+        <v>41.4</v>
       </c>
       <c r="O9" t="n">
-        <v>43.33</v>
+        <v>41.78</v>
       </c>
       <c r="P9" t="n">
+        <v>40.68</v>
+      </c>
+      <c r="Q9" t="n">
         <v>41.5</v>
       </c>
-      <c r="Q9" t="n">
-        <v>41.96</v>
-      </c>
       <c r="R9" t="n">
-        <v>2.9965</v>
+        <v>6.8221</v>
       </c>
       <c r="S9" t="n">
-        <v>17.5552</v>
+        <v>25.4592</v>
       </c>
       <c r="T9" t="n">
-        <v>-4.1893</v>
+        <v>16.0677</v>
       </c>
       <c r="U9" t="n">
-        <v>0.5750999999999999</v>
+        <v>1.1566</v>
       </c>
       <c r="V9" t="n">
-        <v>3.5388</v>
+        <v>6.7325</v>
       </c>
       <c r="W9" t="n">
-        <v>-2.5332</v>
+        <v>3.3183</v>
       </c>
       <c r="X9" t="n">
-        <v>-2.9274</v>
+        <v>-6.7551</v>
       </c>
       <c r="Y9" t="n">
-        <v>-16.6834</v>
+        <v>-22.1551</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.2418</v>
+        <v>-16.2514</v>
       </c>
       <c r="AA9" t="n">
-        <v>-0.5452</v>
+        <v>-1.0963</v>
       </c>
       <c r="AB9" t="n">
-        <v>-3.6288</v>
+        <v>-6.4683</v>
       </c>
       <c r="AC9" t="n">
-        <v>2.167</v>
+        <v>-3.4435</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>184.8</v>
+        <v>211.38</v>
       </c>
       <c r="C10" t="n">
-        <v>195.27</v>
+        <v>228.5</v>
       </c>
       <c r="D10" t="n">
-        <v>183.34</v>
+        <v>209.89</v>
       </c>
       <c r="E10" t="n">
-        <v>190.56</v>
+        <v>225.79</v>
       </c>
       <c r="F10" t="n">
-        <v>78.04000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="G10" t="n">
-        <v>79.33</v>
+        <v>82.27</v>
       </c>
       <c r="H10" t="n">
-        <v>77.33</v>
+        <v>79.98</v>
       </c>
       <c r="I10" t="n">
-        <v>77.84</v>
+        <v>81.95</v>
       </c>
       <c r="J10" t="n">
-        <v>8</v>
+        <v>6.9</v>
       </c>
       <c r="K10" t="n">
-        <v>8.06</v>
+        <v>6.95</v>
       </c>
       <c r="L10" t="n">
-        <v>7.5</v>
+        <v>6.19</v>
       </c>
       <c r="M10" t="n">
-        <v>7.73</v>
+        <v>6.29</v>
       </c>
       <c r="N10" t="n">
-        <v>41.4</v>
+        <v>40.05</v>
       </c>
       <c r="O10" t="n">
-        <v>41.78</v>
+        <v>40.35</v>
       </c>
       <c r="P10" t="n">
-        <v>40.68</v>
+        <v>39.14</v>
       </c>
       <c r="Q10" t="n">
-        <v>41.5</v>
+        <v>39.28</v>
       </c>
       <c r="R10" t="n">
-        <v>6.8221</v>
+        <v>18.4876</v>
       </c>
       <c r="S10" t="n">
-        <v>25.4592</v>
+        <v>30.3637</v>
       </c>
       <c r="T10" t="n">
-        <v>16.0677</v>
+        <v>48.7908</v>
       </c>
       <c r="U10" t="n">
-        <v>1.1566</v>
+        <v>5.2801</v>
       </c>
       <c r="V10" t="n">
-        <v>6.7325</v>
+        <v>7.1102</v>
       </c>
       <c r="W10" t="n">
-        <v>3.3183</v>
+        <v>10.2664</v>
       </c>
       <c r="X10" t="n">
-        <v>-6.7551</v>
+        <v>-18.6287</v>
       </c>
       <c r="Y10" t="n">
-        <v>-22.1551</v>
+        <v>-26.3466</v>
       </c>
       <c r="Z10" t="n">
-        <v>-16.2514</v>
+        <v>-36.7839</v>
       </c>
       <c r="AA10" t="n">
-        <v>-1.0963</v>
+        <v>-5.3494</v>
       </c>
       <c r="AB10" t="n">
-        <v>-6.4683</v>
+        <v>-6.8974</v>
       </c>
       <c r="AC10" t="n">
-        <v>-3.4435</v>
+        <v>-9.7841</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>211.38</v>
+        <v>242.66</v>
       </c>
       <c r="C11" t="n">
-        <v>228.5</v>
+        <v>242.66</v>
       </c>
       <c r="D11" t="n">
-        <v>209.89</v>
+        <v>204</v>
       </c>
       <c r="E11" t="n">
-        <v>225.79</v>
+        <v>217.98</v>
       </c>
       <c r="F11" t="n">
-        <v>80.59</v>
+        <v>82.87</v>
       </c>
       <c r="G11" t="n">
-        <v>82.27</v>
+        <v>82.91</v>
       </c>
       <c r="H11" t="n">
-        <v>79.98</v>
+        <v>80.33</v>
       </c>
       <c r="I11" t="n">
-        <v>81.95</v>
+        <v>81.67</v>
       </c>
       <c r="J11" t="n">
-        <v>6.9</v>
+        <v>5.83</v>
       </c>
       <c r="K11" t="n">
-        <v>6.95</v>
+        <v>6.91</v>
       </c>
       <c r="L11" t="n">
-        <v>6.19</v>
+        <v>5.83</v>
       </c>
       <c r="M11" t="n">
-        <v>6.29</v>
+        <v>6.53</v>
       </c>
       <c r="N11" t="n">
-        <v>40.05</v>
+        <v>38.87</v>
       </c>
       <c r="O11" t="n">
-        <v>40.35</v>
+        <v>40.09</v>
       </c>
       <c r="P11" t="n">
-        <v>39.14</v>
+        <v>38.86</v>
       </c>
       <c r="Q11" t="n">
-        <v>39.28</v>
+        <v>39.44</v>
       </c>
       <c r="R11" t="n">
-        <v>18.4876</v>
+        <v>-3.459</v>
       </c>
       <c r="S11" t="n">
-        <v>30.3637</v>
+        <v>22.1929</v>
       </c>
       <c r="T11" t="n">
-        <v>48.7908</v>
+        <v>43.5118</v>
       </c>
       <c r="U11" t="n">
-        <v>5.2801</v>
+        <v>-0.3417</v>
       </c>
       <c r="V11" t="n">
-        <v>7.1102</v>
+        <v>6.1339</v>
       </c>
       <c r="W11" t="n">
-        <v>10.2664</v>
+        <v>11.9841</v>
       </c>
       <c r="X11" t="n">
-        <v>-18.6287</v>
+        <v>3.8156</v>
       </c>
       <c r="Y11" t="n">
-        <v>-26.3466</v>
+        <v>-21.2304</v>
       </c>
       <c r="Z11" t="n">
-        <v>-36.7839</v>
+        <v>-34.2397</v>
       </c>
       <c r="AA11" t="n">
-        <v>-5.3494</v>
+        <v>0.4073</v>
       </c>
       <c r="AB11" t="n">
-        <v>-6.8974</v>
+        <v>-6.0057</v>
       </c>
       <c r="AC11" t="n">
-        <v>-9.7841</v>
+        <v>-11.1111</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>242.66</v>
+        <v>219</v>
       </c>
       <c r="C12" t="n">
-        <v>242.66</v>
+        <v>231.89</v>
       </c>
       <c r="D12" t="n">
-        <v>204</v>
+        <v>207.56</v>
       </c>
       <c r="E12" t="n">
-        <v>217.98</v>
+        <v>224.63</v>
       </c>
       <c r="F12" t="n">
-        <v>82.87</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="G12" t="n">
-        <v>82.91</v>
+        <v>84.05</v>
       </c>
       <c r="H12" t="n">
-        <v>80.33</v>
+        <v>80.66</v>
       </c>
       <c r="I12" t="n">
-        <v>81.67</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>5.83</v>
+        <v>6.49</v>
       </c>
       <c r="K12" t="n">
-        <v>6.91</v>
+        <v>6.83</v>
       </c>
       <c r="L12" t="n">
-        <v>5.83</v>
+        <v>6.1</v>
       </c>
       <c r="M12" t="n">
-        <v>6.53</v>
+        <v>6.31</v>
       </c>
       <c r="N12" t="n">
-        <v>38.87</v>
+        <v>39.41</v>
       </c>
       <c r="O12" t="n">
-        <v>40.09</v>
+        <v>39.94</v>
       </c>
       <c r="P12" t="n">
-        <v>38.86</v>
+        <v>38.3</v>
       </c>
       <c r="Q12" t="n">
-        <v>39.44</v>
+        <v>38.47</v>
       </c>
       <c r="R12" t="n">
-        <v>-3.459</v>
+        <v>3.0507</v>
       </c>
       <c r="S12" t="n">
-        <v>22.1929</v>
+        <v>17.8789</v>
       </c>
       <c r="T12" t="n">
-        <v>43.5118</v>
+        <v>29.694</v>
       </c>
       <c r="U12" t="n">
-        <v>-0.3417</v>
+        <v>2.4611</v>
       </c>
       <c r="V12" t="n">
-        <v>6.1339</v>
+        <v>7.5026</v>
       </c>
       <c r="W12" t="n">
-        <v>11.9841</v>
+        <v>9.3713</v>
       </c>
       <c r="X12" t="n">
-        <v>3.8156</v>
+        <v>-3.3691</v>
       </c>
       <c r="Y12" t="n">
-        <v>-21.2304</v>
+        <v>-18.37</v>
       </c>
       <c r="Z12" t="n">
-        <v>-34.2397</v>
+        <v>-26.1124</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.4073</v>
+        <v>-2.4594</v>
       </c>
       <c r="AB12" t="n">
-        <v>-6.0057</v>
+        <v>-7.3012</v>
       </c>
       <c r="AC12" t="n">
-        <v>-11.1111</v>
+        <v>-8.817299999999999</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>219</v>
+        <v>231.82</v>
       </c>
       <c r="C13" t="n">
-        <v>231.89</v>
+        <v>239.07</v>
       </c>
       <c r="D13" t="n">
-        <v>207.56</v>
+        <v>218.56</v>
       </c>
       <c r="E13" t="n">
-        <v>224.63</v>
+        <v>224.34</v>
       </c>
       <c r="F13" t="n">
-        <v>81.73999999999999</v>
+        <v>84.41</v>
       </c>
       <c r="G13" t="n">
-        <v>84.05</v>
+        <v>85.7</v>
       </c>
       <c r="H13" t="n">
-        <v>80.66</v>
+        <v>83.53</v>
       </c>
       <c r="I13" t="n">
-        <v>83.68000000000001</v>
+        <v>84.56</v>
       </c>
       <c r="J13" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="K13" t="n">
         <v>6.49</v>
       </c>
-      <c r="K13" t="n">
-        <v>6.83</v>
-      </c>
       <c r="L13" t="n">
-        <v>6.1</v>
+        <v>5.91</v>
       </c>
       <c r="M13" t="n">
-        <v>6.31</v>
+        <v>6.33</v>
       </c>
       <c r="N13" t="n">
-        <v>39.41</v>
+        <v>38.15</v>
       </c>
       <c r="O13" t="n">
-        <v>39.94</v>
+        <v>38.56</v>
       </c>
       <c r="P13" t="n">
-        <v>38.3</v>
+        <v>37.56</v>
       </c>
       <c r="Q13" t="n">
-        <v>38.47</v>
+        <v>38.08</v>
       </c>
       <c r="R13" t="n">
-        <v>3.0507</v>
+        <v>-0.1291</v>
       </c>
       <c r="S13" t="n">
-        <v>17.8789</v>
+        <v>-0.6422</v>
       </c>
       <c r="T13" t="n">
-        <v>29.694</v>
+        <v>25.7582</v>
       </c>
       <c r="U13" t="n">
-        <v>2.4611</v>
+        <v>1.0516</v>
       </c>
       <c r="V13" t="n">
-        <v>7.5026</v>
+        <v>3.1849</v>
       </c>
       <c r="W13" t="n">
-        <v>9.3713</v>
+        <v>9.8895</v>
       </c>
       <c r="X13" t="n">
-        <v>-3.3691</v>
+        <v>0.317</v>
       </c>
       <c r="Y13" t="n">
-        <v>-18.37</v>
+        <v>0.6359</v>
       </c>
       <c r="Z13" t="n">
-        <v>-26.1124</v>
+        <v>-23.6429</v>
       </c>
       <c r="AA13" t="n">
-        <v>-2.4594</v>
+        <v>-1.0138</v>
       </c>
       <c r="AB13" t="n">
-        <v>-7.3012</v>
+        <v>-3.055</v>
       </c>
       <c r="AC13" t="n">
-        <v>-8.817299999999999</v>
+        <v>-9.2469</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>231.82</v>
+        <v>217.27</v>
       </c>
       <c r="C14" t="n">
-        <v>239.07</v>
+        <v>234.06</v>
       </c>
       <c r="D14" t="n">
-        <v>218.56</v>
+        <v>210.14</v>
       </c>
       <c r="E14" t="n">
-        <v>224.34</v>
+        <v>227.03</v>
       </c>
       <c r="F14" t="n">
-        <v>84.41</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>85.7</v>
+        <v>87.06</v>
       </c>
       <c r="H14" t="n">
-        <v>83.53</v>
+        <v>83.75</v>
       </c>
       <c r="I14" t="n">
-        <v>84.56</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="J14" t="n">
-        <v>6.11</v>
+        <v>6.55</v>
       </c>
       <c r="K14" t="n">
-        <v>6.49</v>
+        <v>6.74</v>
       </c>
       <c r="L14" t="n">
-        <v>5.91</v>
+        <v>6.05</v>
       </c>
       <c r="M14" t="n">
-        <v>6.33</v>
+        <v>6.26</v>
       </c>
       <c r="N14" t="n">
-        <v>38.15</v>
+        <v>38.27</v>
       </c>
       <c r="O14" t="n">
-        <v>38.56</v>
+        <v>38.46</v>
       </c>
       <c r="P14" t="n">
-        <v>37.56</v>
+        <v>36.96</v>
       </c>
       <c r="Q14" t="n">
-        <v>38.08</v>
+        <v>37.42</v>
       </c>
       <c r="R14" t="n">
-        <v>-0.1291</v>
+        <v>1.1991</v>
       </c>
       <c r="S14" t="n">
-        <v>-0.6422</v>
+        <v>4.1518</v>
       </c>
       <c r="T14" t="n">
-        <v>25.7582</v>
+        <v>19.1383</v>
       </c>
       <c r="U14" t="n">
-        <v>1.0516</v>
+        <v>1.7502</v>
       </c>
       <c r="V14" t="n">
-        <v>3.1849</v>
+        <v>5.3508</v>
       </c>
       <c r="W14" t="n">
-        <v>9.8895</v>
+        <v>10.5344</v>
       </c>
       <c r="X14" t="n">
-        <v>0.317</v>
+        <v>-1.1058</v>
       </c>
       <c r="Y14" t="n">
-        <v>0.6359</v>
+        <v>-4.1348</v>
       </c>
       <c r="Z14" t="n">
-        <v>-23.6429</v>
+        <v>-19.0168</v>
       </c>
       <c r="AA14" t="n">
-        <v>-1.0138</v>
+        <v>-1.7332</v>
       </c>
       <c r="AB14" t="n">
-        <v>-3.055</v>
+        <v>-5.1217</v>
       </c>
       <c r="AC14" t="n">
-        <v>-9.2469</v>
+        <v>-9.831300000000001</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>217.27</v>
+        <v>243.18</v>
       </c>
       <c r="C15" t="n">
-        <v>234.06</v>
+        <v>267.08</v>
       </c>
       <c r="D15" t="n">
-        <v>210.14</v>
+        <v>238.82</v>
       </c>
       <c r="E15" t="n">
-        <v>227.03</v>
+        <v>266.32</v>
       </c>
       <c r="F15" t="n">
-        <v>84.15000000000001</v>
+        <v>85.94</v>
       </c>
       <c r="G15" t="n">
-        <v>87.06</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="H15" t="n">
-        <v>83.75</v>
+        <v>84.83</v>
       </c>
       <c r="I15" t="n">
-        <v>86.04000000000001</v>
+        <v>87.22</v>
       </c>
       <c r="J15" t="n">
-        <v>6.55</v>
+        <v>5.8</v>
       </c>
       <c r="K15" t="n">
-        <v>6.74</v>
+        <v>5.93</v>
       </c>
       <c r="L15" t="n">
-        <v>6.05</v>
+        <v>5.15</v>
       </c>
       <c r="M15" t="n">
-        <v>6.26</v>
+        <v>5.17</v>
       </c>
       <c r="N15" t="n">
-        <v>38.27</v>
+        <v>37.47</v>
       </c>
       <c r="O15" t="n">
-        <v>38.46</v>
+        <v>37.95</v>
       </c>
       <c r="P15" t="n">
-        <v>36.96</v>
+        <v>36.86</v>
       </c>
       <c r="Q15" t="n">
-        <v>37.42</v>
+        <v>36.91</v>
       </c>
       <c r="R15" t="n">
-        <v>1.1991</v>
+        <v>17.3061</v>
       </c>
       <c r="S15" t="n">
-        <v>4.1518</v>
+        <v>18.5594</v>
       </c>
       <c r="T15" t="n">
-        <v>19.1383</v>
+        <v>17.9503</v>
       </c>
       <c r="U15" t="n">
-        <v>1.7502</v>
+        <v>1.3715</v>
       </c>
       <c r="V15" t="n">
-        <v>5.3508</v>
+        <v>4.2304</v>
       </c>
       <c r="W15" t="n">
-        <v>10.5344</v>
+        <v>6.4308</v>
       </c>
       <c r="X15" t="n">
-        <v>-1.1058</v>
+        <v>-17.4121</v>
       </c>
       <c r="Y15" t="n">
-        <v>-4.1348</v>
+        <v>-18.0666</v>
       </c>
       <c r="Z15" t="n">
-        <v>-19.0168</v>
+        <v>-17.806</v>
       </c>
       <c r="AA15" t="n">
-        <v>-1.7332</v>
+        <v>-1.3629</v>
       </c>
       <c r="AB15" t="n">
-        <v>-5.1217</v>
+        <v>-4.0551</v>
       </c>
       <c r="AC15" t="n">
-        <v>-9.831300000000001</v>
+        <v>-6.0336</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>243.18</v>
+        <v>281.47</v>
       </c>
       <c r="C16" t="n">
-        <v>267.08</v>
+        <v>284.58</v>
       </c>
       <c r="D16" t="n">
-        <v>238.82</v>
+        <v>257.26</v>
       </c>
       <c r="E16" t="n">
-        <v>266.32</v>
+        <v>280.54</v>
       </c>
       <c r="F16" t="n">
-        <v>85.94</v>
+        <v>87.68000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>87.31999999999999</v>
+        <v>88.09</v>
       </c>
       <c r="H16" t="n">
-        <v>84.83</v>
+        <v>85.41</v>
       </c>
       <c r="I16" t="n">
-        <v>87.22</v>
+        <v>86.56</v>
       </c>
       <c r="J16" t="n">
-        <v>5.8</v>
+        <v>4.88</v>
       </c>
       <c r="K16" t="n">
-        <v>5.93</v>
+        <v>5.35</v>
       </c>
       <c r="L16" t="n">
-        <v>5.15</v>
+        <v>4.82</v>
       </c>
       <c r="M16" t="n">
-        <v>5.17</v>
+        <v>4.91</v>
       </c>
       <c r="N16" t="n">
-        <v>37.47</v>
+        <v>36.73</v>
       </c>
       <c r="O16" t="n">
-        <v>37.95</v>
+        <v>37.69</v>
       </c>
       <c r="P16" t="n">
-        <v>36.86</v>
+        <v>36.55</v>
       </c>
       <c r="Q16" t="n">
-        <v>36.91</v>
+        <v>37.19</v>
       </c>
       <c r="R16" t="n">
-        <v>17.3061</v>
+        <v>5.3394</v>
       </c>
       <c r="S16" t="n">
-        <v>18.5594</v>
+        <v>25.0513</v>
       </c>
       <c r="T16" t="n">
-        <v>17.9503</v>
+        <v>28.6999</v>
       </c>
       <c r="U16" t="n">
-        <v>1.3715</v>
+        <v>-0.7567</v>
       </c>
       <c r="V16" t="n">
-        <v>4.2304</v>
+        <v>2.3652</v>
       </c>
       <c r="W16" t="n">
-        <v>6.4308</v>
+        <v>5.9875</v>
       </c>
       <c r="X16" t="n">
-        <v>-17.4121</v>
+        <v>-5.029</v>
       </c>
       <c r="Y16" t="n">
-        <v>-18.0666</v>
+        <v>-22.4329</v>
       </c>
       <c r="Z16" t="n">
-        <v>-17.806</v>
+        <v>-24.8086</v>
       </c>
       <c r="AA16" t="n">
-        <v>-1.3629</v>
+        <v>0.7586000000000001</v>
       </c>
       <c r="AB16" t="n">
-        <v>-4.0551</v>
+        <v>-2.3372</v>
       </c>
       <c r="AC16" t="n">
-        <v>-6.0336</v>
+        <v>-5.7049</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>281.47</v>
+        <v>242.04</v>
       </c>
       <c r="C17" t="n">
-        <v>284.58</v>
+        <v>274.5</v>
       </c>
       <c r="D17" t="n">
-        <v>257.26</v>
+        <v>228.55</v>
       </c>
       <c r="E17" t="n">
-        <v>280.54</v>
+        <v>262.7</v>
       </c>
       <c r="F17" t="n">
-        <v>87.68000000000001</v>
+        <v>83.47</v>
       </c>
       <c r="G17" t="n">
-        <v>88.09</v>
+        <v>86.25</v>
       </c>
       <c r="H17" t="n">
-        <v>85.41</v>
+        <v>82.48</v>
       </c>
       <c r="I17" t="n">
-        <v>86.56</v>
+        <v>85.22</v>
       </c>
       <c r="J17" t="n">
-        <v>4.88</v>
+        <v>5.57</v>
       </c>
       <c r="K17" t="n">
-        <v>5.35</v>
+        <v>5.81</v>
       </c>
       <c r="L17" t="n">
-        <v>4.82</v>
+        <v>5</v>
       </c>
       <c r="M17" t="n">
-        <v>4.91</v>
+        <v>5.2</v>
       </c>
       <c r="N17" t="n">
-        <v>36.73</v>
+        <v>38.53</v>
       </c>
       <c r="O17" t="n">
-        <v>37.69</v>
+        <v>38.96</v>
       </c>
       <c r="P17" t="n">
-        <v>36.55</v>
+        <v>37.33</v>
       </c>
       <c r="Q17" t="n">
-        <v>37.19</v>
+        <v>37.76</v>
       </c>
       <c r="R17" t="n">
-        <v>5.3394</v>
+        <v>-6.3592</v>
       </c>
       <c r="S17" t="n">
-        <v>25.0513</v>
+        <v>15.7116</v>
       </c>
       <c r="T17" t="n">
-        <v>28.6999</v>
+        <v>16.9479</v>
       </c>
       <c r="U17" t="n">
-        <v>-0.7567</v>
+        <v>-1.5481</v>
       </c>
       <c r="V17" t="n">
-        <v>2.3652</v>
+        <v>-0.953</v>
       </c>
       <c r="W17" t="n">
-        <v>5.9875</v>
+        <v>1.8403</v>
       </c>
       <c r="X17" t="n">
-        <v>-5.029</v>
+        <v>5.9063</v>
       </c>
       <c r="Y17" t="n">
-        <v>-22.4329</v>
+        <v>-16.9329</v>
       </c>
       <c r="Z17" t="n">
-        <v>-24.8086</v>
+        <v>-17.5911</v>
       </c>
       <c r="AA17" t="n">
-        <v>0.7586000000000001</v>
+        <v>1.5327</v>
       </c>
       <c r="AB17" t="n">
-        <v>-2.3372</v>
+        <v>0.9086</v>
       </c>
       <c r="AC17" t="n">
-        <v>-5.7049</v>
+        <v>-1.8456</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>242.04</v>
+        <v>230.85</v>
       </c>
       <c r="C18" t="n">
-        <v>274.5</v>
+        <v>233.69</v>
       </c>
       <c r="D18" t="n">
-        <v>228.55</v>
+        <v>181.81</v>
       </c>
       <c r="E18" t="n">
-        <v>262.7</v>
+        <v>182.54</v>
       </c>
       <c r="F18" t="n">
-        <v>83.47</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="G18" t="n">
-        <v>86.25</v>
+        <v>82.08</v>
       </c>
       <c r="H18" t="n">
-        <v>82.48</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="I18" t="n">
-        <v>85.22</v>
+        <v>73.05</v>
       </c>
       <c r="J18" t="n">
-        <v>5.57</v>
+        <v>5.86</v>
       </c>
       <c r="K18" t="n">
-        <v>5.81</v>
+        <v>6.85</v>
       </c>
       <c r="L18" t="n">
-        <v>5</v>
+        <v>5.79</v>
       </c>
       <c r="M18" t="n">
-        <v>5.2</v>
+        <v>6.84</v>
       </c>
       <c r="N18" t="n">
-        <v>38.53</v>
+        <v>39.42</v>
       </c>
       <c r="O18" t="n">
-        <v>38.96</v>
+        <v>43.35</v>
       </c>
       <c r="P18" t="n">
-        <v>37.33</v>
+        <v>39.18</v>
       </c>
       <c r="Q18" t="n">
-        <v>37.76</v>
+        <v>43.19</v>
       </c>
       <c r="R18" t="n">
-        <v>-6.3592</v>
+        <v>-30.5139</v>
       </c>
       <c r="S18" t="n">
-        <v>15.7116</v>
+        <v>-31.4584</v>
       </c>
       <c r="T18" t="n">
-        <v>16.9479</v>
+        <v>-18.6324</v>
       </c>
       <c r="U18" t="n">
-        <v>-1.5481</v>
+        <v>-14.2807</v>
       </c>
       <c r="V18" t="n">
-        <v>-0.953</v>
+        <v>-16.2463</v>
       </c>
       <c r="W18" t="n">
-        <v>1.8403</v>
+        <v>-13.6116</v>
       </c>
       <c r="X18" t="n">
-        <v>5.9063</v>
+        <v>31.5385</v>
       </c>
       <c r="Y18" t="n">
-        <v>-16.9329</v>
+        <v>32.3017</v>
       </c>
       <c r="Z18" t="n">
-        <v>-17.5911</v>
+        <v>8.056900000000001</v>
       </c>
       <c r="AA18" t="n">
-        <v>1.5327</v>
+        <v>14.3803</v>
       </c>
       <c r="AB18" t="n">
-        <v>0.9086</v>
+        <v>17.0144</v>
       </c>
       <c r="AC18" t="n">
-        <v>-1.8456</v>
+        <v>13.4191</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>230.85</v>
+        <v>210.62</v>
       </c>
       <c r="C19" t="n">
-        <v>233.69</v>
+        <v>222.19</v>
       </c>
       <c r="D19" t="n">
-        <v>181.81</v>
+        <v>201.69</v>
       </c>
       <c r="E19" t="n">
-        <v>182.54</v>
+        <v>211.44</v>
       </c>
       <c r="F19" t="n">
-        <v>81.56999999999999</v>
+        <v>76.86</v>
       </c>
       <c r="G19" t="n">
-        <v>82.08</v>
+        <v>78.47</v>
       </c>
       <c r="H19" t="n">
-        <v>72.68000000000001</v>
+        <v>75.38</v>
       </c>
       <c r="I19" t="n">
-        <v>73.05</v>
+        <v>76.27</v>
       </c>
       <c r="J19" t="n">
-        <v>5.86</v>
+        <v>5.71</v>
       </c>
       <c r="K19" t="n">
-        <v>6.85</v>
+        <v>6.05</v>
       </c>
       <c r="L19" t="n">
-        <v>5.79</v>
+        <v>5.27</v>
       </c>
       <c r="M19" t="n">
-        <v>6.84</v>
+        <v>5.69</v>
       </c>
       <c r="N19" t="n">
-        <v>39.42</v>
+        <v>40.92</v>
       </c>
       <c r="O19" t="n">
-        <v>43.35</v>
+        <v>41.78</v>
       </c>
       <c r="P19" t="n">
-        <v>39.18</v>
+        <v>39.96</v>
       </c>
       <c r="Q19" t="n">
-        <v>43.19</v>
+        <v>41.26</v>
       </c>
       <c r="R19" t="n">
-        <v>-30.5139</v>
+        <v>15.8321</v>
       </c>
       <c r="S19" t="n">
-        <v>-31.4584</v>
+        <v>-24.6311</v>
       </c>
       <c r="T19" t="n">
-        <v>-18.6324</v>
+        <v>-6.8669</v>
       </c>
       <c r="U19" t="n">
-        <v>-14.2807</v>
+        <v>4.4079</v>
       </c>
       <c r="V19" t="n">
-        <v>-16.2463</v>
+        <v>-11.8877</v>
       </c>
       <c r="W19" t="n">
-        <v>-13.6116</v>
+        <v>-11.3552</v>
       </c>
       <c r="X19" t="n">
-        <v>31.5385</v>
+        <v>-16.8129</v>
       </c>
       <c r="Y19" t="n">
-        <v>32.3017</v>
+        <v>15.8859</v>
       </c>
       <c r="Z19" t="n">
-        <v>8.056900000000001</v>
+        <v>-9.105399999999999</v>
       </c>
       <c r="AA19" t="n">
-        <v>14.3803</v>
+        <v>-4.4686</v>
       </c>
       <c r="AB19" t="n">
-        <v>17.0144</v>
+        <v>10.9438</v>
       </c>
       <c r="AC19" t="n">
-        <v>13.4191</v>
+        <v>10.2619</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>210.62</v>
+        <v>227.06</v>
       </c>
       <c r="C20" t="n">
-        <v>222.19</v>
+        <v>231.02</v>
       </c>
       <c r="D20" t="n">
-        <v>201.69</v>
+        <v>157.56</v>
       </c>
       <c r="E20" t="n">
-        <v>211.44</v>
+        <v>201.68</v>
       </c>
       <c r="F20" t="n">
-        <v>76.86</v>
+        <v>78.48</v>
       </c>
       <c r="G20" t="n">
-        <v>78.47</v>
+        <v>79.34</v>
       </c>
       <c r="H20" t="n">
-        <v>75.38</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>76.27</v>
+        <v>73.72</v>
       </c>
       <c r="J20" t="n">
-        <v>5.71</v>
+        <v>5.25</v>
       </c>
       <c r="K20" t="n">
-        <v>6.05</v>
+        <v>7.11</v>
       </c>
       <c r="L20" t="n">
-        <v>5.27</v>
+        <v>5.14</v>
       </c>
       <c r="M20" t="n">
-        <v>5.69</v>
+        <v>5.93</v>
       </c>
       <c r="N20" t="n">
-        <v>40.92</v>
+        <v>40.06</v>
       </c>
       <c r="O20" t="n">
-        <v>41.78</v>
+        <v>46.38</v>
       </c>
       <c r="P20" t="n">
-        <v>39.96</v>
+        <v>39.59</v>
       </c>
       <c r="Q20" t="n">
-        <v>41.26</v>
+        <v>42.67</v>
       </c>
       <c r="R20" t="n">
-        <v>15.8321</v>
+        <v>-4.616</v>
       </c>
       <c r="S20" t="n">
-        <v>-24.6311</v>
+        <v>-23.228</v>
       </c>
       <c r="T20" t="n">
-        <v>-6.8669</v>
+        <v>-24.2716</v>
       </c>
       <c r="U20" t="n">
-        <v>4.4079</v>
+        <v>-3.3434</v>
       </c>
       <c r="V20" t="n">
-        <v>-11.8877</v>
+        <v>-13.4945</v>
       </c>
       <c r="W20" t="n">
-        <v>-11.3552</v>
+        <v>-15.4781</v>
       </c>
       <c r="X20" t="n">
-        <v>-16.8129</v>
+        <v>4.2179</v>
       </c>
       <c r="Y20" t="n">
-        <v>15.8859</v>
+        <v>14.0385</v>
       </c>
       <c r="Z20" t="n">
-        <v>-9.105399999999999</v>
+        <v>14.7002</v>
       </c>
       <c r="AA20" t="n">
-        <v>-4.4686</v>
+        <v>3.4174</v>
       </c>
       <c r="AB20" t="n">
-        <v>10.9438</v>
+        <v>13.0032</v>
       </c>
       <c r="AC20" t="n">
-        <v>10.2619</v>
+        <v>15.6055</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>227.06</v>
+        <v>191.54</v>
       </c>
       <c r="C21" t="n">
-        <v>231.02</v>
+        <v>212.99</v>
       </c>
       <c r="D21" t="n">
-        <v>157.56</v>
+        <v>177.3</v>
       </c>
       <c r="E21" t="n">
-        <v>201.68</v>
+        <v>180.65</v>
       </c>
       <c r="F21" t="n">
-        <v>78.48</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>79.34</v>
+        <v>74.7</v>
       </c>
       <c r="H21" t="n">
-        <v>66.79000000000001</v>
+        <v>69</v>
       </c>
       <c r="I21" t="n">
-        <v>73.72</v>
+        <v>69.27</v>
       </c>
       <c r="J21" t="n">
-        <v>5.25</v>
+        <v>6.24</v>
       </c>
       <c r="K21" t="n">
-        <v>7.11</v>
+        <v>6.65</v>
       </c>
       <c r="L21" t="n">
-        <v>5.14</v>
+        <v>5.6</v>
       </c>
       <c r="M21" t="n">
-        <v>5.93</v>
+        <v>6.57</v>
       </c>
       <c r="N21" t="n">
-        <v>40.06</v>
+        <v>43.81</v>
       </c>
       <c r="O21" t="n">
-        <v>46.38</v>
+        <v>45.39</v>
       </c>
       <c r="P21" t="n">
-        <v>39.59</v>
+        <v>42.07</v>
       </c>
       <c r="Q21" t="n">
-        <v>42.67</v>
+        <v>45.25</v>
       </c>
       <c r="R21" t="n">
-        <v>-4.616</v>
+        <v>-10.4274</v>
       </c>
       <c r="S21" t="n">
-        <v>-23.228</v>
+        <v>-1.0354</v>
       </c>
       <c r="T21" t="n">
-        <v>-24.2716</v>
+        <v>-35.6063</v>
       </c>
       <c r="U21" t="n">
-        <v>-3.3434</v>
+        <v>-6.0364</v>
       </c>
       <c r="V21" t="n">
-        <v>-13.4945</v>
+        <v>-5.1745</v>
       </c>
       <c r="W21" t="n">
-        <v>-15.4781</v>
+        <v>-19.9746</v>
       </c>
       <c r="X21" t="n">
-        <v>4.2179</v>
+        <v>10.7926</v>
       </c>
       <c r="Y21" t="n">
-        <v>14.0385</v>
+        <v>-3.9474</v>
       </c>
       <c r="Z21" t="n">
-        <v>14.7002</v>
+        <v>33.8086</v>
       </c>
       <c r="AA21" t="n">
-        <v>3.4174</v>
+        <v>6.0464</v>
       </c>
       <c r="AB21" t="n">
-        <v>13.0032</v>
+        <v>4.7696</v>
       </c>
       <c r="AC21" t="n">
-        <v>15.6055</v>
+        <v>21.6725</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>191.54</v>
+        <v>192.3</v>
       </c>
       <c r="C22" t="n">
-        <v>212.99</v>
+        <v>225.63</v>
       </c>
       <c r="D22" t="n">
-        <v>177.3001</v>
+        <v>192.3</v>
       </c>
       <c r="E22" t="n">
-        <v>180.65</v>
+        <v>223.99</v>
       </c>
       <c r="F22" t="n">
-        <v>71.68000000000001</v>
+        <v>70.84999999999999</v>
       </c>
       <c r="G22" t="n">
-        <v>74.7</v>
+        <v>76.5979</v>
       </c>
       <c r="H22" t="n">
-        <v>69</v>
+        <v>69.59</v>
       </c>
       <c r="I22" t="n">
-        <v>69.27</v>
+        <v>76.01000000000001</v>
       </c>
       <c r="J22" t="n">
-        <v>6.24</v>
+        <v>6.1</v>
       </c>
       <c r="K22" t="n">
-        <v>6.65</v>
+        <v>6.1</v>
       </c>
       <c r="L22" t="n">
-        <v>5.6</v>
+        <v>4.9</v>
       </c>
       <c r="M22" t="n">
-        <v>6.57</v>
+        <v>4.97</v>
       </c>
       <c r="N22" t="n">
-        <v>43.81</v>
+        <v>44.19</v>
       </c>
       <c r="O22" t="n">
-        <v>45.3899</v>
+        <v>45.005</v>
       </c>
       <c r="P22" t="n">
-        <v>42.07</v>
+        <v>40.44</v>
       </c>
       <c r="Q22" t="n">
-        <v>45.25</v>
+        <v>40.83</v>
       </c>
       <c r="R22" t="n">
-        <v>-10.4274</v>
+        <v>23.9911</v>
       </c>
       <c r="S22" t="n">
-        <v>-1.0354</v>
+        <v>5.9355</v>
       </c>
       <c r="T22" t="n">
-        <v>-35.6063</v>
+        <v>-14.7354</v>
       </c>
       <c r="U22" t="n">
-        <v>-6.0364</v>
+        <v>9.73</v>
       </c>
       <c r="V22" t="n">
-        <v>-5.1745</v>
+        <v>-0.3409</v>
       </c>
       <c r="W22" t="n">
-        <v>-19.9746</v>
+        <v>-10.8073</v>
       </c>
       <c r="X22" t="n">
-        <v>10.7926</v>
+        <v>-24.3531</v>
       </c>
       <c r="Y22" t="n">
-        <v>-3.9474</v>
+        <v>-12.6538</v>
       </c>
       <c r="Z22" t="n">
-        <v>33.8086</v>
+        <v>-4.4231</v>
       </c>
       <c r="AA22" t="n">
-        <v>6.0464</v>
+        <v>-9.768000000000001</v>
       </c>
       <c r="AB22" t="n">
-        <v>4.7696</v>
+        <v>-1.0422</v>
       </c>
       <c r="AC22" t="n">
-        <v>21.6725</v>
+        <v>8.1303</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-12 23:17
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>183.84</v>
+        <v>182.67</v>
       </c>
       <c r="C2" t="n">
-        <v>188.49</v>
+        <v>189.56</v>
       </c>
       <c r="D2" t="n">
-        <v>172.26</v>
+        <v>178.28</v>
       </c>
       <c r="E2" t="n">
-        <v>184.24</v>
+        <v>186.19</v>
       </c>
       <c r="F2" t="n">
-        <v>75.81</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>77.94</v>
+        <v>79.68000000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>74.19</v>
+        <v>77.16</v>
       </c>
       <c r="I2" t="n">
-        <v>77.23999999999999</v>
+        <v>78.95</v>
       </c>
       <c r="J2" t="n">
-        <v>8.380000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="K2" t="n">
-        <v>8.98</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L2" t="n">
-        <v>8.140000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M2" t="n">
-        <v>8.35</v>
+        <v>8.27</v>
       </c>
       <c r="N2" t="n">
-        <v>42.83</v>
+        <v>41.98</v>
       </c>
       <c r="O2" t="n">
-        <v>43.77</v>
+        <v>42.06</v>
       </c>
       <c r="P2" t="n">
-        <v>41.6</v>
+        <v>40.68</v>
       </c>
       <c r="Q2" t="n">
-        <v>41.99</v>
+        <v>41.07</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>182.67</v>
+        <v>167</v>
       </c>
       <c r="C3" t="n">
-        <v>189.56</v>
+        <v>174.4</v>
       </c>
       <c r="D3" t="n">
-        <v>178.28</v>
+        <v>161.14</v>
       </c>
       <c r="E3" t="n">
-        <v>186.19</v>
+        <v>164.18</v>
       </c>
       <c r="F3" t="n">
-        <v>77.29000000000001</v>
+        <v>75.73</v>
       </c>
       <c r="G3" t="n">
-        <v>79.68000000000001</v>
+        <v>77.37</v>
       </c>
       <c r="H3" t="n">
-        <v>77.16</v>
+        <v>74.23</v>
       </c>
       <c r="I3" t="n">
-        <v>78.95</v>
+        <v>75.34</v>
       </c>
       <c r="J3" t="n">
-        <v>8.43</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>8.630000000000001</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="L3" t="n">
-        <v>8.119999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M3" t="n">
-        <v>8.27</v>
+        <v>9.23</v>
       </c>
       <c r="N3" t="n">
-        <v>41.98</v>
+        <v>42.77</v>
       </c>
       <c r="O3" t="n">
-        <v>42.06</v>
+        <v>43.57</v>
       </c>
       <c r="P3" t="n">
-        <v>40.68</v>
+        <v>41.93</v>
       </c>
       <c r="Q3" t="n">
-        <v>41.07</v>
+        <v>42.98</v>
       </c>
       <c r="R3" t="n">
-        <v>1.0584</v>
+        <v>-11.8213</v>
       </c>
       <c r="U3" t="n">
-        <v>2.2139</v>
+        <v>-4.5725</v>
       </c>
       <c r="X3" t="n">
-        <v>-0.9581</v>
+        <v>11.6082</v>
       </c>
       <c r="AA3" t="n">
-        <v>-2.191</v>
+        <v>4.6506</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>167</v>
+        <v>172.95</v>
       </c>
       <c r="C4" t="n">
-        <v>174.4</v>
+        <v>174.61</v>
       </c>
       <c r="D4" t="n">
-        <v>161.14</v>
+        <v>142.69</v>
       </c>
       <c r="E4" t="n">
-        <v>164.18</v>
+        <v>151.75</v>
       </c>
       <c r="F4" t="n">
-        <v>75.73</v>
+        <v>76.13</v>
       </c>
       <c r="G4" t="n">
-        <v>77.37</v>
+        <v>76.27</v>
       </c>
       <c r="H4" t="n">
-        <v>74.23</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I4" t="n">
-        <v>75.34</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>9.130000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="K4" t="n">
-        <v>9.390000000000001</v>
+        <v>10.47</v>
       </c>
       <c r="L4" t="n">
-        <v>8.800000000000001</v>
+        <v>8.68</v>
       </c>
       <c r="M4" t="n">
-        <v>9.23</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="N4" t="n">
-        <v>42.77</v>
+        <v>42.51</v>
       </c>
       <c r="O4" t="n">
-        <v>43.57</v>
+        <v>44.82</v>
       </c>
       <c r="P4" t="n">
-        <v>41.93</v>
+        <v>42.44</v>
       </c>
       <c r="Q4" t="n">
-        <v>42.98</v>
+        <v>43.54</v>
       </c>
       <c r="R4" t="n">
-        <v>-11.8213</v>
+        <v>-7.571</v>
       </c>
       <c r="U4" t="n">
-        <v>-4.5725</v>
+        <v>-1.3539</v>
       </c>
       <c r="X4" t="n">
-        <v>11.6082</v>
+        <v>7.8007</v>
       </c>
       <c r="AA4" t="n">
-        <v>4.6506</v>
+        <v>1.3029</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>172.95</v>
+        <v>141.24</v>
       </c>
       <c r="C5" t="n">
-        <v>174.61</v>
+        <v>160.6</v>
       </c>
       <c r="D5" t="n">
-        <v>142.69</v>
+        <v>135.02</v>
       </c>
       <c r="E5" t="n">
-        <v>151.75</v>
+        <v>151.89</v>
       </c>
       <c r="F5" t="n">
-        <v>76.13</v>
+        <v>72.41</v>
       </c>
       <c r="G5" t="n">
-        <v>76.27</v>
+        <v>74.5</v>
       </c>
       <c r="H5" t="n">
-        <v>72.09999999999999</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="I5" t="n">
-        <v>74.31999999999999</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>8.77</v>
+        <v>10.64</v>
       </c>
       <c r="K5" t="n">
-        <v>10.47</v>
+        <v>11.07</v>
       </c>
       <c r="L5" t="n">
-        <v>8.68</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="M5" t="n">
-        <v>9.949999999999999</v>
+        <v>9.93</v>
       </c>
       <c r="N5" t="n">
-        <v>42.51</v>
+        <v>44.68</v>
       </c>
       <c r="O5" t="n">
-        <v>44.82</v>
+        <v>45.53</v>
       </c>
       <c r="P5" t="n">
-        <v>42.44</v>
+        <v>43.46</v>
       </c>
       <c r="Q5" t="n">
-        <v>43.54</v>
+        <v>44.37</v>
       </c>
       <c r="R5" t="n">
-        <v>-7.571</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="S5" t="n">
-        <v>-17.6346</v>
+        <v>-18.422</v>
       </c>
       <c r="U5" t="n">
-        <v>-1.3539</v>
+        <v>-1.8703</v>
       </c>
       <c r="V5" t="n">
-        <v>-3.7804</v>
+        <v>-7.6251</v>
       </c>
       <c r="X5" t="n">
-        <v>7.8007</v>
+        <v>-0.201</v>
       </c>
       <c r="Y5" t="n">
-        <v>19.1617</v>
+        <v>20.0726</v>
       </c>
       <c r="AA5" t="n">
-        <v>1.3029</v>
+        <v>1.9063</v>
       </c>
       <c r="AB5" t="n">
-        <v>3.6914</v>
+        <v>8.0351</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>141.24</v>
+        <v>161</v>
       </c>
       <c r="C6" t="n">
-        <v>160.6</v>
+        <v>173.7</v>
       </c>
       <c r="D6" t="n">
-        <v>135.02</v>
+        <v>161</v>
       </c>
       <c r="E6" t="n">
-        <v>151.89</v>
+        <v>173.2</v>
       </c>
       <c r="F6" t="n">
-        <v>72.41</v>
+        <v>74.09</v>
       </c>
       <c r="G6" t="n">
-        <v>74.5</v>
+        <v>76.53</v>
       </c>
       <c r="H6" t="n">
-        <v>70.95999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="I6" t="n">
-        <v>72.93000000000001</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>10.64</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>11.07</v>
+        <v>9.35</v>
       </c>
       <c r="L6" t="n">
-        <v>9.369999999999999</v>
+        <v>8.51</v>
       </c>
       <c r="M6" t="n">
-        <v>9.93</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N6" t="n">
-        <v>44.68</v>
+        <v>43.67</v>
       </c>
       <c r="O6" t="n">
-        <v>45.53</v>
+        <v>43.97</v>
       </c>
       <c r="P6" t="n">
-        <v>43.46</v>
+        <v>42.19</v>
       </c>
       <c r="Q6" t="n">
-        <v>44.37</v>
+        <v>42.19</v>
       </c>
       <c r="R6" t="n">
-        <v>0.09229999999999999</v>
+        <v>14.0299</v>
       </c>
       <c r="S6" t="n">
-        <v>-18.422</v>
+        <v>5.494</v>
       </c>
       <c r="U6" t="n">
-        <v>-1.8703</v>
+        <v>4.9088</v>
       </c>
       <c r="V6" t="n">
-        <v>-7.6251</v>
+        <v>1.553</v>
       </c>
       <c r="X6" t="n">
-        <v>-0.201</v>
+        <v>-13.998</v>
       </c>
       <c r="Y6" t="n">
-        <v>20.0726</v>
+        <v>-7.4756</v>
       </c>
       <c r="AA6" t="n">
-        <v>1.9063</v>
+        <v>-4.9132</v>
       </c>
       <c r="AB6" t="n">
-        <v>8.0351</v>
+        <v>-1.8381</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>161</v>
+        <v>171.26</v>
       </c>
       <c r="C7" t="n">
-        <v>173.7</v>
+        <v>179.97</v>
       </c>
       <c r="D7" t="n">
-        <v>161</v>
+        <v>168.23</v>
       </c>
       <c r="E7" t="n">
-        <v>173.2</v>
+        <v>178.39</v>
       </c>
       <c r="F7" t="n">
-        <v>74.09</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>76.53</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>73.62</v>
+        <v>74.47</v>
       </c>
       <c r="I7" t="n">
-        <v>76.51000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J7" t="n">
-        <v>9.300000000000001</v>
+        <v>8.65</v>
       </c>
       <c r="K7" t="n">
-        <v>9.35</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L7" t="n">
-        <v>8.51</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M7" t="n">
-        <v>8.539999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N7" t="n">
-        <v>43.67</v>
+        <v>42.94</v>
       </c>
       <c r="O7" t="n">
-        <v>43.97</v>
+        <v>43.33</v>
       </c>
       <c r="P7" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="Q7" t="n">
-        <v>42.19</v>
+        <v>41.96</v>
       </c>
       <c r="R7" t="n">
-        <v>14.0299</v>
+        <v>2.9965</v>
       </c>
       <c r="S7" t="n">
-        <v>5.494</v>
+        <v>17.5552</v>
       </c>
       <c r="T7" t="n">
-        <v>-5.9922</v>
+        <v>-4.1893</v>
       </c>
       <c r="U7" t="n">
-        <v>4.9088</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="V7" t="n">
-        <v>1.553</v>
+        <v>3.5388</v>
       </c>
       <c r="W7" t="n">
-        <v>-0.9451000000000001</v>
+        <v>-2.5332</v>
       </c>
       <c r="X7" t="n">
-        <v>-13.998</v>
+        <v>-2.9274</v>
       </c>
       <c r="Y7" t="n">
-        <v>-7.4756</v>
+        <v>-16.6834</v>
       </c>
       <c r="Z7" t="n">
-        <v>2.2754</v>
+        <v>0.2418</v>
       </c>
       <c r="AA7" t="n">
-        <v>-4.9132</v>
+        <v>-0.5452</v>
       </c>
       <c r="AB7" t="n">
-        <v>-1.8381</v>
+        <v>-3.6288</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.4763</v>
+        <v>2.167</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>171.26</v>
+        <v>184.8</v>
       </c>
       <c r="C8" t="n">
-        <v>179.97</v>
+        <v>195.27</v>
       </c>
       <c r="D8" t="n">
-        <v>168.23</v>
+        <v>183.34</v>
       </c>
       <c r="E8" t="n">
-        <v>178.39</v>
+        <v>190.56</v>
       </c>
       <c r="F8" t="n">
-        <v>75.18000000000001</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>77.79000000000001</v>
+        <v>79.33</v>
       </c>
       <c r="H8" t="n">
-        <v>74.47</v>
+        <v>77.33</v>
       </c>
       <c r="I8" t="n">
-        <v>76.95</v>
+        <v>77.84</v>
       </c>
       <c r="J8" t="n">
-        <v>8.65</v>
+        <v>8</v>
       </c>
       <c r="K8" t="n">
-        <v>8.779999999999999</v>
+        <v>8.06</v>
       </c>
       <c r="L8" t="n">
-        <v>8.210000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="M8" t="n">
-        <v>8.289999999999999</v>
+        <v>7.73</v>
       </c>
       <c r="N8" t="n">
-        <v>42.94</v>
+        <v>41.4</v>
       </c>
       <c r="O8" t="n">
-        <v>43.33</v>
+        <v>41.78</v>
       </c>
       <c r="P8" t="n">
+        <v>40.68</v>
+      </c>
+      <c r="Q8" t="n">
         <v>41.5</v>
       </c>
-      <c r="Q8" t="n">
-        <v>41.96</v>
-      </c>
       <c r="R8" t="n">
-        <v>2.9965</v>
+        <v>6.8221</v>
       </c>
       <c r="S8" t="n">
-        <v>17.5552</v>
+        <v>25.4592</v>
       </c>
       <c r="T8" t="n">
-        <v>-4.1893</v>
+        <v>16.0677</v>
       </c>
       <c r="U8" t="n">
-        <v>0.5750999999999999</v>
+        <v>1.1566</v>
       </c>
       <c r="V8" t="n">
-        <v>3.5388</v>
+        <v>6.7325</v>
       </c>
       <c r="W8" t="n">
-        <v>-2.5332</v>
+        <v>3.3183</v>
       </c>
       <c r="X8" t="n">
-        <v>-2.9274</v>
+        <v>-6.7551</v>
       </c>
       <c r="Y8" t="n">
-        <v>-16.6834</v>
+        <v>-22.1551</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.2418</v>
+        <v>-16.2514</v>
       </c>
       <c r="AA8" t="n">
-        <v>-0.5452</v>
+        <v>-1.0963</v>
       </c>
       <c r="AB8" t="n">
-        <v>-3.6288</v>
+        <v>-6.4683</v>
       </c>
       <c r="AC8" t="n">
-        <v>2.167</v>
+        <v>-3.4435</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>184.8</v>
+        <v>211.38</v>
       </c>
       <c r="C9" t="n">
-        <v>195.27</v>
+        <v>228.5</v>
       </c>
       <c r="D9" t="n">
-        <v>183.34</v>
+        <v>209.89</v>
       </c>
       <c r="E9" t="n">
-        <v>190.56</v>
+        <v>225.79</v>
       </c>
       <c r="F9" t="n">
-        <v>78.04000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="G9" t="n">
-        <v>79.33</v>
+        <v>82.27</v>
       </c>
       <c r="H9" t="n">
-        <v>77.33</v>
+        <v>79.98</v>
       </c>
       <c r="I9" t="n">
-        <v>77.84</v>
+        <v>81.95</v>
       </c>
       <c r="J9" t="n">
-        <v>8</v>
+        <v>6.9</v>
       </c>
       <c r="K9" t="n">
-        <v>8.06</v>
+        <v>6.95</v>
       </c>
       <c r="L9" t="n">
-        <v>7.5</v>
+        <v>6.19</v>
       </c>
       <c r="M9" t="n">
-        <v>7.73</v>
+        <v>6.29</v>
       </c>
       <c r="N9" t="n">
-        <v>41.4</v>
+        <v>40.05</v>
       </c>
       <c r="O9" t="n">
-        <v>41.78</v>
+        <v>40.35</v>
       </c>
       <c r="P9" t="n">
-        <v>40.68</v>
+        <v>39.14</v>
       </c>
       <c r="Q9" t="n">
-        <v>41.5</v>
+        <v>39.28</v>
       </c>
       <c r="R9" t="n">
-        <v>6.8221</v>
+        <v>18.4876</v>
       </c>
       <c r="S9" t="n">
-        <v>25.4592</v>
+        <v>30.3637</v>
       </c>
       <c r="T9" t="n">
-        <v>16.0677</v>
+        <v>48.7908</v>
       </c>
       <c r="U9" t="n">
-        <v>1.1566</v>
+        <v>5.2801</v>
       </c>
       <c r="V9" t="n">
-        <v>6.7325</v>
+        <v>7.1102</v>
       </c>
       <c r="W9" t="n">
-        <v>3.3183</v>
+        <v>10.2664</v>
       </c>
       <c r="X9" t="n">
-        <v>-6.7551</v>
+        <v>-18.6287</v>
       </c>
       <c r="Y9" t="n">
-        <v>-22.1551</v>
+        <v>-26.3466</v>
       </c>
       <c r="Z9" t="n">
-        <v>-16.2514</v>
+        <v>-36.7839</v>
       </c>
       <c r="AA9" t="n">
-        <v>-1.0963</v>
+        <v>-5.3494</v>
       </c>
       <c r="AB9" t="n">
-        <v>-6.4683</v>
+        <v>-6.8974</v>
       </c>
       <c r="AC9" t="n">
-        <v>-3.4435</v>
+        <v>-9.7841</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>211.38</v>
+        <v>242.66</v>
       </c>
       <c r="C10" t="n">
-        <v>228.5</v>
+        <v>242.66</v>
       </c>
       <c r="D10" t="n">
-        <v>209.89</v>
+        <v>204</v>
       </c>
       <c r="E10" t="n">
-        <v>225.79</v>
+        <v>217.98</v>
       </c>
       <c r="F10" t="n">
-        <v>80.59</v>
+        <v>82.87</v>
       </c>
       <c r="G10" t="n">
-        <v>82.27</v>
+        <v>82.91</v>
       </c>
       <c r="H10" t="n">
-        <v>79.98</v>
+        <v>80.33</v>
       </c>
       <c r="I10" t="n">
-        <v>81.95</v>
+        <v>81.67</v>
       </c>
       <c r="J10" t="n">
-        <v>6.9</v>
+        <v>5.83</v>
       </c>
       <c r="K10" t="n">
-        <v>6.95</v>
+        <v>6.91</v>
       </c>
       <c r="L10" t="n">
-        <v>6.19</v>
+        <v>5.83</v>
       </c>
       <c r="M10" t="n">
-        <v>6.29</v>
+        <v>6.53</v>
       </c>
       <c r="N10" t="n">
-        <v>40.05</v>
+        <v>38.87</v>
       </c>
       <c r="O10" t="n">
-        <v>40.35</v>
+        <v>40.09</v>
       </c>
       <c r="P10" t="n">
-        <v>39.14</v>
+        <v>38.86</v>
       </c>
       <c r="Q10" t="n">
-        <v>39.28</v>
+        <v>39.44</v>
       </c>
       <c r="R10" t="n">
-        <v>18.4876</v>
+        <v>-3.459</v>
       </c>
       <c r="S10" t="n">
-        <v>30.3637</v>
+        <v>22.1929</v>
       </c>
       <c r="T10" t="n">
-        <v>48.7908</v>
+        <v>43.5118</v>
       </c>
       <c r="U10" t="n">
-        <v>5.2801</v>
+        <v>-0.3417</v>
       </c>
       <c r="V10" t="n">
-        <v>7.1102</v>
+        <v>6.1339</v>
       </c>
       <c r="W10" t="n">
-        <v>10.2664</v>
+        <v>11.9841</v>
       </c>
       <c r="X10" t="n">
-        <v>-18.6287</v>
+        <v>3.8156</v>
       </c>
       <c r="Y10" t="n">
-        <v>-26.3466</v>
+        <v>-21.2304</v>
       </c>
       <c r="Z10" t="n">
-        <v>-36.7839</v>
+        <v>-34.2397</v>
       </c>
       <c r="AA10" t="n">
-        <v>-5.3494</v>
+        <v>0.4073</v>
       </c>
       <c r="AB10" t="n">
-        <v>-6.8974</v>
+        <v>-6.0057</v>
       </c>
       <c r="AC10" t="n">
-        <v>-9.7841</v>
+        <v>-11.1111</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>242.66</v>
+        <v>219</v>
       </c>
       <c r="C11" t="n">
-        <v>242.66</v>
+        <v>231.89</v>
       </c>
       <c r="D11" t="n">
-        <v>204</v>
+        <v>207.56</v>
       </c>
       <c r="E11" t="n">
-        <v>217.98</v>
+        <v>224.63</v>
       </c>
       <c r="F11" t="n">
-        <v>82.87</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>82.91</v>
+        <v>84.05</v>
       </c>
       <c r="H11" t="n">
-        <v>80.33</v>
+        <v>80.66</v>
       </c>
       <c r="I11" t="n">
-        <v>81.67</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>5.83</v>
+        <v>6.49</v>
       </c>
       <c r="K11" t="n">
-        <v>6.91</v>
+        <v>6.83</v>
       </c>
       <c r="L11" t="n">
-        <v>5.83</v>
+        <v>6.1</v>
       </c>
       <c r="M11" t="n">
-        <v>6.53</v>
+        <v>6.31</v>
       </c>
       <c r="N11" t="n">
-        <v>38.87</v>
+        <v>39.41</v>
       </c>
       <c r="O11" t="n">
-        <v>40.09</v>
+        <v>39.94</v>
       </c>
       <c r="P11" t="n">
-        <v>38.86</v>
+        <v>38.3</v>
       </c>
       <c r="Q11" t="n">
-        <v>39.44</v>
+        <v>38.47</v>
       </c>
       <c r="R11" t="n">
-        <v>-3.459</v>
+        <v>3.0507</v>
       </c>
       <c r="S11" t="n">
-        <v>22.1929</v>
+        <v>17.8789</v>
       </c>
       <c r="T11" t="n">
-        <v>43.5118</v>
+        <v>29.694</v>
       </c>
       <c r="U11" t="n">
-        <v>-0.3417</v>
+        <v>2.4611</v>
       </c>
       <c r="V11" t="n">
-        <v>6.1339</v>
+        <v>7.5026</v>
       </c>
       <c r="W11" t="n">
-        <v>11.9841</v>
+        <v>9.3713</v>
       </c>
       <c r="X11" t="n">
-        <v>3.8156</v>
+        <v>-3.3691</v>
       </c>
       <c r="Y11" t="n">
-        <v>-21.2304</v>
+        <v>-18.37</v>
       </c>
       <c r="Z11" t="n">
-        <v>-34.2397</v>
+        <v>-26.1124</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.4073</v>
+        <v>-2.4594</v>
       </c>
       <c r="AB11" t="n">
-        <v>-6.0057</v>
+        <v>-7.3012</v>
       </c>
       <c r="AC11" t="n">
-        <v>-11.1111</v>
+        <v>-8.817299999999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>219</v>
+        <v>231.82</v>
       </c>
       <c r="C12" t="n">
-        <v>231.89</v>
+        <v>239.07</v>
       </c>
       <c r="D12" t="n">
-        <v>207.56</v>
+        <v>218.56</v>
       </c>
       <c r="E12" t="n">
-        <v>224.63</v>
+        <v>224.34</v>
       </c>
       <c r="F12" t="n">
-        <v>81.73999999999999</v>
+        <v>84.41</v>
       </c>
       <c r="G12" t="n">
-        <v>84.05</v>
+        <v>85.7</v>
       </c>
       <c r="H12" t="n">
-        <v>80.66</v>
+        <v>83.53</v>
       </c>
       <c r="I12" t="n">
-        <v>83.68000000000001</v>
+        <v>84.56</v>
       </c>
       <c r="J12" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="K12" t="n">
         <v>6.49</v>
       </c>
-      <c r="K12" t="n">
-        <v>6.83</v>
-      </c>
       <c r="L12" t="n">
-        <v>6.1</v>
+        <v>5.91</v>
       </c>
       <c r="M12" t="n">
-        <v>6.31</v>
+        <v>6.33</v>
       </c>
       <c r="N12" t="n">
-        <v>39.41</v>
+        <v>38.15</v>
       </c>
       <c r="O12" t="n">
-        <v>39.94</v>
+        <v>38.56</v>
       </c>
       <c r="P12" t="n">
-        <v>38.3</v>
+        <v>37.56</v>
       </c>
       <c r="Q12" t="n">
-        <v>38.47</v>
+        <v>38.08</v>
       </c>
       <c r="R12" t="n">
-        <v>3.0507</v>
+        <v>-0.1291</v>
       </c>
       <c r="S12" t="n">
-        <v>17.8789</v>
+        <v>-0.6422</v>
       </c>
       <c r="T12" t="n">
-        <v>29.694</v>
+        <v>25.7582</v>
       </c>
       <c r="U12" t="n">
-        <v>2.4611</v>
+        <v>1.0516</v>
       </c>
       <c r="V12" t="n">
-        <v>7.5026</v>
+        <v>3.1849</v>
       </c>
       <c r="W12" t="n">
-        <v>9.3713</v>
+        <v>9.8895</v>
       </c>
       <c r="X12" t="n">
-        <v>-3.3691</v>
+        <v>0.317</v>
       </c>
       <c r="Y12" t="n">
-        <v>-18.37</v>
+        <v>0.6359</v>
       </c>
       <c r="Z12" t="n">
-        <v>-26.1124</v>
+        <v>-23.6429</v>
       </c>
       <c r="AA12" t="n">
-        <v>-2.4594</v>
+        <v>-1.0138</v>
       </c>
       <c r="AB12" t="n">
-        <v>-7.3012</v>
+        <v>-3.055</v>
       </c>
       <c r="AC12" t="n">
-        <v>-8.817299999999999</v>
+        <v>-9.2469</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>231.82</v>
+        <v>217.27</v>
       </c>
       <c r="C13" t="n">
-        <v>239.07</v>
+        <v>234.06</v>
       </c>
       <c r="D13" t="n">
-        <v>218.56</v>
+        <v>210.14</v>
       </c>
       <c r="E13" t="n">
-        <v>224.34</v>
+        <v>227.03</v>
       </c>
       <c r="F13" t="n">
-        <v>84.41</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>85.7</v>
+        <v>87.06</v>
       </c>
       <c r="H13" t="n">
-        <v>83.53</v>
+        <v>83.75</v>
       </c>
       <c r="I13" t="n">
-        <v>84.56</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>6.11</v>
+        <v>6.55</v>
       </c>
       <c r="K13" t="n">
-        <v>6.49</v>
+        <v>6.74</v>
       </c>
       <c r="L13" t="n">
-        <v>5.91</v>
+        <v>6.05</v>
       </c>
       <c r="M13" t="n">
-        <v>6.33</v>
+        <v>6.26</v>
       </c>
       <c r="N13" t="n">
-        <v>38.15</v>
+        <v>38.27</v>
       </c>
       <c r="O13" t="n">
-        <v>38.56</v>
+        <v>38.46</v>
       </c>
       <c r="P13" t="n">
-        <v>37.56</v>
+        <v>36.96</v>
       </c>
       <c r="Q13" t="n">
-        <v>38.08</v>
+        <v>37.42</v>
       </c>
       <c r="R13" t="n">
-        <v>-0.1291</v>
+        <v>1.1991</v>
       </c>
       <c r="S13" t="n">
-        <v>-0.6422</v>
+        <v>4.1518</v>
       </c>
       <c r="T13" t="n">
-        <v>25.7582</v>
+        <v>19.1383</v>
       </c>
       <c r="U13" t="n">
-        <v>1.0516</v>
+        <v>1.7502</v>
       </c>
       <c r="V13" t="n">
-        <v>3.1849</v>
+        <v>5.3508</v>
       </c>
       <c r="W13" t="n">
-        <v>9.8895</v>
+        <v>10.5344</v>
       </c>
       <c r="X13" t="n">
-        <v>0.317</v>
+        <v>-1.1058</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.6359</v>
+        <v>-4.1348</v>
       </c>
       <c r="Z13" t="n">
-        <v>-23.6429</v>
+        <v>-19.0168</v>
       </c>
       <c r="AA13" t="n">
-        <v>-1.0138</v>
+        <v>-1.7332</v>
       </c>
       <c r="AB13" t="n">
-        <v>-3.055</v>
+        <v>-5.1217</v>
       </c>
       <c r="AC13" t="n">
-        <v>-9.2469</v>
+        <v>-9.831300000000001</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>217.27</v>
+        <v>243.18</v>
       </c>
       <c r="C14" t="n">
-        <v>234.06</v>
+        <v>267.08</v>
       </c>
       <c r="D14" t="n">
-        <v>210.14</v>
+        <v>238.82</v>
       </c>
       <c r="E14" t="n">
-        <v>227.03</v>
+        <v>266.32</v>
       </c>
       <c r="F14" t="n">
-        <v>84.15000000000001</v>
+        <v>85.94</v>
       </c>
       <c r="G14" t="n">
-        <v>87.06</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>83.75</v>
+        <v>84.83</v>
       </c>
       <c r="I14" t="n">
-        <v>86.04000000000001</v>
+        <v>87.22</v>
       </c>
       <c r="J14" t="n">
-        <v>6.55</v>
+        <v>5.8</v>
       </c>
       <c r="K14" t="n">
-        <v>6.74</v>
+        <v>5.93</v>
       </c>
       <c r="L14" t="n">
-        <v>6.05</v>
+        <v>5.15</v>
       </c>
       <c r="M14" t="n">
-        <v>6.26</v>
+        <v>5.17</v>
       </c>
       <c r="N14" t="n">
-        <v>38.27</v>
+        <v>37.47</v>
       </c>
       <c r="O14" t="n">
-        <v>38.46</v>
+        <v>37.95</v>
       </c>
       <c r="P14" t="n">
-        <v>36.96</v>
+        <v>36.86</v>
       </c>
       <c r="Q14" t="n">
-        <v>37.42</v>
+        <v>36.91</v>
       </c>
       <c r="R14" t="n">
-        <v>1.1991</v>
+        <v>17.3061</v>
       </c>
       <c r="S14" t="n">
-        <v>4.1518</v>
+        <v>18.5594</v>
       </c>
       <c r="T14" t="n">
-        <v>19.1383</v>
+        <v>17.9503</v>
       </c>
       <c r="U14" t="n">
-        <v>1.7502</v>
+        <v>1.3715</v>
       </c>
       <c r="V14" t="n">
-        <v>5.3508</v>
+        <v>4.2304</v>
       </c>
       <c r="W14" t="n">
-        <v>10.5344</v>
+        <v>6.4308</v>
       </c>
       <c r="X14" t="n">
-        <v>-1.1058</v>
+        <v>-17.4121</v>
       </c>
       <c r="Y14" t="n">
-        <v>-4.1348</v>
+        <v>-18.0666</v>
       </c>
       <c r="Z14" t="n">
-        <v>-19.0168</v>
+        <v>-17.806</v>
       </c>
       <c r="AA14" t="n">
-        <v>-1.7332</v>
+        <v>-1.3629</v>
       </c>
       <c r="AB14" t="n">
-        <v>-5.1217</v>
+        <v>-4.0551</v>
       </c>
       <c r="AC14" t="n">
-        <v>-9.831300000000001</v>
+        <v>-6.0336</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>243.18</v>
+        <v>281.47</v>
       </c>
       <c r="C15" t="n">
-        <v>267.08</v>
+        <v>284.58</v>
       </c>
       <c r="D15" t="n">
-        <v>238.82</v>
+        <v>257.26</v>
       </c>
       <c r="E15" t="n">
-        <v>266.32</v>
+        <v>280.54</v>
       </c>
       <c r="F15" t="n">
-        <v>85.94</v>
+        <v>87.68000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>87.31999999999999</v>
+        <v>88.09</v>
       </c>
       <c r="H15" t="n">
-        <v>84.83</v>
+        <v>85.41</v>
       </c>
       <c r="I15" t="n">
-        <v>87.22</v>
+        <v>86.56</v>
       </c>
       <c r="J15" t="n">
-        <v>5.8</v>
+        <v>4.88</v>
       </c>
       <c r="K15" t="n">
-        <v>5.93</v>
+        <v>5.35</v>
       </c>
       <c r="L15" t="n">
-        <v>5.15</v>
+        <v>4.82</v>
       </c>
       <c r="M15" t="n">
-        <v>5.17</v>
+        <v>4.91</v>
       </c>
       <c r="N15" t="n">
-        <v>37.47</v>
+        <v>36.73</v>
       </c>
       <c r="O15" t="n">
-        <v>37.95</v>
+        <v>37.69</v>
       </c>
       <c r="P15" t="n">
-        <v>36.86</v>
+        <v>36.55</v>
       </c>
       <c r="Q15" t="n">
-        <v>36.91</v>
+        <v>37.19</v>
       </c>
       <c r="R15" t="n">
-        <v>17.3061</v>
+        <v>5.3394</v>
       </c>
       <c r="S15" t="n">
-        <v>18.5594</v>
+        <v>25.0513</v>
       </c>
       <c r="T15" t="n">
-        <v>17.9503</v>
+        <v>28.6999</v>
       </c>
       <c r="U15" t="n">
-        <v>1.3715</v>
+        <v>-0.7567</v>
       </c>
       <c r="V15" t="n">
-        <v>4.2304</v>
+        <v>2.3652</v>
       </c>
       <c r="W15" t="n">
-        <v>6.4308</v>
+        <v>5.9875</v>
       </c>
       <c r="X15" t="n">
-        <v>-17.4121</v>
+        <v>-5.029</v>
       </c>
       <c r="Y15" t="n">
-        <v>-18.0666</v>
+        <v>-22.4329</v>
       </c>
       <c r="Z15" t="n">
-        <v>-17.806</v>
+        <v>-24.8086</v>
       </c>
       <c r="AA15" t="n">
-        <v>-1.3629</v>
+        <v>0.7586000000000001</v>
       </c>
       <c r="AB15" t="n">
-        <v>-4.0551</v>
+        <v>-2.3372</v>
       </c>
       <c r="AC15" t="n">
-        <v>-6.0336</v>
+        <v>-5.7049</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>281.47</v>
+        <v>242.04</v>
       </c>
       <c r="C16" t="n">
-        <v>284.58</v>
+        <v>274.5</v>
       </c>
       <c r="D16" t="n">
-        <v>257.26</v>
+        <v>228.55</v>
       </c>
       <c r="E16" t="n">
-        <v>280.54</v>
+        <v>262.7</v>
       </c>
       <c r="F16" t="n">
-        <v>87.68000000000001</v>
+        <v>83.47</v>
       </c>
       <c r="G16" t="n">
-        <v>88.09</v>
+        <v>86.25</v>
       </c>
       <c r="H16" t="n">
-        <v>85.41</v>
+        <v>82.48</v>
       </c>
       <c r="I16" t="n">
-        <v>86.56</v>
+        <v>85.22</v>
       </c>
       <c r="J16" t="n">
-        <v>4.88</v>
+        <v>5.57</v>
       </c>
       <c r="K16" t="n">
-        <v>5.35</v>
+        <v>5.81</v>
       </c>
       <c r="L16" t="n">
-        <v>4.82</v>
+        <v>5</v>
       </c>
       <c r="M16" t="n">
-        <v>4.91</v>
+        <v>5.2</v>
       </c>
       <c r="N16" t="n">
-        <v>36.73</v>
+        <v>38.53</v>
       </c>
       <c r="O16" t="n">
-        <v>37.69</v>
+        <v>38.96</v>
       </c>
       <c r="P16" t="n">
-        <v>36.55</v>
+        <v>37.33</v>
       </c>
       <c r="Q16" t="n">
-        <v>37.19</v>
+        <v>37.76</v>
       </c>
       <c r="R16" t="n">
-        <v>5.3394</v>
+        <v>-6.3592</v>
       </c>
       <c r="S16" t="n">
-        <v>25.0513</v>
+        <v>15.7116</v>
       </c>
       <c r="T16" t="n">
-        <v>28.6999</v>
+        <v>16.9479</v>
       </c>
       <c r="U16" t="n">
-        <v>-0.7567</v>
+        <v>-1.5481</v>
       </c>
       <c r="V16" t="n">
-        <v>2.3652</v>
+        <v>-0.953</v>
       </c>
       <c r="W16" t="n">
-        <v>5.9875</v>
+        <v>1.8403</v>
       </c>
       <c r="X16" t="n">
-        <v>-5.029</v>
+        <v>5.9063</v>
       </c>
       <c r="Y16" t="n">
-        <v>-22.4329</v>
+        <v>-16.9329</v>
       </c>
       <c r="Z16" t="n">
-        <v>-24.8086</v>
+        <v>-17.5911</v>
       </c>
       <c r="AA16" t="n">
-        <v>0.7586000000000001</v>
+        <v>1.5327</v>
       </c>
       <c r="AB16" t="n">
-        <v>-2.3372</v>
+        <v>0.9086</v>
       </c>
       <c r="AC16" t="n">
-        <v>-5.7049</v>
+        <v>-1.8456</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>242.04</v>
+        <v>230.85</v>
       </c>
       <c r="C17" t="n">
-        <v>274.5</v>
+        <v>233.69</v>
       </c>
       <c r="D17" t="n">
-        <v>228.55</v>
+        <v>181.81</v>
       </c>
       <c r="E17" t="n">
-        <v>262.7</v>
+        <v>182.54</v>
       </c>
       <c r="F17" t="n">
-        <v>83.47</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="G17" t="n">
-        <v>86.25</v>
+        <v>82.08</v>
       </c>
       <c r="H17" t="n">
-        <v>82.48</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="I17" t="n">
-        <v>85.22</v>
+        <v>73.05</v>
       </c>
       <c r="J17" t="n">
-        <v>5.57</v>
+        <v>5.86</v>
       </c>
       <c r="K17" t="n">
-        <v>5.81</v>
+        <v>6.85</v>
       </c>
       <c r="L17" t="n">
-        <v>5</v>
+        <v>5.79</v>
       </c>
       <c r="M17" t="n">
-        <v>5.2</v>
+        <v>6.84</v>
       </c>
       <c r="N17" t="n">
-        <v>38.53</v>
+        <v>39.42</v>
       </c>
       <c r="O17" t="n">
-        <v>38.96</v>
+        <v>43.35</v>
       </c>
       <c r="P17" t="n">
-        <v>37.33</v>
+        <v>39.18</v>
       </c>
       <c r="Q17" t="n">
-        <v>37.76</v>
+        <v>43.19</v>
       </c>
       <c r="R17" t="n">
-        <v>-6.3592</v>
+        <v>-30.5139</v>
       </c>
       <c r="S17" t="n">
-        <v>15.7116</v>
+        <v>-31.4584</v>
       </c>
       <c r="T17" t="n">
-        <v>16.9479</v>
+        <v>-18.6324</v>
       </c>
       <c r="U17" t="n">
-        <v>-1.5481</v>
+        <v>-14.2807</v>
       </c>
       <c r="V17" t="n">
-        <v>-0.953</v>
+        <v>-16.2463</v>
       </c>
       <c r="W17" t="n">
-        <v>1.8403</v>
+        <v>-13.6116</v>
       </c>
       <c r="X17" t="n">
-        <v>5.9063</v>
+        <v>31.5385</v>
       </c>
       <c r="Y17" t="n">
-        <v>-16.9329</v>
+        <v>32.3017</v>
       </c>
       <c r="Z17" t="n">
-        <v>-17.5911</v>
+        <v>8.056900000000001</v>
       </c>
       <c r="AA17" t="n">
-        <v>1.5327</v>
+        <v>14.3803</v>
       </c>
       <c r="AB17" t="n">
-        <v>0.9086</v>
+        <v>17.0144</v>
       </c>
       <c r="AC17" t="n">
-        <v>-1.8456</v>
+        <v>13.4191</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>230.85</v>
+        <v>210.62</v>
       </c>
       <c r="C18" t="n">
-        <v>233.69</v>
+        <v>222.19</v>
       </c>
       <c r="D18" t="n">
-        <v>181.81</v>
+        <v>201.69</v>
       </c>
       <c r="E18" t="n">
-        <v>182.54</v>
+        <v>211.44</v>
       </c>
       <c r="F18" t="n">
-        <v>81.56999999999999</v>
+        <v>76.86</v>
       </c>
       <c r="G18" t="n">
-        <v>82.08</v>
+        <v>78.47</v>
       </c>
       <c r="H18" t="n">
-        <v>72.68000000000001</v>
+        <v>75.38</v>
       </c>
       <c r="I18" t="n">
-        <v>73.05</v>
+        <v>76.27</v>
       </c>
       <c r="J18" t="n">
-        <v>5.86</v>
+        <v>5.71</v>
       </c>
       <c r="K18" t="n">
-        <v>6.85</v>
+        <v>6.05</v>
       </c>
       <c r="L18" t="n">
-        <v>5.79</v>
+        <v>5.27</v>
       </c>
       <c r="M18" t="n">
-        <v>6.84</v>
+        <v>5.69</v>
       </c>
       <c r="N18" t="n">
-        <v>39.42</v>
+        <v>40.92</v>
       </c>
       <c r="O18" t="n">
-        <v>43.35</v>
+        <v>41.78</v>
       </c>
       <c r="P18" t="n">
-        <v>39.18</v>
+        <v>39.96</v>
       </c>
       <c r="Q18" t="n">
-        <v>43.19</v>
+        <v>41.26</v>
       </c>
       <c r="R18" t="n">
-        <v>-30.5139</v>
+        <v>15.8321</v>
       </c>
       <c r="S18" t="n">
-        <v>-31.4584</v>
+        <v>-24.6311</v>
       </c>
       <c r="T18" t="n">
-        <v>-18.6324</v>
+        <v>-6.8669</v>
       </c>
       <c r="U18" t="n">
-        <v>-14.2807</v>
+        <v>4.4079</v>
       </c>
       <c r="V18" t="n">
-        <v>-16.2463</v>
+        <v>-11.8877</v>
       </c>
       <c r="W18" t="n">
-        <v>-13.6116</v>
+        <v>-11.3552</v>
       </c>
       <c r="X18" t="n">
-        <v>31.5385</v>
+        <v>-16.8129</v>
       </c>
       <c r="Y18" t="n">
-        <v>32.3017</v>
+        <v>15.8859</v>
       </c>
       <c r="Z18" t="n">
-        <v>8.056900000000001</v>
+        <v>-9.105399999999999</v>
       </c>
       <c r="AA18" t="n">
-        <v>14.3803</v>
+        <v>-4.4686</v>
       </c>
       <c r="AB18" t="n">
-        <v>17.0144</v>
+        <v>10.9438</v>
       </c>
       <c r="AC18" t="n">
-        <v>13.4191</v>
+        <v>10.2619</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>210.62</v>
+        <v>227.06</v>
       </c>
       <c r="C19" t="n">
-        <v>222.19</v>
+        <v>231.02</v>
       </c>
       <c r="D19" t="n">
-        <v>201.69</v>
+        <v>157.56</v>
       </c>
       <c r="E19" t="n">
-        <v>211.44</v>
+        <v>201.68</v>
       </c>
       <c r="F19" t="n">
-        <v>76.86</v>
+        <v>78.48</v>
       </c>
       <c r="G19" t="n">
-        <v>78.47</v>
+        <v>79.34</v>
       </c>
       <c r="H19" t="n">
-        <v>75.38</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="I19" t="n">
-        <v>76.27</v>
+        <v>73.72</v>
       </c>
       <c r="J19" t="n">
-        <v>5.71</v>
+        <v>5.25</v>
       </c>
       <c r="K19" t="n">
-        <v>6.05</v>
+        <v>7.11</v>
       </c>
       <c r="L19" t="n">
-        <v>5.27</v>
+        <v>5.14</v>
       </c>
       <c r="M19" t="n">
-        <v>5.69</v>
+        <v>5.93</v>
       </c>
       <c r="N19" t="n">
-        <v>40.92</v>
+        <v>40.06</v>
       </c>
       <c r="O19" t="n">
-        <v>41.78</v>
+        <v>46.38</v>
       </c>
       <c r="P19" t="n">
-        <v>39.96</v>
+        <v>39.59</v>
       </c>
       <c r="Q19" t="n">
-        <v>41.26</v>
+        <v>42.67</v>
       </c>
       <c r="R19" t="n">
-        <v>15.8321</v>
+        <v>-4.616</v>
       </c>
       <c r="S19" t="n">
-        <v>-24.6311</v>
+        <v>-23.228</v>
       </c>
       <c r="T19" t="n">
-        <v>-6.8669</v>
+        <v>-24.2716</v>
       </c>
       <c r="U19" t="n">
-        <v>4.4079</v>
+        <v>-3.3434</v>
       </c>
       <c r="V19" t="n">
-        <v>-11.8877</v>
+        <v>-13.4945</v>
       </c>
       <c r="W19" t="n">
-        <v>-11.3552</v>
+        <v>-15.4781</v>
       </c>
       <c r="X19" t="n">
-        <v>-16.8129</v>
+        <v>4.2179</v>
       </c>
       <c r="Y19" t="n">
-        <v>15.8859</v>
+        <v>14.0385</v>
       </c>
       <c r="Z19" t="n">
-        <v>-9.105399999999999</v>
+        <v>14.7002</v>
       </c>
       <c r="AA19" t="n">
-        <v>-4.4686</v>
+        <v>3.4174</v>
       </c>
       <c r="AB19" t="n">
-        <v>10.9438</v>
+        <v>13.0032</v>
       </c>
       <c r="AC19" t="n">
-        <v>10.2619</v>
+        <v>15.6055</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>227.06</v>
+        <v>191.54</v>
       </c>
       <c r="C20" t="n">
-        <v>231.02</v>
+        <v>212.99</v>
       </c>
       <c r="D20" t="n">
-        <v>157.56</v>
+        <v>177.3</v>
       </c>
       <c r="E20" t="n">
-        <v>201.68</v>
+        <v>180.65</v>
       </c>
       <c r="F20" t="n">
-        <v>78.48</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>79.34</v>
+        <v>74.7</v>
       </c>
       <c r="H20" t="n">
-        <v>66.79000000000001</v>
+        <v>69</v>
       </c>
       <c r="I20" t="n">
-        <v>73.72</v>
+        <v>69.27</v>
       </c>
       <c r="J20" t="n">
-        <v>5.25</v>
+        <v>6.24</v>
       </c>
       <c r="K20" t="n">
-        <v>7.11</v>
+        <v>6.65</v>
       </c>
       <c r="L20" t="n">
-        <v>5.14</v>
+        <v>5.6</v>
       </c>
       <c r="M20" t="n">
-        <v>5.93</v>
+        <v>6.57</v>
       </c>
       <c r="N20" t="n">
-        <v>40.06</v>
+        <v>43.81</v>
       </c>
       <c r="O20" t="n">
-        <v>46.38</v>
+        <v>45.39</v>
       </c>
       <c r="P20" t="n">
-        <v>39.59</v>
+        <v>42.07</v>
       </c>
       <c r="Q20" t="n">
-        <v>42.67</v>
+        <v>45.25</v>
       </c>
       <c r="R20" t="n">
-        <v>-4.616</v>
+        <v>-10.4274</v>
       </c>
       <c r="S20" t="n">
-        <v>-23.228</v>
+        <v>-1.0354</v>
       </c>
       <c r="T20" t="n">
-        <v>-24.2716</v>
+        <v>-35.6063</v>
       </c>
       <c r="U20" t="n">
-        <v>-3.3434</v>
+        <v>-6.0364</v>
       </c>
       <c r="V20" t="n">
-        <v>-13.4945</v>
+        <v>-5.1745</v>
       </c>
       <c r="W20" t="n">
-        <v>-15.4781</v>
+        <v>-19.9746</v>
       </c>
       <c r="X20" t="n">
-        <v>4.2179</v>
+        <v>10.7926</v>
       </c>
       <c r="Y20" t="n">
-        <v>14.0385</v>
+        <v>-3.9474</v>
       </c>
       <c r="Z20" t="n">
-        <v>14.7002</v>
+        <v>33.8086</v>
       </c>
       <c r="AA20" t="n">
-        <v>3.4174</v>
+        <v>6.0464</v>
       </c>
       <c r="AB20" t="n">
-        <v>13.0032</v>
+        <v>4.7696</v>
       </c>
       <c r="AC20" t="n">
-        <v>15.6055</v>
+        <v>21.6725</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>191.54</v>
+        <v>192.3</v>
       </c>
       <c r="C21" t="n">
-        <v>212.99</v>
+        <v>225.63</v>
       </c>
       <c r="D21" t="n">
-        <v>177.3</v>
+        <v>192.3</v>
       </c>
       <c r="E21" t="n">
-        <v>180.65</v>
+        <v>223.99</v>
       </c>
       <c r="F21" t="n">
-        <v>71.68000000000001</v>
+        <v>70.89</v>
       </c>
       <c r="G21" t="n">
-        <v>74.7</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>69</v>
+        <v>69.59</v>
       </c>
       <c r="I21" t="n">
-        <v>69.27</v>
+        <v>76.01000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>6.24</v>
+        <v>6.1</v>
       </c>
       <c r="K21" t="n">
-        <v>6.65</v>
+        <v>6.1</v>
       </c>
       <c r="L21" t="n">
-        <v>5.6</v>
+        <v>4.9</v>
       </c>
       <c r="M21" t="n">
-        <v>6.57</v>
+        <v>4.97</v>
       </c>
       <c r="N21" t="n">
-        <v>43.81</v>
+        <v>44.18</v>
       </c>
       <c r="O21" t="n">
-        <v>45.39</v>
+        <v>45.01</v>
       </c>
       <c r="P21" t="n">
-        <v>42.07</v>
+        <v>40.44</v>
       </c>
       <c r="Q21" t="n">
-        <v>45.25</v>
+        <v>40.83</v>
       </c>
       <c r="R21" t="n">
-        <v>-10.4274</v>
+        <v>23.9911</v>
       </c>
       <c r="S21" t="n">
-        <v>-1.0354</v>
+        <v>5.9355</v>
       </c>
       <c r="T21" t="n">
-        <v>-35.6063</v>
+        <v>-14.7354</v>
       </c>
       <c r="U21" t="n">
-        <v>-6.0364</v>
+        <v>9.73</v>
       </c>
       <c r="V21" t="n">
-        <v>-5.1745</v>
+        <v>-0.3409</v>
       </c>
       <c r="W21" t="n">
-        <v>-19.9746</v>
+        <v>-10.8073</v>
       </c>
       <c r="X21" t="n">
-        <v>10.7926</v>
+        <v>-24.3531</v>
       </c>
       <c r="Y21" t="n">
-        <v>-3.9474</v>
+        <v>-12.6538</v>
       </c>
       <c r="Z21" t="n">
-        <v>33.8086</v>
+        <v>-4.4231</v>
       </c>
       <c r="AA21" t="n">
-        <v>6.0464</v>
+        <v>-9.768000000000001</v>
       </c>
       <c r="AB21" t="n">
-        <v>4.7696</v>
+        <v>-1.0422</v>
       </c>
       <c r="AC21" t="n">
-        <v>21.6725</v>
+        <v>8.1303</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>192.3</v>
+        <v>222.22</v>
       </c>
       <c r="C22" t="n">
-        <v>225.63</v>
+        <v>242.4</v>
       </c>
       <c r="D22" t="n">
-        <v>192.3</v>
+        <v>214.7406</v>
       </c>
       <c r="E22" t="n">
-        <v>223.99</v>
+        <v>234.68</v>
       </c>
       <c r="F22" t="n">
-        <v>70.84999999999999</v>
+        <v>76.34</v>
       </c>
       <c r="G22" t="n">
-        <v>76.5979</v>
+        <v>78.36</v>
       </c>
       <c r="H22" t="n">
-        <v>69.59</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="I22" t="n">
-        <v>76.01000000000001</v>
+        <v>77.52</v>
       </c>
       <c r="J22" t="n">
-        <v>6.1</v>
+        <v>5.01</v>
       </c>
       <c r="K22" t="n">
-        <v>6.1</v>
+        <v>5.15</v>
       </c>
       <c r="L22" t="n">
-        <v>4.9</v>
+        <v>4.54</v>
       </c>
       <c r="M22" t="n">
-        <v>4.97</v>
+        <v>4.72</v>
       </c>
       <c r="N22" t="n">
-        <v>44.19</v>
+        <v>40.665</v>
       </c>
       <c r="O22" t="n">
-        <v>45.005</v>
+        <v>41.7498</v>
       </c>
       <c r="P22" t="n">
-        <v>40.44</v>
+        <v>39.57</v>
       </c>
       <c r="Q22" t="n">
-        <v>40.83</v>
+        <v>40.04</v>
       </c>
       <c r="R22" t="n">
-        <v>23.9911</v>
+        <v>4.7725</v>
       </c>
       <c r="S22" t="n">
-        <v>5.9355</v>
+        <v>16.3626</v>
       </c>
       <c r="T22" t="n">
-        <v>-14.7354</v>
+        <v>28.5636</v>
       </c>
       <c r="U22" t="n">
-        <v>9.73</v>
+        <v>1.9866</v>
       </c>
       <c r="V22" t="n">
-        <v>-0.3409</v>
+        <v>5.1546</v>
       </c>
       <c r="W22" t="n">
-        <v>-10.8073</v>
+        <v>6.1191</v>
       </c>
       <c r="X22" t="n">
-        <v>-24.3531</v>
+        <v>-5.0302</v>
       </c>
       <c r="Y22" t="n">
-        <v>-12.6538</v>
+        <v>-20.4047</v>
       </c>
       <c r="Z22" t="n">
-        <v>-4.4231</v>
+        <v>-30.9942</v>
       </c>
       <c r="AA22" t="n">
-        <v>-9.768000000000001</v>
+        <v>-1.9349</v>
       </c>
       <c r="AB22" t="n">
-        <v>-1.0422</v>
+        <v>-6.1636</v>
       </c>
       <c r="AC22" t="n">
-        <v>8.1303</v>
+        <v>-7.2934</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-15 23:45
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC22"/>
+  <dimension ref="A1:AC21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1804 +568,1713 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>182.67</v>
+        <v>172.95</v>
       </c>
       <c r="C2" t="n">
-        <v>189.56</v>
+        <v>174.61</v>
       </c>
       <c r="D2" t="n">
-        <v>178.28</v>
+        <v>142.69</v>
       </c>
       <c r="E2" t="n">
-        <v>186.19</v>
+        <v>151.75</v>
       </c>
       <c r="F2" t="n">
-        <v>77.29000000000001</v>
+        <v>76.13</v>
       </c>
       <c r="G2" t="n">
-        <v>79.68000000000001</v>
+        <v>76.27</v>
       </c>
       <c r="H2" t="n">
-        <v>77.16</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>78.95</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>8.43</v>
+        <v>8.77</v>
       </c>
       <c r="K2" t="n">
-        <v>8.630000000000001</v>
+        <v>10.47</v>
       </c>
       <c r="L2" t="n">
-        <v>8.119999999999999</v>
+        <v>8.68</v>
       </c>
       <c r="M2" t="n">
-        <v>8.27</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="N2" t="n">
-        <v>41.98</v>
+        <v>42.51</v>
       </c>
       <c r="O2" t="n">
-        <v>42.06</v>
+        <v>44.82</v>
       </c>
       <c r="P2" t="n">
-        <v>40.68</v>
+        <v>42.44</v>
       </c>
       <c r="Q2" t="n">
-        <v>41.07</v>
+        <v>43.54</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>167</v>
+        <v>141.24</v>
       </c>
       <c r="C3" t="n">
-        <v>174.4</v>
+        <v>160.6</v>
       </c>
       <c r="D3" t="n">
-        <v>161.14</v>
+        <v>135.02</v>
       </c>
       <c r="E3" t="n">
-        <v>164.18</v>
+        <v>151.89</v>
       </c>
       <c r="F3" t="n">
-        <v>75.73</v>
+        <v>72.41</v>
       </c>
       <c r="G3" t="n">
-        <v>77.37</v>
+        <v>74.5</v>
       </c>
       <c r="H3" t="n">
-        <v>74.23</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="I3" t="n">
-        <v>75.34</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>9.130000000000001</v>
+        <v>10.64</v>
       </c>
       <c r="K3" t="n">
-        <v>9.390000000000001</v>
+        <v>11.07</v>
       </c>
       <c r="L3" t="n">
-        <v>8.800000000000001</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="M3" t="n">
-        <v>9.23</v>
+        <v>9.93</v>
       </c>
       <c r="N3" t="n">
-        <v>42.77</v>
+        <v>44.68</v>
       </c>
       <c r="O3" t="n">
-        <v>43.57</v>
+        <v>45.53</v>
       </c>
       <c r="P3" t="n">
-        <v>41.93</v>
+        <v>43.46</v>
       </c>
       <c r="Q3" t="n">
-        <v>42.98</v>
+        <v>44.37</v>
       </c>
       <c r="R3" t="n">
-        <v>-11.8213</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="U3" t="n">
-        <v>-4.5725</v>
+        <v>-1.8703</v>
       </c>
       <c r="X3" t="n">
-        <v>11.6082</v>
+        <v>-0.201</v>
       </c>
       <c r="AA3" t="n">
-        <v>4.6506</v>
+        <v>1.9063</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>172.95</v>
+        <v>161</v>
       </c>
       <c r="C4" t="n">
-        <v>174.61</v>
+        <v>173.7</v>
       </c>
       <c r="D4" t="n">
-        <v>142.69</v>
+        <v>161</v>
       </c>
       <c r="E4" t="n">
-        <v>151.75</v>
+        <v>173.2</v>
       </c>
       <c r="F4" t="n">
-        <v>76.13</v>
+        <v>74.09</v>
       </c>
       <c r="G4" t="n">
-        <v>76.27</v>
+        <v>76.53</v>
       </c>
       <c r="H4" t="n">
-        <v>72.09999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="I4" t="n">
-        <v>74.31999999999999</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>8.77</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>10.47</v>
+        <v>9.35</v>
       </c>
       <c r="L4" t="n">
-        <v>8.68</v>
+        <v>8.51</v>
       </c>
       <c r="M4" t="n">
-        <v>9.949999999999999</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N4" t="n">
-        <v>42.51</v>
+        <v>43.67</v>
       </c>
       <c r="O4" t="n">
-        <v>44.82</v>
+        <v>43.97</v>
       </c>
       <c r="P4" t="n">
-        <v>42.44</v>
+        <v>42.19</v>
       </c>
       <c r="Q4" t="n">
-        <v>43.54</v>
+        <v>42.19</v>
       </c>
       <c r="R4" t="n">
-        <v>-7.571</v>
+        <v>14.0299</v>
       </c>
       <c r="U4" t="n">
-        <v>-1.3539</v>
+        <v>4.9088</v>
       </c>
       <c r="X4" t="n">
-        <v>7.8007</v>
+        <v>-13.998</v>
       </c>
       <c r="AA4" t="n">
-        <v>1.3029</v>
+        <v>-4.9132</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>141.24</v>
+        <v>171.26</v>
       </c>
       <c r="C5" t="n">
-        <v>160.6</v>
+        <v>179.97</v>
       </c>
       <c r="D5" t="n">
-        <v>135.02</v>
+        <v>168.23</v>
       </c>
       <c r="E5" t="n">
-        <v>151.89</v>
+        <v>178.39</v>
       </c>
       <c r="F5" t="n">
-        <v>72.41</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>74.5</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>70.95999999999999</v>
+        <v>74.47</v>
       </c>
       <c r="I5" t="n">
-        <v>72.93000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J5" t="n">
-        <v>10.64</v>
+        <v>8.65</v>
       </c>
       <c r="K5" t="n">
-        <v>11.07</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L5" t="n">
-        <v>9.369999999999999</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>9.93</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N5" t="n">
-        <v>44.68</v>
+        <v>42.94</v>
       </c>
       <c r="O5" t="n">
-        <v>45.53</v>
+        <v>43.33</v>
       </c>
       <c r="P5" t="n">
-        <v>43.46</v>
+        <v>41.5</v>
       </c>
       <c r="Q5" t="n">
-        <v>44.37</v>
+        <v>41.96</v>
       </c>
       <c r="R5" t="n">
-        <v>0.09229999999999999</v>
+        <v>2.9965</v>
       </c>
       <c r="S5" t="n">
-        <v>-18.422</v>
+        <v>17.5552</v>
       </c>
       <c r="U5" t="n">
-        <v>-1.8703</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="V5" t="n">
-        <v>-7.6251</v>
+        <v>3.5388</v>
       </c>
       <c r="X5" t="n">
-        <v>-0.201</v>
+        <v>-2.9274</v>
       </c>
       <c r="Y5" t="n">
-        <v>20.0726</v>
+        <v>-16.6834</v>
       </c>
       <c r="AA5" t="n">
-        <v>1.9063</v>
+        <v>-0.5452</v>
       </c>
       <c r="AB5" t="n">
-        <v>8.0351</v>
+        <v>-3.6288</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>161</v>
+        <v>184.8</v>
       </c>
       <c r="C6" t="n">
-        <v>173.7</v>
+        <v>195.27</v>
       </c>
       <c r="D6" t="n">
-        <v>161</v>
+        <v>183.34</v>
       </c>
       <c r="E6" t="n">
-        <v>173.2</v>
+        <v>190.56</v>
       </c>
       <c r="F6" t="n">
-        <v>74.09</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>76.53</v>
+        <v>79.33</v>
       </c>
       <c r="H6" t="n">
-        <v>73.62</v>
+        <v>77.33</v>
       </c>
       <c r="I6" t="n">
-        <v>76.51000000000001</v>
+        <v>77.84</v>
       </c>
       <c r="J6" t="n">
-        <v>9.300000000000001</v>
+        <v>8</v>
       </c>
       <c r="K6" t="n">
-        <v>9.35</v>
+        <v>8.06</v>
       </c>
       <c r="L6" t="n">
-        <v>8.51</v>
+        <v>7.5</v>
       </c>
       <c r="M6" t="n">
-        <v>8.539999999999999</v>
+        <v>7.73</v>
       </c>
       <c r="N6" t="n">
-        <v>43.67</v>
+        <v>41.4</v>
       </c>
       <c r="O6" t="n">
-        <v>43.97</v>
+        <v>41.78</v>
       </c>
       <c r="P6" t="n">
-        <v>42.19</v>
+        <v>40.68</v>
       </c>
       <c r="Q6" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="R6" t="n">
-        <v>14.0299</v>
+        <v>6.8221</v>
       </c>
       <c r="S6" t="n">
-        <v>5.494</v>
+        <v>25.4592</v>
       </c>
       <c r="U6" t="n">
-        <v>4.9088</v>
+        <v>1.1566</v>
       </c>
       <c r="V6" t="n">
-        <v>1.553</v>
+        <v>6.7325</v>
       </c>
       <c r="X6" t="n">
-        <v>-13.998</v>
+        <v>-6.7551</v>
       </c>
       <c r="Y6" t="n">
-        <v>-7.4756</v>
+        <v>-22.1551</v>
       </c>
       <c r="AA6" t="n">
-        <v>-4.9132</v>
+        <v>-1.0963</v>
       </c>
       <c r="AB6" t="n">
-        <v>-1.8381</v>
+        <v>-6.4683</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>171.26</v>
+        <v>211.38</v>
       </c>
       <c r="C7" t="n">
-        <v>179.97</v>
+        <v>228.5</v>
       </c>
       <c r="D7" t="n">
-        <v>168.23</v>
+        <v>209.89</v>
       </c>
       <c r="E7" t="n">
-        <v>178.39</v>
+        <v>225.79</v>
       </c>
       <c r="F7" t="n">
-        <v>75.18000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="G7" t="n">
-        <v>77.79000000000001</v>
+        <v>82.27</v>
       </c>
       <c r="H7" t="n">
-        <v>74.47</v>
+        <v>79.98</v>
       </c>
       <c r="I7" t="n">
-        <v>76.95</v>
+        <v>81.95</v>
       </c>
       <c r="J7" t="n">
-        <v>8.65</v>
+        <v>6.9</v>
       </c>
       <c r="K7" t="n">
-        <v>8.779999999999999</v>
+        <v>6.95</v>
       </c>
       <c r="L7" t="n">
-        <v>8.210000000000001</v>
+        <v>6.19</v>
       </c>
       <c r="M7" t="n">
-        <v>8.289999999999999</v>
+        <v>6.29</v>
       </c>
       <c r="N7" t="n">
-        <v>42.94</v>
+        <v>40.05</v>
       </c>
       <c r="O7" t="n">
-        <v>43.33</v>
+        <v>40.35</v>
       </c>
       <c r="P7" t="n">
-        <v>41.5</v>
+        <v>39.14</v>
       </c>
       <c r="Q7" t="n">
-        <v>41.96</v>
+        <v>39.28</v>
       </c>
       <c r="R7" t="n">
-        <v>2.9965</v>
+        <v>18.4876</v>
       </c>
       <c r="S7" t="n">
-        <v>17.5552</v>
+        <v>30.3637</v>
       </c>
       <c r="T7" t="n">
-        <v>-4.1893</v>
+        <v>48.7908</v>
       </c>
       <c r="U7" t="n">
-        <v>0.5750999999999999</v>
+        <v>5.2801</v>
       </c>
       <c r="V7" t="n">
-        <v>3.5388</v>
+        <v>7.1102</v>
       </c>
       <c r="W7" t="n">
-        <v>-2.5332</v>
+        <v>10.2664</v>
       </c>
       <c r="X7" t="n">
-        <v>-2.9274</v>
+        <v>-18.6287</v>
       </c>
       <c r="Y7" t="n">
-        <v>-16.6834</v>
+        <v>-26.3466</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.2418</v>
+        <v>-36.7839</v>
       </c>
       <c r="AA7" t="n">
-        <v>-0.5452</v>
+        <v>-5.3494</v>
       </c>
       <c r="AB7" t="n">
-        <v>-3.6288</v>
+        <v>-6.8974</v>
       </c>
       <c r="AC7" t="n">
-        <v>2.167</v>
+        <v>-9.7841</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>184.8</v>
+        <v>242.66</v>
       </c>
       <c r="C8" t="n">
-        <v>195.27</v>
+        <v>242.66</v>
       </c>
       <c r="D8" t="n">
-        <v>183.34</v>
+        <v>204</v>
       </c>
       <c r="E8" t="n">
-        <v>190.56</v>
+        <v>217.98</v>
       </c>
       <c r="F8" t="n">
-        <v>78.04000000000001</v>
+        <v>82.87</v>
       </c>
       <c r="G8" t="n">
-        <v>79.33</v>
+        <v>82.91</v>
       </c>
       <c r="H8" t="n">
-        <v>77.33</v>
+        <v>80.33</v>
       </c>
       <c r="I8" t="n">
-        <v>77.84</v>
+        <v>81.67</v>
       </c>
       <c r="J8" t="n">
-        <v>8</v>
+        <v>5.83</v>
       </c>
       <c r="K8" t="n">
-        <v>8.06</v>
+        <v>6.91</v>
       </c>
       <c r="L8" t="n">
-        <v>7.5</v>
+        <v>5.83</v>
       </c>
       <c r="M8" t="n">
-        <v>7.73</v>
+        <v>6.53</v>
       </c>
       <c r="N8" t="n">
-        <v>41.4</v>
+        <v>38.87</v>
       </c>
       <c r="O8" t="n">
-        <v>41.78</v>
+        <v>40.09</v>
       </c>
       <c r="P8" t="n">
-        <v>40.68</v>
+        <v>38.86</v>
       </c>
       <c r="Q8" t="n">
-        <v>41.5</v>
+        <v>39.44</v>
       </c>
       <c r="R8" t="n">
-        <v>6.8221</v>
+        <v>-3.459</v>
       </c>
       <c r="S8" t="n">
-        <v>25.4592</v>
+        <v>22.1929</v>
       </c>
       <c r="T8" t="n">
-        <v>16.0677</v>
+        <v>43.5118</v>
       </c>
       <c r="U8" t="n">
-        <v>1.1566</v>
+        <v>-0.3417</v>
       </c>
       <c r="V8" t="n">
-        <v>6.7325</v>
+        <v>6.1339</v>
       </c>
       <c r="W8" t="n">
-        <v>3.3183</v>
+        <v>11.9841</v>
       </c>
       <c r="X8" t="n">
-        <v>-6.7551</v>
+        <v>3.8156</v>
       </c>
       <c r="Y8" t="n">
-        <v>-22.1551</v>
+        <v>-21.2304</v>
       </c>
       <c r="Z8" t="n">
-        <v>-16.2514</v>
+        <v>-34.2397</v>
       </c>
       <c r="AA8" t="n">
-        <v>-1.0963</v>
+        <v>0.4073</v>
       </c>
       <c r="AB8" t="n">
-        <v>-6.4683</v>
+        <v>-6.0057</v>
       </c>
       <c r="AC8" t="n">
-        <v>-3.4435</v>
+        <v>-11.1111</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>211.38</v>
+        <v>219</v>
       </c>
       <c r="C9" t="n">
-        <v>228.5</v>
+        <v>231.89</v>
       </c>
       <c r="D9" t="n">
-        <v>209.89</v>
+        <v>207.56</v>
       </c>
       <c r="E9" t="n">
-        <v>225.79</v>
+        <v>224.63</v>
       </c>
       <c r="F9" t="n">
-        <v>80.59</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>82.27</v>
+        <v>84.05</v>
       </c>
       <c r="H9" t="n">
-        <v>79.98</v>
+        <v>80.66</v>
       </c>
       <c r="I9" t="n">
-        <v>81.95</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>6.9</v>
+        <v>6.49</v>
       </c>
       <c r="K9" t="n">
-        <v>6.95</v>
+        <v>6.83</v>
       </c>
       <c r="L9" t="n">
-        <v>6.19</v>
+        <v>6.1</v>
       </c>
       <c r="M9" t="n">
-        <v>6.29</v>
+        <v>6.31</v>
       </c>
       <c r="N9" t="n">
-        <v>40.05</v>
+        <v>39.41</v>
       </c>
       <c r="O9" t="n">
-        <v>40.35</v>
+        <v>39.94</v>
       </c>
       <c r="P9" t="n">
-        <v>39.14</v>
+        <v>38.3</v>
       </c>
       <c r="Q9" t="n">
-        <v>39.28</v>
+        <v>38.47</v>
       </c>
       <c r="R9" t="n">
-        <v>18.4876</v>
+        <v>3.0507</v>
       </c>
       <c r="S9" t="n">
-        <v>30.3637</v>
+        <v>17.8789</v>
       </c>
       <c r="T9" t="n">
-        <v>48.7908</v>
+        <v>29.694</v>
       </c>
       <c r="U9" t="n">
-        <v>5.2801</v>
+        <v>2.4611</v>
       </c>
       <c r="V9" t="n">
-        <v>7.1102</v>
+        <v>7.5026</v>
       </c>
       <c r="W9" t="n">
-        <v>10.2664</v>
+        <v>9.3713</v>
       </c>
       <c r="X9" t="n">
-        <v>-18.6287</v>
+        <v>-3.3691</v>
       </c>
       <c r="Y9" t="n">
-        <v>-26.3466</v>
+        <v>-18.37</v>
       </c>
       <c r="Z9" t="n">
-        <v>-36.7839</v>
+        <v>-26.1124</v>
       </c>
       <c r="AA9" t="n">
-        <v>-5.3494</v>
+        <v>-2.4594</v>
       </c>
       <c r="AB9" t="n">
-        <v>-6.8974</v>
+        <v>-7.3012</v>
       </c>
       <c r="AC9" t="n">
-        <v>-9.7841</v>
+        <v>-8.817299999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>242.66</v>
+        <v>231.82</v>
       </c>
       <c r="C10" t="n">
-        <v>242.66</v>
+        <v>239.07</v>
       </c>
       <c r="D10" t="n">
-        <v>204</v>
+        <v>218.56</v>
       </c>
       <c r="E10" t="n">
-        <v>217.98</v>
+        <v>224.34</v>
       </c>
       <c r="F10" t="n">
-        <v>82.87</v>
+        <v>84.41</v>
       </c>
       <c r="G10" t="n">
-        <v>82.91</v>
+        <v>85.7</v>
       </c>
       <c r="H10" t="n">
-        <v>80.33</v>
+        <v>83.53</v>
       </c>
       <c r="I10" t="n">
-        <v>81.67</v>
+        <v>84.56</v>
       </c>
       <c r="J10" t="n">
-        <v>5.83</v>
+        <v>6.11</v>
       </c>
       <c r="K10" t="n">
-        <v>6.91</v>
+        <v>6.49</v>
       </c>
       <c r="L10" t="n">
-        <v>5.83</v>
+        <v>5.91</v>
       </c>
       <c r="M10" t="n">
-        <v>6.53</v>
+        <v>6.33</v>
       </c>
       <c r="N10" t="n">
-        <v>38.87</v>
+        <v>38.15</v>
       </c>
       <c r="O10" t="n">
-        <v>40.09</v>
+        <v>38.56</v>
       </c>
       <c r="P10" t="n">
-        <v>38.86</v>
+        <v>37.56</v>
       </c>
       <c r="Q10" t="n">
-        <v>39.44</v>
+        <v>38.08</v>
       </c>
       <c r="R10" t="n">
-        <v>-3.459</v>
+        <v>-0.1291</v>
       </c>
       <c r="S10" t="n">
-        <v>22.1929</v>
+        <v>-0.6422</v>
       </c>
       <c r="T10" t="n">
-        <v>43.5118</v>
+        <v>25.7582</v>
       </c>
       <c r="U10" t="n">
-        <v>-0.3417</v>
+        <v>1.0516</v>
       </c>
       <c r="V10" t="n">
-        <v>6.1339</v>
+        <v>3.1849</v>
       </c>
       <c r="W10" t="n">
-        <v>11.9841</v>
+        <v>9.8895</v>
       </c>
       <c r="X10" t="n">
-        <v>3.8156</v>
+        <v>0.317</v>
       </c>
       <c r="Y10" t="n">
-        <v>-21.2304</v>
+        <v>0.6359</v>
       </c>
       <c r="Z10" t="n">
-        <v>-34.2397</v>
+        <v>-23.6429</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.4073</v>
+        <v>-1.0138</v>
       </c>
       <c r="AB10" t="n">
-        <v>-6.0057</v>
+        <v>-3.055</v>
       </c>
       <c r="AC10" t="n">
-        <v>-11.1111</v>
+        <v>-9.2469</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>219</v>
+        <v>217.27</v>
       </c>
       <c r="C11" t="n">
-        <v>231.89</v>
+        <v>234.06</v>
       </c>
       <c r="D11" t="n">
-        <v>207.56</v>
+        <v>210.14</v>
       </c>
       <c r="E11" t="n">
-        <v>224.63</v>
+        <v>227.03</v>
       </c>
       <c r="F11" t="n">
-        <v>81.73999999999999</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>84.05</v>
+        <v>87.06</v>
       </c>
       <c r="H11" t="n">
-        <v>80.66</v>
+        <v>83.75</v>
       </c>
       <c r="I11" t="n">
-        <v>83.68000000000001</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>6.49</v>
+        <v>6.55</v>
       </c>
       <c r="K11" t="n">
-        <v>6.83</v>
+        <v>6.74</v>
       </c>
       <c r="L11" t="n">
-        <v>6.1</v>
+        <v>6.05</v>
       </c>
       <c r="M11" t="n">
-        <v>6.31</v>
+        <v>6.26</v>
       </c>
       <c r="N11" t="n">
-        <v>39.41</v>
+        <v>38.27</v>
       </c>
       <c r="O11" t="n">
-        <v>39.94</v>
+        <v>38.46</v>
       </c>
       <c r="P11" t="n">
-        <v>38.3</v>
+        <v>36.96</v>
       </c>
       <c r="Q11" t="n">
-        <v>38.47</v>
+        <v>37.42</v>
       </c>
       <c r="R11" t="n">
-        <v>3.0507</v>
+        <v>1.1991</v>
       </c>
       <c r="S11" t="n">
-        <v>17.8789</v>
+        <v>4.1518</v>
       </c>
       <c r="T11" t="n">
-        <v>29.694</v>
+        <v>19.1383</v>
       </c>
       <c r="U11" t="n">
-        <v>2.4611</v>
+        <v>1.7502</v>
       </c>
       <c r="V11" t="n">
-        <v>7.5026</v>
+        <v>5.3508</v>
       </c>
       <c r="W11" t="n">
-        <v>9.3713</v>
+        <v>10.5344</v>
       </c>
       <c r="X11" t="n">
-        <v>-3.3691</v>
+        <v>-1.1058</v>
       </c>
       <c r="Y11" t="n">
-        <v>-18.37</v>
+        <v>-4.1348</v>
       </c>
       <c r="Z11" t="n">
-        <v>-26.1124</v>
+        <v>-19.0168</v>
       </c>
       <c r="AA11" t="n">
-        <v>-2.4594</v>
+        <v>-1.7332</v>
       </c>
       <c r="AB11" t="n">
-        <v>-7.3012</v>
+        <v>-5.1217</v>
       </c>
       <c r="AC11" t="n">
-        <v>-8.817299999999999</v>
+        <v>-9.831300000000001</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>231.82</v>
+        <v>243.18</v>
       </c>
       <c r="C12" t="n">
-        <v>239.07</v>
+        <v>267.08</v>
       </c>
       <c r="D12" t="n">
-        <v>218.56</v>
+        <v>238.82</v>
       </c>
       <c r="E12" t="n">
-        <v>224.34</v>
+        <v>266.32</v>
       </c>
       <c r="F12" t="n">
-        <v>84.41</v>
+        <v>85.94</v>
       </c>
       <c r="G12" t="n">
-        <v>85.7</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>83.53</v>
+        <v>84.83</v>
       </c>
       <c r="I12" t="n">
-        <v>84.56</v>
+        <v>87.22</v>
       </c>
       <c r="J12" t="n">
-        <v>6.11</v>
+        <v>5.8</v>
       </c>
       <c r="K12" t="n">
-        <v>6.49</v>
+        <v>5.93</v>
       </c>
       <c r="L12" t="n">
-        <v>5.91</v>
+        <v>5.15</v>
       </c>
       <c r="M12" t="n">
-        <v>6.33</v>
+        <v>5.17</v>
       </c>
       <c r="N12" t="n">
-        <v>38.15</v>
+        <v>37.47</v>
       </c>
       <c r="O12" t="n">
-        <v>38.56</v>
+        <v>37.95</v>
       </c>
       <c r="P12" t="n">
-        <v>37.56</v>
+        <v>36.86</v>
       </c>
       <c r="Q12" t="n">
-        <v>38.08</v>
+        <v>36.91</v>
       </c>
       <c r="R12" t="n">
-        <v>-0.1291</v>
+        <v>17.3061</v>
       </c>
       <c r="S12" t="n">
-        <v>-0.6422</v>
+        <v>18.5594</v>
       </c>
       <c r="T12" t="n">
-        <v>25.7582</v>
+        <v>17.9503</v>
       </c>
       <c r="U12" t="n">
-        <v>1.0516</v>
+        <v>1.3715</v>
       </c>
       <c r="V12" t="n">
-        <v>3.1849</v>
+        <v>4.2304</v>
       </c>
       <c r="W12" t="n">
-        <v>9.8895</v>
+        <v>6.4308</v>
       </c>
       <c r="X12" t="n">
-        <v>0.317</v>
+        <v>-17.4121</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.6359</v>
+        <v>-18.0666</v>
       </c>
       <c r="Z12" t="n">
-        <v>-23.6429</v>
+        <v>-17.806</v>
       </c>
       <c r="AA12" t="n">
-        <v>-1.0138</v>
+        <v>-1.3629</v>
       </c>
       <c r="AB12" t="n">
-        <v>-3.055</v>
+        <v>-4.0551</v>
       </c>
       <c r="AC12" t="n">
-        <v>-9.2469</v>
+        <v>-6.0336</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>217.27</v>
+        <v>281.47</v>
       </c>
       <c r="C13" t="n">
-        <v>234.06</v>
+        <v>284.58</v>
       </c>
       <c r="D13" t="n">
-        <v>210.14</v>
+        <v>257.26</v>
       </c>
       <c r="E13" t="n">
-        <v>227.03</v>
+        <v>280.54</v>
       </c>
       <c r="F13" t="n">
-        <v>84.15000000000001</v>
+        <v>87.68000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>87.06</v>
+        <v>88.09</v>
       </c>
       <c r="H13" t="n">
-        <v>83.75</v>
+        <v>85.41</v>
       </c>
       <c r="I13" t="n">
-        <v>86.04000000000001</v>
+        <v>86.56</v>
       </c>
       <c r="J13" t="n">
-        <v>6.55</v>
+        <v>4.88</v>
       </c>
       <c r="K13" t="n">
-        <v>6.74</v>
+        <v>5.35</v>
       </c>
       <c r="L13" t="n">
-        <v>6.05</v>
+        <v>4.82</v>
       </c>
       <c r="M13" t="n">
-        <v>6.26</v>
+        <v>4.91</v>
       </c>
       <c r="N13" t="n">
-        <v>38.27</v>
+        <v>36.73</v>
       </c>
       <c r="O13" t="n">
-        <v>38.46</v>
+        <v>37.69</v>
       </c>
       <c r="P13" t="n">
-        <v>36.96</v>
+        <v>36.55</v>
       </c>
       <c r="Q13" t="n">
-        <v>37.42</v>
+        <v>37.19</v>
       </c>
       <c r="R13" t="n">
-        <v>1.1991</v>
+        <v>5.3394</v>
       </c>
       <c r="S13" t="n">
-        <v>4.1518</v>
+        <v>25.0513</v>
       </c>
       <c r="T13" t="n">
-        <v>19.1383</v>
+        <v>28.6999</v>
       </c>
       <c r="U13" t="n">
-        <v>1.7502</v>
+        <v>-0.7567</v>
       </c>
       <c r="V13" t="n">
-        <v>5.3508</v>
+        <v>2.3652</v>
       </c>
       <c r="W13" t="n">
-        <v>10.5344</v>
+        <v>5.9875</v>
       </c>
       <c r="X13" t="n">
-        <v>-1.1058</v>
+        <v>-5.029</v>
       </c>
       <c r="Y13" t="n">
-        <v>-4.1348</v>
+        <v>-22.4329</v>
       </c>
       <c r="Z13" t="n">
-        <v>-19.0168</v>
+        <v>-24.8086</v>
       </c>
       <c r="AA13" t="n">
-        <v>-1.7332</v>
+        <v>0.7586000000000001</v>
       </c>
       <c r="AB13" t="n">
-        <v>-5.1217</v>
+        <v>-2.3372</v>
       </c>
       <c r="AC13" t="n">
-        <v>-9.831300000000001</v>
+        <v>-5.7049</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>243.18</v>
+        <v>242.04</v>
       </c>
       <c r="C14" t="n">
-        <v>267.08</v>
+        <v>274.5</v>
       </c>
       <c r="D14" t="n">
-        <v>238.82</v>
+        <v>228.55</v>
       </c>
       <c r="E14" t="n">
-        <v>266.32</v>
+        <v>262.7</v>
       </c>
       <c r="F14" t="n">
-        <v>85.94</v>
+        <v>83.47</v>
       </c>
       <c r="G14" t="n">
-        <v>87.31999999999999</v>
+        <v>86.25</v>
       </c>
       <c r="H14" t="n">
-        <v>84.83</v>
+        <v>82.48</v>
       </c>
       <c r="I14" t="n">
-        <v>87.22</v>
+        <v>85.22</v>
       </c>
       <c r="J14" t="n">
-        <v>5.8</v>
+        <v>5.57</v>
       </c>
       <c r="K14" t="n">
-        <v>5.93</v>
+        <v>5.81</v>
       </c>
       <c r="L14" t="n">
-        <v>5.15</v>
+        <v>5</v>
       </c>
       <c r="M14" t="n">
-        <v>5.17</v>
+        <v>5.2</v>
       </c>
       <c r="N14" t="n">
-        <v>37.47</v>
+        <v>38.53</v>
       </c>
       <c r="O14" t="n">
-        <v>37.95</v>
+        <v>38.96</v>
       </c>
       <c r="P14" t="n">
-        <v>36.86</v>
+        <v>37.33</v>
       </c>
       <c r="Q14" t="n">
-        <v>36.91</v>
+        <v>37.76</v>
       </c>
       <c r="R14" t="n">
-        <v>17.3061</v>
+        <v>-6.3592</v>
       </c>
       <c r="S14" t="n">
-        <v>18.5594</v>
+        <v>15.7116</v>
       </c>
       <c r="T14" t="n">
-        <v>17.9503</v>
+        <v>16.9479</v>
       </c>
       <c r="U14" t="n">
-        <v>1.3715</v>
+        <v>-1.5481</v>
       </c>
       <c r="V14" t="n">
-        <v>4.2304</v>
+        <v>-0.953</v>
       </c>
       <c r="W14" t="n">
-        <v>6.4308</v>
+        <v>1.8403</v>
       </c>
       <c r="X14" t="n">
-        <v>-17.4121</v>
+        <v>5.9063</v>
       </c>
       <c r="Y14" t="n">
-        <v>-18.0666</v>
+        <v>-16.9329</v>
       </c>
       <c r="Z14" t="n">
-        <v>-17.806</v>
+        <v>-17.5911</v>
       </c>
       <c r="AA14" t="n">
-        <v>-1.3629</v>
+        <v>1.5327</v>
       </c>
       <c r="AB14" t="n">
-        <v>-4.0551</v>
+        <v>0.9086</v>
       </c>
       <c r="AC14" t="n">
-        <v>-6.0336</v>
+        <v>-1.8456</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>281.47</v>
+        <v>230.85</v>
       </c>
       <c r="C15" t="n">
-        <v>284.58</v>
+        <v>233.69</v>
       </c>
       <c r="D15" t="n">
-        <v>257.26</v>
+        <v>181.81</v>
       </c>
       <c r="E15" t="n">
-        <v>280.54</v>
+        <v>182.54</v>
       </c>
       <c r="F15" t="n">
-        <v>87.68000000000001</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="G15" t="n">
-        <v>88.09</v>
+        <v>82.08</v>
       </c>
       <c r="H15" t="n">
-        <v>85.41</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="I15" t="n">
-        <v>86.56</v>
+        <v>73.05</v>
       </c>
       <c r="J15" t="n">
-        <v>4.88</v>
+        <v>5.86</v>
       </c>
       <c r="K15" t="n">
-        <v>5.35</v>
+        <v>6.85</v>
       </c>
       <c r="L15" t="n">
-        <v>4.82</v>
+        <v>5.79</v>
       </c>
       <c r="M15" t="n">
-        <v>4.91</v>
+        <v>6.84</v>
       </c>
       <c r="N15" t="n">
-        <v>36.73</v>
+        <v>39.42</v>
       </c>
       <c r="O15" t="n">
-        <v>37.69</v>
+        <v>43.35</v>
       </c>
       <c r="P15" t="n">
-        <v>36.55</v>
+        <v>39.18</v>
       </c>
       <c r="Q15" t="n">
-        <v>37.19</v>
+        <v>43.19</v>
       </c>
       <c r="R15" t="n">
-        <v>5.3394</v>
+        <v>-30.5139</v>
       </c>
       <c r="S15" t="n">
-        <v>25.0513</v>
+        <v>-31.4584</v>
       </c>
       <c r="T15" t="n">
-        <v>28.6999</v>
+        <v>-18.6324</v>
       </c>
       <c r="U15" t="n">
-        <v>-0.7567</v>
+        <v>-14.2807</v>
       </c>
       <c r="V15" t="n">
-        <v>2.3652</v>
+        <v>-16.2463</v>
       </c>
       <c r="W15" t="n">
-        <v>5.9875</v>
+        <v>-13.6116</v>
       </c>
       <c r="X15" t="n">
-        <v>-5.029</v>
+        <v>31.5385</v>
       </c>
       <c r="Y15" t="n">
-        <v>-22.4329</v>
+        <v>32.3017</v>
       </c>
       <c r="Z15" t="n">
-        <v>-24.8086</v>
+        <v>8.056900000000001</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.7586000000000001</v>
+        <v>14.3803</v>
       </c>
       <c r="AB15" t="n">
-        <v>-2.3372</v>
+        <v>17.0144</v>
       </c>
       <c r="AC15" t="n">
-        <v>-5.7049</v>
+        <v>13.4191</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>242.04</v>
+        <v>210.62</v>
       </c>
       <c r="C16" t="n">
-        <v>274.5</v>
+        <v>222.19</v>
       </c>
       <c r="D16" t="n">
-        <v>228.55</v>
+        <v>201.69</v>
       </c>
       <c r="E16" t="n">
-        <v>262.7</v>
+        <v>211.44</v>
       </c>
       <c r="F16" t="n">
-        <v>83.47</v>
+        <v>76.86</v>
       </c>
       <c r="G16" t="n">
-        <v>86.25</v>
+        <v>78.47</v>
       </c>
       <c r="H16" t="n">
-        <v>82.48</v>
+        <v>75.38</v>
       </c>
       <c r="I16" t="n">
-        <v>85.22</v>
+        <v>76.27</v>
       </c>
       <c r="J16" t="n">
-        <v>5.57</v>
+        <v>5.71</v>
       </c>
       <c r="K16" t="n">
-        <v>5.81</v>
+        <v>6.05</v>
       </c>
       <c r="L16" t="n">
-        <v>5</v>
+        <v>5.27</v>
       </c>
       <c r="M16" t="n">
-        <v>5.2</v>
+        <v>5.69</v>
       </c>
       <c r="N16" t="n">
-        <v>38.53</v>
+        <v>40.92</v>
       </c>
       <c r="O16" t="n">
-        <v>38.96</v>
+        <v>41.78</v>
       </c>
       <c r="P16" t="n">
-        <v>37.33</v>
+        <v>39.96</v>
       </c>
       <c r="Q16" t="n">
-        <v>37.76</v>
+        <v>41.26</v>
       </c>
       <c r="R16" t="n">
-        <v>-6.3592</v>
+        <v>15.8321</v>
       </c>
       <c r="S16" t="n">
-        <v>15.7116</v>
+        <v>-24.6311</v>
       </c>
       <c r="T16" t="n">
-        <v>16.9479</v>
+        <v>-6.8669</v>
       </c>
       <c r="U16" t="n">
-        <v>-1.5481</v>
+        <v>4.4079</v>
       </c>
       <c r="V16" t="n">
-        <v>-0.953</v>
+        <v>-11.8877</v>
       </c>
       <c r="W16" t="n">
-        <v>1.8403</v>
+        <v>-11.3552</v>
       </c>
       <c r="X16" t="n">
-        <v>5.9063</v>
+        <v>-16.8129</v>
       </c>
       <c r="Y16" t="n">
-        <v>-16.9329</v>
+        <v>15.8859</v>
       </c>
       <c r="Z16" t="n">
-        <v>-17.5911</v>
+        <v>-9.105399999999999</v>
       </c>
       <c r="AA16" t="n">
-        <v>1.5327</v>
+        <v>-4.4686</v>
       </c>
       <c r="AB16" t="n">
-        <v>0.9086</v>
+        <v>10.9438</v>
       </c>
       <c r="AC16" t="n">
-        <v>-1.8456</v>
+        <v>10.2619</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>230.85</v>
+        <v>227.06</v>
       </c>
       <c r="C17" t="n">
-        <v>233.69</v>
+        <v>231.02</v>
       </c>
       <c r="D17" t="n">
-        <v>181.81</v>
+        <v>157.56</v>
       </c>
       <c r="E17" t="n">
-        <v>182.54</v>
+        <v>201.68</v>
       </c>
       <c r="F17" t="n">
-        <v>81.56999999999999</v>
+        <v>78.48</v>
       </c>
       <c r="G17" t="n">
-        <v>82.08</v>
+        <v>79.34</v>
       </c>
       <c r="H17" t="n">
-        <v>72.68000000000001</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="I17" t="n">
-        <v>73.05</v>
+        <v>73.72</v>
       </c>
       <c r="J17" t="n">
-        <v>5.86</v>
+        <v>5.25</v>
       </c>
       <c r="K17" t="n">
-        <v>6.85</v>
+        <v>7.11</v>
       </c>
       <c r="L17" t="n">
-        <v>5.79</v>
+        <v>5.14</v>
       </c>
       <c r="M17" t="n">
-        <v>6.84</v>
+        <v>5.93</v>
       </c>
       <c r="N17" t="n">
-        <v>39.42</v>
+        <v>40.06</v>
       </c>
       <c r="O17" t="n">
-        <v>43.35</v>
+        <v>46.38</v>
       </c>
       <c r="P17" t="n">
-        <v>39.18</v>
+        <v>39.59</v>
       </c>
       <c r="Q17" t="n">
-        <v>43.19</v>
+        <v>42.67</v>
       </c>
       <c r="R17" t="n">
-        <v>-30.5139</v>
+        <v>-4.616</v>
       </c>
       <c r="S17" t="n">
-        <v>-31.4584</v>
+        <v>-23.228</v>
       </c>
       <c r="T17" t="n">
-        <v>-18.6324</v>
+        <v>-24.2716</v>
       </c>
       <c r="U17" t="n">
-        <v>-14.2807</v>
+        <v>-3.3434</v>
       </c>
       <c r="V17" t="n">
-        <v>-16.2463</v>
+        <v>-13.4945</v>
       </c>
       <c r="W17" t="n">
-        <v>-13.6116</v>
+        <v>-15.4781</v>
       </c>
       <c r="X17" t="n">
-        <v>31.5385</v>
+        <v>4.2179</v>
       </c>
       <c r="Y17" t="n">
-        <v>32.3017</v>
+        <v>14.0385</v>
       </c>
       <c r="Z17" t="n">
-        <v>8.056900000000001</v>
+        <v>14.7002</v>
       </c>
       <c r="AA17" t="n">
-        <v>14.3803</v>
+        <v>3.4174</v>
       </c>
       <c r="AB17" t="n">
-        <v>17.0144</v>
+        <v>13.0032</v>
       </c>
       <c r="AC17" t="n">
-        <v>13.4191</v>
+        <v>15.6055</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>210.62</v>
+        <v>191.54</v>
       </c>
       <c r="C18" t="n">
-        <v>222.19</v>
+        <v>212.99</v>
       </c>
       <c r="D18" t="n">
-        <v>201.69</v>
+        <v>177.3</v>
       </c>
       <c r="E18" t="n">
-        <v>211.44</v>
+        <v>180.65</v>
       </c>
       <c r="F18" t="n">
-        <v>76.86</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>78.47</v>
+        <v>74.7</v>
       </c>
       <c r="H18" t="n">
-        <v>75.38</v>
+        <v>69</v>
       </c>
       <c r="I18" t="n">
-        <v>76.27</v>
+        <v>69.27</v>
       </c>
       <c r="J18" t="n">
-        <v>5.71</v>
+        <v>6.24</v>
       </c>
       <c r="K18" t="n">
-        <v>6.05</v>
+        <v>6.65</v>
       </c>
       <c r="L18" t="n">
-        <v>5.27</v>
+        <v>5.6</v>
       </c>
       <c r="M18" t="n">
-        <v>5.69</v>
+        <v>6.57</v>
       </c>
       <c r="N18" t="n">
-        <v>40.92</v>
+        <v>43.81</v>
       </c>
       <c r="O18" t="n">
-        <v>41.78</v>
+        <v>45.39</v>
       </c>
       <c r="P18" t="n">
-        <v>39.96</v>
+        <v>42.07</v>
       </c>
       <c r="Q18" t="n">
-        <v>41.26</v>
+        <v>45.25</v>
       </c>
       <c r="R18" t="n">
-        <v>15.8321</v>
+        <v>-10.4274</v>
       </c>
       <c r="S18" t="n">
-        <v>-24.6311</v>
+        <v>-1.0354</v>
       </c>
       <c r="T18" t="n">
-        <v>-6.8669</v>
+        <v>-35.6063</v>
       </c>
       <c r="U18" t="n">
-        <v>4.4079</v>
+        <v>-6.0364</v>
       </c>
       <c r="V18" t="n">
-        <v>-11.8877</v>
+        <v>-5.1745</v>
       </c>
       <c r="W18" t="n">
-        <v>-11.3552</v>
+        <v>-19.9746</v>
       </c>
       <c r="X18" t="n">
-        <v>-16.8129</v>
+        <v>10.7926</v>
       </c>
       <c r="Y18" t="n">
-        <v>15.8859</v>
+        <v>-3.9474</v>
       </c>
       <c r="Z18" t="n">
-        <v>-9.105399999999999</v>
+        <v>33.8086</v>
       </c>
       <c r="AA18" t="n">
-        <v>-4.4686</v>
+        <v>6.0464</v>
       </c>
       <c r="AB18" t="n">
-        <v>10.9438</v>
+        <v>4.7696</v>
       </c>
       <c r="AC18" t="n">
-        <v>10.2619</v>
+        <v>21.6725</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>227.06</v>
+        <v>192.3</v>
       </c>
       <c r="C19" t="n">
-        <v>231.02</v>
+        <v>225.63</v>
       </c>
       <c r="D19" t="n">
-        <v>157.56</v>
+        <v>192.3</v>
       </c>
       <c r="E19" t="n">
-        <v>201.68</v>
+        <v>223.99</v>
       </c>
       <c r="F19" t="n">
-        <v>78.48</v>
+        <v>70.89</v>
       </c>
       <c r="G19" t="n">
-        <v>79.34</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>66.79000000000001</v>
+        <v>69.59</v>
       </c>
       <c r="I19" t="n">
-        <v>73.72</v>
+        <v>76.01000000000001</v>
       </c>
       <c r="J19" t="n">
-        <v>5.25</v>
+        <v>6.1</v>
       </c>
       <c r="K19" t="n">
-        <v>7.11</v>
+        <v>6.1</v>
       </c>
       <c r="L19" t="n">
-        <v>5.14</v>
+        <v>4.9</v>
       </c>
       <c r="M19" t="n">
-        <v>5.93</v>
+        <v>4.97</v>
       </c>
       <c r="N19" t="n">
-        <v>40.06</v>
+        <v>44.18</v>
       </c>
       <c r="O19" t="n">
-        <v>46.38</v>
+        <v>45.01</v>
       </c>
       <c r="P19" t="n">
-        <v>39.59</v>
+        <v>40.44</v>
       </c>
       <c r="Q19" t="n">
-        <v>42.67</v>
+        <v>40.83</v>
       </c>
       <c r="R19" t="n">
-        <v>-4.616</v>
+        <v>23.9911</v>
       </c>
       <c r="S19" t="n">
-        <v>-23.228</v>
+        <v>5.9355</v>
       </c>
       <c r="T19" t="n">
-        <v>-24.2716</v>
+        <v>-14.7354</v>
       </c>
       <c r="U19" t="n">
-        <v>-3.3434</v>
+        <v>9.73</v>
       </c>
       <c r="V19" t="n">
-        <v>-13.4945</v>
+        <v>-0.3409</v>
       </c>
       <c r="W19" t="n">
-        <v>-15.4781</v>
+        <v>-10.8073</v>
       </c>
       <c r="X19" t="n">
-        <v>4.2179</v>
+        <v>-24.3531</v>
       </c>
       <c r="Y19" t="n">
-        <v>14.0385</v>
+        <v>-12.6538</v>
       </c>
       <c r="Z19" t="n">
-        <v>14.7002</v>
+        <v>-4.4231</v>
       </c>
       <c r="AA19" t="n">
-        <v>3.4174</v>
+        <v>-9.768000000000001</v>
       </c>
       <c r="AB19" t="n">
-        <v>13.0032</v>
+        <v>-1.0422</v>
       </c>
       <c r="AC19" t="n">
-        <v>15.6055</v>
+        <v>8.1303</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>191.54</v>
+        <v>222.22</v>
       </c>
       <c r="C20" t="n">
-        <v>212.99</v>
+        <v>242.4</v>
       </c>
       <c r="D20" t="n">
-        <v>177.3</v>
+        <v>214.74</v>
       </c>
       <c r="E20" t="n">
-        <v>180.65</v>
+        <v>234.68</v>
       </c>
       <c r="F20" t="n">
-        <v>71.68000000000001</v>
+        <v>76.34</v>
       </c>
       <c r="G20" t="n">
-        <v>74.7</v>
+        <v>78.36</v>
       </c>
       <c r="H20" t="n">
-        <v>69</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>69.27</v>
+        <v>77.52</v>
       </c>
       <c r="J20" t="n">
-        <v>6.24</v>
+        <v>5.01</v>
       </c>
       <c r="K20" t="n">
-        <v>6.65</v>
+        <v>5.15</v>
       </c>
       <c r="L20" t="n">
-        <v>5.6</v>
+        <v>4.54</v>
       </c>
       <c r="M20" t="n">
-        <v>6.57</v>
+        <v>4.72</v>
       </c>
       <c r="N20" t="n">
-        <v>43.81</v>
+        <v>40.65</v>
       </c>
       <c r="O20" t="n">
-        <v>45.39</v>
+        <v>41.75</v>
       </c>
       <c r="P20" t="n">
-        <v>42.07</v>
+        <v>39.57</v>
       </c>
       <c r="Q20" t="n">
-        <v>45.25</v>
+        <v>40.04</v>
       </c>
       <c r="R20" t="n">
-        <v>-10.4274</v>
+        <v>4.7725</v>
       </c>
       <c r="S20" t="n">
-        <v>-1.0354</v>
+        <v>16.3626</v>
       </c>
       <c r="T20" t="n">
-        <v>-35.6063</v>
+        <v>28.5636</v>
       </c>
       <c r="U20" t="n">
-        <v>-6.0364</v>
+        <v>1.9866</v>
       </c>
       <c r="V20" t="n">
-        <v>-5.1745</v>
+        <v>5.1546</v>
       </c>
       <c r="W20" t="n">
-        <v>-19.9746</v>
+        <v>6.1191</v>
       </c>
       <c r="X20" t="n">
-        <v>10.7926</v>
+        <v>-5.0302</v>
       </c>
       <c r="Y20" t="n">
-        <v>-3.9474</v>
+        <v>-20.4047</v>
       </c>
       <c r="Z20" t="n">
-        <v>33.8086</v>
+        <v>-30.9942</v>
       </c>
       <c r="AA20" t="n">
-        <v>6.0464</v>
+        <v>-1.9349</v>
       </c>
       <c r="AB20" t="n">
-        <v>4.7696</v>
+        <v>-6.1636</v>
       </c>
       <c r="AC20" t="n">
-        <v>21.6725</v>
+        <v>-7.2934</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>192.3</v>
+        <v>265.99</v>
       </c>
       <c r="C21" t="n">
-        <v>225.63</v>
+        <v>274.88</v>
       </c>
       <c r="D21" t="n">
-        <v>192.3</v>
+        <v>261.6019</v>
       </c>
       <c r="E21" t="n">
-        <v>223.99</v>
+        <v>272.5</v>
       </c>
       <c r="F21" t="n">
-        <v>70.89</v>
+        <v>82.88</v>
       </c>
       <c r="G21" t="n">
-        <v>76.59999999999999</v>
+        <v>85.03</v>
       </c>
       <c r="H21" t="n">
-        <v>69.59</v>
+        <v>82.64</v>
       </c>
       <c r="I21" t="n">
-        <v>76.01000000000001</v>
+        <v>84.59</v>
       </c>
       <c r="J21" t="n">
-        <v>6.1</v>
+        <v>4.07</v>
       </c>
       <c r="K21" t="n">
-        <v>6.1</v>
+        <v>4.17</v>
       </c>
       <c r="L21" t="n">
-        <v>4.9</v>
+        <v>3.91</v>
       </c>
       <c r="M21" t="n">
-        <v>4.97</v>
+        <v>3.95</v>
       </c>
       <c r="N21" t="n">
-        <v>44.18</v>
+        <v>37.25</v>
       </c>
       <c r="O21" t="n">
-        <v>45.01</v>
+        <v>37.36</v>
       </c>
       <c r="P21" t="n">
-        <v>40.44</v>
+        <v>36.15</v>
       </c>
       <c r="Q21" t="n">
-        <v>40.83</v>
+        <v>36.31</v>
       </c>
       <c r="R21" t="n">
-        <v>23.9911</v>
+        <v>16.1156</v>
       </c>
       <c r="S21" t="n">
-        <v>5.9355</v>
+        <v>50.8442</v>
       </c>
       <c r="T21" t="n">
-        <v>-14.7354</v>
+        <v>28.8782</v>
       </c>
       <c r="U21" t="n">
-        <v>9.73</v>
+        <v>9.120200000000001</v>
       </c>
       <c r="V21" t="n">
-        <v>-0.3409</v>
+        <v>22.1164</v>
       </c>
       <c r="W21" t="n">
-        <v>-10.8073</v>
+        <v>10.9086</v>
       </c>
       <c r="X21" t="n">
-        <v>-24.3531</v>
+        <v>-16.3136</v>
       </c>
       <c r="Y21" t="n">
-        <v>-12.6538</v>
+        <v>-39.8782</v>
       </c>
       <c r="Z21" t="n">
-        <v>-4.4231</v>
+        <v>-30.58</v>
       </c>
       <c r="AA21" t="n">
-        <v>-9.768000000000001</v>
+        <v>-9.3157</v>
       </c>
       <c r="AB21" t="n">
-        <v>-1.0422</v>
+        <v>-19.7569</v>
       </c>
       <c r="AC21" t="n">
-        <v>8.1303</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>222.22</v>
-      </c>
-      <c r="C22" t="n">
-        <v>242.4</v>
-      </c>
-      <c r="D22" t="n">
-        <v>214.7406</v>
-      </c>
-      <c r="E22" t="n">
-        <v>234.68</v>
-      </c>
-      <c r="F22" t="n">
-        <v>76.34</v>
-      </c>
-      <c r="G22" t="n">
-        <v>78.36</v>
-      </c>
-      <c r="H22" t="n">
-        <v>74.29000000000001</v>
-      </c>
-      <c r="I22" t="n">
-        <v>77.52</v>
-      </c>
-      <c r="J22" t="n">
-        <v>5.01</v>
-      </c>
-      <c r="K22" t="n">
-        <v>5.15</v>
-      </c>
-      <c r="L22" t="n">
-        <v>4.54</v>
-      </c>
-      <c r="M22" t="n">
-        <v>4.72</v>
-      </c>
-      <c r="N22" t="n">
-        <v>40.665</v>
-      </c>
-      <c r="O22" t="n">
-        <v>41.7498</v>
-      </c>
-      <c r="P22" t="n">
-        <v>39.57</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>40.04</v>
-      </c>
-      <c r="R22" t="n">
-        <v>4.7725</v>
-      </c>
-      <c r="S22" t="n">
-        <v>16.3626</v>
-      </c>
-      <c r="T22" t="n">
-        <v>28.5636</v>
-      </c>
-      <c r="U22" t="n">
-        <v>1.9866</v>
-      </c>
-      <c r="V22" t="n">
-        <v>5.1546</v>
-      </c>
-      <c r="W22" t="n">
-        <v>6.1191</v>
-      </c>
-      <c r="X22" t="n">
-        <v>-5.0302</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>-20.4047</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>-30.9942</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>-1.9349</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>-6.1636</v>
-      </c>
-      <c r="AC22" t="n">
-        <v>-7.2934</v>
+        <v>-11.9971</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-16 23:24
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC21"/>
+  <dimension ref="A1:AC22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2199,7 +2199,7 @@
         <v>274.88</v>
       </c>
       <c r="D21" t="n">
-        <v>261.6019</v>
+        <v>261.6</v>
       </c>
       <c r="E21" t="n">
         <v>272.5</v>
@@ -2275,6 +2275,97 @@
       </c>
       <c r="AC21" t="n">
         <v>-11.9971</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>267.13</v>
+      </c>
+      <c r="C22" t="n">
+        <v>274.9297</v>
+      </c>
+      <c r="D22" t="n">
+        <v>226.005</v>
+      </c>
+      <c r="E22" t="n">
+        <v>226.19</v>
+      </c>
+      <c r="F22" t="n">
+        <v>84.19</v>
+      </c>
+      <c r="G22" t="n">
+        <v>84.83</v>
+      </c>
+      <c r="H22" t="n">
+        <v>79.86</v>
+      </c>
+      <c r="I22" t="n">
+        <v>79.93000000000001</v>
+      </c>
+      <c r="J22" t="n">
+        <v>4.025</v>
+      </c>
+      <c r="K22" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="L22" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="M22" t="n">
+        <v>4.63</v>
+      </c>
+      <c r="N22" t="n">
+        <v>36.55</v>
+      </c>
+      <c r="O22" t="n">
+        <v>38.39</v>
+      </c>
+      <c r="P22" t="n">
+        <v>36.26</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>38.35</v>
+      </c>
+      <c r="R22" t="n">
+        <v>-16.9945</v>
+      </c>
+      <c r="S22" t="n">
+        <v>0.9822</v>
+      </c>
+      <c r="T22" t="n">
+        <v>12.1529</v>
+      </c>
+      <c r="U22" t="n">
+        <v>-5.5089</v>
+      </c>
+      <c r="V22" t="n">
+        <v>5.1572</v>
+      </c>
+      <c r="W22" t="n">
+        <v>8.4238</v>
+      </c>
+      <c r="X22" t="n">
+        <v>17.2152</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>-6.841</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>-21.9224</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>5.6183</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>-6.074</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>-10.1242</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-17 23:24
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>172.95</v>
+        <v>141.24</v>
       </c>
       <c r="C2" t="n">
-        <v>174.61</v>
+        <v>160.6</v>
       </c>
       <c r="D2" t="n">
-        <v>142.69</v>
+        <v>135.02</v>
       </c>
       <c r="E2" t="n">
-        <v>151.75</v>
+        <v>151.89</v>
       </c>
       <c r="F2" t="n">
-        <v>76.13</v>
+        <v>72.41</v>
       </c>
       <c r="G2" t="n">
-        <v>76.27</v>
+        <v>74.5</v>
       </c>
       <c r="H2" t="n">
-        <v>72.09999999999999</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>74.31999999999999</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>8.77</v>
+        <v>10.64</v>
       </c>
       <c r="K2" t="n">
-        <v>10.47</v>
+        <v>11.07</v>
       </c>
       <c r="L2" t="n">
-        <v>8.68</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="M2" t="n">
-        <v>9.949999999999999</v>
+        <v>9.93</v>
       </c>
       <c r="N2" t="n">
-        <v>42.51</v>
+        <v>44.68</v>
       </c>
       <c r="O2" t="n">
-        <v>44.82</v>
+        <v>45.53</v>
       </c>
       <c r="P2" t="n">
-        <v>42.44</v>
+        <v>43.46</v>
       </c>
       <c r="Q2" t="n">
-        <v>43.54</v>
+        <v>44.37</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>141.24</v>
+        <v>161</v>
       </c>
       <c r="C3" t="n">
-        <v>160.6</v>
+        <v>173.7</v>
       </c>
       <c r="D3" t="n">
-        <v>135.02</v>
+        <v>161</v>
       </c>
       <c r="E3" t="n">
-        <v>151.89</v>
+        <v>173.2</v>
       </c>
       <c r="F3" t="n">
-        <v>72.41</v>
+        <v>74.09</v>
       </c>
       <c r="G3" t="n">
-        <v>74.5</v>
+        <v>76.53</v>
       </c>
       <c r="H3" t="n">
-        <v>70.95999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="I3" t="n">
-        <v>72.93000000000001</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>10.64</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>11.07</v>
+        <v>9.35</v>
       </c>
       <c r="L3" t="n">
-        <v>9.369999999999999</v>
+        <v>8.51</v>
       </c>
       <c r="M3" t="n">
-        <v>9.93</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N3" t="n">
-        <v>44.68</v>
+        <v>43.67</v>
       </c>
       <c r="O3" t="n">
-        <v>45.53</v>
+        <v>43.97</v>
       </c>
       <c r="P3" t="n">
-        <v>43.46</v>
+        <v>42.19</v>
       </c>
       <c r="Q3" t="n">
-        <v>44.37</v>
+        <v>42.19</v>
       </c>
       <c r="R3" t="n">
-        <v>0.09229999999999999</v>
+        <v>14.0299</v>
       </c>
       <c r="U3" t="n">
-        <v>-1.8703</v>
+        <v>4.9088</v>
       </c>
       <c r="X3" t="n">
-        <v>-0.201</v>
+        <v>-13.998</v>
       </c>
       <c r="AA3" t="n">
-        <v>1.9063</v>
+        <v>-4.9132</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>161</v>
+        <v>171.26</v>
       </c>
       <c r="C4" t="n">
-        <v>173.7</v>
+        <v>179.97</v>
       </c>
       <c r="D4" t="n">
-        <v>161</v>
+        <v>168.23</v>
       </c>
       <c r="E4" t="n">
-        <v>173.2</v>
+        <v>178.39</v>
       </c>
       <c r="F4" t="n">
-        <v>74.09</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>76.53</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>73.62</v>
+        <v>74.47</v>
       </c>
       <c r="I4" t="n">
-        <v>76.51000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J4" t="n">
-        <v>9.300000000000001</v>
+        <v>8.65</v>
       </c>
       <c r="K4" t="n">
-        <v>9.35</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L4" t="n">
-        <v>8.51</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>8.539999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N4" t="n">
-        <v>43.67</v>
+        <v>42.94</v>
       </c>
       <c r="O4" t="n">
-        <v>43.97</v>
+        <v>43.33</v>
       </c>
       <c r="P4" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="Q4" t="n">
-        <v>42.19</v>
+        <v>41.96</v>
       </c>
       <c r="R4" t="n">
-        <v>14.0299</v>
+        <v>2.9965</v>
       </c>
       <c r="U4" t="n">
-        <v>4.9088</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="X4" t="n">
-        <v>-13.998</v>
+        <v>-2.9274</v>
       </c>
       <c r="AA4" t="n">
-        <v>-4.9132</v>
+        <v>-0.5452</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>171.26</v>
+        <v>184.8</v>
       </c>
       <c r="C5" t="n">
-        <v>179.97</v>
+        <v>195.27</v>
       </c>
       <c r="D5" t="n">
-        <v>168.23</v>
+        <v>183.34</v>
       </c>
       <c r="E5" t="n">
-        <v>178.39</v>
+        <v>190.56</v>
       </c>
       <c r="F5" t="n">
-        <v>75.18000000000001</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>77.79000000000001</v>
+        <v>79.33</v>
       </c>
       <c r="H5" t="n">
-        <v>74.47</v>
+        <v>77.33</v>
       </c>
       <c r="I5" t="n">
-        <v>76.95</v>
+        <v>77.84</v>
       </c>
       <c r="J5" t="n">
-        <v>8.65</v>
+        <v>8</v>
       </c>
       <c r="K5" t="n">
-        <v>8.779999999999999</v>
+        <v>8.06</v>
       </c>
       <c r="L5" t="n">
-        <v>8.210000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="M5" t="n">
-        <v>8.289999999999999</v>
+        <v>7.73</v>
       </c>
       <c r="N5" t="n">
-        <v>42.94</v>
+        <v>41.4</v>
       </c>
       <c r="O5" t="n">
-        <v>43.33</v>
+        <v>41.78</v>
       </c>
       <c r="P5" t="n">
+        <v>40.68</v>
+      </c>
+      <c r="Q5" t="n">
         <v>41.5</v>
       </c>
-      <c r="Q5" t="n">
-        <v>41.96</v>
-      </c>
       <c r="R5" t="n">
-        <v>2.9965</v>
+        <v>6.8221</v>
       </c>
       <c r="S5" t="n">
-        <v>17.5552</v>
+        <v>25.4592</v>
       </c>
       <c r="U5" t="n">
-        <v>0.5750999999999999</v>
+        <v>1.1566</v>
       </c>
       <c r="V5" t="n">
-        <v>3.5388</v>
+        <v>6.7325</v>
       </c>
       <c r="X5" t="n">
-        <v>-2.9274</v>
+        <v>-6.7551</v>
       </c>
       <c r="Y5" t="n">
-        <v>-16.6834</v>
+        <v>-22.1551</v>
       </c>
       <c r="AA5" t="n">
-        <v>-0.5452</v>
+        <v>-1.0963</v>
       </c>
       <c r="AB5" t="n">
-        <v>-3.6288</v>
+        <v>-6.4683</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>184.8</v>
+        <v>211.38</v>
       </c>
       <c r="C6" t="n">
-        <v>195.27</v>
+        <v>228.5</v>
       </c>
       <c r="D6" t="n">
-        <v>183.34</v>
+        <v>209.89</v>
       </c>
       <c r="E6" t="n">
-        <v>190.56</v>
+        <v>225.79</v>
       </c>
       <c r="F6" t="n">
-        <v>78.04000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="G6" t="n">
-        <v>79.33</v>
+        <v>82.27</v>
       </c>
       <c r="H6" t="n">
-        <v>77.33</v>
+        <v>79.98</v>
       </c>
       <c r="I6" t="n">
-        <v>77.84</v>
+        <v>81.95</v>
       </c>
       <c r="J6" t="n">
-        <v>8</v>
+        <v>6.9</v>
       </c>
       <c r="K6" t="n">
-        <v>8.06</v>
+        <v>6.95</v>
       </c>
       <c r="L6" t="n">
-        <v>7.5</v>
+        <v>6.19</v>
       </c>
       <c r="M6" t="n">
-        <v>7.73</v>
+        <v>6.29</v>
       </c>
       <c r="N6" t="n">
-        <v>41.4</v>
+        <v>40.05</v>
       </c>
       <c r="O6" t="n">
-        <v>41.78</v>
+        <v>40.35</v>
       </c>
       <c r="P6" t="n">
-        <v>40.68</v>
+        <v>39.14</v>
       </c>
       <c r="Q6" t="n">
-        <v>41.5</v>
+        <v>39.28</v>
       </c>
       <c r="R6" t="n">
-        <v>6.8221</v>
+        <v>18.4876</v>
       </c>
       <c r="S6" t="n">
-        <v>25.4592</v>
+        <v>30.3637</v>
       </c>
       <c r="U6" t="n">
-        <v>1.1566</v>
+        <v>5.2801</v>
       </c>
       <c r="V6" t="n">
-        <v>6.7325</v>
+        <v>7.1102</v>
       </c>
       <c r="X6" t="n">
-        <v>-6.7551</v>
+        <v>-18.6287</v>
       </c>
       <c r="Y6" t="n">
-        <v>-22.1551</v>
+        <v>-26.3466</v>
       </c>
       <c r="AA6" t="n">
-        <v>-1.0963</v>
+        <v>-5.3494</v>
       </c>
       <c r="AB6" t="n">
-        <v>-6.4683</v>
+        <v>-6.8974</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>211.38</v>
+        <v>242.66</v>
       </c>
       <c r="C7" t="n">
-        <v>228.5</v>
+        <v>242.66</v>
       </c>
       <c r="D7" t="n">
-        <v>209.89</v>
+        <v>204</v>
       </c>
       <c r="E7" t="n">
-        <v>225.79</v>
+        <v>217.98</v>
       </c>
       <c r="F7" t="n">
-        <v>80.59</v>
+        <v>82.87</v>
       </c>
       <c r="G7" t="n">
-        <v>82.27</v>
+        <v>82.91</v>
       </c>
       <c r="H7" t="n">
-        <v>79.98</v>
+        <v>80.33</v>
       </c>
       <c r="I7" t="n">
-        <v>81.95</v>
+        <v>81.67</v>
       </c>
       <c r="J7" t="n">
-        <v>6.9</v>
+        <v>5.83</v>
       </c>
       <c r="K7" t="n">
-        <v>6.95</v>
+        <v>6.91</v>
       </c>
       <c r="L7" t="n">
-        <v>6.19</v>
+        <v>5.83</v>
       </c>
       <c r="M7" t="n">
-        <v>6.29</v>
+        <v>6.53</v>
       </c>
       <c r="N7" t="n">
-        <v>40.05</v>
+        <v>38.87</v>
       </c>
       <c r="O7" t="n">
-        <v>40.35</v>
+        <v>40.09</v>
       </c>
       <c r="P7" t="n">
-        <v>39.14</v>
+        <v>38.86</v>
       </c>
       <c r="Q7" t="n">
-        <v>39.28</v>
+        <v>39.44</v>
       </c>
       <c r="R7" t="n">
-        <v>18.4876</v>
+        <v>-3.459</v>
       </c>
       <c r="S7" t="n">
-        <v>30.3637</v>
+        <v>22.1929</v>
       </c>
       <c r="T7" t="n">
-        <v>48.7908</v>
+        <v>43.5118</v>
       </c>
       <c r="U7" t="n">
-        <v>5.2801</v>
+        <v>-0.3417</v>
       </c>
       <c r="V7" t="n">
-        <v>7.1102</v>
+        <v>6.1339</v>
       </c>
       <c r="W7" t="n">
-        <v>10.2664</v>
+        <v>11.9841</v>
       </c>
       <c r="X7" t="n">
-        <v>-18.6287</v>
+        <v>3.8156</v>
       </c>
       <c r="Y7" t="n">
-        <v>-26.3466</v>
+        <v>-21.2304</v>
       </c>
       <c r="Z7" t="n">
-        <v>-36.7839</v>
+        <v>-34.2397</v>
       </c>
       <c r="AA7" t="n">
-        <v>-5.3494</v>
+        <v>0.4073</v>
       </c>
       <c r="AB7" t="n">
-        <v>-6.8974</v>
+        <v>-6.0057</v>
       </c>
       <c r="AC7" t="n">
-        <v>-9.7841</v>
+        <v>-11.1111</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>242.66</v>
+        <v>219</v>
       </c>
       <c r="C8" t="n">
-        <v>242.66</v>
+        <v>231.89</v>
       </c>
       <c r="D8" t="n">
-        <v>204</v>
+        <v>207.56</v>
       </c>
       <c r="E8" t="n">
-        <v>217.98</v>
+        <v>224.63</v>
       </c>
       <c r="F8" t="n">
-        <v>82.87</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>82.91</v>
+        <v>84.05</v>
       </c>
       <c r="H8" t="n">
-        <v>80.33</v>
+        <v>80.66</v>
       </c>
       <c r="I8" t="n">
-        <v>81.67</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>5.83</v>
+        <v>6.49</v>
       </c>
       <c r="K8" t="n">
-        <v>6.91</v>
+        <v>6.83</v>
       </c>
       <c r="L8" t="n">
-        <v>5.83</v>
+        <v>6.1</v>
       </c>
       <c r="M8" t="n">
-        <v>6.53</v>
+        <v>6.31</v>
       </c>
       <c r="N8" t="n">
-        <v>38.87</v>
+        <v>39.41</v>
       </c>
       <c r="O8" t="n">
-        <v>40.09</v>
+        <v>39.94</v>
       </c>
       <c r="P8" t="n">
-        <v>38.86</v>
+        <v>38.3</v>
       </c>
       <c r="Q8" t="n">
-        <v>39.44</v>
+        <v>38.47</v>
       </c>
       <c r="R8" t="n">
-        <v>-3.459</v>
+        <v>3.0507</v>
       </c>
       <c r="S8" t="n">
-        <v>22.1929</v>
+        <v>17.8789</v>
       </c>
       <c r="T8" t="n">
-        <v>43.5118</v>
+        <v>29.694</v>
       </c>
       <c r="U8" t="n">
-        <v>-0.3417</v>
+        <v>2.4611</v>
       </c>
       <c r="V8" t="n">
-        <v>6.1339</v>
+        <v>7.5026</v>
       </c>
       <c r="W8" t="n">
-        <v>11.9841</v>
+        <v>9.3713</v>
       </c>
       <c r="X8" t="n">
-        <v>3.8156</v>
+        <v>-3.3691</v>
       </c>
       <c r="Y8" t="n">
-        <v>-21.2304</v>
+        <v>-18.37</v>
       </c>
       <c r="Z8" t="n">
-        <v>-34.2397</v>
+        <v>-26.1124</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.4073</v>
+        <v>-2.4594</v>
       </c>
       <c r="AB8" t="n">
-        <v>-6.0057</v>
+        <v>-7.3012</v>
       </c>
       <c r="AC8" t="n">
-        <v>-11.1111</v>
+        <v>-8.817299999999999</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>219</v>
+        <v>231.82</v>
       </c>
       <c r="C9" t="n">
-        <v>231.89</v>
+        <v>239.07</v>
       </c>
       <c r="D9" t="n">
-        <v>207.56</v>
+        <v>218.56</v>
       </c>
       <c r="E9" t="n">
-        <v>224.63</v>
+        <v>224.34</v>
       </c>
       <c r="F9" t="n">
-        <v>81.73999999999999</v>
+        <v>84.41</v>
       </c>
       <c r="G9" t="n">
-        <v>84.05</v>
+        <v>85.7</v>
       </c>
       <c r="H9" t="n">
-        <v>80.66</v>
+        <v>83.53</v>
       </c>
       <c r="I9" t="n">
-        <v>83.68000000000001</v>
+        <v>84.56</v>
       </c>
       <c r="J9" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="K9" t="n">
         <v>6.49</v>
       </c>
-      <c r="K9" t="n">
-        <v>6.83</v>
-      </c>
       <c r="L9" t="n">
-        <v>6.1</v>
+        <v>5.91</v>
       </c>
       <c r="M9" t="n">
-        <v>6.31</v>
+        <v>6.33</v>
       </c>
       <c r="N9" t="n">
-        <v>39.41</v>
+        <v>38.15</v>
       </c>
       <c r="O9" t="n">
-        <v>39.94</v>
+        <v>38.56</v>
       </c>
       <c r="P9" t="n">
-        <v>38.3</v>
+        <v>37.56</v>
       </c>
       <c r="Q9" t="n">
-        <v>38.47</v>
+        <v>38.08</v>
       </c>
       <c r="R9" t="n">
-        <v>3.0507</v>
+        <v>-0.1291</v>
       </c>
       <c r="S9" t="n">
-        <v>17.8789</v>
+        <v>-0.6422</v>
       </c>
       <c r="T9" t="n">
-        <v>29.694</v>
+        <v>25.7582</v>
       </c>
       <c r="U9" t="n">
-        <v>2.4611</v>
+        <v>1.0516</v>
       </c>
       <c r="V9" t="n">
-        <v>7.5026</v>
+        <v>3.1849</v>
       </c>
       <c r="W9" t="n">
-        <v>9.3713</v>
+        <v>9.8895</v>
       </c>
       <c r="X9" t="n">
-        <v>-3.3691</v>
+        <v>0.317</v>
       </c>
       <c r="Y9" t="n">
-        <v>-18.37</v>
+        <v>0.6359</v>
       </c>
       <c r="Z9" t="n">
-        <v>-26.1124</v>
+        <v>-23.6429</v>
       </c>
       <c r="AA9" t="n">
-        <v>-2.4594</v>
+        <v>-1.0138</v>
       </c>
       <c r="AB9" t="n">
-        <v>-7.3012</v>
+        <v>-3.055</v>
       </c>
       <c r="AC9" t="n">
-        <v>-8.817299999999999</v>
+        <v>-9.2469</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>231.82</v>
+        <v>217.27</v>
       </c>
       <c r="C10" t="n">
-        <v>239.07</v>
+        <v>234.06</v>
       </c>
       <c r="D10" t="n">
-        <v>218.56</v>
+        <v>210.14</v>
       </c>
       <c r="E10" t="n">
-        <v>224.34</v>
+        <v>227.03</v>
       </c>
       <c r="F10" t="n">
-        <v>84.41</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>85.7</v>
+        <v>87.06</v>
       </c>
       <c r="H10" t="n">
-        <v>83.53</v>
+        <v>83.75</v>
       </c>
       <c r="I10" t="n">
-        <v>84.56</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>6.11</v>
+        <v>6.55</v>
       </c>
       <c r="K10" t="n">
-        <v>6.49</v>
+        <v>6.74</v>
       </c>
       <c r="L10" t="n">
-        <v>5.91</v>
+        <v>6.05</v>
       </c>
       <c r="M10" t="n">
-        <v>6.33</v>
+        <v>6.26</v>
       </c>
       <c r="N10" t="n">
-        <v>38.15</v>
+        <v>38.27</v>
       </c>
       <c r="O10" t="n">
-        <v>38.56</v>
+        <v>38.46</v>
       </c>
       <c r="P10" t="n">
-        <v>37.56</v>
+        <v>36.96</v>
       </c>
       <c r="Q10" t="n">
-        <v>38.08</v>
+        <v>37.42</v>
       </c>
       <c r="R10" t="n">
-        <v>-0.1291</v>
+        <v>1.1991</v>
       </c>
       <c r="S10" t="n">
-        <v>-0.6422</v>
+        <v>4.1518</v>
       </c>
       <c r="T10" t="n">
-        <v>25.7582</v>
+        <v>19.1383</v>
       </c>
       <c r="U10" t="n">
-        <v>1.0516</v>
+        <v>1.7502</v>
       </c>
       <c r="V10" t="n">
-        <v>3.1849</v>
+        <v>5.3508</v>
       </c>
       <c r="W10" t="n">
-        <v>9.8895</v>
+        <v>10.5344</v>
       </c>
       <c r="X10" t="n">
-        <v>0.317</v>
+        <v>-1.1058</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.6359</v>
+        <v>-4.1348</v>
       </c>
       <c r="Z10" t="n">
-        <v>-23.6429</v>
+        <v>-19.0168</v>
       </c>
       <c r="AA10" t="n">
-        <v>-1.0138</v>
+        <v>-1.7332</v>
       </c>
       <c r="AB10" t="n">
-        <v>-3.055</v>
+        <v>-5.1217</v>
       </c>
       <c r="AC10" t="n">
-        <v>-9.2469</v>
+        <v>-9.831300000000001</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>217.27</v>
+        <v>243.18</v>
       </c>
       <c r="C11" t="n">
-        <v>234.06</v>
+        <v>267.08</v>
       </c>
       <c r="D11" t="n">
-        <v>210.14</v>
+        <v>238.82</v>
       </c>
       <c r="E11" t="n">
-        <v>227.03</v>
+        <v>266.32</v>
       </c>
       <c r="F11" t="n">
-        <v>84.15000000000001</v>
+        <v>85.94</v>
       </c>
       <c r="G11" t="n">
-        <v>87.06</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="H11" t="n">
-        <v>83.75</v>
+        <v>84.83</v>
       </c>
       <c r="I11" t="n">
-        <v>86.04000000000001</v>
+        <v>87.22</v>
       </c>
       <c r="J11" t="n">
-        <v>6.55</v>
+        <v>5.8</v>
       </c>
       <c r="K11" t="n">
-        <v>6.74</v>
+        <v>5.93</v>
       </c>
       <c r="L11" t="n">
-        <v>6.05</v>
+        <v>5.15</v>
       </c>
       <c r="M11" t="n">
-        <v>6.26</v>
+        <v>5.17</v>
       </c>
       <c r="N11" t="n">
-        <v>38.27</v>
+        <v>37.47</v>
       </c>
       <c r="O11" t="n">
-        <v>38.46</v>
+        <v>37.95</v>
       </c>
       <c r="P11" t="n">
-        <v>36.96</v>
+        <v>36.86</v>
       </c>
       <c r="Q11" t="n">
-        <v>37.42</v>
+        <v>36.91</v>
       </c>
       <c r="R11" t="n">
-        <v>1.1991</v>
+        <v>17.3061</v>
       </c>
       <c r="S11" t="n">
-        <v>4.1518</v>
+        <v>18.5594</v>
       </c>
       <c r="T11" t="n">
-        <v>19.1383</v>
+        <v>17.9503</v>
       </c>
       <c r="U11" t="n">
-        <v>1.7502</v>
+        <v>1.3715</v>
       </c>
       <c r="V11" t="n">
-        <v>5.3508</v>
+        <v>4.2304</v>
       </c>
       <c r="W11" t="n">
-        <v>10.5344</v>
+        <v>6.4308</v>
       </c>
       <c r="X11" t="n">
-        <v>-1.1058</v>
+        <v>-17.4121</v>
       </c>
       <c r="Y11" t="n">
-        <v>-4.1348</v>
+        <v>-18.0666</v>
       </c>
       <c r="Z11" t="n">
-        <v>-19.0168</v>
+        <v>-17.806</v>
       </c>
       <c r="AA11" t="n">
-        <v>-1.7332</v>
+        <v>-1.3629</v>
       </c>
       <c r="AB11" t="n">
-        <v>-5.1217</v>
+        <v>-4.0551</v>
       </c>
       <c r="AC11" t="n">
-        <v>-9.831300000000001</v>
+        <v>-6.0336</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>243.18</v>
+        <v>281.47</v>
       </c>
       <c r="C12" t="n">
-        <v>267.08</v>
+        <v>284.58</v>
       </c>
       <c r="D12" t="n">
-        <v>238.82</v>
+        <v>257.26</v>
       </c>
       <c r="E12" t="n">
-        <v>266.32</v>
+        <v>280.54</v>
       </c>
       <c r="F12" t="n">
-        <v>85.94</v>
+        <v>87.68000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>87.31999999999999</v>
+        <v>88.09</v>
       </c>
       <c r="H12" t="n">
-        <v>84.83</v>
+        <v>85.41</v>
       </c>
       <c r="I12" t="n">
-        <v>87.22</v>
+        <v>86.56</v>
       </c>
       <c r="J12" t="n">
-        <v>5.8</v>
+        <v>4.88</v>
       </c>
       <c r="K12" t="n">
-        <v>5.93</v>
+        <v>5.35</v>
       </c>
       <c r="L12" t="n">
-        <v>5.15</v>
+        <v>4.82</v>
       </c>
       <c r="M12" t="n">
-        <v>5.17</v>
+        <v>4.91</v>
       </c>
       <c r="N12" t="n">
-        <v>37.47</v>
+        <v>36.73</v>
       </c>
       <c r="O12" t="n">
-        <v>37.95</v>
+        <v>37.69</v>
       </c>
       <c r="P12" t="n">
-        <v>36.86</v>
+        <v>36.55</v>
       </c>
       <c r="Q12" t="n">
-        <v>36.91</v>
+        <v>37.19</v>
       </c>
       <c r="R12" t="n">
-        <v>17.3061</v>
+        <v>5.3394</v>
       </c>
       <c r="S12" t="n">
-        <v>18.5594</v>
+        <v>25.0513</v>
       </c>
       <c r="T12" t="n">
-        <v>17.9503</v>
+        <v>28.6999</v>
       </c>
       <c r="U12" t="n">
-        <v>1.3715</v>
+        <v>-0.7567</v>
       </c>
       <c r="V12" t="n">
-        <v>4.2304</v>
+        <v>2.3652</v>
       </c>
       <c r="W12" t="n">
-        <v>6.4308</v>
+        <v>5.9875</v>
       </c>
       <c r="X12" t="n">
-        <v>-17.4121</v>
+        <v>-5.029</v>
       </c>
       <c r="Y12" t="n">
-        <v>-18.0666</v>
+        <v>-22.4329</v>
       </c>
       <c r="Z12" t="n">
-        <v>-17.806</v>
+        <v>-24.8086</v>
       </c>
       <c r="AA12" t="n">
-        <v>-1.3629</v>
+        <v>0.7586000000000001</v>
       </c>
       <c r="AB12" t="n">
-        <v>-4.0551</v>
+        <v>-2.3372</v>
       </c>
       <c r="AC12" t="n">
-        <v>-6.0336</v>
+        <v>-5.7049</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>281.47</v>
+        <v>242.04</v>
       </c>
       <c r="C13" t="n">
-        <v>284.58</v>
+        <v>274.5</v>
       </c>
       <c r="D13" t="n">
-        <v>257.26</v>
+        <v>228.55</v>
       </c>
       <c r="E13" t="n">
-        <v>280.54</v>
+        <v>262.7</v>
       </c>
       <c r="F13" t="n">
-        <v>87.68000000000001</v>
+        <v>83.47</v>
       </c>
       <c r="G13" t="n">
-        <v>88.09</v>
+        <v>86.25</v>
       </c>
       <c r="H13" t="n">
-        <v>85.41</v>
+        <v>82.48</v>
       </c>
       <c r="I13" t="n">
-        <v>86.56</v>
+        <v>85.22</v>
       </c>
       <c r="J13" t="n">
-        <v>4.88</v>
+        <v>5.57</v>
       </c>
       <c r="K13" t="n">
-        <v>5.35</v>
+        <v>5.81</v>
       </c>
       <c r="L13" t="n">
-        <v>4.82</v>
+        <v>5</v>
       </c>
       <c r="M13" t="n">
-        <v>4.91</v>
+        <v>5.2</v>
       </c>
       <c r="N13" t="n">
-        <v>36.73</v>
+        <v>38.53</v>
       </c>
       <c r="O13" t="n">
-        <v>37.69</v>
+        <v>38.96</v>
       </c>
       <c r="P13" t="n">
-        <v>36.55</v>
+        <v>37.33</v>
       </c>
       <c r="Q13" t="n">
-        <v>37.19</v>
+        <v>37.76</v>
       </c>
       <c r="R13" t="n">
-        <v>5.3394</v>
+        <v>-6.3592</v>
       </c>
       <c r="S13" t="n">
-        <v>25.0513</v>
+        <v>15.7116</v>
       </c>
       <c r="T13" t="n">
-        <v>28.6999</v>
+        <v>16.9479</v>
       </c>
       <c r="U13" t="n">
-        <v>-0.7567</v>
+        <v>-1.5481</v>
       </c>
       <c r="V13" t="n">
-        <v>2.3652</v>
+        <v>-0.953</v>
       </c>
       <c r="W13" t="n">
-        <v>5.9875</v>
+        <v>1.8403</v>
       </c>
       <c r="X13" t="n">
-        <v>-5.029</v>
+        <v>5.9063</v>
       </c>
       <c r="Y13" t="n">
-        <v>-22.4329</v>
+        <v>-16.9329</v>
       </c>
       <c r="Z13" t="n">
-        <v>-24.8086</v>
+        <v>-17.5911</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.7586000000000001</v>
+        <v>1.5327</v>
       </c>
       <c r="AB13" t="n">
-        <v>-2.3372</v>
+        <v>0.9086</v>
       </c>
       <c r="AC13" t="n">
-        <v>-5.7049</v>
+        <v>-1.8456</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>242.04</v>
+        <v>230.85</v>
       </c>
       <c r="C14" t="n">
-        <v>274.5</v>
+        <v>233.69</v>
       </c>
       <c r="D14" t="n">
-        <v>228.55</v>
+        <v>181.81</v>
       </c>
       <c r="E14" t="n">
-        <v>262.7</v>
+        <v>182.54</v>
       </c>
       <c r="F14" t="n">
-        <v>83.47</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>86.25</v>
+        <v>82.08</v>
       </c>
       <c r="H14" t="n">
-        <v>82.48</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="I14" t="n">
-        <v>85.22</v>
+        <v>73.05</v>
       </c>
       <c r="J14" t="n">
-        <v>5.57</v>
+        <v>5.86</v>
       </c>
       <c r="K14" t="n">
-        <v>5.81</v>
+        <v>6.85</v>
       </c>
       <c r="L14" t="n">
-        <v>5</v>
+        <v>5.79</v>
       </c>
       <c r="M14" t="n">
-        <v>5.2</v>
+        <v>6.84</v>
       </c>
       <c r="N14" t="n">
-        <v>38.53</v>
+        <v>39.42</v>
       </c>
       <c r="O14" t="n">
-        <v>38.96</v>
+        <v>43.35</v>
       </c>
       <c r="P14" t="n">
-        <v>37.33</v>
+        <v>39.18</v>
       </c>
       <c r="Q14" t="n">
-        <v>37.76</v>
+        <v>43.19</v>
       </c>
       <c r="R14" t="n">
-        <v>-6.3592</v>
+        <v>-30.5139</v>
       </c>
       <c r="S14" t="n">
-        <v>15.7116</v>
+        <v>-31.4584</v>
       </c>
       <c r="T14" t="n">
-        <v>16.9479</v>
+        <v>-18.6324</v>
       </c>
       <c r="U14" t="n">
-        <v>-1.5481</v>
+        <v>-14.2807</v>
       </c>
       <c r="V14" t="n">
-        <v>-0.953</v>
+        <v>-16.2463</v>
       </c>
       <c r="W14" t="n">
-        <v>1.8403</v>
+        <v>-13.6116</v>
       </c>
       <c r="X14" t="n">
-        <v>5.9063</v>
+        <v>31.5385</v>
       </c>
       <c r="Y14" t="n">
-        <v>-16.9329</v>
+        <v>32.3017</v>
       </c>
       <c r="Z14" t="n">
-        <v>-17.5911</v>
+        <v>8.056900000000001</v>
       </c>
       <c r="AA14" t="n">
-        <v>1.5327</v>
+        <v>14.3803</v>
       </c>
       <c r="AB14" t="n">
-        <v>0.9086</v>
+        <v>17.0144</v>
       </c>
       <c r="AC14" t="n">
-        <v>-1.8456</v>
+        <v>13.4191</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>230.85</v>
+        <v>210.62</v>
       </c>
       <c r="C15" t="n">
-        <v>233.69</v>
+        <v>222.19</v>
       </c>
       <c r="D15" t="n">
-        <v>181.81</v>
+        <v>201.69</v>
       </c>
       <c r="E15" t="n">
-        <v>182.54</v>
+        <v>211.44</v>
       </c>
       <c r="F15" t="n">
-        <v>81.56999999999999</v>
+        <v>76.86</v>
       </c>
       <c r="G15" t="n">
-        <v>82.08</v>
+        <v>78.47</v>
       </c>
       <c r="H15" t="n">
-        <v>72.68000000000001</v>
+        <v>75.38</v>
       </c>
       <c r="I15" t="n">
-        <v>73.05</v>
+        <v>76.27</v>
       </c>
       <c r="J15" t="n">
-        <v>5.86</v>
+        <v>5.71</v>
       </c>
       <c r="K15" t="n">
-        <v>6.85</v>
+        <v>6.05</v>
       </c>
       <c r="L15" t="n">
-        <v>5.79</v>
+        <v>5.27</v>
       </c>
       <c r="M15" t="n">
-        <v>6.84</v>
+        <v>5.69</v>
       </c>
       <c r="N15" t="n">
-        <v>39.42</v>
+        <v>40.92</v>
       </c>
       <c r="O15" t="n">
-        <v>43.35</v>
+        <v>41.78</v>
       </c>
       <c r="P15" t="n">
-        <v>39.18</v>
+        <v>39.96</v>
       </c>
       <c r="Q15" t="n">
-        <v>43.19</v>
+        <v>41.26</v>
       </c>
       <c r="R15" t="n">
-        <v>-30.5139</v>
+        <v>15.8321</v>
       </c>
       <c r="S15" t="n">
-        <v>-31.4584</v>
+        <v>-24.6311</v>
       </c>
       <c r="T15" t="n">
-        <v>-18.6324</v>
+        <v>-6.8669</v>
       </c>
       <c r="U15" t="n">
-        <v>-14.2807</v>
+        <v>4.4079</v>
       </c>
       <c r="V15" t="n">
-        <v>-16.2463</v>
+        <v>-11.8877</v>
       </c>
       <c r="W15" t="n">
-        <v>-13.6116</v>
+        <v>-11.3552</v>
       </c>
       <c r="X15" t="n">
-        <v>31.5385</v>
+        <v>-16.8129</v>
       </c>
       <c r="Y15" t="n">
-        <v>32.3017</v>
+        <v>15.8859</v>
       </c>
       <c r="Z15" t="n">
-        <v>8.056900000000001</v>
+        <v>-9.105399999999999</v>
       </c>
       <c r="AA15" t="n">
-        <v>14.3803</v>
+        <v>-4.4686</v>
       </c>
       <c r="AB15" t="n">
-        <v>17.0144</v>
+        <v>10.9438</v>
       </c>
       <c r="AC15" t="n">
-        <v>13.4191</v>
+        <v>10.2619</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>210.62</v>
+        <v>227.06</v>
       </c>
       <c r="C16" t="n">
-        <v>222.19</v>
+        <v>231.02</v>
       </c>
       <c r="D16" t="n">
-        <v>201.69</v>
+        <v>157.56</v>
       </c>
       <c r="E16" t="n">
-        <v>211.44</v>
+        <v>201.68</v>
       </c>
       <c r="F16" t="n">
-        <v>76.86</v>
+        <v>78.48</v>
       </c>
       <c r="G16" t="n">
-        <v>78.47</v>
+        <v>79.34</v>
       </c>
       <c r="H16" t="n">
-        <v>75.38</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="I16" t="n">
-        <v>76.27</v>
+        <v>73.72</v>
       </c>
       <c r="J16" t="n">
-        <v>5.71</v>
+        <v>5.25</v>
       </c>
       <c r="K16" t="n">
-        <v>6.05</v>
+        <v>7.11</v>
       </c>
       <c r="L16" t="n">
-        <v>5.27</v>
+        <v>5.14</v>
       </c>
       <c r="M16" t="n">
-        <v>5.69</v>
+        <v>5.93</v>
       </c>
       <c r="N16" t="n">
-        <v>40.92</v>
+        <v>40.06</v>
       </c>
       <c r="O16" t="n">
-        <v>41.78</v>
+        <v>46.38</v>
       </c>
       <c r="P16" t="n">
-        <v>39.96</v>
+        <v>39.59</v>
       </c>
       <c r="Q16" t="n">
-        <v>41.26</v>
+        <v>42.67</v>
       </c>
       <c r="R16" t="n">
-        <v>15.8321</v>
+        <v>-4.616</v>
       </c>
       <c r="S16" t="n">
-        <v>-24.6311</v>
+        <v>-23.228</v>
       </c>
       <c r="T16" t="n">
-        <v>-6.8669</v>
+        <v>-24.2716</v>
       </c>
       <c r="U16" t="n">
-        <v>4.4079</v>
+        <v>-3.3434</v>
       </c>
       <c r="V16" t="n">
-        <v>-11.8877</v>
+        <v>-13.4945</v>
       </c>
       <c r="W16" t="n">
-        <v>-11.3552</v>
+        <v>-15.4781</v>
       </c>
       <c r="X16" t="n">
-        <v>-16.8129</v>
+        <v>4.2179</v>
       </c>
       <c r="Y16" t="n">
-        <v>15.8859</v>
+        <v>14.0385</v>
       </c>
       <c r="Z16" t="n">
-        <v>-9.105399999999999</v>
+        <v>14.7002</v>
       </c>
       <c r="AA16" t="n">
-        <v>-4.4686</v>
+        <v>3.4174</v>
       </c>
       <c r="AB16" t="n">
-        <v>10.9438</v>
+        <v>13.0032</v>
       </c>
       <c r="AC16" t="n">
-        <v>10.2619</v>
+        <v>15.6055</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>227.06</v>
+        <v>191.54</v>
       </c>
       <c r="C17" t="n">
-        <v>231.02</v>
+        <v>212.99</v>
       </c>
       <c r="D17" t="n">
-        <v>157.56</v>
+        <v>177.3</v>
       </c>
       <c r="E17" t="n">
-        <v>201.68</v>
+        <v>180.65</v>
       </c>
       <c r="F17" t="n">
-        <v>78.48</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>79.34</v>
+        <v>74.7</v>
       </c>
       <c r="H17" t="n">
-        <v>66.79000000000001</v>
+        <v>69</v>
       </c>
       <c r="I17" t="n">
-        <v>73.72</v>
+        <v>69.27</v>
       </c>
       <c r="J17" t="n">
-        <v>5.25</v>
+        <v>6.24</v>
       </c>
       <c r="K17" t="n">
-        <v>7.11</v>
+        <v>6.65</v>
       </c>
       <c r="L17" t="n">
-        <v>5.14</v>
+        <v>5.6</v>
       </c>
       <c r="M17" t="n">
-        <v>5.93</v>
+        <v>6.57</v>
       </c>
       <c r="N17" t="n">
-        <v>40.06</v>
+        <v>43.81</v>
       </c>
       <c r="O17" t="n">
-        <v>46.38</v>
+        <v>45.39</v>
       </c>
       <c r="P17" t="n">
-        <v>39.59</v>
+        <v>42.07</v>
       </c>
       <c r="Q17" t="n">
-        <v>42.67</v>
+        <v>45.25</v>
       </c>
       <c r="R17" t="n">
-        <v>-4.616</v>
+        <v>-10.4274</v>
       </c>
       <c r="S17" t="n">
-        <v>-23.228</v>
+        <v>-1.0354</v>
       </c>
       <c r="T17" t="n">
-        <v>-24.2716</v>
+        <v>-35.6063</v>
       </c>
       <c r="U17" t="n">
-        <v>-3.3434</v>
+        <v>-6.0364</v>
       </c>
       <c r="V17" t="n">
-        <v>-13.4945</v>
+        <v>-5.1745</v>
       </c>
       <c r="W17" t="n">
-        <v>-15.4781</v>
+        <v>-19.9746</v>
       </c>
       <c r="X17" t="n">
-        <v>4.2179</v>
+        <v>10.7926</v>
       </c>
       <c r="Y17" t="n">
-        <v>14.0385</v>
+        <v>-3.9474</v>
       </c>
       <c r="Z17" t="n">
-        <v>14.7002</v>
+        <v>33.8086</v>
       </c>
       <c r="AA17" t="n">
-        <v>3.4174</v>
+        <v>6.0464</v>
       </c>
       <c r="AB17" t="n">
-        <v>13.0032</v>
+        <v>4.7696</v>
       </c>
       <c r="AC17" t="n">
-        <v>15.6055</v>
+        <v>21.6725</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>191.54</v>
+        <v>192.3</v>
       </c>
       <c r="C18" t="n">
-        <v>212.99</v>
+        <v>225.63</v>
       </c>
       <c r="D18" t="n">
-        <v>177.3</v>
+        <v>192.3</v>
       </c>
       <c r="E18" t="n">
-        <v>180.65</v>
+        <v>223.99</v>
       </c>
       <c r="F18" t="n">
-        <v>71.68000000000001</v>
+        <v>70.89</v>
       </c>
       <c r="G18" t="n">
-        <v>74.7</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="H18" t="n">
-        <v>69</v>
+        <v>69.59</v>
       </c>
       <c r="I18" t="n">
-        <v>69.27</v>
+        <v>76.01000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>6.24</v>
+        <v>6.1</v>
       </c>
       <c r="K18" t="n">
-        <v>6.65</v>
+        <v>6.1</v>
       </c>
       <c r="L18" t="n">
-        <v>5.6</v>
+        <v>4.9</v>
       </c>
       <c r="M18" t="n">
-        <v>6.57</v>
+        <v>4.97</v>
       </c>
       <c r="N18" t="n">
-        <v>43.81</v>
+        <v>44.18</v>
       </c>
       <c r="O18" t="n">
-        <v>45.39</v>
+        <v>45.01</v>
       </c>
       <c r="P18" t="n">
-        <v>42.07</v>
+        <v>40.44</v>
       </c>
       <c r="Q18" t="n">
-        <v>45.25</v>
+        <v>40.83</v>
       </c>
       <c r="R18" t="n">
-        <v>-10.4274</v>
+        <v>23.9911</v>
       </c>
       <c r="S18" t="n">
-        <v>-1.0354</v>
+        <v>5.9355</v>
       </c>
       <c r="T18" t="n">
-        <v>-35.6063</v>
+        <v>-14.7354</v>
       </c>
       <c r="U18" t="n">
-        <v>-6.0364</v>
+        <v>9.73</v>
       </c>
       <c r="V18" t="n">
-        <v>-5.1745</v>
+        <v>-0.3409</v>
       </c>
       <c r="W18" t="n">
-        <v>-19.9746</v>
+        <v>-10.8073</v>
       </c>
       <c r="X18" t="n">
-        <v>10.7926</v>
+        <v>-24.3531</v>
       </c>
       <c r="Y18" t="n">
-        <v>-3.9474</v>
+        <v>-12.6538</v>
       </c>
       <c r="Z18" t="n">
-        <v>33.8086</v>
+        <v>-4.4231</v>
       </c>
       <c r="AA18" t="n">
-        <v>6.0464</v>
+        <v>-9.768000000000001</v>
       </c>
       <c r="AB18" t="n">
-        <v>4.7696</v>
+        <v>-1.0422</v>
       </c>
       <c r="AC18" t="n">
-        <v>21.6725</v>
+        <v>8.1303</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>192.3</v>
+        <v>222.22</v>
       </c>
       <c r="C19" t="n">
-        <v>225.63</v>
+        <v>242.4</v>
       </c>
       <c r="D19" t="n">
-        <v>192.3</v>
+        <v>214.74</v>
       </c>
       <c r="E19" t="n">
-        <v>223.99</v>
+        <v>234.68</v>
       </c>
       <c r="F19" t="n">
-        <v>70.89</v>
+        <v>76.34</v>
       </c>
       <c r="G19" t="n">
-        <v>76.59999999999999</v>
+        <v>78.36</v>
       </c>
       <c r="H19" t="n">
-        <v>69.59</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="I19" t="n">
-        <v>76.01000000000001</v>
+        <v>77.52</v>
       </c>
       <c r="J19" t="n">
-        <v>6.1</v>
+        <v>5.01</v>
       </c>
       <c r="K19" t="n">
-        <v>6.1</v>
+        <v>5.15</v>
       </c>
       <c r="L19" t="n">
-        <v>4.9</v>
+        <v>4.54</v>
       </c>
       <c r="M19" t="n">
-        <v>4.97</v>
+        <v>4.72</v>
       </c>
       <c r="N19" t="n">
-        <v>44.18</v>
+        <v>40.65</v>
       </c>
       <c r="O19" t="n">
-        <v>45.01</v>
+        <v>41.75</v>
       </c>
       <c r="P19" t="n">
-        <v>40.44</v>
+        <v>39.57</v>
       </c>
       <c r="Q19" t="n">
-        <v>40.83</v>
+        <v>40.04</v>
       </c>
       <c r="R19" t="n">
-        <v>23.9911</v>
+        <v>4.7725</v>
       </c>
       <c r="S19" t="n">
-        <v>5.9355</v>
+        <v>16.3626</v>
       </c>
       <c r="T19" t="n">
-        <v>-14.7354</v>
+        <v>28.5636</v>
       </c>
       <c r="U19" t="n">
-        <v>9.73</v>
+        <v>1.9866</v>
       </c>
       <c r="V19" t="n">
-        <v>-0.3409</v>
+        <v>5.1546</v>
       </c>
       <c r="W19" t="n">
-        <v>-10.8073</v>
+        <v>6.1191</v>
       </c>
       <c r="X19" t="n">
-        <v>-24.3531</v>
+        <v>-5.0302</v>
       </c>
       <c r="Y19" t="n">
-        <v>-12.6538</v>
+        <v>-20.4047</v>
       </c>
       <c r="Z19" t="n">
-        <v>-4.4231</v>
+        <v>-30.9942</v>
       </c>
       <c r="AA19" t="n">
-        <v>-9.768000000000001</v>
+        <v>-1.9349</v>
       </c>
       <c r="AB19" t="n">
-        <v>-1.0422</v>
+        <v>-6.1636</v>
       </c>
       <c r="AC19" t="n">
-        <v>8.1303</v>
+        <v>-7.2934</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>222.22</v>
+        <v>265.99</v>
       </c>
       <c r="C20" t="n">
-        <v>242.4</v>
+        <v>274.88</v>
       </c>
       <c r="D20" t="n">
-        <v>214.74</v>
+        <v>261.6</v>
       </c>
       <c r="E20" t="n">
-        <v>234.68</v>
+        <v>272.5</v>
       </c>
       <c r="F20" t="n">
-        <v>76.34</v>
+        <v>82.88</v>
       </c>
       <c r="G20" t="n">
-        <v>78.36</v>
+        <v>85.03</v>
       </c>
       <c r="H20" t="n">
-        <v>74.29000000000001</v>
+        <v>82.64</v>
       </c>
       <c r="I20" t="n">
-        <v>77.52</v>
+        <v>84.59</v>
       </c>
       <c r="J20" t="n">
-        <v>5.01</v>
+        <v>4.07</v>
       </c>
       <c r="K20" t="n">
-        <v>5.15</v>
+        <v>4.17</v>
       </c>
       <c r="L20" t="n">
-        <v>4.54</v>
+        <v>3.91</v>
       </c>
       <c r="M20" t="n">
-        <v>4.72</v>
+        <v>3.95</v>
       </c>
       <c r="N20" t="n">
-        <v>40.65</v>
+        <v>37.25</v>
       </c>
       <c r="O20" t="n">
-        <v>41.75</v>
+        <v>37.36</v>
       </c>
       <c r="P20" t="n">
-        <v>39.57</v>
+        <v>36.15</v>
       </c>
       <c r="Q20" t="n">
-        <v>40.04</v>
+        <v>36.31</v>
       </c>
       <c r="R20" t="n">
-        <v>4.7725</v>
+        <v>16.1156</v>
       </c>
       <c r="S20" t="n">
-        <v>16.3626</v>
+        <v>50.8442</v>
       </c>
       <c r="T20" t="n">
-        <v>28.5636</v>
+        <v>28.8782</v>
       </c>
       <c r="U20" t="n">
-        <v>1.9866</v>
+        <v>9.120200000000001</v>
       </c>
       <c r="V20" t="n">
-        <v>5.1546</v>
+        <v>22.1164</v>
       </c>
       <c r="W20" t="n">
-        <v>6.1191</v>
+        <v>10.9086</v>
       </c>
       <c r="X20" t="n">
-        <v>-5.0302</v>
+        <v>-16.3136</v>
       </c>
       <c r="Y20" t="n">
-        <v>-20.4047</v>
+        <v>-39.8782</v>
       </c>
       <c r="Z20" t="n">
-        <v>-30.9942</v>
+        <v>-30.58</v>
       </c>
       <c r="AA20" t="n">
-        <v>-1.9349</v>
+        <v>-9.3157</v>
       </c>
       <c r="AB20" t="n">
-        <v>-6.1636</v>
+        <v>-19.7569</v>
       </c>
       <c r="AC20" t="n">
-        <v>-7.2934</v>
+        <v>-11.9971</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>265.99</v>
+        <v>267.13</v>
       </c>
       <c r="C21" t="n">
-        <v>274.88</v>
+        <v>274.93</v>
       </c>
       <c r="D21" t="n">
-        <v>261.6</v>
+        <v>226</v>
       </c>
       <c r="E21" t="n">
-        <v>272.5</v>
+        <v>226.19</v>
       </c>
       <c r="F21" t="n">
-        <v>82.88</v>
+        <v>84.19</v>
       </c>
       <c r="G21" t="n">
-        <v>85.03</v>
+        <v>84.83</v>
       </c>
       <c r="H21" t="n">
-        <v>82.64</v>
+        <v>79.86</v>
       </c>
       <c r="I21" t="n">
-        <v>84.59</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>4.07</v>
+        <v>4.03</v>
       </c>
       <c r="K21" t="n">
-        <v>4.17</v>
+        <v>4.65</v>
       </c>
       <c r="L21" t="n">
         <v>3.91</v>
       </c>
       <c r="M21" t="n">
-        <v>3.95</v>
+        <v>4.63</v>
       </c>
       <c r="N21" t="n">
-        <v>37.25</v>
+        <v>36.54</v>
       </c>
       <c r="O21" t="n">
-        <v>37.36</v>
+        <v>38.39</v>
       </c>
       <c r="P21" t="n">
-        <v>36.15</v>
+        <v>36.26</v>
       </c>
       <c r="Q21" t="n">
-        <v>36.31</v>
+        <v>38.35</v>
       </c>
       <c r="R21" t="n">
-        <v>16.1156</v>
+        <v>-16.9945</v>
       </c>
       <c r="S21" t="n">
-        <v>50.8442</v>
+        <v>0.9822</v>
       </c>
       <c r="T21" t="n">
-        <v>28.8782</v>
+        <v>12.1529</v>
       </c>
       <c r="U21" t="n">
-        <v>9.120200000000001</v>
+        <v>-5.5089</v>
       </c>
       <c r="V21" t="n">
-        <v>22.1164</v>
+        <v>5.1572</v>
       </c>
       <c r="W21" t="n">
-        <v>10.9086</v>
+        <v>8.4238</v>
       </c>
       <c r="X21" t="n">
-        <v>-16.3136</v>
+        <v>17.2152</v>
       </c>
       <c r="Y21" t="n">
-        <v>-39.8782</v>
+        <v>-6.841</v>
       </c>
       <c r="Z21" t="n">
-        <v>-30.58</v>
+        <v>-21.9224</v>
       </c>
       <c r="AA21" t="n">
-        <v>-9.3157</v>
+        <v>5.6183</v>
       </c>
       <c r="AB21" t="n">
-        <v>-19.7569</v>
+        <v>-6.074</v>
       </c>
       <c r="AC21" t="n">
-        <v>-11.9971</v>
+        <v>-10.1242</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>267.13</v>
+        <v>247.42</v>
       </c>
       <c r="C22" t="n">
-        <v>274.9297</v>
+        <v>259.79</v>
       </c>
       <c r="D22" t="n">
-        <v>226.005</v>
+        <v>233.455</v>
       </c>
       <c r="E22" t="n">
-        <v>226.19</v>
+        <v>233.86</v>
       </c>
       <c r="F22" t="n">
-        <v>84.19</v>
+        <v>81.65000000000001</v>
       </c>
       <c r="G22" t="n">
-        <v>84.83</v>
+        <v>81.80500000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>79.86</v>
+        <v>76.94</v>
       </c>
       <c r="I22" t="n">
-        <v>79.93000000000001</v>
+        <v>77.54000000000001</v>
       </c>
       <c r="J22" t="n">
-        <v>4.025</v>
+        <v>4.17</v>
       </c>
       <c r="K22" t="n">
-        <v>4.65</v>
+        <v>4.45</v>
       </c>
       <c r="L22" t="n">
-        <v>3.91</v>
+        <v>3.92</v>
       </c>
       <c r="M22" t="n">
-        <v>4.63</v>
+        <v>4.46</v>
       </c>
       <c r="N22" t="n">
-        <v>36.55</v>
+        <v>37.54</v>
       </c>
       <c r="O22" t="n">
-        <v>38.39</v>
+        <v>39.79</v>
       </c>
       <c r="P22" t="n">
-        <v>36.26</v>
+        <v>37.46</v>
       </c>
       <c r="Q22" t="n">
-        <v>38.35</v>
+        <v>39.52</v>
       </c>
       <c r="R22" t="n">
-        <v>-16.9945</v>
+        <v>3.391</v>
       </c>
       <c r="S22" t="n">
-        <v>0.9822</v>
+        <v>-0.3494</v>
       </c>
       <c r="T22" t="n">
-        <v>12.1529</v>
+        <v>29.4547</v>
       </c>
       <c r="U22" t="n">
-        <v>-5.5089</v>
+        <v>-2.9901</v>
       </c>
       <c r="V22" t="n">
-        <v>5.1572</v>
+        <v>0.0258</v>
       </c>
       <c r="W22" t="n">
-        <v>8.4238</v>
+        <v>11.9388</v>
       </c>
       <c r="X22" t="n">
-        <v>17.2152</v>
+        <v>-3.6717</v>
       </c>
       <c r="Y22" t="n">
-        <v>-6.841</v>
+        <v>-5.5085</v>
       </c>
       <c r="Z22" t="n">
-        <v>-21.9224</v>
+        <v>-32.1157</v>
       </c>
       <c r="AA22" t="n">
-        <v>5.6183</v>
+        <v>3.0508</v>
       </c>
       <c r="AB22" t="n">
-        <v>-6.074</v>
+        <v>-1.2987</v>
       </c>
       <c r="AC22" t="n">
-        <v>-10.1242</v>
+        <v>-12.663</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-18 23:46
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>141.24</v>
+        <v>161</v>
       </c>
       <c r="C2" t="n">
-        <v>160.6</v>
+        <v>173.7</v>
       </c>
       <c r="D2" t="n">
-        <v>135.02</v>
+        <v>161</v>
       </c>
       <c r="E2" t="n">
-        <v>151.89</v>
+        <v>173.2</v>
       </c>
       <c r="F2" t="n">
-        <v>72.41</v>
+        <v>74.09</v>
       </c>
       <c r="G2" t="n">
-        <v>74.5</v>
+        <v>76.53</v>
       </c>
       <c r="H2" t="n">
-        <v>70.95999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="I2" t="n">
-        <v>72.93000000000001</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>10.64</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>11.07</v>
+        <v>9.35</v>
       </c>
       <c r="L2" t="n">
-        <v>9.369999999999999</v>
+        <v>8.51</v>
       </c>
       <c r="M2" t="n">
-        <v>9.93</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="N2" t="n">
-        <v>44.68</v>
+        <v>43.67</v>
       </c>
       <c r="O2" t="n">
-        <v>45.53</v>
+        <v>43.97</v>
       </c>
       <c r="P2" t="n">
-        <v>43.46</v>
+        <v>42.19</v>
       </c>
       <c r="Q2" t="n">
-        <v>44.37</v>
+        <v>42.19</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>161</v>
+        <v>171.26</v>
       </c>
       <c r="C3" t="n">
-        <v>173.7</v>
+        <v>179.97</v>
       </c>
       <c r="D3" t="n">
-        <v>161</v>
+        <v>168.23</v>
       </c>
       <c r="E3" t="n">
-        <v>173.2</v>
+        <v>178.39</v>
       </c>
       <c r="F3" t="n">
-        <v>74.09</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>76.53</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>73.62</v>
+        <v>74.47</v>
       </c>
       <c r="I3" t="n">
-        <v>76.51000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J3" t="n">
-        <v>9.300000000000001</v>
+        <v>8.65</v>
       </c>
       <c r="K3" t="n">
-        <v>9.35</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L3" t="n">
-        <v>8.51</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M3" t="n">
-        <v>8.539999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N3" t="n">
-        <v>43.67</v>
+        <v>42.94</v>
       </c>
       <c r="O3" t="n">
-        <v>43.97</v>
+        <v>43.33</v>
       </c>
       <c r="P3" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="Q3" t="n">
-        <v>42.19</v>
+        <v>41.96</v>
       </c>
       <c r="R3" t="n">
-        <v>14.0299</v>
+        <v>2.9965</v>
       </c>
       <c r="U3" t="n">
-        <v>4.9088</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="X3" t="n">
-        <v>-13.998</v>
+        <v>-2.9274</v>
       </c>
       <c r="AA3" t="n">
-        <v>-4.9132</v>
+        <v>-0.5452</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>171.26</v>
+        <v>184.8</v>
       </c>
       <c r="C4" t="n">
-        <v>179.97</v>
+        <v>195.27</v>
       </c>
       <c r="D4" t="n">
-        <v>168.23</v>
+        <v>183.34</v>
       </c>
       <c r="E4" t="n">
-        <v>178.39</v>
+        <v>190.56</v>
       </c>
       <c r="F4" t="n">
-        <v>75.18000000000001</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>77.79000000000001</v>
+        <v>79.33</v>
       </c>
       <c r="H4" t="n">
-        <v>74.47</v>
+        <v>77.33</v>
       </c>
       <c r="I4" t="n">
-        <v>76.95</v>
+        <v>77.84</v>
       </c>
       <c r="J4" t="n">
-        <v>8.65</v>
+        <v>8</v>
       </c>
       <c r="K4" t="n">
-        <v>8.779999999999999</v>
+        <v>8.06</v>
       </c>
       <c r="L4" t="n">
-        <v>8.210000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="M4" t="n">
-        <v>8.289999999999999</v>
+        <v>7.73</v>
       </c>
       <c r="N4" t="n">
-        <v>42.94</v>
+        <v>41.4</v>
       </c>
       <c r="O4" t="n">
-        <v>43.33</v>
+        <v>41.78</v>
       </c>
       <c r="P4" t="n">
+        <v>40.68</v>
+      </c>
+      <c r="Q4" t="n">
         <v>41.5</v>
       </c>
-      <c r="Q4" t="n">
-        <v>41.96</v>
-      </c>
       <c r="R4" t="n">
-        <v>2.9965</v>
+        <v>6.8221</v>
       </c>
       <c r="U4" t="n">
-        <v>0.5750999999999999</v>
+        <v>1.1566</v>
       </c>
       <c r="X4" t="n">
-        <v>-2.9274</v>
+        <v>-6.7551</v>
       </c>
       <c r="AA4" t="n">
-        <v>-0.5452</v>
+        <v>-1.0963</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>184.8</v>
+        <v>211.38</v>
       </c>
       <c r="C5" t="n">
-        <v>195.27</v>
+        <v>228.5</v>
       </c>
       <c r="D5" t="n">
-        <v>183.34</v>
+        <v>209.89</v>
       </c>
       <c r="E5" t="n">
-        <v>190.56</v>
+        <v>225.79</v>
       </c>
       <c r="F5" t="n">
-        <v>78.04000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="G5" t="n">
-        <v>79.33</v>
+        <v>82.27</v>
       </c>
       <c r="H5" t="n">
-        <v>77.33</v>
+        <v>79.98</v>
       </c>
       <c r="I5" t="n">
-        <v>77.84</v>
+        <v>81.95</v>
       </c>
       <c r="J5" t="n">
-        <v>8</v>
+        <v>6.9</v>
       </c>
       <c r="K5" t="n">
-        <v>8.06</v>
+        <v>6.95</v>
       </c>
       <c r="L5" t="n">
-        <v>7.5</v>
+        <v>6.19</v>
       </c>
       <c r="M5" t="n">
-        <v>7.73</v>
+        <v>6.29</v>
       </c>
       <c r="N5" t="n">
-        <v>41.4</v>
+        <v>40.05</v>
       </c>
       <c r="O5" t="n">
-        <v>41.78</v>
+        <v>40.35</v>
       </c>
       <c r="P5" t="n">
-        <v>40.68</v>
+        <v>39.14</v>
       </c>
       <c r="Q5" t="n">
-        <v>41.5</v>
+        <v>39.28</v>
       </c>
       <c r="R5" t="n">
-        <v>6.8221</v>
+        <v>18.4876</v>
       </c>
       <c r="S5" t="n">
-        <v>25.4592</v>
+        <v>30.3637</v>
       </c>
       <c r="U5" t="n">
-        <v>1.1566</v>
+        <v>5.2801</v>
       </c>
       <c r="V5" t="n">
-        <v>6.7325</v>
+        <v>7.1102</v>
       </c>
       <c r="X5" t="n">
-        <v>-6.7551</v>
+        <v>-18.6287</v>
       </c>
       <c r="Y5" t="n">
-        <v>-22.1551</v>
+        <v>-26.3466</v>
       </c>
       <c r="AA5" t="n">
-        <v>-1.0963</v>
+        <v>-5.3494</v>
       </c>
       <c r="AB5" t="n">
-        <v>-6.4683</v>
+        <v>-6.8974</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>211.38</v>
+        <v>242.66</v>
       </c>
       <c r="C6" t="n">
-        <v>228.5</v>
+        <v>242.66</v>
       </c>
       <c r="D6" t="n">
-        <v>209.89</v>
+        <v>204</v>
       </c>
       <c r="E6" t="n">
-        <v>225.79</v>
+        <v>217.98</v>
       </c>
       <c r="F6" t="n">
-        <v>80.59</v>
+        <v>82.87</v>
       </c>
       <c r="G6" t="n">
-        <v>82.27</v>
+        <v>82.91</v>
       </c>
       <c r="H6" t="n">
-        <v>79.98</v>
+        <v>80.33</v>
       </c>
       <c r="I6" t="n">
-        <v>81.95</v>
+        <v>81.67</v>
       </c>
       <c r="J6" t="n">
-        <v>6.9</v>
+        <v>5.83</v>
       </c>
       <c r="K6" t="n">
-        <v>6.95</v>
+        <v>6.91</v>
       </c>
       <c r="L6" t="n">
-        <v>6.19</v>
+        <v>5.83</v>
       </c>
       <c r="M6" t="n">
-        <v>6.29</v>
+        <v>6.53</v>
       </c>
       <c r="N6" t="n">
-        <v>40.05</v>
+        <v>38.87</v>
       </c>
       <c r="O6" t="n">
-        <v>40.35</v>
+        <v>40.09</v>
       </c>
       <c r="P6" t="n">
-        <v>39.14</v>
+        <v>38.86</v>
       </c>
       <c r="Q6" t="n">
-        <v>39.28</v>
+        <v>39.44</v>
       </c>
       <c r="R6" t="n">
-        <v>18.4876</v>
+        <v>-3.459</v>
       </c>
       <c r="S6" t="n">
-        <v>30.3637</v>
+        <v>22.1929</v>
       </c>
       <c r="U6" t="n">
-        <v>5.2801</v>
+        <v>-0.3417</v>
       </c>
       <c r="V6" t="n">
-        <v>7.1102</v>
+        <v>6.1339</v>
       </c>
       <c r="X6" t="n">
-        <v>-18.6287</v>
+        <v>3.8156</v>
       </c>
       <c r="Y6" t="n">
-        <v>-26.3466</v>
+        <v>-21.2304</v>
       </c>
       <c r="AA6" t="n">
-        <v>-5.3494</v>
+        <v>0.4073</v>
       </c>
       <c r="AB6" t="n">
-        <v>-6.8974</v>
+        <v>-6.0057</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>242.66</v>
+        <v>219</v>
       </c>
       <c r="C7" t="n">
-        <v>242.66</v>
+        <v>231.89</v>
       </c>
       <c r="D7" t="n">
-        <v>204</v>
+        <v>207.56</v>
       </c>
       <c r="E7" t="n">
-        <v>217.98</v>
+        <v>224.63</v>
       </c>
       <c r="F7" t="n">
-        <v>82.87</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>82.91</v>
+        <v>84.05</v>
       </c>
       <c r="H7" t="n">
-        <v>80.33</v>
+        <v>80.66</v>
       </c>
       <c r="I7" t="n">
-        <v>81.67</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>5.83</v>
+        <v>6.49</v>
       </c>
       <c r="K7" t="n">
-        <v>6.91</v>
+        <v>6.83</v>
       </c>
       <c r="L7" t="n">
-        <v>5.83</v>
+        <v>6.1</v>
       </c>
       <c r="M7" t="n">
-        <v>6.53</v>
+        <v>6.31</v>
       </c>
       <c r="N7" t="n">
-        <v>38.87</v>
+        <v>39.41</v>
       </c>
       <c r="O7" t="n">
-        <v>40.09</v>
+        <v>39.94</v>
       </c>
       <c r="P7" t="n">
-        <v>38.86</v>
+        <v>38.3</v>
       </c>
       <c r="Q7" t="n">
-        <v>39.44</v>
+        <v>38.47</v>
       </c>
       <c r="R7" t="n">
-        <v>-3.459</v>
+        <v>3.0507</v>
       </c>
       <c r="S7" t="n">
-        <v>22.1929</v>
+        <v>17.8789</v>
       </c>
       <c r="T7" t="n">
-        <v>43.5118</v>
+        <v>29.694</v>
       </c>
       <c r="U7" t="n">
-        <v>-0.3417</v>
+        <v>2.4611</v>
       </c>
       <c r="V7" t="n">
-        <v>6.1339</v>
+        <v>7.5026</v>
       </c>
       <c r="W7" t="n">
-        <v>11.9841</v>
+        <v>9.3713</v>
       </c>
       <c r="X7" t="n">
-        <v>3.8156</v>
+        <v>-3.3691</v>
       </c>
       <c r="Y7" t="n">
-        <v>-21.2304</v>
+        <v>-18.37</v>
       </c>
       <c r="Z7" t="n">
-        <v>-34.2397</v>
+        <v>-26.1124</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.4073</v>
+        <v>-2.4594</v>
       </c>
       <c r="AB7" t="n">
-        <v>-6.0057</v>
+        <v>-7.3012</v>
       </c>
       <c r="AC7" t="n">
-        <v>-11.1111</v>
+        <v>-8.817299999999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>219</v>
+        <v>231.82</v>
       </c>
       <c r="C8" t="n">
-        <v>231.89</v>
+        <v>239.07</v>
       </c>
       <c r="D8" t="n">
-        <v>207.56</v>
+        <v>218.56</v>
       </c>
       <c r="E8" t="n">
-        <v>224.63</v>
+        <v>224.34</v>
       </c>
       <c r="F8" t="n">
-        <v>81.73999999999999</v>
+        <v>84.41</v>
       </c>
       <c r="G8" t="n">
-        <v>84.05</v>
+        <v>85.7</v>
       </c>
       <c r="H8" t="n">
-        <v>80.66</v>
+        <v>83.53</v>
       </c>
       <c r="I8" t="n">
-        <v>83.68000000000001</v>
+        <v>84.56</v>
       </c>
       <c r="J8" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="K8" t="n">
         <v>6.49</v>
       </c>
-      <c r="K8" t="n">
-        <v>6.83</v>
-      </c>
       <c r="L8" t="n">
-        <v>6.1</v>
+        <v>5.91</v>
       </c>
       <c r="M8" t="n">
-        <v>6.31</v>
+        <v>6.33</v>
       </c>
       <c r="N8" t="n">
-        <v>39.41</v>
+        <v>38.15</v>
       </c>
       <c r="O8" t="n">
-        <v>39.94</v>
+        <v>38.56</v>
       </c>
       <c r="P8" t="n">
-        <v>38.3</v>
+        <v>37.56</v>
       </c>
       <c r="Q8" t="n">
-        <v>38.47</v>
+        <v>38.08</v>
       </c>
       <c r="R8" t="n">
-        <v>3.0507</v>
+        <v>-0.1291</v>
       </c>
       <c r="S8" t="n">
-        <v>17.8789</v>
+        <v>-0.6422</v>
       </c>
       <c r="T8" t="n">
-        <v>29.694</v>
+        <v>25.7582</v>
       </c>
       <c r="U8" t="n">
-        <v>2.4611</v>
+        <v>1.0516</v>
       </c>
       <c r="V8" t="n">
-        <v>7.5026</v>
+        <v>3.1849</v>
       </c>
       <c r="W8" t="n">
-        <v>9.3713</v>
+        <v>9.8895</v>
       </c>
       <c r="X8" t="n">
-        <v>-3.3691</v>
+        <v>0.317</v>
       </c>
       <c r="Y8" t="n">
-        <v>-18.37</v>
+        <v>0.6359</v>
       </c>
       <c r="Z8" t="n">
-        <v>-26.1124</v>
+        <v>-23.6429</v>
       </c>
       <c r="AA8" t="n">
-        <v>-2.4594</v>
+        <v>-1.0138</v>
       </c>
       <c r="AB8" t="n">
-        <v>-7.3012</v>
+        <v>-3.055</v>
       </c>
       <c r="AC8" t="n">
-        <v>-8.817299999999999</v>
+        <v>-9.2469</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>231.82</v>
+        <v>217.27</v>
       </c>
       <c r="C9" t="n">
-        <v>239.07</v>
+        <v>234.06</v>
       </c>
       <c r="D9" t="n">
-        <v>218.56</v>
+        <v>210.14</v>
       </c>
       <c r="E9" t="n">
-        <v>224.34</v>
+        <v>227.03</v>
       </c>
       <c r="F9" t="n">
-        <v>84.41</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>85.7</v>
+        <v>87.06</v>
       </c>
       <c r="H9" t="n">
-        <v>83.53</v>
+        <v>83.75</v>
       </c>
       <c r="I9" t="n">
-        <v>84.56</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>6.11</v>
+        <v>6.55</v>
       </c>
       <c r="K9" t="n">
-        <v>6.49</v>
+        <v>6.74</v>
       </c>
       <c r="L9" t="n">
-        <v>5.91</v>
+        <v>6.05</v>
       </c>
       <c r="M9" t="n">
-        <v>6.33</v>
+        <v>6.26</v>
       </c>
       <c r="N9" t="n">
-        <v>38.15</v>
+        <v>38.27</v>
       </c>
       <c r="O9" t="n">
-        <v>38.56</v>
+        <v>38.46</v>
       </c>
       <c r="P9" t="n">
-        <v>37.56</v>
+        <v>36.96</v>
       </c>
       <c r="Q9" t="n">
-        <v>38.08</v>
+        <v>37.42</v>
       </c>
       <c r="R9" t="n">
-        <v>-0.1291</v>
+        <v>1.1991</v>
       </c>
       <c r="S9" t="n">
-        <v>-0.6422</v>
+        <v>4.1518</v>
       </c>
       <c r="T9" t="n">
-        <v>25.7582</v>
+        <v>19.1383</v>
       </c>
       <c r="U9" t="n">
-        <v>1.0516</v>
+        <v>1.7502</v>
       </c>
       <c r="V9" t="n">
-        <v>3.1849</v>
+        <v>5.3508</v>
       </c>
       <c r="W9" t="n">
-        <v>9.8895</v>
+        <v>10.5344</v>
       </c>
       <c r="X9" t="n">
-        <v>0.317</v>
+        <v>-1.1058</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.6359</v>
+        <v>-4.1348</v>
       </c>
       <c r="Z9" t="n">
-        <v>-23.6429</v>
+        <v>-19.0168</v>
       </c>
       <c r="AA9" t="n">
-        <v>-1.0138</v>
+        <v>-1.7332</v>
       </c>
       <c r="AB9" t="n">
-        <v>-3.055</v>
+        <v>-5.1217</v>
       </c>
       <c r="AC9" t="n">
-        <v>-9.2469</v>
+        <v>-9.831300000000001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>217.27</v>
+        <v>243.18</v>
       </c>
       <c r="C10" t="n">
-        <v>234.06</v>
+        <v>267.08</v>
       </c>
       <c r="D10" t="n">
-        <v>210.14</v>
+        <v>238.82</v>
       </c>
       <c r="E10" t="n">
-        <v>227.03</v>
+        <v>266.32</v>
       </c>
       <c r="F10" t="n">
-        <v>84.15000000000001</v>
+        <v>85.94</v>
       </c>
       <c r="G10" t="n">
-        <v>87.06</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>83.75</v>
+        <v>84.83</v>
       </c>
       <c r="I10" t="n">
-        <v>86.04000000000001</v>
+        <v>87.22</v>
       </c>
       <c r="J10" t="n">
-        <v>6.55</v>
+        <v>5.8</v>
       </c>
       <c r="K10" t="n">
-        <v>6.74</v>
+        <v>5.93</v>
       </c>
       <c r="L10" t="n">
-        <v>6.05</v>
+        <v>5.15</v>
       </c>
       <c r="M10" t="n">
-        <v>6.26</v>
+        <v>5.17</v>
       </c>
       <c r="N10" t="n">
-        <v>38.27</v>
+        <v>37.47</v>
       </c>
       <c r="O10" t="n">
-        <v>38.46</v>
+        <v>37.95</v>
       </c>
       <c r="P10" t="n">
-        <v>36.96</v>
+        <v>36.86</v>
       </c>
       <c r="Q10" t="n">
-        <v>37.42</v>
+        <v>36.91</v>
       </c>
       <c r="R10" t="n">
-        <v>1.1991</v>
+        <v>17.3061</v>
       </c>
       <c r="S10" t="n">
-        <v>4.1518</v>
+        <v>18.5594</v>
       </c>
       <c r="T10" t="n">
-        <v>19.1383</v>
+        <v>17.9503</v>
       </c>
       <c r="U10" t="n">
-        <v>1.7502</v>
+        <v>1.3715</v>
       </c>
       <c r="V10" t="n">
-        <v>5.3508</v>
+        <v>4.2304</v>
       </c>
       <c r="W10" t="n">
-        <v>10.5344</v>
+        <v>6.4308</v>
       </c>
       <c r="X10" t="n">
-        <v>-1.1058</v>
+        <v>-17.4121</v>
       </c>
       <c r="Y10" t="n">
-        <v>-4.1348</v>
+        <v>-18.0666</v>
       </c>
       <c r="Z10" t="n">
-        <v>-19.0168</v>
+        <v>-17.806</v>
       </c>
       <c r="AA10" t="n">
-        <v>-1.7332</v>
+        <v>-1.3629</v>
       </c>
       <c r="AB10" t="n">
-        <v>-5.1217</v>
+        <v>-4.0551</v>
       </c>
       <c r="AC10" t="n">
-        <v>-9.831300000000001</v>
+        <v>-6.0336</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>243.18</v>
+        <v>281.47</v>
       </c>
       <c r="C11" t="n">
-        <v>267.08</v>
+        <v>284.58</v>
       </c>
       <c r="D11" t="n">
-        <v>238.82</v>
+        <v>257.26</v>
       </c>
       <c r="E11" t="n">
-        <v>266.32</v>
+        <v>280.54</v>
       </c>
       <c r="F11" t="n">
-        <v>85.94</v>
+        <v>87.68000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>87.31999999999999</v>
+        <v>88.09</v>
       </c>
       <c r="H11" t="n">
-        <v>84.83</v>
+        <v>85.41</v>
       </c>
       <c r="I11" t="n">
-        <v>87.22</v>
+        <v>86.56</v>
       </c>
       <c r="J11" t="n">
-        <v>5.8</v>
+        <v>4.88</v>
       </c>
       <c r="K11" t="n">
-        <v>5.93</v>
+        <v>5.35</v>
       </c>
       <c r="L11" t="n">
-        <v>5.15</v>
+        <v>4.82</v>
       </c>
       <c r="M11" t="n">
-        <v>5.17</v>
+        <v>4.91</v>
       </c>
       <c r="N11" t="n">
-        <v>37.47</v>
+        <v>36.73</v>
       </c>
       <c r="O11" t="n">
-        <v>37.95</v>
+        <v>37.69</v>
       </c>
       <c r="P11" t="n">
-        <v>36.86</v>
+        <v>36.55</v>
       </c>
       <c r="Q11" t="n">
-        <v>36.91</v>
+        <v>37.19</v>
       </c>
       <c r="R11" t="n">
-        <v>17.3061</v>
+        <v>5.3394</v>
       </c>
       <c r="S11" t="n">
-        <v>18.5594</v>
+        <v>25.0513</v>
       </c>
       <c r="T11" t="n">
-        <v>17.9503</v>
+        <v>28.6999</v>
       </c>
       <c r="U11" t="n">
-        <v>1.3715</v>
+        <v>-0.7567</v>
       </c>
       <c r="V11" t="n">
-        <v>4.2304</v>
+        <v>2.3652</v>
       </c>
       <c r="W11" t="n">
-        <v>6.4308</v>
+        <v>5.9875</v>
       </c>
       <c r="X11" t="n">
-        <v>-17.4121</v>
+        <v>-5.029</v>
       </c>
       <c r="Y11" t="n">
-        <v>-18.0666</v>
+        <v>-22.4329</v>
       </c>
       <c r="Z11" t="n">
-        <v>-17.806</v>
+        <v>-24.8086</v>
       </c>
       <c r="AA11" t="n">
-        <v>-1.3629</v>
+        <v>0.7586000000000001</v>
       </c>
       <c r="AB11" t="n">
-        <v>-4.0551</v>
+        <v>-2.3372</v>
       </c>
       <c r="AC11" t="n">
-        <v>-6.0336</v>
+        <v>-5.7049</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>281.47</v>
+        <v>242.04</v>
       </c>
       <c r="C12" t="n">
-        <v>284.58</v>
+        <v>274.5</v>
       </c>
       <c r="D12" t="n">
-        <v>257.26</v>
+        <v>228.55</v>
       </c>
       <c r="E12" t="n">
-        <v>280.54</v>
+        <v>262.7</v>
       </c>
       <c r="F12" t="n">
-        <v>87.68000000000001</v>
+        <v>83.47</v>
       </c>
       <c r="G12" t="n">
-        <v>88.09</v>
+        <v>86.25</v>
       </c>
       <c r="H12" t="n">
-        <v>85.41</v>
+        <v>82.48</v>
       </c>
       <c r="I12" t="n">
-        <v>86.56</v>
+        <v>85.22</v>
       </c>
       <c r="J12" t="n">
-        <v>4.88</v>
+        <v>5.57</v>
       </c>
       <c r="K12" t="n">
-        <v>5.35</v>
+        <v>5.81</v>
       </c>
       <c r="L12" t="n">
-        <v>4.82</v>
+        <v>5</v>
       </c>
       <c r="M12" t="n">
-        <v>4.91</v>
+        <v>5.2</v>
       </c>
       <c r="N12" t="n">
-        <v>36.73</v>
+        <v>38.53</v>
       </c>
       <c r="O12" t="n">
-        <v>37.69</v>
+        <v>38.96</v>
       </c>
       <c r="P12" t="n">
-        <v>36.55</v>
+        <v>37.33</v>
       </c>
       <c r="Q12" t="n">
-        <v>37.19</v>
+        <v>37.76</v>
       </c>
       <c r="R12" t="n">
-        <v>5.3394</v>
+        <v>-6.3592</v>
       </c>
       <c r="S12" t="n">
-        <v>25.0513</v>
+        <v>15.7116</v>
       </c>
       <c r="T12" t="n">
-        <v>28.6999</v>
+        <v>16.9479</v>
       </c>
       <c r="U12" t="n">
-        <v>-0.7567</v>
+        <v>-1.5481</v>
       </c>
       <c r="V12" t="n">
-        <v>2.3652</v>
+        <v>-0.953</v>
       </c>
       <c r="W12" t="n">
-        <v>5.9875</v>
+        <v>1.8403</v>
       </c>
       <c r="X12" t="n">
-        <v>-5.029</v>
+        <v>5.9063</v>
       </c>
       <c r="Y12" t="n">
-        <v>-22.4329</v>
+        <v>-16.9329</v>
       </c>
       <c r="Z12" t="n">
-        <v>-24.8086</v>
+        <v>-17.5911</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.7586000000000001</v>
+        <v>1.5327</v>
       </c>
       <c r="AB12" t="n">
-        <v>-2.3372</v>
+        <v>0.9086</v>
       </c>
       <c r="AC12" t="n">
-        <v>-5.7049</v>
+        <v>-1.8456</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>242.04</v>
+        <v>230.85</v>
       </c>
       <c r="C13" t="n">
-        <v>274.5</v>
+        <v>233.69</v>
       </c>
       <c r="D13" t="n">
-        <v>228.55</v>
+        <v>181.81</v>
       </c>
       <c r="E13" t="n">
-        <v>262.7</v>
+        <v>182.54</v>
       </c>
       <c r="F13" t="n">
-        <v>83.47</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>86.25</v>
+        <v>82.08</v>
       </c>
       <c r="H13" t="n">
-        <v>82.48</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="I13" t="n">
-        <v>85.22</v>
+        <v>73.05</v>
       </c>
       <c r="J13" t="n">
-        <v>5.57</v>
+        <v>5.86</v>
       </c>
       <c r="K13" t="n">
-        <v>5.81</v>
+        <v>6.85</v>
       </c>
       <c r="L13" t="n">
-        <v>5</v>
+        <v>5.79</v>
       </c>
       <c r="M13" t="n">
-        <v>5.2</v>
+        <v>6.84</v>
       </c>
       <c r="N13" t="n">
-        <v>38.53</v>
+        <v>39.42</v>
       </c>
       <c r="O13" t="n">
-        <v>38.96</v>
+        <v>43.35</v>
       </c>
       <c r="P13" t="n">
-        <v>37.33</v>
+        <v>39.18</v>
       </c>
       <c r="Q13" t="n">
-        <v>37.76</v>
+        <v>43.19</v>
       </c>
       <c r="R13" t="n">
-        <v>-6.3592</v>
+        <v>-30.5139</v>
       </c>
       <c r="S13" t="n">
-        <v>15.7116</v>
+        <v>-31.4584</v>
       </c>
       <c r="T13" t="n">
-        <v>16.9479</v>
+        <v>-18.6324</v>
       </c>
       <c r="U13" t="n">
-        <v>-1.5481</v>
+        <v>-14.2807</v>
       </c>
       <c r="V13" t="n">
-        <v>-0.953</v>
+        <v>-16.2463</v>
       </c>
       <c r="W13" t="n">
-        <v>1.8403</v>
+        <v>-13.6116</v>
       </c>
       <c r="X13" t="n">
-        <v>5.9063</v>
+        <v>31.5385</v>
       </c>
       <c r="Y13" t="n">
-        <v>-16.9329</v>
+        <v>32.3017</v>
       </c>
       <c r="Z13" t="n">
-        <v>-17.5911</v>
+        <v>8.056900000000001</v>
       </c>
       <c r="AA13" t="n">
-        <v>1.5327</v>
+        <v>14.3803</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.9086</v>
+        <v>17.0144</v>
       </c>
       <c r="AC13" t="n">
-        <v>-1.8456</v>
+        <v>13.4191</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>230.85</v>
+        <v>210.62</v>
       </c>
       <c r="C14" t="n">
-        <v>233.69</v>
+        <v>222.19</v>
       </c>
       <c r="D14" t="n">
-        <v>181.81</v>
+        <v>201.69</v>
       </c>
       <c r="E14" t="n">
-        <v>182.54</v>
+        <v>211.44</v>
       </c>
       <c r="F14" t="n">
-        <v>81.56999999999999</v>
+        <v>76.86</v>
       </c>
       <c r="G14" t="n">
-        <v>82.08</v>
+        <v>78.47</v>
       </c>
       <c r="H14" t="n">
-        <v>72.68000000000001</v>
+        <v>75.38</v>
       </c>
       <c r="I14" t="n">
-        <v>73.05</v>
+        <v>76.27</v>
       </c>
       <c r="J14" t="n">
-        <v>5.86</v>
+        <v>5.71</v>
       </c>
       <c r="K14" t="n">
-        <v>6.85</v>
+        <v>6.05</v>
       </c>
       <c r="L14" t="n">
-        <v>5.79</v>
+        <v>5.27</v>
       </c>
       <c r="M14" t="n">
-        <v>6.84</v>
+        <v>5.69</v>
       </c>
       <c r="N14" t="n">
-        <v>39.42</v>
+        <v>40.92</v>
       </c>
       <c r="O14" t="n">
-        <v>43.35</v>
+        <v>41.78</v>
       </c>
       <c r="P14" t="n">
-        <v>39.18</v>
+        <v>39.96</v>
       </c>
       <c r="Q14" t="n">
-        <v>43.19</v>
+        <v>41.26</v>
       </c>
       <c r="R14" t="n">
-        <v>-30.5139</v>
+        <v>15.8321</v>
       </c>
       <c r="S14" t="n">
-        <v>-31.4584</v>
+        <v>-24.6311</v>
       </c>
       <c r="T14" t="n">
-        <v>-18.6324</v>
+        <v>-6.8669</v>
       </c>
       <c r="U14" t="n">
-        <v>-14.2807</v>
+        <v>4.4079</v>
       </c>
       <c r="V14" t="n">
-        <v>-16.2463</v>
+        <v>-11.8877</v>
       </c>
       <c r="W14" t="n">
-        <v>-13.6116</v>
+        <v>-11.3552</v>
       </c>
       <c r="X14" t="n">
-        <v>31.5385</v>
+        <v>-16.8129</v>
       </c>
       <c r="Y14" t="n">
-        <v>32.3017</v>
+        <v>15.8859</v>
       </c>
       <c r="Z14" t="n">
-        <v>8.056900000000001</v>
+        <v>-9.105399999999999</v>
       </c>
       <c r="AA14" t="n">
-        <v>14.3803</v>
+        <v>-4.4686</v>
       </c>
       <c r="AB14" t="n">
-        <v>17.0144</v>
+        <v>10.9438</v>
       </c>
       <c r="AC14" t="n">
-        <v>13.4191</v>
+        <v>10.2619</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>210.62</v>
+        <v>227.06</v>
       </c>
       <c r="C15" t="n">
-        <v>222.19</v>
+        <v>231.02</v>
       </c>
       <c r="D15" t="n">
-        <v>201.69</v>
+        <v>157.56</v>
       </c>
       <c r="E15" t="n">
-        <v>211.44</v>
+        <v>201.68</v>
       </c>
       <c r="F15" t="n">
-        <v>76.86</v>
+        <v>78.48</v>
       </c>
       <c r="G15" t="n">
-        <v>78.47</v>
+        <v>79.34</v>
       </c>
       <c r="H15" t="n">
-        <v>75.38</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="I15" t="n">
-        <v>76.27</v>
+        <v>73.72</v>
       </c>
       <c r="J15" t="n">
-        <v>5.71</v>
+        <v>5.25</v>
       </c>
       <c r="K15" t="n">
-        <v>6.05</v>
+        <v>7.11</v>
       </c>
       <c r="L15" t="n">
-        <v>5.27</v>
+        <v>5.14</v>
       </c>
       <c r="M15" t="n">
-        <v>5.69</v>
+        <v>5.93</v>
       </c>
       <c r="N15" t="n">
-        <v>40.92</v>
+        <v>40.06</v>
       </c>
       <c r="O15" t="n">
-        <v>41.78</v>
+        <v>46.38</v>
       </c>
       <c r="P15" t="n">
-        <v>39.96</v>
+        <v>39.59</v>
       </c>
       <c r="Q15" t="n">
-        <v>41.26</v>
+        <v>42.67</v>
       </c>
       <c r="R15" t="n">
-        <v>15.8321</v>
+        <v>-4.616</v>
       </c>
       <c r="S15" t="n">
-        <v>-24.6311</v>
+        <v>-23.228</v>
       </c>
       <c r="T15" t="n">
-        <v>-6.8669</v>
+        <v>-24.2716</v>
       </c>
       <c r="U15" t="n">
-        <v>4.4079</v>
+        <v>-3.3434</v>
       </c>
       <c r="V15" t="n">
-        <v>-11.8877</v>
+        <v>-13.4945</v>
       </c>
       <c r="W15" t="n">
-        <v>-11.3552</v>
+        <v>-15.4781</v>
       </c>
       <c r="X15" t="n">
-        <v>-16.8129</v>
+        <v>4.2179</v>
       </c>
       <c r="Y15" t="n">
-        <v>15.8859</v>
+        <v>14.0385</v>
       </c>
       <c r="Z15" t="n">
-        <v>-9.105399999999999</v>
+        <v>14.7002</v>
       </c>
       <c r="AA15" t="n">
-        <v>-4.4686</v>
+        <v>3.4174</v>
       </c>
       <c r="AB15" t="n">
-        <v>10.9438</v>
+        <v>13.0032</v>
       </c>
       <c r="AC15" t="n">
-        <v>10.2619</v>
+        <v>15.6055</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>227.06</v>
+        <v>191.54</v>
       </c>
       <c r="C16" t="n">
-        <v>231.02</v>
+        <v>212.99</v>
       </c>
       <c r="D16" t="n">
-        <v>157.56</v>
+        <v>177.3</v>
       </c>
       <c r="E16" t="n">
-        <v>201.68</v>
+        <v>180.65</v>
       </c>
       <c r="F16" t="n">
-        <v>78.48</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>79.34</v>
+        <v>74.7</v>
       </c>
       <c r="H16" t="n">
-        <v>66.79000000000001</v>
+        <v>69</v>
       </c>
       <c r="I16" t="n">
-        <v>73.72</v>
+        <v>69.27</v>
       </c>
       <c r="J16" t="n">
-        <v>5.25</v>
+        <v>6.24</v>
       </c>
       <c r="K16" t="n">
-        <v>7.11</v>
+        <v>6.65</v>
       </c>
       <c r="L16" t="n">
-        <v>5.14</v>
+        <v>5.6</v>
       </c>
       <c r="M16" t="n">
-        <v>5.93</v>
+        <v>6.57</v>
       </c>
       <c r="N16" t="n">
-        <v>40.06</v>
+        <v>43.81</v>
       </c>
       <c r="O16" t="n">
-        <v>46.38</v>
+        <v>45.39</v>
       </c>
       <c r="P16" t="n">
-        <v>39.59</v>
+        <v>42.07</v>
       </c>
       <c r="Q16" t="n">
-        <v>42.67</v>
+        <v>45.25</v>
       </c>
       <c r="R16" t="n">
-        <v>-4.616</v>
+        <v>-10.4274</v>
       </c>
       <c r="S16" t="n">
-        <v>-23.228</v>
+        <v>-1.0354</v>
       </c>
       <c r="T16" t="n">
-        <v>-24.2716</v>
+        <v>-35.6063</v>
       </c>
       <c r="U16" t="n">
-        <v>-3.3434</v>
+        <v>-6.0364</v>
       </c>
       <c r="V16" t="n">
-        <v>-13.4945</v>
+        <v>-5.1745</v>
       </c>
       <c r="W16" t="n">
-        <v>-15.4781</v>
+        <v>-19.9746</v>
       </c>
       <c r="X16" t="n">
-        <v>4.2179</v>
+        <v>10.7926</v>
       </c>
       <c r="Y16" t="n">
-        <v>14.0385</v>
+        <v>-3.9474</v>
       </c>
       <c r="Z16" t="n">
-        <v>14.7002</v>
+        <v>33.8086</v>
       </c>
       <c r="AA16" t="n">
-        <v>3.4174</v>
+        <v>6.0464</v>
       </c>
       <c r="AB16" t="n">
-        <v>13.0032</v>
+        <v>4.7696</v>
       </c>
       <c r="AC16" t="n">
-        <v>15.6055</v>
+        <v>21.6725</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>191.54</v>
+        <v>192.3</v>
       </c>
       <c r="C17" t="n">
-        <v>212.99</v>
+        <v>225.63</v>
       </c>
       <c r="D17" t="n">
-        <v>177.3</v>
+        <v>192.3</v>
       </c>
       <c r="E17" t="n">
-        <v>180.65</v>
+        <v>223.99</v>
       </c>
       <c r="F17" t="n">
-        <v>71.68000000000001</v>
+        <v>70.89</v>
       </c>
       <c r="G17" t="n">
-        <v>74.7</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="H17" t="n">
-        <v>69</v>
+        <v>69.59</v>
       </c>
       <c r="I17" t="n">
-        <v>69.27</v>
+        <v>76.01000000000001</v>
       </c>
       <c r="J17" t="n">
-        <v>6.24</v>
+        <v>6.1</v>
       </c>
       <c r="K17" t="n">
-        <v>6.65</v>
+        <v>6.1</v>
       </c>
       <c r="L17" t="n">
-        <v>5.6</v>
+        <v>4.9</v>
       </c>
       <c r="M17" t="n">
-        <v>6.57</v>
+        <v>4.97</v>
       </c>
       <c r="N17" t="n">
-        <v>43.81</v>
+        <v>44.18</v>
       </c>
       <c r="O17" t="n">
-        <v>45.39</v>
+        <v>45.01</v>
       </c>
       <c r="P17" t="n">
-        <v>42.07</v>
+        <v>40.44</v>
       </c>
       <c r="Q17" t="n">
-        <v>45.25</v>
+        <v>40.83</v>
       </c>
       <c r="R17" t="n">
-        <v>-10.4274</v>
+        <v>23.9911</v>
       </c>
       <c r="S17" t="n">
-        <v>-1.0354</v>
+        <v>5.9355</v>
       </c>
       <c r="T17" t="n">
-        <v>-35.6063</v>
+        <v>-14.7354</v>
       </c>
       <c r="U17" t="n">
-        <v>-6.0364</v>
+        <v>9.73</v>
       </c>
       <c r="V17" t="n">
-        <v>-5.1745</v>
+        <v>-0.3409</v>
       </c>
       <c r="W17" t="n">
-        <v>-19.9746</v>
+        <v>-10.8073</v>
       </c>
       <c r="X17" t="n">
-        <v>10.7926</v>
+        <v>-24.3531</v>
       </c>
       <c r="Y17" t="n">
-        <v>-3.9474</v>
+        <v>-12.6538</v>
       </c>
       <c r="Z17" t="n">
-        <v>33.8086</v>
+        <v>-4.4231</v>
       </c>
       <c r="AA17" t="n">
-        <v>6.0464</v>
+        <v>-9.768000000000001</v>
       </c>
       <c r="AB17" t="n">
-        <v>4.7696</v>
+        <v>-1.0422</v>
       </c>
       <c r="AC17" t="n">
-        <v>21.6725</v>
+        <v>8.1303</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>192.3</v>
+        <v>222.22</v>
       </c>
       <c r="C18" t="n">
-        <v>225.63</v>
+        <v>242.4</v>
       </c>
       <c r="D18" t="n">
-        <v>192.3</v>
+        <v>214.74</v>
       </c>
       <c r="E18" t="n">
-        <v>223.99</v>
+        <v>234.68</v>
       </c>
       <c r="F18" t="n">
-        <v>70.89</v>
+        <v>76.34</v>
       </c>
       <c r="G18" t="n">
-        <v>76.59999999999999</v>
+        <v>78.36</v>
       </c>
       <c r="H18" t="n">
-        <v>69.59</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="I18" t="n">
-        <v>76.01000000000001</v>
+        <v>77.52</v>
       </c>
       <c r="J18" t="n">
-        <v>6.1</v>
+        <v>5.01</v>
       </c>
       <c r="K18" t="n">
-        <v>6.1</v>
+        <v>5.15</v>
       </c>
       <c r="L18" t="n">
-        <v>4.9</v>
+        <v>4.54</v>
       </c>
       <c r="M18" t="n">
-        <v>4.97</v>
+        <v>4.72</v>
       </c>
       <c r="N18" t="n">
-        <v>44.18</v>
+        <v>40.65</v>
       </c>
       <c r="O18" t="n">
-        <v>45.01</v>
+        <v>41.75</v>
       </c>
       <c r="P18" t="n">
-        <v>40.44</v>
+        <v>39.57</v>
       </c>
       <c r="Q18" t="n">
-        <v>40.83</v>
+        <v>40.04</v>
       </c>
       <c r="R18" t="n">
-        <v>23.9911</v>
+        <v>4.7725</v>
       </c>
       <c r="S18" t="n">
-        <v>5.9355</v>
+        <v>16.3626</v>
       </c>
       <c r="T18" t="n">
-        <v>-14.7354</v>
+        <v>28.5636</v>
       </c>
       <c r="U18" t="n">
-        <v>9.73</v>
+        <v>1.9866</v>
       </c>
       <c r="V18" t="n">
-        <v>-0.3409</v>
+        <v>5.1546</v>
       </c>
       <c r="W18" t="n">
-        <v>-10.8073</v>
+        <v>6.1191</v>
       </c>
       <c r="X18" t="n">
-        <v>-24.3531</v>
+        <v>-5.0302</v>
       </c>
       <c r="Y18" t="n">
-        <v>-12.6538</v>
+        <v>-20.4047</v>
       </c>
       <c r="Z18" t="n">
-        <v>-4.4231</v>
+        <v>-30.9942</v>
       </c>
       <c r="AA18" t="n">
-        <v>-9.768000000000001</v>
+        <v>-1.9349</v>
       </c>
       <c r="AB18" t="n">
-        <v>-1.0422</v>
+        <v>-6.1636</v>
       </c>
       <c r="AC18" t="n">
-        <v>8.1303</v>
+        <v>-7.2934</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>222.22</v>
+        <v>265.99</v>
       </c>
       <c r="C19" t="n">
-        <v>242.4</v>
+        <v>274.88</v>
       </c>
       <c r="D19" t="n">
-        <v>214.74</v>
+        <v>261.6</v>
       </c>
       <c r="E19" t="n">
-        <v>234.68</v>
+        <v>272.5</v>
       </c>
       <c r="F19" t="n">
-        <v>76.34</v>
+        <v>82.88</v>
       </c>
       <c r="G19" t="n">
-        <v>78.36</v>
+        <v>85.03</v>
       </c>
       <c r="H19" t="n">
-        <v>74.29000000000001</v>
+        <v>82.64</v>
       </c>
       <c r="I19" t="n">
-        <v>77.52</v>
+        <v>84.59</v>
       </c>
       <c r="J19" t="n">
-        <v>5.01</v>
+        <v>4.07</v>
       </c>
       <c r="K19" t="n">
-        <v>5.15</v>
+        <v>4.17</v>
       </c>
       <c r="L19" t="n">
-        <v>4.54</v>
+        <v>3.91</v>
       </c>
       <c r="M19" t="n">
-        <v>4.72</v>
+        <v>3.95</v>
       </c>
       <c r="N19" t="n">
-        <v>40.65</v>
+        <v>37.25</v>
       </c>
       <c r="O19" t="n">
-        <v>41.75</v>
+        <v>37.36</v>
       </c>
       <c r="P19" t="n">
-        <v>39.57</v>
+        <v>36.15</v>
       </c>
       <c r="Q19" t="n">
-        <v>40.04</v>
+        <v>36.31</v>
       </c>
       <c r="R19" t="n">
-        <v>4.7725</v>
+        <v>16.1156</v>
       </c>
       <c r="S19" t="n">
-        <v>16.3626</v>
+        <v>50.8442</v>
       </c>
       <c r="T19" t="n">
-        <v>28.5636</v>
+        <v>28.8782</v>
       </c>
       <c r="U19" t="n">
-        <v>1.9866</v>
+        <v>9.120200000000001</v>
       </c>
       <c r="V19" t="n">
-        <v>5.1546</v>
+        <v>22.1164</v>
       </c>
       <c r="W19" t="n">
-        <v>6.1191</v>
+        <v>10.9086</v>
       </c>
       <c r="X19" t="n">
-        <v>-5.0302</v>
+        <v>-16.3136</v>
       </c>
       <c r="Y19" t="n">
-        <v>-20.4047</v>
+        <v>-39.8782</v>
       </c>
       <c r="Z19" t="n">
-        <v>-30.9942</v>
+        <v>-30.58</v>
       </c>
       <c r="AA19" t="n">
-        <v>-1.9349</v>
+        <v>-9.3157</v>
       </c>
       <c r="AB19" t="n">
-        <v>-6.1636</v>
+        <v>-19.7569</v>
       </c>
       <c r="AC19" t="n">
-        <v>-7.2934</v>
+        <v>-11.9971</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>265.99</v>
+        <v>267.13</v>
       </c>
       <c r="C20" t="n">
-        <v>274.88</v>
+        <v>274.93</v>
       </c>
       <c r="D20" t="n">
-        <v>261.6</v>
+        <v>226</v>
       </c>
       <c r="E20" t="n">
-        <v>272.5</v>
+        <v>226.19</v>
       </c>
       <c r="F20" t="n">
-        <v>82.88</v>
+        <v>84.19</v>
       </c>
       <c r="G20" t="n">
-        <v>85.03</v>
+        <v>84.83</v>
       </c>
       <c r="H20" t="n">
-        <v>82.64</v>
+        <v>79.86</v>
       </c>
       <c r="I20" t="n">
-        <v>84.59</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="J20" t="n">
-        <v>4.07</v>
+        <v>4.03</v>
       </c>
       <c r="K20" t="n">
-        <v>4.17</v>
+        <v>4.65</v>
       </c>
       <c r="L20" t="n">
         <v>3.91</v>
       </c>
       <c r="M20" t="n">
-        <v>3.95</v>
+        <v>4.63</v>
       </c>
       <c r="N20" t="n">
-        <v>37.25</v>
+        <v>36.54</v>
       </c>
       <c r="O20" t="n">
-        <v>37.36</v>
+        <v>38.39</v>
       </c>
       <c r="P20" t="n">
-        <v>36.15</v>
+        <v>36.26</v>
       </c>
       <c r="Q20" t="n">
-        <v>36.31</v>
+        <v>38.35</v>
       </c>
       <c r="R20" t="n">
-        <v>16.1156</v>
+        <v>-16.9945</v>
       </c>
       <c r="S20" t="n">
-        <v>50.8442</v>
+        <v>0.9822</v>
       </c>
       <c r="T20" t="n">
-        <v>28.8782</v>
+        <v>12.1529</v>
       </c>
       <c r="U20" t="n">
-        <v>9.120200000000001</v>
+        <v>-5.5089</v>
       </c>
       <c r="V20" t="n">
-        <v>22.1164</v>
+        <v>5.1572</v>
       </c>
       <c r="W20" t="n">
-        <v>10.9086</v>
+        <v>8.4238</v>
       </c>
       <c r="X20" t="n">
-        <v>-16.3136</v>
+        <v>17.2152</v>
       </c>
       <c r="Y20" t="n">
-        <v>-39.8782</v>
+        <v>-6.841</v>
       </c>
       <c r="Z20" t="n">
-        <v>-30.58</v>
+        <v>-21.9224</v>
       </c>
       <c r="AA20" t="n">
-        <v>-9.3157</v>
+        <v>5.6183</v>
       </c>
       <c r="AB20" t="n">
-        <v>-19.7569</v>
+        <v>-6.074</v>
       </c>
       <c r="AC20" t="n">
-        <v>-11.9971</v>
+        <v>-10.1242</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>267.13</v>
+        <v>247.42</v>
       </c>
       <c r="C21" t="n">
-        <v>274.93</v>
+        <v>259.79</v>
       </c>
       <c r="D21" t="n">
-        <v>226</v>
+        <v>233.3</v>
       </c>
       <c r="E21" t="n">
-        <v>226.19</v>
+        <v>233.86</v>
       </c>
       <c r="F21" t="n">
-        <v>84.19</v>
+        <v>81.67</v>
       </c>
       <c r="G21" t="n">
-        <v>84.83</v>
+        <v>81.81</v>
       </c>
       <c r="H21" t="n">
-        <v>79.86</v>
+        <v>76.94</v>
       </c>
       <c r="I21" t="n">
-        <v>79.93000000000001</v>
+        <v>77.54000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>4.03</v>
+        <v>4.17</v>
       </c>
       <c r="K21" t="n">
-        <v>4.65</v>
+        <v>4.46</v>
       </c>
       <c r="L21" t="n">
-        <v>3.91</v>
+        <v>3.92</v>
       </c>
       <c r="M21" t="n">
-        <v>4.63</v>
+        <v>4.46</v>
       </c>
       <c r="N21" t="n">
-        <v>36.54</v>
+        <v>37.53</v>
       </c>
       <c r="O21" t="n">
-        <v>38.39</v>
+        <v>39.79</v>
       </c>
       <c r="P21" t="n">
-        <v>36.26</v>
+        <v>37.46</v>
       </c>
       <c r="Q21" t="n">
-        <v>38.35</v>
+        <v>39.52</v>
       </c>
       <c r="R21" t="n">
-        <v>-16.9945</v>
+        <v>3.391</v>
       </c>
       <c r="S21" t="n">
-        <v>0.9822</v>
+        <v>-0.3494</v>
       </c>
       <c r="T21" t="n">
-        <v>12.1529</v>
+        <v>29.4547</v>
       </c>
       <c r="U21" t="n">
-        <v>-5.5089</v>
+        <v>-2.9901</v>
       </c>
       <c r="V21" t="n">
-        <v>5.1572</v>
+        <v>0.0258</v>
       </c>
       <c r="W21" t="n">
-        <v>8.4238</v>
+        <v>11.9388</v>
       </c>
       <c r="X21" t="n">
-        <v>17.2152</v>
+        <v>-3.6717</v>
       </c>
       <c r="Y21" t="n">
-        <v>-6.841</v>
+        <v>-5.5085</v>
       </c>
       <c r="Z21" t="n">
-        <v>-21.9224</v>
+        <v>-32.1157</v>
       </c>
       <c r="AA21" t="n">
-        <v>5.6183</v>
+        <v>3.0508</v>
       </c>
       <c r="AB21" t="n">
-        <v>-6.074</v>
+        <v>-1.2987</v>
       </c>
       <c r="AC21" t="n">
-        <v>-10.1242</v>
+        <v>-12.663</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>247.42</v>
+        <v>266.035</v>
       </c>
       <c r="C22" t="n">
-        <v>259.79</v>
+        <v>286.1526</v>
       </c>
       <c r="D22" t="n">
-        <v>233.455</v>
+        <v>265</v>
       </c>
       <c r="E22" t="n">
-        <v>233.86</v>
+        <v>279.29</v>
       </c>
       <c r="F22" t="n">
-        <v>81.65000000000001</v>
+        <v>82.09</v>
       </c>
       <c r="G22" t="n">
-        <v>81.80500000000001</v>
+        <v>83.59990000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>76.94</v>
+        <v>80.63</v>
       </c>
       <c r="I22" t="n">
-        <v>77.54000000000001</v>
+        <v>82.87</v>
       </c>
       <c r="J22" t="n">
-        <v>4.17</v>
+        <v>3.855</v>
       </c>
       <c r="K22" t="n">
-        <v>4.45</v>
+        <v>3.865</v>
       </c>
       <c r="L22" t="n">
-        <v>3.92</v>
+        <v>3.45</v>
       </c>
       <c r="M22" t="n">
-        <v>4.46</v>
+        <v>3.59</v>
       </c>
       <c r="N22" t="n">
-        <v>37.54</v>
+        <v>37.2</v>
       </c>
       <c r="O22" t="n">
-        <v>39.79</v>
+        <v>37.95</v>
       </c>
       <c r="P22" t="n">
-        <v>37.46</v>
+        <v>36.4301</v>
       </c>
       <c r="Q22" t="n">
-        <v>39.52</v>
+        <v>36.75</v>
       </c>
       <c r="R22" t="n">
-        <v>3.391</v>
+        <v>19.4262</v>
       </c>
       <c r="S22" t="n">
-        <v>-0.3494</v>
+        <v>2.4917</v>
       </c>
       <c r="T22" t="n">
-        <v>29.4547</v>
+        <v>24.6886</v>
       </c>
       <c r="U22" t="n">
-        <v>-2.9901</v>
+        <v>6.8739</v>
       </c>
       <c r="V22" t="n">
-        <v>0.0258</v>
+        <v>-2.0333</v>
       </c>
       <c r="W22" t="n">
-        <v>11.9388</v>
+        <v>9.0251</v>
       </c>
       <c r="X22" t="n">
-        <v>-3.6717</v>
+        <v>-19.5067</v>
       </c>
       <c r="Y22" t="n">
-        <v>-5.5085</v>
+        <v>-9.113899999999999</v>
       </c>
       <c r="Z22" t="n">
-        <v>-32.1157</v>
+        <v>-27.7666</v>
       </c>
       <c r="AA22" t="n">
-        <v>3.0508</v>
+        <v>-7.0091</v>
       </c>
       <c r="AB22" t="n">
-        <v>-1.2987</v>
+        <v>1.2118</v>
       </c>
       <c r="AC22" t="n">
-        <v>-12.663</v>
+        <v>-9.992699999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-19 22:58
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC22"/>
+  <dimension ref="A1:AC21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1803 +568,1712 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>161</v>
+        <v>171.26</v>
       </c>
       <c r="C2" t="n">
-        <v>173.7</v>
+        <v>179.97</v>
       </c>
       <c r="D2" t="n">
-        <v>161</v>
+        <v>168.23</v>
       </c>
       <c r="E2" t="n">
-        <v>173.2</v>
+        <v>178.39</v>
       </c>
       <c r="F2" t="n">
-        <v>74.09</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>76.53</v>
+        <v>77.79000000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>73.62</v>
+        <v>74.47</v>
       </c>
       <c r="I2" t="n">
-        <v>76.51000000000001</v>
+        <v>76.95</v>
       </c>
       <c r="J2" t="n">
-        <v>9.300000000000001</v>
+        <v>8.65</v>
       </c>
       <c r="K2" t="n">
-        <v>9.35</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="L2" t="n">
-        <v>8.51</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="M2" t="n">
-        <v>8.539999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N2" t="n">
-        <v>43.67</v>
+        <v>42.94</v>
       </c>
       <c r="O2" t="n">
-        <v>43.97</v>
+        <v>43.33</v>
       </c>
       <c r="P2" t="n">
-        <v>42.19</v>
+        <v>41.5</v>
       </c>
       <c r="Q2" t="n">
-        <v>42.19</v>
+        <v>41.96</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>171.26</v>
+        <v>184.8</v>
       </c>
       <c r="C3" t="n">
-        <v>179.97</v>
+        <v>195.27</v>
       </c>
       <c r="D3" t="n">
-        <v>168.23</v>
+        <v>183.34</v>
       </c>
       <c r="E3" t="n">
-        <v>178.39</v>
+        <v>190.56</v>
       </c>
       <c r="F3" t="n">
-        <v>75.18000000000001</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>77.79000000000001</v>
+        <v>79.33</v>
       </c>
       <c r="H3" t="n">
-        <v>74.47</v>
+        <v>77.33</v>
       </c>
       <c r="I3" t="n">
-        <v>76.95</v>
+        <v>77.84</v>
       </c>
       <c r="J3" t="n">
-        <v>8.65</v>
+        <v>8</v>
       </c>
       <c r="K3" t="n">
-        <v>8.779999999999999</v>
+        <v>8.06</v>
       </c>
       <c r="L3" t="n">
-        <v>8.210000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="M3" t="n">
-        <v>8.289999999999999</v>
+        <v>7.73</v>
       </c>
       <c r="N3" t="n">
-        <v>42.94</v>
+        <v>41.4</v>
       </c>
       <c r="O3" t="n">
-        <v>43.33</v>
+        <v>41.78</v>
       </c>
       <c r="P3" t="n">
+        <v>40.68</v>
+      </c>
+      <c r="Q3" t="n">
         <v>41.5</v>
       </c>
-      <c r="Q3" t="n">
-        <v>41.96</v>
-      </c>
       <c r="R3" t="n">
-        <v>2.9965</v>
+        <v>6.8221</v>
       </c>
       <c r="U3" t="n">
-        <v>0.5750999999999999</v>
+        <v>1.1566</v>
       </c>
       <c r="X3" t="n">
-        <v>-2.9274</v>
+        <v>-6.7551</v>
       </c>
       <c r="AA3" t="n">
-        <v>-0.5452</v>
+        <v>-1.0963</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>184.8</v>
+        <v>211.38</v>
       </c>
       <c r="C4" t="n">
-        <v>195.27</v>
+        <v>228.5</v>
       </c>
       <c r="D4" t="n">
-        <v>183.34</v>
+        <v>209.89</v>
       </c>
       <c r="E4" t="n">
-        <v>190.56</v>
+        <v>225.79</v>
       </c>
       <c r="F4" t="n">
-        <v>78.04000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="G4" t="n">
-        <v>79.33</v>
+        <v>82.27</v>
       </c>
       <c r="H4" t="n">
-        <v>77.33</v>
+        <v>79.98</v>
       </c>
       <c r="I4" t="n">
-        <v>77.84</v>
+        <v>81.95</v>
       </c>
       <c r="J4" t="n">
-        <v>8</v>
+        <v>6.9</v>
       </c>
       <c r="K4" t="n">
-        <v>8.06</v>
+        <v>6.95</v>
       </c>
       <c r="L4" t="n">
-        <v>7.5</v>
+        <v>6.19</v>
       </c>
       <c r="M4" t="n">
-        <v>7.73</v>
+        <v>6.29</v>
       </c>
       <c r="N4" t="n">
-        <v>41.4</v>
+        <v>40.05</v>
       </c>
       <c r="O4" t="n">
-        <v>41.78</v>
+        <v>40.35</v>
       </c>
       <c r="P4" t="n">
-        <v>40.68</v>
+        <v>39.14</v>
       </c>
       <c r="Q4" t="n">
-        <v>41.5</v>
+        <v>39.28</v>
       </c>
       <c r="R4" t="n">
-        <v>6.8221</v>
+        <v>18.4876</v>
       </c>
       <c r="U4" t="n">
-        <v>1.1566</v>
+        <v>5.2801</v>
       </c>
       <c r="X4" t="n">
-        <v>-6.7551</v>
+        <v>-18.6287</v>
       </c>
       <c r="AA4" t="n">
-        <v>-1.0963</v>
+        <v>-5.3494</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>211.38</v>
+        <v>242.66</v>
       </c>
       <c r="C5" t="n">
-        <v>228.5</v>
+        <v>242.66</v>
       </c>
       <c r="D5" t="n">
-        <v>209.89</v>
+        <v>204</v>
       </c>
       <c r="E5" t="n">
-        <v>225.79</v>
+        <v>217.98</v>
       </c>
       <c r="F5" t="n">
-        <v>80.59</v>
+        <v>82.87</v>
       </c>
       <c r="G5" t="n">
-        <v>82.27</v>
+        <v>82.91</v>
       </c>
       <c r="H5" t="n">
-        <v>79.98</v>
+        <v>80.33</v>
       </c>
       <c r="I5" t="n">
-        <v>81.95</v>
+        <v>81.67</v>
       </c>
       <c r="J5" t="n">
-        <v>6.9</v>
+        <v>5.83</v>
       </c>
       <c r="K5" t="n">
-        <v>6.95</v>
+        <v>6.91</v>
       </c>
       <c r="L5" t="n">
-        <v>6.19</v>
+        <v>5.83</v>
       </c>
       <c r="M5" t="n">
-        <v>6.29</v>
+        <v>6.53</v>
       </c>
       <c r="N5" t="n">
-        <v>40.05</v>
+        <v>38.87</v>
       </c>
       <c r="O5" t="n">
-        <v>40.35</v>
+        <v>40.09</v>
       </c>
       <c r="P5" t="n">
-        <v>39.14</v>
+        <v>38.86</v>
       </c>
       <c r="Q5" t="n">
-        <v>39.28</v>
+        <v>39.44</v>
       </c>
       <c r="R5" t="n">
-        <v>18.4876</v>
+        <v>-3.459</v>
       </c>
       <c r="S5" t="n">
-        <v>30.3637</v>
+        <v>22.1929</v>
       </c>
       <c r="U5" t="n">
-        <v>5.2801</v>
+        <v>-0.3417</v>
       </c>
       <c r="V5" t="n">
-        <v>7.1102</v>
+        <v>6.1339</v>
       </c>
       <c r="X5" t="n">
-        <v>-18.6287</v>
+        <v>3.8156</v>
       </c>
       <c r="Y5" t="n">
-        <v>-26.3466</v>
+        <v>-21.2304</v>
       </c>
       <c r="AA5" t="n">
-        <v>-5.3494</v>
+        <v>0.4073</v>
       </c>
       <c r="AB5" t="n">
-        <v>-6.8974</v>
+        <v>-6.0057</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>242.66</v>
+        <v>219</v>
       </c>
       <c r="C6" t="n">
-        <v>242.66</v>
+        <v>231.89</v>
       </c>
       <c r="D6" t="n">
-        <v>204</v>
+        <v>207.56</v>
       </c>
       <c r="E6" t="n">
-        <v>217.98</v>
+        <v>224.63</v>
       </c>
       <c r="F6" t="n">
-        <v>82.87</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>82.91</v>
+        <v>84.05</v>
       </c>
       <c r="H6" t="n">
-        <v>80.33</v>
+        <v>80.66</v>
       </c>
       <c r="I6" t="n">
-        <v>81.67</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>5.83</v>
+        <v>6.49</v>
       </c>
       <c r="K6" t="n">
-        <v>6.91</v>
+        <v>6.83</v>
       </c>
       <c r="L6" t="n">
-        <v>5.83</v>
+        <v>6.1</v>
       </c>
       <c r="M6" t="n">
-        <v>6.53</v>
+        <v>6.31</v>
       </c>
       <c r="N6" t="n">
-        <v>38.87</v>
+        <v>39.41</v>
       </c>
       <c r="O6" t="n">
-        <v>40.09</v>
+        <v>39.94</v>
       </c>
       <c r="P6" t="n">
-        <v>38.86</v>
+        <v>38.3</v>
       </c>
       <c r="Q6" t="n">
-        <v>39.44</v>
+        <v>38.47</v>
       </c>
       <c r="R6" t="n">
-        <v>-3.459</v>
+        <v>3.0507</v>
       </c>
       <c r="S6" t="n">
-        <v>22.1929</v>
+        <v>17.8789</v>
       </c>
       <c r="U6" t="n">
-        <v>-0.3417</v>
+        <v>2.4611</v>
       </c>
       <c r="V6" t="n">
-        <v>6.1339</v>
+        <v>7.5026</v>
       </c>
       <c r="X6" t="n">
-        <v>3.8156</v>
+        <v>-3.3691</v>
       </c>
       <c r="Y6" t="n">
-        <v>-21.2304</v>
+        <v>-18.37</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.4073</v>
+        <v>-2.4594</v>
       </c>
       <c r="AB6" t="n">
-        <v>-6.0057</v>
+        <v>-7.3012</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>219</v>
+        <v>231.82</v>
       </c>
       <c r="C7" t="n">
-        <v>231.89</v>
+        <v>239.07</v>
       </c>
       <c r="D7" t="n">
-        <v>207.56</v>
+        <v>218.56</v>
       </c>
       <c r="E7" t="n">
-        <v>224.63</v>
+        <v>224.34</v>
       </c>
       <c r="F7" t="n">
-        <v>81.73999999999999</v>
+        <v>84.41</v>
       </c>
       <c r="G7" t="n">
-        <v>84.05</v>
+        <v>85.7</v>
       </c>
       <c r="H7" t="n">
-        <v>80.66</v>
+        <v>83.53</v>
       </c>
       <c r="I7" t="n">
-        <v>83.68000000000001</v>
+        <v>84.56</v>
       </c>
       <c r="J7" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="K7" t="n">
         <v>6.49</v>
       </c>
-      <c r="K7" t="n">
-        <v>6.83</v>
-      </c>
       <c r="L7" t="n">
-        <v>6.1</v>
+        <v>5.91</v>
       </c>
       <c r="M7" t="n">
-        <v>6.31</v>
+        <v>6.33</v>
       </c>
       <c r="N7" t="n">
-        <v>39.41</v>
+        <v>38.15</v>
       </c>
       <c r="O7" t="n">
-        <v>39.94</v>
+        <v>38.56</v>
       </c>
       <c r="P7" t="n">
-        <v>38.3</v>
+        <v>37.56</v>
       </c>
       <c r="Q7" t="n">
-        <v>38.47</v>
+        <v>38.08</v>
       </c>
       <c r="R7" t="n">
-        <v>3.0507</v>
+        <v>-0.1291</v>
       </c>
       <c r="S7" t="n">
-        <v>17.8789</v>
+        <v>-0.6422</v>
       </c>
       <c r="T7" t="n">
-        <v>29.694</v>
+        <v>25.7582</v>
       </c>
       <c r="U7" t="n">
-        <v>2.4611</v>
+        <v>1.0516</v>
       </c>
       <c r="V7" t="n">
-        <v>7.5026</v>
+        <v>3.1849</v>
       </c>
       <c r="W7" t="n">
-        <v>9.3713</v>
+        <v>9.8895</v>
       </c>
       <c r="X7" t="n">
-        <v>-3.3691</v>
+        <v>0.317</v>
       </c>
       <c r="Y7" t="n">
-        <v>-18.37</v>
+        <v>0.6359</v>
       </c>
       <c r="Z7" t="n">
-        <v>-26.1124</v>
+        <v>-23.6429</v>
       </c>
       <c r="AA7" t="n">
-        <v>-2.4594</v>
+        <v>-1.0138</v>
       </c>
       <c r="AB7" t="n">
-        <v>-7.3012</v>
+        <v>-3.055</v>
       </c>
       <c r="AC7" t="n">
-        <v>-8.817299999999999</v>
+        <v>-9.2469</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>231.82</v>
+        <v>217.27</v>
       </c>
       <c r="C8" t="n">
-        <v>239.07</v>
+        <v>234.06</v>
       </c>
       <c r="D8" t="n">
-        <v>218.56</v>
+        <v>210.14</v>
       </c>
       <c r="E8" t="n">
-        <v>224.34</v>
+        <v>227.03</v>
       </c>
       <c r="F8" t="n">
-        <v>84.41</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>85.7</v>
+        <v>87.06</v>
       </c>
       <c r="H8" t="n">
-        <v>83.53</v>
+        <v>83.75</v>
       </c>
       <c r="I8" t="n">
-        <v>84.56</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>6.11</v>
+        <v>6.55</v>
       </c>
       <c r="K8" t="n">
-        <v>6.49</v>
+        <v>6.74</v>
       </c>
       <c r="L8" t="n">
-        <v>5.91</v>
+        <v>6.05</v>
       </c>
       <c r="M8" t="n">
-        <v>6.33</v>
+        <v>6.26</v>
       </c>
       <c r="N8" t="n">
-        <v>38.15</v>
+        <v>38.27</v>
       </c>
       <c r="O8" t="n">
-        <v>38.56</v>
+        <v>38.46</v>
       </c>
       <c r="P8" t="n">
-        <v>37.56</v>
+        <v>36.96</v>
       </c>
       <c r="Q8" t="n">
-        <v>38.08</v>
+        <v>37.42</v>
       </c>
       <c r="R8" t="n">
-        <v>-0.1291</v>
+        <v>1.1991</v>
       </c>
       <c r="S8" t="n">
-        <v>-0.6422</v>
+        <v>4.1518</v>
       </c>
       <c r="T8" t="n">
-        <v>25.7582</v>
+        <v>19.1383</v>
       </c>
       <c r="U8" t="n">
-        <v>1.0516</v>
+        <v>1.7502</v>
       </c>
       <c r="V8" t="n">
-        <v>3.1849</v>
+        <v>5.3508</v>
       </c>
       <c r="W8" t="n">
-        <v>9.8895</v>
+        <v>10.5344</v>
       </c>
       <c r="X8" t="n">
-        <v>0.317</v>
+        <v>-1.1058</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.6359</v>
+        <v>-4.1348</v>
       </c>
       <c r="Z8" t="n">
-        <v>-23.6429</v>
+        <v>-19.0168</v>
       </c>
       <c r="AA8" t="n">
-        <v>-1.0138</v>
+        <v>-1.7332</v>
       </c>
       <c r="AB8" t="n">
-        <v>-3.055</v>
+        <v>-5.1217</v>
       </c>
       <c r="AC8" t="n">
-        <v>-9.2469</v>
+        <v>-9.831300000000001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>217.27</v>
+        <v>243.18</v>
       </c>
       <c r="C9" t="n">
-        <v>234.06</v>
+        <v>267.08</v>
       </c>
       <c r="D9" t="n">
-        <v>210.14</v>
+        <v>238.82</v>
       </c>
       <c r="E9" t="n">
-        <v>227.03</v>
+        <v>266.32</v>
       </c>
       <c r="F9" t="n">
-        <v>84.15000000000001</v>
+        <v>85.94</v>
       </c>
       <c r="G9" t="n">
-        <v>87.06</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>83.75</v>
+        <v>84.83</v>
       </c>
       <c r="I9" t="n">
-        <v>86.04000000000001</v>
+        <v>87.22</v>
       </c>
       <c r="J9" t="n">
-        <v>6.55</v>
+        <v>5.8</v>
       </c>
       <c r="K9" t="n">
-        <v>6.74</v>
+        <v>5.93</v>
       </c>
       <c r="L9" t="n">
-        <v>6.05</v>
+        <v>5.15</v>
       </c>
       <c r="M9" t="n">
-        <v>6.26</v>
+        <v>5.17</v>
       </c>
       <c r="N9" t="n">
-        <v>38.27</v>
+        <v>37.47</v>
       </c>
       <c r="O9" t="n">
-        <v>38.46</v>
+        <v>37.95</v>
       </c>
       <c r="P9" t="n">
-        <v>36.96</v>
+        <v>36.86</v>
       </c>
       <c r="Q9" t="n">
-        <v>37.42</v>
+        <v>36.91</v>
       </c>
       <c r="R9" t="n">
-        <v>1.1991</v>
+        <v>17.3061</v>
       </c>
       <c r="S9" t="n">
-        <v>4.1518</v>
+        <v>18.5594</v>
       </c>
       <c r="T9" t="n">
-        <v>19.1383</v>
+        <v>17.9503</v>
       </c>
       <c r="U9" t="n">
-        <v>1.7502</v>
+        <v>1.3715</v>
       </c>
       <c r="V9" t="n">
-        <v>5.3508</v>
+        <v>4.2304</v>
       </c>
       <c r="W9" t="n">
-        <v>10.5344</v>
+        <v>6.4308</v>
       </c>
       <c r="X9" t="n">
-        <v>-1.1058</v>
+        <v>-17.4121</v>
       </c>
       <c r="Y9" t="n">
-        <v>-4.1348</v>
+        <v>-18.0666</v>
       </c>
       <c r="Z9" t="n">
-        <v>-19.0168</v>
+        <v>-17.806</v>
       </c>
       <c r="AA9" t="n">
-        <v>-1.7332</v>
+        <v>-1.3629</v>
       </c>
       <c r="AB9" t="n">
-        <v>-5.1217</v>
+        <v>-4.0551</v>
       </c>
       <c r="AC9" t="n">
-        <v>-9.831300000000001</v>
+        <v>-6.0336</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>243.18</v>
+        <v>281.47</v>
       </c>
       <c r="C10" t="n">
-        <v>267.08</v>
+        <v>284.58</v>
       </c>
       <c r="D10" t="n">
-        <v>238.82</v>
+        <v>257.26</v>
       </c>
       <c r="E10" t="n">
-        <v>266.32</v>
+        <v>280.54</v>
       </c>
       <c r="F10" t="n">
-        <v>85.94</v>
+        <v>87.68000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>87.31999999999999</v>
+        <v>88.09</v>
       </c>
       <c r="H10" t="n">
-        <v>84.83</v>
+        <v>85.41</v>
       </c>
       <c r="I10" t="n">
-        <v>87.22</v>
+        <v>86.56</v>
       </c>
       <c r="J10" t="n">
-        <v>5.8</v>
+        <v>4.88</v>
       </c>
       <c r="K10" t="n">
-        <v>5.93</v>
+        <v>5.35</v>
       </c>
       <c r="L10" t="n">
-        <v>5.15</v>
+        <v>4.82</v>
       </c>
       <c r="M10" t="n">
-        <v>5.17</v>
+        <v>4.91</v>
       </c>
       <c r="N10" t="n">
-        <v>37.47</v>
+        <v>36.73</v>
       </c>
       <c r="O10" t="n">
-        <v>37.95</v>
+        <v>37.69</v>
       </c>
       <c r="P10" t="n">
-        <v>36.86</v>
+        <v>36.55</v>
       </c>
       <c r="Q10" t="n">
-        <v>36.91</v>
+        <v>37.19</v>
       </c>
       <c r="R10" t="n">
-        <v>17.3061</v>
+        <v>5.3394</v>
       </c>
       <c r="S10" t="n">
-        <v>18.5594</v>
+        <v>25.0513</v>
       </c>
       <c r="T10" t="n">
-        <v>17.9503</v>
+        <v>28.6999</v>
       </c>
       <c r="U10" t="n">
-        <v>1.3715</v>
+        <v>-0.7567</v>
       </c>
       <c r="V10" t="n">
-        <v>4.2304</v>
+        <v>2.3652</v>
       </c>
       <c r="W10" t="n">
-        <v>6.4308</v>
+        <v>5.9875</v>
       </c>
       <c r="X10" t="n">
-        <v>-17.4121</v>
+        <v>-5.029</v>
       </c>
       <c r="Y10" t="n">
-        <v>-18.0666</v>
+        <v>-22.4329</v>
       </c>
       <c r="Z10" t="n">
-        <v>-17.806</v>
+        <v>-24.8086</v>
       </c>
       <c r="AA10" t="n">
-        <v>-1.3629</v>
+        <v>0.7586000000000001</v>
       </c>
       <c r="AB10" t="n">
-        <v>-4.0551</v>
+        <v>-2.3372</v>
       </c>
       <c r="AC10" t="n">
-        <v>-6.0336</v>
+        <v>-5.7049</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>281.47</v>
+        <v>242.04</v>
       </c>
       <c r="C11" t="n">
-        <v>284.58</v>
+        <v>274.5</v>
       </c>
       <c r="D11" t="n">
-        <v>257.26</v>
+        <v>228.55</v>
       </c>
       <c r="E11" t="n">
-        <v>280.54</v>
+        <v>262.7</v>
       </c>
       <c r="F11" t="n">
-        <v>87.68000000000001</v>
+        <v>83.47</v>
       </c>
       <c r="G11" t="n">
-        <v>88.09</v>
+        <v>86.25</v>
       </c>
       <c r="H11" t="n">
-        <v>85.41</v>
+        <v>82.48</v>
       </c>
       <c r="I11" t="n">
-        <v>86.56</v>
+        <v>85.22</v>
       </c>
       <c r="J11" t="n">
-        <v>4.88</v>
+        <v>5.57</v>
       </c>
       <c r="K11" t="n">
-        <v>5.35</v>
+        <v>5.81</v>
       </c>
       <c r="L11" t="n">
-        <v>4.82</v>
+        <v>5</v>
       </c>
       <c r="M11" t="n">
-        <v>4.91</v>
+        <v>5.2</v>
       </c>
       <c r="N11" t="n">
-        <v>36.73</v>
+        <v>38.53</v>
       </c>
       <c r="O11" t="n">
-        <v>37.69</v>
+        <v>38.96</v>
       </c>
       <c r="P11" t="n">
-        <v>36.55</v>
+        <v>37.33</v>
       </c>
       <c r="Q11" t="n">
-        <v>37.19</v>
+        <v>37.76</v>
       </c>
       <c r="R11" t="n">
-        <v>5.3394</v>
+        <v>-6.3592</v>
       </c>
       <c r="S11" t="n">
-        <v>25.0513</v>
+        <v>15.7116</v>
       </c>
       <c r="T11" t="n">
-        <v>28.6999</v>
+        <v>16.9479</v>
       </c>
       <c r="U11" t="n">
-        <v>-0.7567</v>
+        <v>-1.5481</v>
       </c>
       <c r="V11" t="n">
-        <v>2.3652</v>
+        <v>-0.953</v>
       </c>
       <c r="W11" t="n">
-        <v>5.9875</v>
+        <v>1.8403</v>
       </c>
       <c r="X11" t="n">
-        <v>-5.029</v>
+        <v>5.9063</v>
       </c>
       <c r="Y11" t="n">
-        <v>-22.4329</v>
+        <v>-16.9329</v>
       </c>
       <c r="Z11" t="n">
-        <v>-24.8086</v>
+        <v>-17.5911</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.7586000000000001</v>
+        <v>1.5327</v>
       </c>
       <c r="AB11" t="n">
-        <v>-2.3372</v>
+        <v>0.9086</v>
       </c>
       <c r="AC11" t="n">
-        <v>-5.7049</v>
+        <v>-1.8456</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>242.04</v>
+        <v>230.85</v>
       </c>
       <c r="C12" t="n">
-        <v>274.5</v>
+        <v>233.69</v>
       </c>
       <c r="D12" t="n">
-        <v>228.55</v>
+        <v>181.81</v>
       </c>
       <c r="E12" t="n">
-        <v>262.7</v>
+        <v>182.54</v>
       </c>
       <c r="F12" t="n">
-        <v>83.47</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="G12" t="n">
-        <v>86.25</v>
+        <v>82.08</v>
       </c>
       <c r="H12" t="n">
-        <v>82.48</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="I12" t="n">
-        <v>85.22</v>
+        <v>73.05</v>
       </c>
       <c r="J12" t="n">
-        <v>5.57</v>
+        <v>5.86</v>
       </c>
       <c r="K12" t="n">
-        <v>5.81</v>
+        <v>6.85</v>
       </c>
       <c r="L12" t="n">
-        <v>5</v>
+        <v>5.79</v>
       </c>
       <c r="M12" t="n">
-        <v>5.2</v>
+        <v>6.84</v>
       </c>
       <c r="N12" t="n">
-        <v>38.53</v>
+        <v>39.42</v>
       </c>
       <c r="O12" t="n">
-        <v>38.96</v>
+        <v>43.35</v>
       </c>
       <c r="P12" t="n">
-        <v>37.33</v>
+        <v>39.18</v>
       </c>
       <c r="Q12" t="n">
-        <v>37.76</v>
+        <v>43.19</v>
       </c>
       <c r="R12" t="n">
-        <v>-6.3592</v>
+        <v>-30.5139</v>
       </c>
       <c r="S12" t="n">
-        <v>15.7116</v>
+        <v>-31.4584</v>
       </c>
       <c r="T12" t="n">
-        <v>16.9479</v>
+        <v>-18.6324</v>
       </c>
       <c r="U12" t="n">
-        <v>-1.5481</v>
+        <v>-14.2807</v>
       </c>
       <c r="V12" t="n">
-        <v>-0.953</v>
+        <v>-16.2463</v>
       </c>
       <c r="W12" t="n">
-        <v>1.8403</v>
+        <v>-13.6116</v>
       </c>
       <c r="X12" t="n">
-        <v>5.9063</v>
+        <v>31.5385</v>
       </c>
       <c r="Y12" t="n">
-        <v>-16.9329</v>
+        <v>32.3017</v>
       </c>
       <c r="Z12" t="n">
-        <v>-17.5911</v>
+        <v>8.056900000000001</v>
       </c>
       <c r="AA12" t="n">
-        <v>1.5327</v>
+        <v>14.3803</v>
       </c>
       <c r="AB12" t="n">
-        <v>0.9086</v>
+        <v>17.0144</v>
       </c>
       <c r="AC12" t="n">
-        <v>-1.8456</v>
+        <v>13.4191</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>230.85</v>
+        <v>210.62</v>
       </c>
       <c r="C13" t="n">
-        <v>233.69</v>
+        <v>222.19</v>
       </c>
       <c r="D13" t="n">
-        <v>181.81</v>
+        <v>201.69</v>
       </c>
       <c r="E13" t="n">
-        <v>182.54</v>
+        <v>211.44</v>
       </c>
       <c r="F13" t="n">
-        <v>81.56999999999999</v>
+        <v>76.86</v>
       </c>
       <c r="G13" t="n">
-        <v>82.08</v>
+        <v>78.47</v>
       </c>
       <c r="H13" t="n">
-        <v>72.68000000000001</v>
+        <v>75.38</v>
       </c>
       <c r="I13" t="n">
-        <v>73.05</v>
+        <v>76.27</v>
       </c>
       <c r="J13" t="n">
-        <v>5.86</v>
+        <v>5.71</v>
       </c>
       <c r="K13" t="n">
-        <v>6.85</v>
+        <v>6.05</v>
       </c>
       <c r="L13" t="n">
-        <v>5.79</v>
+        <v>5.27</v>
       </c>
       <c r="M13" t="n">
-        <v>6.84</v>
+        <v>5.69</v>
       </c>
       <c r="N13" t="n">
-        <v>39.42</v>
+        <v>40.92</v>
       </c>
       <c r="O13" t="n">
-        <v>43.35</v>
+        <v>41.78</v>
       </c>
       <c r="P13" t="n">
-        <v>39.18</v>
+        <v>39.96</v>
       </c>
       <c r="Q13" t="n">
-        <v>43.19</v>
+        <v>41.26</v>
       </c>
       <c r="R13" t="n">
-        <v>-30.5139</v>
+        <v>15.8321</v>
       </c>
       <c r="S13" t="n">
-        <v>-31.4584</v>
+        <v>-24.6311</v>
       </c>
       <c r="T13" t="n">
-        <v>-18.6324</v>
+        <v>-6.8669</v>
       </c>
       <c r="U13" t="n">
-        <v>-14.2807</v>
+        <v>4.4079</v>
       </c>
       <c r="V13" t="n">
-        <v>-16.2463</v>
+        <v>-11.8877</v>
       </c>
       <c r="W13" t="n">
-        <v>-13.6116</v>
+        <v>-11.3552</v>
       </c>
       <c r="X13" t="n">
-        <v>31.5385</v>
+        <v>-16.8129</v>
       </c>
       <c r="Y13" t="n">
-        <v>32.3017</v>
+        <v>15.8859</v>
       </c>
       <c r="Z13" t="n">
-        <v>8.056900000000001</v>
+        <v>-9.105399999999999</v>
       </c>
       <c r="AA13" t="n">
-        <v>14.3803</v>
+        <v>-4.4686</v>
       </c>
       <c r="AB13" t="n">
-        <v>17.0144</v>
+        <v>10.9438</v>
       </c>
       <c r="AC13" t="n">
-        <v>13.4191</v>
+        <v>10.2619</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>210.62</v>
+        <v>227.06</v>
       </c>
       <c r="C14" t="n">
-        <v>222.19</v>
+        <v>231.02</v>
       </c>
       <c r="D14" t="n">
-        <v>201.69</v>
+        <v>157.56</v>
       </c>
       <c r="E14" t="n">
-        <v>211.44</v>
+        <v>201.68</v>
       </c>
       <c r="F14" t="n">
-        <v>76.86</v>
+        <v>78.48</v>
       </c>
       <c r="G14" t="n">
-        <v>78.47</v>
+        <v>79.34</v>
       </c>
       <c r="H14" t="n">
-        <v>75.38</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="I14" t="n">
-        <v>76.27</v>
+        <v>73.72</v>
       </c>
       <c r="J14" t="n">
-        <v>5.71</v>
+        <v>5.25</v>
       </c>
       <c r="K14" t="n">
-        <v>6.05</v>
+        <v>7.11</v>
       </c>
       <c r="L14" t="n">
-        <v>5.27</v>
+        <v>5.14</v>
       </c>
       <c r="M14" t="n">
-        <v>5.69</v>
+        <v>5.93</v>
       </c>
       <c r="N14" t="n">
-        <v>40.92</v>
+        <v>40.06</v>
       </c>
       <c r="O14" t="n">
-        <v>41.78</v>
+        <v>46.38</v>
       </c>
       <c r="P14" t="n">
-        <v>39.96</v>
+        <v>39.59</v>
       </c>
       <c r="Q14" t="n">
-        <v>41.26</v>
+        <v>42.67</v>
       </c>
       <c r="R14" t="n">
-        <v>15.8321</v>
+        <v>-4.616</v>
       </c>
       <c r="S14" t="n">
-        <v>-24.6311</v>
+        <v>-23.228</v>
       </c>
       <c r="T14" t="n">
-        <v>-6.8669</v>
+        <v>-24.2716</v>
       </c>
       <c r="U14" t="n">
-        <v>4.4079</v>
+        <v>-3.3434</v>
       </c>
       <c r="V14" t="n">
-        <v>-11.8877</v>
+        <v>-13.4945</v>
       </c>
       <c r="W14" t="n">
-        <v>-11.3552</v>
+        <v>-15.4781</v>
       </c>
       <c r="X14" t="n">
-        <v>-16.8129</v>
+        <v>4.2179</v>
       </c>
       <c r="Y14" t="n">
-        <v>15.8859</v>
+        <v>14.0385</v>
       </c>
       <c r="Z14" t="n">
-        <v>-9.105399999999999</v>
+        <v>14.7002</v>
       </c>
       <c r="AA14" t="n">
-        <v>-4.4686</v>
+        <v>3.4174</v>
       </c>
       <c r="AB14" t="n">
-        <v>10.9438</v>
+        <v>13.0032</v>
       </c>
       <c r="AC14" t="n">
-        <v>10.2619</v>
+        <v>15.6055</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>227.06</v>
+        <v>191.54</v>
       </c>
       <c r="C15" t="n">
-        <v>231.02</v>
+        <v>212.99</v>
       </c>
       <c r="D15" t="n">
-        <v>157.56</v>
+        <v>177.3</v>
       </c>
       <c r="E15" t="n">
-        <v>201.68</v>
+        <v>180.65</v>
       </c>
       <c r="F15" t="n">
-        <v>78.48</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>79.34</v>
+        <v>74.7</v>
       </c>
       <c r="H15" t="n">
-        <v>66.79000000000001</v>
+        <v>69</v>
       </c>
       <c r="I15" t="n">
-        <v>73.72</v>
+        <v>69.27</v>
       </c>
       <c r="J15" t="n">
-        <v>5.25</v>
+        <v>6.24</v>
       </c>
       <c r="K15" t="n">
-        <v>7.11</v>
+        <v>6.65</v>
       </c>
       <c r="L15" t="n">
-        <v>5.14</v>
+        <v>5.6</v>
       </c>
       <c r="M15" t="n">
-        <v>5.93</v>
+        <v>6.57</v>
       </c>
       <c r="N15" t="n">
-        <v>40.06</v>
+        <v>43.81</v>
       </c>
       <c r="O15" t="n">
-        <v>46.38</v>
+        <v>45.39</v>
       </c>
       <c r="P15" t="n">
-        <v>39.59</v>
+        <v>42.07</v>
       </c>
       <c r="Q15" t="n">
-        <v>42.67</v>
+        <v>45.25</v>
       </c>
       <c r="R15" t="n">
-        <v>-4.616</v>
+        <v>-10.4274</v>
       </c>
       <c r="S15" t="n">
-        <v>-23.228</v>
+        <v>-1.0354</v>
       </c>
       <c r="T15" t="n">
-        <v>-24.2716</v>
+        <v>-35.6063</v>
       </c>
       <c r="U15" t="n">
-        <v>-3.3434</v>
+        <v>-6.0364</v>
       </c>
       <c r="V15" t="n">
-        <v>-13.4945</v>
+        <v>-5.1745</v>
       </c>
       <c r="W15" t="n">
-        <v>-15.4781</v>
+        <v>-19.9746</v>
       </c>
       <c r="X15" t="n">
-        <v>4.2179</v>
+        <v>10.7926</v>
       </c>
       <c r="Y15" t="n">
-        <v>14.0385</v>
+        <v>-3.9474</v>
       </c>
       <c r="Z15" t="n">
-        <v>14.7002</v>
+        <v>33.8086</v>
       </c>
       <c r="AA15" t="n">
-        <v>3.4174</v>
+        <v>6.0464</v>
       </c>
       <c r="AB15" t="n">
-        <v>13.0032</v>
+        <v>4.7696</v>
       </c>
       <c r="AC15" t="n">
-        <v>15.6055</v>
+        <v>21.6725</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>191.54</v>
+        <v>192.3</v>
       </c>
       <c r="C16" t="n">
-        <v>212.99</v>
+        <v>225.63</v>
       </c>
       <c r="D16" t="n">
-        <v>177.3</v>
+        <v>192.3</v>
       </c>
       <c r="E16" t="n">
-        <v>180.65</v>
+        <v>223.99</v>
       </c>
       <c r="F16" t="n">
-        <v>71.68000000000001</v>
+        <v>70.89</v>
       </c>
       <c r="G16" t="n">
-        <v>74.7</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>69</v>
+        <v>69.59</v>
       </c>
       <c r="I16" t="n">
-        <v>69.27</v>
+        <v>76.01000000000001</v>
       </c>
       <c r="J16" t="n">
-        <v>6.24</v>
+        <v>6.1</v>
       </c>
       <c r="K16" t="n">
-        <v>6.65</v>
+        <v>6.1</v>
       </c>
       <c r="L16" t="n">
-        <v>5.6</v>
+        <v>4.9</v>
       </c>
       <c r="M16" t="n">
-        <v>6.57</v>
+        <v>4.97</v>
       </c>
       <c r="N16" t="n">
-        <v>43.81</v>
+        <v>44.18</v>
       </c>
       <c r="O16" t="n">
-        <v>45.39</v>
+        <v>45.01</v>
       </c>
       <c r="P16" t="n">
-        <v>42.07</v>
+        <v>40.44</v>
       </c>
       <c r="Q16" t="n">
-        <v>45.25</v>
+        <v>40.83</v>
       </c>
       <c r="R16" t="n">
-        <v>-10.4274</v>
+        <v>23.9911</v>
       </c>
       <c r="S16" t="n">
-        <v>-1.0354</v>
+        <v>5.9355</v>
       </c>
       <c r="T16" t="n">
-        <v>-35.6063</v>
+        <v>-14.7354</v>
       </c>
       <c r="U16" t="n">
-        <v>-6.0364</v>
+        <v>9.73</v>
       </c>
       <c r="V16" t="n">
-        <v>-5.1745</v>
+        <v>-0.3409</v>
       </c>
       <c r="W16" t="n">
-        <v>-19.9746</v>
+        <v>-10.8073</v>
       </c>
       <c r="X16" t="n">
-        <v>10.7926</v>
+        <v>-24.3531</v>
       </c>
       <c r="Y16" t="n">
-        <v>-3.9474</v>
+        <v>-12.6538</v>
       </c>
       <c r="Z16" t="n">
-        <v>33.8086</v>
+        <v>-4.4231</v>
       </c>
       <c r="AA16" t="n">
-        <v>6.0464</v>
+        <v>-9.768000000000001</v>
       </c>
       <c r="AB16" t="n">
-        <v>4.7696</v>
+        <v>-1.0422</v>
       </c>
       <c r="AC16" t="n">
-        <v>21.6725</v>
+        <v>8.1303</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>192.3</v>
+        <v>222.22</v>
       </c>
       <c r="C17" t="n">
-        <v>225.63</v>
+        <v>242.4</v>
       </c>
       <c r="D17" t="n">
-        <v>192.3</v>
+        <v>214.74</v>
       </c>
       <c r="E17" t="n">
-        <v>223.99</v>
+        <v>234.68</v>
       </c>
       <c r="F17" t="n">
-        <v>70.89</v>
+        <v>76.34</v>
       </c>
       <c r="G17" t="n">
-        <v>76.59999999999999</v>
+        <v>78.36</v>
       </c>
       <c r="H17" t="n">
-        <v>69.59</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="I17" t="n">
-        <v>76.01000000000001</v>
+        <v>77.52</v>
       </c>
       <c r="J17" t="n">
-        <v>6.1</v>
+        <v>5.01</v>
       </c>
       <c r="K17" t="n">
-        <v>6.1</v>
+        <v>5.15</v>
       </c>
       <c r="L17" t="n">
-        <v>4.9</v>
+        <v>4.54</v>
       </c>
       <c r="M17" t="n">
-        <v>4.97</v>
+        <v>4.72</v>
       </c>
       <c r="N17" t="n">
-        <v>44.18</v>
+        <v>40.65</v>
       </c>
       <c r="O17" t="n">
-        <v>45.01</v>
+        <v>41.75</v>
       </c>
       <c r="P17" t="n">
-        <v>40.44</v>
+        <v>39.57</v>
       </c>
       <c r="Q17" t="n">
-        <v>40.83</v>
+        <v>40.04</v>
       </c>
       <c r="R17" t="n">
-        <v>23.9911</v>
+        <v>4.7725</v>
       </c>
       <c r="S17" t="n">
-        <v>5.9355</v>
+        <v>16.3626</v>
       </c>
       <c r="T17" t="n">
-        <v>-14.7354</v>
+        <v>28.5636</v>
       </c>
       <c r="U17" t="n">
-        <v>9.73</v>
+        <v>1.9866</v>
       </c>
       <c r="V17" t="n">
-        <v>-0.3409</v>
+        <v>5.1546</v>
       </c>
       <c r="W17" t="n">
-        <v>-10.8073</v>
+        <v>6.1191</v>
       </c>
       <c r="X17" t="n">
-        <v>-24.3531</v>
+        <v>-5.0302</v>
       </c>
       <c r="Y17" t="n">
-        <v>-12.6538</v>
+        <v>-20.4047</v>
       </c>
       <c r="Z17" t="n">
-        <v>-4.4231</v>
+        <v>-30.9942</v>
       </c>
       <c r="AA17" t="n">
-        <v>-9.768000000000001</v>
+        <v>-1.9349</v>
       </c>
       <c r="AB17" t="n">
-        <v>-1.0422</v>
+        <v>-6.1636</v>
       </c>
       <c r="AC17" t="n">
-        <v>8.1303</v>
+        <v>-7.2934</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>222.22</v>
+        <v>265.99</v>
       </c>
       <c r="C18" t="n">
-        <v>242.4</v>
+        <v>274.88</v>
       </c>
       <c r="D18" t="n">
-        <v>214.74</v>
+        <v>261.6</v>
       </c>
       <c r="E18" t="n">
-        <v>234.68</v>
+        <v>272.5</v>
       </c>
       <c r="F18" t="n">
-        <v>76.34</v>
+        <v>82.88</v>
       </c>
       <c r="G18" t="n">
-        <v>78.36</v>
+        <v>85.03</v>
       </c>
       <c r="H18" t="n">
-        <v>74.29000000000001</v>
+        <v>82.64</v>
       </c>
       <c r="I18" t="n">
-        <v>77.52</v>
+        <v>84.59</v>
       </c>
       <c r="J18" t="n">
-        <v>5.01</v>
+        <v>4.07</v>
       </c>
       <c r="K18" t="n">
-        <v>5.15</v>
+        <v>4.17</v>
       </c>
       <c r="L18" t="n">
-        <v>4.54</v>
+        <v>3.91</v>
       </c>
       <c r="M18" t="n">
-        <v>4.72</v>
+        <v>3.95</v>
       </c>
       <c r="N18" t="n">
-        <v>40.65</v>
+        <v>37.25</v>
       </c>
       <c r="O18" t="n">
-        <v>41.75</v>
+        <v>37.36</v>
       </c>
       <c r="P18" t="n">
-        <v>39.57</v>
+        <v>36.15</v>
       </c>
       <c r="Q18" t="n">
-        <v>40.04</v>
+        <v>36.31</v>
       </c>
       <c r="R18" t="n">
-        <v>4.7725</v>
+        <v>16.1156</v>
       </c>
       <c r="S18" t="n">
-        <v>16.3626</v>
+        <v>50.8442</v>
       </c>
       <c r="T18" t="n">
-        <v>28.5636</v>
+        <v>28.8782</v>
       </c>
       <c r="U18" t="n">
-        <v>1.9866</v>
+        <v>9.120200000000001</v>
       </c>
       <c r="V18" t="n">
-        <v>5.1546</v>
+        <v>22.1164</v>
       </c>
       <c r="W18" t="n">
-        <v>6.1191</v>
+        <v>10.9086</v>
       </c>
       <c r="X18" t="n">
-        <v>-5.0302</v>
+        <v>-16.3136</v>
       </c>
       <c r="Y18" t="n">
-        <v>-20.4047</v>
+        <v>-39.8782</v>
       </c>
       <c r="Z18" t="n">
-        <v>-30.9942</v>
+        <v>-30.58</v>
       </c>
       <c r="AA18" t="n">
-        <v>-1.9349</v>
+        <v>-9.3157</v>
       </c>
       <c r="AB18" t="n">
-        <v>-6.1636</v>
+        <v>-19.7569</v>
       </c>
       <c r="AC18" t="n">
-        <v>-7.2934</v>
+        <v>-11.9971</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>265.99</v>
+        <v>267.13</v>
       </c>
       <c r="C19" t="n">
-        <v>274.88</v>
+        <v>274.93</v>
       </c>
       <c r="D19" t="n">
-        <v>261.6</v>
+        <v>226</v>
       </c>
       <c r="E19" t="n">
-        <v>272.5</v>
+        <v>226.19</v>
       </c>
       <c r="F19" t="n">
-        <v>82.88</v>
+        <v>84.19</v>
       </c>
       <c r="G19" t="n">
-        <v>85.03</v>
+        <v>84.83</v>
       </c>
       <c r="H19" t="n">
-        <v>82.64</v>
+        <v>79.86</v>
       </c>
       <c r="I19" t="n">
-        <v>84.59</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="J19" t="n">
-        <v>4.07</v>
+        <v>4.03</v>
       </c>
       <c r="K19" t="n">
-        <v>4.17</v>
+        <v>4.65</v>
       </c>
       <c r="L19" t="n">
         <v>3.91</v>
       </c>
       <c r="M19" t="n">
-        <v>3.95</v>
+        <v>4.63</v>
       </c>
       <c r="N19" t="n">
-        <v>37.25</v>
+        <v>36.54</v>
       </c>
       <c r="O19" t="n">
-        <v>37.36</v>
+        <v>38.39</v>
       </c>
       <c r="P19" t="n">
-        <v>36.15</v>
+        <v>36.26</v>
       </c>
       <c r="Q19" t="n">
-        <v>36.31</v>
+        <v>38.35</v>
       </c>
       <c r="R19" t="n">
-        <v>16.1156</v>
+        <v>-16.9945</v>
       </c>
       <c r="S19" t="n">
-        <v>50.8442</v>
+        <v>0.9822</v>
       </c>
       <c r="T19" t="n">
-        <v>28.8782</v>
+        <v>12.1529</v>
       </c>
       <c r="U19" t="n">
-        <v>9.120200000000001</v>
+        <v>-5.5089</v>
       </c>
       <c r="V19" t="n">
-        <v>22.1164</v>
+        <v>5.1572</v>
       </c>
       <c r="W19" t="n">
-        <v>10.9086</v>
+        <v>8.4238</v>
       </c>
       <c r="X19" t="n">
-        <v>-16.3136</v>
+        <v>17.2152</v>
       </c>
       <c r="Y19" t="n">
-        <v>-39.8782</v>
+        <v>-6.841</v>
       </c>
       <c r="Z19" t="n">
-        <v>-30.58</v>
+        <v>-21.9224</v>
       </c>
       <c r="AA19" t="n">
-        <v>-9.3157</v>
+        <v>5.6183</v>
       </c>
       <c r="AB19" t="n">
-        <v>-19.7569</v>
+        <v>-6.074</v>
       </c>
       <c r="AC19" t="n">
-        <v>-11.9971</v>
+        <v>-10.1242</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>267.13</v>
+        <v>247.42</v>
       </c>
       <c r="C20" t="n">
-        <v>274.93</v>
+        <v>259.79</v>
       </c>
       <c r="D20" t="n">
-        <v>226</v>
+        <v>233.3</v>
       </c>
       <c r="E20" t="n">
-        <v>226.19</v>
+        <v>233.86</v>
       </c>
       <c r="F20" t="n">
-        <v>84.19</v>
+        <v>81.67</v>
       </c>
       <c r="G20" t="n">
-        <v>84.83</v>
+        <v>81.81</v>
       </c>
       <c r="H20" t="n">
-        <v>79.86</v>
+        <v>76.94</v>
       </c>
       <c r="I20" t="n">
-        <v>79.93000000000001</v>
+        <v>77.54000000000001</v>
       </c>
       <c r="J20" t="n">
-        <v>4.03</v>
+        <v>4.17</v>
       </c>
       <c r="K20" t="n">
-        <v>4.65</v>
+        <v>4.46</v>
       </c>
       <c r="L20" t="n">
-        <v>3.91</v>
+        <v>3.92</v>
       </c>
       <c r="M20" t="n">
-        <v>4.63</v>
+        <v>4.46</v>
       </c>
       <c r="N20" t="n">
-        <v>36.54</v>
+        <v>37.53</v>
       </c>
       <c r="O20" t="n">
-        <v>38.39</v>
+        <v>39.79</v>
       </c>
       <c r="P20" t="n">
-        <v>36.26</v>
+        <v>37.46</v>
       </c>
       <c r="Q20" t="n">
-        <v>38.35</v>
+        <v>39.52</v>
       </c>
       <c r="R20" t="n">
-        <v>-16.9945</v>
+        <v>3.391</v>
       </c>
       <c r="S20" t="n">
-        <v>0.9822</v>
+        <v>-0.3494</v>
       </c>
       <c r="T20" t="n">
-        <v>12.1529</v>
+        <v>29.4547</v>
       </c>
       <c r="U20" t="n">
-        <v>-5.5089</v>
+        <v>-2.9901</v>
       </c>
       <c r="V20" t="n">
-        <v>5.1572</v>
+        <v>0.0258</v>
       </c>
       <c r="W20" t="n">
-        <v>8.4238</v>
+        <v>11.9388</v>
       </c>
       <c r="X20" t="n">
-        <v>17.2152</v>
+        <v>-3.6717</v>
       </c>
       <c r="Y20" t="n">
-        <v>-6.841</v>
+        <v>-5.5085</v>
       </c>
       <c r="Z20" t="n">
-        <v>-21.9224</v>
+        <v>-32.1157</v>
       </c>
       <c r="AA20" t="n">
-        <v>5.6183</v>
+        <v>3.0508</v>
       </c>
       <c r="AB20" t="n">
-        <v>-6.074</v>
+        <v>-1.2987</v>
       </c>
       <c r="AC20" t="n">
-        <v>-10.1242</v>
+        <v>-12.663</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>247.42</v>
+        <v>266.04</v>
       </c>
       <c r="C21" t="n">
-        <v>259.79</v>
+        <v>286.15</v>
       </c>
       <c r="D21" t="n">
-        <v>233.3</v>
+        <v>265</v>
       </c>
       <c r="E21" t="n">
-        <v>233.86</v>
+        <v>279.29</v>
       </c>
       <c r="F21" t="n">
-        <v>81.67</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="G21" t="n">
-        <v>81.81</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>76.94</v>
+        <v>80.63</v>
       </c>
       <c r="I21" t="n">
-        <v>77.54000000000001</v>
+        <v>82.87</v>
       </c>
       <c r="J21" t="n">
-        <v>4.17</v>
+        <v>3.86</v>
       </c>
       <c r="K21" t="n">
-        <v>4.46</v>
+        <v>3.87</v>
       </c>
       <c r="L21" t="n">
-        <v>3.92</v>
+        <v>3.45</v>
       </c>
       <c r="M21" t="n">
-        <v>4.46</v>
+        <v>3.59</v>
       </c>
       <c r="N21" t="n">
-        <v>37.53</v>
+        <v>37.2</v>
       </c>
       <c r="O21" t="n">
-        <v>39.79</v>
+        <v>37.95</v>
       </c>
       <c r="P21" t="n">
-        <v>37.46</v>
+        <v>36.43</v>
       </c>
       <c r="Q21" t="n">
-        <v>39.52</v>
+        <v>36.75</v>
       </c>
       <c r="R21" t="n">
-        <v>3.391</v>
+        <v>19.4262</v>
       </c>
       <c r="S21" t="n">
-        <v>-0.3494</v>
+        <v>2.4917</v>
       </c>
       <c r="T21" t="n">
-        <v>29.4547</v>
+        <v>24.6886</v>
       </c>
       <c r="U21" t="n">
-        <v>-2.9901</v>
+        <v>6.8739</v>
       </c>
       <c r="V21" t="n">
-        <v>0.0258</v>
+        <v>-2.0333</v>
       </c>
       <c r="W21" t="n">
-        <v>11.9388</v>
+        <v>9.0251</v>
       </c>
       <c r="X21" t="n">
-        <v>-3.6717</v>
+        <v>-19.5067</v>
       </c>
       <c r="Y21" t="n">
-        <v>-5.5085</v>
+        <v>-9.113899999999999</v>
       </c>
       <c r="Z21" t="n">
-        <v>-32.1157</v>
+        <v>-27.7666</v>
       </c>
       <c r="AA21" t="n">
-        <v>3.0508</v>
+        <v>-7.0091</v>
       </c>
       <c r="AB21" t="n">
-        <v>-1.2987</v>
+        <v>1.2118</v>
       </c>
       <c r="AC21" t="n">
-        <v>-12.663</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>266.035</v>
-      </c>
-      <c r="C22" t="n">
-        <v>286.1526</v>
-      </c>
-      <c r="D22" t="n">
-        <v>265</v>
-      </c>
-      <c r="E22" t="n">
-        <v>279.29</v>
-      </c>
-      <c r="F22" t="n">
-        <v>82.09</v>
-      </c>
-      <c r="G22" t="n">
-        <v>83.59990000000001</v>
-      </c>
-      <c r="H22" t="n">
-        <v>80.63</v>
-      </c>
-      <c r="I22" t="n">
-        <v>82.87</v>
-      </c>
-      <c r="J22" t="n">
-        <v>3.855</v>
-      </c>
-      <c r="K22" t="n">
-        <v>3.865</v>
-      </c>
-      <c r="L22" t="n">
-        <v>3.45</v>
-      </c>
-      <c r="M22" t="n">
-        <v>3.59</v>
-      </c>
-      <c r="N22" t="n">
-        <v>37.2</v>
-      </c>
-      <c r="O22" t="n">
-        <v>37.95</v>
-      </c>
-      <c r="P22" t="n">
-        <v>36.4301</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>36.75</v>
-      </c>
-      <c r="R22" t="n">
-        <v>19.4262</v>
-      </c>
-      <c r="S22" t="n">
-        <v>2.4917</v>
-      </c>
-      <c r="T22" t="n">
-        <v>24.6886</v>
-      </c>
-      <c r="U22" t="n">
-        <v>6.8739</v>
-      </c>
-      <c r="V22" t="n">
-        <v>-2.0333</v>
-      </c>
-      <c r="W22" t="n">
-        <v>9.0251</v>
-      </c>
-      <c r="X22" t="n">
-        <v>-19.5067</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>-9.113899999999999</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>-27.7666</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>-7.0091</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>1.2118</v>
-      </c>
-      <c r="AC22" t="n">
         <v>-9.992699999999999</v>
       </c>
     </row>
@@ -2412,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-22 23:20
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC21"/>
+  <dimension ref="A1:AC20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1713 +568,1622 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>171.26</v>
+        <v>211.38</v>
       </c>
       <c r="C2" t="n">
-        <v>179.97</v>
+        <v>228.5</v>
       </c>
       <c r="D2" t="n">
-        <v>168.23</v>
+        <v>209.89</v>
       </c>
       <c r="E2" t="n">
-        <v>178.39</v>
+        <v>225.79</v>
       </c>
       <c r="F2" t="n">
-        <v>75.18000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="G2" t="n">
-        <v>77.79000000000001</v>
+        <v>82.27</v>
       </c>
       <c r="H2" t="n">
-        <v>74.47</v>
+        <v>79.98</v>
       </c>
       <c r="I2" t="n">
-        <v>76.95</v>
+        <v>81.95</v>
       </c>
       <c r="J2" t="n">
-        <v>8.65</v>
+        <v>6.9</v>
       </c>
       <c r="K2" t="n">
-        <v>8.779999999999999</v>
+        <v>6.95</v>
       </c>
       <c r="L2" t="n">
-        <v>8.210000000000001</v>
+        <v>6.19</v>
       </c>
       <c r="M2" t="n">
-        <v>8.289999999999999</v>
+        <v>6.29</v>
       </c>
       <c r="N2" t="n">
-        <v>42.94</v>
+        <v>40.05</v>
       </c>
       <c r="O2" t="n">
-        <v>43.33</v>
+        <v>40.35</v>
       </c>
       <c r="P2" t="n">
-        <v>41.5</v>
+        <v>39.14</v>
       </c>
       <c r="Q2" t="n">
-        <v>41.96</v>
+        <v>39.28</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>184.8</v>
+        <v>242.66</v>
       </c>
       <c r="C3" t="n">
-        <v>195.27</v>
+        <v>242.66</v>
       </c>
       <c r="D3" t="n">
-        <v>183.34</v>
+        <v>204</v>
       </c>
       <c r="E3" t="n">
-        <v>190.56</v>
+        <v>217.98</v>
       </c>
       <c r="F3" t="n">
-        <v>78.04000000000001</v>
+        <v>82.87</v>
       </c>
       <c r="G3" t="n">
-        <v>79.33</v>
+        <v>82.91</v>
       </c>
       <c r="H3" t="n">
-        <v>77.33</v>
+        <v>80.33</v>
       </c>
       <c r="I3" t="n">
-        <v>77.84</v>
+        <v>81.67</v>
       </c>
       <c r="J3" t="n">
-        <v>8</v>
+        <v>5.83</v>
       </c>
       <c r="K3" t="n">
-        <v>8.06</v>
+        <v>6.91</v>
       </c>
       <c r="L3" t="n">
-        <v>7.5</v>
+        <v>5.83</v>
       </c>
       <c r="M3" t="n">
-        <v>7.73</v>
+        <v>6.53</v>
       </c>
       <c r="N3" t="n">
-        <v>41.4</v>
+        <v>38.87</v>
       </c>
       <c r="O3" t="n">
-        <v>41.78</v>
+        <v>40.09</v>
       </c>
       <c r="P3" t="n">
-        <v>40.68</v>
+        <v>38.86</v>
       </c>
       <c r="Q3" t="n">
-        <v>41.5</v>
+        <v>39.44</v>
       </c>
       <c r="R3" t="n">
-        <v>6.8221</v>
+        <v>-3.459</v>
       </c>
       <c r="U3" t="n">
-        <v>1.1566</v>
+        <v>-0.3417</v>
       </c>
       <c r="X3" t="n">
-        <v>-6.7551</v>
+        <v>3.8156</v>
       </c>
       <c r="AA3" t="n">
-        <v>-1.0963</v>
+        <v>0.4073</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>211.38</v>
+        <v>219</v>
       </c>
       <c r="C4" t="n">
-        <v>228.5</v>
+        <v>231.89</v>
       </c>
       <c r="D4" t="n">
-        <v>209.89</v>
+        <v>207.56</v>
       </c>
       <c r="E4" t="n">
-        <v>225.79</v>
+        <v>224.63</v>
       </c>
       <c r="F4" t="n">
-        <v>80.59</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>82.27</v>
+        <v>84.05</v>
       </c>
       <c r="H4" t="n">
-        <v>79.98</v>
+        <v>80.66</v>
       </c>
       <c r="I4" t="n">
-        <v>81.95</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>6.9</v>
+        <v>6.49</v>
       </c>
       <c r="K4" t="n">
-        <v>6.95</v>
+        <v>6.83</v>
       </c>
       <c r="L4" t="n">
-        <v>6.19</v>
+        <v>6.1</v>
       </c>
       <c r="M4" t="n">
-        <v>6.29</v>
+        <v>6.31</v>
       </c>
       <c r="N4" t="n">
-        <v>40.05</v>
+        <v>39.41</v>
       </c>
       <c r="O4" t="n">
-        <v>40.35</v>
+        <v>39.94</v>
       </c>
       <c r="P4" t="n">
-        <v>39.14</v>
+        <v>38.3</v>
       </c>
       <c r="Q4" t="n">
-        <v>39.28</v>
+        <v>38.47</v>
       </c>
       <c r="R4" t="n">
-        <v>18.4876</v>
+        <v>3.0507</v>
       </c>
       <c r="U4" t="n">
-        <v>5.2801</v>
+        <v>2.4611</v>
       </c>
       <c r="X4" t="n">
-        <v>-18.6287</v>
+        <v>-3.3691</v>
       </c>
       <c r="AA4" t="n">
-        <v>-5.3494</v>
+        <v>-2.4594</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>242.66</v>
+        <v>231.82</v>
       </c>
       <c r="C5" t="n">
-        <v>242.66</v>
+        <v>239.07</v>
       </c>
       <c r="D5" t="n">
-        <v>204</v>
+        <v>218.56</v>
       </c>
       <c r="E5" t="n">
-        <v>217.98</v>
+        <v>224.34</v>
       </c>
       <c r="F5" t="n">
-        <v>82.87</v>
+        <v>84.41</v>
       </c>
       <c r="G5" t="n">
-        <v>82.91</v>
+        <v>85.7</v>
       </c>
       <c r="H5" t="n">
-        <v>80.33</v>
+        <v>83.53</v>
       </c>
       <c r="I5" t="n">
-        <v>81.67</v>
+        <v>84.56</v>
       </c>
       <c r="J5" t="n">
-        <v>5.83</v>
+        <v>6.11</v>
       </c>
       <c r="K5" t="n">
-        <v>6.91</v>
+        <v>6.49</v>
       </c>
       <c r="L5" t="n">
-        <v>5.83</v>
+        <v>5.91</v>
       </c>
       <c r="M5" t="n">
-        <v>6.53</v>
+        <v>6.33</v>
       </c>
       <c r="N5" t="n">
-        <v>38.87</v>
+        <v>38.15</v>
       </c>
       <c r="O5" t="n">
-        <v>40.09</v>
+        <v>38.56</v>
       </c>
       <c r="P5" t="n">
-        <v>38.86</v>
+        <v>37.56</v>
       </c>
       <c r="Q5" t="n">
-        <v>39.44</v>
+        <v>38.08</v>
       </c>
       <c r="R5" t="n">
-        <v>-3.459</v>
+        <v>-0.1291</v>
       </c>
       <c r="S5" t="n">
-        <v>22.1929</v>
+        <v>-0.6422</v>
       </c>
       <c r="U5" t="n">
-        <v>-0.3417</v>
+        <v>1.0516</v>
       </c>
       <c r="V5" t="n">
-        <v>6.1339</v>
+        <v>3.1849</v>
       </c>
       <c r="X5" t="n">
-        <v>3.8156</v>
+        <v>0.317</v>
       </c>
       <c r="Y5" t="n">
-        <v>-21.2304</v>
+        <v>0.6359</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.4073</v>
+        <v>-1.0138</v>
       </c>
       <c r="AB5" t="n">
-        <v>-6.0057</v>
+        <v>-3.055</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>219</v>
+        <v>217.27</v>
       </c>
       <c r="C6" t="n">
-        <v>231.89</v>
+        <v>234.06</v>
       </c>
       <c r="D6" t="n">
-        <v>207.56</v>
+        <v>210.14</v>
       </c>
       <c r="E6" t="n">
-        <v>224.63</v>
+        <v>227.03</v>
       </c>
       <c r="F6" t="n">
-        <v>81.73999999999999</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>84.05</v>
+        <v>87.06</v>
       </c>
       <c r="H6" t="n">
-        <v>80.66</v>
+        <v>83.75</v>
       </c>
       <c r="I6" t="n">
-        <v>83.68000000000001</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>6.49</v>
+        <v>6.55</v>
       </c>
       <c r="K6" t="n">
-        <v>6.83</v>
+        <v>6.74</v>
       </c>
       <c r="L6" t="n">
-        <v>6.1</v>
+        <v>6.05</v>
       </c>
       <c r="M6" t="n">
-        <v>6.31</v>
+        <v>6.26</v>
       </c>
       <c r="N6" t="n">
-        <v>39.41</v>
+        <v>38.27</v>
       </c>
       <c r="O6" t="n">
-        <v>39.94</v>
+        <v>38.46</v>
       </c>
       <c r="P6" t="n">
-        <v>38.3</v>
+        <v>36.96</v>
       </c>
       <c r="Q6" t="n">
-        <v>38.47</v>
+        <v>37.42</v>
       </c>
       <c r="R6" t="n">
-        <v>3.0507</v>
+        <v>1.1991</v>
       </c>
       <c r="S6" t="n">
-        <v>17.8789</v>
+        <v>4.1518</v>
       </c>
       <c r="U6" t="n">
-        <v>2.4611</v>
+        <v>1.7502</v>
       </c>
       <c r="V6" t="n">
-        <v>7.5026</v>
+        <v>5.3508</v>
       </c>
       <c r="X6" t="n">
-        <v>-3.3691</v>
+        <v>-1.1058</v>
       </c>
       <c r="Y6" t="n">
-        <v>-18.37</v>
+        <v>-4.1348</v>
       </c>
       <c r="AA6" t="n">
-        <v>-2.4594</v>
+        <v>-1.7332</v>
       </c>
       <c r="AB6" t="n">
-        <v>-7.3012</v>
+        <v>-5.1217</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>231.82</v>
+        <v>243.18</v>
       </c>
       <c r="C7" t="n">
-        <v>239.07</v>
+        <v>267.08</v>
       </c>
       <c r="D7" t="n">
-        <v>218.56</v>
+        <v>238.82</v>
       </c>
       <c r="E7" t="n">
-        <v>224.34</v>
+        <v>266.32</v>
       </c>
       <c r="F7" t="n">
-        <v>84.41</v>
+        <v>85.94</v>
       </c>
       <c r="G7" t="n">
-        <v>85.7</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>83.53</v>
+        <v>84.83</v>
       </c>
       <c r="I7" t="n">
-        <v>84.56</v>
+        <v>87.22</v>
       </c>
       <c r="J7" t="n">
-        <v>6.11</v>
+        <v>5.8</v>
       </c>
       <c r="K7" t="n">
-        <v>6.49</v>
+        <v>5.93</v>
       </c>
       <c r="L7" t="n">
-        <v>5.91</v>
+        <v>5.15</v>
       </c>
       <c r="M7" t="n">
-        <v>6.33</v>
+        <v>5.17</v>
       </c>
       <c r="N7" t="n">
-        <v>38.15</v>
+        <v>37.47</v>
       </c>
       <c r="O7" t="n">
-        <v>38.56</v>
+        <v>37.95</v>
       </c>
       <c r="P7" t="n">
-        <v>37.56</v>
+        <v>36.86</v>
       </c>
       <c r="Q7" t="n">
-        <v>38.08</v>
+        <v>36.91</v>
       </c>
       <c r="R7" t="n">
-        <v>-0.1291</v>
+        <v>17.3061</v>
       </c>
       <c r="S7" t="n">
-        <v>-0.6422</v>
+        <v>18.5594</v>
       </c>
       <c r="T7" t="n">
-        <v>25.7582</v>
+        <v>17.9503</v>
       </c>
       <c r="U7" t="n">
-        <v>1.0516</v>
+        <v>1.3715</v>
       </c>
       <c r="V7" t="n">
-        <v>3.1849</v>
+        <v>4.2304</v>
       </c>
       <c r="W7" t="n">
-        <v>9.8895</v>
+        <v>6.4308</v>
       </c>
       <c r="X7" t="n">
-        <v>0.317</v>
+        <v>-17.4121</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.6359</v>
+        <v>-18.0666</v>
       </c>
       <c r="Z7" t="n">
-        <v>-23.6429</v>
+        <v>-17.806</v>
       </c>
       <c r="AA7" t="n">
-        <v>-1.0138</v>
+        <v>-1.3629</v>
       </c>
       <c r="AB7" t="n">
-        <v>-3.055</v>
+        <v>-4.0551</v>
       </c>
       <c r="AC7" t="n">
-        <v>-9.2469</v>
+        <v>-6.0336</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>217.27</v>
+        <v>281.47</v>
       </c>
       <c r="C8" t="n">
-        <v>234.06</v>
+        <v>284.58</v>
       </c>
       <c r="D8" t="n">
-        <v>210.14</v>
+        <v>257.26</v>
       </c>
       <c r="E8" t="n">
-        <v>227.03</v>
+        <v>280.54</v>
       </c>
       <c r="F8" t="n">
-        <v>84.15000000000001</v>
+        <v>87.68000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>87.06</v>
+        <v>88.09</v>
       </c>
       <c r="H8" t="n">
-        <v>83.75</v>
+        <v>85.41</v>
       </c>
       <c r="I8" t="n">
-        <v>86.04000000000001</v>
+        <v>86.56</v>
       </c>
       <c r="J8" t="n">
-        <v>6.55</v>
+        <v>4.88</v>
       </c>
       <c r="K8" t="n">
-        <v>6.74</v>
+        <v>5.35</v>
       </c>
       <c r="L8" t="n">
-        <v>6.05</v>
+        <v>4.82</v>
       </c>
       <c r="M8" t="n">
-        <v>6.26</v>
+        <v>4.91</v>
       </c>
       <c r="N8" t="n">
-        <v>38.27</v>
+        <v>36.73</v>
       </c>
       <c r="O8" t="n">
-        <v>38.46</v>
+        <v>37.69</v>
       </c>
       <c r="P8" t="n">
-        <v>36.96</v>
+        <v>36.55</v>
       </c>
       <c r="Q8" t="n">
-        <v>37.42</v>
+        <v>37.19</v>
       </c>
       <c r="R8" t="n">
-        <v>1.1991</v>
+        <v>5.3394</v>
       </c>
       <c r="S8" t="n">
-        <v>4.1518</v>
+        <v>25.0513</v>
       </c>
       <c r="T8" t="n">
-        <v>19.1383</v>
+        <v>28.6999</v>
       </c>
       <c r="U8" t="n">
-        <v>1.7502</v>
+        <v>-0.7567</v>
       </c>
       <c r="V8" t="n">
-        <v>5.3508</v>
+        <v>2.3652</v>
       </c>
       <c r="W8" t="n">
-        <v>10.5344</v>
+        <v>5.9875</v>
       </c>
       <c r="X8" t="n">
-        <v>-1.1058</v>
+        <v>-5.029</v>
       </c>
       <c r="Y8" t="n">
-        <v>-4.1348</v>
+        <v>-22.4329</v>
       </c>
       <c r="Z8" t="n">
-        <v>-19.0168</v>
+        <v>-24.8086</v>
       </c>
       <c r="AA8" t="n">
-        <v>-1.7332</v>
+        <v>0.7586000000000001</v>
       </c>
       <c r="AB8" t="n">
-        <v>-5.1217</v>
+        <v>-2.3372</v>
       </c>
       <c r="AC8" t="n">
-        <v>-9.831300000000001</v>
+        <v>-5.7049</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>243.18</v>
+        <v>242.04</v>
       </c>
       <c r="C9" t="n">
-        <v>267.08</v>
+        <v>274.5</v>
       </c>
       <c r="D9" t="n">
-        <v>238.82</v>
+        <v>228.55</v>
       </c>
       <c r="E9" t="n">
-        <v>266.32</v>
+        <v>262.7</v>
       </c>
       <c r="F9" t="n">
-        <v>85.94</v>
+        <v>83.47</v>
       </c>
       <c r="G9" t="n">
-        <v>87.31999999999999</v>
+        <v>86.25</v>
       </c>
       <c r="H9" t="n">
-        <v>84.83</v>
+        <v>82.48</v>
       </c>
       <c r="I9" t="n">
-        <v>87.22</v>
+        <v>85.22</v>
       </c>
       <c r="J9" t="n">
-        <v>5.8</v>
+        <v>5.57</v>
       </c>
       <c r="K9" t="n">
-        <v>5.93</v>
+        <v>5.81</v>
       </c>
       <c r="L9" t="n">
-        <v>5.15</v>
+        <v>5</v>
       </c>
       <c r="M9" t="n">
-        <v>5.17</v>
+        <v>5.2</v>
       </c>
       <c r="N9" t="n">
-        <v>37.47</v>
+        <v>38.53</v>
       </c>
       <c r="O9" t="n">
-        <v>37.95</v>
+        <v>38.96</v>
       </c>
       <c r="P9" t="n">
-        <v>36.86</v>
+        <v>37.33</v>
       </c>
       <c r="Q9" t="n">
-        <v>36.91</v>
+        <v>37.76</v>
       </c>
       <c r="R9" t="n">
-        <v>17.3061</v>
+        <v>-6.3592</v>
       </c>
       <c r="S9" t="n">
-        <v>18.5594</v>
+        <v>15.7116</v>
       </c>
       <c r="T9" t="n">
-        <v>17.9503</v>
+        <v>16.9479</v>
       </c>
       <c r="U9" t="n">
-        <v>1.3715</v>
+        <v>-1.5481</v>
       </c>
       <c r="V9" t="n">
-        <v>4.2304</v>
+        <v>-0.953</v>
       </c>
       <c r="W9" t="n">
-        <v>6.4308</v>
+        <v>1.8403</v>
       </c>
       <c r="X9" t="n">
-        <v>-17.4121</v>
+        <v>5.9063</v>
       </c>
       <c r="Y9" t="n">
-        <v>-18.0666</v>
+        <v>-16.9329</v>
       </c>
       <c r="Z9" t="n">
-        <v>-17.806</v>
+        <v>-17.5911</v>
       </c>
       <c r="AA9" t="n">
-        <v>-1.3629</v>
+        <v>1.5327</v>
       </c>
       <c r="AB9" t="n">
-        <v>-4.0551</v>
+        <v>0.9086</v>
       </c>
       <c r="AC9" t="n">
-        <v>-6.0336</v>
+        <v>-1.8456</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>281.47</v>
+        <v>230.85</v>
       </c>
       <c r="C10" t="n">
-        <v>284.58</v>
+        <v>233.69</v>
       </c>
       <c r="D10" t="n">
-        <v>257.26</v>
+        <v>181.81</v>
       </c>
       <c r="E10" t="n">
-        <v>280.54</v>
+        <v>182.54</v>
       </c>
       <c r="F10" t="n">
-        <v>87.68000000000001</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="G10" t="n">
-        <v>88.09</v>
+        <v>82.08</v>
       </c>
       <c r="H10" t="n">
-        <v>85.41</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="I10" t="n">
-        <v>86.56</v>
+        <v>73.05</v>
       </c>
       <c r="J10" t="n">
-        <v>4.88</v>
+        <v>5.86</v>
       </c>
       <c r="K10" t="n">
-        <v>5.35</v>
+        <v>6.85</v>
       </c>
       <c r="L10" t="n">
-        <v>4.82</v>
+        <v>5.79</v>
       </c>
       <c r="M10" t="n">
-        <v>4.91</v>
+        <v>6.84</v>
       </c>
       <c r="N10" t="n">
-        <v>36.73</v>
+        <v>39.42</v>
       </c>
       <c r="O10" t="n">
-        <v>37.69</v>
+        <v>43.35</v>
       </c>
       <c r="P10" t="n">
-        <v>36.55</v>
+        <v>39.18</v>
       </c>
       <c r="Q10" t="n">
-        <v>37.19</v>
+        <v>43.19</v>
       </c>
       <c r="R10" t="n">
-        <v>5.3394</v>
+        <v>-30.5139</v>
       </c>
       <c r="S10" t="n">
-        <v>25.0513</v>
+        <v>-31.4584</v>
       </c>
       <c r="T10" t="n">
-        <v>28.6999</v>
+        <v>-18.6324</v>
       </c>
       <c r="U10" t="n">
-        <v>-0.7567</v>
+        <v>-14.2807</v>
       </c>
       <c r="V10" t="n">
-        <v>2.3652</v>
+        <v>-16.2463</v>
       </c>
       <c r="W10" t="n">
-        <v>5.9875</v>
+        <v>-13.6116</v>
       </c>
       <c r="X10" t="n">
-        <v>-5.029</v>
+        <v>31.5385</v>
       </c>
       <c r="Y10" t="n">
-        <v>-22.4329</v>
+        <v>32.3017</v>
       </c>
       <c r="Z10" t="n">
-        <v>-24.8086</v>
+        <v>8.056900000000001</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.7586000000000001</v>
+        <v>14.3803</v>
       </c>
       <c r="AB10" t="n">
-        <v>-2.3372</v>
+        <v>17.0144</v>
       </c>
       <c r="AC10" t="n">
-        <v>-5.7049</v>
+        <v>13.4191</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>242.04</v>
+        <v>210.62</v>
       </c>
       <c r="C11" t="n">
-        <v>274.5</v>
+        <v>222.19</v>
       </c>
       <c r="D11" t="n">
-        <v>228.55</v>
+        <v>201.69</v>
       </c>
       <c r="E11" t="n">
-        <v>262.7</v>
+        <v>211.44</v>
       </c>
       <c r="F11" t="n">
-        <v>83.47</v>
+        <v>76.86</v>
       </c>
       <c r="G11" t="n">
-        <v>86.25</v>
+        <v>78.47</v>
       </c>
       <c r="H11" t="n">
-        <v>82.48</v>
+        <v>75.38</v>
       </c>
       <c r="I11" t="n">
-        <v>85.22</v>
+        <v>76.27</v>
       </c>
       <c r="J11" t="n">
-        <v>5.57</v>
+        <v>5.71</v>
       </c>
       <c r="K11" t="n">
-        <v>5.81</v>
+        <v>6.05</v>
       </c>
       <c r="L11" t="n">
-        <v>5</v>
+        <v>5.27</v>
       </c>
       <c r="M11" t="n">
-        <v>5.2</v>
+        <v>5.69</v>
       </c>
       <c r="N11" t="n">
-        <v>38.53</v>
+        <v>40.92</v>
       </c>
       <c r="O11" t="n">
-        <v>38.96</v>
+        <v>41.78</v>
       </c>
       <c r="P11" t="n">
-        <v>37.33</v>
+        <v>39.96</v>
       </c>
       <c r="Q11" t="n">
-        <v>37.76</v>
+        <v>41.26</v>
       </c>
       <c r="R11" t="n">
-        <v>-6.3592</v>
+        <v>15.8321</v>
       </c>
       <c r="S11" t="n">
-        <v>15.7116</v>
+        <v>-24.6311</v>
       </c>
       <c r="T11" t="n">
-        <v>16.9479</v>
+        <v>-6.8669</v>
       </c>
       <c r="U11" t="n">
-        <v>-1.5481</v>
+        <v>4.4079</v>
       </c>
       <c r="V11" t="n">
-        <v>-0.953</v>
+        <v>-11.8877</v>
       </c>
       <c r="W11" t="n">
-        <v>1.8403</v>
+        <v>-11.3552</v>
       </c>
       <c r="X11" t="n">
-        <v>5.9063</v>
+        <v>-16.8129</v>
       </c>
       <c r="Y11" t="n">
-        <v>-16.9329</v>
+        <v>15.8859</v>
       </c>
       <c r="Z11" t="n">
-        <v>-17.5911</v>
+        <v>-9.105399999999999</v>
       </c>
       <c r="AA11" t="n">
-        <v>1.5327</v>
+        <v>-4.4686</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.9086</v>
+        <v>10.9438</v>
       </c>
       <c r="AC11" t="n">
-        <v>-1.8456</v>
+        <v>10.2619</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>230.85</v>
+        <v>227.06</v>
       </c>
       <c r="C12" t="n">
-        <v>233.69</v>
+        <v>231.02</v>
       </c>
       <c r="D12" t="n">
-        <v>181.81</v>
+        <v>157.56</v>
       </c>
       <c r="E12" t="n">
-        <v>182.54</v>
+        <v>201.68</v>
       </c>
       <c r="F12" t="n">
-        <v>81.56999999999999</v>
+        <v>78.48</v>
       </c>
       <c r="G12" t="n">
-        <v>82.08</v>
+        <v>79.34</v>
       </c>
       <c r="H12" t="n">
-        <v>72.68000000000001</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="I12" t="n">
-        <v>73.05</v>
+        <v>73.72</v>
       </c>
       <c r="J12" t="n">
-        <v>5.86</v>
+        <v>5.25</v>
       </c>
       <c r="K12" t="n">
-        <v>6.85</v>
+        <v>7.11</v>
       </c>
       <c r="L12" t="n">
-        <v>5.79</v>
+        <v>5.14</v>
       </c>
       <c r="M12" t="n">
-        <v>6.84</v>
+        <v>5.93</v>
       </c>
       <c r="N12" t="n">
-        <v>39.42</v>
+        <v>40.06</v>
       </c>
       <c r="O12" t="n">
-        <v>43.35</v>
+        <v>46.38</v>
       </c>
       <c r="P12" t="n">
-        <v>39.18</v>
+        <v>39.59</v>
       </c>
       <c r="Q12" t="n">
-        <v>43.19</v>
+        <v>42.67</v>
       </c>
       <c r="R12" t="n">
-        <v>-30.5139</v>
+        <v>-4.616</v>
       </c>
       <c r="S12" t="n">
-        <v>-31.4584</v>
+        <v>-23.228</v>
       </c>
       <c r="T12" t="n">
-        <v>-18.6324</v>
+        <v>-24.2716</v>
       </c>
       <c r="U12" t="n">
-        <v>-14.2807</v>
+        <v>-3.3434</v>
       </c>
       <c r="V12" t="n">
-        <v>-16.2463</v>
+        <v>-13.4945</v>
       </c>
       <c r="W12" t="n">
-        <v>-13.6116</v>
+        <v>-15.4781</v>
       </c>
       <c r="X12" t="n">
-        <v>31.5385</v>
+        <v>4.2179</v>
       </c>
       <c r="Y12" t="n">
-        <v>32.3017</v>
+        <v>14.0385</v>
       </c>
       <c r="Z12" t="n">
-        <v>8.056900000000001</v>
+        <v>14.7002</v>
       </c>
       <c r="AA12" t="n">
-        <v>14.3803</v>
+        <v>3.4174</v>
       </c>
       <c r="AB12" t="n">
-        <v>17.0144</v>
+        <v>13.0032</v>
       </c>
       <c r="AC12" t="n">
-        <v>13.4191</v>
+        <v>15.6055</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>210.62</v>
+        <v>191.54</v>
       </c>
       <c r="C13" t="n">
-        <v>222.19</v>
+        <v>212.99</v>
       </c>
       <c r="D13" t="n">
-        <v>201.69</v>
+        <v>177.3</v>
       </c>
       <c r="E13" t="n">
-        <v>211.44</v>
+        <v>180.65</v>
       </c>
       <c r="F13" t="n">
-        <v>76.86</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>78.47</v>
+        <v>74.7</v>
       </c>
       <c r="H13" t="n">
-        <v>75.38</v>
+        <v>69</v>
       </c>
       <c r="I13" t="n">
-        <v>76.27</v>
+        <v>69.27</v>
       </c>
       <c r="J13" t="n">
-        <v>5.71</v>
+        <v>6.24</v>
       </c>
       <c r="K13" t="n">
-        <v>6.05</v>
+        <v>6.65</v>
       </c>
       <c r="L13" t="n">
-        <v>5.27</v>
+        <v>5.6</v>
       </c>
       <c r="M13" t="n">
-        <v>5.69</v>
+        <v>6.57</v>
       </c>
       <c r="N13" t="n">
-        <v>40.92</v>
+        <v>43.81</v>
       </c>
       <c r="O13" t="n">
-        <v>41.78</v>
+        <v>45.39</v>
       </c>
       <c r="P13" t="n">
-        <v>39.96</v>
+        <v>42.07</v>
       </c>
       <c r="Q13" t="n">
-        <v>41.26</v>
+        <v>45.25</v>
       </c>
       <c r="R13" t="n">
-        <v>15.8321</v>
+        <v>-10.4274</v>
       </c>
       <c r="S13" t="n">
-        <v>-24.6311</v>
+        <v>-1.0354</v>
       </c>
       <c r="T13" t="n">
-        <v>-6.8669</v>
+        <v>-35.6063</v>
       </c>
       <c r="U13" t="n">
-        <v>4.4079</v>
+        <v>-6.0364</v>
       </c>
       <c r="V13" t="n">
-        <v>-11.8877</v>
+        <v>-5.1745</v>
       </c>
       <c r="W13" t="n">
-        <v>-11.3552</v>
+        <v>-19.9746</v>
       </c>
       <c r="X13" t="n">
-        <v>-16.8129</v>
+        <v>10.7926</v>
       </c>
       <c r="Y13" t="n">
-        <v>15.8859</v>
+        <v>-3.9474</v>
       </c>
       <c r="Z13" t="n">
-        <v>-9.105399999999999</v>
+        <v>33.8086</v>
       </c>
       <c r="AA13" t="n">
-        <v>-4.4686</v>
+        <v>6.0464</v>
       </c>
       <c r="AB13" t="n">
-        <v>10.9438</v>
+        <v>4.7696</v>
       </c>
       <c r="AC13" t="n">
-        <v>10.2619</v>
+        <v>21.6725</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>227.06</v>
+        <v>192.3</v>
       </c>
       <c r="C14" t="n">
-        <v>231.02</v>
+        <v>225.63</v>
       </c>
       <c r="D14" t="n">
-        <v>157.56</v>
+        <v>192.3</v>
       </c>
       <c r="E14" t="n">
-        <v>201.68</v>
+        <v>223.99</v>
       </c>
       <c r="F14" t="n">
-        <v>78.48</v>
+        <v>70.89</v>
       </c>
       <c r="G14" t="n">
-        <v>79.34</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>66.79000000000001</v>
+        <v>69.59</v>
       </c>
       <c r="I14" t="n">
-        <v>73.72</v>
+        <v>76.01000000000001</v>
       </c>
       <c r="J14" t="n">
-        <v>5.25</v>
+        <v>6.1</v>
       </c>
       <c r="K14" t="n">
-        <v>7.11</v>
+        <v>6.1</v>
       </c>
       <c r="L14" t="n">
-        <v>5.14</v>
+        <v>4.9</v>
       </c>
       <c r="M14" t="n">
-        <v>5.93</v>
+        <v>4.97</v>
       </c>
       <c r="N14" t="n">
-        <v>40.06</v>
+        <v>44.18</v>
       </c>
       <c r="O14" t="n">
-        <v>46.38</v>
+        <v>45.01</v>
       </c>
       <c r="P14" t="n">
-        <v>39.59</v>
+        <v>40.44</v>
       </c>
       <c r="Q14" t="n">
-        <v>42.67</v>
+        <v>40.83</v>
       </c>
       <c r="R14" t="n">
-        <v>-4.616</v>
+        <v>23.9911</v>
       </c>
       <c r="S14" t="n">
-        <v>-23.228</v>
+        <v>5.9355</v>
       </c>
       <c r="T14" t="n">
-        <v>-24.2716</v>
+        <v>-14.7354</v>
       </c>
       <c r="U14" t="n">
-        <v>-3.3434</v>
+        <v>9.73</v>
       </c>
       <c r="V14" t="n">
-        <v>-13.4945</v>
+        <v>-0.3409</v>
       </c>
       <c r="W14" t="n">
-        <v>-15.4781</v>
+        <v>-10.8073</v>
       </c>
       <c r="X14" t="n">
-        <v>4.2179</v>
+        <v>-24.3531</v>
       </c>
       <c r="Y14" t="n">
-        <v>14.0385</v>
+        <v>-12.6538</v>
       </c>
       <c r="Z14" t="n">
-        <v>14.7002</v>
+        <v>-4.4231</v>
       </c>
       <c r="AA14" t="n">
-        <v>3.4174</v>
+        <v>-9.768000000000001</v>
       </c>
       <c r="AB14" t="n">
-        <v>13.0032</v>
+        <v>-1.0422</v>
       </c>
       <c r="AC14" t="n">
-        <v>15.6055</v>
+        <v>8.1303</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>191.54</v>
+        <v>222.22</v>
       </c>
       <c r="C15" t="n">
-        <v>212.99</v>
+        <v>242.4</v>
       </c>
       <c r="D15" t="n">
-        <v>177.3</v>
+        <v>214.74</v>
       </c>
       <c r="E15" t="n">
-        <v>180.65</v>
+        <v>234.68</v>
       </c>
       <c r="F15" t="n">
-        <v>71.68000000000001</v>
+        <v>76.34</v>
       </c>
       <c r="G15" t="n">
-        <v>74.7</v>
+        <v>78.36</v>
       </c>
       <c r="H15" t="n">
-        <v>69</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="I15" t="n">
-        <v>69.27</v>
+        <v>77.52</v>
       </c>
       <c r="J15" t="n">
-        <v>6.24</v>
+        <v>5.01</v>
       </c>
       <c r="K15" t="n">
-        <v>6.65</v>
+        <v>5.15</v>
       </c>
       <c r="L15" t="n">
-        <v>5.6</v>
+        <v>4.54</v>
       </c>
       <c r="M15" t="n">
-        <v>6.57</v>
+        <v>4.72</v>
       </c>
       <c r="N15" t="n">
-        <v>43.81</v>
+        <v>40.65</v>
       </c>
       <c r="O15" t="n">
-        <v>45.39</v>
+        <v>41.75</v>
       </c>
       <c r="P15" t="n">
-        <v>42.07</v>
+        <v>39.57</v>
       </c>
       <c r="Q15" t="n">
-        <v>45.25</v>
+        <v>40.04</v>
       </c>
       <c r="R15" t="n">
-        <v>-10.4274</v>
+        <v>4.7725</v>
       </c>
       <c r="S15" t="n">
-        <v>-1.0354</v>
+        <v>16.3626</v>
       </c>
       <c r="T15" t="n">
-        <v>-35.6063</v>
+        <v>28.5636</v>
       </c>
       <c r="U15" t="n">
-        <v>-6.0364</v>
+        <v>1.9866</v>
       </c>
       <c r="V15" t="n">
-        <v>-5.1745</v>
+        <v>5.1546</v>
       </c>
       <c r="W15" t="n">
-        <v>-19.9746</v>
+        <v>6.1191</v>
       </c>
       <c r="X15" t="n">
-        <v>10.7926</v>
+        <v>-5.0302</v>
       </c>
       <c r="Y15" t="n">
-        <v>-3.9474</v>
+        <v>-20.4047</v>
       </c>
       <c r="Z15" t="n">
-        <v>33.8086</v>
+        <v>-30.9942</v>
       </c>
       <c r="AA15" t="n">
-        <v>6.0464</v>
+        <v>-1.9349</v>
       </c>
       <c r="AB15" t="n">
-        <v>4.7696</v>
+        <v>-6.1636</v>
       </c>
       <c r="AC15" t="n">
-        <v>21.6725</v>
+        <v>-7.2934</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>192.3</v>
+        <v>265.99</v>
       </c>
       <c r="C16" t="n">
-        <v>225.63</v>
+        <v>274.88</v>
       </c>
       <c r="D16" t="n">
-        <v>192.3</v>
+        <v>261.6</v>
       </c>
       <c r="E16" t="n">
-        <v>223.99</v>
+        <v>272.5</v>
       </c>
       <c r="F16" t="n">
-        <v>70.89</v>
+        <v>82.88</v>
       </c>
       <c r="G16" t="n">
-        <v>76.59999999999999</v>
+        <v>85.03</v>
       </c>
       <c r="H16" t="n">
-        <v>69.59</v>
+        <v>82.64</v>
       </c>
       <c r="I16" t="n">
-        <v>76.01000000000001</v>
+        <v>84.59</v>
       </c>
       <c r="J16" t="n">
-        <v>6.1</v>
+        <v>4.07</v>
       </c>
       <c r="K16" t="n">
-        <v>6.1</v>
+        <v>4.17</v>
       </c>
       <c r="L16" t="n">
-        <v>4.9</v>
+        <v>3.91</v>
       </c>
       <c r="M16" t="n">
-        <v>4.97</v>
+        <v>3.95</v>
       </c>
       <c r="N16" t="n">
-        <v>44.18</v>
+        <v>37.25</v>
       </c>
       <c r="O16" t="n">
-        <v>45.01</v>
+        <v>37.36</v>
       </c>
       <c r="P16" t="n">
-        <v>40.44</v>
+        <v>36.15</v>
       </c>
       <c r="Q16" t="n">
-        <v>40.83</v>
+        <v>36.31</v>
       </c>
       <c r="R16" t="n">
-        <v>23.9911</v>
+        <v>16.1156</v>
       </c>
       <c r="S16" t="n">
-        <v>5.9355</v>
+        <v>50.8442</v>
       </c>
       <c r="T16" t="n">
-        <v>-14.7354</v>
+        <v>28.8782</v>
       </c>
       <c r="U16" t="n">
-        <v>9.73</v>
+        <v>9.120200000000001</v>
       </c>
       <c r="V16" t="n">
-        <v>-0.3409</v>
+        <v>22.1164</v>
       </c>
       <c r="W16" t="n">
-        <v>-10.8073</v>
+        <v>10.9086</v>
       </c>
       <c r="X16" t="n">
-        <v>-24.3531</v>
+        <v>-16.3136</v>
       </c>
       <c r="Y16" t="n">
-        <v>-12.6538</v>
+        <v>-39.8782</v>
       </c>
       <c r="Z16" t="n">
-        <v>-4.4231</v>
+        <v>-30.58</v>
       </c>
       <c r="AA16" t="n">
-        <v>-9.768000000000001</v>
+        <v>-9.3157</v>
       </c>
       <c r="AB16" t="n">
-        <v>-1.0422</v>
+        <v>-19.7569</v>
       </c>
       <c r="AC16" t="n">
-        <v>8.1303</v>
+        <v>-11.9971</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>222.22</v>
+        <v>267.13</v>
       </c>
       <c r="C17" t="n">
-        <v>242.4</v>
+        <v>274.93</v>
       </c>
       <c r="D17" t="n">
-        <v>214.74</v>
+        <v>226</v>
       </c>
       <c r="E17" t="n">
-        <v>234.68</v>
+        <v>226.19</v>
       </c>
       <c r="F17" t="n">
-        <v>76.34</v>
+        <v>84.19</v>
       </c>
       <c r="G17" t="n">
-        <v>78.36</v>
+        <v>84.83</v>
       </c>
       <c r="H17" t="n">
-        <v>74.29000000000001</v>
+        <v>79.86</v>
       </c>
       <c r="I17" t="n">
-        <v>77.52</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="J17" t="n">
-        <v>5.01</v>
+        <v>4.03</v>
       </c>
       <c r="K17" t="n">
-        <v>5.15</v>
+        <v>4.65</v>
       </c>
       <c r="L17" t="n">
-        <v>4.54</v>
+        <v>3.91</v>
       </c>
       <c r="M17" t="n">
-        <v>4.72</v>
+        <v>4.63</v>
       </c>
       <c r="N17" t="n">
-        <v>40.65</v>
+        <v>36.54</v>
       </c>
       <c r="O17" t="n">
-        <v>41.75</v>
+        <v>38.39</v>
       </c>
       <c r="P17" t="n">
-        <v>39.57</v>
+        <v>36.26</v>
       </c>
       <c r="Q17" t="n">
-        <v>40.04</v>
+        <v>38.35</v>
       </c>
       <c r="R17" t="n">
-        <v>4.7725</v>
+        <v>-16.9945</v>
       </c>
       <c r="S17" t="n">
-        <v>16.3626</v>
+        <v>0.9822</v>
       </c>
       <c r="T17" t="n">
-        <v>28.5636</v>
+        <v>12.1529</v>
       </c>
       <c r="U17" t="n">
-        <v>1.9866</v>
+        <v>-5.5089</v>
       </c>
       <c r="V17" t="n">
-        <v>5.1546</v>
+        <v>5.1572</v>
       </c>
       <c r="W17" t="n">
-        <v>6.1191</v>
+        <v>8.4238</v>
       </c>
       <c r="X17" t="n">
-        <v>-5.0302</v>
+        <v>17.2152</v>
       </c>
       <c r="Y17" t="n">
-        <v>-20.4047</v>
+        <v>-6.841</v>
       </c>
       <c r="Z17" t="n">
-        <v>-30.9942</v>
+        <v>-21.9224</v>
       </c>
       <c r="AA17" t="n">
-        <v>-1.9349</v>
+        <v>5.6183</v>
       </c>
       <c r="AB17" t="n">
-        <v>-6.1636</v>
+        <v>-6.074</v>
       </c>
       <c r="AC17" t="n">
-        <v>-7.2934</v>
+        <v>-10.1242</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>265.99</v>
+        <v>247.42</v>
       </c>
       <c r="C18" t="n">
-        <v>274.88</v>
+        <v>259.79</v>
       </c>
       <c r="D18" t="n">
-        <v>261.6</v>
+        <v>233.3</v>
       </c>
       <c r="E18" t="n">
-        <v>272.5</v>
+        <v>233.86</v>
       </c>
       <c r="F18" t="n">
-        <v>82.88</v>
+        <v>81.67</v>
       </c>
       <c r="G18" t="n">
-        <v>85.03</v>
+        <v>81.81</v>
       </c>
       <c r="H18" t="n">
-        <v>82.64</v>
+        <v>76.94</v>
       </c>
       <c r="I18" t="n">
-        <v>84.59</v>
+        <v>77.54000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>4.07</v>
+        <v>4.17</v>
       </c>
       <c r="K18" t="n">
-        <v>4.17</v>
+        <v>4.46</v>
       </c>
       <c r="L18" t="n">
-        <v>3.91</v>
+        <v>3.92</v>
       </c>
       <c r="M18" t="n">
-        <v>3.95</v>
+        <v>4.46</v>
       </c>
       <c r="N18" t="n">
-        <v>37.25</v>
+        <v>37.53</v>
       </c>
       <c r="O18" t="n">
-        <v>37.36</v>
+        <v>39.79</v>
       </c>
       <c r="P18" t="n">
-        <v>36.15</v>
+        <v>37.46</v>
       </c>
       <c r="Q18" t="n">
-        <v>36.31</v>
+        <v>39.52</v>
       </c>
       <c r="R18" t="n">
-        <v>16.1156</v>
+        <v>3.391</v>
       </c>
       <c r="S18" t="n">
-        <v>50.8442</v>
+        <v>-0.3494</v>
       </c>
       <c r="T18" t="n">
-        <v>28.8782</v>
+        <v>29.4547</v>
       </c>
       <c r="U18" t="n">
-        <v>9.120200000000001</v>
+        <v>-2.9901</v>
       </c>
       <c r="V18" t="n">
-        <v>22.1164</v>
+        <v>0.0258</v>
       </c>
       <c r="W18" t="n">
-        <v>10.9086</v>
+        <v>11.9388</v>
       </c>
       <c r="X18" t="n">
-        <v>-16.3136</v>
+        <v>-3.6717</v>
       </c>
       <c r="Y18" t="n">
-        <v>-39.8782</v>
+        <v>-5.5085</v>
       </c>
       <c r="Z18" t="n">
-        <v>-30.58</v>
+        <v>-32.1157</v>
       </c>
       <c r="AA18" t="n">
-        <v>-9.3157</v>
+        <v>3.0508</v>
       </c>
       <c r="AB18" t="n">
-        <v>-19.7569</v>
+        <v>-1.2987</v>
       </c>
       <c r="AC18" t="n">
-        <v>-11.9971</v>
+        <v>-12.663</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>267.13</v>
+        <v>266.04</v>
       </c>
       <c r="C19" t="n">
-        <v>274.93</v>
+        <v>286.15</v>
       </c>
       <c r="D19" t="n">
-        <v>226</v>
+        <v>265</v>
       </c>
       <c r="E19" t="n">
-        <v>226.19</v>
+        <v>279.29</v>
       </c>
       <c r="F19" t="n">
-        <v>84.19</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="G19" t="n">
-        <v>84.83</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>79.86</v>
+        <v>80.63</v>
       </c>
       <c r="I19" t="n">
-        <v>79.93000000000001</v>
+        <v>82.87</v>
       </c>
       <c r="J19" t="n">
-        <v>4.03</v>
+        <v>3.86</v>
       </c>
       <c r="K19" t="n">
-        <v>4.65</v>
+        <v>3.87</v>
       </c>
       <c r="L19" t="n">
-        <v>3.91</v>
+        <v>3.45</v>
       </c>
       <c r="M19" t="n">
-        <v>4.63</v>
+        <v>3.59</v>
       </c>
       <c r="N19" t="n">
-        <v>36.54</v>
+        <v>37.2</v>
       </c>
       <c r="O19" t="n">
-        <v>38.39</v>
+        <v>37.95</v>
       </c>
       <c r="P19" t="n">
-        <v>36.26</v>
+        <v>36.43</v>
       </c>
       <c r="Q19" t="n">
-        <v>38.35</v>
+        <v>36.75</v>
       </c>
       <c r="R19" t="n">
-        <v>-16.9945</v>
+        <v>19.4262</v>
       </c>
       <c r="S19" t="n">
-        <v>0.9822</v>
+        <v>2.4917</v>
       </c>
       <c r="T19" t="n">
-        <v>12.1529</v>
+        <v>24.6886</v>
       </c>
       <c r="U19" t="n">
-        <v>-5.5089</v>
+        <v>6.8739</v>
       </c>
       <c r="V19" t="n">
-        <v>5.1572</v>
+        <v>-2.0333</v>
       </c>
       <c r="W19" t="n">
-        <v>8.4238</v>
+        <v>9.0251</v>
       </c>
       <c r="X19" t="n">
-        <v>17.2152</v>
+        <v>-19.5067</v>
       </c>
       <c r="Y19" t="n">
-        <v>-6.841</v>
+        <v>-9.113899999999999</v>
       </c>
       <c r="Z19" t="n">
-        <v>-21.9224</v>
+        <v>-27.7666</v>
       </c>
       <c r="AA19" t="n">
-        <v>5.6183</v>
+        <v>-7.0091</v>
       </c>
       <c r="AB19" t="n">
-        <v>-6.074</v>
+        <v>1.2118</v>
       </c>
       <c r="AC19" t="n">
-        <v>-10.1242</v>
+        <v>-9.992699999999999</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>247.42</v>
+        <v>299.26</v>
       </c>
       <c r="C20" t="n">
-        <v>259.79</v>
+        <v>302</v>
       </c>
       <c r="D20" t="n">
-        <v>233.3</v>
+        <v>286.2401</v>
       </c>
       <c r="E20" t="n">
-        <v>233.86</v>
+        <v>300.77</v>
       </c>
       <c r="F20" t="n">
-        <v>81.67</v>
+        <v>83.97</v>
       </c>
       <c r="G20" t="n">
-        <v>81.81</v>
+        <v>85.1099</v>
       </c>
       <c r="H20" t="n">
-        <v>76.94</v>
+        <v>81.39</v>
       </c>
       <c r="I20" t="n">
-        <v>77.54000000000001</v>
+        <v>82.58</v>
       </c>
       <c r="J20" t="n">
-        <v>4.17</v>
+        <v>3.33</v>
       </c>
       <c r="K20" t="n">
-        <v>4.46</v>
+        <v>3.49</v>
       </c>
       <c r="L20" t="n">
-        <v>3.92</v>
+        <v>3.29</v>
       </c>
       <c r="M20" t="n">
-        <v>4.46</v>
+        <v>3.3</v>
       </c>
       <c r="N20" t="n">
-        <v>37.53</v>
+        <v>36.31</v>
       </c>
       <c r="O20" t="n">
-        <v>39.79</v>
+        <v>37.44</v>
       </c>
       <c r="P20" t="n">
-        <v>37.46</v>
+        <v>35.8</v>
       </c>
       <c r="Q20" t="n">
-        <v>39.52</v>
+        <v>36.93</v>
       </c>
       <c r="R20" t="n">
-        <v>3.391</v>
+        <v>7.6909</v>
       </c>
       <c r="S20" t="n">
-        <v>-0.3494</v>
+        <v>32.9723</v>
       </c>
       <c r="T20" t="n">
-        <v>29.4547</v>
+        <v>28.1618</v>
       </c>
       <c r="U20" t="n">
-        <v>-2.9901</v>
+        <v>-0.3499</v>
       </c>
       <c r="V20" t="n">
-        <v>0.0258</v>
+        <v>3.3154</v>
       </c>
       <c r="W20" t="n">
-        <v>11.9388</v>
+        <v>6.5273</v>
       </c>
       <c r="X20" t="n">
-        <v>-3.6717</v>
+        <v>-8.077999999999999</v>
       </c>
       <c r="Y20" t="n">
-        <v>-5.5085</v>
+        <v>-28.7257</v>
       </c>
       <c r="Z20" t="n">
-        <v>-32.1157</v>
+        <v>-30.0847</v>
       </c>
       <c r="AA20" t="n">
-        <v>3.0508</v>
+        <v>0.4898</v>
       </c>
       <c r="AB20" t="n">
-        <v>-1.2987</v>
+        <v>-3.7027</v>
       </c>
       <c r="AC20" t="n">
-        <v>-12.663</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>266.04</v>
-      </c>
-      <c r="C21" t="n">
-        <v>286.15</v>
-      </c>
-      <c r="D21" t="n">
-        <v>265</v>
-      </c>
-      <c r="E21" t="n">
-        <v>279.29</v>
-      </c>
-      <c r="F21" t="n">
-        <v>82.09999999999999</v>
-      </c>
-      <c r="G21" t="n">
-        <v>83.59999999999999</v>
-      </c>
-      <c r="H21" t="n">
-        <v>80.63</v>
-      </c>
-      <c r="I21" t="n">
-        <v>82.87</v>
-      </c>
-      <c r="J21" t="n">
-        <v>3.86</v>
-      </c>
-      <c r="K21" t="n">
-        <v>3.87</v>
-      </c>
-      <c r="L21" t="n">
-        <v>3.45</v>
-      </c>
-      <c r="M21" t="n">
-        <v>3.59</v>
-      </c>
-      <c r="N21" t="n">
-        <v>37.2</v>
-      </c>
-      <c r="O21" t="n">
-        <v>37.95</v>
-      </c>
-      <c r="P21" t="n">
-        <v>36.43</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>36.75</v>
-      </c>
-      <c r="R21" t="n">
-        <v>19.4262</v>
-      </c>
-      <c r="S21" t="n">
-        <v>2.4917</v>
-      </c>
-      <c r="T21" t="n">
-        <v>24.6886</v>
-      </c>
-      <c r="U21" t="n">
-        <v>6.8739</v>
-      </c>
-      <c r="V21" t="n">
-        <v>-2.0333</v>
-      </c>
-      <c r="W21" t="n">
-        <v>9.0251</v>
-      </c>
-      <c r="X21" t="n">
-        <v>-19.5067</v>
-      </c>
-      <c r="Y21" t="n">
-        <v>-9.113899999999999</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>-27.7666</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>-7.0091</v>
-      </c>
-      <c r="AB21" t="n">
-        <v>1.2118</v>
-      </c>
-      <c r="AC21" t="n">
-        <v>-9.992699999999999</v>
+        <v>-7.7672</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2230,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-23 23:08
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC20"/>
+  <dimension ref="A1:AC21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2108,16 +2108,16 @@
         <v>302</v>
       </c>
       <c r="D20" t="n">
-        <v>286.2401</v>
+        <v>286.24</v>
       </c>
       <c r="E20" t="n">
         <v>300.77</v>
       </c>
       <c r="F20" t="n">
-        <v>83.97</v>
+        <v>83.95</v>
       </c>
       <c r="G20" t="n">
-        <v>85.1099</v>
+        <v>85.11</v>
       </c>
       <c r="H20" t="n">
         <v>81.39</v>
@@ -2184,6 +2184,97 @@
       </c>
       <c r="AC20" t="n">
         <v>-7.7672</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>236</v>
+      </c>
+      <c r="C21" t="n">
+        <v>252.98</v>
+      </c>
+      <c r="D21" t="n">
+        <v>223</v>
+      </c>
+      <c r="E21" t="n">
+        <v>231.42</v>
+      </c>
+      <c r="F21" t="n">
+        <v>75.12</v>
+      </c>
+      <c r="G21" t="n">
+        <v>77.73999999999999</v>
+      </c>
+      <c r="H21" t="n">
+        <v>73.9101</v>
+      </c>
+      <c r="I21" t="n">
+        <v>74.44</v>
+      </c>
+      <c r="J21" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="K21" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="L21" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M21" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="N21" t="n">
+        <v>40.31</v>
+      </c>
+      <c r="O21" t="n">
+        <v>40.7999</v>
+      </c>
+      <c r="P21" t="n">
+        <v>39.0899</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>40.56</v>
+      </c>
+      <c r="R21" t="n">
+        <v>-23.0575</v>
+      </c>
+      <c r="S21" t="n">
+        <v>-1.0434</v>
+      </c>
+      <c r="T21" t="n">
+        <v>-15.0752</v>
+      </c>
+      <c r="U21" t="n">
+        <v>-9.857100000000001</v>
+      </c>
+      <c r="V21" t="n">
+        <v>-3.9979</v>
+      </c>
+      <c r="W21" t="n">
+        <v>-11.9991</v>
+      </c>
+      <c r="X21" t="n">
+        <v>22.4242</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>-9.417</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>2.2785</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>9.8294</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>2.6316</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>11.7048</v>
       </c>
     </row>
   </sheetData>
@@ -2230,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-24 23:03
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC21"/>
+  <dimension ref="A1:AC22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -596,16 +596,16 @@
         <v>81.95</v>
       </c>
       <c r="J2" t="n">
-        <v>6.9</v>
+        <v>6.8205</v>
       </c>
       <c r="K2" t="n">
-        <v>6.95</v>
+        <v>6.87</v>
       </c>
       <c r="L2" t="n">
-        <v>6.19</v>
+        <v>6.1187</v>
       </c>
       <c r="M2" t="n">
-        <v>6.29</v>
+        <v>6.2176</v>
       </c>
       <c r="N2" t="n">
         <v>40.05</v>
@@ -651,16 +651,16 @@
         <v>81.67</v>
       </c>
       <c r="J3" t="n">
-        <v>5.83</v>
+        <v>5.7629</v>
       </c>
       <c r="K3" t="n">
-        <v>6.91</v>
+        <v>6.8304</v>
       </c>
       <c r="L3" t="n">
-        <v>5.83</v>
+        <v>5.7629</v>
       </c>
       <c r="M3" t="n">
-        <v>6.53</v>
+        <v>6.4548</v>
       </c>
       <c r="N3" t="n">
         <v>38.87</v>
@@ -681,7 +681,7 @@
         <v>-0.3417</v>
       </c>
       <c r="X3" t="n">
-        <v>3.8156</v>
+        <v>3.815</v>
       </c>
       <c r="AA3" t="n">
         <v>0.4073</v>
@@ -718,16 +718,16 @@
         <v>83.68000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>6.49</v>
+        <v>6.4153</v>
       </c>
       <c r="K4" t="n">
-        <v>6.83</v>
+        <v>6.7514</v>
       </c>
       <c r="L4" t="n">
-        <v>6.1</v>
+        <v>6.0298</v>
       </c>
       <c r="M4" t="n">
-        <v>6.31</v>
+        <v>6.2373</v>
       </c>
       <c r="N4" t="n">
         <v>39.41</v>
@@ -748,7 +748,7 @@
         <v>2.4611</v>
       </c>
       <c r="X4" t="n">
-        <v>-3.3691</v>
+        <v>-3.3696</v>
       </c>
       <c r="AA4" t="n">
         <v>-2.4594</v>
@@ -785,16 +785,16 @@
         <v>84.56</v>
       </c>
       <c r="J5" t="n">
-        <v>6.11</v>
+        <v>6.0396</v>
       </c>
       <c r="K5" t="n">
-        <v>6.49</v>
+        <v>6.4153</v>
       </c>
       <c r="L5" t="n">
-        <v>5.91</v>
+        <v>5.8419</v>
       </c>
       <c r="M5" t="n">
-        <v>6.33</v>
+        <v>6.2571</v>
       </c>
       <c r="N5" t="n">
         <v>38.15</v>
@@ -821,10 +821,10 @@
         <v>3.1849</v>
       </c>
       <c r="X5" t="n">
-        <v>0.317</v>
+        <v>0.3174</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.6359</v>
+        <v>0.6353</v>
       </c>
       <c r="AA5" t="n">
         <v>-1.0138</v>
@@ -864,16 +864,16 @@
         <v>86.04000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>6.55</v>
+        <v>6.4746</v>
       </c>
       <c r="K6" t="n">
-        <v>6.74</v>
+        <v>6.6624</v>
       </c>
       <c r="L6" t="n">
-        <v>6.05</v>
+        <v>5.9803</v>
       </c>
       <c r="M6" t="n">
-        <v>6.26</v>
+        <v>6.1879</v>
       </c>
       <c r="N6" t="n">
         <v>38.27</v>
@@ -900,10 +900,10 @@
         <v>5.3508</v>
       </c>
       <c r="X6" t="n">
-        <v>-1.1058</v>
+        <v>-1.1059</v>
       </c>
       <c r="Y6" t="n">
-        <v>-4.1348</v>
+        <v>-4.1349</v>
       </c>
       <c r="AA6" t="n">
         <v>-1.7332</v>
@@ -943,16 +943,16 @@
         <v>87.22</v>
       </c>
       <c r="J7" t="n">
-        <v>5.8</v>
+        <v>5.7332</v>
       </c>
       <c r="K7" t="n">
-        <v>5.93</v>
+        <v>5.8617</v>
       </c>
       <c r="L7" t="n">
-        <v>5.15</v>
+        <v>5.0907</v>
       </c>
       <c r="M7" t="n">
-        <v>5.17</v>
+        <v>5.1105</v>
       </c>
       <c r="N7" t="n">
         <v>37.47</v>
@@ -985,13 +985,13 @@
         <v>6.4308</v>
       </c>
       <c r="X7" t="n">
-        <v>-17.4121</v>
+        <v>-17.4114</v>
       </c>
       <c r="Y7" t="n">
-        <v>-18.0666</v>
+        <v>-18.0655</v>
       </c>
       <c r="Z7" t="n">
-        <v>-17.806</v>
+        <v>-17.8059</v>
       </c>
       <c r="AA7" t="n">
         <v>-1.3629</v>
@@ -1034,16 +1034,16 @@
         <v>86.56</v>
       </c>
       <c r="J8" t="n">
-        <v>4.88</v>
+        <v>4.8238</v>
       </c>
       <c r="K8" t="n">
-        <v>5.35</v>
+        <v>5.2884</v>
       </c>
       <c r="L8" t="n">
-        <v>4.82</v>
+        <v>4.7645</v>
       </c>
       <c r="M8" t="n">
-        <v>4.91</v>
+        <v>4.8535</v>
       </c>
       <c r="N8" t="n">
         <v>36.73</v>
@@ -1076,13 +1076,13 @@
         <v>5.9875</v>
       </c>
       <c r="X8" t="n">
-        <v>-5.029</v>
+        <v>-5.0289</v>
       </c>
       <c r="Y8" t="n">
-        <v>-22.4329</v>
+        <v>-22.4321</v>
       </c>
       <c r="Z8" t="n">
-        <v>-24.8086</v>
+        <v>-24.8079</v>
       </c>
       <c r="AA8" t="n">
         <v>0.7586000000000001</v>
@@ -1125,16 +1125,16 @@
         <v>85.22</v>
       </c>
       <c r="J9" t="n">
-        <v>5.57</v>
+        <v>5.5059</v>
       </c>
       <c r="K9" t="n">
-        <v>5.81</v>
+        <v>5.7431</v>
       </c>
       <c r="L9" t="n">
-        <v>5</v>
+        <v>4.9424</v>
       </c>
       <c r="M9" t="n">
-        <v>5.2</v>
+        <v>5.1401</v>
       </c>
       <c r="N9" t="n">
         <v>38.53</v>
@@ -1167,13 +1167,13 @@
         <v>1.8403</v>
       </c>
       <c r="X9" t="n">
-        <v>5.9063</v>
+        <v>5.905</v>
       </c>
       <c r="Y9" t="n">
-        <v>-16.9329</v>
+        <v>-16.933</v>
       </c>
       <c r="Z9" t="n">
-        <v>-17.5911</v>
+        <v>-17.5909</v>
       </c>
       <c r="AA9" t="n">
         <v>1.5327</v>
@@ -1216,16 +1216,16 @@
         <v>73.05</v>
       </c>
       <c r="J10" t="n">
-        <v>5.86</v>
+        <v>5.7925</v>
       </c>
       <c r="K10" t="n">
-        <v>6.85</v>
+        <v>6.7711</v>
       </c>
       <c r="L10" t="n">
-        <v>5.79</v>
+        <v>5.7233</v>
       </c>
       <c r="M10" t="n">
-        <v>6.84</v>
+        <v>6.7612</v>
       </c>
       <c r="N10" t="n">
         <v>39.42</v>
@@ -1258,13 +1258,13 @@
         <v>-13.6116</v>
       </c>
       <c r="X10" t="n">
-        <v>31.5385</v>
+        <v>31.5383</v>
       </c>
       <c r="Y10" t="n">
-        <v>32.3017</v>
+        <v>32.3002</v>
       </c>
       <c r="Z10" t="n">
-        <v>8.056900000000001</v>
+        <v>8.0564</v>
       </c>
       <c r="AA10" t="n">
         <v>14.3803</v>
@@ -1307,16 +1307,16 @@
         <v>76.27</v>
       </c>
       <c r="J11" t="n">
-        <v>5.71</v>
+        <v>5.6442</v>
       </c>
       <c r="K11" t="n">
-        <v>6.05</v>
+        <v>5.9803</v>
       </c>
       <c r="L11" t="n">
-        <v>5.27</v>
+        <v>5.2093</v>
       </c>
       <c r="M11" t="n">
-        <v>5.69</v>
+        <v>5.6245</v>
       </c>
       <c r="N11" t="n">
         <v>40.92</v>
@@ -1349,13 +1349,13 @@
         <v>-11.3552</v>
       </c>
       <c r="X11" t="n">
-        <v>-16.8129</v>
+        <v>-16.8121</v>
       </c>
       <c r="Y11" t="n">
-        <v>15.8859</v>
+        <v>15.8854</v>
       </c>
       <c r="Z11" t="n">
-        <v>-9.105399999999999</v>
+        <v>-9.104900000000001</v>
       </c>
       <c r="AA11" t="n">
         <v>-4.4686</v>
@@ -1398,16 +1398,16 @@
         <v>73.72</v>
       </c>
       <c r="J12" t="n">
-        <v>5.25</v>
+        <v>5.1895</v>
       </c>
       <c r="K12" t="n">
-        <v>7.11</v>
+        <v>7.0281</v>
       </c>
       <c r="L12" t="n">
-        <v>5.14</v>
+        <v>5.0808</v>
       </c>
       <c r="M12" t="n">
-        <v>5.93</v>
+        <v>5.8617</v>
       </c>
       <c r="N12" t="n">
         <v>40.06</v>
@@ -1440,13 +1440,13 @@
         <v>-15.4781</v>
       </c>
       <c r="X12" t="n">
-        <v>4.2179</v>
+        <v>4.2173</v>
       </c>
       <c r="Y12" t="n">
-        <v>14.0385</v>
+        <v>14.0386</v>
       </c>
       <c r="Z12" t="n">
-        <v>14.7002</v>
+        <v>14.6991</v>
       </c>
       <c r="AA12" t="n">
         <v>3.4174</v>
@@ -1489,16 +1489,16 @@
         <v>69.27</v>
       </c>
       <c r="J13" t="n">
-        <v>6.24</v>
+        <v>6.1681</v>
       </c>
       <c r="K13" t="n">
-        <v>6.65</v>
+        <v>6.5734</v>
       </c>
       <c r="L13" t="n">
-        <v>5.6</v>
+        <v>5.5355</v>
       </c>
       <c r="M13" t="n">
-        <v>6.57</v>
+        <v>6.4943</v>
       </c>
       <c r="N13" t="n">
         <v>43.81</v>
@@ -1531,13 +1531,13 @@
         <v>-19.9746</v>
       </c>
       <c r="X13" t="n">
-        <v>10.7926</v>
+        <v>10.7921</v>
       </c>
       <c r="Y13" t="n">
-        <v>-3.9474</v>
+        <v>-3.9475</v>
       </c>
       <c r="Z13" t="n">
-        <v>33.8086</v>
+        <v>33.8065</v>
       </c>
       <c r="AA13" t="n">
         <v>6.0464</v>
@@ -1580,16 +1580,16 @@
         <v>76.01000000000001</v>
       </c>
       <c r="J14" t="n">
-        <v>6.1</v>
+        <v>6.0298</v>
       </c>
       <c r="K14" t="n">
-        <v>6.1</v>
+        <v>6.0298</v>
       </c>
       <c r="L14" t="n">
-        <v>4.9</v>
+        <v>4.8436</v>
       </c>
       <c r="M14" t="n">
-        <v>4.97</v>
+        <v>4.9128</v>
       </c>
       <c r="N14" t="n">
         <v>44.18</v>
@@ -1622,13 +1622,13 @@
         <v>-10.8073</v>
       </c>
       <c r="X14" t="n">
-        <v>-24.3531</v>
+        <v>-24.3521</v>
       </c>
       <c r="Y14" t="n">
-        <v>-12.6538</v>
+        <v>-12.6536</v>
       </c>
       <c r="Z14" t="n">
-        <v>-4.4231</v>
+        <v>-4.4221</v>
       </c>
       <c r="AA14" t="n">
         <v>-9.768000000000001</v>
@@ -1671,16 +1671,16 @@
         <v>77.52</v>
       </c>
       <c r="J15" t="n">
-        <v>5.01</v>
+        <v>4.9523</v>
       </c>
       <c r="K15" t="n">
-        <v>5.15</v>
+        <v>5.0907</v>
       </c>
       <c r="L15" t="n">
-        <v>4.54</v>
+        <v>4.4877</v>
       </c>
       <c r="M15" t="n">
-        <v>4.72</v>
+        <v>4.6656</v>
       </c>
       <c r="N15" t="n">
         <v>40.65</v>
@@ -1713,13 +1713,13 @@
         <v>6.1191</v>
       </c>
       <c r="X15" t="n">
-        <v>-5.0302</v>
+        <v>-5.0318</v>
       </c>
       <c r="Y15" t="n">
-        <v>-20.4047</v>
+        <v>-20.4053</v>
       </c>
       <c r="Z15" t="n">
-        <v>-30.9942</v>
+        <v>-30.9945</v>
       </c>
       <c r="AA15" t="n">
         <v>-1.9349</v>
@@ -1762,16 +1762,16 @@
         <v>84.59</v>
       </c>
       <c r="J16" t="n">
-        <v>4.07</v>
+        <v>4.0231</v>
       </c>
       <c r="K16" t="n">
-        <v>4.17</v>
+        <v>4.122</v>
       </c>
       <c r="L16" t="n">
-        <v>3.91</v>
+        <v>3.865</v>
       </c>
       <c r="M16" t="n">
-        <v>3.95</v>
+        <v>3.9045</v>
       </c>
       <c r="N16" t="n">
         <v>37.25</v>
@@ -1804,13 +1804,13 @@
         <v>10.9086</v>
       </c>
       <c r="X16" t="n">
-        <v>-16.3136</v>
+        <v>-16.313</v>
       </c>
       <c r="Y16" t="n">
-        <v>-39.8782</v>
+        <v>-39.878</v>
       </c>
       <c r="Z16" t="n">
-        <v>-30.58</v>
+        <v>-30.5805</v>
       </c>
       <c r="AA16" t="n">
         <v>-9.3157</v>
@@ -1853,16 +1853,16 @@
         <v>79.93000000000001</v>
       </c>
       <c r="J17" t="n">
-        <v>4.03</v>
+        <v>3.9836</v>
       </c>
       <c r="K17" t="n">
-        <v>4.65</v>
+        <v>4.5965</v>
       </c>
       <c r="L17" t="n">
-        <v>3.91</v>
+        <v>3.865</v>
       </c>
       <c r="M17" t="n">
-        <v>4.63</v>
+        <v>4.5767</v>
       </c>
       <c r="N17" t="n">
         <v>36.54</v>
@@ -1895,13 +1895,13 @@
         <v>8.4238</v>
       </c>
       <c r="X17" t="n">
-        <v>17.2152</v>
+        <v>17.216</v>
       </c>
       <c r="Y17" t="n">
-        <v>-6.841</v>
+        <v>-6.8413</v>
       </c>
       <c r="Z17" t="n">
-        <v>-21.9224</v>
+        <v>-21.922</v>
       </c>
       <c r="AA17" t="n">
         <v>5.6183</v>
@@ -1944,16 +1944,16 @@
         <v>77.54000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>4.17</v>
+        <v>4.122</v>
       </c>
       <c r="K18" t="n">
-        <v>4.46</v>
+        <v>4.4086</v>
       </c>
       <c r="L18" t="n">
-        <v>3.92</v>
+        <v>3.8749</v>
       </c>
       <c r="M18" t="n">
-        <v>4.46</v>
+        <v>4.4086</v>
       </c>
       <c r="N18" t="n">
         <v>37.53</v>
@@ -1986,13 +1986,13 @@
         <v>11.9388</v>
       </c>
       <c r="X18" t="n">
-        <v>-3.6717</v>
+        <v>-3.673</v>
       </c>
       <c r="Y18" t="n">
-        <v>-5.5085</v>
+        <v>-5.5084</v>
       </c>
       <c r="Z18" t="n">
-        <v>-32.1157</v>
+        <v>-32.1159</v>
       </c>
       <c r="AA18" t="n">
         <v>3.0508</v>
@@ -2035,16 +2035,16 @@
         <v>82.87</v>
       </c>
       <c r="J19" t="n">
-        <v>3.86</v>
+        <v>3.8156</v>
       </c>
       <c r="K19" t="n">
-        <v>3.87</v>
+        <v>3.8254</v>
       </c>
       <c r="L19" t="n">
-        <v>3.45</v>
+        <v>3.4103</v>
       </c>
       <c r="M19" t="n">
-        <v>3.59</v>
+        <v>3.5487</v>
       </c>
       <c r="N19" t="n">
         <v>37.2</v>
@@ -2077,13 +2077,13 @@
         <v>9.0251</v>
       </c>
       <c r="X19" t="n">
-        <v>-19.5067</v>
+        <v>-19.5051</v>
       </c>
       <c r="Y19" t="n">
-        <v>-9.113899999999999</v>
+        <v>-9.1126</v>
       </c>
       <c r="Z19" t="n">
-        <v>-27.7666</v>
+        <v>-27.7662</v>
       </c>
       <c r="AA19" t="n">
         <v>-7.0091</v>
@@ -2126,16 +2126,16 @@
         <v>82.58</v>
       </c>
       <c r="J20" t="n">
-        <v>3.33</v>
+        <v>3.2917</v>
       </c>
       <c r="K20" t="n">
-        <v>3.49</v>
+        <v>3.4498</v>
       </c>
       <c r="L20" t="n">
-        <v>3.29</v>
+        <v>3.2521</v>
       </c>
       <c r="M20" t="n">
-        <v>3.3</v>
+        <v>3.262</v>
       </c>
       <c r="N20" t="n">
         <v>36.31</v>
@@ -2168,13 +2168,13 @@
         <v>6.5273</v>
       </c>
       <c r="X20" t="n">
-        <v>-8.077999999999999</v>
+        <v>-8.079000000000001</v>
       </c>
       <c r="Y20" t="n">
-        <v>-28.7257</v>
+        <v>-28.7259</v>
       </c>
       <c r="Z20" t="n">
-        <v>-30.0847</v>
+        <v>-30.084</v>
       </c>
       <c r="AA20" t="n">
         <v>0.4898</v>
@@ -2211,7 +2211,7 @@
         <v>77.73999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>73.9101</v>
+        <v>73.91</v>
       </c>
       <c r="I21" t="n">
         <v>74.44</v>
@@ -2229,13 +2229,13 @@
         <v>4.04</v>
       </c>
       <c r="N21" t="n">
-        <v>40.31</v>
+        <v>40.26</v>
       </c>
       <c r="O21" t="n">
-        <v>40.7999</v>
+        <v>40.8</v>
       </c>
       <c r="P21" t="n">
-        <v>39.0899</v>
+        <v>39.08</v>
       </c>
       <c r="Q21" t="n">
         <v>40.56</v>
@@ -2259,13 +2259,13 @@
         <v>-11.9991</v>
       </c>
       <c r="X21" t="n">
-        <v>22.4242</v>
+        <v>23.8504</v>
       </c>
       <c r="Y21" t="n">
-        <v>-9.417</v>
+        <v>-8.360900000000001</v>
       </c>
       <c r="Z21" t="n">
-        <v>2.2785</v>
+        <v>3.4704</v>
       </c>
       <c r="AA21" t="n">
         <v>9.8294</v>
@@ -2275,6 +2275,97 @@
       </c>
       <c r="AC21" t="n">
         <v>11.7048</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>233.11</v>
+      </c>
+      <c r="C22" t="n">
+        <v>237</v>
+      </c>
+      <c r="D22" t="n">
+        <v>211.13</v>
+      </c>
+      <c r="E22" t="n">
+        <v>229.57</v>
+      </c>
+      <c r="F22" t="n">
+        <v>74.78</v>
+      </c>
+      <c r="G22" t="n">
+        <v>76.18000000000001</v>
+      </c>
+      <c r="H22" t="n">
+        <v>71.34999999999999</v>
+      </c>
+      <c r="I22" t="n">
+        <v>73.3</v>
+      </c>
+      <c r="J22" t="n">
+        <v>4</v>
+      </c>
+      <c r="K22" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="L22" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="M22" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="N22" t="n">
+        <v>39.67</v>
+      </c>
+      <c r="O22" t="n">
+        <v>41.49</v>
+      </c>
+      <c r="P22" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>40.45</v>
+      </c>
+      <c r="R22" t="n">
+        <v>-0.7994</v>
+      </c>
+      <c r="S22" t="n">
+        <v>-17.8023</v>
+      </c>
+      <c r="T22" t="n">
+        <v>1.4943</v>
+      </c>
+      <c r="U22" t="n">
+        <v>-1.5314</v>
+      </c>
+      <c r="V22" t="n">
+        <v>-11.5482</v>
+      </c>
+      <c r="W22" t="n">
+        <v>-8.2948</v>
+      </c>
+      <c r="X22" t="n">
+        <v>0.9901</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>14.9717</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>-10.8528</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>-0.2712</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>10.068</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>5.4759</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-25 23:18
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>211.38</v>
+        <v>242.66</v>
       </c>
       <c r="C2" t="n">
-        <v>228.5</v>
+        <v>242.66</v>
       </c>
       <c r="D2" t="n">
-        <v>209.89</v>
+        <v>204</v>
       </c>
       <c r="E2" t="n">
-        <v>225.79</v>
+        <v>217.98</v>
       </c>
       <c r="F2" t="n">
-        <v>80.59</v>
+        <v>82.87</v>
       </c>
       <c r="G2" t="n">
-        <v>82.27</v>
+        <v>82.91</v>
       </c>
       <c r="H2" t="n">
-        <v>79.98</v>
+        <v>80.33</v>
       </c>
       <c r="I2" t="n">
-        <v>81.95</v>
+        <v>81.67</v>
       </c>
       <c r="J2" t="n">
-        <v>6.8205</v>
+        <v>5.7629</v>
       </c>
       <c r="K2" t="n">
-        <v>6.87</v>
+        <v>6.8304</v>
       </c>
       <c r="L2" t="n">
-        <v>6.1187</v>
+        <v>5.7629</v>
       </c>
       <c r="M2" t="n">
-        <v>6.2176</v>
+        <v>6.4548</v>
       </c>
       <c r="N2" t="n">
-        <v>40.05</v>
+        <v>38.2586</v>
       </c>
       <c r="O2" t="n">
-        <v>40.35</v>
+        <v>39.4594</v>
       </c>
       <c r="P2" t="n">
-        <v>39.14</v>
+        <v>38.2487</v>
       </c>
       <c r="Q2" t="n">
-        <v>39.28</v>
+        <v>38.8196</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>242.66</v>
+        <v>219</v>
       </c>
       <c r="C3" t="n">
-        <v>242.66</v>
+        <v>231.89</v>
       </c>
       <c r="D3" t="n">
-        <v>204</v>
+        <v>207.56</v>
       </c>
       <c r="E3" t="n">
-        <v>217.98</v>
+        <v>224.63</v>
       </c>
       <c r="F3" t="n">
-        <v>82.87</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>82.91</v>
+        <v>84.05</v>
       </c>
       <c r="H3" t="n">
-        <v>80.33</v>
+        <v>80.66</v>
       </c>
       <c r="I3" t="n">
-        <v>81.67</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>5.7629</v>
+        <v>6.4153</v>
       </c>
       <c r="K3" t="n">
-        <v>6.8304</v>
+        <v>6.7514</v>
       </c>
       <c r="L3" t="n">
-        <v>5.7629</v>
+        <v>6.0298</v>
       </c>
       <c r="M3" t="n">
-        <v>6.4548</v>
+        <v>6.2373</v>
       </c>
       <c r="N3" t="n">
-        <v>38.87</v>
+        <v>38.7901</v>
       </c>
       <c r="O3" t="n">
-        <v>40.09</v>
+        <v>39.3118</v>
       </c>
       <c r="P3" t="n">
-        <v>38.86</v>
+        <v>37.6975</v>
       </c>
       <c r="Q3" t="n">
-        <v>39.44</v>
+        <v>37.8649</v>
       </c>
       <c r="R3" t="n">
-        <v>-3.459</v>
+        <v>3.0507</v>
       </c>
       <c r="U3" t="n">
-        <v>-0.3417</v>
+        <v>2.4611</v>
       </c>
       <c r="X3" t="n">
-        <v>3.815</v>
+        <v>-3.3696</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.4073</v>
+        <v>-2.4593</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>219</v>
+        <v>231.82</v>
       </c>
       <c r="C4" t="n">
-        <v>231.89</v>
+        <v>239.07</v>
       </c>
       <c r="D4" t="n">
-        <v>207.56</v>
+        <v>218.56</v>
       </c>
       <c r="E4" t="n">
-        <v>224.63</v>
+        <v>224.34</v>
       </c>
       <c r="F4" t="n">
-        <v>81.73999999999999</v>
+        <v>84.41</v>
       </c>
       <c r="G4" t="n">
-        <v>84.05</v>
+        <v>85.7</v>
       </c>
       <c r="H4" t="n">
-        <v>80.66</v>
+        <v>83.53</v>
       </c>
       <c r="I4" t="n">
-        <v>83.68000000000001</v>
+        <v>84.56</v>
       </c>
       <c r="J4" t="n">
+        <v>6.0396</v>
+      </c>
+      <c r="K4" t="n">
         <v>6.4153</v>
       </c>
-      <c r="K4" t="n">
-        <v>6.7514</v>
-      </c>
       <c r="L4" t="n">
-        <v>6.0298</v>
+        <v>5.8419</v>
       </c>
       <c r="M4" t="n">
-        <v>6.2373</v>
+        <v>6.2571</v>
       </c>
       <c r="N4" t="n">
-        <v>39.41</v>
+        <v>37.5499</v>
       </c>
       <c r="O4" t="n">
-        <v>39.94</v>
+        <v>37.9535</v>
       </c>
       <c r="P4" t="n">
-        <v>38.3</v>
+        <v>36.9692</v>
       </c>
       <c r="Q4" t="n">
-        <v>38.47</v>
+        <v>37.481</v>
       </c>
       <c r="R4" t="n">
-        <v>3.0507</v>
+        <v>-0.1291</v>
       </c>
       <c r="U4" t="n">
-        <v>2.4611</v>
+        <v>1.0516</v>
       </c>
       <c r="X4" t="n">
-        <v>-3.3696</v>
+        <v>0.3174</v>
       </c>
       <c r="AA4" t="n">
-        <v>-2.4594</v>
+        <v>-1.0139</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>231.82</v>
+        <v>217.27</v>
       </c>
       <c r="C5" t="n">
-        <v>239.07</v>
+        <v>234.06</v>
       </c>
       <c r="D5" t="n">
-        <v>218.56</v>
+        <v>210.14</v>
       </c>
       <c r="E5" t="n">
-        <v>224.34</v>
+        <v>227.03</v>
       </c>
       <c r="F5" t="n">
-        <v>84.41</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>85.7</v>
+        <v>87.06</v>
       </c>
       <c r="H5" t="n">
-        <v>83.53</v>
+        <v>83.75</v>
       </c>
       <c r="I5" t="n">
-        <v>84.56</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>6.0396</v>
+        <v>6.4746</v>
       </c>
       <c r="K5" t="n">
-        <v>6.4153</v>
+        <v>6.6624</v>
       </c>
       <c r="L5" t="n">
-        <v>5.8419</v>
+        <v>5.9803</v>
       </c>
       <c r="M5" t="n">
-        <v>6.2571</v>
+        <v>6.1879</v>
       </c>
       <c r="N5" t="n">
-        <v>38.15</v>
+        <v>37.668</v>
       </c>
       <c r="O5" t="n">
-        <v>38.56</v>
+        <v>37.855</v>
       </c>
       <c r="P5" t="n">
-        <v>37.56</v>
+        <v>36.3786</v>
       </c>
       <c r="Q5" t="n">
-        <v>38.08</v>
+        <v>36.8314</v>
       </c>
       <c r="R5" t="n">
-        <v>-0.1291</v>
+        <v>1.1991</v>
       </c>
       <c r="S5" t="n">
-        <v>-0.6422</v>
+        <v>4.1518</v>
       </c>
       <c r="U5" t="n">
-        <v>1.0516</v>
+        <v>1.7502</v>
       </c>
       <c r="V5" t="n">
-        <v>3.1849</v>
+        <v>5.3508</v>
       </c>
       <c r="X5" t="n">
-        <v>0.3174</v>
+        <v>-1.1059</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.6353</v>
+        <v>-4.1349</v>
       </c>
       <c r="AA5" t="n">
-        <v>-1.0138</v>
+        <v>-1.7331</v>
       </c>
       <c r="AB5" t="n">
-        <v>-3.055</v>
+        <v>-5.1216</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>217.27</v>
+        <v>243.18</v>
       </c>
       <c r="C6" t="n">
-        <v>234.06</v>
+        <v>267.08</v>
       </c>
       <c r="D6" t="n">
-        <v>210.14</v>
+        <v>238.82</v>
       </c>
       <c r="E6" t="n">
-        <v>227.03</v>
+        <v>266.32</v>
       </c>
       <c r="F6" t="n">
-        <v>84.15000000000001</v>
+        <v>85.94</v>
       </c>
       <c r="G6" t="n">
-        <v>87.06</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>83.75</v>
+        <v>84.83</v>
       </c>
       <c r="I6" t="n">
-        <v>86.04000000000001</v>
+        <v>87.22</v>
       </c>
       <c r="J6" t="n">
-        <v>6.4746</v>
+        <v>5.7332</v>
       </c>
       <c r="K6" t="n">
-        <v>6.6624</v>
+        <v>5.8617</v>
       </c>
       <c r="L6" t="n">
-        <v>5.9803</v>
+        <v>5.0907</v>
       </c>
       <c r="M6" t="n">
-        <v>6.1879</v>
+        <v>5.1105</v>
       </c>
       <c r="N6" t="n">
-        <v>38.27</v>
+        <v>36.8806</v>
       </c>
       <c r="O6" t="n">
-        <v>38.46</v>
+        <v>37.3531</v>
       </c>
       <c r="P6" t="n">
-        <v>36.96</v>
+        <v>36.2802</v>
       </c>
       <c r="Q6" t="n">
-        <v>37.42</v>
+        <v>36.3294</v>
       </c>
       <c r="R6" t="n">
-        <v>1.1991</v>
+        <v>17.3061</v>
       </c>
       <c r="S6" t="n">
-        <v>4.1518</v>
+        <v>18.5594</v>
       </c>
       <c r="U6" t="n">
-        <v>1.7502</v>
+        <v>1.3715</v>
       </c>
       <c r="V6" t="n">
-        <v>5.3508</v>
+        <v>4.2304</v>
       </c>
       <c r="X6" t="n">
-        <v>-1.1059</v>
+        <v>-17.4114</v>
       </c>
       <c r="Y6" t="n">
-        <v>-4.1349</v>
+        <v>-18.0655</v>
       </c>
       <c r="AA6" t="n">
-        <v>-1.7332</v>
+        <v>-1.363</v>
       </c>
       <c r="AB6" t="n">
-        <v>-5.1217</v>
+        <v>-4.0552</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>243.18</v>
+        <v>281.47</v>
       </c>
       <c r="C7" t="n">
-        <v>267.08</v>
+        <v>284.58</v>
       </c>
       <c r="D7" t="n">
-        <v>238.82</v>
+        <v>257.26</v>
       </c>
       <c r="E7" t="n">
-        <v>266.32</v>
+        <v>280.54</v>
       </c>
       <c r="F7" t="n">
-        <v>85.94</v>
+        <v>87.68000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>87.31999999999999</v>
+        <v>88.09</v>
       </c>
       <c r="H7" t="n">
-        <v>84.83</v>
+        <v>85.41</v>
       </c>
       <c r="I7" t="n">
-        <v>87.22</v>
+        <v>86.56</v>
       </c>
       <c r="J7" t="n">
-        <v>5.7332</v>
+        <v>4.8238</v>
       </c>
       <c r="K7" t="n">
-        <v>5.8617</v>
+        <v>5.2884</v>
       </c>
       <c r="L7" t="n">
-        <v>5.0907</v>
+        <v>4.7645</v>
       </c>
       <c r="M7" t="n">
-        <v>5.1105</v>
+        <v>4.8535</v>
       </c>
       <c r="N7" t="n">
-        <v>37.47</v>
+        <v>36.1522</v>
       </c>
       <c r="O7" t="n">
-        <v>37.95</v>
+        <v>37.0971</v>
       </c>
       <c r="P7" t="n">
-        <v>36.86</v>
+        <v>35.9751</v>
       </c>
       <c r="Q7" t="n">
-        <v>36.91</v>
+        <v>36.605</v>
       </c>
       <c r="R7" t="n">
-        <v>17.3061</v>
+        <v>5.3394</v>
       </c>
       <c r="S7" t="n">
-        <v>18.5594</v>
+        <v>25.0513</v>
       </c>
       <c r="T7" t="n">
-        <v>17.9503</v>
+        <v>28.6999</v>
       </c>
       <c r="U7" t="n">
-        <v>1.3715</v>
+        <v>-0.7567</v>
       </c>
       <c r="V7" t="n">
-        <v>4.2304</v>
+        <v>2.3652</v>
       </c>
       <c r="W7" t="n">
-        <v>6.4308</v>
+        <v>5.9875</v>
       </c>
       <c r="X7" t="n">
-        <v>-17.4114</v>
+        <v>-5.0289</v>
       </c>
       <c r="Y7" t="n">
-        <v>-18.0655</v>
+        <v>-22.4321</v>
       </c>
       <c r="Z7" t="n">
-        <v>-17.8059</v>
+        <v>-24.8079</v>
       </c>
       <c r="AA7" t="n">
-        <v>-1.3629</v>
+        <v>0.7586000000000001</v>
       </c>
       <c r="AB7" t="n">
-        <v>-4.0551</v>
+        <v>-2.3372</v>
       </c>
       <c r="AC7" t="n">
-        <v>-6.0336</v>
+        <v>-5.7049</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>281.47</v>
+        <v>242.04</v>
       </c>
       <c r="C8" t="n">
-        <v>284.58</v>
+        <v>274.5</v>
       </c>
       <c r="D8" t="n">
-        <v>257.26</v>
+        <v>228.55</v>
       </c>
       <c r="E8" t="n">
-        <v>280.54</v>
+        <v>262.7</v>
       </c>
       <c r="F8" t="n">
-        <v>87.68000000000001</v>
+        <v>83.47</v>
       </c>
       <c r="G8" t="n">
-        <v>88.09</v>
+        <v>86.25</v>
       </c>
       <c r="H8" t="n">
-        <v>85.41</v>
+        <v>82.48</v>
       </c>
       <c r="I8" t="n">
-        <v>86.56</v>
+        <v>85.22</v>
       </c>
       <c r="J8" t="n">
-        <v>4.8238</v>
+        <v>5.5059</v>
       </c>
       <c r="K8" t="n">
-        <v>5.2884</v>
+        <v>5.7431</v>
       </c>
       <c r="L8" t="n">
-        <v>4.7645</v>
+        <v>4.9424</v>
       </c>
       <c r="M8" t="n">
-        <v>4.8535</v>
+        <v>5.1401</v>
       </c>
       <c r="N8" t="n">
-        <v>36.73</v>
+        <v>37.9239</v>
       </c>
       <c r="O8" t="n">
-        <v>37.69</v>
+        <v>38.3472</v>
       </c>
       <c r="P8" t="n">
-        <v>36.55</v>
+        <v>36.7428</v>
       </c>
       <c r="Q8" t="n">
-        <v>37.19</v>
+        <v>37.166</v>
       </c>
       <c r="R8" t="n">
-        <v>5.3394</v>
+        <v>-6.3592</v>
       </c>
       <c r="S8" t="n">
-        <v>25.0513</v>
+        <v>15.7116</v>
       </c>
       <c r="T8" t="n">
-        <v>28.6999</v>
+        <v>16.9479</v>
       </c>
       <c r="U8" t="n">
-        <v>-0.7567</v>
+        <v>-1.5481</v>
       </c>
       <c r="V8" t="n">
-        <v>2.3652</v>
+        <v>-0.953</v>
       </c>
       <c r="W8" t="n">
-        <v>5.9875</v>
+        <v>1.8403</v>
       </c>
       <c r="X8" t="n">
-        <v>-5.0289</v>
+        <v>5.905</v>
       </c>
       <c r="Y8" t="n">
-        <v>-22.4321</v>
+        <v>-16.933</v>
       </c>
       <c r="Z8" t="n">
-        <v>-24.8079</v>
+        <v>-17.5909</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.7586000000000001</v>
+        <v>1.5326</v>
       </c>
       <c r="AB8" t="n">
-        <v>-2.3372</v>
+        <v>0.9085</v>
       </c>
       <c r="AC8" t="n">
-        <v>-5.7049</v>
+        <v>-1.8458</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>242.04</v>
+        <v>230.85</v>
       </c>
       <c r="C9" t="n">
-        <v>274.5</v>
+        <v>233.69</v>
       </c>
       <c r="D9" t="n">
-        <v>228.55</v>
+        <v>181.81</v>
       </c>
       <c r="E9" t="n">
-        <v>262.7</v>
+        <v>182.54</v>
       </c>
       <c r="F9" t="n">
-        <v>83.47</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>86.25</v>
+        <v>82.08</v>
       </c>
       <c r="H9" t="n">
-        <v>82.48</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="I9" t="n">
-        <v>85.22</v>
+        <v>73.05</v>
       </c>
       <c r="J9" t="n">
-        <v>5.5059</v>
+        <v>5.7925</v>
       </c>
       <c r="K9" t="n">
-        <v>5.7431</v>
+        <v>6.7711</v>
       </c>
       <c r="L9" t="n">
-        <v>4.9424</v>
+        <v>5.7233</v>
       </c>
       <c r="M9" t="n">
-        <v>5.1401</v>
+        <v>6.7612</v>
       </c>
       <c r="N9" t="n">
-        <v>38.53</v>
+        <v>38.7999</v>
       </c>
       <c r="O9" t="n">
-        <v>38.96</v>
+        <v>42.6681</v>
       </c>
       <c r="P9" t="n">
-        <v>37.33</v>
+        <v>38.5637</v>
       </c>
       <c r="Q9" t="n">
-        <v>37.76</v>
+        <v>42.5106</v>
       </c>
       <c r="R9" t="n">
-        <v>-6.3592</v>
+        <v>-30.5139</v>
       </c>
       <c r="S9" t="n">
-        <v>15.7116</v>
+        <v>-31.4584</v>
       </c>
       <c r="T9" t="n">
-        <v>16.9479</v>
+        <v>-18.6324</v>
       </c>
       <c r="U9" t="n">
-        <v>-1.5481</v>
+        <v>-14.2807</v>
       </c>
       <c r="V9" t="n">
-        <v>-0.953</v>
+        <v>-16.2463</v>
       </c>
       <c r="W9" t="n">
-        <v>1.8403</v>
+        <v>-13.6116</v>
       </c>
       <c r="X9" t="n">
-        <v>5.905</v>
+        <v>31.5383</v>
       </c>
       <c r="Y9" t="n">
-        <v>-16.933</v>
+        <v>32.3002</v>
       </c>
       <c r="Z9" t="n">
-        <v>-17.5909</v>
+        <v>8.0564</v>
       </c>
       <c r="AA9" t="n">
-        <v>1.5327</v>
+        <v>14.3803</v>
       </c>
       <c r="AB9" t="n">
-        <v>0.9086</v>
+        <v>17.0143</v>
       </c>
       <c r="AC9" t="n">
-        <v>-1.8456</v>
+        <v>13.4191</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>230.85</v>
+        <v>210.62</v>
       </c>
       <c r="C10" t="n">
-        <v>233.69</v>
+        <v>222.19</v>
       </c>
       <c r="D10" t="n">
-        <v>181.81</v>
+        <v>201.69</v>
       </c>
       <c r="E10" t="n">
-        <v>182.54</v>
+        <v>211.44</v>
       </c>
       <c r="F10" t="n">
-        <v>81.56999999999999</v>
+        <v>76.86</v>
       </c>
       <c r="G10" t="n">
-        <v>82.08</v>
+        <v>78.47</v>
       </c>
       <c r="H10" t="n">
-        <v>72.68000000000001</v>
+        <v>75.38</v>
       </c>
       <c r="I10" t="n">
-        <v>73.05</v>
+        <v>76.27</v>
       </c>
       <c r="J10" t="n">
-        <v>5.7925</v>
+        <v>5.6442</v>
       </c>
       <c r="K10" t="n">
-        <v>6.7711</v>
+        <v>5.9803</v>
       </c>
       <c r="L10" t="n">
-        <v>5.7233</v>
+        <v>5.2093</v>
       </c>
       <c r="M10" t="n">
-        <v>6.7612</v>
+        <v>5.6245</v>
       </c>
       <c r="N10" t="n">
-        <v>39.42</v>
+        <v>40.2763</v>
       </c>
       <c r="O10" t="n">
-        <v>43.35</v>
+        <v>41.1228</v>
       </c>
       <c r="P10" t="n">
-        <v>39.18</v>
+        <v>39.3314</v>
       </c>
       <c r="Q10" t="n">
-        <v>43.19</v>
+        <v>40.611</v>
       </c>
       <c r="R10" t="n">
-        <v>-30.5139</v>
+        <v>15.8321</v>
       </c>
       <c r="S10" t="n">
-        <v>-31.4584</v>
+        <v>-24.6311</v>
       </c>
       <c r="T10" t="n">
-        <v>-18.6324</v>
+        <v>-6.8669</v>
       </c>
       <c r="U10" t="n">
-        <v>-14.2807</v>
+        <v>4.4079</v>
       </c>
       <c r="V10" t="n">
-        <v>-16.2463</v>
+        <v>-11.8877</v>
       </c>
       <c r="W10" t="n">
-        <v>-13.6116</v>
+        <v>-11.3552</v>
       </c>
       <c r="X10" t="n">
-        <v>31.5383</v>
+        <v>-16.8121</v>
       </c>
       <c r="Y10" t="n">
-        <v>32.3002</v>
+        <v>15.8854</v>
       </c>
       <c r="Z10" t="n">
-        <v>8.0564</v>
+        <v>-9.104900000000001</v>
       </c>
       <c r="AA10" t="n">
-        <v>14.3803</v>
+        <v>-4.4685</v>
       </c>
       <c r="AB10" t="n">
-        <v>17.0144</v>
+        <v>10.9439</v>
       </c>
       <c r="AC10" t="n">
-        <v>13.4191</v>
+        <v>10.2619</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>210.62</v>
+        <v>227.06</v>
       </c>
       <c r="C11" t="n">
-        <v>222.19</v>
+        <v>231.02</v>
       </c>
       <c r="D11" t="n">
-        <v>201.69</v>
+        <v>157.56</v>
       </c>
       <c r="E11" t="n">
-        <v>211.44</v>
+        <v>201.68</v>
       </c>
       <c r="F11" t="n">
-        <v>76.86</v>
+        <v>78.48</v>
       </c>
       <c r="G11" t="n">
-        <v>78.47</v>
+        <v>79.34</v>
       </c>
       <c r="H11" t="n">
-        <v>75.38</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="I11" t="n">
-        <v>76.27</v>
+        <v>73.72</v>
       </c>
       <c r="J11" t="n">
-        <v>5.6442</v>
+        <v>5.1895</v>
       </c>
       <c r="K11" t="n">
-        <v>5.9803</v>
+        <v>7.0281</v>
       </c>
       <c r="L11" t="n">
-        <v>5.2093</v>
+        <v>5.0808</v>
       </c>
       <c r="M11" t="n">
-        <v>5.6245</v>
+        <v>5.8617</v>
       </c>
       <c r="N11" t="n">
-        <v>40.92</v>
+        <v>39.4299</v>
       </c>
       <c r="O11" t="n">
-        <v>41.78</v>
+        <v>45.6505</v>
       </c>
       <c r="P11" t="n">
-        <v>39.96</v>
+        <v>38.9673</v>
       </c>
       <c r="Q11" t="n">
-        <v>41.26</v>
+        <v>41.9988</v>
       </c>
       <c r="R11" t="n">
-        <v>15.8321</v>
+        <v>-4.616</v>
       </c>
       <c r="S11" t="n">
-        <v>-24.6311</v>
+        <v>-23.228</v>
       </c>
       <c r="T11" t="n">
-        <v>-6.8669</v>
+        <v>-24.2716</v>
       </c>
       <c r="U11" t="n">
-        <v>4.4079</v>
+        <v>-3.3434</v>
       </c>
       <c r="V11" t="n">
-        <v>-11.8877</v>
+        <v>-13.4945</v>
       </c>
       <c r="W11" t="n">
-        <v>-11.3552</v>
+        <v>-15.4781</v>
       </c>
       <c r="X11" t="n">
-        <v>-16.8121</v>
+        <v>4.2173</v>
       </c>
       <c r="Y11" t="n">
-        <v>15.8854</v>
+        <v>14.0386</v>
       </c>
       <c r="Z11" t="n">
-        <v>-9.104900000000001</v>
+        <v>14.6991</v>
       </c>
       <c r="AA11" t="n">
-        <v>-4.4686</v>
+        <v>3.4173</v>
       </c>
       <c r="AB11" t="n">
-        <v>10.9438</v>
+        <v>13.0033</v>
       </c>
       <c r="AC11" t="n">
-        <v>10.2619</v>
+        <v>15.6055</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>227.06</v>
+        <v>191.54</v>
       </c>
       <c r="C12" t="n">
-        <v>231.02</v>
+        <v>212.99</v>
       </c>
       <c r="D12" t="n">
-        <v>157.56</v>
+        <v>177.3</v>
       </c>
       <c r="E12" t="n">
-        <v>201.68</v>
+        <v>180.65</v>
       </c>
       <c r="F12" t="n">
-        <v>78.48</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>79.34</v>
+        <v>74.7</v>
       </c>
       <c r="H12" t="n">
-        <v>66.79000000000001</v>
+        <v>69</v>
       </c>
       <c r="I12" t="n">
-        <v>73.72</v>
+        <v>69.27</v>
       </c>
       <c r="J12" t="n">
-        <v>5.1895</v>
+        <v>6.1681</v>
       </c>
       <c r="K12" t="n">
-        <v>7.0281</v>
+        <v>6.5734</v>
       </c>
       <c r="L12" t="n">
-        <v>5.0808</v>
+        <v>5.5355</v>
       </c>
       <c r="M12" t="n">
-        <v>5.8617</v>
+        <v>6.4943</v>
       </c>
       <c r="N12" t="n">
-        <v>40.06</v>
+        <v>43.1209</v>
       </c>
       <c r="O12" t="n">
-        <v>46.38</v>
+        <v>44.676</v>
       </c>
       <c r="P12" t="n">
-        <v>39.59</v>
+        <v>41.4082</v>
       </c>
       <c r="Q12" t="n">
-        <v>42.67</v>
+        <v>44.5382</v>
       </c>
       <c r="R12" t="n">
-        <v>-4.616</v>
+        <v>-10.4274</v>
       </c>
       <c r="S12" t="n">
-        <v>-23.228</v>
+        <v>-1.0354</v>
       </c>
       <c r="T12" t="n">
-        <v>-24.2716</v>
+        <v>-35.6063</v>
       </c>
       <c r="U12" t="n">
-        <v>-3.3434</v>
+        <v>-6.0364</v>
       </c>
       <c r="V12" t="n">
-        <v>-13.4945</v>
+        <v>-5.1745</v>
       </c>
       <c r="W12" t="n">
-        <v>-15.4781</v>
+        <v>-19.9746</v>
       </c>
       <c r="X12" t="n">
-        <v>4.2173</v>
+        <v>10.7921</v>
       </c>
       <c r="Y12" t="n">
-        <v>14.0386</v>
+        <v>-3.9475</v>
       </c>
       <c r="Z12" t="n">
-        <v>14.6991</v>
+        <v>33.8065</v>
       </c>
       <c r="AA12" t="n">
-        <v>3.4174</v>
+        <v>6.0464</v>
       </c>
       <c r="AB12" t="n">
-        <v>13.0032</v>
+        <v>4.7696</v>
       </c>
       <c r="AC12" t="n">
-        <v>15.6055</v>
+        <v>21.6724</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>191.54</v>
+        <v>192.3</v>
       </c>
       <c r="C13" t="n">
-        <v>212.99</v>
+        <v>225.63</v>
       </c>
       <c r="D13" t="n">
-        <v>177.3</v>
+        <v>192.3</v>
       </c>
       <c r="E13" t="n">
-        <v>180.65</v>
+        <v>223.99</v>
       </c>
       <c r="F13" t="n">
-        <v>71.68000000000001</v>
+        <v>70.89</v>
       </c>
       <c r="G13" t="n">
-        <v>74.7</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>69</v>
+        <v>69.59</v>
       </c>
       <c r="I13" t="n">
-        <v>69.27</v>
+        <v>76.01000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>6.1681</v>
+        <v>6.0298</v>
       </c>
       <c r="K13" t="n">
-        <v>6.5734</v>
+        <v>6.0298</v>
       </c>
       <c r="L13" t="n">
-        <v>5.5355</v>
+        <v>4.8436</v>
       </c>
       <c r="M13" t="n">
-        <v>6.4943</v>
+        <v>4.9128</v>
       </c>
       <c r="N13" t="n">
-        <v>43.81</v>
+        <v>43.4851</v>
       </c>
       <c r="O13" t="n">
-        <v>45.39</v>
+        <v>44.302</v>
       </c>
       <c r="P13" t="n">
-        <v>42.07</v>
+        <v>39.8039</v>
       </c>
       <c r="Q13" t="n">
-        <v>45.25</v>
+        <v>40.1878</v>
       </c>
       <c r="R13" t="n">
-        <v>-10.4274</v>
+        <v>23.9911</v>
       </c>
       <c r="S13" t="n">
-        <v>-1.0354</v>
+        <v>5.9355</v>
       </c>
       <c r="T13" t="n">
-        <v>-35.6063</v>
+        <v>-14.7354</v>
       </c>
       <c r="U13" t="n">
-        <v>-6.0364</v>
+        <v>9.73</v>
       </c>
       <c r="V13" t="n">
-        <v>-5.1745</v>
+        <v>-0.3409</v>
       </c>
       <c r="W13" t="n">
-        <v>-19.9746</v>
+        <v>-10.8073</v>
       </c>
       <c r="X13" t="n">
-        <v>10.7921</v>
+        <v>-24.3521</v>
       </c>
       <c r="Y13" t="n">
-        <v>-3.9475</v>
+        <v>-12.6536</v>
       </c>
       <c r="Z13" t="n">
-        <v>33.8065</v>
+        <v>-4.4221</v>
       </c>
       <c r="AA13" t="n">
-        <v>6.0464</v>
+        <v>-9.767799999999999</v>
       </c>
       <c r="AB13" t="n">
-        <v>4.7696</v>
+        <v>-1.0421</v>
       </c>
       <c r="AC13" t="n">
-        <v>21.6725</v>
+        <v>8.1305</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>192.3</v>
+        <v>222.22</v>
       </c>
       <c r="C14" t="n">
-        <v>225.63</v>
+        <v>242.4</v>
       </c>
       <c r="D14" t="n">
-        <v>192.3</v>
+        <v>214.74</v>
       </c>
       <c r="E14" t="n">
-        <v>223.99</v>
+        <v>234.68</v>
       </c>
       <c r="F14" t="n">
-        <v>70.89</v>
+        <v>76.34</v>
       </c>
       <c r="G14" t="n">
-        <v>76.59999999999999</v>
+        <v>78.36</v>
       </c>
       <c r="H14" t="n">
-        <v>69.59</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="I14" t="n">
-        <v>76.01000000000001</v>
+        <v>77.52</v>
       </c>
       <c r="J14" t="n">
-        <v>6.0298</v>
+        <v>4.9523</v>
       </c>
       <c r="K14" t="n">
-        <v>6.0298</v>
+        <v>5.0907</v>
       </c>
       <c r="L14" t="n">
-        <v>4.8436</v>
+        <v>4.4877</v>
       </c>
       <c r="M14" t="n">
-        <v>4.9128</v>
+        <v>4.6656</v>
       </c>
       <c r="N14" t="n">
-        <v>44.18</v>
+        <v>40.0106</v>
       </c>
       <c r="O14" t="n">
-        <v>45.01</v>
+        <v>41.0933</v>
       </c>
       <c r="P14" t="n">
-        <v>40.44</v>
+        <v>38.9476</v>
       </c>
       <c r="Q14" t="n">
-        <v>40.83</v>
+        <v>39.4102</v>
       </c>
       <c r="R14" t="n">
-        <v>23.9911</v>
+        <v>4.7725</v>
       </c>
       <c r="S14" t="n">
-        <v>5.9355</v>
+        <v>16.3626</v>
       </c>
       <c r="T14" t="n">
-        <v>-14.7354</v>
+        <v>28.5636</v>
       </c>
       <c r="U14" t="n">
-        <v>9.73</v>
+        <v>1.9866</v>
       </c>
       <c r="V14" t="n">
-        <v>-0.3409</v>
+        <v>5.1546</v>
       </c>
       <c r="W14" t="n">
-        <v>-10.8073</v>
+        <v>6.1191</v>
       </c>
       <c r="X14" t="n">
-        <v>-24.3521</v>
+        <v>-5.0318</v>
       </c>
       <c r="Y14" t="n">
-        <v>-12.6536</v>
+        <v>-20.4053</v>
       </c>
       <c r="Z14" t="n">
-        <v>-4.4221</v>
+        <v>-30.9945</v>
       </c>
       <c r="AA14" t="n">
-        <v>-9.768000000000001</v>
+        <v>-1.9349</v>
       </c>
       <c r="AB14" t="n">
-        <v>-1.0422</v>
+        <v>-6.1635</v>
       </c>
       <c r="AC14" t="n">
-        <v>8.1303</v>
+        <v>-7.2932</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>222.22</v>
+        <v>265.99</v>
       </c>
       <c r="C15" t="n">
-        <v>242.4</v>
+        <v>274.88</v>
       </c>
       <c r="D15" t="n">
-        <v>214.74</v>
+        <v>261.6</v>
       </c>
       <c r="E15" t="n">
-        <v>234.68</v>
+        <v>272.5</v>
       </c>
       <c r="F15" t="n">
-        <v>76.34</v>
+        <v>82.88</v>
       </c>
       <c r="G15" t="n">
-        <v>78.36</v>
+        <v>85.03</v>
       </c>
       <c r="H15" t="n">
-        <v>74.29000000000001</v>
+        <v>82.64</v>
       </c>
       <c r="I15" t="n">
-        <v>77.52</v>
+        <v>84.59</v>
       </c>
       <c r="J15" t="n">
-        <v>4.9523</v>
+        <v>4.0231</v>
       </c>
       <c r="K15" t="n">
-        <v>5.0907</v>
+        <v>4.122</v>
       </c>
       <c r="L15" t="n">
-        <v>4.4877</v>
+        <v>3.865</v>
       </c>
       <c r="M15" t="n">
-        <v>4.6656</v>
+        <v>3.9045</v>
       </c>
       <c r="N15" t="n">
-        <v>40.65</v>
+        <v>36.6641</v>
       </c>
       <c r="O15" t="n">
-        <v>41.75</v>
+        <v>36.7723</v>
       </c>
       <c r="P15" t="n">
-        <v>39.57</v>
+        <v>35.5814</v>
       </c>
       <c r="Q15" t="n">
-        <v>40.04</v>
+        <v>35.7389</v>
       </c>
       <c r="R15" t="n">
-        <v>4.7725</v>
+        <v>16.1156</v>
       </c>
       <c r="S15" t="n">
-        <v>16.3626</v>
+        <v>50.8442</v>
       </c>
       <c r="T15" t="n">
-        <v>28.5636</v>
+        <v>28.8782</v>
       </c>
       <c r="U15" t="n">
-        <v>1.9866</v>
+        <v>9.120200000000001</v>
       </c>
       <c r="V15" t="n">
-        <v>5.1546</v>
+        <v>22.1164</v>
       </c>
       <c r="W15" t="n">
-        <v>6.1191</v>
+        <v>10.9086</v>
       </c>
       <c r="X15" t="n">
-        <v>-5.0318</v>
+        <v>-16.313</v>
       </c>
       <c r="Y15" t="n">
-        <v>-20.4053</v>
+        <v>-39.878</v>
       </c>
       <c r="Z15" t="n">
-        <v>-30.9945</v>
+        <v>-30.5805</v>
       </c>
       <c r="AA15" t="n">
-        <v>-1.9349</v>
+        <v>-9.3156</v>
       </c>
       <c r="AB15" t="n">
-        <v>-6.1636</v>
+        <v>-19.7567</v>
       </c>
       <c r="AC15" t="n">
-        <v>-7.2934</v>
+        <v>-11.997</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>265.99</v>
+        <v>267.13</v>
       </c>
       <c r="C16" t="n">
-        <v>274.88</v>
+        <v>274.93</v>
       </c>
       <c r="D16" t="n">
-        <v>261.6</v>
+        <v>226</v>
       </c>
       <c r="E16" t="n">
-        <v>272.5</v>
+        <v>226.19</v>
       </c>
       <c r="F16" t="n">
-        <v>82.88</v>
+        <v>84.19</v>
       </c>
       <c r="G16" t="n">
-        <v>85.03</v>
+        <v>84.83</v>
       </c>
       <c r="H16" t="n">
-        <v>82.64</v>
+        <v>79.86</v>
       </c>
       <c r="I16" t="n">
-        <v>84.59</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="J16" t="n">
-        <v>4.0231</v>
+        <v>3.9836</v>
       </c>
       <c r="K16" t="n">
-        <v>4.122</v>
+        <v>4.5965</v>
       </c>
       <c r="L16" t="n">
         <v>3.865</v>
       </c>
       <c r="M16" t="n">
-        <v>3.9045</v>
+        <v>4.5767</v>
       </c>
       <c r="N16" t="n">
-        <v>37.25</v>
+        <v>35.9652</v>
       </c>
       <c r="O16" t="n">
-        <v>37.36</v>
+        <v>37.7861</v>
       </c>
       <c r="P16" t="n">
-        <v>36.15</v>
+        <v>35.6896</v>
       </c>
       <c r="Q16" t="n">
-        <v>36.31</v>
+        <v>37.7468</v>
       </c>
       <c r="R16" t="n">
-        <v>16.1156</v>
+        <v>-16.9945</v>
       </c>
       <c r="S16" t="n">
-        <v>50.8442</v>
+        <v>0.9822</v>
       </c>
       <c r="T16" t="n">
-        <v>28.8782</v>
+        <v>12.1529</v>
       </c>
       <c r="U16" t="n">
-        <v>9.120200000000001</v>
+        <v>-5.5089</v>
       </c>
       <c r="V16" t="n">
-        <v>22.1164</v>
+        <v>5.1572</v>
       </c>
       <c r="W16" t="n">
-        <v>10.9086</v>
+        <v>8.4238</v>
       </c>
       <c r="X16" t="n">
-        <v>-16.313</v>
+        <v>17.216</v>
       </c>
       <c r="Y16" t="n">
-        <v>-39.878</v>
+        <v>-6.8413</v>
       </c>
       <c r="Z16" t="n">
-        <v>-30.5805</v>
+        <v>-21.922</v>
       </c>
       <c r="AA16" t="n">
-        <v>-9.3157</v>
+        <v>5.6182</v>
       </c>
       <c r="AB16" t="n">
-        <v>-19.7569</v>
+        <v>-6.074</v>
       </c>
       <c r="AC16" t="n">
-        <v>-11.9971</v>
+        <v>-10.1241</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>267.13</v>
+        <v>247.42</v>
       </c>
       <c r="C17" t="n">
-        <v>274.93</v>
+        <v>259.79</v>
       </c>
       <c r="D17" t="n">
-        <v>226</v>
+        <v>233.3</v>
       </c>
       <c r="E17" t="n">
-        <v>226.19</v>
+        <v>233.86</v>
       </c>
       <c r="F17" t="n">
-        <v>84.19</v>
+        <v>81.67</v>
       </c>
       <c r="G17" t="n">
-        <v>84.83</v>
+        <v>81.81</v>
       </c>
       <c r="H17" t="n">
-        <v>79.86</v>
+        <v>76.94</v>
       </c>
       <c r="I17" t="n">
-        <v>79.93000000000001</v>
+        <v>77.54000000000001</v>
       </c>
       <c r="J17" t="n">
-        <v>3.9836</v>
+        <v>4.122</v>
       </c>
       <c r="K17" t="n">
-        <v>4.5965</v>
+        <v>4.4086</v>
       </c>
       <c r="L17" t="n">
-        <v>3.865</v>
+        <v>3.8749</v>
       </c>
       <c r="M17" t="n">
-        <v>4.5767</v>
+        <v>4.4086</v>
       </c>
       <c r="N17" t="n">
-        <v>36.54</v>
+        <v>36.9397</v>
       </c>
       <c r="O17" t="n">
-        <v>38.39</v>
+        <v>39.1641</v>
       </c>
       <c r="P17" t="n">
-        <v>36.26</v>
+        <v>36.8708</v>
       </c>
       <c r="Q17" t="n">
-        <v>38.35</v>
+        <v>38.8984</v>
       </c>
       <c r="R17" t="n">
-        <v>-16.9945</v>
+        <v>3.391</v>
       </c>
       <c r="S17" t="n">
-        <v>0.9822</v>
+        <v>-0.3494</v>
       </c>
       <c r="T17" t="n">
-        <v>12.1529</v>
+        <v>29.4547</v>
       </c>
       <c r="U17" t="n">
-        <v>-5.5089</v>
+        <v>-2.9901</v>
       </c>
       <c r="V17" t="n">
-        <v>5.1572</v>
+        <v>0.0258</v>
       </c>
       <c r="W17" t="n">
-        <v>8.4238</v>
+        <v>11.9388</v>
       </c>
       <c r="X17" t="n">
-        <v>17.216</v>
+        <v>-3.673</v>
       </c>
       <c r="Y17" t="n">
-        <v>-6.8413</v>
+        <v>-5.5084</v>
       </c>
       <c r="Z17" t="n">
-        <v>-21.922</v>
+        <v>-32.1159</v>
       </c>
       <c r="AA17" t="n">
-        <v>5.6183</v>
+        <v>3.0509</v>
       </c>
       <c r="AB17" t="n">
-        <v>-6.074</v>
+        <v>-1.2986</v>
       </c>
       <c r="AC17" t="n">
-        <v>-10.1242</v>
+        <v>-12.6628</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>247.42</v>
+        <v>266.04</v>
       </c>
       <c r="C18" t="n">
-        <v>259.79</v>
+        <v>286.15</v>
       </c>
       <c r="D18" t="n">
-        <v>233.3</v>
+        <v>265</v>
       </c>
       <c r="E18" t="n">
-        <v>233.86</v>
+        <v>279.29</v>
       </c>
       <c r="F18" t="n">
-        <v>81.67</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="G18" t="n">
-        <v>81.81</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="H18" t="n">
-        <v>76.94</v>
+        <v>80.63</v>
       </c>
       <c r="I18" t="n">
-        <v>77.54000000000001</v>
+        <v>82.87</v>
       </c>
       <c r="J18" t="n">
-        <v>4.122</v>
+        <v>3.8156</v>
       </c>
       <c r="K18" t="n">
-        <v>4.4086</v>
+        <v>3.8254</v>
       </c>
       <c r="L18" t="n">
-        <v>3.8749</v>
+        <v>3.4103</v>
       </c>
       <c r="M18" t="n">
-        <v>4.4086</v>
+        <v>3.5487</v>
       </c>
       <c r="N18" t="n">
-        <v>37.53</v>
+        <v>36.6149</v>
       </c>
       <c r="O18" t="n">
-        <v>39.79</v>
+        <v>37.3531</v>
       </c>
       <c r="P18" t="n">
-        <v>37.46</v>
+        <v>35.857</v>
       </c>
       <c r="Q18" t="n">
-        <v>39.52</v>
+        <v>36.1719</v>
       </c>
       <c r="R18" t="n">
-        <v>3.391</v>
+        <v>19.4262</v>
       </c>
       <c r="S18" t="n">
-        <v>-0.3494</v>
+        <v>2.4917</v>
       </c>
       <c r="T18" t="n">
-        <v>29.4547</v>
+        <v>24.6886</v>
       </c>
       <c r="U18" t="n">
-        <v>-2.9901</v>
+        <v>6.8739</v>
       </c>
       <c r="V18" t="n">
-        <v>0.0258</v>
+        <v>-2.0333</v>
       </c>
       <c r="W18" t="n">
-        <v>11.9388</v>
+        <v>9.0251</v>
       </c>
       <c r="X18" t="n">
-        <v>-3.673</v>
+        <v>-19.5051</v>
       </c>
       <c r="Y18" t="n">
-        <v>-5.5084</v>
+        <v>-9.1126</v>
       </c>
       <c r="Z18" t="n">
-        <v>-32.1159</v>
+        <v>-27.7662</v>
       </c>
       <c r="AA18" t="n">
-        <v>3.0508</v>
+        <v>-7.0093</v>
       </c>
       <c r="AB18" t="n">
-        <v>-1.2987</v>
+        <v>1.2116</v>
       </c>
       <c r="AC18" t="n">
-        <v>-12.663</v>
+        <v>-9.992800000000001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>266.04</v>
+        <v>299.26</v>
       </c>
       <c r="C19" t="n">
-        <v>286.15</v>
+        <v>302</v>
       </c>
       <c r="D19" t="n">
-        <v>265</v>
+        <v>286.24</v>
       </c>
       <c r="E19" t="n">
-        <v>279.29</v>
+        <v>300.77</v>
       </c>
       <c r="F19" t="n">
-        <v>82.09999999999999</v>
+        <v>83.95</v>
       </c>
       <c r="G19" t="n">
-        <v>83.59999999999999</v>
+        <v>85.11</v>
       </c>
       <c r="H19" t="n">
-        <v>80.63</v>
+        <v>81.39</v>
       </c>
       <c r="I19" t="n">
-        <v>82.87</v>
+        <v>82.58</v>
       </c>
       <c r="J19" t="n">
-        <v>3.8156</v>
+        <v>3.2917</v>
       </c>
       <c r="K19" t="n">
-        <v>3.8254</v>
+        <v>3.4498</v>
       </c>
       <c r="L19" t="n">
-        <v>3.4103</v>
+        <v>3.2521</v>
       </c>
       <c r="M19" t="n">
-        <v>3.5487</v>
+        <v>3.262</v>
       </c>
       <c r="N19" t="n">
-        <v>37.2</v>
+        <v>35.7389</v>
       </c>
       <c r="O19" t="n">
-        <v>37.95</v>
+        <v>36.8511</v>
       </c>
       <c r="P19" t="n">
-        <v>36.43</v>
+        <v>35.2369</v>
       </c>
       <c r="Q19" t="n">
-        <v>36.75</v>
+        <v>36.3491</v>
       </c>
       <c r="R19" t="n">
-        <v>19.4262</v>
+        <v>7.6909</v>
       </c>
       <c r="S19" t="n">
-        <v>2.4917</v>
+        <v>32.9723</v>
       </c>
       <c r="T19" t="n">
-        <v>24.6886</v>
+        <v>28.1618</v>
       </c>
       <c r="U19" t="n">
-        <v>6.8739</v>
+        <v>-0.3499</v>
       </c>
       <c r="V19" t="n">
-        <v>-2.0333</v>
+        <v>3.3154</v>
       </c>
       <c r="W19" t="n">
-        <v>9.0251</v>
+        <v>6.5273</v>
       </c>
       <c r="X19" t="n">
-        <v>-19.5051</v>
+        <v>-8.079000000000001</v>
       </c>
       <c r="Y19" t="n">
-        <v>-9.1126</v>
+        <v>-28.7259</v>
       </c>
       <c r="Z19" t="n">
-        <v>-27.7662</v>
+        <v>-30.084</v>
       </c>
       <c r="AA19" t="n">
-        <v>-7.0091</v>
+        <v>0.4899</v>
       </c>
       <c r="AB19" t="n">
-        <v>1.2118</v>
+        <v>-3.7028</v>
       </c>
       <c r="AC19" t="n">
-        <v>-9.992699999999999</v>
+        <v>-7.7673</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>299.26</v>
+        <v>236</v>
       </c>
       <c r="C20" t="n">
-        <v>302</v>
+        <v>252.98</v>
       </c>
       <c r="D20" t="n">
-        <v>286.24</v>
+        <v>223</v>
       </c>
       <c r="E20" t="n">
-        <v>300.77</v>
+        <v>231.42</v>
       </c>
       <c r="F20" t="n">
-        <v>83.95</v>
+        <v>75.12</v>
       </c>
       <c r="G20" t="n">
-        <v>85.11</v>
+        <v>77.73999999999999</v>
       </c>
       <c r="H20" t="n">
-        <v>81.39</v>
+        <v>73.91</v>
       </c>
       <c r="I20" t="n">
-        <v>82.58</v>
+        <v>74.44</v>
       </c>
       <c r="J20" t="n">
-        <v>3.2917</v>
+        <v>3.99</v>
       </c>
       <c r="K20" t="n">
-        <v>3.4498</v>
+        <v>4.13</v>
       </c>
       <c r="L20" t="n">
-        <v>3.2521</v>
+        <v>3.8</v>
       </c>
       <c r="M20" t="n">
-        <v>3.262</v>
+        <v>4.04</v>
       </c>
       <c r="N20" t="n">
-        <v>36.31</v>
+        <v>39.6267</v>
       </c>
       <c r="O20" t="n">
-        <v>37.44</v>
+        <v>40.1582</v>
       </c>
       <c r="P20" t="n">
-        <v>35.8</v>
+        <v>38.4653</v>
       </c>
       <c r="Q20" t="n">
-        <v>36.93</v>
+        <v>39.922</v>
       </c>
       <c r="R20" t="n">
-        <v>7.6909</v>
+        <v>-23.0575</v>
       </c>
       <c r="S20" t="n">
-        <v>32.9723</v>
+        <v>-1.0434</v>
       </c>
       <c r="T20" t="n">
-        <v>28.1618</v>
+        <v>-15.0752</v>
       </c>
       <c r="U20" t="n">
-        <v>-0.3499</v>
+        <v>-9.857100000000001</v>
       </c>
       <c r="V20" t="n">
-        <v>3.3154</v>
+        <v>-3.9979</v>
       </c>
       <c r="W20" t="n">
-        <v>6.5273</v>
+        <v>-11.9991</v>
       </c>
       <c r="X20" t="n">
-        <v>-8.079000000000001</v>
+        <v>23.8504</v>
       </c>
       <c r="Y20" t="n">
-        <v>-28.7259</v>
+        <v>-8.360900000000001</v>
       </c>
       <c r="Z20" t="n">
-        <v>-30.084</v>
+        <v>3.4704</v>
       </c>
       <c r="AA20" t="n">
-        <v>0.4898</v>
+        <v>9.8294</v>
       </c>
       <c r="AB20" t="n">
-        <v>-3.7027</v>
+        <v>2.6315</v>
       </c>
       <c r="AC20" t="n">
-        <v>-7.7672</v>
+        <v>11.7046</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>236</v>
+        <v>233.11</v>
       </c>
       <c r="C21" t="n">
-        <v>252.98</v>
+        <v>237</v>
       </c>
       <c r="D21" t="n">
-        <v>223</v>
+        <v>211.13</v>
       </c>
       <c r="E21" t="n">
-        <v>231.42</v>
+        <v>229.57</v>
       </c>
       <c r="F21" t="n">
-        <v>75.12</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>77.73999999999999</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="H21" t="n">
-        <v>73.91</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="I21" t="n">
-        <v>74.44</v>
+        <v>73.3</v>
       </c>
       <c r="J21" t="n">
-        <v>3.99</v>
+        <v>4</v>
       </c>
       <c r="K21" t="n">
-        <v>4.13</v>
+        <v>4.39</v>
       </c>
       <c r="L21" t="n">
-        <v>3.8</v>
+        <v>3.92</v>
       </c>
       <c r="M21" t="n">
-        <v>4.04</v>
+        <v>4.08</v>
       </c>
       <c r="N21" t="n">
-        <v>40.26</v>
+        <v>39.66</v>
       </c>
       <c r="O21" t="n">
-        <v>40.8</v>
+        <v>41.49</v>
       </c>
       <c r="P21" t="n">
-        <v>39.08</v>
+        <v>38.9</v>
       </c>
       <c r="Q21" t="n">
-        <v>40.56</v>
+        <v>40.45</v>
       </c>
       <c r="R21" t="n">
-        <v>-23.0575</v>
+        <v>-0.7994</v>
       </c>
       <c r="S21" t="n">
-        <v>-1.0434</v>
+        <v>-17.8023</v>
       </c>
       <c r="T21" t="n">
-        <v>-15.0752</v>
+        <v>1.4943</v>
       </c>
       <c r="U21" t="n">
-        <v>-9.857100000000001</v>
+        <v>-1.5314</v>
       </c>
       <c r="V21" t="n">
-        <v>-3.9979</v>
+        <v>-11.5482</v>
       </c>
       <c r="W21" t="n">
-        <v>-11.9991</v>
+        <v>-8.2948</v>
       </c>
       <c r="X21" t="n">
-        <v>23.8504</v>
+        <v>0.9901</v>
       </c>
       <c r="Y21" t="n">
-        <v>-8.360900000000001</v>
+        <v>14.9717</v>
       </c>
       <c r="Z21" t="n">
-        <v>3.4704</v>
+        <v>-10.8528</v>
       </c>
       <c r="AA21" t="n">
-        <v>9.8294</v>
+        <v>1.3226</v>
       </c>
       <c r="AB21" t="n">
-        <v>2.6316</v>
+        <v>11.8271</v>
       </c>
       <c r="AC21" t="n">
-        <v>11.7048</v>
+        <v>7.1614</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>233.11</v>
+        <v>268.05</v>
       </c>
       <c r="C22" t="n">
-        <v>237</v>
+        <v>268.33</v>
       </c>
       <c r="D22" t="n">
-        <v>211.13</v>
+        <v>225.7441</v>
       </c>
       <c r="E22" t="n">
-        <v>229.57</v>
+        <v>252.61</v>
       </c>
       <c r="F22" t="n">
-        <v>74.78</v>
+        <v>77.94</v>
       </c>
       <c r="G22" t="n">
-        <v>76.18000000000001</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="H22" t="n">
-        <v>71.34999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I22" t="n">
-        <v>73.3</v>
+        <v>74.95</v>
       </c>
       <c r="J22" t="n">
-        <v>4</v>
+        <v>3.38</v>
       </c>
       <c r="K22" t="n">
-        <v>4.39</v>
+        <v>4.15</v>
       </c>
       <c r="L22" t="n">
-        <v>3.92</v>
+        <v>3.37</v>
       </c>
       <c r="M22" t="n">
-        <v>4.08</v>
+        <v>3.63</v>
       </c>
       <c r="N22" t="n">
-        <v>39.67</v>
+        <v>37.86</v>
       </c>
       <c r="O22" t="n">
-        <v>41.49</v>
+        <v>41.3699</v>
       </c>
       <c r="P22" t="n">
-        <v>38.9</v>
+        <v>37.7101</v>
       </c>
       <c r="Q22" t="n">
-        <v>40.45</v>
+        <v>39.47</v>
       </c>
       <c r="R22" t="n">
-        <v>-0.7994</v>
+        <v>10.0362</v>
       </c>
       <c r="S22" t="n">
-        <v>-17.8023</v>
+        <v>-16.0122</v>
       </c>
       <c r="T22" t="n">
-        <v>1.4943</v>
+        <v>8.0176</v>
       </c>
       <c r="U22" t="n">
-        <v>-1.5314</v>
+        <v>2.251</v>
       </c>
       <c r="V22" t="n">
-        <v>-11.5482</v>
+        <v>-9.2395</v>
       </c>
       <c r="W22" t="n">
-        <v>-8.2948</v>
+        <v>-3.3402</v>
       </c>
       <c r="X22" t="n">
-        <v>0.9901</v>
+        <v>-11.0294</v>
       </c>
       <c r="Y22" t="n">
-        <v>14.9717</v>
+        <v>11.2814</v>
       </c>
       <c r="Z22" t="n">
-        <v>-10.8528</v>
+        <v>-17.6609</v>
       </c>
       <c r="AA22" t="n">
-        <v>-0.2712</v>
+        <v>-2.4227</v>
       </c>
       <c r="AB22" t="n">
-        <v>10.068</v>
+        <v>8.585900000000001</v>
       </c>
       <c r="AC22" t="n">
-        <v>5.4759</v>
+        <v>1.4695</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-26 23:06
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>242.66</v>
+        <v>219</v>
       </c>
       <c r="C2" t="n">
-        <v>242.66</v>
+        <v>231.89</v>
       </c>
       <c r="D2" t="n">
-        <v>204</v>
+        <v>207.56</v>
       </c>
       <c r="E2" t="n">
-        <v>217.98</v>
+        <v>224.63</v>
       </c>
       <c r="F2" t="n">
-        <v>82.87</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>82.91</v>
+        <v>84.05</v>
       </c>
       <c r="H2" t="n">
-        <v>80.33</v>
+        <v>80.66</v>
       </c>
       <c r="I2" t="n">
-        <v>81.67</v>
+        <v>83.68000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>5.7629</v>
+        <v>6.4153</v>
       </c>
       <c r="K2" t="n">
-        <v>6.8304</v>
+        <v>6.7514</v>
       </c>
       <c r="L2" t="n">
-        <v>5.7629</v>
+        <v>6.0298</v>
       </c>
       <c r="M2" t="n">
-        <v>6.4548</v>
+        <v>6.2373</v>
       </c>
       <c r="N2" t="n">
-        <v>38.2586</v>
+        <v>38.7901</v>
       </c>
       <c r="O2" t="n">
-        <v>39.4594</v>
+        <v>39.3118</v>
       </c>
       <c r="P2" t="n">
-        <v>38.2487</v>
+        <v>37.6975</v>
       </c>
       <c r="Q2" t="n">
-        <v>38.8196</v>
+        <v>37.8649</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>219</v>
+        <v>231.82</v>
       </c>
       <c r="C3" t="n">
-        <v>231.89</v>
+        <v>239.07</v>
       </c>
       <c r="D3" t="n">
-        <v>207.56</v>
+        <v>218.56</v>
       </c>
       <c r="E3" t="n">
-        <v>224.63</v>
+        <v>224.34</v>
       </c>
       <c r="F3" t="n">
-        <v>81.73999999999999</v>
+        <v>84.41</v>
       </c>
       <c r="G3" t="n">
-        <v>84.05</v>
+        <v>85.7</v>
       </c>
       <c r="H3" t="n">
-        <v>80.66</v>
+        <v>83.53</v>
       </c>
       <c r="I3" t="n">
-        <v>83.68000000000001</v>
+        <v>84.56</v>
       </c>
       <c r="J3" t="n">
+        <v>6.0396</v>
+      </c>
+      <c r="K3" t="n">
         <v>6.4153</v>
       </c>
-      <c r="K3" t="n">
-        <v>6.7514</v>
-      </c>
       <c r="L3" t="n">
-        <v>6.0298</v>
+        <v>5.8419</v>
       </c>
       <c r="M3" t="n">
-        <v>6.2373</v>
+        <v>6.2571</v>
       </c>
       <c r="N3" t="n">
-        <v>38.7901</v>
+        <v>37.5499</v>
       </c>
       <c r="O3" t="n">
-        <v>39.3118</v>
+        <v>37.9535</v>
       </c>
       <c r="P3" t="n">
-        <v>37.6975</v>
+        <v>36.9692</v>
       </c>
       <c r="Q3" t="n">
-        <v>37.8649</v>
+        <v>37.481</v>
       </c>
       <c r="R3" t="n">
-        <v>3.0507</v>
+        <v>-0.1291</v>
       </c>
       <c r="U3" t="n">
-        <v>2.4611</v>
+        <v>1.0516</v>
       </c>
       <c r="X3" t="n">
-        <v>-3.3696</v>
+        <v>0.3174</v>
       </c>
       <c r="AA3" t="n">
-        <v>-2.4593</v>
+        <v>-1.0139</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>231.82</v>
+        <v>217.27</v>
       </c>
       <c r="C4" t="n">
-        <v>239.07</v>
+        <v>234.06</v>
       </c>
       <c r="D4" t="n">
-        <v>218.56</v>
+        <v>210.14</v>
       </c>
       <c r="E4" t="n">
-        <v>224.34</v>
+        <v>227.03</v>
       </c>
       <c r="F4" t="n">
-        <v>84.41</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>85.7</v>
+        <v>87.06</v>
       </c>
       <c r="H4" t="n">
-        <v>83.53</v>
+        <v>83.75</v>
       </c>
       <c r="I4" t="n">
-        <v>84.56</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>6.0396</v>
+        <v>6.4746</v>
       </c>
       <c r="K4" t="n">
-        <v>6.4153</v>
+        <v>6.6624</v>
       </c>
       <c r="L4" t="n">
-        <v>5.8419</v>
+        <v>5.9803</v>
       </c>
       <c r="M4" t="n">
-        <v>6.2571</v>
+        <v>6.1879</v>
       </c>
       <c r="N4" t="n">
-        <v>37.5499</v>
+        <v>37.668</v>
       </c>
       <c r="O4" t="n">
-        <v>37.9535</v>
+        <v>37.855</v>
       </c>
       <c r="P4" t="n">
-        <v>36.9692</v>
+        <v>36.3786</v>
       </c>
       <c r="Q4" t="n">
-        <v>37.481</v>
+        <v>36.8314</v>
       </c>
       <c r="R4" t="n">
-        <v>-0.1291</v>
+        <v>1.1991</v>
       </c>
       <c r="U4" t="n">
-        <v>1.0516</v>
+        <v>1.7502</v>
       </c>
       <c r="X4" t="n">
-        <v>0.3174</v>
+        <v>-1.1059</v>
       </c>
       <c r="AA4" t="n">
-        <v>-1.0139</v>
+        <v>-1.7331</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>217.27</v>
+        <v>243.18</v>
       </c>
       <c r="C5" t="n">
-        <v>234.06</v>
+        <v>267.08</v>
       </c>
       <c r="D5" t="n">
-        <v>210.14</v>
+        <v>238.82</v>
       </c>
       <c r="E5" t="n">
-        <v>227.03</v>
+        <v>266.32</v>
       </c>
       <c r="F5" t="n">
-        <v>84.15000000000001</v>
+        <v>85.94</v>
       </c>
       <c r="G5" t="n">
-        <v>87.06</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>83.75</v>
+        <v>84.83</v>
       </c>
       <c r="I5" t="n">
-        <v>86.04000000000001</v>
+        <v>87.22</v>
       </c>
       <c r="J5" t="n">
-        <v>6.4746</v>
+        <v>5.7332</v>
       </c>
       <c r="K5" t="n">
-        <v>6.6624</v>
+        <v>5.8617</v>
       </c>
       <c r="L5" t="n">
-        <v>5.9803</v>
+        <v>5.0907</v>
       </c>
       <c r="M5" t="n">
-        <v>6.1879</v>
+        <v>5.1105</v>
       </c>
       <c r="N5" t="n">
-        <v>37.668</v>
+        <v>36.8806</v>
       </c>
       <c r="O5" t="n">
-        <v>37.855</v>
+        <v>37.3531</v>
       </c>
       <c r="P5" t="n">
-        <v>36.3786</v>
+        <v>36.2802</v>
       </c>
       <c r="Q5" t="n">
-        <v>36.8314</v>
+        <v>36.3294</v>
       </c>
       <c r="R5" t="n">
-        <v>1.1991</v>
+        <v>17.3061</v>
       </c>
       <c r="S5" t="n">
-        <v>4.1518</v>
+        <v>18.5594</v>
       </c>
       <c r="U5" t="n">
-        <v>1.7502</v>
+        <v>1.3715</v>
       </c>
       <c r="V5" t="n">
-        <v>5.3508</v>
+        <v>4.2304</v>
       </c>
       <c r="X5" t="n">
-        <v>-1.1059</v>
+        <v>-17.4114</v>
       </c>
       <c r="Y5" t="n">
-        <v>-4.1349</v>
+        <v>-18.0655</v>
       </c>
       <c r="AA5" t="n">
-        <v>-1.7331</v>
+        <v>-1.363</v>
       </c>
       <c r="AB5" t="n">
-        <v>-5.1216</v>
+        <v>-4.0552</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>243.18</v>
+        <v>281.47</v>
       </c>
       <c r="C6" t="n">
-        <v>267.08</v>
+        <v>284.58</v>
       </c>
       <c r="D6" t="n">
-        <v>238.82</v>
+        <v>257.26</v>
       </c>
       <c r="E6" t="n">
-        <v>266.32</v>
+        <v>280.54</v>
       </c>
       <c r="F6" t="n">
-        <v>85.94</v>
+        <v>87.68000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>87.31999999999999</v>
+        <v>88.09</v>
       </c>
       <c r="H6" t="n">
-        <v>84.83</v>
+        <v>85.41</v>
       </c>
       <c r="I6" t="n">
-        <v>87.22</v>
+        <v>86.56</v>
       </c>
       <c r="J6" t="n">
-        <v>5.7332</v>
+        <v>4.8238</v>
       </c>
       <c r="K6" t="n">
-        <v>5.8617</v>
+        <v>5.2884</v>
       </c>
       <c r="L6" t="n">
-        <v>5.0907</v>
+        <v>4.7645</v>
       </c>
       <c r="M6" t="n">
-        <v>5.1105</v>
+        <v>4.8535</v>
       </c>
       <c r="N6" t="n">
-        <v>36.8806</v>
+        <v>36.1522</v>
       </c>
       <c r="O6" t="n">
-        <v>37.3531</v>
+        <v>37.0971</v>
       </c>
       <c r="P6" t="n">
-        <v>36.2802</v>
+        <v>35.9751</v>
       </c>
       <c r="Q6" t="n">
-        <v>36.3294</v>
+        <v>36.605</v>
       </c>
       <c r="R6" t="n">
-        <v>17.3061</v>
+        <v>5.3394</v>
       </c>
       <c r="S6" t="n">
-        <v>18.5594</v>
+        <v>25.0513</v>
       </c>
       <c r="U6" t="n">
-        <v>1.3715</v>
+        <v>-0.7567</v>
       </c>
       <c r="V6" t="n">
-        <v>4.2304</v>
+        <v>2.3652</v>
       </c>
       <c r="X6" t="n">
-        <v>-17.4114</v>
+        <v>-5.0289</v>
       </c>
       <c r="Y6" t="n">
-        <v>-18.0655</v>
+        <v>-22.4321</v>
       </c>
       <c r="AA6" t="n">
-        <v>-1.363</v>
+        <v>0.7586000000000001</v>
       </c>
       <c r="AB6" t="n">
-        <v>-4.0552</v>
+        <v>-2.3372</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>281.47</v>
+        <v>242.04</v>
       </c>
       <c r="C7" t="n">
-        <v>284.58</v>
+        <v>274.5</v>
       </c>
       <c r="D7" t="n">
-        <v>257.26</v>
+        <v>228.55</v>
       </c>
       <c r="E7" t="n">
-        <v>280.54</v>
+        <v>262.7</v>
       </c>
       <c r="F7" t="n">
-        <v>87.68000000000001</v>
+        <v>83.47</v>
       </c>
       <c r="G7" t="n">
-        <v>88.09</v>
+        <v>86.25</v>
       </c>
       <c r="H7" t="n">
-        <v>85.41</v>
+        <v>82.48</v>
       </c>
       <c r="I7" t="n">
-        <v>86.56</v>
+        <v>85.22</v>
       </c>
       <c r="J7" t="n">
-        <v>4.8238</v>
+        <v>5.5059</v>
       </c>
       <c r="K7" t="n">
-        <v>5.2884</v>
+        <v>5.7431</v>
       </c>
       <c r="L7" t="n">
-        <v>4.7645</v>
+        <v>4.9424</v>
       </c>
       <c r="M7" t="n">
-        <v>4.8535</v>
+        <v>5.1401</v>
       </c>
       <c r="N7" t="n">
-        <v>36.1522</v>
+        <v>37.9239</v>
       </c>
       <c r="O7" t="n">
-        <v>37.0971</v>
+        <v>38.3472</v>
       </c>
       <c r="P7" t="n">
-        <v>35.9751</v>
+        <v>36.7428</v>
       </c>
       <c r="Q7" t="n">
-        <v>36.605</v>
+        <v>37.166</v>
       </c>
       <c r="R7" t="n">
-        <v>5.3394</v>
+        <v>-6.3592</v>
       </c>
       <c r="S7" t="n">
-        <v>25.0513</v>
+        <v>15.7116</v>
       </c>
       <c r="T7" t="n">
-        <v>28.6999</v>
+        <v>16.9479</v>
       </c>
       <c r="U7" t="n">
-        <v>-0.7567</v>
+        <v>-1.5481</v>
       </c>
       <c r="V7" t="n">
-        <v>2.3652</v>
+        <v>-0.953</v>
       </c>
       <c r="W7" t="n">
-        <v>5.9875</v>
+        <v>1.8403</v>
       </c>
       <c r="X7" t="n">
-        <v>-5.0289</v>
+        <v>5.905</v>
       </c>
       <c r="Y7" t="n">
-        <v>-22.4321</v>
+        <v>-16.933</v>
       </c>
       <c r="Z7" t="n">
-        <v>-24.8079</v>
+        <v>-17.5909</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.7586000000000001</v>
+        <v>1.5326</v>
       </c>
       <c r="AB7" t="n">
-        <v>-2.3372</v>
+        <v>0.9085</v>
       </c>
       <c r="AC7" t="n">
-        <v>-5.7049</v>
+        <v>-1.8458</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>242.04</v>
+        <v>230.85</v>
       </c>
       <c r="C8" t="n">
-        <v>274.5</v>
+        <v>233.69</v>
       </c>
       <c r="D8" t="n">
-        <v>228.55</v>
+        <v>181.81</v>
       </c>
       <c r="E8" t="n">
-        <v>262.7</v>
+        <v>182.54</v>
       </c>
       <c r="F8" t="n">
-        <v>83.47</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>86.25</v>
+        <v>82.08</v>
       </c>
       <c r="H8" t="n">
-        <v>82.48</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="I8" t="n">
-        <v>85.22</v>
+        <v>73.05</v>
       </c>
       <c r="J8" t="n">
-        <v>5.5059</v>
+        <v>5.7925</v>
       </c>
       <c r="K8" t="n">
-        <v>5.7431</v>
+        <v>6.7711</v>
       </c>
       <c r="L8" t="n">
-        <v>4.9424</v>
+        <v>5.7233</v>
       </c>
       <c r="M8" t="n">
-        <v>5.1401</v>
+        <v>6.7612</v>
       </c>
       <c r="N8" t="n">
-        <v>37.9239</v>
+        <v>38.7999</v>
       </c>
       <c r="O8" t="n">
-        <v>38.3472</v>
+        <v>42.6681</v>
       </c>
       <c r="P8" t="n">
-        <v>36.7428</v>
+        <v>38.5637</v>
       </c>
       <c r="Q8" t="n">
-        <v>37.166</v>
+        <v>42.5106</v>
       </c>
       <c r="R8" t="n">
-        <v>-6.3592</v>
+        <v>-30.5139</v>
       </c>
       <c r="S8" t="n">
-        <v>15.7116</v>
+        <v>-31.4584</v>
       </c>
       <c r="T8" t="n">
-        <v>16.9479</v>
+        <v>-18.6324</v>
       </c>
       <c r="U8" t="n">
-        <v>-1.5481</v>
+        <v>-14.2807</v>
       </c>
       <c r="V8" t="n">
-        <v>-0.953</v>
+        <v>-16.2463</v>
       </c>
       <c r="W8" t="n">
-        <v>1.8403</v>
+        <v>-13.6116</v>
       </c>
       <c r="X8" t="n">
-        <v>5.905</v>
+        <v>31.5383</v>
       </c>
       <c r="Y8" t="n">
-        <v>-16.933</v>
+        <v>32.3002</v>
       </c>
       <c r="Z8" t="n">
-        <v>-17.5909</v>
+        <v>8.0564</v>
       </c>
       <c r="AA8" t="n">
-        <v>1.5326</v>
+        <v>14.3803</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.9085</v>
+        <v>17.0143</v>
       </c>
       <c r="AC8" t="n">
-        <v>-1.8458</v>
+        <v>13.4191</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>230.85</v>
+        <v>210.62</v>
       </c>
       <c r="C9" t="n">
-        <v>233.69</v>
+        <v>222.19</v>
       </c>
       <c r="D9" t="n">
-        <v>181.81</v>
+        <v>201.69</v>
       </c>
       <c r="E9" t="n">
-        <v>182.54</v>
+        <v>211.44</v>
       </c>
       <c r="F9" t="n">
-        <v>81.56999999999999</v>
+        <v>76.86</v>
       </c>
       <c r="G9" t="n">
-        <v>82.08</v>
+        <v>78.47</v>
       </c>
       <c r="H9" t="n">
-        <v>72.68000000000001</v>
+        <v>75.38</v>
       </c>
       <c r="I9" t="n">
-        <v>73.05</v>
+        <v>76.27</v>
       </c>
       <c r="J9" t="n">
-        <v>5.7925</v>
+        <v>5.6442</v>
       </c>
       <c r="K9" t="n">
-        <v>6.7711</v>
+        <v>5.9803</v>
       </c>
       <c r="L9" t="n">
-        <v>5.7233</v>
+        <v>5.2093</v>
       </c>
       <c r="M9" t="n">
-        <v>6.7612</v>
+        <v>5.6245</v>
       </c>
       <c r="N9" t="n">
-        <v>38.7999</v>
+        <v>40.2763</v>
       </c>
       <c r="O9" t="n">
-        <v>42.6681</v>
+        <v>41.1228</v>
       </c>
       <c r="P9" t="n">
-        <v>38.5637</v>
+        <v>39.3314</v>
       </c>
       <c r="Q9" t="n">
-        <v>42.5106</v>
+        <v>40.611</v>
       </c>
       <c r="R9" t="n">
-        <v>-30.5139</v>
+        <v>15.8321</v>
       </c>
       <c r="S9" t="n">
-        <v>-31.4584</v>
+        <v>-24.6311</v>
       </c>
       <c r="T9" t="n">
-        <v>-18.6324</v>
+        <v>-6.8669</v>
       </c>
       <c r="U9" t="n">
-        <v>-14.2807</v>
+        <v>4.4079</v>
       </c>
       <c r="V9" t="n">
-        <v>-16.2463</v>
+        <v>-11.8877</v>
       </c>
       <c r="W9" t="n">
-        <v>-13.6116</v>
+        <v>-11.3552</v>
       </c>
       <c r="X9" t="n">
-        <v>31.5383</v>
+        <v>-16.8121</v>
       </c>
       <c r="Y9" t="n">
-        <v>32.3002</v>
+        <v>15.8854</v>
       </c>
       <c r="Z9" t="n">
-        <v>8.0564</v>
+        <v>-9.104900000000001</v>
       </c>
       <c r="AA9" t="n">
-        <v>14.3803</v>
+        <v>-4.4685</v>
       </c>
       <c r="AB9" t="n">
-        <v>17.0143</v>
+        <v>10.9439</v>
       </c>
       <c r="AC9" t="n">
-        <v>13.4191</v>
+        <v>10.2619</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>210.62</v>
+        <v>227.06</v>
       </c>
       <c r="C10" t="n">
-        <v>222.19</v>
+        <v>231.02</v>
       </c>
       <c r="D10" t="n">
-        <v>201.69</v>
+        <v>157.56</v>
       </c>
       <c r="E10" t="n">
-        <v>211.44</v>
+        <v>201.68</v>
       </c>
       <c r="F10" t="n">
-        <v>76.86</v>
+        <v>78.48</v>
       </c>
       <c r="G10" t="n">
-        <v>78.47</v>
+        <v>79.34</v>
       </c>
       <c r="H10" t="n">
-        <v>75.38</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="I10" t="n">
-        <v>76.27</v>
+        <v>73.72</v>
       </c>
       <c r="J10" t="n">
-        <v>5.6442</v>
+        <v>5.1895</v>
       </c>
       <c r="K10" t="n">
-        <v>5.9803</v>
+        <v>7.0281</v>
       </c>
       <c r="L10" t="n">
-        <v>5.2093</v>
+        <v>5.0808</v>
       </c>
       <c r="M10" t="n">
-        <v>5.6245</v>
+        <v>5.8617</v>
       </c>
       <c r="N10" t="n">
-        <v>40.2763</v>
+        <v>39.4299</v>
       </c>
       <c r="O10" t="n">
-        <v>41.1228</v>
+        <v>45.6505</v>
       </c>
       <c r="P10" t="n">
-        <v>39.3314</v>
+        <v>38.9673</v>
       </c>
       <c r="Q10" t="n">
-        <v>40.611</v>
+        <v>41.9988</v>
       </c>
       <c r="R10" t="n">
-        <v>15.8321</v>
+        <v>-4.616</v>
       </c>
       <c r="S10" t="n">
-        <v>-24.6311</v>
+        <v>-23.228</v>
       </c>
       <c r="T10" t="n">
-        <v>-6.8669</v>
+        <v>-24.2716</v>
       </c>
       <c r="U10" t="n">
-        <v>4.4079</v>
+        <v>-3.3434</v>
       </c>
       <c r="V10" t="n">
-        <v>-11.8877</v>
+        <v>-13.4945</v>
       </c>
       <c r="W10" t="n">
-        <v>-11.3552</v>
+        <v>-15.4781</v>
       </c>
       <c r="X10" t="n">
-        <v>-16.8121</v>
+        <v>4.2173</v>
       </c>
       <c r="Y10" t="n">
-        <v>15.8854</v>
+        <v>14.0386</v>
       </c>
       <c r="Z10" t="n">
-        <v>-9.104900000000001</v>
+        <v>14.6991</v>
       </c>
       <c r="AA10" t="n">
-        <v>-4.4685</v>
+        <v>3.4173</v>
       </c>
       <c r="AB10" t="n">
-        <v>10.9439</v>
+        <v>13.0033</v>
       </c>
       <c r="AC10" t="n">
-        <v>10.2619</v>
+        <v>15.6055</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>227.06</v>
+        <v>191.54</v>
       </c>
       <c r="C11" t="n">
-        <v>231.02</v>
+        <v>212.99</v>
       </c>
       <c r="D11" t="n">
-        <v>157.56</v>
+        <v>177.3</v>
       </c>
       <c r="E11" t="n">
-        <v>201.68</v>
+        <v>180.65</v>
       </c>
       <c r="F11" t="n">
-        <v>78.48</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>79.34</v>
+        <v>74.7</v>
       </c>
       <c r="H11" t="n">
-        <v>66.79000000000001</v>
+        <v>69</v>
       </c>
       <c r="I11" t="n">
-        <v>73.72</v>
+        <v>69.27</v>
       </c>
       <c r="J11" t="n">
-        <v>5.1895</v>
+        <v>6.1681</v>
       </c>
       <c r="K11" t="n">
-        <v>7.0281</v>
+        <v>6.5734</v>
       </c>
       <c r="L11" t="n">
-        <v>5.0808</v>
+        <v>5.5355</v>
       </c>
       <c r="M11" t="n">
-        <v>5.8617</v>
+        <v>6.4943</v>
       </c>
       <c r="N11" t="n">
-        <v>39.4299</v>
+        <v>43.1209</v>
       </c>
       <c r="O11" t="n">
-        <v>45.6505</v>
+        <v>44.676</v>
       </c>
       <c r="P11" t="n">
-        <v>38.9673</v>
+        <v>41.4082</v>
       </c>
       <c r="Q11" t="n">
-        <v>41.9988</v>
+        <v>44.5382</v>
       </c>
       <c r="R11" t="n">
-        <v>-4.616</v>
+        <v>-10.4274</v>
       </c>
       <c r="S11" t="n">
-        <v>-23.228</v>
+        <v>-1.0354</v>
       </c>
       <c r="T11" t="n">
-        <v>-24.2716</v>
+        <v>-35.6063</v>
       </c>
       <c r="U11" t="n">
-        <v>-3.3434</v>
+        <v>-6.0364</v>
       </c>
       <c r="V11" t="n">
-        <v>-13.4945</v>
+        <v>-5.1745</v>
       </c>
       <c r="W11" t="n">
-        <v>-15.4781</v>
+        <v>-19.9746</v>
       </c>
       <c r="X11" t="n">
-        <v>4.2173</v>
+        <v>10.7921</v>
       </c>
       <c r="Y11" t="n">
-        <v>14.0386</v>
+        <v>-3.9475</v>
       </c>
       <c r="Z11" t="n">
-        <v>14.6991</v>
+        <v>33.8065</v>
       </c>
       <c r="AA11" t="n">
-        <v>3.4173</v>
+        <v>6.0464</v>
       </c>
       <c r="AB11" t="n">
-        <v>13.0033</v>
+        <v>4.7696</v>
       </c>
       <c r="AC11" t="n">
-        <v>15.6055</v>
+        <v>21.6724</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>191.54</v>
+        <v>192.3</v>
       </c>
       <c r="C12" t="n">
-        <v>212.99</v>
+        <v>225.63</v>
       </c>
       <c r="D12" t="n">
-        <v>177.3</v>
+        <v>192.3</v>
       </c>
       <c r="E12" t="n">
-        <v>180.65</v>
+        <v>223.99</v>
       </c>
       <c r="F12" t="n">
-        <v>71.68000000000001</v>
+        <v>70.89</v>
       </c>
       <c r="G12" t="n">
-        <v>74.7</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>69</v>
+        <v>69.59</v>
       </c>
       <c r="I12" t="n">
-        <v>69.27</v>
+        <v>76.01000000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>6.1681</v>
+        <v>6.0298</v>
       </c>
       <c r="K12" t="n">
-        <v>6.5734</v>
+        <v>6.0298</v>
       </c>
       <c r="L12" t="n">
-        <v>5.5355</v>
+        <v>4.8436</v>
       </c>
       <c r="M12" t="n">
-        <v>6.4943</v>
+        <v>4.9128</v>
       </c>
       <c r="N12" t="n">
-        <v>43.1209</v>
+        <v>43.4851</v>
       </c>
       <c r="O12" t="n">
-        <v>44.676</v>
+        <v>44.302</v>
       </c>
       <c r="P12" t="n">
-        <v>41.4082</v>
+        <v>39.8039</v>
       </c>
       <c r="Q12" t="n">
-        <v>44.5382</v>
+        <v>40.1878</v>
       </c>
       <c r="R12" t="n">
-        <v>-10.4274</v>
+        <v>23.9911</v>
       </c>
       <c r="S12" t="n">
-        <v>-1.0354</v>
+        <v>5.9355</v>
       </c>
       <c r="T12" t="n">
-        <v>-35.6063</v>
+        <v>-14.7354</v>
       </c>
       <c r="U12" t="n">
-        <v>-6.0364</v>
+        <v>9.73</v>
       </c>
       <c r="V12" t="n">
-        <v>-5.1745</v>
+        <v>-0.3409</v>
       </c>
       <c r="W12" t="n">
-        <v>-19.9746</v>
+        <v>-10.8073</v>
       </c>
       <c r="X12" t="n">
-        <v>10.7921</v>
+        <v>-24.3521</v>
       </c>
       <c r="Y12" t="n">
-        <v>-3.9475</v>
+        <v>-12.6536</v>
       </c>
       <c r="Z12" t="n">
-        <v>33.8065</v>
+        <v>-4.4221</v>
       </c>
       <c r="AA12" t="n">
-        <v>6.0464</v>
+        <v>-9.767799999999999</v>
       </c>
       <c r="AB12" t="n">
-        <v>4.7696</v>
+        <v>-1.0421</v>
       </c>
       <c r="AC12" t="n">
-        <v>21.6724</v>
+        <v>8.1305</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>192.3</v>
+        <v>222.22</v>
       </c>
       <c r="C13" t="n">
-        <v>225.63</v>
+        <v>242.4</v>
       </c>
       <c r="D13" t="n">
-        <v>192.3</v>
+        <v>214.74</v>
       </c>
       <c r="E13" t="n">
-        <v>223.99</v>
+        <v>234.68</v>
       </c>
       <c r="F13" t="n">
-        <v>70.89</v>
+        <v>76.34</v>
       </c>
       <c r="G13" t="n">
-        <v>76.59999999999999</v>
+        <v>78.36</v>
       </c>
       <c r="H13" t="n">
-        <v>69.59</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="I13" t="n">
-        <v>76.01000000000001</v>
+        <v>77.52</v>
       </c>
       <c r="J13" t="n">
-        <v>6.0298</v>
+        <v>4.9523</v>
       </c>
       <c r="K13" t="n">
-        <v>6.0298</v>
+        <v>5.0907</v>
       </c>
       <c r="L13" t="n">
-        <v>4.8436</v>
+        <v>4.4877</v>
       </c>
       <c r="M13" t="n">
-        <v>4.9128</v>
+        <v>4.6656</v>
       </c>
       <c r="N13" t="n">
-        <v>43.4851</v>
+        <v>40.0106</v>
       </c>
       <c r="O13" t="n">
-        <v>44.302</v>
+        <v>41.0933</v>
       </c>
       <c r="P13" t="n">
-        <v>39.8039</v>
+        <v>38.9476</v>
       </c>
       <c r="Q13" t="n">
-        <v>40.1878</v>
+        <v>39.4102</v>
       </c>
       <c r="R13" t="n">
-        <v>23.9911</v>
+        <v>4.7725</v>
       </c>
       <c r="S13" t="n">
-        <v>5.9355</v>
+        <v>16.3626</v>
       </c>
       <c r="T13" t="n">
-        <v>-14.7354</v>
+        <v>28.5636</v>
       </c>
       <c r="U13" t="n">
-        <v>9.73</v>
+        <v>1.9866</v>
       </c>
       <c r="V13" t="n">
-        <v>-0.3409</v>
+        <v>5.1546</v>
       </c>
       <c r="W13" t="n">
-        <v>-10.8073</v>
+        <v>6.1191</v>
       </c>
       <c r="X13" t="n">
-        <v>-24.3521</v>
+        <v>-5.0318</v>
       </c>
       <c r="Y13" t="n">
-        <v>-12.6536</v>
+        <v>-20.4053</v>
       </c>
       <c r="Z13" t="n">
-        <v>-4.4221</v>
+        <v>-30.9945</v>
       </c>
       <c r="AA13" t="n">
-        <v>-9.767799999999999</v>
+        <v>-1.9349</v>
       </c>
       <c r="AB13" t="n">
-        <v>-1.0421</v>
+        <v>-6.1635</v>
       </c>
       <c r="AC13" t="n">
-        <v>8.1305</v>
+        <v>-7.2932</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>222.22</v>
+        <v>265.99</v>
       </c>
       <c r="C14" t="n">
-        <v>242.4</v>
+        <v>274.88</v>
       </c>
       <c r="D14" t="n">
-        <v>214.74</v>
+        <v>261.6</v>
       </c>
       <c r="E14" t="n">
-        <v>234.68</v>
+        <v>272.5</v>
       </c>
       <c r="F14" t="n">
-        <v>76.34</v>
+        <v>82.88</v>
       </c>
       <c r="G14" t="n">
-        <v>78.36</v>
+        <v>85.03</v>
       </c>
       <c r="H14" t="n">
-        <v>74.29000000000001</v>
+        <v>82.64</v>
       </c>
       <c r="I14" t="n">
-        <v>77.52</v>
+        <v>84.59</v>
       </c>
       <c r="J14" t="n">
-        <v>4.9523</v>
+        <v>4.0231</v>
       </c>
       <c r="K14" t="n">
-        <v>5.0907</v>
+        <v>4.122</v>
       </c>
       <c r="L14" t="n">
-        <v>4.4877</v>
+        <v>3.865</v>
       </c>
       <c r="M14" t="n">
-        <v>4.6656</v>
+        <v>3.9045</v>
       </c>
       <c r="N14" t="n">
-        <v>40.0106</v>
+        <v>36.6641</v>
       </c>
       <c r="O14" t="n">
-        <v>41.0933</v>
+        <v>36.7723</v>
       </c>
       <c r="P14" t="n">
-        <v>38.9476</v>
+        <v>35.5814</v>
       </c>
       <c r="Q14" t="n">
-        <v>39.4102</v>
+        <v>35.7389</v>
       </c>
       <c r="R14" t="n">
-        <v>4.7725</v>
+        <v>16.1156</v>
       </c>
       <c r="S14" t="n">
-        <v>16.3626</v>
+        <v>50.8442</v>
       </c>
       <c r="T14" t="n">
-        <v>28.5636</v>
+        <v>28.8782</v>
       </c>
       <c r="U14" t="n">
-        <v>1.9866</v>
+        <v>9.120200000000001</v>
       </c>
       <c r="V14" t="n">
-        <v>5.1546</v>
+        <v>22.1164</v>
       </c>
       <c r="W14" t="n">
-        <v>6.1191</v>
+        <v>10.9086</v>
       </c>
       <c r="X14" t="n">
-        <v>-5.0318</v>
+        <v>-16.313</v>
       </c>
       <c r="Y14" t="n">
-        <v>-20.4053</v>
+        <v>-39.878</v>
       </c>
       <c r="Z14" t="n">
-        <v>-30.9945</v>
+        <v>-30.5805</v>
       </c>
       <c r="AA14" t="n">
-        <v>-1.9349</v>
+        <v>-9.3156</v>
       </c>
       <c r="AB14" t="n">
-        <v>-6.1635</v>
+        <v>-19.7567</v>
       </c>
       <c r="AC14" t="n">
-        <v>-7.2932</v>
+        <v>-11.997</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>265.99</v>
+        <v>267.13</v>
       </c>
       <c r="C15" t="n">
-        <v>274.88</v>
+        <v>274.93</v>
       </c>
       <c r="D15" t="n">
-        <v>261.6</v>
+        <v>226</v>
       </c>
       <c r="E15" t="n">
-        <v>272.5</v>
+        <v>226.19</v>
       </c>
       <c r="F15" t="n">
-        <v>82.88</v>
+        <v>84.19</v>
       </c>
       <c r="G15" t="n">
-        <v>85.03</v>
+        <v>84.83</v>
       </c>
       <c r="H15" t="n">
-        <v>82.64</v>
+        <v>79.86</v>
       </c>
       <c r="I15" t="n">
-        <v>84.59</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="J15" t="n">
-        <v>4.0231</v>
+        <v>3.9836</v>
       </c>
       <c r="K15" t="n">
-        <v>4.122</v>
+        <v>4.5965</v>
       </c>
       <c r="L15" t="n">
         <v>3.865</v>
       </c>
       <c r="M15" t="n">
-        <v>3.9045</v>
+        <v>4.5767</v>
       </c>
       <c r="N15" t="n">
-        <v>36.6641</v>
+        <v>35.9652</v>
       </c>
       <c r="O15" t="n">
-        <v>36.7723</v>
+        <v>37.7861</v>
       </c>
       <c r="P15" t="n">
-        <v>35.5814</v>
+        <v>35.6896</v>
       </c>
       <c r="Q15" t="n">
-        <v>35.7389</v>
+        <v>37.7468</v>
       </c>
       <c r="R15" t="n">
-        <v>16.1156</v>
+        <v>-16.9945</v>
       </c>
       <c r="S15" t="n">
-        <v>50.8442</v>
+        <v>0.9822</v>
       </c>
       <c r="T15" t="n">
-        <v>28.8782</v>
+        <v>12.1529</v>
       </c>
       <c r="U15" t="n">
-        <v>9.120200000000001</v>
+        <v>-5.5089</v>
       </c>
       <c r="V15" t="n">
-        <v>22.1164</v>
+        <v>5.1572</v>
       </c>
       <c r="W15" t="n">
-        <v>10.9086</v>
+        <v>8.4238</v>
       </c>
       <c r="X15" t="n">
-        <v>-16.313</v>
+        <v>17.216</v>
       </c>
       <c r="Y15" t="n">
-        <v>-39.878</v>
+        <v>-6.8413</v>
       </c>
       <c r="Z15" t="n">
-        <v>-30.5805</v>
+        <v>-21.922</v>
       </c>
       <c r="AA15" t="n">
-        <v>-9.3156</v>
+        <v>5.6182</v>
       </c>
       <c r="AB15" t="n">
-        <v>-19.7567</v>
+        <v>-6.074</v>
       </c>
       <c r="AC15" t="n">
-        <v>-11.997</v>
+        <v>-10.1241</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>267.13</v>
+        <v>247.42</v>
       </c>
       <c r="C16" t="n">
-        <v>274.93</v>
+        <v>259.79</v>
       </c>
       <c r="D16" t="n">
-        <v>226</v>
+        <v>233.3</v>
       </c>
       <c r="E16" t="n">
-        <v>226.19</v>
+        <v>233.86</v>
       </c>
       <c r="F16" t="n">
-        <v>84.19</v>
+        <v>81.67</v>
       </c>
       <c r="G16" t="n">
-        <v>84.83</v>
+        <v>81.81</v>
       </c>
       <c r="H16" t="n">
-        <v>79.86</v>
+        <v>76.94</v>
       </c>
       <c r="I16" t="n">
-        <v>79.93000000000001</v>
+        <v>77.54000000000001</v>
       </c>
       <c r="J16" t="n">
-        <v>3.9836</v>
+        <v>4.122</v>
       </c>
       <c r="K16" t="n">
-        <v>4.5965</v>
+        <v>4.4086</v>
       </c>
       <c r="L16" t="n">
-        <v>3.865</v>
+        <v>3.8749</v>
       </c>
       <c r="M16" t="n">
-        <v>4.5767</v>
+        <v>4.4086</v>
       </c>
       <c r="N16" t="n">
-        <v>35.9652</v>
+        <v>36.9397</v>
       </c>
       <c r="O16" t="n">
-        <v>37.7861</v>
+        <v>39.1641</v>
       </c>
       <c r="P16" t="n">
-        <v>35.6896</v>
+        <v>36.8708</v>
       </c>
       <c r="Q16" t="n">
-        <v>37.7468</v>
+        <v>38.8984</v>
       </c>
       <c r="R16" t="n">
-        <v>-16.9945</v>
+        <v>3.391</v>
       </c>
       <c r="S16" t="n">
-        <v>0.9822</v>
+        <v>-0.3494</v>
       </c>
       <c r="T16" t="n">
-        <v>12.1529</v>
+        <v>29.4547</v>
       </c>
       <c r="U16" t="n">
-        <v>-5.5089</v>
+        <v>-2.9901</v>
       </c>
       <c r="V16" t="n">
-        <v>5.1572</v>
+        <v>0.0258</v>
       </c>
       <c r="W16" t="n">
-        <v>8.4238</v>
+        <v>11.9388</v>
       </c>
       <c r="X16" t="n">
-        <v>17.216</v>
+        <v>-3.673</v>
       </c>
       <c r="Y16" t="n">
-        <v>-6.8413</v>
+        <v>-5.5084</v>
       </c>
       <c r="Z16" t="n">
-        <v>-21.922</v>
+        <v>-32.1159</v>
       </c>
       <c r="AA16" t="n">
-        <v>5.6182</v>
+        <v>3.0509</v>
       </c>
       <c r="AB16" t="n">
-        <v>-6.074</v>
+        <v>-1.2986</v>
       </c>
       <c r="AC16" t="n">
-        <v>-10.1241</v>
+        <v>-12.6628</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>247.42</v>
+        <v>266.04</v>
       </c>
       <c r="C17" t="n">
-        <v>259.79</v>
+        <v>286.15</v>
       </c>
       <c r="D17" t="n">
-        <v>233.3</v>
+        <v>265</v>
       </c>
       <c r="E17" t="n">
-        <v>233.86</v>
+        <v>279.29</v>
       </c>
       <c r="F17" t="n">
-        <v>81.67</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="G17" t="n">
-        <v>81.81</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="H17" t="n">
-        <v>76.94</v>
+        <v>80.63</v>
       </c>
       <c r="I17" t="n">
-        <v>77.54000000000001</v>
+        <v>82.87</v>
       </c>
       <c r="J17" t="n">
-        <v>4.122</v>
+        <v>3.8156</v>
       </c>
       <c r="K17" t="n">
-        <v>4.4086</v>
+        <v>3.8254</v>
       </c>
       <c r="L17" t="n">
-        <v>3.8749</v>
+        <v>3.4103</v>
       </c>
       <c r="M17" t="n">
-        <v>4.4086</v>
+        <v>3.5487</v>
       </c>
       <c r="N17" t="n">
-        <v>36.9397</v>
+        <v>36.6149</v>
       </c>
       <c r="O17" t="n">
-        <v>39.1641</v>
+        <v>37.3531</v>
       </c>
       <c r="P17" t="n">
-        <v>36.8708</v>
+        <v>35.857</v>
       </c>
       <c r="Q17" t="n">
-        <v>38.8984</v>
+        <v>36.1719</v>
       </c>
       <c r="R17" t="n">
-        <v>3.391</v>
+        <v>19.4262</v>
       </c>
       <c r="S17" t="n">
-        <v>-0.3494</v>
+        <v>2.4917</v>
       </c>
       <c r="T17" t="n">
-        <v>29.4547</v>
+        <v>24.6886</v>
       </c>
       <c r="U17" t="n">
-        <v>-2.9901</v>
+        <v>6.8739</v>
       </c>
       <c r="V17" t="n">
-        <v>0.0258</v>
+        <v>-2.0333</v>
       </c>
       <c r="W17" t="n">
-        <v>11.9388</v>
+        <v>9.0251</v>
       </c>
       <c r="X17" t="n">
-        <v>-3.673</v>
+        <v>-19.5051</v>
       </c>
       <c r="Y17" t="n">
-        <v>-5.5084</v>
+        <v>-9.1126</v>
       </c>
       <c r="Z17" t="n">
-        <v>-32.1159</v>
+        <v>-27.7662</v>
       </c>
       <c r="AA17" t="n">
-        <v>3.0509</v>
+        <v>-7.0093</v>
       </c>
       <c r="AB17" t="n">
-        <v>-1.2986</v>
+        <v>1.2116</v>
       </c>
       <c r="AC17" t="n">
-        <v>-12.6628</v>
+        <v>-9.992800000000001</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>266.04</v>
+        <v>299.26</v>
       </c>
       <c r="C18" t="n">
-        <v>286.15</v>
+        <v>302</v>
       </c>
       <c r="D18" t="n">
-        <v>265</v>
+        <v>286.24</v>
       </c>
       <c r="E18" t="n">
-        <v>279.29</v>
+        <v>300.77</v>
       </c>
       <c r="F18" t="n">
-        <v>82.09999999999999</v>
+        <v>83.95</v>
       </c>
       <c r="G18" t="n">
-        <v>83.59999999999999</v>
+        <v>85.11</v>
       </c>
       <c r="H18" t="n">
-        <v>80.63</v>
+        <v>81.39</v>
       </c>
       <c r="I18" t="n">
-        <v>82.87</v>
+        <v>82.58</v>
       </c>
       <c r="J18" t="n">
-        <v>3.8156</v>
+        <v>3.2917</v>
       </c>
       <c r="K18" t="n">
-        <v>3.8254</v>
+        <v>3.4498</v>
       </c>
       <c r="L18" t="n">
-        <v>3.4103</v>
+        <v>3.2521</v>
       </c>
       <c r="M18" t="n">
-        <v>3.5487</v>
+        <v>3.262</v>
       </c>
       <c r="N18" t="n">
-        <v>36.6149</v>
+        <v>35.7389</v>
       </c>
       <c r="O18" t="n">
-        <v>37.3531</v>
+        <v>36.8511</v>
       </c>
       <c r="P18" t="n">
-        <v>35.857</v>
+        <v>35.2369</v>
       </c>
       <c r="Q18" t="n">
-        <v>36.1719</v>
+        <v>36.3491</v>
       </c>
       <c r="R18" t="n">
-        <v>19.4262</v>
+        <v>7.6909</v>
       </c>
       <c r="S18" t="n">
-        <v>2.4917</v>
+        <v>32.9723</v>
       </c>
       <c r="T18" t="n">
-        <v>24.6886</v>
+        <v>28.1618</v>
       </c>
       <c r="U18" t="n">
-        <v>6.8739</v>
+        <v>-0.3499</v>
       </c>
       <c r="V18" t="n">
-        <v>-2.0333</v>
+        <v>3.3154</v>
       </c>
       <c r="W18" t="n">
-        <v>9.0251</v>
+        <v>6.5273</v>
       </c>
       <c r="X18" t="n">
-        <v>-19.5051</v>
+        <v>-8.079000000000001</v>
       </c>
       <c r="Y18" t="n">
-        <v>-9.1126</v>
+        <v>-28.7259</v>
       </c>
       <c r="Z18" t="n">
-        <v>-27.7662</v>
+        <v>-30.084</v>
       </c>
       <c r="AA18" t="n">
-        <v>-7.0093</v>
+        <v>0.4899</v>
       </c>
       <c r="AB18" t="n">
-        <v>1.2116</v>
+        <v>-3.7028</v>
       </c>
       <c r="AC18" t="n">
-        <v>-9.992800000000001</v>
+        <v>-7.7673</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>299.26</v>
+        <v>236</v>
       </c>
       <c r="C19" t="n">
-        <v>302</v>
+        <v>252.98</v>
       </c>
       <c r="D19" t="n">
-        <v>286.24</v>
+        <v>223</v>
       </c>
       <c r="E19" t="n">
-        <v>300.77</v>
+        <v>231.42</v>
       </c>
       <c r="F19" t="n">
-        <v>83.95</v>
+        <v>75.12</v>
       </c>
       <c r="G19" t="n">
-        <v>85.11</v>
+        <v>77.73999999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>81.39</v>
+        <v>73.91</v>
       </c>
       <c r="I19" t="n">
-        <v>82.58</v>
+        <v>74.44</v>
       </c>
       <c r="J19" t="n">
-        <v>3.2917</v>
+        <v>3.99</v>
       </c>
       <c r="K19" t="n">
-        <v>3.4498</v>
+        <v>4.13</v>
       </c>
       <c r="L19" t="n">
-        <v>3.2521</v>
+        <v>3.8</v>
       </c>
       <c r="M19" t="n">
-        <v>3.262</v>
+        <v>4.04</v>
       </c>
       <c r="N19" t="n">
-        <v>35.7389</v>
+        <v>39.6267</v>
       </c>
       <c r="O19" t="n">
-        <v>36.8511</v>
+        <v>40.1582</v>
       </c>
       <c r="P19" t="n">
-        <v>35.2369</v>
+        <v>38.4653</v>
       </c>
       <c r="Q19" t="n">
-        <v>36.3491</v>
+        <v>39.922</v>
       </c>
       <c r="R19" t="n">
-        <v>7.6909</v>
+        <v>-23.0575</v>
       </c>
       <c r="S19" t="n">
-        <v>32.9723</v>
+        <v>-1.0434</v>
       </c>
       <c r="T19" t="n">
-        <v>28.1618</v>
+        <v>-15.0752</v>
       </c>
       <c r="U19" t="n">
-        <v>-0.3499</v>
+        <v>-9.857100000000001</v>
       </c>
       <c r="V19" t="n">
-        <v>3.3154</v>
+        <v>-3.9979</v>
       </c>
       <c r="W19" t="n">
-        <v>6.5273</v>
+        <v>-11.9991</v>
       </c>
       <c r="X19" t="n">
-        <v>-8.079000000000001</v>
+        <v>23.8504</v>
       </c>
       <c r="Y19" t="n">
-        <v>-28.7259</v>
+        <v>-8.360900000000001</v>
       </c>
       <c r="Z19" t="n">
-        <v>-30.084</v>
+        <v>3.4704</v>
       </c>
       <c r="AA19" t="n">
-        <v>0.4899</v>
+        <v>9.8294</v>
       </c>
       <c r="AB19" t="n">
-        <v>-3.7028</v>
+        <v>2.6315</v>
       </c>
       <c r="AC19" t="n">
-        <v>-7.7673</v>
+        <v>11.7046</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>236</v>
+        <v>233.11</v>
       </c>
       <c r="C20" t="n">
-        <v>252.98</v>
+        <v>237</v>
       </c>
       <c r="D20" t="n">
-        <v>223</v>
+        <v>211.13</v>
       </c>
       <c r="E20" t="n">
-        <v>231.42</v>
+        <v>229.57</v>
       </c>
       <c r="F20" t="n">
-        <v>75.12</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>77.73999999999999</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="H20" t="n">
-        <v>73.91</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>74.44</v>
+        <v>73.3</v>
       </c>
       <c r="J20" t="n">
-        <v>3.99</v>
+        <v>4</v>
       </c>
       <c r="K20" t="n">
-        <v>4.13</v>
+        <v>4.39</v>
       </c>
       <c r="L20" t="n">
-        <v>3.8</v>
+        <v>3.92</v>
       </c>
       <c r="M20" t="n">
-        <v>4.04</v>
+        <v>4.08</v>
       </c>
       <c r="N20" t="n">
-        <v>39.6267</v>
+        <v>39.66</v>
       </c>
       <c r="O20" t="n">
-        <v>40.1582</v>
+        <v>41.49</v>
       </c>
       <c r="P20" t="n">
-        <v>38.4653</v>
+        <v>38.9</v>
       </c>
       <c r="Q20" t="n">
-        <v>39.922</v>
+        <v>40.45</v>
       </c>
       <c r="R20" t="n">
-        <v>-23.0575</v>
+        <v>-0.7994</v>
       </c>
       <c r="S20" t="n">
-        <v>-1.0434</v>
+        <v>-17.8023</v>
       </c>
       <c r="T20" t="n">
-        <v>-15.0752</v>
+        <v>1.4943</v>
       </c>
       <c r="U20" t="n">
-        <v>-9.857100000000001</v>
+        <v>-1.5314</v>
       </c>
       <c r="V20" t="n">
-        <v>-3.9979</v>
+        <v>-11.5482</v>
       </c>
       <c r="W20" t="n">
-        <v>-11.9991</v>
+        <v>-8.2948</v>
       </c>
       <c r="X20" t="n">
-        <v>23.8504</v>
+        <v>0.9901</v>
       </c>
       <c r="Y20" t="n">
-        <v>-8.360900000000001</v>
+        <v>14.9717</v>
       </c>
       <c r="Z20" t="n">
-        <v>3.4704</v>
+        <v>-10.8528</v>
       </c>
       <c r="AA20" t="n">
-        <v>9.8294</v>
+        <v>1.3226</v>
       </c>
       <c r="AB20" t="n">
-        <v>2.6315</v>
+        <v>11.8271</v>
       </c>
       <c r="AC20" t="n">
-        <v>11.7046</v>
+        <v>7.1614</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>233.11</v>
+        <v>268.05</v>
       </c>
       <c r="C21" t="n">
-        <v>237</v>
+        <v>268.4</v>
       </c>
       <c r="D21" t="n">
-        <v>211.13</v>
+        <v>225.74</v>
       </c>
       <c r="E21" t="n">
-        <v>229.57</v>
+        <v>252.61</v>
       </c>
       <c r="F21" t="n">
-        <v>74.79000000000001</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="G21" t="n">
-        <v>76.18000000000001</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>71.34999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I21" t="n">
-        <v>73.3</v>
+        <v>74.95</v>
       </c>
       <c r="J21" t="n">
-        <v>4</v>
+        <v>3.38</v>
       </c>
       <c r="K21" t="n">
-        <v>4.39</v>
+        <v>4.15</v>
       </c>
       <c r="L21" t="n">
-        <v>3.92</v>
+        <v>3.37</v>
       </c>
       <c r="M21" t="n">
-        <v>4.08</v>
+        <v>3.63</v>
       </c>
       <c r="N21" t="n">
-        <v>39.66</v>
+        <v>37.87</v>
       </c>
       <c r="O21" t="n">
-        <v>41.49</v>
+        <v>41.37</v>
       </c>
       <c r="P21" t="n">
-        <v>38.9</v>
+        <v>37.71</v>
       </c>
       <c r="Q21" t="n">
-        <v>40.45</v>
+        <v>39.47</v>
       </c>
       <c r="R21" t="n">
-        <v>-0.7994</v>
+        <v>10.0362</v>
       </c>
       <c r="S21" t="n">
-        <v>-17.8023</v>
+        <v>-16.0122</v>
       </c>
       <c r="T21" t="n">
-        <v>1.4943</v>
+        <v>8.0176</v>
       </c>
       <c r="U21" t="n">
-        <v>-1.5314</v>
+        <v>2.251</v>
       </c>
       <c r="V21" t="n">
-        <v>-11.5482</v>
+        <v>-9.2395</v>
       </c>
       <c r="W21" t="n">
-        <v>-8.2948</v>
+        <v>-3.3402</v>
       </c>
       <c r="X21" t="n">
-        <v>0.9901</v>
+        <v>-11.0294</v>
       </c>
       <c r="Y21" t="n">
-        <v>14.9717</v>
+        <v>11.2814</v>
       </c>
       <c r="Z21" t="n">
-        <v>-10.8528</v>
+        <v>-17.6609</v>
       </c>
       <c r="AA21" t="n">
-        <v>1.3226</v>
+        <v>-2.4227</v>
       </c>
       <c r="AB21" t="n">
-        <v>11.8271</v>
+        <v>8.585900000000001</v>
       </c>
       <c r="AC21" t="n">
-        <v>7.1614</v>
+        <v>1.4695</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>268.05</v>
+        <v>226.24</v>
       </c>
       <c r="C22" t="n">
-        <v>268.33</v>
+        <v>231.21</v>
       </c>
       <c r="D22" t="n">
-        <v>225.7441</v>
+        <v>212.1</v>
       </c>
       <c r="E22" t="n">
-        <v>252.61</v>
+        <v>215.6</v>
       </c>
       <c r="F22" t="n">
-        <v>77.94</v>
+        <v>72.065</v>
       </c>
       <c r="G22" t="n">
-        <v>78.23999999999999</v>
+        <v>74.69</v>
       </c>
       <c r="H22" t="n">
-        <v>71.59999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="I22" t="n">
-        <v>74.95</v>
+        <v>71.83</v>
       </c>
       <c r="J22" t="n">
-        <v>3.38</v>
+        <v>4.035</v>
       </c>
       <c r="K22" t="n">
-        <v>4.15</v>
+        <v>4.25</v>
       </c>
       <c r="L22" t="n">
-        <v>3.37</v>
+        <v>3.95</v>
       </c>
       <c r="M22" t="n">
-        <v>3.63</v>
+        <v>4.24</v>
       </c>
       <c r="N22" t="n">
-        <v>37.86</v>
+        <v>41.085</v>
       </c>
       <c r="O22" t="n">
-        <v>41.3699</v>
+        <v>41.79</v>
       </c>
       <c r="P22" t="n">
-        <v>37.7101</v>
+        <v>39.69</v>
       </c>
       <c r="Q22" t="n">
-        <v>39.47</v>
+        <v>41.31</v>
       </c>
       <c r="R22" t="n">
-        <v>10.0362</v>
+        <v>-14.651</v>
       </c>
       <c r="S22" t="n">
-        <v>-16.0122</v>
+        <v>-6.8361</v>
       </c>
       <c r="T22" t="n">
-        <v>8.0176</v>
+        <v>-22.8043</v>
       </c>
       <c r="U22" t="n">
-        <v>2.251</v>
+        <v>-4.1628</v>
       </c>
       <c r="V22" t="n">
-        <v>-9.2395</v>
+        <v>-3.5062</v>
       </c>
       <c r="W22" t="n">
-        <v>-3.3402</v>
+        <v>-13.3221</v>
       </c>
       <c r="X22" t="n">
-        <v>-11.0294</v>
+        <v>16.8044</v>
       </c>
       <c r="Y22" t="n">
-        <v>11.2814</v>
+        <v>4.9505</v>
       </c>
       <c r="Z22" t="n">
-        <v>-17.6609</v>
+        <v>19.4804</v>
       </c>
       <c r="AA22" t="n">
-        <v>-2.4227</v>
+        <v>4.6618</v>
       </c>
       <c r="AB22" t="n">
-        <v>8.585900000000001</v>
+        <v>3.4768</v>
       </c>
       <c r="AC22" t="n">
-        <v>1.4695</v>
+        <v>14.2047</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-29 22:57
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC22"/>
+  <dimension ref="A1:AC21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1804 +568,1713 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>219</v>
+        <v>217.27</v>
       </c>
       <c r="C2" t="n">
-        <v>231.89</v>
+        <v>234.06</v>
       </c>
       <c r="D2" t="n">
-        <v>207.56</v>
+        <v>210.14</v>
       </c>
       <c r="E2" t="n">
-        <v>224.63</v>
+        <v>227.03</v>
       </c>
       <c r="F2" t="n">
-        <v>81.73999999999999</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>84.05</v>
+        <v>87.06</v>
       </c>
       <c r="H2" t="n">
-        <v>80.66</v>
+        <v>83.75</v>
       </c>
       <c r="I2" t="n">
-        <v>83.68000000000001</v>
+        <v>86.04000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>6.4153</v>
+        <v>6.4746</v>
       </c>
       <c r="K2" t="n">
-        <v>6.7514</v>
+        <v>6.6624</v>
       </c>
       <c r="L2" t="n">
-        <v>6.0298</v>
+        <v>5.9803</v>
       </c>
       <c r="M2" t="n">
-        <v>6.2373</v>
+        <v>6.1879</v>
       </c>
       <c r="N2" t="n">
-        <v>38.7901</v>
+        <v>37.668</v>
       </c>
       <c r="O2" t="n">
-        <v>39.3118</v>
+        <v>37.855</v>
       </c>
       <c r="P2" t="n">
-        <v>37.6975</v>
+        <v>36.3786</v>
       </c>
       <c r="Q2" t="n">
-        <v>37.8649</v>
+        <v>36.8314</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>231.82</v>
+        <v>243.18</v>
       </c>
       <c r="C3" t="n">
-        <v>239.07</v>
+        <v>267.08</v>
       </c>
       <c r="D3" t="n">
-        <v>218.56</v>
+        <v>238.82</v>
       </c>
       <c r="E3" t="n">
-        <v>224.34</v>
+        <v>266.32</v>
       </c>
       <c r="F3" t="n">
-        <v>84.41</v>
+        <v>85.94</v>
       </c>
       <c r="G3" t="n">
-        <v>85.7</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>83.53</v>
+        <v>84.83</v>
       </c>
       <c r="I3" t="n">
-        <v>84.56</v>
+        <v>87.22</v>
       </c>
       <c r="J3" t="n">
-        <v>6.0396</v>
+        <v>5.7332</v>
       </c>
       <c r="K3" t="n">
-        <v>6.4153</v>
+        <v>5.8617</v>
       </c>
       <c r="L3" t="n">
-        <v>5.8419</v>
+        <v>5.0907</v>
       </c>
       <c r="M3" t="n">
-        <v>6.2571</v>
+        <v>5.1105</v>
       </c>
       <c r="N3" t="n">
-        <v>37.5499</v>
+        <v>36.8806</v>
       </c>
       <c r="O3" t="n">
-        <v>37.9535</v>
+        <v>37.3531</v>
       </c>
       <c r="P3" t="n">
-        <v>36.9692</v>
+        <v>36.2802</v>
       </c>
       <c r="Q3" t="n">
-        <v>37.481</v>
+        <v>36.3294</v>
       </c>
       <c r="R3" t="n">
-        <v>-0.1291</v>
+        <v>17.3061</v>
       </c>
       <c r="U3" t="n">
-        <v>1.0516</v>
+        <v>1.3715</v>
       </c>
       <c r="X3" t="n">
-        <v>0.3174</v>
+        <v>-17.4114</v>
       </c>
       <c r="AA3" t="n">
-        <v>-1.0139</v>
+        <v>-1.363</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>217.27</v>
+        <v>281.47</v>
       </c>
       <c r="C4" t="n">
-        <v>234.06</v>
+        <v>284.58</v>
       </c>
       <c r="D4" t="n">
-        <v>210.14</v>
+        <v>257.26</v>
       </c>
       <c r="E4" t="n">
-        <v>227.03</v>
+        <v>280.54</v>
       </c>
       <c r="F4" t="n">
-        <v>84.15000000000001</v>
+        <v>87.68000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>87.06</v>
+        <v>88.09</v>
       </c>
       <c r="H4" t="n">
-        <v>83.75</v>
+        <v>85.41</v>
       </c>
       <c r="I4" t="n">
-        <v>86.04000000000001</v>
+        <v>86.56</v>
       </c>
       <c r="J4" t="n">
-        <v>6.4746</v>
+        <v>4.8238</v>
       </c>
       <c r="K4" t="n">
-        <v>6.6624</v>
+        <v>5.2884</v>
       </c>
       <c r="L4" t="n">
-        <v>5.9803</v>
+        <v>4.7645</v>
       </c>
       <c r="M4" t="n">
-        <v>6.1879</v>
+        <v>4.8535</v>
       </c>
       <c r="N4" t="n">
-        <v>37.668</v>
+        <v>36.1522</v>
       </c>
       <c r="O4" t="n">
-        <v>37.855</v>
+        <v>37.0971</v>
       </c>
       <c r="P4" t="n">
-        <v>36.3786</v>
+        <v>35.9751</v>
       </c>
       <c r="Q4" t="n">
-        <v>36.8314</v>
+        <v>36.605</v>
       </c>
       <c r="R4" t="n">
-        <v>1.1991</v>
+        <v>5.3394</v>
       </c>
       <c r="U4" t="n">
-        <v>1.7502</v>
+        <v>-0.7567</v>
       </c>
       <c r="X4" t="n">
-        <v>-1.1059</v>
+        <v>-5.0289</v>
       </c>
       <c r="AA4" t="n">
-        <v>-1.7331</v>
+        <v>0.7586000000000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>243.18</v>
+        <v>242.04</v>
       </c>
       <c r="C5" t="n">
-        <v>267.08</v>
+        <v>274.5</v>
       </c>
       <c r="D5" t="n">
-        <v>238.82</v>
+        <v>228.55</v>
       </c>
       <c r="E5" t="n">
-        <v>266.32</v>
+        <v>262.7</v>
       </c>
       <c r="F5" t="n">
-        <v>85.94</v>
+        <v>83.47</v>
       </c>
       <c r="G5" t="n">
-        <v>87.31999999999999</v>
+        <v>86.25</v>
       </c>
       <c r="H5" t="n">
-        <v>84.83</v>
+        <v>82.48</v>
       </c>
       <c r="I5" t="n">
-        <v>87.22</v>
+        <v>85.22</v>
       </c>
       <c r="J5" t="n">
-        <v>5.7332</v>
+        <v>5.5059</v>
       </c>
       <c r="K5" t="n">
-        <v>5.8617</v>
+        <v>5.7431</v>
       </c>
       <c r="L5" t="n">
-        <v>5.0907</v>
+        <v>4.9424</v>
       </c>
       <c r="M5" t="n">
-        <v>5.1105</v>
+        <v>5.1401</v>
       </c>
       <c r="N5" t="n">
-        <v>36.8806</v>
+        <v>37.9239</v>
       </c>
       <c r="O5" t="n">
-        <v>37.3531</v>
+        <v>38.3472</v>
       </c>
       <c r="P5" t="n">
-        <v>36.2802</v>
+        <v>36.7428</v>
       </c>
       <c r="Q5" t="n">
-        <v>36.3294</v>
+        <v>37.166</v>
       </c>
       <c r="R5" t="n">
-        <v>17.3061</v>
+        <v>-6.3592</v>
       </c>
       <c r="S5" t="n">
-        <v>18.5594</v>
+        <v>15.7116</v>
       </c>
       <c r="U5" t="n">
-        <v>1.3715</v>
+        <v>-1.5481</v>
       </c>
       <c r="V5" t="n">
-        <v>4.2304</v>
+        <v>-0.953</v>
       </c>
       <c r="X5" t="n">
-        <v>-17.4114</v>
+        <v>5.905</v>
       </c>
       <c r="Y5" t="n">
-        <v>-18.0655</v>
+        <v>-16.933</v>
       </c>
       <c r="AA5" t="n">
-        <v>-1.363</v>
+        <v>1.5326</v>
       </c>
       <c r="AB5" t="n">
-        <v>-4.0552</v>
+        <v>0.9085</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>281.47</v>
+        <v>230.85</v>
       </c>
       <c r="C6" t="n">
-        <v>284.58</v>
+        <v>233.69</v>
       </c>
       <c r="D6" t="n">
-        <v>257.26</v>
+        <v>181.81</v>
       </c>
       <c r="E6" t="n">
-        <v>280.54</v>
+        <v>182.54</v>
       </c>
       <c r="F6" t="n">
-        <v>87.68000000000001</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>88.09</v>
+        <v>82.08</v>
       </c>
       <c r="H6" t="n">
-        <v>85.41</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="I6" t="n">
-        <v>86.56</v>
+        <v>73.05</v>
       </c>
       <c r="J6" t="n">
-        <v>4.8238</v>
+        <v>5.7925</v>
       </c>
       <c r="K6" t="n">
-        <v>5.2884</v>
+        <v>6.7711</v>
       </c>
       <c r="L6" t="n">
-        <v>4.7645</v>
+        <v>5.7233</v>
       </c>
       <c r="M6" t="n">
-        <v>4.8535</v>
+        <v>6.7612</v>
       </c>
       <c r="N6" t="n">
-        <v>36.1522</v>
+        <v>38.7999</v>
       </c>
       <c r="O6" t="n">
-        <v>37.0971</v>
+        <v>42.6681</v>
       </c>
       <c r="P6" t="n">
-        <v>35.9751</v>
+        <v>38.5637</v>
       </c>
       <c r="Q6" t="n">
-        <v>36.605</v>
+        <v>42.5106</v>
       </c>
       <c r="R6" t="n">
-        <v>5.3394</v>
+        <v>-30.5139</v>
       </c>
       <c r="S6" t="n">
-        <v>25.0513</v>
+        <v>-31.4584</v>
       </c>
       <c r="U6" t="n">
-        <v>-0.7567</v>
+        <v>-14.2807</v>
       </c>
       <c r="V6" t="n">
-        <v>2.3652</v>
+        <v>-16.2463</v>
       </c>
       <c r="X6" t="n">
-        <v>-5.0289</v>
+        <v>31.5383</v>
       </c>
       <c r="Y6" t="n">
-        <v>-22.4321</v>
+        <v>32.3002</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.7586000000000001</v>
+        <v>14.3803</v>
       </c>
       <c r="AB6" t="n">
-        <v>-2.3372</v>
+        <v>17.0143</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>242.04</v>
+        <v>210.62</v>
       </c>
       <c r="C7" t="n">
-        <v>274.5</v>
+        <v>222.19</v>
       </c>
       <c r="D7" t="n">
-        <v>228.55</v>
+        <v>201.69</v>
       </c>
       <c r="E7" t="n">
-        <v>262.7</v>
+        <v>211.44</v>
       </c>
       <c r="F7" t="n">
-        <v>83.47</v>
+        <v>76.86</v>
       </c>
       <c r="G7" t="n">
-        <v>86.25</v>
+        <v>78.47</v>
       </c>
       <c r="H7" t="n">
-        <v>82.48</v>
+        <v>75.38</v>
       </c>
       <c r="I7" t="n">
-        <v>85.22</v>
+        <v>76.27</v>
       </c>
       <c r="J7" t="n">
-        <v>5.5059</v>
+        <v>5.6442</v>
       </c>
       <c r="K7" t="n">
-        <v>5.7431</v>
+        <v>5.9803</v>
       </c>
       <c r="L7" t="n">
-        <v>4.9424</v>
+        <v>5.2093</v>
       </c>
       <c r="M7" t="n">
-        <v>5.1401</v>
+        <v>5.6245</v>
       </c>
       <c r="N7" t="n">
-        <v>37.9239</v>
+        <v>40.2763</v>
       </c>
       <c r="O7" t="n">
-        <v>38.3472</v>
+        <v>41.1228</v>
       </c>
       <c r="P7" t="n">
-        <v>36.7428</v>
+        <v>39.3314</v>
       </c>
       <c r="Q7" t="n">
-        <v>37.166</v>
+        <v>40.611</v>
       </c>
       <c r="R7" t="n">
-        <v>-6.3592</v>
+        <v>15.8321</v>
       </c>
       <c r="S7" t="n">
-        <v>15.7116</v>
+        <v>-24.6311</v>
       </c>
       <c r="T7" t="n">
-        <v>16.9479</v>
+        <v>-6.8669</v>
       </c>
       <c r="U7" t="n">
-        <v>-1.5481</v>
+        <v>4.4079</v>
       </c>
       <c r="V7" t="n">
-        <v>-0.953</v>
+        <v>-11.8877</v>
       </c>
       <c r="W7" t="n">
-        <v>1.8403</v>
+        <v>-11.3552</v>
       </c>
       <c r="X7" t="n">
-        <v>5.905</v>
+        <v>-16.8121</v>
       </c>
       <c r="Y7" t="n">
-        <v>-16.933</v>
+        <v>15.8854</v>
       </c>
       <c r="Z7" t="n">
-        <v>-17.5909</v>
+        <v>-9.104900000000001</v>
       </c>
       <c r="AA7" t="n">
-        <v>1.5326</v>
+        <v>-4.4685</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.9085</v>
+        <v>10.9439</v>
       </c>
       <c r="AC7" t="n">
-        <v>-1.8458</v>
+        <v>10.2619</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>230.85</v>
+        <v>227.06</v>
       </c>
       <c r="C8" t="n">
-        <v>233.69</v>
+        <v>231.02</v>
       </c>
       <c r="D8" t="n">
-        <v>181.81</v>
+        <v>157.56</v>
       </c>
       <c r="E8" t="n">
-        <v>182.54</v>
+        <v>201.68</v>
       </c>
       <c r="F8" t="n">
-        <v>81.56999999999999</v>
+        <v>78.48</v>
       </c>
       <c r="G8" t="n">
-        <v>82.08</v>
+        <v>79.34</v>
       </c>
       <c r="H8" t="n">
-        <v>72.68000000000001</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="I8" t="n">
-        <v>73.05</v>
+        <v>73.72</v>
       </c>
       <c r="J8" t="n">
-        <v>5.7925</v>
+        <v>5.1895</v>
       </c>
       <c r="K8" t="n">
-        <v>6.7711</v>
+        <v>7.0281</v>
       </c>
       <c r="L8" t="n">
-        <v>5.7233</v>
+        <v>5.0808</v>
       </c>
       <c r="M8" t="n">
-        <v>6.7612</v>
+        <v>5.8617</v>
       </c>
       <c r="N8" t="n">
-        <v>38.7999</v>
+        <v>39.4299</v>
       </c>
       <c r="O8" t="n">
-        <v>42.6681</v>
+        <v>45.6505</v>
       </c>
       <c r="P8" t="n">
-        <v>38.5637</v>
+        <v>38.9673</v>
       </c>
       <c r="Q8" t="n">
-        <v>42.5106</v>
+        <v>41.9988</v>
       </c>
       <c r="R8" t="n">
-        <v>-30.5139</v>
+        <v>-4.616</v>
       </c>
       <c r="S8" t="n">
-        <v>-31.4584</v>
+        <v>-23.228</v>
       </c>
       <c r="T8" t="n">
-        <v>-18.6324</v>
+        <v>-24.2716</v>
       </c>
       <c r="U8" t="n">
-        <v>-14.2807</v>
+        <v>-3.3434</v>
       </c>
       <c r="V8" t="n">
-        <v>-16.2463</v>
+        <v>-13.4945</v>
       </c>
       <c r="W8" t="n">
-        <v>-13.6116</v>
+        <v>-15.4781</v>
       </c>
       <c r="X8" t="n">
-        <v>31.5383</v>
+        <v>4.2173</v>
       </c>
       <c r="Y8" t="n">
-        <v>32.3002</v>
+        <v>14.0386</v>
       </c>
       <c r="Z8" t="n">
-        <v>8.0564</v>
+        <v>14.6991</v>
       </c>
       <c r="AA8" t="n">
-        <v>14.3803</v>
+        <v>3.4173</v>
       </c>
       <c r="AB8" t="n">
-        <v>17.0143</v>
+        <v>13.0033</v>
       </c>
       <c r="AC8" t="n">
-        <v>13.4191</v>
+        <v>15.6055</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>210.62</v>
+        <v>191.54</v>
       </c>
       <c r="C9" t="n">
-        <v>222.19</v>
+        <v>212.99</v>
       </c>
       <c r="D9" t="n">
-        <v>201.69</v>
+        <v>177.3</v>
       </c>
       <c r="E9" t="n">
-        <v>211.44</v>
+        <v>180.65</v>
       </c>
       <c r="F9" t="n">
-        <v>76.86</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>78.47</v>
+        <v>74.7</v>
       </c>
       <c r="H9" t="n">
-        <v>75.38</v>
+        <v>69</v>
       </c>
       <c r="I9" t="n">
-        <v>76.27</v>
+        <v>69.27</v>
       </c>
       <c r="J9" t="n">
-        <v>5.6442</v>
+        <v>6.1681</v>
       </c>
       <c r="K9" t="n">
-        <v>5.9803</v>
+        <v>6.5734</v>
       </c>
       <c r="L9" t="n">
-        <v>5.2093</v>
+        <v>5.5355</v>
       </c>
       <c r="M9" t="n">
-        <v>5.6245</v>
+        <v>6.4943</v>
       </c>
       <c r="N9" t="n">
-        <v>40.2763</v>
+        <v>43.1209</v>
       </c>
       <c r="O9" t="n">
-        <v>41.1228</v>
+        <v>44.676</v>
       </c>
       <c r="P9" t="n">
-        <v>39.3314</v>
+        <v>41.4082</v>
       </c>
       <c r="Q9" t="n">
-        <v>40.611</v>
+        <v>44.5382</v>
       </c>
       <c r="R9" t="n">
-        <v>15.8321</v>
+        <v>-10.4274</v>
       </c>
       <c r="S9" t="n">
-        <v>-24.6311</v>
+        <v>-1.0354</v>
       </c>
       <c r="T9" t="n">
-        <v>-6.8669</v>
+        <v>-35.6063</v>
       </c>
       <c r="U9" t="n">
-        <v>4.4079</v>
+        <v>-6.0364</v>
       </c>
       <c r="V9" t="n">
-        <v>-11.8877</v>
+        <v>-5.1745</v>
       </c>
       <c r="W9" t="n">
-        <v>-11.3552</v>
+        <v>-19.9746</v>
       </c>
       <c r="X9" t="n">
-        <v>-16.8121</v>
+        <v>10.7921</v>
       </c>
       <c r="Y9" t="n">
-        <v>15.8854</v>
+        <v>-3.9475</v>
       </c>
       <c r="Z9" t="n">
-        <v>-9.104900000000001</v>
+        <v>33.8065</v>
       </c>
       <c r="AA9" t="n">
-        <v>-4.4685</v>
+        <v>6.0464</v>
       </c>
       <c r="AB9" t="n">
-        <v>10.9439</v>
+        <v>4.7696</v>
       </c>
       <c r="AC9" t="n">
-        <v>10.2619</v>
+        <v>21.6724</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>227.06</v>
+        <v>192.3</v>
       </c>
       <c r="C10" t="n">
-        <v>231.02</v>
+        <v>225.63</v>
       </c>
       <c r="D10" t="n">
-        <v>157.56</v>
+        <v>192.3</v>
       </c>
       <c r="E10" t="n">
-        <v>201.68</v>
+        <v>223.99</v>
       </c>
       <c r="F10" t="n">
-        <v>78.48</v>
+        <v>70.89</v>
       </c>
       <c r="G10" t="n">
-        <v>79.34</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>66.79000000000001</v>
+        <v>69.59</v>
       </c>
       <c r="I10" t="n">
-        <v>73.72</v>
+        <v>76.01000000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>5.1895</v>
+        <v>6.0298</v>
       </c>
       <c r="K10" t="n">
-        <v>7.0281</v>
+        <v>6.0298</v>
       </c>
       <c r="L10" t="n">
-        <v>5.0808</v>
+        <v>4.8436</v>
       </c>
       <c r="M10" t="n">
-        <v>5.8617</v>
+        <v>4.9128</v>
       </c>
       <c r="N10" t="n">
-        <v>39.4299</v>
+        <v>43.4851</v>
       </c>
       <c r="O10" t="n">
-        <v>45.6505</v>
+        <v>44.302</v>
       </c>
       <c r="P10" t="n">
-        <v>38.9673</v>
+        <v>39.8039</v>
       </c>
       <c r="Q10" t="n">
-        <v>41.9988</v>
+        <v>40.1878</v>
       </c>
       <c r="R10" t="n">
-        <v>-4.616</v>
+        <v>23.9911</v>
       </c>
       <c r="S10" t="n">
-        <v>-23.228</v>
+        <v>5.9355</v>
       </c>
       <c r="T10" t="n">
-        <v>-24.2716</v>
+        <v>-14.7354</v>
       </c>
       <c r="U10" t="n">
-        <v>-3.3434</v>
+        <v>9.73</v>
       </c>
       <c r="V10" t="n">
-        <v>-13.4945</v>
+        <v>-0.3409</v>
       </c>
       <c r="W10" t="n">
-        <v>-15.4781</v>
+        <v>-10.8073</v>
       </c>
       <c r="X10" t="n">
-        <v>4.2173</v>
+        <v>-24.3521</v>
       </c>
       <c r="Y10" t="n">
-        <v>14.0386</v>
+        <v>-12.6536</v>
       </c>
       <c r="Z10" t="n">
-        <v>14.6991</v>
+        <v>-4.4221</v>
       </c>
       <c r="AA10" t="n">
-        <v>3.4173</v>
+        <v>-9.767799999999999</v>
       </c>
       <c r="AB10" t="n">
-        <v>13.0033</v>
+        <v>-1.0421</v>
       </c>
       <c r="AC10" t="n">
-        <v>15.6055</v>
+        <v>8.1305</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>191.54</v>
+        <v>222.22</v>
       </c>
       <c r="C11" t="n">
-        <v>212.99</v>
+        <v>242.4</v>
       </c>
       <c r="D11" t="n">
-        <v>177.3</v>
+        <v>214.74</v>
       </c>
       <c r="E11" t="n">
-        <v>180.65</v>
+        <v>234.68</v>
       </c>
       <c r="F11" t="n">
-        <v>71.68000000000001</v>
+        <v>76.34</v>
       </c>
       <c r="G11" t="n">
-        <v>74.7</v>
+        <v>78.36</v>
       </c>
       <c r="H11" t="n">
-        <v>69</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="I11" t="n">
-        <v>69.27</v>
+        <v>77.52</v>
       </c>
       <c r="J11" t="n">
-        <v>6.1681</v>
+        <v>4.9523</v>
       </c>
       <c r="K11" t="n">
-        <v>6.5734</v>
+        <v>5.0907</v>
       </c>
       <c r="L11" t="n">
-        <v>5.5355</v>
+        <v>4.4877</v>
       </c>
       <c r="M11" t="n">
-        <v>6.4943</v>
+        <v>4.6656</v>
       </c>
       <c r="N11" t="n">
-        <v>43.1209</v>
+        <v>40.0106</v>
       </c>
       <c r="O11" t="n">
-        <v>44.676</v>
+        <v>41.0933</v>
       </c>
       <c r="P11" t="n">
-        <v>41.4082</v>
+        <v>38.9476</v>
       </c>
       <c r="Q11" t="n">
-        <v>44.5382</v>
+        <v>39.4102</v>
       </c>
       <c r="R11" t="n">
-        <v>-10.4274</v>
+        <v>4.7725</v>
       </c>
       <c r="S11" t="n">
-        <v>-1.0354</v>
+        <v>16.3626</v>
       </c>
       <c r="T11" t="n">
-        <v>-35.6063</v>
+        <v>28.5636</v>
       </c>
       <c r="U11" t="n">
-        <v>-6.0364</v>
+        <v>1.9866</v>
       </c>
       <c r="V11" t="n">
-        <v>-5.1745</v>
+        <v>5.1546</v>
       </c>
       <c r="W11" t="n">
-        <v>-19.9746</v>
+        <v>6.1191</v>
       </c>
       <c r="X11" t="n">
-        <v>10.7921</v>
+        <v>-5.0318</v>
       </c>
       <c r="Y11" t="n">
-        <v>-3.9475</v>
+        <v>-20.4053</v>
       </c>
       <c r="Z11" t="n">
-        <v>33.8065</v>
+        <v>-30.9945</v>
       </c>
       <c r="AA11" t="n">
-        <v>6.0464</v>
+        <v>-1.9349</v>
       </c>
       <c r="AB11" t="n">
-        <v>4.7696</v>
+        <v>-6.1635</v>
       </c>
       <c r="AC11" t="n">
-        <v>21.6724</v>
+        <v>-7.2932</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>192.3</v>
+        <v>265.99</v>
       </c>
       <c r="C12" t="n">
-        <v>225.63</v>
+        <v>274.88</v>
       </c>
       <c r="D12" t="n">
-        <v>192.3</v>
+        <v>261.6</v>
       </c>
       <c r="E12" t="n">
-        <v>223.99</v>
+        <v>272.5</v>
       </c>
       <c r="F12" t="n">
-        <v>70.89</v>
+        <v>82.88</v>
       </c>
       <c r="G12" t="n">
-        <v>76.59999999999999</v>
+        <v>85.03</v>
       </c>
       <c r="H12" t="n">
-        <v>69.59</v>
+        <v>82.64</v>
       </c>
       <c r="I12" t="n">
-        <v>76.01000000000001</v>
+        <v>84.59</v>
       </c>
       <c r="J12" t="n">
-        <v>6.0298</v>
+        <v>4.0231</v>
       </c>
       <c r="K12" t="n">
-        <v>6.0298</v>
+        <v>4.122</v>
       </c>
       <c r="L12" t="n">
-        <v>4.8436</v>
+        <v>3.865</v>
       </c>
       <c r="M12" t="n">
-        <v>4.9128</v>
+        <v>3.9045</v>
       </c>
       <c r="N12" t="n">
-        <v>43.4851</v>
+        <v>36.6641</v>
       </c>
       <c r="O12" t="n">
-        <v>44.302</v>
+        <v>36.7723</v>
       </c>
       <c r="P12" t="n">
-        <v>39.8039</v>
+        <v>35.5814</v>
       </c>
       <c r="Q12" t="n">
-        <v>40.1878</v>
+        <v>35.7389</v>
       </c>
       <c r="R12" t="n">
-        <v>23.9911</v>
+        <v>16.1156</v>
       </c>
       <c r="S12" t="n">
-        <v>5.9355</v>
+        <v>50.8442</v>
       </c>
       <c r="T12" t="n">
-        <v>-14.7354</v>
+        <v>28.8782</v>
       </c>
       <c r="U12" t="n">
-        <v>9.73</v>
+        <v>9.120200000000001</v>
       </c>
       <c r="V12" t="n">
-        <v>-0.3409</v>
+        <v>22.1164</v>
       </c>
       <c r="W12" t="n">
-        <v>-10.8073</v>
+        <v>10.9086</v>
       </c>
       <c r="X12" t="n">
-        <v>-24.3521</v>
+        <v>-16.313</v>
       </c>
       <c r="Y12" t="n">
-        <v>-12.6536</v>
+        <v>-39.878</v>
       </c>
       <c r="Z12" t="n">
-        <v>-4.4221</v>
+        <v>-30.5805</v>
       </c>
       <c r="AA12" t="n">
-        <v>-9.767799999999999</v>
+        <v>-9.3156</v>
       </c>
       <c r="AB12" t="n">
-        <v>-1.0421</v>
+        <v>-19.7567</v>
       </c>
       <c r="AC12" t="n">
-        <v>8.1305</v>
+        <v>-11.997</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>222.22</v>
+        <v>267.13</v>
       </c>
       <c r="C13" t="n">
-        <v>242.4</v>
+        <v>274.93</v>
       </c>
       <c r="D13" t="n">
-        <v>214.74</v>
+        <v>226</v>
       </c>
       <c r="E13" t="n">
-        <v>234.68</v>
+        <v>226.19</v>
       </c>
       <c r="F13" t="n">
-        <v>76.34</v>
+        <v>84.19</v>
       </c>
       <c r="G13" t="n">
-        <v>78.36</v>
+        <v>84.83</v>
       </c>
       <c r="H13" t="n">
-        <v>74.29000000000001</v>
+        <v>79.86</v>
       </c>
       <c r="I13" t="n">
-        <v>77.52</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>4.9523</v>
+        <v>3.9836</v>
       </c>
       <c r="K13" t="n">
-        <v>5.0907</v>
+        <v>4.5965</v>
       </c>
       <c r="L13" t="n">
-        <v>4.4877</v>
+        <v>3.865</v>
       </c>
       <c r="M13" t="n">
-        <v>4.6656</v>
+        <v>4.5767</v>
       </c>
       <c r="N13" t="n">
-        <v>40.0106</v>
+        <v>35.9652</v>
       </c>
       <c r="O13" t="n">
-        <v>41.0933</v>
+        <v>37.7861</v>
       </c>
       <c r="P13" t="n">
-        <v>38.9476</v>
+        <v>35.6896</v>
       </c>
       <c r="Q13" t="n">
-        <v>39.4102</v>
+        <v>37.7468</v>
       </c>
       <c r="R13" t="n">
-        <v>4.7725</v>
+        <v>-16.9945</v>
       </c>
       <c r="S13" t="n">
-        <v>16.3626</v>
+        <v>0.9822</v>
       </c>
       <c r="T13" t="n">
-        <v>28.5636</v>
+        <v>12.1529</v>
       </c>
       <c r="U13" t="n">
-        <v>1.9866</v>
+        <v>-5.5089</v>
       </c>
       <c r="V13" t="n">
-        <v>5.1546</v>
+        <v>5.1572</v>
       </c>
       <c r="W13" t="n">
-        <v>6.1191</v>
+        <v>8.4238</v>
       </c>
       <c r="X13" t="n">
-        <v>-5.0318</v>
+        <v>17.216</v>
       </c>
       <c r="Y13" t="n">
-        <v>-20.4053</v>
+        <v>-6.8413</v>
       </c>
       <c r="Z13" t="n">
-        <v>-30.9945</v>
+        <v>-21.922</v>
       </c>
       <c r="AA13" t="n">
-        <v>-1.9349</v>
+        <v>5.6182</v>
       </c>
       <c r="AB13" t="n">
-        <v>-6.1635</v>
+        <v>-6.074</v>
       </c>
       <c r="AC13" t="n">
-        <v>-7.2932</v>
+        <v>-10.1241</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>265.99</v>
+        <v>247.42</v>
       </c>
       <c r="C14" t="n">
-        <v>274.88</v>
+        <v>259.79</v>
       </c>
       <c r="D14" t="n">
-        <v>261.6</v>
+        <v>233.3</v>
       </c>
       <c r="E14" t="n">
-        <v>272.5</v>
+        <v>233.86</v>
       </c>
       <c r="F14" t="n">
-        <v>82.88</v>
+        <v>81.67</v>
       </c>
       <c r="G14" t="n">
-        <v>85.03</v>
+        <v>81.81</v>
       </c>
       <c r="H14" t="n">
-        <v>82.64</v>
+        <v>76.94</v>
       </c>
       <c r="I14" t="n">
-        <v>84.59</v>
+        <v>77.54000000000001</v>
       </c>
       <c r="J14" t="n">
-        <v>4.0231</v>
+        <v>4.122</v>
       </c>
       <c r="K14" t="n">
-        <v>4.122</v>
+        <v>4.4086</v>
       </c>
       <c r="L14" t="n">
-        <v>3.865</v>
+        <v>3.8749</v>
       </c>
       <c r="M14" t="n">
-        <v>3.9045</v>
+        <v>4.4086</v>
       </c>
       <c r="N14" t="n">
-        <v>36.6641</v>
+        <v>36.9397</v>
       </c>
       <c r="O14" t="n">
-        <v>36.7723</v>
+        <v>39.1641</v>
       </c>
       <c r="P14" t="n">
-        <v>35.5814</v>
+        <v>36.8708</v>
       </c>
       <c r="Q14" t="n">
-        <v>35.7389</v>
+        <v>38.8984</v>
       </c>
       <c r="R14" t="n">
-        <v>16.1156</v>
+        <v>3.391</v>
       </c>
       <c r="S14" t="n">
-        <v>50.8442</v>
+        <v>-0.3494</v>
       </c>
       <c r="T14" t="n">
-        <v>28.8782</v>
+        <v>29.4547</v>
       </c>
       <c r="U14" t="n">
-        <v>9.120200000000001</v>
+        <v>-2.9901</v>
       </c>
       <c r="V14" t="n">
-        <v>22.1164</v>
+        <v>0.0258</v>
       </c>
       <c r="W14" t="n">
-        <v>10.9086</v>
+        <v>11.9388</v>
       </c>
       <c r="X14" t="n">
-        <v>-16.313</v>
+        <v>-3.673</v>
       </c>
       <c r="Y14" t="n">
-        <v>-39.878</v>
+        <v>-5.5084</v>
       </c>
       <c r="Z14" t="n">
-        <v>-30.5805</v>
+        <v>-32.1159</v>
       </c>
       <c r="AA14" t="n">
-        <v>-9.3156</v>
+        <v>3.0509</v>
       </c>
       <c r="AB14" t="n">
-        <v>-19.7567</v>
+        <v>-1.2986</v>
       </c>
       <c r="AC14" t="n">
-        <v>-11.997</v>
+        <v>-12.6628</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>267.13</v>
+        <v>266.04</v>
       </c>
       <c r="C15" t="n">
-        <v>274.93</v>
+        <v>286.15</v>
       </c>
       <c r="D15" t="n">
-        <v>226</v>
+        <v>265</v>
       </c>
       <c r="E15" t="n">
-        <v>226.19</v>
+        <v>279.29</v>
       </c>
       <c r="F15" t="n">
-        <v>84.19</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="G15" t="n">
-        <v>84.83</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="H15" t="n">
-        <v>79.86</v>
+        <v>80.63</v>
       </c>
       <c r="I15" t="n">
-        <v>79.93000000000001</v>
+        <v>82.87</v>
       </c>
       <c r="J15" t="n">
-        <v>3.9836</v>
+        <v>3.8156</v>
       </c>
       <c r="K15" t="n">
-        <v>4.5965</v>
+        <v>3.8254</v>
       </c>
       <c r="L15" t="n">
-        <v>3.865</v>
+        <v>3.4103</v>
       </c>
       <c r="M15" t="n">
-        <v>4.5767</v>
+        <v>3.5487</v>
       </c>
       <c r="N15" t="n">
-        <v>35.9652</v>
+        <v>36.6149</v>
       </c>
       <c r="O15" t="n">
-        <v>37.7861</v>
+        <v>37.3531</v>
       </c>
       <c r="P15" t="n">
-        <v>35.6896</v>
+        <v>35.857</v>
       </c>
       <c r="Q15" t="n">
-        <v>37.7468</v>
+        <v>36.1719</v>
       </c>
       <c r="R15" t="n">
-        <v>-16.9945</v>
+        <v>19.4262</v>
       </c>
       <c r="S15" t="n">
-        <v>0.9822</v>
+        <v>2.4917</v>
       </c>
       <c r="T15" t="n">
-        <v>12.1529</v>
+        <v>24.6886</v>
       </c>
       <c r="U15" t="n">
-        <v>-5.5089</v>
+        <v>6.8739</v>
       </c>
       <c r="V15" t="n">
-        <v>5.1572</v>
+        <v>-2.0333</v>
       </c>
       <c r="W15" t="n">
-        <v>8.4238</v>
+        <v>9.0251</v>
       </c>
       <c r="X15" t="n">
-        <v>17.216</v>
+        <v>-19.5051</v>
       </c>
       <c r="Y15" t="n">
-        <v>-6.8413</v>
+        <v>-9.1126</v>
       </c>
       <c r="Z15" t="n">
-        <v>-21.922</v>
+        <v>-27.7662</v>
       </c>
       <c r="AA15" t="n">
-        <v>5.6182</v>
+        <v>-7.0093</v>
       </c>
       <c r="AB15" t="n">
-        <v>-6.074</v>
+        <v>1.2116</v>
       </c>
       <c r="AC15" t="n">
-        <v>-10.1241</v>
+        <v>-9.992800000000001</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>247.42</v>
+        <v>299.26</v>
       </c>
       <c r="C16" t="n">
-        <v>259.79</v>
+        <v>302</v>
       </c>
       <c r="D16" t="n">
-        <v>233.3</v>
+        <v>286.24</v>
       </c>
       <c r="E16" t="n">
-        <v>233.86</v>
+        <v>300.77</v>
       </c>
       <c r="F16" t="n">
-        <v>81.67</v>
+        <v>83.95</v>
       </c>
       <c r="G16" t="n">
-        <v>81.81</v>
+        <v>85.11</v>
       </c>
       <c r="H16" t="n">
-        <v>76.94</v>
+        <v>81.39</v>
       </c>
       <c r="I16" t="n">
-        <v>77.54000000000001</v>
+        <v>82.58</v>
       </c>
       <c r="J16" t="n">
-        <v>4.122</v>
+        <v>3.2917</v>
       </c>
       <c r="K16" t="n">
-        <v>4.4086</v>
+        <v>3.4498</v>
       </c>
       <c r="L16" t="n">
-        <v>3.8749</v>
+        <v>3.2521</v>
       </c>
       <c r="M16" t="n">
-        <v>4.4086</v>
+        <v>3.262</v>
       </c>
       <c r="N16" t="n">
-        <v>36.9397</v>
+        <v>35.7389</v>
       </c>
       <c r="O16" t="n">
-        <v>39.1641</v>
+        <v>36.8511</v>
       </c>
       <c r="P16" t="n">
-        <v>36.8708</v>
+        <v>35.2369</v>
       </c>
       <c r="Q16" t="n">
-        <v>38.8984</v>
+        <v>36.3491</v>
       </c>
       <c r="R16" t="n">
-        <v>3.391</v>
+        <v>7.6909</v>
       </c>
       <c r="S16" t="n">
-        <v>-0.3494</v>
+        <v>32.9723</v>
       </c>
       <c r="T16" t="n">
-        <v>29.4547</v>
+        <v>28.1618</v>
       </c>
       <c r="U16" t="n">
-        <v>-2.9901</v>
+        <v>-0.3499</v>
       </c>
       <c r="V16" t="n">
-        <v>0.0258</v>
+        <v>3.3154</v>
       </c>
       <c r="W16" t="n">
-        <v>11.9388</v>
+        <v>6.5273</v>
       </c>
       <c r="X16" t="n">
-        <v>-3.673</v>
+        <v>-8.079000000000001</v>
       </c>
       <c r="Y16" t="n">
-        <v>-5.5084</v>
+        <v>-28.7259</v>
       </c>
       <c r="Z16" t="n">
-        <v>-32.1159</v>
+        <v>-30.084</v>
       </c>
       <c r="AA16" t="n">
-        <v>3.0509</v>
+        <v>0.4899</v>
       </c>
       <c r="AB16" t="n">
-        <v>-1.2986</v>
+        <v>-3.7028</v>
       </c>
       <c r="AC16" t="n">
-        <v>-12.6628</v>
+        <v>-7.7673</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>266.04</v>
+        <v>236</v>
       </c>
       <c r="C17" t="n">
-        <v>286.15</v>
+        <v>252.98</v>
       </c>
       <c r="D17" t="n">
-        <v>265</v>
+        <v>223</v>
       </c>
       <c r="E17" t="n">
-        <v>279.29</v>
+        <v>231.42</v>
       </c>
       <c r="F17" t="n">
-        <v>82.09999999999999</v>
+        <v>75.12</v>
       </c>
       <c r="G17" t="n">
-        <v>83.59999999999999</v>
+        <v>77.73999999999999</v>
       </c>
       <c r="H17" t="n">
-        <v>80.63</v>
+        <v>73.91</v>
       </c>
       <c r="I17" t="n">
-        <v>82.87</v>
+        <v>74.44</v>
       </c>
       <c r="J17" t="n">
-        <v>3.8156</v>
+        <v>3.99</v>
       </c>
       <c r="K17" t="n">
-        <v>3.8254</v>
+        <v>4.13</v>
       </c>
       <c r="L17" t="n">
-        <v>3.4103</v>
+        <v>3.8</v>
       </c>
       <c r="M17" t="n">
-        <v>3.5487</v>
+        <v>4.04</v>
       </c>
       <c r="N17" t="n">
-        <v>36.6149</v>
+        <v>39.6267</v>
       </c>
       <c r="O17" t="n">
-        <v>37.3531</v>
+        <v>40.1582</v>
       </c>
       <c r="P17" t="n">
-        <v>35.857</v>
+        <v>38.4653</v>
       </c>
       <c r="Q17" t="n">
-        <v>36.1719</v>
+        <v>39.922</v>
       </c>
       <c r="R17" t="n">
-        <v>19.4262</v>
+        <v>-23.0575</v>
       </c>
       <c r="S17" t="n">
-        <v>2.4917</v>
+        <v>-1.0434</v>
       </c>
       <c r="T17" t="n">
-        <v>24.6886</v>
+        <v>-15.0752</v>
       </c>
       <c r="U17" t="n">
-        <v>6.8739</v>
+        <v>-9.857100000000001</v>
       </c>
       <c r="V17" t="n">
-        <v>-2.0333</v>
+        <v>-3.9979</v>
       </c>
       <c r="W17" t="n">
-        <v>9.0251</v>
+        <v>-11.9991</v>
       </c>
       <c r="X17" t="n">
-        <v>-19.5051</v>
+        <v>23.8504</v>
       </c>
       <c r="Y17" t="n">
-        <v>-9.1126</v>
+        <v>-8.360900000000001</v>
       </c>
       <c r="Z17" t="n">
-        <v>-27.7662</v>
+        <v>3.4704</v>
       </c>
       <c r="AA17" t="n">
-        <v>-7.0093</v>
+        <v>9.8294</v>
       </c>
       <c r="AB17" t="n">
-        <v>1.2116</v>
+        <v>2.6315</v>
       </c>
       <c r="AC17" t="n">
-        <v>-9.992800000000001</v>
+        <v>11.7046</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>299.26</v>
+        <v>233.11</v>
       </c>
       <c r="C18" t="n">
-        <v>302</v>
+        <v>237</v>
       </c>
       <c r="D18" t="n">
-        <v>286.24</v>
+        <v>211.13</v>
       </c>
       <c r="E18" t="n">
-        <v>300.77</v>
+        <v>229.57</v>
       </c>
       <c r="F18" t="n">
-        <v>83.95</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>85.11</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="H18" t="n">
-        <v>81.39</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="I18" t="n">
-        <v>82.58</v>
+        <v>73.3</v>
       </c>
       <c r="J18" t="n">
-        <v>3.2917</v>
+        <v>4</v>
       </c>
       <c r="K18" t="n">
-        <v>3.4498</v>
+        <v>4.39</v>
       </c>
       <c r="L18" t="n">
-        <v>3.2521</v>
+        <v>3.92</v>
       </c>
       <c r="M18" t="n">
-        <v>3.262</v>
+        <v>4.08</v>
       </c>
       <c r="N18" t="n">
-        <v>35.7389</v>
+        <v>39.66</v>
       </c>
       <c r="O18" t="n">
-        <v>36.8511</v>
+        <v>41.49</v>
       </c>
       <c r="P18" t="n">
-        <v>35.2369</v>
+        <v>38.9</v>
       </c>
       <c r="Q18" t="n">
-        <v>36.3491</v>
+        <v>40.45</v>
       </c>
       <c r="R18" t="n">
-        <v>7.6909</v>
+        <v>-0.7994</v>
       </c>
       <c r="S18" t="n">
-        <v>32.9723</v>
+        <v>-17.8023</v>
       </c>
       <c r="T18" t="n">
-        <v>28.1618</v>
+        <v>1.4943</v>
       </c>
       <c r="U18" t="n">
-        <v>-0.3499</v>
+        <v>-1.5314</v>
       </c>
       <c r="V18" t="n">
-        <v>3.3154</v>
+        <v>-11.5482</v>
       </c>
       <c r="W18" t="n">
-        <v>6.5273</v>
+        <v>-8.2948</v>
       </c>
       <c r="X18" t="n">
-        <v>-8.079000000000001</v>
+        <v>0.9901</v>
       </c>
       <c r="Y18" t="n">
-        <v>-28.7259</v>
+        <v>14.9717</v>
       </c>
       <c r="Z18" t="n">
-        <v>-30.084</v>
+        <v>-10.8528</v>
       </c>
       <c r="AA18" t="n">
-        <v>0.4899</v>
+        <v>1.3226</v>
       </c>
       <c r="AB18" t="n">
-        <v>-3.7028</v>
+        <v>11.8271</v>
       </c>
       <c r="AC18" t="n">
-        <v>-7.7673</v>
+        <v>7.1614</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>236</v>
+        <v>268.05</v>
       </c>
       <c r="C19" t="n">
-        <v>252.98</v>
+        <v>268.4</v>
       </c>
       <c r="D19" t="n">
-        <v>223</v>
+        <v>225.74</v>
       </c>
       <c r="E19" t="n">
-        <v>231.42</v>
+        <v>252.61</v>
       </c>
       <c r="F19" t="n">
-        <v>75.12</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="G19" t="n">
-        <v>77.73999999999999</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>73.91</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>74.44</v>
+        <v>74.95</v>
       </c>
       <c r="J19" t="n">
-        <v>3.99</v>
+        <v>3.38</v>
       </c>
       <c r="K19" t="n">
-        <v>4.13</v>
+        <v>4.15</v>
       </c>
       <c r="L19" t="n">
-        <v>3.8</v>
+        <v>3.37</v>
       </c>
       <c r="M19" t="n">
-        <v>4.04</v>
+        <v>3.63</v>
       </c>
       <c r="N19" t="n">
-        <v>39.6267</v>
+        <v>37.87</v>
       </c>
       <c r="O19" t="n">
-        <v>40.1582</v>
+        <v>41.37</v>
       </c>
       <c r="P19" t="n">
-        <v>38.4653</v>
+        <v>37.71</v>
       </c>
       <c r="Q19" t="n">
-        <v>39.922</v>
+        <v>39.47</v>
       </c>
       <c r="R19" t="n">
-        <v>-23.0575</v>
+        <v>10.0362</v>
       </c>
       <c r="S19" t="n">
-        <v>-1.0434</v>
+        <v>-16.0122</v>
       </c>
       <c r="T19" t="n">
-        <v>-15.0752</v>
+        <v>8.0176</v>
       </c>
       <c r="U19" t="n">
-        <v>-9.857100000000001</v>
+        <v>2.251</v>
       </c>
       <c r="V19" t="n">
-        <v>-3.9979</v>
+        <v>-9.2395</v>
       </c>
       <c r="W19" t="n">
-        <v>-11.9991</v>
+        <v>-3.3402</v>
       </c>
       <c r="X19" t="n">
-        <v>23.8504</v>
+        <v>-11.0294</v>
       </c>
       <c r="Y19" t="n">
-        <v>-8.360900000000001</v>
+        <v>11.2814</v>
       </c>
       <c r="Z19" t="n">
-        <v>3.4704</v>
+        <v>-17.6609</v>
       </c>
       <c r="AA19" t="n">
-        <v>9.8294</v>
+        <v>-2.4227</v>
       </c>
       <c r="AB19" t="n">
-        <v>2.6315</v>
+        <v>8.585900000000001</v>
       </c>
       <c r="AC19" t="n">
-        <v>11.7046</v>
+        <v>1.4695</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>233.11</v>
+        <v>226.24</v>
       </c>
       <c r="C20" t="n">
-        <v>237</v>
+        <v>231.25</v>
       </c>
       <c r="D20" t="n">
-        <v>211.13</v>
+        <v>212.1</v>
       </c>
       <c r="E20" t="n">
-        <v>229.57</v>
+        <v>215.6</v>
       </c>
       <c r="F20" t="n">
-        <v>74.79000000000001</v>
+        <v>72.09</v>
       </c>
       <c r="G20" t="n">
-        <v>76.18000000000001</v>
+        <v>74.69</v>
       </c>
       <c r="H20" t="n">
-        <v>71.34999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="I20" t="n">
-        <v>73.3</v>
+        <v>71.83</v>
       </c>
       <c r="J20" t="n">
-        <v>4</v>
+        <v>4.04</v>
       </c>
       <c r="K20" t="n">
-        <v>4.39</v>
+        <v>4.25</v>
       </c>
       <c r="L20" t="n">
-        <v>3.92</v>
+        <v>3.95</v>
       </c>
       <c r="M20" t="n">
-        <v>4.08</v>
+        <v>4.24</v>
       </c>
       <c r="N20" t="n">
-        <v>39.66</v>
+        <v>41.08</v>
       </c>
       <c r="O20" t="n">
-        <v>41.49</v>
+        <v>41.79</v>
       </c>
       <c r="P20" t="n">
-        <v>38.9</v>
+        <v>39.69</v>
       </c>
       <c r="Q20" t="n">
-        <v>40.45</v>
+        <v>41.31</v>
       </c>
       <c r="R20" t="n">
-        <v>-0.7994</v>
+        <v>-14.651</v>
       </c>
       <c r="S20" t="n">
-        <v>-17.8023</v>
+        <v>-6.8361</v>
       </c>
       <c r="T20" t="n">
-        <v>1.4943</v>
+        <v>-22.8043</v>
       </c>
       <c r="U20" t="n">
-        <v>-1.5314</v>
+        <v>-4.1628</v>
       </c>
       <c r="V20" t="n">
-        <v>-11.5482</v>
+        <v>-3.5062</v>
       </c>
       <c r="W20" t="n">
-        <v>-8.2948</v>
+        <v>-13.3221</v>
       </c>
       <c r="X20" t="n">
-        <v>0.9901</v>
+        <v>16.8044</v>
       </c>
       <c r="Y20" t="n">
-        <v>14.9717</v>
+        <v>4.9505</v>
       </c>
       <c r="Z20" t="n">
-        <v>-10.8528</v>
+        <v>19.4804</v>
       </c>
       <c r="AA20" t="n">
-        <v>1.3226</v>
+        <v>4.6618</v>
       </c>
       <c r="AB20" t="n">
-        <v>11.8271</v>
+        <v>3.4768</v>
       </c>
       <c r="AC20" t="n">
-        <v>7.1614</v>
+        <v>14.2047</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>268.05</v>
+        <v>216.36</v>
       </c>
       <c r="C21" t="n">
-        <v>268.4</v>
+        <v>238.6533</v>
       </c>
       <c r="D21" t="n">
-        <v>225.74</v>
+        <v>192.3</v>
       </c>
       <c r="E21" t="n">
-        <v>252.61</v>
+        <v>236.52</v>
       </c>
       <c r="F21" t="n">
-        <v>77.95999999999999</v>
+        <v>74.12</v>
       </c>
       <c r="G21" t="n">
-        <v>78.23999999999999</v>
+        <v>77.375</v>
       </c>
       <c r="H21" t="n">
-        <v>71.59999999999999</v>
+        <v>71.45</v>
       </c>
       <c r="I21" t="n">
-        <v>74.95</v>
+        <v>77.19</v>
       </c>
       <c r="J21" t="n">
-        <v>3.38</v>
+        <v>4.1597</v>
       </c>
       <c r="K21" t="n">
-        <v>4.15</v>
+        <v>4.63</v>
       </c>
       <c r="L21" t="n">
-        <v>3.37</v>
+        <v>3.7</v>
       </c>
       <c r="M21" t="n">
-        <v>3.63</v>
+        <v>3.72</v>
       </c>
       <c r="N21" t="n">
-        <v>37.87</v>
+        <v>39.89</v>
       </c>
       <c r="O21" t="n">
-        <v>41.37</v>
+        <v>41.4299</v>
       </c>
       <c r="P21" t="n">
-        <v>37.71</v>
+        <v>38.08</v>
       </c>
       <c r="Q21" t="n">
-        <v>39.47</v>
+        <v>38.16</v>
       </c>
       <c r="R21" t="n">
-        <v>10.0362</v>
+        <v>9.703200000000001</v>
       </c>
       <c r="S21" t="n">
-        <v>-16.0122</v>
+        <v>3.0274</v>
       </c>
       <c r="T21" t="n">
-        <v>8.0176</v>
+        <v>-21.3618</v>
       </c>
       <c r="U21" t="n">
-        <v>2.251</v>
+        <v>7.4621</v>
       </c>
       <c r="V21" t="n">
-        <v>-9.2395</v>
+        <v>5.307</v>
       </c>
       <c r="W21" t="n">
-        <v>-3.3402</v>
+        <v>-6.527</v>
       </c>
       <c r="X21" t="n">
-        <v>-11.0294</v>
+        <v>-12.2642</v>
       </c>
       <c r="Y21" t="n">
-        <v>11.2814</v>
+        <v>-8.823499999999999</v>
       </c>
       <c r="Z21" t="n">
-        <v>-17.6609</v>
+        <v>14.0405</v>
       </c>
       <c r="AA21" t="n">
-        <v>-2.4227</v>
+        <v>-7.6253</v>
       </c>
       <c r="AB21" t="n">
-        <v>8.585900000000001</v>
+        <v>-5.6613</v>
       </c>
       <c r="AC21" t="n">
-        <v>1.4695</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-06-26</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>226.24</v>
-      </c>
-      <c r="C22" t="n">
-        <v>231.21</v>
-      </c>
-      <c r="D22" t="n">
-        <v>212.1</v>
-      </c>
-      <c r="E22" t="n">
-        <v>215.6</v>
-      </c>
-      <c r="F22" t="n">
-        <v>72.065</v>
-      </c>
-      <c r="G22" t="n">
-        <v>74.69</v>
-      </c>
-      <c r="H22" t="n">
-        <v>70.72</v>
-      </c>
-      <c r="I22" t="n">
-        <v>71.83</v>
-      </c>
-      <c r="J22" t="n">
-        <v>4.035</v>
-      </c>
-      <c r="K22" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="L22" t="n">
-        <v>3.95</v>
-      </c>
-      <c r="M22" t="n">
-        <v>4.24</v>
-      </c>
-      <c r="N22" t="n">
-        <v>41.085</v>
-      </c>
-      <c r="O22" t="n">
-        <v>41.79</v>
-      </c>
-      <c r="P22" t="n">
-        <v>39.69</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>41.31</v>
-      </c>
-      <c r="R22" t="n">
-        <v>-14.651</v>
-      </c>
-      <c r="S22" t="n">
-        <v>-6.8361</v>
-      </c>
-      <c r="T22" t="n">
-        <v>-22.8043</v>
-      </c>
-      <c r="U22" t="n">
-        <v>-4.1628</v>
-      </c>
-      <c r="V22" t="n">
-        <v>-3.5062</v>
-      </c>
-      <c r="W22" t="n">
-        <v>-13.3221</v>
-      </c>
-      <c r="X22" t="n">
-        <v>16.8044</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>4.9505</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>19.4804</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>4.6618</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>3.4768</v>
-      </c>
-      <c r="AC22" t="n">
-        <v>14.2047</v>
+        <v>4.982</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-06-30 23:13
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC21"/>
+  <dimension ref="A1:AC22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2196,7 +2196,7 @@
         <v>216.36</v>
       </c>
       <c r="C21" t="n">
-        <v>238.6533</v>
+        <v>238.65</v>
       </c>
       <c r="D21" t="n">
         <v>192.3</v>
@@ -2208,7 +2208,7 @@
         <v>74.12</v>
       </c>
       <c r="G21" t="n">
-        <v>77.375</v>
+        <v>77.38</v>
       </c>
       <c r="H21" t="n">
         <v>71.45</v>
@@ -2217,7 +2217,7 @@
         <v>77.19</v>
       </c>
       <c r="J21" t="n">
-        <v>4.1597</v>
+        <v>4.16</v>
       </c>
       <c r="K21" t="n">
         <v>4.63</v>
@@ -2229,10 +2229,10 @@
         <v>3.72</v>
       </c>
       <c r="N21" t="n">
-        <v>39.89</v>
+        <v>39.91</v>
       </c>
       <c r="O21" t="n">
-        <v>41.4299</v>
+        <v>41.43</v>
       </c>
       <c r="P21" t="n">
         <v>38.08</v>
@@ -2275,6 +2275,97 @@
       </c>
       <c r="AC21" t="n">
         <v>4.982</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>241.45</v>
+      </c>
+      <c r="C22" t="n">
+        <v>272</v>
+      </c>
+      <c r="D22" t="n">
+        <v>240.601</v>
+      </c>
+      <c r="E22" t="n">
+        <v>266.71</v>
+      </c>
+      <c r="F22" t="n">
+        <v>77.262</v>
+      </c>
+      <c r="G22" t="n">
+        <v>81.54000000000001</v>
+      </c>
+      <c r="H22" t="n">
+        <v>77.15000000000001</v>
+      </c>
+      <c r="I22" t="n">
+        <v>81</v>
+      </c>
+      <c r="J22" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="K22" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="L22" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="M22" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="N22" t="n">
+        <v>38.16</v>
+      </c>
+      <c r="O22" t="n">
+        <v>38.195</v>
+      </c>
+      <c r="P22" t="n">
+        <v>36.03</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>36.31</v>
+      </c>
+      <c r="R22" t="n">
+        <v>12.7642</v>
+      </c>
+      <c r="S22" t="n">
+        <v>5.5817</v>
+      </c>
+      <c r="T22" t="n">
+        <v>15.2493</v>
+      </c>
+      <c r="U22" t="n">
+        <v>4.9359</v>
+      </c>
+      <c r="V22" t="n">
+        <v>8.071999999999999</v>
+      </c>
+      <c r="W22" t="n">
+        <v>8.8125</v>
+      </c>
+      <c r="X22" t="n">
+        <v>-12.9032</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>-10.7438</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>-19.802</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>-4.848</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>-8.0061</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>-9.047599999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-07-01 23:15
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>217.27</v>
+        <v>243.18</v>
       </c>
       <c r="C2" t="n">
-        <v>234.06</v>
+        <v>267.08</v>
       </c>
       <c r="D2" t="n">
-        <v>210.14</v>
+        <v>238.82</v>
       </c>
       <c r="E2" t="n">
-        <v>227.03</v>
+        <v>266.32</v>
       </c>
       <c r="F2" t="n">
-        <v>84.15000000000001</v>
+        <v>85.94</v>
       </c>
       <c r="G2" t="n">
-        <v>87.06</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>83.75</v>
+        <v>84.83</v>
       </c>
       <c r="I2" t="n">
-        <v>86.04000000000001</v>
+        <v>87.22</v>
       </c>
       <c r="J2" t="n">
-        <v>6.4746</v>
+        <v>5.7332</v>
       </c>
       <c r="K2" t="n">
-        <v>6.6624</v>
+        <v>5.8617</v>
       </c>
       <c r="L2" t="n">
-        <v>5.9803</v>
+        <v>5.0907</v>
       </c>
       <c r="M2" t="n">
-        <v>6.1879</v>
+        <v>5.1105</v>
       </c>
       <c r="N2" t="n">
-        <v>37.668</v>
+        <v>36.8806</v>
       </c>
       <c r="O2" t="n">
-        <v>37.855</v>
+        <v>37.3531</v>
       </c>
       <c r="P2" t="n">
-        <v>36.3786</v>
+        <v>36.2802</v>
       </c>
       <c r="Q2" t="n">
-        <v>36.8314</v>
+        <v>36.3294</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>243.18</v>
+        <v>281.47</v>
       </c>
       <c r="C3" t="n">
-        <v>267.08</v>
+        <v>284.58</v>
       </c>
       <c r="D3" t="n">
-        <v>238.82</v>
+        <v>257.26</v>
       </c>
       <c r="E3" t="n">
-        <v>266.32</v>
+        <v>280.54</v>
       </c>
       <c r="F3" t="n">
-        <v>85.94</v>
+        <v>87.68000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>87.31999999999999</v>
+        <v>88.09</v>
       </c>
       <c r="H3" t="n">
-        <v>84.83</v>
+        <v>85.41</v>
       </c>
       <c r="I3" t="n">
-        <v>87.22</v>
+        <v>86.56</v>
       </c>
       <c r="J3" t="n">
-        <v>5.7332</v>
+        <v>4.8238</v>
       </c>
       <c r="K3" t="n">
-        <v>5.8617</v>
+        <v>5.2884</v>
       </c>
       <c r="L3" t="n">
-        <v>5.0907</v>
+        <v>4.7645</v>
       </c>
       <c r="M3" t="n">
-        <v>5.1105</v>
+        <v>4.8535</v>
       </c>
       <c r="N3" t="n">
-        <v>36.8806</v>
+        <v>36.1522</v>
       </c>
       <c r="O3" t="n">
-        <v>37.3531</v>
+        <v>37.0971</v>
       </c>
       <c r="P3" t="n">
-        <v>36.2802</v>
+        <v>35.9751</v>
       </c>
       <c r="Q3" t="n">
-        <v>36.3294</v>
+        <v>36.605</v>
       </c>
       <c r="R3" t="n">
-        <v>17.3061</v>
+        <v>5.3394</v>
       </c>
       <c r="U3" t="n">
-        <v>1.3715</v>
+        <v>-0.7567</v>
       </c>
       <c r="X3" t="n">
-        <v>-17.4114</v>
+        <v>-5.0289</v>
       </c>
       <c r="AA3" t="n">
-        <v>-1.363</v>
+        <v>0.7586000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>281.47</v>
+        <v>242.04</v>
       </c>
       <c r="C4" t="n">
-        <v>284.58</v>
+        <v>274.5</v>
       </c>
       <c r="D4" t="n">
-        <v>257.26</v>
+        <v>228.55</v>
       </c>
       <c r="E4" t="n">
-        <v>280.54</v>
+        <v>262.7</v>
       </c>
       <c r="F4" t="n">
-        <v>87.68000000000001</v>
+        <v>83.47</v>
       </c>
       <c r="G4" t="n">
-        <v>88.09</v>
+        <v>86.25</v>
       </c>
       <c r="H4" t="n">
-        <v>85.41</v>
+        <v>82.48</v>
       </c>
       <c r="I4" t="n">
-        <v>86.56</v>
+        <v>85.22</v>
       </c>
       <c r="J4" t="n">
-        <v>4.8238</v>
+        <v>5.5059</v>
       </c>
       <c r="K4" t="n">
-        <v>5.2884</v>
+        <v>5.7431</v>
       </c>
       <c r="L4" t="n">
-        <v>4.7645</v>
+        <v>4.9424</v>
       </c>
       <c r="M4" t="n">
-        <v>4.8535</v>
+        <v>5.1401</v>
       </c>
       <c r="N4" t="n">
-        <v>36.1522</v>
+        <v>37.9239</v>
       </c>
       <c r="O4" t="n">
-        <v>37.0971</v>
+        <v>38.3472</v>
       </c>
       <c r="P4" t="n">
-        <v>35.9751</v>
+        <v>36.7428</v>
       </c>
       <c r="Q4" t="n">
-        <v>36.605</v>
+        <v>37.166</v>
       </c>
       <c r="R4" t="n">
-        <v>5.3394</v>
+        <v>-6.3592</v>
       </c>
       <c r="U4" t="n">
-        <v>-0.7567</v>
+        <v>-1.5481</v>
       </c>
       <c r="X4" t="n">
-        <v>-5.0289</v>
+        <v>5.905</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.7586000000000001</v>
+        <v>1.5326</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>242.04</v>
+        <v>230.85</v>
       </c>
       <c r="C5" t="n">
-        <v>274.5</v>
+        <v>233.69</v>
       </c>
       <c r="D5" t="n">
-        <v>228.55</v>
+        <v>181.81</v>
       </c>
       <c r="E5" t="n">
-        <v>262.7</v>
+        <v>182.54</v>
       </c>
       <c r="F5" t="n">
-        <v>83.47</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>86.25</v>
+        <v>82.08</v>
       </c>
       <c r="H5" t="n">
-        <v>82.48</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="I5" t="n">
-        <v>85.22</v>
+        <v>73.05</v>
       </c>
       <c r="J5" t="n">
-        <v>5.5059</v>
+        <v>5.7925</v>
       </c>
       <c r="K5" t="n">
-        <v>5.7431</v>
+        <v>6.7711</v>
       </c>
       <c r="L5" t="n">
-        <v>4.9424</v>
+        <v>5.7233</v>
       </c>
       <c r="M5" t="n">
-        <v>5.1401</v>
+        <v>6.7612</v>
       </c>
       <c r="N5" t="n">
-        <v>37.9239</v>
+        <v>38.7999</v>
       </c>
       <c r="O5" t="n">
-        <v>38.3472</v>
+        <v>42.6681</v>
       </c>
       <c r="P5" t="n">
-        <v>36.7428</v>
+        <v>38.5637</v>
       </c>
       <c r="Q5" t="n">
-        <v>37.166</v>
+        <v>42.5106</v>
       </c>
       <c r="R5" t="n">
-        <v>-6.3592</v>
+        <v>-30.5139</v>
       </c>
       <c r="S5" t="n">
-        <v>15.7116</v>
+        <v>-31.4584</v>
       </c>
       <c r="U5" t="n">
-        <v>-1.5481</v>
+        <v>-14.2807</v>
       </c>
       <c r="V5" t="n">
-        <v>-0.953</v>
+        <v>-16.2463</v>
       </c>
       <c r="X5" t="n">
-        <v>5.905</v>
+        <v>31.5383</v>
       </c>
       <c r="Y5" t="n">
-        <v>-16.933</v>
+        <v>32.3002</v>
       </c>
       <c r="AA5" t="n">
-        <v>1.5326</v>
+        <v>14.3803</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.9085</v>
+        <v>17.0143</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>230.85</v>
+        <v>210.62</v>
       </c>
       <c r="C6" t="n">
-        <v>233.69</v>
+        <v>222.19</v>
       </c>
       <c r="D6" t="n">
-        <v>181.81</v>
+        <v>201.69</v>
       </c>
       <c r="E6" t="n">
-        <v>182.54</v>
+        <v>211.44</v>
       </c>
       <c r="F6" t="n">
-        <v>81.56999999999999</v>
+        <v>76.86</v>
       </c>
       <c r="G6" t="n">
-        <v>82.08</v>
+        <v>78.47</v>
       </c>
       <c r="H6" t="n">
-        <v>72.68000000000001</v>
+        <v>75.38</v>
       </c>
       <c r="I6" t="n">
-        <v>73.05</v>
+        <v>76.27</v>
       </c>
       <c r="J6" t="n">
-        <v>5.7925</v>
+        <v>5.6442</v>
       </c>
       <c r="K6" t="n">
-        <v>6.7711</v>
+        <v>5.9803</v>
       </c>
       <c r="L6" t="n">
-        <v>5.7233</v>
+        <v>5.2093</v>
       </c>
       <c r="M6" t="n">
-        <v>6.7612</v>
+        <v>5.6245</v>
       </c>
       <c r="N6" t="n">
-        <v>38.7999</v>
+        <v>40.2763</v>
       </c>
       <c r="O6" t="n">
-        <v>42.6681</v>
+        <v>41.1228</v>
       </c>
       <c r="P6" t="n">
-        <v>38.5637</v>
+        <v>39.3314</v>
       </c>
       <c r="Q6" t="n">
-        <v>42.5106</v>
+        <v>40.611</v>
       </c>
       <c r="R6" t="n">
-        <v>-30.5139</v>
+        <v>15.8321</v>
       </c>
       <c r="S6" t="n">
-        <v>-31.4584</v>
+        <v>-24.6311</v>
       </c>
       <c r="U6" t="n">
-        <v>-14.2807</v>
+        <v>4.4079</v>
       </c>
       <c r="V6" t="n">
-        <v>-16.2463</v>
+        <v>-11.8877</v>
       </c>
       <c r="X6" t="n">
-        <v>31.5383</v>
+        <v>-16.8121</v>
       </c>
       <c r="Y6" t="n">
-        <v>32.3002</v>
+        <v>15.8854</v>
       </c>
       <c r="AA6" t="n">
-        <v>14.3803</v>
+        <v>-4.4685</v>
       </c>
       <c r="AB6" t="n">
-        <v>17.0143</v>
+        <v>10.9439</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>210.62</v>
+        <v>227.06</v>
       </c>
       <c r="C7" t="n">
-        <v>222.19</v>
+        <v>231.02</v>
       </c>
       <c r="D7" t="n">
-        <v>201.69</v>
+        <v>157.56</v>
       </c>
       <c r="E7" t="n">
-        <v>211.44</v>
+        <v>201.68</v>
       </c>
       <c r="F7" t="n">
-        <v>76.86</v>
+        <v>78.48</v>
       </c>
       <c r="G7" t="n">
-        <v>78.47</v>
+        <v>79.34</v>
       </c>
       <c r="H7" t="n">
-        <v>75.38</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="I7" t="n">
-        <v>76.27</v>
+        <v>73.72</v>
       </c>
       <c r="J7" t="n">
-        <v>5.6442</v>
+        <v>5.1895</v>
       </c>
       <c r="K7" t="n">
-        <v>5.9803</v>
+        <v>7.0281</v>
       </c>
       <c r="L7" t="n">
-        <v>5.2093</v>
+        <v>5.0808</v>
       </c>
       <c r="M7" t="n">
-        <v>5.6245</v>
+        <v>5.8617</v>
       </c>
       <c r="N7" t="n">
-        <v>40.2763</v>
+        <v>39.4299</v>
       </c>
       <c r="O7" t="n">
-        <v>41.1228</v>
+        <v>45.6505</v>
       </c>
       <c r="P7" t="n">
-        <v>39.3314</v>
+        <v>38.9673</v>
       </c>
       <c r="Q7" t="n">
-        <v>40.611</v>
+        <v>41.9988</v>
       </c>
       <c r="R7" t="n">
-        <v>15.8321</v>
+        <v>-4.616</v>
       </c>
       <c r="S7" t="n">
-        <v>-24.6311</v>
+        <v>-23.228</v>
       </c>
       <c r="T7" t="n">
-        <v>-6.8669</v>
+        <v>-24.2716</v>
       </c>
       <c r="U7" t="n">
-        <v>4.4079</v>
+        <v>-3.3434</v>
       </c>
       <c r="V7" t="n">
-        <v>-11.8877</v>
+        <v>-13.4945</v>
       </c>
       <c r="W7" t="n">
-        <v>-11.3552</v>
+        <v>-15.4781</v>
       </c>
       <c r="X7" t="n">
-        <v>-16.8121</v>
+        <v>4.2173</v>
       </c>
       <c r="Y7" t="n">
-        <v>15.8854</v>
+        <v>14.0386</v>
       </c>
       <c r="Z7" t="n">
-        <v>-9.104900000000001</v>
+        <v>14.6991</v>
       </c>
       <c r="AA7" t="n">
-        <v>-4.4685</v>
+        <v>3.4173</v>
       </c>
       <c r="AB7" t="n">
-        <v>10.9439</v>
+        <v>13.0033</v>
       </c>
       <c r="AC7" t="n">
-        <v>10.2619</v>
+        <v>15.6055</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>227.06</v>
+        <v>191.54</v>
       </c>
       <c r="C8" t="n">
-        <v>231.02</v>
+        <v>212.99</v>
       </c>
       <c r="D8" t="n">
-        <v>157.56</v>
+        <v>177.3</v>
       </c>
       <c r="E8" t="n">
-        <v>201.68</v>
+        <v>180.65</v>
       </c>
       <c r="F8" t="n">
-        <v>78.48</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>79.34</v>
+        <v>74.7</v>
       </c>
       <c r="H8" t="n">
-        <v>66.79000000000001</v>
+        <v>69</v>
       </c>
       <c r="I8" t="n">
-        <v>73.72</v>
+        <v>69.27</v>
       </c>
       <c r="J8" t="n">
-        <v>5.1895</v>
+        <v>6.1681</v>
       </c>
       <c r="K8" t="n">
-        <v>7.0281</v>
+        <v>6.5734</v>
       </c>
       <c r="L8" t="n">
-        <v>5.0808</v>
+        <v>5.5355</v>
       </c>
       <c r="M8" t="n">
-        <v>5.8617</v>
+        <v>6.4943</v>
       </c>
       <c r="N8" t="n">
-        <v>39.4299</v>
+        <v>43.1209</v>
       </c>
       <c r="O8" t="n">
-        <v>45.6505</v>
+        <v>44.676</v>
       </c>
       <c r="P8" t="n">
-        <v>38.9673</v>
+        <v>41.4082</v>
       </c>
       <c r="Q8" t="n">
-        <v>41.9988</v>
+        <v>44.5382</v>
       </c>
       <c r="R8" t="n">
-        <v>-4.616</v>
+        <v>-10.4274</v>
       </c>
       <c r="S8" t="n">
-        <v>-23.228</v>
+        <v>-1.0354</v>
       </c>
       <c r="T8" t="n">
-        <v>-24.2716</v>
+        <v>-35.6063</v>
       </c>
       <c r="U8" t="n">
-        <v>-3.3434</v>
+        <v>-6.0364</v>
       </c>
       <c r="V8" t="n">
-        <v>-13.4945</v>
+        <v>-5.1745</v>
       </c>
       <c r="W8" t="n">
-        <v>-15.4781</v>
+        <v>-19.9746</v>
       </c>
       <c r="X8" t="n">
-        <v>4.2173</v>
+        <v>10.7921</v>
       </c>
       <c r="Y8" t="n">
-        <v>14.0386</v>
+        <v>-3.9475</v>
       </c>
       <c r="Z8" t="n">
-        <v>14.6991</v>
+        <v>33.8065</v>
       </c>
       <c r="AA8" t="n">
-        <v>3.4173</v>
+        <v>6.0464</v>
       </c>
       <c r="AB8" t="n">
-        <v>13.0033</v>
+        <v>4.7696</v>
       </c>
       <c r="AC8" t="n">
-        <v>15.6055</v>
+        <v>21.6724</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>191.54</v>
+        <v>192.3</v>
       </c>
       <c r="C9" t="n">
-        <v>212.99</v>
+        <v>225.63</v>
       </c>
       <c r="D9" t="n">
-        <v>177.3</v>
+        <v>192.3</v>
       </c>
       <c r="E9" t="n">
-        <v>180.65</v>
+        <v>223.99</v>
       </c>
       <c r="F9" t="n">
-        <v>71.68000000000001</v>
+        <v>70.89</v>
       </c>
       <c r="G9" t="n">
-        <v>74.7</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>69</v>
+        <v>69.59</v>
       </c>
       <c r="I9" t="n">
-        <v>69.27</v>
+        <v>76.01000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>6.1681</v>
+        <v>6.0298</v>
       </c>
       <c r="K9" t="n">
-        <v>6.5734</v>
+        <v>6.0298</v>
       </c>
       <c r="L9" t="n">
-        <v>5.5355</v>
+        <v>4.8436</v>
       </c>
       <c r="M9" t="n">
-        <v>6.4943</v>
+        <v>4.9128</v>
       </c>
       <c r="N9" t="n">
-        <v>43.1209</v>
+        <v>43.4851</v>
       </c>
       <c r="O9" t="n">
-        <v>44.676</v>
+        <v>44.302</v>
       </c>
       <c r="P9" t="n">
-        <v>41.4082</v>
+        <v>39.8039</v>
       </c>
       <c r="Q9" t="n">
-        <v>44.5382</v>
+        <v>40.1878</v>
       </c>
       <c r="R9" t="n">
-        <v>-10.4274</v>
+        <v>23.9911</v>
       </c>
       <c r="S9" t="n">
-        <v>-1.0354</v>
+        <v>5.9355</v>
       </c>
       <c r="T9" t="n">
-        <v>-35.6063</v>
+        <v>-14.7354</v>
       </c>
       <c r="U9" t="n">
-        <v>-6.0364</v>
+        <v>9.73</v>
       </c>
       <c r="V9" t="n">
-        <v>-5.1745</v>
+        <v>-0.3409</v>
       </c>
       <c r="W9" t="n">
-        <v>-19.9746</v>
+        <v>-10.8073</v>
       </c>
       <c r="X9" t="n">
-        <v>10.7921</v>
+        <v>-24.3521</v>
       </c>
       <c r="Y9" t="n">
-        <v>-3.9475</v>
+        <v>-12.6536</v>
       </c>
       <c r="Z9" t="n">
-        <v>33.8065</v>
+        <v>-4.4221</v>
       </c>
       <c r="AA9" t="n">
-        <v>6.0464</v>
+        <v>-9.767799999999999</v>
       </c>
       <c r="AB9" t="n">
-        <v>4.7696</v>
+        <v>-1.0421</v>
       </c>
       <c r="AC9" t="n">
-        <v>21.6724</v>
+        <v>8.1305</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>192.3</v>
+        <v>222.22</v>
       </c>
       <c r="C10" t="n">
-        <v>225.63</v>
+        <v>242.4</v>
       </c>
       <c r="D10" t="n">
-        <v>192.3</v>
+        <v>214.74</v>
       </c>
       <c r="E10" t="n">
-        <v>223.99</v>
+        <v>234.68</v>
       </c>
       <c r="F10" t="n">
-        <v>70.89</v>
+        <v>76.34</v>
       </c>
       <c r="G10" t="n">
-        <v>76.59999999999999</v>
+        <v>78.36</v>
       </c>
       <c r="H10" t="n">
-        <v>69.59</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="I10" t="n">
-        <v>76.01000000000001</v>
+        <v>77.52</v>
       </c>
       <c r="J10" t="n">
-        <v>6.0298</v>
+        <v>4.9523</v>
       </c>
       <c r="K10" t="n">
-        <v>6.0298</v>
+        <v>5.0907</v>
       </c>
       <c r="L10" t="n">
-        <v>4.8436</v>
+        <v>4.4877</v>
       </c>
       <c r="M10" t="n">
-        <v>4.9128</v>
+        <v>4.6656</v>
       </c>
       <c r="N10" t="n">
-        <v>43.4851</v>
+        <v>40.0106</v>
       </c>
       <c r="O10" t="n">
-        <v>44.302</v>
+        <v>41.0933</v>
       </c>
       <c r="P10" t="n">
-        <v>39.8039</v>
+        <v>38.9476</v>
       </c>
       <c r="Q10" t="n">
-        <v>40.1878</v>
+        <v>39.4102</v>
       </c>
       <c r="R10" t="n">
-        <v>23.9911</v>
+        <v>4.7725</v>
       </c>
       <c r="S10" t="n">
-        <v>5.9355</v>
+        <v>16.3626</v>
       </c>
       <c r="T10" t="n">
-        <v>-14.7354</v>
+        <v>28.5636</v>
       </c>
       <c r="U10" t="n">
-        <v>9.73</v>
+        <v>1.9866</v>
       </c>
       <c r="V10" t="n">
-        <v>-0.3409</v>
+        <v>5.1546</v>
       </c>
       <c r="W10" t="n">
-        <v>-10.8073</v>
+        <v>6.1191</v>
       </c>
       <c r="X10" t="n">
-        <v>-24.3521</v>
+        <v>-5.0318</v>
       </c>
       <c r="Y10" t="n">
-        <v>-12.6536</v>
+        <v>-20.4053</v>
       </c>
       <c r="Z10" t="n">
-        <v>-4.4221</v>
+        <v>-30.9945</v>
       </c>
       <c r="AA10" t="n">
-        <v>-9.767799999999999</v>
+        <v>-1.9349</v>
       </c>
       <c r="AB10" t="n">
-        <v>-1.0421</v>
+        <v>-6.1635</v>
       </c>
       <c r="AC10" t="n">
-        <v>8.1305</v>
+        <v>-7.2932</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>222.22</v>
+        <v>265.99</v>
       </c>
       <c r="C11" t="n">
-        <v>242.4</v>
+        <v>274.88</v>
       </c>
       <c r="D11" t="n">
-        <v>214.74</v>
+        <v>261.6</v>
       </c>
       <c r="E11" t="n">
-        <v>234.68</v>
+        <v>272.5</v>
       </c>
       <c r="F11" t="n">
-        <v>76.34</v>
+        <v>82.88</v>
       </c>
       <c r="G11" t="n">
-        <v>78.36</v>
+        <v>85.03</v>
       </c>
       <c r="H11" t="n">
-        <v>74.29000000000001</v>
+        <v>82.64</v>
       </c>
       <c r="I11" t="n">
-        <v>77.52</v>
+        <v>84.59</v>
       </c>
       <c r="J11" t="n">
-        <v>4.9523</v>
+        <v>4.0231</v>
       </c>
       <c r="K11" t="n">
-        <v>5.0907</v>
+        <v>4.122</v>
       </c>
       <c r="L11" t="n">
-        <v>4.4877</v>
+        <v>3.865</v>
       </c>
       <c r="M11" t="n">
-        <v>4.6656</v>
+        <v>3.9045</v>
       </c>
       <c r="N11" t="n">
-        <v>40.0106</v>
+        <v>36.6641</v>
       </c>
       <c r="O11" t="n">
-        <v>41.0933</v>
+        <v>36.7723</v>
       </c>
       <c r="P11" t="n">
-        <v>38.9476</v>
+        <v>35.5814</v>
       </c>
       <c r="Q11" t="n">
-        <v>39.4102</v>
+        <v>35.7389</v>
       </c>
       <c r="R11" t="n">
-        <v>4.7725</v>
+        <v>16.1156</v>
       </c>
       <c r="S11" t="n">
-        <v>16.3626</v>
+        <v>50.8442</v>
       </c>
       <c r="T11" t="n">
-        <v>28.5636</v>
+        <v>28.8782</v>
       </c>
       <c r="U11" t="n">
-        <v>1.9866</v>
+        <v>9.120200000000001</v>
       </c>
       <c r="V11" t="n">
-        <v>5.1546</v>
+        <v>22.1164</v>
       </c>
       <c r="W11" t="n">
-        <v>6.1191</v>
+        <v>10.9086</v>
       </c>
       <c r="X11" t="n">
-        <v>-5.0318</v>
+        <v>-16.313</v>
       </c>
       <c r="Y11" t="n">
-        <v>-20.4053</v>
+        <v>-39.878</v>
       </c>
       <c r="Z11" t="n">
-        <v>-30.9945</v>
+        <v>-30.5805</v>
       </c>
       <c r="AA11" t="n">
-        <v>-1.9349</v>
+        <v>-9.3156</v>
       </c>
       <c r="AB11" t="n">
-        <v>-6.1635</v>
+        <v>-19.7567</v>
       </c>
       <c r="AC11" t="n">
-        <v>-7.2932</v>
+        <v>-11.997</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>265.99</v>
+        <v>267.13</v>
       </c>
       <c r="C12" t="n">
-        <v>274.88</v>
+        <v>274.93</v>
       </c>
       <c r="D12" t="n">
-        <v>261.6</v>
+        <v>226</v>
       </c>
       <c r="E12" t="n">
-        <v>272.5</v>
+        <v>226.19</v>
       </c>
       <c r="F12" t="n">
-        <v>82.88</v>
+        <v>84.19</v>
       </c>
       <c r="G12" t="n">
-        <v>85.03</v>
+        <v>84.83</v>
       </c>
       <c r="H12" t="n">
-        <v>82.64</v>
+        <v>79.86</v>
       </c>
       <c r="I12" t="n">
-        <v>84.59</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>4.0231</v>
+        <v>3.9836</v>
       </c>
       <c r="K12" t="n">
-        <v>4.122</v>
+        <v>4.5965</v>
       </c>
       <c r="L12" t="n">
         <v>3.865</v>
       </c>
       <c r="M12" t="n">
-        <v>3.9045</v>
+        <v>4.5767</v>
       </c>
       <c r="N12" t="n">
-        <v>36.6641</v>
+        <v>35.9652</v>
       </c>
       <c r="O12" t="n">
-        <v>36.7723</v>
+        <v>37.7861</v>
       </c>
       <c r="P12" t="n">
-        <v>35.5814</v>
+        <v>35.6896</v>
       </c>
       <c r="Q12" t="n">
-        <v>35.7389</v>
+        <v>37.7468</v>
       </c>
       <c r="R12" t="n">
-        <v>16.1156</v>
+        <v>-16.9945</v>
       </c>
       <c r="S12" t="n">
-        <v>50.8442</v>
+        <v>0.9822</v>
       </c>
       <c r="T12" t="n">
-        <v>28.8782</v>
+        <v>12.1529</v>
       </c>
       <c r="U12" t="n">
-        <v>9.120200000000001</v>
+        <v>-5.5089</v>
       </c>
       <c r="V12" t="n">
-        <v>22.1164</v>
+        <v>5.1572</v>
       </c>
       <c r="W12" t="n">
-        <v>10.9086</v>
+        <v>8.4238</v>
       </c>
       <c r="X12" t="n">
-        <v>-16.313</v>
+        <v>17.216</v>
       </c>
       <c r="Y12" t="n">
-        <v>-39.878</v>
+        <v>-6.8413</v>
       </c>
       <c r="Z12" t="n">
-        <v>-30.5805</v>
+        <v>-21.922</v>
       </c>
       <c r="AA12" t="n">
-        <v>-9.3156</v>
+        <v>5.6182</v>
       </c>
       <c r="AB12" t="n">
-        <v>-19.7567</v>
+        <v>-6.074</v>
       </c>
       <c r="AC12" t="n">
-        <v>-11.997</v>
+        <v>-10.1241</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>267.13</v>
+        <v>247.42</v>
       </c>
       <c r="C13" t="n">
-        <v>274.93</v>
+        <v>259.79</v>
       </c>
       <c r="D13" t="n">
-        <v>226</v>
+        <v>233.3</v>
       </c>
       <c r="E13" t="n">
-        <v>226.19</v>
+        <v>233.86</v>
       </c>
       <c r="F13" t="n">
-        <v>84.19</v>
+        <v>81.67</v>
       </c>
       <c r="G13" t="n">
-        <v>84.83</v>
+        <v>81.81</v>
       </c>
       <c r="H13" t="n">
-        <v>79.86</v>
+        <v>76.94</v>
       </c>
       <c r="I13" t="n">
-        <v>79.93000000000001</v>
+        <v>77.54000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>3.9836</v>
+        <v>4.122</v>
       </c>
       <c r="K13" t="n">
-        <v>4.5965</v>
+        <v>4.4086</v>
       </c>
       <c r="L13" t="n">
-        <v>3.865</v>
+        <v>3.8749</v>
       </c>
       <c r="M13" t="n">
-        <v>4.5767</v>
+        <v>4.4086</v>
       </c>
       <c r="N13" t="n">
-        <v>35.9652</v>
+        <v>36.9397</v>
       </c>
       <c r="O13" t="n">
-        <v>37.7861</v>
+        <v>39.1641</v>
       </c>
       <c r="P13" t="n">
-        <v>35.6896</v>
+        <v>36.8708</v>
       </c>
       <c r="Q13" t="n">
-        <v>37.7468</v>
+        <v>38.8984</v>
       </c>
       <c r="R13" t="n">
-        <v>-16.9945</v>
+        <v>3.391</v>
       </c>
       <c r="S13" t="n">
-        <v>0.9822</v>
+        <v>-0.3494</v>
       </c>
       <c r="T13" t="n">
-        <v>12.1529</v>
+        <v>29.4547</v>
       </c>
       <c r="U13" t="n">
-        <v>-5.5089</v>
+        <v>-2.9901</v>
       </c>
       <c r="V13" t="n">
-        <v>5.1572</v>
+        <v>0.0258</v>
       </c>
       <c r="W13" t="n">
-        <v>8.4238</v>
+        <v>11.9388</v>
       </c>
       <c r="X13" t="n">
-        <v>17.216</v>
+        <v>-3.673</v>
       </c>
       <c r="Y13" t="n">
-        <v>-6.8413</v>
+        <v>-5.5084</v>
       </c>
       <c r="Z13" t="n">
-        <v>-21.922</v>
+        <v>-32.1159</v>
       </c>
       <c r="AA13" t="n">
-        <v>5.6182</v>
+        <v>3.0509</v>
       </c>
       <c r="AB13" t="n">
-        <v>-6.074</v>
+        <v>-1.2986</v>
       </c>
       <c r="AC13" t="n">
-        <v>-10.1241</v>
+        <v>-12.6628</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>247.42</v>
+        <v>266.04</v>
       </c>
       <c r="C14" t="n">
-        <v>259.79</v>
+        <v>286.15</v>
       </c>
       <c r="D14" t="n">
-        <v>233.3</v>
+        <v>265</v>
       </c>
       <c r="E14" t="n">
-        <v>233.86</v>
+        <v>279.29</v>
       </c>
       <c r="F14" t="n">
-        <v>81.67</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>81.81</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>76.94</v>
+        <v>80.63</v>
       </c>
       <c r="I14" t="n">
-        <v>77.54000000000001</v>
+        <v>82.87</v>
       </c>
       <c r="J14" t="n">
-        <v>4.122</v>
+        <v>3.8156</v>
       </c>
       <c r="K14" t="n">
-        <v>4.4086</v>
+        <v>3.8254</v>
       </c>
       <c r="L14" t="n">
-        <v>3.8749</v>
+        <v>3.4103</v>
       </c>
       <c r="M14" t="n">
-        <v>4.4086</v>
+        <v>3.5487</v>
       </c>
       <c r="N14" t="n">
-        <v>36.9397</v>
+        <v>36.6149</v>
       </c>
       <c r="O14" t="n">
-        <v>39.1641</v>
+        <v>37.3531</v>
       </c>
       <c r="P14" t="n">
-        <v>36.8708</v>
+        <v>35.857</v>
       </c>
       <c r="Q14" t="n">
-        <v>38.8984</v>
+        <v>36.1719</v>
       </c>
       <c r="R14" t="n">
-        <v>3.391</v>
+        <v>19.4262</v>
       </c>
       <c r="S14" t="n">
-        <v>-0.3494</v>
+        <v>2.4917</v>
       </c>
       <c r="T14" t="n">
-        <v>29.4547</v>
+        <v>24.6886</v>
       </c>
       <c r="U14" t="n">
-        <v>-2.9901</v>
+        <v>6.8739</v>
       </c>
       <c r="V14" t="n">
-        <v>0.0258</v>
+        <v>-2.0333</v>
       </c>
       <c r="W14" t="n">
-        <v>11.9388</v>
+        <v>9.0251</v>
       </c>
       <c r="X14" t="n">
-        <v>-3.673</v>
+        <v>-19.5051</v>
       </c>
       <c r="Y14" t="n">
-        <v>-5.5084</v>
+        <v>-9.1126</v>
       </c>
       <c r="Z14" t="n">
-        <v>-32.1159</v>
+        <v>-27.7662</v>
       </c>
       <c r="AA14" t="n">
-        <v>3.0509</v>
+        <v>-7.0093</v>
       </c>
       <c r="AB14" t="n">
-        <v>-1.2986</v>
+        <v>1.2116</v>
       </c>
       <c r="AC14" t="n">
-        <v>-12.6628</v>
+        <v>-9.992800000000001</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>266.04</v>
+        <v>299.26</v>
       </c>
       <c r="C15" t="n">
-        <v>286.15</v>
+        <v>302</v>
       </c>
       <c r="D15" t="n">
-        <v>265</v>
+        <v>286.24</v>
       </c>
       <c r="E15" t="n">
-        <v>279.29</v>
+        <v>300.77</v>
       </c>
       <c r="F15" t="n">
-        <v>82.09999999999999</v>
+        <v>83.95</v>
       </c>
       <c r="G15" t="n">
-        <v>83.59999999999999</v>
+        <v>85.11</v>
       </c>
       <c r="H15" t="n">
-        <v>80.63</v>
+        <v>81.39</v>
       </c>
       <c r="I15" t="n">
-        <v>82.87</v>
+        <v>82.58</v>
       </c>
       <c r="J15" t="n">
-        <v>3.8156</v>
+        <v>3.2917</v>
       </c>
       <c r="K15" t="n">
-        <v>3.8254</v>
+        <v>3.4498</v>
       </c>
       <c r="L15" t="n">
-        <v>3.4103</v>
+        <v>3.2521</v>
       </c>
       <c r="M15" t="n">
-        <v>3.5487</v>
+        <v>3.262</v>
       </c>
       <c r="N15" t="n">
-        <v>36.6149</v>
+        <v>35.7389</v>
       </c>
       <c r="O15" t="n">
-        <v>37.3531</v>
+        <v>36.8511</v>
       </c>
       <c r="P15" t="n">
-        <v>35.857</v>
+        <v>35.2369</v>
       </c>
       <c r="Q15" t="n">
-        <v>36.1719</v>
+        <v>36.3491</v>
       </c>
       <c r="R15" t="n">
-        <v>19.4262</v>
+        <v>7.6909</v>
       </c>
       <c r="S15" t="n">
-        <v>2.4917</v>
+        <v>32.9723</v>
       </c>
       <c r="T15" t="n">
-        <v>24.6886</v>
+        <v>28.1618</v>
       </c>
       <c r="U15" t="n">
-        <v>6.8739</v>
+        <v>-0.3499</v>
       </c>
       <c r="V15" t="n">
-        <v>-2.0333</v>
+        <v>3.3154</v>
       </c>
       <c r="W15" t="n">
-        <v>9.0251</v>
+        <v>6.5273</v>
       </c>
       <c r="X15" t="n">
-        <v>-19.5051</v>
+        <v>-8.079000000000001</v>
       </c>
       <c r="Y15" t="n">
-        <v>-9.1126</v>
+        <v>-28.7259</v>
       </c>
       <c r="Z15" t="n">
-        <v>-27.7662</v>
+        <v>-30.084</v>
       </c>
       <c r="AA15" t="n">
-        <v>-7.0093</v>
+        <v>0.4899</v>
       </c>
       <c r="AB15" t="n">
-        <v>1.2116</v>
+        <v>-3.7028</v>
       </c>
       <c r="AC15" t="n">
-        <v>-9.992800000000001</v>
+        <v>-7.7673</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>299.26</v>
+        <v>236</v>
       </c>
       <c r="C16" t="n">
-        <v>302</v>
+        <v>252.98</v>
       </c>
       <c r="D16" t="n">
-        <v>286.24</v>
+        <v>223</v>
       </c>
       <c r="E16" t="n">
-        <v>300.77</v>
+        <v>231.42</v>
       </c>
       <c r="F16" t="n">
-        <v>83.95</v>
+        <v>75.12</v>
       </c>
       <c r="G16" t="n">
-        <v>85.11</v>
+        <v>77.73999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>81.39</v>
+        <v>73.91</v>
       </c>
       <c r="I16" t="n">
-        <v>82.58</v>
+        <v>74.44</v>
       </c>
       <c r="J16" t="n">
-        <v>3.2917</v>
+        <v>3.99</v>
       </c>
       <c r="K16" t="n">
-        <v>3.4498</v>
+        <v>4.13</v>
       </c>
       <c r="L16" t="n">
-        <v>3.2521</v>
+        <v>3.8</v>
       </c>
       <c r="M16" t="n">
-        <v>3.262</v>
+        <v>4.04</v>
       </c>
       <c r="N16" t="n">
-        <v>35.7389</v>
+        <v>39.6267</v>
       </c>
       <c r="O16" t="n">
-        <v>36.8511</v>
+        <v>40.1582</v>
       </c>
       <c r="P16" t="n">
-        <v>35.2369</v>
+        <v>38.4653</v>
       </c>
       <c r="Q16" t="n">
-        <v>36.3491</v>
+        <v>39.922</v>
       </c>
       <c r="R16" t="n">
-        <v>7.6909</v>
+        <v>-23.0575</v>
       </c>
       <c r="S16" t="n">
-        <v>32.9723</v>
+        <v>-1.0434</v>
       </c>
       <c r="T16" t="n">
-        <v>28.1618</v>
+        <v>-15.0752</v>
       </c>
       <c r="U16" t="n">
-        <v>-0.3499</v>
+        <v>-9.857100000000001</v>
       </c>
       <c r="V16" t="n">
-        <v>3.3154</v>
+        <v>-3.9979</v>
       </c>
       <c r="W16" t="n">
-        <v>6.5273</v>
+        <v>-11.9991</v>
       </c>
       <c r="X16" t="n">
-        <v>-8.079000000000001</v>
+        <v>23.8504</v>
       </c>
       <c r="Y16" t="n">
-        <v>-28.7259</v>
+        <v>-8.360900000000001</v>
       </c>
       <c r="Z16" t="n">
-        <v>-30.084</v>
+        <v>3.4704</v>
       </c>
       <c r="AA16" t="n">
-        <v>0.4899</v>
+        <v>9.8294</v>
       </c>
       <c r="AB16" t="n">
-        <v>-3.7028</v>
+        <v>2.6315</v>
       </c>
       <c r="AC16" t="n">
-        <v>-7.7673</v>
+        <v>11.7046</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>236</v>
+        <v>233.11</v>
       </c>
       <c r="C17" t="n">
-        <v>252.98</v>
+        <v>237</v>
       </c>
       <c r="D17" t="n">
-        <v>223</v>
+        <v>211.13</v>
       </c>
       <c r="E17" t="n">
-        <v>231.42</v>
+        <v>229.57</v>
       </c>
       <c r="F17" t="n">
-        <v>75.12</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>77.73999999999999</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="H17" t="n">
-        <v>73.91</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="I17" t="n">
-        <v>74.44</v>
+        <v>73.3</v>
       </c>
       <c r="J17" t="n">
-        <v>3.99</v>
+        <v>4</v>
       </c>
       <c r="K17" t="n">
-        <v>4.13</v>
+        <v>4.39</v>
       </c>
       <c r="L17" t="n">
-        <v>3.8</v>
+        <v>3.92</v>
       </c>
       <c r="M17" t="n">
-        <v>4.04</v>
+        <v>4.08</v>
       </c>
       <c r="N17" t="n">
-        <v>39.6267</v>
+        <v>39.66</v>
       </c>
       <c r="O17" t="n">
-        <v>40.1582</v>
+        <v>41.49</v>
       </c>
       <c r="P17" t="n">
-        <v>38.4653</v>
+        <v>38.9</v>
       </c>
       <c r="Q17" t="n">
-        <v>39.922</v>
+        <v>40.45</v>
       </c>
       <c r="R17" t="n">
-        <v>-23.0575</v>
+        <v>-0.7994</v>
       </c>
       <c r="S17" t="n">
-        <v>-1.0434</v>
+        <v>-17.8023</v>
       </c>
       <c r="T17" t="n">
-        <v>-15.0752</v>
+        <v>1.4943</v>
       </c>
       <c r="U17" t="n">
-        <v>-9.857100000000001</v>
+        <v>-1.5314</v>
       </c>
       <c r="V17" t="n">
-        <v>-3.9979</v>
+        <v>-11.5482</v>
       </c>
       <c r="W17" t="n">
-        <v>-11.9991</v>
+        <v>-8.2948</v>
       </c>
       <c r="X17" t="n">
-        <v>23.8504</v>
+        <v>0.9901</v>
       </c>
       <c r="Y17" t="n">
-        <v>-8.360900000000001</v>
+        <v>14.9717</v>
       </c>
       <c r="Z17" t="n">
-        <v>3.4704</v>
+        <v>-10.8528</v>
       </c>
       <c r="AA17" t="n">
-        <v>9.8294</v>
+        <v>1.3226</v>
       </c>
       <c r="AB17" t="n">
-        <v>2.6315</v>
+        <v>11.8271</v>
       </c>
       <c r="AC17" t="n">
-        <v>11.7046</v>
+        <v>7.1614</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>233.11</v>
+        <v>268.05</v>
       </c>
       <c r="C18" t="n">
-        <v>237</v>
+        <v>268.4</v>
       </c>
       <c r="D18" t="n">
-        <v>211.13</v>
+        <v>225.74</v>
       </c>
       <c r="E18" t="n">
-        <v>229.57</v>
+        <v>252.61</v>
       </c>
       <c r="F18" t="n">
-        <v>74.79000000000001</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="G18" t="n">
-        <v>76.18000000000001</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="H18" t="n">
-        <v>71.34999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I18" t="n">
-        <v>73.3</v>
+        <v>74.95</v>
       </c>
       <c r="J18" t="n">
-        <v>4</v>
+        <v>3.38</v>
       </c>
       <c r="K18" t="n">
-        <v>4.39</v>
+        <v>4.15</v>
       </c>
       <c r="L18" t="n">
-        <v>3.92</v>
+        <v>3.37</v>
       </c>
       <c r="M18" t="n">
-        <v>4.08</v>
+        <v>3.63</v>
       </c>
       <c r="N18" t="n">
-        <v>39.66</v>
+        <v>37.87</v>
       </c>
       <c r="O18" t="n">
-        <v>41.49</v>
+        <v>41.37</v>
       </c>
       <c r="P18" t="n">
-        <v>38.9</v>
+        <v>37.71</v>
       </c>
       <c r="Q18" t="n">
-        <v>40.45</v>
+        <v>39.47</v>
       </c>
       <c r="R18" t="n">
-        <v>-0.7994</v>
+        <v>10.0362</v>
       </c>
       <c r="S18" t="n">
-        <v>-17.8023</v>
+        <v>-16.0122</v>
       </c>
       <c r="T18" t="n">
-        <v>1.4943</v>
+        <v>8.0176</v>
       </c>
       <c r="U18" t="n">
-        <v>-1.5314</v>
+        <v>2.251</v>
       </c>
       <c r="V18" t="n">
-        <v>-11.5482</v>
+        <v>-9.2395</v>
       </c>
       <c r="W18" t="n">
-        <v>-8.2948</v>
+        <v>-3.3402</v>
       </c>
       <c r="X18" t="n">
-        <v>0.9901</v>
+        <v>-11.0294</v>
       </c>
       <c r="Y18" t="n">
-        <v>14.9717</v>
+        <v>11.2814</v>
       </c>
       <c r="Z18" t="n">
-        <v>-10.8528</v>
+        <v>-17.6609</v>
       </c>
       <c r="AA18" t="n">
-        <v>1.3226</v>
+        <v>-2.4227</v>
       </c>
       <c r="AB18" t="n">
-        <v>11.8271</v>
+        <v>8.585900000000001</v>
       </c>
       <c r="AC18" t="n">
-        <v>7.1614</v>
+        <v>1.4695</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>268.05</v>
+        <v>226.24</v>
       </c>
       <c r="C19" t="n">
-        <v>268.4</v>
+        <v>231.25</v>
       </c>
       <c r="D19" t="n">
-        <v>225.74</v>
+        <v>212.1</v>
       </c>
       <c r="E19" t="n">
-        <v>252.61</v>
+        <v>215.6</v>
       </c>
       <c r="F19" t="n">
-        <v>77.95999999999999</v>
+        <v>72.09</v>
       </c>
       <c r="G19" t="n">
-        <v>78.23999999999999</v>
+        <v>74.69</v>
       </c>
       <c r="H19" t="n">
-        <v>71.59999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="I19" t="n">
-        <v>74.95</v>
+        <v>71.83</v>
       </c>
       <c r="J19" t="n">
-        <v>3.38</v>
+        <v>4.04</v>
       </c>
       <c r="K19" t="n">
-        <v>4.15</v>
+        <v>4.25</v>
       </c>
       <c r="L19" t="n">
-        <v>3.37</v>
+        <v>3.95</v>
       </c>
       <c r="M19" t="n">
-        <v>3.63</v>
+        <v>4.24</v>
       </c>
       <c r="N19" t="n">
-        <v>37.87</v>
+        <v>41.08</v>
       </c>
       <c r="O19" t="n">
-        <v>41.37</v>
+        <v>41.79</v>
       </c>
       <c r="P19" t="n">
-        <v>37.71</v>
+        <v>39.69</v>
       </c>
       <c r="Q19" t="n">
-        <v>39.47</v>
+        <v>41.31</v>
       </c>
       <c r="R19" t="n">
-        <v>10.0362</v>
+        <v>-14.651</v>
       </c>
       <c r="S19" t="n">
-        <v>-16.0122</v>
+        <v>-6.8361</v>
       </c>
       <c r="T19" t="n">
-        <v>8.0176</v>
+        <v>-22.8043</v>
       </c>
       <c r="U19" t="n">
-        <v>2.251</v>
+        <v>-4.1628</v>
       </c>
       <c r="V19" t="n">
-        <v>-9.2395</v>
+        <v>-3.5062</v>
       </c>
       <c r="W19" t="n">
-        <v>-3.3402</v>
+        <v>-13.3221</v>
       </c>
       <c r="X19" t="n">
-        <v>-11.0294</v>
+        <v>16.8044</v>
       </c>
       <c r="Y19" t="n">
-        <v>11.2814</v>
+        <v>4.9505</v>
       </c>
       <c r="Z19" t="n">
-        <v>-17.6609</v>
+        <v>19.4804</v>
       </c>
       <c r="AA19" t="n">
-        <v>-2.4227</v>
+        <v>4.6618</v>
       </c>
       <c r="AB19" t="n">
-        <v>8.585900000000001</v>
+        <v>3.4768</v>
       </c>
       <c r="AC19" t="n">
-        <v>1.4695</v>
+        <v>14.2047</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>226.24</v>
+        <v>216.36</v>
       </c>
       <c r="C20" t="n">
-        <v>231.25</v>
+        <v>238.65</v>
       </c>
       <c r="D20" t="n">
-        <v>212.1</v>
+        <v>192.3</v>
       </c>
       <c r="E20" t="n">
-        <v>215.6</v>
+        <v>236.52</v>
       </c>
       <c r="F20" t="n">
-        <v>72.09</v>
+        <v>74.12</v>
       </c>
       <c r="G20" t="n">
-        <v>74.69</v>
+        <v>77.38</v>
       </c>
       <c r="H20" t="n">
-        <v>70.72</v>
+        <v>71.45</v>
       </c>
       <c r="I20" t="n">
-        <v>71.83</v>
+        <v>77.19</v>
       </c>
       <c r="J20" t="n">
-        <v>4.04</v>
+        <v>4.16</v>
       </c>
       <c r="K20" t="n">
-        <v>4.25</v>
+        <v>4.63</v>
       </c>
       <c r="L20" t="n">
-        <v>3.95</v>
+        <v>3.7</v>
       </c>
       <c r="M20" t="n">
-        <v>4.24</v>
+        <v>3.72</v>
       </c>
       <c r="N20" t="n">
-        <v>41.08</v>
+        <v>39.91</v>
       </c>
       <c r="O20" t="n">
-        <v>41.79</v>
+        <v>41.43</v>
       </c>
       <c r="P20" t="n">
-        <v>39.69</v>
+        <v>38.08</v>
       </c>
       <c r="Q20" t="n">
-        <v>41.31</v>
+        <v>38.16</v>
       </c>
       <c r="R20" t="n">
-        <v>-14.651</v>
+        <v>9.703200000000001</v>
       </c>
       <c r="S20" t="n">
-        <v>-6.8361</v>
+        <v>3.0274</v>
       </c>
       <c r="T20" t="n">
-        <v>-22.8043</v>
+        <v>-21.3618</v>
       </c>
       <c r="U20" t="n">
-        <v>-4.1628</v>
+        <v>7.4621</v>
       </c>
       <c r="V20" t="n">
-        <v>-3.5062</v>
+        <v>5.307</v>
       </c>
       <c r="W20" t="n">
-        <v>-13.3221</v>
+        <v>-6.527</v>
       </c>
       <c r="X20" t="n">
-        <v>16.8044</v>
+        <v>-12.2642</v>
       </c>
       <c r="Y20" t="n">
-        <v>4.9505</v>
+        <v>-8.823499999999999</v>
       </c>
       <c r="Z20" t="n">
-        <v>19.4804</v>
+        <v>14.0405</v>
       </c>
       <c r="AA20" t="n">
-        <v>4.6618</v>
+        <v>-7.6253</v>
       </c>
       <c r="AB20" t="n">
-        <v>3.4768</v>
+        <v>-5.6613</v>
       </c>
       <c r="AC20" t="n">
-        <v>14.2047</v>
+        <v>4.982</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>216.36</v>
+        <v>241.45</v>
       </c>
       <c r="C21" t="n">
-        <v>238.65</v>
+        <v>272</v>
       </c>
       <c r="D21" t="n">
-        <v>192.3</v>
+        <v>240.59</v>
       </c>
       <c r="E21" t="n">
-        <v>236.52</v>
+        <v>266.71</v>
       </c>
       <c r="F21" t="n">
-        <v>74.12</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="G21" t="n">
-        <v>77.38</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="H21" t="n">
-        <v>71.45</v>
+        <v>77.15000000000001</v>
       </c>
       <c r="I21" t="n">
-        <v>77.19</v>
+        <v>81</v>
       </c>
       <c r="J21" t="n">
-        <v>4.16</v>
+        <v>3.66</v>
       </c>
       <c r="K21" t="n">
-        <v>4.63</v>
+        <v>3.68</v>
       </c>
       <c r="L21" t="n">
-        <v>3.7</v>
+        <v>3.17</v>
       </c>
       <c r="M21" t="n">
-        <v>3.72</v>
+        <v>3.24</v>
       </c>
       <c r="N21" t="n">
-        <v>39.91</v>
+        <v>38.16</v>
       </c>
       <c r="O21" t="n">
-        <v>41.43</v>
+        <v>38.2</v>
       </c>
       <c r="P21" t="n">
-        <v>38.08</v>
+        <v>36.03</v>
       </c>
       <c r="Q21" t="n">
-        <v>38.16</v>
+        <v>36.31</v>
       </c>
       <c r="R21" t="n">
-        <v>9.703200000000001</v>
+        <v>12.7642</v>
       </c>
       <c r="S21" t="n">
-        <v>3.0274</v>
+        <v>5.5817</v>
       </c>
       <c r="T21" t="n">
-        <v>-21.3618</v>
+        <v>15.2493</v>
       </c>
       <c r="U21" t="n">
-        <v>7.4621</v>
+        <v>4.9359</v>
       </c>
       <c r="V21" t="n">
-        <v>5.307</v>
+        <v>8.071999999999999</v>
       </c>
       <c r="W21" t="n">
-        <v>-6.527</v>
+        <v>8.8125</v>
       </c>
       <c r="X21" t="n">
-        <v>-12.2642</v>
+        <v>-12.9032</v>
       </c>
       <c r="Y21" t="n">
-        <v>-8.823499999999999</v>
+        <v>-10.7438</v>
       </c>
       <c r="Z21" t="n">
-        <v>14.0405</v>
+        <v>-19.802</v>
       </c>
       <c r="AA21" t="n">
-        <v>-7.6253</v>
+        <v>-4.848</v>
       </c>
       <c r="AB21" t="n">
-        <v>-5.6613</v>
+        <v>-8.0061</v>
       </c>
       <c r="AC21" t="n">
-        <v>4.982</v>
+        <v>-9.047599999999999</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>241.45</v>
+        <v>237.785</v>
       </c>
       <c r="C22" t="n">
-        <v>272</v>
+        <v>246.44</v>
       </c>
       <c r="D22" t="n">
-        <v>240.601</v>
+        <v>215.3807</v>
       </c>
       <c r="E22" t="n">
-        <v>266.71</v>
+        <v>217.55</v>
       </c>
       <c r="F22" t="n">
-        <v>77.262</v>
+        <v>78.72</v>
       </c>
       <c r="G22" t="n">
-        <v>81.54000000000001</v>
+        <v>79.64</v>
       </c>
       <c r="H22" t="n">
-        <v>77.15000000000001</v>
+        <v>77.23</v>
       </c>
       <c r="I22" t="n">
-        <v>81</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J22" t="n">
-        <v>3.66</v>
+        <v>3.5903</v>
       </c>
       <c r="K22" t="n">
-        <v>3.68</v>
+        <v>3.89</v>
       </c>
       <c r="L22" t="n">
-        <v>3.17</v>
+        <v>3.51</v>
       </c>
       <c r="M22" t="n">
-        <v>3.24</v>
+        <v>3.86</v>
       </c>
       <c r="N22" t="n">
-        <v>38.16</v>
+        <v>37.31</v>
       </c>
       <c r="O22" t="n">
-        <v>38.195</v>
+        <v>37.975</v>
       </c>
       <c r="P22" t="n">
-        <v>36.03</v>
+        <v>36.9</v>
       </c>
       <c r="Q22" t="n">
-        <v>36.31</v>
+        <v>37.88</v>
       </c>
       <c r="R22" t="n">
-        <v>12.7642</v>
+        <v>-18.432</v>
       </c>
       <c r="S22" t="n">
-        <v>5.5817</v>
+        <v>0.9045</v>
       </c>
       <c r="T22" t="n">
-        <v>15.2493</v>
+        <v>-5.2359</v>
       </c>
       <c r="U22" t="n">
-        <v>4.9359</v>
+        <v>-4.3704</v>
       </c>
       <c r="V22" t="n">
-        <v>8.071999999999999</v>
+        <v>7.838</v>
       </c>
       <c r="W22" t="n">
-        <v>8.8125</v>
+        <v>5.6753</v>
       </c>
       <c r="X22" t="n">
-        <v>-12.9032</v>
+        <v>19.1358</v>
       </c>
       <c r="Y22" t="n">
-        <v>-10.7438</v>
+        <v>-8.962300000000001</v>
       </c>
       <c r="Z22" t="n">
-        <v>-19.802</v>
+        <v>-5.3922</v>
       </c>
       <c r="AA22" t="n">
-        <v>-4.848</v>
+        <v>4.3239</v>
       </c>
       <c r="AB22" t="n">
-        <v>-8.0061</v>
+        <v>-8.303100000000001</v>
       </c>
       <c r="AC22" t="n">
-        <v>-9.047599999999999</v>
+        <v>-6.3535</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-07-02 23:07
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>243.18</v>
+        <v>281.47</v>
       </c>
       <c r="C2" t="n">
-        <v>267.08</v>
+        <v>284.58</v>
       </c>
       <c r="D2" t="n">
-        <v>238.82</v>
+        <v>257.26</v>
       </c>
       <c r="E2" t="n">
-        <v>266.32</v>
+        <v>280.54</v>
       </c>
       <c r="F2" t="n">
-        <v>85.94</v>
+        <v>87.68000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>87.31999999999999</v>
+        <v>88.09</v>
       </c>
       <c r="H2" t="n">
-        <v>84.83</v>
+        <v>85.41</v>
       </c>
       <c r="I2" t="n">
-        <v>87.22</v>
+        <v>86.56</v>
       </c>
       <c r="J2" t="n">
-        <v>5.7332</v>
+        <v>4.8238</v>
       </c>
       <c r="K2" t="n">
-        <v>5.8617</v>
+        <v>5.2884</v>
       </c>
       <c r="L2" t="n">
-        <v>5.0907</v>
+        <v>4.7645</v>
       </c>
       <c r="M2" t="n">
-        <v>5.1105</v>
+        <v>4.8535</v>
       </c>
       <c r="N2" t="n">
-        <v>36.8806</v>
+        <v>36.1522</v>
       </c>
       <c r="O2" t="n">
-        <v>37.3531</v>
+        <v>37.0971</v>
       </c>
       <c r="P2" t="n">
-        <v>36.2802</v>
+        <v>35.9751</v>
       </c>
       <c r="Q2" t="n">
-        <v>36.3294</v>
+        <v>36.605</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>281.47</v>
+        <v>242.04</v>
       </c>
       <c r="C3" t="n">
-        <v>284.58</v>
+        <v>274.5</v>
       </c>
       <c r="D3" t="n">
-        <v>257.26</v>
+        <v>228.55</v>
       </c>
       <c r="E3" t="n">
-        <v>280.54</v>
+        <v>262.7</v>
       </c>
       <c r="F3" t="n">
-        <v>87.68000000000001</v>
+        <v>83.47</v>
       </c>
       <c r="G3" t="n">
-        <v>88.09</v>
+        <v>86.25</v>
       </c>
       <c r="H3" t="n">
-        <v>85.41</v>
+        <v>82.48</v>
       </c>
       <c r="I3" t="n">
-        <v>86.56</v>
+        <v>85.22</v>
       </c>
       <c r="J3" t="n">
-        <v>4.8238</v>
+        <v>5.5059</v>
       </c>
       <c r="K3" t="n">
-        <v>5.2884</v>
+        <v>5.7431</v>
       </c>
       <c r="L3" t="n">
-        <v>4.7645</v>
+        <v>4.9424</v>
       </c>
       <c r="M3" t="n">
-        <v>4.8535</v>
+        <v>5.1401</v>
       </c>
       <c r="N3" t="n">
-        <v>36.1522</v>
+        <v>37.9239</v>
       </c>
       <c r="O3" t="n">
-        <v>37.0971</v>
+        <v>38.3472</v>
       </c>
       <c r="P3" t="n">
-        <v>35.9751</v>
+        <v>36.7428</v>
       </c>
       <c r="Q3" t="n">
-        <v>36.605</v>
+        <v>37.166</v>
       </c>
       <c r="R3" t="n">
-        <v>5.3394</v>
+        <v>-6.3592</v>
       </c>
       <c r="U3" t="n">
-        <v>-0.7567</v>
+        <v>-1.5481</v>
       </c>
       <c r="X3" t="n">
-        <v>-5.0289</v>
+        <v>5.905</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.7586000000000001</v>
+        <v>1.5326</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>242.04</v>
+        <v>230.85</v>
       </c>
       <c r="C4" t="n">
-        <v>274.5</v>
+        <v>233.69</v>
       </c>
       <c r="D4" t="n">
-        <v>228.55</v>
+        <v>181.81</v>
       </c>
       <c r="E4" t="n">
-        <v>262.7</v>
+        <v>182.54</v>
       </c>
       <c r="F4" t="n">
-        <v>83.47</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>86.25</v>
+        <v>82.08</v>
       </c>
       <c r="H4" t="n">
-        <v>82.48</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>85.22</v>
+        <v>73.05</v>
       </c>
       <c r="J4" t="n">
-        <v>5.5059</v>
+        <v>5.7925</v>
       </c>
       <c r="K4" t="n">
-        <v>5.7431</v>
+        <v>6.7711</v>
       </c>
       <c r="L4" t="n">
-        <v>4.9424</v>
+        <v>5.7233</v>
       </c>
       <c r="M4" t="n">
-        <v>5.1401</v>
+        <v>6.7612</v>
       </c>
       <c r="N4" t="n">
-        <v>37.9239</v>
+        <v>38.7999</v>
       </c>
       <c r="O4" t="n">
-        <v>38.3472</v>
+        <v>42.6681</v>
       </c>
       <c r="P4" t="n">
-        <v>36.7428</v>
+        <v>38.5637</v>
       </c>
       <c r="Q4" t="n">
-        <v>37.166</v>
+        <v>42.5106</v>
       </c>
       <c r="R4" t="n">
-        <v>-6.3592</v>
+        <v>-30.5139</v>
       </c>
       <c r="U4" t="n">
-        <v>-1.5481</v>
+        <v>-14.2807</v>
       </c>
       <c r="X4" t="n">
-        <v>5.905</v>
+        <v>31.5383</v>
       </c>
       <c r="AA4" t="n">
-        <v>1.5326</v>
+        <v>14.3803</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>230.85</v>
+        <v>210.62</v>
       </c>
       <c r="C5" t="n">
-        <v>233.69</v>
+        <v>222.19</v>
       </c>
       <c r="D5" t="n">
-        <v>181.81</v>
+        <v>201.69</v>
       </c>
       <c r="E5" t="n">
-        <v>182.54</v>
+        <v>211.44</v>
       </c>
       <c r="F5" t="n">
-        <v>81.56999999999999</v>
+        <v>76.86</v>
       </c>
       <c r="G5" t="n">
-        <v>82.08</v>
+        <v>78.47</v>
       </c>
       <c r="H5" t="n">
-        <v>72.68000000000001</v>
+        <v>75.38</v>
       </c>
       <c r="I5" t="n">
-        <v>73.05</v>
+        <v>76.27</v>
       </c>
       <c r="J5" t="n">
-        <v>5.7925</v>
+        <v>5.6442</v>
       </c>
       <c r="K5" t="n">
-        <v>6.7711</v>
+        <v>5.9803</v>
       </c>
       <c r="L5" t="n">
-        <v>5.7233</v>
+        <v>5.2093</v>
       </c>
       <c r="M5" t="n">
-        <v>6.7612</v>
+        <v>5.6245</v>
       </c>
       <c r="N5" t="n">
-        <v>38.7999</v>
+        <v>40.2763</v>
       </c>
       <c r="O5" t="n">
-        <v>42.6681</v>
+        <v>41.1228</v>
       </c>
       <c r="P5" t="n">
-        <v>38.5637</v>
+        <v>39.3314</v>
       </c>
       <c r="Q5" t="n">
-        <v>42.5106</v>
+        <v>40.611</v>
       </c>
       <c r="R5" t="n">
-        <v>-30.5139</v>
+        <v>15.8321</v>
       </c>
       <c r="S5" t="n">
-        <v>-31.4584</v>
+        <v>-24.6311</v>
       </c>
       <c r="U5" t="n">
-        <v>-14.2807</v>
+        <v>4.4079</v>
       </c>
       <c r="V5" t="n">
-        <v>-16.2463</v>
+        <v>-11.8877</v>
       </c>
       <c r="X5" t="n">
-        <v>31.5383</v>
+        <v>-16.8121</v>
       </c>
       <c r="Y5" t="n">
-        <v>32.3002</v>
+        <v>15.8854</v>
       </c>
       <c r="AA5" t="n">
-        <v>14.3803</v>
+        <v>-4.4685</v>
       </c>
       <c r="AB5" t="n">
-        <v>17.0143</v>
+        <v>10.9439</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>210.62</v>
+        <v>227.06</v>
       </c>
       <c r="C6" t="n">
-        <v>222.19</v>
+        <v>231.02</v>
       </c>
       <c r="D6" t="n">
-        <v>201.69</v>
+        <v>157.56</v>
       </c>
       <c r="E6" t="n">
-        <v>211.44</v>
+        <v>201.68</v>
       </c>
       <c r="F6" t="n">
-        <v>76.86</v>
+        <v>78.48</v>
       </c>
       <c r="G6" t="n">
-        <v>78.47</v>
+        <v>79.34</v>
       </c>
       <c r="H6" t="n">
-        <v>75.38</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="I6" t="n">
-        <v>76.27</v>
+        <v>73.72</v>
       </c>
       <c r="J6" t="n">
-        <v>5.6442</v>
+        <v>5.1895</v>
       </c>
       <c r="K6" t="n">
-        <v>5.9803</v>
+        <v>7.0281</v>
       </c>
       <c r="L6" t="n">
-        <v>5.2093</v>
+        <v>5.0808</v>
       </c>
       <c r="M6" t="n">
-        <v>5.6245</v>
+        <v>5.8617</v>
       </c>
       <c r="N6" t="n">
-        <v>40.2763</v>
+        <v>39.4299</v>
       </c>
       <c r="O6" t="n">
-        <v>41.1228</v>
+        <v>45.6505</v>
       </c>
       <c r="P6" t="n">
-        <v>39.3314</v>
+        <v>38.9673</v>
       </c>
       <c r="Q6" t="n">
-        <v>40.611</v>
+        <v>41.9988</v>
       </c>
       <c r="R6" t="n">
-        <v>15.8321</v>
+        <v>-4.616</v>
       </c>
       <c r="S6" t="n">
-        <v>-24.6311</v>
+        <v>-23.228</v>
       </c>
       <c r="U6" t="n">
-        <v>4.4079</v>
+        <v>-3.3434</v>
       </c>
       <c r="V6" t="n">
-        <v>-11.8877</v>
+        <v>-13.4945</v>
       </c>
       <c r="X6" t="n">
-        <v>-16.8121</v>
+        <v>4.2173</v>
       </c>
       <c r="Y6" t="n">
-        <v>15.8854</v>
+        <v>14.0386</v>
       </c>
       <c r="AA6" t="n">
-        <v>-4.4685</v>
+        <v>3.4173</v>
       </c>
       <c r="AB6" t="n">
-        <v>10.9439</v>
+        <v>13.0033</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>227.06</v>
+        <v>191.54</v>
       </c>
       <c r="C7" t="n">
-        <v>231.02</v>
+        <v>212.99</v>
       </c>
       <c r="D7" t="n">
-        <v>157.56</v>
+        <v>177.3</v>
       </c>
       <c r="E7" t="n">
-        <v>201.68</v>
+        <v>180.65</v>
       </c>
       <c r="F7" t="n">
-        <v>78.48</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>79.34</v>
+        <v>74.7</v>
       </c>
       <c r="H7" t="n">
-        <v>66.79000000000001</v>
+        <v>69</v>
       </c>
       <c r="I7" t="n">
-        <v>73.72</v>
+        <v>69.27</v>
       </c>
       <c r="J7" t="n">
-        <v>5.1895</v>
+        <v>6.1681</v>
       </c>
       <c r="K7" t="n">
-        <v>7.0281</v>
+        <v>6.5734</v>
       </c>
       <c r="L7" t="n">
-        <v>5.0808</v>
+        <v>5.5355</v>
       </c>
       <c r="M7" t="n">
-        <v>5.8617</v>
+        <v>6.4943</v>
       </c>
       <c r="N7" t="n">
-        <v>39.4299</v>
+        <v>43.1209</v>
       </c>
       <c r="O7" t="n">
-        <v>45.6505</v>
+        <v>44.676</v>
       </c>
       <c r="P7" t="n">
-        <v>38.9673</v>
+        <v>41.4082</v>
       </c>
       <c r="Q7" t="n">
-        <v>41.9988</v>
+        <v>44.5382</v>
       </c>
       <c r="R7" t="n">
-        <v>-4.616</v>
+        <v>-10.4274</v>
       </c>
       <c r="S7" t="n">
-        <v>-23.228</v>
+        <v>-1.0354</v>
       </c>
       <c r="T7" t="n">
-        <v>-24.2716</v>
+        <v>-35.6063</v>
       </c>
       <c r="U7" t="n">
-        <v>-3.3434</v>
+        <v>-6.0364</v>
       </c>
       <c r="V7" t="n">
-        <v>-13.4945</v>
+        <v>-5.1745</v>
       </c>
       <c r="W7" t="n">
-        <v>-15.4781</v>
+        <v>-19.9746</v>
       </c>
       <c r="X7" t="n">
-        <v>4.2173</v>
+        <v>10.7921</v>
       </c>
       <c r="Y7" t="n">
-        <v>14.0386</v>
+        <v>-3.9475</v>
       </c>
       <c r="Z7" t="n">
-        <v>14.6991</v>
+        <v>33.8065</v>
       </c>
       <c r="AA7" t="n">
-        <v>3.4173</v>
+        <v>6.0464</v>
       </c>
       <c r="AB7" t="n">
-        <v>13.0033</v>
+        <v>4.7696</v>
       </c>
       <c r="AC7" t="n">
-        <v>15.6055</v>
+        <v>21.6724</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>191.54</v>
+        <v>192.3</v>
       </c>
       <c r="C8" t="n">
-        <v>212.99</v>
+        <v>225.63</v>
       </c>
       <c r="D8" t="n">
-        <v>177.3</v>
+        <v>192.3</v>
       </c>
       <c r="E8" t="n">
-        <v>180.65</v>
+        <v>223.99</v>
       </c>
       <c r="F8" t="n">
-        <v>71.68000000000001</v>
+        <v>70.89</v>
       </c>
       <c r="G8" t="n">
-        <v>74.7</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>69</v>
+        <v>69.59</v>
       </c>
       <c r="I8" t="n">
-        <v>69.27</v>
+        <v>76.01000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>6.1681</v>
+        <v>6.0298</v>
       </c>
       <c r="K8" t="n">
-        <v>6.5734</v>
+        <v>6.0298</v>
       </c>
       <c r="L8" t="n">
-        <v>5.5355</v>
+        <v>4.8436</v>
       </c>
       <c r="M8" t="n">
-        <v>6.4943</v>
+        <v>4.9128</v>
       </c>
       <c r="N8" t="n">
-        <v>43.1209</v>
+        <v>43.4851</v>
       </c>
       <c r="O8" t="n">
-        <v>44.676</v>
+        <v>44.302</v>
       </c>
       <c r="P8" t="n">
-        <v>41.4082</v>
+        <v>39.8039</v>
       </c>
       <c r="Q8" t="n">
-        <v>44.5382</v>
+        <v>40.1878</v>
       </c>
       <c r="R8" t="n">
-        <v>-10.4274</v>
+        <v>23.9911</v>
       </c>
       <c r="S8" t="n">
-        <v>-1.0354</v>
+        <v>5.9355</v>
       </c>
       <c r="T8" t="n">
-        <v>-35.6063</v>
+        <v>-14.7354</v>
       </c>
       <c r="U8" t="n">
-        <v>-6.0364</v>
+        <v>9.73</v>
       </c>
       <c r="V8" t="n">
-        <v>-5.1745</v>
+        <v>-0.3409</v>
       </c>
       <c r="W8" t="n">
-        <v>-19.9746</v>
+        <v>-10.8073</v>
       </c>
       <c r="X8" t="n">
-        <v>10.7921</v>
+        <v>-24.3521</v>
       </c>
       <c r="Y8" t="n">
-        <v>-3.9475</v>
+        <v>-12.6536</v>
       </c>
       <c r="Z8" t="n">
-        <v>33.8065</v>
+        <v>-4.4221</v>
       </c>
       <c r="AA8" t="n">
-        <v>6.0464</v>
+        <v>-9.767799999999999</v>
       </c>
       <c r="AB8" t="n">
-        <v>4.7696</v>
+        <v>-1.0421</v>
       </c>
       <c r="AC8" t="n">
-        <v>21.6724</v>
+        <v>8.1305</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>192.3</v>
+        <v>222.22</v>
       </c>
       <c r="C9" t="n">
-        <v>225.63</v>
+        <v>242.4</v>
       </c>
       <c r="D9" t="n">
-        <v>192.3</v>
+        <v>214.74</v>
       </c>
       <c r="E9" t="n">
-        <v>223.99</v>
+        <v>234.68</v>
       </c>
       <c r="F9" t="n">
-        <v>70.89</v>
+        <v>76.34</v>
       </c>
       <c r="G9" t="n">
-        <v>76.59999999999999</v>
+        <v>78.36</v>
       </c>
       <c r="H9" t="n">
-        <v>69.59</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="I9" t="n">
-        <v>76.01000000000001</v>
+        <v>77.52</v>
       </c>
       <c r="J9" t="n">
-        <v>6.0298</v>
+        <v>4.9523</v>
       </c>
       <c r="K9" t="n">
-        <v>6.0298</v>
+        <v>5.0907</v>
       </c>
       <c r="L9" t="n">
-        <v>4.8436</v>
+        <v>4.4877</v>
       </c>
       <c r="M9" t="n">
-        <v>4.9128</v>
+        <v>4.6656</v>
       </c>
       <c r="N9" t="n">
-        <v>43.4851</v>
+        <v>40.0106</v>
       </c>
       <c r="O9" t="n">
-        <v>44.302</v>
+        <v>41.0933</v>
       </c>
       <c r="P9" t="n">
-        <v>39.8039</v>
+        <v>38.9476</v>
       </c>
       <c r="Q9" t="n">
-        <v>40.1878</v>
+        <v>39.4102</v>
       </c>
       <c r="R9" t="n">
-        <v>23.9911</v>
+        <v>4.7725</v>
       </c>
       <c r="S9" t="n">
-        <v>5.9355</v>
+        <v>16.3626</v>
       </c>
       <c r="T9" t="n">
-        <v>-14.7354</v>
+        <v>28.5636</v>
       </c>
       <c r="U9" t="n">
-        <v>9.73</v>
+        <v>1.9866</v>
       </c>
       <c r="V9" t="n">
-        <v>-0.3409</v>
+        <v>5.1546</v>
       </c>
       <c r="W9" t="n">
-        <v>-10.8073</v>
+        <v>6.1191</v>
       </c>
       <c r="X9" t="n">
-        <v>-24.3521</v>
+        <v>-5.0318</v>
       </c>
       <c r="Y9" t="n">
-        <v>-12.6536</v>
+        <v>-20.4053</v>
       </c>
       <c r="Z9" t="n">
-        <v>-4.4221</v>
+        <v>-30.9945</v>
       </c>
       <c r="AA9" t="n">
-        <v>-9.767799999999999</v>
+        <v>-1.9349</v>
       </c>
       <c r="AB9" t="n">
-        <v>-1.0421</v>
+        <v>-6.1635</v>
       </c>
       <c r="AC9" t="n">
-        <v>8.1305</v>
+        <v>-7.2932</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>222.22</v>
+        <v>265.99</v>
       </c>
       <c r="C10" t="n">
-        <v>242.4</v>
+        <v>274.88</v>
       </c>
       <c r="D10" t="n">
-        <v>214.74</v>
+        <v>261.6</v>
       </c>
       <c r="E10" t="n">
-        <v>234.68</v>
+        <v>272.5</v>
       </c>
       <c r="F10" t="n">
-        <v>76.34</v>
+        <v>82.88</v>
       </c>
       <c r="G10" t="n">
-        <v>78.36</v>
+        <v>85.03</v>
       </c>
       <c r="H10" t="n">
-        <v>74.29000000000001</v>
+        <v>82.64</v>
       </c>
       <c r="I10" t="n">
-        <v>77.52</v>
+        <v>84.59</v>
       </c>
       <c r="J10" t="n">
-        <v>4.9523</v>
+        <v>4.0231</v>
       </c>
       <c r="K10" t="n">
-        <v>5.0907</v>
+        <v>4.122</v>
       </c>
       <c r="L10" t="n">
-        <v>4.4877</v>
+        <v>3.865</v>
       </c>
       <c r="M10" t="n">
-        <v>4.6656</v>
+        <v>3.9045</v>
       </c>
       <c r="N10" t="n">
-        <v>40.0106</v>
+        <v>36.6641</v>
       </c>
       <c r="O10" t="n">
-        <v>41.0933</v>
+        <v>36.7723</v>
       </c>
       <c r="P10" t="n">
-        <v>38.9476</v>
+        <v>35.5814</v>
       </c>
       <c r="Q10" t="n">
-        <v>39.4102</v>
+        <v>35.7389</v>
       </c>
       <c r="R10" t="n">
-        <v>4.7725</v>
+        <v>16.1156</v>
       </c>
       <c r="S10" t="n">
-        <v>16.3626</v>
+        <v>50.8442</v>
       </c>
       <c r="T10" t="n">
-        <v>28.5636</v>
+        <v>28.8782</v>
       </c>
       <c r="U10" t="n">
-        <v>1.9866</v>
+        <v>9.120200000000001</v>
       </c>
       <c r="V10" t="n">
-        <v>5.1546</v>
+        <v>22.1164</v>
       </c>
       <c r="W10" t="n">
-        <v>6.1191</v>
+        <v>10.9086</v>
       </c>
       <c r="X10" t="n">
-        <v>-5.0318</v>
+        <v>-16.313</v>
       </c>
       <c r="Y10" t="n">
-        <v>-20.4053</v>
+        <v>-39.878</v>
       </c>
       <c r="Z10" t="n">
-        <v>-30.9945</v>
+        <v>-30.5805</v>
       </c>
       <c r="AA10" t="n">
-        <v>-1.9349</v>
+        <v>-9.3156</v>
       </c>
       <c r="AB10" t="n">
-        <v>-6.1635</v>
+        <v>-19.7567</v>
       </c>
       <c r="AC10" t="n">
-        <v>-7.2932</v>
+        <v>-11.997</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>265.99</v>
+        <v>267.13</v>
       </c>
       <c r="C11" t="n">
-        <v>274.88</v>
+        <v>274.93</v>
       </c>
       <c r="D11" t="n">
-        <v>261.6</v>
+        <v>226</v>
       </c>
       <c r="E11" t="n">
-        <v>272.5</v>
+        <v>226.19</v>
       </c>
       <c r="F11" t="n">
-        <v>82.88</v>
+        <v>84.19</v>
       </c>
       <c r="G11" t="n">
-        <v>85.03</v>
+        <v>84.83</v>
       </c>
       <c r="H11" t="n">
-        <v>82.64</v>
+        <v>79.86</v>
       </c>
       <c r="I11" t="n">
-        <v>84.59</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>4.0231</v>
+        <v>3.9836</v>
       </c>
       <c r="K11" t="n">
-        <v>4.122</v>
+        <v>4.5965</v>
       </c>
       <c r="L11" t="n">
         <v>3.865</v>
       </c>
       <c r="M11" t="n">
-        <v>3.9045</v>
+        <v>4.5767</v>
       </c>
       <c r="N11" t="n">
-        <v>36.6641</v>
+        <v>35.9652</v>
       </c>
       <c r="O11" t="n">
-        <v>36.7723</v>
+        <v>37.7861</v>
       </c>
       <c r="P11" t="n">
-        <v>35.5814</v>
+        <v>35.6896</v>
       </c>
       <c r="Q11" t="n">
-        <v>35.7389</v>
+        <v>37.7468</v>
       </c>
       <c r="R11" t="n">
-        <v>16.1156</v>
+        <v>-16.9945</v>
       </c>
       <c r="S11" t="n">
-        <v>50.8442</v>
+        <v>0.9822</v>
       </c>
       <c r="T11" t="n">
-        <v>28.8782</v>
+        <v>12.1529</v>
       </c>
       <c r="U11" t="n">
-        <v>9.120200000000001</v>
+        <v>-5.5089</v>
       </c>
       <c r="V11" t="n">
-        <v>22.1164</v>
+        <v>5.1572</v>
       </c>
       <c r="W11" t="n">
-        <v>10.9086</v>
+        <v>8.4238</v>
       </c>
       <c r="X11" t="n">
-        <v>-16.313</v>
+        <v>17.216</v>
       </c>
       <c r="Y11" t="n">
-        <v>-39.878</v>
+        <v>-6.8413</v>
       </c>
       <c r="Z11" t="n">
-        <v>-30.5805</v>
+        <v>-21.922</v>
       </c>
       <c r="AA11" t="n">
-        <v>-9.3156</v>
+        <v>5.6182</v>
       </c>
       <c r="AB11" t="n">
-        <v>-19.7567</v>
+        <v>-6.074</v>
       </c>
       <c r="AC11" t="n">
-        <v>-11.997</v>
+        <v>-10.1241</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>267.13</v>
+        <v>247.42</v>
       </c>
       <c r="C12" t="n">
-        <v>274.93</v>
+        <v>259.79</v>
       </c>
       <c r="D12" t="n">
-        <v>226</v>
+        <v>233.3</v>
       </c>
       <c r="E12" t="n">
-        <v>226.19</v>
+        <v>233.86</v>
       </c>
       <c r="F12" t="n">
-        <v>84.19</v>
+        <v>81.67</v>
       </c>
       <c r="G12" t="n">
-        <v>84.83</v>
+        <v>81.81</v>
       </c>
       <c r="H12" t="n">
-        <v>79.86</v>
+        <v>76.94</v>
       </c>
       <c r="I12" t="n">
-        <v>79.93000000000001</v>
+        <v>77.54000000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>3.9836</v>
+        <v>4.122</v>
       </c>
       <c r="K12" t="n">
-        <v>4.5965</v>
+        <v>4.4086</v>
       </c>
       <c r="L12" t="n">
-        <v>3.865</v>
+        <v>3.8749</v>
       </c>
       <c r="M12" t="n">
-        <v>4.5767</v>
+        <v>4.4086</v>
       </c>
       <c r="N12" t="n">
-        <v>35.9652</v>
+        <v>36.9397</v>
       </c>
       <c r="O12" t="n">
-        <v>37.7861</v>
+        <v>39.1641</v>
       </c>
       <c r="P12" t="n">
-        <v>35.6896</v>
+        <v>36.8708</v>
       </c>
       <c r="Q12" t="n">
-        <v>37.7468</v>
+        <v>38.8984</v>
       </c>
       <c r="R12" t="n">
-        <v>-16.9945</v>
+        <v>3.391</v>
       </c>
       <c r="S12" t="n">
-        <v>0.9822</v>
+        <v>-0.3494</v>
       </c>
       <c r="T12" t="n">
-        <v>12.1529</v>
+        <v>29.4547</v>
       </c>
       <c r="U12" t="n">
-        <v>-5.5089</v>
+        <v>-2.9901</v>
       </c>
       <c r="V12" t="n">
-        <v>5.1572</v>
+        <v>0.0258</v>
       </c>
       <c r="W12" t="n">
-        <v>8.4238</v>
+        <v>11.9388</v>
       </c>
       <c r="X12" t="n">
-        <v>17.216</v>
+        <v>-3.673</v>
       </c>
       <c r="Y12" t="n">
-        <v>-6.8413</v>
+        <v>-5.5084</v>
       </c>
       <c r="Z12" t="n">
-        <v>-21.922</v>
+        <v>-32.1159</v>
       </c>
       <c r="AA12" t="n">
-        <v>5.6182</v>
+        <v>3.0509</v>
       </c>
       <c r="AB12" t="n">
-        <v>-6.074</v>
+        <v>-1.2986</v>
       </c>
       <c r="AC12" t="n">
-        <v>-10.1241</v>
+        <v>-12.6628</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>247.42</v>
+        <v>266.04</v>
       </c>
       <c r="C13" t="n">
-        <v>259.79</v>
+        <v>286.15</v>
       </c>
       <c r="D13" t="n">
-        <v>233.3</v>
+        <v>265</v>
       </c>
       <c r="E13" t="n">
-        <v>233.86</v>
+        <v>279.29</v>
       </c>
       <c r="F13" t="n">
-        <v>81.67</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>81.81</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>76.94</v>
+        <v>80.63</v>
       </c>
       <c r="I13" t="n">
-        <v>77.54000000000001</v>
+        <v>82.87</v>
       </c>
       <c r="J13" t="n">
-        <v>4.122</v>
+        <v>3.8156</v>
       </c>
       <c r="K13" t="n">
-        <v>4.4086</v>
+        <v>3.8254</v>
       </c>
       <c r="L13" t="n">
-        <v>3.8749</v>
+        <v>3.4103</v>
       </c>
       <c r="M13" t="n">
-        <v>4.4086</v>
+        <v>3.5487</v>
       </c>
       <c r="N13" t="n">
-        <v>36.9397</v>
+        <v>36.6149</v>
       </c>
       <c r="O13" t="n">
-        <v>39.1641</v>
+        <v>37.3531</v>
       </c>
       <c r="P13" t="n">
-        <v>36.8708</v>
+        <v>35.857</v>
       </c>
       <c r="Q13" t="n">
-        <v>38.8984</v>
+        <v>36.1719</v>
       </c>
       <c r="R13" t="n">
-        <v>3.391</v>
+        <v>19.4262</v>
       </c>
       <c r="S13" t="n">
-        <v>-0.3494</v>
+        <v>2.4917</v>
       </c>
       <c r="T13" t="n">
-        <v>29.4547</v>
+        <v>24.6886</v>
       </c>
       <c r="U13" t="n">
-        <v>-2.9901</v>
+        <v>6.8739</v>
       </c>
       <c r="V13" t="n">
-        <v>0.0258</v>
+        <v>-2.0333</v>
       </c>
       <c r="W13" t="n">
-        <v>11.9388</v>
+        <v>9.0251</v>
       </c>
       <c r="X13" t="n">
-        <v>-3.673</v>
+        <v>-19.5051</v>
       </c>
       <c r="Y13" t="n">
-        <v>-5.5084</v>
+        <v>-9.1126</v>
       </c>
       <c r="Z13" t="n">
-        <v>-32.1159</v>
+        <v>-27.7662</v>
       </c>
       <c r="AA13" t="n">
-        <v>3.0509</v>
+        <v>-7.0093</v>
       </c>
       <c r="AB13" t="n">
-        <v>-1.2986</v>
+        <v>1.2116</v>
       </c>
       <c r="AC13" t="n">
-        <v>-12.6628</v>
+        <v>-9.992800000000001</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>266.04</v>
+        <v>299.26</v>
       </c>
       <c r="C14" t="n">
-        <v>286.15</v>
+        <v>302</v>
       </c>
       <c r="D14" t="n">
-        <v>265</v>
+        <v>286.24</v>
       </c>
       <c r="E14" t="n">
-        <v>279.29</v>
+        <v>300.77</v>
       </c>
       <c r="F14" t="n">
-        <v>82.09999999999999</v>
+        <v>83.95</v>
       </c>
       <c r="G14" t="n">
-        <v>83.59999999999999</v>
+        <v>85.11</v>
       </c>
       <c r="H14" t="n">
-        <v>80.63</v>
+        <v>81.39</v>
       </c>
       <c r="I14" t="n">
-        <v>82.87</v>
+        <v>82.58</v>
       </c>
       <c r="J14" t="n">
-        <v>3.8156</v>
+        <v>3.2917</v>
       </c>
       <c r="K14" t="n">
-        <v>3.8254</v>
+        <v>3.4498</v>
       </c>
       <c r="L14" t="n">
-        <v>3.4103</v>
+        <v>3.2521</v>
       </c>
       <c r="M14" t="n">
-        <v>3.5487</v>
+        <v>3.262</v>
       </c>
       <c r="N14" t="n">
-        <v>36.6149</v>
+        <v>35.7389</v>
       </c>
       <c r="O14" t="n">
-        <v>37.3531</v>
+        <v>36.8511</v>
       </c>
       <c r="P14" t="n">
-        <v>35.857</v>
+        <v>35.2369</v>
       </c>
       <c r="Q14" t="n">
-        <v>36.1719</v>
+        <v>36.3491</v>
       </c>
       <c r="R14" t="n">
-        <v>19.4262</v>
+        <v>7.6909</v>
       </c>
       <c r="S14" t="n">
-        <v>2.4917</v>
+        <v>32.9723</v>
       </c>
       <c r="T14" t="n">
-        <v>24.6886</v>
+        <v>28.1618</v>
       </c>
       <c r="U14" t="n">
-        <v>6.8739</v>
+        <v>-0.3499</v>
       </c>
       <c r="V14" t="n">
-        <v>-2.0333</v>
+        <v>3.3154</v>
       </c>
       <c r="W14" t="n">
-        <v>9.0251</v>
+        <v>6.5273</v>
       </c>
       <c r="X14" t="n">
-        <v>-19.5051</v>
+        <v>-8.079000000000001</v>
       </c>
       <c r="Y14" t="n">
-        <v>-9.1126</v>
+        <v>-28.7259</v>
       </c>
       <c r="Z14" t="n">
-        <v>-27.7662</v>
+        <v>-30.084</v>
       </c>
       <c r="AA14" t="n">
-        <v>-7.0093</v>
+        <v>0.4899</v>
       </c>
       <c r="AB14" t="n">
-        <v>1.2116</v>
+        <v>-3.7028</v>
       </c>
       <c r="AC14" t="n">
-        <v>-9.992800000000001</v>
+        <v>-7.7673</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>299.26</v>
+        <v>236</v>
       </c>
       <c r="C15" t="n">
-        <v>302</v>
+        <v>252.98</v>
       </c>
       <c r="D15" t="n">
-        <v>286.24</v>
+        <v>223</v>
       </c>
       <c r="E15" t="n">
-        <v>300.77</v>
+        <v>231.42</v>
       </c>
       <c r="F15" t="n">
-        <v>83.95</v>
+        <v>75.12</v>
       </c>
       <c r="G15" t="n">
-        <v>85.11</v>
+        <v>77.73999999999999</v>
       </c>
       <c r="H15" t="n">
-        <v>81.39</v>
+        <v>73.91</v>
       </c>
       <c r="I15" t="n">
-        <v>82.58</v>
+        <v>74.44</v>
       </c>
       <c r="J15" t="n">
-        <v>3.2917</v>
+        <v>3.99</v>
       </c>
       <c r="K15" t="n">
-        <v>3.4498</v>
+        <v>4.13</v>
       </c>
       <c r="L15" t="n">
-        <v>3.2521</v>
+        <v>3.8</v>
       </c>
       <c r="M15" t="n">
-        <v>3.262</v>
+        <v>4.04</v>
       </c>
       <c r="N15" t="n">
-        <v>35.7389</v>
+        <v>39.6267</v>
       </c>
       <c r="O15" t="n">
-        <v>36.8511</v>
+        <v>40.1582</v>
       </c>
       <c r="P15" t="n">
-        <v>35.2369</v>
+        <v>38.4653</v>
       </c>
       <c r="Q15" t="n">
-        <v>36.3491</v>
+        <v>39.922</v>
       </c>
       <c r="R15" t="n">
-        <v>7.6909</v>
+        <v>-23.0575</v>
       </c>
       <c r="S15" t="n">
-        <v>32.9723</v>
+        <v>-1.0434</v>
       </c>
       <c r="T15" t="n">
-        <v>28.1618</v>
+        <v>-15.0752</v>
       </c>
       <c r="U15" t="n">
-        <v>-0.3499</v>
+        <v>-9.857100000000001</v>
       </c>
       <c r="V15" t="n">
-        <v>3.3154</v>
+        <v>-3.9979</v>
       </c>
       <c r="W15" t="n">
-        <v>6.5273</v>
+        <v>-11.9991</v>
       </c>
       <c r="X15" t="n">
-        <v>-8.079000000000001</v>
+        <v>23.8504</v>
       </c>
       <c r="Y15" t="n">
-        <v>-28.7259</v>
+        <v>-8.360900000000001</v>
       </c>
       <c r="Z15" t="n">
-        <v>-30.084</v>
+        <v>3.4704</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.4899</v>
+        <v>9.8294</v>
       </c>
       <c r="AB15" t="n">
-        <v>-3.7028</v>
+        <v>2.6315</v>
       </c>
       <c r="AC15" t="n">
-        <v>-7.7673</v>
+        <v>11.7046</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>236</v>
+        <v>233.11</v>
       </c>
       <c r="C16" t="n">
-        <v>252.98</v>
+        <v>237</v>
       </c>
       <c r="D16" t="n">
-        <v>223</v>
+        <v>211.13</v>
       </c>
       <c r="E16" t="n">
-        <v>231.42</v>
+        <v>229.57</v>
       </c>
       <c r="F16" t="n">
-        <v>75.12</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>77.73999999999999</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="H16" t="n">
-        <v>73.91</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="I16" t="n">
-        <v>74.44</v>
+        <v>73.3</v>
       </c>
       <c r="J16" t="n">
-        <v>3.99</v>
+        <v>4</v>
       </c>
       <c r="K16" t="n">
-        <v>4.13</v>
+        <v>4.39</v>
       </c>
       <c r="L16" t="n">
-        <v>3.8</v>
+        <v>3.92</v>
       </c>
       <c r="M16" t="n">
-        <v>4.04</v>
+        <v>4.08</v>
       </c>
       <c r="N16" t="n">
-        <v>39.6267</v>
+        <v>39.66</v>
       </c>
       <c r="O16" t="n">
-        <v>40.1582</v>
+        <v>41.49</v>
       </c>
       <c r="P16" t="n">
-        <v>38.4653</v>
+        <v>38.9</v>
       </c>
       <c r="Q16" t="n">
-        <v>39.922</v>
+        <v>40.45</v>
       </c>
       <c r="R16" t="n">
-        <v>-23.0575</v>
+        <v>-0.7994</v>
       </c>
       <c r="S16" t="n">
-        <v>-1.0434</v>
+        <v>-17.8023</v>
       </c>
       <c r="T16" t="n">
-        <v>-15.0752</v>
+        <v>1.4943</v>
       </c>
       <c r="U16" t="n">
-        <v>-9.857100000000001</v>
+        <v>-1.5314</v>
       </c>
       <c r="V16" t="n">
-        <v>-3.9979</v>
+        <v>-11.5482</v>
       </c>
       <c r="W16" t="n">
-        <v>-11.9991</v>
+        <v>-8.2948</v>
       </c>
       <c r="X16" t="n">
-        <v>23.8504</v>
+        <v>0.9901</v>
       </c>
       <c r="Y16" t="n">
-        <v>-8.360900000000001</v>
+        <v>14.9717</v>
       </c>
       <c r="Z16" t="n">
-        <v>3.4704</v>
+        <v>-10.8528</v>
       </c>
       <c r="AA16" t="n">
-        <v>9.8294</v>
+        <v>1.3226</v>
       </c>
       <c r="AB16" t="n">
-        <v>2.6315</v>
+        <v>11.8271</v>
       </c>
       <c r="AC16" t="n">
-        <v>11.7046</v>
+        <v>7.1614</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>233.11</v>
+        <v>268.05</v>
       </c>
       <c r="C17" t="n">
-        <v>237</v>
+        <v>268.4</v>
       </c>
       <c r="D17" t="n">
-        <v>211.13</v>
+        <v>225.74</v>
       </c>
       <c r="E17" t="n">
-        <v>229.57</v>
+        <v>252.61</v>
       </c>
       <c r="F17" t="n">
-        <v>74.79000000000001</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="G17" t="n">
-        <v>76.18000000000001</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="H17" t="n">
-        <v>71.34999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I17" t="n">
-        <v>73.3</v>
+        <v>74.95</v>
       </c>
       <c r="J17" t="n">
-        <v>4</v>
+        <v>3.38</v>
       </c>
       <c r="K17" t="n">
-        <v>4.39</v>
+        <v>4.15</v>
       </c>
       <c r="L17" t="n">
-        <v>3.92</v>
+        <v>3.37</v>
       </c>
       <c r="M17" t="n">
-        <v>4.08</v>
+        <v>3.63</v>
       </c>
       <c r="N17" t="n">
-        <v>39.66</v>
+        <v>37.87</v>
       </c>
       <c r="O17" t="n">
-        <v>41.49</v>
+        <v>41.37</v>
       </c>
       <c r="P17" t="n">
-        <v>38.9</v>
+        <v>37.71</v>
       </c>
       <c r="Q17" t="n">
-        <v>40.45</v>
+        <v>39.47</v>
       </c>
       <c r="R17" t="n">
-        <v>-0.7994</v>
+        <v>10.0362</v>
       </c>
       <c r="S17" t="n">
-        <v>-17.8023</v>
+        <v>-16.0122</v>
       </c>
       <c r="T17" t="n">
-        <v>1.4943</v>
+        <v>8.0176</v>
       </c>
       <c r="U17" t="n">
-        <v>-1.5314</v>
+        <v>2.251</v>
       </c>
       <c r="V17" t="n">
-        <v>-11.5482</v>
+        <v>-9.2395</v>
       </c>
       <c r="W17" t="n">
-        <v>-8.2948</v>
+        <v>-3.3402</v>
       </c>
       <c r="X17" t="n">
-        <v>0.9901</v>
+        <v>-11.0294</v>
       </c>
       <c r="Y17" t="n">
-        <v>14.9717</v>
+        <v>11.2814</v>
       </c>
       <c r="Z17" t="n">
-        <v>-10.8528</v>
+        <v>-17.6609</v>
       </c>
       <c r="AA17" t="n">
-        <v>1.3226</v>
+        <v>-2.4227</v>
       </c>
       <c r="AB17" t="n">
-        <v>11.8271</v>
+        <v>8.585900000000001</v>
       </c>
       <c r="AC17" t="n">
-        <v>7.1614</v>
+        <v>1.4695</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>268.05</v>
+        <v>226.24</v>
       </c>
       <c r="C18" t="n">
-        <v>268.4</v>
+        <v>231.25</v>
       </c>
       <c r="D18" t="n">
-        <v>225.74</v>
+        <v>212.1</v>
       </c>
       <c r="E18" t="n">
-        <v>252.61</v>
+        <v>215.6</v>
       </c>
       <c r="F18" t="n">
-        <v>77.95999999999999</v>
+        <v>72.09</v>
       </c>
       <c r="G18" t="n">
-        <v>78.23999999999999</v>
+        <v>74.69</v>
       </c>
       <c r="H18" t="n">
-        <v>71.59999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="I18" t="n">
-        <v>74.95</v>
+        <v>71.83</v>
       </c>
       <c r="J18" t="n">
-        <v>3.38</v>
+        <v>4.04</v>
       </c>
       <c r="K18" t="n">
-        <v>4.15</v>
+        <v>4.25</v>
       </c>
       <c r="L18" t="n">
-        <v>3.37</v>
+        <v>3.95</v>
       </c>
       <c r="M18" t="n">
-        <v>3.63</v>
+        <v>4.24</v>
       </c>
       <c r="N18" t="n">
-        <v>37.87</v>
+        <v>41.08</v>
       </c>
       <c r="O18" t="n">
-        <v>41.37</v>
+        <v>41.79</v>
       </c>
       <c r="P18" t="n">
-        <v>37.71</v>
+        <v>39.69</v>
       </c>
       <c r="Q18" t="n">
-        <v>39.47</v>
+        <v>41.31</v>
       </c>
       <c r="R18" t="n">
-        <v>10.0362</v>
+        <v>-14.651</v>
       </c>
       <c r="S18" t="n">
-        <v>-16.0122</v>
+        <v>-6.8361</v>
       </c>
       <c r="T18" t="n">
-        <v>8.0176</v>
+        <v>-22.8043</v>
       </c>
       <c r="U18" t="n">
-        <v>2.251</v>
+        <v>-4.1628</v>
       </c>
       <c r="V18" t="n">
-        <v>-9.2395</v>
+        <v>-3.5062</v>
       </c>
       <c r="W18" t="n">
-        <v>-3.3402</v>
+        <v>-13.3221</v>
       </c>
       <c r="X18" t="n">
-        <v>-11.0294</v>
+        <v>16.8044</v>
       </c>
       <c r="Y18" t="n">
-        <v>11.2814</v>
+        <v>4.9505</v>
       </c>
       <c r="Z18" t="n">
-        <v>-17.6609</v>
+        <v>19.4804</v>
       </c>
       <c r="AA18" t="n">
-        <v>-2.4227</v>
+        <v>4.6618</v>
       </c>
       <c r="AB18" t="n">
-        <v>8.585900000000001</v>
+        <v>3.4768</v>
       </c>
       <c r="AC18" t="n">
-        <v>1.4695</v>
+        <v>14.2047</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>226.24</v>
+        <v>216.36</v>
       </c>
       <c r="C19" t="n">
-        <v>231.25</v>
+        <v>238.65</v>
       </c>
       <c r="D19" t="n">
-        <v>212.1</v>
+        <v>192.3</v>
       </c>
       <c r="E19" t="n">
-        <v>215.6</v>
+        <v>236.52</v>
       </c>
       <c r="F19" t="n">
-        <v>72.09</v>
+        <v>74.12</v>
       </c>
       <c r="G19" t="n">
-        <v>74.69</v>
+        <v>77.38</v>
       </c>
       <c r="H19" t="n">
-        <v>70.72</v>
+        <v>71.45</v>
       </c>
       <c r="I19" t="n">
-        <v>71.83</v>
+        <v>77.19</v>
       </c>
       <c r="J19" t="n">
-        <v>4.04</v>
+        <v>4.16</v>
       </c>
       <c r="K19" t="n">
-        <v>4.25</v>
+        <v>4.63</v>
       </c>
       <c r="L19" t="n">
-        <v>3.95</v>
+        <v>3.7</v>
       </c>
       <c r="M19" t="n">
-        <v>4.24</v>
+        <v>3.72</v>
       </c>
       <c r="N19" t="n">
-        <v>41.08</v>
+        <v>39.91</v>
       </c>
       <c r="O19" t="n">
-        <v>41.79</v>
+        <v>41.43</v>
       </c>
       <c r="P19" t="n">
-        <v>39.69</v>
+        <v>38.08</v>
       </c>
       <c r="Q19" t="n">
-        <v>41.31</v>
+        <v>38.16</v>
       </c>
       <c r="R19" t="n">
-        <v>-14.651</v>
+        <v>9.703200000000001</v>
       </c>
       <c r="S19" t="n">
-        <v>-6.8361</v>
+        <v>3.0274</v>
       </c>
       <c r="T19" t="n">
-        <v>-22.8043</v>
+        <v>-21.3618</v>
       </c>
       <c r="U19" t="n">
-        <v>-4.1628</v>
+        <v>7.4621</v>
       </c>
       <c r="V19" t="n">
-        <v>-3.5062</v>
+        <v>5.307</v>
       </c>
       <c r="W19" t="n">
-        <v>-13.3221</v>
+        <v>-6.527</v>
       </c>
       <c r="X19" t="n">
-        <v>16.8044</v>
+        <v>-12.2642</v>
       </c>
       <c r="Y19" t="n">
-        <v>4.9505</v>
+        <v>-8.823499999999999</v>
       </c>
       <c r="Z19" t="n">
-        <v>19.4804</v>
+        <v>14.0405</v>
       </c>
       <c r="AA19" t="n">
-        <v>4.6618</v>
+        <v>-7.6253</v>
       </c>
       <c r="AB19" t="n">
-        <v>3.4768</v>
+        <v>-5.6613</v>
       </c>
       <c r="AC19" t="n">
-        <v>14.2047</v>
+        <v>4.982</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>216.36</v>
+        <v>241.45</v>
       </c>
       <c r="C20" t="n">
-        <v>238.65</v>
+        <v>272</v>
       </c>
       <c r="D20" t="n">
-        <v>192.3</v>
+        <v>240.59</v>
       </c>
       <c r="E20" t="n">
-        <v>236.52</v>
+        <v>266.71</v>
       </c>
       <c r="F20" t="n">
-        <v>74.12</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="G20" t="n">
-        <v>77.38</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="H20" t="n">
-        <v>71.45</v>
+        <v>77.15000000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>77.19</v>
+        <v>81</v>
       </c>
       <c r="J20" t="n">
-        <v>4.16</v>
+        <v>3.66</v>
       </c>
       <c r="K20" t="n">
-        <v>4.63</v>
+        <v>3.68</v>
       </c>
       <c r="L20" t="n">
-        <v>3.7</v>
+        <v>3.17</v>
       </c>
       <c r="M20" t="n">
-        <v>3.72</v>
+        <v>3.24</v>
       </c>
       <c r="N20" t="n">
-        <v>39.91</v>
+        <v>38.16</v>
       </c>
       <c r="O20" t="n">
-        <v>41.43</v>
+        <v>38.2</v>
       </c>
       <c r="P20" t="n">
-        <v>38.08</v>
+        <v>36.03</v>
       </c>
       <c r="Q20" t="n">
-        <v>38.16</v>
+        <v>36.31</v>
       </c>
       <c r="R20" t="n">
-        <v>9.703200000000001</v>
+        <v>12.7642</v>
       </c>
       <c r="S20" t="n">
-        <v>3.0274</v>
+        <v>5.5817</v>
       </c>
       <c r="T20" t="n">
-        <v>-21.3618</v>
+        <v>15.2493</v>
       </c>
       <c r="U20" t="n">
-        <v>7.4621</v>
+        <v>4.9359</v>
       </c>
       <c r="V20" t="n">
-        <v>5.307</v>
+        <v>8.071999999999999</v>
       </c>
       <c r="W20" t="n">
-        <v>-6.527</v>
+        <v>8.8125</v>
       </c>
       <c r="X20" t="n">
-        <v>-12.2642</v>
+        <v>-12.9032</v>
       </c>
       <c r="Y20" t="n">
-        <v>-8.823499999999999</v>
+        <v>-10.7438</v>
       </c>
       <c r="Z20" t="n">
-        <v>14.0405</v>
+        <v>-19.802</v>
       </c>
       <c r="AA20" t="n">
-        <v>-7.6253</v>
+        <v>-4.848</v>
       </c>
       <c r="AB20" t="n">
-        <v>-5.6613</v>
+        <v>-8.0061</v>
       </c>
       <c r="AC20" t="n">
-        <v>4.982</v>
+        <v>-9.047599999999999</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>241.45</v>
+        <v>237.79</v>
       </c>
       <c r="C21" t="n">
-        <v>272</v>
+        <v>246.47</v>
       </c>
       <c r="D21" t="n">
-        <v>240.59</v>
+        <v>215.38</v>
       </c>
       <c r="E21" t="n">
-        <v>266.71</v>
+        <v>217.55</v>
       </c>
       <c r="F21" t="n">
-        <v>77.23999999999999</v>
+        <v>78.72</v>
       </c>
       <c r="G21" t="n">
-        <v>81.54000000000001</v>
+        <v>79.64</v>
       </c>
       <c r="H21" t="n">
-        <v>77.15000000000001</v>
+        <v>77.23</v>
       </c>
       <c r="I21" t="n">
-        <v>81</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J21" t="n">
-        <v>3.66</v>
+        <v>3.59</v>
       </c>
       <c r="K21" t="n">
-        <v>3.68</v>
+        <v>3.89</v>
       </c>
       <c r="L21" t="n">
-        <v>3.17</v>
+        <v>3.51</v>
       </c>
       <c r="M21" t="n">
-        <v>3.24</v>
+        <v>3.86</v>
       </c>
       <c r="N21" t="n">
-        <v>38.16</v>
+        <v>37.31</v>
       </c>
       <c r="O21" t="n">
-        <v>38.2</v>
+        <v>37.98</v>
       </c>
       <c r="P21" t="n">
-        <v>36.03</v>
+        <v>36.9</v>
       </c>
       <c r="Q21" t="n">
-        <v>36.31</v>
+        <v>37.88</v>
       </c>
       <c r="R21" t="n">
-        <v>12.7642</v>
+        <v>-18.432</v>
       </c>
       <c r="S21" t="n">
-        <v>5.5817</v>
+        <v>0.9045</v>
       </c>
       <c r="T21" t="n">
-        <v>15.2493</v>
+        <v>-5.2359</v>
       </c>
       <c r="U21" t="n">
-        <v>4.9359</v>
+        <v>-4.3704</v>
       </c>
       <c r="V21" t="n">
-        <v>8.071999999999999</v>
+        <v>7.838</v>
       </c>
       <c r="W21" t="n">
-        <v>8.8125</v>
+        <v>5.6753</v>
       </c>
       <c r="X21" t="n">
-        <v>-12.9032</v>
+        <v>19.1358</v>
       </c>
       <c r="Y21" t="n">
-        <v>-10.7438</v>
+        <v>-8.962300000000001</v>
       </c>
       <c r="Z21" t="n">
-        <v>-19.802</v>
+        <v>-5.3922</v>
       </c>
       <c r="AA21" t="n">
-        <v>-4.848</v>
+        <v>4.3239</v>
       </c>
       <c r="AB21" t="n">
-        <v>-8.0061</v>
+        <v>-8.303100000000001</v>
       </c>
       <c r="AC21" t="n">
-        <v>-9.047599999999999</v>
+        <v>-6.3535</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>237.785</v>
+        <v>219.23</v>
       </c>
       <c r="C22" t="n">
-        <v>246.44</v>
+        <v>226.13</v>
       </c>
       <c r="D22" t="n">
-        <v>215.3807</v>
+        <v>168.88</v>
       </c>
       <c r="E22" t="n">
-        <v>217.55</v>
+        <v>181.47</v>
       </c>
       <c r="F22" t="n">
-        <v>78.72</v>
+        <v>77.47</v>
       </c>
       <c r="G22" t="n">
-        <v>79.64</v>
+        <v>79.13500000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>77.23</v>
+        <v>71.72</v>
       </c>
       <c r="I22" t="n">
-        <v>77.45999999999999</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="J22" t="n">
-        <v>3.5903</v>
+        <v>3.84</v>
       </c>
       <c r="K22" t="n">
-        <v>3.89</v>
+        <v>4.74</v>
       </c>
       <c r="L22" t="n">
-        <v>3.51</v>
+        <v>3.71</v>
       </c>
       <c r="M22" t="n">
-        <v>3.86</v>
+        <v>4.51</v>
       </c>
       <c r="N22" t="n">
-        <v>37.31</v>
+        <v>37.91</v>
       </c>
       <c r="O22" t="n">
-        <v>37.975</v>
+        <v>40.72</v>
       </c>
       <c r="P22" t="n">
-        <v>36.9</v>
+        <v>37.08</v>
       </c>
       <c r="Q22" t="n">
-        <v>37.88</v>
+        <v>39.95</v>
       </c>
       <c r="R22" t="n">
-        <v>-18.432</v>
+        <v>-16.5847</v>
       </c>
       <c r="S22" t="n">
-        <v>0.9045</v>
+        <v>-23.275</v>
       </c>
       <c r="T22" t="n">
-        <v>-5.2359</v>
+        <v>-28.162</v>
       </c>
       <c r="U22" t="n">
-        <v>-4.3704</v>
+        <v>-5.306</v>
       </c>
       <c r="V22" t="n">
-        <v>7.838</v>
+        <v>-4.9747</v>
       </c>
       <c r="W22" t="n">
-        <v>5.6753</v>
+        <v>-2.1348</v>
       </c>
       <c r="X22" t="n">
-        <v>19.1358</v>
+        <v>16.8394</v>
       </c>
       <c r="Y22" t="n">
-        <v>-8.962300000000001</v>
+        <v>21.2366</v>
       </c>
       <c r="Z22" t="n">
-        <v>-5.3922</v>
+        <v>24.2424</v>
       </c>
       <c r="AA22" t="n">
-        <v>4.3239</v>
+        <v>5.4646</v>
       </c>
       <c r="AB22" t="n">
-        <v>-8.303100000000001</v>
+        <v>4.6908</v>
       </c>
       <c r="AC22" t="n">
-        <v>-6.3535</v>
+        <v>1.2161</v>
       </c>
     </row>
   </sheetData>
@@ -2412,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-07-03 23:04
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC22"/>
+  <dimension ref="A1:AC21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1803 +568,1712 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>281.47</v>
+        <v>242.04</v>
       </c>
       <c r="C2" t="n">
-        <v>284.58</v>
+        <v>274.5</v>
       </c>
       <c r="D2" t="n">
-        <v>257.26</v>
+        <v>228.55</v>
       </c>
       <c r="E2" t="n">
-        <v>280.54</v>
+        <v>262.7</v>
       </c>
       <c r="F2" t="n">
-        <v>87.68000000000001</v>
+        <v>83.47</v>
       </c>
       <c r="G2" t="n">
-        <v>88.09</v>
+        <v>86.25</v>
       </c>
       <c r="H2" t="n">
-        <v>85.41</v>
+        <v>82.48</v>
       </c>
       <c r="I2" t="n">
-        <v>86.56</v>
+        <v>85.22</v>
       </c>
       <c r="J2" t="n">
-        <v>4.8238</v>
+        <v>5.5059</v>
       </c>
       <c r="K2" t="n">
-        <v>5.2884</v>
+        <v>5.7431</v>
       </c>
       <c r="L2" t="n">
-        <v>4.7645</v>
+        <v>4.9424</v>
       </c>
       <c r="M2" t="n">
-        <v>4.8535</v>
+        <v>5.1401</v>
       </c>
       <c r="N2" t="n">
-        <v>36.1522</v>
+        <v>37.9239</v>
       </c>
       <c r="O2" t="n">
-        <v>37.0971</v>
+        <v>38.3472</v>
       </c>
       <c r="P2" t="n">
-        <v>35.9751</v>
+        <v>36.7428</v>
       </c>
       <c r="Q2" t="n">
-        <v>36.605</v>
+        <v>37.166</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>242.04</v>
+        <v>230.85</v>
       </c>
       <c r="C3" t="n">
-        <v>274.5</v>
+        <v>233.69</v>
       </c>
       <c r="D3" t="n">
-        <v>228.55</v>
+        <v>181.81</v>
       </c>
       <c r="E3" t="n">
-        <v>262.7</v>
+        <v>182.54</v>
       </c>
       <c r="F3" t="n">
-        <v>83.47</v>
+        <v>81.56999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>86.25</v>
+        <v>82.08</v>
       </c>
       <c r="H3" t="n">
-        <v>82.48</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>85.22</v>
+        <v>73.05</v>
       </c>
       <c r="J3" t="n">
-        <v>5.5059</v>
+        <v>5.7925</v>
       </c>
       <c r="K3" t="n">
-        <v>5.7431</v>
+        <v>6.7711</v>
       </c>
       <c r="L3" t="n">
-        <v>4.9424</v>
+        <v>5.7233</v>
       </c>
       <c r="M3" t="n">
-        <v>5.1401</v>
+        <v>6.7612</v>
       </c>
       <c r="N3" t="n">
-        <v>37.9239</v>
+        <v>38.7999</v>
       </c>
       <c r="O3" t="n">
-        <v>38.3472</v>
+        <v>42.6681</v>
       </c>
       <c r="P3" t="n">
-        <v>36.7428</v>
+        <v>38.5637</v>
       </c>
       <c r="Q3" t="n">
-        <v>37.166</v>
+        <v>42.5106</v>
       </c>
       <c r="R3" t="n">
-        <v>-6.3592</v>
+        <v>-30.5139</v>
       </c>
       <c r="U3" t="n">
-        <v>-1.5481</v>
+        <v>-14.2807</v>
       </c>
       <c r="X3" t="n">
-        <v>5.905</v>
+        <v>31.5383</v>
       </c>
       <c r="AA3" t="n">
-        <v>1.5326</v>
+        <v>14.3803</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>230.85</v>
+        <v>210.62</v>
       </c>
       <c r="C4" t="n">
-        <v>233.69</v>
+        <v>222.19</v>
       </c>
       <c r="D4" t="n">
-        <v>181.81</v>
+        <v>201.69</v>
       </c>
       <c r="E4" t="n">
-        <v>182.54</v>
+        <v>211.44</v>
       </c>
       <c r="F4" t="n">
-        <v>81.56999999999999</v>
+        <v>76.86</v>
       </c>
       <c r="G4" t="n">
-        <v>82.08</v>
+        <v>78.47</v>
       </c>
       <c r="H4" t="n">
-        <v>72.68000000000001</v>
+        <v>75.38</v>
       </c>
       <c r="I4" t="n">
-        <v>73.05</v>
+        <v>76.27</v>
       </c>
       <c r="J4" t="n">
-        <v>5.7925</v>
+        <v>5.6442</v>
       </c>
       <c r="K4" t="n">
-        <v>6.7711</v>
+        <v>5.9803</v>
       </c>
       <c r="L4" t="n">
-        <v>5.7233</v>
+        <v>5.2093</v>
       </c>
       <c r="M4" t="n">
-        <v>6.7612</v>
+        <v>5.6245</v>
       </c>
       <c r="N4" t="n">
-        <v>38.7999</v>
+        <v>40.2763</v>
       </c>
       <c r="O4" t="n">
-        <v>42.6681</v>
+        <v>41.1228</v>
       </c>
       <c r="P4" t="n">
-        <v>38.5637</v>
+        <v>39.3314</v>
       </c>
       <c r="Q4" t="n">
-        <v>42.5106</v>
+        <v>40.611</v>
       </c>
       <c r="R4" t="n">
-        <v>-30.5139</v>
+        <v>15.8321</v>
       </c>
       <c r="U4" t="n">
-        <v>-14.2807</v>
+        <v>4.4079</v>
       </c>
       <c r="X4" t="n">
-        <v>31.5383</v>
+        <v>-16.8121</v>
       </c>
       <c r="AA4" t="n">
-        <v>14.3803</v>
+        <v>-4.4685</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>210.62</v>
+        <v>227.06</v>
       </c>
       <c r="C5" t="n">
-        <v>222.19</v>
+        <v>231.02</v>
       </c>
       <c r="D5" t="n">
-        <v>201.69</v>
+        <v>157.56</v>
       </c>
       <c r="E5" t="n">
-        <v>211.44</v>
+        <v>201.68</v>
       </c>
       <c r="F5" t="n">
-        <v>76.86</v>
+        <v>78.48</v>
       </c>
       <c r="G5" t="n">
-        <v>78.47</v>
+        <v>79.34</v>
       </c>
       <c r="H5" t="n">
-        <v>75.38</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="I5" t="n">
-        <v>76.27</v>
+        <v>73.72</v>
       </c>
       <c r="J5" t="n">
-        <v>5.6442</v>
+        <v>5.1895</v>
       </c>
       <c r="K5" t="n">
-        <v>5.9803</v>
+        <v>7.0281</v>
       </c>
       <c r="L5" t="n">
-        <v>5.2093</v>
+        <v>5.0808</v>
       </c>
       <c r="M5" t="n">
-        <v>5.6245</v>
+        <v>5.8617</v>
       </c>
       <c r="N5" t="n">
-        <v>40.2763</v>
+        <v>39.4299</v>
       </c>
       <c r="O5" t="n">
-        <v>41.1228</v>
+        <v>45.6505</v>
       </c>
       <c r="P5" t="n">
-        <v>39.3314</v>
+        <v>38.9673</v>
       </c>
       <c r="Q5" t="n">
-        <v>40.611</v>
+        <v>41.9988</v>
       </c>
       <c r="R5" t="n">
-        <v>15.8321</v>
+        <v>-4.616</v>
       </c>
       <c r="S5" t="n">
-        <v>-24.6311</v>
+        <v>-23.228</v>
       </c>
       <c r="U5" t="n">
-        <v>4.4079</v>
+        <v>-3.3434</v>
       </c>
       <c r="V5" t="n">
-        <v>-11.8877</v>
+        <v>-13.4945</v>
       </c>
       <c r="X5" t="n">
-        <v>-16.8121</v>
+        <v>4.2173</v>
       </c>
       <c r="Y5" t="n">
-        <v>15.8854</v>
+        <v>14.0386</v>
       </c>
       <c r="AA5" t="n">
-        <v>-4.4685</v>
+        <v>3.4173</v>
       </c>
       <c r="AB5" t="n">
-        <v>10.9439</v>
+        <v>13.0033</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>227.06</v>
+        <v>191.54</v>
       </c>
       <c r="C6" t="n">
-        <v>231.02</v>
+        <v>212.99</v>
       </c>
       <c r="D6" t="n">
-        <v>157.56</v>
+        <v>177.3</v>
       </c>
       <c r="E6" t="n">
-        <v>201.68</v>
+        <v>180.65</v>
       </c>
       <c r="F6" t="n">
-        <v>78.48</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>79.34</v>
+        <v>74.7</v>
       </c>
       <c r="H6" t="n">
-        <v>66.79000000000001</v>
+        <v>69</v>
       </c>
       <c r="I6" t="n">
-        <v>73.72</v>
+        <v>69.27</v>
       </c>
       <c r="J6" t="n">
-        <v>5.1895</v>
+        <v>6.1681</v>
       </c>
       <c r="K6" t="n">
-        <v>7.0281</v>
+        <v>6.5734</v>
       </c>
       <c r="L6" t="n">
-        <v>5.0808</v>
+        <v>5.5355</v>
       </c>
       <c r="M6" t="n">
-        <v>5.8617</v>
+        <v>6.4943</v>
       </c>
       <c r="N6" t="n">
-        <v>39.4299</v>
+        <v>43.1209</v>
       </c>
       <c r="O6" t="n">
-        <v>45.6505</v>
+        <v>44.676</v>
       </c>
       <c r="P6" t="n">
-        <v>38.9673</v>
+        <v>41.4082</v>
       </c>
       <c r="Q6" t="n">
-        <v>41.9988</v>
+        <v>44.5382</v>
       </c>
       <c r="R6" t="n">
-        <v>-4.616</v>
+        <v>-10.4274</v>
       </c>
       <c r="S6" t="n">
-        <v>-23.228</v>
+        <v>-1.0354</v>
       </c>
       <c r="U6" t="n">
-        <v>-3.3434</v>
+        <v>-6.0364</v>
       </c>
       <c r="V6" t="n">
-        <v>-13.4945</v>
+        <v>-5.1745</v>
       </c>
       <c r="X6" t="n">
-        <v>4.2173</v>
+        <v>10.7921</v>
       </c>
       <c r="Y6" t="n">
-        <v>14.0386</v>
+        <v>-3.9475</v>
       </c>
       <c r="AA6" t="n">
-        <v>3.4173</v>
+        <v>6.0464</v>
       </c>
       <c r="AB6" t="n">
-        <v>13.0033</v>
+        <v>4.7696</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>191.54</v>
+        <v>192.3</v>
       </c>
       <c r="C7" t="n">
-        <v>212.99</v>
+        <v>225.63</v>
       </c>
       <c r="D7" t="n">
-        <v>177.3</v>
+        <v>192.3</v>
       </c>
       <c r="E7" t="n">
-        <v>180.65</v>
+        <v>223.99</v>
       </c>
       <c r="F7" t="n">
-        <v>71.68000000000001</v>
+        <v>70.89</v>
       </c>
       <c r="G7" t="n">
-        <v>74.7</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>69</v>
+        <v>69.59</v>
       </c>
       <c r="I7" t="n">
-        <v>69.27</v>
+        <v>76.01000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>6.1681</v>
+        <v>6.0298</v>
       </c>
       <c r="K7" t="n">
-        <v>6.5734</v>
+        <v>6.0298</v>
       </c>
       <c r="L7" t="n">
-        <v>5.5355</v>
+        <v>4.8436</v>
       </c>
       <c r="M7" t="n">
-        <v>6.4943</v>
+        <v>4.9128</v>
       </c>
       <c r="N7" t="n">
-        <v>43.1209</v>
+        <v>43.4851</v>
       </c>
       <c r="O7" t="n">
-        <v>44.676</v>
+        <v>44.302</v>
       </c>
       <c r="P7" t="n">
-        <v>41.4082</v>
+        <v>39.8039</v>
       </c>
       <c r="Q7" t="n">
-        <v>44.5382</v>
+        <v>40.1878</v>
       </c>
       <c r="R7" t="n">
-        <v>-10.4274</v>
+        <v>23.9911</v>
       </c>
       <c r="S7" t="n">
-        <v>-1.0354</v>
+        <v>5.9355</v>
       </c>
       <c r="T7" t="n">
-        <v>-35.6063</v>
+        <v>-14.7354</v>
       </c>
       <c r="U7" t="n">
-        <v>-6.0364</v>
+        <v>9.73</v>
       </c>
       <c r="V7" t="n">
-        <v>-5.1745</v>
+        <v>-0.3409</v>
       </c>
       <c r="W7" t="n">
-        <v>-19.9746</v>
+        <v>-10.8073</v>
       </c>
       <c r="X7" t="n">
-        <v>10.7921</v>
+        <v>-24.3521</v>
       </c>
       <c r="Y7" t="n">
-        <v>-3.9475</v>
+        <v>-12.6536</v>
       </c>
       <c r="Z7" t="n">
-        <v>33.8065</v>
+        <v>-4.4221</v>
       </c>
       <c r="AA7" t="n">
-        <v>6.0464</v>
+        <v>-9.767799999999999</v>
       </c>
       <c r="AB7" t="n">
-        <v>4.7696</v>
+        <v>-1.0421</v>
       </c>
       <c r="AC7" t="n">
-        <v>21.6724</v>
+        <v>8.1305</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>192.3</v>
+        <v>222.22</v>
       </c>
       <c r="C8" t="n">
-        <v>225.63</v>
+        <v>242.4</v>
       </c>
       <c r="D8" t="n">
-        <v>192.3</v>
+        <v>214.74</v>
       </c>
       <c r="E8" t="n">
-        <v>223.99</v>
+        <v>234.68</v>
       </c>
       <c r="F8" t="n">
-        <v>70.89</v>
+        <v>76.34</v>
       </c>
       <c r="G8" t="n">
-        <v>76.59999999999999</v>
+        <v>78.36</v>
       </c>
       <c r="H8" t="n">
-        <v>69.59</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="I8" t="n">
-        <v>76.01000000000001</v>
+        <v>77.52</v>
       </c>
       <c r="J8" t="n">
-        <v>6.0298</v>
+        <v>4.9523</v>
       </c>
       <c r="K8" t="n">
-        <v>6.0298</v>
+        <v>5.0907</v>
       </c>
       <c r="L8" t="n">
-        <v>4.8436</v>
+        <v>4.4877</v>
       </c>
       <c r="M8" t="n">
-        <v>4.9128</v>
+        <v>4.6656</v>
       </c>
       <c r="N8" t="n">
-        <v>43.4851</v>
+        <v>40.0106</v>
       </c>
       <c r="O8" t="n">
-        <v>44.302</v>
+        <v>41.0933</v>
       </c>
       <c r="P8" t="n">
-        <v>39.8039</v>
+        <v>38.9476</v>
       </c>
       <c r="Q8" t="n">
-        <v>40.1878</v>
+        <v>39.4102</v>
       </c>
       <c r="R8" t="n">
-        <v>23.9911</v>
+        <v>4.7725</v>
       </c>
       <c r="S8" t="n">
-        <v>5.9355</v>
+        <v>16.3626</v>
       </c>
       <c r="T8" t="n">
-        <v>-14.7354</v>
+        <v>28.5636</v>
       </c>
       <c r="U8" t="n">
-        <v>9.73</v>
+        <v>1.9866</v>
       </c>
       <c r="V8" t="n">
-        <v>-0.3409</v>
+        <v>5.1546</v>
       </c>
       <c r="W8" t="n">
-        <v>-10.8073</v>
+        <v>6.1191</v>
       </c>
       <c r="X8" t="n">
-        <v>-24.3521</v>
+        <v>-5.0318</v>
       </c>
       <c r="Y8" t="n">
-        <v>-12.6536</v>
+        <v>-20.4053</v>
       </c>
       <c r="Z8" t="n">
-        <v>-4.4221</v>
+        <v>-30.9945</v>
       </c>
       <c r="AA8" t="n">
-        <v>-9.767799999999999</v>
+        <v>-1.9349</v>
       </c>
       <c r="AB8" t="n">
-        <v>-1.0421</v>
+        <v>-6.1635</v>
       </c>
       <c r="AC8" t="n">
-        <v>8.1305</v>
+        <v>-7.2932</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>222.22</v>
+        <v>265.99</v>
       </c>
       <c r="C9" t="n">
-        <v>242.4</v>
+        <v>274.88</v>
       </c>
       <c r="D9" t="n">
-        <v>214.74</v>
+        <v>261.6</v>
       </c>
       <c r="E9" t="n">
-        <v>234.68</v>
+        <v>272.5</v>
       </c>
       <c r="F9" t="n">
-        <v>76.34</v>
+        <v>82.88</v>
       </c>
       <c r="G9" t="n">
-        <v>78.36</v>
+        <v>85.03</v>
       </c>
       <c r="H9" t="n">
-        <v>74.29000000000001</v>
+        <v>82.64</v>
       </c>
       <c r="I9" t="n">
-        <v>77.52</v>
+        <v>84.59</v>
       </c>
       <c r="J9" t="n">
-        <v>4.9523</v>
+        <v>4.0231</v>
       </c>
       <c r="K9" t="n">
-        <v>5.0907</v>
+        <v>4.122</v>
       </c>
       <c r="L9" t="n">
-        <v>4.4877</v>
+        <v>3.865</v>
       </c>
       <c r="M9" t="n">
-        <v>4.6656</v>
+        <v>3.9045</v>
       </c>
       <c r="N9" t="n">
-        <v>40.0106</v>
+        <v>36.6641</v>
       </c>
       <c r="O9" t="n">
-        <v>41.0933</v>
+        <v>36.7723</v>
       </c>
       <c r="P9" t="n">
-        <v>38.9476</v>
+        <v>35.5814</v>
       </c>
       <c r="Q9" t="n">
-        <v>39.4102</v>
+        <v>35.7389</v>
       </c>
       <c r="R9" t="n">
-        <v>4.7725</v>
+        <v>16.1156</v>
       </c>
       <c r="S9" t="n">
-        <v>16.3626</v>
+        <v>50.8442</v>
       </c>
       <c r="T9" t="n">
-        <v>28.5636</v>
+        <v>28.8782</v>
       </c>
       <c r="U9" t="n">
-        <v>1.9866</v>
+        <v>9.120200000000001</v>
       </c>
       <c r="V9" t="n">
-        <v>5.1546</v>
+        <v>22.1164</v>
       </c>
       <c r="W9" t="n">
-        <v>6.1191</v>
+        <v>10.9086</v>
       </c>
       <c r="X9" t="n">
-        <v>-5.0318</v>
+        <v>-16.313</v>
       </c>
       <c r="Y9" t="n">
-        <v>-20.4053</v>
+        <v>-39.878</v>
       </c>
       <c r="Z9" t="n">
-        <v>-30.9945</v>
+        <v>-30.5805</v>
       </c>
       <c r="AA9" t="n">
-        <v>-1.9349</v>
+        <v>-9.3156</v>
       </c>
       <c r="AB9" t="n">
-        <v>-6.1635</v>
+        <v>-19.7567</v>
       </c>
       <c r="AC9" t="n">
-        <v>-7.2932</v>
+        <v>-11.997</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>265.99</v>
+        <v>267.13</v>
       </c>
       <c r="C10" t="n">
-        <v>274.88</v>
+        <v>274.93</v>
       </c>
       <c r="D10" t="n">
-        <v>261.6</v>
+        <v>226</v>
       </c>
       <c r="E10" t="n">
-        <v>272.5</v>
+        <v>226.19</v>
       </c>
       <c r="F10" t="n">
-        <v>82.88</v>
+        <v>84.19</v>
       </c>
       <c r="G10" t="n">
-        <v>85.03</v>
+        <v>84.83</v>
       </c>
       <c r="H10" t="n">
-        <v>82.64</v>
+        <v>79.86</v>
       </c>
       <c r="I10" t="n">
-        <v>84.59</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>4.0231</v>
+        <v>3.9836</v>
       </c>
       <c r="K10" t="n">
-        <v>4.122</v>
+        <v>4.5965</v>
       </c>
       <c r="L10" t="n">
         <v>3.865</v>
       </c>
       <c r="M10" t="n">
-        <v>3.9045</v>
+        <v>4.5767</v>
       </c>
       <c r="N10" t="n">
-        <v>36.6641</v>
+        <v>35.9652</v>
       </c>
       <c r="O10" t="n">
-        <v>36.7723</v>
+        <v>37.7861</v>
       </c>
       <c r="P10" t="n">
-        <v>35.5814</v>
+        <v>35.6896</v>
       </c>
       <c r="Q10" t="n">
-        <v>35.7389</v>
+        <v>37.7468</v>
       </c>
       <c r="R10" t="n">
-        <v>16.1156</v>
+        <v>-16.9945</v>
       </c>
       <c r="S10" t="n">
-        <v>50.8442</v>
+        <v>0.9822</v>
       </c>
       <c r="T10" t="n">
-        <v>28.8782</v>
+        <v>12.1529</v>
       </c>
       <c r="U10" t="n">
-        <v>9.120200000000001</v>
+        <v>-5.5089</v>
       </c>
       <c r="V10" t="n">
-        <v>22.1164</v>
+        <v>5.1572</v>
       </c>
       <c r="W10" t="n">
-        <v>10.9086</v>
+        <v>8.4238</v>
       </c>
       <c r="X10" t="n">
-        <v>-16.313</v>
+        <v>17.216</v>
       </c>
       <c r="Y10" t="n">
-        <v>-39.878</v>
+        <v>-6.8413</v>
       </c>
       <c r="Z10" t="n">
-        <v>-30.5805</v>
+        <v>-21.922</v>
       </c>
       <c r="AA10" t="n">
-        <v>-9.3156</v>
+        <v>5.6182</v>
       </c>
       <c r="AB10" t="n">
-        <v>-19.7567</v>
+        <v>-6.074</v>
       </c>
       <c r="AC10" t="n">
-        <v>-11.997</v>
+        <v>-10.1241</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>267.13</v>
+        <v>247.42</v>
       </c>
       <c r="C11" t="n">
-        <v>274.93</v>
+        <v>259.79</v>
       </c>
       <c r="D11" t="n">
-        <v>226</v>
+        <v>233.3</v>
       </c>
       <c r="E11" t="n">
-        <v>226.19</v>
+        <v>233.86</v>
       </c>
       <c r="F11" t="n">
-        <v>84.19</v>
+        <v>81.67</v>
       </c>
       <c r="G11" t="n">
-        <v>84.83</v>
+        <v>81.81</v>
       </c>
       <c r="H11" t="n">
-        <v>79.86</v>
+        <v>76.94</v>
       </c>
       <c r="I11" t="n">
-        <v>79.93000000000001</v>
+        <v>77.54000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>3.9836</v>
+        <v>4.122</v>
       </c>
       <c r="K11" t="n">
-        <v>4.5965</v>
+        <v>4.4086</v>
       </c>
       <c r="L11" t="n">
-        <v>3.865</v>
+        <v>3.8749</v>
       </c>
       <c r="M11" t="n">
-        <v>4.5767</v>
+        <v>4.4086</v>
       </c>
       <c r="N11" t="n">
-        <v>35.9652</v>
+        <v>36.9397</v>
       </c>
       <c r="O11" t="n">
-        <v>37.7861</v>
+        <v>39.1641</v>
       </c>
       <c r="P11" t="n">
-        <v>35.6896</v>
+        <v>36.8708</v>
       </c>
       <c r="Q11" t="n">
-        <v>37.7468</v>
+        <v>38.8984</v>
       </c>
       <c r="R11" t="n">
-        <v>-16.9945</v>
+        <v>3.391</v>
       </c>
       <c r="S11" t="n">
-        <v>0.9822</v>
+        <v>-0.3494</v>
       </c>
       <c r="T11" t="n">
-        <v>12.1529</v>
+        <v>29.4547</v>
       </c>
       <c r="U11" t="n">
-        <v>-5.5089</v>
+        <v>-2.9901</v>
       </c>
       <c r="V11" t="n">
-        <v>5.1572</v>
+        <v>0.0258</v>
       </c>
       <c r="W11" t="n">
-        <v>8.4238</v>
+        <v>11.9388</v>
       </c>
       <c r="X11" t="n">
-        <v>17.216</v>
+        <v>-3.673</v>
       </c>
       <c r="Y11" t="n">
-        <v>-6.8413</v>
+        <v>-5.5084</v>
       </c>
       <c r="Z11" t="n">
-        <v>-21.922</v>
+        <v>-32.1159</v>
       </c>
       <c r="AA11" t="n">
-        <v>5.6182</v>
+        <v>3.0509</v>
       </c>
       <c r="AB11" t="n">
-        <v>-6.074</v>
+        <v>-1.2986</v>
       </c>
       <c r="AC11" t="n">
-        <v>-10.1241</v>
+        <v>-12.6628</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>247.42</v>
+        <v>266.04</v>
       </c>
       <c r="C12" t="n">
-        <v>259.79</v>
+        <v>286.15</v>
       </c>
       <c r="D12" t="n">
-        <v>233.3</v>
+        <v>265</v>
       </c>
       <c r="E12" t="n">
-        <v>233.86</v>
+        <v>279.29</v>
       </c>
       <c r="F12" t="n">
-        <v>81.67</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="G12" t="n">
-        <v>81.81</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>76.94</v>
+        <v>80.63</v>
       </c>
       <c r="I12" t="n">
-        <v>77.54000000000001</v>
+        <v>82.87</v>
       </c>
       <c r="J12" t="n">
-        <v>4.122</v>
+        <v>3.8156</v>
       </c>
       <c r="K12" t="n">
-        <v>4.4086</v>
+        <v>3.8254</v>
       </c>
       <c r="L12" t="n">
-        <v>3.8749</v>
+        <v>3.4103</v>
       </c>
       <c r="M12" t="n">
-        <v>4.4086</v>
+        <v>3.5487</v>
       </c>
       <c r="N12" t="n">
-        <v>36.9397</v>
+        <v>36.6149</v>
       </c>
       <c r="O12" t="n">
-        <v>39.1641</v>
+        <v>37.3531</v>
       </c>
       <c r="P12" t="n">
-        <v>36.8708</v>
+        <v>35.857</v>
       </c>
       <c r="Q12" t="n">
-        <v>38.8984</v>
+        <v>36.1719</v>
       </c>
       <c r="R12" t="n">
-        <v>3.391</v>
+        <v>19.4262</v>
       </c>
       <c r="S12" t="n">
-        <v>-0.3494</v>
+        <v>2.4917</v>
       </c>
       <c r="T12" t="n">
-        <v>29.4547</v>
+        <v>24.6886</v>
       </c>
       <c r="U12" t="n">
-        <v>-2.9901</v>
+        <v>6.8739</v>
       </c>
       <c r="V12" t="n">
-        <v>0.0258</v>
+        <v>-2.0333</v>
       </c>
       <c r="W12" t="n">
-        <v>11.9388</v>
+        <v>9.0251</v>
       </c>
       <c r="X12" t="n">
-        <v>-3.673</v>
+        <v>-19.5051</v>
       </c>
       <c r="Y12" t="n">
-        <v>-5.5084</v>
+        <v>-9.1126</v>
       </c>
       <c r="Z12" t="n">
-        <v>-32.1159</v>
+        <v>-27.7662</v>
       </c>
       <c r="AA12" t="n">
-        <v>3.0509</v>
+        <v>-7.0093</v>
       </c>
       <c r="AB12" t="n">
-        <v>-1.2986</v>
+        <v>1.2116</v>
       </c>
       <c r="AC12" t="n">
-        <v>-12.6628</v>
+        <v>-9.992800000000001</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>266.04</v>
+        <v>299.26</v>
       </c>
       <c r="C13" t="n">
-        <v>286.15</v>
+        <v>302</v>
       </c>
       <c r="D13" t="n">
-        <v>265</v>
+        <v>286.24</v>
       </c>
       <c r="E13" t="n">
-        <v>279.29</v>
+        <v>300.77</v>
       </c>
       <c r="F13" t="n">
-        <v>82.09999999999999</v>
+        <v>83.95</v>
       </c>
       <c r="G13" t="n">
-        <v>83.59999999999999</v>
+        <v>85.11</v>
       </c>
       <c r="H13" t="n">
-        <v>80.63</v>
+        <v>81.39</v>
       </c>
       <c r="I13" t="n">
-        <v>82.87</v>
+        <v>82.58</v>
       </c>
       <c r="J13" t="n">
-        <v>3.8156</v>
+        <v>3.2917</v>
       </c>
       <c r="K13" t="n">
-        <v>3.8254</v>
+        <v>3.4498</v>
       </c>
       <c r="L13" t="n">
-        <v>3.4103</v>
+        <v>3.2521</v>
       </c>
       <c r="M13" t="n">
-        <v>3.5487</v>
+        <v>3.262</v>
       </c>
       <c r="N13" t="n">
-        <v>36.6149</v>
+        <v>35.7389</v>
       </c>
       <c r="O13" t="n">
-        <v>37.3531</v>
+        <v>36.8511</v>
       </c>
       <c r="P13" t="n">
-        <v>35.857</v>
+        <v>35.2369</v>
       </c>
       <c r="Q13" t="n">
-        <v>36.1719</v>
+        <v>36.3491</v>
       </c>
       <c r="R13" t="n">
-        <v>19.4262</v>
+        <v>7.6909</v>
       </c>
       <c r="S13" t="n">
-        <v>2.4917</v>
+        <v>32.9723</v>
       </c>
       <c r="T13" t="n">
-        <v>24.6886</v>
+        <v>28.1618</v>
       </c>
       <c r="U13" t="n">
-        <v>6.8739</v>
+        <v>-0.3499</v>
       </c>
       <c r="V13" t="n">
-        <v>-2.0333</v>
+        <v>3.3154</v>
       </c>
       <c r="W13" t="n">
-        <v>9.0251</v>
+        <v>6.5273</v>
       </c>
       <c r="X13" t="n">
-        <v>-19.5051</v>
+        <v>-8.079000000000001</v>
       </c>
       <c r="Y13" t="n">
-        <v>-9.1126</v>
+        <v>-28.7259</v>
       </c>
       <c r="Z13" t="n">
-        <v>-27.7662</v>
+        <v>-30.084</v>
       </c>
       <c r="AA13" t="n">
-        <v>-7.0093</v>
+        <v>0.4899</v>
       </c>
       <c r="AB13" t="n">
-        <v>1.2116</v>
+        <v>-3.7028</v>
       </c>
       <c r="AC13" t="n">
-        <v>-9.992800000000001</v>
+        <v>-7.7673</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>299.26</v>
+        <v>236</v>
       </c>
       <c r="C14" t="n">
-        <v>302</v>
+        <v>252.98</v>
       </c>
       <c r="D14" t="n">
-        <v>286.24</v>
+        <v>223</v>
       </c>
       <c r="E14" t="n">
-        <v>300.77</v>
+        <v>231.42</v>
       </c>
       <c r="F14" t="n">
-        <v>83.95</v>
+        <v>75.12</v>
       </c>
       <c r="G14" t="n">
-        <v>85.11</v>
+        <v>77.73999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>81.39</v>
+        <v>73.91</v>
       </c>
       <c r="I14" t="n">
-        <v>82.58</v>
+        <v>74.44</v>
       </c>
       <c r="J14" t="n">
-        <v>3.2917</v>
+        <v>3.99</v>
       </c>
       <c r="K14" t="n">
-        <v>3.4498</v>
+        <v>4.13</v>
       </c>
       <c r="L14" t="n">
-        <v>3.2521</v>
+        <v>3.8</v>
       </c>
       <c r="M14" t="n">
-        <v>3.262</v>
+        <v>4.04</v>
       </c>
       <c r="N14" t="n">
-        <v>35.7389</v>
+        <v>39.6267</v>
       </c>
       <c r="O14" t="n">
-        <v>36.8511</v>
+        <v>40.1582</v>
       </c>
       <c r="P14" t="n">
-        <v>35.2369</v>
+        <v>38.4653</v>
       </c>
       <c r="Q14" t="n">
-        <v>36.3491</v>
+        <v>39.922</v>
       </c>
       <c r="R14" t="n">
-        <v>7.6909</v>
+        <v>-23.0575</v>
       </c>
       <c r="S14" t="n">
-        <v>32.9723</v>
+        <v>-1.0434</v>
       </c>
       <c r="T14" t="n">
-        <v>28.1618</v>
+        <v>-15.0752</v>
       </c>
       <c r="U14" t="n">
-        <v>-0.3499</v>
+        <v>-9.857100000000001</v>
       </c>
       <c r="V14" t="n">
-        <v>3.3154</v>
+        <v>-3.9979</v>
       </c>
       <c r="W14" t="n">
-        <v>6.5273</v>
+        <v>-11.9991</v>
       </c>
       <c r="X14" t="n">
-        <v>-8.079000000000001</v>
+        <v>23.8504</v>
       </c>
       <c r="Y14" t="n">
-        <v>-28.7259</v>
+        <v>-8.360900000000001</v>
       </c>
       <c r="Z14" t="n">
-        <v>-30.084</v>
+        <v>3.4704</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.4899</v>
+        <v>9.8294</v>
       </c>
       <c r="AB14" t="n">
-        <v>-3.7028</v>
+        <v>2.6315</v>
       </c>
       <c r="AC14" t="n">
-        <v>-7.7673</v>
+        <v>11.7046</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>236</v>
+        <v>233.11</v>
       </c>
       <c r="C15" t="n">
-        <v>252.98</v>
+        <v>237</v>
       </c>
       <c r="D15" t="n">
-        <v>223</v>
+        <v>211.13</v>
       </c>
       <c r="E15" t="n">
-        <v>231.42</v>
+        <v>229.57</v>
       </c>
       <c r="F15" t="n">
-        <v>75.12</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>77.73999999999999</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="H15" t="n">
-        <v>73.91</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="I15" t="n">
-        <v>74.44</v>
+        <v>73.3</v>
       </c>
       <c r="J15" t="n">
-        <v>3.99</v>
+        <v>4</v>
       </c>
       <c r="K15" t="n">
-        <v>4.13</v>
+        <v>4.39</v>
       </c>
       <c r="L15" t="n">
-        <v>3.8</v>
+        <v>3.92</v>
       </c>
       <c r="M15" t="n">
-        <v>4.04</v>
+        <v>4.08</v>
       </c>
       <c r="N15" t="n">
-        <v>39.6267</v>
+        <v>39.66</v>
       </c>
       <c r="O15" t="n">
-        <v>40.1582</v>
+        <v>41.49</v>
       </c>
       <c r="P15" t="n">
-        <v>38.4653</v>
+        <v>38.9</v>
       </c>
       <c r="Q15" t="n">
-        <v>39.922</v>
+        <v>40.45</v>
       </c>
       <c r="R15" t="n">
-        <v>-23.0575</v>
+        <v>-0.7994</v>
       </c>
       <c r="S15" t="n">
-        <v>-1.0434</v>
+        <v>-17.8023</v>
       </c>
       <c r="T15" t="n">
-        <v>-15.0752</v>
+        <v>1.4943</v>
       </c>
       <c r="U15" t="n">
-        <v>-9.857100000000001</v>
+        <v>-1.5314</v>
       </c>
       <c r="V15" t="n">
-        <v>-3.9979</v>
+        <v>-11.5482</v>
       </c>
       <c r="W15" t="n">
-        <v>-11.9991</v>
+        <v>-8.2948</v>
       </c>
       <c r="X15" t="n">
-        <v>23.8504</v>
+        <v>0.9901</v>
       </c>
       <c r="Y15" t="n">
-        <v>-8.360900000000001</v>
+        <v>14.9717</v>
       </c>
       <c r="Z15" t="n">
-        <v>3.4704</v>
+        <v>-10.8528</v>
       </c>
       <c r="AA15" t="n">
-        <v>9.8294</v>
+        <v>1.3226</v>
       </c>
       <c r="AB15" t="n">
-        <v>2.6315</v>
+        <v>11.8271</v>
       </c>
       <c r="AC15" t="n">
-        <v>11.7046</v>
+        <v>7.1614</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>233.11</v>
+        <v>268.05</v>
       </c>
       <c r="C16" t="n">
-        <v>237</v>
+        <v>268.4</v>
       </c>
       <c r="D16" t="n">
-        <v>211.13</v>
+        <v>225.74</v>
       </c>
       <c r="E16" t="n">
-        <v>229.57</v>
+        <v>252.61</v>
       </c>
       <c r="F16" t="n">
-        <v>74.79000000000001</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>76.18000000000001</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>71.34999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I16" t="n">
-        <v>73.3</v>
+        <v>74.95</v>
       </c>
       <c r="J16" t="n">
-        <v>4</v>
+        <v>3.38</v>
       </c>
       <c r="K16" t="n">
-        <v>4.39</v>
+        <v>4.15</v>
       </c>
       <c r="L16" t="n">
-        <v>3.92</v>
+        <v>3.37</v>
       </c>
       <c r="M16" t="n">
-        <v>4.08</v>
+        <v>3.63</v>
       </c>
       <c r="N16" t="n">
-        <v>39.66</v>
+        <v>37.87</v>
       </c>
       <c r="O16" t="n">
-        <v>41.49</v>
+        <v>41.37</v>
       </c>
       <c r="P16" t="n">
-        <v>38.9</v>
+        <v>37.71</v>
       </c>
       <c r="Q16" t="n">
-        <v>40.45</v>
+        <v>39.47</v>
       </c>
       <c r="R16" t="n">
-        <v>-0.7994</v>
+        <v>10.0362</v>
       </c>
       <c r="S16" t="n">
-        <v>-17.8023</v>
+        <v>-16.0122</v>
       </c>
       <c r="T16" t="n">
-        <v>1.4943</v>
+        <v>8.0176</v>
       </c>
       <c r="U16" t="n">
-        <v>-1.5314</v>
+        <v>2.251</v>
       </c>
       <c r="V16" t="n">
-        <v>-11.5482</v>
+        <v>-9.2395</v>
       </c>
       <c r="W16" t="n">
-        <v>-8.2948</v>
+        <v>-3.3402</v>
       </c>
       <c r="X16" t="n">
-        <v>0.9901</v>
+        <v>-11.0294</v>
       </c>
       <c r="Y16" t="n">
-        <v>14.9717</v>
+        <v>11.2814</v>
       </c>
       <c r="Z16" t="n">
-        <v>-10.8528</v>
+        <v>-17.6609</v>
       </c>
       <c r="AA16" t="n">
-        <v>1.3226</v>
+        <v>-2.4227</v>
       </c>
       <c r="AB16" t="n">
-        <v>11.8271</v>
+        <v>8.585900000000001</v>
       </c>
       <c r="AC16" t="n">
-        <v>7.1614</v>
+        <v>1.4695</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>268.05</v>
+        <v>226.24</v>
       </c>
       <c r="C17" t="n">
-        <v>268.4</v>
+        <v>231.25</v>
       </c>
       <c r="D17" t="n">
-        <v>225.74</v>
+        <v>212.1</v>
       </c>
       <c r="E17" t="n">
-        <v>252.61</v>
+        <v>215.6</v>
       </c>
       <c r="F17" t="n">
-        <v>77.95999999999999</v>
+        <v>72.09</v>
       </c>
       <c r="G17" t="n">
-        <v>78.23999999999999</v>
+        <v>74.69</v>
       </c>
       <c r="H17" t="n">
-        <v>71.59999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="I17" t="n">
-        <v>74.95</v>
+        <v>71.83</v>
       </c>
       <c r="J17" t="n">
-        <v>3.38</v>
+        <v>4.04</v>
       </c>
       <c r="K17" t="n">
-        <v>4.15</v>
+        <v>4.25</v>
       </c>
       <c r="L17" t="n">
-        <v>3.37</v>
+        <v>3.95</v>
       </c>
       <c r="M17" t="n">
-        <v>3.63</v>
+        <v>4.24</v>
       </c>
       <c r="N17" t="n">
-        <v>37.87</v>
+        <v>41.08</v>
       </c>
       <c r="O17" t="n">
-        <v>41.37</v>
+        <v>41.79</v>
       </c>
       <c r="P17" t="n">
-        <v>37.71</v>
+        <v>39.69</v>
       </c>
       <c r="Q17" t="n">
-        <v>39.47</v>
+        <v>41.31</v>
       </c>
       <c r="R17" t="n">
-        <v>10.0362</v>
+        <v>-14.651</v>
       </c>
       <c r="S17" t="n">
-        <v>-16.0122</v>
+        <v>-6.8361</v>
       </c>
       <c r="T17" t="n">
-        <v>8.0176</v>
+        <v>-22.8043</v>
       </c>
       <c r="U17" t="n">
-        <v>2.251</v>
+        <v>-4.1628</v>
       </c>
       <c r="V17" t="n">
-        <v>-9.2395</v>
+        <v>-3.5062</v>
       </c>
       <c r="W17" t="n">
-        <v>-3.3402</v>
+        <v>-13.3221</v>
       </c>
       <c r="X17" t="n">
-        <v>-11.0294</v>
+        <v>16.8044</v>
       </c>
       <c r="Y17" t="n">
-        <v>11.2814</v>
+        <v>4.9505</v>
       </c>
       <c r="Z17" t="n">
-        <v>-17.6609</v>
+        <v>19.4804</v>
       </c>
       <c r="AA17" t="n">
-        <v>-2.4227</v>
+        <v>4.6618</v>
       </c>
       <c r="AB17" t="n">
-        <v>8.585900000000001</v>
+        <v>3.4768</v>
       </c>
       <c r="AC17" t="n">
-        <v>1.4695</v>
+        <v>14.2047</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>226.24</v>
+        <v>216.36</v>
       </c>
       <c r="C18" t="n">
-        <v>231.25</v>
+        <v>238.65</v>
       </c>
       <c r="D18" t="n">
-        <v>212.1</v>
+        <v>192.3</v>
       </c>
       <c r="E18" t="n">
-        <v>215.6</v>
+        <v>236.52</v>
       </c>
       <c r="F18" t="n">
-        <v>72.09</v>
+        <v>74.12</v>
       </c>
       <c r="G18" t="n">
-        <v>74.69</v>
+        <v>77.38</v>
       </c>
       <c r="H18" t="n">
-        <v>70.72</v>
+        <v>71.45</v>
       </c>
       <c r="I18" t="n">
-        <v>71.83</v>
+        <v>77.19</v>
       </c>
       <c r="J18" t="n">
-        <v>4.04</v>
+        <v>4.16</v>
       </c>
       <c r="K18" t="n">
-        <v>4.25</v>
+        <v>4.63</v>
       </c>
       <c r="L18" t="n">
-        <v>3.95</v>
+        <v>3.7</v>
       </c>
       <c r="M18" t="n">
-        <v>4.24</v>
+        <v>3.72</v>
       </c>
       <c r="N18" t="n">
-        <v>41.08</v>
+        <v>39.91</v>
       </c>
       <c r="O18" t="n">
-        <v>41.79</v>
+        <v>41.43</v>
       </c>
       <c r="P18" t="n">
-        <v>39.69</v>
+        <v>38.08</v>
       </c>
       <c r="Q18" t="n">
-        <v>41.31</v>
+        <v>38.16</v>
       </c>
       <c r="R18" t="n">
-        <v>-14.651</v>
+        <v>9.703200000000001</v>
       </c>
       <c r="S18" t="n">
-        <v>-6.8361</v>
+        <v>3.0274</v>
       </c>
       <c r="T18" t="n">
-        <v>-22.8043</v>
+        <v>-21.3618</v>
       </c>
       <c r="U18" t="n">
-        <v>-4.1628</v>
+        <v>7.4621</v>
       </c>
       <c r="V18" t="n">
-        <v>-3.5062</v>
+        <v>5.307</v>
       </c>
       <c r="W18" t="n">
-        <v>-13.3221</v>
+        <v>-6.527</v>
       </c>
       <c r="X18" t="n">
-        <v>16.8044</v>
+        <v>-12.2642</v>
       </c>
       <c r="Y18" t="n">
-        <v>4.9505</v>
+        <v>-8.823499999999999</v>
       </c>
       <c r="Z18" t="n">
-        <v>19.4804</v>
+        <v>14.0405</v>
       </c>
       <c r="AA18" t="n">
-        <v>4.6618</v>
+        <v>-7.6253</v>
       </c>
       <c r="AB18" t="n">
-        <v>3.4768</v>
+        <v>-5.6613</v>
       </c>
       <c r="AC18" t="n">
-        <v>14.2047</v>
+        <v>4.982</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>216.36</v>
+        <v>241.45</v>
       </c>
       <c r="C19" t="n">
-        <v>238.65</v>
+        <v>272</v>
       </c>
       <c r="D19" t="n">
-        <v>192.3</v>
+        <v>240.59</v>
       </c>
       <c r="E19" t="n">
-        <v>236.52</v>
+        <v>266.71</v>
       </c>
       <c r="F19" t="n">
-        <v>74.12</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="G19" t="n">
-        <v>77.38</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>71.45</v>
+        <v>77.15000000000001</v>
       </c>
       <c r="I19" t="n">
-        <v>77.19</v>
+        <v>81</v>
       </c>
       <c r="J19" t="n">
-        <v>4.16</v>
+        <v>3.66</v>
       </c>
       <c r="K19" t="n">
-        <v>4.63</v>
+        <v>3.68</v>
       </c>
       <c r="L19" t="n">
-        <v>3.7</v>
+        <v>3.17</v>
       </c>
       <c r="M19" t="n">
-        <v>3.72</v>
+        <v>3.24</v>
       </c>
       <c r="N19" t="n">
-        <v>39.91</v>
+        <v>38.16</v>
       </c>
       <c r="O19" t="n">
-        <v>41.43</v>
+        <v>38.2</v>
       </c>
       <c r="P19" t="n">
-        <v>38.08</v>
+        <v>36.03</v>
       </c>
       <c r="Q19" t="n">
-        <v>38.16</v>
+        <v>36.31</v>
       </c>
       <c r="R19" t="n">
-        <v>9.703200000000001</v>
+        <v>12.7642</v>
       </c>
       <c r="S19" t="n">
-        <v>3.0274</v>
+        <v>5.5817</v>
       </c>
       <c r="T19" t="n">
-        <v>-21.3618</v>
+        <v>15.2493</v>
       </c>
       <c r="U19" t="n">
-        <v>7.4621</v>
+        <v>4.9359</v>
       </c>
       <c r="V19" t="n">
-        <v>5.307</v>
+        <v>8.071999999999999</v>
       </c>
       <c r="W19" t="n">
-        <v>-6.527</v>
+        <v>8.8125</v>
       </c>
       <c r="X19" t="n">
-        <v>-12.2642</v>
+        <v>-12.9032</v>
       </c>
       <c r="Y19" t="n">
-        <v>-8.823499999999999</v>
+        <v>-10.7438</v>
       </c>
       <c r="Z19" t="n">
-        <v>14.0405</v>
+        <v>-19.802</v>
       </c>
       <c r="AA19" t="n">
-        <v>-7.6253</v>
+        <v>-4.848</v>
       </c>
       <c r="AB19" t="n">
-        <v>-5.6613</v>
+        <v>-8.0061</v>
       </c>
       <c r="AC19" t="n">
-        <v>4.982</v>
+        <v>-9.047599999999999</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>241.45</v>
+        <v>237.79</v>
       </c>
       <c r="C20" t="n">
-        <v>272</v>
+        <v>246.47</v>
       </c>
       <c r="D20" t="n">
-        <v>240.59</v>
+        <v>215.38</v>
       </c>
       <c r="E20" t="n">
-        <v>266.71</v>
+        <v>217.55</v>
       </c>
       <c r="F20" t="n">
-        <v>77.23999999999999</v>
+        <v>78.72</v>
       </c>
       <c r="G20" t="n">
-        <v>81.54000000000001</v>
+        <v>79.64</v>
       </c>
       <c r="H20" t="n">
-        <v>77.15000000000001</v>
+        <v>77.23</v>
       </c>
       <c r="I20" t="n">
-        <v>81</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J20" t="n">
-        <v>3.66</v>
+        <v>3.59</v>
       </c>
       <c r="K20" t="n">
-        <v>3.68</v>
+        <v>3.89</v>
       </c>
       <c r="L20" t="n">
-        <v>3.17</v>
+        <v>3.51</v>
       </c>
       <c r="M20" t="n">
-        <v>3.24</v>
+        <v>3.86</v>
       </c>
       <c r="N20" t="n">
-        <v>38.16</v>
+        <v>37.31</v>
       </c>
       <c r="O20" t="n">
-        <v>38.2</v>
+        <v>37.98</v>
       </c>
       <c r="P20" t="n">
-        <v>36.03</v>
+        <v>36.9</v>
       </c>
       <c r="Q20" t="n">
-        <v>36.31</v>
+        <v>37.88</v>
       </c>
       <c r="R20" t="n">
-        <v>12.7642</v>
+        <v>-18.432</v>
       </c>
       <c r="S20" t="n">
-        <v>5.5817</v>
+        <v>0.9045</v>
       </c>
       <c r="T20" t="n">
-        <v>15.2493</v>
+        <v>-5.2359</v>
       </c>
       <c r="U20" t="n">
-        <v>4.9359</v>
+        <v>-4.3704</v>
       </c>
       <c r="V20" t="n">
-        <v>8.071999999999999</v>
+        <v>7.838</v>
       </c>
       <c r="W20" t="n">
-        <v>8.8125</v>
+        <v>5.6753</v>
       </c>
       <c r="X20" t="n">
-        <v>-12.9032</v>
+        <v>19.1358</v>
       </c>
       <c r="Y20" t="n">
-        <v>-10.7438</v>
+        <v>-8.962300000000001</v>
       </c>
       <c r="Z20" t="n">
-        <v>-19.802</v>
+        <v>-5.3922</v>
       </c>
       <c r="AA20" t="n">
-        <v>-4.848</v>
+        <v>4.3239</v>
       </c>
       <c r="AB20" t="n">
-        <v>-8.0061</v>
+        <v>-8.303100000000001</v>
       </c>
       <c r="AC20" t="n">
-        <v>-9.047599999999999</v>
+        <v>-6.3535</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>237.79</v>
+        <v>219.23</v>
       </c>
       <c r="C21" t="n">
-        <v>246.47</v>
+        <v>226.13</v>
       </c>
       <c r="D21" t="n">
-        <v>215.38</v>
+        <v>168.88</v>
       </c>
       <c r="E21" t="n">
-        <v>217.55</v>
+        <v>181.47</v>
       </c>
       <c r="F21" t="n">
-        <v>78.72</v>
+        <v>77.45</v>
       </c>
       <c r="G21" t="n">
-        <v>79.64</v>
+        <v>79.14</v>
       </c>
       <c r="H21" t="n">
-        <v>77.23</v>
+        <v>71.72</v>
       </c>
       <c r="I21" t="n">
-        <v>77.45999999999999</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="J21" t="n">
-        <v>3.59</v>
+        <v>3.84</v>
       </c>
       <c r="K21" t="n">
-        <v>3.89</v>
+        <v>4.74</v>
       </c>
       <c r="L21" t="n">
-        <v>3.51</v>
+        <v>3.71</v>
       </c>
       <c r="M21" t="n">
-        <v>3.86</v>
+        <v>4.51</v>
       </c>
       <c r="N21" t="n">
-        <v>37.31</v>
+        <v>37.91</v>
       </c>
       <c r="O21" t="n">
-        <v>37.98</v>
+        <v>40.72</v>
       </c>
       <c r="P21" t="n">
-        <v>36.9</v>
+        <v>37.08</v>
       </c>
       <c r="Q21" t="n">
-        <v>37.88</v>
+        <v>39.95</v>
       </c>
       <c r="R21" t="n">
-        <v>-18.432</v>
+        <v>-16.5847</v>
       </c>
       <c r="S21" t="n">
-        <v>0.9045</v>
+        <v>-23.275</v>
       </c>
       <c r="T21" t="n">
-        <v>-5.2359</v>
+        <v>-28.162</v>
       </c>
       <c r="U21" t="n">
-        <v>-4.3704</v>
+        <v>-5.306</v>
       </c>
       <c r="V21" t="n">
-        <v>7.838</v>
+        <v>-4.9747</v>
       </c>
       <c r="W21" t="n">
-        <v>5.6753</v>
+        <v>-2.1348</v>
       </c>
       <c r="X21" t="n">
-        <v>19.1358</v>
+        <v>16.8394</v>
       </c>
       <c r="Y21" t="n">
-        <v>-8.962300000000001</v>
+        <v>21.2366</v>
       </c>
       <c r="Z21" t="n">
-        <v>-5.3922</v>
+        <v>24.2424</v>
       </c>
       <c r="AA21" t="n">
-        <v>4.3239</v>
+        <v>5.4646</v>
       </c>
       <c r="AB21" t="n">
-        <v>-8.303100000000001</v>
+        <v>4.6908</v>
       </c>
       <c r="AC21" t="n">
-        <v>-6.3535</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>219.23</v>
-      </c>
-      <c r="C22" t="n">
-        <v>226.13</v>
-      </c>
-      <c r="D22" t="n">
-        <v>168.88</v>
-      </c>
-      <c r="E22" t="n">
-        <v>181.47</v>
-      </c>
-      <c r="F22" t="n">
-        <v>77.47</v>
-      </c>
-      <c r="G22" t="n">
-        <v>79.13500000000001</v>
-      </c>
-      <c r="H22" t="n">
-        <v>71.72</v>
-      </c>
-      <c r="I22" t="n">
-        <v>73.34999999999999</v>
-      </c>
-      <c r="J22" t="n">
-        <v>3.84</v>
-      </c>
-      <c r="K22" t="n">
-        <v>4.74</v>
-      </c>
-      <c r="L22" t="n">
-        <v>3.71</v>
-      </c>
-      <c r="M22" t="n">
-        <v>4.51</v>
-      </c>
-      <c r="N22" t="n">
-        <v>37.91</v>
-      </c>
-      <c r="O22" t="n">
-        <v>40.72</v>
-      </c>
-      <c r="P22" t="n">
-        <v>37.08</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>39.95</v>
-      </c>
-      <c r="R22" t="n">
-        <v>-16.5847</v>
-      </c>
-      <c r="S22" t="n">
-        <v>-23.275</v>
-      </c>
-      <c r="T22" t="n">
-        <v>-28.162</v>
-      </c>
-      <c r="U22" t="n">
-        <v>-5.306</v>
-      </c>
-      <c r="V22" t="n">
-        <v>-4.9747</v>
-      </c>
-      <c r="W22" t="n">
-        <v>-2.1348</v>
-      </c>
-      <c r="X22" t="n">
-        <v>16.8394</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>21.2366</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>24.2424</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>5.4646</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>4.6908</v>
-      </c>
-      <c r="AC22" t="n">
         <v>1.2161</v>
       </c>
     </row>
@@ -2412,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-07-06 23:07
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC21"/>
+  <dimension ref="A1:AC20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1713 +568,1622 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>242.04</v>
+        <v>210.62</v>
       </c>
       <c r="C2" t="n">
-        <v>274.5</v>
+        <v>222.19</v>
       </c>
       <c r="D2" t="n">
-        <v>228.55</v>
+        <v>201.69</v>
       </c>
       <c r="E2" t="n">
-        <v>262.7</v>
+        <v>211.44</v>
       </c>
       <c r="F2" t="n">
-        <v>83.47</v>
+        <v>76.86</v>
       </c>
       <c r="G2" t="n">
-        <v>86.25</v>
+        <v>78.47</v>
       </c>
       <c r="H2" t="n">
-        <v>82.48</v>
+        <v>75.38</v>
       </c>
       <c r="I2" t="n">
-        <v>85.22</v>
+        <v>76.27</v>
       </c>
       <c r="J2" t="n">
-        <v>5.5059</v>
+        <v>5.6442</v>
       </c>
       <c r="K2" t="n">
-        <v>5.7431</v>
+        <v>5.9803</v>
       </c>
       <c r="L2" t="n">
-        <v>4.9424</v>
+        <v>5.2093</v>
       </c>
       <c r="M2" t="n">
-        <v>5.1401</v>
+        <v>5.6245</v>
       </c>
       <c r="N2" t="n">
-        <v>37.9239</v>
+        <v>40.2763</v>
       </c>
       <c r="O2" t="n">
-        <v>38.3472</v>
+        <v>41.1228</v>
       </c>
       <c r="P2" t="n">
-        <v>36.7428</v>
+        <v>39.3314</v>
       </c>
       <c r="Q2" t="n">
-        <v>37.166</v>
+        <v>40.611</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>230.85</v>
+        <v>227.06</v>
       </c>
       <c r="C3" t="n">
-        <v>233.69</v>
+        <v>231.02</v>
       </c>
       <c r="D3" t="n">
-        <v>181.81</v>
+        <v>157.56</v>
       </c>
       <c r="E3" t="n">
-        <v>182.54</v>
+        <v>201.68</v>
       </c>
       <c r="F3" t="n">
-        <v>81.56999999999999</v>
+        <v>78.48</v>
       </c>
       <c r="G3" t="n">
-        <v>82.08</v>
+        <v>79.34</v>
       </c>
       <c r="H3" t="n">
-        <v>72.68000000000001</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>73.05</v>
+        <v>73.72</v>
       </c>
       <c r="J3" t="n">
-        <v>5.7925</v>
+        <v>5.1895</v>
       </c>
       <c r="K3" t="n">
-        <v>6.7711</v>
+        <v>7.0281</v>
       </c>
       <c r="L3" t="n">
-        <v>5.7233</v>
+        <v>5.0808</v>
       </c>
       <c r="M3" t="n">
-        <v>6.7612</v>
+        <v>5.8617</v>
       </c>
       <c r="N3" t="n">
-        <v>38.7999</v>
+        <v>39.4299</v>
       </c>
       <c r="O3" t="n">
-        <v>42.6681</v>
+        <v>45.6505</v>
       </c>
       <c r="P3" t="n">
-        <v>38.5637</v>
+        <v>38.9673</v>
       </c>
       <c r="Q3" t="n">
-        <v>42.5106</v>
+        <v>41.9988</v>
       </c>
       <c r="R3" t="n">
-        <v>-30.5139</v>
+        <v>-4.616</v>
       </c>
       <c r="U3" t="n">
-        <v>-14.2807</v>
+        <v>-3.3434</v>
       </c>
       <c r="X3" t="n">
-        <v>31.5383</v>
+        <v>4.2173</v>
       </c>
       <c r="AA3" t="n">
-        <v>14.3803</v>
+        <v>3.4173</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>210.62</v>
+        <v>191.54</v>
       </c>
       <c r="C4" t="n">
-        <v>222.19</v>
+        <v>212.99</v>
       </c>
       <c r="D4" t="n">
-        <v>201.69</v>
+        <v>177.3</v>
       </c>
       <c r="E4" t="n">
-        <v>211.44</v>
+        <v>180.65</v>
       </c>
       <c r="F4" t="n">
-        <v>76.86</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>78.47</v>
+        <v>74.7</v>
       </c>
       <c r="H4" t="n">
-        <v>75.38</v>
+        <v>69</v>
       </c>
       <c r="I4" t="n">
-        <v>76.27</v>
+        <v>69.27</v>
       </c>
       <c r="J4" t="n">
-        <v>5.6442</v>
+        <v>6.1681</v>
       </c>
       <c r="K4" t="n">
-        <v>5.9803</v>
+        <v>6.5734</v>
       </c>
       <c r="L4" t="n">
-        <v>5.2093</v>
+        <v>5.5355</v>
       </c>
       <c r="M4" t="n">
-        <v>5.6245</v>
+        <v>6.4943</v>
       </c>
       <c r="N4" t="n">
-        <v>40.2763</v>
+        <v>43.1209</v>
       </c>
       <c r="O4" t="n">
-        <v>41.1228</v>
+        <v>44.676</v>
       </c>
       <c r="P4" t="n">
-        <v>39.3314</v>
+        <v>41.4082</v>
       </c>
       <c r="Q4" t="n">
-        <v>40.611</v>
+        <v>44.5382</v>
       </c>
       <c r="R4" t="n">
-        <v>15.8321</v>
+        <v>-10.4274</v>
       </c>
       <c r="U4" t="n">
-        <v>4.4079</v>
+        <v>-6.0364</v>
       </c>
       <c r="X4" t="n">
-        <v>-16.8121</v>
+        <v>10.7921</v>
       </c>
       <c r="AA4" t="n">
-        <v>-4.4685</v>
+        <v>6.0464</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>227.06</v>
+        <v>192.3</v>
       </c>
       <c r="C5" t="n">
-        <v>231.02</v>
+        <v>225.63</v>
       </c>
       <c r="D5" t="n">
-        <v>157.56</v>
+        <v>192.3</v>
       </c>
       <c r="E5" t="n">
-        <v>201.68</v>
+        <v>223.99</v>
       </c>
       <c r="F5" t="n">
-        <v>78.48</v>
+        <v>70.89</v>
       </c>
       <c r="G5" t="n">
-        <v>79.34</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>66.79000000000001</v>
+        <v>69.59</v>
       </c>
       <c r="I5" t="n">
-        <v>73.72</v>
+        <v>76.01000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>5.1895</v>
+        <v>6.0298</v>
       </c>
       <c r="K5" t="n">
-        <v>7.0281</v>
+        <v>6.0298</v>
       </c>
       <c r="L5" t="n">
-        <v>5.0808</v>
+        <v>4.8436</v>
       </c>
       <c r="M5" t="n">
-        <v>5.8617</v>
+        <v>4.9128</v>
       </c>
       <c r="N5" t="n">
-        <v>39.4299</v>
+        <v>43.4851</v>
       </c>
       <c r="O5" t="n">
-        <v>45.6505</v>
+        <v>44.302</v>
       </c>
       <c r="P5" t="n">
-        <v>38.9673</v>
+        <v>39.8039</v>
       </c>
       <c r="Q5" t="n">
-        <v>41.9988</v>
+        <v>40.1878</v>
       </c>
       <c r="R5" t="n">
-        <v>-4.616</v>
+        <v>23.9911</v>
       </c>
       <c r="S5" t="n">
-        <v>-23.228</v>
+        <v>5.9355</v>
       </c>
       <c r="U5" t="n">
-        <v>-3.3434</v>
+        <v>9.73</v>
       </c>
       <c r="V5" t="n">
-        <v>-13.4945</v>
+        <v>-0.3409</v>
       </c>
       <c r="X5" t="n">
-        <v>4.2173</v>
+        <v>-24.3521</v>
       </c>
       <c r="Y5" t="n">
-        <v>14.0386</v>
+        <v>-12.6536</v>
       </c>
       <c r="AA5" t="n">
-        <v>3.4173</v>
+        <v>-9.767799999999999</v>
       </c>
       <c r="AB5" t="n">
-        <v>13.0033</v>
+        <v>-1.0421</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>191.54</v>
+        <v>222.22</v>
       </c>
       <c r="C6" t="n">
-        <v>212.99</v>
+        <v>242.4</v>
       </c>
       <c r="D6" t="n">
-        <v>177.3</v>
+        <v>214.74</v>
       </c>
       <c r="E6" t="n">
-        <v>180.65</v>
+        <v>234.68</v>
       </c>
       <c r="F6" t="n">
-        <v>71.68000000000001</v>
+        <v>76.34</v>
       </c>
       <c r="G6" t="n">
-        <v>74.7</v>
+        <v>78.36</v>
       </c>
       <c r="H6" t="n">
-        <v>69</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="I6" t="n">
-        <v>69.27</v>
+        <v>77.52</v>
       </c>
       <c r="J6" t="n">
-        <v>6.1681</v>
+        <v>4.9523</v>
       </c>
       <c r="K6" t="n">
-        <v>6.5734</v>
+        <v>5.0907</v>
       </c>
       <c r="L6" t="n">
-        <v>5.5355</v>
+        <v>4.4877</v>
       </c>
       <c r="M6" t="n">
-        <v>6.4943</v>
+        <v>4.6656</v>
       </c>
       <c r="N6" t="n">
-        <v>43.1209</v>
+        <v>40.0106</v>
       </c>
       <c r="O6" t="n">
-        <v>44.676</v>
+        <v>41.0933</v>
       </c>
       <c r="P6" t="n">
-        <v>41.4082</v>
+        <v>38.9476</v>
       </c>
       <c r="Q6" t="n">
-        <v>44.5382</v>
+        <v>39.4102</v>
       </c>
       <c r="R6" t="n">
-        <v>-10.4274</v>
+        <v>4.7725</v>
       </c>
       <c r="S6" t="n">
-        <v>-1.0354</v>
+        <v>16.3626</v>
       </c>
       <c r="U6" t="n">
-        <v>-6.0364</v>
+        <v>1.9866</v>
       </c>
       <c r="V6" t="n">
-        <v>-5.1745</v>
+        <v>5.1546</v>
       </c>
       <c r="X6" t="n">
-        <v>10.7921</v>
+        <v>-5.0318</v>
       </c>
       <c r="Y6" t="n">
-        <v>-3.9475</v>
+        <v>-20.4053</v>
       </c>
       <c r="AA6" t="n">
-        <v>6.0464</v>
+        <v>-1.9349</v>
       </c>
       <c r="AB6" t="n">
-        <v>4.7696</v>
+        <v>-6.1635</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>192.3</v>
+        <v>265.99</v>
       </c>
       <c r="C7" t="n">
-        <v>225.63</v>
+        <v>274.88</v>
       </c>
       <c r="D7" t="n">
-        <v>192.3</v>
+        <v>261.6</v>
       </c>
       <c r="E7" t="n">
-        <v>223.99</v>
+        <v>272.5</v>
       </c>
       <c r="F7" t="n">
-        <v>70.89</v>
+        <v>82.88</v>
       </c>
       <c r="G7" t="n">
-        <v>76.59999999999999</v>
+        <v>85.03</v>
       </c>
       <c r="H7" t="n">
-        <v>69.59</v>
+        <v>82.64</v>
       </c>
       <c r="I7" t="n">
-        <v>76.01000000000001</v>
+        <v>84.59</v>
       </c>
       <c r="J7" t="n">
-        <v>6.0298</v>
+        <v>4.0231</v>
       </c>
       <c r="K7" t="n">
-        <v>6.0298</v>
+        <v>4.122</v>
       </c>
       <c r="L7" t="n">
-        <v>4.8436</v>
+        <v>3.865</v>
       </c>
       <c r="M7" t="n">
-        <v>4.9128</v>
+        <v>3.9045</v>
       </c>
       <c r="N7" t="n">
-        <v>43.4851</v>
+        <v>36.6641</v>
       </c>
       <c r="O7" t="n">
-        <v>44.302</v>
+        <v>36.7723</v>
       </c>
       <c r="P7" t="n">
-        <v>39.8039</v>
+        <v>35.5814</v>
       </c>
       <c r="Q7" t="n">
-        <v>40.1878</v>
+        <v>35.7389</v>
       </c>
       <c r="R7" t="n">
-        <v>23.9911</v>
+        <v>16.1156</v>
       </c>
       <c r="S7" t="n">
-        <v>5.9355</v>
+        <v>50.8442</v>
       </c>
       <c r="T7" t="n">
-        <v>-14.7354</v>
+        <v>28.8782</v>
       </c>
       <c r="U7" t="n">
-        <v>9.73</v>
+        <v>9.120200000000001</v>
       </c>
       <c r="V7" t="n">
-        <v>-0.3409</v>
+        <v>22.1164</v>
       </c>
       <c r="W7" t="n">
-        <v>-10.8073</v>
+        <v>10.9086</v>
       </c>
       <c r="X7" t="n">
-        <v>-24.3521</v>
+        <v>-16.313</v>
       </c>
       <c r="Y7" t="n">
-        <v>-12.6536</v>
+        <v>-39.878</v>
       </c>
       <c r="Z7" t="n">
-        <v>-4.4221</v>
+        <v>-30.5805</v>
       </c>
       <c r="AA7" t="n">
-        <v>-9.767799999999999</v>
+        <v>-9.3156</v>
       </c>
       <c r="AB7" t="n">
-        <v>-1.0421</v>
+        <v>-19.7567</v>
       </c>
       <c r="AC7" t="n">
-        <v>8.1305</v>
+        <v>-11.997</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>222.22</v>
+        <v>267.13</v>
       </c>
       <c r="C8" t="n">
-        <v>242.4</v>
+        <v>274.93</v>
       </c>
       <c r="D8" t="n">
-        <v>214.74</v>
+        <v>226</v>
       </c>
       <c r="E8" t="n">
-        <v>234.68</v>
+        <v>226.19</v>
       </c>
       <c r="F8" t="n">
-        <v>76.34</v>
+        <v>84.19</v>
       </c>
       <c r="G8" t="n">
-        <v>78.36</v>
+        <v>84.83</v>
       </c>
       <c r="H8" t="n">
-        <v>74.29000000000001</v>
+        <v>79.86</v>
       </c>
       <c r="I8" t="n">
-        <v>77.52</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>4.9523</v>
+        <v>3.9836</v>
       </c>
       <c r="K8" t="n">
-        <v>5.0907</v>
+        <v>4.5965</v>
       </c>
       <c r="L8" t="n">
-        <v>4.4877</v>
+        <v>3.865</v>
       </c>
       <c r="M8" t="n">
-        <v>4.6656</v>
+        <v>4.5767</v>
       </c>
       <c r="N8" t="n">
-        <v>40.0106</v>
+        <v>35.9652</v>
       </c>
       <c r="O8" t="n">
-        <v>41.0933</v>
+        <v>37.7861</v>
       </c>
       <c r="P8" t="n">
-        <v>38.9476</v>
+        <v>35.6896</v>
       </c>
       <c r="Q8" t="n">
-        <v>39.4102</v>
+        <v>37.7468</v>
       </c>
       <c r="R8" t="n">
-        <v>4.7725</v>
+        <v>-16.9945</v>
       </c>
       <c r="S8" t="n">
-        <v>16.3626</v>
+        <v>0.9822</v>
       </c>
       <c r="T8" t="n">
-        <v>28.5636</v>
+        <v>12.1529</v>
       </c>
       <c r="U8" t="n">
-        <v>1.9866</v>
+        <v>-5.5089</v>
       </c>
       <c r="V8" t="n">
-        <v>5.1546</v>
+        <v>5.1572</v>
       </c>
       <c r="W8" t="n">
-        <v>6.1191</v>
+        <v>8.4238</v>
       </c>
       <c r="X8" t="n">
-        <v>-5.0318</v>
+        <v>17.216</v>
       </c>
       <c r="Y8" t="n">
-        <v>-20.4053</v>
+        <v>-6.8413</v>
       </c>
       <c r="Z8" t="n">
-        <v>-30.9945</v>
+        <v>-21.922</v>
       </c>
       <c r="AA8" t="n">
-        <v>-1.9349</v>
+        <v>5.6182</v>
       </c>
       <c r="AB8" t="n">
-        <v>-6.1635</v>
+        <v>-6.074</v>
       </c>
       <c r="AC8" t="n">
-        <v>-7.2932</v>
+        <v>-10.1241</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>265.99</v>
+        <v>247.42</v>
       </c>
       <c r="C9" t="n">
-        <v>274.88</v>
+        <v>259.79</v>
       </c>
       <c r="D9" t="n">
-        <v>261.6</v>
+        <v>233.3</v>
       </c>
       <c r="E9" t="n">
-        <v>272.5</v>
+        <v>233.86</v>
       </c>
       <c r="F9" t="n">
-        <v>82.88</v>
+        <v>81.67</v>
       </c>
       <c r="G9" t="n">
-        <v>85.03</v>
+        <v>81.81</v>
       </c>
       <c r="H9" t="n">
-        <v>82.64</v>
+        <v>76.94</v>
       </c>
       <c r="I9" t="n">
-        <v>84.59</v>
+        <v>77.54000000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>4.0231</v>
+        <v>4.122</v>
       </c>
       <c r="K9" t="n">
-        <v>4.122</v>
+        <v>4.4086</v>
       </c>
       <c r="L9" t="n">
-        <v>3.865</v>
+        <v>3.8749</v>
       </c>
       <c r="M9" t="n">
-        <v>3.9045</v>
+        <v>4.4086</v>
       </c>
       <c r="N9" t="n">
-        <v>36.6641</v>
+        <v>36.9397</v>
       </c>
       <c r="O9" t="n">
-        <v>36.7723</v>
+        <v>39.1641</v>
       </c>
       <c r="P9" t="n">
-        <v>35.5814</v>
+        <v>36.8708</v>
       </c>
       <c r="Q9" t="n">
-        <v>35.7389</v>
+        <v>38.8984</v>
       </c>
       <c r="R9" t="n">
-        <v>16.1156</v>
+        <v>3.391</v>
       </c>
       <c r="S9" t="n">
-        <v>50.8442</v>
+        <v>-0.3494</v>
       </c>
       <c r="T9" t="n">
-        <v>28.8782</v>
+        <v>29.4547</v>
       </c>
       <c r="U9" t="n">
-        <v>9.120200000000001</v>
+        <v>-2.9901</v>
       </c>
       <c r="V9" t="n">
-        <v>22.1164</v>
+        <v>0.0258</v>
       </c>
       <c r="W9" t="n">
-        <v>10.9086</v>
+        <v>11.9388</v>
       </c>
       <c r="X9" t="n">
-        <v>-16.313</v>
+        <v>-3.673</v>
       </c>
       <c r="Y9" t="n">
-        <v>-39.878</v>
+        <v>-5.5084</v>
       </c>
       <c r="Z9" t="n">
-        <v>-30.5805</v>
+        <v>-32.1159</v>
       </c>
       <c r="AA9" t="n">
-        <v>-9.3156</v>
+        <v>3.0509</v>
       </c>
       <c r="AB9" t="n">
-        <v>-19.7567</v>
+        <v>-1.2986</v>
       </c>
       <c r="AC9" t="n">
-        <v>-11.997</v>
+        <v>-12.6628</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>267.13</v>
+        <v>266.04</v>
       </c>
       <c r="C10" t="n">
-        <v>274.93</v>
+        <v>286.15</v>
       </c>
       <c r="D10" t="n">
-        <v>226</v>
+        <v>265</v>
       </c>
       <c r="E10" t="n">
-        <v>226.19</v>
+        <v>279.29</v>
       </c>
       <c r="F10" t="n">
-        <v>84.19</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="G10" t="n">
-        <v>84.83</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>79.86</v>
+        <v>80.63</v>
       </c>
       <c r="I10" t="n">
-        <v>79.93000000000001</v>
+        <v>82.87</v>
       </c>
       <c r="J10" t="n">
-        <v>3.9836</v>
+        <v>3.8156</v>
       </c>
       <c r="K10" t="n">
-        <v>4.5965</v>
+        <v>3.8254</v>
       </c>
       <c r="L10" t="n">
-        <v>3.865</v>
+        <v>3.4103</v>
       </c>
       <c r="M10" t="n">
-        <v>4.5767</v>
+        <v>3.5487</v>
       </c>
       <c r="N10" t="n">
-        <v>35.9652</v>
+        <v>36.6149</v>
       </c>
       <c r="O10" t="n">
-        <v>37.7861</v>
+        <v>37.3531</v>
       </c>
       <c r="P10" t="n">
-        <v>35.6896</v>
+        <v>35.857</v>
       </c>
       <c r="Q10" t="n">
-        <v>37.7468</v>
+        <v>36.1719</v>
       </c>
       <c r="R10" t="n">
-        <v>-16.9945</v>
+        <v>19.4262</v>
       </c>
       <c r="S10" t="n">
-        <v>0.9822</v>
+        <v>2.4917</v>
       </c>
       <c r="T10" t="n">
-        <v>12.1529</v>
+        <v>24.6886</v>
       </c>
       <c r="U10" t="n">
-        <v>-5.5089</v>
+        <v>6.8739</v>
       </c>
       <c r="V10" t="n">
-        <v>5.1572</v>
+        <v>-2.0333</v>
       </c>
       <c r="W10" t="n">
-        <v>8.4238</v>
+        <v>9.0251</v>
       </c>
       <c r="X10" t="n">
-        <v>17.216</v>
+        <v>-19.5051</v>
       </c>
       <c r="Y10" t="n">
-        <v>-6.8413</v>
+        <v>-9.1126</v>
       </c>
       <c r="Z10" t="n">
-        <v>-21.922</v>
+        <v>-27.7662</v>
       </c>
       <c r="AA10" t="n">
-        <v>5.6182</v>
+        <v>-7.0093</v>
       </c>
       <c r="AB10" t="n">
-        <v>-6.074</v>
+        <v>1.2116</v>
       </c>
       <c r="AC10" t="n">
-        <v>-10.1241</v>
+        <v>-9.992800000000001</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>247.42</v>
+        <v>299.26</v>
       </c>
       <c r="C11" t="n">
-        <v>259.79</v>
+        <v>302</v>
       </c>
       <c r="D11" t="n">
-        <v>233.3</v>
+        <v>286.24</v>
       </c>
       <c r="E11" t="n">
-        <v>233.86</v>
+        <v>300.77</v>
       </c>
       <c r="F11" t="n">
-        <v>81.67</v>
+        <v>83.95</v>
       </c>
       <c r="G11" t="n">
-        <v>81.81</v>
+        <v>85.11</v>
       </c>
       <c r="H11" t="n">
-        <v>76.94</v>
+        <v>81.39</v>
       </c>
       <c r="I11" t="n">
-        <v>77.54000000000001</v>
+        <v>82.58</v>
       </c>
       <c r="J11" t="n">
-        <v>4.122</v>
+        <v>3.2917</v>
       </c>
       <c r="K11" t="n">
-        <v>4.4086</v>
+        <v>3.4498</v>
       </c>
       <c r="L11" t="n">
-        <v>3.8749</v>
+        <v>3.2521</v>
       </c>
       <c r="M11" t="n">
-        <v>4.4086</v>
+        <v>3.262</v>
       </c>
       <c r="N11" t="n">
-        <v>36.9397</v>
+        <v>35.7389</v>
       </c>
       <c r="O11" t="n">
-        <v>39.1641</v>
+        <v>36.8511</v>
       </c>
       <c r="P11" t="n">
-        <v>36.8708</v>
+        <v>35.2369</v>
       </c>
       <c r="Q11" t="n">
-        <v>38.8984</v>
+        <v>36.3491</v>
       </c>
       <c r="R11" t="n">
-        <v>3.391</v>
+        <v>7.6909</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.3494</v>
+        <v>32.9723</v>
       </c>
       <c r="T11" t="n">
-        <v>29.4547</v>
+        <v>28.1618</v>
       </c>
       <c r="U11" t="n">
-        <v>-2.9901</v>
+        <v>-0.3499</v>
       </c>
       <c r="V11" t="n">
-        <v>0.0258</v>
+        <v>3.3154</v>
       </c>
       <c r="W11" t="n">
-        <v>11.9388</v>
+        <v>6.5273</v>
       </c>
       <c r="X11" t="n">
-        <v>-3.673</v>
+        <v>-8.079000000000001</v>
       </c>
       <c r="Y11" t="n">
-        <v>-5.5084</v>
+        <v>-28.7259</v>
       </c>
       <c r="Z11" t="n">
-        <v>-32.1159</v>
+        <v>-30.084</v>
       </c>
       <c r="AA11" t="n">
-        <v>3.0509</v>
+        <v>0.4899</v>
       </c>
       <c r="AB11" t="n">
-        <v>-1.2986</v>
+        <v>-3.7028</v>
       </c>
       <c r="AC11" t="n">
-        <v>-12.6628</v>
+        <v>-7.7673</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>266.04</v>
+        <v>236</v>
       </c>
       <c r="C12" t="n">
-        <v>286.15</v>
+        <v>252.98</v>
       </c>
       <c r="D12" t="n">
-        <v>265</v>
+        <v>223</v>
       </c>
       <c r="E12" t="n">
-        <v>279.29</v>
+        <v>231.42</v>
       </c>
       <c r="F12" t="n">
-        <v>82.09999999999999</v>
+        <v>75.12</v>
       </c>
       <c r="G12" t="n">
-        <v>83.59999999999999</v>
+        <v>77.73999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>80.63</v>
+        <v>73.91</v>
       </c>
       <c r="I12" t="n">
-        <v>82.87</v>
+        <v>74.44</v>
       </c>
       <c r="J12" t="n">
-        <v>3.8156</v>
+        <v>3.99</v>
       </c>
       <c r="K12" t="n">
-        <v>3.8254</v>
+        <v>4.13</v>
       </c>
       <c r="L12" t="n">
-        <v>3.4103</v>
+        <v>3.8</v>
       </c>
       <c r="M12" t="n">
-        <v>3.5487</v>
+        <v>4.04</v>
       </c>
       <c r="N12" t="n">
-        <v>36.6149</v>
+        <v>39.6267</v>
       </c>
       <c r="O12" t="n">
-        <v>37.3531</v>
+        <v>40.1582</v>
       </c>
       <c r="P12" t="n">
-        <v>35.857</v>
+        <v>38.4653</v>
       </c>
       <c r="Q12" t="n">
-        <v>36.1719</v>
+        <v>39.922</v>
       </c>
       <c r="R12" t="n">
-        <v>19.4262</v>
+        <v>-23.0575</v>
       </c>
       <c r="S12" t="n">
-        <v>2.4917</v>
+        <v>-1.0434</v>
       </c>
       <c r="T12" t="n">
-        <v>24.6886</v>
+        <v>-15.0752</v>
       </c>
       <c r="U12" t="n">
-        <v>6.8739</v>
+        <v>-9.857100000000001</v>
       </c>
       <c r="V12" t="n">
-        <v>-2.0333</v>
+        <v>-3.9979</v>
       </c>
       <c r="W12" t="n">
-        <v>9.0251</v>
+        <v>-11.9991</v>
       </c>
       <c r="X12" t="n">
-        <v>-19.5051</v>
+        <v>23.8504</v>
       </c>
       <c r="Y12" t="n">
-        <v>-9.1126</v>
+        <v>-8.360900000000001</v>
       </c>
       <c r="Z12" t="n">
-        <v>-27.7662</v>
+        <v>3.4704</v>
       </c>
       <c r="AA12" t="n">
-        <v>-7.0093</v>
+        <v>9.8294</v>
       </c>
       <c r="AB12" t="n">
-        <v>1.2116</v>
+        <v>2.6315</v>
       </c>
       <c r="AC12" t="n">
-        <v>-9.992800000000001</v>
+        <v>11.7046</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>299.26</v>
+        <v>233.11</v>
       </c>
       <c r="C13" t="n">
-        <v>302</v>
+        <v>237</v>
       </c>
       <c r="D13" t="n">
-        <v>286.24</v>
+        <v>211.13</v>
       </c>
       <c r="E13" t="n">
-        <v>300.77</v>
+        <v>229.57</v>
       </c>
       <c r="F13" t="n">
-        <v>83.95</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>85.11</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="H13" t="n">
-        <v>81.39</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>82.58</v>
+        <v>73.3</v>
       </c>
       <c r="J13" t="n">
-        <v>3.2917</v>
+        <v>4</v>
       </c>
       <c r="K13" t="n">
-        <v>3.4498</v>
+        <v>4.39</v>
       </c>
       <c r="L13" t="n">
-        <v>3.2521</v>
+        <v>3.92</v>
       </c>
       <c r="M13" t="n">
-        <v>3.262</v>
+        <v>4.08</v>
       </c>
       <c r="N13" t="n">
-        <v>35.7389</v>
+        <v>39.66</v>
       </c>
       <c r="O13" t="n">
-        <v>36.8511</v>
+        <v>41.49</v>
       </c>
       <c r="P13" t="n">
-        <v>35.2369</v>
+        <v>38.9</v>
       </c>
       <c r="Q13" t="n">
-        <v>36.3491</v>
+        <v>40.45</v>
       </c>
       <c r="R13" t="n">
-        <v>7.6909</v>
+        <v>-0.7994</v>
       </c>
       <c r="S13" t="n">
-        <v>32.9723</v>
+        <v>-17.8023</v>
       </c>
       <c r="T13" t="n">
-        <v>28.1618</v>
+        <v>1.4943</v>
       </c>
       <c r="U13" t="n">
-        <v>-0.3499</v>
+        <v>-1.5314</v>
       </c>
       <c r="V13" t="n">
-        <v>3.3154</v>
+        <v>-11.5482</v>
       </c>
       <c r="W13" t="n">
-        <v>6.5273</v>
+        <v>-8.2948</v>
       </c>
       <c r="X13" t="n">
-        <v>-8.079000000000001</v>
+        <v>0.9901</v>
       </c>
       <c r="Y13" t="n">
-        <v>-28.7259</v>
+        <v>14.9717</v>
       </c>
       <c r="Z13" t="n">
-        <v>-30.084</v>
+        <v>-10.8528</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.4899</v>
+        <v>1.3226</v>
       </c>
       <c r="AB13" t="n">
-        <v>-3.7028</v>
+        <v>11.8271</v>
       </c>
       <c r="AC13" t="n">
-        <v>-7.7673</v>
+        <v>7.1614</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>236</v>
+        <v>268.05</v>
       </c>
       <c r="C14" t="n">
-        <v>252.98</v>
+        <v>268.4</v>
       </c>
       <c r="D14" t="n">
-        <v>223</v>
+        <v>225.74</v>
       </c>
       <c r="E14" t="n">
-        <v>231.42</v>
+        <v>252.61</v>
       </c>
       <c r="F14" t="n">
-        <v>75.12</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>77.73999999999999</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>73.91</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I14" t="n">
-        <v>74.44</v>
+        <v>74.95</v>
       </c>
       <c r="J14" t="n">
-        <v>3.99</v>
+        <v>3.38</v>
       </c>
       <c r="K14" t="n">
-        <v>4.13</v>
+        <v>4.15</v>
       </c>
       <c r="L14" t="n">
-        <v>3.8</v>
+        <v>3.37</v>
       </c>
       <c r="M14" t="n">
-        <v>4.04</v>
+        <v>3.63</v>
       </c>
       <c r="N14" t="n">
-        <v>39.6267</v>
+        <v>37.87</v>
       </c>
       <c r="O14" t="n">
-        <v>40.1582</v>
+        <v>41.37</v>
       </c>
       <c r="P14" t="n">
-        <v>38.4653</v>
+        <v>37.71</v>
       </c>
       <c r="Q14" t="n">
-        <v>39.922</v>
+        <v>39.47</v>
       </c>
       <c r="R14" t="n">
-        <v>-23.0575</v>
+        <v>10.0362</v>
       </c>
       <c r="S14" t="n">
-        <v>-1.0434</v>
+        <v>-16.0122</v>
       </c>
       <c r="T14" t="n">
-        <v>-15.0752</v>
+        <v>8.0176</v>
       </c>
       <c r="U14" t="n">
-        <v>-9.857100000000001</v>
+        <v>2.251</v>
       </c>
       <c r="V14" t="n">
-        <v>-3.9979</v>
+        <v>-9.2395</v>
       </c>
       <c r="W14" t="n">
-        <v>-11.9991</v>
+        <v>-3.3402</v>
       </c>
       <c r="X14" t="n">
-        <v>23.8504</v>
+        <v>-11.0294</v>
       </c>
       <c r="Y14" t="n">
-        <v>-8.360900000000001</v>
+        <v>11.2814</v>
       </c>
       <c r="Z14" t="n">
-        <v>3.4704</v>
+        <v>-17.6609</v>
       </c>
       <c r="AA14" t="n">
-        <v>9.8294</v>
+        <v>-2.4227</v>
       </c>
       <c r="AB14" t="n">
-        <v>2.6315</v>
+        <v>8.585900000000001</v>
       </c>
       <c r="AC14" t="n">
-        <v>11.7046</v>
+        <v>1.4695</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>233.11</v>
+        <v>226.24</v>
       </c>
       <c r="C15" t="n">
-        <v>237</v>
+        <v>231.25</v>
       </c>
       <c r="D15" t="n">
-        <v>211.13</v>
+        <v>212.1</v>
       </c>
       <c r="E15" t="n">
-        <v>229.57</v>
+        <v>215.6</v>
       </c>
       <c r="F15" t="n">
-        <v>74.79000000000001</v>
+        <v>72.09</v>
       </c>
       <c r="G15" t="n">
-        <v>76.18000000000001</v>
+        <v>74.69</v>
       </c>
       <c r="H15" t="n">
-        <v>71.34999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="I15" t="n">
-        <v>73.3</v>
+        <v>71.83</v>
       </c>
       <c r="J15" t="n">
-        <v>4</v>
+        <v>4.04</v>
       </c>
       <c r="K15" t="n">
-        <v>4.39</v>
+        <v>4.25</v>
       </c>
       <c r="L15" t="n">
-        <v>3.92</v>
+        <v>3.95</v>
       </c>
       <c r="M15" t="n">
-        <v>4.08</v>
+        <v>4.24</v>
       </c>
       <c r="N15" t="n">
-        <v>39.66</v>
+        <v>41.08</v>
       </c>
       <c r="O15" t="n">
-        <v>41.49</v>
+        <v>41.79</v>
       </c>
       <c r="P15" t="n">
-        <v>38.9</v>
+        <v>39.69</v>
       </c>
       <c r="Q15" t="n">
-        <v>40.45</v>
+        <v>41.31</v>
       </c>
       <c r="R15" t="n">
-        <v>-0.7994</v>
+        <v>-14.651</v>
       </c>
       <c r="S15" t="n">
-        <v>-17.8023</v>
+        <v>-6.8361</v>
       </c>
       <c r="T15" t="n">
-        <v>1.4943</v>
+        <v>-22.8043</v>
       </c>
       <c r="U15" t="n">
-        <v>-1.5314</v>
+        <v>-4.1628</v>
       </c>
       <c r="V15" t="n">
-        <v>-11.5482</v>
+        <v>-3.5062</v>
       </c>
       <c r="W15" t="n">
-        <v>-8.2948</v>
+        <v>-13.3221</v>
       </c>
       <c r="X15" t="n">
-        <v>0.9901</v>
+        <v>16.8044</v>
       </c>
       <c r="Y15" t="n">
-        <v>14.9717</v>
+        <v>4.9505</v>
       </c>
       <c r="Z15" t="n">
-        <v>-10.8528</v>
+        <v>19.4804</v>
       </c>
       <c r="AA15" t="n">
-        <v>1.3226</v>
+        <v>4.6618</v>
       </c>
       <c r="AB15" t="n">
-        <v>11.8271</v>
+        <v>3.4768</v>
       </c>
       <c r="AC15" t="n">
-        <v>7.1614</v>
+        <v>14.2047</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>268.05</v>
+        <v>216.36</v>
       </c>
       <c r="C16" t="n">
-        <v>268.4</v>
+        <v>238.65</v>
       </c>
       <c r="D16" t="n">
-        <v>225.74</v>
+        <v>192.3</v>
       </c>
       <c r="E16" t="n">
-        <v>252.61</v>
+        <v>236.52</v>
       </c>
       <c r="F16" t="n">
-        <v>77.95999999999999</v>
+        <v>74.12</v>
       </c>
       <c r="G16" t="n">
-        <v>78.23999999999999</v>
+        <v>77.38</v>
       </c>
       <c r="H16" t="n">
-        <v>71.59999999999999</v>
+        <v>71.45</v>
       </c>
       <c r="I16" t="n">
-        <v>74.95</v>
+        <v>77.19</v>
       </c>
       <c r="J16" t="n">
-        <v>3.38</v>
+        <v>4.16</v>
       </c>
       <c r="K16" t="n">
-        <v>4.15</v>
+        <v>4.63</v>
       </c>
       <c r="L16" t="n">
-        <v>3.37</v>
+        <v>3.7</v>
       </c>
       <c r="M16" t="n">
-        <v>3.63</v>
+        <v>3.72</v>
       </c>
       <c r="N16" t="n">
-        <v>37.87</v>
+        <v>39.91</v>
       </c>
       <c r="O16" t="n">
-        <v>41.37</v>
+        <v>41.43</v>
       </c>
       <c r="P16" t="n">
-        <v>37.71</v>
+        <v>38.08</v>
       </c>
       <c r="Q16" t="n">
-        <v>39.47</v>
+        <v>38.16</v>
       </c>
       <c r="R16" t="n">
-        <v>10.0362</v>
+        <v>9.703200000000001</v>
       </c>
       <c r="S16" t="n">
-        <v>-16.0122</v>
+        <v>3.0274</v>
       </c>
       <c r="T16" t="n">
-        <v>8.0176</v>
+        <v>-21.3618</v>
       </c>
       <c r="U16" t="n">
-        <v>2.251</v>
+        <v>7.4621</v>
       </c>
       <c r="V16" t="n">
-        <v>-9.2395</v>
+        <v>5.307</v>
       </c>
       <c r="W16" t="n">
-        <v>-3.3402</v>
+        <v>-6.527</v>
       </c>
       <c r="X16" t="n">
-        <v>-11.0294</v>
+        <v>-12.2642</v>
       </c>
       <c r="Y16" t="n">
-        <v>11.2814</v>
+        <v>-8.823499999999999</v>
       </c>
       <c r="Z16" t="n">
-        <v>-17.6609</v>
+        <v>14.0405</v>
       </c>
       <c r="AA16" t="n">
-        <v>-2.4227</v>
+        <v>-7.6253</v>
       </c>
       <c r="AB16" t="n">
-        <v>8.585900000000001</v>
+        <v>-5.6613</v>
       </c>
       <c r="AC16" t="n">
-        <v>1.4695</v>
+        <v>4.982</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>226.24</v>
+        <v>241.45</v>
       </c>
       <c r="C17" t="n">
-        <v>231.25</v>
+        <v>272</v>
       </c>
       <c r="D17" t="n">
-        <v>212.1</v>
+        <v>240.59</v>
       </c>
       <c r="E17" t="n">
-        <v>215.6</v>
+        <v>266.71</v>
       </c>
       <c r="F17" t="n">
-        <v>72.09</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="G17" t="n">
-        <v>74.69</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="H17" t="n">
-        <v>70.72</v>
+        <v>77.15000000000001</v>
       </c>
       <c r="I17" t="n">
-        <v>71.83</v>
+        <v>81</v>
       </c>
       <c r="J17" t="n">
-        <v>4.04</v>
+        <v>3.66</v>
       </c>
       <c r="K17" t="n">
-        <v>4.25</v>
+        <v>3.68</v>
       </c>
       <c r="L17" t="n">
-        <v>3.95</v>
+        <v>3.17</v>
       </c>
       <c r="M17" t="n">
-        <v>4.24</v>
+        <v>3.24</v>
       </c>
       <c r="N17" t="n">
-        <v>41.08</v>
+        <v>38.16</v>
       </c>
       <c r="O17" t="n">
-        <v>41.79</v>
+        <v>38.2</v>
       </c>
       <c r="P17" t="n">
-        <v>39.69</v>
+        <v>36.03</v>
       </c>
       <c r="Q17" t="n">
-        <v>41.31</v>
+        <v>36.31</v>
       </c>
       <c r="R17" t="n">
-        <v>-14.651</v>
+        <v>12.7642</v>
       </c>
       <c r="S17" t="n">
-        <v>-6.8361</v>
+        <v>5.5817</v>
       </c>
       <c r="T17" t="n">
-        <v>-22.8043</v>
+        <v>15.2493</v>
       </c>
       <c r="U17" t="n">
-        <v>-4.1628</v>
+        <v>4.9359</v>
       </c>
       <c r="V17" t="n">
-        <v>-3.5062</v>
+        <v>8.071999999999999</v>
       </c>
       <c r="W17" t="n">
-        <v>-13.3221</v>
+        <v>8.8125</v>
       </c>
       <c r="X17" t="n">
-        <v>16.8044</v>
+        <v>-12.9032</v>
       </c>
       <c r="Y17" t="n">
-        <v>4.9505</v>
+        <v>-10.7438</v>
       </c>
       <c r="Z17" t="n">
-        <v>19.4804</v>
+        <v>-19.802</v>
       </c>
       <c r="AA17" t="n">
-        <v>4.6618</v>
+        <v>-4.848</v>
       </c>
       <c r="AB17" t="n">
-        <v>3.4768</v>
+        <v>-8.0061</v>
       </c>
       <c r="AC17" t="n">
-        <v>14.2047</v>
+        <v>-9.047599999999999</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>216.36</v>
+        <v>237.79</v>
       </c>
       <c r="C18" t="n">
-        <v>238.65</v>
+        <v>246.47</v>
       </c>
       <c r="D18" t="n">
-        <v>192.3</v>
+        <v>215.38</v>
       </c>
       <c r="E18" t="n">
-        <v>236.52</v>
+        <v>217.55</v>
       </c>
       <c r="F18" t="n">
-        <v>74.12</v>
+        <v>78.72</v>
       </c>
       <c r="G18" t="n">
-        <v>77.38</v>
+        <v>79.64</v>
       </c>
       <c r="H18" t="n">
-        <v>71.45</v>
+        <v>77.23</v>
       </c>
       <c r="I18" t="n">
-        <v>77.19</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J18" t="n">
-        <v>4.16</v>
+        <v>3.59</v>
       </c>
       <c r="K18" t="n">
-        <v>4.63</v>
+        <v>3.89</v>
       </c>
       <c r="L18" t="n">
-        <v>3.7</v>
+        <v>3.51</v>
       </c>
       <c r="M18" t="n">
-        <v>3.72</v>
+        <v>3.86</v>
       </c>
       <c r="N18" t="n">
-        <v>39.91</v>
+        <v>37.31</v>
       </c>
       <c r="O18" t="n">
-        <v>41.43</v>
+        <v>37.98</v>
       </c>
       <c r="P18" t="n">
-        <v>38.08</v>
+        <v>36.9</v>
       </c>
       <c r="Q18" t="n">
-        <v>38.16</v>
+        <v>37.88</v>
       </c>
       <c r="R18" t="n">
-        <v>9.703200000000001</v>
+        <v>-18.432</v>
       </c>
       <c r="S18" t="n">
-        <v>3.0274</v>
+        <v>0.9045</v>
       </c>
       <c r="T18" t="n">
-        <v>-21.3618</v>
+        <v>-5.2359</v>
       </c>
       <c r="U18" t="n">
-        <v>7.4621</v>
+        <v>-4.3704</v>
       </c>
       <c r="V18" t="n">
-        <v>5.307</v>
+        <v>7.838</v>
       </c>
       <c r="W18" t="n">
-        <v>-6.527</v>
+        <v>5.6753</v>
       </c>
       <c r="X18" t="n">
-        <v>-12.2642</v>
+        <v>19.1358</v>
       </c>
       <c r="Y18" t="n">
-        <v>-8.823499999999999</v>
+        <v>-8.962300000000001</v>
       </c>
       <c r="Z18" t="n">
-        <v>14.0405</v>
+        <v>-5.3922</v>
       </c>
       <c r="AA18" t="n">
-        <v>-7.6253</v>
+        <v>4.3239</v>
       </c>
       <c r="AB18" t="n">
-        <v>-5.6613</v>
+        <v>-8.303100000000001</v>
       </c>
       <c r="AC18" t="n">
-        <v>4.982</v>
+        <v>-6.3535</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>241.45</v>
+        <v>219.23</v>
       </c>
       <c r="C19" t="n">
-        <v>272</v>
+        <v>226.13</v>
       </c>
       <c r="D19" t="n">
-        <v>240.59</v>
+        <v>168.88</v>
       </c>
       <c r="E19" t="n">
-        <v>266.71</v>
+        <v>181.47</v>
       </c>
       <c r="F19" t="n">
-        <v>77.23999999999999</v>
+        <v>77.45</v>
       </c>
       <c r="G19" t="n">
-        <v>81.54000000000001</v>
+        <v>79.14</v>
       </c>
       <c r="H19" t="n">
-        <v>77.15000000000001</v>
+        <v>71.72</v>
       </c>
       <c r="I19" t="n">
-        <v>81</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="J19" t="n">
-        <v>3.66</v>
+        <v>3.84</v>
       </c>
       <c r="K19" t="n">
-        <v>3.68</v>
+        <v>4.74</v>
       </c>
       <c r="L19" t="n">
-        <v>3.17</v>
+        <v>3.71</v>
       </c>
       <c r="M19" t="n">
-        <v>3.24</v>
+        <v>4.51</v>
       </c>
       <c r="N19" t="n">
-        <v>38.16</v>
+        <v>37.91</v>
       </c>
       <c r="O19" t="n">
-        <v>38.2</v>
+        <v>40.72</v>
       </c>
       <c r="P19" t="n">
-        <v>36.03</v>
+        <v>37.08</v>
       </c>
       <c r="Q19" t="n">
-        <v>36.31</v>
+        <v>39.95</v>
       </c>
       <c r="R19" t="n">
-        <v>12.7642</v>
+        <v>-16.5847</v>
       </c>
       <c r="S19" t="n">
-        <v>5.5817</v>
+        <v>-23.275</v>
       </c>
       <c r="T19" t="n">
-        <v>15.2493</v>
+        <v>-28.162</v>
       </c>
       <c r="U19" t="n">
-        <v>4.9359</v>
+        <v>-5.306</v>
       </c>
       <c r="V19" t="n">
-        <v>8.071999999999999</v>
+        <v>-4.9747</v>
       </c>
       <c r="W19" t="n">
-        <v>8.8125</v>
+        <v>-2.1348</v>
       </c>
       <c r="X19" t="n">
-        <v>-12.9032</v>
+        <v>16.8394</v>
       </c>
       <c r="Y19" t="n">
-        <v>-10.7438</v>
+        <v>21.2366</v>
       </c>
       <c r="Z19" t="n">
-        <v>-19.802</v>
+        <v>24.2424</v>
       </c>
       <c r="AA19" t="n">
-        <v>-4.848</v>
+        <v>5.4646</v>
       </c>
       <c r="AB19" t="n">
-        <v>-8.0061</v>
+        <v>4.6908</v>
       </c>
       <c r="AC19" t="n">
-        <v>-9.047599999999999</v>
+        <v>1.2161</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>237.79</v>
+        <v>197.21</v>
       </c>
       <c r="C20" t="n">
-        <v>246.47</v>
+        <v>210.8</v>
       </c>
       <c r="D20" t="n">
-        <v>215.38</v>
+        <v>194.22</v>
       </c>
       <c r="E20" t="n">
-        <v>217.55</v>
+        <v>194.65</v>
       </c>
       <c r="F20" t="n">
-        <v>78.72</v>
+        <v>75.53</v>
       </c>
       <c r="G20" t="n">
-        <v>79.64</v>
+        <v>77.45</v>
       </c>
       <c r="H20" t="n">
-        <v>77.23</v>
+        <v>75.11</v>
       </c>
       <c r="I20" t="n">
-        <v>77.45999999999999</v>
+        <v>76.42</v>
       </c>
       <c r="J20" t="n">
-        <v>3.59</v>
+        <v>4.11</v>
       </c>
       <c r="K20" t="n">
-        <v>3.89</v>
+        <v>4.18</v>
       </c>
       <c r="L20" t="n">
-        <v>3.51</v>
+        <v>3.77</v>
       </c>
       <c r="M20" t="n">
-        <v>3.86</v>
+        <v>4.17</v>
       </c>
       <c r="N20" t="n">
-        <v>37.31</v>
+        <v>38.75</v>
       </c>
       <c r="O20" t="n">
-        <v>37.98</v>
+        <v>38.97</v>
       </c>
       <c r="P20" t="n">
-        <v>36.9</v>
+        <v>37.705</v>
       </c>
       <c r="Q20" t="n">
-        <v>37.88</v>
+        <v>38.28</v>
       </c>
       <c r="R20" t="n">
-        <v>-18.432</v>
+        <v>7.2629</v>
       </c>
       <c r="S20" t="n">
-        <v>0.9045</v>
+        <v>-27.0181</v>
       </c>
       <c r="T20" t="n">
-        <v>-5.2359</v>
+        <v>-9.7171</v>
       </c>
       <c r="U20" t="n">
-        <v>-4.3704</v>
+        <v>4.1854</v>
       </c>
       <c r="V20" t="n">
-        <v>7.838</v>
+        <v>-5.6543</v>
       </c>
       <c r="W20" t="n">
-        <v>5.6753</v>
+        <v>6.3901</v>
       </c>
       <c r="X20" t="n">
-        <v>19.1358</v>
+        <v>-7.5388</v>
       </c>
       <c r="Y20" t="n">
-        <v>-8.962300000000001</v>
+        <v>28.7037</v>
       </c>
       <c r="Z20" t="n">
-        <v>-5.3922</v>
+        <v>-1.6509</v>
       </c>
       <c r="AA20" t="n">
-        <v>4.3239</v>
+        <v>-4.1802</v>
       </c>
       <c r="AB20" t="n">
-        <v>-8.303100000000001</v>
+        <v>5.4255</v>
       </c>
       <c r="AC20" t="n">
-        <v>-6.3535</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>219.23</v>
-      </c>
-      <c r="C21" t="n">
-        <v>226.13</v>
-      </c>
-      <c r="D21" t="n">
-        <v>168.88</v>
-      </c>
-      <c r="E21" t="n">
-        <v>181.47</v>
-      </c>
-      <c r="F21" t="n">
-        <v>77.45</v>
-      </c>
-      <c r="G21" t="n">
-        <v>79.14</v>
-      </c>
-      <c r="H21" t="n">
-        <v>71.72</v>
-      </c>
-      <c r="I21" t="n">
-        <v>73.34999999999999</v>
-      </c>
-      <c r="J21" t="n">
-        <v>3.84</v>
-      </c>
-      <c r="K21" t="n">
-        <v>4.74</v>
-      </c>
-      <c r="L21" t="n">
-        <v>3.71</v>
-      </c>
-      <c r="M21" t="n">
-        <v>4.51</v>
-      </c>
-      <c r="N21" t="n">
-        <v>37.91</v>
-      </c>
-      <c r="O21" t="n">
-        <v>40.72</v>
-      </c>
-      <c r="P21" t="n">
-        <v>37.08</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>39.95</v>
-      </c>
-      <c r="R21" t="n">
-        <v>-16.5847</v>
-      </c>
-      <c r="S21" t="n">
-        <v>-23.275</v>
-      </c>
-      <c r="T21" t="n">
-        <v>-28.162</v>
-      </c>
-      <c r="U21" t="n">
-        <v>-5.306</v>
-      </c>
-      <c r="V21" t="n">
-        <v>-4.9747</v>
-      </c>
-      <c r="W21" t="n">
-        <v>-2.1348</v>
-      </c>
-      <c r="X21" t="n">
-        <v>16.8394</v>
-      </c>
-      <c r="Y21" t="n">
-        <v>21.2366</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>24.2424</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>5.4646</v>
-      </c>
-      <c r="AB21" t="n">
-        <v>4.6908</v>
-      </c>
-      <c r="AC21" t="n">
-        <v>1.2161</v>
+        <v>-7.3348</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2230,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-07-07 23:01
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC20"/>
+  <dimension ref="A1:AC21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -584,16 +584,16 @@
         <v>211.44</v>
       </c>
       <c r="F2" t="n">
-        <v>76.86</v>
+        <v>76.68340000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>78.47</v>
+        <v>78.2897</v>
       </c>
       <c r="H2" t="n">
-        <v>75.38</v>
+        <v>75.2068</v>
       </c>
       <c r="I2" t="n">
-        <v>76.27</v>
+        <v>76.09480000000001</v>
       </c>
       <c r="J2" t="n">
         <v>5.6442</v>
@@ -639,16 +639,16 @@
         <v>201.68</v>
       </c>
       <c r="F3" t="n">
-        <v>78.48</v>
+        <v>78.2997</v>
       </c>
       <c r="G3" t="n">
-        <v>79.34</v>
+        <v>79.15770000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>66.79000000000001</v>
+        <v>66.6366</v>
       </c>
       <c r="I3" t="n">
-        <v>73.72</v>
+        <v>73.55070000000001</v>
       </c>
       <c r="J3" t="n">
         <v>5.1895</v>
@@ -678,7 +678,7 @@
         <v>-4.616</v>
       </c>
       <c r="U3" t="n">
-        <v>-3.3434</v>
+        <v>-3.3433</v>
       </c>
       <c r="X3" t="n">
         <v>4.2173</v>
@@ -706,16 +706,16 @@
         <v>180.65</v>
       </c>
       <c r="F4" t="n">
-        <v>71.68000000000001</v>
+        <v>71.5153</v>
       </c>
       <c r="G4" t="n">
-        <v>74.7</v>
+        <v>74.5284</v>
       </c>
       <c r="H4" t="n">
-        <v>69</v>
+        <v>68.8415</v>
       </c>
       <c r="I4" t="n">
-        <v>69.27</v>
+        <v>69.1109</v>
       </c>
       <c r="J4" t="n">
         <v>6.1681</v>
@@ -773,16 +773,16 @@
         <v>223.99</v>
       </c>
       <c r="F5" t="n">
-        <v>70.89</v>
+        <v>70.7272</v>
       </c>
       <c r="G5" t="n">
-        <v>76.59999999999999</v>
+        <v>76.42400000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>69.59</v>
+        <v>69.4301</v>
       </c>
       <c r="I5" t="n">
-        <v>76.01000000000001</v>
+        <v>75.83540000000001</v>
       </c>
       <c r="J5" t="n">
         <v>6.0298</v>
@@ -852,16 +852,16 @@
         <v>234.68</v>
       </c>
       <c r="F6" t="n">
-        <v>76.34</v>
+        <v>76.16459999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>78.36</v>
+        <v>78.18000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>74.29000000000001</v>
+        <v>74.1193</v>
       </c>
       <c r="I6" t="n">
-        <v>77.52</v>
+        <v>77.3419</v>
       </c>
       <c r="J6" t="n">
         <v>4.9523</v>
@@ -894,10 +894,10 @@
         <v>16.3626</v>
       </c>
       <c r="U6" t="n">
-        <v>1.9866</v>
+        <v>1.9865</v>
       </c>
       <c r="V6" t="n">
-        <v>5.1546</v>
+        <v>5.1545</v>
       </c>
       <c r="X6" t="n">
         <v>-5.0318</v>
@@ -931,16 +931,16 @@
         <v>272.5</v>
       </c>
       <c r="F7" t="n">
-        <v>82.88</v>
+        <v>82.6896</v>
       </c>
       <c r="G7" t="n">
-        <v>85.03</v>
+        <v>84.8347</v>
       </c>
       <c r="H7" t="n">
-        <v>82.64</v>
+        <v>82.4502</v>
       </c>
       <c r="I7" t="n">
-        <v>84.59</v>
+        <v>84.39570000000001</v>
       </c>
       <c r="J7" t="n">
         <v>4.0231</v>
@@ -976,10 +976,10 @@
         <v>28.8782</v>
       </c>
       <c r="U7" t="n">
-        <v>9.120200000000001</v>
+        <v>9.1203</v>
       </c>
       <c r="V7" t="n">
-        <v>22.1164</v>
+        <v>22.1163</v>
       </c>
       <c r="W7" t="n">
         <v>10.9086</v>
@@ -1022,16 +1022,16 @@
         <v>226.19</v>
       </c>
       <c r="F8" t="n">
-        <v>84.19</v>
+        <v>83.9966</v>
       </c>
       <c r="G8" t="n">
-        <v>84.83</v>
+        <v>84.63509999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>79.86</v>
+        <v>79.67659999999999</v>
       </c>
       <c r="I8" t="n">
-        <v>79.93000000000001</v>
+        <v>79.74639999999999</v>
       </c>
       <c r="J8" t="n">
         <v>3.9836</v>
@@ -1073,7 +1073,7 @@
         <v>5.1572</v>
       </c>
       <c r="W8" t="n">
-        <v>8.4238</v>
+        <v>8.4237</v>
       </c>
       <c r="X8" t="n">
         <v>17.216</v>
@@ -1113,16 +1113,16 @@
         <v>233.86</v>
       </c>
       <c r="F9" t="n">
-        <v>81.67</v>
+        <v>81.4824</v>
       </c>
       <c r="G9" t="n">
-        <v>81.81</v>
+        <v>81.6221</v>
       </c>
       <c r="H9" t="n">
-        <v>76.94</v>
+        <v>76.7633</v>
       </c>
       <c r="I9" t="n">
-        <v>77.54000000000001</v>
+        <v>77.36190000000001</v>
       </c>
       <c r="J9" t="n">
         <v>4.122</v>
@@ -1161,7 +1161,7 @@
         <v>-2.9901</v>
       </c>
       <c r="V9" t="n">
-        <v>0.0258</v>
+        <v>0.0259</v>
       </c>
       <c r="W9" t="n">
         <v>11.9388</v>
@@ -1204,16 +1204,16 @@
         <v>279.29</v>
       </c>
       <c r="F10" t="n">
-        <v>82.09999999999999</v>
+        <v>81.9114</v>
       </c>
       <c r="G10" t="n">
-        <v>83.59999999999999</v>
+        <v>83.408</v>
       </c>
       <c r="H10" t="n">
-        <v>80.63</v>
+        <v>80.4448</v>
       </c>
       <c r="I10" t="n">
-        <v>82.87</v>
+        <v>82.67959999999999</v>
       </c>
       <c r="J10" t="n">
         <v>3.8156</v>
@@ -1249,10 +1249,10 @@
         <v>24.6886</v>
       </c>
       <c r="U10" t="n">
-        <v>6.8739</v>
+        <v>6.8738</v>
       </c>
       <c r="V10" t="n">
-        <v>-2.0333</v>
+        <v>-2.0334</v>
       </c>
       <c r="W10" t="n">
         <v>9.0251</v>
@@ -1295,16 +1295,16 @@
         <v>300.77</v>
       </c>
       <c r="F11" t="n">
-        <v>83.95</v>
+        <v>83.7572</v>
       </c>
       <c r="G11" t="n">
-        <v>85.11</v>
+        <v>84.9145</v>
       </c>
       <c r="H11" t="n">
-        <v>81.39</v>
+        <v>81.203</v>
       </c>
       <c r="I11" t="n">
-        <v>82.58</v>
+        <v>82.3903</v>
       </c>
       <c r="J11" t="n">
         <v>3.2917</v>
@@ -1346,7 +1346,7 @@
         <v>3.3154</v>
       </c>
       <c r="W11" t="n">
-        <v>6.5273</v>
+        <v>6.5274</v>
       </c>
       <c r="X11" t="n">
         <v>-8.079000000000001</v>
@@ -1386,16 +1386,16 @@
         <v>231.42</v>
       </c>
       <c r="F12" t="n">
-        <v>75.12</v>
+        <v>74.9474</v>
       </c>
       <c r="G12" t="n">
-        <v>77.73999999999999</v>
+        <v>77.56140000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>73.91</v>
+        <v>73.7402</v>
       </c>
       <c r="I12" t="n">
-        <v>74.44</v>
+        <v>74.26900000000001</v>
       </c>
       <c r="J12" t="n">
         <v>3.99</v>
@@ -1434,7 +1434,7 @@
         <v>-9.857100000000001</v>
       </c>
       <c r="V12" t="n">
-        <v>-3.9979</v>
+        <v>-3.998</v>
       </c>
       <c r="W12" t="n">
         <v>-11.9991</v>
@@ -1522,13 +1522,13 @@
         <v>1.4943</v>
       </c>
       <c r="U13" t="n">
-        <v>-1.5314</v>
+        <v>-1.3047</v>
       </c>
       <c r="V13" t="n">
-        <v>-11.5482</v>
+        <v>-11.3445</v>
       </c>
       <c r="W13" t="n">
-        <v>-8.2948</v>
+        <v>-8.083600000000001</v>
       </c>
       <c r="X13" t="n">
         <v>0.9901</v>
@@ -1616,10 +1616,10 @@
         <v>2.251</v>
       </c>
       <c r="V14" t="n">
-        <v>-9.2395</v>
+        <v>-9.0306</v>
       </c>
       <c r="W14" t="n">
-        <v>-3.3402</v>
+        <v>-3.1177</v>
       </c>
       <c r="X14" t="n">
         <v>-11.0294</v>
@@ -1707,10 +1707,10 @@
         <v>-4.1628</v>
       </c>
       <c r="V15" t="n">
-        <v>-3.5062</v>
+        <v>-3.284</v>
       </c>
       <c r="W15" t="n">
-        <v>-13.3221</v>
+        <v>-13.1225</v>
       </c>
       <c r="X15" t="n">
         <v>16.8044</v>
@@ -1801,7 +1801,7 @@
         <v>5.307</v>
       </c>
       <c r="W16" t="n">
-        <v>-6.527</v>
+        <v>-6.3118</v>
       </c>
       <c r="X16" t="n">
         <v>-12.2642</v>
@@ -1892,7 +1892,7 @@
         <v>8.071999999999999</v>
       </c>
       <c r="W17" t="n">
-        <v>8.8125</v>
+        <v>9.063000000000001</v>
       </c>
       <c r="X17" t="n">
         <v>-12.9032</v>
@@ -2114,7 +2114,7 @@
         <v>194.65</v>
       </c>
       <c r="F20" t="n">
-        <v>75.53</v>
+        <v>75.54000000000001</v>
       </c>
       <c r="G20" t="n">
         <v>77.45</v>
@@ -2141,10 +2141,10 @@
         <v>38.75</v>
       </c>
       <c r="O20" t="n">
-        <v>38.97</v>
+        <v>38.98</v>
       </c>
       <c r="P20" t="n">
-        <v>37.705</v>
+        <v>37.71</v>
       </c>
       <c r="Q20" t="n">
         <v>38.28</v>
@@ -2184,6 +2184,97 @@
       </c>
       <c r="AC20" t="n">
         <v>-7.3348</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>165.4</v>
+      </c>
+      <c r="C21" t="n">
+        <v>171.88</v>
+      </c>
+      <c r="D21" t="n">
+        <v>150.08</v>
+      </c>
+      <c r="E21" t="n">
+        <v>165.28</v>
+      </c>
+      <c r="F21" t="n">
+        <v>73.7</v>
+      </c>
+      <c r="G21" t="n">
+        <v>74.38</v>
+      </c>
+      <c r="H21" t="n">
+        <v>70.76000000000001</v>
+      </c>
+      <c r="I21" t="n">
+        <v>72.23</v>
+      </c>
+      <c r="J21" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="K21" t="n">
+        <v>5.14</v>
+      </c>
+      <c r="L21" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="M21" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="N21" t="n">
+        <v>39.64</v>
+      </c>
+      <c r="O21" t="n">
+        <v>41.1065</v>
+      </c>
+      <c r="P21" t="n">
+        <v>39.29</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>40.38</v>
+      </c>
+      <c r="R21" t="n">
+        <v>-15.0886</v>
+      </c>
+      <c r="S21" t="n">
+        <v>-24.0267</v>
+      </c>
+      <c r="T21" t="n">
+        <v>-30.1201</v>
+      </c>
+      <c r="U21" t="n">
+        <v>-5.4829</v>
+      </c>
+      <c r="V21" t="n">
+        <v>-6.7519</v>
+      </c>
+      <c r="W21" t="n">
+        <v>-6.4257</v>
+      </c>
+      <c r="X21" t="n">
+        <v>15.1079</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>24.3523</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>29.0323</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>5.4859</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>6.5998</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>5.8176</v>
       </c>
     </row>
   </sheetData>
@@ -2230,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-07-08 23:07
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1713 +568,1713 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>210.62</v>
+        <v>227.06</v>
       </c>
       <c r="C2" t="n">
-        <v>222.19</v>
+        <v>231.02</v>
       </c>
       <c r="D2" t="n">
-        <v>201.69</v>
+        <v>157.56</v>
       </c>
       <c r="E2" t="n">
-        <v>211.44</v>
+        <v>201.68</v>
       </c>
       <c r="F2" t="n">
-        <v>76.68340000000001</v>
+        <v>78.2997</v>
       </c>
       <c r="G2" t="n">
-        <v>78.2897</v>
+        <v>79.15770000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>75.2068</v>
+        <v>66.6366</v>
       </c>
       <c r="I2" t="n">
-        <v>76.09480000000001</v>
+        <v>73.55070000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>5.6442</v>
+        <v>5.1895</v>
       </c>
       <c r="K2" t="n">
-        <v>5.9803</v>
+        <v>7.0281</v>
       </c>
       <c r="L2" t="n">
-        <v>5.2093</v>
+        <v>5.0808</v>
       </c>
       <c r="M2" t="n">
-        <v>5.6245</v>
+        <v>5.8617</v>
       </c>
       <c r="N2" t="n">
-        <v>40.2763</v>
+        <v>39.4299</v>
       </c>
       <c r="O2" t="n">
-        <v>41.1228</v>
+        <v>45.6505</v>
       </c>
       <c r="P2" t="n">
-        <v>39.3314</v>
+        <v>38.9673</v>
       </c>
       <c r="Q2" t="n">
-        <v>40.611</v>
+        <v>41.9988</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>227.06</v>
+        <v>191.54</v>
       </c>
       <c r="C3" t="n">
-        <v>231.02</v>
+        <v>212.99</v>
       </c>
       <c r="D3" t="n">
-        <v>157.56</v>
+        <v>177.3</v>
       </c>
       <c r="E3" t="n">
-        <v>201.68</v>
+        <v>180.65</v>
       </c>
       <c r="F3" t="n">
-        <v>78.2997</v>
+        <v>71.5153</v>
       </c>
       <c r="G3" t="n">
-        <v>79.15770000000001</v>
+        <v>74.5284</v>
       </c>
       <c r="H3" t="n">
-        <v>66.6366</v>
+        <v>68.8415</v>
       </c>
       <c r="I3" t="n">
-        <v>73.55070000000001</v>
+        <v>69.1109</v>
       </c>
       <c r="J3" t="n">
-        <v>5.1895</v>
+        <v>6.1681</v>
       </c>
       <c r="K3" t="n">
-        <v>7.0281</v>
+        <v>6.5734</v>
       </c>
       <c r="L3" t="n">
-        <v>5.0808</v>
+        <v>5.5355</v>
       </c>
       <c r="M3" t="n">
-        <v>5.8617</v>
+        <v>6.4943</v>
       </c>
       <c r="N3" t="n">
-        <v>39.4299</v>
+        <v>43.1209</v>
       </c>
       <c r="O3" t="n">
-        <v>45.6505</v>
+        <v>44.676</v>
       </c>
       <c r="P3" t="n">
-        <v>38.9673</v>
+        <v>41.4082</v>
       </c>
       <c r="Q3" t="n">
-        <v>41.9988</v>
+        <v>44.5382</v>
       </c>
       <c r="R3" t="n">
-        <v>-4.616</v>
+        <v>-10.4274</v>
       </c>
       <c r="U3" t="n">
-        <v>-3.3433</v>
+        <v>-6.0364</v>
       </c>
       <c r="X3" t="n">
-        <v>4.2173</v>
+        <v>10.7921</v>
       </c>
       <c r="AA3" t="n">
-        <v>3.4173</v>
+        <v>6.0464</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>191.54</v>
+        <v>192.3</v>
       </c>
       <c r="C4" t="n">
-        <v>212.99</v>
+        <v>225.63</v>
       </c>
       <c r="D4" t="n">
-        <v>177.3</v>
+        <v>192.3</v>
       </c>
       <c r="E4" t="n">
-        <v>180.65</v>
+        <v>223.99</v>
       </c>
       <c r="F4" t="n">
-        <v>71.5153</v>
+        <v>70.7272</v>
       </c>
       <c r="G4" t="n">
-        <v>74.5284</v>
+        <v>76.42400000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>68.8415</v>
+        <v>69.4301</v>
       </c>
       <c r="I4" t="n">
-        <v>69.1109</v>
+        <v>75.83540000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>6.1681</v>
+        <v>6.0298</v>
       </c>
       <c r="K4" t="n">
-        <v>6.5734</v>
+        <v>6.0298</v>
       </c>
       <c r="L4" t="n">
-        <v>5.5355</v>
+        <v>4.8436</v>
       </c>
       <c r="M4" t="n">
-        <v>6.4943</v>
+        <v>4.9128</v>
       </c>
       <c r="N4" t="n">
-        <v>43.1209</v>
+        <v>43.4851</v>
       </c>
       <c r="O4" t="n">
-        <v>44.676</v>
+        <v>44.302</v>
       </c>
       <c r="P4" t="n">
-        <v>41.4082</v>
+        <v>39.8039</v>
       </c>
       <c r="Q4" t="n">
-        <v>44.5382</v>
+        <v>40.1878</v>
       </c>
       <c r="R4" t="n">
-        <v>-10.4274</v>
+        <v>23.9911</v>
       </c>
       <c r="U4" t="n">
-        <v>-6.0364</v>
+        <v>9.73</v>
       </c>
       <c r="X4" t="n">
-        <v>10.7921</v>
+        <v>-24.3521</v>
       </c>
       <c r="AA4" t="n">
-        <v>6.0464</v>
+        <v>-9.767799999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>192.3</v>
+        <v>222.22</v>
       </c>
       <c r="C5" t="n">
-        <v>225.63</v>
+        <v>242.4</v>
       </c>
       <c r="D5" t="n">
-        <v>192.3</v>
+        <v>214.74</v>
       </c>
       <c r="E5" t="n">
-        <v>223.99</v>
+        <v>234.68</v>
       </c>
       <c r="F5" t="n">
-        <v>70.7272</v>
+        <v>76.16459999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>76.42400000000001</v>
+        <v>78.18000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>69.4301</v>
+        <v>74.1193</v>
       </c>
       <c r="I5" t="n">
-        <v>75.83540000000001</v>
+        <v>77.3419</v>
       </c>
       <c r="J5" t="n">
-        <v>6.0298</v>
+        <v>4.9523</v>
       </c>
       <c r="K5" t="n">
-        <v>6.0298</v>
+        <v>5.0907</v>
       </c>
       <c r="L5" t="n">
-        <v>4.8436</v>
+        <v>4.4877</v>
       </c>
       <c r="M5" t="n">
-        <v>4.9128</v>
+        <v>4.6656</v>
       </c>
       <c r="N5" t="n">
-        <v>43.4851</v>
+        <v>40.0106</v>
       </c>
       <c r="O5" t="n">
-        <v>44.302</v>
+        <v>41.0933</v>
       </c>
       <c r="P5" t="n">
-        <v>39.8039</v>
+        <v>38.9476</v>
       </c>
       <c r="Q5" t="n">
-        <v>40.1878</v>
+        <v>39.4102</v>
       </c>
       <c r="R5" t="n">
-        <v>23.9911</v>
+        <v>4.7725</v>
       </c>
       <c r="S5" t="n">
-        <v>5.9355</v>
+        <v>16.3626</v>
       </c>
       <c r="U5" t="n">
-        <v>9.73</v>
+        <v>1.9865</v>
       </c>
       <c r="V5" t="n">
-        <v>-0.3409</v>
+        <v>5.1545</v>
       </c>
       <c r="X5" t="n">
-        <v>-24.3521</v>
+        <v>-5.0318</v>
       </c>
       <c r="Y5" t="n">
-        <v>-12.6536</v>
+        <v>-20.4053</v>
       </c>
       <c r="AA5" t="n">
-        <v>-9.767799999999999</v>
+        <v>-1.9349</v>
       </c>
       <c r="AB5" t="n">
-        <v>-1.0421</v>
+        <v>-6.1635</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>222.22</v>
+        <v>265.99</v>
       </c>
       <c r="C6" t="n">
-        <v>242.4</v>
+        <v>274.88</v>
       </c>
       <c r="D6" t="n">
-        <v>214.74</v>
+        <v>261.6</v>
       </c>
       <c r="E6" t="n">
-        <v>234.68</v>
+        <v>272.5</v>
       </c>
       <c r="F6" t="n">
-        <v>76.16459999999999</v>
+        <v>82.6896</v>
       </c>
       <c r="G6" t="n">
-        <v>78.18000000000001</v>
+        <v>84.8347</v>
       </c>
       <c r="H6" t="n">
-        <v>74.1193</v>
+        <v>82.4502</v>
       </c>
       <c r="I6" t="n">
-        <v>77.3419</v>
+        <v>84.39570000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>4.9523</v>
+        <v>4.0231</v>
       </c>
       <c r="K6" t="n">
-        <v>5.0907</v>
+        <v>4.122</v>
       </c>
       <c r="L6" t="n">
-        <v>4.4877</v>
+        <v>3.865</v>
       </c>
       <c r="M6" t="n">
-        <v>4.6656</v>
+        <v>3.9045</v>
       </c>
       <c r="N6" t="n">
-        <v>40.0106</v>
+        <v>36.6641</v>
       </c>
       <c r="O6" t="n">
-        <v>41.0933</v>
+        <v>36.7723</v>
       </c>
       <c r="P6" t="n">
-        <v>38.9476</v>
+        <v>35.5814</v>
       </c>
       <c r="Q6" t="n">
-        <v>39.4102</v>
+        <v>35.7389</v>
       </c>
       <c r="R6" t="n">
-        <v>4.7725</v>
+        <v>16.1156</v>
       </c>
       <c r="S6" t="n">
-        <v>16.3626</v>
+        <v>50.8442</v>
       </c>
       <c r="U6" t="n">
-        <v>1.9865</v>
+        <v>9.1203</v>
       </c>
       <c r="V6" t="n">
-        <v>5.1545</v>
+        <v>22.1163</v>
       </c>
       <c r="X6" t="n">
-        <v>-5.0318</v>
+        <v>-16.313</v>
       </c>
       <c r="Y6" t="n">
-        <v>-20.4053</v>
+        <v>-39.878</v>
       </c>
       <c r="AA6" t="n">
-        <v>-1.9349</v>
+        <v>-9.3156</v>
       </c>
       <c r="AB6" t="n">
-        <v>-6.1635</v>
+        <v>-19.7567</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>265.99</v>
+        <v>267.13</v>
       </c>
       <c r="C7" t="n">
-        <v>274.88</v>
+        <v>274.93</v>
       </c>
       <c r="D7" t="n">
-        <v>261.6</v>
+        <v>226</v>
       </c>
       <c r="E7" t="n">
-        <v>272.5</v>
+        <v>226.19</v>
       </c>
       <c r="F7" t="n">
-        <v>82.6896</v>
+        <v>83.9966</v>
       </c>
       <c r="G7" t="n">
-        <v>84.8347</v>
+        <v>84.63509999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>82.4502</v>
+        <v>79.67659999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>84.39570000000001</v>
+        <v>79.74639999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>4.0231</v>
+        <v>3.9836</v>
       </c>
       <c r="K7" t="n">
-        <v>4.122</v>
+        <v>4.5965</v>
       </c>
       <c r="L7" t="n">
         <v>3.865</v>
       </c>
       <c r="M7" t="n">
-        <v>3.9045</v>
+        <v>4.5767</v>
       </c>
       <c r="N7" t="n">
-        <v>36.6641</v>
+        <v>35.9652</v>
       </c>
       <c r="O7" t="n">
-        <v>36.7723</v>
+        <v>37.7861</v>
       </c>
       <c r="P7" t="n">
-        <v>35.5814</v>
+        <v>35.6896</v>
       </c>
       <c r="Q7" t="n">
-        <v>35.7389</v>
+        <v>37.7468</v>
       </c>
       <c r="R7" t="n">
-        <v>16.1156</v>
+        <v>-16.9945</v>
       </c>
       <c r="S7" t="n">
-        <v>50.8442</v>
+        <v>0.9822</v>
       </c>
       <c r="T7" t="n">
-        <v>28.8782</v>
+        <v>12.1529</v>
       </c>
       <c r="U7" t="n">
-        <v>9.1203</v>
+        <v>-5.5089</v>
       </c>
       <c r="V7" t="n">
-        <v>22.1163</v>
+        <v>5.1572</v>
       </c>
       <c r="W7" t="n">
-        <v>10.9086</v>
+        <v>8.4237</v>
       </c>
       <c r="X7" t="n">
-        <v>-16.313</v>
+        <v>17.216</v>
       </c>
       <c r="Y7" t="n">
-        <v>-39.878</v>
+        <v>-6.8413</v>
       </c>
       <c r="Z7" t="n">
-        <v>-30.5805</v>
+        <v>-21.922</v>
       </c>
       <c r="AA7" t="n">
-        <v>-9.3156</v>
+        <v>5.6182</v>
       </c>
       <c r="AB7" t="n">
-        <v>-19.7567</v>
+        <v>-6.074</v>
       </c>
       <c r="AC7" t="n">
-        <v>-11.997</v>
+        <v>-10.1241</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>267.13</v>
+        <v>247.42</v>
       </c>
       <c r="C8" t="n">
-        <v>274.93</v>
+        <v>259.79</v>
       </c>
       <c r="D8" t="n">
-        <v>226</v>
+        <v>233.3</v>
       </c>
       <c r="E8" t="n">
-        <v>226.19</v>
+        <v>233.86</v>
       </c>
       <c r="F8" t="n">
-        <v>83.9966</v>
+        <v>81.4824</v>
       </c>
       <c r="G8" t="n">
-        <v>84.63509999999999</v>
+        <v>81.6221</v>
       </c>
       <c r="H8" t="n">
-        <v>79.67659999999999</v>
+        <v>76.7633</v>
       </c>
       <c r="I8" t="n">
-        <v>79.74639999999999</v>
+        <v>77.36190000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>3.9836</v>
+        <v>4.122</v>
       </c>
       <c r="K8" t="n">
-        <v>4.5965</v>
+        <v>4.4086</v>
       </c>
       <c r="L8" t="n">
-        <v>3.865</v>
+        <v>3.8749</v>
       </c>
       <c r="M8" t="n">
-        <v>4.5767</v>
+        <v>4.4086</v>
       </c>
       <c r="N8" t="n">
-        <v>35.9652</v>
+        <v>36.9397</v>
       </c>
       <c r="O8" t="n">
-        <v>37.7861</v>
+        <v>39.1641</v>
       </c>
       <c r="P8" t="n">
-        <v>35.6896</v>
+        <v>36.8708</v>
       </c>
       <c r="Q8" t="n">
-        <v>37.7468</v>
+        <v>38.8984</v>
       </c>
       <c r="R8" t="n">
-        <v>-16.9945</v>
+        <v>3.391</v>
       </c>
       <c r="S8" t="n">
-        <v>0.9822</v>
+        <v>-0.3494</v>
       </c>
       <c r="T8" t="n">
-        <v>12.1529</v>
+        <v>29.4547</v>
       </c>
       <c r="U8" t="n">
-        <v>-5.5089</v>
+        <v>-2.9901</v>
       </c>
       <c r="V8" t="n">
-        <v>5.1572</v>
+        <v>0.0259</v>
       </c>
       <c r="W8" t="n">
-        <v>8.4237</v>
+        <v>11.9388</v>
       </c>
       <c r="X8" t="n">
-        <v>17.216</v>
+        <v>-3.673</v>
       </c>
       <c r="Y8" t="n">
-        <v>-6.8413</v>
+        <v>-5.5084</v>
       </c>
       <c r="Z8" t="n">
-        <v>-21.922</v>
+        <v>-32.1159</v>
       </c>
       <c r="AA8" t="n">
-        <v>5.6182</v>
+        <v>3.0509</v>
       </c>
       <c r="AB8" t="n">
-        <v>-6.074</v>
+        <v>-1.2986</v>
       </c>
       <c r="AC8" t="n">
-        <v>-10.1241</v>
+        <v>-12.6628</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>247.42</v>
+        <v>266.04</v>
       </c>
       <c r="C9" t="n">
-        <v>259.79</v>
+        <v>286.15</v>
       </c>
       <c r="D9" t="n">
-        <v>233.3</v>
+        <v>265</v>
       </c>
       <c r="E9" t="n">
-        <v>233.86</v>
+        <v>279.29</v>
       </c>
       <c r="F9" t="n">
-        <v>81.4824</v>
+        <v>81.9114</v>
       </c>
       <c r="G9" t="n">
-        <v>81.6221</v>
+        <v>83.408</v>
       </c>
       <c r="H9" t="n">
-        <v>76.7633</v>
+        <v>80.4448</v>
       </c>
       <c r="I9" t="n">
-        <v>77.36190000000001</v>
+        <v>82.67959999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>4.122</v>
+        <v>3.8156</v>
       </c>
       <c r="K9" t="n">
-        <v>4.4086</v>
+        <v>3.8254</v>
       </c>
       <c r="L9" t="n">
-        <v>3.8749</v>
+        <v>3.4103</v>
       </c>
       <c r="M9" t="n">
-        <v>4.4086</v>
+        <v>3.5487</v>
       </c>
       <c r="N9" t="n">
-        <v>36.9397</v>
+        <v>36.6149</v>
       </c>
       <c r="O9" t="n">
-        <v>39.1641</v>
+        <v>37.3531</v>
       </c>
       <c r="P9" t="n">
-        <v>36.8708</v>
+        <v>35.857</v>
       </c>
       <c r="Q9" t="n">
-        <v>38.8984</v>
+        <v>36.1719</v>
       </c>
       <c r="R9" t="n">
-        <v>3.391</v>
+        <v>19.4262</v>
       </c>
       <c r="S9" t="n">
-        <v>-0.3494</v>
+        <v>2.4917</v>
       </c>
       <c r="T9" t="n">
-        <v>29.4547</v>
+        <v>24.6886</v>
       </c>
       <c r="U9" t="n">
-        <v>-2.9901</v>
+        <v>6.8738</v>
       </c>
       <c r="V9" t="n">
-        <v>0.0259</v>
+        <v>-2.0334</v>
       </c>
       <c r="W9" t="n">
-        <v>11.9388</v>
+        <v>9.0251</v>
       </c>
       <c r="X9" t="n">
-        <v>-3.673</v>
+        <v>-19.5051</v>
       </c>
       <c r="Y9" t="n">
-        <v>-5.5084</v>
+        <v>-9.1126</v>
       </c>
       <c r="Z9" t="n">
-        <v>-32.1159</v>
+        <v>-27.7662</v>
       </c>
       <c r="AA9" t="n">
-        <v>3.0509</v>
+        <v>-7.0093</v>
       </c>
       <c r="AB9" t="n">
-        <v>-1.2986</v>
+        <v>1.2116</v>
       </c>
       <c r="AC9" t="n">
-        <v>-12.6628</v>
+        <v>-9.992800000000001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>266.04</v>
+        <v>299.26</v>
       </c>
       <c r="C10" t="n">
-        <v>286.15</v>
+        <v>302</v>
       </c>
       <c r="D10" t="n">
-        <v>265</v>
+        <v>286.24</v>
       </c>
       <c r="E10" t="n">
-        <v>279.29</v>
+        <v>300.77</v>
       </c>
       <c r="F10" t="n">
-        <v>81.9114</v>
+        <v>83.7572</v>
       </c>
       <c r="G10" t="n">
-        <v>83.408</v>
+        <v>84.9145</v>
       </c>
       <c r="H10" t="n">
-        <v>80.4448</v>
+        <v>81.203</v>
       </c>
       <c r="I10" t="n">
-        <v>82.67959999999999</v>
+        <v>82.3903</v>
       </c>
       <c r="J10" t="n">
-        <v>3.8156</v>
+        <v>3.2917</v>
       </c>
       <c r="K10" t="n">
-        <v>3.8254</v>
+        <v>3.4498</v>
       </c>
       <c r="L10" t="n">
-        <v>3.4103</v>
+        <v>3.2521</v>
       </c>
       <c r="M10" t="n">
-        <v>3.5487</v>
+        <v>3.262</v>
       </c>
       <c r="N10" t="n">
-        <v>36.6149</v>
+        <v>35.7389</v>
       </c>
       <c r="O10" t="n">
-        <v>37.3531</v>
+        <v>36.8511</v>
       </c>
       <c r="P10" t="n">
-        <v>35.857</v>
+        <v>35.2369</v>
       </c>
       <c r="Q10" t="n">
-        <v>36.1719</v>
+        <v>36.3491</v>
       </c>
       <c r="R10" t="n">
-        <v>19.4262</v>
+        <v>7.6909</v>
       </c>
       <c r="S10" t="n">
-        <v>2.4917</v>
+        <v>32.9723</v>
       </c>
       <c r="T10" t="n">
-        <v>24.6886</v>
+        <v>28.1618</v>
       </c>
       <c r="U10" t="n">
-        <v>6.8738</v>
+        <v>-0.3499</v>
       </c>
       <c r="V10" t="n">
-        <v>-2.0334</v>
+        <v>3.3154</v>
       </c>
       <c r="W10" t="n">
-        <v>9.0251</v>
+        <v>6.5274</v>
       </c>
       <c r="X10" t="n">
-        <v>-19.5051</v>
+        <v>-8.079000000000001</v>
       </c>
       <c r="Y10" t="n">
-        <v>-9.1126</v>
+        <v>-28.7259</v>
       </c>
       <c r="Z10" t="n">
-        <v>-27.7662</v>
+        <v>-30.084</v>
       </c>
       <c r="AA10" t="n">
-        <v>-7.0093</v>
+        <v>0.4899</v>
       </c>
       <c r="AB10" t="n">
-        <v>1.2116</v>
+        <v>-3.7028</v>
       </c>
       <c r="AC10" t="n">
-        <v>-9.992800000000001</v>
+        <v>-7.7673</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>299.26</v>
+        <v>236</v>
       </c>
       <c r="C11" t="n">
-        <v>302</v>
+        <v>252.98</v>
       </c>
       <c r="D11" t="n">
-        <v>286.24</v>
+        <v>223</v>
       </c>
       <c r="E11" t="n">
-        <v>300.77</v>
+        <v>231.42</v>
       </c>
       <c r="F11" t="n">
-        <v>83.7572</v>
+        <v>74.9474</v>
       </c>
       <c r="G11" t="n">
-        <v>84.9145</v>
+        <v>77.56140000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>81.203</v>
+        <v>73.7402</v>
       </c>
       <c r="I11" t="n">
-        <v>82.3903</v>
+        <v>74.26900000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>3.2917</v>
+        <v>3.99</v>
       </c>
       <c r="K11" t="n">
-        <v>3.4498</v>
+        <v>4.13</v>
       </c>
       <c r="L11" t="n">
-        <v>3.2521</v>
+        <v>3.8</v>
       </c>
       <c r="M11" t="n">
-        <v>3.262</v>
+        <v>4.04</v>
       </c>
       <c r="N11" t="n">
-        <v>35.7389</v>
+        <v>39.6267</v>
       </c>
       <c r="O11" t="n">
-        <v>36.8511</v>
+        <v>40.1582</v>
       </c>
       <c r="P11" t="n">
-        <v>35.2369</v>
+        <v>38.4653</v>
       </c>
       <c r="Q11" t="n">
-        <v>36.3491</v>
+        <v>39.922</v>
       </c>
       <c r="R11" t="n">
-        <v>7.6909</v>
+        <v>-23.0575</v>
       </c>
       <c r="S11" t="n">
-        <v>32.9723</v>
+        <v>-1.0434</v>
       </c>
       <c r="T11" t="n">
-        <v>28.1618</v>
+        <v>-15.0752</v>
       </c>
       <c r="U11" t="n">
-        <v>-0.3499</v>
+        <v>-9.857100000000001</v>
       </c>
       <c r="V11" t="n">
-        <v>3.3154</v>
+        <v>-3.998</v>
       </c>
       <c r="W11" t="n">
-        <v>6.5274</v>
+        <v>-11.9991</v>
       </c>
       <c r="X11" t="n">
-        <v>-8.079000000000001</v>
+        <v>23.8504</v>
       </c>
       <c r="Y11" t="n">
-        <v>-28.7259</v>
+        <v>-8.360900000000001</v>
       </c>
       <c r="Z11" t="n">
-        <v>-30.084</v>
+        <v>3.4704</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.4899</v>
+        <v>9.8294</v>
       </c>
       <c r="AB11" t="n">
-        <v>-3.7028</v>
+        <v>2.6315</v>
       </c>
       <c r="AC11" t="n">
-        <v>-7.7673</v>
+        <v>11.7046</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>236</v>
+        <v>233.11</v>
       </c>
       <c r="C12" t="n">
-        <v>252.98</v>
+        <v>237</v>
       </c>
       <c r="D12" t="n">
-        <v>223</v>
+        <v>211.13</v>
       </c>
       <c r="E12" t="n">
-        <v>231.42</v>
+        <v>229.57</v>
       </c>
       <c r="F12" t="n">
-        <v>74.9474</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>77.56140000000001</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>73.7402</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>74.26900000000001</v>
+        <v>73.3</v>
       </c>
       <c r="J12" t="n">
-        <v>3.99</v>
+        <v>4</v>
       </c>
       <c r="K12" t="n">
-        <v>4.13</v>
+        <v>4.39</v>
       </c>
       <c r="L12" t="n">
-        <v>3.8</v>
+        <v>3.92</v>
       </c>
       <c r="M12" t="n">
-        <v>4.04</v>
+        <v>4.08</v>
       </c>
       <c r="N12" t="n">
-        <v>39.6267</v>
+        <v>39.66</v>
       </c>
       <c r="O12" t="n">
-        <v>40.1582</v>
+        <v>41.49</v>
       </c>
       <c r="P12" t="n">
-        <v>38.4653</v>
+        <v>38.9</v>
       </c>
       <c r="Q12" t="n">
-        <v>39.922</v>
+        <v>40.45</v>
       </c>
       <c r="R12" t="n">
-        <v>-23.0575</v>
+        <v>-0.7994</v>
       </c>
       <c r="S12" t="n">
-        <v>-1.0434</v>
+        <v>-17.8023</v>
       </c>
       <c r="T12" t="n">
-        <v>-15.0752</v>
+        <v>1.4943</v>
       </c>
       <c r="U12" t="n">
-        <v>-9.857100000000001</v>
+        <v>-1.3047</v>
       </c>
       <c r="V12" t="n">
-        <v>-3.998</v>
+        <v>-11.3445</v>
       </c>
       <c r="W12" t="n">
-        <v>-11.9991</v>
+        <v>-8.083600000000001</v>
       </c>
       <c r="X12" t="n">
-        <v>23.8504</v>
+        <v>0.9901</v>
       </c>
       <c r="Y12" t="n">
-        <v>-8.360900000000001</v>
+        <v>14.9717</v>
       </c>
       <c r="Z12" t="n">
-        <v>3.4704</v>
+        <v>-10.8528</v>
       </c>
       <c r="AA12" t="n">
-        <v>9.8294</v>
+        <v>1.3226</v>
       </c>
       <c r="AB12" t="n">
-        <v>2.6315</v>
+        <v>11.8271</v>
       </c>
       <c r="AC12" t="n">
-        <v>11.7046</v>
+        <v>7.1614</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>233.11</v>
+        <v>268.05</v>
       </c>
       <c r="C13" t="n">
-        <v>237</v>
+        <v>268.4</v>
       </c>
       <c r="D13" t="n">
-        <v>211.13</v>
+        <v>225.74</v>
       </c>
       <c r="E13" t="n">
-        <v>229.57</v>
+        <v>252.61</v>
       </c>
       <c r="F13" t="n">
-        <v>74.79000000000001</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>76.18000000000001</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>71.34999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>73.3</v>
+        <v>74.95</v>
       </c>
       <c r="J13" t="n">
-        <v>4</v>
+        <v>3.38</v>
       </c>
       <c r="K13" t="n">
-        <v>4.39</v>
+        <v>4.15</v>
       </c>
       <c r="L13" t="n">
-        <v>3.92</v>
+        <v>3.37</v>
       </c>
       <c r="M13" t="n">
-        <v>4.08</v>
+        <v>3.63</v>
       </c>
       <c r="N13" t="n">
-        <v>39.66</v>
+        <v>37.87</v>
       </c>
       <c r="O13" t="n">
-        <v>41.49</v>
+        <v>41.37</v>
       </c>
       <c r="P13" t="n">
-        <v>38.9</v>
+        <v>37.71</v>
       </c>
       <c r="Q13" t="n">
-        <v>40.45</v>
+        <v>39.47</v>
       </c>
       <c r="R13" t="n">
-        <v>-0.7994</v>
+        <v>10.0362</v>
       </c>
       <c r="S13" t="n">
-        <v>-17.8023</v>
+        <v>-16.0122</v>
       </c>
       <c r="T13" t="n">
-        <v>1.4943</v>
+        <v>8.0176</v>
       </c>
       <c r="U13" t="n">
-        <v>-1.3047</v>
+        <v>2.251</v>
       </c>
       <c r="V13" t="n">
-        <v>-11.3445</v>
+        <v>-9.0306</v>
       </c>
       <c r="W13" t="n">
-        <v>-8.083600000000001</v>
+        <v>-3.1177</v>
       </c>
       <c r="X13" t="n">
-        <v>0.9901</v>
+        <v>-11.0294</v>
       </c>
       <c r="Y13" t="n">
-        <v>14.9717</v>
+        <v>11.2814</v>
       </c>
       <c r="Z13" t="n">
-        <v>-10.8528</v>
+        <v>-17.6609</v>
       </c>
       <c r="AA13" t="n">
-        <v>1.3226</v>
+        <v>-2.4227</v>
       </c>
       <c r="AB13" t="n">
-        <v>11.8271</v>
+        <v>8.585900000000001</v>
       </c>
       <c r="AC13" t="n">
-        <v>7.1614</v>
+        <v>1.4695</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>268.05</v>
+        <v>226.24</v>
       </c>
       <c r="C14" t="n">
-        <v>268.4</v>
+        <v>231.25</v>
       </c>
       <c r="D14" t="n">
-        <v>225.74</v>
+        <v>212.1</v>
       </c>
       <c r="E14" t="n">
-        <v>252.61</v>
+        <v>215.6</v>
       </c>
       <c r="F14" t="n">
-        <v>77.95999999999999</v>
+        <v>72.09</v>
       </c>
       <c r="G14" t="n">
-        <v>78.23999999999999</v>
+        <v>74.69</v>
       </c>
       <c r="H14" t="n">
-        <v>71.59999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="I14" t="n">
-        <v>74.95</v>
+        <v>71.83</v>
       </c>
       <c r="J14" t="n">
-        <v>3.38</v>
+        <v>4.04</v>
       </c>
       <c r="K14" t="n">
-        <v>4.15</v>
+        <v>4.25</v>
       </c>
       <c r="L14" t="n">
-        <v>3.37</v>
+        <v>3.95</v>
       </c>
       <c r="M14" t="n">
-        <v>3.63</v>
+        <v>4.24</v>
       </c>
       <c r="N14" t="n">
-        <v>37.87</v>
+        <v>41.08</v>
       </c>
       <c r="O14" t="n">
-        <v>41.37</v>
+        <v>41.79</v>
       </c>
       <c r="P14" t="n">
-        <v>37.71</v>
+        <v>39.69</v>
       </c>
       <c r="Q14" t="n">
-        <v>39.47</v>
+        <v>41.31</v>
       </c>
       <c r="R14" t="n">
-        <v>10.0362</v>
+        <v>-14.651</v>
       </c>
       <c r="S14" t="n">
-        <v>-16.0122</v>
+        <v>-6.8361</v>
       </c>
       <c r="T14" t="n">
-        <v>8.0176</v>
+        <v>-22.8043</v>
       </c>
       <c r="U14" t="n">
-        <v>2.251</v>
+        <v>-4.1628</v>
       </c>
       <c r="V14" t="n">
-        <v>-9.0306</v>
+        <v>-3.284</v>
       </c>
       <c r="W14" t="n">
-        <v>-3.1177</v>
+        <v>-13.1225</v>
       </c>
       <c r="X14" t="n">
-        <v>-11.0294</v>
+        <v>16.8044</v>
       </c>
       <c r="Y14" t="n">
-        <v>11.2814</v>
+        <v>4.9505</v>
       </c>
       <c r="Z14" t="n">
-        <v>-17.6609</v>
+        <v>19.4804</v>
       </c>
       <c r="AA14" t="n">
-        <v>-2.4227</v>
+        <v>4.6618</v>
       </c>
       <c r="AB14" t="n">
-        <v>8.585900000000001</v>
+        <v>3.4768</v>
       </c>
       <c r="AC14" t="n">
-        <v>1.4695</v>
+        <v>14.2047</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>226.24</v>
+        <v>216.36</v>
       </c>
       <c r="C15" t="n">
-        <v>231.25</v>
+        <v>238.65</v>
       </c>
       <c r="D15" t="n">
-        <v>212.1</v>
+        <v>192.3</v>
       </c>
       <c r="E15" t="n">
-        <v>215.6</v>
+        <v>236.52</v>
       </c>
       <c r="F15" t="n">
-        <v>72.09</v>
+        <v>74.12</v>
       </c>
       <c r="G15" t="n">
-        <v>74.69</v>
+        <v>77.38</v>
       </c>
       <c r="H15" t="n">
-        <v>70.72</v>
+        <v>71.45</v>
       </c>
       <c r="I15" t="n">
-        <v>71.83</v>
+        <v>77.19</v>
       </c>
       <c r="J15" t="n">
-        <v>4.04</v>
+        <v>4.16</v>
       </c>
       <c r="K15" t="n">
-        <v>4.25</v>
+        <v>4.63</v>
       </c>
       <c r="L15" t="n">
-        <v>3.95</v>
+        <v>3.7</v>
       </c>
       <c r="M15" t="n">
-        <v>4.24</v>
+        <v>3.72</v>
       </c>
       <c r="N15" t="n">
-        <v>41.08</v>
+        <v>39.91</v>
       </c>
       <c r="O15" t="n">
-        <v>41.79</v>
+        <v>41.43</v>
       </c>
       <c r="P15" t="n">
-        <v>39.69</v>
+        <v>38.08</v>
       </c>
       <c r="Q15" t="n">
-        <v>41.31</v>
+        <v>38.16</v>
       </c>
       <c r="R15" t="n">
-        <v>-14.651</v>
+        <v>9.703200000000001</v>
       </c>
       <c r="S15" t="n">
-        <v>-6.8361</v>
+        <v>3.0274</v>
       </c>
       <c r="T15" t="n">
-        <v>-22.8043</v>
+        <v>-21.3618</v>
       </c>
       <c r="U15" t="n">
-        <v>-4.1628</v>
+        <v>7.4621</v>
       </c>
       <c r="V15" t="n">
-        <v>-3.284</v>
+        <v>5.307</v>
       </c>
       <c r="W15" t="n">
-        <v>-13.1225</v>
+        <v>-6.3118</v>
       </c>
       <c r="X15" t="n">
-        <v>16.8044</v>
+        <v>-12.2642</v>
       </c>
       <c r="Y15" t="n">
-        <v>4.9505</v>
+        <v>-8.823499999999999</v>
       </c>
       <c r="Z15" t="n">
-        <v>19.4804</v>
+        <v>14.0405</v>
       </c>
       <c r="AA15" t="n">
-        <v>4.6618</v>
+        <v>-7.6253</v>
       </c>
       <c r="AB15" t="n">
-        <v>3.4768</v>
+        <v>-5.6613</v>
       </c>
       <c r="AC15" t="n">
-        <v>14.2047</v>
+        <v>4.982</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>216.36</v>
+        <v>241.45</v>
       </c>
       <c r="C16" t="n">
-        <v>238.65</v>
+        <v>272</v>
       </c>
       <c r="D16" t="n">
-        <v>192.3</v>
+        <v>240.59</v>
       </c>
       <c r="E16" t="n">
-        <v>236.52</v>
+        <v>266.71</v>
       </c>
       <c r="F16" t="n">
-        <v>74.12</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>77.38</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="H16" t="n">
-        <v>71.45</v>
+        <v>77.15000000000001</v>
       </c>
       <c r="I16" t="n">
-        <v>77.19</v>
+        <v>81</v>
       </c>
       <c r="J16" t="n">
-        <v>4.16</v>
+        <v>3.66</v>
       </c>
       <c r="K16" t="n">
-        <v>4.63</v>
+        <v>3.68</v>
       </c>
       <c r="L16" t="n">
-        <v>3.7</v>
+        <v>3.17</v>
       </c>
       <c r="M16" t="n">
-        <v>3.72</v>
+        <v>3.24</v>
       </c>
       <c r="N16" t="n">
-        <v>39.91</v>
+        <v>38.16</v>
       </c>
       <c r="O16" t="n">
-        <v>41.43</v>
+        <v>38.2</v>
       </c>
       <c r="P16" t="n">
-        <v>38.08</v>
+        <v>36.03</v>
       </c>
       <c r="Q16" t="n">
-        <v>38.16</v>
+        <v>36.31</v>
       </c>
       <c r="R16" t="n">
-        <v>9.703200000000001</v>
+        <v>12.7642</v>
       </c>
       <c r="S16" t="n">
-        <v>3.0274</v>
+        <v>5.5817</v>
       </c>
       <c r="T16" t="n">
-        <v>-21.3618</v>
+        <v>15.2493</v>
       </c>
       <c r="U16" t="n">
-        <v>7.4621</v>
+        <v>4.9359</v>
       </c>
       <c r="V16" t="n">
-        <v>5.307</v>
+        <v>8.071999999999999</v>
       </c>
       <c r="W16" t="n">
-        <v>-6.3118</v>
+        <v>9.063000000000001</v>
       </c>
       <c r="X16" t="n">
-        <v>-12.2642</v>
+        <v>-12.9032</v>
       </c>
       <c r="Y16" t="n">
-        <v>-8.823499999999999</v>
+        <v>-10.7438</v>
       </c>
       <c r="Z16" t="n">
-        <v>14.0405</v>
+        <v>-19.802</v>
       </c>
       <c r="AA16" t="n">
-        <v>-7.6253</v>
+        <v>-4.848</v>
       </c>
       <c r="AB16" t="n">
-        <v>-5.6613</v>
+        <v>-8.0061</v>
       </c>
       <c r="AC16" t="n">
-        <v>4.982</v>
+        <v>-9.047599999999999</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>241.45</v>
+        <v>237.79</v>
       </c>
       <c r="C17" t="n">
-        <v>272</v>
+        <v>246.47</v>
       </c>
       <c r="D17" t="n">
-        <v>240.59</v>
+        <v>215.38</v>
       </c>
       <c r="E17" t="n">
-        <v>266.71</v>
+        <v>217.55</v>
       </c>
       <c r="F17" t="n">
-        <v>77.23999999999999</v>
+        <v>78.72</v>
       </c>
       <c r="G17" t="n">
-        <v>81.54000000000001</v>
+        <v>79.64</v>
       </c>
       <c r="H17" t="n">
-        <v>77.15000000000001</v>
+        <v>77.23</v>
       </c>
       <c r="I17" t="n">
-        <v>81</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>3.66</v>
+        <v>3.59</v>
       </c>
       <c r="K17" t="n">
-        <v>3.68</v>
+        <v>3.89</v>
       </c>
       <c r="L17" t="n">
-        <v>3.17</v>
+        <v>3.51</v>
       </c>
       <c r="M17" t="n">
-        <v>3.24</v>
+        <v>3.86</v>
       </c>
       <c r="N17" t="n">
-        <v>38.16</v>
+        <v>37.31</v>
       </c>
       <c r="O17" t="n">
-        <v>38.2</v>
+        <v>37.98</v>
       </c>
       <c r="P17" t="n">
-        <v>36.03</v>
+        <v>36.9</v>
       </c>
       <c r="Q17" t="n">
-        <v>36.31</v>
+        <v>37.88</v>
       </c>
       <c r="R17" t="n">
-        <v>12.7642</v>
+        <v>-18.432</v>
       </c>
       <c r="S17" t="n">
-        <v>5.5817</v>
+        <v>0.9045</v>
       </c>
       <c r="T17" t="n">
-        <v>15.2493</v>
+        <v>-5.2359</v>
       </c>
       <c r="U17" t="n">
-        <v>4.9359</v>
+        <v>-4.3704</v>
       </c>
       <c r="V17" t="n">
-        <v>8.071999999999999</v>
+        <v>7.838</v>
       </c>
       <c r="W17" t="n">
-        <v>9.063000000000001</v>
+        <v>5.6753</v>
       </c>
       <c r="X17" t="n">
-        <v>-12.9032</v>
+        <v>19.1358</v>
       </c>
       <c r="Y17" t="n">
-        <v>-10.7438</v>
+        <v>-8.962300000000001</v>
       </c>
       <c r="Z17" t="n">
-        <v>-19.802</v>
+        <v>-5.3922</v>
       </c>
       <c r="AA17" t="n">
-        <v>-4.848</v>
+        <v>4.3239</v>
       </c>
       <c r="AB17" t="n">
-        <v>-8.0061</v>
+        <v>-8.303100000000001</v>
       </c>
       <c r="AC17" t="n">
-        <v>-9.047599999999999</v>
+        <v>-6.3535</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>237.79</v>
+        <v>219.23</v>
       </c>
       <c r="C18" t="n">
-        <v>246.47</v>
+        <v>226.13</v>
       </c>
       <c r="D18" t="n">
-        <v>215.38</v>
+        <v>168.88</v>
       </c>
       <c r="E18" t="n">
-        <v>217.55</v>
+        <v>181.47</v>
       </c>
       <c r="F18" t="n">
-        <v>78.72</v>
+        <v>77.45</v>
       </c>
       <c r="G18" t="n">
-        <v>79.64</v>
+        <v>79.14</v>
       </c>
       <c r="H18" t="n">
-        <v>77.23</v>
+        <v>71.72</v>
       </c>
       <c r="I18" t="n">
-        <v>77.45999999999999</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="J18" t="n">
-        <v>3.59</v>
+        <v>3.84</v>
       </c>
       <c r="K18" t="n">
-        <v>3.89</v>
+        <v>4.74</v>
       </c>
       <c r="L18" t="n">
-        <v>3.51</v>
+        <v>3.71</v>
       </c>
       <c r="M18" t="n">
-        <v>3.86</v>
+        <v>4.51</v>
       </c>
       <c r="N18" t="n">
-        <v>37.31</v>
+        <v>37.91</v>
       </c>
       <c r="O18" t="n">
-        <v>37.98</v>
+        <v>40.72</v>
       </c>
       <c r="P18" t="n">
-        <v>36.9</v>
+        <v>37.08</v>
       </c>
       <c r="Q18" t="n">
-        <v>37.88</v>
+        <v>39.95</v>
       </c>
       <c r="R18" t="n">
-        <v>-18.432</v>
+        <v>-16.5847</v>
       </c>
       <c r="S18" t="n">
-        <v>0.9045</v>
+        <v>-23.275</v>
       </c>
       <c r="T18" t="n">
-        <v>-5.2359</v>
+        <v>-28.162</v>
       </c>
       <c r="U18" t="n">
-        <v>-4.3704</v>
+        <v>-5.306</v>
       </c>
       <c r="V18" t="n">
-        <v>7.838</v>
+        <v>-4.9747</v>
       </c>
       <c r="W18" t="n">
-        <v>5.6753</v>
+        <v>-2.1348</v>
       </c>
       <c r="X18" t="n">
-        <v>19.1358</v>
+        <v>16.8394</v>
       </c>
       <c r="Y18" t="n">
-        <v>-8.962300000000001</v>
+        <v>21.2366</v>
       </c>
       <c r="Z18" t="n">
-        <v>-5.3922</v>
+        <v>24.2424</v>
       </c>
       <c r="AA18" t="n">
-        <v>4.3239</v>
+        <v>5.4646</v>
       </c>
       <c r="AB18" t="n">
-        <v>-8.303100000000001</v>
+        <v>4.6908</v>
       </c>
       <c r="AC18" t="n">
-        <v>-6.3535</v>
+        <v>1.2161</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>219.23</v>
+        <v>197.21</v>
       </c>
       <c r="C19" t="n">
-        <v>226.13</v>
+        <v>210.8</v>
       </c>
       <c r="D19" t="n">
-        <v>168.88</v>
+        <v>194.22</v>
       </c>
       <c r="E19" t="n">
-        <v>181.47</v>
+        <v>194.65</v>
       </c>
       <c r="F19" t="n">
+        <v>75.54000000000001</v>
+      </c>
+      <c r="G19" t="n">
         <v>77.45</v>
       </c>
-      <c r="G19" t="n">
-        <v>79.14</v>
-      </c>
       <c r="H19" t="n">
-        <v>71.72</v>
+        <v>75.11</v>
       </c>
       <c r="I19" t="n">
-        <v>73.34999999999999</v>
+        <v>76.42</v>
       </c>
       <c r="J19" t="n">
-        <v>3.84</v>
+        <v>4.11</v>
       </c>
       <c r="K19" t="n">
-        <v>4.74</v>
+        <v>4.18</v>
       </c>
       <c r="L19" t="n">
-        <v>3.71</v>
+        <v>3.77</v>
       </c>
       <c r="M19" t="n">
-        <v>4.51</v>
+        <v>4.17</v>
       </c>
       <c r="N19" t="n">
-        <v>37.91</v>
+        <v>38.75</v>
       </c>
       <c r="O19" t="n">
-        <v>40.72</v>
+        <v>38.98</v>
       </c>
       <c r="P19" t="n">
-        <v>37.08</v>
+        <v>37.71</v>
       </c>
       <c r="Q19" t="n">
-        <v>39.95</v>
+        <v>38.28</v>
       </c>
       <c r="R19" t="n">
-        <v>-16.5847</v>
+        <v>7.2629</v>
       </c>
       <c r="S19" t="n">
-        <v>-23.275</v>
+        <v>-27.0181</v>
       </c>
       <c r="T19" t="n">
-        <v>-28.162</v>
+        <v>-9.7171</v>
       </c>
       <c r="U19" t="n">
-        <v>-5.306</v>
+        <v>4.1854</v>
       </c>
       <c r="V19" t="n">
-        <v>-4.9747</v>
+        <v>-5.6543</v>
       </c>
       <c r="W19" t="n">
-        <v>-2.1348</v>
+        <v>6.3901</v>
       </c>
       <c r="X19" t="n">
-        <v>16.8394</v>
+        <v>-7.5388</v>
       </c>
       <c r="Y19" t="n">
-        <v>21.2366</v>
+        <v>28.7037</v>
       </c>
       <c r="Z19" t="n">
-        <v>24.2424</v>
+        <v>-1.6509</v>
       </c>
       <c r="AA19" t="n">
-        <v>5.4646</v>
+        <v>-4.1802</v>
       </c>
       <c r="AB19" t="n">
-        <v>4.6908</v>
+        <v>5.4255</v>
       </c>
       <c r="AC19" t="n">
-        <v>1.2161</v>
+        <v>-7.3348</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>197.21</v>
+        <v>165.4</v>
       </c>
       <c r="C20" t="n">
-        <v>210.8</v>
+        <v>171.88</v>
       </c>
       <c r="D20" t="n">
-        <v>194.22</v>
+        <v>150.08</v>
       </c>
       <c r="E20" t="n">
-        <v>194.65</v>
+        <v>165.28</v>
       </c>
       <c r="F20" t="n">
-        <v>75.54000000000001</v>
+        <v>73.7</v>
       </c>
       <c r="G20" t="n">
-        <v>77.45</v>
+        <v>74.39</v>
       </c>
       <c r="H20" t="n">
-        <v>75.11</v>
+        <v>70.76000000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>76.42</v>
+        <v>72.23</v>
       </c>
       <c r="J20" t="n">
-        <v>4.11</v>
+        <v>4.8</v>
       </c>
       <c r="K20" t="n">
-        <v>4.18</v>
+        <v>5.14</v>
       </c>
       <c r="L20" t="n">
-        <v>3.77</v>
+        <v>4.66</v>
       </c>
       <c r="M20" t="n">
-        <v>4.17</v>
+        <v>4.8</v>
       </c>
       <c r="N20" t="n">
-        <v>38.75</v>
+        <v>39.64</v>
       </c>
       <c r="O20" t="n">
-        <v>38.98</v>
+        <v>41.11</v>
       </c>
       <c r="P20" t="n">
-        <v>37.71</v>
+        <v>39.29</v>
       </c>
       <c r="Q20" t="n">
-        <v>38.28</v>
+        <v>40.38</v>
       </c>
       <c r="R20" t="n">
-        <v>7.2629</v>
+        <v>-15.0886</v>
       </c>
       <c r="S20" t="n">
-        <v>-27.0181</v>
+        <v>-24.0267</v>
       </c>
       <c r="T20" t="n">
-        <v>-9.7171</v>
+        <v>-30.1201</v>
       </c>
       <c r="U20" t="n">
-        <v>4.1854</v>
+        <v>-5.4829</v>
       </c>
       <c r="V20" t="n">
-        <v>-5.6543</v>
+        <v>-6.7519</v>
       </c>
       <c r="W20" t="n">
-        <v>6.3901</v>
+        <v>-6.4257</v>
       </c>
       <c r="X20" t="n">
-        <v>-7.5388</v>
+        <v>15.1079</v>
       </c>
       <c r="Y20" t="n">
-        <v>28.7037</v>
+        <v>24.3523</v>
       </c>
       <c r="Z20" t="n">
-        <v>-1.6509</v>
+        <v>29.0323</v>
       </c>
       <c r="AA20" t="n">
-        <v>-4.1802</v>
+        <v>5.4859</v>
       </c>
       <c r="AB20" t="n">
-        <v>5.4255</v>
+        <v>6.5998</v>
       </c>
       <c r="AC20" t="n">
-        <v>-7.3348</v>
+        <v>5.8176</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>165.4</v>
+        <v>159.21</v>
       </c>
       <c r="C21" t="n">
-        <v>171.88</v>
+        <v>176.75</v>
       </c>
       <c r="D21" t="n">
-        <v>150.08</v>
+        <v>158.8749</v>
       </c>
       <c r="E21" t="n">
-        <v>165.28</v>
+        <v>174.82</v>
       </c>
       <c r="F21" t="n">
-        <v>73.7</v>
+        <v>70.795</v>
       </c>
       <c r="G21" t="n">
-        <v>74.38</v>
+        <v>73.015</v>
       </c>
       <c r="H21" t="n">
-        <v>70.76000000000001</v>
+        <v>69.56999999999999</v>
       </c>
       <c r="I21" t="n">
-        <v>72.23</v>
+        <v>72.72</v>
       </c>
       <c r="J21" t="n">
-        <v>4.8</v>
+        <v>4.98</v>
       </c>
       <c r="K21" t="n">
-        <v>5.14</v>
+        <v>4.99</v>
       </c>
       <c r="L21" t="n">
-        <v>4.66</v>
+        <v>4.46</v>
       </c>
       <c r="M21" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="N21" t="n">
-        <v>39.64</v>
+        <v>41.18</v>
       </c>
       <c r="O21" t="n">
-        <v>41.1065</v>
+        <v>41.855</v>
       </c>
       <c r="P21" t="n">
-        <v>39.29</v>
+        <v>39.93</v>
       </c>
       <c r="Q21" t="n">
-        <v>40.38</v>
+        <v>40.08</v>
       </c>
       <c r="R21" t="n">
-        <v>-15.0886</v>
+        <v>5.772</v>
       </c>
       <c r="S21" t="n">
-        <v>-24.0267</v>
+        <v>-3.6645</v>
       </c>
       <c r="T21" t="n">
-        <v>-30.1201</v>
+        <v>-34.4532</v>
       </c>
       <c r="U21" t="n">
-        <v>-5.4829</v>
+        <v>0.6784</v>
       </c>
       <c r="V21" t="n">
-        <v>-6.7519</v>
+        <v>-0.8589</v>
       </c>
       <c r="W21" t="n">
-        <v>-6.4257</v>
+        <v>-10.2222</v>
       </c>
       <c r="X21" t="n">
-        <v>15.1079</v>
+        <v>-6.25</v>
       </c>
       <c r="Y21" t="n">
-        <v>24.3523</v>
+        <v>-0.2217</v>
       </c>
       <c r="Z21" t="n">
-        <v>29.0323</v>
+        <v>38.8889</v>
       </c>
       <c r="AA21" t="n">
-        <v>5.4859</v>
+        <v>-0.7429</v>
       </c>
       <c r="AB21" t="n">
-        <v>6.5998</v>
+        <v>0.3254</v>
       </c>
       <c r="AC21" t="n">
-        <v>5.8176</v>
+        <v>10.3828</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-07-09 23:11
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1713 +568,1713 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>227.06</v>
+        <v>191.54</v>
       </c>
       <c r="C2" t="n">
-        <v>231.02</v>
+        <v>212.99</v>
       </c>
       <c r="D2" t="n">
-        <v>157.56</v>
+        <v>177.3</v>
       </c>
       <c r="E2" t="n">
-        <v>201.68</v>
+        <v>180.65</v>
       </c>
       <c r="F2" t="n">
-        <v>78.2997</v>
+        <v>71.5153</v>
       </c>
       <c r="G2" t="n">
-        <v>79.15770000000001</v>
+        <v>74.5284</v>
       </c>
       <c r="H2" t="n">
-        <v>66.6366</v>
+        <v>68.8415</v>
       </c>
       <c r="I2" t="n">
-        <v>73.55070000000001</v>
+        <v>69.1109</v>
       </c>
       <c r="J2" t="n">
-        <v>5.1895</v>
+        <v>6.1681</v>
       </c>
       <c r="K2" t="n">
-        <v>7.0281</v>
+        <v>6.5734</v>
       </c>
       <c r="L2" t="n">
-        <v>5.0808</v>
+        <v>5.5355</v>
       </c>
       <c r="M2" t="n">
-        <v>5.8617</v>
+        <v>6.4943</v>
       </c>
       <c r="N2" t="n">
-        <v>39.4299</v>
+        <v>43.1209</v>
       </c>
       <c r="O2" t="n">
-        <v>45.6505</v>
+        <v>44.676</v>
       </c>
       <c r="P2" t="n">
-        <v>38.9673</v>
+        <v>41.4082</v>
       </c>
       <c r="Q2" t="n">
-        <v>41.9988</v>
+        <v>44.5382</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>191.54</v>
+        <v>192.3</v>
       </c>
       <c r="C3" t="n">
-        <v>212.99</v>
+        <v>225.63</v>
       </c>
       <c r="D3" t="n">
-        <v>177.3</v>
+        <v>192.3</v>
       </c>
       <c r="E3" t="n">
-        <v>180.65</v>
+        <v>223.99</v>
       </c>
       <c r="F3" t="n">
-        <v>71.5153</v>
+        <v>70.7272</v>
       </c>
       <c r="G3" t="n">
-        <v>74.5284</v>
+        <v>76.42400000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>68.8415</v>
+        <v>69.4301</v>
       </c>
       <c r="I3" t="n">
-        <v>69.1109</v>
+        <v>75.83540000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>6.1681</v>
+        <v>6.0298</v>
       </c>
       <c r="K3" t="n">
-        <v>6.5734</v>
+        <v>6.0298</v>
       </c>
       <c r="L3" t="n">
-        <v>5.5355</v>
+        <v>4.8436</v>
       </c>
       <c r="M3" t="n">
-        <v>6.4943</v>
+        <v>4.9128</v>
       </c>
       <c r="N3" t="n">
-        <v>43.1209</v>
+        <v>43.4851</v>
       </c>
       <c r="O3" t="n">
-        <v>44.676</v>
+        <v>44.302</v>
       </c>
       <c r="P3" t="n">
-        <v>41.4082</v>
+        <v>39.8039</v>
       </c>
       <c r="Q3" t="n">
-        <v>44.5382</v>
+        <v>40.1878</v>
       </c>
       <c r="R3" t="n">
-        <v>-10.4274</v>
+        <v>23.9911</v>
       </c>
       <c r="U3" t="n">
-        <v>-6.0364</v>
+        <v>9.73</v>
       </c>
       <c r="X3" t="n">
-        <v>10.7921</v>
+        <v>-24.3521</v>
       </c>
       <c r="AA3" t="n">
-        <v>6.0464</v>
+        <v>-9.767799999999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>192.3</v>
+        <v>222.22</v>
       </c>
       <c r="C4" t="n">
-        <v>225.63</v>
+        <v>242.4</v>
       </c>
       <c r="D4" t="n">
-        <v>192.3</v>
+        <v>214.74</v>
       </c>
       <c r="E4" t="n">
-        <v>223.99</v>
+        <v>234.68</v>
       </c>
       <c r="F4" t="n">
-        <v>70.7272</v>
+        <v>76.16459999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>76.42400000000001</v>
+        <v>78.18000000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>69.4301</v>
+        <v>74.1193</v>
       </c>
       <c r="I4" t="n">
-        <v>75.83540000000001</v>
+        <v>77.3419</v>
       </c>
       <c r="J4" t="n">
-        <v>6.0298</v>
+        <v>4.9523</v>
       </c>
       <c r="K4" t="n">
-        <v>6.0298</v>
+        <v>5.0907</v>
       </c>
       <c r="L4" t="n">
-        <v>4.8436</v>
+        <v>4.4877</v>
       </c>
       <c r="M4" t="n">
-        <v>4.9128</v>
+        <v>4.6656</v>
       </c>
       <c r="N4" t="n">
-        <v>43.4851</v>
+        <v>40.0106</v>
       </c>
       <c r="O4" t="n">
-        <v>44.302</v>
+        <v>41.0933</v>
       </c>
       <c r="P4" t="n">
-        <v>39.8039</v>
+        <v>38.9476</v>
       </c>
       <c r="Q4" t="n">
-        <v>40.1878</v>
+        <v>39.4102</v>
       </c>
       <c r="R4" t="n">
-        <v>23.9911</v>
+        <v>4.7725</v>
       </c>
       <c r="U4" t="n">
-        <v>9.73</v>
+        <v>1.9865</v>
       </c>
       <c r="X4" t="n">
-        <v>-24.3521</v>
+        <v>-5.0318</v>
       </c>
       <c r="AA4" t="n">
-        <v>-9.767799999999999</v>
+        <v>-1.9349</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>222.22</v>
+        <v>265.99</v>
       </c>
       <c r="C5" t="n">
-        <v>242.4</v>
+        <v>274.88</v>
       </c>
       <c r="D5" t="n">
-        <v>214.74</v>
+        <v>261.6</v>
       </c>
       <c r="E5" t="n">
-        <v>234.68</v>
+        <v>272.5</v>
       </c>
       <c r="F5" t="n">
-        <v>76.16459999999999</v>
+        <v>82.6896</v>
       </c>
       <c r="G5" t="n">
-        <v>78.18000000000001</v>
+        <v>84.8347</v>
       </c>
       <c r="H5" t="n">
-        <v>74.1193</v>
+        <v>82.4502</v>
       </c>
       <c r="I5" t="n">
-        <v>77.3419</v>
+        <v>84.39570000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>4.9523</v>
+        <v>4.0231</v>
       </c>
       <c r="K5" t="n">
-        <v>5.0907</v>
+        <v>4.122</v>
       </c>
       <c r="L5" t="n">
-        <v>4.4877</v>
+        <v>3.865</v>
       </c>
       <c r="M5" t="n">
-        <v>4.6656</v>
+        <v>3.9045</v>
       </c>
       <c r="N5" t="n">
-        <v>40.0106</v>
+        <v>36.6641</v>
       </c>
       <c r="O5" t="n">
-        <v>41.0933</v>
+        <v>36.7723</v>
       </c>
       <c r="P5" t="n">
-        <v>38.9476</v>
+        <v>35.5814</v>
       </c>
       <c r="Q5" t="n">
-        <v>39.4102</v>
+        <v>35.7389</v>
       </c>
       <c r="R5" t="n">
-        <v>4.7725</v>
+        <v>16.1156</v>
       </c>
       <c r="S5" t="n">
-        <v>16.3626</v>
+        <v>50.8442</v>
       </c>
       <c r="U5" t="n">
-        <v>1.9865</v>
+        <v>9.1203</v>
       </c>
       <c r="V5" t="n">
-        <v>5.1545</v>
+        <v>22.1163</v>
       </c>
       <c r="X5" t="n">
-        <v>-5.0318</v>
+        <v>-16.313</v>
       </c>
       <c r="Y5" t="n">
-        <v>-20.4053</v>
+        <v>-39.878</v>
       </c>
       <c r="AA5" t="n">
-        <v>-1.9349</v>
+        <v>-9.3156</v>
       </c>
       <c r="AB5" t="n">
-        <v>-6.1635</v>
+        <v>-19.7567</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>265.99</v>
+        <v>267.13</v>
       </c>
       <c r="C6" t="n">
-        <v>274.88</v>
+        <v>274.93</v>
       </c>
       <c r="D6" t="n">
-        <v>261.6</v>
+        <v>226</v>
       </c>
       <c r="E6" t="n">
-        <v>272.5</v>
+        <v>226.19</v>
       </c>
       <c r="F6" t="n">
-        <v>82.6896</v>
+        <v>83.9966</v>
       </c>
       <c r="G6" t="n">
-        <v>84.8347</v>
+        <v>84.63509999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>82.4502</v>
+        <v>79.67659999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>84.39570000000001</v>
+        <v>79.74639999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>4.0231</v>
+        <v>3.9836</v>
       </c>
       <c r="K6" t="n">
-        <v>4.122</v>
+        <v>4.5965</v>
       </c>
       <c r="L6" t="n">
         <v>3.865</v>
       </c>
       <c r="M6" t="n">
-        <v>3.9045</v>
+        <v>4.5767</v>
       </c>
       <c r="N6" t="n">
-        <v>36.6641</v>
+        <v>35.9652</v>
       </c>
       <c r="O6" t="n">
-        <v>36.7723</v>
+        <v>37.7861</v>
       </c>
       <c r="P6" t="n">
-        <v>35.5814</v>
+        <v>35.6896</v>
       </c>
       <c r="Q6" t="n">
-        <v>35.7389</v>
+        <v>37.7468</v>
       </c>
       <c r="R6" t="n">
-        <v>16.1156</v>
+        <v>-16.9945</v>
       </c>
       <c r="S6" t="n">
-        <v>50.8442</v>
+        <v>0.9822</v>
       </c>
       <c r="U6" t="n">
-        <v>9.1203</v>
+        <v>-5.5089</v>
       </c>
       <c r="V6" t="n">
-        <v>22.1163</v>
+        <v>5.1572</v>
       </c>
       <c r="X6" t="n">
-        <v>-16.313</v>
+        <v>17.216</v>
       </c>
       <c r="Y6" t="n">
-        <v>-39.878</v>
+        <v>-6.8413</v>
       </c>
       <c r="AA6" t="n">
-        <v>-9.3156</v>
+        <v>5.6182</v>
       </c>
       <c r="AB6" t="n">
-        <v>-19.7567</v>
+        <v>-6.074</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>267.13</v>
+        <v>247.42</v>
       </c>
       <c r="C7" t="n">
-        <v>274.93</v>
+        <v>259.79</v>
       </c>
       <c r="D7" t="n">
-        <v>226</v>
+        <v>233.3</v>
       </c>
       <c r="E7" t="n">
-        <v>226.19</v>
+        <v>233.86</v>
       </c>
       <c r="F7" t="n">
-        <v>83.9966</v>
+        <v>81.4824</v>
       </c>
       <c r="G7" t="n">
-        <v>84.63509999999999</v>
+        <v>81.6221</v>
       </c>
       <c r="H7" t="n">
-        <v>79.67659999999999</v>
+        <v>76.7633</v>
       </c>
       <c r="I7" t="n">
-        <v>79.74639999999999</v>
+        <v>77.36190000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>3.9836</v>
+        <v>4.122</v>
       </c>
       <c r="K7" t="n">
-        <v>4.5965</v>
+        <v>4.4086</v>
       </c>
       <c r="L7" t="n">
-        <v>3.865</v>
+        <v>3.8749</v>
       </c>
       <c r="M7" t="n">
-        <v>4.5767</v>
+        <v>4.4086</v>
       </c>
       <c r="N7" t="n">
-        <v>35.9652</v>
+        <v>36.9397</v>
       </c>
       <c r="O7" t="n">
-        <v>37.7861</v>
+        <v>39.1641</v>
       </c>
       <c r="P7" t="n">
-        <v>35.6896</v>
+        <v>36.8708</v>
       </c>
       <c r="Q7" t="n">
-        <v>37.7468</v>
+        <v>38.8984</v>
       </c>
       <c r="R7" t="n">
-        <v>-16.9945</v>
+        <v>3.391</v>
       </c>
       <c r="S7" t="n">
-        <v>0.9822</v>
+        <v>-0.3494</v>
       </c>
       <c r="T7" t="n">
-        <v>12.1529</v>
+        <v>29.4547</v>
       </c>
       <c r="U7" t="n">
-        <v>-5.5089</v>
+        <v>-2.9901</v>
       </c>
       <c r="V7" t="n">
-        <v>5.1572</v>
+        <v>0.0259</v>
       </c>
       <c r="W7" t="n">
-        <v>8.4237</v>
+        <v>11.9388</v>
       </c>
       <c r="X7" t="n">
-        <v>17.216</v>
+        <v>-3.673</v>
       </c>
       <c r="Y7" t="n">
-        <v>-6.8413</v>
+        <v>-5.5084</v>
       </c>
       <c r="Z7" t="n">
-        <v>-21.922</v>
+        <v>-32.1159</v>
       </c>
       <c r="AA7" t="n">
-        <v>5.6182</v>
+        <v>3.0509</v>
       </c>
       <c r="AB7" t="n">
-        <v>-6.074</v>
+        <v>-1.2986</v>
       </c>
       <c r="AC7" t="n">
-        <v>-10.1241</v>
+        <v>-12.6628</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>247.42</v>
+        <v>266.04</v>
       </c>
       <c r="C8" t="n">
-        <v>259.79</v>
+        <v>286.15</v>
       </c>
       <c r="D8" t="n">
-        <v>233.3</v>
+        <v>265</v>
       </c>
       <c r="E8" t="n">
-        <v>233.86</v>
+        <v>279.29</v>
       </c>
       <c r="F8" t="n">
-        <v>81.4824</v>
+        <v>81.9114</v>
       </c>
       <c r="G8" t="n">
-        <v>81.6221</v>
+        <v>83.408</v>
       </c>
       <c r="H8" t="n">
-        <v>76.7633</v>
+        <v>80.4448</v>
       </c>
       <c r="I8" t="n">
-        <v>77.36190000000001</v>
+        <v>82.67959999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>4.122</v>
+        <v>3.8156</v>
       </c>
       <c r="K8" t="n">
-        <v>4.4086</v>
+        <v>3.8254</v>
       </c>
       <c r="L8" t="n">
-        <v>3.8749</v>
+        <v>3.4103</v>
       </c>
       <c r="M8" t="n">
-        <v>4.4086</v>
+        <v>3.5487</v>
       </c>
       <c r="N8" t="n">
-        <v>36.9397</v>
+        <v>36.6149</v>
       </c>
       <c r="O8" t="n">
-        <v>39.1641</v>
+        <v>37.3531</v>
       </c>
       <c r="P8" t="n">
-        <v>36.8708</v>
+        <v>35.857</v>
       </c>
       <c r="Q8" t="n">
-        <v>38.8984</v>
+        <v>36.1719</v>
       </c>
       <c r="R8" t="n">
-        <v>3.391</v>
+        <v>19.4262</v>
       </c>
       <c r="S8" t="n">
-        <v>-0.3494</v>
+        <v>2.4917</v>
       </c>
       <c r="T8" t="n">
-        <v>29.4547</v>
+        <v>24.6886</v>
       </c>
       <c r="U8" t="n">
-        <v>-2.9901</v>
+        <v>6.8738</v>
       </c>
       <c r="V8" t="n">
-        <v>0.0259</v>
+        <v>-2.0334</v>
       </c>
       <c r="W8" t="n">
-        <v>11.9388</v>
+        <v>9.0251</v>
       </c>
       <c r="X8" t="n">
-        <v>-3.673</v>
+        <v>-19.5051</v>
       </c>
       <c r="Y8" t="n">
-        <v>-5.5084</v>
+        <v>-9.1126</v>
       </c>
       <c r="Z8" t="n">
-        <v>-32.1159</v>
+        <v>-27.7662</v>
       </c>
       <c r="AA8" t="n">
-        <v>3.0509</v>
+        <v>-7.0093</v>
       </c>
       <c r="AB8" t="n">
-        <v>-1.2986</v>
+        <v>1.2116</v>
       </c>
       <c r="AC8" t="n">
-        <v>-12.6628</v>
+        <v>-9.992800000000001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>266.04</v>
+        <v>299.26</v>
       </c>
       <c r="C9" t="n">
-        <v>286.15</v>
+        <v>302</v>
       </c>
       <c r="D9" t="n">
-        <v>265</v>
+        <v>286.24</v>
       </c>
       <c r="E9" t="n">
-        <v>279.29</v>
+        <v>300.77</v>
       </c>
       <c r="F9" t="n">
-        <v>81.9114</v>
+        <v>83.7572</v>
       </c>
       <c r="G9" t="n">
-        <v>83.408</v>
+        <v>84.9145</v>
       </c>
       <c r="H9" t="n">
-        <v>80.4448</v>
+        <v>81.203</v>
       </c>
       <c r="I9" t="n">
-        <v>82.67959999999999</v>
+        <v>82.3903</v>
       </c>
       <c r="J9" t="n">
-        <v>3.8156</v>
+        <v>3.2917</v>
       </c>
       <c r="K9" t="n">
-        <v>3.8254</v>
+        <v>3.4498</v>
       </c>
       <c r="L9" t="n">
-        <v>3.4103</v>
+        <v>3.2521</v>
       </c>
       <c r="M9" t="n">
-        <v>3.5487</v>
+        <v>3.262</v>
       </c>
       <c r="N9" t="n">
-        <v>36.6149</v>
+        <v>35.7389</v>
       </c>
       <c r="O9" t="n">
-        <v>37.3531</v>
+        <v>36.8511</v>
       </c>
       <c r="P9" t="n">
-        <v>35.857</v>
+        <v>35.2369</v>
       </c>
       <c r="Q9" t="n">
-        <v>36.1719</v>
+        <v>36.3491</v>
       </c>
       <c r="R9" t="n">
-        <v>19.4262</v>
+        <v>7.6909</v>
       </c>
       <c r="S9" t="n">
-        <v>2.4917</v>
+        <v>32.9723</v>
       </c>
       <c r="T9" t="n">
-        <v>24.6886</v>
+        <v>28.1618</v>
       </c>
       <c r="U9" t="n">
-        <v>6.8738</v>
+        <v>-0.3499</v>
       </c>
       <c r="V9" t="n">
-        <v>-2.0334</v>
+        <v>3.3154</v>
       </c>
       <c r="W9" t="n">
-        <v>9.0251</v>
+        <v>6.5274</v>
       </c>
       <c r="X9" t="n">
-        <v>-19.5051</v>
+        <v>-8.079000000000001</v>
       </c>
       <c r="Y9" t="n">
-        <v>-9.1126</v>
+        <v>-28.7259</v>
       </c>
       <c r="Z9" t="n">
-        <v>-27.7662</v>
+        <v>-30.084</v>
       </c>
       <c r="AA9" t="n">
-        <v>-7.0093</v>
+        <v>0.4899</v>
       </c>
       <c r="AB9" t="n">
-        <v>1.2116</v>
+        <v>-3.7028</v>
       </c>
       <c r="AC9" t="n">
-        <v>-9.992800000000001</v>
+        <v>-7.7673</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>299.26</v>
+        <v>236</v>
       </c>
       <c r="C10" t="n">
-        <v>302</v>
+        <v>252.98</v>
       </c>
       <c r="D10" t="n">
-        <v>286.24</v>
+        <v>223</v>
       </c>
       <c r="E10" t="n">
-        <v>300.77</v>
+        <v>231.42</v>
       </c>
       <c r="F10" t="n">
-        <v>83.7572</v>
+        <v>74.9474</v>
       </c>
       <c r="G10" t="n">
-        <v>84.9145</v>
+        <v>77.56140000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>81.203</v>
+        <v>73.7402</v>
       </c>
       <c r="I10" t="n">
-        <v>82.3903</v>
+        <v>74.26900000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>3.2917</v>
+        <v>3.99</v>
       </c>
       <c r="K10" t="n">
-        <v>3.4498</v>
+        <v>4.13</v>
       </c>
       <c r="L10" t="n">
-        <v>3.2521</v>
+        <v>3.8</v>
       </c>
       <c r="M10" t="n">
-        <v>3.262</v>
+        <v>4.04</v>
       </c>
       <c r="N10" t="n">
-        <v>35.7389</v>
+        <v>39.6267</v>
       </c>
       <c r="O10" t="n">
-        <v>36.8511</v>
+        <v>40.1582</v>
       </c>
       <c r="P10" t="n">
-        <v>35.2369</v>
+        <v>38.4653</v>
       </c>
       <c r="Q10" t="n">
-        <v>36.3491</v>
+        <v>39.922</v>
       </c>
       <c r="R10" t="n">
-        <v>7.6909</v>
+        <v>-23.0575</v>
       </c>
       <c r="S10" t="n">
-        <v>32.9723</v>
+        <v>-1.0434</v>
       </c>
       <c r="T10" t="n">
-        <v>28.1618</v>
+        <v>-15.0752</v>
       </c>
       <c r="U10" t="n">
-        <v>-0.3499</v>
+        <v>-9.857100000000001</v>
       </c>
       <c r="V10" t="n">
-        <v>3.3154</v>
+        <v>-3.998</v>
       </c>
       <c r="W10" t="n">
-        <v>6.5274</v>
+        <v>-11.9991</v>
       </c>
       <c r="X10" t="n">
-        <v>-8.079000000000001</v>
+        <v>23.8504</v>
       </c>
       <c r="Y10" t="n">
-        <v>-28.7259</v>
+        <v>-8.360900000000001</v>
       </c>
       <c r="Z10" t="n">
-        <v>-30.084</v>
+        <v>3.4704</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.4899</v>
+        <v>9.8294</v>
       </c>
       <c r="AB10" t="n">
-        <v>-3.7028</v>
+        <v>2.6315</v>
       </c>
       <c r="AC10" t="n">
-        <v>-7.7673</v>
+        <v>11.7046</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>236</v>
+        <v>233.11</v>
       </c>
       <c r="C11" t="n">
-        <v>252.98</v>
+        <v>237</v>
       </c>
       <c r="D11" t="n">
-        <v>223</v>
+        <v>211.13</v>
       </c>
       <c r="E11" t="n">
-        <v>231.42</v>
+        <v>229.57</v>
       </c>
       <c r="F11" t="n">
-        <v>74.9474</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>77.56140000000001</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>73.7402</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>74.26900000000001</v>
+        <v>73.3</v>
       </c>
       <c r="J11" t="n">
-        <v>3.99</v>
+        <v>4</v>
       </c>
       <c r="K11" t="n">
-        <v>4.13</v>
+        <v>4.39</v>
       </c>
       <c r="L11" t="n">
-        <v>3.8</v>
+        <v>3.92</v>
       </c>
       <c r="M11" t="n">
-        <v>4.04</v>
+        <v>4.08</v>
       </c>
       <c r="N11" t="n">
-        <v>39.6267</v>
+        <v>39.66</v>
       </c>
       <c r="O11" t="n">
-        <v>40.1582</v>
+        <v>41.49</v>
       </c>
       <c r="P11" t="n">
-        <v>38.4653</v>
+        <v>38.9</v>
       </c>
       <c r="Q11" t="n">
-        <v>39.922</v>
+        <v>40.45</v>
       </c>
       <c r="R11" t="n">
-        <v>-23.0575</v>
+        <v>-0.7994</v>
       </c>
       <c r="S11" t="n">
-        <v>-1.0434</v>
+        <v>-17.8023</v>
       </c>
       <c r="T11" t="n">
-        <v>-15.0752</v>
+        <v>1.4943</v>
       </c>
       <c r="U11" t="n">
-        <v>-9.857100000000001</v>
+        <v>-1.3047</v>
       </c>
       <c r="V11" t="n">
-        <v>-3.998</v>
+        <v>-11.3445</v>
       </c>
       <c r="W11" t="n">
-        <v>-11.9991</v>
+        <v>-8.083600000000001</v>
       </c>
       <c r="X11" t="n">
-        <v>23.8504</v>
+        <v>0.9901</v>
       </c>
       <c r="Y11" t="n">
-        <v>-8.360900000000001</v>
+        <v>14.9717</v>
       </c>
       <c r="Z11" t="n">
-        <v>3.4704</v>
+        <v>-10.8528</v>
       </c>
       <c r="AA11" t="n">
-        <v>9.8294</v>
+        <v>1.3226</v>
       </c>
       <c r="AB11" t="n">
-        <v>2.6315</v>
+        <v>11.8271</v>
       </c>
       <c r="AC11" t="n">
-        <v>11.7046</v>
+        <v>7.1614</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>233.11</v>
+        <v>268.05</v>
       </c>
       <c r="C12" t="n">
-        <v>237</v>
+        <v>268.4</v>
       </c>
       <c r="D12" t="n">
-        <v>211.13</v>
+        <v>225.74</v>
       </c>
       <c r="E12" t="n">
-        <v>229.57</v>
+        <v>252.61</v>
       </c>
       <c r="F12" t="n">
-        <v>74.79000000000001</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="G12" t="n">
-        <v>76.18000000000001</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>71.34999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>73.3</v>
+        <v>74.95</v>
       </c>
       <c r="J12" t="n">
-        <v>4</v>
+        <v>3.38</v>
       </c>
       <c r="K12" t="n">
-        <v>4.39</v>
+        <v>4.15</v>
       </c>
       <c r="L12" t="n">
-        <v>3.92</v>
+        <v>3.37</v>
       </c>
       <c r="M12" t="n">
-        <v>4.08</v>
+        <v>3.63</v>
       </c>
       <c r="N12" t="n">
-        <v>39.66</v>
+        <v>37.87</v>
       </c>
       <c r="O12" t="n">
-        <v>41.49</v>
+        <v>41.37</v>
       </c>
       <c r="P12" t="n">
-        <v>38.9</v>
+        <v>37.71</v>
       </c>
       <c r="Q12" t="n">
-        <v>40.45</v>
+        <v>39.47</v>
       </c>
       <c r="R12" t="n">
-        <v>-0.7994</v>
+        <v>10.0362</v>
       </c>
       <c r="S12" t="n">
-        <v>-17.8023</v>
+        <v>-16.0122</v>
       </c>
       <c r="T12" t="n">
-        <v>1.4943</v>
+        <v>8.0176</v>
       </c>
       <c r="U12" t="n">
-        <v>-1.3047</v>
+        <v>2.251</v>
       </c>
       <c r="V12" t="n">
-        <v>-11.3445</v>
+        <v>-9.0306</v>
       </c>
       <c r="W12" t="n">
-        <v>-8.083600000000001</v>
+        <v>-3.1177</v>
       </c>
       <c r="X12" t="n">
-        <v>0.9901</v>
+        <v>-11.0294</v>
       </c>
       <c r="Y12" t="n">
-        <v>14.9717</v>
+        <v>11.2814</v>
       </c>
       <c r="Z12" t="n">
-        <v>-10.8528</v>
+        <v>-17.6609</v>
       </c>
       <c r="AA12" t="n">
-        <v>1.3226</v>
+        <v>-2.4227</v>
       </c>
       <c r="AB12" t="n">
-        <v>11.8271</v>
+        <v>8.585900000000001</v>
       </c>
       <c r="AC12" t="n">
-        <v>7.1614</v>
+        <v>1.4695</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>268.05</v>
+        <v>226.24</v>
       </c>
       <c r="C13" t="n">
-        <v>268.4</v>
+        <v>231.25</v>
       </c>
       <c r="D13" t="n">
-        <v>225.74</v>
+        <v>212.1</v>
       </c>
       <c r="E13" t="n">
-        <v>252.61</v>
+        <v>215.6</v>
       </c>
       <c r="F13" t="n">
-        <v>77.95999999999999</v>
+        <v>72.09</v>
       </c>
       <c r="G13" t="n">
-        <v>78.23999999999999</v>
+        <v>74.69</v>
       </c>
       <c r="H13" t="n">
-        <v>71.59999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="I13" t="n">
-        <v>74.95</v>
+        <v>71.83</v>
       </c>
       <c r="J13" t="n">
-        <v>3.38</v>
+        <v>4.04</v>
       </c>
       <c r="K13" t="n">
-        <v>4.15</v>
+        <v>4.25</v>
       </c>
       <c r="L13" t="n">
-        <v>3.37</v>
+        <v>3.95</v>
       </c>
       <c r="M13" t="n">
-        <v>3.63</v>
+        <v>4.24</v>
       </c>
       <c r="N13" t="n">
-        <v>37.87</v>
+        <v>41.08</v>
       </c>
       <c r="O13" t="n">
-        <v>41.37</v>
+        <v>41.79</v>
       </c>
       <c r="P13" t="n">
-        <v>37.71</v>
+        <v>39.69</v>
       </c>
       <c r="Q13" t="n">
-        <v>39.47</v>
+        <v>41.31</v>
       </c>
       <c r="R13" t="n">
-        <v>10.0362</v>
+        <v>-14.651</v>
       </c>
       <c r="S13" t="n">
-        <v>-16.0122</v>
+        <v>-6.8361</v>
       </c>
       <c r="T13" t="n">
-        <v>8.0176</v>
+        <v>-22.8043</v>
       </c>
       <c r="U13" t="n">
-        <v>2.251</v>
+        <v>-4.1628</v>
       </c>
       <c r="V13" t="n">
-        <v>-9.0306</v>
+        <v>-3.284</v>
       </c>
       <c r="W13" t="n">
-        <v>-3.1177</v>
+        <v>-13.1225</v>
       </c>
       <c r="X13" t="n">
-        <v>-11.0294</v>
+        <v>16.8044</v>
       </c>
       <c r="Y13" t="n">
-        <v>11.2814</v>
+        <v>4.9505</v>
       </c>
       <c r="Z13" t="n">
-        <v>-17.6609</v>
+        <v>19.4804</v>
       </c>
       <c r="AA13" t="n">
-        <v>-2.4227</v>
+        <v>4.6618</v>
       </c>
       <c r="AB13" t="n">
-        <v>8.585900000000001</v>
+        <v>3.4768</v>
       </c>
       <c r="AC13" t="n">
-        <v>1.4695</v>
+        <v>14.2047</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>226.24</v>
+        <v>216.36</v>
       </c>
       <c r="C14" t="n">
-        <v>231.25</v>
+        <v>238.65</v>
       </c>
       <c r="D14" t="n">
-        <v>212.1</v>
+        <v>192.3</v>
       </c>
       <c r="E14" t="n">
-        <v>215.6</v>
+        <v>236.52</v>
       </c>
       <c r="F14" t="n">
-        <v>72.09</v>
+        <v>74.12</v>
       </c>
       <c r="G14" t="n">
-        <v>74.69</v>
+        <v>77.38</v>
       </c>
       <c r="H14" t="n">
-        <v>70.72</v>
+        <v>71.45</v>
       </c>
       <c r="I14" t="n">
-        <v>71.83</v>
+        <v>77.19</v>
       </c>
       <c r="J14" t="n">
-        <v>4.04</v>
+        <v>4.16</v>
       </c>
       <c r="K14" t="n">
-        <v>4.25</v>
+        <v>4.63</v>
       </c>
       <c r="L14" t="n">
-        <v>3.95</v>
+        <v>3.7</v>
       </c>
       <c r="M14" t="n">
-        <v>4.24</v>
+        <v>3.72</v>
       </c>
       <c r="N14" t="n">
-        <v>41.08</v>
+        <v>39.91</v>
       </c>
       <c r="O14" t="n">
-        <v>41.79</v>
+        <v>41.43</v>
       </c>
       <c r="P14" t="n">
-        <v>39.69</v>
+        <v>38.08</v>
       </c>
       <c r="Q14" t="n">
-        <v>41.31</v>
+        <v>38.16</v>
       </c>
       <c r="R14" t="n">
-        <v>-14.651</v>
+        <v>9.703200000000001</v>
       </c>
       <c r="S14" t="n">
-        <v>-6.8361</v>
+        <v>3.0274</v>
       </c>
       <c r="T14" t="n">
-        <v>-22.8043</v>
+        <v>-21.3618</v>
       </c>
       <c r="U14" t="n">
-        <v>-4.1628</v>
+        <v>7.4621</v>
       </c>
       <c r="V14" t="n">
-        <v>-3.284</v>
+        <v>5.307</v>
       </c>
       <c r="W14" t="n">
-        <v>-13.1225</v>
+        <v>-6.3118</v>
       </c>
       <c r="X14" t="n">
-        <v>16.8044</v>
+        <v>-12.2642</v>
       </c>
       <c r="Y14" t="n">
-        <v>4.9505</v>
+        <v>-8.823499999999999</v>
       </c>
       <c r="Z14" t="n">
-        <v>19.4804</v>
+        <v>14.0405</v>
       </c>
       <c r="AA14" t="n">
-        <v>4.6618</v>
+        <v>-7.6253</v>
       </c>
       <c r="AB14" t="n">
-        <v>3.4768</v>
+        <v>-5.6613</v>
       </c>
       <c r="AC14" t="n">
-        <v>14.2047</v>
+        <v>4.982</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>216.36</v>
+        <v>241.45</v>
       </c>
       <c r="C15" t="n">
-        <v>238.65</v>
+        <v>272</v>
       </c>
       <c r="D15" t="n">
-        <v>192.3</v>
+        <v>240.59</v>
       </c>
       <c r="E15" t="n">
-        <v>236.52</v>
+        <v>266.71</v>
       </c>
       <c r="F15" t="n">
-        <v>74.12</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="G15" t="n">
-        <v>77.38</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="H15" t="n">
-        <v>71.45</v>
+        <v>77.15000000000001</v>
       </c>
       <c r="I15" t="n">
-        <v>77.19</v>
+        <v>81</v>
       </c>
       <c r="J15" t="n">
-        <v>4.16</v>
+        <v>3.66</v>
       </c>
       <c r="K15" t="n">
-        <v>4.63</v>
+        <v>3.68</v>
       </c>
       <c r="L15" t="n">
-        <v>3.7</v>
+        <v>3.17</v>
       </c>
       <c r="M15" t="n">
-        <v>3.72</v>
+        <v>3.24</v>
       </c>
       <c r="N15" t="n">
-        <v>39.91</v>
+        <v>38.16</v>
       </c>
       <c r="O15" t="n">
-        <v>41.43</v>
+        <v>38.2</v>
       </c>
       <c r="P15" t="n">
-        <v>38.08</v>
+        <v>36.03</v>
       </c>
       <c r="Q15" t="n">
-        <v>38.16</v>
+        <v>36.31</v>
       </c>
       <c r="R15" t="n">
-        <v>9.703200000000001</v>
+        <v>12.7642</v>
       </c>
       <c r="S15" t="n">
-        <v>3.0274</v>
+        <v>5.5817</v>
       </c>
       <c r="T15" t="n">
-        <v>-21.3618</v>
+        <v>15.2493</v>
       </c>
       <c r="U15" t="n">
-        <v>7.4621</v>
+        <v>4.9359</v>
       </c>
       <c r="V15" t="n">
-        <v>5.307</v>
+        <v>8.071999999999999</v>
       </c>
       <c r="W15" t="n">
-        <v>-6.3118</v>
+        <v>9.063000000000001</v>
       </c>
       <c r="X15" t="n">
-        <v>-12.2642</v>
+        <v>-12.9032</v>
       </c>
       <c r="Y15" t="n">
-        <v>-8.823499999999999</v>
+        <v>-10.7438</v>
       </c>
       <c r="Z15" t="n">
-        <v>14.0405</v>
+        <v>-19.802</v>
       </c>
       <c r="AA15" t="n">
-        <v>-7.6253</v>
+        <v>-4.848</v>
       </c>
       <c r="AB15" t="n">
-        <v>-5.6613</v>
+        <v>-8.0061</v>
       </c>
       <c r="AC15" t="n">
-        <v>4.982</v>
+        <v>-9.047599999999999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>241.45</v>
+        <v>237.79</v>
       </c>
       <c r="C16" t="n">
-        <v>272</v>
+        <v>246.47</v>
       </c>
       <c r="D16" t="n">
-        <v>240.59</v>
+        <v>215.38</v>
       </c>
       <c r="E16" t="n">
-        <v>266.71</v>
+        <v>217.55</v>
       </c>
       <c r="F16" t="n">
-        <v>77.23999999999999</v>
+        <v>78.72</v>
       </c>
       <c r="G16" t="n">
-        <v>81.54000000000001</v>
+        <v>79.64</v>
       </c>
       <c r="H16" t="n">
-        <v>77.15000000000001</v>
+        <v>77.23</v>
       </c>
       <c r="I16" t="n">
-        <v>81</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J16" t="n">
-        <v>3.66</v>
+        <v>3.59</v>
       </c>
       <c r="K16" t="n">
-        <v>3.68</v>
+        <v>3.89</v>
       </c>
       <c r="L16" t="n">
-        <v>3.17</v>
+        <v>3.51</v>
       </c>
       <c r="M16" t="n">
-        <v>3.24</v>
+        <v>3.86</v>
       </c>
       <c r="N16" t="n">
-        <v>38.16</v>
+        <v>37.31</v>
       </c>
       <c r="O16" t="n">
-        <v>38.2</v>
+        <v>37.98</v>
       </c>
       <c r="P16" t="n">
-        <v>36.03</v>
+        <v>36.9</v>
       </c>
       <c r="Q16" t="n">
-        <v>36.31</v>
+        <v>37.88</v>
       </c>
       <c r="R16" t="n">
-        <v>12.7642</v>
+        <v>-18.432</v>
       </c>
       <c r="S16" t="n">
-        <v>5.5817</v>
+        <v>0.9045</v>
       </c>
       <c r="T16" t="n">
-        <v>15.2493</v>
+        <v>-5.2359</v>
       </c>
       <c r="U16" t="n">
-        <v>4.9359</v>
+        <v>-4.3704</v>
       </c>
       <c r="V16" t="n">
-        <v>8.071999999999999</v>
+        <v>7.838</v>
       </c>
       <c r="W16" t="n">
-        <v>9.063000000000001</v>
+        <v>5.6753</v>
       </c>
       <c r="X16" t="n">
-        <v>-12.9032</v>
+        <v>19.1358</v>
       </c>
       <c r="Y16" t="n">
-        <v>-10.7438</v>
+        <v>-8.962300000000001</v>
       </c>
       <c r="Z16" t="n">
-        <v>-19.802</v>
+        <v>-5.3922</v>
       </c>
       <c r="AA16" t="n">
-        <v>-4.848</v>
+        <v>4.3239</v>
       </c>
       <c r="AB16" t="n">
-        <v>-8.0061</v>
+        <v>-8.303100000000001</v>
       </c>
       <c r="AC16" t="n">
-        <v>-9.047599999999999</v>
+        <v>-6.3535</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>237.79</v>
+        <v>219.23</v>
       </c>
       <c r="C17" t="n">
-        <v>246.47</v>
+        <v>226.13</v>
       </c>
       <c r="D17" t="n">
-        <v>215.38</v>
+        <v>168.88</v>
       </c>
       <c r="E17" t="n">
-        <v>217.55</v>
+        <v>181.47</v>
       </c>
       <c r="F17" t="n">
-        <v>78.72</v>
+        <v>77.45</v>
       </c>
       <c r="G17" t="n">
-        <v>79.64</v>
+        <v>79.14</v>
       </c>
       <c r="H17" t="n">
-        <v>77.23</v>
+        <v>71.72</v>
       </c>
       <c r="I17" t="n">
-        <v>77.45999999999999</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="J17" t="n">
-        <v>3.59</v>
+        <v>3.84</v>
       </c>
       <c r="K17" t="n">
-        <v>3.89</v>
+        <v>4.74</v>
       </c>
       <c r="L17" t="n">
-        <v>3.51</v>
+        <v>3.71</v>
       </c>
       <c r="M17" t="n">
-        <v>3.86</v>
+        <v>4.51</v>
       </c>
       <c r="N17" t="n">
-        <v>37.31</v>
+        <v>37.91</v>
       </c>
       <c r="O17" t="n">
-        <v>37.98</v>
+        <v>40.72</v>
       </c>
       <c r="P17" t="n">
-        <v>36.9</v>
+        <v>37.08</v>
       </c>
       <c r="Q17" t="n">
-        <v>37.88</v>
+        <v>39.95</v>
       </c>
       <c r="R17" t="n">
-        <v>-18.432</v>
+        <v>-16.5847</v>
       </c>
       <c r="S17" t="n">
-        <v>0.9045</v>
+        <v>-23.275</v>
       </c>
       <c r="T17" t="n">
-        <v>-5.2359</v>
+        <v>-28.162</v>
       </c>
       <c r="U17" t="n">
-        <v>-4.3704</v>
+        <v>-5.306</v>
       </c>
       <c r="V17" t="n">
-        <v>7.838</v>
+        <v>-4.9747</v>
       </c>
       <c r="W17" t="n">
-        <v>5.6753</v>
+        <v>-2.1348</v>
       </c>
       <c r="X17" t="n">
-        <v>19.1358</v>
+        <v>16.8394</v>
       </c>
       <c r="Y17" t="n">
-        <v>-8.962300000000001</v>
+        <v>21.2366</v>
       </c>
       <c r="Z17" t="n">
-        <v>-5.3922</v>
+        <v>24.2424</v>
       </c>
       <c r="AA17" t="n">
-        <v>4.3239</v>
+        <v>5.4646</v>
       </c>
       <c r="AB17" t="n">
-        <v>-8.303100000000001</v>
+        <v>4.6908</v>
       </c>
       <c r="AC17" t="n">
-        <v>-6.3535</v>
+        <v>1.2161</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>219.23</v>
+        <v>197.21</v>
       </c>
       <c r="C18" t="n">
-        <v>226.13</v>
+        <v>210.8</v>
       </c>
       <c r="D18" t="n">
-        <v>168.88</v>
+        <v>194.22</v>
       </c>
       <c r="E18" t="n">
-        <v>181.47</v>
+        <v>194.65</v>
       </c>
       <c r="F18" t="n">
+        <v>75.54000000000001</v>
+      </c>
+      <c r="G18" t="n">
         <v>77.45</v>
       </c>
-      <c r="G18" t="n">
-        <v>79.14</v>
-      </c>
       <c r="H18" t="n">
-        <v>71.72</v>
+        <v>75.11</v>
       </c>
       <c r="I18" t="n">
-        <v>73.34999999999999</v>
+        <v>76.42</v>
       </c>
       <c r="J18" t="n">
-        <v>3.84</v>
+        <v>4.11</v>
       </c>
       <c r="K18" t="n">
-        <v>4.74</v>
+        <v>4.18</v>
       </c>
       <c r="L18" t="n">
-        <v>3.71</v>
+        <v>3.77</v>
       </c>
       <c r="M18" t="n">
-        <v>4.51</v>
+        <v>4.17</v>
       </c>
       <c r="N18" t="n">
-        <v>37.91</v>
+        <v>38.75</v>
       </c>
       <c r="O18" t="n">
-        <v>40.72</v>
+        <v>38.98</v>
       </c>
       <c r="P18" t="n">
-        <v>37.08</v>
+        <v>37.71</v>
       </c>
       <c r="Q18" t="n">
-        <v>39.95</v>
+        <v>38.28</v>
       </c>
       <c r="R18" t="n">
-        <v>-16.5847</v>
+        <v>7.2629</v>
       </c>
       <c r="S18" t="n">
-        <v>-23.275</v>
+        <v>-27.0181</v>
       </c>
       <c r="T18" t="n">
-        <v>-28.162</v>
+        <v>-9.7171</v>
       </c>
       <c r="U18" t="n">
-        <v>-5.306</v>
+        <v>4.1854</v>
       </c>
       <c r="V18" t="n">
-        <v>-4.9747</v>
+        <v>-5.6543</v>
       </c>
       <c r="W18" t="n">
-        <v>-2.1348</v>
+        <v>6.3901</v>
       </c>
       <c r="X18" t="n">
-        <v>16.8394</v>
+        <v>-7.5388</v>
       </c>
       <c r="Y18" t="n">
-        <v>21.2366</v>
+        <v>28.7037</v>
       </c>
       <c r="Z18" t="n">
-        <v>24.2424</v>
+        <v>-1.6509</v>
       </c>
       <c r="AA18" t="n">
-        <v>5.4646</v>
+        <v>-4.1802</v>
       </c>
       <c r="AB18" t="n">
-        <v>4.6908</v>
+        <v>5.4255</v>
       </c>
       <c r="AC18" t="n">
-        <v>1.2161</v>
+        <v>-7.3348</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>197.21</v>
+        <v>165.4</v>
       </c>
       <c r="C19" t="n">
-        <v>210.8</v>
+        <v>171.88</v>
       </c>
       <c r="D19" t="n">
-        <v>194.22</v>
+        <v>150.08</v>
       </c>
       <c r="E19" t="n">
-        <v>194.65</v>
+        <v>165.28</v>
       </c>
       <c r="F19" t="n">
-        <v>75.54000000000001</v>
+        <v>73.7</v>
       </c>
       <c r="G19" t="n">
-        <v>77.45</v>
+        <v>74.39</v>
       </c>
       <c r="H19" t="n">
-        <v>75.11</v>
+        <v>70.76000000000001</v>
       </c>
       <c r="I19" t="n">
-        <v>76.42</v>
+        <v>72.23</v>
       </c>
       <c r="J19" t="n">
-        <v>4.11</v>
+        <v>4.8</v>
       </c>
       <c r="K19" t="n">
-        <v>4.18</v>
+        <v>5.14</v>
       </c>
       <c r="L19" t="n">
-        <v>3.77</v>
+        <v>4.66</v>
       </c>
       <c r="M19" t="n">
-        <v>4.17</v>
+        <v>4.8</v>
       </c>
       <c r="N19" t="n">
-        <v>38.75</v>
+        <v>39.64</v>
       </c>
       <c r="O19" t="n">
-        <v>38.98</v>
+        <v>41.11</v>
       </c>
       <c r="P19" t="n">
-        <v>37.71</v>
+        <v>39.29</v>
       </c>
       <c r="Q19" t="n">
-        <v>38.28</v>
+        <v>40.38</v>
       </c>
       <c r="R19" t="n">
-        <v>7.2629</v>
+        <v>-15.0886</v>
       </c>
       <c r="S19" t="n">
-        <v>-27.0181</v>
+        <v>-24.0267</v>
       </c>
       <c r="T19" t="n">
-        <v>-9.7171</v>
+        <v>-30.1201</v>
       </c>
       <c r="U19" t="n">
-        <v>4.1854</v>
+        <v>-5.4829</v>
       </c>
       <c r="V19" t="n">
-        <v>-5.6543</v>
+        <v>-6.7519</v>
       </c>
       <c r="W19" t="n">
-        <v>6.3901</v>
+        <v>-6.4257</v>
       </c>
       <c r="X19" t="n">
-        <v>-7.5388</v>
+        <v>15.1079</v>
       </c>
       <c r="Y19" t="n">
-        <v>28.7037</v>
+        <v>24.3523</v>
       </c>
       <c r="Z19" t="n">
-        <v>-1.6509</v>
+        <v>29.0323</v>
       </c>
       <c r="AA19" t="n">
-        <v>-4.1802</v>
+        <v>5.4859</v>
       </c>
       <c r="AB19" t="n">
-        <v>5.4255</v>
+        <v>6.5998</v>
       </c>
       <c r="AC19" t="n">
-        <v>-7.3348</v>
+        <v>5.8176</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>165.4</v>
+        <v>159.21</v>
       </c>
       <c r="C20" t="n">
-        <v>171.88</v>
+        <v>176.75</v>
       </c>
       <c r="D20" t="n">
-        <v>150.08</v>
+        <v>158.87</v>
       </c>
       <c r="E20" t="n">
-        <v>165.28</v>
+        <v>174.82</v>
       </c>
       <c r="F20" t="n">
-        <v>73.7</v>
+        <v>70.8</v>
       </c>
       <c r="G20" t="n">
-        <v>74.39</v>
+        <v>73.02</v>
       </c>
       <c r="H20" t="n">
-        <v>70.76000000000001</v>
+        <v>69.56999999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>72.23</v>
+        <v>72.72</v>
       </c>
       <c r="J20" t="n">
-        <v>4.8</v>
+        <v>4.98</v>
       </c>
       <c r="K20" t="n">
-        <v>5.14</v>
+        <v>4.99</v>
       </c>
       <c r="L20" t="n">
-        <v>4.66</v>
+        <v>4.46</v>
       </c>
       <c r="M20" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="N20" t="n">
-        <v>39.64</v>
+        <v>41.18</v>
       </c>
       <c r="O20" t="n">
-        <v>41.11</v>
+        <v>41.86</v>
       </c>
       <c r="P20" t="n">
-        <v>39.29</v>
+        <v>39.93</v>
       </c>
       <c r="Q20" t="n">
-        <v>40.38</v>
+        <v>40.08</v>
       </c>
       <c r="R20" t="n">
-        <v>-15.0886</v>
+        <v>5.772</v>
       </c>
       <c r="S20" t="n">
-        <v>-24.0267</v>
+        <v>-3.6645</v>
       </c>
       <c r="T20" t="n">
-        <v>-30.1201</v>
+        <v>-34.4532</v>
       </c>
       <c r="U20" t="n">
-        <v>-5.4829</v>
+        <v>0.6784</v>
       </c>
       <c r="V20" t="n">
-        <v>-6.7519</v>
+        <v>-0.8589</v>
       </c>
       <c r="W20" t="n">
-        <v>-6.4257</v>
+        <v>-10.2222</v>
       </c>
       <c r="X20" t="n">
-        <v>15.1079</v>
+        <v>-6.25</v>
       </c>
       <c r="Y20" t="n">
-        <v>24.3523</v>
+        <v>-0.2217</v>
       </c>
       <c r="Z20" t="n">
-        <v>29.0323</v>
+        <v>38.8889</v>
       </c>
       <c r="AA20" t="n">
-        <v>5.4859</v>
+        <v>-0.7429</v>
       </c>
       <c r="AB20" t="n">
-        <v>6.5998</v>
+        <v>0.3254</v>
       </c>
       <c r="AC20" t="n">
-        <v>5.8176</v>
+        <v>10.3828</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>159.21</v>
+        <v>199.81</v>
       </c>
       <c r="C21" t="n">
-        <v>176.75</v>
+        <v>204.52</v>
       </c>
       <c r="D21" t="n">
-        <v>158.8749</v>
+        <v>189.46</v>
       </c>
       <c r="E21" t="n">
-        <v>174.82</v>
+        <v>192.45</v>
       </c>
       <c r="F21" t="n">
-        <v>70.795</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="G21" t="n">
-        <v>73.015</v>
+        <v>76.685</v>
       </c>
       <c r="H21" t="n">
-        <v>69.56999999999999</v>
+        <v>73.89</v>
       </c>
       <c r="I21" t="n">
-        <v>72.72</v>
+        <v>76.34</v>
       </c>
       <c r="J21" t="n">
-        <v>4.98</v>
+        <v>3.87</v>
       </c>
       <c r="K21" t="n">
-        <v>4.99</v>
+        <v>4.12</v>
       </c>
       <c r="L21" t="n">
-        <v>4.46</v>
+        <v>3.75</v>
       </c>
       <c r="M21" t="n">
-        <v>4.5</v>
+        <v>4.07</v>
       </c>
       <c r="N21" t="n">
-        <v>41.18</v>
+        <v>38.98</v>
       </c>
       <c r="O21" t="n">
-        <v>41.855</v>
+        <v>39.465</v>
       </c>
       <c r="P21" t="n">
-        <v>39.93</v>
+        <v>37.93</v>
       </c>
       <c r="Q21" t="n">
-        <v>40.08</v>
+        <v>38.1</v>
       </c>
       <c r="R21" t="n">
-        <v>5.772</v>
+        <v>10.0847</v>
       </c>
       <c r="S21" t="n">
-        <v>-3.6645</v>
+        <v>-1.1302</v>
       </c>
       <c r="T21" t="n">
-        <v>-34.4532</v>
+        <v>-11.5376</v>
       </c>
       <c r="U21" t="n">
-        <v>0.6784</v>
+        <v>4.978</v>
       </c>
       <c r="V21" t="n">
-        <v>-0.8589</v>
+        <v>-0.1047</v>
       </c>
       <c r="W21" t="n">
-        <v>-10.2222</v>
+        <v>-1.4459</v>
       </c>
       <c r="X21" t="n">
-        <v>-6.25</v>
+        <v>-9.5556</v>
       </c>
       <c r="Y21" t="n">
-        <v>-0.2217</v>
+        <v>-2.3981</v>
       </c>
       <c r="Z21" t="n">
-        <v>38.8889</v>
+        <v>5.4404</v>
       </c>
       <c r="AA21" t="n">
-        <v>-0.7429</v>
+        <v>-4.9401</v>
       </c>
       <c r="AB21" t="n">
-        <v>0.3254</v>
+        <v>-0.4702</v>
       </c>
       <c r="AC21" t="n">
-        <v>10.3828</v>
+        <v>0.5808</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-07-10 22:59
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1713 +568,1713 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>191.54</v>
+        <v>192.3</v>
       </c>
       <c r="C2" t="n">
-        <v>212.99</v>
+        <v>225.63</v>
       </c>
       <c r="D2" t="n">
-        <v>177.3</v>
+        <v>192.3</v>
       </c>
       <c r="E2" t="n">
-        <v>180.65</v>
+        <v>223.99</v>
       </c>
       <c r="F2" t="n">
-        <v>71.5153</v>
+        <v>70.7272</v>
       </c>
       <c r="G2" t="n">
-        <v>74.5284</v>
+        <v>76.42400000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>68.8415</v>
+        <v>69.4301</v>
       </c>
       <c r="I2" t="n">
-        <v>69.1109</v>
+        <v>75.83540000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>6.1681</v>
+        <v>6.0298</v>
       </c>
       <c r="K2" t="n">
-        <v>6.5734</v>
+        <v>6.0298</v>
       </c>
       <c r="L2" t="n">
-        <v>5.5355</v>
+        <v>4.8436</v>
       </c>
       <c r="M2" t="n">
-        <v>6.4943</v>
+        <v>4.9128</v>
       </c>
       <c r="N2" t="n">
-        <v>43.1209</v>
+        <v>43.4851</v>
       </c>
       <c r="O2" t="n">
-        <v>44.676</v>
+        <v>44.302</v>
       </c>
       <c r="P2" t="n">
-        <v>41.4082</v>
+        <v>39.8039</v>
       </c>
       <c r="Q2" t="n">
-        <v>44.5382</v>
+        <v>40.1878</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>192.3</v>
+        <v>222.22</v>
       </c>
       <c r="C3" t="n">
-        <v>225.63</v>
+        <v>242.4</v>
       </c>
       <c r="D3" t="n">
-        <v>192.3</v>
+        <v>214.74</v>
       </c>
       <c r="E3" t="n">
-        <v>223.99</v>
+        <v>234.68</v>
       </c>
       <c r="F3" t="n">
-        <v>70.7272</v>
+        <v>76.16459999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>76.42400000000001</v>
+        <v>78.18000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>69.4301</v>
+        <v>74.1193</v>
       </c>
       <c r="I3" t="n">
-        <v>75.83540000000001</v>
+        <v>77.3419</v>
       </c>
       <c r="J3" t="n">
-        <v>6.0298</v>
+        <v>4.9523</v>
       </c>
       <c r="K3" t="n">
-        <v>6.0298</v>
+        <v>5.0907</v>
       </c>
       <c r="L3" t="n">
-        <v>4.8436</v>
+        <v>4.4877</v>
       </c>
       <c r="M3" t="n">
-        <v>4.9128</v>
+        <v>4.6656</v>
       </c>
       <c r="N3" t="n">
-        <v>43.4851</v>
+        <v>40.0106</v>
       </c>
       <c r="O3" t="n">
-        <v>44.302</v>
+        <v>41.0933</v>
       </c>
       <c r="P3" t="n">
-        <v>39.8039</v>
+        <v>38.9476</v>
       </c>
       <c r="Q3" t="n">
-        <v>40.1878</v>
+        <v>39.4102</v>
       </c>
       <c r="R3" t="n">
-        <v>23.9911</v>
+        <v>4.7725</v>
       </c>
       <c r="U3" t="n">
-        <v>9.73</v>
+        <v>1.9865</v>
       </c>
       <c r="X3" t="n">
-        <v>-24.3521</v>
+        <v>-5.0318</v>
       </c>
       <c r="AA3" t="n">
-        <v>-9.767799999999999</v>
+        <v>-1.9349</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>222.22</v>
+        <v>265.99</v>
       </c>
       <c r="C4" t="n">
-        <v>242.4</v>
+        <v>274.88</v>
       </c>
       <c r="D4" t="n">
-        <v>214.74</v>
+        <v>261.6</v>
       </c>
       <c r="E4" t="n">
-        <v>234.68</v>
+        <v>272.5</v>
       </c>
       <c r="F4" t="n">
-        <v>76.16459999999999</v>
+        <v>82.6896</v>
       </c>
       <c r="G4" t="n">
-        <v>78.18000000000001</v>
+        <v>84.8347</v>
       </c>
       <c r="H4" t="n">
-        <v>74.1193</v>
+        <v>82.4502</v>
       </c>
       <c r="I4" t="n">
-        <v>77.3419</v>
+        <v>84.39570000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>4.9523</v>
+        <v>4.0231</v>
       </c>
       <c r="K4" t="n">
-        <v>5.0907</v>
+        <v>4.122</v>
       </c>
       <c r="L4" t="n">
-        <v>4.4877</v>
+        <v>3.865</v>
       </c>
       <c r="M4" t="n">
-        <v>4.6656</v>
+        <v>3.9045</v>
       </c>
       <c r="N4" t="n">
-        <v>40.0106</v>
+        <v>36.6641</v>
       </c>
       <c r="O4" t="n">
-        <v>41.0933</v>
+        <v>36.7723</v>
       </c>
       <c r="P4" t="n">
-        <v>38.9476</v>
+        <v>35.5814</v>
       </c>
       <c r="Q4" t="n">
-        <v>39.4102</v>
+        <v>35.7389</v>
       </c>
       <c r="R4" t="n">
-        <v>4.7725</v>
+        <v>16.1156</v>
       </c>
       <c r="U4" t="n">
-        <v>1.9865</v>
+        <v>9.1203</v>
       </c>
       <c r="X4" t="n">
-        <v>-5.0318</v>
+        <v>-16.313</v>
       </c>
       <c r="AA4" t="n">
-        <v>-1.9349</v>
+        <v>-9.3156</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>265.99</v>
+        <v>267.13</v>
       </c>
       <c r="C5" t="n">
-        <v>274.88</v>
+        <v>274.93</v>
       </c>
       <c r="D5" t="n">
-        <v>261.6</v>
+        <v>226</v>
       </c>
       <c r="E5" t="n">
-        <v>272.5</v>
+        <v>226.19</v>
       </c>
       <c r="F5" t="n">
-        <v>82.6896</v>
+        <v>83.9966</v>
       </c>
       <c r="G5" t="n">
-        <v>84.8347</v>
+        <v>84.63509999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>82.4502</v>
+        <v>79.67659999999999</v>
       </c>
       <c r="I5" t="n">
-        <v>84.39570000000001</v>
+        <v>79.74639999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>4.0231</v>
+        <v>3.9836</v>
       </c>
       <c r="K5" t="n">
-        <v>4.122</v>
+        <v>4.5965</v>
       </c>
       <c r="L5" t="n">
         <v>3.865</v>
       </c>
       <c r="M5" t="n">
-        <v>3.9045</v>
+        <v>4.5767</v>
       </c>
       <c r="N5" t="n">
-        <v>36.6641</v>
+        <v>35.9652</v>
       </c>
       <c r="O5" t="n">
-        <v>36.7723</v>
+        <v>37.7861</v>
       </c>
       <c r="P5" t="n">
-        <v>35.5814</v>
+        <v>35.6896</v>
       </c>
       <c r="Q5" t="n">
-        <v>35.7389</v>
+        <v>37.7468</v>
       </c>
       <c r="R5" t="n">
-        <v>16.1156</v>
+        <v>-16.9945</v>
       </c>
       <c r="S5" t="n">
-        <v>50.8442</v>
+        <v>0.9822</v>
       </c>
       <c r="U5" t="n">
-        <v>9.1203</v>
+        <v>-5.5089</v>
       </c>
       <c r="V5" t="n">
-        <v>22.1163</v>
+        <v>5.1572</v>
       </c>
       <c r="X5" t="n">
-        <v>-16.313</v>
+        <v>17.216</v>
       </c>
       <c r="Y5" t="n">
-        <v>-39.878</v>
+        <v>-6.8413</v>
       </c>
       <c r="AA5" t="n">
-        <v>-9.3156</v>
+        <v>5.6182</v>
       </c>
       <c r="AB5" t="n">
-        <v>-19.7567</v>
+        <v>-6.074</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>267.13</v>
+        <v>247.42</v>
       </c>
       <c r="C6" t="n">
-        <v>274.93</v>
+        <v>259.79</v>
       </c>
       <c r="D6" t="n">
-        <v>226</v>
+        <v>233.3</v>
       </c>
       <c r="E6" t="n">
-        <v>226.19</v>
+        <v>233.86</v>
       </c>
       <c r="F6" t="n">
-        <v>83.9966</v>
+        <v>81.4824</v>
       </c>
       <c r="G6" t="n">
-        <v>84.63509999999999</v>
+        <v>81.6221</v>
       </c>
       <c r="H6" t="n">
-        <v>79.67659999999999</v>
+        <v>76.7633</v>
       </c>
       <c r="I6" t="n">
-        <v>79.74639999999999</v>
+        <v>77.36190000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>3.9836</v>
+        <v>4.122</v>
       </c>
       <c r="K6" t="n">
-        <v>4.5965</v>
+        <v>4.4086</v>
       </c>
       <c r="L6" t="n">
-        <v>3.865</v>
+        <v>3.8749</v>
       </c>
       <c r="M6" t="n">
-        <v>4.5767</v>
+        <v>4.4086</v>
       </c>
       <c r="N6" t="n">
-        <v>35.9652</v>
+        <v>36.9397</v>
       </c>
       <c r="O6" t="n">
-        <v>37.7861</v>
+        <v>39.1641</v>
       </c>
       <c r="P6" t="n">
-        <v>35.6896</v>
+        <v>36.8708</v>
       </c>
       <c r="Q6" t="n">
-        <v>37.7468</v>
+        <v>38.8984</v>
       </c>
       <c r="R6" t="n">
-        <v>-16.9945</v>
+        <v>3.391</v>
       </c>
       <c r="S6" t="n">
-        <v>0.9822</v>
+        <v>-0.3494</v>
       </c>
       <c r="U6" t="n">
-        <v>-5.5089</v>
+        <v>-2.9901</v>
       </c>
       <c r="V6" t="n">
-        <v>5.1572</v>
+        <v>0.0259</v>
       </c>
       <c r="X6" t="n">
-        <v>17.216</v>
+        <v>-3.673</v>
       </c>
       <c r="Y6" t="n">
-        <v>-6.8413</v>
+        <v>-5.5084</v>
       </c>
       <c r="AA6" t="n">
-        <v>5.6182</v>
+        <v>3.0509</v>
       </c>
       <c r="AB6" t="n">
-        <v>-6.074</v>
+        <v>-1.2986</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>247.42</v>
+        <v>266.04</v>
       </c>
       <c r="C7" t="n">
-        <v>259.79</v>
+        <v>286.15</v>
       </c>
       <c r="D7" t="n">
-        <v>233.3</v>
+        <v>265</v>
       </c>
       <c r="E7" t="n">
-        <v>233.86</v>
+        <v>279.29</v>
       </c>
       <c r="F7" t="n">
-        <v>81.4824</v>
+        <v>81.9114</v>
       </c>
       <c r="G7" t="n">
-        <v>81.6221</v>
+        <v>83.408</v>
       </c>
       <c r="H7" t="n">
-        <v>76.7633</v>
+        <v>80.4448</v>
       </c>
       <c r="I7" t="n">
-        <v>77.36190000000001</v>
+        <v>82.67959999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>4.122</v>
+        <v>3.8156</v>
       </c>
       <c r="K7" t="n">
-        <v>4.4086</v>
+        <v>3.8254</v>
       </c>
       <c r="L7" t="n">
-        <v>3.8749</v>
+        <v>3.4103</v>
       </c>
       <c r="M7" t="n">
-        <v>4.4086</v>
+        <v>3.5487</v>
       </c>
       <c r="N7" t="n">
-        <v>36.9397</v>
+        <v>36.6149</v>
       </c>
       <c r="O7" t="n">
-        <v>39.1641</v>
+        <v>37.3531</v>
       </c>
       <c r="P7" t="n">
-        <v>36.8708</v>
+        <v>35.857</v>
       </c>
       <c r="Q7" t="n">
-        <v>38.8984</v>
+        <v>36.1719</v>
       </c>
       <c r="R7" t="n">
-        <v>3.391</v>
+        <v>19.4262</v>
       </c>
       <c r="S7" t="n">
-        <v>-0.3494</v>
+        <v>2.4917</v>
       </c>
       <c r="T7" t="n">
-        <v>29.4547</v>
+        <v>24.6886</v>
       </c>
       <c r="U7" t="n">
-        <v>-2.9901</v>
+        <v>6.8738</v>
       </c>
       <c r="V7" t="n">
-        <v>0.0259</v>
+        <v>-2.0334</v>
       </c>
       <c r="W7" t="n">
-        <v>11.9388</v>
+        <v>9.0251</v>
       </c>
       <c r="X7" t="n">
-        <v>-3.673</v>
+        <v>-19.5051</v>
       </c>
       <c r="Y7" t="n">
-        <v>-5.5084</v>
+        <v>-9.1126</v>
       </c>
       <c r="Z7" t="n">
-        <v>-32.1159</v>
+        <v>-27.7662</v>
       </c>
       <c r="AA7" t="n">
-        <v>3.0509</v>
+        <v>-7.0093</v>
       </c>
       <c r="AB7" t="n">
-        <v>-1.2986</v>
+        <v>1.2116</v>
       </c>
       <c r="AC7" t="n">
-        <v>-12.6628</v>
+        <v>-9.992800000000001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>266.04</v>
+        <v>299.26</v>
       </c>
       <c r="C8" t="n">
-        <v>286.15</v>
+        <v>302</v>
       </c>
       <c r="D8" t="n">
-        <v>265</v>
+        <v>286.24</v>
       </c>
       <c r="E8" t="n">
-        <v>279.29</v>
+        <v>300.77</v>
       </c>
       <c r="F8" t="n">
-        <v>81.9114</v>
+        <v>83.7572</v>
       </c>
       <c r="G8" t="n">
-        <v>83.408</v>
+        <v>84.9145</v>
       </c>
       <c r="H8" t="n">
-        <v>80.4448</v>
+        <v>81.203</v>
       </c>
       <c r="I8" t="n">
-        <v>82.67959999999999</v>
+        <v>82.3903</v>
       </c>
       <c r="J8" t="n">
-        <v>3.8156</v>
+        <v>3.2917</v>
       </c>
       <c r="K8" t="n">
-        <v>3.8254</v>
+        <v>3.4498</v>
       </c>
       <c r="L8" t="n">
-        <v>3.4103</v>
+        <v>3.2521</v>
       </c>
       <c r="M8" t="n">
-        <v>3.5487</v>
+        <v>3.262</v>
       </c>
       <c r="N8" t="n">
-        <v>36.6149</v>
+        <v>35.7389</v>
       </c>
       <c r="O8" t="n">
-        <v>37.3531</v>
+        <v>36.8511</v>
       </c>
       <c r="P8" t="n">
-        <v>35.857</v>
+        <v>35.2369</v>
       </c>
       <c r="Q8" t="n">
-        <v>36.1719</v>
+        <v>36.3491</v>
       </c>
       <c r="R8" t="n">
-        <v>19.4262</v>
+        <v>7.6909</v>
       </c>
       <c r="S8" t="n">
-        <v>2.4917</v>
+        <v>32.9723</v>
       </c>
       <c r="T8" t="n">
-        <v>24.6886</v>
+        <v>28.1618</v>
       </c>
       <c r="U8" t="n">
-        <v>6.8738</v>
+        <v>-0.3499</v>
       </c>
       <c r="V8" t="n">
-        <v>-2.0334</v>
+        <v>3.3154</v>
       </c>
       <c r="W8" t="n">
-        <v>9.0251</v>
+        <v>6.5274</v>
       </c>
       <c r="X8" t="n">
-        <v>-19.5051</v>
+        <v>-8.079000000000001</v>
       </c>
       <c r="Y8" t="n">
-        <v>-9.1126</v>
+        <v>-28.7259</v>
       </c>
       <c r="Z8" t="n">
-        <v>-27.7662</v>
+        <v>-30.084</v>
       </c>
       <c r="AA8" t="n">
-        <v>-7.0093</v>
+        <v>0.4899</v>
       </c>
       <c r="AB8" t="n">
-        <v>1.2116</v>
+        <v>-3.7028</v>
       </c>
       <c r="AC8" t="n">
-        <v>-9.992800000000001</v>
+        <v>-7.7673</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>299.26</v>
+        <v>236</v>
       </c>
       <c r="C9" t="n">
-        <v>302</v>
+        <v>252.98</v>
       </c>
       <c r="D9" t="n">
-        <v>286.24</v>
+        <v>223</v>
       </c>
       <c r="E9" t="n">
-        <v>300.77</v>
+        <v>231.42</v>
       </c>
       <c r="F9" t="n">
-        <v>83.7572</v>
+        <v>74.9474</v>
       </c>
       <c r="G9" t="n">
-        <v>84.9145</v>
+        <v>77.56140000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>81.203</v>
+        <v>73.7402</v>
       </c>
       <c r="I9" t="n">
-        <v>82.3903</v>
+        <v>74.26900000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>3.2917</v>
+        <v>3.99</v>
       </c>
       <c r="K9" t="n">
-        <v>3.4498</v>
+        <v>4.13</v>
       </c>
       <c r="L9" t="n">
-        <v>3.2521</v>
+        <v>3.8</v>
       </c>
       <c r="M9" t="n">
-        <v>3.262</v>
+        <v>4.04</v>
       </c>
       <c r="N9" t="n">
-        <v>35.7389</v>
+        <v>39.6267</v>
       </c>
       <c r="O9" t="n">
-        <v>36.8511</v>
+        <v>40.1582</v>
       </c>
       <c r="P9" t="n">
-        <v>35.2369</v>
+        <v>38.4653</v>
       </c>
       <c r="Q9" t="n">
-        <v>36.3491</v>
+        <v>39.922</v>
       </c>
       <c r="R9" t="n">
-        <v>7.6909</v>
+        <v>-23.0575</v>
       </c>
       <c r="S9" t="n">
-        <v>32.9723</v>
+        <v>-1.0434</v>
       </c>
       <c r="T9" t="n">
-        <v>28.1618</v>
+        <v>-15.0752</v>
       </c>
       <c r="U9" t="n">
-        <v>-0.3499</v>
+        <v>-9.857100000000001</v>
       </c>
       <c r="V9" t="n">
-        <v>3.3154</v>
+        <v>-3.998</v>
       </c>
       <c r="W9" t="n">
-        <v>6.5274</v>
+        <v>-11.9991</v>
       </c>
       <c r="X9" t="n">
-        <v>-8.079000000000001</v>
+        <v>23.8504</v>
       </c>
       <c r="Y9" t="n">
-        <v>-28.7259</v>
+        <v>-8.360900000000001</v>
       </c>
       <c r="Z9" t="n">
-        <v>-30.084</v>
+        <v>3.4704</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.4899</v>
+        <v>9.8294</v>
       </c>
       <c r="AB9" t="n">
-        <v>-3.7028</v>
+        <v>2.6315</v>
       </c>
       <c r="AC9" t="n">
-        <v>-7.7673</v>
+        <v>11.7046</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>236</v>
+        <v>233.11</v>
       </c>
       <c r="C10" t="n">
-        <v>252.98</v>
+        <v>237</v>
       </c>
       <c r="D10" t="n">
-        <v>223</v>
+        <v>211.13</v>
       </c>
       <c r="E10" t="n">
-        <v>231.42</v>
+        <v>229.57</v>
       </c>
       <c r="F10" t="n">
-        <v>74.9474</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>77.56140000000001</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>73.7402</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>74.26900000000001</v>
+        <v>73.3</v>
       </c>
       <c r="J10" t="n">
-        <v>3.99</v>
+        <v>4</v>
       </c>
       <c r="K10" t="n">
-        <v>4.13</v>
+        <v>4.39</v>
       </c>
       <c r="L10" t="n">
-        <v>3.8</v>
+        <v>3.92</v>
       </c>
       <c r="M10" t="n">
-        <v>4.04</v>
+        <v>4.08</v>
       </c>
       <c r="N10" t="n">
-        <v>39.6267</v>
+        <v>39.66</v>
       </c>
       <c r="O10" t="n">
-        <v>40.1582</v>
+        <v>41.49</v>
       </c>
       <c r="P10" t="n">
-        <v>38.4653</v>
+        <v>38.9</v>
       </c>
       <c r="Q10" t="n">
-        <v>39.922</v>
+        <v>40.45</v>
       </c>
       <c r="R10" t="n">
-        <v>-23.0575</v>
+        <v>-0.7994</v>
       </c>
       <c r="S10" t="n">
-        <v>-1.0434</v>
+        <v>-17.8023</v>
       </c>
       <c r="T10" t="n">
-        <v>-15.0752</v>
+        <v>1.4943</v>
       </c>
       <c r="U10" t="n">
-        <v>-9.857100000000001</v>
+        <v>-1.3047</v>
       </c>
       <c r="V10" t="n">
-        <v>-3.998</v>
+        <v>-11.3445</v>
       </c>
       <c r="W10" t="n">
-        <v>-11.9991</v>
+        <v>-8.083600000000001</v>
       </c>
       <c r="X10" t="n">
-        <v>23.8504</v>
+        <v>0.9901</v>
       </c>
       <c r="Y10" t="n">
-        <v>-8.360900000000001</v>
+        <v>14.9717</v>
       </c>
       <c r="Z10" t="n">
-        <v>3.4704</v>
+        <v>-10.8528</v>
       </c>
       <c r="AA10" t="n">
-        <v>9.8294</v>
+        <v>1.3226</v>
       </c>
       <c r="AB10" t="n">
-        <v>2.6315</v>
+        <v>11.8271</v>
       </c>
       <c r="AC10" t="n">
-        <v>11.7046</v>
+        <v>7.1614</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>233.11</v>
+        <v>268.05</v>
       </c>
       <c r="C11" t="n">
-        <v>237</v>
+        <v>268.4</v>
       </c>
       <c r="D11" t="n">
-        <v>211.13</v>
+        <v>225.74</v>
       </c>
       <c r="E11" t="n">
-        <v>229.57</v>
+        <v>252.61</v>
       </c>
       <c r="F11" t="n">
-        <v>74.79000000000001</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>76.18000000000001</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="H11" t="n">
-        <v>71.34999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>73.3</v>
+        <v>74.95</v>
       </c>
       <c r="J11" t="n">
-        <v>4</v>
+        <v>3.38</v>
       </c>
       <c r="K11" t="n">
-        <v>4.39</v>
+        <v>4.15</v>
       </c>
       <c r="L11" t="n">
-        <v>3.92</v>
+        <v>3.37</v>
       </c>
       <c r="M11" t="n">
-        <v>4.08</v>
+        <v>3.63</v>
       </c>
       <c r="N11" t="n">
-        <v>39.66</v>
+        <v>37.87</v>
       </c>
       <c r="O11" t="n">
-        <v>41.49</v>
+        <v>41.37</v>
       </c>
       <c r="P11" t="n">
-        <v>38.9</v>
+        <v>37.71</v>
       </c>
       <c r="Q11" t="n">
-        <v>40.45</v>
+        <v>39.47</v>
       </c>
       <c r="R11" t="n">
-        <v>-0.7994</v>
+        <v>10.0362</v>
       </c>
       <c r="S11" t="n">
-        <v>-17.8023</v>
+        <v>-16.0122</v>
       </c>
       <c r="T11" t="n">
-        <v>1.4943</v>
+        <v>8.0176</v>
       </c>
       <c r="U11" t="n">
-        <v>-1.3047</v>
+        <v>2.251</v>
       </c>
       <c r="V11" t="n">
-        <v>-11.3445</v>
+        <v>-9.0306</v>
       </c>
       <c r="W11" t="n">
-        <v>-8.083600000000001</v>
+        <v>-3.1177</v>
       </c>
       <c r="X11" t="n">
-        <v>0.9901</v>
+        <v>-11.0294</v>
       </c>
       <c r="Y11" t="n">
-        <v>14.9717</v>
+        <v>11.2814</v>
       </c>
       <c r="Z11" t="n">
-        <v>-10.8528</v>
+        <v>-17.6609</v>
       </c>
       <c r="AA11" t="n">
-        <v>1.3226</v>
+        <v>-2.4227</v>
       </c>
       <c r="AB11" t="n">
-        <v>11.8271</v>
+        <v>8.585900000000001</v>
       </c>
       <c r="AC11" t="n">
-        <v>7.1614</v>
+        <v>1.4695</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>268.05</v>
+        <v>226.24</v>
       </c>
       <c r="C12" t="n">
-        <v>268.4</v>
+        <v>231.25</v>
       </c>
       <c r="D12" t="n">
-        <v>225.74</v>
+        <v>212.1</v>
       </c>
       <c r="E12" t="n">
-        <v>252.61</v>
+        <v>215.6</v>
       </c>
       <c r="F12" t="n">
-        <v>77.95999999999999</v>
+        <v>72.09</v>
       </c>
       <c r="G12" t="n">
-        <v>78.23999999999999</v>
+        <v>74.69</v>
       </c>
       <c r="H12" t="n">
-        <v>71.59999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="I12" t="n">
-        <v>74.95</v>
+        <v>71.83</v>
       </c>
       <c r="J12" t="n">
-        <v>3.38</v>
+        <v>4.04</v>
       </c>
       <c r="K12" t="n">
-        <v>4.15</v>
+        <v>4.25</v>
       </c>
       <c r="L12" t="n">
-        <v>3.37</v>
+        <v>3.95</v>
       </c>
       <c r="M12" t="n">
-        <v>3.63</v>
+        <v>4.24</v>
       </c>
       <c r="N12" t="n">
-        <v>37.87</v>
+        <v>41.08</v>
       </c>
       <c r="O12" t="n">
-        <v>41.37</v>
+        <v>41.79</v>
       </c>
       <c r="P12" t="n">
-        <v>37.71</v>
+        <v>39.69</v>
       </c>
       <c r="Q12" t="n">
-        <v>39.47</v>
+        <v>41.31</v>
       </c>
       <c r="R12" t="n">
-        <v>10.0362</v>
+        <v>-14.651</v>
       </c>
       <c r="S12" t="n">
-        <v>-16.0122</v>
+        <v>-6.8361</v>
       </c>
       <c r="T12" t="n">
-        <v>8.0176</v>
+        <v>-22.8043</v>
       </c>
       <c r="U12" t="n">
-        <v>2.251</v>
+        <v>-4.1628</v>
       </c>
       <c r="V12" t="n">
-        <v>-9.0306</v>
+        <v>-3.284</v>
       </c>
       <c r="W12" t="n">
-        <v>-3.1177</v>
+        <v>-13.1225</v>
       </c>
       <c r="X12" t="n">
-        <v>-11.0294</v>
+        <v>16.8044</v>
       </c>
       <c r="Y12" t="n">
-        <v>11.2814</v>
+        <v>4.9505</v>
       </c>
       <c r="Z12" t="n">
-        <v>-17.6609</v>
+        <v>19.4804</v>
       </c>
       <c r="AA12" t="n">
-        <v>-2.4227</v>
+        <v>4.6618</v>
       </c>
       <c r="AB12" t="n">
-        <v>8.585900000000001</v>
+        <v>3.4768</v>
       </c>
       <c r="AC12" t="n">
-        <v>1.4695</v>
+        <v>14.2047</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>226.24</v>
+        <v>216.36</v>
       </c>
       <c r="C13" t="n">
-        <v>231.25</v>
+        <v>238.65</v>
       </c>
       <c r="D13" t="n">
-        <v>212.1</v>
+        <v>192.3</v>
       </c>
       <c r="E13" t="n">
-        <v>215.6</v>
+        <v>236.52</v>
       </c>
       <c r="F13" t="n">
-        <v>72.09</v>
+        <v>74.12</v>
       </c>
       <c r="G13" t="n">
-        <v>74.69</v>
+        <v>77.38</v>
       </c>
       <c r="H13" t="n">
-        <v>70.72</v>
+        <v>71.45</v>
       </c>
       <c r="I13" t="n">
-        <v>71.83</v>
+        <v>77.19</v>
       </c>
       <c r="J13" t="n">
-        <v>4.04</v>
+        <v>4.16</v>
       </c>
       <c r="K13" t="n">
-        <v>4.25</v>
+        <v>4.63</v>
       </c>
       <c r="L13" t="n">
-        <v>3.95</v>
+        <v>3.7</v>
       </c>
       <c r="M13" t="n">
-        <v>4.24</v>
+        <v>3.72</v>
       </c>
       <c r="N13" t="n">
-        <v>41.08</v>
+        <v>39.91</v>
       </c>
       <c r="O13" t="n">
-        <v>41.79</v>
+        <v>41.43</v>
       </c>
       <c r="P13" t="n">
-        <v>39.69</v>
+        <v>38.08</v>
       </c>
       <c r="Q13" t="n">
-        <v>41.31</v>
+        <v>38.16</v>
       </c>
       <c r="R13" t="n">
-        <v>-14.651</v>
+        <v>9.703200000000001</v>
       </c>
       <c r="S13" t="n">
-        <v>-6.8361</v>
+        <v>3.0274</v>
       </c>
       <c r="T13" t="n">
-        <v>-22.8043</v>
+        <v>-21.3618</v>
       </c>
       <c r="U13" t="n">
-        <v>-4.1628</v>
+        <v>7.4621</v>
       </c>
       <c r="V13" t="n">
-        <v>-3.284</v>
+        <v>5.307</v>
       </c>
       <c r="W13" t="n">
-        <v>-13.1225</v>
+        <v>-6.3118</v>
       </c>
       <c r="X13" t="n">
-        <v>16.8044</v>
+        <v>-12.2642</v>
       </c>
       <c r="Y13" t="n">
-        <v>4.9505</v>
+        <v>-8.823499999999999</v>
       </c>
       <c r="Z13" t="n">
-        <v>19.4804</v>
+        <v>14.0405</v>
       </c>
       <c r="AA13" t="n">
-        <v>4.6618</v>
+        <v>-7.6253</v>
       </c>
       <c r="AB13" t="n">
-        <v>3.4768</v>
+        <v>-5.6613</v>
       </c>
       <c r="AC13" t="n">
-        <v>14.2047</v>
+        <v>4.982</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>216.36</v>
+        <v>241.45</v>
       </c>
       <c r="C14" t="n">
-        <v>238.65</v>
+        <v>272</v>
       </c>
       <c r="D14" t="n">
-        <v>192.3</v>
+        <v>240.59</v>
       </c>
       <c r="E14" t="n">
-        <v>236.52</v>
+        <v>266.71</v>
       </c>
       <c r="F14" t="n">
-        <v>74.12</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>77.38</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="H14" t="n">
-        <v>71.45</v>
+        <v>77.15000000000001</v>
       </c>
       <c r="I14" t="n">
-        <v>77.19</v>
+        <v>81</v>
       </c>
       <c r="J14" t="n">
-        <v>4.16</v>
+        <v>3.66</v>
       </c>
       <c r="K14" t="n">
-        <v>4.63</v>
+        <v>3.68</v>
       </c>
       <c r="L14" t="n">
-        <v>3.7</v>
+        <v>3.17</v>
       </c>
       <c r="M14" t="n">
-        <v>3.72</v>
+        <v>3.24</v>
       </c>
       <c r="N14" t="n">
-        <v>39.91</v>
+        <v>38.16</v>
       </c>
       <c r="O14" t="n">
-        <v>41.43</v>
+        <v>38.2</v>
       </c>
       <c r="P14" t="n">
-        <v>38.08</v>
+        <v>36.03</v>
       </c>
       <c r="Q14" t="n">
-        <v>38.16</v>
+        <v>36.31</v>
       </c>
       <c r="R14" t="n">
-        <v>9.703200000000001</v>
+        <v>12.7642</v>
       </c>
       <c r="S14" t="n">
-        <v>3.0274</v>
+        <v>5.5817</v>
       </c>
       <c r="T14" t="n">
-        <v>-21.3618</v>
+        <v>15.2493</v>
       </c>
       <c r="U14" t="n">
-        <v>7.4621</v>
+        <v>4.9359</v>
       </c>
       <c r="V14" t="n">
-        <v>5.307</v>
+        <v>8.071999999999999</v>
       </c>
       <c r="W14" t="n">
-        <v>-6.3118</v>
+        <v>9.063000000000001</v>
       </c>
       <c r="X14" t="n">
-        <v>-12.2642</v>
+        <v>-12.9032</v>
       </c>
       <c r="Y14" t="n">
-        <v>-8.823499999999999</v>
+        <v>-10.7438</v>
       </c>
       <c r="Z14" t="n">
-        <v>14.0405</v>
+        <v>-19.802</v>
       </c>
       <c r="AA14" t="n">
-        <v>-7.6253</v>
+        <v>-4.848</v>
       </c>
       <c r="AB14" t="n">
-        <v>-5.6613</v>
+        <v>-8.0061</v>
       </c>
       <c r="AC14" t="n">
-        <v>4.982</v>
+        <v>-9.047599999999999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>241.45</v>
+        <v>237.79</v>
       </c>
       <c r="C15" t="n">
-        <v>272</v>
+        <v>246.47</v>
       </c>
       <c r="D15" t="n">
-        <v>240.59</v>
+        <v>215.38</v>
       </c>
       <c r="E15" t="n">
-        <v>266.71</v>
+        <v>217.55</v>
       </c>
       <c r="F15" t="n">
-        <v>77.23999999999999</v>
+        <v>78.72</v>
       </c>
       <c r="G15" t="n">
-        <v>81.54000000000001</v>
+        <v>79.64</v>
       </c>
       <c r="H15" t="n">
-        <v>77.15000000000001</v>
+        <v>77.23</v>
       </c>
       <c r="I15" t="n">
-        <v>81</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>3.66</v>
+        <v>3.59</v>
       </c>
       <c r="K15" t="n">
-        <v>3.68</v>
+        <v>3.89</v>
       </c>
       <c r="L15" t="n">
-        <v>3.17</v>
+        <v>3.51</v>
       </c>
       <c r="M15" t="n">
-        <v>3.24</v>
+        <v>3.86</v>
       </c>
       <c r="N15" t="n">
-        <v>38.16</v>
+        <v>37.31</v>
       </c>
       <c r="O15" t="n">
-        <v>38.2</v>
+        <v>37.98</v>
       </c>
       <c r="P15" t="n">
-        <v>36.03</v>
+        <v>36.9</v>
       </c>
       <c r="Q15" t="n">
-        <v>36.31</v>
+        <v>37.88</v>
       </c>
       <c r="R15" t="n">
-        <v>12.7642</v>
+        <v>-18.432</v>
       </c>
       <c r="S15" t="n">
-        <v>5.5817</v>
+        <v>0.9045</v>
       </c>
       <c r="T15" t="n">
-        <v>15.2493</v>
+        <v>-5.2359</v>
       </c>
       <c r="U15" t="n">
-        <v>4.9359</v>
+        <v>-4.3704</v>
       </c>
       <c r="V15" t="n">
-        <v>8.071999999999999</v>
+        <v>7.838</v>
       </c>
       <c r="W15" t="n">
-        <v>9.063000000000001</v>
+        <v>5.6753</v>
       </c>
       <c r="X15" t="n">
-        <v>-12.9032</v>
+        <v>19.1358</v>
       </c>
       <c r="Y15" t="n">
-        <v>-10.7438</v>
+        <v>-8.962300000000001</v>
       </c>
       <c r="Z15" t="n">
-        <v>-19.802</v>
+        <v>-5.3922</v>
       </c>
       <c r="AA15" t="n">
-        <v>-4.848</v>
+        <v>4.3239</v>
       </c>
       <c r="AB15" t="n">
-        <v>-8.0061</v>
+        <v>-8.303100000000001</v>
       </c>
       <c r="AC15" t="n">
-        <v>-9.047599999999999</v>
+        <v>-6.3535</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>237.79</v>
+        <v>219.23</v>
       </c>
       <c r="C16" t="n">
-        <v>246.47</v>
+        <v>226.13</v>
       </c>
       <c r="D16" t="n">
-        <v>215.38</v>
+        <v>168.88</v>
       </c>
       <c r="E16" t="n">
-        <v>217.55</v>
+        <v>181.47</v>
       </c>
       <c r="F16" t="n">
-        <v>78.72</v>
+        <v>77.45</v>
       </c>
       <c r="G16" t="n">
-        <v>79.64</v>
+        <v>79.14</v>
       </c>
       <c r="H16" t="n">
-        <v>77.23</v>
+        <v>71.72</v>
       </c>
       <c r="I16" t="n">
-        <v>77.45999999999999</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="J16" t="n">
-        <v>3.59</v>
+        <v>3.84</v>
       </c>
       <c r="K16" t="n">
-        <v>3.89</v>
+        <v>4.74</v>
       </c>
       <c r="L16" t="n">
-        <v>3.51</v>
+        <v>3.71</v>
       </c>
       <c r="M16" t="n">
-        <v>3.86</v>
+        <v>4.51</v>
       </c>
       <c r="N16" t="n">
-        <v>37.31</v>
+        <v>37.91</v>
       </c>
       <c r="O16" t="n">
-        <v>37.98</v>
+        <v>40.72</v>
       </c>
       <c r="P16" t="n">
-        <v>36.9</v>
+        <v>37.08</v>
       </c>
       <c r="Q16" t="n">
-        <v>37.88</v>
+        <v>39.95</v>
       </c>
       <c r="R16" t="n">
-        <v>-18.432</v>
+        <v>-16.5847</v>
       </c>
       <c r="S16" t="n">
-        <v>0.9045</v>
+        <v>-23.275</v>
       </c>
       <c r="T16" t="n">
-        <v>-5.2359</v>
+        <v>-28.162</v>
       </c>
       <c r="U16" t="n">
-        <v>-4.3704</v>
+        <v>-5.306</v>
       </c>
       <c r="V16" t="n">
-        <v>7.838</v>
+        <v>-4.9747</v>
       </c>
       <c r="W16" t="n">
-        <v>5.6753</v>
+        <v>-2.1348</v>
       </c>
       <c r="X16" t="n">
-        <v>19.1358</v>
+        <v>16.8394</v>
       </c>
       <c r="Y16" t="n">
-        <v>-8.962300000000001</v>
+        <v>21.2366</v>
       </c>
       <c r="Z16" t="n">
-        <v>-5.3922</v>
+        <v>24.2424</v>
       </c>
       <c r="AA16" t="n">
-        <v>4.3239</v>
+        <v>5.4646</v>
       </c>
       <c r="AB16" t="n">
-        <v>-8.303100000000001</v>
+        <v>4.6908</v>
       </c>
       <c r="AC16" t="n">
-        <v>-6.3535</v>
+        <v>1.2161</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>219.23</v>
+        <v>197.21</v>
       </c>
       <c r="C17" t="n">
-        <v>226.13</v>
+        <v>210.8</v>
       </c>
       <c r="D17" t="n">
-        <v>168.88</v>
+        <v>194.22</v>
       </c>
       <c r="E17" t="n">
-        <v>181.47</v>
+        <v>194.65</v>
       </c>
       <c r="F17" t="n">
+        <v>75.54000000000001</v>
+      </c>
+      <c r="G17" t="n">
         <v>77.45</v>
       </c>
-      <c r="G17" t="n">
-        <v>79.14</v>
-      </c>
       <c r="H17" t="n">
-        <v>71.72</v>
+        <v>75.11</v>
       </c>
       <c r="I17" t="n">
-        <v>73.34999999999999</v>
+        <v>76.42</v>
       </c>
       <c r="J17" t="n">
-        <v>3.84</v>
+        <v>4.11</v>
       </c>
       <c r="K17" t="n">
-        <v>4.74</v>
+        <v>4.18</v>
       </c>
       <c r="L17" t="n">
-        <v>3.71</v>
+        <v>3.77</v>
       </c>
       <c r="M17" t="n">
-        <v>4.51</v>
+        <v>4.17</v>
       </c>
       <c r="N17" t="n">
-        <v>37.91</v>
+        <v>38.75</v>
       </c>
       <c r="O17" t="n">
-        <v>40.72</v>
+        <v>38.98</v>
       </c>
       <c r="P17" t="n">
-        <v>37.08</v>
+        <v>37.71</v>
       </c>
       <c r="Q17" t="n">
-        <v>39.95</v>
+        <v>38.28</v>
       </c>
       <c r="R17" t="n">
-        <v>-16.5847</v>
+        <v>7.2629</v>
       </c>
       <c r="S17" t="n">
-        <v>-23.275</v>
+        <v>-27.0181</v>
       </c>
       <c r="T17" t="n">
-        <v>-28.162</v>
+        <v>-9.7171</v>
       </c>
       <c r="U17" t="n">
-        <v>-5.306</v>
+        <v>4.1854</v>
       </c>
       <c r="V17" t="n">
-        <v>-4.9747</v>
+        <v>-5.6543</v>
       </c>
       <c r="W17" t="n">
-        <v>-2.1348</v>
+        <v>6.3901</v>
       </c>
       <c r="X17" t="n">
-        <v>16.8394</v>
+        <v>-7.5388</v>
       </c>
       <c r="Y17" t="n">
-        <v>21.2366</v>
+        <v>28.7037</v>
       </c>
       <c r="Z17" t="n">
-        <v>24.2424</v>
+        <v>-1.6509</v>
       </c>
       <c r="AA17" t="n">
-        <v>5.4646</v>
+        <v>-4.1802</v>
       </c>
       <c r="AB17" t="n">
-        <v>4.6908</v>
+        <v>5.4255</v>
       </c>
       <c r="AC17" t="n">
-        <v>1.2161</v>
+        <v>-7.3348</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>197.21</v>
+        <v>165.4</v>
       </c>
       <c r="C18" t="n">
-        <v>210.8</v>
+        <v>171.88</v>
       </c>
       <c r="D18" t="n">
-        <v>194.22</v>
+        <v>150.08</v>
       </c>
       <c r="E18" t="n">
-        <v>194.65</v>
+        <v>165.28</v>
       </c>
       <c r="F18" t="n">
-        <v>75.54000000000001</v>
+        <v>73.7</v>
       </c>
       <c r="G18" t="n">
-        <v>77.45</v>
+        <v>74.39</v>
       </c>
       <c r="H18" t="n">
-        <v>75.11</v>
+        <v>70.76000000000001</v>
       </c>
       <c r="I18" t="n">
-        <v>76.42</v>
+        <v>72.23</v>
       </c>
       <c r="J18" t="n">
-        <v>4.11</v>
+        <v>4.8</v>
       </c>
       <c r="K18" t="n">
-        <v>4.18</v>
+        <v>5.14</v>
       </c>
       <c r="L18" t="n">
-        <v>3.77</v>
+        <v>4.66</v>
       </c>
       <c r="M18" t="n">
-        <v>4.17</v>
+        <v>4.8</v>
       </c>
       <c r="N18" t="n">
-        <v>38.75</v>
+        <v>39.64</v>
       </c>
       <c r="O18" t="n">
-        <v>38.98</v>
+        <v>41.11</v>
       </c>
       <c r="P18" t="n">
-        <v>37.71</v>
+        <v>39.29</v>
       </c>
       <c r="Q18" t="n">
-        <v>38.28</v>
+        <v>40.38</v>
       </c>
       <c r="R18" t="n">
-        <v>7.2629</v>
+        <v>-15.0886</v>
       </c>
       <c r="S18" t="n">
-        <v>-27.0181</v>
+        <v>-24.0267</v>
       </c>
       <c r="T18" t="n">
-        <v>-9.7171</v>
+        <v>-30.1201</v>
       </c>
       <c r="U18" t="n">
-        <v>4.1854</v>
+        <v>-5.4829</v>
       </c>
       <c r="V18" t="n">
-        <v>-5.6543</v>
+        <v>-6.7519</v>
       </c>
       <c r="W18" t="n">
-        <v>6.3901</v>
+        <v>-6.4257</v>
       </c>
       <c r="X18" t="n">
-        <v>-7.5388</v>
+        <v>15.1079</v>
       </c>
       <c r="Y18" t="n">
-        <v>28.7037</v>
+        <v>24.3523</v>
       </c>
       <c r="Z18" t="n">
-        <v>-1.6509</v>
+        <v>29.0323</v>
       </c>
       <c r="AA18" t="n">
-        <v>-4.1802</v>
+        <v>5.4859</v>
       </c>
       <c r="AB18" t="n">
-        <v>5.4255</v>
+        <v>6.5998</v>
       </c>
       <c r="AC18" t="n">
-        <v>-7.3348</v>
+        <v>5.8176</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>165.4</v>
+        <v>159.21</v>
       </c>
       <c r="C19" t="n">
-        <v>171.88</v>
+        <v>176.75</v>
       </c>
       <c r="D19" t="n">
-        <v>150.08</v>
+        <v>158.87</v>
       </c>
       <c r="E19" t="n">
-        <v>165.28</v>
+        <v>174.82</v>
       </c>
       <c r="F19" t="n">
-        <v>73.7</v>
+        <v>70.8</v>
       </c>
       <c r="G19" t="n">
-        <v>74.39</v>
+        <v>73.02</v>
       </c>
       <c r="H19" t="n">
-        <v>70.76000000000001</v>
+        <v>69.56999999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>72.23</v>
+        <v>72.72</v>
       </c>
       <c r="J19" t="n">
-        <v>4.8</v>
+        <v>4.98</v>
       </c>
       <c r="K19" t="n">
-        <v>5.14</v>
+        <v>4.99</v>
       </c>
       <c r="L19" t="n">
-        <v>4.66</v>
+        <v>4.46</v>
       </c>
       <c r="M19" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="N19" t="n">
-        <v>39.64</v>
+        <v>41.18</v>
       </c>
       <c r="O19" t="n">
-        <v>41.11</v>
+        <v>41.86</v>
       </c>
       <c r="P19" t="n">
-        <v>39.29</v>
+        <v>39.93</v>
       </c>
       <c r="Q19" t="n">
-        <v>40.38</v>
+        <v>40.08</v>
       </c>
       <c r="R19" t="n">
-        <v>-15.0886</v>
+        <v>5.772</v>
       </c>
       <c r="S19" t="n">
-        <v>-24.0267</v>
+        <v>-3.6645</v>
       </c>
       <c r="T19" t="n">
-        <v>-30.1201</v>
+        <v>-34.4532</v>
       </c>
       <c r="U19" t="n">
-        <v>-5.4829</v>
+        <v>0.6784</v>
       </c>
       <c r="V19" t="n">
-        <v>-6.7519</v>
+        <v>-0.8589</v>
       </c>
       <c r="W19" t="n">
-        <v>-6.4257</v>
+        <v>-10.2222</v>
       </c>
       <c r="X19" t="n">
-        <v>15.1079</v>
+        <v>-6.25</v>
       </c>
       <c r="Y19" t="n">
-        <v>24.3523</v>
+        <v>-0.2217</v>
       </c>
       <c r="Z19" t="n">
-        <v>29.0323</v>
+        <v>38.8889</v>
       </c>
       <c r="AA19" t="n">
-        <v>5.4859</v>
+        <v>-0.7429</v>
       </c>
       <c r="AB19" t="n">
-        <v>6.5998</v>
+        <v>0.3254</v>
       </c>
       <c r="AC19" t="n">
-        <v>5.8176</v>
+        <v>10.3828</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>159.21</v>
+        <v>199.81</v>
       </c>
       <c r="C20" t="n">
-        <v>176.75</v>
+        <v>204.55</v>
       </c>
       <c r="D20" t="n">
-        <v>158.87</v>
+        <v>189.46</v>
       </c>
       <c r="E20" t="n">
-        <v>174.82</v>
+        <v>192.45</v>
       </c>
       <c r="F20" t="n">
-        <v>70.8</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="G20" t="n">
-        <v>73.02</v>
+        <v>76.69</v>
       </c>
       <c r="H20" t="n">
-        <v>69.56999999999999</v>
+        <v>73.89</v>
       </c>
       <c r="I20" t="n">
-        <v>72.72</v>
+        <v>76.34</v>
       </c>
       <c r="J20" t="n">
-        <v>4.98</v>
+        <v>3.87</v>
       </c>
       <c r="K20" t="n">
-        <v>4.99</v>
+        <v>4.12</v>
       </c>
       <c r="L20" t="n">
-        <v>4.46</v>
+        <v>3.75</v>
       </c>
       <c r="M20" t="n">
-        <v>4.5</v>
+        <v>4.07</v>
       </c>
       <c r="N20" t="n">
-        <v>41.18</v>
+        <v>38.93</v>
       </c>
       <c r="O20" t="n">
-        <v>41.86</v>
+        <v>39.47</v>
       </c>
       <c r="P20" t="n">
-        <v>39.93</v>
+        <v>37.93</v>
       </c>
       <c r="Q20" t="n">
-        <v>40.08</v>
+        <v>38.1</v>
       </c>
       <c r="R20" t="n">
-        <v>5.772</v>
+        <v>10.0847</v>
       </c>
       <c r="S20" t="n">
-        <v>-3.6645</v>
+        <v>-1.1302</v>
       </c>
       <c r="T20" t="n">
-        <v>-34.4532</v>
+        <v>-11.5376</v>
       </c>
       <c r="U20" t="n">
-        <v>0.6784</v>
+        <v>4.978</v>
       </c>
       <c r="V20" t="n">
-        <v>-0.8589</v>
+        <v>-0.1047</v>
       </c>
       <c r="W20" t="n">
-        <v>-10.2222</v>
+        <v>-1.4459</v>
       </c>
       <c r="X20" t="n">
-        <v>-6.25</v>
+        <v>-9.5556</v>
       </c>
       <c r="Y20" t="n">
-        <v>-0.2217</v>
+        <v>-2.3981</v>
       </c>
       <c r="Z20" t="n">
-        <v>38.8889</v>
+        <v>5.4404</v>
       </c>
       <c r="AA20" t="n">
-        <v>-0.7429</v>
+        <v>-4.9401</v>
       </c>
       <c r="AB20" t="n">
-        <v>0.3254</v>
+        <v>-0.4702</v>
       </c>
       <c r="AC20" t="n">
-        <v>10.3828</v>
+        <v>0.5808</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>199.81</v>
+        <v>182.4</v>
       </c>
       <c r="C21" t="n">
-        <v>204.52</v>
+        <v>195.94</v>
       </c>
       <c r="D21" t="n">
-        <v>189.46</v>
+        <v>176.83</v>
       </c>
       <c r="E21" t="n">
-        <v>192.45</v>
+        <v>192.26</v>
       </c>
       <c r="F21" t="n">
-        <v>74.84999999999999</v>
+        <v>75.529</v>
       </c>
       <c r="G21" t="n">
-        <v>76.685</v>
+        <v>77.31999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>73.89</v>
+        <v>74.33</v>
       </c>
       <c r="I21" t="n">
-        <v>76.34</v>
+        <v>77.03</v>
       </c>
       <c r="J21" t="n">
-        <v>3.87</v>
+        <v>4.27</v>
       </c>
       <c r="K21" t="n">
-        <v>4.12</v>
+        <v>4.39</v>
       </c>
       <c r="L21" t="n">
-        <v>3.75</v>
+        <v>3.99</v>
       </c>
       <c r="M21" t="n">
-        <v>4.07</v>
+        <v>4.08</v>
       </c>
       <c r="N21" t="n">
-        <v>38.98</v>
+        <v>38.485</v>
       </c>
       <c r="O21" t="n">
-        <v>39.465</v>
+        <v>39.14</v>
       </c>
       <c r="P21" t="n">
-        <v>37.93</v>
+        <v>37.64</v>
       </c>
       <c r="Q21" t="n">
-        <v>38.1</v>
+        <v>37.78</v>
       </c>
       <c r="R21" t="n">
-        <v>10.0847</v>
+        <v>-0.0987</v>
       </c>
       <c r="S21" t="n">
-        <v>-1.1302</v>
+        <v>16.3238</v>
       </c>
       <c r="T21" t="n">
-        <v>-11.5376</v>
+        <v>5.9459</v>
       </c>
       <c r="U21" t="n">
-        <v>4.978</v>
+        <v>0.9039</v>
       </c>
       <c r="V21" t="n">
-        <v>-0.1047</v>
+        <v>6.6454</v>
       </c>
       <c r="W21" t="n">
-        <v>-1.4459</v>
+        <v>5.017</v>
       </c>
       <c r="X21" t="n">
-        <v>-9.5556</v>
+        <v>0.2457</v>
       </c>
       <c r="Y21" t="n">
-        <v>-2.3981</v>
+        <v>-15</v>
       </c>
       <c r="Z21" t="n">
-        <v>5.4404</v>
+        <v>-9.5344</v>
       </c>
       <c r="AA21" t="n">
-        <v>-4.9401</v>
+        <v>-0.8399</v>
       </c>
       <c r="AB21" t="n">
-        <v>-0.4702</v>
+        <v>-6.4388</v>
       </c>
       <c r="AC21" t="n">
-        <v>0.5808</v>
+        <v>-5.4318</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-07-13 22:56
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC21"/>
+  <dimension ref="A1:AC20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,1713 +568,1622 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>192.3</v>
+        <v>265.99</v>
       </c>
       <c r="C2" t="n">
-        <v>225.63</v>
+        <v>274.88</v>
       </c>
       <c r="D2" t="n">
-        <v>192.3</v>
+        <v>261.6</v>
       </c>
       <c r="E2" t="n">
-        <v>223.99</v>
+        <v>272.5</v>
       </c>
       <c r="F2" t="n">
-        <v>70.7272</v>
+        <v>82.6896</v>
       </c>
       <c r="G2" t="n">
-        <v>76.42400000000001</v>
+        <v>84.8347</v>
       </c>
       <c r="H2" t="n">
-        <v>69.4301</v>
+        <v>82.4502</v>
       </c>
       <c r="I2" t="n">
-        <v>75.83540000000001</v>
+        <v>84.39570000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>6.0298</v>
+        <v>4.0231</v>
       </c>
       <c r="K2" t="n">
-        <v>6.0298</v>
+        <v>4.122</v>
       </c>
       <c r="L2" t="n">
-        <v>4.8436</v>
+        <v>3.865</v>
       </c>
       <c r="M2" t="n">
-        <v>4.9128</v>
+        <v>3.9045</v>
       </c>
       <c r="N2" t="n">
-        <v>43.4851</v>
+        <v>36.6641</v>
       </c>
       <c r="O2" t="n">
-        <v>44.302</v>
+        <v>36.7723</v>
       </c>
       <c r="P2" t="n">
-        <v>39.8039</v>
+        <v>35.5814</v>
       </c>
       <c r="Q2" t="n">
-        <v>40.1878</v>
+        <v>35.7389</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>222.22</v>
+        <v>267.13</v>
       </c>
       <c r="C3" t="n">
-        <v>242.4</v>
+        <v>274.93</v>
       </c>
       <c r="D3" t="n">
-        <v>214.74</v>
+        <v>226</v>
       </c>
       <c r="E3" t="n">
-        <v>234.68</v>
+        <v>226.19</v>
       </c>
       <c r="F3" t="n">
-        <v>76.16459999999999</v>
+        <v>83.9966</v>
       </c>
       <c r="G3" t="n">
-        <v>78.18000000000001</v>
+        <v>84.63509999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>74.1193</v>
+        <v>79.67659999999999</v>
       </c>
       <c r="I3" t="n">
-        <v>77.3419</v>
+        <v>79.74639999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>4.9523</v>
+        <v>3.9836</v>
       </c>
       <c r="K3" t="n">
-        <v>5.0907</v>
+        <v>4.5965</v>
       </c>
       <c r="L3" t="n">
-        <v>4.4877</v>
+        <v>3.865</v>
       </c>
       <c r="M3" t="n">
-        <v>4.6656</v>
+        <v>4.5767</v>
       </c>
       <c r="N3" t="n">
-        <v>40.0106</v>
+        <v>35.9652</v>
       </c>
       <c r="O3" t="n">
-        <v>41.0933</v>
+        <v>37.7861</v>
       </c>
       <c r="P3" t="n">
-        <v>38.9476</v>
+        <v>35.6896</v>
       </c>
       <c r="Q3" t="n">
-        <v>39.4102</v>
+        <v>37.7468</v>
       </c>
       <c r="R3" t="n">
-        <v>4.7725</v>
+        <v>-16.9945</v>
       </c>
       <c r="U3" t="n">
-        <v>1.9865</v>
+        <v>-5.5089</v>
       </c>
       <c r="X3" t="n">
-        <v>-5.0318</v>
+        <v>17.216</v>
       </c>
       <c r="AA3" t="n">
-        <v>-1.9349</v>
+        <v>5.6182</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>265.99</v>
+        <v>247.42</v>
       </c>
       <c r="C4" t="n">
-        <v>274.88</v>
+        <v>259.79</v>
       </c>
       <c r="D4" t="n">
-        <v>261.6</v>
+        <v>233.3</v>
       </c>
       <c r="E4" t="n">
-        <v>272.5</v>
+        <v>233.86</v>
       </c>
       <c r="F4" t="n">
-        <v>82.6896</v>
+        <v>81.4824</v>
       </c>
       <c r="G4" t="n">
-        <v>84.8347</v>
+        <v>81.6221</v>
       </c>
       <c r="H4" t="n">
-        <v>82.4502</v>
+        <v>76.7633</v>
       </c>
       <c r="I4" t="n">
-        <v>84.39570000000001</v>
+        <v>77.36190000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>4.0231</v>
+        <v>4.122</v>
       </c>
       <c r="K4" t="n">
-        <v>4.122</v>
+        <v>4.4086</v>
       </c>
       <c r="L4" t="n">
-        <v>3.865</v>
+        <v>3.8749</v>
       </c>
       <c r="M4" t="n">
-        <v>3.9045</v>
+        <v>4.4086</v>
       </c>
       <c r="N4" t="n">
-        <v>36.6641</v>
+        <v>36.9397</v>
       </c>
       <c r="O4" t="n">
-        <v>36.7723</v>
+        <v>39.1641</v>
       </c>
       <c r="P4" t="n">
-        <v>35.5814</v>
+        <v>36.8708</v>
       </c>
       <c r="Q4" t="n">
-        <v>35.7389</v>
+        <v>38.8984</v>
       </c>
       <c r="R4" t="n">
-        <v>16.1156</v>
+        <v>3.391</v>
       </c>
       <c r="U4" t="n">
-        <v>9.1203</v>
+        <v>-2.9901</v>
       </c>
       <c r="X4" t="n">
-        <v>-16.313</v>
+        <v>-3.673</v>
       </c>
       <c r="AA4" t="n">
-        <v>-9.3156</v>
+        <v>3.0509</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>267.13</v>
+        <v>266.04</v>
       </c>
       <c r="C5" t="n">
-        <v>274.93</v>
+        <v>286.15</v>
       </c>
       <c r="D5" t="n">
-        <v>226</v>
+        <v>265</v>
       </c>
       <c r="E5" t="n">
-        <v>226.19</v>
+        <v>279.29</v>
       </c>
       <c r="F5" t="n">
-        <v>83.9966</v>
+        <v>81.9114</v>
       </c>
       <c r="G5" t="n">
-        <v>84.63509999999999</v>
+        <v>83.408</v>
       </c>
       <c r="H5" t="n">
-        <v>79.67659999999999</v>
+        <v>80.4448</v>
       </c>
       <c r="I5" t="n">
-        <v>79.74639999999999</v>
+        <v>82.67959999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>3.9836</v>
+        <v>3.8156</v>
       </c>
       <c r="K5" t="n">
-        <v>4.5965</v>
+        <v>3.8254</v>
       </c>
       <c r="L5" t="n">
-        <v>3.865</v>
+        <v>3.4103</v>
       </c>
       <c r="M5" t="n">
-        <v>4.5767</v>
+        <v>3.5487</v>
       </c>
       <c r="N5" t="n">
-        <v>35.9652</v>
+        <v>36.6149</v>
       </c>
       <c r="O5" t="n">
-        <v>37.7861</v>
+        <v>37.3531</v>
       </c>
       <c r="P5" t="n">
-        <v>35.6896</v>
+        <v>35.857</v>
       </c>
       <c r="Q5" t="n">
-        <v>37.7468</v>
+        <v>36.1719</v>
       </c>
       <c r="R5" t="n">
-        <v>-16.9945</v>
+        <v>19.4262</v>
       </c>
       <c r="S5" t="n">
-        <v>0.9822</v>
+        <v>2.4917</v>
       </c>
       <c r="U5" t="n">
-        <v>-5.5089</v>
+        <v>6.8738</v>
       </c>
       <c r="V5" t="n">
-        <v>5.1572</v>
+        <v>-2.0334</v>
       </c>
       <c r="X5" t="n">
-        <v>17.216</v>
+        <v>-19.5051</v>
       </c>
       <c r="Y5" t="n">
-        <v>-6.8413</v>
+        <v>-9.1126</v>
       </c>
       <c r="AA5" t="n">
-        <v>5.6182</v>
+        <v>-7.0093</v>
       </c>
       <c r="AB5" t="n">
-        <v>-6.074</v>
+        <v>1.2116</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>247.42</v>
+        <v>299.26</v>
       </c>
       <c r="C6" t="n">
-        <v>259.79</v>
+        <v>302</v>
       </c>
       <c r="D6" t="n">
-        <v>233.3</v>
+        <v>286.24</v>
       </c>
       <c r="E6" t="n">
-        <v>233.86</v>
+        <v>300.77</v>
       </c>
       <c r="F6" t="n">
-        <v>81.4824</v>
+        <v>83.7572</v>
       </c>
       <c r="G6" t="n">
-        <v>81.6221</v>
+        <v>84.9145</v>
       </c>
       <c r="H6" t="n">
-        <v>76.7633</v>
+        <v>81.203</v>
       </c>
       <c r="I6" t="n">
-        <v>77.36190000000001</v>
+        <v>82.3903</v>
       </c>
       <c r="J6" t="n">
-        <v>4.122</v>
+        <v>3.2917</v>
       </c>
       <c r="K6" t="n">
-        <v>4.4086</v>
+        <v>3.4498</v>
       </c>
       <c r="L6" t="n">
-        <v>3.8749</v>
+        <v>3.2521</v>
       </c>
       <c r="M6" t="n">
-        <v>4.4086</v>
+        <v>3.262</v>
       </c>
       <c r="N6" t="n">
-        <v>36.9397</v>
+        <v>35.7389</v>
       </c>
       <c r="O6" t="n">
-        <v>39.1641</v>
+        <v>36.8511</v>
       </c>
       <c r="P6" t="n">
-        <v>36.8708</v>
+        <v>35.2369</v>
       </c>
       <c r="Q6" t="n">
-        <v>38.8984</v>
+        <v>36.3491</v>
       </c>
       <c r="R6" t="n">
-        <v>3.391</v>
+        <v>7.6909</v>
       </c>
       <c r="S6" t="n">
-        <v>-0.3494</v>
+        <v>32.9723</v>
       </c>
       <c r="U6" t="n">
-        <v>-2.9901</v>
+        <v>-0.3499</v>
       </c>
       <c r="V6" t="n">
-        <v>0.0259</v>
+        <v>3.3154</v>
       </c>
       <c r="X6" t="n">
-        <v>-3.673</v>
+        <v>-8.079000000000001</v>
       </c>
       <c r="Y6" t="n">
-        <v>-5.5084</v>
+        <v>-28.7259</v>
       </c>
       <c r="AA6" t="n">
-        <v>3.0509</v>
+        <v>0.4899</v>
       </c>
       <c r="AB6" t="n">
-        <v>-1.2986</v>
+        <v>-3.7028</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>266.04</v>
+        <v>236</v>
       </c>
       <c r="C7" t="n">
-        <v>286.15</v>
+        <v>252.98</v>
       </c>
       <c r="D7" t="n">
-        <v>265</v>
+        <v>223</v>
       </c>
       <c r="E7" t="n">
-        <v>279.29</v>
+        <v>231.42</v>
       </c>
       <c r="F7" t="n">
-        <v>81.9114</v>
+        <v>74.9474</v>
       </c>
       <c r="G7" t="n">
-        <v>83.408</v>
+        <v>77.56140000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>80.4448</v>
+        <v>73.7402</v>
       </c>
       <c r="I7" t="n">
-        <v>82.67959999999999</v>
+        <v>74.26900000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>3.8156</v>
+        <v>3.99</v>
       </c>
       <c r="K7" t="n">
-        <v>3.8254</v>
+        <v>4.13</v>
       </c>
       <c r="L7" t="n">
-        <v>3.4103</v>
+        <v>3.8</v>
       </c>
       <c r="M7" t="n">
-        <v>3.5487</v>
+        <v>4.04</v>
       </c>
       <c r="N7" t="n">
-        <v>36.6149</v>
+        <v>39.6267</v>
       </c>
       <c r="O7" t="n">
-        <v>37.3531</v>
+        <v>40.1582</v>
       </c>
       <c r="P7" t="n">
-        <v>35.857</v>
+        <v>38.4653</v>
       </c>
       <c r="Q7" t="n">
-        <v>36.1719</v>
+        <v>39.922</v>
       </c>
       <c r="R7" t="n">
-        <v>19.4262</v>
+        <v>-23.0575</v>
       </c>
       <c r="S7" t="n">
-        <v>2.4917</v>
+        <v>-1.0434</v>
       </c>
       <c r="T7" t="n">
-        <v>24.6886</v>
+        <v>-15.0752</v>
       </c>
       <c r="U7" t="n">
-        <v>6.8738</v>
+        <v>-9.857100000000001</v>
       </c>
       <c r="V7" t="n">
-        <v>-2.0334</v>
+        <v>-3.998</v>
       </c>
       <c r="W7" t="n">
-        <v>9.0251</v>
+        <v>-11.9991</v>
       </c>
       <c r="X7" t="n">
-        <v>-19.5051</v>
+        <v>23.8504</v>
       </c>
       <c r="Y7" t="n">
-        <v>-9.1126</v>
+        <v>-8.360900000000001</v>
       </c>
       <c r="Z7" t="n">
-        <v>-27.7662</v>
+        <v>3.4704</v>
       </c>
       <c r="AA7" t="n">
-        <v>-7.0093</v>
+        <v>9.8294</v>
       </c>
       <c r="AB7" t="n">
-        <v>1.2116</v>
+        <v>2.6315</v>
       </c>
       <c r="AC7" t="n">
-        <v>-9.992800000000001</v>
+        <v>11.7046</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>299.26</v>
+        <v>233.11</v>
       </c>
       <c r="C8" t="n">
-        <v>302</v>
+        <v>237</v>
       </c>
       <c r="D8" t="n">
-        <v>286.24</v>
+        <v>211.13</v>
       </c>
       <c r="E8" t="n">
-        <v>300.77</v>
+        <v>229.57</v>
       </c>
       <c r="F8" t="n">
-        <v>83.7572</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>84.9145</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="H8" t="n">
-        <v>81.203</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="I8" t="n">
-        <v>82.3903</v>
+        <v>73.3</v>
       </c>
       <c r="J8" t="n">
-        <v>3.2917</v>
+        <v>4</v>
       </c>
       <c r="K8" t="n">
-        <v>3.4498</v>
+        <v>4.39</v>
       </c>
       <c r="L8" t="n">
-        <v>3.2521</v>
+        <v>3.92</v>
       </c>
       <c r="M8" t="n">
-        <v>3.262</v>
+        <v>4.08</v>
       </c>
       <c r="N8" t="n">
-        <v>35.7389</v>
+        <v>39.66</v>
       </c>
       <c r="O8" t="n">
-        <v>36.8511</v>
+        <v>41.49</v>
       </c>
       <c r="P8" t="n">
-        <v>35.2369</v>
+        <v>38.9</v>
       </c>
       <c r="Q8" t="n">
-        <v>36.3491</v>
+        <v>40.45</v>
       </c>
       <c r="R8" t="n">
-        <v>7.6909</v>
+        <v>-0.7994</v>
       </c>
       <c r="S8" t="n">
-        <v>32.9723</v>
+        <v>-17.8023</v>
       </c>
       <c r="T8" t="n">
-        <v>28.1618</v>
+        <v>1.4943</v>
       </c>
       <c r="U8" t="n">
-        <v>-0.3499</v>
+        <v>-1.3047</v>
       </c>
       <c r="V8" t="n">
-        <v>3.3154</v>
+        <v>-11.3445</v>
       </c>
       <c r="W8" t="n">
-        <v>6.5274</v>
+        <v>-8.083600000000001</v>
       </c>
       <c r="X8" t="n">
-        <v>-8.079000000000001</v>
+        <v>0.9901</v>
       </c>
       <c r="Y8" t="n">
-        <v>-28.7259</v>
+        <v>14.9717</v>
       </c>
       <c r="Z8" t="n">
-        <v>-30.084</v>
+        <v>-10.8528</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.4899</v>
+        <v>1.3226</v>
       </c>
       <c r="AB8" t="n">
-        <v>-3.7028</v>
+        <v>11.8271</v>
       </c>
       <c r="AC8" t="n">
-        <v>-7.7673</v>
+        <v>7.1614</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>236</v>
+        <v>268.05</v>
       </c>
       <c r="C9" t="n">
-        <v>252.98</v>
+        <v>268.4</v>
       </c>
       <c r="D9" t="n">
-        <v>223</v>
+        <v>225.74</v>
       </c>
       <c r="E9" t="n">
-        <v>231.42</v>
+        <v>252.61</v>
       </c>
       <c r="F9" t="n">
-        <v>74.9474</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>77.56140000000001</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>73.7402</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I9" t="n">
-        <v>74.26900000000001</v>
+        <v>74.95</v>
       </c>
       <c r="J9" t="n">
-        <v>3.99</v>
+        <v>3.38</v>
       </c>
       <c r="K9" t="n">
-        <v>4.13</v>
+        <v>4.15</v>
       </c>
       <c r="L9" t="n">
-        <v>3.8</v>
+        <v>3.37</v>
       </c>
       <c r="M9" t="n">
-        <v>4.04</v>
+        <v>3.63</v>
       </c>
       <c r="N9" t="n">
-        <v>39.6267</v>
+        <v>37.87</v>
       </c>
       <c r="O9" t="n">
-        <v>40.1582</v>
+        <v>41.37</v>
       </c>
       <c r="P9" t="n">
-        <v>38.4653</v>
+        <v>37.71</v>
       </c>
       <c r="Q9" t="n">
-        <v>39.922</v>
+        <v>39.47</v>
       </c>
       <c r="R9" t="n">
-        <v>-23.0575</v>
+        <v>10.0362</v>
       </c>
       <c r="S9" t="n">
-        <v>-1.0434</v>
+        <v>-16.0122</v>
       </c>
       <c r="T9" t="n">
-        <v>-15.0752</v>
+        <v>8.0176</v>
       </c>
       <c r="U9" t="n">
-        <v>-9.857100000000001</v>
+        <v>2.251</v>
       </c>
       <c r="V9" t="n">
-        <v>-3.998</v>
+        <v>-9.0306</v>
       </c>
       <c r="W9" t="n">
-        <v>-11.9991</v>
+        <v>-3.1177</v>
       </c>
       <c r="X9" t="n">
-        <v>23.8504</v>
+        <v>-11.0294</v>
       </c>
       <c r="Y9" t="n">
-        <v>-8.360900000000001</v>
+        <v>11.2814</v>
       </c>
       <c r="Z9" t="n">
-        <v>3.4704</v>
+        <v>-17.6609</v>
       </c>
       <c r="AA9" t="n">
-        <v>9.8294</v>
+        <v>-2.4227</v>
       </c>
       <c r="AB9" t="n">
-        <v>2.6315</v>
+        <v>8.585900000000001</v>
       </c>
       <c r="AC9" t="n">
-        <v>11.7046</v>
+        <v>1.4695</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>233.11</v>
+        <v>226.24</v>
       </c>
       <c r="C10" t="n">
-        <v>237</v>
+        <v>231.25</v>
       </c>
       <c r="D10" t="n">
-        <v>211.13</v>
+        <v>212.1</v>
       </c>
       <c r="E10" t="n">
-        <v>229.57</v>
+        <v>215.6</v>
       </c>
       <c r="F10" t="n">
-        <v>74.79000000000001</v>
+        <v>72.09</v>
       </c>
       <c r="G10" t="n">
-        <v>76.18000000000001</v>
+        <v>74.69</v>
       </c>
       <c r="H10" t="n">
-        <v>71.34999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="I10" t="n">
-        <v>73.3</v>
+        <v>71.83</v>
       </c>
       <c r="J10" t="n">
-        <v>4</v>
+        <v>4.04</v>
       </c>
       <c r="K10" t="n">
-        <v>4.39</v>
+        <v>4.25</v>
       </c>
       <c r="L10" t="n">
-        <v>3.92</v>
+        <v>3.95</v>
       </c>
       <c r="M10" t="n">
-        <v>4.08</v>
+        <v>4.24</v>
       </c>
       <c r="N10" t="n">
-        <v>39.66</v>
+        <v>41.08</v>
       </c>
       <c r="O10" t="n">
-        <v>41.49</v>
+        <v>41.79</v>
       </c>
       <c r="P10" t="n">
-        <v>38.9</v>
+        <v>39.69</v>
       </c>
       <c r="Q10" t="n">
-        <v>40.45</v>
+        <v>41.31</v>
       </c>
       <c r="R10" t="n">
-        <v>-0.7994</v>
+        <v>-14.651</v>
       </c>
       <c r="S10" t="n">
-        <v>-17.8023</v>
+        <v>-6.8361</v>
       </c>
       <c r="T10" t="n">
-        <v>1.4943</v>
+        <v>-22.8043</v>
       </c>
       <c r="U10" t="n">
-        <v>-1.3047</v>
+        <v>-4.1628</v>
       </c>
       <c r="V10" t="n">
-        <v>-11.3445</v>
+        <v>-3.284</v>
       </c>
       <c r="W10" t="n">
-        <v>-8.083600000000001</v>
+        <v>-13.1225</v>
       </c>
       <c r="X10" t="n">
-        <v>0.9901</v>
+        <v>16.8044</v>
       </c>
       <c r="Y10" t="n">
-        <v>14.9717</v>
+        <v>4.9505</v>
       </c>
       <c r="Z10" t="n">
-        <v>-10.8528</v>
+        <v>19.4804</v>
       </c>
       <c r="AA10" t="n">
-        <v>1.3226</v>
+        <v>4.6618</v>
       </c>
       <c r="AB10" t="n">
-        <v>11.8271</v>
+        <v>3.4768</v>
       </c>
       <c r="AC10" t="n">
-        <v>7.1614</v>
+        <v>14.2047</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>268.05</v>
+        <v>216.36</v>
       </c>
       <c r="C11" t="n">
-        <v>268.4</v>
+        <v>238.65</v>
       </c>
       <c r="D11" t="n">
-        <v>225.74</v>
+        <v>192.3</v>
       </c>
       <c r="E11" t="n">
-        <v>252.61</v>
+        <v>236.52</v>
       </c>
       <c r="F11" t="n">
-        <v>77.95999999999999</v>
+        <v>74.12</v>
       </c>
       <c r="G11" t="n">
-        <v>78.23999999999999</v>
+        <v>77.38</v>
       </c>
       <c r="H11" t="n">
-        <v>71.59999999999999</v>
+        <v>71.45</v>
       </c>
       <c r="I11" t="n">
-        <v>74.95</v>
+        <v>77.19</v>
       </c>
       <c r="J11" t="n">
-        <v>3.38</v>
+        <v>4.16</v>
       </c>
       <c r="K11" t="n">
-        <v>4.15</v>
+        <v>4.63</v>
       </c>
       <c r="L11" t="n">
-        <v>3.37</v>
+        <v>3.7</v>
       </c>
       <c r="M11" t="n">
-        <v>3.63</v>
+        <v>3.72</v>
       </c>
       <c r="N11" t="n">
-        <v>37.87</v>
+        <v>39.91</v>
       </c>
       <c r="O11" t="n">
-        <v>41.37</v>
+        <v>41.43</v>
       </c>
       <c r="P11" t="n">
-        <v>37.71</v>
+        <v>38.08</v>
       </c>
       <c r="Q11" t="n">
-        <v>39.47</v>
+        <v>38.16</v>
       </c>
       <c r="R11" t="n">
-        <v>10.0362</v>
+        <v>9.703200000000001</v>
       </c>
       <c r="S11" t="n">
-        <v>-16.0122</v>
+        <v>3.0274</v>
       </c>
       <c r="T11" t="n">
-        <v>8.0176</v>
+        <v>-21.3618</v>
       </c>
       <c r="U11" t="n">
-        <v>2.251</v>
+        <v>7.4621</v>
       </c>
       <c r="V11" t="n">
-        <v>-9.0306</v>
+        <v>5.307</v>
       </c>
       <c r="W11" t="n">
-        <v>-3.1177</v>
+        <v>-6.3118</v>
       </c>
       <c r="X11" t="n">
-        <v>-11.0294</v>
+        <v>-12.2642</v>
       </c>
       <c r="Y11" t="n">
-        <v>11.2814</v>
+        <v>-8.823499999999999</v>
       </c>
       <c r="Z11" t="n">
-        <v>-17.6609</v>
+        <v>14.0405</v>
       </c>
       <c r="AA11" t="n">
-        <v>-2.4227</v>
+        <v>-7.6253</v>
       </c>
       <c r="AB11" t="n">
-        <v>8.585900000000001</v>
+        <v>-5.6613</v>
       </c>
       <c r="AC11" t="n">
-        <v>1.4695</v>
+        <v>4.982</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>226.24</v>
+        <v>241.45</v>
       </c>
       <c r="C12" t="n">
-        <v>231.25</v>
+        <v>272</v>
       </c>
       <c r="D12" t="n">
-        <v>212.1</v>
+        <v>240.59</v>
       </c>
       <c r="E12" t="n">
-        <v>215.6</v>
+        <v>266.71</v>
       </c>
       <c r="F12" t="n">
-        <v>72.09</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="G12" t="n">
-        <v>74.69</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>70.72</v>
+        <v>77.15000000000001</v>
       </c>
       <c r="I12" t="n">
-        <v>71.83</v>
+        <v>81</v>
       </c>
       <c r="J12" t="n">
-        <v>4.04</v>
+        <v>3.66</v>
       </c>
       <c r="K12" t="n">
-        <v>4.25</v>
+        <v>3.68</v>
       </c>
       <c r="L12" t="n">
-        <v>3.95</v>
+        <v>3.17</v>
       </c>
       <c r="M12" t="n">
-        <v>4.24</v>
+        <v>3.24</v>
       </c>
       <c r="N12" t="n">
-        <v>41.08</v>
+        <v>38.16</v>
       </c>
       <c r="O12" t="n">
-        <v>41.79</v>
+        <v>38.2</v>
       </c>
       <c r="P12" t="n">
-        <v>39.69</v>
+        <v>36.03</v>
       </c>
       <c r="Q12" t="n">
-        <v>41.31</v>
+        <v>36.31</v>
       </c>
       <c r="R12" t="n">
-        <v>-14.651</v>
+        <v>12.7642</v>
       </c>
       <c r="S12" t="n">
-        <v>-6.8361</v>
+        <v>5.5817</v>
       </c>
       <c r="T12" t="n">
-        <v>-22.8043</v>
+        <v>15.2493</v>
       </c>
       <c r="U12" t="n">
-        <v>-4.1628</v>
+        <v>4.9359</v>
       </c>
       <c r="V12" t="n">
-        <v>-3.284</v>
+        <v>8.071999999999999</v>
       </c>
       <c r="W12" t="n">
-        <v>-13.1225</v>
+        <v>9.063000000000001</v>
       </c>
       <c r="X12" t="n">
-        <v>16.8044</v>
+        <v>-12.9032</v>
       </c>
       <c r="Y12" t="n">
-        <v>4.9505</v>
+        <v>-10.7438</v>
       </c>
       <c r="Z12" t="n">
-        <v>19.4804</v>
+        <v>-19.802</v>
       </c>
       <c r="AA12" t="n">
-        <v>4.6618</v>
+        <v>-4.848</v>
       </c>
       <c r="AB12" t="n">
-        <v>3.4768</v>
+        <v>-8.0061</v>
       </c>
       <c r="AC12" t="n">
-        <v>14.2047</v>
+        <v>-9.047599999999999</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>216.36</v>
+        <v>237.79</v>
       </c>
       <c r="C13" t="n">
-        <v>238.65</v>
+        <v>246.47</v>
       </c>
       <c r="D13" t="n">
-        <v>192.3</v>
+        <v>215.38</v>
       </c>
       <c r="E13" t="n">
-        <v>236.52</v>
+        <v>217.55</v>
       </c>
       <c r="F13" t="n">
-        <v>74.12</v>
+        <v>78.72</v>
       </c>
       <c r="G13" t="n">
-        <v>77.38</v>
+        <v>79.64</v>
       </c>
       <c r="H13" t="n">
-        <v>71.45</v>
+        <v>77.23</v>
       </c>
       <c r="I13" t="n">
-        <v>77.19</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>4.16</v>
+        <v>3.59</v>
       </c>
       <c r="K13" t="n">
-        <v>4.63</v>
+        <v>3.89</v>
       </c>
       <c r="L13" t="n">
-        <v>3.7</v>
+        <v>3.51</v>
       </c>
       <c r="M13" t="n">
-        <v>3.72</v>
+        <v>3.86</v>
       </c>
       <c r="N13" t="n">
-        <v>39.91</v>
+        <v>37.31</v>
       </c>
       <c r="O13" t="n">
-        <v>41.43</v>
+        <v>37.98</v>
       </c>
       <c r="P13" t="n">
-        <v>38.08</v>
+        <v>36.9</v>
       </c>
       <c r="Q13" t="n">
-        <v>38.16</v>
+        <v>37.88</v>
       </c>
       <c r="R13" t="n">
-        <v>9.703200000000001</v>
+        <v>-18.432</v>
       </c>
       <c r="S13" t="n">
-        <v>3.0274</v>
+        <v>0.9045</v>
       </c>
       <c r="T13" t="n">
-        <v>-21.3618</v>
+        <v>-5.2359</v>
       </c>
       <c r="U13" t="n">
-        <v>7.4621</v>
+        <v>-4.3704</v>
       </c>
       <c r="V13" t="n">
-        <v>5.307</v>
+        <v>7.838</v>
       </c>
       <c r="W13" t="n">
-        <v>-6.3118</v>
+        <v>5.6753</v>
       </c>
       <c r="X13" t="n">
-        <v>-12.2642</v>
+        <v>19.1358</v>
       </c>
       <c r="Y13" t="n">
-        <v>-8.823499999999999</v>
+        <v>-8.962300000000001</v>
       </c>
       <c r="Z13" t="n">
-        <v>14.0405</v>
+        <v>-5.3922</v>
       </c>
       <c r="AA13" t="n">
-        <v>-7.6253</v>
+        <v>4.3239</v>
       </c>
       <c r="AB13" t="n">
-        <v>-5.6613</v>
+        <v>-8.303100000000001</v>
       </c>
       <c r="AC13" t="n">
-        <v>4.982</v>
+        <v>-6.3535</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>241.45</v>
+        <v>219.23</v>
       </c>
       <c r="C14" t="n">
-        <v>272</v>
+        <v>226.13</v>
       </c>
       <c r="D14" t="n">
-        <v>240.59</v>
+        <v>168.88</v>
       </c>
       <c r="E14" t="n">
-        <v>266.71</v>
+        <v>181.47</v>
       </c>
       <c r="F14" t="n">
-        <v>77.23999999999999</v>
+        <v>77.45</v>
       </c>
       <c r="G14" t="n">
-        <v>81.54000000000001</v>
+        <v>79.14</v>
       </c>
       <c r="H14" t="n">
-        <v>77.15000000000001</v>
+        <v>71.72</v>
       </c>
       <c r="I14" t="n">
-        <v>81</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>3.66</v>
+        <v>3.84</v>
       </c>
       <c r="K14" t="n">
-        <v>3.68</v>
+        <v>4.74</v>
       </c>
       <c r="L14" t="n">
-        <v>3.17</v>
+        <v>3.71</v>
       </c>
       <c r="M14" t="n">
-        <v>3.24</v>
+        <v>4.51</v>
       </c>
       <c r="N14" t="n">
-        <v>38.16</v>
+        <v>37.91</v>
       </c>
       <c r="O14" t="n">
-        <v>38.2</v>
+        <v>40.72</v>
       </c>
       <c r="P14" t="n">
-        <v>36.03</v>
+        <v>37.08</v>
       </c>
       <c r="Q14" t="n">
-        <v>36.31</v>
+        <v>39.95</v>
       </c>
       <c r="R14" t="n">
-        <v>12.7642</v>
+        <v>-16.5847</v>
       </c>
       <c r="S14" t="n">
-        <v>5.5817</v>
+        <v>-23.275</v>
       </c>
       <c r="T14" t="n">
-        <v>15.2493</v>
+        <v>-28.162</v>
       </c>
       <c r="U14" t="n">
-        <v>4.9359</v>
+        <v>-5.306</v>
       </c>
       <c r="V14" t="n">
-        <v>8.071999999999999</v>
+        <v>-4.9747</v>
       </c>
       <c r="W14" t="n">
-        <v>9.063000000000001</v>
+        <v>-2.1348</v>
       </c>
       <c r="X14" t="n">
-        <v>-12.9032</v>
+        <v>16.8394</v>
       </c>
       <c r="Y14" t="n">
-        <v>-10.7438</v>
+        <v>21.2366</v>
       </c>
       <c r="Z14" t="n">
-        <v>-19.802</v>
+        <v>24.2424</v>
       </c>
       <c r="AA14" t="n">
-        <v>-4.848</v>
+        <v>5.4646</v>
       </c>
       <c r="AB14" t="n">
-        <v>-8.0061</v>
+        <v>4.6908</v>
       </c>
       <c r="AC14" t="n">
-        <v>-9.047599999999999</v>
+        <v>1.2161</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>237.79</v>
+        <v>197.21</v>
       </c>
       <c r="C15" t="n">
-        <v>246.47</v>
+        <v>210.8</v>
       </c>
       <c r="D15" t="n">
-        <v>215.38</v>
+        <v>194.22</v>
       </c>
       <c r="E15" t="n">
-        <v>217.55</v>
+        <v>194.65</v>
       </c>
       <c r="F15" t="n">
-        <v>78.72</v>
+        <v>75.54000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>79.64</v>
+        <v>77.45</v>
       </c>
       <c r="H15" t="n">
-        <v>77.23</v>
+        <v>75.11</v>
       </c>
       <c r="I15" t="n">
-        <v>77.45999999999999</v>
+        <v>76.42</v>
       </c>
       <c r="J15" t="n">
-        <v>3.59</v>
+        <v>4.11</v>
       </c>
       <c r="K15" t="n">
-        <v>3.89</v>
+        <v>4.18</v>
       </c>
       <c r="L15" t="n">
-        <v>3.51</v>
+        <v>3.77</v>
       </c>
       <c r="M15" t="n">
-        <v>3.86</v>
+        <v>4.17</v>
       </c>
       <c r="N15" t="n">
-        <v>37.31</v>
+        <v>38.75</v>
       </c>
       <c r="O15" t="n">
-        <v>37.98</v>
+        <v>38.98</v>
       </c>
       <c r="P15" t="n">
-        <v>36.9</v>
+        <v>37.71</v>
       </c>
       <c r="Q15" t="n">
-        <v>37.88</v>
+        <v>38.28</v>
       </c>
       <c r="R15" t="n">
-        <v>-18.432</v>
+        <v>7.2629</v>
       </c>
       <c r="S15" t="n">
-        <v>0.9045</v>
+        <v>-27.0181</v>
       </c>
       <c r="T15" t="n">
-        <v>-5.2359</v>
+        <v>-9.7171</v>
       </c>
       <c r="U15" t="n">
-        <v>-4.3704</v>
+        <v>4.1854</v>
       </c>
       <c r="V15" t="n">
-        <v>7.838</v>
+        <v>-5.6543</v>
       </c>
       <c r="W15" t="n">
-        <v>5.6753</v>
+        <v>6.3901</v>
       </c>
       <c r="X15" t="n">
-        <v>19.1358</v>
+        <v>-7.5388</v>
       </c>
       <c r="Y15" t="n">
-        <v>-8.962300000000001</v>
+        <v>28.7037</v>
       </c>
       <c r="Z15" t="n">
-        <v>-5.3922</v>
+        <v>-1.6509</v>
       </c>
       <c r="AA15" t="n">
-        <v>4.3239</v>
+        <v>-4.1802</v>
       </c>
       <c r="AB15" t="n">
-        <v>-8.303100000000001</v>
+        <v>5.4255</v>
       </c>
       <c r="AC15" t="n">
-        <v>-6.3535</v>
+        <v>-7.3348</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>219.23</v>
+        <v>165.4</v>
       </c>
       <c r="C16" t="n">
-        <v>226.13</v>
+        <v>171.88</v>
       </c>
       <c r="D16" t="n">
-        <v>168.88</v>
+        <v>150.08</v>
       </c>
       <c r="E16" t="n">
-        <v>181.47</v>
+        <v>165.28</v>
       </c>
       <c r="F16" t="n">
-        <v>77.45</v>
+        <v>73.7</v>
       </c>
       <c r="G16" t="n">
-        <v>79.14</v>
+        <v>74.39</v>
       </c>
       <c r="H16" t="n">
-        <v>71.72</v>
+        <v>70.76000000000001</v>
       </c>
       <c r="I16" t="n">
-        <v>73.34999999999999</v>
+        <v>72.23</v>
       </c>
       <c r="J16" t="n">
-        <v>3.84</v>
+        <v>4.8</v>
       </c>
       <c r="K16" t="n">
-        <v>4.74</v>
+        <v>5.14</v>
       </c>
       <c r="L16" t="n">
-        <v>3.71</v>
+        <v>4.66</v>
       </c>
       <c r="M16" t="n">
-        <v>4.51</v>
+        <v>4.8</v>
       </c>
       <c r="N16" t="n">
-        <v>37.91</v>
+        <v>39.64</v>
       </c>
       <c r="O16" t="n">
-        <v>40.72</v>
+        <v>41.11</v>
       </c>
       <c r="P16" t="n">
-        <v>37.08</v>
+        <v>39.29</v>
       </c>
       <c r="Q16" t="n">
-        <v>39.95</v>
+        <v>40.38</v>
       </c>
       <c r="R16" t="n">
-        <v>-16.5847</v>
+        <v>-15.0886</v>
       </c>
       <c r="S16" t="n">
-        <v>-23.275</v>
+        <v>-24.0267</v>
       </c>
       <c r="T16" t="n">
-        <v>-28.162</v>
+        <v>-30.1201</v>
       </c>
       <c r="U16" t="n">
-        <v>-5.306</v>
+        <v>-5.4829</v>
       </c>
       <c r="V16" t="n">
-        <v>-4.9747</v>
+        <v>-6.7519</v>
       </c>
       <c r="W16" t="n">
-        <v>-2.1348</v>
+        <v>-6.4257</v>
       </c>
       <c r="X16" t="n">
-        <v>16.8394</v>
+        <v>15.1079</v>
       </c>
       <c r="Y16" t="n">
-        <v>21.2366</v>
+        <v>24.3523</v>
       </c>
       <c r="Z16" t="n">
-        <v>24.2424</v>
+        <v>29.0323</v>
       </c>
       <c r="AA16" t="n">
-        <v>5.4646</v>
+        <v>5.4859</v>
       </c>
       <c r="AB16" t="n">
-        <v>4.6908</v>
+        <v>6.5998</v>
       </c>
       <c r="AC16" t="n">
-        <v>1.2161</v>
+        <v>5.8176</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>197.21</v>
+        <v>159.21</v>
       </c>
       <c r="C17" t="n">
-        <v>210.8</v>
+        <v>176.75</v>
       </c>
       <c r="D17" t="n">
-        <v>194.22</v>
+        <v>158.87</v>
       </c>
       <c r="E17" t="n">
-        <v>194.65</v>
+        <v>174.82</v>
       </c>
       <c r="F17" t="n">
-        <v>75.54000000000001</v>
+        <v>70.8</v>
       </c>
       <c r="G17" t="n">
-        <v>77.45</v>
+        <v>73.02</v>
       </c>
       <c r="H17" t="n">
-        <v>75.11</v>
+        <v>69.56999999999999</v>
       </c>
       <c r="I17" t="n">
-        <v>76.42</v>
+        <v>72.72</v>
       </c>
       <c r="J17" t="n">
-        <v>4.11</v>
+        <v>4.98</v>
       </c>
       <c r="K17" t="n">
-        <v>4.18</v>
+        <v>4.99</v>
       </c>
       <c r="L17" t="n">
-        <v>3.77</v>
+        <v>4.46</v>
       </c>
       <c r="M17" t="n">
-        <v>4.17</v>
+        <v>4.5</v>
       </c>
       <c r="N17" t="n">
-        <v>38.75</v>
+        <v>41.18</v>
       </c>
       <c r="O17" t="n">
-        <v>38.98</v>
+        <v>41.86</v>
       </c>
       <c r="P17" t="n">
-        <v>37.71</v>
+        <v>39.93</v>
       </c>
       <c r="Q17" t="n">
-        <v>38.28</v>
+        <v>40.08</v>
       </c>
       <c r="R17" t="n">
-        <v>7.2629</v>
+        <v>5.772</v>
       </c>
       <c r="S17" t="n">
-        <v>-27.0181</v>
+        <v>-3.6645</v>
       </c>
       <c r="T17" t="n">
-        <v>-9.7171</v>
+        <v>-34.4532</v>
       </c>
       <c r="U17" t="n">
-        <v>4.1854</v>
+        <v>0.6784</v>
       </c>
       <c r="V17" t="n">
-        <v>-5.6543</v>
+        <v>-0.8589</v>
       </c>
       <c r="W17" t="n">
-        <v>6.3901</v>
+        <v>-10.2222</v>
       </c>
       <c r="X17" t="n">
-        <v>-7.5388</v>
+        <v>-6.25</v>
       </c>
       <c r="Y17" t="n">
-        <v>28.7037</v>
+        <v>-0.2217</v>
       </c>
       <c r="Z17" t="n">
-        <v>-1.6509</v>
+        <v>38.8889</v>
       </c>
       <c r="AA17" t="n">
-        <v>-4.1802</v>
+        <v>-0.7429</v>
       </c>
       <c r="AB17" t="n">
-        <v>5.4255</v>
+        <v>0.3254</v>
       </c>
       <c r="AC17" t="n">
-        <v>-7.3348</v>
+        <v>10.3828</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>165.4</v>
+        <v>199.81</v>
       </c>
       <c r="C18" t="n">
-        <v>171.88</v>
+        <v>204.55</v>
       </c>
       <c r="D18" t="n">
-        <v>150.08</v>
+        <v>189.46</v>
       </c>
       <c r="E18" t="n">
-        <v>165.28</v>
+        <v>192.45</v>
       </c>
       <c r="F18" t="n">
-        <v>73.7</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="G18" t="n">
-        <v>74.39</v>
+        <v>76.69</v>
       </c>
       <c r="H18" t="n">
-        <v>70.76000000000001</v>
+        <v>73.89</v>
       </c>
       <c r="I18" t="n">
-        <v>72.23</v>
+        <v>76.34</v>
       </c>
       <c r="J18" t="n">
-        <v>4.8</v>
+        <v>3.87</v>
       </c>
       <c r="K18" t="n">
-        <v>5.14</v>
+        <v>4.12</v>
       </c>
       <c r="L18" t="n">
-        <v>4.66</v>
+        <v>3.75</v>
       </c>
       <c r="M18" t="n">
-        <v>4.8</v>
+        <v>4.07</v>
       </c>
       <c r="N18" t="n">
-        <v>39.64</v>
+        <v>38.93</v>
       </c>
       <c r="O18" t="n">
-        <v>41.11</v>
+        <v>39.47</v>
       </c>
       <c r="P18" t="n">
-        <v>39.29</v>
+        <v>37.93</v>
       </c>
       <c r="Q18" t="n">
-        <v>40.38</v>
+        <v>38.1</v>
       </c>
       <c r="R18" t="n">
-        <v>-15.0886</v>
+        <v>10.0847</v>
       </c>
       <c r="S18" t="n">
-        <v>-24.0267</v>
+        <v>-1.1302</v>
       </c>
       <c r="T18" t="n">
-        <v>-30.1201</v>
+        <v>-11.5376</v>
       </c>
       <c r="U18" t="n">
-        <v>-5.4829</v>
+        <v>4.978</v>
       </c>
       <c r="V18" t="n">
-        <v>-6.7519</v>
+        <v>-0.1047</v>
       </c>
       <c r="W18" t="n">
-        <v>-6.4257</v>
+        <v>-1.4459</v>
       </c>
       <c r="X18" t="n">
-        <v>15.1079</v>
+        <v>-9.5556</v>
       </c>
       <c r="Y18" t="n">
-        <v>24.3523</v>
+        <v>-2.3981</v>
       </c>
       <c r="Z18" t="n">
-        <v>29.0323</v>
+        <v>5.4404</v>
       </c>
       <c r="AA18" t="n">
-        <v>5.4859</v>
+        <v>-4.9401</v>
       </c>
       <c r="AB18" t="n">
-        <v>6.5998</v>
+        <v>-0.4702</v>
       </c>
       <c r="AC18" t="n">
-        <v>5.8176</v>
+        <v>0.5808</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>159.21</v>
+        <v>182.4</v>
       </c>
       <c r="C19" t="n">
-        <v>176.75</v>
+        <v>195.94</v>
       </c>
       <c r="D19" t="n">
-        <v>158.87</v>
+        <v>176.8</v>
       </c>
       <c r="E19" t="n">
-        <v>174.82</v>
+        <v>192.26</v>
       </c>
       <c r="F19" t="n">
-        <v>70.8</v>
+        <v>75.53</v>
       </c>
       <c r="G19" t="n">
-        <v>73.02</v>
+        <v>77.31999999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>69.56999999999999</v>
+        <v>74.33</v>
       </c>
       <c r="I19" t="n">
-        <v>72.72</v>
+        <v>77.03</v>
       </c>
       <c r="J19" t="n">
-        <v>4.98</v>
+        <v>4.27</v>
       </c>
       <c r="K19" t="n">
-        <v>4.99</v>
+        <v>4.39</v>
       </c>
       <c r="L19" t="n">
-        <v>4.46</v>
+        <v>3.99</v>
       </c>
       <c r="M19" t="n">
-        <v>4.5</v>
+        <v>4.08</v>
       </c>
       <c r="N19" t="n">
-        <v>41.18</v>
+        <v>38.49</v>
       </c>
       <c r="O19" t="n">
-        <v>41.86</v>
+        <v>39.14</v>
       </c>
       <c r="P19" t="n">
-        <v>39.93</v>
+        <v>37.64</v>
       </c>
       <c r="Q19" t="n">
-        <v>40.08</v>
+        <v>37.78</v>
       </c>
       <c r="R19" t="n">
-        <v>5.772</v>
+        <v>-0.0987</v>
       </c>
       <c r="S19" t="n">
-        <v>-3.6645</v>
+        <v>16.3238</v>
       </c>
       <c r="T19" t="n">
-        <v>-34.4532</v>
+        <v>5.9459</v>
       </c>
       <c r="U19" t="n">
-        <v>0.6784</v>
+        <v>0.9039</v>
       </c>
       <c r="V19" t="n">
-        <v>-0.8589</v>
+        <v>6.6454</v>
       </c>
       <c r="W19" t="n">
-        <v>-10.2222</v>
+        <v>5.017</v>
       </c>
       <c r="X19" t="n">
-        <v>-6.25</v>
+        <v>0.2457</v>
       </c>
       <c r="Y19" t="n">
-        <v>-0.2217</v>
+        <v>-15</v>
       </c>
       <c r="Z19" t="n">
-        <v>38.8889</v>
+        <v>-9.5344</v>
       </c>
       <c r="AA19" t="n">
-        <v>-0.7429</v>
+        <v>-0.8399</v>
       </c>
       <c r="AB19" t="n">
-        <v>0.3254</v>
+        <v>-6.4388</v>
       </c>
       <c r="AC19" t="n">
-        <v>10.3828</v>
+        <v>-5.4318</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>199.81</v>
+        <v>174.61</v>
       </c>
       <c r="C20" t="n">
-        <v>204.55</v>
+        <v>177.66</v>
       </c>
       <c r="D20" t="n">
-        <v>189.46</v>
+        <v>161.55</v>
       </c>
       <c r="E20" t="n">
-        <v>192.45</v>
+        <v>165.37</v>
       </c>
       <c r="F20" t="n">
-        <v>74.84999999999999</v>
+        <v>74.54000000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>76.69</v>
+        <v>74.845</v>
       </c>
       <c r="H20" t="n">
-        <v>73.89</v>
+        <v>72.0903</v>
       </c>
       <c r="I20" t="n">
-        <v>76.34</v>
+        <v>72.64</v>
       </c>
       <c r="J20" t="n">
-        <v>3.87</v>
+        <v>4.435</v>
       </c>
       <c r="K20" t="n">
-        <v>4.12</v>
+        <v>4.73</v>
       </c>
       <c r="L20" t="n">
-        <v>3.75</v>
+        <v>4.38</v>
       </c>
       <c r="M20" t="n">
-        <v>4.07</v>
+        <v>4.65</v>
       </c>
       <c r="N20" t="n">
-        <v>38.93</v>
+        <v>39.005</v>
       </c>
       <c r="O20" t="n">
-        <v>39.47</v>
+        <v>40.21</v>
       </c>
       <c r="P20" t="n">
-        <v>37.93</v>
+        <v>38.85</v>
       </c>
       <c r="Q20" t="n">
-        <v>38.1</v>
+        <v>39.95</v>
       </c>
       <c r="R20" t="n">
-        <v>10.0847</v>
+        <v>-13.9863</v>
       </c>
       <c r="S20" t="n">
-        <v>-1.1302</v>
+        <v>-5.4056</v>
       </c>
       <c r="T20" t="n">
-        <v>-11.5376</v>
+        <v>-15.0424</v>
       </c>
       <c r="U20" t="n">
-        <v>4.978</v>
+        <v>-5.6991</v>
       </c>
       <c r="V20" t="n">
-        <v>-0.1047</v>
+        <v>-0.11</v>
       </c>
       <c r="W20" t="n">
-        <v>-1.4459</v>
+        <v>-4.9463</v>
       </c>
       <c r="X20" t="n">
-        <v>-9.5556</v>
+        <v>13.9706</v>
       </c>
       <c r="Y20" t="n">
-        <v>-2.3981</v>
+        <v>3.3333</v>
       </c>
       <c r="Z20" t="n">
-        <v>5.4404</v>
+        <v>11.5108</v>
       </c>
       <c r="AA20" t="n">
-        <v>-4.9401</v>
+        <v>5.7438</v>
       </c>
       <c r="AB20" t="n">
-        <v>-0.4702</v>
+        <v>-0.3244</v>
       </c>
       <c r="AC20" t="n">
-        <v>0.5808</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>182.4</v>
-      </c>
-      <c r="C21" t="n">
-        <v>195.94</v>
-      </c>
-      <c r="D21" t="n">
-        <v>176.83</v>
-      </c>
-      <c r="E21" t="n">
-        <v>192.26</v>
-      </c>
-      <c r="F21" t="n">
-        <v>75.529</v>
-      </c>
-      <c r="G21" t="n">
-        <v>77.31999999999999</v>
-      </c>
-      <c r="H21" t="n">
-        <v>74.33</v>
-      </c>
-      <c r="I21" t="n">
-        <v>77.03</v>
-      </c>
-      <c r="J21" t="n">
-        <v>4.27</v>
-      </c>
-      <c r="K21" t="n">
-        <v>4.39</v>
-      </c>
-      <c r="L21" t="n">
-        <v>3.99</v>
-      </c>
-      <c r="M21" t="n">
-        <v>4.08</v>
-      </c>
-      <c r="N21" t="n">
-        <v>38.485</v>
-      </c>
-      <c r="O21" t="n">
-        <v>39.14</v>
-      </c>
-      <c r="P21" t="n">
-        <v>37.64</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>37.78</v>
-      </c>
-      <c r="R21" t="n">
-        <v>-0.0987</v>
-      </c>
-      <c r="S21" t="n">
-        <v>16.3238</v>
-      </c>
-      <c r="T21" t="n">
-        <v>5.9459</v>
-      </c>
-      <c r="U21" t="n">
-        <v>0.9039</v>
-      </c>
-      <c r="V21" t="n">
-        <v>6.6454</v>
-      </c>
-      <c r="W21" t="n">
-        <v>5.017</v>
-      </c>
-      <c r="X21" t="n">
-        <v>0.2457</v>
-      </c>
-      <c r="Y21" t="n">
-        <v>-15</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>-9.5344</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>-0.8399</v>
-      </c>
-      <c r="AB21" t="n">
-        <v>-6.4388</v>
-      </c>
-      <c r="AC21" t="n">
-        <v>-5.4318</v>
+        <v>4.3626</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2230,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-07-14 22:56
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC20"/>
+  <dimension ref="A1:AC21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2105,7 +2105,7 @@
         <v>174.61</v>
       </c>
       <c r="C20" t="n">
-        <v>177.66</v>
+        <v>177.67</v>
       </c>
       <c r="D20" t="n">
         <v>161.55</v>
@@ -2117,16 +2117,16 @@
         <v>74.54000000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>74.845</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="H20" t="n">
-        <v>72.0903</v>
+        <v>72.09</v>
       </c>
       <c r="I20" t="n">
         <v>72.64</v>
       </c>
       <c r="J20" t="n">
-        <v>4.435</v>
+        <v>4.44</v>
       </c>
       <c r="K20" t="n">
         <v>4.73</v>
@@ -2138,7 +2138,7 @@
         <v>4.65</v>
       </c>
       <c r="N20" t="n">
-        <v>39.005</v>
+        <v>39.01</v>
       </c>
       <c r="O20" t="n">
         <v>40.21</v>
@@ -2184,6 +2184,97 @@
       </c>
       <c r="AC20" t="n">
         <v>4.3626</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>187.69</v>
+      </c>
+      <c r="C21" t="n">
+        <v>188.426</v>
+      </c>
+      <c r="D21" t="n">
+        <v>170.26</v>
+      </c>
+      <c r="E21" t="n">
+        <v>176.66</v>
+      </c>
+      <c r="F21" t="n">
+        <v>75.19</v>
+      </c>
+      <c r="G21" t="n">
+        <v>75.84</v>
+      </c>
+      <c r="H21" t="n">
+        <v>73.41500000000001</v>
+      </c>
+      <c r="I21" t="n">
+        <v>75.02</v>
+      </c>
+      <c r="J21" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="K21" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L21" t="n">
+        <v>3.9698</v>
+      </c>
+      <c r="M21" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="N21" t="n">
+        <v>38.53</v>
+      </c>
+      <c r="O21" t="n">
+        <v>39.5299</v>
+      </c>
+      <c r="P21" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>38.63</v>
+      </c>
+      <c r="R21" t="n">
+        <v>6.8271</v>
+      </c>
+      <c r="S21" t="n">
+        <v>-8.204700000000001</v>
+      </c>
+      <c r="T21" t="n">
+        <v>6.8853</v>
+      </c>
+      <c r="U21" t="n">
+        <v>3.2764</v>
+      </c>
+      <c r="V21" t="n">
+        <v>-1.7291</v>
+      </c>
+      <c r="W21" t="n">
+        <v>3.8627</v>
+      </c>
+      <c r="X21" t="n">
+        <v>-7.957</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>5.1597</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>-10.8333</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>-3.3041</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>1.3911</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>-4.3338</v>
       </c>
     </row>
   </sheetData>
@@ -2230,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-07-15 22:58
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1713 +568,1713 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>265.99</v>
+        <v>267.13</v>
       </c>
       <c r="C2" t="n">
-        <v>274.88</v>
+        <v>274.93</v>
       </c>
       <c r="D2" t="n">
-        <v>261.6</v>
+        <v>226</v>
       </c>
       <c r="E2" t="n">
-        <v>272.5</v>
+        <v>226.19</v>
       </c>
       <c r="F2" t="n">
-        <v>82.6896</v>
+        <v>83.9966</v>
       </c>
       <c r="G2" t="n">
-        <v>84.8347</v>
+        <v>84.63509999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>82.4502</v>
+        <v>79.67659999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>84.39570000000001</v>
+        <v>79.74639999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>4.0231</v>
+        <v>3.9836</v>
       </c>
       <c r="K2" t="n">
-        <v>4.122</v>
+        <v>4.5965</v>
       </c>
       <c r="L2" t="n">
         <v>3.865</v>
       </c>
       <c r="M2" t="n">
-        <v>3.9045</v>
+        <v>4.5767</v>
       </c>
       <c r="N2" t="n">
-        <v>36.6641</v>
+        <v>35.9652</v>
       </c>
       <c r="O2" t="n">
-        <v>36.7723</v>
+        <v>37.7861</v>
       </c>
       <c r="P2" t="n">
-        <v>35.5814</v>
+        <v>35.6896</v>
       </c>
       <c r="Q2" t="n">
-        <v>35.7389</v>
+        <v>37.7468</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>267.13</v>
+        <v>247.42</v>
       </c>
       <c r="C3" t="n">
-        <v>274.93</v>
+        <v>259.79</v>
       </c>
       <c r="D3" t="n">
-        <v>226</v>
+        <v>233.3</v>
       </c>
       <c r="E3" t="n">
-        <v>226.19</v>
+        <v>233.86</v>
       </c>
       <c r="F3" t="n">
-        <v>83.9966</v>
+        <v>81.4824</v>
       </c>
       <c r="G3" t="n">
-        <v>84.63509999999999</v>
+        <v>81.6221</v>
       </c>
       <c r="H3" t="n">
-        <v>79.67659999999999</v>
+        <v>76.7633</v>
       </c>
       <c r="I3" t="n">
-        <v>79.74639999999999</v>
+        <v>77.36190000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>3.9836</v>
+        <v>4.122</v>
       </c>
       <c r="K3" t="n">
-        <v>4.5965</v>
+        <v>4.4086</v>
       </c>
       <c r="L3" t="n">
-        <v>3.865</v>
+        <v>3.8749</v>
       </c>
       <c r="M3" t="n">
-        <v>4.5767</v>
+        <v>4.4086</v>
       </c>
       <c r="N3" t="n">
-        <v>35.9652</v>
+        <v>36.9397</v>
       </c>
       <c r="O3" t="n">
-        <v>37.7861</v>
+        <v>39.1641</v>
       </c>
       <c r="P3" t="n">
-        <v>35.6896</v>
+        <v>36.8708</v>
       </c>
       <c r="Q3" t="n">
-        <v>37.7468</v>
+        <v>38.8984</v>
       </c>
       <c r="R3" t="n">
-        <v>-16.9945</v>
+        <v>3.391</v>
       </c>
       <c r="U3" t="n">
-        <v>-5.5089</v>
+        <v>-2.9901</v>
       </c>
       <c r="X3" t="n">
-        <v>17.216</v>
+        <v>-3.673</v>
       </c>
       <c r="AA3" t="n">
-        <v>5.6182</v>
+        <v>3.0509</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>247.42</v>
+        <v>266.04</v>
       </c>
       <c r="C4" t="n">
-        <v>259.79</v>
+        <v>286.15</v>
       </c>
       <c r="D4" t="n">
-        <v>233.3</v>
+        <v>265</v>
       </c>
       <c r="E4" t="n">
-        <v>233.86</v>
+        <v>279.29</v>
       </c>
       <c r="F4" t="n">
-        <v>81.4824</v>
+        <v>81.9114</v>
       </c>
       <c r="G4" t="n">
-        <v>81.6221</v>
+        <v>83.408</v>
       </c>
       <c r="H4" t="n">
-        <v>76.7633</v>
+        <v>80.4448</v>
       </c>
       <c r="I4" t="n">
-        <v>77.36190000000001</v>
+        <v>82.67959999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>4.122</v>
+        <v>3.8156</v>
       </c>
       <c r="K4" t="n">
-        <v>4.4086</v>
+        <v>3.8254</v>
       </c>
       <c r="L4" t="n">
-        <v>3.8749</v>
+        <v>3.4103</v>
       </c>
       <c r="M4" t="n">
-        <v>4.4086</v>
+        <v>3.5487</v>
       </c>
       <c r="N4" t="n">
-        <v>36.9397</v>
+        <v>36.6149</v>
       </c>
       <c r="O4" t="n">
-        <v>39.1641</v>
+        <v>37.3531</v>
       </c>
       <c r="P4" t="n">
-        <v>36.8708</v>
+        <v>35.857</v>
       </c>
       <c r="Q4" t="n">
-        <v>38.8984</v>
+        <v>36.1719</v>
       </c>
       <c r="R4" t="n">
-        <v>3.391</v>
+        <v>19.4262</v>
       </c>
       <c r="U4" t="n">
-        <v>-2.9901</v>
+        <v>6.8738</v>
       </c>
       <c r="X4" t="n">
-        <v>-3.673</v>
+        <v>-19.5051</v>
       </c>
       <c r="AA4" t="n">
-        <v>3.0509</v>
+        <v>-7.0093</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>266.04</v>
+        <v>299.26</v>
       </c>
       <c r="C5" t="n">
-        <v>286.15</v>
+        <v>302</v>
       </c>
       <c r="D5" t="n">
-        <v>265</v>
+        <v>286.24</v>
       </c>
       <c r="E5" t="n">
-        <v>279.29</v>
+        <v>300.77</v>
       </c>
       <c r="F5" t="n">
-        <v>81.9114</v>
+        <v>83.7572</v>
       </c>
       <c r="G5" t="n">
-        <v>83.408</v>
+        <v>84.9145</v>
       </c>
       <c r="H5" t="n">
-        <v>80.4448</v>
+        <v>81.203</v>
       </c>
       <c r="I5" t="n">
-        <v>82.67959999999999</v>
+        <v>82.3903</v>
       </c>
       <c r="J5" t="n">
-        <v>3.8156</v>
+        <v>3.2917</v>
       </c>
       <c r="K5" t="n">
-        <v>3.8254</v>
+        <v>3.4498</v>
       </c>
       <c r="L5" t="n">
-        <v>3.4103</v>
+        <v>3.2521</v>
       </c>
       <c r="M5" t="n">
-        <v>3.5487</v>
+        <v>3.262</v>
       </c>
       <c r="N5" t="n">
-        <v>36.6149</v>
+        <v>35.7389</v>
       </c>
       <c r="O5" t="n">
-        <v>37.3531</v>
+        <v>36.8511</v>
       </c>
       <c r="P5" t="n">
-        <v>35.857</v>
+        <v>35.2369</v>
       </c>
       <c r="Q5" t="n">
-        <v>36.1719</v>
+        <v>36.3491</v>
       </c>
       <c r="R5" t="n">
-        <v>19.4262</v>
+        <v>7.6909</v>
       </c>
       <c r="S5" t="n">
-        <v>2.4917</v>
+        <v>32.9723</v>
       </c>
       <c r="U5" t="n">
-        <v>6.8738</v>
+        <v>-0.3499</v>
       </c>
       <c r="V5" t="n">
-        <v>-2.0334</v>
+        <v>3.3154</v>
       </c>
       <c r="X5" t="n">
-        <v>-19.5051</v>
+        <v>-8.079000000000001</v>
       </c>
       <c r="Y5" t="n">
-        <v>-9.1126</v>
+        <v>-28.7259</v>
       </c>
       <c r="AA5" t="n">
-        <v>-7.0093</v>
+        <v>0.4899</v>
       </c>
       <c r="AB5" t="n">
-        <v>1.2116</v>
+        <v>-3.7028</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>299.26</v>
+        <v>236</v>
       </c>
       <c r="C6" t="n">
-        <v>302</v>
+        <v>252.98</v>
       </c>
       <c r="D6" t="n">
-        <v>286.24</v>
+        <v>223</v>
       </c>
       <c r="E6" t="n">
-        <v>300.77</v>
+        <v>231.42</v>
       </c>
       <c r="F6" t="n">
-        <v>83.7572</v>
+        <v>74.9474</v>
       </c>
       <c r="G6" t="n">
-        <v>84.9145</v>
+        <v>77.56140000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>81.203</v>
+        <v>73.7402</v>
       </c>
       <c r="I6" t="n">
-        <v>82.3903</v>
+        <v>74.26900000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>3.2917</v>
+        <v>3.99</v>
       </c>
       <c r="K6" t="n">
-        <v>3.4498</v>
+        <v>4.13</v>
       </c>
       <c r="L6" t="n">
-        <v>3.2521</v>
+        <v>3.8</v>
       </c>
       <c r="M6" t="n">
-        <v>3.262</v>
+        <v>4.04</v>
       </c>
       <c r="N6" t="n">
-        <v>35.7389</v>
+        <v>39.6267</v>
       </c>
       <c r="O6" t="n">
-        <v>36.8511</v>
+        <v>40.1582</v>
       </c>
       <c r="P6" t="n">
-        <v>35.2369</v>
+        <v>38.4653</v>
       </c>
       <c r="Q6" t="n">
-        <v>36.3491</v>
+        <v>39.922</v>
       </c>
       <c r="R6" t="n">
-        <v>7.6909</v>
+        <v>-23.0575</v>
       </c>
       <c r="S6" t="n">
-        <v>32.9723</v>
+        <v>-1.0434</v>
       </c>
       <c r="U6" t="n">
-        <v>-0.3499</v>
+        <v>-9.857100000000001</v>
       </c>
       <c r="V6" t="n">
-        <v>3.3154</v>
+        <v>-3.998</v>
       </c>
       <c r="X6" t="n">
-        <v>-8.079000000000001</v>
+        <v>23.8504</v>
       </c>
       <c r="Y6" t="n">
-        <v>-28.7259</v>
+        <v>-8.360900000000001</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.4899</v>
+        <v>9.8294</v>
       </c>
       <c r="AB6" t="n">
-        <v>-3.7028</v>
+        <v>2.6315</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>236</v>
+        <v>233.11</v>
       </c>
       <c r="C7" t="n">
-        <v>252.98</v>
+        <v>237</v>
       </c>
       <c r="D7" t="n">
-        <v>223</v>
+        <v>211.13</v>
       </c>
       <c r="E7" t="n">
-        <v>231.42</v>
+        <v>229.57</v>
       </c>
       <c r="F7" t="n">
-        <v>74.9474</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>77.56140000000001</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>73.7402</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>74.26900000000001</v>
+        <v>73.3</v>
       </c>
       <c r="J7" t="n">
-        <v>3.99</v>
+        <v>4</v>
       </c>
       <c r="K7" t="n">
-        <v>4.13</v>
+        <v>4.39</v>
       </c>
       <c r="L7" t="n">
-        <v>3.8</v>
+        <v>3.92</v>
       </c>
       <c r="M7" t="n">
-        <v>4.04</v>
+        <v>4.08</v>
       </c>
       <c r="N7" t="n">
-        <v>39.6267</v>
+        <v>39.66</v>
       </c>
       <c r="O7" t="n">
-        <v>40.1582</v>
+        <v>41.49</v>
       </c>
       <c r="P7" t="n">
-        <v>38.4653</v>
+        <v>38.9</v>
       </c>
       <c r="Q7" t="n">
-        <v>39.922</v>
+        <v>40.45</v>
       </c>
       <c r="R7" t="n">
-        <v>-23.0575</v>
+        <v>-0.7994</v>
       </c>
       <c r="S7" t="n">
-        <v>-1.0434</v>
+        <v>-17.8023</v>
       </c>
       <c r="T7" t="n">
-        <v>-15.0752</v>
+        <v>1.4943</v>
       </c>
       <c r="U7" t="n">
-        <v>-9.857100000000001</v>
+        <v>-1.3047</v>
       </c>
       <c r="V7" t="n">
-        <v>-3.998</v>
+        <v>-11.3445</v>
       </c>
       <c r="W7" t="n">
-        <v>-11.9991</v>
+        <v>-8.083600000000001</v>
       </c>
       <c r="X7" t="n">
-        <v>23.8504</v>
+        <v>0.9901</v>
       </c>
       <c r="Y7" t="n">
-        <v>-8.360900000000001</v>
+        <v>14.9717</v>
       </c>
       <c r="Z7" t="n">
-        <v>3.4704</v>
+        <v>-10.8528</v>
       </c>
       <c r="AA7" t="n">
-        <v>9.8294</v>
+        <v>1.3226</v>
       </c>
       <c r="AB7" t="n">
-        <v>2.6315</v>
+        <v>11.8271</v>
       </c>
       <c r="AC7" t="n">
-        <v>11.7046</v>
+        <v>7.1614</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>233.11</v>
+        <v>268.05</v>
       </c>
       <c r="C8" t="n">
-        <v>237</v>
+        <v>268.4</v>
       </c>
       <c r="D8" t="n">
-        <v>211.13</v>
+        <v>225.74</v>
       </c>
       <c r="E8" t="n">
-        <v>229.57</v>
+        <v>252.61</v>
       </c>
       <c r="F8" t="n">
-        <v>74.79000000000001</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>76.18000000000001</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>71.34999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I8" t="n">
-        <v>73.3</v>
+        <v>74.95</v>
       </c>
       <c r="J8" t="n">
-        <v>4</v>
+        <v>3.38</v>
       </c>
       <c r="K8" t="n">
-        <v>4.39</v>
+        <v>4.15</v>
       </c>
       <c r="L8" t="n">
-        <v>3.92</v>
+        <v>3.37</v>
       </c>
       <c r="M8" t="n">
-        <v>4.08</v>
+        <v>3.63</v>
       </c>
       <c r="N8" t="n">
-        <v>39.66</v>
+        <v>37.87</v>
       </c>
       <c r="O8" t="n">
-        <v>41.49</v>
+        <v>41.37</v>
       </c>
       <c r="P8" t="n">
-        <v>38.9</v>
+        <v>37.71</v>
       </c>
       <c r="Q8" t="n">
-        <v>40.45</v>
+        <v>39.47</v>
       </c>
       <c r="R8" t="n">
-        <v>-0.7994</v>
+        <v>10.0362</v>
       </c>
       <c r="S8" t="n">
-        <v>-17.8023</v>
+        <v>-16.0122</v>
       </c>
       <c r="T8" t="n">
-        <v>1.4943</v>
+        <v>8.0176</v>
       </c>
       <c r="U8" t="n">
-        <v>-1.3047</v>
+        <v>2.251</v>
       </c>
       <c r="V8" t="n">
-        <v>-11.3445</v>
+        <v>-9.0306</v>
       </c>
       <c r="W8" t="n">
-        <v>-8.083600000000001</v>
+        <v>-3.1177</v>
       </c>
       <c r="X8" t="n">
-        <v>0.9901</v>
+        <v>-11.0294</v>
       </c>
       <c r="Y8" t="n">
-        <v>14.9717</v>
+        <v>11.2814</v>
       </c>
       <c r="Z8" t="n">
-        <v>-10.8528</v>
+        <v>-17.6609</v>
       </c>
       <c r="AA8" t="n">
-        <v>1.3226</v>
+        <v>-2.4227</v>
       </c>
       <c r="AB8" t="n">
-        <v>11.8271</v>
+        <v>8.585900000000001</v>
       </c>
       <c r="AC8" t="n">
-        <v>7.1614</v>
+        <v>1.4695</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>268.05</v>
+        <v>226.24</v>
       </c>
       <c r="C9" t="n">
-        <v>268.4</v>
+        <v>231.25</v>
       </c>
       <c r="D9" t="n">
-        <v>225.74</v>
+        <v>212.1</v>
       </c>
       <c r="E9" t="n">
-        <v>252.61</v>
+        <v>215.6</v>
       </c>
       <c r="F9" t="n">
-        <v>77.95999999999999</v>
+        <v>72.09</v>
       </c>
       <c r="G9" t="n">
-        <v>78.23999999999999</v>
+        <v>74.69</v>
       </c>
       <c r="H9" t="n">
-        <v>71.59999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="I9" t="n">
-        <v>74.95</v>
+        <v>71.83</v>
       </c>
       <c r="J9" t="n">
-        <v>3.38</v>
+        <v>4.04</v>
       </c>
       <c r="K9" t="n">
-        <v>4.15</v>
+        <v>4.25</v>
       </c>
       <c r="L9" t="n">
-        <v>3.37</v>
+        <v>3.95</v>
       </c>
       <c r="M9" t="n">
-        <v>3.63</v>
+        <v>4.24</v>
       </c>
       <c r="N9" t="n">
-        <v>37.87</v>
+        <v>41.08</v>
       </c>
       <c r="O9" t="n">
-        <v>41.37</v>
+        <v>41.79</v>
       </c>
       <c r="P9" t="n">
-        <v>37.71</v>
+        <v>39.69</v>
       </c>
       <c r="Q9" t="n">
-        <v>39.47</v>
+        <v>41.31</v>
       </c>
       <c r="R9" t="n">
-        <v>10.0362</v>
+        <v>-14.651</v>
       </c>
       <c r="S9" t="n">
-        <v>-16.0122</v>
+        <v>-6.8361</v>
       </c>
       <c r="T9" t="n">
-        <v>8.0176</v>
+        <v>-22.8043</v>
       </c>
       <c r="U9" t="n">
-        <v>2.251</v>
+        <v>-4.1628</v>
       </c>
       <c r="V9" t="n">
-        <v>-9.0306</v>
+        <v>-3.284</v>
       </c>
       <c r="W9" t="n">
-        <v>-3.1177</v>
+        <v>-13.1225</v>
       </c>
       <c r="X9" t="n">
-        <v>-11.0294</v>
+        <v>16.8044</v>
       </c>
       <c r="Y9" t="n">
-        <v>11.2814</v>
+        <v>4.9505</v>
       </c>
       <c r="Z9" t="n">
-        <v>-17.6609</v>
+        <v>19.4804</v>
       </c>
       <c r="AA9" t="n">
-        <v>-2.4227</v>
+        <v>4.6618</v>
       </c>
       <c r="AB9" t="n">
-        <v>8.585900000000001</v>
+        <v>3.4768</v>
       </c>
       <c r="AC9" t="n">
-        <v>1.4695</v>
+        <v>14.2047</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>226.24</v>
+        <v>216.36</v>
       </c>
       <c r="C10" t="n">
-        <v>231.25</v>
+        <v>238.65</v>
       </c>
       <c r="D10" t="n">
-        <v>212.1</v>
+        <v>192.3</v>
       </c>
       <c r="E10" t="n">
-        <v>215.6</v>
+        <v>236.52</v>
       </c>
       <c r="F10" t="n">
-        <v>72.09</v>
+        <v>74.12</v>
       </c>
       <c r="G10" t="n">
-        <v>74.69</v>
+        <v>77.38</v>
       </c>
       <c r="H10" t="n">
-        <v>70.72</v>
+        <v>71.45</v>
       </c>
       <c r="I10" t="n">
-        <v>71.83</v>
+        <v>77.19</v>
       </c>
       <c r="J10" t="n">
-        <v>4.04</v>
+        <v>4.16</v>
       </c>
       <c r="K10" t="n">
-        <v>4.25</v>
+        <v>4.63</v>
       </c>
       <c r="L10" t="n">
-        <v>3.95</v>
+        <v>3.7</v>
       </c>
       <c r="M10" t="n">
-        <v>4.24</v>
+        <v>3.72</v>
       </c>
       <c r="N10" t="n">
-        <v>41.08</v>
+        <v>39.91</v>
       </c>
       <c r="O10" t="n">
-        <v>41.79</v>
+        <v>41.43</v>
       </c>
       <c r="P10" t="n">
-        <v>39.69</v>
+        <v>38.08</v>
       </c>
       <c r="Q10" t="n">
-        <v>41.31</v>
+        <v>38.16</v>
       </c>
       <c r="R10" t="n">
-        <v>-14.651</v>
+        <v>9.703200000000001</v>
       </c>
       <c r="S10" t="n">
-        <v>-6.8361</v>
+        <v>3.0274</v>
       </c>
       <c r="T10" t="n">
-        <v>-22.8043</v>
+        <v>-21.3618</v>
       </c>
       <c r="U10" t="n">
-        <v>-4.1628</v>
+        <v>7.4621</v>
       </c>
       <c r="V10" t="n">
-        <v>-3.284</v>
+        <v>5.307</v>
       </c>
       <c r="W10" t="n">
-        <v>-13.1225</v>
+        <v>-6.3118</v>
       </c>
       <c r="X10" t="n">
-        <v>16.8044</v>
+        <v>-12.2642</v>
       </c>
       <c r="Y10" t="n">
-        <v>4.9505</v>
+        <v>-8.823499999999999</v>
       </c>
       <c r="Z10" t="n">
-        <v>19.4804</v>
+        <v>14.0405</v>
       </c>
       <c r="AA10" t="n">
-        <v>4.6618</v>
+        <v>-7.6253</v>
       </c>
       <c r="AB10" t="n">
-        <v>3.4768</v>
+        <v>-5.6613</v>
       </c>
       <c r="AC10" t="n">
-        <v>14.2047</v>
+        <v>4.982</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>216.36</v>
+        <v>241.45</v>
       </c>
       <c r="C11" t="n">
-        <v>238.65</v>
+        <v>272</v>
       </c>
       <c r="D11" t="n">
-        <v>192.3</v>
+        <v>240.59</v>
       </c>
       <c r="E11" t="n">
-        <v>236.52</v>
+        <v>266.71</v>
       </c>
       <c r="F11" t="n">
-        <v>74.12</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>77.38</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>71.45</v>
+        <v>77.15000000000001</v>
       </c>
       <c r="I11" t="n">
-        <v>77.19</v>
+        <v>81</v>
       </c>
       <c r="J11" t="n">
-        <v>4.16</v>
+        <v>3.66</v>
       </c>
       <c r="K11" t="n">
-        <v>4.63</v>
+        <v>3.68</v>
       </c>
       <c r="L11" t="n">
-        <v>3.7</v>
+        <v>3.17</v>
       </c>
       <c r="M11" t="n">
-        <v>3.72</v>
+        <v>3.24</v>
       </c>
       <c r="N11" t="n">
-        <v>39.91</v>
+        <v>38.16</v>
       </c>
       <c r="O11" t="n">
-        <v>41.43</v>
+        <v>38.2</v>
       </c>
       <c r="P11" t="n">
-        <v>38.08</v>
+        <v>36.03</v>
       </c>
       <c r="Q11" t="n">
-        <v>38.16</v>
+        <v>36.31</v>
       </c>
       <c r="R11" t="n">
-        <v>9.703200000000001</v>
+        <v>12.7642</v>
       </c>
       <c r="S11" t="n">
-        <v>3.0274</v>
+        <v>5.5817</v>
       </c>
       <c r="T11" t="n">
-        <v>-21.3618</v>
+        <v>15.2493</v>
       </c>
       <c r="U11" t="n">
-        <v>7.4621</v>
+        <v>4.9359</v>
       </c>
       <c r="V11" t="n">
-        <v>5.307</v>
+        <v>8.071999999999999</v>
       </c>
       <c r="W11" t="n">
-        <v>-6.3118</v>
+        <v>9.063000000000001</v>
       </c>
       <c r="X11" t="n">
-        <v>-12.2642</v>
+        <v>-12.9032</v>
       </c>
       <c r="Y11" t="n">
-        <v>-8.823499999999999</v>
+        <v>-10.7438</v>
       </c>
       <c r="Z11" t="n">
-        <v>14.0405</v>
+        <v>-19.802</v>
       </c>
       <c r="AA11" t="n">
-        <v>-7.6253</v>
+        <v>-4.848</v>
       </c>
       <c r="AB11" t="n">
-        <v>-5.6613</v>
+        <v>-8.0061</v>
       </c>
       <c r="AC11" t="n">
-        <v>4.982</v>
+        <v>-9.047599999999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>241.45</v>
+        <v>237.79</v>
       </c>
       <c r="C12" t="n">
-        <v>272</v>
+        <v>246.47</v>
       </c>
       <c r="D12" t="n">
-        <v>240.59</v>
+        <v>215.38</v>
       </c>
       <c r="E12" t="n">
-        <v>266.71</v>
+        <v>217.55</v>
       </c>
       <c r="F12" t="n">
-        <v>77.23999999999999</v>
+        <v>78.72</v>
       </c>
       <c r="G12" t="n">
-        <v>81.54000000000001</v>
+        <v>79.64</v>
       </c>
       <c r="H12" t="n">
-        <v>77.15000000000001</v>
+        <v>77.23</v>
       </c>
       <c r="I12" t="n">
-        <v>81</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>3.66</v>
+        <v>3.59</v>
       </c>
       <c r="K12" t="n">
-        <v>3.68</v>
+        <v>3.89</v>
       </c>
       <c r="L12" t="n">
-        <v>3.17</v>
+        <v>3.51</v>
       </c>
       <c r="M12" t="n">
-        <v>3.24</v>
+        <v>3.86</v>
       </c>
       <c r="N12" t="n">
-        <v>38.16</v>
+        <v>37.31</v>
       </c>
       <c r="O12" t="n">
-        <v>38.2</v>
+        <v>37.98</v>
       </c>
       <c r="P12" t="n">
-        <v>36.03</v>
+        <v>36.9</v>
       </c>
       <c r="Q12" t="n">
-        <v>36.31</v>
+        <v>37.88</v>
       </c>
       <c r="R12" t="n">
-        <v>12.7642</v>
+        <v>-18.432</v>
       </c>
       <c r="S12" t="n">
-        <v>5.5817</v>
+        <v>0.9045</v>
       </c>
       <c r="T12" t="n">
-        <v>15.2493</v>
+        <v>-5.2359</v>
       </c>
       <c r="U12" t="n">
-        <v>4.9359</v>
+        <v>-4.3704</v>
       </c>
       <c r="V12" t="n">
-        <v>8.071999999999999</v>
+        <v>7.838</v>
       </c>
       <c r="W12" t="n">
-        <v>9.063000000000001</v>
+        <v>5.6753</v>
       </c>
       <c r="X12" t="n">
-        <v>-12.9032</v>
+        <v>19.1358</v>
       </c>
       <c r="Y12" t="n">
-        <v>-10.7438</v>
+        <v>-8.962300000000001</v>
       </c>
       <c r="Z12" t="n">
-        <v>-19.802</v>
+        <v>-5.3922</v>
       </c>
       <c r="AA12" t="n">
-        <v>-4.848</v>
+        <v>4.3239</v>
       </c>
       <c r="AB12" t="n">
-        <v>-8.0061</v>
+        <v>-8.303100000000001</v>
       </c>
       <c r="AC12" t="n">
-        <v>-9.047599999999999</v>
+        <v>-6.3535</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>237.79</v>
+        <v>219.23</v>
       </c>
       <c r="C13" t="n">
-        <v>246.47</v>
+        <v>226.13</v>
       </c>
       <c r="D13" t="n">
-        <v>215.38</v>
+        <v>168.88</v>
       </c>
       <c r="E13" t="n">
-        <v>217.55</v>
+        <v>181.47</v>
       </c>
       <c r="F13" t="n">
-        <v>78.72</v>
+        <v>77.45</v>
       </c>
       <c r="G13" t="n">
-        <v>79.64</v>
+        <v>79.14</v>
       </c>
       <c r="H13" t="n">
-        <v>77.23</v>
+        <v>71.72</v>
       </c>
       <c r="I13" t="n">
-        <v>77.45999999999999</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>3.59</v>
+        <v>3.84</v>
       </c>
       <c r="K13" t="n">
-        <v>3.89</v>
+        <v>4.74</v>
       </c>
       <c r="L13" t="n">
-        <v>3.51</v>
+        <v>3.71</v>
       </c>
       <c r="M13" t="n">
-        <v>3.86</v>
+        <v>4.51</v>
       </c>
       <c r="N13" t="n">
-        <v>37.31</v>
+        <v>37.91</v>
       </c>
       <c r="O13" t="n">
-        <v>37.98</v>
+        <v>40.72</v>
       </c>
       <c r="P13" t="n">
-        <v>36.9</v>
+        <v>37.08</v>
       </c>
       <c r="Q13" t="n">
-        <v>37.88</v>
+        <v>39.95</v>
       </c>
       <c r="R13" t="n">
-        <v>-18.432</v>
+        <v>-16.5847</v>
       </c>
       <c r="S13" t="n">
-        <v>0.9045</v>
+        <v>-23.275</v>
       </c>
       <c r="T13" t="n">
-        <v>-5.2359</v>
+        <v>-28.162</v>
       </c>
       <c r="U13" t="n">
-        <v>-4.3704</v>
+        <v>-5.306</v>
       </c>
       <c r="V13" t="n">
-        <v>7.838</v>
+        <v>-4.9747</v>
       </c>
       <c r="W13" t="n">
-        <v>5.6753</v>
+        <v>-2.1348</v>
       </c>
       <c r="X13" t="n">
-        <v>19.1358</v>
+        <v>16.8394</v>
       </c>
       <c r="Y13" t="n">
-        <v>-8.962300000000001</v>
+        <v>21.2366</v>
       </c>
       <c r="Z13" t="n">
-        <v>-5.3922</v>
+        <v>24.2424</v>
       </c>
       <c r="AA13" t="n">
-        <v>4.3239</v>
+        <v>5.4646</v>
       </c>
       <c r="AB13" t="n">
-        <v>-8.303100000000001</v>
+        <v>4.6908</v>
       </c>
       <c r="AC13" t="n">
-        <v>-6.3535</v>
+        <v>1.2161</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>219.23</v>
+        <v>197.21</v>
       </c>
       <c r="C14" t="n">
-        <v>226.13</v>
+        <v>210.8</v>
       </c>
       <c r="D14" t="n">
-        <v>168.88</v>
+        <v>194.22</v>
       </c>
       <c r="E14" t="n">
-        <v>181.47</v>
+        <v>194.65</v>
       </c>
       <c r="F14" t="n">
+        <v>75.54000000000001</v>
+      </c>
+      <c r="G14" t="n">
         <v>77.45</v>
       </c>
-      <c r="G14" t="n">
-        <v>79.14</v>
-      </c>
       <c r="H14" t="n">
-        <v>71.72</v>
+        <v>75.11</v>
       </c>
       <c r="I14" t="n">
-        <v>73.34999999999999</v>
+        <v>76.42</v>
       </c>
       <c r="J14" t="n">
-        <v>3.84</v>
+        <v>4.11</v>
       </c>
       <c r="K14" t="n">
-        <v>4.74</v>
+        <v>4.18</v>
       </c>
       <c r="L14" t="n">
-        <v>3.71</v>
+        <v>3.77</v>
       </c>
       <c r="M14" t="n">
-        <v>4.51</v>
+        <v>4.17</v>
       </c>
       <c r="N14" t="n">
-        <v>37.91</v>
+        <v>38.75</v>
       </c>
       <c r="O14" t="n">
-        <v>40.72</v>
+        <v>38.98</v>
       </c>
       <c r="P14" t="n">
-        <v>37.08</v>
+        <v>37.71</v>
       </c>
       <c r="Q14" t="n">
-        <v>39.95</v>
+        <v>38.28</v>
       </c>
       <c r="R14" t="n">
-        <v>-16.5847</v>
+        <v>7.2629</v>
       </c>
       <c r="S14" t="n">
-        <v>-23.275</v>
+        <v>-27.0181</v>
       </c>
       <c r="T14" t="n">
-        <v>-28.162</v>
+        <v>-9.7171</v>
       </c>
       <c r="U14" t="n">
-        <v>-5.306</v>
+        <v>4.1854</v>
       </c>
       <c r="V14" t="n">
-        <v>-4.9747</v>
+        <v>-5.6543</v>
       </c>
       <c r="W14" t="n">
-        <v>-2.1348</v>
+        <v>6.3901</v>
       </c>
       <c r="X14" t="n">
-        <v>16.8394</v>
+        <v>-7.5388</v>
       </c>
       <c r="Y14" t="n">
-        <v>21.2366</v>
+        <v>28.7037</v>
       </c>
       <c r="Z14" t="n">
-        <v>24.2424</v>
+        <v>-1.6509</v>
       </c>
       <c r="AA14" t="n">
-        <v>5.4646</v>
+        <v>-4.1802</v>
       </c>
       <c r="AB14" t="n">
-        <v>4.6908</v>
+        <v>5.4255</v>
       </c>
       <c r="AC14" t="n">
-        <v>1.2161</v>
+        <v>-7.3348</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>197.21</v>
+        <v>165.4</v>
       </c>
       <c r="C15" t="n">
-        <v>210.8</v>
+        <v>171.88</v>
       </c>
       <c r="D15" t="n">
-        <v>194.22</v>
+        <v>150.08</v>
       </c>
       <c r="E15" t="n">
-        <v>194.65</v>
+        <v>165.28</v>
       </c>
       <c r="F15" t="n">
-        <v>75.54000000000001</v>
+        <v>73.7</v>
       </c>
       <c r="G15" t="n">
-        <v>77.45</v>
+        <v>74.39</v>
       </c>
       <c r="H15" t="n">
-        <v>75.11</v>
+        <v>70.76000000000001</v>
       </c>
       <c r="I15" t="n">
-        <v>76.42</v>
+        <v>72.23</v>
       </c>
       <c r="J15" t="n">
-        <v>4.11</v>
+        <v>4.8</v>
       </c>
       <c r="K15" t="n">
-        <v>4.18</v>
+        <v>5.14</v>
       </c>
       <c r="L15" t="n">
-        <v>3.77</v>
+        <v>4.66</v>
       </c>
       <c r="M15" t="n">
-        <v>4.17</v>
+        <v>4.8</v>
       </c>
       <c r="N15" t="n">
-        <v>38.75</v>
+        <v>39.64</v>
       </c>
       <c r="O15" t="n">
-        <v>38.98</v>
+        <v>41.11</v>
       </c>
       <c r="P15" t="n">
-        <v>37.71</v>
+        <v>39.29</v>
       </c>
       <c r="Q15" t="n">
-        <v>38.28</v>
+        <v>40.38</v>
       </c>
       <c r="R15" t="n">
-        <v>7.2629</v>
+        <v>-15.0886</v>
       </c>
       <c r="S15" t="n">
-        <v>-27.0181</v>
+        <v>-24.0267</v>
       </c>
       <c r="T15" t="n">
-        <v>-9.7171</v>
+        <v>-30.1201</v>
       </c>
       <c r="U15" t="n">
-        <v>4.1854</v>
+        <v>-5.4829</v>
       </c>
       <c r="V15" t="n">
-        <v>-5.6543</v>
+        <v>-6.7519</v>
       </c>
       <c r="W15" t="n">
-        <v>6.3901</v>
+        <v>-6.4257</v>
       </c>
       <c r="X15" t="n">
-        <v>-7.5388</v>
+        <v>15.1079</v>
       </c>
       <c r="Y15" t="n">
-        <v>28.7037</v>
+        <v>24.3523</v>
       </c>
       <c r="Z15" t="n">
-        <v>-1.6509</v>
+        <v>29.0323</v>
       </c>
       <c r="AA15" t="n">
-        <v>-4.1802</v>
+        <v>5.4859</v>
       </c>
       <c r="AB15" t="n">
-        <v>5.4255</v>
+        <v>6.5998</v>
       </c>
       <c r="AC15" t="n">
-        <v>-7.3348</v>
+        <v>5.8176</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>165.4</v>
+        <v>159.21</v>
       </c>
       <c r="C16" t="n">
-        <v>171.88</v>
+        <v>176.75</v>
       </c>
       <c r="D16" t="n">
-        <v>150.08</v>
+        <v>158.87</v>
       </c>
       <c r="E16" t="n">
-        <v>165.28</v>
+        <v>174.82</v>
       </c>
       <c r="F16" t="n">
-        <v>73.7</v>
+        <v>70.8</v>
       </c>
       <c r="G16" t="n">
-        <v>74.39</v>
+        <v>73.02</v>
       </c>
       <c r="H16" t="n">
-        <v>70.76000000000001</v>
+        <v>69.56999999999999</v>
       </c>
       <c r="I16" t="n">
-        <v>72.23</v>
+        <v>72.72</v>
       </c>
       <c r="J16" t="n">
-        <v>4.8</v>
+        <v>4.98</v>
       </c>
       <c r="K16" t="n">
-        <v>5.14</v>
+        <v>4.99</v>
       </c>
       <c r="L16" t="n">
-        <v>4.66</v>
+        <v>4.46</v>
       </c>
       <c r="M16" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="N16" t="n">
-        <v>39.64</v>
+        <v>41.18</v>
       </c>
       <c r="O16" t="n">
-        <v>41.11</v>
+        <v>41.86</v>
       </c>
       <c r="P16" t="n">
-        <v>39.29</v>
+        <v>39.93</v>
       </c>
       <c r="Q16" t="n">
-        <v>40.38</v>
+        <v>40.08</v>
       </c>
       <c r="R16" t="n">
-        <v>-15.0886</v>
+        <v>5.772</v>
       </c>
       <c r="S16" t="n">
-        <v>-24.0267</v>
+        <v>-3.6645</v>
       </c>
       <c r="T16" t="n">
-        <v>-30.1201</v>
+        <v>-34.4532</v>
       </c>
       <c r="U16" t="n">
-        <v>-5.4829</v>
+        <v>0.6784</v>
       </c>
       <c r="V16" t="n">
-        <v>-6.7519</v>
+        <v>-0.8589</v>
       </c>
       <c r="W16" t="n">
-        <v>-6.4257</v>
+        <v>-10.2222</v>
       </c>
       <c r="X16" t="n">
-        <v>15.1079</v>
+        <v>-6.25</v>
       </c>
       <c r="Y16" t="n">
-        <v>24.3523</v>
+        <v>-0.2217</v>
       </c>
       <c r="Z16" t="n">
-        <v>29.0323</v>
+        <v>38.8889</v>
       </c>
       <c r="AA16" t="n">
-        <v>5.4859</v>
+        <v>-0.7429</v>
       </c>
       <c r="AB16" t="n">
-        <v>6.5998</v>
+        <v>0.3254</v>
       </c>
       <c r="AC16" t="n">
-        <v>5.8176</v>
+        <v>10.3828</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>159.21</v>
+        <v>199.81</v>
       </c>
       <c r="C17" t="n">
-        <v>176.75</v>
+        <v>204.55</v>
       </c>
       <c r="D17" t="n">
-        <v>158.87</v>
+        <v>189.46</v>
       </c>
       <c r="E17" t="n">
-        <v>174.82</v>
+        <v>192.45</v>
       </c>
       <c r="F17" t="n">
-        <v>70.8</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="G17" t="n">
-        <v>73.02</v>
+        <v>76.69</v>
       </c>
       <c r="H17" t="n">
-        <v>69.56999999999999</v>
+        <v>73.89</v>
       </c>
       <c r="I17" t="n">
-        <v>72.72</v>
+        <v>76.34</v>
       </c>
       <c r="J17" t="n">
-        <v>4.98</v>
+        <v>3.87</v>
       </c>
       <c r="K17" t="n">
-        <v>4.99</v>
+        <v>4.12</v>
       </c>
       <c r="L17" t="n">
-        <v>4.46</v>
+        <v>3.75</v>
       </c>
       <c r="M17" t="n">
-        <v>4.5</v>
+        <v>4.07</v>
       </c>
       <c r="N17" t="n">
-        <v>41.18</v>
+        <v>38.93</v>
       </c>
       <c r="O17" t="n">
-        <v>41.86</v>
+        <v>39.47</v>
       </c>
       <c r="P17" t="n">
-        <v>39.93</v>
+        <v>37.93</v>
       </c>
       <c r="Q17" t="n">
-        <v>40.08</v>
+        <v>38.1</v>
       </c>
       <c r="R17" t="n">
-        <v>5.772</v>
+        <v>10.0847</v>
       </c>
       <c r="S17" t="n">
-        <v>-3.6645</v>
+        <v>-1.1302</v>
       </c>
       <c r="T17" t="n">
-        <v>-34.4532</v>
+        <v>-11.5376</v>
       </c>
       <c r="U17" t="n">
-        <v>0.6784</v>
+        <v>4.978</v>
       </c>
       <c r="V17" t="n">
-        <v>-0.8589</v>
+        <v>-0.1047</v>
       </c>
       <c r="W17" t="n">
-        <v>-10.2222</v>
+        <v>-1.4459</v>
       </c>
       <c r="X17" t="n">
-        <v>-6.25</v>
+        <v>-9.5556</v>
       </c>
       <c r="Y17" t="n">
-        <v>-0.2217</v>
+        <v>-2.3981</v>
       </c>
       <c r="Z17" t="n">
-        <v>38.8889</v>
+        <v>5.4404</v>
       </c>
       <c r="AA17" t="n">
-        <v>-0.7429</v>
+        <v>-4.9401</v>
       </c>
       <c r="AB17" t="n">
-        <v>0.3254</v>
+        <v>-0.4702</v>
       </c>
       <c r="AC17" t="n">
-        <v>10.3828</v>
+        <v>0.5808</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>199.81</v>
+        <v>182.4</v>
       </c>
       <c r="C18" t="n">
-        <v>204.55</v>
+        <v>195.94</v>
       </c>
       <c r="D18" t="n">
-        <v>189.46</v>
+        <v>176.8</v>
       </c>
       <c r="E18" t="n">
-        <v>192.45</v>
+        <v>192.26</v>
       </c>
       <c r="F18" t="n">
-        <v>74.84999999999999</v>
+        <v>75.53</v>
       </c>
       <c r="G18" t="n">
-        <v>76.69</v>
+        <v>77.31999999999999</v>
       </c>
       <c r="H18" t="n">
-        <v>73.89</v>
+        <v>74.33</v>
       </c>
       <c r="I18" t="n">
-        <v>76.34</v>
+        <v>77.03</v>
       </c>
       <c r="J18" t="n">
-        <v>3.87</v>
+        <v>4.27</v>
       </c>
       <c r="K18" t="n">
-        <v>4.12</v>
+        <v>4.39</v>
       </c>
       <c r="L18" t="n">
-        <v>3.75</v>
+        <v>3.99</v>
       </c>
       <c r="M18" t="n">
-        <v>4.07</v>
+        <v>4.08</v>
       </c>
       <c r="N18" t="n">
-        <v>38.93</v>
+        <v>38.49</v>
       </c>
       <c r="O18" t="n">
-        <v>39.47</v>
+        <v>39.14</v>
       </c>
       <c r="P18" t="n">
-        <v>37.93</v>
+        <v>37.64</v>
       </c>
       <c r="Q18" t="n">
-        <v>38.1</v>
+        <v>37.78</v>
       </c>
       <c r="R18" t="n">
-        <v>10.0847</v>
+        <v>-0.0987</v>
       </c>
       <c r="S18" t="n">
-        <v>-1.1302</v>
+        <v>16.3238</v>
       </c>
       <c r="T18" t="n">
-        <v>-11.5376</v>
+        <v>5.9459</v>
       </c>
       <c r="U18" t="n">
-        <v>4.978</v>
+        <v>0.9039</v>
       </c>
       <c r="V18" t="n">
-        <v>-0.1047</v>
+        <v>6.6454</v>
       </c>
       <c r="W18" t="n">
-        <v>-1.4459</v>
+        <v>5.017</v>
       </c>
       <c r="X18" t="n">
-        <v>-9.5556</v>
+        <v>0.2457</v>
       </c>
       <c r="Y18" t="n">
-        <v>-2.3981</v>
+        <v>-15</v>
       </c>
       <c r="Z18" t="n">
-        <v>5.4404</v>
+        <v>-9.5344</v>
       </c>
       <c r="AA18" t="n">
-        <v>-4.9401</v>
+        <v>-0.8399</v>
       </c>
       <c r="AB18" t="n">
-        <v>-0.4702</v>
+        <v>-6.4388</v>
       </c>
       <c r="AC18" t="n">
-        <v>0.5808</v>
+        <v>-5.4318</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>182.4</v>
+        <v>174.61</v>
       </c>
       <c r="C19" t="n">
-        <v>195.94</v>
+        <v>177.67</v>
       </c>
       <c r="D19" t="n">
-        <v>176.8</v>
+        <v>161.55</v>
       </c>
       <c r="E19" t="n">
-        <v>192.26</v>
+        <v>165.37</v>
       </c>
       <c r="F19" t="n">
-        <v>75.53</v>
+        <v>74.54000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>77.31999999999999</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>74.33</v>
+        <v>72.09</v>
       </c>
       <c r="I19" t="n">
-        <v>77.03</v>
+        <v>72.64</v>
       </c>
       <c r="J19" t="n">
-        <v>4.27</v>
+        <v>4.44</v>
       </c>
       <c r="K19" t="n">
-        <v>4.39</v>
+        <v>4.73</v>
       </c>
       <c r="L19" t="n">
-        <v>3.99</v>
+        <v>4.38</v>
       </c>
       <c r="M19" t="n">
-        <v>4.08</v>
+        <v>4.65</v>
       </c>
       <c r="N19" t="n">
-        <v>38.49</v>
+        <v>39.01</v>
       </c>
       <c r="O19" t="n">
-        <v>39.14</v>
+        <v>40.21</v>
       </c>
       <c r="P19" t="n">
-        <v>37.64</v>
+        <v>38.85</v>
       </c>
       <c r="Q19" t="n">
-        <v>37.78</v>
+        <v>39.95</v>
       </c>
       <c r="R19" t="n">
-        <v>-0.0987</v>
+        <v>-13.9863</v>
       </c>
       <c r="S19" t="n">
-        <v>16.3238</v>
+        <v>-5.4056</v>
       </c>
       <c r="T19" t="n">
-        <v>5.9459</v>
+        <v>-15.0424</v>
       </c>
       <c r="U19" t="n">
-        <v>0.9039</v>
+        <v>-5.6991</v>
       </c>
       <c r="V19" t="n">
-        <v>6.6454</v>
+        <v>-0.11</v>
       </c>
       <c r="W19" t="n">
-        <v>5.017</v>
+        <v>-4.9463</v>
       </c>
       <c r="X19" t="n">
-        <v>0.2457</v>
+        <v>13.9706</v>
       </c>
       <c r="Y19" t="n">
-        <v>-15</v>
+        <v>3.3333</v>
       </c>
       <c r="Z19" t="n">
-        <v>-9.5344</v>
+        <v>11.5108</v>
       </c>
       <c r="AA19" t="n">
-        <v>-0.8399</v>
+        <v>5.7438</v>
       </c>
       <c r="AB19" t="n">
-        <v>-6.4388</v>
+        <v>-0.3244</v>
       </c>
       <c r="AC19" t="n">
-        <v>-5.4318</v>
+        <v>4.3626</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>174.61</v>
+        <v>187.69</v>
       </c>
       <c r="C20" t="n">
-        <v>177.67</v>
+        <v>188.43</v>
       </c>
       <c r="D20" t="n">
-        <v>161.55</v>
+        <v>170.26</v>
       </c>
       <c r="E20" t="n">
-        <v>165.37</v>
+        <v>176.66</v>
       </c>
       <c r="F20" t="n">
-        <v>74.54000000000001</v>
+        <v>75.2</v>
       </c>
       <c r="G20" t="n">
-        <v>74.84999999999999</v>
+        <v>75.84999999999999</v>
       </c>
       <c r="H20" t="n">
-        <v>72.09</v>
+        <v>73.41</v>
       </c>
       <c r="I20" t="n">
-        <v>72.64</v>
+        <v>75.02</v>
       </c>
       <c r="J20" t="n">
-        <v>4.44</v>
+        <v>3.97</v>
       </c>
       <c r="K20" t="n">
-        <v>4.73</v>
+        <v>4.5</v>
       </c>
       <c r="L20" t="n">
-        <v>4.38</v>
+        <v>3.97</v>
       </c>
       <c r="M20" t="n">
-        <v>4.65</v>
+        <v>4.28</v>
       </c>
       <c r="N20" t="n">
-        <v>39.01</v>
+        <v>38.54</v>
       </c>
       <c r="O20" t="n">
-        <v>40.21</v>
+        <v>39.53</v>
       </c>
       <c r="P20" t="n">
-        <v>38.85</v>
+        <v>38.19</v>
       </c>
       <c r="Q20" t="n">
-        <v>39.95</v>
+        <v>38.63</v>
       </c>
       <c r="R20" t="n">
-        <v>-13.9863</v>
+        <v>6.8271</v>
       </c>
       <c r="S20" t="n">
-        <v>-5.4056</v>
+        <v>-8.204700000000001</v>
       </c>
       <c r="T20" t="n">
-        <v>-15.0424</v>
+        <v>6.8853</v>
       </c>
       <c r="U20" t="n">
-        <v>-5.6991</v>
+        <v>3.2764</v>
       </c>
       <c r="V20" t="n">
-        <v>-0.11</v>
+        <v>-1.7291</v>
       </c>
       <c r="W20" t="n">
-        <v>-4.9463</v>
+        <v>3.8627</v>
       </c>
       <c r="X20" t="n">
-        <v>13.9706</v>
+        <v>-7.957</v>
       </c>
       <c r="Y20" t="n">
-        <v>3.3333</v>
+        <v>5.1597</v>
       </c>
       <c r="Z20" t="n">
-        <v>11.5108</v>
+        <v>-10.8333</v>
       </c>
       <c r="AA20" t="n">
-        <v>5.7438</v>
+        <v>-3.3041</v>
       </c>
       <c r="AB20" t="n">
-        <v>-0.3244</v>
+        <v>1.3911</v>
       </c>
       <c r="AC20" t="n">
-        <v>4.3626</v>
+        <v>-4.3338</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>187.69</v>
+        <v>183.77</v>
       </c>
       <c r="C21" t="n">
-        <v>188.426</v>
+        <v>183.935</v>
       </c>
       <c r="D21" t="n">
-        <v>170.26</v>
+        <v>150</v>
       </c>
       <c r="E21" t="n">
-        <v>176.66</v>
+        <v>165.55</v>
       </c>
       <c r="F21" t="n">
-        <v>75.19</v>
+        <v>76.33</v>
       </c>
       <c r="G21" t="n">
-        <v>75.84</v>
+        <v>76.4699</v>
       </c>
       <c r="H21" t="n">
-        <v>73.41500000000001</v>
+        <v>72.06</v>
       </c>
       <c r="I21" t="n">
-        <v>75.02</v>
+        <v>74.44</v>
       </c>
       <c r="J21" t="n">
-        <v>3.97</v>
+        <v>41.23</v>
       </c>
       <c r="K21" t="n">
-        <v>4.5</v>
+        <v>49.69</v>
       </c>
       <c r="L21" t="n">
-        <v>3.9698</v>
+        <v>41.17</v>
       </c>
       <c r="M21" t="n">
-        <v>4.28</v>
+        <v>45.98</v>
       </c>
       <c r="N21" t="n">
-        <v>38.53</v>
+        <v>37.99</v>
       </c>
       <c r="O21" t="n">
-        <v>39.5299</v>
+        <v>40.1669</v>
       </c>
       <c r="P21" t="n">
-        <v>38.2</v>
+        <v>37.895</v>
       </c>
       <c r="Q21" t="n">
-        <v>38.63</v>
+        <v>38.94</v>
       </c>
       <c r="R21" t="n">
-        <v>6.8271</v>
+        <v>-6.2889</v>
       </c>
       <c r="S21" t="n">
-        <v>-8.204700000000001</v>
+        <v>-13.8926</v>
       </c>
       <c r="T21" t="n">
-        <v>6.8853</v>
+        <v>-5.3026</v>
       </c>
       <c r="U21" t="n">
-        <v>3.2764</v>
+        <v>-0.7731</v>
       </c>
       <c r="V21" t="n">
-        <v>-1.7291</v>
+        <v>-3.3623</v>
       </c>
       <c r="W21" t="n">
-        <v>3.8627</v>
+        <v>2.3652</v>
       </c>
       <c r="X21" t="n">
-        <v>-7.957</v>
+        <v>974.2991</v>
       </c>
       <c r="Y21" t="n">
-        <v>5.1597</v>
+        <v>1026.9608</v>
       </c>
       <c r="Z21" t="n">
-        <v>-10.8333</v>
+        <v>921.7778</v>
       </c>
       <c r="AA21" t="n">
-        <v>-3.3041</v>
+        <v>0.8025</v>
       </c>
       <c r="AB21" t="n">
-        <v>1.3911</v>
+        <v>3.0704</v>
       </c>
       <c r="AC21" t="n">
-        <v>-4.3338</v>
+        <v>-2.8443</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-07-16 22:56
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1713 +568,1713 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>267.13</v>
+        <v>247.42</v>
       </c>
       <c r="C2" t="n">
-        <v>274.93</v>
+        <v>259.79</v>
       </c>
       <c r="D2" t="n">
-        <v>226</v>
+        <v>233.3</v>
       </c>
       <c r="E2" t="n">
-        <v>226.19</v>
+        <v>233.86</v>
       </c>
       <c r="F2" t="n">
-        <v>83.9966</v>
+        <v>81.4824</v>
       </c>
       <c r="G2" t="n">
-        <v>84.63509999999999</v>
+        <v>81.6221</v>
       </c>
       <c r="H2" t="n">
-        <v>79.67659999999999</v>
+        <v>76.7633</v>
       </c>
       <c r="I2" t="n">
-        <v>79.74639999999999</v>
+        <v>77.36190000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>3.9836</v>
+        <v>41.2198</v>
       </c>
       <c r="K2" t="n">
-        <v>4.5965</v>
+        <v>44.0864</v>
       </c>
       <c r="L2" t="n">
-        <v>3.865</v>
+        <v>38.7486</v>
       </c>
       <c r="M2" t="n">
-        <v>4.5767</v>
+        <v>44.0864</v>
       </c>
       <c r="N2" t="n">
-        <v>35.9652</v>
+        <v>36.9397</v>
       </c>
       <c r="O2" t="n">
-        <v>37.7861</v>
+        <v>39.1641</v>
       </c>
       <c r="P2" t="n">
-        <v>35.6896</v>
+        <v>36.8708</v>
       </c>
       <c r="Q2" t="n">
-        <v>37.7468</v>
+        <v>38.8984</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>247.42</v>
+        <v>266.04</v>
       </c>
       <c r="C3" t="n">
-        <v>259.79</v>
+        <v>286.15</v>
       </c>
       <c r="D3" t="n">
-        <v>233.3</v>
+        <v>265</v>
       </c>
       <c r="E3" t="n">
-        <v>233.86</v>
+        <v>279.29</v>
       </c>
       <c r="F3" t="n">
-        <v>81.4824</v>
+        <v>81.9114</v>
       </c>
       <c r="G3" t="n">
-        <v>81.6221</v>
+        <v>83.408</v>
       </c>
       <c r="H3" t="n">
-        <v>76.7633</v>
+        <v>80.4448</v>
       </c>
       <c r="I3" t="n">
-        <v>77.36190000000001</v>
+        <v>82.67959999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>4.122</v>
+        <v>38.1555</v>
       </c>
       <c r="K3" t="n">
-        <v>4.4086</v>
+        <v>38.2544</v>
       </c>
       <c r="L3" t="n">
-        <v>3.8749</v>
+        <v>34.1027</v>
       </c>
       <c r="M3" t="n">
-        <v>4.4086</v>
+        <v>35.4866</v>
       </c>
       <c r="N3" t="n">
-        <v>36.9397</v>
+        <v>36.6149</v>
       </c>
       <c r="O3" t="n">
-        <v>39.1641</v>
+        <v>37.3531</v>
       </c>
       <c r="P3" t="n">
-        <v>36.8708</v>
+        <v>35.857</v>
       </c>
       <c r="Q3" t="n">
-        <v>38.8984</v>
+        <v>36.1719</v>
       </c>
       <c r="R3" t="n">
-        <v>3.391</v>
+        <v>19.4262</v>
       </c>
       <c r="U3" t="n">
-        <v>-2.9901</v>
+        <v>6.8738</v>
       </c>
       <c r="X3" t="n">
-        <v>-3.673</v>
+        <v>-19.5067</v>
       </c>
       <c r="AA3" t="n">
-        <v>3.0509</v>
+        <v>-7.0093</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>266.04</v>
+        <v>299.26</v>
       </c>
       <c r="C4" t="n">
-        <v>286.15</v>
+        <v>302</v>
       </c>
       <c r="D4" t="n">
-        <v>265</v>
+        <v>286.24</v>
       </c>
       <c r="E4" t="n">
-        <v>279.29</v>
+        <v>300.77</v>
       </c>
       <c r="F4" t="n">
-        <v>81.9114</v>
+        <v>83.7572</v>
       </c>
       <c r="G4" t="n">
-        <v>83.408</v>
+        <v>84.9145</v>
       </c>
       <c r="H4" t="n">
-        <v>80.4448</v>
+        <v>81.203</v>
       </c>
       <c r="I4" t="n">
-        <v>82.67959999999999</v>
+        <v>82.3903</v>
       </c>
       <c r="J4" t="n">
-        <v>3.8156</v>
+        <v>32.9165</v>
       </c>
       <c r="K4" t="n">
-        <v>3.8254</v>
+        <v>34.4981</v>
       </c>
       <c r="L4" t="n">
-        <v>3.4103</v>
+        <v>32.5212</v>
       </c>
       <c r="M4" t="n">
-        <v>3.5487</v>
+        <v>32.62</v>
       </c>
       <c r="N4" t="n">
-        <v>36.6149</v>
+        <v>35.7389</v>
       </c>
       <c r="O4" t="n">
-        <v>37.3531</v>
+        <v>36.8511</v>
       </c>
       <c r="P4" t="n">
-        <v>35.857</v>
+        <v>35.2369</v>
       </c>
       <c r="Q4" t="n">
-        <v>36.1719</v>
+        <v>36.3491</v>
       </c>
       <c r="R4" t="n">
-        <v>19.4262</v>
+        <v>7.6909</v>
       </c>
       <c r="U4" t="n">
-        <v>6.8738</v>
+        <v>-0.3499</v>
       </c>
       <c r="X4" t="n">
-        <v>-19.5051</v>
+        <v>-8.077999999999999</v>
       </c>
       <c r="AA4" t="n">
-        <v>-7.0093</v>
+        <v>0.4899</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>299.26</v>
+        <v>236</v>
       </c>
       <c r="C5" t="n">
-        <v>302</v>
+        <v>252.98</v>
       </c>
       <c r="D5" t="n">
-        <v>286.24</v>
+        <v>223</v>
       </c>
       <c r="E5" t="n">
-        <v>300.77</v>
+        <v>231.42</v>
       </c>
       <c r="F5" t="n">
-        <v>83.7572</v>
+        <v>74.9474</v>
       </c>
       <c r="G5" t="n">
-        <v>84.9145</v>
+        <v>77.56140000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>81.203</v>
+        <v>73.7402</v>
       </c>
       <c r="I5" t="n">
-        <v>82.3903</v>
+        <v>74.26900000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>3.2917</v>
+        <v>39.9</v>
       </c>
       <c r="K5" t="n">
-        <v>3.4498</v>
+        <v>41.3</v>
       </c>
       <c r="L5" t="n">
-        <v>3.2521</v>
+        <v>38</v>
       </c>
       <c r="M5" t="n">
-        <v>3.262</v>
+        <v>40.4</v>
       </c>
       <c r="N5" t="n">
-        <v>35.7389</v>
+        <v>39.6267</v>
       </c>
       <c r="O5" t="n">
-        <v>36.8511</v>
+        <v>40.1582</v>
       </c>
       <c r="P5" t="n">
-        <v>35.2369</v>
+        <v>38.4653</v>
       </c>
       <c r="Q5" t="n">
-        <v>36.3491</v>
+        <v>39.922</v>
       </c>
       <c r="R5" t="n">
-        <v>7.6909</v>
+        <v>-23.0575</v>
       </c>
       <c r="S5" t="n">
-        <v>32.9723</v>
+        <v>-1.0434</v>
       </c>
       <c r="U5" t="n">
-        <v>-0.3499</v>
+        <v>-9.857100000000001</v>
       </c>
       <c r="V5" t="n">
-        <v>3.3154</v>
+        <v>-3.998</v>
       </c>
       <c r="X5" t="n">
-        <v>-8.079000000000001</v>
+        <v>23.8504</v>
       </c>
       <c r="Y5" t="n">
-        <v>-28.7259</v>
+        <v>-8.361800000000001</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.4899</v>
+        <v>9.8294</v>
       </c>
       <c r="AB5" t="n">
-        <v>-3.7028</v>
+        <v>2.6315</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>236</v>
+        <v>233.11</v>
       </c>
       <c r="C6" t="n">
-        <v>252.98</v>
+        <v>237</v>
       </c>
       <c r="D6" t="n">
-        <v>223</v>
+        <v>211.13</v>
       </c>
       <c r="E6" t="n">
-        <v>231.42</v>
+        <v>229.57</v>
       </c>
       <c r="F6" t="n">
-        <v>74.9474</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>77.56140000000001</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>73.7402</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>74.26900000000001</v>
+        <v>73.3</v>
       </c>
       <c r="J6" t="n">
-        <v>3.99</v>
+        <v>40</v>
       </c>
       <c r="K6" t="n">
-        <v>4.13</v>
+        <v>43.9</v>
       </c>
       <c r="L6" t="n">
-        <v>3.8</v>
+        <v>39.2</v>
       </c>
       <c r="M6" t="n">
-        <v>4.04</v>
+        <v>40.8</v>
       </c>
       <c r="N6" t="n">
-        <v>39.6267</v>
+        <v>39.66</v>
       </c>
       <c r="O6" t="n">
-        <v>40.1582</v>
+        <v>41.49</v>
       </c>
       <c r="P6" t="n">
-        <v>38.4653</v>
+        <v>38.9</v>
       </c>
       <c r="Q6" t="n">
-        <v>39.922</v>
+        <v>40.45</v>
       </c>
       <c r="R6" t="n">
-        <v>-23.0575</v>
+        <v>-0.7994</v>
       </c>
       <c r="S6" t="n">
-        <v>-1.0434</v>
+        <v>-17.8023</v>
       </c>
       <c r="U6" t="n">
-        <v>-9.857100000000001</v>
+        <v>-1.3047</v>
       </c>
       <c r="V6" t="n">
-        <v>-3.998</v>
+        <v>-11.3445</v>
       </c>
       <c r="X6" t="n">
-        <v>23.8504</v>
+        <v>0.9901</v>
       </c>
       <c r="Y6" t="n">
-        <v>-8.360900000000001</v>
+        <v>14.973</v>
       </c>
       <c r="AA6" t="n">
-        <v>9.8294</v>
+        <v>1.3226</v>
       </c>
       <c r="AB6" t="n">
-        <v>2.6315</v>
+        <v>11.8271</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>233.11</v>
+        <v>268.05</v>
       </c>
       <c r="C7" t="n">
-        <v>237</v>
+        <v>268.4</v>
       </c>
       <c r="D7" t="n">
-        <v>211.13</v>
+        <v>225.74</v>
       </c>
       <c r="E7" t="n">
-        <v>229.57</v>
+        <v>252.61</v>
       </c>
       <c r="F7" t="n">
-        <v>74.79000000000001</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>76.18000000000001</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>71.34999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>73.3</v>
+        <v>74.95</v>
       </c>
       <c r="J7" t="n">
-        <v>4</v>
+        <v>33.8</v>
       </c>
       <c r="K7" t="n">
-        <v>4.39</v>
+        <v>41.5</v>
       </c>
       <c r="L7" t="n">
-        <v>3.92</v>
+        <v>33.7</v>
       </c>
       <c r="M7" t="n">
-        <v>4.08</v>
+        <v>36.3</v>
       </c>
       <c r="N7" t="n">
-        <v>39.66</v>
+        <v>37.87</v>
       </c>
       <c r="O7" t="n">
-        <v>41.49</v>
+        <v>41.37</v>
       </c>
       <c r="P7" t="n">
-        <v>38.9</v>
+        <v>37.71</v>
       </c>
       <c r="Q7" t="n">
-        <v>40.45</v>
+        <v>39.47</v>
       </c>
       <c r="R7" t="n">
-        <v>-0.7994</v>
+        <v>10.0362</v>
       </c>
       <c r="S7" t="n">
-        <v>-17.8023</v>
+        <v>-16.0122</v>
       </c>
       <c r="T7" t="n">
-        <v>1.4943</v>
+        <v>8.0176</v>
       </c>
       <c r="U7" t="n">
-        <v>-1.3047</v>
+        <v>2.251</v>
       </c>
       <c r="V7" t="n">
-        <v>-11.3445</v>
+        <v>-9.0306</v>
       </c>
       <c r="W7" t="n">
-        <v>-8.083600000000001</v>
+        <v>-3.1177</v>
       </c>
       <c r="X7" t="n">
-        <v>0.9901</v>
+        <v>-11.0294</v>
       </c>
       <c r="Y7" t="n">
-        <v>14.9717</v>
+        <v>11.2814</v>
       </c>
       <c r="Z7" t="n">
-        <v>-10.8528</v>
+        <v>-17.6617</v>
       </c>
       <c r="AA7" t="n">
-        <v>1.3226</v>
+        <v>-2.4227</v>
       </c>
       <c r="AB7" t="n">
-        <v>11.8271</v>
+        <v>8.585900000000001</v>
       </c>
       <c r="AC7" t="n">
-        <v>7.1614</v>
+        <v>1.4695</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>268.05</v>
+        <v>226.24</v>
       </c>
       <c r="C8" t="n">
-        <v>268.4</v>
+        <v>231.25</v>
       </c>
       <c r="D8" t="n">
-        <v>225.74</v>
+        <v>212.1</v>
       </c>
       <c r="E8" t="n">
-        <v>252.61</v>
+        <v>215.6</v>
       </c>
       <c r="F8" t="n">
-        <v>77.95999999999999</v>
+        <v>72.09</v>
       </c>
       <c r="G8" t="n">
-        <v>78.23999999999999</v>
+        <v>74.69</v>
       </c>
       <c r="H8" t="n">
-        <v>71.59999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="I8" t="n">
-        <v>74.95</v>
+        <v>71.83</v>
       </c>
       <c r="J8" t="n">
-        <v>3.38</v>
+        <v>40.4</v>
       </c>
       <c r="K8" t="n">
-        <v>4.15</v>
+        <v>42.5</v>
       </c>
       <c r="L8" t="n">
-        <v>3.37</v>
+        <v>39.5</v>
       </c>
       <c r="M8" t="n">
-        <v>3.63</v>
+        <v>42.4</v>
       </c>
       <c r="N8" t="n">
-        <v>37.87</v>
+        <v>41.08</v>
       </c>
       <c r="O8" t="n">
-        <v>41.37</v>
+        <v>41.79</v>
       </c>
       <c r="P8" t="n">
-        <v>37.71</v>
+        <v>39.69</v>
       </c>
       <c r="Q8" t="n">
-        <v>39.47</v>
+        <v>41.31</v>
       </c>
       <c r="R8" t="n">
-        <v>10.0362</v>
+        <v>-14.651</v>
       </c>
       <c r="S8" t="n">
-        <v>-16.0122</v>
+        <v>-6.8361</v>
       </c>
       <c r="T8" t="n">
-        <v>8.0176</v>
+        <v>-22.8043</v>
       </c>
       <c r="U8" t="n">
-        <v>2.251</v>
+        <v>-4.1628</v>
       </c>
       <c r="V8" t="n">
-        <v>-9.0306</v>
+        <v>-3.284</v>
       </c>
       <c r="W8" t="n">
-        <v>-3.1177</v>
+        <v>-13.1225</v>
       </c>
       <c r="X8" t="n">
-        <v>-11.0294</v>
+        <v>16.8044</v>
       </c>
       <c r="Y8" t="n">
-        <v>11.2814</v>
+        <v>4.9505</v>
       </c>
       <c r="Z8" t="n">
-        <v>-17.6609</v>
+        <v>19.4817</v>
       </c>
       <c r="AA8" t="n">
-        <v>-2.4227</v>
+        <v>4.6618</v>
       </c>
       <c r="AB8" t="n">
-        <v>8.585900000000001</v>
+        <v>3.4768</v>
       </c>
       <c r="AC8" t="n">
-        <v>1.4695</v>
+        <v>14.2047</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>226.24</v>
+        <v>216.36</v>
       </c>
       <c r="C9" t="n">
-        <v>231.25</v>
+        <v>238.65</v>
       </c>
       <c r="D9" t="n">
-        <v>212.1</v>
+        <v>192.3</v>
       </c>
       <c r="E9" t="n">
-        <v>215.6</v>
+        <v>236.52</v>
       </c>
       <c r="F9" t="n">
-        <v>72.09</v>
+        <v>74.12</v>
       </c>
       <c r="G9" t="n">
-        <v>74.69</v>
+        <v>77.38</v>
       </c>
       <c r="H9" t="n">
-        <v>70.72</v>
+        <v>71.45</v>
       </c>
       <c r="I9" t="n">
-        <v>71.83</v>
+        <v>77.19</v>
       </c>
       <c r="J9" t="n">
-        <v>4.04</v>
+        <v>41.6</v>
       </c>
       <c r="K9" t="n">
-        <v>4.25</v>
+        <v>46.3</v>
       </c>
       <c r="L9" t="n">
-        <v>3.95</v>
+        <v>37</v>
       </c>
       <c r="M9" t="n">
-        <v>4.24</v>
+        <v>37.2</v>
       </c>
       <c r="N9" t="n">
-        <v>41.08</v>
+        <v>39.91</v>
       </c>
       <c r="O9" t="n">
-        <v>41.79</v>
+        <v>41.43</v>
       </c>
       <c r="P9" t="n">
-        <v>39.69</v>
+        <v>38.08</v>
       </c>
       <c r="Q9" t="n">
-        <v>41.31</v>
+        <v>38.16</v>
       </c>
       <c r="R9" t="n">
-        <v>-14.651</v>
+        <v>9.703200000000001</v>
       </c>
       <c r="S9" t="n">
-        <v>-6.8361</v>
+        <v>3.0274</v>
       </c>
       <c r="T9" t="n">
-        <v>-22.8043</v>
+        <v>-21.3618</v>
       </c>
       <c r="U9" t="n">
-        <v>-4.1628</v>
+        <v>7.4621</v>
       </c>
       <c r="V9" t="n">
-        <v>-3.284</v>
+        <v>5.307</v>
       </c>
       <c r="W9" t="n">
-        <v>-13.1225</v>
+        <v>-6.3118</v>
       </c>
       <c r="X9" t="n">
-        <v>16.8044</v>
+        <v>-12.2642</v>
       </c>
       <c r="Y9" t="n">
-        <v>4.9505</v>
+        <v>-8.823499999999999</v>
       </c>
       <c r="Z9" t="n">
-        <v>19.4804</v>
+        <v>14.0405</v>
       </c>
       <c r="AA9" t="n">
-        <v>4.6618</v>
+        <v>-7.6253</v>
       </c>
       <c r="AB9" t="n">
-        <v>3.4768</v>
+        <v>-5.6613</v>
       </c>
       <c r="AC9" t="n">
-        <v>14.2047</v>
+        <v>4.982</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>216.36</v>
+        <v>241.45</v>
       </c>
       <c r="C10" t="n">
-        <v>238.65</v>
+        <v>272</v>
       </c>
       <c r="D10" t="n">
-        <v>192.3</v>
+        <v>240.59</v>
       </c>
       <c r="E10" t="n">
-        <v>236.52</v>
+        <v>266.71</v>
       </c>
       <c r="F10" t="n">
-        <v>74.12</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="G10" t="n">
-        <v>77.38</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>71.45</v>
+        <v>77.15000000000001</v>
       </c>
       <c r="I10" t="n">
-        <v>77.19</v>
+        <v>81</v>
       </c>
       <c r="J10" t="n">
-        <v>4.16</v>
+        <v>36.6</v>
       </c>
       <c r="K10" t="n">
-        <v>4.63</v>
+        <v>36.8</v>
       </c>
       <c r="L10" t="n">
-        <v>3.7</v>
+        <v>31.7</v>
       </c>
       <c r="M10" t="n">
-        <v>3.72</v>
+        <v>32.4</v>
       </c>
       <c r="N10" t="n">
-        <v>39.91</v>
+        <v>38.16</v>
       </c>
       <c r="O10" t="n">
-        <v>41.43</v>
+        <v>38.2</v>
       </c>
       <c r="P10" t="n">
-        <v>38.08</v>
+        <v>36.03</v>
       </c>
       <c r="Q10" t="n">
-        <v>38.16</v>
+        <v>36.31</v>
       </c>
       <c r="R10" t="n">
-        <v>9.703200000000001</v>
+        <v>12.7642</v>
       </c>
       <c r="S10" t="n">
-        <v>3.0274</v>
+        <v>5.5817</v>
       </c>
       <c r="T10" t="n">
-        <v>-21.3618</v>
+        <v>15.2493</v>
       </c>
       <c r="U10" t="n">
-        <v>7.4621</v>
+        <v>4.9359</v>
       </c>
       <c r="V10" t="n">
-        <v>5.307</v>
+        <v>8.071999999999999</v>
       </c>
       <c r="W10" t="n">
-        <v>-6.3118</v>
+        <v>9.063000000000001</v>
       </c>
       <c r="X10" t="n">
-        <v>-12.2642</v>
+        <v>-12.9032</v>
       </c>
       <c r="Y10" t="n">
-        <v>-8.823499999999999</v>
+        <v>-10.7438</v>
       </c>
       <c r="Z10" t="n">
-        <v>14.0405</v>
+        <v>-19.802</v>
       </c>
       <c r="AA10" t="n">
-        <v>-7.6253</v>
+        <v>-4.848</v>
       </c>
       <c r="AB10" t="n">
-        <v>-5.6613</v>
+        <v>-8.0061</v>
       </c>
       <c r="AC10" t="n">
-        <v>4.982</v>
+        <v>-9.047599999999999</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>241.45</v>
+        <v>237.79</v>
       </c>
       <c r="C11" t="n">
-        <v>272</v>
+        <v>246.47</v>
       </c>
       <c r="D11" t="n">
-        <v>240.59</v>
+        <v>215.38</v>
       </c>
       <c r="E11" t="n">
-        <v>266.71</v>
+        <v>217.55</v>
       </c>
       <c r="F11" t="n">
-        <v>77.23999999999999</v>
+        <v>78.72</v>
       </c>
       <c r="G11" t="n">
-        <v>81.54000000000001</v>
+        <v>79.64</v>
       </c>
       <c r="H11" t="n">
-        <v>77.15000000000001</v>
+        <v>77.23</v>
       </c>
       <c r="I11" t="n">
-        <v>81</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>3.66</v>
+        <v>35.9</v>
       </c>
       <c r="K11" t="n">
-        <v>3.68</v>
+        <v>38.9</v>
       </c>
       <c r="L11" t="n">
-        <v>3.17</v>
+        <v>35.1</v>
       </c>
       <c r="M11" t="n">
-        <v>3.24</v>
+        <v>38.6</v>
       </c>
       <c r="N11" t="n">
-        <v>38.16</v>
+        <v>37.31</v>
       </c>
       <c r="O11" t="n">
-        <v>38.2</v>
+        <v>37.98</v>
       </c>
       <c r="P11" t="n">
-        <v>36.03</v>
+        <v>36.9</v>
       </c>
       <c r="Q11" t="n">
-        <v>36.31</v>
+        <v>37.88</v>
       </c>
       <c r="R11" t="n">
-        <v>12.7642</v>
+        <v>-18.432</v>
       </c>
       <c r="S11" t="n">
-        <v>5.5817</v>
+        <v>0.9045</v>
       </c>
       <c r="T11" t="n">
-        <v>15.2493</v>
+        <v>-5.2359</v>
       </c>
       <c r="U11" t="n">
-        <v>4.9359</v>
+        <v>-4.3704</v>
       </c>
       <c r="V11" t="n">
-        <v>8.071999999999999</v>
+        <v>7.838</v>
       </c>
       <c r="W11" t="n">
-        <v>9.063000000000001</v>
+        <v>5.6753</v>
       </c>
       <c r="X11" t="n">
-        <v>-12.9032</v>
+        <v>19.1358</v>
       </c>
       <c r="Y11" t="n">
-        <v>-10.7438</v>
+        <v>-8.962300000000001</v>
       </c>
       <c r="Z11" t="n">
-        <v>-19.802</v>
+        <v>-5.3922</v>
       </c>
       <c r="AA11" t="n">
-        <v>-4.848</v>
+        <v>4.3239</v>
       </c>
       <c r="AB11" t="n">
-        <v>-8.0061</v>
+        <v>-8.303100000000001</v>
       </c>
       <c r="AC11" t="n">
-        <v>-9.047599999999999</v>
+        <v>-6.3535</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>237.79</v>
+        <v>219.23</v>
       </c>
       <c r="C12" t="n">
-        <v>246.47</v>
+        <v>226.13</v>
       </c>
       <c r="D12" t="n">
-        <v>215.38</v>
+        <v>168.88</v>
       </c>
       <c r="E12" t="n">
-        <v>217.55</v>
+        <v>181.47</v>
       </c>
       <c r="F12" t="n">
-        <v>78.72</v>
+        <v>77.45</v>
       </c>
       <c r="G12" t="n">
-        <v>79.64</v>
+        <v>79.14</v>
       </c>
       <c r="H12" t="n">
-        <v>77.23</v>
+        <v>71.72</v>
       </c>
       <c r="I12" t="n">
-        <v>77.45999999999999</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>3.59</v>
+        <v>38.4</v>
       </c>
       <c r="K12" t="n">
-        <v>3.89</v>
+        <v>47.4</v>
       </c>
       <c r="L12" t="n">
-        <v>3.51</v>
+        <v>37.1</v>
       </c>
       <c r="M12" t="n">
-        <v>3.86</v>
+        <v>45.1</v>
       </c>
       <c r="N12" t="n">
-        <v>37.31</v>
+        <v>37.91</v>
       </c>
       <c r="O12" t="n">
-        <v>37.98</v>
+        <v>40.72</v>
       </c>
       <c r="P12" t="n">
-        <v>36.9</v>
+        <v>37.08</v>
       </c>
       <c r="Q12" t="n">
-        <v>37.88</v>
+        <v>39.95</v>
       </c>
       <c r="R12" t="n">
-        <v>-18.432</v>
+        <v>-16.5847</v>
       </c>
       <c r="S12" t="n">
-        <v>0.9045</v>
+        <v>-23.275</v>
       </c>
       <c r="T12" t="n">
-        <v>-5.2359</v>
+        <v>-28.162</v>
       </c>
       <c r="U12" t="n">
-        <v>-4.3704</v>
+        <v>-5.306</v>
       </c>
       <c r="V12" t="n">
-        <v>7.838</v>
+        <v>-4.9747</v>
       </c>
       <c r="W12" t="n">
-        <v>5.6753</v>
+        <v>-2.1348</v>
       </c>
       <c r="X12" t="n">
-        <v>19.1358</v>
+        <v>16.8394</v>
       </c>
       <c r="Y12" t="n">
-        <v>-8.962300000000001</v>
+        <v>21.2366</v>
       </c>
       <c r="Z12" t="n">
-        <v>-5.3922</v>
+        <v>24.2424</v>
       </c>
       <c r="AA12" t="n">
-        <v>4.3239</v>
+        <v>5.4646</v>
       </c>
       <c r="AB12" t="n">
-        <v>-8.303100000000001</v>
+        <v>4.6908</v>
       </c>
       <c r="AC12" t="n">
-        <v>-6.3535</v>
+        <v>1.2161</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>219.23</v>
+        <v>197.21</v>
       </c>
       <c r="C13" t="n">
-        <v>226.13</v>
+        <v>210.8</v>
       </c>
       <c r="D13" t="n">
-        <v>168.88</v>
+        <v>194.22</v>
       </c>
       <c r="E13" t="n">
-        <v>181.47</v>
+        <v>194.65</v>
       </c>
       <c r="F13" t="n">
+        <v>75.54000000000001</v>
+      </c>
+      <c r="G13" t="n">
         <v>77.45</v>
       </c>
-      <c r="G13" t="n">
-        <v>79.14</v>
-      </c>
       <c r="H13" t="n">
-        <v>71.72</v>
+        <v>75.11</v>
       </c>
       <c r="I13" t="n">
-        <v>73.34999999999999</v>
+        <v>76.42</v>
       </c>
       <c r="J13" t="n">
-        <v>3.84</v>
+        <v>41.1</v>
       </c>
       <c r="K13" t="n">
-        <v>4.74</v>
+        <v>41.8</v>
       </c>
       <c r="L13" t="n">
-        <v>3.71</v>
+        <v>37.7</v>
       </c>
       <c r="M13" t="n">
-        <v>4.51</v>
+        <v>41.7</v>
       </c>
       <c r="N13" t="n">
-        <v>37.91</v>
+        <v>38.75</v>
       </c>
       <c r="O13" t="n">
-        <v>40.72</v>
+        <v>38.98</v>
       </c>
       <c r="P13" t="n">
-        <v>37.08</v>
+        <v>37.71</v>
       </c>
       <c r="Q13" t="n">
-        <v>39.95</v>
+        <v>38.28</v>
       </c>
       <c r="R13" t="n">
-        <v>-16.5847</v>
+        <v>7.2629</v>
       </c>
       <c r="S13" t="n">
-        <v>-23.275</v>
+        <v>-27.0181</v>
       </c>
       <c r="T13" t="n">
-        <v>-28.162</v>
+        <v>-9.7171</v>
       </c>
       <c r="U13" t="n">
-        <v>-5.306</v>
+        <v>4.1854</v>
       </c>
       <c r="V13" t="n">
-        <v>-4.9747</v>
+        <v>-5.6543</v>
       </c>
       <c r="W13" t="n">
-        <v>-2.1348</v>
+        <v>6.3901</v>
       </c>
       <c r="X13" t="n">
-        <v>16.8394</v>
+        <v>-7.5388</v>
       </c>
       <c r="Y13" t="n">
-        <v>21.2366</v>
+        <v>28.7037</v>
       </c>
       <c r="Z13" t="n">
-        <v>24.2424</v>
+        <v>-1.6509</v>
       </c>
       <c r="AA13" t="n">
-        <v>5.4646</v>
+        <v>-4.1802</v>
       </c>
       <c r="AB13" t="n">
-        <v>4.6908</v>
+        <v>5.4255</v>
       </c>
       <c r="AC13" t="n">
-        <v>1.2161</v>
+        <v>-7.3348</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>197.21</v>
+        <v>165.4</v>
       </c>
       <c r="C14" t="n">
-        <v>210.8</v>
+        <v>171.88</v>
       </c>
       <c r="D14" t="n">
-        <v>194.22</v>
+        <v>150.08</v>
       </c>
       <c r="E14" t="n">
-        <v>194.65</v>
+        <v>165.28</v>
       </c>
       <c r="F14" t="n">
-        <v>75.54000000000001</v>
+        <v>73.7</v>
       </c>
       <c r="G14" t="n">
-        <v>77.45</v>
+        <v>74.39</v>
       </c>
       <c r="H14" t="n">
-        <v>75.11</v>
+        <v>70.76000000000001</v>
       </c>
       <c r="I14" t="n">
-        <v>76.42</v>
+        <v>72.23</v>
       </c>
       <c r="J14" t="n">
-        <v>4.11</v>
+        <v>48</v>
       </c>
       <c r="K14" t="n">
-        <v>4.18</v>
+        <v>51.4</v>
       </c>
       <c r="L14" t="n">
-        <v>3.77</v>
+        <v>46.6</v>
       </c>
       <c r="M14" t="n">
-        <v>4.17</v>
+        <v>48</v>
       </c>
       <c r="N14" t="n">
-        <v>38.75</v>
+        <v>39.64</v>
       </c>
       <c r="O14" t="n">
-        <v>38.98</v>
+        <v>41.11</v>
       </c>
       <c r="P14" t="n">
-        <v>37.71</v>
+        <v>39.29</v>
       </c>
       <c r="Q14" t="n">
-        <v>38.28</v>
+        <v>40.38</v>
       </c>
       <c r="R14" t="n">
-        <v>7.2629</v>
+        <v>-15.0886</v>
       </c>
       <c r="S14" t="n">
-        <v>-27.0181</v>
+        <v>-24.0267</v>
       </c>
       <c r="T14" t="n">
-        <v>-9.7171</v>
+        <v>-30.1201</v>
       </c>
       <c r="U14" t="n">
-        <v>4.1854</v>
+        <v>-5.4829</v>
       </c>
       <c r="V14" t="n">
-        <v>-5.6543</v>
+        <v>-6.7519</v>
       </c>
       <c r="W14" t="n">
-        <v>6.3901</v>
+        <v>-6.4257</v>
       </c>
       <c r="X14" t="n">
-        <v>-7.5388</v>
+        <v>15.1079</v>
       </c>
       <c r="Y14" t="n">
-        <v>28.7037</v>
+        <v>24.3523</v>
       </c>
       <c r="Z14" t="n">
-        <v>-1.6509</v>
+        <v>29.0323</v>
       </c>
       <c r="AA14" t="n">
-        <v>-4.1802</v>
+        <v>5.4859</v>
       </c>
       <c r="AB14" t="n">
-        <v>5.4255</v>
+        <v>6.5998</v>
       </c>
       <c r="AC14" t="n">
-        <v>-7.3348</v>
+        <v>5.8176</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>165.4</v>
+        <v>159.21</v>
       </c>
       <c r="C15" t="n">
-        <v>171.88</v>
+        <v>176.75</v>
       </c>
       <c r="D15" t="n">
-        <v>150.08</v>
+        <v>158.87</v>
       </c>
       <c r="E15" t="n">
-        <v>165.28</v>
+        <v>174.82</v>
       </c>
       <c r="F15" t="n">
-        <v>73.7</v>
+        <v>70.8</v>
       </c>
       <c r="G15" t="n">
-        <v>74.39</v>
+        <v>73.02</v>
       </c>
       <c r="H15" t="n">
-        <v>70.76000000000001</v>
+        <v>69.56999999999999</v>
       </c>
       <c r="I15" t="n">
-        <v>72.23</v>
+        <v>72.72</v>
       </c>
       <c r="J15" t="n">
-        <v>4.8</v>
+        <v>49.8</v>
       </c>
       <c r="K15" t="n">
-        <v>5.14</v>
+        <v>49.9</v>
       </c>
       <c r="L15" t="n">
-        <v>4.66</v>
+        <v>44.6</v>
       </c>
       <c r="M15" t="n">
-        <v>4.8</v>
+        <v>45</v>
       </c>
       <c r="N15" t="n">
-        <v>39.64</v>
+        <v>41.18</v>
       </c>
       <c r="O15" t="n">
-        <v>41.11</v>
+        <v>41.86</v>
       </c>
       <c r="P15" t="n">
-        <v>39.29</v>
+        <v>39.93</v>
       </c>
       <c r="Q15" t="n">
-        <v>40.38</v>
+        <v>40.08</v>
       </c>
       <c r="R15" t="n">
-        <v>-15.0886</v>
+        <v>5.772</v>
       </c>
       <c r="S15" t="n">
-        <v>-24.0267</v>
+        <v>-3.6645</v>
       </c>
       <c r="T15" t="n">
-        <v>-30.1201</v>
+        <v>-34.4532</v>
       </c>
       <c r="U15" t="n">
-        <v>-5.4829</v>
+        <v>0.6784</v>
       </c>
       <c r="V15" t="n">
-        <v>-6.7519</v>
+        <v>-0.8589</v>
       </c>
       <c r="W15" t="n">
-        <v>-6.4257</v>
+        <v>-10.2222</v>
       </c>
       <c r="X15" t="n">
-        <v>15.1079</v>
+        <v>-6.25</v>
       </c>
       <c r="Y15" t="n">
-        <v>24.3523</v>
+        <v>-0.2217</v>
       </c>
       <c r="Z15" t="n">
-        <v>29.0323</v>
+        <v>38.8889</v>
       </c>
       <c r="AA15" t="n">
-        <v>5.4859</v>
+        <v>-0.7429</v>
       </c>
       <c r="AB15" t="n">
-        <v>6.5998</v>
+        <v>0.3254</v>
       </c>
       <c r="AC15" t="n">
-        <v>5.8176</v>
+        <v>10.3828</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>159.21</v>
+        <v>199.81</v>
       </c>
       <c r="C16" t="n">
-        <v>176.75</v>
+        <v>204.55</v>
       </c>
       <c r="D16" t="n">
-        <v>158.87</v>
+        <v>189.46</v>
       </c>
       <c r="E16" t="n">
-        <v>174.82</v>
+        <v>192.45</v>
       </c>
       <c r="F16" t="n">
-        <v>70.8</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>73.02</v>
+        <v>76.69</v>
       </c>
       <c r="H16" t="n">
-        <v>69.56999999999999</v>
+        <v>73.89</v>
       </c>
       <c r="I16" t="n">
-        <v>72.72</v>
+        <v>76.34</v>
       </c>
       <c r="J16" t="n">
-        <v>4.98</v>
+        <v>38.7</v>
       </c>
       <c r="K16" t="n">
-        <v>4.99</v>
+        <v>41.2</v>
       </c>
       <c r="L16" t="n">
-        <v>4.46</v>
+        <v>37.5</v>
       </c>
       <c r="M16" t="n">
-        <v>4.5</v>
+        <v>40.7</v>
       </c>
       <c r="N16" t="n">
-        <v>41.18</v>
+        <v>38.93</v>
       </c>
       <c r="O16" t="n">
-        <v>41.86</v>
+        <v>39.47</v>
       </c>
       <c r="P16" t="n">
-        <v>39.93</v>
+        <v>37.93</v>
       </c>
       <c r="Q16" t="n">
-        <v>40.08</v>
+        <v>38.1</v>
       </c>
       <c r="R16" t="n">
-        <v>5.772</v>
+        <v>10.0847</v>
       </c>
       <c r="S16" t="n">
-        <v>-3.6645</v>
+        <v>-1.1302</v>
       </c>
       <c r="T16" t="n">
-        <v>-34.4532</v>
+        <v>-11.5376</v>
       </c>
       <c r="U16" t="n">
-        <v>0.6784</v>
+        <v>4.978</v>
       </c>
       <c r="V16" t="n">
-        <v>-0.8589</v>
+        <v>-0.1047</v>
       </c>
       <c r="W16" t="n">
-        <v>-10.2222</v>
+        <v>-1.4459</v>
       </c>
       <c r="X16" t="n">
-        <v>-6.25</v>
+        <v>-9.5556</v>
       </c>
       <c r="Y16" t="n">
-        <v>-0.2217</v>
+        <v>-2.3981</v>
       </c>
       <c r="Z16" t="n">
-        <v>38.8889</v>
+        <v>5.4404</v>
       </c>
       <c r="AA16" t="n">
-        <v>-0.7429</v>
+        <v>-4.9401</v>
       </c>
       <c r="AB16" t="n">
-        <v>0.3254</v>
+        <v>-0.4702</v>
       </c>
       <c r="AC16" t="n">
-        <v>10.3828</v>
+        <v>0.5808</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>199.81</v>
+        <v>182.4</v>
       </c>
       <c r="C17" t="n">
-        <v>204.55</v>
+        <v>195.94</v>
       </c>
       <c r="D17" t="n">
-        <v>189.46</v>
+        <v>176.8</v>
       </c>
       <c r="E17" t="n">
-        <v>192.45</v>
+        <v>192.26</v>
       </c>
       <c r="F17" t="n">
-        <v>74.84999999999999</v>
+        <v>75.53</v>
       </c>
       <c r="G17" t="n">
-        <v>76.69</v>
+        <v>77.31999999999999</v>
       </c>
       <c r="H17" t="n">
-        <v>73.89</v>
+        <v>74.33</v>
       </c>
       <c r="I17" t="n">
-        <v>76.34</v>
+        <v>77.03</v>
       </c>
       <c r="J17" t="n">
-        <v>3.87</v>
+        <v>42.7</v>
       </c>
       <c r="K17" t="n">
-        <v>4.12</v>
+        <v>43.9</v>
       </c>
       <c r="L17" t="n">
-        <v>3.75</v>
+        <v>39.9</v>
       </c>
       <c r="M17" t="n">
-        <v>4.07</v>
+        <v>40.8</v>
       </c>
       <c r="N17" t="n">
-        <v>38.93</v>
+        <v>38.49</v>
       </c>
       <c r="O17" t="n">
-        <v>39.47</v>
+        <v>39.14</v>
       </c>
       <c r="P17" t="n">
-        <v>37.93</v>
+        <v>37.64</v>
       </c>
       <c r="Q17" t="n">
-        <v>38.1</v>
+        <v>37.78</v>
       </c>
       <c r="R17" t="n">
-        <v>10.0847</v>
+        <v>-0.0987</v>
       </c>
       <c r="S17" t="n">
-        <v>-1.1302</v>
+        <v>16.3238</v>
       </c>
       <c r="T17" t="n">
-        <v>-11.5376</v>
+        <v>5.9459</v>
       </c>
       <c r="U17" t="n">
-        <v>4.978</v>
+        <v>0.9039</v>
       </c>
       <c r="V17" t="n">
-        <v>-0.1047</v>
+        <v>6.6454</v>
       </c>
       <c r="W17" t="n">
-        <v>-1.4459</v>
+        <v>5.017</v>
       </c>
       <c r="X17" t="n">
-        <v>-9.5556</v>
+        <v>0.2457</v>
       </c>
       <c r="Y17" t="n">
-        <v>-2.3981</v>
+        <v>-15</v>
       </c>
       <c r="Z17" t="n">
-        <v>5.4404</v>
+        <v>-9.5344</v>
       </c>
       <c r="AA17" t="n">
-        <v>-4.9401</v>
+        <v>-0.8399</v>
       </c>
       <c r="AB17" t="n">
-        <v>-0.4702</v>
+        <v>-6.4388</v>
       </c>
       <c r="AC17" t="n">
-        <v>0.5808</v>
+        <v>-5.4318</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>182.4</v>
+        <v>174.61</v>
       </c>
       <c r="C18" t="n">
-        <v>195.94</v>
+        <v>177.67</v>
       </c>
       <c r="D18" t="n">
-        <v>176.8</v>
+        <v>161.55</v>
       </c>
       <c r="E18" t="n">
-        <v>192.26</v>
+        <v>165.37</v>
       </c>
       <c r="F18" t="n">
-        <v>75.53</v>
+        <v>74.54000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>77.31999999999999</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="H18" t="n">
-        <v>74.33</v>
+        <v>72.09</v>
       </c>
       <c r="I18" t="n">
-        <v>77.03</v>
+        <v>72.64</v>
       </c>
       <c r="J18" t="n">
-        <v>4.27</v>
+        <v>44.4</v>
       </c>
       <c r="K18" t="n">
-        <v>4.39</v>
+        <v>47.3</v>
       </c>
       <c r="L18" t="n">
-        <v>3.99</v>
+        <v>43.8</v>
       </c>
       <c r="M18" t="n">
-        <v>4.08</v>
+        <v>46.5</v>
       </c>
       <c r="N18" t="n">
-        <v>38.49</v>
+        <v>39.01</v>
       </c>
       <c r="O18" t="n">
-        <v>39.14</v>
+        <v>40.21</v>
       </c>
       <c r="P18" t="n">
-        <v>37.64</v>
+        <v>38.85</v>
       </c>
       <c r="Q18" t="n">
-        <v>37.78</v>
+        <v>39.95</v>
       </c>
       <c r="R18" t="n">
-        <v>-0.0987</v>
+        <v>-13.9863</v>
       </c>
       <c r="S18" t="n">
-        <v>16.3238</v>
+        <v>-5.4056</v>
       </c>
       <c r="T18" t="n">
-        <v>5.9459</v>
+        <v>-15.0424</v>
       </c>
       <c r="U18" t="n">
-        <v>0.9039</v>
+        <v>-5.6991</v>
       </c>
       <c r="V18" t="n">
-        <v>6.6454</v>
+        <v>-0.11</v>
       </c>
       <c r="W18" t="n">
-        <v>5.017</v>
+        <v>-4.9463</v>
       </c>
       <c r="X18" t="n">
-        <v>0.2457</v>
+        <v>13.9706</v>
       </c>
       <c r="Y18" t="n">
-        <v>-15</v>
+        <v>3.3333</v>
       </c>
       <c r="Z18" t="n">
-        <v>-9.5344</v>
+        <v>11.5108</v>
       </c>
       <c r="AA18" t="n">
-        <v>-0.8399</v>
+        <v>5.7438</v>
       </c>
       <c r="AB18" t="n">
-        <v>-6.4388</v>
+        <v>-0.3244</v>
       </c>
       <c r="AC18" t="n">
-        <v>-5.4318</v>
+        <v>4.3626</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>174.61</v>
+        <v>187.69</v>
       </c>
       <c r="C19" t="n">
-        <v>177.67</v>
+        <v>188.43</v>
       </c>
       <c r="D19" t="n">
-        <v>161.55</v>
+        <v>170.26</v>
       </c>
       <c r="E19" t="n">
-        <v>165.37</v>
+        <v>176.66</v>
       </c>
       <c r="F19" t="n">
-        <v>74.54000000000001</v>
+        <v>75.2</v>
       </c>
       <c r="G19" t="n">
-        <v>74.84999999999999</v>
+        <v>75.84999999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>72.09</v>
+        <v>73.41</v>
       </c>
       <c r="I19" t="n">
-        <v>72.64</v>
+        <v>75.02</v>
       </c>
       <c r="J19" t="n">
-        <v>4.44</v>
+        <v>39.7</v>
       </c>
       <c r="K19" t="n">
-        <v>4.73</v>
+        <v>45</v>
       </c>
       <c r="L19" t="n">
-        <v>4.38</v>
+        <v>39.7</v>
       </c>
       <c r="M19" t="n">
-        <v>4.65</v>
+        <v>42.8</v>
       </c>
       <c r="N19" t="n">
-        <v>39.01</v>
+        <v>38.54</v>
       </c>
       <c r="O19" t="n">
-        <v>40.21</v>
+        <v>39.53</v>
       </c>
       <c r="P19" t="n">
-        <v>38.85</v>
+        <v>38.19</v>
       </c>
       <c r="Q19" t="n">
-        <v>39.95</v>
+        <v>38.63</v>
       </c>
       <c r="R19" t="n">
-        <v>-13.9863</v>
+        <v>6.8271</v>
       </c>
       <c r="S19" t="n">
-        <v>-5.4056</v>
+        <v>-8.204700000000001</v>
       </c>
       <c r="T19" t="n">
-        <v>-15.0424</v>
+        <v>6.8853</v>
       </c>
       <c r="U19" t="n">
-        <v>-5.6991</v>
+        <v>3.2764</v>
       </c>
       <c r="V19" t="n">
-        <v>-0.11</v>
+        <v>-1.7291</v>
       </c>
       <c r="W19" t="n">
-        <v>-4.9463</v>
+        <v>3.8627</v>
       </c>
       <c r="X19" t="n">
-        <v>13.9706</v>
+        <v>-7.957</v>
       </c>
       <c r="Y19" t="n">
-        <v>3.3333</v>
+        <v>5.1597</v>
       </c>
       <c r="Z19" t="n">
-        <v>11.5108</v>
+        <v>-10.8333</v>
       </c>
       <c r="AA19" t="n">
-        <v>5.7438</v>
+        <v>-3.3041</v>
       </c>
       <c r="AB19" t="n">
-        <v>-0.3244</v>
+        <v>1.3911</v>
       </c>
       <c r="AC19" t="n">
-        <v>4.3626</v>
+        <v>-4.3338</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>187.69</v>
+        <v>183.77</v>
       </c>
       <c r="C20" t="n">
-        <v>188.43</v>
+        <v>184</v>
       </c>
       <c r="D20" t="n">
-        <v>170.26</v>
+        <v>150</v>
       </c>
       <c r="E20" t="n">
-        <v>176.66</v>
+        <v>165.55</v>
       </c>
       <c r="F20" t="n">
-        <v>75.2</v>
+        <v>76.29000000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>75.84999999999999</v>
+        <v>76.47</v>
       </c>
       <c r="H20" t="n">
-        <v>73.41</v>
+        <v>72.06</v>
       </c>
       <c r="I20" t="n">
-        <v>75.02</v>
+        <v>74.44</v>
       </c>
       <c r="J20" t="n">
-        <v>3.97</v>
+        <v>41.23</v>
       </c>
       <c r="K20" t="n">
-        <v>4.5</v>
+        <v>49.69</v>
       </c>
       <c r="L20" t="n">
-        <v>3.97</v>
+        <v>41.16</v>
       </c>
       <c r="M20" t="n">
-        <v>4.28</v>
+        <v>45.98</v>
       </c>
       <c r="N20" t="n">
-        <v>38.54</v>
+        <v>37.98</v>
       </c>
       <c r="O20" t="n">
-        <v>39.53</v>
+        <v>40.17</v>
       </c>
       <c r="P20" t="n">
-        <v>38.19</v>
+        <v>37.89</v>
       </c>
       <c r="Q20" t="n">
-        <v>38.63</v>
+        <v>38.94</v>
       </c>
       <c r="R20" t="n">
-        <v>6.8271</v>
+        <v>-6.2889</v>
       </c>
       <c r="S20" t="n">
-        <v>-8.204700000000001</v>
+        <v>-13.8926</v>
       </c>
       <c r="T20" t="n">
-        <v>6.8853</v>
+        <v>-5.3026</v>
       </c>
       <c r="U20" t="n">
-        <v>3.2764</v>
+        <v>-0.7731</v>
       </c>
       <c r="V20" t="n">
-        <v>-1.7291</v>
+        <v>-3.3623</v>
       </c>
       <c r="W20" t="n">
-        <v>3.8627</v>
+        <v>2.3652</v>
       </c>
       <c r="X20" t="n">
-        <v>-7.957</v>
+        <v>7.4299</v>
       </c>
       <c r="Y20" t="n">
-        <v>5.1597</v>
+        <v>12.6961</v>
       </c>
       <c r="Z20" t="n">
-        <v>-10.8333</v>
+        <v>2.1778</v>
       </c>
       <c r="AA20" t="n">
-        <v>-3.3041</v>
+        <v>0.8025</v>
       </c>
       <c r="AB20" t="n">
-        <v>1.3911</v>
+        <v>3.0704</v>
       </c>
       <c r="AC20" t="n">
-        <v>-4.3338</v>
+        <v>-2.8443</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>183.77</v>
+        <v>150.44</v>
       </c>
       <c r="C21" t="n">
-        <v>183.935</v>
+        <v>155.81</v>
       </c>
       <c r="D21" t="n">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="E21" t="n">
-        <v>165.55</v>
+        <v>142.48</v>
       </c>
       <c r="F21" t="n">
-        <v>76.33</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="G21" t="n">
-        <v>76.4699</v>
+        <v>73.11669999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>72.06</v>
+        <v>69.69</v>
       </c>
       <c r="I21" t="n">
-        <v>74.44</v>
+        <v>70.73999999999999</v>
       </c>
       <c r="J21" t="n">
-        <v>41.23</v>
+        <v>49.77</v>
       </c>
       <c r="K21" t="n">
-        <v>49.69</v>
+        <v>53.3375</v>
       </c>
       <c r="L21" t="n">
-        <v>41.17</v>
+        <v>48.31</v>
       </c>
       <c r="M21" t="n">
-        <v>45.98</v>
+        <v>52.02</v>
       </c>
       <c r="N21" t="n">
-        <v>37.99</v>
+        <v>39.905</v>
       </c>
       <c r="O21" t="n">
-        <v>40.1669</v>
+        <v>41.4378</v>
       </c>
       <c r="P21" t="n">
-        <v>37.895</v>
+        <v>39.645</v>
       </c>
       <c r="Q21" t="n">
-        <v>38.94</v>
+        <v>40.89</v>
       </c>
       <c r="R21" t="n">
-        <v>-6.2889</v>
+        <v>-13.9354</v>
       </c>
       <c r="S21" t="n">
-        <v>-13.8926</v>
+        <v>-13.8417</v>
       </c>
       <c r="T21" t="n">
-        <v>-5.3026</v>
+        <v>-25.9652</v>
       </c>
       <c r="U21" t="n">
-        <v>-0.7731</v>
+        <v>-4.9704</v>
       </c>
       <c r="V21" t="n">
-        <v>-3.3623</v>
+        <v>-2.6156</v>
       </c>
       <c r="W21" t="n">
-        <v>2.3652</v>
+        <v>-7.3356</v>
       </c>
       <c r="X21" t="n">
-        <v>974.2991</v>
+        <v>13.1361</v>
       </c>
       <c r="Y21" t="n">
-        <v>1026.9608</v>
+        <v>11.871</v>
       </c>
       <c r="Z21" t="n">
-        <v>921.7778</v>
+        <v>27.8133</v>
       </c>
       <c r="AA21" t="n">
-        <v>0.8025</v>
+        <v>5.0077</v>
       </c>
       <c r="AB21" t="n">
-        <v>3.0704</v>
+        <v>2.3529</v>
       </c>
       <c r="AC21" t="n">
-        <v>-2.8443</v>
+        <v>7.3228</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-07-17 22:51
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1713 +568,1713 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>247.42</v>
+        <v>266.04</v>
       </c>
       <c r="C2" t="n">
-        <v>259.79</v>
+        <v>286.15</v>
       </c>
       <c r="D2" t="n">
-        <v>233.3</v>
+        <v>265</v>
       </c>
       <c r="E2" t="n">
-        <v>233.86</v>
+        <v>279.29</v>
       </c>
       <c r="F2" t="n">
-        <v>81.4824</v>
+        <v>81.9114</v>
       </c>
       <c r="G2" t="n">
-        <v>81.6221</v>
+        <v>83.408</v>
       </c>
       <c r="H2" t="n">
-        <v>76.7633</v>
+        <v>80.4448</v>
       </c>
       <c r="I2" t="n">
-        <v>77.36190000000001</v>
+        <v>82.67959999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>41.2198</v>
+        <v>38.1555</v>
       </c>
       <c r="K2" t="n">
-        <v>44.0864</v>
+        <v>38.2544</v>
       </c>
       <c r="L2" t="n">
-        <v>38.7486</v>
+        <v>34.1027</v>
       </c>
       <c r="M2" t="n">
-        <v>44.0864</v>
+        <v>35.4866</v>
       </c>
       <c r="N2" t="n">
-        <v>36.9397</v>
+        <v>36.6149</v>
       </c>
       <c r="O2" t="n">
-        <v>39.1641</v>
+        <v>37.3531</v>
       </c>
       <c r="P2" t="n">
-        <v>36.8708</v>
+        <v>35.857</v>
       </c>
       <c r="Q2" t="n">
-        <v>38.8984</v>
+        <v>36.1719</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>266.04</v>
+        <v>299.26</v>
       </c>
       <c r="C3" t="n">
-        <v>286.15</v>
+        <v>302</v>
       </c>
       <c r="D3" t="n">
-        <v>265</v>
+        <v>286.24</v>
       </c>
       <c r="E3" t="n">
-        <v>279.29</v>
+        <v>300.77</v>
       </c>
       <c r="F3" t="n">
-        <v>81.9114</v>
+        <v>83.7572</v>
       </c>
       <c r="G3" t="n">
-        <v>83.408</v>
+        <v>84.9145</v>
       </c>
       <c r="H3" t="n">
-        <v>80.4448</v>
+        <v>81.203</v>
       </c>
       <c r="I3" t="n">
-        <v>82.67959999999999</v>
+        <v>82.3903</v>
       </c>
       <c r="J3" t="n">
-        <v>38.1555</v>
+        <v>32.9165</v>
       </c>
       <c r="K3" t="n">
-        <v>38.2544</v>
+        <v>34.4981</v>
       </c>
       <c r="L3" t="n">
-        <v>34.1027</v>
+        <v>32.5212</v>
       </c>
       <c r="M3" t="n">
-        <v>35.4866</v>
+        <v>32.62</v>
       </c>
       <c r="N3" t="n">
-        <v>36.6149</v>
+        <v>35.7389</v>
       </c>
       <c r="O3" t="n">
-        <v>37.3531</v>
+        <v>36.8511</v>
       </c>
       <c r="P3" t="n">
-        <v>35.857</v>
+        <v>35.2369</v>
       </c>
       <c r="Q3" t="n">
-        <v>36.1719</v>
+        <v>36.3491</v>
       </c>
       <c r="R3" t="n">
-        <v>19.4262</v>
+        <v>7.6909</v>
       </c>
       <c r="U3" t="n">
-        <v>6.8738</v>
+        <v>-0.3499</v>
       </c>
       <c r="X3" t="n">
-        <v>-19.5067</v>
+        <v>-8.077999999999999</v>
       </c>
       <c r="AA3" t="n">
-        <v>-7.0093</v>
+        <v>0.4899</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>299.26</v>
+        <v>236</v>
       </c>
       <c r="C4" t="n">
-        <v>302</v>
+        <v>252.98</v>
       </c>
       <c r="D4" t="n">
-        <v>286.24</v>
+        <v>223</v>
       </c>
       <c r="E4" t="n">
-        <v>300.77</v>
+        <v>231.42</v>
       </c>
       <c r="F4" t="n">
-        <v>83.7572</v>
+        <v>74.9474</v>
       </c>
       <c r="G4" t="n">
-        <v>84.9145</v>
+        <v>77.56140000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>81.203</v>
+        <v>73.7402</v>
       </c>
       <c r="I4" t="n">
-        <v>82.3903</v>
+        <v>74.26900000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>32.9165</v>
+        <v>39.9</v>
       </c>
       <c r="K4" t="n">
-        <v>34.4981</v>
+        <v>41.3</v>
       </c>
       <c r="L4" t="n">
-        <v>32.5212</v>
+        <v>38</v>
       </c>
       <c r="M4" t="n">
-        <v>32.62</v>
+        <v>40.4</v>
       </c>
       <c r="N4" t="n">
-        <v>35.7389</v>
+        <v>39.6267</v>
       </c>
       <c r="O4" t="n">
-        <v>36.8511</v>
+        <v>40.1582</v>
       </c>
       <c r="P4" t="n">
-        <v>35.2369</v>
+        <v>38.4653</v>
       </c>
       <c r="Q4" t="n">
-        <v>36.3491</v>
+        <v>39.922</v>
       </c>
       <c r="R4" t="n">
-        <v>7.6909</v>
+        <v>-23.0575</v>
       </c>
       <c r="U4" t="n">
-        <v>-0.3499</v>
+        <v>-9.857100000000001</v>
       </c>
       <c r="X4" t="n">
-        <v>-8.077999999999999</v>
+        <v>23.8504</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.4899</v>
+        <v>9.8294</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>236</v>
+        <v>233.11</v>
       </c>
       <c r="C5" t="n">
-        <v>252.98</v>
+        <v>237</v>
       </c>
       <c r="D5" t="n">
-        <v>223</v>
+        <v>211.13</v>
       </c>
       <c r="E5" t="n">
-        <v>231.42</v>
+        <v>229.57</v>
       </c>
       <c r="F5" t="n">
-        <v>74.9474</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>77.56140000000001</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>73.7402</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="I5" t="n">
-        <v>74.26900000000001</v>
+        <v>73.3</v>
       </c>
       <c r="J5" t="n">
-        <v>39.9</v>
+        <v>40</v>
       </c>
       <c r="K5" t="n">
-        <v>41.3</v>
+        <v>43.9</v>
       </c>
       <c r="L5" t="n">
-        <v>38</v>
+        <v>39.2</v>
       </c>
       <c r="M5" t="n">
-        <v>40.4</v>
+        <v>40.8</v>
       </c>
       <c r="N5" t="n">
-        <v>39.6267</v>
+        <v>39.66</v>
       </c>
       <c r="O5" t="n">
-        <v>40.1582</v>
+        <v>41.49</v>
       </c>
       <c r="P5" t="n">
-        <v>38.4653</v>
+        <v>38.9</v>
       </c>
       <c r="Q5" t="n">
-        <v>39.922</v>
+        <v>40.45</v>
       </c>
       <c r="R5" t="n">
-        <v>-23.0575</v>
+        <v>-0.7994</v>
       </c>
       <c r="S5" t="n">
-        <v>-1.0434</v>
+        <v>-17.8023</v>
       </c>
       <c r="U5" t="n">
-        <v>-9.857100000000001</v>
+        <v>-1.3047</v>
       </c>
       <c r="V5" t="n">
-        <v>-3.998</v>
+        <v>-11.3445</v>
       </c>
       <c r="X5" t="n">
-        <v>23.8504</v>
+        <v>0.9901</v>
       </c>
       <c r="Y5" t="n">
-        <v>-8.361800000000001</v>
+        <v>14.973</v>
       </c>
       <c r="AA5" t="n">
-        <v>9.8294</v>
+        <v>1.3226</v>
       </c>
       <c r="AB5" t="n">
-        <v>2.6315</v>
+        <v>11.8271</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>233.11</v>
+        <v>268.05</v>
       </c>
       <c r="C6" t="n">
-        <v>237</v>
+        <v>268.4</v>
       </c>
       <c r="D6" t="n">
-        <v>211.13</v>
+        <v>225.74</v>
       </c>
       <c r="E6" t="n">
-        <v>229.57</v>
+        <v>252.61</v>
       </c>
       <c r="F6" t="n">
-        <v>74.79000000000001</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>76.18000000000001</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>71.34999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>73.3</v>
+        <v>74.95</v>
       </c>
       <c r="J6" t="n">
-        <v>40</v>
+        <v>33.8</v>
       </c>
       <c r="K6" t="n">
-        <v>43.9</v>
+        <v>41.5</v>
       </c>
       <c r="L6" t="n">
-        <v>39.2</v>
+        <v>33.7</v>
       </c>
       <c r="M6" t="n">
-        <v>40.8</v>
+        <v>36.3</v>
       </c>
       <c r="N6" t="n">
-        <v>39.66</v>
+        <v>37.87</v>
       </c>
       <c r="O6" t="n">
-        <v>41.49</v>
+        <v>41.37</v>
       </c>
       <c r="P6" t="n">
-        <v>38.9</v>
+        <v>37.71</v>
       </c>
       <c r="Q6" t="n">
-        <v>40.45</v>
+        <v>39.47</v>
       </c>
       <c r="R6" t="n">
-        <v>-0.7994</v>
+        <v>10.0362</v>
       </c>
       <c r="S6" t="n">
-        <v>-17.8023</v>
+        <v>-16.0122</v>
       </c>
       <c r="U6" t="n">
-        <v>-1.3047</v>
+        <v>2.251</v>
       </c>
       <c r="V6" t="n">
-        <v>-11.3445</v>
+        <v>-9.0306</v>
       </c>
       <c r="X6" t="n">
-        <v>0.9901</v>
+        <v>-11.0294</v>
       </c>
       <c r="Y6" t="n">
-        <v>14.973</v>
+        <v>11.2814</v>
       </c>
       <c r="AA6" t="n">
-        <v>1.3226</v>
+        <v>-2.4227</v>
       </c>
       <c r="AB6" t="n">
-        <v>11.8271</v>
+        <v>8.585900000000001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>268.05</v>
+        <v>226.24</v>
       </c>
       <c r="C7" t="n">
-        <v>268.4</v>
+        <v>231.25</v>
       </c>
       <c r="D7" t="n">
-        <v>225.74</v>
+        <v>212.1</v>
       </c>
       <c r="E7" t="n">
-        <v>252.61</v>
+        <v>215.6</v>
       </c>
       <c r="F7" t="n">
-        <v>77.95999999999999</v>
+        <v>72.09</v>
       </c>
       <c r="G7" t="n">
-        <v>78.23999999999999</v>
+        <v>74.69</v>
       </c>
       <c r="H7" t="n">
-        <v>71.59999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="I7" t="n">
-        <v>74.95</v>
+        <v>71.83</v>
       </c>
       <c r="J7" t="n">
-        <v>33.8</v>
+        <v>40.4</v>
       </c>
       <c r="K7" t="n">
-        <v>41.5</v>
+        <v>42.5</v>
       </c>
       <c r="L7" t="n">
-        <v>33.7</v>
+        <v>39.5</v>
       </c>
       <c r="M7" t="n">
-        <v>36.3</v>
+        <v>42.4</v>
       </c>
       <c r="N7" t="n">
-        <v>37.87</v>
+        <v>41.08</v>
       </c>
       <c r="O7" t="n">
-        <v>41.37</v>
+        <v>41.79</v>
       </c>
       <c r="P7" t="n">
-        <v>37.71</v>
+        <v>39.69</v>
       </c>
       <c r="Q7" t="n">
-        <v>39.47</v>
+        <v>41.31</v>
       </c>
       <c r="R7" t="n">
-        <v>10.0362</v>
+        <v>-14.651</v>
       </c>
       <c r="S7" t="n">
-        <v>-16.0122</v>
+        <v>-6.8361</v>
       </c>
       <c r="T7" t="n">
-        <v>8.0176</v>
+        <v>-22.8043</v>
       </c>
       <c r="U7" t="n">
-        <v>2.251</v>
+        <v>-4.1628</v>
       </c>
       <c r="V7" t="n">
-        <v>-9.0306</v>
+        <v>-3.284</v>
       </c>
       <c r="W7" t="n">
-        <v>-3.1177</v>
+        <v>-13.1225</v>
       </c>
       <c r="X7" t="n">
-        <v>-11.0294</v>
+        <v>16.8044</v>
       </c>
       <c r="Y7" t="n">
-        <v>11.2814</v>
+        <v>4.9505</v>
       </c>
       <c r="Z7" t="n">
-        <v>-17.6617</v>
+        <v>19.4817</v>
       </c>
       <c r="AA7" t="n">
-        <v>-2.4227</v>
+        <v>4.6618</v>
       </c>
       <c r="AB7" t="n">
-        <v>8.585900000000001</v>
+        <v>3.4768</v>
       </c>
       <c r="AC7" t="n">
-        <v>1.4695</v>
+        <v>14.2047</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>226.24</v>
+        <v>216.36</v>
       </c>
       <c r="C8" t="n">
-        <v>231.25</v>
+        <v>238.65</v>
       </c>
       <c r="D8" t="n">
-        <v>212.1</v>
+        <v>192.3</v>
       </c>
       <c r="E8" t="n">
-        <v>215.6</v>
+        <v>236.52</v>
       </c>
       <c r="F8" t="n">
-        <v>72.09</v>
+        <v>74.12</v>
       </c>
       <c r="G8" t="n">
-        <v>74.69</v>
+        <v>77.38</v>
       </c>
       <c r="H8" t="n">
-        <v>70.72</v>
+        <v>71.45</v>
       </c>
       <c r="I8" t="n">
-        <v>71.83</v>
+        <v>77.19</v>
       </c>
       <c r="J8" t="n">
-        <v>40.4</v>
+        <v>41.6</v>
       </c>
       <c r="K8" t="n">
-        <v>42.5</v>
+        <v>46.3</v>
       </c>
       <c r="L8" t="n">
-        <v>39.5</v>
+        <v>37</v>
       </c>
       <c r="M8" t="n">
-        <v>42.4</v>
+        <v>37.2</v>
       </c>
       <c r="N8" t="n">
-        <v>41.08</v>
+        <v>39.91</v>
       </c>
       <c r="O8" t="n">
-        <v>41.79</v>
+        <v>41.43</v>
       </c>
       <c r="P8" t="n">
-        <v>39.69</v>
+        <v>38.08</v>
       </c>
       <c r="Q8" t="n">
-        <v>41.31</v>
+        <v>38.16</v>
       </c>
       <c r="R8" t="n">
-        <v>-14.651</v>
+        <v>9.703200000000001</v>
       </c>
       <c r="S8" t="n">
-        <v>-6.8361</v>
+        <v>3.0274</v>
       </c>
       <c r="T8" t="n">
-        <v>-22.8043</v>
+        <v>-21.3618</v>
       </c>
       <c r="U8" t="n">
-        <v>-4.1628</v>
+        <v>7.4621</v>
       </c>
       <c r="V8" t="n">
-        <v>-3.284</v>
+        <v>5.307</v>
       </c>
       <c r="W8" t="n">
-        <v>-13.1225</v>
+        <v>-6.3118</v>
       </c>
       <c r="X8" t="n">
-        <v>16.8044</v>
+        <v>-12.2642</v>
       </c>
       <c r="Y8" t="n">
-        <v>4.9505</v>
+        <v>-8.823499999999999</v>
       </c>
       <c r="Z8" t="n">
-        <v>19.4817</v>
+        <v>14.0405</v>
       </c>
       <c r="AA8" t="n">
-        <v>4.6618</v>
+        <v>-7.6253</v>
       </c>
       <c r="AB8" t="n">
-        <v>3.4768</v>
+        <v>-5.6613</v>
       </c>
       <c r="AC8" t="n">
-        <v>14.2047</v>
+        <v>4.982</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>216.36</v>
+        <v>241.45</v>
       </c>
       <c r="C9" t="n">
-        <v>238.65</v>
+        <v>272</v>
       </c>
       <c r="D9" t="n">
-        <v>192.3</v>
+        <v>240.59</v>
       </c>
       <c r="E9" t="n">
-        <v>236.52</v>
+        <v>266.71</v>
       </c>
       <c r="F9" t="n">
-        <v>74.12</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>77.38</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>71.45</v>
+        <v>77.15000000000001</v>
       </c>
       <c r="I9" t="n">
-        <v>77.19</v>
+        <v>81</v>
       </c>
       <c r="J9" t="n">
-        <v>41.6</v>
+        <v>36.6</v>
       </c>
       <c r="K9" t="n">
-        <v>46.3</v>
+        <v>36.8</v>
       </c>
       <c r="L9" t="n">
-        <v>37</v>
+        <v>31.7</v>
       </c>
       <c r="M9" t="n">
-        <v>37.2</v>
+        <v>32.4</v>
       </c>
       <c r="N9" t="n">
-        <v>39.91</v>
+        <v>38.16</v>
       </c>
       <c r="O9" t="n">
-        <v>41.43</v>
+        <v>38.2</v>
       </c>
       <c r="P9" t="n">
-        <v>38.08</v>
+        <v>36.03</v>
       </c>
       <c r="Q9" t="n">
-        <v>38.16</v>
+        <v>36.31</v>
       </c>
       <c r="R9" t="n">
-        <v>9.703200000000001</v>
+        <v>12.7642</v>
       </c>
       <c r="S9" t="n">
-        <v>3.0274</v>
+        <v>5.5817</v>
       </c>
       <c r="T9" t="n">
-        <v>-21.3618</v>
+        <v>15.2493</v>
       </c>
       <c r="U9" t="n">
-        <v>7.4621</v>
+        <v>4.9359</v>
       </c>
       <c r="V9" t="n">
-        <v>5.307</v>
+        <v>8.071999999999999</v>
       </c>
       <c r="W9" t="n">
-        <v>-6.3118</v>
+        <v>9.063000000000001</v>
       </c>
       <c r="X9" t="n">
-        <v>-12.2642</v>
+        <v>-12.9032</v>
       </c>
       <c r="Y9" t="n">
-        <v>-8.823499999999999</v>
+        <v>-10.7438</v>
       </c>
       <c r="Z9" t="n">
-        <v>14.0405</v>
+        <v>-19.802</v>
       </c>
       <c r="AA9" t="n">
-        <v>-7.6253</v>
+        <v>-4.848</v>
       </c>
       <c r="AB9" t="n">
-        <v>-5.6613</v>
+        <v>-8.0061</v>
       </c>
       <c r="AC9" t="n">
-        <v>4.982</v>
+        <v>-9.047599999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>241.45</v>
+        <v>237.79</v>
       </c>
       <c r="C10" t="n">
-        <v>272</v>
+        <v>246.47</v>
       </c>
       <c r="D10" t="n">
-        <v>240.59</v>
+        <v>215.38</v>
       </c>
       <c r="E10" t="n">
-        <v>266.71</v>
+        <v>217.55</v>
       </c>
       <c r="F10" t="n">
-        <v>77.23999999999999</v>
+        <v>78.72</v>
       </c>
       <c r="G10" t="n">
-        <v>81.54000000000001</v>
+        <v>79.64</v>
       </c>
       <c r="H10" t="n">
-        <v>77.15000000000001</v>
+        <v>77.23</v>
       </c>
       <c r="I10" t="n">
-        <v>81</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>36.6</v>
+        <v>35.9</v>
       </c>
       <c r="K10" t="n">
-        <v>36.8</v>
+        <v>38.9</v>
       </c>
       <c r="L10" t="n">
-        <v>31.7</v>
+        <v>35.1</v>
       </c>
       <c r="M10" t="n">
-        <v>32.4</v>
+        <v>38.6</v>
       </c>
       <c r="N10" t="n">
-        <v>38.16</v>
+        <v>37.31</v>
       </c>
       <c r="O10" t="n">
-        <v>38.2</v>
+        <v>37.98</v>
       </c>
       <c r="P10" t="n">
-        <v>36.03</v>
+        <v>36.9</v>
       </c>
       <c r="Q10" t="n">
-        <v>36.31</v>
+        <v>37.88</v>
       </c>
       <c r="R10" t="n">
-        <v>12.7642</v>
+        <v>-18.432</v>
       </c>
       <c r="S10" t="n">
-        <v>5.5817</v>
+        <v>0.9045</v>
       </c>
       <c r="T10" t="n">
-        <v>15.2493</v>
+        <v>-5.2359</v>
       </c>
       <c r="U10" t="n">
-        <v>4.9359</v>
+        <v>-4.3704</v>
       </c>
       <c r="V10" t="n">
-        <v>8.071999999999999</v>
+        <v>7.838</v>
       </c>
       <c r="W10" t="n">
-        <v>9.063000000000001</v>
+        <v>5.6753</v>
       </c>
       <c r="X10" t="n">
-        <v>-12.9032</v>
+        <v>19.1358</v>
       </c>
       <c r="Y10" t="n">
-        <v>-10.7438</v>
+        <v>-8.962300000000001</v>
       </c>
       <c r="Z10" t="n">
-        <v>-19.802</v>
+        <v>-5.3922</v>
       </c>
       <c r="AA10" t="n">
-        <v>-4.848</v>
+        <v>4.3239</v>
       </c>
       <c r="AB10" t="n">
-        <v>-8.0061</v>
+        <v>-8.303100000000001</v>
       </c>
       <c r="AC10" t="n">
-        <v>-9.047599999999999</v>
+        <v>-6.3535</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>237.79</v>
+        <v>219.23</v>
       </c>
       <c r="C11" t="n">
-        <v>246.47</v>
+        <v>226.13</v>
       </c>
       <c r="D11" t="n">
-        <v>215.38</v>
+        <v>168.88</v>
       </c>
       <c r="E11" t="n">
-        <v>217.55</v>
+        <v>181.47</v>
       </c>
       <c r="F11" t="n">
-        <v>78.72</v>
+        <v>77.45</v>
       </c>
       <c r="G11" t="n">
-        <v>79.64</v>
+        <v>79.14</v>
       </c>
       <c r="H11" t="n">
-        <v>77.23</v>
+        <v>71.72</v>
       </c>
       <c r="I11" t="n">
-        <v>77.45999999999999</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>35.9</v>
+        <v>38.4</v>
       </c>
       <c r="K11" t="n">
-        <v>38.9</v>
+        <v>47.4</v>
       </c>
       <c r="L11" t="n">
-        <v>35.1</v>
+        <v>37.1</v>
       </c>
       <c r="M11" t="n">
-        <v>38.6</v>
+        <v>45.1</v>
       </c>
       <c r="N11" t="n">
-        <v>37.31</v>
+        <v>37.91</v>
       </c>
       <c r="O11" t="n">
-        <v>37.98</v>
+        <v>40.72</v>
       </c>
       <c r="P11" t="n">
-        <v>36.9</v>
+        <v>37.08</v>
       </c>
       <c r="Q11" t="n">
-        <v>37.88</v>
+        <v>39.95</v>
       </c>
       <c r="R11" t="n">
-        <v>-18.432</v>
+        <v>-16.5847</v>
       </c>
       <c r="S11" t="n">
-        <v>0.9045</v>
+        <v>-23.275</v>
       </c>
       <c r="T11" t="n">
-        <v>-5.2359</v>
+        <v>-28.162</v>
       </c>
       <c r="U11" t="n">
-        <v>-4.3704</v>
+        <v>-5.306</v>
       </c>
       <c r="V11" t="n">
-        <v>7.838</v>
+        <v>-4.9747</v>
       </c>
       <c r="W11" t="n">
-        <v>5.6753</v>
+        <v>-2.1348</v>
       </c>
       <c r="X11" t="n">
-        <v>19.1358</v>
+        <v>16.8394</v>
       </c>
       <c r="Y11" t="n">
-        <v>-8.962300000000001</v>
+        <v>21.2366</v>
       </c>
       <c r="Z11" t="n">
-        <v>-5.3922</v>
+        <v>24.2424</v>
       </c>
       <c r="AA11" t="n">
-        <v>4.3239</v>
+        <v>5.4646</v>
       </c>
       <c r="AB11" t="n">
-        <v>-8.303100000000001</v>
+        <v>4.6908</v>
       </c>
       <c r="AC11" t="n">
-        <v>-6.3535</v>
+        <v>1.2161</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>219.23</v>
+        <v>197.21</v>
       </c>
       <c r="C12" t="n">
-        <v>226.13</v>
+        <v>210.8</v>
       </c>
       <c r="D12" t="n">
-        <v>168.88</v>
+        <v>194.22</v>
       </c>
       <c r="E12" t="n">
-        <v>181.47</v>
+        <v>194.65</v>
       </c>
       <c r="F12" t="n">
+        <v>75.54000000000001</v>
+      </c>
+      <c r="G12" t="n">
         <v>77.45</v>
       </c>
-      <c r="G12" t="n">
-        <v>79.14</v>
-      </c>
       <c r="H12" t="n">
-        <v>71.72</v>
+        <v>75.11</v>
       </c>
       <c r="I12" t="n">
-        <v>73.34999999999999</v>
+        <v>76.42</v>
       </c>
       <c r="J12" t="n">
-        <v>38.4</v>
+        <v>41.1</v>
       </c>
       <c r="K12" t="n">
-        <v>47.4</v>
+        <v>41.8</v>
       </c>
       <c r="L12" t="n">
-        <v>37.1</v>
+        <v>37.7</v>
       </c>
       <c r="M12" t="n">
-        <v>45.1</v>
+        <v>41.7</v>
       </c>
       <c r="N12" t="n">
-        <v>37.91</v>
+        <v>38.75</v>
       </c>
       <c r="O12" t="n">
-        <v>40.72</v>
+        <v>38.98</v>
       </c>
       <c r="P12" t="n">
-        <v>37.08</v>
+        <v>37.71</v>
       </c>
       <c r="Q12" t="n">
-        <v>39.95</v>
+        <v>38.28</v>
       </c>
       <c r="R12" t="n">
-        <v>-16.5847</v>
+        <v>7.2629</v>
       </c>
       <c r="S12" t="n">
-        <v>-23.275</v>
+        <v>-27.0181</v>
       </c>
       <c r="T12" t="n">
-        <v>-28.162</v>
+        <v>-9.7171</v>
       </c>
       <c r="U12" t="n">
-        <v>-5.306</v>
+        <v>4.1854</v>
       </c>
       <c r="V12" t="n">
-        <v>-4.9747</v>
+        <v>-5.6543</v>
       </c>
       <c r="W12" t="n">
-        <v>-2.1348</v>
+        <v>6.3901</v>
       </c>
       <c r="X12" t="n">
-        <v>16.8394</v>
+        <v>-7.5388</v>
       </c>
       <c r="Y12" t="n">
-        <v>21.2366</v>
+        <v>28.7037</v>
       </c>
       <c r="Z12" t="n">
-        <v>24.2424</v>
+        <v>-1.6509</v>
       </c>
       <c r="AA12" t="n">
-        <v>5.4646</v>
+        <v>-4.1802</v>
       </c>
       <c r="AB12" t="n">
-        <v>4.6908</v>
+        <v>5.4255</v>
       </c>
       <c r="AC12" t="n">
-        <v>1.2161</v>
+        <v>-7.3348</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>197.21</v>
+        <v>165.4</v>
       </c>
       <c r="C13" t="n">
-        <v>210.8</v>
+        <v>171.88</v>
       </c>
       <c r="D13" t="n">
-        <v>194.22</v>
+        <v>150.08</v>
       </c>
       <c r="E13" t="n">
-        <v>194.65</v>
+        <v>165.28</v>
       </c>
       <c r="F13" t="n">
-        <v>75.54000000000001</v>
+        <v>73.7</v>
       </c>
       <c r="G13" t="n">
-        <v>77.45</v>
+        <v>74.39</v>
       </c>
       <c r="H13" t="n">
-        <v>75.11</v>
+        <v>70.76000000000001</v>
       </c>
       <c r="I13" t="n">
-        <v>76.42</v>
+        <v>72.23</v>
       </c>
       <c r="J13" t="n">
-        <v>41.1</v>
+        <v>48</v>
       </c>
       <c r="K13" t="n">
-        <v>41.8</v>
+        <v>51.4</v>
       </c>
       <c r="L13" t="n">
-        <v>37.7</v>
+        <v>46.6</v>
       </c>
       <c r="M13" t="n">
-        <v>41.7</v>
+        <v>48</v>
       </c>
       <c r="N13" t="n">
-        <v>38.75</v>
+        <v>39.64</v>
       </c>
       <c r="O13" t="n">
-        <v>38.98</v>
+        <v>41.11</v>
       </c>
       <c r="P13" t="n">
-        <v>37.71</v>
+        <v>39.29</v>
       </c>
       <c r="Q13" t="n">
-        <v>38.28</v>
+        <v>40.38</v>
       </c>
       <c r="R13" t="n">
-        <v>7.2629</v>
+        <v>-15.0886</v>
       </c>
       <c r="S13" t="n">
-        <v>-27.0181</v>
+        <v>-24.0267</v>
       </c>
       <c r="T13" t="n">
-        <v>-9.7171</v>
+        <v>-30.1201</v>
       </c>
       <c r="U13" t="n">
-        <v>4.1854</v>
+        <v>-5.4829</v>
       </c>
       <c r="V13" t="n">
-        <v>-5.6543</v>
+        <v>-6.7519</v>
       </c>
       <c r="W13" t="n">
-        <v>6.3901</v>
+        <v>-6.4257</v>
       </c>
       <c r="X13" t="n">
-        <v>-7.5388</v>
+        <v>15.1079</v>
       </c>
       <c r="Y13" t="n">
-        <v>28.7037</v>
+        <v>24.3523</v>
       </c>
       <c r="Z13" t="n">
-        <v>-1.6509</v>
+        <v>29.0323</v>
       </c>
       <c r="AA13" t="n">
-        <v>-4.1802</v>
+        <v>5.4859</v>
       </c>
       <c r="AB13" t="n">
-        <v>5.4255</v>
+        <v>6.5998</v>
       </c>
       <c r="AC13" t="n">
-        <v>-7.3348</v>
+        <v>5.8176</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>165.4</v>
+        <v>159.21</v>
       </c>
       <c r="C14" t="n">
-        <v>171.88</v>
+        <v>176.75</v>
       </c>
       <c r="D14" t="n">
-        <v>150.08</v>
+        <v>158.87</v>
       </c>
       <c r="E14" t="n">
-        <v>165.28</v>
+        <v>174.82</v>
       </c>
       <c r="F14" t="n">
-        <v>73.7</v>
+        <v>70.8</v>
       </c>
       <c r="G14" t="n">
-        <v>74.39</v>
+        <v>73.02</v>
       </c>
       <c r="H14" t="n">
-        <v>70.76000000000001</v>
+        <v>69.56999999999999</v>
       </c>
       <c r="I14" t="n">
-        <v>72.23</v>
+        <v>72.72</v>
       </c>
       <c r="J14" t="n">
-        <v>48</v>
+        <v>49.8</v>
       </c>
       <c r="K14" t="n">
-        <v>51.4</v>
+        <v>49.9</v>
       </c>
       <c r="L14" t="n">
-        <v>46.6</v>
+        <v>44.6</v>
       </c>
       <c r="M14" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="N14" t="n">
-        <v>39.64</v>
+        <v>41.18</v>
       </c>
       <c r="O14" t="n">
-        <v>41.11</v>
+        <v>41.86</v>
       </c>
       <c r="P14" t="n">
-        <v>39.29</v>
+        <v>39.93</v>
       </c>
       <c r="Q14" t="n">
-        <v>40.38</v>
+        <v>40.08</v>
       </c>
       <c r="R14" t="n">
-        <v>-15.0886</v>
+        <v>5.772</v>
       </c>
       <c r="S14" t="n">
-        <v>-24.0267</v>
+        <v>-3.6645</v>
       </c>
       <c r="T14" t="n">
-        <v>-30.1201</v>
+        <v>-34.4532</v>
       </c>
       <c r="U14" t="n">
-        <v>-5.4829</v>
+        <v>0.6784</v>
       </c>
       <c r="V14" t="n">
-        <v>-6.7519</v>
+        <v>-0.8589</v>
       </c>
       <c r="W14" t="n">
-        <v>-6.4257</v>
+        <v>-10.2222</v>
       </c>
       <c r="X14" t="n">
-        <v>15.1079</v>
+        <v>-6.25</v>
       </c>
       <c r="Y14" t="n">
-        <v>24.3523</v>
+        <v>-0.2217</v>
       </c>
       <c r="Z14" t="n">
-        <v>29.0323</v>
+        <v>38.8889</v>
       </c>
       <c r="AA14" t="n">
-        <v>5.4859</v>
+        <v>-0.7429</v>
       </c>
       <c r="AB14" t="n">
-        <v>6.5998</v>
+        <v>0.3254</v>
       </c>
       <c r="AC14" t="n">
-        <v>5.8176</v>
+        <v>10.3828</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>159.21</v>
+        <v>199.81</v>
       </c>
       <c r="C15" t="n">
-        <v>176.75</v>
+        <v>204.55</v>
       </c>
       <c r="D15" t="n">
-        <v>158.87</v>
+        <v>189.46</v>
       </c>
       <c r="E15" t="n">
-        <v>174.82</v>
+        <v>192.45</v>
       </c>
       <c r="F15" t="n">
-        <v>70.8</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="G15" t="n">
-        <v>73.02</v>
+        <v>76.69</v>
       </c>
       <c r="H15" t="n">
-        <v>69.56999999999999</v>
+        <v>73.89</v>
       </c>
       <c r="I15" t="n">
-        <v>72.72</v>
+        <v>76.34</v>
       </c>
       <c r="J15" t="n">
-        <v>49.8</v>
+        <v>38.7</v>
       </c>
       <c r="K15" t="n">
-        <v>49.9</v>
+        <v>41.2</v>
       </c>
       <c r="L15" t="n">
-        <v>44.6</v>
+        <v>37.5</v>
       </c>
       <c r="M15" t="n">
-        <v>45</v>
+        <v>40.7</v>
       </c>
       <c r="N15" t="n">
-        <v>41.18</v>
+        <v>38.93</v>
       </c>
       <c r="O15" t="n">
-        <v>41.86</v>
+        <v>39.47</v>
       </c>
       <c r="P15" t="n">
-        <v>39.93</v>
+        <v>37.93</v>
       </c>
       <c r="Q15" t="n">
-        <v>40.08</v>
+        <v>38.1</v>
       </c>
       <c r="R15" t="n">
-        <v>5.772</v>
+        <v>10.0847</v>
       </c>
       <c r="S15" t="n">
-        <v>-3.6645</v>
+        <v>-1.1302</v>
       </c>
       <c r="T15" t="n">
-        <v>-34.4532</v>
+        <v>-11.5376</v>
       </c>
       <c r="U15" t="n">
-        <v>0.6784</v>
+        <v>4.978</v>
       </c>
       <c r="V15" t="n">
-        <v>-0.8589</v>
+        <v>-0.1047</v>
       </c>
       <c r="W15" t="n">
-        <v>-10.2222</v>
+        <v>-1.4459</v>
       </c>
       <c r="X15" t="n">
-        <v>-6.25</v>
+        <v>-9.5556</v>
       </c>
       <c r="Y15" t="n">
-        <v>-0.2217</v>
+        <v>-2.3981</v>
       </c>
       <c r="Z15" t="n">
-        <v>38.8889</v>
+        <v>5.4404</v>
       </c>
       <c r="AA15" t="n">
-        <v>-0.7429</v>
+        <v>-4.9401</v>
       </c>
       <c r="AB15" t="n">
-        <v>0.3254</v>
+        <v>-0.4702</v>
       </c>
       <c r="AC15" t="n">
-        <v>10.3828</v>
+        <v>0.5808</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>199.81</v>
+        <v>182.4</v>
       </c>
       <c r="C16" t="n">
-        <v>204.55</v>
+        <v>195.94</v>
       </c>
       <c r="D16" t="n">
-        <v>189.46</v>
+        <v>176.8</v>
       </c>
       <c r="E16" t="n">
-        <v>192.45</v>
+        <v>192.26</v>
       </c>
       <c r="F16" t="n">
-        <v>74.84999999999999</v>
+        <v>75.53</v>
       </c>
       <c r="G16" t="n">
-        <v>76.69</v>
+        <v>77.31999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>73.89</v>
+        <v>74.33</v>
       </c>
       <c r="I16" t="n">
-        <v>76.34</v>
+        <v>77.03</v>
       </c>
       <c r="J16" t="n">
-        <v>38.7</v>
+        <v>42.7</v>
       </c>
       <c r="K16" t="n">
-        <v>41.2</v>
+        <v>43.9</v>
       </c>
       <c r="L16" t="n">
-        <v>37.5</v>
+        <v>39.9</v>
       </c>
       <c r="M16" t="n">
-        <v>40.7</v>
+        <v>40.8</v>
       </c>
       <c r="N16" t="n">
-        <v>38.93</v>
+        <v>38.49</v>
       </c>
       <c r="O16" t="n">
-        <v>39.47</v>
+        <v>39.14</v>
       </c>
       <c r="P16" t="n">
-        <v>37.93</v>
+        <v>37.64</v>
       </c>
       <c r="Q16" t="n">
-        <v>38.1</v>
+        <v>37.78</v>
       </c>
       <c r="R16" t="n">
-        <v>10.0847</v>
+        <v>-0.0987</v>
       </c>
       <c r="S16" t="n">
-        <v>-1.1302</v>
+        <v>16.3238</v>
       </c>
       <c r="T16" t="n">
-        <v>-11.5376</v>
+        <v>5.9459</v>
       </c>
       <c r="U16" t="n">
-        <v>4.978</v>
+        <v>0.9039</v>
       </c>
       <c r="V16" t="n">
-        <v>-0.1047</v>
+        <v>6.6454</v>
       </c>
       <c r="W16" t="n">
-        <v>-1.4459</v>
+        <v>5.017</v>
       </c>
       <c r="X16" t="n">
-        <v>-9.5556</v>
+        <v>0.2457</v>
       </c>
       <c r="Y16" t="n">
-        <v>-2.3981</v>
+        <v>-15</v>
       </c>
       <c r="Z16" t="n">
-        <v>5.4404</v>
+        <v>-9.5344</v>
       </c>
       <c r="AA16" t="n">
-        <v>-4.9401</v>
+        <v>-0.8399</v>
       </c>
       <c r="AB16" t="n">
-        <v>-0.4702</v>
+        <v>-6.4388</v>
       </c>
       <c r="AC16" t="n">
-        <v>0.5808</v>
+        <v>-5.4318</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>182.4</v>
+        <v>174.61</v>
       </c>
       <c r="C17" t="n">
-        <v>195.94</v>
+        <v>177.67</v>
       </c>
       <c r="D17" t="n">
-        <v>176.8</v>
+        <v>161.55</v>
       </c>
       <c r="E17" t="n">
-        <v>192.26</v>
+        <v>165.37</v>
       </c>
       <c r="F17" t="n">
-        <v>75.53</v>
+        <v>74.54000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>77.31999999999999</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="H17" t="n">
-        <v>74.33</v>
+        <v>72.09</v>
       </c>
       <c r="I17" t="n">
-        <v>77.03</v>
+        <v>72.64</v>
       </c>
       <c r="J17" t="n">
-        <v>42.7</v>
+        <v>44.4</v>
       </c>
       <c r="K17" t="n">
-        <v>43.9</v>
+        <v>47.3</v>
       </c>
       <c r="L17" t="n">
-        <v>39.9</v>
+        <v>43.8</v>
       </c>
       <c r="M17" t="n">
-        <v>40.8</v>
+        <v>46.5</v>
       </c>
       <c r="N17" t="n">
-        <v>38.49</v>
+        <v>39.01</v>
       </c>
       <c r="O17" t="n">
-        <v>39.14</v>
+        <v>40.21</v>
       </c>
       <c r="P17" t="n">
-        <v>37.64</v>
+        <v>38.85</v>
       </c>
       <c r="Q17" t="n">
-        <v>37.78</v>
+        <v>39.95</v>
       </c>
       <c r="R17" t="n">
-        <v>-0.0987</v>
+        <v>-13.9863</v>
       </c>
       <c r="S17" t="n">
-        <v>16.3238</v>
+        <v>-5.4056</v>
       </c>
       <c r="T17" t="n">
-        <v>5.9459</v>
+        <v>-15.0424</v>
       </c>
       <c r="U17" t="n">
-        <v>0.9039</v>
+        <v>-5.6991</v>
       </c>
       <c r="V17" t="n">
-        <v>6.6454</v>
+        <v>-0.11</v>
       </c>
       <c r="W17" t="n">
-        <v>5.017</v>
+        <v>-4.9463</v>
       </c>
       <c r="X17" t="n">
-        <v>0.2457</v>
+        <v>13.9706</v>
       </c>
       <c r="Y17" t="n">
-        <v>-15</v>
+        <v>3.3333</v>
       </c>
       <c r="Z17" t="n">
-        <v>-9.5344</v>
+        <v>11.5108</v>
       </c>
       <c r="AA17" t="n">
-        <v>-0.8399</v>
+        <v>5.7438</v>
       </c>
       <c r="AB17" t="n">
-        <v>-6.4388</v>
+        <v>-0.3244</v>
       </c>
       <c r="AC17" t="n">
-        <v>-5.4318</v>
+        <v>4.3626</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>174.61</v>
+        <v>187.69</v>
       </c>
       <c r="C18" t="n">
-        <v>177.67</v>
+        <v>188.43</v>
       </c>
       <c r="D18" t="n">
-        <v>161.55</v>
+        <v>170.26</v>
       </c>
       <c r="E18" t="n">
-        <v>165.37</v>
+        <v>176.66</v>
       </c>
       <c r="F18" t="n">
-        <v>74.54000000000001</v>
+        <v>75.2</v>
       </c>
       <c r="G18" t="n">
-        <v>74.84999999999999</v>
+        <v>75.84999999999999</v>
       </c>
       <c r="H18" t="n">
-        <v>72.09</v>
+        <v>73.41</v>
       </c>
       <c r="I18" t="n">
-        <v>72.64</v>
+        <v>75.02</v>
       </c>
       <c r="J18" t="n">
-        <v>44.4</v>
+        <v>39.7</v>
       </c>
       <c r="K18" t="n">
-        <v>47.3</v>
+        <v>45</v>
       </c>
       <c r="L18" t="n">
-        <v>43.8</v>
+        <v>39.7</v>
       </c>
       <c r="M18" t="n">
-        <v>46.5</v>
+        <v>42.8</v>
       </c>
       <c r="N18" t="n">
-        <v>39.01</v>
+        <v>38.54</v>
       </c>
       <c r="O18" t="n">
-        <v>40.21</v>
+        <v>39.53</v>
       </c>
       <c r="P18" t="n">
-        <v>38.85</v>
+        <v>38.19</v>
       </c>
       <c r="Q18" t="n">
-        <v>39.95</v>
+        <v>38.63</v>
       </c>
       <c r="R18" t="n">
-        <v>-13.9863</v>
+        <v>6.8271</v>
       </c>
       <c r="S18" t="n">
-        <v>-5.4056</v>
+        <v>-8.204700000000001</v>
       </c>
       <c r="T18" t="n">
-        <v>-15.0424</v>
+        <v>6.8853</v>
       </c>
       <c r="U18" t="n">
-        <v>-5.6991</v>
+        <v>3.2764</v>
       </c>
       <c r="V18" t="n">
-        <v>-0.11</v>
+        <v>-1.7291</v>
       </c>
       <c r="W18" t="n">
-        <v>-4.9463</v>
+        <v>3.8627</v>
       </c>
       <c r="X18" t="n">
-        <v>13.9706</v>
+        <v>-7.957</v>
       </c>
       <c r="Y18" t="n">
-        <v>3.3333</v>
+        <v>5.1597</v>
       </c>
       <c r="Z18" t="n">
-        <v>11.5108</v>
+        <v>-10.8333</v>
       </c>
       <c r="AA18" t="n">
-        <v>5.7438</v>
+        <v>-3.3041</v>
       </c>
       <c r="AB18" t="n">
-        <v>-0.3244</v>
+        <v>1.3911</v>
       </c>
       <c r="AC18" t="n">
-        <v>4.3626</v>
+        <v>-4.3338</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>187.69</v>
+        <v>183.77</v>
       </c>
       <c r="C19" t="n">
-        <v>188.43</v>
+        <v>184</v>
       </c>
       <c r="D19" t="n">
-        <v>170.26</v>
+        <v>150</v>
       </c>
       <c r="E19" t="n">
-        <v>176.66</v>
+        <v>165.55</v>
       </c>
       <c r="F19" t="n">
-        <v>75.2</v>
+        <v>76.29000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>75.84999999999999</v>
+        <v>76.47</v>
       </c>
       <c r="H19" t="n">
-        <v>73.41</v>
+        <v>72.06</v>
       </c>
       <c r="I19" t="n">
-        <v>75.02</v>
+        <v>74.44</v>
       </c>
       <c r="J19" t="n">
-        <v>39.7</v>
+        <v>41.23</v>
       </c>
       <c r="K19" t="n">
-        <v>45</v>
+        <v>49.69</v>
       </c>
       <c r="L19" t="n">
-        <v>39.7</v>
+        <v>41.16</v>
       </c>
       <c r="M19" t="n">
-        <v>42.8</v>
+        <v>45.98</v>
       </c>
       <c r="N19" t="n">
-        <v>38.54</v>
+        <v>37.98</v>
       </c>
       <c r="O19" t="n">
-        <v>39.53</v>
+        <v>40.17</v>
       </c>
       <c r="P19" t="n">
-        <v>38.19</v>
+        <v>37.89</v>
       </c>
       <c r="Q19" t="n">
-        <v>38.63</v>
+        <v>38.94</v>
       </c>
       <c r="R19" t="n">
-        <v>6.8271</v>
+        <v>-6.2889</v>
       </c>
       <c r="S19" t="n">
-        <v>-8.204700000000001</v>
+        <v>-13.8926</v>
       </c>
       <c r="T19" t="n">
-        <v>6.8853</v>
+        <v>-5.3026</v>
       </c>
       <c r="U19" t="n">
-        <v>3.2764</v>
+        <v>-0.7731</v>
       </c>
       <c r="V19" t="n">
-        <v>-1.7291</v>
+        <v>-3.3623</v>
       </c>
       <c r="W19" t="n">
-        <v>3.8627</v>
+        <v>2.3652</v>
       </c>
       <c r="X19" t="n">
-        <v>-7.957</v>
+        <v>7.4299</v>
       </c>
       <c r="Y19" t="n">
-        <v>5.1597</v>
+        <v>12.6961</v>
       </c>
       <c r="Z19" t="n">
-        <v>-10.8333</v>
+        <v>2.1778</v>
       </c>
       <c r="AA19" t="n">
-        <v>-3.3041</v>
+        <v>0.8025</v>
       </c>
       <c r="AB19" t="n">
-        <v>1.3911</v>
+        <v>3.0704</v>
       </c>
       <c r="AC19" t="n">
-        <v>-4.3338</v>
+        <v>-2.8443</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>183.77</v>
+        <v>150.44</v>
       </c>
       <c r="C20" t="n">
-        <v>184</v>
+        <v>155.83</v>
       </c>
       <c r="D20" t="n">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="E20" t="n">
-        <v>165.55</v>
+        <v>142.48</v>
       </c>
       <c r="F20" t="n">
-        <v>76.29000000000001</v>
+        <v>72.61</v>
       </c>
       <c r="G20" t="n">
-        <v>76.47</v>
+        <v>73.12</v>
       </c>
       <c r="H20" t="n">
-        <v>72.06</v>
+        <v>69.69</v>
       </c>
       <c r="I20" t="n">
-        <v>74.44</v>
+        <v>70.73999999999999</v>
       </c>
       <c r="J20" t="n">
-        <v>41.23</v>
+        <v>49.77</v>
       </c>
       <c r="K20" t="n">
-        <v>49.69</v>
+        <v>53.34</v>
       </c>
       <c r="L20" t="n">
-        <v>41.16</v>
+        <v>48.31</v>
       </c>
       <c r="M20" t="n">
-        <v>45.98</v>
+        <v>52.02</v>
       </c>
       <c r="N20" t="n">
-        <v>37.98</v>
+        <v>39.9</v>
       </c>
       <c r="O20" t="n">
-        <v>40.17</v>
+        <v>41.44</v>
       </c>
       <c r="P20" t="n">
-        <v>37.89</v>
+        <v>39.65</v>
       </c>
       <c r="Q20" t="n">
-        <v>38.94</v>
+        <v>40.89</v>
       </c>
       <c r="R20" t="n">
-        <v>-6.2889</v>
+        <v>-13.9354</v>
       </c>
       <c r="S20" t="n">
-        <v>-13.8926</v>
+        <v>-13.8417</v>
       </c>
       <c r="T20" t="n">
-        <v>-5.3026</v>
+        <v>-25.9652</v>
       </c>
       <c r="U20" t="n">
-        <v>-0.7731</v>
+        <v>-4.9704</v>
       </c>
       <c r="V20" t="n">
-        <v>-3.3623</v>
+        <v>-2.6156</v>
       </c>
       <c r="W20" t="n">
-        <v>2.3652</v>
+        <v>-7.3356</v>
       </c>
       <c r="X20" t="n">
-        <v>7.4299</v>
+        <v>13.1361</v>
       </c>
       <c r="Y20" t="n">
-        <v>12.6961</v>
+        <v>11.871</v>
       </c>
       <c r="Z20" t="n">
-        <v>2.1778</v>
+        <v>27.8133</v>
       </c>
       <c r="AA20" t="n">
-        <v>0.8025</v>
+        <v>5.0077</v>
       </c>
       <c r="AB20" t="n">
-        <v>3.0704</v>
+        <v>2.3529</v>
       </c>
       <c r="AC20" t="n">
-        <v>-2.8443</v>
+        <v>7.3228</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>150.44</v>
+        <v>124.73</v>
       </c>
       <c r="C21" t="n">
-        <v>155.81</v>
+        <v>144.3999</v>
       </c>
       <c r="D21" t="n">
-        <v>138</v>
+        <v>116.47</v>
       </c>
       <c r="E21" t="n">
-        <v>142.48</v>
+        <v>135.47</v>
       </c>
       <c r="F21" t="n">
-        <v>72.59999999999999</v>
+        <v>66.38</v>
       </c>
       <c r="G21" t="n">
-        <v>73.11669999999999</v>
+        <v>69.55500000000001</v>
       </c>
       <c r="H21" t="n">
-        <v>69.69</v>
+        <v>64.91</v>
       </c>
       <c r="I21" t="n">
-        <v>70.73999999999999</v>
+        <v>67.53</v>
       </c>
       <c r="J21" t="n">
-        <v>49.77</v>
+        <v>58.59</v>
       </c>
       <c r="K21" t="n">
-        <v>53.3375</v>
+        <v>61.5932</v>
       </c>
       <c r="L21" t="n">
-        <v>48.31</v>
+        <v>51.34</v>
       </c>
       <c r="M21" t="n">
-        <v>52.02</v>
+        <v>54.85</v>
       </c>
       <c r="N21" t="n">
-        <v>39.905</v>
+        <v>43.43</v>
       </c>
       <c r="O21" t="n">
-        <v>41.4378</v>
+        <v>44.2714</v>
       </c>
       <c r="P21" t="n">
-        <v>39.645</v>
+        <v>41.585</v>
       </c>
       <c r="Q21" t="n">
-        <v>40.89</v>
+        <v>42.79</v>
       </c>
       <c r="R21" t="n">
-        <v>-13.9354</v>
+        <v>-4.92</v>
       </c>
       <c r="S21" t="n">
-        <v>-13.8417</v>
+        <v>-23.316</v>
       </c>
       <c r="T21" t="n">
-        <v>-25.9652</v>
+        <v>-29.5381</v>
       </c>
       <c r="U21" t="n">
-        <v>-4.9704</v>
+        <v>-4.5377</v>
       </c>
       <c r="V21" t="n">
-        <v>-2.6156</v>
+        <v>-9.984</v>
       </c>
       <c r="W21" t="n">
-        <v>-7.3356</v>
+        <v>-12.3329</v>
       </c>
       <c r="X21" t="n">
-        <v>13.1361</v>
+        <v>5.4402</v>
       </c>
       <c r="Y21" t="n">
-        <v>11.871</v>
+        <v>28.1542</v>
       </c>
       <c r="Z21" t="n">
-        <v>27.8133</v>
+        <v>34.4363</v>
       </c>
       <c r="AA21" t="n">
-        <v>5.0077</v>
+        <v>4.6466</v>
       </c>
       <c r="AB21" t="n">
-        <v>2.3529</v>
+        <v>10.7688</v>
       </c>
       <c r="AC21" t="n">
-        <v>7.3228</v>
+        <v>13.261</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-07-20 23:00
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1713 +568,1713 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>266.04</v>
+        <v>299.26</v>
       </c>
       <c r="C2" t="n">
-        <v>286.15</v>
+        <v>302</v>
       </c>
       <c r="D2" t="n">
-        <v>265</v>
+        <v>286.24</v>
       </c>
       <c r="E2" t="n">
-        <v>279.29</v>
+        <v>300.77</v>
       </c>
       <c r="F2" t="n">
-        <v>81.9114</v>
+        <v>83.7572</v>
       </c>
       <c r="G2" t="n">
-        <v>83.408</v>
+        <v>84.9145</v>
       </c>
       <c r="H2" t="n">
-        <v>80.4448</v>
+        <v>81.203</v>
       </c>
       <c r="I2" t="n">
-        <v>82.67959999999999</v>
+        <v>82.3903</v>
       </c>
       <c r="J2" t="n">
-        <v>38.1555</v>
+        <v>32.9165</v>
       </c>
       <c r="K2" t="n">
-        <v>38.2544</v>
+        <v>34.4981</v>
       </c>
       <c r="L2" t="n">
-        <v>34.1027</v>
+        <v>32.5212</v>
       </c>
       <c r="M2" t="n">
-        <v>35.4866</v>
+        <v>32.62</v>
       </c>
       <c r="N2" t="n">
-        <v>36.6149</v>
+        <v>35.7389</v>
       </c>
       <c r="O2" t="n">
-        <v>37.3531</v>
+        <v>36.8511</v>
       </c>
       <c r="P2" t="n">
-        <v>35.857</v>
+        <v>35.2369</v>
       </c>
       <c r="Q2" t="n">
-        <v>36.1719</v>
+        <v>36.3491</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>299.26</v>
+        <v>236</v>
       </c>
       <c r="C3" t="n">
-        <v>302</v>
+        <v>252.98</v>
       </c>
       <c r="D3" t="n">
-        <v>286.24</v>
+        <v>223</v>
       </c>
       <c r="E3" t="n">
-        <v>300.77</v>
+        <v>231.42</v>
       </c>
       <c r="F3" t="n">
-        <v>83.7572</v>
+        <v>74.9474</v>
       </c>
       <c r="G3" t="n">
-        <v>84.9145</v>
+        <v>77.56140000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>81.203</v>
+        <v>73.7402</v>
       </c>
       <c r="I3" t="n">
-        <v>82.3903</v>
+        <v>74.26900000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>32.9165</v>
+        <v>39.9</v>
       </c>
       <c r="K3" t="n">
-        <v>34.4981</v>
+        <v>41.3</v>
       </c>
       <c r="L3" t="n">
-        <v>32.5212</v>
+        <v>38</v>
       </c>
       <c r="M3" t="n">
-        <v>32.62</v>
+        <v>40.4</v>
       </c>
       <c r="N3" t="n">
-        <v>35.7389</v>
+        <v>39.6267</v>
       </c>
       <c r="O3" t="n">
-        <v>36.8511</v>
+        <v>40.1582</v>
       </c>
       <c r="P3" t="n">
-        <v>35.2369</v>
+        <v>38.4653</v>
       </c>
       <c r="Q3" t="n">
-        <v>36.3491</v>
+        <v>39.922</v>
       </c>
       <c r="R3" t="n">
-        <v>7.6909</v>
+        <v>-23.0575</v>
       </c>
       <c r="U3" t="n">
-        <v>-0.3499</v>
+        <v>-9.857100000000001</v>
       </c>
       <c r="X3" t="n">
-        <v>-8.077999999999999</v>
+        <v>23.8504</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.4899</v>
+        <v>9.8294</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>236</v>
+        <v>233.11</v>
       </c>
       <c r="C4" t="n">
-        <v>252.98</v>
+        <v>237</v>
       </c>
       <c r="D4" t="n">
-        <v>223</v>
+        <v>211.13</v>
       </c>
       <c r="E4" t="n">
-        <v>231.42</v>
+        <v>229.57</v>
       </c>
       <c r="F4" t="n">
-        <v>74.9474</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>77.56140000000001</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>73.7402</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="I4" t="n">
-        <v>74.26900000000001</v>
+        <v>73.3</v>
       </c>
       <c r="J4" t="n">
-        <v>39.9</v>
+        <v>40</v>
       </c>
       <c r="K4" t="n">
-        <v>41.3</v>
+        <v>43.9</v>
       </c>
       <c r="L4" t="n">
-        <v>38</v>
+        <v>39.2</v>
       </c>
       <c r="M4" t="n">
-        <v>40.4</v>
+        <v>40.8</v>
       </c>
       <c r="N4" t="n">
-        <v>39.6267</v>
+        <v>39.66</v>
       </c>
       <c r="O4" t="n">
-        <v>40.1582</v>
+        <v>41.49</v>
       </c>
       <c r="P4" t="n">
-        <v>38.4653</v>
+        <v>38.9</v>
       </c>
       <c r="Q4" t="n">
-        <v>39.922</v>
+        <v>40.45</v>
       </c>
       <c r="R4" t="n">
-        <v>-23.0575</v>
+        <v>-0.7994</v>
       </c>
       <c r="U4" t="n">
-        <v>-9.857100000000001</v>
+        <v>-1.3047</v>
       </c>
       <c r="X4" t="n">
-        <v>23.8504</v>
+        <v>0.9901</v>
       </c>
       <c r="AA4" t="n">
-        <v>9.8294</v>
+        <v>1.3226</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>233.11</v>
+        <v>268.05</v>
       </c>
       <c r="C5" t="n">
-        <v>237</v>
+        <v>268.4</v>
       </c>
       <c r="D5" t="n">
-        <v>211.13</v>
+        <v>225.74</v>
       </c>
       <c r="E5" t="n">
-        <v>229.57</v>
+        <v>252.61</v>
       </c>
       <c r="F5" t="n">
-        <v>74.79000000000001</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>76.18000000000001</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>71.34999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I5" t="n">
-        <v>73.3</v>
+        <v>74.95</v>
       </c>
       <c r="J5" t="n">
-        <v>40</v>
+        <v>33.8</v>
       </c>
       <c r="K5" t="n">
-        <v>43.9</v>
+        <v>41.5</v>
       </c>
       <c r="L5" t="n">
-        <v>39.2</v>
+        <v>33.7</v>
       </c>
       <c r="M5" t="n">
-        <v>40.8</v>
+        <v>36.3</v>
       </c>
       <c r="N5" t="n">
-        <v>39.66</v>
+        <v>37.87</v>
       </c>
       <c r="O5" t="n">
-        <v>41.49</v>
+        <v>41.37</v>
       </c>
       <c r="P5" t="n">
-        <v>38.9</v>
+        <v>37.71</v>
       </c>
       <c r="Q5" t="n">
-        <v>40.45</v>
+        <v>39.47</v>
       </c>
       <c r="R5" t="n">
-        <v>-0.7994</v>
+        <v>10.0362</v>
       </c>
       <c r="S5" t="n">
-        <v>-17.8023</v>
+        <v>-16.0122</v>
       </c>
       <c r="U5" t="n">
-        <v>-1.3047</v>
+        <v>2.251</v>
       </c>
       <c r="V5" t="n">
-        <v>-11.3445</v>
+        <v>-9.0306</v>
       </c>
       <c r="X5" t="n">
-        <v>0.9901</v>
+        <v>-11.0294</v>
       </c>
       <c r="Y5" t="n">
-        <v>14.973</v>
+        <v>11.2814</v>
       </c>
       <c r="AA5" t="n">
-        <v>1.3226</v>
+        <v>-2.4227</v>
       </c>
       <c r="AB5" t="n">
-        <v>11.8271</v>
+        <v>8.585900000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>268.05</v>
+        <v>226.24</v>
       </c>
       <c r="C6" t="n">
-        <v>268.4</v>
+        <v>231.25</v>
       </c>
       <c r="D6" t="n">
-        <v>225.74</v>
+        <v>212.1</v>
       </c>
       <c r="E6" t="n">
-        <v>252.61</v>
+        <v>215.6</v>
       </c>
       <c r="F6" t="n">
-        <v>77.95999999999999</v>
+        <v>72.09</v>
       </c>
       <c r="G6" t="n">
-        <v>78.23999999999999</v>
+        <v>74.69</v>
       </c>
       <c r="H6" t="n">
-        <v>71.59999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="I6" t="n">
-        <v>74.95</v>
+        <v>71.83</v>
       </c>
       <c r="J6" t="n">
-        <v>33.8</v>
+        <v>40.4</v>
       </c>
       <c r="K6" t="n">
-        <v>41.5</v>
+        <v>42.5</v>
       </c>
       <c r="L6" t="n">
-        <v>33.7</v>
+        <v>39.5</v>
       </c>
       <c r="M6" t="n">
-        <v>36.3</v>
+        <v>42.4</v>
       </c>
       <c r="N6" t="n">
-        <v>37.87</v>
+        <v>41.08</v>
       </c>
       <c r="O6" t="n">
-        <v>41.37</v>
+        <v>41.79</v>
       </c>
       <c r="P6" t="n">
-        <v>37.71</v>
+        <v>39.69</v>
       </c>
       <c r="Q6" t="n">
-        <v>39.47</v>
+        <v>41.31</v>
       </c>
       <c r="R6" t="n">
-        <v>10.0362</v>
+        <v>-14.651</v>
       </c>
       <c r="S6" t="n">
-        <v>-16.0122</v>
+        <v>-6.8361</v>
       </c>
       <c r="U6" t="n">
-        <v>2.251</v>
+        <v>-4.1628</v>
       </c>
       <c r="V6" t="n">
-        <v>-9.0306</v>
+        <v>-3.284</v>
       </c>
       <c r="X6" t="n">
-        <v>-11.0294</v>
+        <v>16.8044</v>
       </c>
       <c r="Y6" t="n">
-        <v>11.2814</v>
+        <v>4.9505</v>
       </c>
       <c r="AA6" t="n">
-        <v>-2.4227</v>
+        <v>4.6618</v>
       </c>
       <c r="AB6" t="n">
-        <v>8.585900000000001</v>
+        <v>3.4768</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>226.24</v>
+        <v>216.36</v>
       </c>
       <c r="C7" t="n">
-        <v>231.25</v>
+        <v>238.65</v>
       </c>
       <c r="D7" t="n">
-        <v>212.1</v>
+        <v>192.3</v>
       </c>
       <c r="E7" t="n">
-        <v>215.6</v>
+        <v>236.52</v>
       </c>
       <c r="F7" t="n">
-        <v>72.09</v>
+        <v>74.12</v>
       </c>
       <c r="G7" t="n">
-        <v>74.69</v>
+        <v>77.38</v>
       </c>
       <c r="H7" t="n">
-        <v>70.72</v>
+        <v>71.45</v>
       </c>
       <c r="I7" t="n">
-        <v>71.83</v>
+        <v>77.19</v>
       </c>
       <c r="J7" t="n">
-        <v>40.4</v>
+        <v>41.6</v>
       </c>
       <c r="K7" t="n">
-        <v>42.5</v>
+        <v>46.3</v>
       </c>
       <c r="L7" t="n">
-        <v>39.5</v>
+        <v>37</v>
       </c>
       <c r="M7" t="n">
-        <v>42.4</v>
+        <v>37.2</v>
       </c>
       <c r="N7" t="n">
-        <v>41.08</v>
+        <v>39.91</v>
       </c>
       <c r="O7" t="n">
-        <v>41.79</v>
+        <v>41.43</v>
       </c>
       <c r="P7" t="n">
-        <v>39.69</v>
+        <v>38.08</v>
       </c>
       <c r="Q7" t="n">
-        <v>41.31</v>
+        <v>38.16</v>
       </c>
       <c r="R7" t="n">
-        <v>-14.651</v>
+        <v>9.703200000000001</v>
       </c>
       <c r="S7" t="n">
-        <v>-6.8361</v>
+        <v>3.0274</v>
       </c>
       <c r="T7" t="n">
-        <v>-22.8043</v>
+        <v>-21.3618</v>
       </c>
       <c r="U7" t="n">
-        <v>-4.1628</v>
+        <v>7.4621</v>
       </c>
       <c r="V7" t="n">
-        <v>-3.284</v>
+        <v>5.307</v>
       </c>
       <c r="W7" t="n">
-        <v>-13.1225</v>
+        <v>-6.3118</v>
       </c>
       <c r="X7" t="n">
-        <v>16.8044</v>
+        <v>-12.2642</v>
       </c>
       <c r="Y7" t="n">
-        <v>4.9505</v>
+        <v>-8.823499999999999</v>
       </c>
       <c r="Z7" t="n">
-        <v>19.4817</v>
+        <v>14.0405</v>
       </c>
       <c r="AA7" t="n">
-        <v>4.6618</v>
+        <v>-7.6253</v>
       </c>
       <c r="AB7" t="n">
-        <v>3.4768</v>
+        <v>-5.6613</v>
       </c>
       <c r="AC7" t="n">
-        <v>14.2047</v>
+        <v>4.982</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>216.36</v>
+        <v>241.45</v>
       </c>
       <c r="C8" t="n">
-        <v>238.65</v>
+        <v>272</v>
       </c>
       <c r="D8" t="n">
-        <v>192.3</v>
+        <v>240.59</v>
       </c>
       <c r="E8" t="n">
-        <v>236.52</v>
+        <v>266.71</v>
       </c>
       <c r="F8" t="n">
-        <v>74.12</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>77.38</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="H8" t="n">
-        <v>71.45</v>
+        <v>77.15000000000001</v>
       </c>
       <c r="I8" t="n">
-        <v>77.19</v>
+        <v>81</v>
       </c>
       <c r="J8" t="n">
-        <v>41.6</v>
+        <v>36.6</v>
       </c>
       <c r="K8" t="n">
-        <v>46.3</v>
+        <v>36.8</v>
       </c>
       <c r="L8" t="n">
-        <v>37</v>
+        <v>31.7</v>
       </c>
       <c r="M8" t="n">
-        <v>37.2</v>
+        <v>32.4</v>
       </c>
       <c r="N8" t="n">
-        <v>39.91</v>
+        <v>38.16</v>
       </c>
       <c r="O8" t="n">
-        <v>41.43</v>
+        <v>38.2</v>
       </c>
       <c r="P8" t="n">
-        <v>38.08</v>
+        <v>36.03</v>
       </c>
       <c r="Q8" t="n">
-        <v>38.16</v>
+        <v>36.31</v>
       </c>
       <c r="R8" t="n">
-        <v>9.703200000000001</v>
+        <v>12.7642</v>
       </c>
       <c r="S8" t="n">
-        <v>3.0274</v>
+        <v>5.5817</v>
       </c>
       <c r="T8" t="n">
-        <v>-21.3618</v>
+        <v>15.2493</v>
       </c>
       <c r="U8" t="n">
-        <v>7.4621</v>
+        <v>4.9359</v>
       </c>
       <c r="V8" t="n">
-        <v>5.307</v>
+        <v>8.071999999999999</v>
       </c>
       <c r="W8" t="n">
-        <v>-6.3118</v>
+        <v>9.063000000000001</v>
       </c>
       <c r="X8" t="n">
-        <v>-12.2642</v>
+        <v>-12.9032</v>
       </c>
       <c r="Y8" t="n">
-        <v>-8.823499999999999</v>
+        <v>-10.7438</v>
       </c>
       <c r="Z8" t="n">
-        <v>14.0405</v>
+        <v>-19.802</v>
       </c>
       <c r="AA8" t="n">
-        <v>-7.6253</v>
+        <v>-4.848</v>
       </c>
       <c r="AB8" t="n">
-        <v>-5.6613</v>
+        <v>-8.0061</v>
       </c>
       <c r="AC8" t="n">
-        <v>4.982</v>
+        <v>-9.047599999999999</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>241.45</v>
+        <v>237.79</v>
       </c>
       <c r="C9" t="n">
-        <v>272</v>
+        <v>246.47</v>
       </c>
       <c r="D9" t="n">
-        <v>240.59</v>
+        <v>215.38</v>
       </c>
       <c r="E9" t="n">
-        <v>266.71</v>
+        <v>217.55</v>
       </c>
       <c r="F9" t="n">
-        <v>77.23999999999999</v>
+        <v>78.72</v>
       </c>
       <c r="G9" t="n">
-        <v>81.54000000000001</v>
+        <v>79.64</v>
       </c>
       <c r="H9" t="n">
-        <v>77.15000000000001</v>
+        <v>77.23</v>
       </c>
       <c r="I9" t="n">
-        <v>81</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>36.6</v>
+        <v>35.9</v>
       </c>
       <c r="K9" t="n">
-        <v>36.8</v>
+        <v>38.9</v>
       </c>
       <c r="L9" t="n">
-        <v>31.7</v>
+        <v>35.1</v>
       </c>
       <c r="M9" t="n">
-        <v>32.4</v>
+        <v>38.6</v>
       </c>
       <c r="N9" t="n">
-        <v>38.16</v>
+        <v>37.31</v>
       </c>
       <c r="O9" t="n">
-        <v>38.2</v>
+        <v>37.98</v>
       </c>
       <c r="P9" t="n">
-        <v>36.03</v>
+        <v>36.9</v>
       </c>
       <c r="Q9" t="n">
-        <v>36.31</v>
+        <v>37.88</v>
       </c>
       <c r="R9" t="n">
-        <v>12.7642</v>
+        <v>-18.432</v>
       </c>
       <c r="S9" t="n">
-        <v>5.5817</v>
+        <v>0.9045</v>
       </c>
       <c r="T9" t="n">
-        <v>15.2493</v>
+        <v>-5.2359</v>
       </c>
       <c r="U9" t="n">
-        <v>4.9359</v>
+        <v>-4.3704</v>
       </c>
       <c r="V9" t="n">
-        <v>8.071999999999999</v>
+        <v>7.838</v>
       </c>
       <c r="W9" t="n">
-        <v>9.063000000000001</v>
+        <v>5.6753</v>
       </c>
       <c r="X9" t="n">
-        <v>-12.9032</v>
+        <v>19.1358</v>
       </c>
       <c r="Y9" t="n">
-        <v>-10.7438</v>
+        <v>-8.962300000000001</v>
       </c>
       <c r="Z9" t="n">
-        <v>-19.802</v>
+        <v>-5.3922</v>
       </c>
       <c r="AA9" t="n">
-        <v>-4.848</v>
+        <v>4.3239</v>
       </c>
       <c r="AB9" t="n">
-        <v>-8.0061</v>
+        <v>-8.303100000000001</v>
       </c>
       <c r="AC9" t="n">
-        <v>-9.047599999999999</v>
+        <v>-6.3535</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>237.79</v>
+        <v>219.23</v>
       </c>
       <c r="C10" t="n">
-        <v>246.47</v>
+        <v>226.13</v>
       </c>
       <c r="D10" t="n">
-        <v>215.38</v>
+        <v>168.88</v>
       </c>
       <c r="E10" t="n">
-        <v>217.55</v>
+        <v>181.47</v>
       </c>
       <c r="F10" t="n">
-        <v>78.72</v>
+        <v>77.45</v>
       </c>
       <c r="G10" t="n">
-        <v>79.64</v>
+        <v>79.14</v>
       </c>
       <c r="H10" t="n">
-        <v>77.23</v>
+        <v>71.72</v>
       </c>
       <c r="I10" t="n">
-        <v>77.45999999999999</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>35.9</v>
+        <v>38.4</v>
       </c>
       <c r="K10" t="n">
-        <v>38.9</v>
+        <v>47.4</v>
       </c>
       <c r="L10" t="n">
-        <v>35.1</v>
+        <v>37.1</v>
       </c>
       <c r="M10" t="n">
-        <v>38.6</v>
+        <v>45.1</v>
       </c>
       <c r="N10" t="n">
-        <v>37.31</v>
+        <v>37.91</v>
       </c>
       <c r="O10" t="n">
-        <v>37.98</v>
+        <v>40.72</v>
       </c>
       <c r="P10" t="n">
-        <v>36.9</v>
+        <v>37.08</v>
       </c>
       <c r="Q10" t="n">
-        <v>37.88</v>
+        <v>39.95</v>
       </c>
       <c r="R10" t="n">
-        <v>-18.432</v>
+        <v>-16.5847</v>
       </c>
       <c r="S10" t="n">
-        <v>0.9045</v>
+        <v>-23.275</v>
       </c>
       <c r="T10" t="n">
-        <v>-5.2359</v>
+        <v>-28.162</v>
       </c>
       <c r="U10" t="n">
-        <v>-4.3704</v>
+        <v>-5.306</v>
       </c>
       <c r="V10" t="n">
-        <v>7.838</v>
+        <v>-4.9747</v>
       </c>
       <c r="W10" t="n">
-        <v>5.6753</v>
+        <v>-2.1348</v>
       </c>
       <c r="X10" t="n">
-        <v>19.1358</v>
+        <v>16.8394</v>
       </c>
       <c r="Y10" t="n">
-        <v>-8.962300000000001</v>
+        <v>21.2366</v>
       </c>
       <c r="Z10" t="n">
-        <v>-5.3922</v>
+        <v>24.2424</v>
       </c>
       <c r="AA10" t="n">
-        <v>4.3239</v>
+        <v>5.4646</v>
       </c>
       <c r="AB10" t="n">
-        <v>-8.303100000000001</v>
+        <v>4.6908</v>
       </c>
       <c r="AC10" t="n">
-        <v>-6.3535</v>
+        <v>1.2161</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>219.23</v>
+        <v>197.21</v>
       </c>
       <c r="C11" t="n">
-        <v>226.13</v>
+        <v>210.8</v>
       </c>
       <c r="D11" t="n">
-        <v>168.88</v>
+        <v>194.22</v>
       </c>
       <c r="E11" t="n">
-        <v>181.47</v>
+        <v>194.65</v>
       </c>
       <c r="F11" t="n">
+        <v>75.54000000000001</v>
+      </c>
+      <c r="G11" t="n">
         <v>77.45</v>
       </c>
-      <c r="G11" t="n">
-        <v>79.14</v>
-      </c>
       <c r="H11" t="n">
-        <v>71.72</v>
+        <v>75.11</v>
       </c>
       <c r="I11" t="n">
-        <v>73.34999999999999</v>
+        <v>76.42</v>
       </c>
       <c r="J11" t="n">
-        <v>38.4</v>
+        <v>41.1</v>
       </c>
       <c r="K11" t="n">
-        <v>47.4</v>
+        <v>41.8</v>
       </c>
       <c r="L11" t="n">
-        <v>37.1</v>
+        <v>37.7</v>
       </c>
       <c r="M11" t="n">
-        <v>45.1</v>
+        <v>41.7</v>
       </c>
       <c r="N11" t="n">
-        <v>37.91</v>
+        <v>38.75</v>
       </c>
       <c r="O11" t="n">
-        <v>40.72</v>
+        <v>38.98</v>
       </c>
       <c r="P11" t="n">
-        <v>37.08</v>
+        <v>37.71</v>
       </c>
       <c r="Q11" t="n">
-        <v>39.95</v>
+        <v>38.28</v>
       </c>
       <c r="R11" t="n">
-        <v>-16.5847</v>
+        <v>7.2629</v>
       </c>
       <c r="S11" t="n">
-        <v>-23.275</v>
+        <v>-27.0181</v>
       </c>
       <c r="T11" t="n">
-        <v>-28.162</v>
+        <v>-9.7171</v>
       </c>
       <c r="U11" t="n">
-        <v>-5.306</v>
+        <v>4.1854</v>
       </c>
       <c r="V11" t="n">
-        <v>-4.9747</v>
+        <v>-5.6543</v>
       </c>
       <c r="W11" t="n">
-        <v>-2.1348</v>
+        <v>6.3901</v>
       </c>
       <c r="X11" t="n">
-        <v>16.8394</v>
+        <v>-7.5388</v>
       </c>
       <c r="Y11" t="n">
-        <v>21.2366</v>
+        <v>28.7037</v>
       </c>
       <c r="Z11" t="n">
-        <v>24.2424</v>
+        <v>-1.6509</v>
       </c>
       <c r="AA11" t="n">
-        <v>5.4646</v>
+        <v>-4.1802</v>
       </c>
       <c r="AB11" t="n">
-        <v>4.6908</v>
+        <v>5.4255</v>
       </c>
       <c r="AC11" t="n">
-        <v>1.2161</v>
+        <v>-7.3348</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>197.21</v>
+        <v>165.4</v>
       </c>
       <c r="C12" t="n">
-        <v>210.8</v>
+        <v>171.88</v>
       </c>
       <c r="D12" t="n">
-        <v>194.22</v>
+        <v>150.08</v>
       </c>
       <c r="E12" t="n">
-        <v>194.65</v>
+        <v>165.28</v>
       </c>
       <c r="F12" t="n">
-        <v>75.54000000000001</v>
+        <v>73.7</v>
       </c>
       <c r="G12" t="n">
-        <v>77.45</v>
+        <v>74.39</v>
       </c>
       <c r="H12" t="n">
-        <v>75.11</v>
+        <v>70.76000000000001</v>
       </c>
       <c r="I12" t="n">
-        <v>76.42</v>
+        <v>72.23</v>
       </c>
       <c r="J12" t="n">
-        <v>41.1</v>
+        <v>48</v>
       </c>
       <c r="K12" t="n">
-        <v>41.8</v>
+        <v>51.4</v>
       </c>
       <c r="L12" t="n">
-        <v>37.7</v>
+        <v>46.6</v>
       </c>
       <c r="M12" t="n">
-        <v>41.7</v>
+        <v>48</v>
       </c>
       <c r="N12" t="n">
-        <v>38.75</v>
+        <v>39.64</v>
       </c>
       <c r="O12" t="n">
-        <v>38.98</v>
+        <v>41.11</v>
       </c>
       <c r="P12" t="n">
-        <v>37.71</v>
+        <v>39.29</v>
       </c>
       <c r="Q12" t="n">
-        <v>38.28</v>
+        <v>40.38</v>
       </c>
       <c r="R12" t="n">
-        <v>7.2629</v>
+        <v>-15.0886</v>
       </c>
       <c r="S12" t="n">
-        <v>-27.0181</v>
+        <v>-24.0267</v>
       </c>
       <c r="T12" t="n">
-        <v>-9.7171</v>
+        <v>-30.1201</v>
       </c>
       <c r="U12" t="n">
-        <v>4.1854</v>
+        <v>-5.4829</v>
       </c>
       <c r="V12" t="n">
-        <v>-5.6543</v>
+        <v>-6.7519</v>
       </c>
       <c r="W12" t="n">
-        <v>6.3901</v>
+        <v>-6.4257</v>
       </c>
       <c r="X12" t="n">
-        <v>-7.5388</v>
+        <v>15.1079</v>
       </c>
       <c r="Y12" t="n">
-        <v>28.7037</v>
+        <v>24.3523</v>
       </c>
       <c r="Z12" t="n">
-        <v>-1.6509</v>
+        <v>29.0323</v>
       </c>
       <c r="AA12" t="n">
-        <v>-4.1802</v>
+        <v>5.4859</v>
       </c>
       <c r="AB12" t="n">
-        <v>5.4255</v>
+        <v>6.5998</v>
       </c>
       <c r="AC12" t="n">
-        <v>-7.3348</v>
+        <v>5.8176</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>165.4</v>
+        <v>159.21</v>
       </c>
       <c r="C13" t="n">
-        <v>171.88</v>
+        <v>176.75</v>
       </c>
       <c r="D13" t="n">
-        <v>150.08</v>
+        <v>158.87</v>
       </c>
       <c r="E13" t="n">
-        <v>165.28</v>
+        <v>174.82</v>
       </c>
       <c r="F13" t="n">
-        <v>73.7</v>
+        <v>70.8</v>
       </c>
       <c r="G13" t="n">
-        <v>74.39</v>
+        <v>73.02</v>
       </c>
       <c r="H13" t="n">
-        <v>70.76000000000001</v>
+        <v>69.56999999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>72.23</v>
+        <v>72.72</v>
       </c>
       <c r="J13" t="n">
-        <v>48</v>
+        <v>49.8</v>
       </c>
       <c r="K13" t="n">
-        <v>51.4</v>
+        <v>49.9</v>
       </c>
       <c r="L13" t="n">
-        <v>46.6</v>
+        <v>44.6</v>
       </c>
       <c r="M13" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="N13" t="n">
-        <v>39.64</v>
+        <v>41.18</v>
       </c>
       <c r="O13" t="n">
-        <v>41.11</v>
+        <v>41.86</v>
       </c>
       <c r="P13" t="n">
-        <v>39.29</v>
+        <v>39.93</v>
       </c>
       <c r="Q13" t="n">
-        <v>40.38</v>
+        <v>40.08</v>
       </c>
       <c r="R13" t="n">
-        <v>-15.0886</v>
+        <v>5.772</v>
       </c>
       <c r="S13" t="n">
-        <v>-24.0267</v>
+        <v>-3.6645</v>
       </c>
       <c r="T13" t="n">
-        <v>-30.1201</v>
+        <v>-34.4532</v>
       </c>
       <c r="U13" t="n">
-        <v>-5.4829</v>
+        <v>0.6784</v>
       </c>
       <c r="V13" t="n">
-        <v>-6.7519</v>
+        <v>-0.8589</v>
       </c>
       <c r="W13" t="n">
-        <v>-6.4257</v>
+        <v>-10.2222</v>
       </c>
       <c r="X13" t="n">
-        <v>15.1079</v>
+        <v>-6.25</v>
       </c>
       <c r="Y13" t="n">
-        <v>24.3523</v>
+        <v>-0.2217</v>
       </c>
       <c r="Z13" t="n">
-        <v>29.0323</v>
+        <v>38.8889</v>
       </c>
       <c r="AA13" t="n">
-        <v>5.4859</v>
+        <v>-0.7429</v>
       </c>
       <c r="AB13" t="n">
-        <v>6.5998</v>
+        <v>0.3254</v>
       </c>
       <c r="AC13" t="n">
-        <v>5.8176</v>
+        <v>10.3828</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>159.21</v>
+        <v>199.81</v>
       </c>
       <c r="C14" t="n">
-        <v>176.75</v>
+        <v>204.55</v>
       </c>
       <c r="D14" t="n">
-        <v>158.87</v>
+        <v>189.46</v>
       </c>
       <c r="E14" t="n">
-        <v>174.82</v>
+        <v>192.45</v>
       </c>
       <c r="F14" t="n">
-        <v>70.8</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>73.02</v>
+        <v>76.69</v>
       </c>
       <c r="H14" t="n">
-        <v>69.56999999999999</v>
+        <v>73.89</v>
       </c>
       <c r="I14" t="n">
-        <v>72.72</v>
+        <v>76.34</v>
       </c>
       <c r="J14" t="n">
-        <v>49.8</v>
+        <v>38.7</v>
       </c>
       <c r="K14" t="n">
-        <v>49.9</v>
+        <v>41.2</v>
       </c>
       <c r="L14" t="n">
-        <v>44.6</v>
+        <v>37.5</v>
       </c>
       <c r="M14" t="n">
-        <v>45</v>
+        <v>40.7</v>
       </c>
       <c r="N14" t="n">
-        <v>41.18</v>
+        <v>38.93</v>
       </c>
       <c r="O14" t="n">
-        <v>41.86</v>
+        <v>39.47</v>
       </c>
       <c r="P14" t="n">
-        <v>39.93</v>
+        <v>37.93</v>
       </c>
       <c r="Q14" t="n">
-        <v>40.08</v>
+        <v>38.1</v>
       </c>
       <c r="R14" t="n">
-        <v>5.772</v>
+        <v>10.0847</v>
       </c>
       <c r="S14" t="n">
-        <v>-3.6645</v>
+        <v>-1.1302</v>
       </c>
       <c r="T14" t="n">
-        <v>-34.4532</v>
+        <v>-11.5376</v>
       </c>
       <c r="U14" t="n">
-        <v>0.6784</v>
+        <v>4.978</v>
       </c>
       <c r="V14" t="n">
-        <v>-0.8589</v>
+        <v>-0.1047</v>
       </c>
       <c r="W14" t="n">
-        <v>-10.2222</v>
+        <v>-1.4459</v>
       </c>
       <c r="X14" t="n">
-        <v>-6.25</v>
+        <v>-9.5556</v>
       </c>
       <c r="Y14" t="n">
-        <v>-0.2217</v>
+        <v>-2.3981</v>
       </c>
       <c r="Z14" t="n">
-        <v>38.8889</v>
+        <v>5.4404</v>
       </c>
       <c r="AA14" t="n">
-        <v>-0.7429</v>
+        <v>-4.9401</v>
       </c>
       <c r="AB14" t="n">
-        <v>0.3254</v>
+        <v>-0.4702</v>
       </c>
       <c r="AC14" t="n">
-        <v>10.3828</v>
+        <v>0.5808</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>199.81</v>
+        <v>182.4</v>
       </c>
       <c r="C15" t="n">
-        <v>204.55</v>
+        <v>195.94</v>
       </c>
       <c r="D15" t="n">
-        <v>189.46</v>
+        <v>176.8</v>
       </c>
       <c r="E15" t="n">
-        <v>192.45</v>
+        <v>192.26</v>
       </c>
       <c r="F15" t="n">
-        <v>74.84999999999999</v>
+        <v>75.53</v>
       </c>
       <c r="G15" t="n">
-        <v>76.69</v>
+        <v>77.31999999999999</v>
       </c>
       <c r="H15" t="n">
-        <v>73.89</v>
+        <v>74.33</v>
       </c>
       <c r="I15" t="n">
-        <v>76.34</v>
+        <v>77.03</v>
       </c>
       <c r="J15" t="n">
-        <v>38.7</v>
+        <v>42.7</v>
       </c>
       <c r="K15" t="n">
-        <v>41.2</v>
+        <v>43.9</v>
       </c>
       <c r="L15" t="n">
-        <v>37.5</v>
+        <v>39.9</v>
       </c>
       <c r="M15" t="n">
-        <v>40.7</v>
+        <v>40.8</v>
       </c>
       <c r="N15" t="n">
-        <v>38.93</v>
+        <v>38.49</v>
       </c>
       <c r="O15" t="n">
-        <v>39.47</v>
+        <v>39.14</v>
       </c>
       <c r="P15" t="n">
-        <v>37.93</v>
+        <v>37.64</v>
       </c>
       <c r="Q15" t="n">
-        <v>38.1</v>
+        <v>37.78</v>
       </c>
       <c r="R15" t="n">
-        <v>10.0847</v>
+        <v>-0.0987</v>
       </c>
       <c r="S15" t="n">
-        <v>-1.1302</v>
+        <v>16.3238</v>
       </c>
       <c r="T15" t="n">
-        <v>-11.5376</v>
+        <v>5.9459</v>
       </c>
       <c r="U15" t="n">
-        <v>4.978</v>
+        <v>0.9039</v>
       </c>
       <c r="V15" t="n">
-        <v>-0.1047</v>
+        <v>6.6454</v>
       </c>
       <c r="W15" t="n">
-        <v>-1.4459</v>
+        <v>5.017</v>
       </c>
       <c r="X15" t="n">
-        <v>-9.5556</v>
+        <v>0.2457</v>
       </c>
       <c r="Y15" t="n">
-        <v>-2.3981</v>
+        <v>-15</v>
       </c>
       <c r="Z15" t="n">
-        <v>5.4404</v>
+        <v>-9.5344</v>
       </c>
       <c r="AA15" t="n">
-        <v>-4.9401</v>
+        <v>-0.8399</v>
       </c>
       <c r="AB15" t="n">
-        <v>-0.4702</v>
+        <v>-6.4388</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.5808</v>
+        <v>-5.4318</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>182.4</v>
+        <v>174.61</v>
       </c>
       <c r="C16" t="n">
-        <v>195.94</v>
+        <v>177.67</v>
       </c>
       <c r="D16" t="n">
-        <v>176.8</v>
+        <v>161.55</v>
       </c>
       <c r="E16" t="n">
-        <v>192.26</v>
+        <v>165.37</v>
       </c>
       <c r="F16" t="n">
-        <v>75.53</v>
+        <v>74.54000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>77.31999999999999</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>74.33</v>
+        <v>72.09</v>
       </c>
       <c r="I16" t="n">
-        <v>77.03</v>
+        <v>72.64</v>
       </c>
       <c r="J16" t="n">
-        <v>42.7</v>
+        <v>44.4</v>
       </c>
       <c r="K16" t="n">
-        <v>43.9</v>
+        <v>47.3</v>
       </c>
       <c r="L16" t="n">
-        <v>39.9</v>
+        <v>43.8</v>
       </c>
       <c r="M16" t="n">
-        <v>40.8</v>
+        <v>46.5</v>
       </c>
       <c r="N16" t="n">
-        <v>38.49</v>
+        <v>39.01</v>
       </c>
       <c r="O16" t="n">
-        <v>39.14</v>
+        <v>40.21</v>
       </c>
       <c r="P16" t="n">
-        <v>37.64</v>
+        <v>38.85</v>
       </c>
       <c r="Q16" t="n">
-        <v>37.78</v>
+        <v>39.95</v>
       </c>
       <c r="R16" t="n">
-        <v>-0.0987</v>
+        <v>-13.9863</v>
       </c>
       <c r="S16" t="n">
-        <v>16.3238</v>
+        <v>-5.4056</v>
       </c>
       <c r="T16" t="n">
-        <v>5.9459</v>
+        <v>-15.0424</v>
       </c>
       <c r="U16" t="n">
-        <v>0.9039</v>
+        <v>-5.6991</v>
       </c>
       <c r="V16" t="n">
-        <v>6.6454</v>
+        <v>-0.11</v>
       </c>
       <c r="W16" t="n">
-        <v>5.017</v>
+        <v>-4.9463</v>
       </c>
       <c r="X16" t="n">
-        <v>0.2457</v>
+        <v>13.9706</v>
       </c>
       <c r="Y16" t="n">
-        <v>-15</v>
+        <v>3.3333</v>
       </c>
       <c r="Z16" t="n">
-        <v>-9.5344</v>
+        <v>11.5108</v>
       </c>
       <c r="AA16" t="n">
-        <v>-0.8399</v>
+        <v>5.7438</v>
       </c>
       <c r="AB16" t="n">
-        <v>-6.4388</v>
+        <v>-0.3244</v>
       </c>
       <c r="AC16" t="n">
-        <v>-5.4318</v>
+        <v>4.3626</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>174.61</v>
+        <v>187.69</v>
       </c>
       <c r="C17" t="n">
-        <v>177.67</v>
+        <v>188.43</v>
       </c>
       <c r="D17" t="n">
-        <v>161.55</v>
+        <v>170.26</v>
       </c>
       <c r="E17" t="n">
-        <v>165.37</v>
+        <v>176.66</v>
       </c>
       <c r="F17" t="n">
-        <v>74.54000000000001</v>
+        <v>75.2</v>
       </c>
       <c r="G17" t="n">
-        <v>74.84999999999999</v>
+        <v>75.84999999999999</v>
       </c>
       <c r="H17" t="n">
-        <v>72.09</v>
+        <v>73.41</v>
       </c>
       <c r="I17" t="n">
-        <v>72.64</v>
+        <v>75.02</v>
       </c>
       <c r="J17" t="n">
-        <v>44.4</v>
+        <v>39.7</v>
       </c>
       <c r="K17" t="n">
-        <v>47.3</v>
+        <v>45</v>
       </c>
       <c r="L17" t="n">
-        <v>43.8</v>
+        <v>39.7</v>
       </c>
       <c r="M17" t="n">
-        <v>46.5</v>
+        <v>42.8</v>
       </c>
       <c r="N17" t="n">
-        <v>39.01</v>
+        <v>38.54</v>
       </c>
       <c r="O17" t="n">
-        <v>40.21</v>
+        <v>39.53</v>
       </c>
       <c r="P17" t="n">
-        <v>38.85</v>
+        <v>38.19</v>
       </c>
       <c r="Q17" t="n">
-        <v>39.95</v>
+        <v>38.63</v>
       </c>
       <c r="R17" t="n">
-        <v>-13.9863</v>
+        <v>6.8271</v>
       </c>
       <c r="S17" t="n">
-        <v>-5.4056</v>
+        <v>-8.204700000000001</v>
       </c>
       <c r="T17" t="n">
-        <v>-15.0424</v>
+        <v>6.8853</v>
       </c>
       <c r="U17" t="n">
-        <v>-5.6991</v>
+        <v>3.2764</v>
       </c>
       <c r="V17" t="n">
-        <v>-0.11</v>
+        <v>-1.7291</v>
       </c>
       <c r="W17" t="n">
-        <v>-4.9463</v>
+        <v>3.8627</v>
       </c>
       <c r="X17" t="n">
-        <v>13.9706</v>
+        <v>-7.957</v>
       </c>
       <c r="Y17" t="n">
-        <v>3.3333</v>
+        <v>5.1597</v>
       </c>
       <c r="Z17" t="n">
-        <v>11.5108</v>
+        <v>-10.8333</v>
       </c>
       <c r="AA17" t="n">
-        <v>5.7438</v>
+        <v>-3.3041</v>
       </c>
       <c r="AB17" t="n">
-        <v>-0.3244</v>
+        <v>1.3911</v>
       </c>
       <c r="AC17" t="n">
-        <v>4.3626</v>
+        <v>-4.3338</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>187.69</v>
+        <v>183.77</v>
       </c>
       <c r="C18" t="n">
-        <v>188.43</v>
+        <v>184</v>
       </c>
       <c r="D18" t="n">
-        <v>170.26</v>
+        <v>150</v>
       </c>
       <c r="E18" t="n">
-        <v>176.66</v>
+        <v>165.55</v>
       </c>
       <c r="F18" t="n">
-        <v>75.2</v>
+        <v>76.29000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>75.84999999999999</v>
+        <v>76.47</v>
       </c>
       <c r="H18" t="n">
-        <v>73.41</v>
+        <v>72.06</v>
       </c>
       <c r="I18" t="n">
-        <v>75.02</v>
+        <v>74.44</v>
       </c>
       <c r="J18" t="n">
-        <v>39.7</v>
+        <v>41.23</v>
       </c>
       <c r="K18" t="n">
-        <v>45</v>
+        <v>49.69</v>
       </c>
       <c r="L18" t="n">
-        <v>39.7</v>
+        <v>41.16</v>
       </c>
       <c r="M18" t="n">
-        <v>42.8</v>
+        <v>45.98</v>
       </c>
       <c r="N18" t="n">
-        <v>38.54</v>
+        <v>37.98</v>
       </c>
       <c r="O18" t="n">
-        <v>39.53</v>
+        <v>40.17</v>
       </c>
       <c r="P18" t="n">
-        <v>38.19</v>
+        <v>37.89</v>
       </c>
       <c r="Q18" t="n">
-        <v>38.63</v>
+        <v>38.94</v>
       </c>
       <c r="R18" t="n">
-        <v>6.8271</v>
+        <v>-6.2889</v>
       </c>
       <c r="S18" t="n">
-        <v>-8.204700000000001</v>
+        <v>-13.8926</v>
       </c>
       <c r="T18" t="n">
-        <v>6.8853</v>
+        <v>-5.3026</v>
       </c>
       <c r="U18" t="n">
-        <v>3.2764</v>
+        <v>-0.7731</v>
       </c>
       <c r="V18" t="n">
-        <v>-1.7291</v>
+        <v>-3.3623</v>
       </c>
       <c r="W18" t="n">
-        <v>3.8627</v>
+        <v>2.3652</v>
       </c>
       <c r="X18" t="n">
-        <v>-7.957</v>
+        <v>7.4299</v>
       </c>
       <c r="Y18" t="n">
-        <v>5.1597</v>
+        <v>12.6961</v>
       </c>
       <c r="Z18" t="n">
-        <v>-10.8333</v>
+        <v>2.1778</v>
       </c>
       <c r="AA18" t="n">
-        <v>-3.3041</v>
+        <v>0.8025</v>
       </c>
       <c r="AB18" t="n">
-        <v>1.3911</v>
+        <v>3.0704</v>
       </c>
       <c r="AC18" t="n">
-        <v>-4.3338</v>
+        <v>-2.8443</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>183.77</v>
+        <v>150.44</v>
       </c>
       <c r="C19" t="n">
-        <v>184</v>
+        <v>155.83</v>
       </c>
       <c r="D19" t="n">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="E19" t="n">
-        <v>165.55</v>
+        <v>142.48</v>
       </c>
       <c r="F19" t="n">
-        <v>76.29000000000001</v>
+        <v>72.61</v>
       </c>
       <c r="G19" t="n">
-        <v>76.47</v>
+        <v>73.12</v>
       </c>
       <c r="H19" t="n">
-        <v>72.06</v>
+        <v>69.69</v>
       </c>
       <c r="I19" t="n">
-        <v>74.44</v>
+        <v>70.73999999999999</v>
       </c>
       <c r="J19" t="n">
-        <v>41.23</v>
+        <v>49.77</v>
       </c>
       <c r="K19" t="n">
-        <v>49.69</v>
+        <v>53.34</v>
       </c>
       <c r="L19" t="n">
-        <v>41.16</v>
+        <v>48.31</v>
       </c>
       <c r="M19" t="n">
-        <v>45.98</v>
+        <v>52.02</v>
       </c>
       <c r="N19" t="n">
-        <v>37.98</v>
+        <v>39.9</v>
       </c>
       <c r="O19" t="n">
-        <v>40.17</v>
+        <v>41.44</v>
       </c>
       <c r="P19" t="n">
-        <v>37.89</v>
+        <v>39.65</v>
       </c>
       <c r="Q19" t="n">
-        <v>38.94</v>
+        <v>40.89</v>
       </c>
       <c r="R19" t="n">
-        <v>-6.2889</v>
+        <v>-13.9354</v>
       </c>
       <c r="S19" t="n">
-        <v>-13.8926</v>
+        <v>-13.8417</v>
       </c>
       <c r="T19" t="n">
-        <v>-5.3026</v>
+        <v>-25.9652</v>
       </c>
       <c r="U19" t="n">
-        <v>-0.7731</v>
+        <v>-4.9704</v>
       </c>
       <c r="V19" t="n">
-        <v>-3.3623</v>
+        <v>-2.6156</v>
       </c>
       <c r="W19" t="n">
-        <v>2.3652</v>
+        <v>-7.3356</v>
       </c>
       <c r="X19" t="n">
-        <v>7.4299</v>
+        <v>13.1361</v>
       </c>
       <c r="Y19" t="n">
-        <v>12.6961</v>
+        <v>11.871</v>
       </c>
       <c r="Z19" t="n">
-        <v>2.1778</v>
+        <v>27.8133</v>
       </c>
       <c r="AA19" t="n">
-        <v>0.8025</v>
+        <v>5.0077</v>
       </c>
       <c r="AB19" t="n">
-        <v>3.0704</v>
+        <v>2.3529</v>
       </c>
       <c r="AC19" t="n">
-        <v>-2.8443</v>
+        <v>7.3228</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>150.44</v>
+        <v>124.73</v>
       </c>
       <c r="C20" t="n">
-        <v>155.83</v>
+        <v>144.4</v>
       </c>
       <c r="D20" t="n">
-        <v>138</v>
+        <v>116.47</v>
       </c>
       <c r="E20" t="n">
-        <v>142.48</v>
+        <v>135.47</v>
       </c>
       <c r="F20" t="n">
-        <v>72.61</v>
+        <v>66.38</v>
       </c>
       <c r="G20" t="n">
-        <v>73.12</v>
+        <v>69.56</v>
       </c>
       <c r="H20" t="n">
-        <v>69.69</v>
+        <v>64.91</v>
       </c>
       <c r="I20" t="n">
-        <v>70.73999999999999</v>
+        <v>67.53</v>
       </c>
       <c r="J20" t="n">
-        <v>49.77</v>
+        <v>58.59</v>
       </c>
       <c r="K20" t="n">
-        <v>53.34</v>
+        <v>61.6</v>
       </c>
       <c r="L20" t="n">
-        <v>48.31</v>
+        <v>51.34</v>
       </c>
       <c r="M20" t="n">
-        <v>52.02</v>
+        <v>54.85</v>
       </c>
       <c r="N20" t="n">
-        <v>39.9</v>
+        <v>43.43</v>
       </c>
       <c r="O20" t="n">
-        <v>41.44</v>
+        <v>44.27</v>
       </c>
       <c r="P20" t="n">
-        <v>39.65</v>
+        <v>41.59</v>
       </c>
       <c r="Q20" t="n">
-        <v>40.89</v>
+        <v>42.79</v>
       </c>
       <c r="R20" t="n">
-        <v>-13.9354</v>
+        <v>-4.92</v>
       </c>
       <c r="S20" t="n">
-        <v>-13.8417</v>
+        <v>-23.316</v>
       </c>
       <c r="T20" t="n">
-        <v>-25.9652</v>
+        <v>-29.5381</v>
       </c>
       <c r="U20" t="n">
-        <v>-4.9704</v>
+        <v>-4.5377</v>
       </c>
       <c r="V20" t="n">
-        <v>-2.6156</v>
+        <v>-9.984</v>
       </c>
       <c r="W20" t="n">
-        <v>-7.3356</v>
+        <v>-12.3329</v>
       </c>
       <c r="X20" t="n">
-        <v>13.1361</v>
+        <v>5.4402</v>
       </c>
       <c r="Y20" t="n">
-        <v>11.871</v>
+        <v>28.1542</v>
       </c>
       <c r="Z20" t="n">
-        <v>27.8133</v>
+        <v>34.4363</v>
       </c>
       <c r="AA20" t="n">
-        <v>5.0077</v>
+        <v>4.6466</v>
       </c>
       <c r="AB20" t="n">
-        <v>2.3529</v>
+        <v>10.7688</v>
       </c>
       <c r="AC20" t="n">
-        <v>7.3228</v>
+        <v>13.261</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>124.73</v>
+        <v>143.52</v>
       </c>
       <c r="C21" t="n">
-        <v>144.3999</v>
+        <v>148.74</v>
       </c>
       <c r="D21" t="n">
-        <v>116.47</v>
+        <v>135.665</v>
       </c>
       <c r="E21" t="n">
-        <v>135.47</v>
+        <v>136.81</v>
       </c>
       <c r="F21" t="n">
-        <v>66.38</v>
+        <v>69.47</v>
       </c>
       <c r="G21" t="n">
-        <v>69.55500000000001</v>
+        <v>70.505</v>
       </c>
       <c r="H21" t="n">
-        <v>64.91</v>
+        <v>67.5</v>
       </c>
       <c r="I21" t="n">
-        <v>67.53</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>58.59</v>
+        <v>51.19</v>
       </c>
       <c r="K21" t="n">
-        <v>61.5932</v>
+        <v>54.41</v>
       </c>
       <c r="L21" t="n">
-        <v>51.34</v>
+        <v>49.11</v>
       </c>
       <c r="M21" t="n">
-        <v>54.85</v>
+        <v>53.99</v>
       </c>
       <c r="N21" t="n">
-        <v>43.43</v>
+        <v>41.52</v>
       </c>
       <c r="O21" t="n">
-        <v>44.2714</v>
+        <v>42.7615</v>
       </c>
       <c r="P21" t="n">
-        <v>41.585</v>
+        <v>40.87</v>
       </c>
       <c r="Q21" t="n">
-        <v>42.79</v>
+        <v>42.68</v>
       </c>
       <c r="R21" t="n">
-        <v>-4.92</v>
+        <v>0.9891</v>
       </c>
       <c r="S21" t="n">
-        <v>-23.316</v>
+        <v>-17.3603</v>
       </c>
       <c r="T21" t="n">
-        <v>-29.5381</v>
+        <v>-17.2704</v>
       </c>
       <c r="U21" t="n">
-        <v>-4.5377</v>
+        <v>0.1777</v>
       </c>
       <c r="V21" t="n">
-        <v>-9.984</v>
+        <v>-9.1214</v>
       </c>
       <c r="W21" t="n">
-        <v>-12.3329</v>
+        <v>-6.8695</v>
       </c>
       <c r="X21" t="n">
-        <v>5.4402</v>
+        <v>-1.5679</v>
       </c>
       <c r="Y21" t="n">
-        <v>28.1542</v>
+        <v>17.4206</v>
       </c>
       <c r="Z21" t="n">
-        <v>34.4363</v>
+        <v>16.1075</v>
       </c>
       <c r="AA21" t="n">
-        <v>4.6466</v>
+        <v>-0.2571</v>
       </c>
       <c r="AB21" t="n">
-        <v>10.7688</v>
+        <v>9.6045</v>
       </c>
       <c r="AC21" t="n">
-        <v>13.261</v>
+        <v>6.8335</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2321,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-07-21 22:57
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC21"/>
+  <dimension ref="A1:AC22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2199,7 +2199,7 @@
         <v>148.74</v>
       </c>
       <c r="D21" t="n">
-        <v>135.665</v>
+        <v>135.67</v>
       </c>
       <c r="E21" t="n">
         <v>136.81</v>
@@ -2208,7 +2208,7 @@
         <v>69.47</v>
       </c>
       <c r="G21" t="n">
-        <v>70.505</v>
+        <v>70.51000000000001</v>
       </c>
       <c r="H21" t="n">
         <v>67.5</v>
@@ -2229,10 +2229,10 @@
         <v>53.99</v>
       </c>
       <c r="N21" t="n">
-        <v>41.52</v>
+        <v>41.54</v>
       </c>
       <c r="O21" t="n">
-        <v>42.7615</v>
+        <v>42.76</v>
       </c>
       <c r="P21" t="n">
         <v>40.87</v>
@@ -2275,6 +2275,97 @@
       </c>
       <c r="AC21" t="n">
         <v>6.8335</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>155.84</v>
+      </c>
+      <c r="C22" t="n">
+        <v>160.64</v>
+      </c>
+      <c r="D22" t="n">
+        <v>148.87</v>
+      </c>
+      <c r="E22" t="n">
+        <v>158.54</v>
+      </c>
+      <c r="F22" t="n">
+        <v>70.709</v>
+      </c>
+      <c r="G22" t="n">
+        <v>71.7199</v>
+      </c>
+      <c r="H22" t="n">
+        <v>69.61</v>
+      </c>
+      <c r="I22" t="n">
+        <v>71.37</v>
+      </c>
+      <c r="J22" t="n">
+        <v>46.34</v>
+      </c>
+      <c r="K22" t="n">
+        <v>49.09</v>
+      </c>
+      <c r="L22" t="n">
+        <v>44.44</v>
+      </c>
+      <c r="M22" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="N22" t="n">
+        <v>40.75</v>
+      </c>
+      <c r="O22" t="n">
+        <v>41.445</v>
+      </c>
+      <c r="P22" t="n">
+        <v>40.11</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>40.31</v>
+      </c>
+      <c r="R22" t="n">
+        <v>15.8833</v>
+      </c>
+      <c r="S22" t="n">
+        <v>11.2718</v>
+      </c>
+      <c r="T22" t="n">
+        <v>-10.257</v>
+      </c>
+      <c r="U22" t="n">
+        <v>5.4989</v>
+      </c>
+      <c r="V22" t="n">
+        <v>0.8905999999999999</v>
+      </c>
+      <c r="W22" t="n">
+        <v>-4.8654</v>
+      </c>
+      <c r="X22" t="n">
+        <v>-16.4104</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>-13.2449</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>5.4439</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>-5.553</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>-1.4184</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>4.349</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2412,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master system update 2026-07-22 23:03
</commit_message>
<xml_diff>
--- a/data/4_etf/4_ETF_Workbook.xlsx
+++ b/data/4_etf/4_ETF_Workbook.xlsx
@@ -568,1804 +568,1804 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>299.26</v>
+        <v>236</v>
       </c>
       <c r="C2" t="n">
-        <v>302</v>
+        <v>252.98</v>
       </c>
       <c r="D2" t="n">
-        <v>286.24</v>
+        <v>223</v>
       </c>
       <c r="E2" t="n">
-        <v>300.77</v>
+        <v>231.42</v>
       </c>
       <c r="F2" t="n">
-        <v>83.7572</v>
+        <v>74.9474</v>
       </c>
       <c r="G2" t="n">
-        <v>84.9145</v>
+        <v>77.56140000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>81.203</v>
+        <v>73.7402</v>
       </c>
       <c r="I2" t="n">
-        <v>82.3903</v>
+        <v>74.26900000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>32.9165</v>
+        <v>39.9</v>
       </c>
       <c r="K2" t="n">
-        <v>34.4981</v>
+        <v>41.3</v>
       </c>
       <c r="L2" t="n">
-        <v>32.5212</v>
+        <v>38</v>
       </c>
       <c r="M2" t="n">
-        <v>32.62</v>
+        <v>40.4</v>
       </c>
       <c r="N2" t="n">
-        <v>35.7389</v>
+        <v>39.6267</v>
       </c>
       <c r="O2" t="n">
-        <v>36.8511</v>
+        <v>40.1582</v>
       </c>
       <c r="P2" t="n">
-        <v>35.2369</v>
+        <v>38.4653</v>
       </c>
       <c r="Q2" t="n">
-        <v>36.3491</v>
+        <v>39.922</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>236</v>
+        <v>233.11</v>
       </c>
       <c r="C3" t="n">
-        <v>252.98</v>
+        <v>237</v>
       </c>
       <c r="D3" t="n">
-        <v>223</v>
+        <v>211.13</v>
       </c>
       <c r="E3" t="n">
-        <v>231.42</v>
+        <v>229.57</v>
       </c>
       <c r="F3" t="n">
-        <v>74.9474</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>77.56140000000001</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>73.7402</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="I3" t="n">
-        <v>74.26900000000001</v>
+        <v>73.3</v>
       </c>
       <c r="J3" t="n">
-        <v>39.9</v>
+        <v>40</v>
       </c>
       <c r="K3" t="n">
-        <v>41.3</v>
+        <v>43.9</v>
       </c>
       <c r="L3" t="n">
-        <v>38</v>
+        <v>39.2</v>
       </c>
       <c r="M3" t="n">
-        <v>40.4</v>
+        <v>40.8</v>
       </c>
       <c r="N3" t="n">
-        <v>39.6267</v>
+        <v>39.66</v>
       </c>
       <c r="O3" t="n">
-        <v>40.1582</v>
+        <v>41.49</v>
       </c>
       <c r="P3" t="n">
-        <v>38.4653</v>
+        <v>38.9</v>
       </c>
       <c r="Q3" t="n">
-        <v>39.922</v>
+        <v>40.45</v>
       </c>
       <c r="R3" t="n">
-        <v>-23.0575</v>
+        <v>-0.7994</v>
       </c>
       <c r="U3" t="n">
-        <v>-9.857100000000001</v>
+        <v>-1.3047</v>
       </c>
       <c r="X3" t="n">
-        <v>23.8504</v>
+        <v>0.9901</v>
       </c>
       <c r="AA3" t="n">
-        <v>9.8294</v>
+        <v>1.3226</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>233.11</v>
+        <v>268.05</v>
       </c>
       <c r="C4" t="n">
-        <v>237</v>
+        <v>268.4</v>
       </c>
       <c r="D4" t="n">
-        <v>211.13</v>
+        <v>225.74</v>
       </c>
       <c r="E4" t="n">
-        <v>229.57</v>
+        <v>252.61</v>
       </c>
       <c r="F4" t="n">
-        <v>74.79000000000001</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>76.18000000000001</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>71.34999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I4" t="n">
-        <v>73.3</v>
+        <v>74.95</v>
       </c>
       <c r="J4" t="n">
-        <v>40</v>
+        <v>33.8</v>
       </c>
       <c r="K4" t="n">
-        <v>43.9</v>
+        <v>41.5</v>
       </c>
       <c r="L4" t="n">
-        <v>39.2</v>
+        <v>33.7</v>
       </c>
       <c r="M4" t="n">
-        <v>40.8</v>
+        <v>36.3</v>
       </c>
       <c r="N4" t="n">
-        <v>39.66</v>
+        <v>37.87</v>
       </c>
       <c r="O4" t="n">
-        <v>41.49</v>
+        <v>41.37</v>
       </c>
       <c r="P4" t="n">
-        <v>38.9</v>
+        <v>37.71</v>
       </c>
       <c r="Q4" t="n">
-        <v>40.45</v>
+        <v>39.47</v>
       </c>
       <c r="R4" t="n">
-        <v>-0.7994</v>
+        <v>10.0362</v>
       </c>
       <c r="U4" t="n">
-        <v>-1.3047</v>
+        <v>2.251</v>
       </c>
       <c r="X4" t="n">
-        <v>0.9901</v>
+        <v>-11.0294</v>
       </c>
       <c r="AA4" t="n">
-        <v>1.3226</v>
+        <v>-2.4227</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>268.05</v>
+        <v>226.24</v>
       </c>
       <c r="C5" t="n">
-        <v>268.4</v>
+        <v>231.25</v>
       </c>
       <c r="D5" t="n">
-        <v>225.74</v>
+        <v>212.1</v>
       </c>
       <c r="E5" t="n">
-        <v>252.61</v>
+        <v>215.6</v>
       </c>
       <c r="F5" t="n">
-        <v>77.95999999999999</v>
+        <v>72.09</v>
       </c>
       <c r="G5" t="n">
-        <v>78.23999999999999</v>
+        <v>74.69</v>
       </c>
       <c r="H5" t="n">
-        <v>71.59999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="I5" t="n">
-        <v>74.95</v>
+        <v>71.83</v>
       </c>
       <c r="J5" t="n">
-        <v>33.8</v>
+        <v>40.4</v>
       </c>
       <c r="K5" t="n">
-        <v>41.5</v>
+        <v>42.5</v>
       </c>
       <c r="L5" t="n">
-        <v>33.7</v>
+        <v>39.5</v>
       </c>
       <c r="M5" t="n">
-        <v>36.3</v>
+        <v>42.4</v>
       </c>
       <c r="N5" t="n">
-        <v>37.87</v>
+        <v>41.08</v>
       </c>
       <c r="O5" t="n">
-        <v>41.37</v>
+        <v>41.79</v>
       </c>
       <c r="P5" t="n">
-        <v>37.71</v>
+        <v>39.69</v>
       </c>
       <c r="Q5" t="n">
-        <v>39.47</v>
+        <v>41.31</v>
       </c>
       <c r="R5" t="n">
-        <v>10.0362</v>
+        <v>-14.651</v>
       </c>
       <c r="S5" t="n">
-        <v>-16.0122</v>
+        <v>-6.8361</v>
       </c>
       <c r="U5" t="n">
-        <v>2.251</v>
+        <v>-4.1628</v>
       </c>
       <c r="V5" t="n">
-        <v>-9.0306</v>
+        <v>-3.284</v>
       </c>
       <c r="X5" t="n">
-        <v>-11.0294</v>
+        <v>16.8044</v>
       </c>
       <c r="Y5" t="n">
-        <v>11.2814</v>
+        <v>4.9505</v>
       </c>
       <c r="AA5" t="n">
-        <v>-2.4227</v>
+        <v>4.6618</v>
       </c>
       <c r="AB5" t="n">
-        <v>8.585900000000001</v>
+        <v>3.4768</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>226.24</v>
+        <v>216.36</v>
       </c>
       <c r="C6" t="n">
-        <v>231.25</v>
+        <v>238.65</v>
       </c>
       <c r="D6" t="n">
-        <v>212.1</v>
+        <v>192.3</v>
       </c>
       <c r="E6" t="n">
-        <v>215.6</v>
+        <v>236.52</v>
       </c>
       <c r="F6" t="n">
-        <v>72.09</v>
+        <v>74.12</v>
       </c>
       <c r="G6" t="n">
-        <v>74.69</v>
+        <v>77.38</v>
       </c>
       <c r="H6" t="n">
-        <v>70.72</v>
+        <v>71.45</v>
       </c>
       <c r="I6" t="n">
-        <v>71.83</v>
+        <v>77.19</v>
       </c>
       <c r="J6" t="n">
-        <v>40.4</v>
+        <v>41.6</v>
       </c>
       <c r="K6" t="n">
-        <v>42.5</v>
+        <v>46.3</v>
       </c>
       <c r="L6" t="n">
-        <v>39.5</v>
+        <v>37</v>
       </c>
       <c r="M6" t="n">
-        <v>42.4</v>
+        <v>37.2</v>
       </c>
       <c r="N6" t="n">
-        <v>41.08</v>
+        <v>39.91</v>
       </c>
       <c r="O6" t="n">
-        <v>41.79</v>
+        <v>41.43</v>
       </c>
       <c r="P6" t="n">
-        <v>39.69</v>
+        <v>38.08</v>
       </c>
       <c r="Q6" t="n">
-        <v>41.31</v>
+        <v>38.16</v>
       </c>
       <c r="R6" t="n">
-        <v>-14.651</v>
+        <v>9.703200000000001</v>
       </c>
       <c r="S6" t="n">
-        <v>-6.8361</v>
+        <v>3.0274</v>
       </c>
       <c r="U6" t="n">
-        <v>-4.1628</v>
+        <v>7.4621</v>
       </c>
       <c r="V6" t="n">
-        <v>-3.284</v>
+        <v>5.307</v>
       </c>
       <c r="X6" t="n">
-        <v>16.8044</v>
+        <v>-12.2642</v>
       </c>
       <c r="Y6" t="n">
-        <v>4.9505</v>
+        <v>-8.823499999999999</v>
       </c>
       <c r="AA6" t="n">
-        <v>4.6618</v>
+        <v>-7.6253</v>
       </c>
       <c r="AB6" t="n">
-        <v>3.4768</v>
+        <v>-5.6613</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>216.36</v>
+        <v>241.45</v>
       </c>
       <c r="C7" t="n">
-        <v>238.65</v>
+        <v>272</v>
       </c>
       <c r="D7" t="n">
-        <v>192.3</v>
+        <v>240.59</v>
       </c>
       <c r="E7" t="n">
-        <v>236.52</v>
+        <v>266.71</v>
       </c>
       <c r="F7" t="n">
-        <v>74.12</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>77.38</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>71.45</v>
+        <v>77.15000000000001</v>
       </c>
       <c r="I7" t="n">
-        <v>77.19</v>
+        <v>81</v>
       </c>
       <c r="J7" t="n">
-        <v>41.6</v>
+        <v>36.6</v>
       </c>
       <c r="K7" t="n">
-        <v>46.3</v>
+        <v>36.8</v>
       </c>
       <c r="L7" t="n">
-        <v>37</v>
+        <v>31.7</v>
       </c>
       <c r="M7" t="n">
-        <v>37.2</v>
+        <v>32.4</v>
       </c>
       <c r="N7" t="n">
-        <v>39.91</v>
+        <v>38.16</v>
       </c>
       <c r="O7" t="n">
-        <v>41.43</v>
+        <v>38.2</v>
       </c>
       <c r="P7" t="n">
-        <v>38.08</v>
+        <v>36.03</v>
       </c>
       <c r="Q7" t="n">
-        <v>38.16</v>
+        <v>36.31</v>
       </c>
       <c r="R7" t="n">
-        <v>9.703200000000001</v>
+        <v>12.7642</v>
       </c>
       <c r="S7" t="n">
-        <v>3.0274</v>
+        <v>5.5817</v>
       </c>
       <c r="T7" t="n">
-        <v>-21.3618</v>
+        <v>15.2493</v>
       </c>
       <c r="U7" t="n">
-        <v>7.4621</v>
+        <v>4.9359</v>
       </c>
       <c r="V7" t="n">
-        <v>5.307</v>
+        <v>8.071999999999999</v>
       </c>
       <c r="W7" t="n">
-        <v>-6.3118</v>
+        <v>9.063000000000001</v>
       </c>
       <c r="X7" t="n">
-        <v>-12.2642</v>
+        <v>-12.9032</v>
       </c>
       <c r="Y7" t="n">
-        <v>-8.823499999999999</v>
+        <v>-10.7438</v>
       </c>
       <c r="Z7" t="n">
-        <v>14.0405</v>
+        <v>-19.802</v>
       </c>
       <c r="AA7" t="n">
-        <v>-7.6253</v>
+        <v>-4.848</v>
       </c>
       <c r="AB7" t="n">
-        <v>-5.6613</v>
+        <v>-8.0061</v>
       </c>
       <c r="AC7" t="n">
-        <v>4.982</v>
+        <v>-9.047599999999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>241.45</v>
+        <v>237.79</v>
       </c>
       <c r="C8" t="n">
-        <v>272</v>
+        <v>246.47</v>
       </c>
       <c r="D8" t="n">
-        <v>240.59</v>
+        <v>215.38</v>
       </c>
       <c r="E8" t="n">
-        <v>266.71</v>
+        <v>217.55</v>
       </c>
       <c r="F8" t="n">
-        <v>77.23999999999999</v>
+        <v>78.72</v>
       </c>
       <c r="G8" t="n">
-        <v>81.54000000000001</v>
+        <v>79.64</v>
       </c>
       <c r="H8" t="n">
-        <v>77.15000000000001</v>
+        <v>77.23</v>
       </c>
       <c r="I8" t="n">
-        <v>81</v>
+        <v>77.45999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>36.6</v>
+        <v>35.9</v>
       </c>
       <c r="K8" t="n">
-        <v>36.8</v>
+        <v>38.9</v>
       </c>
       <c r="L8" t="n">
-        <v>31.7</v>
+        <v>35.1</v>
       </c>
       <c r="M8" t="n">
-        <v>32.4</v>
+        <v>38.6</v>
       </c>
       <c r="N8" t="n">
-        <v>38.16</v>
+        <v>37.31</v>
       </c>
       <c r="O8" t="n">
-        <v>38.2</v>
+        <v>37.98</v>
       </c>
       <c r="P8" t="n">
-        <v>36.03</v>
+        <v>36.9</v>
       </c>
       <c r="Q8" t="n">
-        <v>36.31</v>
+        <v>37.88</v>
       </c>
       <c r="R8" t="n">
-        <v>12.7642</v>
+        <v>-18.432</v>
       </c>
       <c r="S8" t="n">
-        <v>5.5817</v>
+        <v>0.9045</v>
       </c>
       <c r="T8" t="n">
-        <v>15.2493</v>
+        <v>-5.2359</v>
       </c>
       <c r="U8" t="n">
-        <v>4.9359</v>
+        <v>-4.3704</v>
       </c>
       <c r="V8" t="n">
-        <v>8.071999999999999</v>
+        <v>7.838</v>
       </c>
       <c r="W8" t="n">
-        <v>9.063000000000001</v>
+        <v>5.6753</v>
       </c>
       <c r="X8" t="n">
-        <v>-12.9032</v>
+        <v>19.1358</v>
       </c>
       <c r="Y8" t="n">
-        <v>-10.7438</v>
+        <v>-8.962300000000001</v>
       </c>
       <c r="Z8" t="n">
-        <v>-19.802</v>
+        <v>-5.3922</v>
       </c>
       <c r="AA8" t="n">
-        <v>-4.848</v>
+        <v>4.3239</v>
       </c>
       <c r="AB8" t="n">
-        <v>-8.0061</v>
+        <v>-8.303100000000001</v>
       </c>
       <c r="AC8" t="n">
-        <v>-9.047599999999999</v>
+        <v>-6.3535</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>237.79</v>
+        <v>219.23</v>
       </c>
       <c r="C9" t="n">
-        <v>246.47</v>
+        <v>226.13</v>
       </c>
       <c r="D9" t="n">
-        <v>215.38</v>
+        <v>168.88</v>
       </c>
       <c r="E9" t="n">
-        <v>217.55</v>
+        <v>181.47</v>
       </c>
       <c r="F9" t="n">
-        <v>78.72</v>
+        <v>77.45</v>
       </c>
       <c r="G9" t="n">
-        <v>79.64</v>
+        <v>79.14</v>
       </c>
       <c r="H9" t="n">
-        <v>77.23</v>
+        <v>71.72</v>
       </c>
       <c r="I9" t="n">
-        <v>77.45999999999999</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>35.9</v>
+        <v>38.4</v>
       </c>
       <c r="K9" t="n">
-        <v>38.9</v>
+        <v>47.4</v>
       </c>
       <c r="L9" t="n">
-        <v>35.1</v>
+        <v>37.1</v>
       </c>
       <c r="M9" t="n">
-        <v>38.6</v>
+        <v>45.1</v>
       </c>
       <c r="N9" t="n">
-        <v>37.31</v>
+        <v>37.91</v>
       </c>
       <c r="O9" t="n">
-        <v>37.98</v>
+        <v>40.72</v>
       </c>
       <c r="P9" t="n">
-        <v>36.9</v>
+        <v>37.08</v>
       </c>
       <c r="Q9" t="n">
-        <v>37.88</v>
+        <v>39.95</v>
       </c>
       <c r="R9" t="n">
-        <v>-18.432</v>
+        <v>-16.5847</v>
       </c>
       <c r="S9" t="n">
-        <v>0.9045</v>
+        <v>-23.275</v>
       </c>
       <c r="T9" t="n">
-        <v>-5.2359</v>
+        <v>-28.162</v>
       </c>
       <c r="U9" t="n">
-        <v>-4.3704</v>
+        <v>-5.306</v>
       </c>
       <c r="V9" t="n">
-        <v>7.838</v>
+        <v>-4.9747</v>
       </c>
       <c r="W9" t="n">
-        <v>5.6753</v>
+        <v>-2.1348</v>
       </c>
       <c r="X9" t="n">
-        <v>19.1358</v>
+        <v>16.8394</v>
       </c>
       <c r="Y9" t="n">
-        <v>-8.962300000000001</v>
+        <v>21.2366</v>
       </c>
       <c r="Z9" t="n">
-        <v>-5.3922</v>
+        <v>24.2424</v>
       </c>
       <c r="AA9" t="n">
-        <v>4.3239</v>
+        <v>5.4646</v>
       </c>
       <c r="AB9" t="n">
-        <v>-8.303100000000001</v>
+        <v>4.6908</v>
       </c>
       <c r="AC9" t="n">
-        <v>-6.3535</v>
+        <v>1.2161</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>219.23</v>
+        <v>197.21</v>
       </c>
       <c r="C10" t="n">
-        <v>226.13</v>
+        <v>210.8</v>
       </c>
       <c r="D10" t="n">
-        <v>168.88</v>
+        <v>194.22</v>
       </c>
       <c r="E10" t="n">
-        <v>181.47</v>
+        <v>194.65</v>
       </c>
       <c r="F10" t="n">
+        <v>75.54000000000001</v>
+      </c>
+      <c r="G10" t="n">
         <v>77.45</v>
       </c>
-      <c r="G10" t="n">
-        <v>79.14</v>
-      </c>
       <c r="H10" t="n">
-        <v>71.72</v>
+        <v>75.11</v>
       </c>
       <c r="I10" t="n">
-        <v>73.34999999999999</v>
+        <v>76.42</v>
       </c>
       <c r="J10" t="n">
-        <v>38.4</v>
+        <v>41.1</v>
       </c>
       <c r="K10" t="n">
-        <v>47.4</v>
+        <v>41.8</v>
       </c>
       <c r="L10" t="n">
-        <v>37.1</v>
+        <v>37.7</v>
       </c>
       <c r="M10" t="n">
-        <v>45.1</v>
+        <v>41.7</v>
       </c>
       <c r="N10" t="n">
-        <v>37.91</v>
+        <v>38.75</v>
       </c>
       <c r="O10" t="n">
-        <v>40.72</v>
+        <v>38.98</v>
       </c>
       <c r="P10" t="n">
-        <v>37.08</v>
+        <v>37.71</v>
       </c>
       <c r="Q10" t="n">
-        <v>39.95</v>
+        <v>38.28</v>
       </c>
       <c r="R10" t="n">
-        <v>-16.5847</v>
+        <v>7.2629</v>
       </c>
       <c r="S10" t="n">
-        <v>-23.275</v>
+        <v>-27.0181</v>
       </c>
       <c r="T10" t="n">
-        <v>-28.162</v>
+        <v>-9.7171</v>
       </c>
       <c r="U10" t="n">
-        <v>-5.306</v>
+        <v>4.1854</v>
       </c>
       <c r="V10" t="n">
-        <v>-4.9747</v>
+        <v>-5.6543</v>
       </c>
       <c r="W10" t="n">
-        <v>-2.1348</v>
+        <v>6.3901</v>
       </c>
       <c r="X10" t="n">
-        <v>16.8394</v>
+        <v>-7.5388</v>
       </c>
       <c r="Y10" t="n">
-        <v>21.2366</v>
+        <v>28.7037</v>
       </c>
       <c r="Z10" t="n">
-        <v>24.2424</v>
+        <v>-1.6509</v>
       </c>
       <c r="AA10" t="n">
-        <v>5.4646</v>
+        <v>-4.1802</v>
       </c>
       <c r="AB10" t="n">
-        <v>4.6908</v>
+        <v>5.4255</v>
       </c>
       <c r="AC10" t="n">
-        <v>1.2161</v>
+        <v>-7.3348</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>197.21</v>
+        <v>165.4</v>
       </c>
       <c r="C11" t="n">
-        <v>210.8</v>
+        <v>171.88</v>
       </c>
       <c r="D11" t="n">
-        <v>194.22</v>
+        <v>150.08</v>
       </c>
       <c r="E11" t="n">
-        <v>194.65</v>
+        <v>165.28</v>
       </c>
       <c r="F11" t="n">
-        <v>75.54000000000001</v>
+        <v>73.7</v>
       </c>
       <c r="G11" t="n">
-        <v>77.45</v>
+        <v>74.39</v>
       </c>
       <c r="H11" t="n">
-        <v>75.11</v>
+        <v>70.76000000000001</v>
       </c>
       <c r="I11" t="n">
-        <v>76.42</v>
+        <v>72.23</v>
       </c>
       <c r="J11" t="n">
-        <v>41.1</v>
+        <v>48</v>
       </c>
       <c r="K11" t="n">
-        <v>41.8</v>
+        <v>51.4</v>
       </c>
       <c r="L11" t="n">
-        <v>37.7</v>
+        <v>46.6</v>
       </c>
       <c r="M11" t="n">
-        <v>41.7</v>
+        <v>48</v>
       </c>
       <c r="N11" t="n">
-        <v>38.75</v>
+        <v>39.64</v>
       </c>
       <c r="O11" t="n">
-        <v>38.98</v>
+        <v>41.11</v>
       </c>
       <c r="P11" t="n">
-        <v>37.71</v>
+        <v>39.29</v>
       </c>
       <c r="Q11" t="n">
-        <v>38.28</v>
+        <v>40.38</v>
       </c>
       <c r="R11" t="n">
-        <v>7.2629</v>
+        <v>-15.0886</v>
       </c>
       <c r="S11" t="n">
-        <v>-27.0181</v>
+        <v>-24.0267</v>
       </c>
       <c r="T11" t="n">
-        <v>-9.7171</v>
+        <v>-30.1201</v>
       </c>
       <c r="U11" t="n">
-        <v>4.1854</v>
+        <v>-5.4829</v>
       </c>
       <c r="V11" t="n">
-        <v>-5.6543</v>
+        <v>-6.7519</v>
       </c>
       <c r="W11" t="n">
-        <v>6.3901</v>
+        <v>-6.4257</v>
       </c>
       <c r="X11" t="n">
-        <v>-7.5388</v>
+        <v>15.1079</v>
       </c>
       <c r="Y11" t="n">
-        <v>28.7037</v>
+        <v>24.3523</v>
       </c>
       <c r="Z11" t="n">
-        <v>-1.6509</v>
+        <v>29.0323</v>
       </c>
       <c r="AA11" t="n">
-        <v>-4.1802</v>
+        <v>5.4859</v>
       </c>
       <c r="AB11" t="n">
-        <v>5.4255</v>
+        <v>6.5998</v>
       </c>
       <c r="AC11" t="n">
-        <v>-7.3348</v>
+        <v>5.8176</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>165.4</v>
+        <v>159.21</v>
       </c>
       <c r="C12" t="n">
-        <v>171.88</v>
+        <v>176.75</v>
       </c>
       <c r="D12" t="n">
-        <v>150.08</v>
+        <v>158.87</v>
       </c>
       <c r="E12" t="n">
-        <v>165.28</v>
+        <v>174.82</v>
       </c>
       <c r="F12" t="n">
-        <v>73.7</v>
+        <v>70.8</v>
       </c>
       <c r="G12" t="n">
-        <v>74.39</v>
+        <v>73.02</v>
       </c>
       <c r="H12" t="n">
-        <v>70.76000000000001</v>
+        <v>69.56999999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>72.23</v>
+        <v>72.72</v>
       </c>
       <c r="J12" t="n">
-        <v>48</v>
+        <v>49.8</v>
       </c>
       <c r="K12" t="n">
-        <v>51.4</v>
+        <v>49.9</v>
       </c>
       <c r="L12" t="n">
-        <v>46.6</v>
+        <v>44.6</v>
       </c>
       <c r="M12" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="N12" t="n">
-        <v>39.64</v>
+        <v>41.18</v>
       </c>
       <c r="O12" t="n">
-        <v>41.11</v>
+        <v>41.86</v>
       </c>
       <c r="P12" t="n">
-        <v>39.29</v>
+        <v>39.93</v>
       </c>
       <c r="Q12" t="n">
-        <v>40.38</v>
+        <v>40.08</v>
       </c>
       <c r="R12" t="n">
-        <v>-15.0886</v>
+        <v>5.772</v>
       </c>
       <c r="S12" t="n">
-        <v>-24.0267</v>
+        <v>-3.6645</v>
       </c>
       <c r="T12" t="n">
-        <v>-30.1201</v>
+        <v>-34.4532</v>
       </c>
       <c r="U12" t="n">
-        <v>-5.4829</v>
+        <v>0.6784</v>
       </c>
       <c r="V12" t="n">
-        <v>-6.7519</v>
+        <v>-0.8589</v>
       </c>
       <c r="W12" t="n">
-        <v>-6.4257</v>
+        <v>-10.2222</v>
       </c>
       <c r="X12" t="n">
-        <v>15.1079</v>
+        <v>-6.25</v>
       </c>
       <c r="Y12" t="n">
-        <v>24.3523</v>
+        <v>-0.2217</v>
       </c>
       <c r="Z12" t="n">
-        <v>29.0323</v>
+        <v>38.8889</v>
       </c>
       <c r="AA12" t="n">
-        <v>5.4859</v>
+        <v>-0.7429</v>
       </c>
       <c r="AB12" t="n">
-        <v>6.5998</v>
+        <v>0.3254</v>
       </c>
       <c r="AC12" t="n">
-        <v>5.8176</v>
+        <v>10.3828</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>159.21</v>
+        <v>199.81</v>
       </c>
       <c r="C13" t="n">
-        <v>176.75</v>
+        <v>204.55</v>
       </c>
       <c r="D13" t="n">
-        <v>158.87</v>
+        <v>189.46</v>
       </c>
       <c r="E13" t="n">
-        <v>174.82</v>
+        <v>192.45</v>
       </c>
       <c r="F13" t="n">
-        <v>70.8</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>73.02</v>
+        <v>76.69</v>
       </c>
       <c r="H13" t="n">
-        <v>69.56999999999999</v>
+        <v>73.89</v>
       </c>
       <c r="I13" t="n">
-        <v>72.72</v>
+        <v>76.34</v>
       </c>
       <c r="J13" t="n">
-        <v>49.8</v>
+        <v>38.7</v>
       </c>
       <c r="K13" t="n">
-        <v>49.9</v>
+        <v>41.2</v>
       </c>
       <c r="L13" t="n">
-        <v>44.6</v>
+        <v>37.5</v>
       </c>
       <c r="M13" t="n">
-        <v>45</v>
+        <v>40.7</v>
       </c>
       <c r="N13" t="n">
-        <v>41.18</v>
+        <v>38.93</v>
       </c>
       <c r="O13" t="n">
-        <v>41.86</v>
+        <v>39.47</v>
       </c>
       <c r="P13" t="n">
-        <v>39.93</v>
+        <v>37.93</v>
       </c>
       <c r="Q13" t="n">
-        <v>40.08</v>
+        <v>38.1</v>
       </c>
       <c r="R13" t="n">
-        <v>5.772</v>
+        <v>10.0847</v>
       </c>
       <c r="S13" t="n">
-        <v>-3.6645</v>
+        <v>-1.1302</v>
       </c>
       <c r="T13" t="n">
-        <v>-34.4532</v>
+        <v>-11.5376</v>
       </c>
       <c r="U13" t="n">
-        <v>0.6784</v>
+        <v>4.978</v>
       </c>
       <c r="V13" t="n">
-        <v>-0.8589</v>
+        <v>-0.1047</v>
       </c>
       <c r="W13" t="n">
-        <v>-10.2222</v>
+        <v>-1.4459</v>
       </c>
       <c r="X13" t="n">
-        <v>-6.25</v>
+        <v>-9.5556</v>
       </c>
       <c r="Y13" t="n">
-        <v>-0.2217</v>
+        <v>-2.3981</v>
       </c>
       <c r="Z13" t="n">
-        <v>38.8889</v>
+        <v>5.4404</v>
       </c>
       <c r="AA13" t="n">
-        <v>-0.7429</v>
+        <v>-4.9401</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.3254</v>
+        <v>-0.4702</v>
       </c>
       <c r="AC13" t="n">
-        <v>10.3828</v>
+        <v>0.5808</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>199.81</v>
+        <v>182.4</v>
       </c>
       <c r="C14" t="n">
-        <v>204.55</v>
+        <v>195.94</v>
       </c>
       <c r="D14" t="n">
-        <v>189.46</v>
+        <v>176.8</v>
       </c>
       <c r="E14" t="n">
-        <v>192.45</v>
+        <v>192.26</v>
       </c>
       <c r="F14" t="n">
-        <v>74.84999999999999</v>
+        <v>75.53</v>
       </c>
       <c r="G14" t="n">
-        <v>76.69</v>
+        <v>77.31999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>73.89</v>
+        <v>74.33</v>
       </c>
       <c r="I14" t="n">
-        <v>76.34</v>
+        <v>77.03</v>
       </c>
       <c r="J14" t="n">
-        <v>38.7</v>
+        <v>42.7</v>
       </c>
       <c r="K14" t="n">
-        <v>41.2</v>
+        <v>43.9</v>
       </c>
       <c r="L14" t="n">
-        <v>37.5</v>
+        <v>39.9</v>
       </c>
       <c r="M14" t="n">
-        <v>40.7</v>
+        <v>40.8</v>
       </c>
       <c r="N14" t="n">
-        <v>38.93</v>
+        <v>38.49</v>
       </c>
       <c r="O14" t="n">
-        <v>39.47</v>
+        <v>39.14</v>
       </c>
       <c r="P14" t="n">
-        <v>37.93</v>
+        <v>37.64</v>
       </c>
       <c r="Q14" t="n">
-        <v>38.1</v>
+        <v>37.78</v>
       </c>
       <c r="R14" t="n">
-        <v>10.0847</v>
+        <v>-0.0987</v>
       </c>
       <c r="S14" t="n">
-        <v>-1.1302</v>
+        <v>16.3238</v>
       </c>
       <c r="T14" t="n">
-        <v>-11.5376</v>
+        <v>5.9459</v>
       </c>
       <c r="U14" t="n">
-        <v>4.978</v>
+        <v>0.9039</v>
       </c>
       <c r="V14" t="n">
-        <v>-0.1047</v>
+        <v>6.6454</v>
       </c>
       <c r="W14" t="n">
-        <v>-1.4459</v>
+        <v>5.017</v>
       </c>
       <c r="X14" t="n">
-        <v>-9.5556</v>
+        <v>0.2457</v>
       </c>
       <c r="Y14" t="n">
-        <v>-2.3981</v>
+        <v>-15</v>
       </c>
       <c r="Z14" t="n">
-        <v>5.4404</v>
+        <v>-9.5344</v>
       </c>
       <c r="AA14" t="n">
-        <v>-4.9401</v>
+        <v>-0.8399</v>
       </c>
       <c r="AB14" t="n">
-        <v>-0.4702</v>
+        <v>-6.4388</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.5808</v>
+        <v>-5.4318</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>182.4</v>
+        <v>174.61</v>
       </c>
       <c r="C15" t="n">
-        <v>195.94</v>
+        <v>177.67</v>
       </c>
       <c r="D15" t="n">
-        <v>176.8</v>
+        <v>161.55</v>
       </c>
       <c r="E15" t="n">
-        <v>192.26</v>
+        <v>165.37</v>
       </c>
       <c r="F15" t="n">
-        <v>75.53</v>
+        <v>74.54000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>77.31999999999999</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="H15" t="n">
-        <v>74.33</v>
+        <v>72.09</v>
       </c>
       <c r="I15" t="n">
-        <v>77.03</v>
+        <v>72.64</v>
       </c>
       <c r="J15" t="n">
-        <v>42.7</v>
+        <v>44.4</v>
       </c>
       <c r="K15" t="n">
-        <v>43.9</v>
+        <v>47.3</v>
       </c>
       <c r="L15" t="n">
-        <v>39.9</v>
+        <v>43.8</v>
       </c>
       <c r="M15" t="n">
-        <v>40.8</v>
+        <v>46.5</v>
       </c>
       <c r="N15" t="n">
-        <v>38.49</v>
+        <v>39.01</v>
       </c>
       <c r="O15" t="n">
-        <v>39.14</v>
+        <v>40.21</v>
       </c>
       <c r="P15" t="n">
-        <v>37.64</v>
+        <v>38.85</v>
       </c>
       <c r="Q15" t="n">
-        <v>37.78</v>
+        <v>39.95</v>
       </c>
       <c r="R15" t="n">
-        <v>-0.0987</v>
+        <v>-13.9863</v>
       </c>
       <c r="S15" t="n">
-        <v>16.3238</v>
+        <v>-5.4056</v>
       </c>
       <c r="T15" t="n">
-        <v>5.9459</v>
+        <v>-15.0424</v>
       </c>
       <c r="U15" t="n">
-        <v>0.9039</v>
+        <v>-5.6991</v>
       </c>
       <c r="V15" t="n">
-        <v>6.6454</v>
+        <v>-0.11</v>
       </c>
       <c r="W15" t="n">
-        <v>5.017</v>
+        <v>-4.9463</v>
       </c>
       <c r="X15" t="n">
-        <v>0.2457</v>
+        <v>13.9706</v>
       </c>
       <c r="Y15" t="n">
-        <v>-15</v>
+        <v>3.3333</v>
       </c>
       <c r="Z15" t="n">
-        <v>-9.5344</v>
+        <v>11.5108</v>
       </c>
       <c r="AA15" t="n">
-        <v>-0.8399</v>
+        <v>5.7438</v>
       </c>
       <c r="AB15" t="n">
-        <v>-6.4388</v>
+        <v>-0.3244</v>
       </c>
       <c r="AC15" t="n">
-        <v>-5.4318</v>
+        <v>4.3626</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>174.61</v>
+        <v>187.69</v>
       </c>
       <c r="C16" t="n">
-        <v>177.67</v>
+        <v>188.43</v>
       </c>
       <c r="D16" t="n">
-        <v>161.55</v>
+        <v>170.26</v>
       </c>
       <c r="E16" t="n">
-        <v>165.37</v>
+        <v>176.66</v>
       </c>
       <c r="F16" t="n">
-        <v>74.54000000000001</v>
+        <v>75.2</v>
       </c>
       <c r="G16" t="n">
-        <v>74.84999999999999</v>
+        <v>75.84999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>72.09</v>
+        <v>73.41</v>
       </c>
       <c r="I16" t="n">
-        <v>72.64</v>
+        <v>75.02</v>
       </c>
       <c r="J16" t="n">
-        <v>44.4</v>
+        <v>39.7</v>
       </c>
       <c r="K16" t="n">
-        <v>47.3</v>
+        <v>45</v>
       </c>
       <c r="L16" t="n">
-        <v>43.8</v>
+        <v>39.7</v>
       </c>
       <c r="M16" t="n">
-        <v>46.5</v>
+        <v>42.8</v>
       </c>
       <c r="N16" t="n">
-        <v>39.01</v>
+        <v>38.54</v>
       </c>
       <c r="O16" t="n">
-        <v>40.21</v>
+        <v>39.53</v>
       </c>
       <c r="P16" t="n">
-        <v>38.85</v>
+        <v>38.19</v>
       </c>
       <c r="Q16" t="n">
-        <v>39.95</v>
+        <v>38.63</v>
       </c>
       <c r="R16" t="n">
-        <v>-13.9863</v>
+        <v>6.8271</v>
       </c>
       <c r="S16" t="n">
-        <v>-5.4056</v>
+        <v>-8.204700000000001</v>
       </c>
       <c r="T16" t="n">
-        <v>-15.0424</v>
+        <v>6.8853</v>
       </c>
       <c r="U16" t="n">
-        <v>-5.6991</v>
+        <v>3.2764</v>
       </c>
       <c r="V16" t="n">
-        <v>-0.11</v>
+        <v>-1.7291</v>
       </c>
       <c r="W16" t="n">
-        <v>-4.9463</v>
+        <v>3.8627</v>
       </c>
       <c r="X16" t="n">
-        <v>13.9706</v>
+        <v>-7.957</v>
       </c>
       <c r="Y16" t="n">
-        <v>3.3333</v>
+        <v>5.1597</v>
       </c>
       <c r="Z16" t="n">
-        <v>11.5108</v>
+        <v>-10.8333</v>
       </c>
       <c r="AA16" t="n">
-        <v>5.7438</v>
+        <v>-3.3041</v>
       </c>
       <c r="AB16" t="n">
-        <v>-0.3244</v>
+        <v>1.3911</v>
       </c>
       <c r="AC16" t="n">
-        <v>4.3626</v>
+        <v>-4.3338</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>187.69</v>
+        <v>183.77</v>
       </c>
       <c r="C17" t="n">
-        <v>188.43</v>
+        <v>184</v>
       </c>
       <c r="D17" t="n">
-        <v>170.26</v>
+        <v>150</v>
       </c>
       <c r="E17" t="n">
-        <v>176.66</v>
+        <v>165.55</v>
       </c>
       <c r="F17" t="n">
-        <v>75.2</v>
+        <v>76.29000000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>75.84999999999999</v>
+        <v>76.47</v>
       </c>
       <c r="H17" t="n">
-        <v>73.41</v>
+        <v>72.06</v>
       </c>
       <c r="I17" t="n">
-        <v>75.02</v>
+        <v>74.44</v>
       </c>
       <c r="J17" t="n">
-        <v>39.7</v>
+        <v>41.23</v>
       </c>
       <c r="K17" t="n">
-        <v>45</v>
+        <v>49.69</v>
       </c>
       <c r="L17" t="n">
-        <v>39.7</v>
+        <v>41.16</v>
       </c>
       <c r="M17" t="n">
-        <v>42.8</v>
+        <v>45.98</v>
       </c>
       <c r="N17" t="n">
-        <v>38.54</v>
+        <v>37.98</v>
       </c>
       <c r="O17" t="n">
-        <v>39.53</v>
+        <v>40.17</v>
       </c>
       <c r="P17" t="n">
-        <v>38.19</v>
+        <v>37.89</v>
       </c>
       <c r="Q17" t="n">
-        <v>38.63</v>
+        <v>38.94</v>
       </c>
       <c r="R17" t="n">
-        <v>6.8271</v>
+        <v>-6.2889</v>
       </c>
       <c r="S17" t="n">
-        <v>-8.204700000000001</v>
+        <v>-13.8926</v>
       </c>
       <c r="T17" t="n">
-        <v>6.8853</v>
+        <v>-5.3026</v>
       </c>
       <c r="U17" t="n">
-        <v>3.2764</v>
+        <v>-0.7731</v>
       </c>
       <c r="V17" t="n">
-        <v>-1.7291</v>
+        <v>-3.3623</v>
       </c>
       <c r="W17" t="n">
-        <v>3.8627</v>
+        <v>2.3652</v>
       </c>
       <c r="X17" t="n">
-        <v>-7.957</v>
+        <v>7.4299</v>
       </c>
       <c r="Y17" t="n">
-        <v>5.1597</v>
+        <v>12.6961</v>
       </c>
       <c r="Z17" t="n">
-        <v>-10.8333</v>
+        <v>2.1778</v>
       </c>
       <c r="AA17" t="n">
-        <v>-3.3041</v>
+        <v>0.8025</v>
       </c>
       <c r="AB17" t="n">
-        <v>1.3911</v>
+        <v>3.0704</v>
       </c>
       <c r="AC17" t="n">
-        <v>-4.3338</v>
+        <v>-2.8443</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>183.77</v>
+        <v>150.44</v>
       </c>
       <c r="C18" t="n">
-        <v>184</v>
+        <v>155.83</v>
       </c>
       <c r="D18" t="n">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="E18" t="n">
-        <v>165.55</v>
+        <v>142.48</v>
       </c>
       <c r="F18" t="n">
-        <v>76.29000000000001</v>
+        <v>72.61</v>
       </c>
       <c r="G18" t="n">
-        <v>76.47</v>
+        <v>73.12</v>
       </c>
       <c r="H18" t="n">
-        <v>72.06</v>
+        <v>69.69</v>
       </c>
       <c r="I18" t="n">
-        <v>74.44</v>
+        <v>70.73999999999999</v>
       </c>
       <c r="J18" t="n">
-        <v>41.23</v>
+        <v>49.77</v>
       </c>
       <c r="K18" t="n">
-        <v>49.69</v>
+        <v>53.34</v>
       </c>
       <c r="L18" t="n">
-        <v>41.16</v>
+        <v>48.31</v>
       </c>
       <c r="M18" t="n">
-        <v>45.98</v>
+        <v>52.02</v>
       </c>
       <c r="N18" t="n">
-        <v>37.98</v>
+        <v>39.9</v>
       </c>
       <c r="O18" t="n">
-        <v>40.17</v>
+        <v>41.44</v>
       </c>
       <c r="P18" t="n">
-        <v>37.89</v>
+        <v>39.65</v>
       </c>
       <c r="Q18" t="n">
-        <v>38.94</v>
+        <v>40.89</v>
       </c>
       <c r="R18" t="n">
-        <v>-6.2889</v>
+        <v>-13.9354</v>
       </c>
       <c r="S18" t="n">
-        <v>-13.8926</v>
+        <v>-13.8417</v>
       </c>
       <c r="T18" t="n">
-        <v>-5.3026</v>
+        <v>-25.9652</v>
       </c>
       <c r="U18" t="n">
-        <v>-0.7731</v>
+        <v>-4.9704</v>
       </c>
       <c r="V18" t="n">
-        <v>-3.3623</v>
+        <v>-2.6156</v>
       </c>
       <c r="W18" t="n">
-        <v>2.3652</v>
+        <v>-7.3356</v>
       </c>
       <c r="X18" t="n">
-        <v>7.4299</v>
+        <v>13.1361</v>
       </c>
       <c r="Y18" t="n">
-        <v>12.6961</v>
+        <v>11.871</v>
       </c>
       <c r="Z18" t="n">
-        <v>2.1778</v>
+        <v>27.8133</v>
       </c>
       <c r="AA18" t="n">
-        <v>0.8025</v>
+        <v>5.0077</v>
       </c>
       <c r="AB18" t="n">
-        <v>3.0704</v>
+        <v>2.3529</v>
       </c>
       <c r="AC18" t="n">
-        <v>-2.8443</v>
+        <v>7.3228</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>150.44</v>
+        <v>124.73</v>
       </c>
       <c r="C19" t="n">
-        <v>155.83</v>
+        <v>144.4</v>
       </c>
       <c r="D19" t="n">
-        <v>138</v>
+        <v>116.47</v>
       </c>
       <c r="E19" t="n">
-        <v>142.48</v>
+        <v>135.47</v>
       </c>
       <c r="F19" t="n">
-        <v>72.61</v>
+        <v>66.38</v>
       </c>
       <c r="G19" t="n">
-        <v>73.12</v>
+        <v>69.56</v>
       </c>
       <c r="H19" t="n">
-        <v>69.69</v>
+        <v>64.91</v>
       </c>
       <c r="I19" t="n">
-        <v>70.73999999999999</v>
+        <v>67.53</v>
       </c>
       <c r="J19" t="n">
-        <v>49.77</v>
+        <v>58.59</v>
       </c>
       <c r="K19" t="n">
-        <v>53.34</v>
+        <v>61.6</v>
       </c>
       <c r="L19" t="n">
-        <v>48.31</v>
+        <v>51.34</v>
       </c>
       <c r="M19" t="n">
-        <v>52.02</v>
+        <v>54.85</v>
       </c>
       <c r="N19" t="n">
-        <v>39.9</v>
+        <v>43.43</v>
       </c>
       <c r="O19" t="n">
-        <v>41.44</v>
+        <v>44.27</v>
       </c>
       <c r="P19" t="n">
-        <v>39.65</v>
+        <v>41.59</v>
       </c>
       <c r="Q19" t="n">
-        <v>40.89</v>
+        <v>42.79</v>
       </c>
       <c r="R19" t="n">
-        <v>-13.9354</v>
+        <v>-4.92</v>
       </c>
       <c r="S19" t="n">
-        <v>-13.8417</v>
+        <v>-23.316</v>
       </c>
       <c r="T19" t="n">
-        <v>-25.9652</v>
+        <v>-29.5381</v>
       </c>
       <c r="U19" t="n">
-        <v>-4.9704</v>
+        <v>-4.5377</v>
       </c>
       <c r="V19" t="n">
-        <v>-2.6156</v>
+        <v>-9.984</v>
       </c>
       <c r="W19" t="n">
-        <v>-7.3356</v>
+        <v>-12.3329</v>
       </c>
       <c r="X19" t="n">
-        <v>13.1361</v>
+        <v>5.4402</v>
       </c>
       <c r="Y19" t="n">
-        <v>11.871</v>
+        <v>28.1542</v>
       </c>
       <c r="Z19" t="n">
-        <v>27.8133</v>
+        <v>34.4363</v>
       </c>
       <c r="AA19" t="n">
-        <v>5.0077</v>
+        <v>4.6466</v>
       </c>
       <c r="AB19" t="n">
-        <v>2.3529</v>
+        <v>10.7688</v>
       </c>
       <c r="AC19" t="n">
-        <v>7.3228</v>
+        <v>13.261</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>124.73</v>
+        <v>143.52</v>
       </c>
 